<commit_message>
Record P2-10 progress: provider pinning and the output guard.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/production-readiness.xlsx
+++ b/docs/production-readiness.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'任務清單'!$A$1:$P$56</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'待確認問題'!$A$1:$G$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$115</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$117</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -641,7 +641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I79"/>
+  <dimension ref="A1:I80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -665,7 +665,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>最後更新：2026-10-07 21:39　·　本頁由 tracker.py 自動生成，請勿手動編輯</t>
+          <t>最後更新：2026-10-07 22:04　·　本頁由 tracker.py 自動生成，請勿手動編輯</t>
         </is>
       </c>
     </row>
@@ -820,11 +820,11 @@
       </c>
       <c r="D8" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A8,'任務清單'!$F:$F,D$5)</f>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E8" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A8,'任務清單'!$F:$F,E$5)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F8" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A8,'任務清單'!$F:$F,F$5)</f>
@@ -896,11 +896,11 @@
       </c>
       <c r="D10" s="5">
         <f>SUM(D6:D9)</f>
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E10" s="5">
         <f>SUM(E6:E9)</f>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F10" s="5">
         <f>SUM(F6:F9)</f>
@@ -983,11 +983,11 @@
       </c>
       <c r="D13" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A13,'任務清單'!$F:$F,D$12)</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E13" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A13,'任務清單'!$F:$F,E$12)</f>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F13" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A13,'任務清單'!$F:$F,F$12)</f>
@@ -1139,11 +1139,11 @@
       </c>
       <c r="D17" s="5">
         <f>SUM(D13:D16)</f>
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E17" s="5">
         <f>SUM(E13:E16)</f>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F17" s="5">
         <f>SUM(F13:F16)</f>
@@ -1584,15 +1584,15 @@
       <c r="H32" s="11" t="n"/>
       <c r="I32" s="12" t="n"/>
     </row>
-    <row r="33" ht="60" customHeight="1">
+    <row r="33" ht="228" customHeight="1">
       <c r="A33" s="13" t="inlineStr">
         <is>
-          <t>R-01</t>
+          <t>P2-10</t>
         </is>
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>選定量產板子</t>
+          <t>DeepSeek v4 flash 經 OpenRouter 時固定可用的供應商</t>
         </is>
       </c>
       <c r="C33" s="13" t="inlineStr">
@@ -1607,7 +1607,8 @@
       </c>
       <c r="E33" s="6" t="inlineStr">
         <is>
-          <t>已定案 Spotpear AI Toy（用戶 10/07 決定）；評分表 ①–⑦ 在 Spotpear 上實測並記錄結果，沒有否決性問題（如 2 小時內 OOM 重啟、C3 無法啟用 Secure Boot v2＋Flash 加密、無認證模組）。</t>
+          <t>上次測試：部分通過 — ① 16 家供應商各 20 次真實 session prompt（含開場白，串流，order=[x]+allow_fallbacks=false）：建議清單 azure/alibaba/novita/siliconflow/gmicloud 各 20/20，0 空內容 0 特殊 token，首字 p50 1.25/2.33/2.59/2.56/3.25s；只設 order 時 order=[deepinfra] 實際由 Relace 回應（回過 content=None）→ 已改為 allow_fallbacks=false。伺服器端 LLMOutputGuard：pytest 8 項（尾部/跨 chunk 拆開的 token、空回應記警告）全套 203 passed；真實 LLM 串流經 guard 6 角色 12/12 正常、無誤觸發。② 實機 5 次開場白未做
+線上用 DeepSeek 時，provider_order 只列實測正常的供應商（例如 StreamLake、SiliconFlow、GMICloud、Novita），並開 reasoning；或線上改用 gemma-4-26b。伺服器遇到空回應或特殊 token 時不把它送去 TTS。</t>
         </is>
       </c>
       <c r="F33" s="11" t="n"/>
@@ -1615,15 +1616,15 @@
       <c r="H33" s="11" t="n"/>
       <c r="I33" s="12" t="n"/>
     </row>
-    <row r="34" ht="172" customHeight="1">
+    <row r="34" ht="60" customHeight="1">
       <c r="A34" s="13" t="inlineStr">
         <is>
-          <t>R-02</t>
+          <t>R-01</t>
         </is>
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>角色收窄到 5–8 個粵語陪伴角色</t>
+          <t>選定量產板子</t>
         </is>
       </c>
       <c r="C34" s="13" t="inlineStr">
@@ -1638,8 +1639,7 @@
       </c>
       <c r="E34" s="6" t="inlineStr">
         <is>
-          <t>上次測試：通過 — 用戶已確認角色陣容。本地 DB：① 未隱藏內建角色只剩 hk_ 6 個 ② localhost:3100 Children 頁只見 6 個、Story 頁只見叮叮兔/咪咪貓 ③ 每角色 10 句粵語，prompt 用伺服器同一套組裝、開場白按 pipecat 以 user 角色送出：gemma-4-26b 65/66 合格（1 句 4 句/2 問）；DeepSeek v4 flash 預設 reasoning 61/66（超標都只多 1–2 句）；全部無簡體、恐怖、拼字
-只保留 5–8 個自己設計的粵語陪伴角色，其餘設為 is_hidden；每個角色按 3–6 歲設計：句子短、用詞簡單、一次只問一個問題，不講恐怖、暴力或需要識字的內容。</t>
+          <t>已定案 Spotpear AI Toy（用戶 10/07 決定）；評分表 ①–⑦ 在 Spotpear 上實測並記錄結果，沒有否決性問題（如 2 小時內 OOM 重啟、C3 無法啟用 Secure Boot v2＋Flash 加密、無認證模組）。</t>
         </is>
       </c>
       <c r="F34" s="11" t="n"/>
@@ -1647,15 +1647,15 @@
       <c r="H34" s="11" t="n"/>
       <c r="I34" s="12" t="n"/>
     </row>
-    <row r="35" ht="74" customHeight="1">
+    <row r="35" ht="172" customHeight="1">
       <c r="A35" s="13" t="inlineStr">
         <is>
-          <t>P2-10</t>
+          <t>R-02</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>DeepSeek v4 flash 經 OpenRouter 時固定可用的供應商</t>
+          <t>角色收窄到 5–8 個粵語陪伴角色</t>
         </is>
       </c>
       <c r="C35" s="13" t="inlineStr">
@@ -1665,12 +1665,13 @@
       </c>
       <c r="D35" s="13" t="inlineStr">
         <is>
-          <t>未開始</t>
+          <t>進行中</t>
         </is>
       </c>
       <c r="E35" s="6" t="inlineStr">
         <is>
-          <t>線上用 DeepSeek 時，provider_order 只列實測正常的供應商（例如 StreamLake、SiliconFlow、GMICloud、Novita），並開 reasoning；或線上改用 gemma-4-26b。伺服器遇到空回應或特殊 token 時不把它送去 TTS。</t>
+          <t>上次測試：通過 — 用戶已確認角色陣容。本地 DB：① 未隱藏內建角色只剩 hk_ 6 個 ② localhost:3100 Children 頁只見 6 個、Story 頁只見叮叮兔/咪咪貓 ③ 每角色 10 句粵語，prompt 用伺服器同一套組裝、開場白按 pipecat 以 user 角色送出：gemma-4-26b 65/66 合格（1 句 4 句/2 問）；DeepSeek v4 flash 預設 reasoning 61/66（超標都只多 1–2 句）；全部無簡體、恐怖、拼字
+只保留 5–8 個自己設計的粵語陪伴角色，其餘設為 is_hidden；每個角色按 3–6 歲設計：句子短、用詞簡單、一次只問一個問題，不講恐怖、暴力或需要識字的內容。</t>
         </is>
       </c>
       <c r="F35" s="11" t="n"/>
@@ -1833,68 +1834,68 @@
       <c r="H40" s="11" t="n"/>
       <c r="I40" s="12" t="n"/>
     </row>
-    <row r="42">
-      <c r="A42" s="10" t="inlineStr">
+    <row r="41" ht="46" customHeight="1">
+      <c r="A41" s="13" t="inlineStr">
+        <is>
+          <t>P2-02</t>
+        </is>
+      </c>
+      <c r="B41" s="6" t="inlineStr">
+        <is>
+          <t>CI 跑測試與靜態檢查</t>
+        </is>
+      </c>
+      <c r="C41" s="13" t="inlineStr">
+        <is>
+          <t>2 內測準備</t>
+        </is>
+      </c>
+      <c r="D41" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E41" s="6" t="inlineStr">
+        <is>
+          <t>推送與 PR 時跑 pytest、ruff、pyright、next lint、tsc --noEmit、pio run；任何一項失敗就不發佈 image。</t>
+        </is>
+      </c>
+      <c r="F41" s="11" t="n"/>
+      <c r="G41" s="11" t="n"/>
+      <c r="H41" s="11" t="n"/>
+      <c r="I41" s="12" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="10" t="inlineStr">
         <is>
           <t>✅ 最近完成與測試效果</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="4" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
         <is>
           <t>編號</t>
         </is>
       </c>
-      <c r="B43" s="4" t="inlineStr">
+      <c r="B44" s="4" t="inlineStr">
         <is>
           <t>任務</t>
         </is>
       </c>
-      <c r="C43" s="4" t="inlineStr">
+      <c r="C44" s="4" t="inlineStr">
         <is>
           <t>測試結果</t>
         </is>
       </c>
-      <c r="D43" s="4" t="inlineStr">
+      <c r="D44" s="4" t="inlineStr">
         <is>
           <t>完成日期</t>
         </is>
       </c>
-      <c r="E43" s="4" t="inlineStr">
+      <c r="E44" s="4" t="inlineStr">
         <is>
           <t>測試證據</t>
-        </is>
-      </c>
-      <c r="F43" s="11" t="n"/>
-      <c r="G43" s="11" t="n"/>
-      <c r="H43" s="11" t="n"/>
-      <c r="I43" s="12" t="n"/>
-    </row>
-    <row r="44" ht="88" customHeight="1">
-      <c r="A44" s="13" t="inlineStr">
-        <is>
-          <t>R-03</t>
-        </is>
-      </c>
-      <c r="B44" s="6" t="inlineStr">
-        <is>
-          <t>移除不用的 Deno／Cloudflare 後端與上游預設主機</t>
-        </is>
-      </c>
-      <c r="C44" s="13" t="inlineStr">
-        <is>
-          <t>通過</t>
-        </is>
-      </c>
-      <c r="D44" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-07</t>
-        </is>
-      </c>
-      <c r="E44" s="6" t="inlineStr">
-        <is>
-          <t>① grep deno.dev|workers.dev|railway.app|VOICE_SERVER_DENO|VOICE_SERVER_CLOUDFLARE 全 repo → 只剩 seed.json 的任務描述本身 ② pio run 18 個 env 全 SUCCESS（S3 devkit/Waveshare/xmini-c3/Spotpear 各變體）③ FastAPI pytest 182 passed；另 tsc --noEmit 通過</t>
         </is>
       </c>
       <c r="F44" s="11" t="n"/>
@@ -1905,12 +1906,12 @@
     <row r="45" ht="88" customHeight="1">
       <c r="A45" s="13" t="inlineStr">
         <is>
-          <t>P2-01</t>
+          <t>R-03</t>
         </is>
       </c>
       <c r="B45" s="6" t="inlineStr">
         <is>
-          <t>修好後端測試環境</t>
+          <t>移除不用的 Deno／Cloudflare 後端與上游預設主機</t>
         </is>
       </c>
       <c r="C45" s="13" t="inlineStr">
@@ -1925,7 +1926,7 @@
       </c>
       <c r="E45" s="6" t="inlineStr">
         <is>
-          <t>cd server/fastapi &amp;&amp; .venv/bin/python -m pytest -q → 173 passed（原本 60 個 async 測試報「not natively supported」）；pyproject dev group 加 pytest&gt;=9,&lt;10、pytest-asyncio&gt;=1.4,&lt;2，asyncio_mode=auto；pip install --dry-run --group dev 可解析</t>
+          <t>① grep deno.dev|workers.dev|railway.app|VOICE_SERVER_DENO|VOICE_SERVER_CLOUDFLARE 全 repo → 只剩 seed.json 的任務描述本身 ② pio run 18 個 env 全 SUCCESS（S3 devkit/Waveshare/xmini-c3/Spotpear 各變體）③ FastAPI pytest 182 passed；另 tsc --noEmit 通過</t>
         </is>
       </c>
       <c r="F45" s="11" t="n"/>
@@ -1933,15 +1934,15 @@
       <c r="H45" s="11" t="n"/>
       <c r="I45" s="12" t="n"/>
     </row>
-    <row r="46" ht="60" customHeight="1">
+    <row r="46" ht="88" customHeight="1">
       <c r="A46" s="13" t="inlineStr">
         <is>
-          <t>P2-03</t>
+          <t>P2-01</t>
         </is>
       </c>
       <c r="B46" s="6" t="inlineStr">
         <is>
-          <t>提交目前未提交的改動</t>
+          <t>修好後端測試環境</t>
         </is>
       </c>
       <c r="C46" s="13" t="inlineStr">
@@ -1951,12 +1952,12 @@
       </c>
       <c r="D46" s="13" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="E46" s="6" t="inlineStr">
         <is>
-          <t>git status --short → 0 行；3bc7119..b322375 按主題拆成 5 個 commit（50 檔：xmini-c3 電量、facts 記憶層、日期時間天氣、BEAM 評測、進度追蹤）；git ls-remote mygithub main = HEAD = b322375</t>
+          <t>cd server/fastapi &amp;&amp; .venv/bin/python -m pytest -q → 173 passed（原本 60 個 async 測試報「not natively supported」）；pyproject dev group 加 pytest&gt;=9,&lt;10、pytest-asyncio&gt;=1.4,&lt;2，asyncio_mode=auto；pip install --dry-run --group dev 可解析</t>
         </is>
       </c>
       <c r="F46" s="11" t="n"/>
@@ -1964,50 +1965,58 @@
       <c r="H46" s="11" t="n"/>
       <c r="I46" s="12" t="n"/>
     </row>
-    <row r="48">
-      <c r="A48" s="10" t="inlineStr">
+    <row r="47" ht="60" customHeight="1">
+      <c r="A47" s="13" t="inlineStr">
+        <is>
+          <t>P2-03</t>
+        </is>
+      </c>
+      <c r="B47" s="6" t="inlineStr">
+        <is>
+          <t>提交目前未提交的改動</t>
+        </is>
+      </c>
+      <c r="C47" s="13" t="inlineStr">
+        <is>
+          <t>通過</t>
+        </is>
+      </c>
+      <c r="D47" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="E47" s="6" t="inlineStr">
+        <is>
+          <t>git status --short → 0 行；3bc7119..b322375 按主題拆成 5 個 commit（50 檔：xmini-c3 電量、facts 記憶層、日期時間天氣、BEAM 評測、進度追蹤）；git ls-remote mygithub main = HEAD = b322375</t>
+        </is>
+      </c>
+      <c r="F47" s="11" t="n"/>
+      <c r="G47" s="11" t="n"/>
+      <c r="H47" s="11" t="n"/>
+      <c r="I47" s="12" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="10" t="inlineStr">
         <is>
           <t>⏳ 等待依賴 / ⛔ 阻塞</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="4" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
         <is>
           <t>編號</t>
         </is>
       </c>
-      <c r="B49" s="4" t="inlineStr">
+      <c r="B50" s="4" t="inlineStr">
         <is>
           <t>任務</t>
         </is>
       </c>
-      <c r="C49" s="4" t="inlineStr">
+      <c r="C50" s="4" t="inlineStr">
         <is>
           <t>在等什麼</t>
-        </is>
-      </c>
-      <c r="D49" s="11" t="n"/>
-      <c r="E49" s="11" t="n"/>
-      <c r="F49" s="11" t="n"/>
-      <c r="G49" s="11" t="n"/>
-      <c r="H49" s="11" t="n"/>
-      <c r="I49" s="12" t="n"/>
-    </row>
-    <row r="50" ht="60" customHeight="1">
-      <c r="A50" s="13" t="inlineStr">
-        <is>
-          <t>R-16</t>
-        </is>
-      </c>
-      <c r="B50" s="6" t="inlineStr">
-        <is>
-          <t>Spotpear 量產版加電池電壓檢測（GPIO0 分壓）</t>
-        </is>
-      </c>
-      <c r="C50" s="6" t="inlineStr">
-        <is>
-          <t>阻塞：[2026-10-07] 仍按 10/06 決定暫緩：等用戶做充滿再放電測試（與 R-17 同一次），看 VDD 低電提醒在關機前多久觸發；太遲或不觸發才向 Spotpear 提改板。已把分壓改板的問題一併放進給 Spotpear 的草稿，方便同一封發出</t>
         </is>
       </c>
       <c r="D50" s="11" t="n"/>
@@ -2017,20 +2026,20 @@
       <c r="H50" s="11" t="n"/>
       <c r="I50" s="12" t="n"/>
     </row>
-    <row r="51" ht="88" customHeight="1">
+    <row r="51" ht="60" customHeight="1">
       <c r="A51" s="13" t="inlineStr">
         <is>
-          <t>R-17</t>
+          <t>R-16</t>
         </is>
       </c>
       <c r="B51" s="6" t="inlineStr">
         <is>
-          <t>Spotpear 電池耗盡時插電能否正常開機（供電路徑）</t>
+          <t>Spotpear 量產版加電池電壓檢測（GPIO0 分壓）</t>
         </is>
       </c>
       <c r="C51" s="6" t="inlineStr">
         <is>
-          <t>阻塞：[2026-10-07] 等兩件事：(1) Spotpear 回覆充電芯片型號、充電電流、有沒有 power path（問題已草擬給用戶發送）(2) 用戶做一次實物放電：拔 USB 用到自動關機 → 插 USB 計時到能對話 → 插住用 30 分鐘。與 R-16 的放電測試同一次完成。韌體現況：brownout 重啟會補播低電提醒，運行記錄（開機時 Supply log）會記每次重啟原因，可據此判斷有沒有反覆 brownout；『掉電後先深睡充電』的緩解要等測試證明需要才做</t>
+          <t>阻塞：[2026-10-07] 仍按 10/06 決定暫緩：等用戶做充滿再放電測試（與 R-17 同一次），看 VDD 低電提醒在關機前多久觸發；太遲或不觸發才向 Spotpear 提改板。已把分壓改板的問題一併放進給 Spotpear 的草稿，方便同一封發出</t>
         </is>
       </c>
       <c r="D51" s="11" t="n"/>
@@ -2040,20 +2049,20 @@
       <c r="H51" s="11" t="n"/>
       <c r="I51" s="12" t="n"/>
     </row>
-    <row r="52" ht="18" customHeight="1">
+    <row r="52" ht="88" customHeight="1">
       <c r="A52" s="13" t="inlineStr">
         <is>
-          <t>P0-07</t>
+          <t>R-17</t>
         </is>
       </c>
       <c r="B52" s="6" t="inlineStr">
         <is>
-          <t>輪換 JWT secret，作廢已發出的 token</t>
+          <t>Spotpear 電池耗盡時插電能否正常開機（供電路徑）</t>
         </is>
       </c>
       <c r="C52" s="6" t="inlineStr">
         <is>
-          <t>等 P0-06</t>
+          <t>阻塞：[2026-10-07] 等兩件事：(1) Spotpear 回覆充電芯片型號、充電電流、有沒有 power path（問題已草擬給用戶發送）(2) 用戶做一次實物放電：拔 USB 用到自動關機 → 插 USB 計時到能對話 → 插住用 30 分鐘。與 R-16 的放電測試同一次完成。韌體現況：brownout 重啟會補播低電提醒，運行記錄（開機時 Supply log）會記每次重啟原因，可據此判斷有沒有反覆 brownout；『掉電後先深睡充電』的緩解要等測試證明需要才做</t>
         </is>
       </c>
       <c r="D52" s="11" t="n"/>
@@ -2066,12 +2075,12 @@
     <row r="53" ht="18" customHeight="1">
       <c r="A53" s="13" t="inlineStr">
         <is>
-          <t>P0-11</t>
+          <t>P0-07</t>
         </is>
       </c>
       <c r="B53" s="6" t="inlineStr">
         <is>
-          <t>設備認領要求持有證明</t>
+          <t>輪換 JWT secret，作廢已發出的 token</t>
         </is>
       </c>
       <c r="C53" s="6" t="inlineStr">
@@ -2089,17 +2098,17 @@
     <row r="54" ht="18" customHeight="1">
       <c r="A54" s="13" t="inlineStr">
         <is>
-          <t>P1-10</t>
+          <t>P0-11</t>
         </is>
       </c>
       <c r="B54" s="6" t="inlineStr">
         <is>
-          <t>管理操作審計記錄</t>
+          <t>設備認領要求持有證明</t>
         </is>
       </c>
       <c r="C54" s="6" t="inlineStr">
         <is>
-          <t>等 P0-12</t>
+          <t>等 P0-06</t>
         </is>
       </c>
       <c r="D54" s="11" t="n"/>
@@ -2112,17 +2121,17 @@
     <row r="55" ht="18" customHeight="1">
       <c r="A55" s="13" t="inlineStr">
         <is>
-          <t>R-05</t>
+          <t>P1-10</t>
         </is>
       </c>
       <c r="B55" s="6" t="inlineStr">
         <is>
-          <t>內測版外殼（3D 打印 20 台）</t>
+          <t>管理操作審計記錄</t>
         </is>
       </c>
       <c r="C55" s="6" t="inlineStr">
         <is>
-          <t>等 R-01</t>
+          <t>等 P0-12</t>
         </is>
       </c>
       <c r="D55" s="11" t="n"/>
@@ -2135,17 +2144,17 @@
     <row r="56" ht="18" customHeight="1">
       <c r="A56" s="13" t="inlineStr">
         <is>
-          <t>R-06</t>
+          <t>R-05</t>
         </is>
       </c>
       <c r="B56" s="6" t="inlineStr">
         <is>
-          <t>家長自助上手流程</t>
+          <t>內測版外殼（3D 打印 20 台）</t>
         </is>
       </c>
       <c r="C56" s="6" t="inlineStr">
         <is>
-          <t>等 P0-11</t>
+          <t>等 R-01</t>
         </is>
       </c>
       <c r="D56" s="11" t="n"/>
@@ -2155,20 +2164,20 @@
       <c r="H56" s="11" t="n"/>
       <c r="I56" s="12" t="n"/>
     </row>
-    <row r="57" ht="46" customHeight="1">
+    <row r="57" ht="18" customHeight="1">
       <c r="A57" s="13" t="inlineStr">
         <is>
-          <t>R-13</t>
+          <t>R-06</t>
         </is>
       </c>
       <c r="B57" s="6" t="inlineStr">
         <is>
-          <t>CP1 內測就緒檢查（10/30）</t>
+          <t>家長自助上手流程</t>
         </is>
       </c>
       <c r="C57" s="6" t="inlineStr">
         <is>
-          <t>等 P0-02、P0-03、P0-04、P0-05、P0-06、P0-07、P0-08、P0-09、P0-10、P0-11、P0-12、P0-13、P1-01、P1-02、P2-09、R-01、R-02、R-04、R-05、R-06、P0-15、P0-16、P1-09、P1-11</t>
+          <t>等 P0-11</t>
         </is>
       </c>
       <c r="D57" s="11" t="n"/>
@@ -2178,20 +2187,20 @@
       <c r="H57" s="11" t="n"/>
       <c r="I57" s="12" t="n"/>
     </row>
-    <row r="58" ht="18" customHeight="1">
+    <row r="58" ht="46" customHeight="1">
       <c r="A58" s="13" t="inlineStr">
         <is>
-          <t>P0-14</t>
+          <t>R-13</t>
         </is>
       </c>
       <c r="B58" s="6" t="inlineStr">
         <is>
-          <t>韌體簽章、Secure Boot 與 Flash 加密</t>
+          <t>CP1 內測就緒檢查（10/30）</t>
         </is>
       </c>
       <c r="C58" s="6" t="inlineStr">
         <is>
-          <t>等 P0-13、R-01</t>
+          <t>等 P0-02、P0-03、P0-04、P0-05、P0-06、P0-07、P0-08、P0-09、P0-10、P0-11、P0-12、P0-13、P1-01、P1-02、P2-09、R-01、R-02、R-04、R-05、R-06、P0-15、P0-16、P1-09、P1-11</t>
         </is>
       </c>
       <c r="D58" s="11" t="n"/>
@@ -2204,17 +2213,17 @@
     <row r="59" ht="18" customHeight="1">
       <c r="A59" s="13" t="inlineStr">
         <is>
-          <t>P1-06</t>
+          <t>P0-14</t>
         </is>
       </c>
       <c r="B59" s="6" t="inlineStr">
         <is>
-          <t>處理 GPL-3.0 依賴（arduino-audio-tools）</t>
+          <t>韌體簽章、Secure Boot 與 Flash 加密</t>
         </is>
       </c>
       <c r="C59" s="6" t="inlineStr">
         <is>
-          <t>等 Q3</t>
+          <t>等 P0-13、R-01</t>
         </is>
       </c>
       <c r="D59" s="11" t="n"/>
@@ -2227,12 +2236,12 @@
     <row r="60" ht="18" customHeight="1">
       <c r="A60" s="13" t="inlineStr">
         <is>
-          <t>P1-07</t>
+          <t>P1-06</t>
         </is>
       </c>
       <c r="B60" s="6" t="inlineStr">
         <is>
-          <t>LGPL 合規與第三方授權聲明</t>
+          <t>處理 GPL-3.0 依賴（arduino-audio-tools）</t>
         </is>
       </c>
       <c r="C60" s="6" t="inlineStr">
@@ -2250,17 +2259,17 @@
     <row r="61" ht="18" customHeight="1">
       <c r="A61" s="13" t="inlineStr">
         <is>
-          <t>P1-08</t>
+          <t>P1-07</t>
         </is>
       </c>
       <c r="B61" s="6" t="inlineStr">
         <is>
-          <t>硬件認證</t>
+          <t>LGPL 合規與第三方授權聲明</t>
         </is>
       </c>
       <c r="C61" s="6" t="inlineStr">
         <is>
-          <t>等 R-01、R-05</t>
+          <t>等 Q3</t>
         </is>
       </c>
       <c r="D61" s="11" t="n"/>
@@ -2273,17 +2282,17 @@
     <row r="62" ht="18" customHeight="1">
       <c r="A62" s="13" t="inlineStr">
         <is>
-          <t>R-07</t>
+          <t>P1-08</t>
         </is>
       </c>
       <c r="B62" s="6" t="inlineStr">
         <is>
-          <t>20 個家庭封閉內測</t>
+          <t>硬件認證</t>
         </is>
       </c>
       <c r="C62" s="6" t="inlineStr">
         <is>
-          <t>等 R-13</t>
+          <t>等 R-01、R-05</t>
         </is>
       </c>
       <c r="D62" s="11" t="n"/>
@@ -2296,17 +2305,17 @@
     <row r="63" ht="18" customHeight="1">
       <c r="A63" s="13" t="inlineStr">
         <is>
-          <t>R-08</t>
+          <t>R-07</t>
         </is>
       </c>
       <c r="B63" s="6" t="inlineStr">
         <is>
-          <t>第 8 週關卡決策</t>
+          <t>20 個家庭封閉內測</t>
         </is>
       </c>
       <c r="C63" s="6" t="inlineStr">
         <is>
-          <t>等 R-07、P2-09、P1-08</t>
+          <t>等 R-13</t>
         </is>
       </c>
       <c r="D63" s="11" t="n"/>
@@ -2319,17 +2328,17 @@
     <row r="64" ht="18" customHeight="1">
       <c r="A64" s="13" t="inlineStr">
         <is>
-          <t>R-14</t>
+          <t>R-08</t>
         </is>
       </c>
       <c r="B64" s="6" t="inlineStr">
         <is>
-          <t>離線兒歌與故事</t>
+          <t>第 8 週關卡決策</t>
         </is>
       </c>
       <c r="C64" s="6" t="inlineStr">
         <is>
-          <t>等 R-01</t>
+          <t>等 R-07、P2-09、P1-08</t>
         </is>
       </c>
       <c r="D64" s="11" t="n"/>
@@ -2342,17 +2351,17 @@
     <row r="65" ht="18" customHeight="1">
       <c r="A65" s="13" t="inlineStr">
         <is>
-          <t>P2-05</t>
+          <t>R-14</t>
         </is>
       </c>
       <c r="B65" s="6" t="inlineStr">
         <is>
-          <t>拒絕未知設備並限制用量</t>
+          <t>離線兒歌與故事</t>
         </is>
       </c>
       <c r="C65" s="6" t="inlineStr">
         <is>
-          <t>等 P0-08</t>
+          <t>等 R-01</t>
         </is>
       </c>
       <c r="D65" s="11" t="n"/>
@@ -2365,17 +2374,17 @@
     <row r="66" ht="18" customHeight="1">
       <c r="A66" s="13" t="inlineStr">
         <is>
-          <t>R-09</t>
+          <t>P2-05</t>
         </is>
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
-          <t>量產外殼（真空複模）</t>
+          <t>拒絕未知設備並限制用量</t>
         </is>
       </c>
       <c r="C66" s="6" t="inlineStr">
         <is>
-          <t>等 R-08、R-05</t>
+          <t>等 P0-08</t>
         </is>
       </c>
       <c r="D66" s="11" t="n"/>
@@ -2388,17 +2397,17 @@
     <row r="67" ht="18" customHeight="1">
       <c r="A67" s="13" t="inlineStr">
         <is>
-          <t>R-10</t>
+          <t>R-09</t>
         </is>
       </c>
       <c r="B67" s="6" t="inlineStr">
         <is>
-          <t>出廠流程</t>
+          <t>量產外殼（真空複模）</t>
         </is>
       </c>
       <c r="C67" s="6" t="inlineStr">
         <is>
-          <t>等 P0-06、P0-14、R-01</t>
+          <t>等 R-08、R-05</t>
         </is>
       </c>
       <c r="D67" s="11" t="n"/>
@@ -2411,17 +2420,17 @@
     <row r="68" ht="18" customHeight="1">
       <c r="A68" s="13" t="inlineStr">
         <is>
-          <t>R-15</t>
+          <t>R-10</t>
         </is>
       </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t>農曆新年前交付（生產 1/15、送達 1/29）</t>
+          <t>出廠流程</t>
         </is>
       </c>
       <c r="C68" s="6" t="inlineStr">
         <is>
-          <t>等 R-09、R-10</t>
+          <t>等 P0-06、P0-14、R-01</t>
         </is>
       </c>
       <c r="D68" s="11" t="n"/>
@@ -2431,50 +2440,50 @@
       <c r="H68" s="11" t="n"/>
       <c r="I68" s="12" t="n"/>
     </row>
-    <row r="70">
-      <c r="A70" s="10" t="inlineStr">
+    <row r="69" ht="18" customHeight="1">
+      <c r="A69" s="13" t="inlineStr">
+        <is>
+          <t>R-15</t>
+        </is>
+      </c>
+      <c r="B69" s="6" t="inlineStr">
+        <is>
+          <t>農曆新年前交付（生產 1/15、送達 1/29）</t>
+        </is>
+      </c>
+      <c r="C69" s="6" t="inlineStr">
+        <is>
+          <t>等 R-09、R-10</t>
+        </is>
+      </c>
+      <c r="D69" s="11" t="n"/>
+      <c r="E69" s="11" t="n"/>
+      <c r="F69" s="11" t="n"/>
+      <c r="G69" s="11" t="n"/>
+      <c r="H69" s="11" t="n"/>
+      <c r="I69" s="12" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="10" t="inlineStr">
         <is>
           <t>❓ 待確認問題</t>
         </is>
       </c>
     </row>
-    <row r="71">
-      <c r="A71" s="4" t="inlineStr">
+    <row r="72">
+      <c r="A72" s="4" t="inlineStr">
         <is>
           <t>編號</t>
         </is>
       </c>
-      <c r="B71" s="4" t="inlineStr">
+      <c r="B72" s="4" t="inlineStr">
         <is>
           <t>問題</t>
         </is>
       </c>
-      <c r="C71" s="4" t="inlineStr">
+      <c r="C72" s="4" t="inlineStr">
         <is>
           <t>影響的任務 / 為什麼重要</t>
-        </is>
-      </c>
-      <c r="D71" s="11" t="n"/>
-      <c r="E71" s="11" t="n"/>
-      <c r="F71" s="11" t="n"/>
-      <c r="G71" s="11" t="n"/>
-      <c r="H71" s="11" t="n"/>
-      <c r="I71" s="12" t="n"/>
-    </row>
-    <row r="72" ht="18" customHeight="1">
-      <c r="A72" s="13" t="inlineStr">
-        <is>
-          <t>Q3</t>
-        </is>
-      </c>
-      <c r="B72" s="6" t="inlineStr">
-        <is>
-          <t>韌體打算閉源商業銷售嗎？</t>
-        </is>
-      </c>
-      <c r="C72" s="6" t="inlineStr">
-        <is>
-          <t>P1-06, P1-07：決定 GPL／LGPL 依賴要開源還是替換。</t>
         </is>
       </c>
       <c r="D72" s="11" t="n"/>
@@ -2484,63 +2493,85 @@
       <c r="H72" s="11" t="n"/>
       <c r="I72" s="12" t="n"/>
     </row>
-    <row r="74">
-      <c r="A74" s="10" t="inlineStr">
+    <row r="73" ht="18" customHeight="1">
+      <c r="A73" s="13" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="B73" s="6" t="inlineStr">
+        <is>
+          <t>韌體打算閉源商業銷售嗎？</t>
+        </is>
+      </c>
+      <c r="C73" s="6" t="inlineStr">
+        <is>
+          <t>P1-06, P1-07：決定 GPL／LGPL 依賴要開源還是替換。</t>
+        </is>
+      </c>
+      <c r="D73" s="11" t="n"/>
+      <c r="E73" s="11" t="n"/>
+      <c r="F73" s="11" t="n"/>
+      <c r="G73" s="11" t="n"/>
+      <c r="H73" s="11" t="n"/>
+      <c r="I73" s="12" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="10" t="inlineStr">
         <is>
           <t>說明</t>
         </is>
       </c>
     </row>
-    <row r="75" ht="32" customHeight="1">
-      <c r="A75" s="14" t="inlineStr">
+    <row r="76" ht="32" customHeight="1">
+      <c r="A76" s="14" t="inlineStr">
         <is>
           <t>・狀態：未開始 → 進行中 → 已完成。只有測試真的跑過而且通過才算已完成；阻塞要在備註寫原因；不再需要的任務標不適用，不要刪。</t>
-        </is>
-      </c>
-    </row>
-    <row r="76" ht="18" customHeight="1">
-      <c r="A76" s="14" t="inlineStr">
-        <is>
-          <t>・測試結果：未測試 / 通過 / 失敗 / 部分通過。測試證據寫跑了什麼、看到什麼，完整歷史在「更新記錄」。</t>
         </is>
       </c>
     </row>
     <row r="77" ht="18" customHeight="1">
       <c r="A77" s="14" t="inlineStr">
         <is>
-          <t>・「接下來」按階段排序，同一階段內再按優先級；依賴還沒滿足的任務不會出現在「接下來」。</t>
+          <t>・測試結果：未測試 / 通過 / 失敗 / 部分通過。測試證據寫跑了什麼、看到什麼，完整歷史在「更新記錄」。</t>
         </is>
       </c>
     </row>
     <row r="78" ht="18" customHeight="1">
       <c r="A78" s="14" t="inlineStr">
         <is>
+          <t>・「接下來」按階段排序，同一階段內再按優先級；依賴還沒滿足的任務不會出現在「接下來」。</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="18" customHeight="1">
+      <c r="A79" s="14" t="inlineStr">
+        <is>
           <t>・可以手動改：「任務清單」的狀態、測試結果、測試證據、Commit、備註，以及「待確認問題」的回答。其餘欄位和本頁由腳本維護。</t>
         </is>
       </c>
     </row>
-    <row r="79" ht="32" customHeight="1">
-      <c r="A79" s="14" t="inlineStr">
+    <row r="80" ht="32" customHeight="1">
+      <c r="A80" s="14" t="inlineStr">
         <is>
           <t>・建議用法：在 Claude Code 對 Claude 說「P0-02 做完了」或輸入 /prod-readiness。Claude 會先跑測試再更新，並寫進「更新記錄」。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="60">
+  <mergeCells count="61">
     <mergeCell ref="E21:I21"/>
     <mergeCell ref="C61:I61"/>
-    <mergeCell ref="E43:I43"/>
     <mergeCell ref="C52:I52"/>
     <mergeCell ref="A75:I75"/>
     <mergeCell ref="E24:I24"/>
+    <mergeCell ref="A80:I80"/>
     <mergeCell ref="E33:I33"/>
     <mergeCell ref="A3:I3"/>
     <mergeCell ref="E23:I23"/>
     <mergeCell ref="C72:I72"/>
     <mergeCell ref="E39:I39"/>
     <mergeCell ref="C67:I67"/>
-    <mergeCell ref="A74:I74"/>
     <mergeCell ref="C57:I57"/>
     <mergeCell ref="C53:I53"/>
     <mergeCell ref="C66:I66"/>
@@ -2550,9 +2581,9 @@
     <mergeCell ref="E35:I35"/>
     <mergeCell ref="E20:I20"/>
     <mergeCell ref="E38:I38"/>
-    <mergeCell ref="A42:I42"/>
+    <mergeCell ref="C69:I69"/>
+    <mergeCell ref="A71:I71"/>
     <mergeCell ref="A76:I76"/>
-    <mergeCell ref="C49:I49"/>
     <mergeCell ref="E28:I28"/>
     <mergeCell ref="C62:I62"/>
     <mergeCell ref="C68:I68"/>
@@ -2560,34 +2591,36 @@
     <mergeCell ref="E40:I40"/>
     <mergeCell ref="C58:I58"/>
     <mergeCell ref="E30:I30"/>
+    <mergeCell ref="A43:I43"/>
     <mergeCell ref="E34:I34"/>
     <mergeCell ref="A19:I19"/>
     <mergeCell ref="C64:I64"/>
+    <mergeCell ref="C51:I51"/>
     <mergeCell ref="E46:I46"/>
+    <mergeCell ref="C73:I73"/>
     <mergeCell ref="E27:I27"/>
     <mergeCell ref="E45:I45"/>
     <mergeCell ref="C54:I54"/>
     <mergeCell ref="A77:I77"/>
     <mergeCell ref="E36:I36"/>
     <mergeCell ref="C63:I63"/>
-    <mergeCell ref="A48:I48"/>
     <mergeCell ref="C65:I65"/>
     <mergeCell ref="E26:I26"/>
     <mergeCell ref="C55:I55"/>
     <mergeCell ref="C50:I50"/>
+    <mergeCell ref="A49:I49"/>
     <mergeCell ref="C56:I56"/>
     <mergeCell ref="E32:I32"/>
     <mergeCell ref="E25:I25"/>
     <mergeCell ref="C59:I59"/>
     <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A70:I70"/>
+    <mergeCell ref="E41:I41"/>
     <mergeCell ref="A79:I79"/>
     <mergeCell ref="E37:I37"/>
     <mergeCell ref="C60:I60"/>
     <mergeCell ref="E22:I22"/>
-    <mergeCell ref="C51:I51"/>
+    <mergeCell ref="E47:I47"/>
     <mergeCell ref="A78:I78"/>
-    <mergeCell ref="C71:I71"/>
   </mergeCells>
   <conditionalFormatting sqref="I6:I10">
     <cfRule type="dataBar" priority="1">
@@ -6563,7 +6596,7 @@
         </is>
       </c>
     </row>
-    <row r="56" ht="74" customHeight="1">
+    <row r="56" ht="172" customHeight="1">
       <c r="A56" s="13" t="inlineStr">
         <is>
           <t>P2-10</t>
@@ -6591,12 +6624,12 @@
       </c>
       <c r="F56" s="13" t="inlineStr">
         <is>
-          <t>未開始</t>
+          <t>進行中</t>
         </is>
       </c>
       <c r="G56" s="13" t="inlineStr">
         <is>
-          <t>未測試</t>
+          <t>部分通過</t>
         </is>
       </c>
       <c r="I56" s="6" t="inlineStr">
@@ -6620,9 +6653,20 @@
         </is>
       </c>
       <c r="M56" s="13" t="n"/>
+      <c r="N56" s="6" t="inlineStr">
+        <is>
+          <t>① 16 家供應商各 20 次真實 session prompt（含開場白，串流，order=[x]+allow_fallbacks=false）：建議清單 azure/alibaba/novita/siliconflow/gmicloud 各 20/20，0 空內容 0 特殊 token，首字 p50 1.25/2.33/2.59/2.56/3.25s；只設 order 時 order=[deepinfra] 實際由 Relace 回應（回過 content=None）→ 已改為 allow_fallbacks=false。伺服器端 LLMOutputGuard：pytest 8 項（尾部/跨 chunk 拆開的 token、空回應記警告）全套 203 passed；真實 LLM 串流經 guard 6 角色 12/12 正常、無誤觸發。② 實機 5 次開場白未做</t>
+        </is>
+      </c>
+      <c r="O56" s="13" t="inlineStr">
+        <is>
+          <t>58bc82b</t>
+        </is>
+      </c>
       <c r="P56" s="6" t="inlineStr">
         <is>
-          <t>[2026-10-07] 新增</t>
+          <t>[2026-10-07] 新增
+[2026-10-07] 2026-10-07 58bc82b（分支 p2-10-provider-pinning，未合併、未部署）。上線後在管理頁設 provider_order=azure,alibaba,novita,siliconflow,gmicloud（或繼續用 gemma）。Azure 20 次中 1 次把孩子叫成「小柔」（prompt 無此名），屬模型偶發，非供應商問題</t>
         </is>
       </c>
     </row>
@@ -7090,7 +7134,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I115"/>
+  <dimension ref="A1:I117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -11124,8 +11168,86 @@
         </is>
       </c>
     </row>
+    <row r="116" ht="32" customHeight="1">
+      <c r="A116" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-07 21:47</t>
+        </is>
+      </c>
+      <c r="B116" s="13" t="inlineStr">
+        <is>
+          <t>P2-10</t>
+        </is>
+      </c>
+      <c r="C116" s="6" t="inlineStr">
+        <is>
+          <t>DeepSeek v4 flash 經 OpenRouter 時固定可用的供應商</t>
+        </is>
+      </c>
+      <c r="D116" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E116" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F116" s="13" t="n"/>
+      <c r="G116" s="6" t="n"/>
+      <c r="H116" s="13" t="n"/>
+      <c r="I116" s="6" t="n"/>
+    </row>
+    <row r="117" ht="144" customHeight="1">
+      <c r="A117" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-07 22:04</t>
+        </is>
+      </c>
+      <c r="B117" s="13" t="inlineStr">
+        <is>
+          <t>P2-10</t>
+        </is>
+      </c>
+      <c r="C117" s="6" t="inlineStr">
+        <is>
+          <t>DeepSeek v4 flash 經 OpenRouter 時固定可用的供應商</t>
+        </is>
+      </c>
+      <c r="D117" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="E117" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F117" s="13" t="inlineStr">
+        <is>
+          <t>部分通過</t>
+        </is>
+      </c>
+      <c r="G117" s="6" t="inlineStr">
+        <is>
+          <t>① 16 家供應商各 20 次真實 session prompt（含開場白，串流，order=[x]+allow_fallbacks=false）：建議清單 azure/alibaba/novita/siliconflow/gmicloud 各 20/20，0 空內容 0 特殊 token，首字 p50 1.25/2.33/2.59/2.56/3.25s；只設 order 時 order=[deepinfra] 實際由 Relace 回應（回過 content=None）→ 已改為 allow_fallbacks=false。伺服器端 LLMOutputGuard：pytest 8 項（尾部/跨 chunk 拆開的 token、空回應記警告）全套 203 passed；真實 LLM 串流經 guard 6 角色 12/12 正常、無誤觸發。② 實機 5 次開場白未做</t>
+        </is>
+      </c>
+      <c r="H117" s="13" t="inlineStr">
+        <is>
+          <t>58bc82b</t>
+        </is>
+      </c>
+      <c r="I117" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-07 58bc82b（分支 p2-10-provider-pinning，未合併、未部署）。上線後在管理頁設 provider_order=azure,alibaba,novita,siliconflow,gmicloud（或繼續用 gemma）。Azure 20 次中 1 次把孩子叫成「小柔」（prompt 無此名），屬模型偶發，非供應商問題</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I115"/>
+  <autoFilter ref="A1:I117"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record P0-13 progress: OTA built and tested on the server side.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/production-readiness.xlsx
+++ b/docs/production-readiness.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'任務清單'!$A$1:$P$56</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'待確認問題'!$A$1:$G$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$117</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$119</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -641,7 +641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I80"/>
+  <dimension ref="A1:I81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -665,7 +665,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>最後更新：2026-10-07 22:04　·　本頁由 tracker.py 自動生成，請勿手動編輯</t>
+          <t>最後更新：2026-10-08 09:04　·　本頁由 tracker.py 自動生成，請勿手動編輯</t>
         </is>
       </c>
     </row>
@@ -740,11 +740,11 @@
       </c>
       <c r="D6" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A6,'任務清單'!$F:$F,D$5)</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E6" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A6,'任務清單'!$F:$F,E$5)</f>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F6" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A6,'任務清單'!$F:$F,F$5)</f>
@@ -896,11 +896,11 @@
       </c>
       <c r="D10" s="5">
         <f>SUM(D6:D9)</f>
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E10" s="5">
         <f>SUM(E6:E9)</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F10" s="5">
         <f>SUM(F6:F9)</f>
@@ -1023,11 +1023,11 @@
       </c>
       <c r="D14" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A14,'任務清單'!$F:$F,D$12)</f>
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E14" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A14,'任務清單'!$F:$F,E$12)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F14" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A14,'任務清單'!$F:$F,F$12)</f>
@@ -1139,11 +1139,11 @@
       </c>
       <c r="D17" s="5">
         <f>SUM(D13:D16)</f>
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E17" s="5">
         <f>SUM(E13:E16)</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F17" s="5">
         <f>SUM(F13:F16)</f>
@@ -1679,7 +1679,7 @@
       <c r="H35" s="11" t="n"/>
       <c r="I35" s="12" t="n"/>
     </row>
-    <row r="36" ht="32" customHeight="1">
+    <row r="36" ht="172" customHeight="1">
       <c r="A36" s="13" t="inlineStr">
         <is>
           <t>P0-13</t>
@@ -1697,12 +1697,13 @@
       </c>
       <c r="D36" s="13" t="inlineStr">
         <is>
-          <t>未開始</t>
+          <t>進行中</t>
         </is>
       </c>
       <c r="E36" s="6" t="inlineStr">
         <is>
-          <t>填入真實 URL 與 CA；新韌體啟動自檢通過才標記有效，否則自動回滾；設備上報韌體版本。</t>
+          <t>上次測試：部分通過 — 本機：firmware_releases + 私有 bucket + /api/ota/check + /api/ota/firmware/[id]，API 16/16（無 token/web token/過期 → 401；只提供本板 current release；下載 1654400 bytes 與 build sha256 一致；回滾過的版本不再提供並記在 devices）；release_firmware.py 拒 localws build、拒重複版本；pio 18 個 env 全 SUCCESS，spotpear 1.58MB/2MB；Arduino 2.0.17 bootloader 已開 CONFIG_BOOTLOADER_APP_ROLLBACK_ENABLE（C3/S3）。①② 實機未做
+填入真實 URL 與 CA；新韌體啟動自檢通過才標記有效，否則自動回滾；設備上報韌體版本。</t>
         </is>
       </c>
       <c r="F36" s="11" t="n"/>
@@ -1865,68 +1866,68 @@
       <c r="H41" s="11" t="n"/>
       <c r="I41" s="12" t="n"/>
     </row>
-    <row r="43">
-      <c r="A43" s="10" t="inlineStr">
+    <row r="42" ht="32" customHeight="1">
+      <c r="A42" s="13" t="inlineStr">
+        <is>
+          <t>P2-04</t>
+        </is>
+      </c>
+      <c r="B42" s="6" t="inlineStr">
+        <is>
+          <t>容器改用非 root 用戶</t>
+        </is>
+      </c>
+      <c r="C42" s="13" t="inlineStr">
+        <is>
+          <t>2 內測準備</t>
+        </is>
+      </c>
+      <c r="D42" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E42" s="6" t="inlineStr">
+        <is>
+          <t>兩個 Dockerfile 都設定非 root 的 USER。</t>
+        </is>
+      </c>
+      <c r="F42" s="11" t="n"/>
+      <c r="G42" s="11" t="n"/>
+      <c r="H42" s="11" t="n"/>
+      <c r="I42" s="12" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="10" t="inlineStr">
         <is>
           <t>✅ 最近完成與測試效果</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="4" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
         <is>
           <t>編號</t>
         </is>
       </c>
-      <c r="B44" s="4" t="inlineStr">
+      <c r="B45" s="4" t="inlineStr">
         <is>
           <t>任務</t>
         </is>
       </c>
-      <c r="C44" s="4" t="inlineStr">
+      <c r="C45" s="4" t="inlineStr">
         <is>
           <t>測試結果</t>
         </is>
       </c>
-      <c r="D44" s="4" t="inlineStr">
+      <c r="D45" s="4" t="inlineStr">
         <is>
           <t>完成日期</t>
         </is>
       </c>
-      <c r="E44" s="4" t="inlineStr">
+      <c r="E45" s="4" t="inlineStr">
         <is>
           <t>測試證據</t>
-        </is>
-      </c>
-      <c r="F44" s="11" t="n"/>
-      <c r="G44" s="11" t="n"/>
-      <c r="H44" s="11" t="n"/>
-      <c r="I44" s="12" t="n"/>
-    </row>
-    <row r="45" ht="88" customHeight="1">
-      <c r="A45" s="13" t="inlineStr">
-        <is>
-          <t>R-03</t>
-        </is>
-      </c>
-      <c r="B45" s="6" t="inlineStr">
-        <is>
-          <t>移除不用的 Deno／Cloudflare 後端與上游預設主機</t>
-        </is>
-      </c>
-      <c r="C45" s="13" t="inlineStr">
-        <is>
-          <t>通過</t>
-        </is>
-      </c>
-      <c r="D45" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-07</t>
-        </is>
-      </c>
-      <c r="E45" s="6" t="inlineStr">
-        <is>
-          <t>① grep deno.dev|workers.dev|railway.app|VOICE_SERVER_DENO|VOICE_SERVER_CLOUDFLARE 全 repo → 只剩 seed.json 的任務描述本身 ② pio run 18 個 env 全 SUCCESS（S3 devkit/Waveshare/xmini-c3/Spotpear 各變體）③ FastAPI pytest 182 passed；另 tsc --noEmit 通過</t>
         </is>
       </c>
       <c r="F45" s="11" t="n"/>
@@ -1937,12 +1938,12 @@
     <row r="46" ht="88" customHeight="1">
       <c r="A46" s="13" t="inlineStr">
         <is>
-          <t>P2-01</t>
+          <t>R-03</t>
         </is>
       </c>
       <c r="B46" s="6" t="inlineStr">
         <is>
-          <t>修好後端測試環境</t>
+          <t>移除不用的 Deno／Cloudflare 後端與上游預設主機</t>
         </is>
       </c>
       <c r="C46" s="13" t="inlineStr">
@@ -1957,7 +1958,7 @@
       </c>
       <c r="E46" s="6" t="inlineStr">
         <is>
-          <t>cd server/fastapi &amp;&amp; .venv/bin/python -m pytest -q → 173 passed（原本 60 個 async 測試報「not natively supported」）；pyproject dev group 加 pytest&gt;=9,&lt;10、pytest-asyncio&gt;=1.4,&lt;2，asyncio_mode=auto；pip install --dry-run --group dev 可解析</t>
+          <t>① grep deno.dev|workers.dev|railway.app|VOICE_SERVER_DENO|VOICE_SERVER_CLOUDFLARE 全 repo → 只剩 seed.json 的任務描述本身 ② pio run 18 個 env 全 SUCCESS（S3 devkit/Waveshare/xmini-c3/Spotpear 各變體）③ FastAPI pytest 182 passed；另 tsc --noEmit 通過</t>
         </is>
       </c>
       <c r="F46" s="11" t="n"/>
@@ -1965,15 +1966,15 @@
       <c r="H46" s="11" t="n"/>
       <c r="I46" s="12" t="n"/>
     </row>
-    <row r="47" ht="60" customHeight="1">
+    <row r="47" ht="88" customHeight="1">
       <c r="A47" s="13" t="inlineStr">
         <is>
-          <t>P2-03</t>
+          <t>P2-01</t>
         </is>
       </c>
       <c r="B47" s="6" t="inlineStr">
         <is>
-          <t>提交目前未提交的改動</t>
+          <t>修好後端測試環境</t>
         </is>
       </c>
       <c r="C47" s="13" t="inlineStr">
@@ -1983,12 +1984,12 @@
       </c>
       <c r="D47" s="13" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="E47" s="6" t="inlineStr">
         <is>
-          <t>git status --short → 0 行；3bc7119..b322375 按主題拆成 5 個 commit（50 檔：xmini-c3 電量、facts 記憶層、日期時間天氣、BEAM 評測、進度追蹤）；git ls-remote mygithub main = HEAD = b322375</t>
+          <t>cd server/fastapi &amp;&amp; .venv/bin/python -m pytest -q → 173 passed（原本 60 個 async 測試報「not natively supported」）；pyproject dev group 加 pytest&gt;=9,&lt;10、pytest-asyncio&gt;=1.4,&lt;2，asyncio_mode=auto；pip install --dry-run --group dev 可解析</t>
         </is>
       </c>
       <c r="F47" s="11" t="n"/>
@@ -1996,50 +1997,58 @@
       <c r="H47" s="11" t="n"/>
       <c r="I47" s="12" t="n"/>
     </row>
-    <row r="49">
-      <c r="A49" s="10" t="inlineStr">
+    <row r="48" ht="60" customHeight="1">
+      <c r="A48" s="13" t="inlineStr">
+        <is>
+          <t>P2-03</t>
+        </is>
+      </c>
+      <c r="B48" s="6" t="inlineStr">
+        <is>
+          <t>提交目前未提交的改動</t>
+        </is>
+      </c>
+      <c r="C48" s="13" t="inlineStr">
+        <is>
+          <t>通過</t>
+        </is>
+      </c>
+      <c r="D48" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="E48" s="6" t="inlineStr">
+        <is>
+          <t>git status --short → 0 行；3bc7119..b322375 按主題拆成 5 個 commit（50 檔：xmini-c3 電量、facts 記憶層、日期時間天氣、BEAM 評測、進度追蹤）；git ls-remote mygithub main = HEAD = b322375</t>
+        </is>
+      </c>
+      <c r="F48" s="11" t="n"/>
+      <c r="G48" s="11" t="n"/>
+      <c r="H48" s="11" t="n"/>
+      <c r="I48" s="12" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="10" t="inlineStr">
         <is>
           <t>⏳ 等待依賴 / ⛔ 阻塞</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="4" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
         <is>
           <t>編號</t>
         </is>
       </c>
-      <c r="B50" s="4" t="inlineStr">
+      <c r="B51" s="4" t="inlineStr">
         <is>
           <t>任務</t>
         </is>
       </c>
-      <c r="C50" s="4" t="inlineStr">
+      <c r="C51" s="4" t="inlineStr">
         <is>
           <t>在等什麼</t>
-        </is>
-      </c>
-      <c r="D50" s="11" t="n"/>
-      <c r="E50" s="11" t="n"/>
-      <c r="F50" s="11" t="n"/>
-      <c r="G50" s="11" t="n"/>
-      <c r="H50" s="11" t="n"/>
-      <c r="I50" s="12" t="n"/>
-    </row>
-    <row r="51" ht="60" customHeight="1">
-      <c r="A51" s="13" t="inlineStr">
-        <is>
-          <t>R-16</t>
-        </is>
-      </c>
-      <c r="B51" s="6" t="inlineStr">
-        <is>
-          <t>Spotpear 量產版加電池電壓檢測（GPIO0 分壓）</t>
-        </is>
-      </c>
-      <c r="C51" s="6" t="inlineStr">
-        <is>
-          <t>阻塞：[2026-10-07] 仍按 10/06 決定暫緩：等用戶做充滿再放電測試（與 R-17 同一次），看 VDD 低電提醒在關機前多久觸發；太遲或不觸發才向 Spotpear 提改板。已把分壓改板的問題一併放進給 Spotpear 的草稿，方便同一封發出</t>
         </is>
       </c>
       <c r="D51" s="11" t="n"/>
@@ -2049,20 +2058,20 @@
       <c r="H51" s="11" t="n"/>
       <c r="I51" s="12" t="n"/>
     </row>
-    <row r="52" ht="88" customHeight="1">
+    <row r="52" ht="60" customHeight="1">
       <c r="A52" s="13" t="inlineStr">
         <is>
-          <t>R-17</t>
+          <t>R-16</t>
         </is>
       </c>
       <c r="B52" s="6" t="inlineStr">
         <is>
-          <t>Spotpear 電池耗盡時插電能否正常開機（供電路徑）</t>
+          <t>Spotpear 量產版加電池電壓檢測（GPIO0 分壓）</t>
         </is>
       </c>
       <c r="C52" s="6" t="inlineStr">
         <is>
-          <t>阻塞：[2026-10-07] 等兩件事：(1) Spotpear 回覆充電芯片型號、充電電流、有沒有 power path（問題已草擬給用戶發送）(2) 用戶做一次實物放電：拔 USB 用到自動關機 → 插 USB 計時到能對話 → 插住用 30 分鐘。與 R-16 的放電測試同一次完成。韌體現況：brownout 重啟會補播低電提醒，運行記錄（開機時 Supply log）會記每次重啟原因，可據此判斷有沒有反覆 brownout；『掉電後先深睡充電』的緩解要等測試證明需要才做</t>
+          <t>阻塞：[2026-10-07] 仍按 10/06 決定暫緩：等用戶做充滿再放電測試（與 R-17 同一次），看 VDD 低電提醒在關機前多久觸發；太遲或不觸發才向 Spotpear 提改板。已把分壓改板的問題一併放進給 Spotpear 的草稿，方便同一封發出</t>
         </is>
       </c>
       <c r="D52" s="11" t="n"/>
@@ -2072,20 +2081,20 @@
       <c r="H52" s="11" t="n"/>
       <c r="I52" s="12" t="n"/>
     </row>
-    <row r="53" ht="18" customHeight="1">
+    <row r="53" ht="88" customHeight="1">
       <c r="A53" s="13" t="inlineStr">
         <is>
-          <t>P0-07</t>
+          <t>R-17</t>
         </is>
       </c>
       <c r="B53" s="6" t="inlineStr">
         <is>
-          <t>輪換 JWT secret，作廢已發出的 token</t>
+          <t>Spotpear 電池耗盡時插電能否正常開機（供電路徑）</t>
         </is>
       </c>
       <c r="C53" s="6" t="inlineStr">
         <is>
-          <t>等 P0-06</t>
+          <t>阻塞：[2026-10-07] 等兩件事：(1) Spotpear 回覆充電芯片型號、充電電流、有沒有 power path（問題已草擬給用戶發送）(2) 用戶做一次實物放電：拔 USB 用到自動關機 → 插 USB 計時到能對話 → 插住用 30 分鐘。與 R-16 的放電測試同一次完成。韌體現況：brownout 重啟會補播低電提醒，運行記錄（開機時 Supply log）會記每次重啟原因，可據此判斷有沒有反覆 brownout；『掉電後先深睡充電』的緩解要等測試證明需要才做</t>
         </is>
       </c>
       <c r="D53" s="11" t="n"/>
@@ -2098,12 +2107,12 @@
     <row r="54" ht="18" customHeight="1">
       <c r="A54" s="13" t="inlineStr">
         <is>
-          <t>P0-11</t>
+          <t>P0-07</t>
         </is>
       </c>
       <c r="B54" s="6" t="inlineStr">
         <is>
-          <t>設備認領要求持有證明</t>
+          <t>輪換 JWT secret，作廢已發出的 token</t>
         </is>
       </c>
       <c r="C54" s="6" t="inlineStr">
@@ -2121,17 +2130,17 @@
     <row r="55" ht="18" customHeight="1">
       <c r="A55" s="13" t="inlineStr">
         <is>
-          <t>P1-10</t>
+          <t>P0-11</t>
         </is>
       </c>
       <c r="B55" s="6" t="inlineStr">
         <is>
-          <t>管理操作審計記錄</t>
+          <t>設備認領要求持有證明</t>
         </is>
       </c>
       <c r="C55" s="6" t="inlineStr">
         <is>
-          <t>等 P0-12</t>
+          <t>等 P0-06</t>
         </is>
       </c>
       <c r="D55" s="11" t="n"/>
@@ -2144,17 +2153,17 @@
     <row r="56" ht="18" customHeight="1">
       <c r="A56" s="13" t="inlineStr">
         <is>
-          <t>R-05</t>
+          <t>P1-10</t>
         </is>
       </c>
       <c r="B56" s="6" t="inlineStr">
         <is>
-          <t>內測版外殼（3D 打印 20 台）</t>
+          <t>管理操作審計記錄</t>
         </is>
       </c>
       <c r="C56" s="6" t="inlineStr">
         <is>
-          <t>等 R-01</t>
+          <t>等 P0-12</t>
         </is>
       </c>
       <c r="D56" s="11" t="n"/>
@@ -2167,17 +2176,17 @@
     <row r="57" ht="18" customHeight="1">
       <c r="A57" s="13" t="inlineStr">
         <is>
-          <t>R-06</t>
+          <t>R-05</t>
         </is>
       </c>
       <c r="B57" s="6" t="inlineStr">
         <is>
-          <t>家長自助上手流程</t>
+          <t>內測版外殼（3D 打印 20 台）</t>
         </is>
       </c>
       <c r="C57" s="6" t="inlineStr">
         <is>
-          <t>等 P0-11</t>
+          <t>等 R-01</t>
         </is>
       </c>
       <c r="D57" s="11" t="n"/>
@@ -2187,20 +2196,20 @@
       <c r="H57" s="11" t="n"/>
       <c r="I57" s="12" t="n"/>
     </row>
-    <row r="58" ht="46" customHeight="1">
+    <row r="58" ht="18" customHeight="1">
       <c r="A58" s="13" t="inlineStr">
         <is>
-          <t>R-13</t>
+          <t>R-06</t>
         </is>
       </c>
       <c r="B58" s="6" t="inlineStr">
         <is>
-          <t>CP1 內測就緒檢查（10/30）</t>
+          <t>家長自助上手流程</t>
         </is>
       </c>
       <c r="C58" s="6" t="inlineStr">
         <is>
-          <t>等 P0-02、P0-03、P0-04、P0-05、P0-06、P0-07、P0-08、P0-09、P0-10、P0-11、P0-12、P0-13、P1-01、P1-02、P2-09、R-01、R-02、R-04、R-05、R-06、P0-15、P0-16、P1-09、P1-11</t>
+          <t>等 P0-11</t>
         </is>
       </c>
       <c r="D58" s="11" t="n"/>
@@ -2210,20 +2219,20 @@
       <c r="H58" s="11" t="n"/>
       <c r="I58" s="12" t="n"/>
     </row>
-    <row r="59" ht="18" customHeight="1">
+    <row r="59" ht="46" customHeight="1">
       <c r="A59" s="13" t="inlineStr">
         <is>
-          <t>P0-14</t>
+          <t>R-13</t>
         </is>
       </c>
       <c r="B59" s="6" t="inlineStr">
         <is>
-          <t>韌體簽章、Secure Boot 與 Flash 加密</t>
+          <t>CP1 內測就緒檢查（10/30）</t>
         </is>
       </c>
       <c r="C59" s="6" t="inlineStr">
         <is>
-          <t>等 P0-13、R-01</t>
+          <t>等 P0-02、P0-03、P0-04、P0-05、P0-06、P0-07、P0-08、P0-09、P0-10、P0-11、P0-12、P0-13、P1-01、P1-02、P2-09、R-01、R-02、R-04、R-05、R-06、P0-15、P0-16、P1-09、P1-11</t>
         </is>
       </c>
       <c r="D59" s="11" t="n"/>
@@ -2236,17 +2245,17 @@
     <row r="60" ht="18" customHeight="1">
       <c r="A60" s="13" t="inlineStr">
         <is>
-          <t>P1-06</t>
+          <t>P0-14</t>
         </is>
       </c>
       <c r="B60" s="6" t="inlineStr">
         <is>
-          <t>處理 GPL-3.0 依賴（arduino-audio-tools）</t>
+          <t>韌體簽章、Secure Boot 與 Flash 加密</t>
         </is>
       </c>
       <c r="C60" s="6" t="inlineStr">
         <is>
-          <t>等 Q3</t>
+          <t>等 P0-13、R-01</t>
         </is>
       </c>
       <c r="D60" s="11" t="n"/>
@@ -2259,12 +2268,12 @@
     <row r="61" ht="18" customHeight="1">
       <c r="A61" s="13" t="inlineStr">
         <is>
-          <t>P1-07</t>
+          <t>P1-06</t>
         </is>
       </c>
       <c r="B61" s="6" t="inlineStr">
         <is>
-          <t>LGPL 合規與第三方授權聲明</t>
+          <t>處理 GPL-3.0 依賴（arduino-audio-tools）</t>
         </is>
       </c>
       <c r="C61" s="6" t="inlineStr">
@@ -2282,17 +2291,17 @@
     <row r="62" ht="18" customHeight="1">
       <c r="A62" s="13" t="inlineStr">
         <is>
-          <t>P1-08</t>
+          <t>P1-07</t>
         </is>
       </c>
       <c r="B62" s="6" t="inlineStr">
         <is>
-          <t>硬件認證</t>
+          <t>LGPL 合規與第三方授權聲明</t>
         </is>
       </c>
       <c r="C62" s="6" t="inlineStr">
         <is>
-          <t>等 R-01、R-05</t>
+          <t>等 Q3</t>
         </is>
       </c>
       <c r="D62" s="11" t="n"/>
@@ -2305,17 +2314,17 @@
     <row r="63" ht="18" customHeight="1">
       <c r="A63" s="13" t="inlineStr">
         <is>
-          <t>R-07</t>
+          <t>P1-08</t>
         </is>
       </c>
       <c r="B63" s="6" t="inlineStr">
         <is>
-          <t>20 個家庭封閉內測</t>
+          <t>硬件認證</t>
         </is>
       </c>
       <c r="C63" s="6" t="inlineStr">
         <is>
-          <t>等 R-13</t>
+          <t>等 R-01、R-05</t>
         </is>
       </c>
       <c r="D63" s="11" t="n"/>
@@ -2328,17 +2337,17 @@
     <row r="64" ht="18" customHeight="1">
       <c r="A64" s="13" t="inlineStr">
         <is>
-          <t>R-08</t>
+          <t>R-07</t>
         </is>
       </c>
       <c r="B64" s="6" t="inlineStr">
         <is>
-          <t>第 8 週關卡決策</t>
+          <t>20 個家庭封閉內測</t>
         </is>
       </c>
       <c r="C64" s="6" t="inlineStr">
         <is>
-          <t>等 R-07、P2-09、P1-08</t>
+          <t>等 R-13</t>
         </is>
       </c>
       <c r="D64" s="11" t="n"/>
@@ -2351,17 +2360,17 @@
     <row r="65" ht="18" customHeight="1">
       <c r="A65" s="13" t="inlineStr">
         <is>
-          <t>R-14</t>
+          <t>R-08</t>
         </is>
       </c>
       <c r="B65" s="6" t="inlineStr">
         <is>
-          <t>離線兒歌與故事</t>
+          <t>第 8 週關卡決策</t>
         </is>
       </c>
       <c r="C65" s="6" t="inlineStr">
         <is>
-          <t>等 R-01</t>
+          <t>等 R-07、P2-09、P1-08</t>
         </is>
       </c>
       <c r="D65" s="11" t="n"/>
@@ -2374,17 +2383,17 @@
     <row r="66" ht="18" customHeight="1">
       <c r="A66" s="13" t="inlineStr">
         <is>
-          <t>P2-05</t>
+          <t>R-14</t>
         </is>
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
-          <t>拒絕未知設備並限制用量</t>
+          <t>離線兒歌與故事</t>
         </is>
       </c>
       <c r="C66" s="6" t="inlineStr">
         <is>
-          <t>等 P0-08</t>
+          <t>等 R-01</t>
         </is>
       </c>
       <c r="D66" s="11" t="n"/>
@@ -2397,17 +2406,17 @@
     <row r="67" ht="18" customHeight="1">
       <c r="A67" s="13" t="inlineStr">
         <is>
-          <t>R-09</t>
+          <t>P2-05</t>
         </is>
       </c>
       <c r="B67" s="6" t="inlineStr">
         <is>
-          <t>量產外殼（真空複模）</t>
+          <t>拒絕未知設備並限制用量</t>
         </is>
       </c>
       <c r="C67" s="6" t="inlineStr">
         <is>
-          <t>等 R-08、R-05</t>
+          <t>等 P0-08</t>
         </is>
       </c>
       <c r="D67" s="11" t="n"/>
@@ -2420,17 +2429,17 @@
     <row r="68" ht="18" customHeight="1">
       <c r="A68" s="13" t="inlineStr">
         <is>
-          <t>R-10</t>
+          <t>R-09</t>
         </is>
       </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t>出廠流程</t>
+          <t>量產外殼（真空複模）</t>
         </is>
       </c>
       <c r="C68" s="6" t="inlineStr">
         <is>
-          <t>等 P0-06、P0-14、R-01</t>
+          <t>等 R-08、R-05</t>
         </is>
       </c>
       <c r="D68" s="11" t="n"/>
@@ -2443,17 +2452,17 @@
     <row r="69" ht="18" customHeight="1">
       <c r="A69" s="13" t="inlineStr">
         <is>
-          <t>R-15</t>
+          <t>R-10</t>
         </is>
       </c>
       <c r="B69" s="6" t="inlineStr">
         <is>
-          <t>農曆新年前交付（生產 1/15、送達 1/29）</t>
+          <t>出廠流程</t>
         </is>
       </c>
       <c r="C69" s="6" t="inlineStr">
         <is>
-          <t>等 R-09、R-10</t>
+          <t>等 P0-06、P0-14、R-01</t>
         </is>
       </c>
       <c r="D69" s="11" t="n"/>
@@ -2463,50 +2472,50 @@
       <c r="H69" s="11" t="n"/>
       <c r="I69" s="12" t="n"/>
     </row>
-    <row r="71">
-      <c r="A71" s="10" t="inlineStr">
+    <row r="70" ht="18" customHeight="1">
+      <c r="A70" s="13" t="inlineStr">
+        <is>
+          <t>R-15</t>
+        </is>
+      </c>
+      <c r="B70" s="6" t="inlineStr">
+        <is>
+          <t>農曆新年前交付（生產 1/15、送達 1/29）</t>
+        </is>
+      </c>
+      <c r="C70" s="6" t="inlineStr">
+        <is>
+          <t>等 R-09、R-10</t>
+        </is>
+      </c>
+      <c r="D70" s="11" t="n"/>
+      <c r="E70" s="11" t="n"/>
+      <c r="F70" s="11" t="n"/>
+      <c r="G70" s="11" t="n"/>
+      <c r="H70" s="11" t="n"/>
+      <c r="I70" s="12" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="10" t="inlineStr">
         <is>
           <t>❓ 待確認問題</t>
         </is>
       </c>
     </row>
-    <row r="72">
-      <c r="A72" s="4" t="inlineStr">
+    <row r="73">
+      <c r="A73" s="4" t="inlineStr">
         <is>
           <t>編號</t>
         </is>
       </c>
-      <c r="B72" s="4" t="inlineStr">
+      <c r="B73" s="4" t="inlineStr">
         <is>
           <t>問題</t>
         </is>
       </c>
-      <c r="C72" s="4" t="inlineStr">
+      <c r="C73" s="4" t="inlineStr">
         <is>
           <t>影響的任務 / 為什麼重要</t>
-        </is>
-      </c>
-      <c r="D72" s="11" t="n"/>
-      <c r="E72" s="11" t="n"/>
-      <c r="F72" s="11" t="n"/>
-      <c r="G72" s="11" t="n"/>
-      <c r="H72" s="11" t="n"/>
-      <c r="I72" s="12" t="n"/>
-    </row>
-    <row r="73" ht="18" customHeight="1">
-      <c r="A73" s="13" t="inlineStr">
-        <is>
-          <t>Q3</t>
-        </is>
-      </c>
-      <c r="B73" s="6" t="inlineStr">
-        <is>
-          <t>韌體打算閉源商業銷售嗎？</t>
-        </is>
-      </c>
-      <c r="C73" s="6" t="inlineStr">
-        <is>
-          <t>P1-06, P1-07：決定 GPL／LGPL 依賴要開源還是替換。</t>
         </is>
       </c>
       <c r="D73" s="11" t="n"/>
@@ -2516,73 +2525,96 @@
       <c r="H73" s="11" t="n"/>
       <c r="I73" s="12" t="n"/>
     </row>
-    <row r="75">
-      <c r="A75" s="10" t="inlineStr">
+    <row r="74" ht="18" customHeight="1">
+      <c r="A74" s="13" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="B74" s="6" t="inlineStr">
+        <is>
+          <t>韌體打算閉源商業銷售嗎？</t>
+        </is>
+      </c>
+      <c r="C74" s="6" t="inlineStr">
+        <is>
+          <t>P1-06, P1-07：決定 GPL／LGPL 依賴要開源還是替換。</t>
+        </is>
+      </c>
+      <c r="D74" s="11" t="n"/>
+      <c r="E74" s="11" t="n"/>
+      <c r="F74" s="11" t="n"/>
+      <c r="G74" s="11" t="n"/>
+      <c r="H74" s="11" t="n"/>
+      <c r="I74" s="12" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="10" t="inlineStr">
         <is>
           <t>說明</t>
         </is>
       </c>
     </row>
-    <row r="76" ht="32" customHeight="1">
-      <c r="A76" s="14" t="inlineStr">
+    <row r="77" ht="32" customHeight="1">
+      <c r="A77" s="14" t="inlineStr">
         <is>
           <t>・狀態：未開始 → 進行中 → 已完成。只有測試真的跑過而且通過才算已完成；阻塞要在備註寫原因；不再需要的任務標不適用，不要刪。</t>
-        </is>
-      </c>
-    </row>
-    <row r="77" ht="18" customHeight="1">
-      <c r="A77" s="14" t="inlineStr">
-        <is>
-          <t>・測試結果：未測試 / 通過 / 失敗 / 部分通過。測試證據寫跑了什麼、看到什麼，完整歷史在「更新記錄」。</t>
         </is>
       </c>
     </row>
     <row r="78" ht="18" customHeight="1">
       <c r="A78" s="14" t="inlineStr">
         <is>
-          <t>・「接下來」按階段排序，同一階段內再按優先級；依賴還沒滿足的任務不會出現在「接下來」。</t>
+          <t>・測試結果：未測試 / 通過 / 失敗 / 部分通過。測試證據寫跑了什麼、看到什麼，完整歷史在「更新記錄」。</t>
         </is>
       </c>
     </row>
     <row r="79" ht="18" customHeight="1">
       <c r="A79" s="14" t="inlineStr">
         <is>
+          <t>・「接下來」按階段排序，同一階段內再按優先級；依賴還沒滿足的任務不會出現在「接下來」。</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="18" customHeight="1">
+      <c r="A80" s="14" t="inlineStr">
+        <is>
           <t>・可以手動改：「任務清單」的狀態、測試結果、測試證據、Commit、備註，以及「待確認問題」的回答。其餘欄位和本頁由腳本維護。</t>
         </is>
       </c>
     </row>
-    <row r="80" ht="32" customHeight="1">
-      <c r="A80" s="14" t="inlineStr">
+    <row r="81" ht="32" customHeight="1">
+      <c r="A81" s="14" t="inlineStr">
         <is>
           <t>・建議用法：在 Claude Code 對 Claude 說「P0-02 做完了」或輸入 /prod-readiness。Claude 會先跑測試再更新，並寫進「更新記錄」。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="61">
+  <mergeCells count="62">
     <mergeCell ref="E21:I21"/>
     <mergeCell ref="C61:I61"/>
     <mergeCell ref="C52:I52"/>
-    <mergeCell ref="A75:I75"/>
+    <mergeCell ref="C70:I70"/>
     <mergeCell ref="E24:I24"/>
+    <mergeCell ref="E42:I42"/>
     <mergeCell ref="A80:I80"/>
     <mergeCell ref="E33:I33"/>
     <mergeCell ref="A3:I3"/>
     <mergeCell ref="E23:I23"/>
-    <mergeCell ref="C72:I72"/>
     <mergeCell ref="E39:I39"/>
+    <mergeCell ref="A50:I50"/>
     <mergeCell ref="C67:I67"/>
+    <mergeCell ref="E48:I48"/>
     <mergeCell ref="C57:I57"/>
     <mergeCell ref="C53:I53"/>
     <mergeCell ref="C66:I66"/>
-    <mergeCell ref="E44:I44"/>
     <mergeCell ref="A2:I2"/>
     <mergeCell ref="E29:I29"/>
     <mergeCell ref="E35:I35"/>
     <mergeCell ref="E20:I20"/>
     <mergeCell ref="E38:I38"/>
     <mergeCell ref="C69:I69"/>
-    <mergeCell ref="A71:I71"/>
     <mergeCell ref="A76:I76"/>
     <mergeCell ref="E28:I28"/>
     <mergeCell ref="C62:I62"/>
@@ -2590,14 +2622,17 @@
     <mergeCell ref="E31:I31"/>
     <mergeCell ref="E40:I40"/>
     <mergeCell ref="C58:I58"/>
+    <mergeCell ref="A72:I72"/>
     <mergeCell ref="E30:I30"/>
-    <mergeCell ref="A43:I43"/>
+    <mergeCell ref="A81:I81"/>
     <mergeCell ref="E34:I34"/>
     <mergeCell ref="A19:I19"/>
+    <mergeCell ref="C74:I74"/>
     <mergeCell ref="C64:I64"/>
     <mergeCell ref="C51:I51"/>
     <mergeCell ref="E46:I46"/>
     <mergeCell ref="C73:I73"/>
+    <mergeCell ref="A44:I44"/>
     <mergeCell ref="E27:I27"/>
     <mergeCell ref="E45:I45"/>
     <mergeCell ref="C54:I54"/>
@@ -2607,8 +2642,6 @@
     <mergeCell ref="C65:I65"/>
     <mergeCell ref="E26:I26"/>
     <mergeCell ref="C55:I55"/>
-    <mergeCell ref="C50:I50"/>
-    <mergeCell ref="A49:I49"/>
     <mergeCell ref="C56:I56"/>
     <mergeCell ref="E32:I32"/>
     <mergeCell ref="E25:I25"/>
@@ -3663,7 +3696,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="32" customHeight="1">
+    <row r="14" ht="144" customHeight="1">
       <c r="A14" s="13" t="inlineStr">
         <is>
           <t>P0-13</t>
@@ -3691,12 +3724,12 @@
       </c>
       <c r="F14" s="13" t="inlineStr">
         <is>
-          <t>未開始</t>
+          <t>進行中</t>
         </is>
       </c>
       <c r="G14" s="13" t="inlineStr">
         <is>
-          <t>未測試</t>
+          <t>部分通過</t>
         </is>
       </c>
       <c r="H14" s="13" t="n"/>
@@ -3722,9 +3755,21 @@
         </is>
       </c>
       <c r="M14" s="13" t="n"/>
-      <c r="N14" s="6" t="n"/>
-      <c r="O14" s="13" t="n"/>
-      <c r="P14" s="6" t="n"/>
+      <c r="N14" s="6" t="inlineStr">
+        <is>
+          <t>本機：firmware_releases + 私有 bucket + /api/ota/check + /api/ota/firmware/[id]，API 16/16（無 token/web token/過期 → 401；只提供本板 current release；下載 1654400 bytes 與 build sha256 一致；回滾過的版本不再提供並記在 devices）；release_firmware.py 拒 localws build、拒重複版本；pio 18 個 env 全 SUCCESS，spotpear 1.58MB/2MB；Arduino 2.0.17 bootloader 已開 CONFIG_BOOTLOADER_APP_ROLLBACK_ENABLE（C3/S3）。①② 實機未做</t>
+        </is>
+      </c>
+      <c r="O14" s="13" t="inlineStr">
+        <is>
+          <t>b27cc07</t>
+        </is>
+      </c>
+      <c r="P14" s="6" t="inlineStr">
+        <is>
+          <t>[2026-10-08] 2026-10-08 b27cc07（分支 p0-13-ota）。部署時要套 20261008100000_firmware_releases.sql，發佈要用 SUPABASE_URL+service key 跑 tools/release_firmware.py</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="60" customHeight="1">
       <c r="A15" s="13" t="inlineStr">
@@ -7134,7 +7179,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I117"/>
+  <dimension ref="A1:I119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -11246,8 +11291,86 @@
         </is>
       </c>
     </row>
+    <row r="118" ht="32" customHeight="1">
+      <c r="A118" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-07 22:06</t>
+        </is>
+      </c>
+      <c r="B118" s="13" t="inlineStr">
+        <is>
+          <t>P0-13</t>
+        </is>
+      </c>
+      <c r="C118" s="6" t="inlineStr">
+        <is>
+          <t>讓 OTA 真正可用並能回滾</t>
+        </is>
+      </c>
+      <c r="D118" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E118" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F118" s="13" t="n"/>
+      <c r="G118" s="6" t="n"/>
+      <c r="H118" s="13" t="n"/>
+      <c r="I118" s="6" t="n"/>
+    </row>
+    <row r="119" ht="130" customHeight="1">
+      <c r="A119" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-08 09:04</t>
+        </is>
+      </c>
+      <c r="B119" s="13" t="inlineStr">
+        <is>
+          <t>P0-13</t>
+        </is>
+      </c>
+      <c r="C119" s="6" t="inlineStr">
+        <is>
+          <t>讓 OTA 真正可用並能回滾</t>
+        </is>
+      </c>
+      <c r="D119" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="E119" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F119" s="13" t="inlineStr">
+        <is>
+          <t>部分通過</t>
+        </is>
+      </c>
+      <c r="G119" s="6" t="inlineStr">
+        <is>
+          <t>本機：firmware_releases + 私有 bucket + /api/ota/check + /api/ota/firmware/[id]，API 16/16（無 token/web token/過期 → 401；只提供本板 current release；下載 1654400 bytes 與 build sha256 一致；回滾過的版本不再提供並記在 devices）；release_firmware.py 拒 localws build、拒重複版本；pio 18 個 env 全 SUCCESS，spotpear 1.58MB/2MB；Arduino 2.0.17 bootloader 已開 CONFIG_BOOTLOADER_APP_ROLLBACK_ENABLE（C3/S3）。①② 實機未做</t>
+        </is>
+      </c>
+      <c r="H119" s="13" t="inlineStr">
+        <is>
+          <t>b27cc07</t>
+        </is>
+      </c>
+      <c r="I119" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-08 b27cc07（分支 p0-13-ota）。部署時要套 20261008100000_firmware_releases.sql，發佈要用 SUPABASE_URL+service key 跑 tools/release_firmware.py</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I117"/>
+  <autoFilter ref="A1:I119"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record P0-13: OTA upgrade and rollback pass on the dev board.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/production-readiness.xlsx
+++ b/docs/production-readiness.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'任務清單'!$A$1:$P$56</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'待確認問題'!$A$1:$G$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$119</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$120</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -665,7 +665,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>最後更新：2026-10-08 09:04　·　本頁由 tracker.py 自動生成，請勿手動編輯</t>
+          <t>最後更新：2026-10-08 09:30　·　本頁由 tracker.py 自動生成，請勿手動編輯</t>
         </is>
       </c>
     </row>
@@ -1679,7 +1679,7 @@
       <c r="H35" s="11" t="n"/>
       <c r="I35" s="12" t="n"/>
     </row>
-    <row r="36" ht="172" customHeight="1">
+    <row r="36" ht="186" customHeight="1">
       <c r="A36" s="13" t="inlineStr">
         <is>
           <t>P0-13</t>
@@ -1702,7 +1702,7 @@
       </c>
       <c r="E36" s="6" t="inlineStr">
         <is>
-          <t>上次測試：部分通過 — 本機：firmware_releases + 私有 bucket + /api/ota/check + /api/ota/firmware/[id]，API 16/16（無 token/web token/過期 → 401；只提供本板 current release；下載 1654400 bytes 與 build sha256 一致；回滾過的版本不再提供並記在 devices）；release_firmware.py 拒 localws build、拒重複版本；pio 18 個 env 全 SUCCESS，spotpear 1.58MB/2MB；Arduino 2.0.17 bootloader 已開 CONFIG_BOOTLOADER_APP_ROLLBACK_ENABLE（C3/S3）。①② 實機未做
+          <t>上次測試：通過 — 實機開發板 63:64（localall，本機後端）：① 1.1.0→1.2.1 OTA 下載 14s、sha256 過、重啟到 app1 試用、連上語音伺服器後穩定 120s 才 confirmed、開場白播完、devices 記 1.2.1 ② 推開機 3s 崩潰的 1.2.2：安裝→崩潰→bootloader 1s 內回到 1.2.1『rolled back from 1.2.2』→上報 ota_failed_version=1.2.2→再重啟不再下載。過程中測出並修好 2 個 bug：收到 auth 即確認太早（1.0.2 確認後崩潰循環，887b769 改為穩定 2 分鐘）；millis()|1 計時繞回導致誤回滾（3a874dd）。API 16/16，pio 全 env 通過
 填入真實 URL 與 CA；新韌體啟動自檢通過才標記有效，否則自動回滾；設備上報韌體版本。</t>
         </is>
       </c>
@@ -3696,7 +3696,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="144" customHeight="1">
+    <row r="14" ht="214" customHeight="1">
       <c r="A14" s="13" t="inlineStr">
         <is>
           <t>P0-13</t>
@@ -3729,7 +3729,7 @@
       </c>
       <c r="G14" s="13" t="inlineStr">
         <is>
-          <t>部分通過</t>
+          <t>通過</t>
         </is>
       </c>
       <c r="H14" s="13" t="n"/>
@@ -3757,17 +3757,18 @@
       <c r="M14" s="13" t="n"/>
       <c r="N14" s="6" t="inlineStr">
         <is>
-          <t>本機：firmware_releases + 私有 bucket + /api/ota/check + /api/ota/firmware/[id]，API 16/16（無 token/web token/過期 → 401；只提供本板 current release；下載 1654400 bytes 與 build sha256 一致；回滾過的版本不再提供並記在 devices）；release_firmware.py 拒 localws build、拒重複版本；pio 18 個 env 全 SUCCESS，spotpear 1.58MB/2MB；Arduino 2.0.17 bootloader 已開 CONFIG_BOOTLOADER_APP_ROLLBACK_ENABLE（C3/S3）。①② 實機未做</t>
+          <t>實機開發板 63:64（localall，本機後端）：① 1.1.0→1.2.1 OTA 下載 14s、sha256 過、重啟到 app1 試用、連上語音伺服器後穩定 120s 才 confirmed、開場白播完、devices 記 1.2.1 ② 推開機 3s 崩潰的 1.2.2：安裝→崩潰→bootloader 1s 內回到 1.2.1『rolled back from 1.2.2』→上報 ota_failed_version=1.2.2→再重啟不再下載。過程中測出並修好 2 個 bug：收到 auth 即確認太早（1.0.2 確認後崩潰循環，887b769 改為穩定 2 分鐘）；millis()|1 計時繞回導致誤回滾（3a874dd）。API 16/16，pio 全 env 通過</t>
         </is>
       </c>
       <c r="O14" s="13" t="inlineStr">
         <is>
-          <t>b27cc07</t>
+          <t>3a874dd</t>
         </is>
       </c>
       <c r="P14" s="6" t="inlineStr">
         <is>
-          <t>[2026-10-08] 2026-10-08 b27cc07（分支 p0-13-ota）。部署時要套 20261008100000_firmware_releases.sql，發佈要用 SUPABASE_URL+service key 跑 tools/release_firmware.py</t>
+          <t>[2026-10-08] 2026-10-08 b27cc07（分支 p0-13-ota）。部署時要套 20261008100000_firmware_releases.sql，發佈要用 SUPABASE_URL+service key 跑 tools/release_firmware.py
+[2026-10-08] 2026-10-08 實機①②通過，未部署。上線要：套 20261008100000、部署前端、用 release_firmware.py 發佈正式 build；生產 HTTPS（同 CF CA）的 1.6MB 下載尚未在線上驗證。開發板現跑 1.2.1 localall。未做：已確認版本日後若崩潰循環不會自動切回舊槽，需 USB 救（可另立任務）</t>
         </is>
       </c>
     </row>
@@ -7179,7 +7180,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I119"/>
+  <dimension ref="A1:I120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -11369,8 +11370,55 @@
         </is>
       </c>
     </row>
+    <row r="120" ht="144" customHeight="1">
+      <c r="A120" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-08 09:30</t>
+        </is>
+      </c>
+      <c r="B120" s="13" t="inlineStr">
+        <is>
+          <t>P0-13</t>
+        </is>
+      </c>
+      <c r="C120" s="6" t="inlineStr">
+        <is>
+          <t>讓 OTA 真正可用並能回滾</t>
+        </is>
+      </c>
+      <c r="D120" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="E120" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F120" s="13" t="inlineStr">
+        <is>
+          <t>通過</t>
+        </is>
+      </c>
+      <c r="G120" s="6" t="inlineStr">
+        <is>
+          <t>實機開發板 63:64（localall，本機後端）：① 1.1.0→1.2.1 OTA 下載 14s、sha256 過、重啟到 app1 試用、連上語音伺服器後穩定 120s 才 confirmed、開場白播完、devices 記 1.2.1 ② 推開機 3s 崩潰的 1.2.2：安裝→崩潰→bootloader 1s 內回到 1.2.1『rolled back from 1.2.2』→上報 ota_failed_version=1.2.2→再重啟不再下載。過程中測出並修好 2 個 bug：收到 auth 即確認太早（1.0.2 確認後崩潰循環，887b769 改為穩定 2 分鐘）；millis()|1 計時繞回導致誤回滾（3a874dd）。API 16/16，pio 全 env 通過</t>
+        </is>
+      </c>
+      <c r="H120" s="13" t="inlineStr">
+        <is>
+          <t>3a874dd</t>
+        </is>
+      </c>
+      <c r="I120" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-08 實機①②通過，未部署。上線要：套 20261008100000、部署前端、用 release_firmware.py 發佈正式 build；生產 HTTPS（同 CF CA）的 1.6MB 下載尚未在線上驗證。開發板現跑 1.2.1 localall。未做：已確認版本日後若崩潰循環不會自動切回舊槽，需 USB 救（可另立任務）</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I119"/>
+  <autoFilter ref="A1:I120"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Track the C3 async_tcp watchdog reset found during the OTA test.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/production-readiness.xlsx
+++ b/docs/production-readiness.xlsx
@@ -13,9 +13,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="更新記錄" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'任務清單'!$A$1:$P$56</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'任務清單'!$A$1:$P$57</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'待確認問題'!$A$1:$G$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$120</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$122</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -665,14 +665,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>最後更新：2026-10-08 09:30　·　本頁由 tracker.py 自動生成，請勿手動編輯</t>
+          <t>最後更新：2026-10-08 09:45　·　本頁由 tracker.py 自動生成，請勿手動編輯</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>總進度：3/54 已完成（6%）　·　目前階段：1 止血定案（10/5–10/16）</t>
+          <t>總進度：3/55 已完成（5%）　·　目前階段：1 止血定案（10/5–10/16）</t>
         </is>
       </c>
     </row>
@@ -816,11 +816,11 @@
       </c>
       <c r="C8" s="7">
         <f>COUNTIF('任務清單'!$B:$B,$A8)</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D8" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A8,'任務清單'!$F:$F,D$5)</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E8" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A8,'任務清單'!$F:$F,E$5)</f>
@@ -840,7 +840,7 @@
       </c>
       <c r="I8" s="8">
         <f>IFERROR(F8/(C8-H8),0)</f>
-        <v>0.2</v>
+        <v>0.18181818181818182</v>
       </c>
     </row>
     <row r="9" ht="18" customHeight="1">
@@ -892,11 +892,11 @@
       <c r="B10" s="6" t="n"/>
       <c r="C10" s="5">
         <f>SUM(C6:C9)</f>
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D10" s="5">
         <f>SUM(D6:D9)</f>
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E10" s="5">
         <f>SUM(E6:E9)</f>
@@ -916,7 +916,7 @@
       </c>
       <c r="I10" s="9">
         <f>IFERROR(F10/(C10-H10),0)</f>
-        <v>0.05555555555555555</v>
+        <v>0.05454545454545454</v>
       </c>
     </row>
     <row r="12">
@@ -1019,11 +1019,11 @@
       </c>
       <c r="C14" s="7">
         <f>COUNTIF('任務清單'!$C:$C,$A14)</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D14" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A14,'任務清單'!$F:$F,D$12)</f>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E14" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A14,'任務清單'!$F:$F,E$12)</f>
@@ -1135,11 +1135,11 @@
       <c r="B17" s="6" t="n"/>
       <c r="C17" s="5">
         <f>SUM(C13:C16)</f>
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D17" s="5">
         <f>SUM(D13:D16)</f>
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E17" s="5">
         <f>SUM(E13:E16)</f>
@@ -1159,7 +1159,7 @@
       </c>
       <c r="I17" s="9">
         <f>IFERROR(F17/(C17-H17),0)</f>
-        <v>0.05555555555555555</v>
+        <v>0.05454545454545454</v>
       </c>
     </row>
     <row r="19">
@@ -2683,7 +2683,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P56"/>
+  <dimension ref="A1:P57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3696,7 +3696,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="214" customHeight="1">
+    <row r="14" ht="382" customHeight="1">
       <c r="A14" s="13" t="inlineStr">
         <is>
           <t>P0-13</t>
@@ -3762,13 +3762,14 @@
       </c>
       <c r="O14" s="13" t="inlineStr">
         <is>
-          <t>3a874dd</t>
+          <t>68b9550</t>
         </is>
       </c>
       <c r="P14" s="6" t="inlineStr">
         <is>
           <t>[2026-10-08] 2026-10-08 b27cc07（分支 p0-13-ota）。部署時要套 20261008100000_firmware_releases.sql，發佈要用 SUPABASE_URL+service key 跑 tools/release_firmware.py
-[2026-10-08] 2026-10-08 實機①②通過，未部署。上線要：套 20261008100000、部署前端、用 release_firmware.py 發佈正式 build；生產 HTTPS（同 CF CA）的 1.6MB 下載尚未在線上驗證。開發板現跑 1.2.1 localall。未做：已確認版本日後若崩潰循環不會自動切回舊槽，需 USB 救（可另立任務）</t>
+[2026-10-08] 2026-10-08 實機①②通過，未部署。上線要：套 20261008100000、部署前端、用 release_firmware.py 發佈正式 build；生產 HTTPS（同 CF CA）的 1.6MB 下載尚未在線上驗證。開發板現跑 1.2.1 localall。未做：已確認版本日後若崩潰循環不會自動切回舊槽，需 USB 救（可另立任務）
+[2026-10-08] 2026-10-08 OTA 檢查併入 /api/generate_auth_token（68b9550），開機回到一次 TLS 握手；/api/ota/check 移除。token 路徑 API 11/11（舊韌體無 ota、格式錯仍發 token、回滾版本不再提供）；實機 1.3.0→1.3.1 經 token 回應安裝、試用、播完開場白、120s 確認。第一次升級 1.3.1 被 async_tcp 任務看門狗觸發重啟並正確回滾——是既有韌體 bug，見新任務</t>
         </is>
       </c>
     </row>
@@ -6716,8 +6717,71 @@
         </is>
       </c>
     </row>
+    <row r="57" ht="102" customHeight="1">
+      <c r="A57" s="13" t="inlineStr">
+        <is>
+          <t>P2-11</t>
+        </is>
+      </c>
+      <c r="B57" s="13" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C57" s="13" t="inlineStr">
+        <is>
+          <t>2 內測準備</t>
+        </is>
+      </c>
+      <c r="D57" s="6" t="inlineStr">
+        <is>
+          <t>工程</t>
+        </is>
+      </c>
+      <c r="E57" s="6" t="inlineStr">
+        <is>
+          <t>C3 播放時 async_tcp 觸發任務看門狗重啟</t>
+        </is>
+      </c>
+      <c r="F57" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="G57" s="13" t="inlineStr">
+        <is>
+          <t>未測試</t>
+        </is>
+      </c>
+      <c r="I57" s="6" t="inlineStr">
+        <is>
+          <t>AsyncTCP 在 ESP32 預設把 async_tcp task 加入 5 秒任務看門狗（CONFIG_ASYNC_TCP_USE_WDT=1）。C3 單核，播開場白時 Opus Decode 連續佔用 CPU，async_tcp 超過 5 秒輪不到 → abort 重啟。2026-10-08 開發板實測出現一次（播開場白第 5 秒）。孩子聽回覆時玩具會突然重啟；落在 OTA 試用期內時，好版本會被回滾並記為失敗</t>
+        </is>
+      </c>
+      <c r="J57" s="6" t="inlineStr">
+        <is>
+          <t>firmware-arduino/platformio.ini（AsyncTCP 3.5.0）；src/Audio.cpp decodeTask 優先級與讓出</t>
+        </is>
+      </c>
+      <c r="K57" s="6" t="inlineStr">
+        <is>
+          <t>C3 env 不再因 async_tcp 觸發看門狗：關閉 AsyncTCP 的 WDT 訂閱（-D CONFIG_ASYNC_TCP_USE_WDT=0）或讓解碼 task 定期讓出 CPU；播放與 SoftAP 配網都仍正常</t>
+        </is>
+      </c>
+      <c r="L57" s="6" t="inlineStr">
+        <is>
+          <t>① Spotpear 開發板連續開機 30 次並播完開場白、再進行 20 輪對話，串口 0 次 task_wdt ② SoftAP 配網頁面仍能打開並保存 WiFi</t>
+        </is>
+      </c>
+      <c r="M57" s="13" t="n"/>
+      <c r="P57" s="6" t="inlineStr">
+        <is>
+          <t>[2026-10-08] 新增</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P56"/>
+  <autoFilter ref="A1:P57"/>
   <conditionalFormatting sqref="F2:F1000">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"已完成"</formula>
@@ -7180,7 +7244,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I120"/>
+  <dimension ref="A1:I122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -11417,8 +11481,74 @@
         </is>
       </c>
     </row>
+    <row r="121" ht="144" customHeight="1">
+      <c r="A121" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-08 09:45</t>
+        </is>
+      </c>
+      <c r="B121" s="13" t="inlineStr">
+        <is>
+          <t>P0-13</t>
+        </is>
+      </c>
+      <c r="C121" s="6" t="inlineStr">
+        <is>
+          <t>讓 OTA 真正可用並能回滾</t>
+        </is>
+      </c>
+      <c r="D121" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="E121" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F121" s="13" t="n"/>
+      <c r="G121" s="6" t="n"/>
+      <c r="H121" s="13" t="inlineStr">
+        <is>
+          <t>68b9550</t>
+        </is>
+      </c>
+      <c r="I121" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-08 OTA 檢查併入 /api/generate_auth_token（68b9550），開機回到一次 TLS 握手；/api/ota/check 移除。token 路徑 API 11/11（舊韌體無 ota、格式錯仍發 token、回滾版本不再提供）；實機 1.3.0→1.3.1 經 token 回應安裝、試用、播完開場白、120s 確認。第一次升級 1.3.1 被 async_tcp 任務看門狗觸發重啟並正確回滾——是既有韌體 bug，見新任務</t>
+        </is>
+      </c>
+    </row>
+    <row r="122" ht="32" customHeight="1">
+      <c r="A122" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-08 09:45</t>
+        </is>
+      </c>
+      <c r="B122" s="13" t="inlineStr">
+        <is>
+          <t>P2-11</t>
+        </is>
+      </c>
+      <c r="C122" s="6" t="inlineStr">
+        <is>
+          <t>C3 播放時 async_tcp 觸發任務看門狗重啟</t>
+        </is>
+      </c>
+      <c r="E122" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="I122" s="6" t="inlineStr">
+        <is>
+          <t>新增任務</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I120"/>
+  <autoFilter ref="A1:I122"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record P2-11: decode-sample freeze found and fixed, 30 boots clean.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/production-readiness.xlsx
+++ b/docs/production-readiness.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'任務清單'!$A$1:$P$57</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'待確認問題'!$A$1:$G$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$122</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$125</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -641,7 +641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I81"/>
+  <dimension ref="A1:I82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -665,7 +665,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>最後更新：2026-10-08 09:45　·　本頁由 tracker.py 自動生成，請勿手動編輯</t>
+          <t>最後更新：2026-10-08 10:42　·　本頁由 tracker.py 自動生成，請勿手動編輯</t>
         </is>
       </c>
     </row>
@@ -820,11 +820,11 @@
       </c>
       <c r="D8" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A8,'任務清單'!$F:$F,D$5)</f>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E8" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A8,'任務清單'!$F:$F,E$5)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F8" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A8,'任務清單'!$F:$F,F$5)</f>
@@ -896,11 +896,11 @@
       </c>
       <c r="D10" s="5">
         <f>SUM(D6:D9)</f>
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E10" s="5">
         <f>SUM(E6:E9)</f>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F10" s="5">
         <f>SUM(F6:F9)</f>
@@ -1023,11 +1023,11 @@
       </c>
       <c r="D14" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A14,'任務清單'!$F:$F,D$12)</f>
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E14" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A14,'任務清單'!$F:$F,E$12)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F14" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A14,'任務清單'!$F:$F,F$12)</f>
@@ -1139,11 +1139,11 @@
       </c>
       <c r="D17" s="5">
         <f>SUM(D13:D16)</f>
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E17" s="5">
         <f>SUM(E13:E16)</f>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F17" s="5">
         <f>SUM(F13:F16)</f>
@@ -1711,15 +1711,15 @@
       <c r="H36" s="11" t="n"/>
       <c r="I36" s="12" t="n"/>
     </row>
-    <row r="37" ht="60" customHeight="1">
+    <row r="37" ht="144" customHeight="1">
       <c r="A37" s="13" t="inlineStr">
         <is>
-          <t>P1-01</t>
+          <t>P2-11</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>加入內容審核層（輸入與輸出）</t>
+          <t>C3 播放時 async_tcp 觸發任務看門狗重啟</t>
         </is>
       </c>
       <c r="C37" s="13" t="inlineStr">
@@ -1729,12 +1729,13 @@
       </c>
       <c r="D37" s="13" t="inlineStr">
         <is>
-          <t>未開始</t>
+          <t>進行中</t>
         </is>
       </c>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>STT 文字與 LLM 輸出都經審核，尺度按 3–6 歲；命中時換成安全回覆並記錄事件，事件只記類別、時間、角色，不記原文（管理員不能看兒童內容，見 Q7）；首字延遲增加 ≤150ms。</t>
+          <t>上次測試：部分通過 — ① 1.3.4 localall 連續重啟 30 次：開場白 30/30、task_wdt 0、panic 0（修正前 19 次 4 次）；CPU 抽樣仍每輪 2–7 次，解碼約 8.6–9.3ms/封包。排除過程：關 AsyncTCP WDT 只把重啟變成卡住（30 次 3 次靜默&gt;17s）；Serial.setTxTimeoutMs(0) 仍 30 次 2 次 → 均撤回。② 20 輪對話待用戶
+排程器暫停期間不可呼叫會阻塞的寫入：只在環形緩衝區放得下最大解碼封包（120ms）時才做 CPU 抽樣；AsyncTCP 看門狗保持開啟以便抓到同類問題</t>
         </is>
       </c>
       <c r="F37" s="11" t="n"/>
@@ -1742,15 +1743,15 @@
       <c r="H37" s="11" t="n"/>
       <c r="I37" s="12" t="n"/>
     </row>
-    <row r="38" ht="32" customHeight="1">
+    <row r="38" ht="60" customHeight="1">
       <c r="A38" s="13" t="inlineStr">
         <is>
-          <t>P1-02</t>
+          <t>P1-01</t>
         </is>
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>日誌移除兒童個人資料</t>
+          <t>加入內容審核層（輸入與輸出）</t>
         </is>
       </c>
       <c r="C38" s="13" t="inlineStr">
@@ -1765,7 +1766,7 @@
       </c>
       <c r="E38" s="6" t="inlineStr">
         <is>
-          <t>生產日誌只記 ID、長度、類別，不記內容；內容只在 DEBUG 等級輸出，生產不開 DEBUG。</t>
+          <t>STT 文字與 LLM 輸出都經審核，尺度按 3–6 歲；命中時換成安全回覆並記錄事件，事件只記類別、時間、角色，不記原文（管理員不能看兒童內容，見 Q7）；首字延遲增加 ≤150ms。</t>
         </is>
       </c>
       <c r="F38" s="11" t="n"/>
@@ -1773,15 +1774,15 @@
       <c r="H38" s="11" t="n"/>
       <c r="I38" s="12" t="n"/>
     </row>
-    <row r="39" ht="46" customHeight="1">
+    <row r="39" ht="32" customHeight="1">
       <c r="A39" s="13" t="inlineStr">
         <is>
-          <t>P1-09</t>
+          <t>P1-02</t>
         </is>
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>家長鎖：孩子模式進設定要輸入 PIN</t>
+          <t>日誌移除兒童個人資料</t>
         </is>
       </c>
       <c r="C39" s="13" t="inlineStr">
@@ -1796,7 +1797,7 @@
       </c>
       <c r="E39" s="6" t="inlineStr">
         <is>
-          <t>從孩子模式進入設定、家長控制、記憶、設備頁面前，都要先輸入家長 PIN（第一次使用時設定）；連錯 5 次鎖定 5 分鐘；忘記 PIN 可用帳號密碼重設。</t>
+          <t>生產日誌只記 ID、長度、類別，不記內容；內容只在 DEBUG 等級輸出，生產不開 DEBUG。</t>
         </is>
       </c>
       <c r="F39" s="11" t="n"/>
@@ -1807,12 +1808,12 @@
     <row r="40" ht="46" customHeight="1">
       <c r="A40" s="13" t="inlineStr">
         <is>
-          <t>P1-11</t>
+          <t>P1-09</t>
         </is>
       </c>
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>伺服器與資料庫直接存取的管控</t>
+          <t>家長鎖：孩子模式進設定要輸入 PIN</t>
         </is>
       </c>
       <c r="C40" s="13" t="inlineStr">
@@ -1827,7 +1828,7 @@
       </c>
       <c r="E40" s="6" t="inlineStr">
         <is>
-          <t>列出誰有 SSH 與資料庫直連權限（越少越好）；service_role key 只存在伺服器的 env；私隱政策寫明這類存取的範圍；每次直接查看生產資料都留記錄。</t>
+          <t>從孩子模式進入設定、家長控制、記憶、設備頁面前，都要先輸入家長 PIN（第一次使用時設定）；連錯 5 次鎖定 5 分鐘；忘記 PIN 可用帳號密碼重設。</t>
         </is>
       </c>
       <c r="F40" s="11" t="n"/>
@@ -1838,12 +1839,12 @@
     <row r="41" ht="46" customHeight="1">
       <c r="A41" s="13" t="inlineStr">
         <is>
-          <t>P2-02</t>
+          <t>P1-11</t>
         </is>
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>CI 跑測試與靜態檢查</t>
+          <t>伺服器與資料庫直接存取的管控</t>
         </is>
       </c>
       <c r="C41" s="13" t="inlineStr">
@@ -1858,7 +1859,7 @@
       </c>
       <c r="E41" s="6" t="inlineStr">
         <is>
-          <t>推送與 PR 時跑 pytest、ruff、pyright、next lint、tsc --noEmit、pio run；任何一項失敗就不發佈 image。</t>
+          <t>列出誰有 SSH 與資料庫直連權限（越少越好）；service_role key 只存在伺服器的 env；私隱政策寫明這類存取的範圍；每次直接查看生產資料都留記錄。</t>
         </is>
       </c>
       <c r="F41" s="11" t="n"/>
@@ -1866,15 +1867,15 @@
       <c r="H41" s="11" t="n"/>
       <c r="I41" s="12" t="n"/>
     </row>
-    <row r="42" ht="32" customHeight="1">
+    <row r="42" ht="46" customHeight="1">
       <c r="A42" s="13" t="inlineStr">
         <is>
-          <t>P2-04</t>
+          <t>P2-02</t>
         </is>
       </c>
       <c r="B42" s="6" t="inlineStr">
         <is>
-          <t>容器改用非 root 用戶</t>
+          <t>CI 跑測試與靜態檢查</t>
         </is>
       </c>
       <c r="C42" s="13" t="inlineStr">
@@ -1889,7 +1890,7 @@
       </c>
       <c r="E42" s="6" t="inlineStr">
         <is>
-          <t>兩個 Dockerfile 都設定非 root 的 USER。</t>
+          <t>推送與 PR 時跑 pytest、ruff、pyright、next lint、tsc --noEmit、pio run；任何一項失敗就不發佈 image。</t>
         </is>
       </c>
       <c r="F42" s="11" t="n"/>
@@ -1897,68 +1898,68 @@
       <c r="H42" s="11" t="n"/>
       <c r="I42" s="12" t="n"/>
     </row>
-    <row r="44">
-      <c r="A44" s="10" t="inlineStr">
+    <row r="43" ht="32" customHeight="1">
+      <c r="A43" s="13" t="inlineStr">
+        <is>
+          <t>P2-04</t>
+        </is>
+      </c>
+      <c r="B43" s="6" t="inlineStr">
+        <is>
+          <t>容器改用非 root 用戶</t>
+        </is>
+      </c>
+      <c r="C43" s="13" t="inlineStr">
+        <is>
+          <t>2 內測準備</t>
+        </is>
+      </c>
+      <c r="D43" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E43" s="6" t="inlineStr">
+        <is>
+          <t>兩個 Dockerfile 都設定非 root 的 USER。</t>
+        </is>
+      </c>
+      <c r="F43" s="11" t="n"/>
+      <c r="G43" s="11" t="n"/>
+      <c r="H43" s="11" t="n"/>
+      <c r="I43" s="12" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="10" t="inlineStr">
         <is>
           <t>✅ 最近完成與測試效果</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="4" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
         <is>
           <t>編號</t>
         </is>
       </c>
-      <c r="B45" s="4" t="inlineStr">
+      <c r="B46" s="4" t="inlineStr">
         <is>
           <t>任務</t>
         </is>
       </c>
-      <c r="C45" s="4" t="inlineStr">
+      <c r="C46" s="4" t="inlineStr">
         <is>
           <t>測試結果</t>
         </is>
       </c>
-      <c r="D45" s="4" t="inlineStr">
+      <c r="D46" s="4" t="inlineStr">
         <is>
           <t>完成日期</t>
         </is>
       </c>
-      <c r="E45" s="4" t="inlineStr">
+      <c r="E46" s="4" t="inlineStr">
         <is>
           <t>測試證據</t>
-        </is>
-      </c>
-      <c r="F45" s="11" t="n"/>
-      <c r="G45" s="11" t="n"/>
-      <c r="H45" s="11" t="n"/>
-      <c r="I45" s="12" t="n"/>
-    </row>
-    <row r="46" ht="88" customHeight="1">
-      <c r="A46" s="13" t="inlineStr">
-        <is>
-          <t>R-03</t>
-        </is>
-      </c>
-      <c r="B46" s="6" t="inlineStr">
-        <is>
-          <t>移除不用的 Deno／Cloudflare 後端與上游預設主機</t>
-        </is>
-      </c>
-      <c r="C46" s="13" t="inlineStr">
-        <is>
-          <t>通過</t>
-        </is>
-      </c>
-      <c r="D46" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-07</t>
-        </is>
-      </c>
-      <c r="E46" s="6" t="inlineStr">
-        <is>
-          <t>① grep deno.dev|workers.dev|railway.app|VOICE_SERVER_DENO|VOICE_SERVER_CLOUDFLARE 全 repo → 只剩 seed.json 的任務描述本身 ② pio run 18 個 env 全 SUCCESS（S3 devkit/Waveshare/xmini-c3/Spotpear 各變體）③ FastAPI pytest 182 passed；另 tsc --noEmit 通過</t>
         </is>
       </c>
       <c r="F46" s="11" t="n"/>
@@ -1969,12 +1970,12 @@
     <row r="47" ht="88" customHeight="1">
       <c r="A47" s="13" t="inlineStr">
         <is>
-          <t>P2-01</t>
+          <t>R-03</t>
         </is>
       </c>
       <c r="B47" s="6" t="inlineStr">
         <is>
-          <t>修好後端測試環境</t>
+          <t>移除不用的 Deno／Cloudflare 後端與上游預設主機</t>
         </is>
       </c>
       <c r="C47" s="13" t="inlineStr">
@@ -1989,7 +1990,7 @@
       </c>
       <c r="E47" s="6" t="inlineStr">
         <is>
-          <t>cd server/fastapi &amp;&amp; .venv/bin/python -m pytest -q → 173 passed（原本 60 個 async 測試報「not natively supported」）；pyproject dev group 加 pytest&gt;=9,&lt;10、pytest-asyncio&gt;=1.4,&lt;2，asyncio_mode=auto；pip install --dry-run --group dev 可解析</t>
+          <t>① grep deno.dev|workers.dev|railway.app|VOICE_SERVER_DENO|VOICE_SERVER_CLOUDFLARE 全 repo → 只剩 seed.json 的任務描述本身 ② pio run 18 個 env 全 SUCCESS（S3 devkit/Waveshare/xmini-c3/Spotpear 各變體）③ FastAPI pytest 182 passed；另 tsc --noEmit 通過</t>
         </is>
       </c>
       <c r="F47" s="11" t="n"/>
@@ -1997,15 +1998,15 @@
       <c r="H47" s="11" t="n"/>
       <c r="I47" s="12" t="n"/>
     </row>
-    <row r="48" ht="60" customHeight="1">
+    <row r="48" ht="88" customHeight="1">
       <c r="A48" s="13" t="inlineStr">
         <is>
-          <t>P2-03</t>
+          <t>P2-01</t>
         </is>
       </c>
       <c r="B48" s="6" t="inlineStr">
         <is>
-          <t>提交目前未提交的改動</t>
+          <t>修好後端測試環境</t>
         </is>
       </c>
       <c r="C48" s="13" t="inlineStr">
@@ -2015,12 +2016,12 @@
       </c>
       <c r="D48" s="13" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="E48" s="6" t="inlineStr">
         <is>
-          <t>git status --short → 0 行；3bc7119..b322375 按主題拆成 5 個 commit（50 檔：xmini-c3 電量、facts 記憶層、日期時間天氣、BEAM 評測、進度追蹤）；git ls-remote mygithub main = HEAD = b322375</t>
+          <t>cd server/fastapi &amp;&amp; .venv/bin/python -m pytest -q → 173 passed（原本 60 個 async 測試報「not natively supported」）；pyproject dev group 加 pytest&gt;=9,&lt;10、pytest-asyncio&gt;=1.4,&lt;2，asyncio_mode=auto；pip install --dry-run --group dev 可解析</t>
         </is>
       </c>
       <c r="F48" s="11" t="n"/>
@@ -2028,50 +2029,58 @@
       <c r="H48" s="11" t="n"/>
       <c r="I48" s="12" t="n"/>
     </row>
-    <row r="50">
-      <c r="A50" s="10" t="inlineStr">
+    <row r="49" ht="60" customHeight="1">
+      <c r="A49" s="13" t="inlineStr">
+        <is>
+          <t>P2-03</t>
+        </is>
+      </c>
+      <c r="B49" s="6" t="inlineStr">
+        <is>
+          <t>提交目前未提交的改動</t>
+        </is>
+      </c>
+      <c r="C49" s="13" t="inlineStr">
+        <is>
+          <t>通過</t>
+        </is>
+      </c>
+      <c r="D49" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="E49" s="6" t="inlineStr">
+        <is>
+          <t>git status --short → 0 行；3bc7119..b322375 按主題拆成 5 個 commit（50 檔：xmini-c3 電量、facts 記憶層、日期時間天氣、BEAM 評測、進度追蹤）；git ls-remote mygithub main = HEAD = b322375</t>
+        </is>
+      </c>
+      <c r="F49" s="11" t="n"/>
+      <c r="G49" s="11" t="n"/>
+      <c r="H49" s="11" t="n"/>
+      <c r="I49" s="12" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="10" t="inlineStr">
         <is>
           <t>⏳ 等待依賴 / ⛔ 阻塞</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="4" t="inlineStr">
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
         <is>
           <t>編號</t>
         </is>
       </c>
-      <c r="B51" s="4" t="inlineStr">
+      <c r="B52" s="4" t="inlineStr">
         <is>
           <t>任務</t>
         </is>
       </c>
-      <c r="C51" s="4" t="inlineStr">
+      <c r="C52" s="4" t="inlineStr">
         <is>
           <t>在等什麼</t>
-        </is>
-      </c>
-      <c r="D51" s="11" t="n"/>
-      <c r="E51" s="11" t="n"/>
-      <c r="F51" s="11" t="n"/>
-      <c r="G51" s="11" t="n"/>
-      <c r="H51" s="11" t="n"/>
-      <c r="I51" s="12" t="n"/>
-    </row>
-    <row r="52" ht="60" customHeight="1">
-      <c r="A52" s="13" t="inlineStr">
-        <is>
-          <t>R-16</t>
-        </is>
-      </c>
-      <c r="B52" s="6" t="inlineStr">
-        <is>
-          <t>Spotpear 量產版加電池電壓檢測（GPIO0 分壓）</t>
-        </is>
-      </c>
-      <c r="C52" s="6" t="inlineStr">
-        <is>
-          <t>阻塞：[2026-10-07] 仍按 10/06 決定暫緩：等用戶做充滿再放電測試（與 R-17 同一次），看 VDD 低電提醒在關機前多久觸發；太遲或不觸發才向 Spotpear 提改板。已把分壓改板的問題一併放進給 Spotpear 的草稿，方便同一封發出</t>
         </is>
       </c>
       <c r="D52" s="11" t="n"/>
@@ -2081,20 +2090,20 @@
       <c r="H52" s="11" t="n"/>
       <c r="I52" s="12" t="n"/>
     </row>
-    <row r="53" ht="88" customHeight="1">
+    <row r="53" ht="60" customHeight="1">
       <c r="A53" s="13" t="inlineStr">
         <is>
-          <t>R-17</t>
+          <t>R-16</t>
         </is>
       </c>
       <c r="B53" s="6" t="inlineStr">
         <is>
-          <t>Spotpear 電池耗盡時插電能否正常開機（供電路徑）</t>
+          <t>Spotpear 量產版加電池電壓檢測（GPIO0 分壓）</t>
         </is>
       </c>
       <c r="C53" s="6" t="inlineStr">
         <is>
-          <t>阻塞：[2026-10-07] 等兩件事：(1) Spotpear 回覆充電芯片型號、充電電流、有沒有 power path（問題已草擬給用戶發送）(2) 用戶做一次實物放電：拔 USB 用到自動關機 → 插 USB 計時到能對話 → 插住用 30 分鐘。與 R-16 的放電測試同一次完成。韌體現況：brownout 重啟會補播低電提醒，運行記錄（開機時 Supply log）會記每次重啟原因，可據此判斷有沒有反覆 brownout；『掉電後先深睡充電』的緩解要等測試證明需要才做</t>
+          <t>阻塞：[2026-10-07] 仍按 10/06 決定暫緩：等用戶做充滿再放電測試（與 R-17 同一次），看 VDD 低電提醒在關機前多久觸發；太遲或不觸發才向 Spotpear 提改板。已把分壓改板的問題一併放進給 Spotpear 的草稿，方便同一封發出</t>
         </is>
       </c>
       <c r="D53" s="11" t="n"/>
@@ -2104,20 +2113,20 @@
       <c r="H53" s="11" t="n"/>
       <c r="I53" s="12" t="n"/>
     </row>
-    <row r="54" ht="18" customHeight="1">
+    <row r="54" ht="88" customHeight="1">
       <c r="A54" s="13" t="inlineStr">
         <is>
-          <t>P0-07</t>
+          <t>R-17</t>
         </is>
       </c>
       <c r="B54" s="6" t="inlineStr">
         <is>
-          <t>輪換 JWT secret，作廢已發出的 token</t>
+          <t>Spotpear 電池耗盡時插電能否正常開機（供電路徑）</t>
         </is>
       </c>
       <c r="C54" s="6" t="inlineStr">
         <is>
-          <t>等 P0-06</t>
+          <t>阻塞：[2026-10-07] 等兩件事：(1) Spotpear 回覆充電芯片型號、充電電流、有沒有 power path（問題已草擬給用戶發送）(2) 用戶做一次實物放電：拔 USB 用到自動關機 → 插 USB 計時到能對話 → 插住用 30 分鐘。與 R-16 的放電測試同一次完成。韌體現況：brownout 重啟會補播低電提醒，運行記錄（開機時 Supply log）會記每次重啟原因，可據此判斷有沒有反覆 brownout；『掉電後先深睡充電』的緩解要等測試證明需要才做</t>
         </is>
       </c>
       <c r="D54" s="11" t="n"/>
@@ -2130,12 +2139,12 @@
     <row r="55" ht="18" customHeight="1">
       <c r="A55" s="13" t="inlineStr">
         <is>
-          <t>P0-11</t>
+          <t>P0-07</t>
         </is>
       </c>
       <c r="B55" s="6" t="inlineStr">
         <is>
-          <t>設備認領要求持有證明</t>
+          <t>輪換 JWT secret，作廢已發出的 token</t>
         </is>
       </c>
       <c r="C55" s="6" t="inlineStr">
@@ -2153,17 +2162,17 @@
     <row r="56" ht="18" customHeight="1">
       <c r="A56" s="13" t="inlineStr">
         <is>
-          <t>P1-10</t>
+          <t>P0-11</t>
         </is>
       </c>
       <c r="B56" s="6" t="inlineStr">
         <is>
-          <t>管理操作審計記錄</t>
+          <t>設備認領要求持有證明</t>
         </is>
       </c>
       <c r="C56" s="6" t="inlineStr">
         <is>
-          <t>等 P0-12</t>
+          <t>等 P0-06</t>
         </is>
       </c>
       <c r="D56" s="11" t="n"/>
@@ -2176,17 +2185,17 @@
     <row r="57" ht="18" customHeight="1">
       <c r="A57" s="13" t="inlineStr">
         <is>
-          <t>R-05</t>
+          <t>P1-10</t>
         </is>
       </c>
       <c r="B57" s="6" t="inlineStr">
         <is>
-          <t>內測版外殼（3D 打印 20 台）</t>
+          <t>管理操作審計記錄</t>
         </is>
       </c>
       <c r="C57" s="6" t="inlineStr">
         <is>
-          <t>等 R-01</t>
+          <t>等 P0-12</t>
         </is>
       </c>
       <c r="D57" s="11" t="n"/>
@@ -2199,17 +2208,17 @@
     <row r="58" ht="18" customHeight="1">
       <c r="A58" s="13" t="inlineStr">
         <is>
-          <t>R-06</t>
+          <t>R-05</t>
         </is>
       </c>
       <c r="B58" s="6" t="inlineStr">
         <is>
-          <t>家長自助上手流程</t>
+          <t>內測版外殼（3D 打印 20 台）</t>
         </is>
       </c>
       <c r="C58" s="6" t="inlineStr">
         <is>
-          <t>等 P0-11</t>
+          <t>等 R-01</t>
         </is>
       </c>
       <c r="D58" s="11" t="n"/>
@@ -2219,20 +2228,20 @@
       <c r="H58" s="11" t="n"/>
       <c r="I58" s="12" t="n"/>
     </row>
-    <row r="59" ht="46" customHeight="1">
+    <row r="59" ht="18" customHeight="1">
       <c r="A59" s="13" t="inlineStr">
         <is>
-          <t>R-13</t>
+          <t>R-06</t>
         </is>
       </c>
       <c r="B59" s="6" t="inlineStr">
         <is>
-          <t>CP1 內測就緒檢查（10/30）</t>
+          <t>家長自助上手流程</t>
         </is>
       </c>
       <c r="C59" s="6" t="inlineStr">
         <is>
-          <t>等 P0-02、P0-03、P0-04、P0-05、P0-06、P0-07、P0-08、P0-09、P0-10、P0-11、P0-12、P0-13、P1-01、P1-02、P2-09、R-01、R-02、R-04、R-05、R-06、P0-15、P0-16、P1-09、P1-11</t>
+          <t>等 P0-11</t>
         </is>
       </c>
       <c r="D59" s="11" t="n"/>
@@ -2242,20 +2251,20 @@
       <c r="H59" s="11" t="n"/>
       <c r="I59" s="12" t="n"/>
     </row>
-    <row r="60" ht="18" customHeight="1">
+    <row r="60" ht="46" customHeight="1">
       <c r="A60" s="13" t="inlineStr">
         <is>
-          <t>P0-14</t>
+          <t>R-13</t>
         </is>
       </c>
       <c r="B60" s="6" t="inlineStr">
         <is>
-          <t>韌體簽章、Secure Boot 與 Flash 加密</t>
+          <t>CP1 內測就緒檢查（10/30）</t>
         </is>
       </c>
       <c r="C60" s="6" t="inlineStr">
         <is>
-          <t>等 P0-13、R-01</t>
+          <t>等 P0-02、P0-03、P0-04、P0-05、P0-06、P0-07、P0-08、P0-09、P0-10、P0-11、P0-12、P0-13、P1-01、P1-02、P2-09、R-01、R-02、R-04、R-05、R-06、P0-15、P0-16、P1-09、P1-11</t>
         </is>
       </c>
       <c r="D60" s="11" t="n"/>
@@ -2268,17 +2277,17 @@
     <row r="61" ht="18" customHeight="1">
       <c r="A61" s="13" t="inlineStr">
         <is>
-          <t>P1-06</t>
+          <t>P0-14</t>
         </is>
       </c>
       <c r="B61" s="6" t="inlineStr">
         <is>
-          <t>處理 GPL-3.0 依賴（arduino-audio-tools）</t>
+          <t>韌體簽章、Secure Boot 與 Flash 加密</t>
         </is>
       </c>
       <c r="C61" s="6" t="inlineStr">
         <is>
-          <t>等 Q3</t>
+          <t>等 P0-13、R-01</t>
         </is>
       </c>
       <c r="D61" s="11" t="n"/>
@@ -2291,12 +2300,12 @@
     <row r="62" ht="18" customHeight="1">
       <c r="A62" s="13" t="inlineStr">
         <is>
-          <t>P1-07</t>
+          <t>P1-06</t>
         </is>
       </c>
       <c r="B62" s="6" t="inlineStr">
         <is>
-          <t>LGPL 合規與第三方授權聲明</t>
+          <t>處理 GPL-3.0 依賴（arduino-audio-tools）</t>
         </is>
       </c>
       <c r="C62" s="6" t="inlineStr">
@@ -2314,17 +2323,17 @@
     <row r="63" ht="18" customHeight="1">
       <c r="A63" s="13" t="inlineStr">
         <is>
-          <t>P1-08</t>
+          <t>P1-07</t>
         </is>
       </c>
       <c r="B63" s="6" t="inlineStr">
         <is>
-          <t>硬件認證</t>
+          <t>LGPL 合規與第三方授權聲明</t>
         </is>
       </c>
       <c r="C63" s="6" t="inlineStr">
         <is>
-          <t>等 R-01、R-05</t>
+          <t>等 Q3</t>
         </is>
       </c>
       <c r="D63" s="11" t="n"/>
@@ -2337,17 +2346,17 @@
     <row r="64" ht="18" customHeight="1">
       <c r="A64" s="13" t="inlineStr">
         <is>
-          <t>R-07</t>
+          <t>P1-08</t>
         </is>
       </c>
       <c r="B64" s="6" t="inlineStr">
         <is>
-          <t>20 個家庭封閉內測</t>
+          <t>硬件認證</t>
         </is>
       </c>
       <c r="C64" s="6" t="inlineStr">
         <is>
-          <t>等 R-13</t>
+          <t>等 R-01、R-05</t>
         </is>
       </c>
       <c r="D64" s="11" t="n"/>
@@ -2360,17 +2369,17 @@
     <row r="65" ht="18" customHeight="1">
       <c r="A65" s="13" t="inlineStr">
         <is>
-          <t>R-08</t>
+          <t>R-07</t>
         </is>
       </c>
       <c r="B65" s="6" t="inlineStr">
         <is>
-          <t>第 8 週關卡決策</t>
+          <t>20 個家庭封閉內測</t>
         </is>
       </c>
       <c r="C65" s="6" t="inlineStr">
         <is>
-          <t>等 R-07、P2-09、P1-08</t>
+          <t>等 R-13</t>
         </is>
       </c>
       <c r="D65" s="11" t="n"/>
@@ -2383,17 +2392,17 @@
     <row r="66" ht="18" customHeight="1">
       <c r="A66" s="13" t="inlineStr">
         <is>
-          <t>R-14</t>
+          <t>R-08</t>
         </is>
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
-          <t>離線兒歌與故事</t>
+          <t>第 8 週關卡決策</t>
         </is>
       </c>
       <c r="C66" s="6" t="inlineStr">
         <is>
-          <t>等 R-01</t>
+          <t>等 R-07、P2-09、P1-08</t>
         </is>
       </c>
       <c r="D66" s="11" t="n"/>
@@ -2406,17 +2415,17 @@
     <row r="67" ht="18" customHeight="1">
       <c r="A67" s="13" t="inlineStr">
         <is>
-          <t>P2-05</t>
+          <t>R-14</t>
         </is>
       </c>
       <c r="B67" s="6" t="inlineStr">
         <is>
-          <t>拒絕未知設備並限制用量</t>
+          <t>離線兒歌與故事</t>
         </is>
       </c>
       <c r="C67" s="6" t="inlineStr">
         <is>
-          <t>等 P0-08</t>
+          <t>等 R-01</t>
         </is>
       </c>
       <c r="D67" s="11" t="n"/>
@@ -2429,17 +2438,17 @@
     <row r="68" ht="18" customHeight="1">
       <c r="A68" s="13" t="inlineStr">
         <is>
-          <t>R-09</t>
+          <t>P2-05</t>
         </is>
       </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t>量產外殼（真空複模）</t>
+          <t>拒絕未知設備並限制用量</t>
         </is>
       </c>
       <c r="C68" s="6" t="inlineStr">
         <is>
-          <t>等 R-08、R-05</t>
+          <t>等 P0-08</t>
         </is>
       </c>
       <c r="D68" s="11" t="n"/>
@@ -2452,17 +2461,17 @@
     <row r="69" ht="18" customHeight="1">
       <c r="A69" s="13" t="inlineStr">
         <is>
-          <t>R-10</t>
+          <t>R-09</t>
         </is>
       </c>
       <c r="B69" s="6" t="inlineStr">
         <is>
-          <t>出廠流程</t>
+          <t>量產外殼（真空複模）</t>
         </is>
       </c>
       <c r="C69" s="6" t="inlineStr">
         <is>
-          <t>等 P0-06、P0-14、R-01</t>
+          <t>等 R-08、R-05</t>
         </is>
       </c>
       <c r="D69" s="11" t="n"/>
@@ -2475,17 +2484,17 @@
     <row r="70" ht="18" customHeight="1">
       <c r="A70" s="13" t="inlineStr">
         <is>
-          <t>R-15</t>
+          <t>R-10</t>
         </is>
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>農曆新年前交付（生產 1/15、送達 1/29）</t>
+          <t>出廠流程</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr">
         <is>
-          <t>等 R-09、R-10</t>
+          <t>等 P0-06、P0-14、R-01</t>
         </is>
       </c>
       <c r="D70" s="11" t="n"/>
@@ -2495,50 +2504,50 @@
       <c r="H70" s="11" t="n"/>
       <c r="I70" s="12" t="n"/>
     </row>
-    <row r="72">
-      <c r="A72" s="10" t="inlineStr">
+    <row r="71" ht="18" customHeight="1">
+      <c r="A71" s="13" t="inlineStr">
+        <is>
+          <t>R-15</t>
+        </is>
+      </c>
+      <c r="B71" s="6" t="inlineStr">
+        <is>
+          <t>農曆新年前交付（生產 1/15、送達 1/29）</t>
+        </is>
+      </c>
+      <c r="C71" s="6" t="inlineStr">
+        <is>
+          <t>等 R-09、R-10</t>
+        </is>
+      </c>
+      <c r="D71" s="11" t="n"/>
+      <c r="E71" s="11" t="n"/>
+      <c r="F71" s="11" t="n"/>
+      <c r="G71" s="11" t="n"/>
+      <c r="H71" s="11" t="n"/>
+      <c r="I71" s="12" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="10" t="inlineStr">
         <is>
           <t>❓ 待確認問題</t>
         </is>
       </c>
     </row>
-    <row r="73">
-      <c r="A73" s="4" t="inlineStr">
+    <row r="74">
+      <c r="A74" s="4" t="inlineStr">
         <is>
           <t>編號</t>
         </is>
       </c>
-      <c r="B73" s="4" t="inlineStr">
+      <c r="B74" s="4" t="inlineStr">
         <is>
           <t>問題</t>
         </is>
       </c>
-      <c r="C73" s="4" t="inlineStr">
+      <c r="C74" s="4" t="inlineStr">
         <is>
           <t>影響的任務 / 為什麼重要</t>
-        </is>
-      </c>
-      <c r="D73" s="11" t="n"/>
-      <c r="E73" s="11" t="n"/>
-      <c r="F73" s="11" t="n"/>
-      <c r="G73" s="11" t="n"/>
-      <c r="H73" s="11" t="n"/>
-      <c r="I73" s="12" t="n"/>
-    </row>
-    <row r="74" ht="18" customHeight="1">
-      <c r="A74" s="13" t="inlineStr">
-        <is>
-          <t>Q3</t>
-        </is>
-      </c>
-      <c r="B74" s="6" t="inlineStr">
-        <is>
-          <t>韌體打算閉源商業銷售嗎？</t>
-        </is>
-      </c>
-      <c r="C74" s="6" t="inlineStr">
-        <is>
-          <t>P1-06, P1-07：決定 GPL／LGPL 依賴要開源還是替換。</t>
         </is>
       </c>
       <c r="D74" s="11" t="n"/>
@@ -2548,52 +2557,76 @@
       <c r="H74" s="11" t="n"/>
       <c r="I74" s="12" t="n"/>
     </row>
-    <row r="76">
-      <c r="A76" s="10" t="inlineStr">
+    <row r="75" ht="18" customHeight="1">
+      <c r="A75" s="13" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="B75" s="6" t="inlineStr">
+        <is>
+          <t>韌體打算閉源商業銷售嗎？</t>
+        </is>
+      </c>
+      <c r="C75" s="6" t="inlineStr">
+        <is>
+          <t>P1-06, P1-07：決定 GPL／LGPL 依賴要開源還是替換。</t>
+        </is>
+      </c>
+      <c r="D75" s="11" t="n"/>
+      <c r="E75" s="11" t="n"/>
+      <c r="F75" s="11" t="n"/>
+      <c r="G75" s="11" t="n"/>
+      <c r="H75" s="11" t="n"/>
+      <c r="I75" s="12" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="10" t="inlineStr">
         <is>
           <t>說明</t>
         </is>
       </c>
     </row>
-    <row r="77" ht="32" customHeight="1">
-      <c r="A77" s="14" t="inlineStr">
+    <row r="78" ht="32" customHeight="1">
+      <c r="A78" s="14" t="inlineStr">
         <is>
           <t>・狀態：未開始 → 進行中 → 已完成。只有測試真的跑過而且通過才算已完成；阻塞要在備註寫原因；不再需要的任務標不適用，不要刪。</t>
-        </is>
-      </c>
-    </row>
-    <row r="78" ht="18" customHeight="1">
-      <c r="A78" s="14" t="inlineStr">
-        <is>
-          <t>・測試結果：未測試 / 通過 / 失敗 / 部分通過。測試證據寫跑了什麼、看到什麼，完整歷史在「更新記錄」。</t>
         </is>
       </c>
     </row>
     <row r="79" ht="18" customHeight="1">
       <c r="A79" s="14" t="inlineStr">
         <is>
-          <t>・「接下來」按階段排序，同一階段內再按優先級；依賴還沒滿足的任務不會出現在「接下來」。</t>
+          <t>・測試結果：未測試 / 通過 / 失敗 / 部分通過。測試證據寫跑了什麼、看到什麼，完整歷史在「更新記錄」。</t>
         </is>
       </c>
     </row>
     <row r="80" ht="18" customHeight="1">
       <c r="A80" s="14" t="inlineStr">
         <is>
+          <t>・「接下來」按階段排序，同一階段內再按優先級；依賴還沒滿足的任務不會出現在「接下來」。</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="18" customHeight="1">
+      <c r="A81" s="14" t="inlineStr">
+        <is>
           <t>・可以手動改：「任務清單」的狀態、測試結果、測試證據、Commit、備註，以及「待確認問題」的回答。其餘欄位和本頁由腳本維護。</t>
         </is>
       </c>
     </row>
-    <row r="81" ht="32" customHeight="1">
-      <c r="A81" s="14" t="inlineStr">
+    <row r="82" ht="32" customHeight="1">
+      <c r="A82" s="14" t="inlineStr">
         <is>
           <t>・建議用法：在 Claude Code 對 Claude 說「P0-02 做完了」或輸入 /prod-readiness。Claude 會先跑測試再更新，並寫進「更新記錄」。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="62">
+  <mergeCells count="63">
     <mergeCell ref="E21:I21"/>
     <mergeCell ref="C61:I61"/>
+    <mergeCell ref="E43:I43"/>
     <mergeCell ref="C52:I52"/>
     <mergeCell ref="C70:I70"/>
     <mergeCell ref="E24:I24"/>
@@ -2603,7 +2636,6 @@
     <mergeCell ref="A3:I3"/>
     <mergeCell ref="E23:I23"/>
     <mergeCell ref="E39:I39"/>
-    <mergeCell ref="A50:I50"/>
     <mergeCell ref="C67:I67"/>
     <mergeCell ref="E48:I48"/>
     <mergeCell ref="C57:I57"/>
@@ -2615,26 +2647,21 @@
     <mergeCell ref="E20:I20"/>
     <mergeCell ref="E38:I38"/>
     <mergeCell ref="C69:I69"/>
-    <mergeCell ref="A76:I76"/>
     <mergeCell ref="E28:I28"/>
     <mergeCell ref="C62:I62"/>
     <mergeCell ref="C68:I68"/>
     <mergeCell ref="E31:I31"/>
     <mergeCell ref="E40:I40"/>
     <mergeCell ref="C58:I58"/>
-    <mergeCell ref="A72:I72"/>
     <mergeCell ref="E30:I30"/>
     <mergeCell ref="A81:I81"/>
     <mergeCell ref="E34:I34"/>
     <mergeCell ref="A19:I19"/>
     <mergeCell ref="C74:I74"/>
     <mergeCell ref="C64:I64"/>
-    <mergeCell ref="C51:I51"/>
     <mergeCell ref="E46:I46"/>
-    <mergeCell ref="C73:I73"/>
-    <mergeCell ref="A44:I44"/>
+    <mergeCell ref="E49:I49"/>
     <mergeCell ref="E27:I27"/>
-    <mergeCell ref="E45:I45"/>
     <mergeCell ref="C54:I54"/>
     <mergeCell ref="A77:I77"/>
     <mergeCell ref="E36:I36"/>
@@ -2642,18 +2669,24 @@
     <mergeCell ref="C65:I65"/>
     <mergeCell ref="E26:I26"/>
     <mergeCell ref="C55:I55"/>
+    <mergeCell ref="A82:I82"/>
+    <mergeCell ref="C75:I75"/>
+    <mergeCell ref="A73:I73"/>
+    <mergeCell ref="A51:I51"/>
     <mergeCell ref="C56:I56"/>
     <mergeCell ref="E32:I32"/>
     <mergeCell ref="E25:I25"/>
     <mergeCell ref="C59:I59"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="E41:I41"/>
+    <mergeCell ref="A45:I45"/>
     <mergeCell ref="A79:I79"/>
     <mergeCell ref="E37:I37"/>
     <mergeCell ref="C60:I60"/>
     <mergeCell ref="E22:I22"/>
     <mergeCell ref="E47:I47"/>
     <mergeCell ref="A78:I78"/>
+    <mergeCell ref="C71:I71"/>
   </mergeCells>
   <conditionalFormatting sqref="I6:I10">
     <cfRule type="dataBar" priority="1">
@@ -6717,7 +6750,7 @@
         </is>
       </c>
     </row>
-    <row r="57" ht="102" customHeight="1">
+    <row r="57" ht="186" customHeight="1">
       <c r="A57" s="13" t="inlineStr">
         <is>
           <t>P2-11</t>
@@ -6745,12 +6778,12 @@
       </c>
       <c r="F57" s="13" t="inlineStr">
         <is>
-          <t>未開始</t>
+          <t>進行中</t>
         </is>
       </c>
       <c r="G57" s="13" t="inlineStr">
         <is>
-          <t>未測試</t>
+          <t>部分通過</t>
         </is>
       </c>
       <c r="I57" s="6" t="inlineStr">
@@ -6765,18 +6798,29 @@
       </c>
       <c r="K57" s="6" t="inlineStr">
         <is>
-          <t>C3 env 不再因 async_tcp 觸發看門狗：關閉 AsyncTCP 的 WDT 訂閱（-D CONFIG_ASYNC_TCP_USE_WDT=0）或讓解碼 task 定期讓出 CPU；播放與 SoftAP 配網都仍正常</t>
+          <t>排程器暫停期間不可呼叫會阻塞的寫入：只在環形緩衝區放得下最大解碼封包（120ms）時才做 CPU 抽樣；AsyncTCP 看門狗保持開啟以便抓到同類問題</t>
         </is>
       </c>
       <c r="L57" s="6" t="inlineStr">
         <is>
-          <t>① Spotpear 開發板連續開機 30 次並播完開場白、再進行 20 輪對話，串口 0 次 task_wdt ② SoftAP 配網頁面仍能打開並保存 WiFi</t>
+          <t>① Spotpear 開發板連續開機 30 次並播完開場白，串口 0 次 task_wdt / panic ② 20 輪實際對話，串口 0 次 task_wdt</t>
         </is>
       </c>
       <c r="M57" s="13" t="n"/>
+      <c r="N57" s="6" t="inlineStr">
+        <is>
+          <t>① 1.3.4 localall 連續重啟 30 次：開場白 30/30、task_wdt 0、panic 0（修正前 19 次 4 次）；CPU 抽樣仍每輪 2–7 次，解碼約 8.6–9.3ms/封包。排除過程：關 AsyncTCP WDT 只把重啟變成卡住（30 次 3 次靜默&gt;17s）；Serial.setTxTimeoutMs(0) 仍 30 次 2 次 → 均撤回。② 20 輪對話待用戶</t>
+        </is>
+      </c>
+      <c r="O57" s="13" t="inlineStr">
+        <is>
+          <t>8e8b449</t>
+        </is>
+      </c>
       <c r="P57" s="6" t="inlineStr">
         <is>
-          <t>[2026-10-08] 新增</t>
+          <t>[2026-10-08] 新增
+[2026-10-08] 2026-10-08 查明真正原因：不是 async_tcp 被搶 CPU。decodeTask 每輪在 vTaskSuspendAll() 下解碼一個封包量 CPU，解碼寫入已滿的播放環形緩衝區時 writeArray() 等空位，但排程器已停、揚聲器 task 無法消耗 → 卡死，看門狗報 async_tcp（唯一訂閱者）未回報。原驗收（關 AsyncTCP WDT / SoftAP 測試）按錯誤猜測寫，已改；關 WDT 只會把重啟變成永久卡住</t>
         </is>
       </c>
     </row>
@@ -7244,7 +7288,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I122"/>
+  <dimension ref="A1:I125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -11547,8 +11591,117 @@
         </is>
       </c>
     </row>
+    <row r="123" ht="32" customHeight="1">
+      <c r="A123" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-08 09:47</t>
+        </is>
+      </c>
+      <c r="B123" s="13" t="inlineStr">
+        <is>
+          <t>P2-11</t>
+        </is>
+      </c>
+      <c r="C123" s="6" t="inlineStr">
+        <is>
+          <t>C3 播放時 async_tcp 觸發任務看門狗重啟</t>
+        </is>
+      </c>
+      <c r="D123" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E123" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F123" s="13" t="n"/>
+      <c r="G123" s="6" t="n"/>
+      <c r="H123" s="13" t="n"/>
+      <c r="I123" s="6" t="n"/>
+    </row>
+    <row r="124" ht="158" customHeight="1">
+      <c r="A124" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-08 10:42</t>
+        </is>
+      </c>
+      <c r="B124" s="13" t="inlineStr">
+        <is>
+          <t>P2-11</t>
+        </is>
+      </c>
+      <c r="C124" s="6" t="inlineStr">
+        <is>
+          <t>C3 播放時 async_tcp 觸發任務看門狗重啟</t>
+        </is>
+      </c>
+      <c r="D124" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="E124" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F124" s="13" t="n"/>
+      <c r="G124" s="6" t="n"/>
+      <c r="H124" s="13" t="n"/>
+      <c r="I124" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-08 查明真正原因：不是 async_tcp 被搶 CPU。decodeTask 每輪在 vTaskSuspendAll() 下解碼一個封包量 CPU，解碼寫入已滿的播放環形緩衝區時 writeArray() 等空位，但排程器已停、揚聲器 task 無法消耗 → 卡死，看門狗報 async_tcp（唯一訂閱者）未回報。原驗收（關 AsyncTCP WDT / SoftAP 測試）按錯誤猜測寫，已改；關 WDT 只會把重啟變成永久卡住；修改了驗收標準、測試方法</t>
+        </is>
+      </c>
+    </row>
+    <row r="125" ht="88" customHeight="1">
+      <c r="A125" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-08 10:42</t>
+        </is>
+      </c>
+      <c r="B125" s="13" t="inlineStr">
+        <is>
+          <t>P2-11</t>
+        </is>
+      </c>
+      <c r="C125" s="6" t="inlineStr">
+        <is>
+          <t>C3 播放時 async_tcp 觸發任務看門狗重啟</t>
+        </is>
+      </c>
+      <c r="D125" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="E125" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F125" s="13" t="inlineStr">
+        <is>
+          <t>部分通過</t>
+        </is>
+      </c>
+      <c r="G125" s="6" t="inlineStr">
+        <is>
+          <t>① 1.3.4 localall 連續重啟 30 次：開場白 30/30、task_wdt 0、panic 0（修正前 19 次 4 次）；CPU 抽樣仍每輪 2–7 次，解碼約 8.6–9.3ms/封包。排除過程：關 AsyncTCP WDT 只把重啟變成卡住（30 次 3 次靜默&gt;17s）；Serial.setTxTimeoutMs(0) 仍 30 次 2 次 → 均撤回。② 20 輪對話待用戶</t>
+        </is>
+      </c>
+      <c r="H125" s="13" t="inlineStr">
+        <is>
+          <t>8e8b449</t>
+        </is>
+      </c>
+      <c r="I125" s="6" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I122"/>
+  <autoFilter ref="A1:I125"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record P2-11 done: 30 boots and 20 conversation turns without a reset.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/production-readiness.xlsx
+++ b/docs/production-readiness.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'任務清單'!$A$1:$P$57</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'待確認問題'!$A$1:$G$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$125</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$126</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -665,14 +665,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>最後更新：2026-10-08 10:42　·　本頁由 tracker.py 自動生成，請勿手動編輯</t>
+          <t>最後更新：2026-10-08 10:51　·　本頁由 tracker.py 自動生成，請勿手動編輯</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>總進度：3/55 已完成（5%）　·　目前階段：1 止血定案（10/5–10/16）</t>
+          <t>總進度：4/55 已完成（7%）　·　目前階段：1 止血定案（10/5–10/16）</t>
         </is>
       </c>
     </row>
@@ -824,11 +824,11 @@
       </c>
       <c r="E8" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A8,'任務清單'!$F:$F,E$5)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F8" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A8,'任務清單'!$F:$F,F$5)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G8" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A8,'任務清單'!$F:$F,G$5)</f>
@@ -840,7 +840,7 @@
       </c>
       <c r="I8" s="8">
         <f>IFERROR(F8/(C8-H8),0)</f>
-        <v>0.18181818181818182</v>
+        <v>0.2727272727272727</v>
       </c>
     </row>
     <row r="9" ht="18" customHeight="1">
@@ -900,11 +900,11 @@
       </c>
       <c r="E10" s="5">
         <f>SUM(E6:E9)</f>
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F10" s="5">
         <f>SUM(F6:F9)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G10" s="5">
         <f>SUM(G6:G9)</f>
@@ -916,7 +916,7 @@
       </c>
       <c r="I10" s="9">
         <f>IFERROR(F10/(C10-H10),0)</f>
-        <v>0.05454545454545454</v>
+        <v>0.07272727272727272</v>
       </c>
     </row>
     <row r="12">
@@ -1027,11 +1027,11 @@
       </c>
       <c r="E14" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A14,'任務清單'!$F:$F,E$12)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F14" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A14,'任務清單'!$F:$F,F$12)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G14" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A14,'任務清單'!$F:$F,G$12)</f>
@@ -1043,7 +1043,7 @@
       </c>
       <c r="I14" s="8">
         <f>IFERROR(F14/(C14-H14),0)</f>
-        <v>0.0</v>
+        <v>0.07142857142857142</v>
       </c>
     </row>
     <row r="15" ht="32" customHeight="1">
@@ -1143,11 +1143,11 @@
       </c>
       <c r="E17" s="5">
         <f>SUM(E13:E16)</f>
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F17" s="5">
         <f>SUM(F13:F16)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G17" s="5">
         <f>SUM(G13:G16)</f>
@@ -1159,7 +1159,7 @@
       </c>
       <c r="I17" s="9">
         <f>IFERROR(F17/(C17-H17),0)</f>
-        <v>0.05454545454545454</v>
+        <v>0.07272727272727272</v>
       </c>
     </row>
     <row r="19">
@@ -1711,15 +1711,15 @@
       <c r="H36" s="11" t="n"/>
       <c r="I36" s="12" t="n"/>
     </row>
-    <row r="37" ht="144" customHeight="1">
+    <row r="37" ht="60" customHeight="1">
       <c r="A37" s="13" t="inlineStr">
         <is>
-          <t>P2-11</t>
+          <t>P1-01</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>C3 播放時 async_tcp 觸發任務看門狗重啟</t>
+          <t>加入內容審核層（輸入與輸出）</t>
         </is>
       </c>
       <c r="C37" s="13" t="inlineStr">
@@ -1729,13 +1729,12 @@
       </c>
       <c r="D37" s="13" t="inlineStr">
         <is>
-          <t>進行中</t>
+          <t>未開始</t>
         </is>
       </c>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>上次測試：部分通過 — ① 1.3.4 localall 連續重啟 30 次：開場白 30/30、task_wdt 0、panic 0（修正前 19 次 4 次）；CPU 抽樣仍每輪 2–7 次，解碼約 8.6–9.3ms/封包。排除過程：關 AsyncTCP WDT 只把重啟變成卡住（30 次 3 次靜默&gt;17s）；Serial.setTxTimeoutMs(0) 仍 30 次 2 次 → 均撤回。② 20 輪對話待用戶
-排程器暫停期間不可呼叫會阻塞的寫入：只在環形緩衝區放得下最大解碼封包（120ms）時才做 CPU 抽樣；AsyncTCP 看門狗保持開啟以便抓到同類問題</t>
+          <t>STT 文字與 LLM 輸出都經審核，尺度按 3–6 歲；命中時換成安全回覆並記錄事件，事件只記類別、時間、角色，不記原文（管理員不能看兒童內容，見 Q7）；首字延遲增加 ≤150ms。</t>
         </is>
       </c>
       <c r="F37" s="11" t="n"/>
@@ -1743,15 +1742,15 @@
       <c r="H37" s="11" t="n"/>
       <c r="I37" s="12" t="n"/>
     </row>
-    <row r="38" ht="60" customHeight="1">
+    <row r="38" ht="32" customHeight="1">
       <c r="A38" s="13" t="inlineStr">
         <is>
-          <t>P1-01</t>
+          <t>P1-02</t>
         </is>
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>加入內容審核層（輸入與輸出）</t>
+          <t>日誌移除兒童個人資料</t>
         </is>
       </c>
       <c r="C38" s="13" t="inlineStr">
@@ -1766,7 +1765,7 @@
       </c>
       <c r="E38" s="6" t="inlineStr">
         <is>
-          <t>STT 文字與 LLM 輸出都經審核，尺度按 3–6 歲；命中時換成安全回覆並記錄事件，事件只記類別、時間、角色，不記原文（管理員不能看兒童內容，見 Q7）；首字延遲增加 ≤150ms。</t>
+          <t>生產日誌只記 ID、長度、類別，不記內容；內容只在 DEBUG 等級輸出，生產不開 DEBUG。</t>
         </is>
       </c>
       <c r="F38" s="11" t="n"/>
@@ -1774,15 +1773,15 @@
       <c r="H38" s="11" t="n"/>
       <c r="I38" s="12" t="n"/>
     </row>
-    <row r="39" ht="32" customHeight="1">
+    <row r="39" ht="46" customHeight="1">
       <c r="A39" s="13" t="inlineStr">
         <is>
-          <t>P1-02</t>
+          <t>P1-09</t>
         </is>
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>日誌移除兒童個人資料</t>
+          <t>家長鎖：孩子模式進設定要輸入 PIN</t>
         </is>
       </c>
       <c r="C39" s="13" t="inlineStr">
@@ -1797,7 +1796,7 @@
       </c>
       <c r="E39" s="6" t="inlineStr">
         <is>
-          <t>生產日誌只記 ID、長度、類別，不記內容；內容只在 DEBUG 等級輸出，生產不開 DEBUG。</t>
+          <t>從孩子模式進入設定、家長控制、記憶、設備頁面前，都要先輸入家長 PIN（第一次使用時設定）；連錯 5 次鎖定 5 分鐘；忘記 PIN 可用帳號密碼重設。</t>
         </is>
       </c>
       <c r="F39" s="11" t="n"/>
@@ -1808,12 +1807,12 @@
     <row r="40" ht="46" customHeight="1">
       <c r="A40" s="13" t="inlineStr">
         <is>
-          <t>P1-09</t>
+          <t>P1-11</t>
         </is>
       </c>
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>家長鎖：孩子模式進設定要輸入 PIN</t>
+          <t>伺服器與資料庫直接存取的管控</t>
         </is>
       </c>
       <c r="C40" s="13" t="inlineStr">
@@ -1828,7 +1827,7 @@
       </c>
       <c r="E40" s="6" t="inlineStr">
         <is>
-          <t>從孩子模式進入設定、家長控制、記憶、設備頁面前，都要先輸入家長 PIN（第一次使用時設定）；連錯 5 次鎖定 5 分鐘；忘記 PIN 可用帳號密碼重設。</t>
+          <t>列出誰有 SSH 與資料庫直連權限（越少越好）；service_role key 只存在伺服器的 env；私隱政策寫明這類存取的範圍；每次直接查看生產資料都留記錄。</t>
         </is>
       </c>
       <c r="F40" s="11" t="n"/>
@@ -1839,12 +1838,12 @@
     <row r="41" ht="46" customHeight="1">
       <c r="A41" s="13" t="inlineStr">
         <is>
-          <t>P1-11</t>
+          <t>P2-02</t>
         </is>
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>伺服器與資料庫直接存取的管控</t>
+          <t>CI 跑測試與靜態檢查</t>
         </is>
       </c>
       <c r="C41" s="13" t="inlineStr">
@@ -1859,7 +1858,7 @@
       </c>
       <c r="E41" s="6" t="inlineStr">
         <is>
-          <t>列出誰有 SSH 與資料庫直連權限（越少越好）；service_role key 只存在伺服器的 env；私隱政策寫明這類存取的範圍；每次直接查看生產資料都留記錄。</t>
+          <t>推送與 PR 時跑 pytest、ruff、pyright、next lint、tsc --noEmit、pio run；任何一項失敗就不發佈 image。</t>
         </is>
       </c>
       <c r="F41" s="11" t="n"/>
@@ -1867,15 +1866,15 @@
       <c r="H41" s="11" t="n"/>
       <c r="I41" s="12" t="n"/>
     </row>
-    <row r="42" ht="46" customHeight="1">
+    <row r="42" ht="32" customHeight="1">
       <c r="A42" s="13" t="inlineStr">
         <is>
-          <t>P2-02</t>
+          <t>P2-04</t>
         </is>
       </c>
       <c r="B42" s="6" t="inlineStr">
         <is>
-          <t>CI 跑測試與靜態檢查</t>
+          <t>容器改用非 root 用戶</t>
         </is>
       </c>
       <c r="C42" s="13" t="inlineStr">
@@ -1890,7 +1889,7 @@
       </c>
       <c r="E42" s="6" t="inlineStr">
         <is>
-          <t>推送與 PR 時跑 pytest、ruff、pyright、next lint、tsc --noEmit、pio run；任何一項失敗就不發佈 image。</t>
+          <t>兩個 Dockerfile 都設定非 root 的 USER。</t>
         </is>
       </c>
       <c r="F42" s="11" t="n"/>
@@ -1898,68 +1897,68 @@
       <c r="H42" s="11" t="n"/>
       <c r="I42" s="12" t="n"/>
     </row>
-    <row r="43" ht="32" customHeight="1">
-      <c r="A43" s="13" t="inlineStr">
-        <is>
-          <t>P2-04</t>
-        </is>
-      </c>
-      <c r="B43" s="6" t="inlineStr">
-        <is>
-          <t>容器改用非 root 用戶</t>
-        </is>
-      </c>
-      <c r="C43" s="13" t="inlineStr">
-        <is>
-          <t>2 內測準備</t>
-        </is>
-      </c>
-      <c r="D43" s="13" t="inlineStr">
-        <is>
-          <t>未開始</t>
-        </is>
-      </c>
-      <c r="E43" s="6" t="inlineStr">
-        <is>
-          <t>兩個 Dockerfile 都設定非 root 的 USER。</t>
-        </is>
-      </c>
-      <c r="F43" s="11" t="n"/>
-      <c r="G43" s="11" t="n"/>
-      <c r="H43" s="11" t="n"/>
-      <c r="I43" s="12" t="n"/>
+    <row r="44">
+      <c r="A44" s="10" t="inlineStr">
+        <is>
+          <t>✅ 最近完成與測試效果</t>
+        </is>
+      </c>
     </row>
     <row r="45">
-      <c r="A45" s="10" t="inlineStr">
-        <is>
-          <t>✅ 最近完成與測試效果</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="4" t="inlineStr">
+      <c r="A45" s="4" t="inlineStr">
         <is>
           <t>編號</t>
         </is>
       </c>
-      <c r="B46" s="4" t="inlineStr">
+      <c r="B45" s="4" t="inlineStr">
         <is>
           <t>任務</t>
         </is>
       </c>
-      <c r="C46" s="4" t="inlineStr">
+      <c r="C45" s="4" t="inlineStr">
         <is>
           <t>測試結果</t>
         </is>
       </c>
-      <c r="D46" s="4" t="inlineStr">
+      <c r="D45" s="4" t="inlineStr">
         <is>
           <t>完成日期</t>
         </is>
       </c>
-      <c r="E46" s="4" t="inlineStr">
+      <c r="E45" s="4" t="inlineStr">
         <is>
           <t>測試證據</t>
+        </is>
+      </c>
+      <c r="F45" s="11" t="n"/>
+      <c r="G45" s="11" t="n"/>
+      <c r="H45" s="11" t="n"/>
+      <c r="I45" s="12" t="n"/>
+    </row>
+    <row r="46" ht="88" customHeight="1">
+      <c r="A46" s="13" t="inlineStr">
+        <is>
+          <t>P2-11</t>
+        </is>
+      </c>
+      <c r="B46" s="6" t="inlineStr">
+        <is>
+          <t>C3 播放時 async_tcp 觸發任務看門狗重啟</t>
+        </is>
+      </c>
+      <c r="C46" s="13" t="inlineStr">
+        <is>
+          <t>通過</t>
+        </is>
+      </c>
+      <c r="D46" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="E46" s="6" t="inlineStr">
+        <is>
+          <t>① 1.3.4 連續重啟 30 次：開場白 30/30、task_wdt 0、panic 0（修正前 19 次 4 次）② 用戶實際對話 20 輪（10:44–10:50）：20 輪都有回應，3 次未完成皆為用戶插話打斷且隨即恢復，短按合併為單輪；task_wdt 0、panic 0；CPU 抽樣照常（每輪 9–13 個）</t>
         </is>
       </c>
       <c r="F46" s="11" t="n"/>
@@ -2626,7 +2625,6 @@
   <mergeCells count="63">
     <mergeCell ref="E21:I21"/>
     <mergeCell ref="C61:I61"/>
-    <mergeCell ref="E43:I43"/>
     <mergeCell ref="C52:I52"/>
     <mergeCell ref="C70:I70"/>
     <mergeCell ref="E24:I24"/>
@@ -2660,8 +2658,10 @@
     <mergeCell ref="C74:I74"/>
     <mergeCell ref="C64:I64"/>
     <mergeCell ref="E46:I46"/>
+    <mergeCell ref="A44:I44"/>
     <mergeCell ref="E49:I49"/>
     <mergeCell ref="E27:I27"/>
+    <mergeCell ref="E45:I45"/>
     <mergeCell ref="C54:I54"/>
     <mergeCell ref="A77:I77"/>
     <mergeCell ref="E36:I36"/>
@@ -2679,7 +2679,6 @@
     <mergeCell ref="C59:I59"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="E41:I41"/>
-    <mergeCell ref="A45:I45"/>
     <mergeCell ref="A79:I79"/>
     <mergeCell ref="E37:I37"/>
     <mergeCell ref="C60:I60"/>
@@ -6778,12 +6777,17 @@
       </c>
       <c r="F57" s="13" t="inlineStr">
         <is>
-          <t>進行中</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="G57" s="13" t="inlineStr">
         <is>
-          <t>部分通過</t>
+          <t>通過</t>
+        </is>
+      </c>
+      <c r="H57" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="I57" s="6" t="inlineStr">
@@ -6809,7 +6813,7 @@
       <c r="M57" s="13" t="n"/>
       <c r="N57" s="6" t="inlineStr">
         <is>
-          <t>① 1.3.4 localall 連續重啟 30 次：開場白 30/30、task_wdt 0、panic 0（修正前 19 次 4 次）；CPU 抽樣仍每輪 2–7 次，解碼約 8.6–9.3ms/封包。排除過程：關 AsyncTCP WDT 只把重啟變成卡住（30 次 3 次靜默&gt;17s）；Serial.setTxTimeoutMs(0) 仍 30 次 2 次 → 均撤回。② 20 輪對話待用戶</t>
+          <t>① 1.3.4 連續重啟 30 次：開場白 30/30、task_wdt 0、panic 0（修正前 19 次 4 次）② 用戶實際對話 20 輪（10:44–10:50）：20 輪都有回應，3 次未完成皆為用戶插話打斷且隨即恢復，短按合併為單輪；task_wdt 0、panic 0；CPU 抽樣照常（每輪 9–13 個）</t>
         </is>
       </c>
       <c r="O57" s="13" t="inlineStr">
@@ -7288,7 +7292,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I125"/>
+  <dimension ref="A1:I126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -11700,8 +11704,51 @@
       </c>
       <c r="I125" s="6" t="n"/>
     </row>
+    <row r="126" ht="74" customHeight="1">
+      <c r="A126" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-08 10:51</t>
+        </is>
+      </c>
+      <c r="B126" s="13" t="inlineStr">
+        <is>
+          <t>P2-11</t>
+        </is>
+      </c>
+      <c r="C126" s="6" t="inlineStr">
+        <is>
+          <t>C3 播放時 async_tcp 觸發任務看門狗重啟</t>
+        </is>
+      </c>
+      <c r="D126" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="E126" s="13" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="F126" s="13" t="inlineStr">
+        <is>
+          <t>通過</t>
+        </is>
+      </c>
+      <c r="G126" s="6" t="inlineStr">
+        <is>
+          <t>① 1.3.4 連續重啟 30 次：開場白 30/30、task_wdt 0、panic 0（修正前 19 次 4 次）② 用戶實際對話 20 輪（10:44–10:50）：20 輪都有回應，3 次未完成皆為用戶插話打斷且隨即恢復，短按合併為單輪；task_wdt 0、panic 0；CPU 抽樣照常（每輪 9–13 個）</t>
+        </is>
+      </c>
+      <c r="H126" s="13" t="inlineStr">
+        <is>
+          <t>8e8b449</t>
+        </is>
+      </c>
+      <c r="I126" s="6" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I125"/>
+  <autoFilter ref="A1:I126"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Note two unexplained power-on resets on USB under R-17.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/production-readiness.xlsx
+++ b/docs/production-readiness.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'任務清單'!$A$1:$P$57</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'待確認問題'!$A$1:$G$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$126</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$127</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -665,7 +665,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>最後更新：2026-10-08 10:51　·　本頁由 tracker.py 自動生成，請勿手動編輯</t>
+          <t>最後更新：2026-10-08 11:05　·　本頁由 tracker.py 自動生成，請勿手動編輯</t>
         </is>
       </c>
     </row>
@@ -2125,7 +2125,7 @@
       </c>
       <c r="C54" s="6" t="inlineStr">
         <is>
-          <t>阻塞：[2026-10-07] 等兩件事：(1) Spotpear 回覆充電芯片型號、充電電流、有沒有 power path（問題已草擬給用戶發送）(2) 用戶做一次實物放電：拔 USB 用到自動關機 → 插 USB 計時到能對話 → 插住用 30 分鐘。與 R-16 的放電測試同一次完成。韌體現況：brownout 重啟會補播低電提醒，運行記錄（開機時 Supply log）會記每次重啟原因，可據此判斷有沒有反覆 brownout；『掉電後先深睡充電』的緩解要等測試證明需要才做</t>
+          <t>阻塞：[2026-10-08] 2026-10-08 開發板 63:64 插著 USB 時兩次無法解釋的完全斷電重開：09:13:26（崩潰循環中）、10:44:33（閒置、用戶確認沒碰）。都是 USB 先斷線再以 ESP_RST_POWERON 開機，非 brownout；斷電前 6 秒 GPIO0 讀數 99.9% 參考值，屬突然切斷而非緩降（SupplyMonitor 取樣太疏抓不到瞬間）。韌體無法造成 POWERON，指向充電芯片/電池保護/供電路徑，應一併問 Spotpear；放電實測時留意插 USB 閒置時是否也會斷電</t>
         </is>
       </c>
       <c r="D54" s="11" t="n"/>
@@ -6542,7 +6542,7 @@
         </is>
       </c>
     </row>
-    <row r="54" ht="200" customHeight="1">
+    <row r="54" ht="382" customHeight="1">
       <c r="A54" s="13" t="inlineStr">
         <is>
           <t>R-17</t>
@@ -6602,7 +6602,8 @@
       <c r="P54" s="6" t="inlineStr">
         <is>
           <t>[2026-10-06] 新增
-[2026-10-07] 等兩件事：(1) Spotpear 回覆充電芯片型號、充電電流、有沒有 power path（問題已草擬給用戶發送）(2) 用戶做一次實物放電：拔 USB 用到自動關機 → 插 USB 計時到能對話 → 插住用 30 分鐘。與 R-16 的放電測試同一次完成。韌體現況：brownout 重啟會補播低電提醒，運行記錄（開機時 Supply log）會記每次重啟原因，可據此判斷有沒有反覆 brownout；『掉電後先深睡充電』的緩解要等測試證明需要才做</t>
+[2026-10-07] 等兩件事：(1) Spotpear 回覆充電芯片型號、充電電流、有沒有 power path（問題已草擬給用戶發送）(2) 用戶做一次實物放電：拔 USB 用到自動關機 → 插 USB 計時到能對話 → 插住用 30 分鐘。與 R-16 的放電測試同一次完成。韌體現況：brownout 重啟會補播低電提醒，運行記錄（開機時 Supply log）會記每次重啟原因，可據此判斷有沒有反覆 brownout；『掉電後先深睡充電』的緩解要等測試證明需要才做
+[2026-10-08] 2026-10-08 開發板 63:64 插著 USB 時兩次無法解釋的完全斷電重開：09:13:26（崩潰循環中）、10:44:33（閒置、用戶確認沒碰）。都是 USB 先斷線再以 ESP_RST_POWERON 開機，非 brownout；斷電前 6 秒 GPIO0 讀數 99.9% 參考值，屬突然切斷而非緩降（SupplyMonitor 取樣太疏抓不到瞬間）。韌體無法造成 POWERON，指向充電芯片/電池保護/供電路徑，應一併問 Spotpear；放電實測時留意插 USB 閒置時是否也會斷電</t>
         </is>
       </c>
     </row>
@@ -7292,7 +7293,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I126"/>
+  <dimension ref="A1:I127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -11747,8 +11748,43 @@
       </c>
       <c r="I126" s="6" t="n"/>
     </row>
+    <row r="127" ht="158" customHeight="1">
+      <c r="A127" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-08 11:05</t>
+        </is>
+      </c>
+      <c r="B127" s="13" t="inlineStr">
+        <is>
+          <t>R-17</t>
+        </is>
+      </c>
+      <c r="C127" s="6" t="inlineStr">
+        <is>
+          <t>Spotpear 電池耗盡時插電能否正常開機（供電路徑）</t>
+        </is>
+      </c>
+      <c r="D127" s="13" t="inlineStr">
+        <is>
+          <t>阻塞</t>
+        </is>
+      </c>
+      <c r="E127" s="13" t="inlineStr">
+        <is>
+          <t>阻塞</t>
+        </is>
+      </c>
+      <c r="F127" s="13" t="n"/>
+      <c r="G127" s="6" t="n"/>
+      <c r="H127" s="13" t="n"/>
+      <c r="I127" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-08 開發板 63:64 插著 USB 時兩次無法解釋的完全斷電重開：09:13:26（崩潰循環中）、10:44:33（閒置、用戶確認沒碰）。都是 USB 先斷線再以 ESP_RST_POWERON 開機，非 brownout；斷電前 6 秒 GPIO0 讀數 99.9% 參考值，屬突然切斷而非緩降（SupplyMonitor 取樣太疏抓不到瞬間）。韌體無法造成 POWERON，指向充電芯片/電池保護/供電路徑，應一併問 Spotpear；放電實測時留意插 USB 閒置時是否也會斷電</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I126"/>
+  <autoFilter ref="A1:I127"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record the OTA fall-back and reset-reason verdicts under P0-13.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/production-readiness.xlsx
+++ b/docs/production-readiness.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'任務清單'!$A$1:$P$57</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'待確認問題'!$A$1:$G$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$127</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$128</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -665,7 +665,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>最後更新：2026-10-08 11:05　·　本頁由 tracker.py 自動生成，請勿手動編輯</t>
+          <t>最後更新：2026-10-08 18:02　·　本頁由 tracker.py 自動生成，請勿手動編輯</t>
         </is>
       </c>
     </row>
@@ -3728,7 +3728,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="382" customHeight="1">
+    <row r="14" ht="409" customHeight="1">
       <c r="A14" s="13" t="inlineStr">
         <is>
           <t>P0-13</t>
@@ -3794,14 +3794,15 @@
       </c>
       <c r="O14" s="13" t="inlineStr">
         <is>
-          <t>68b9550</t>
+          <t>682f3b4</t>
         </is>
       </c>
       <c r="P14" s="6" t="inlineStr">
         <is>
           <t>[2026-10-08] 2026-10-08 b27cc07（分支 p0-13-ota）。部署時要套 20261008100000_firmware_releases.sql，發佈要用 SUPABASE_URL+service key 跑 tools/release_firmware.py
 [2026-10-08] 2026-10-08 實機①②通過，未部署。上線要：套 20261008100000、部署前端、用 release_firmware.py 發佈正式 build；生產 HTTPS（同 CF CA）的 1.6MB 下載尚未在線上驗證。開發板現跑 1.2.1 localall。未做：已確認版本日後若崩潰循環不會自動切回舊槽，需 USB 救（可另立任務）
-[2026-10-08] 2026-10-08 OTA 檢查併入 /api/generate_auth_token（68b9550），開機回到一次 TLS 握手；/api/ota/check 移除。token 路徑 API 11/11（舊韌體無 ota、格式錯仍發 token、回滾版本不再提供）；實機 1.3.0→1.3.1 經 token 回應安裝、試用、播完開場白、120s 確認。第一次升級 1.3.1 被 async_tcp 任務看門狗觸發重啟並正確回滾——是既有韌體 bug，見新任務</t>
+[2026-10-08] 2026-10-08 OTA 檢查併入 /api/generate_auth_token（68b9550），開機回到一次 TLS 握手；/api/ota/check 移除。token 路徑 API 11/11（舊韌體無 ota、格式錯仍發 token、回滾版本不再提供）；實機 1.3.0→1.3.1 經 token 回應安裝、試用、播完開場白、120s 確認。第一次升級 1.3.1 被 async_tcp 任務看門狗觸發重啟並正確回滾——是既有韌體 bug，見新任務
+[2026-10-08] 2026-10-08 交板前強化（682f3b4）：① 確認後連續崩潰 3 次 → 切回另一槽位（每段崩潰期一次）、立即重新確認、上報失敗 ② 回滾按重啟原因判定：崩潰/看門狗即失敗，斷電等非崩潰原因可重試 2 次（R-17 會自己斷電）。實機 1.5.x：試用期內 EN 重啟 → 重試第 2 次並確認；1.5.2 確認後崩潰 3 次 → 回 1.5.1、重新確認、報失敗；1.5.3 試用期崩潰 → 回滾、reason 4 即報失敗。runbook 已加 20261008100000 與 OTA 檢查（3aa632a）。上線後須用開發板對雲端走一次 HTTPS OTA 再交板</t>
         </is>
       </c>
     </row>
@@ -7293,7 +7294,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I127"/>
+  <dimension ref="A1:I128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -11783,8 +11784,47 @@
         </is>
       </c>
     </row>
+    <row r="128" ht="186" customHeight="1">
+      <c r="A128" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-08 18:02</t>
+        </is>
+      </c>
+      <c r="B128" s="13" t="inlineStr">
+        <is>
+          <t>P0-13</t>
+        </is>
+      </c>
+      <c r="C128" s="6" t="inlineStr">
+        <is>
+          <t>讓 OTA 真正可用並能回滾</t>
+        </is>
+      </c>
+      <c r="D128" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="E128" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F128" s="13" t="n"/>
+      <c r="G128" s="6" t="n"/>
+      <c r="H128" s="13" t="inlineStr">
+        <is>
+          <t>682f3b4</t>
+        </is>
+      </c>
+      <c r="I128" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-08 交板前強化（682f3b4）：① 確認後連續崩潰 3 次 → 切回另一槽位（每段崩潰期一次）、立即重新確認、上報失敗 ② 回滾按重啟原因判定：崩潰/看門狗即失敗，斷電等非崩潰原因可重試 2 次（R-17 會自己斷電）。實機 1.5.x：試用期內 EN 重啟 → 重試第 2 次並確認；1.5.2 確認後崩潰 3 次 → 回 1.5.1、重新確認、報失敗；1.5.3 試用期崩潰 → 回滾、reason 4 即報失敗。runbook 已加 20261008100000 與 OTA 檢查（3aa632a）。上線後須用開發板對雲端走一次 HTTPS OTA 再交板</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I127"/>
+  <autoFilter ref="A1:I128"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Track P1-12 (per-device memory, unbind dialog) and add R-20.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/production-readiness.xlsx
+++ b/docs/production-readiness.xlsx
@@ -13,9 +13,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="更新記錄" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'任務清單'!$A$1:$P$57</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'任務清單'!$A$1:$P$62</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'待確認問題'!$A$1:$G$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$128</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$144</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -641,7 +641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I82"/>
+  <dimension ref="A1:I86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -665,14 +665,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>最後更新：2026-10-08 18:02　·　本頁由 tracker.py 自動生成，請勿手動編輯</t>
+          <t>最後更新：2026-10-09 21:54　·　本頁由 tracker.py 自動生成，請勿手動編輯</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>總進度：4/55 已完成（7%）　·　目前階段：1 止血定案（10/5–10/16）</t>
+          <t>總進度：5/60 已完成（8%）　·　目前階段：1 止血定案（10/5–10/16）</t>
         </is>
       </c>
     </row>
@@ -744,11 +744,11 @@
       </c>
       <c r="E6" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A6,'任務清單'!$F:$F,E$5)</f>
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F6" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A6,'任務清單'!$F:$F,F$5)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G6" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A6,'任務清單'!$F:$F,G$5)</f>
@@ -760,7 +760,7 @@
       </c>
       <c r="I6" s="8">
         <f>IFERROR(F6/(C6-H6),0)</f>
-        <v>0.0</v>
+        <v>0.0625</v>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1">
@@ -776,7 +776,7 @@
       </c>
       <c r="C7" s="7">
         <f>COUNTIF('任務清單'!$B:$B,$A7)</f>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D7" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A7,'任務清單'!$F:$F,D$5)</f>
@@ -784,7 +784,7 @@
       </c>
       <c r="E7" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A7,'任務清單'!$F:$F,E$5)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F7" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A7,'任務清單'!$F:$F,F$5)</f>
@@ -816,11 +816,11 @@
       </c>
       <c r="C8" s="7">
         <f>COUNTIF('任務清單'!$B:$B,$A8)</f>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D8" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A8,'任務清單'!$F:$F,D$5)</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E8" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A8,'任務清單'!$F:$F,E$5)</f>
@@ -840,7 +840,7 @@
       </c>
       <c r="I8" s="8">
         <f>IFERROR(F8/(C8-H8),0)</f>
-        <v>0.2727272727272727</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="9" ht="18" customHeight="1">
@@ -856,11 +856,11 @@
       </c>
       <c r="C9" s="7">
         <f>COUNTIF('任務清單'!$B:$B,$A9)</f>
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D9" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A9,'任務清單'!$F:$F,D$5)</f>
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="E9" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A9,'任務清單'!$F:$F,E$5)</f>
@@ -880,7 +880,7 @@
       </c>
       <c r="I9" s="8">
         <f>IFERROR(F9/(C9-H9),0)</f>
-        <v>0.058823529411764705</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="10">
@@ -892,11 +892,11 @@
       <c r="B10" s="6" t="n"/>
       <c r="C10" s="5">
         <f>SUM(C6:C9)</f>
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="D10" s="5">
         <f>SUM(D6:D9)</f>
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="E10" s="5">
         <f>SUM(E6:E9)</f>
@@ -904,7 +904,7 @@
       </c>
       <c r="F10" s="5">
         <f>SUM(F6:F9)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G10" s="5">
         <f>SUM(G6:G9)</f>
@@ -916,7 +916,7 @@
       </c>
       <c r="I10" s="9">
         <f>IFERROR(F10/(C10-H10),0)</f>
-        <v>0.07272727272727272</v>
+        <v>0.08333333333333333</v>
       </c>
     </row>
     <row r="12">
@@ -1019,11 +1019,11 @@
       </c>
       <c r="C14" s="7">
         <f>COUNTIF('任務清單'!$C:$C,$A14)</f>
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="D14" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A14,'任務清單'!$F:$F,D$12)</f>
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="E14" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A14,'任務清單'!$F:$F,E$12)</f>
@@ -1031,7 +1031,7 @@
       </c>
       <c r="F14" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A14,'任務清單'!$F:$F,F$12)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G14" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A14,'任務清單'!$F:$F,G$12)</f>
@@ -1043,7 +1043,7 @@
       </c>
       <c r="I14" s="8">
         <f>IFERROR(F14/(C14-H14),0)</f>
-        <v>0.07142857142857142</v>
+        <v>0.1111111111111111</v>
       </c>
     </row>
     <row r="15" ht="32" customHeight="1">
@@ -1059,11 +1059,11 @@
       </c>
       <c r="C15" s="7">
         <f>COUNTIF('任務清單'!$C:$C,$A15)</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D15" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A15,'任務清單'!$F:$F,D$12)</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E15" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A15,'任務清單'!$F:$F,E$12)</f>
@@ -1135,11 +1135,11 @@
       <c r="B17" s="6" t="n"/>
       <c r="C17" s="5">
         <f>SUM(C13:C16)</f>
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="D17" s="5">
         <f>SUM(D13:D16)</f>
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="E17" s="5">
         <f>SUM(E13:E16)</f>
@@ -1147,7 +1147,7 @@
       </c>
       <c r="F17" s="5">
         <f>SUM(F13:F16)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G17" s="5">
         <f>SUM(G13:G16)</f>
@@ -1159,7 +1159,7 @@
       </c>
       <c r="I17" s="9">
         <f>IFERROR(F17/(C17-H17),0)</f>
-        <v>0.07272727272727272</v>
+        <v>0.08333333333333333</v>
       </c>
     </row>
     <row r="19">
@@ -1679,15 +1679,15 @@
       <c r="H35" s="11" t="n"/>
       <c r="I35" s="12" t="n"/>
     </row>
-    <row r="36" ht="186" customHeight="1">
+    <row r="36" ht="409" customHeight="1">
       <c r="A36" s="13" t="inlineStr">
         <is>
-          <t>P0-13</t>
+          <t>P1-12</t>
         </is>
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>讓 OTA 真正可用並能回滾</t>
+          <t>設備解綁時的記憶處理：確認、預設保留、可選清除</t>
         </is>
       </c>
       <c r="C36" s="13" t="inlineStr">
@@ -1702,8 +1702,8 @@
       </c>
       <c r="E36" s="6" t="inlineStr">
         <is>
-          <t>上次測試：通過 — 實機開發板 63:64（localall，本機後端）：① 1.1.0→1.2.1 OTA 下載 14s、sha256 過、重啟到 app1 試用、連上語音伺服器後穩定 120s 才 confirmed、開場白播完、devices 記 1.2.1 ② 推開機 3s 崩潰的 1.2.2：安裝→崩潰→bootloader 1s 內回到 1.2.1『rolled back from 1.2.2』→上報 ota_failed_version=1.2.2→再重啟不再下載。過程中測出並修好 2 個 bug：收到 auth 即確認太早（1.0.2 確認後崩潰循環，887b769 改為穩定 2 分鐘）；millis()|1 計時繞回導致誤回滾（3a874dd）。API 16/16，pio 全 env 通過
-填入真實 URL 與 CA；新韌體啟動自檢通過才標記有效，否則自動回滾；設備上報韌體版本。</t>
+          <t>上次測試：部分通過 — 本機（開發板 DEV636 身份的模擬裝置 + 網頁）：TC1/2/5/6/7/8/10/11/13 通過；TC3 重綁後 log『Loaded 2 fact(s)』；TC4 第二台 starts cold、設定頁可切換；TC9 DB 層 B 解綁回 NULL、清除報錯，anon/authenticated 無 EXECUTE；TC10 舊代數寫入三表皆 HTTP 400、清除後 40 秒仍 0 行；TC12 伺服器端 4401 通過；pytest 214 passed。未做：TC12 真機 202/配對、TC3 真機問答、TC14 網頁語音。
+① 按「解綁」先彈出確認對話框，取消則什麼都不改。② 對話框預設保留記憶；「同時清除記憶」要主動勾選，並寫明無法復原。③ 記憶跟設備：鍵是 (user_id, device_id, ip_key)。同一帳號的每台設備各自一份記憶；保留時，同帳號重綁同一台會接著用；換新設備從空白開始（搬記憶交給 R-11）。④ 清除在伺服器端一個交易完成：先刪該設備的 memory_facts、memory_segments、conversations（連帳號的舊 memories），再解綁；任何一步失敗就不解綁，並顯示錯誤。⑤ 其他帳號認領同一台設備，看不到舊記憶（靠 user_id 隔離，不靠刪除成功）。⑥ 設定頁按設備顯示記憶；「清除全部」只清所選設備，連 conversations 一起刪。⑦ 對話中清除，之後的寫入和 consolidation 不會把記憶寫回（devices.memories_revision + trigger）。⑧ 未認領的設備不能對話：/ws/esp32 查到設備沒有 user_id 就在 auth 前以 4401 關閉，即使 24 小時 token 未過期；韌體重新取 token 拿到 202，回到配對狀態。⑨ 解綁時立即中斷該設備正在進行的語音 session。⑩ 網頁語音（playground）沒有設備，不讀也不寫記憶。</t>
         </is>
       </c>
       <c r="F36" s="11" t="n"/>
@@ -1935,15 +1935,15 @@
       <c r="H45" s="11" t="n"/>
       <c r="I45" s="12" t="n"/>
     </row>
-    <row r="46" ht="88" customHeight="1">
+    <row r="46" ht="130" customHeight="1">
       <c r="A46" s="13" t="inlineStr">
         <is>
-          <t>P2-11</t>
+          <t>P0-13</t>
         </is>
       </c>
       <c r="B46" s="6" t="inlineStr">
         <is>
-          <t>C3 播放時 async_tcp 觸發任務看門狗重啟</t>
+          <t>讓 OTA 真正可用並能回滾</t>
         </is>
       </c>
       <c r="C46" s="13" t="inlineStr">
@@ -1953,12 +1953,12 @@
       </c>
       <c r="D46" s="13" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="E46" s="6" t="inlineStr">
         <is>
-          <t>① 1.3.4 連續重啟 30 次：開場白 30/30、task_wdt 0、panic 0（修正前 19 次 4 次）② 用戶實際對話 20 輪（10:44–10:50）：20 輪都有回應，3 次未完成皆為用戶插話打斷且隨即恢復，短按合併為單輪；task_wdt 0、panic 0；CPU 抽樣照常（每輪 9–13 個）</t>
+          <t>生產雲端 HTTPS OTA（2026-10-09）：release_firmware.py publish spotpear-ai-toy --current → 1.0.1 現行；42:34 開機 1.0.0 → token 回應 Installing 1.0.1 (1655776 bytes) → 經 Cloudflare+nginx 下載 100% → 重啟到 app1 on probation → 連上語音伺服器 → 120s 後『Firmware 1.0.1 confirmed』。②崩潰回滾沿用 10-08 開發板實測（1.2.2/1.5.3 回滾、1.5.2 切回舊槽）；本機 63:64 1.5.1→1.6.1 亦確認</t>
         </is>
       </c>
       <c r="F46" s="11" t="n"/>
@@ -1969,12 +1969,12 @@
     <row r="47" ht="88" customHeight="1">
       <c r="A47" s="13" t="inlineStr">
         <is>
-          <t>R-03</t>
+          <t>P2-11</t>
         </is>
       </c>
       <c r="B47" s="6" t="inlineStr">
         <is>
-          <t>移除不用的 Deno／Cloudflare 後端與上游預設主機</t>
+          <t>C3 播放時 async_tcp 觸發任務看門狗重啟</t>
         </is>
       </c>
       <c r="C47" s="13" t="inlineStr">
@@ -1984,12 +1984,12 @@
       </c>
       <c r="D47" s="13" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="E47" s="6" t="inlineStr">
         <is>
-          <t>① grep deno.dev|workers.dev|railway.app|VOICE_SERVER_DENO|VOICE_SERVER_CLOUDFLARE 全 repo → 只剩 seed.json 的任務描述本身 ② pio run 18 個 env 全 SUCCESS（S3 devkit/Waveshare/xmini-c3/Spotpear 各變體）③ FastAPI pytest 182 passed；另 tsc --noEmit 通過</t>
+          <t>① 1.3.4 連續重啟 30 次：開場白 30/30、task_wdt 0、panic 0（修正前 19 次 4 次）② 用戶實際對話 20 輪（10:44–10:50）：20 輪都有回應，3 次未完成皆為用戶插話打斷且隨即恢復，短按合併為單輪；task_wdt 0、panic 0；CPU 抽樣照常（每輪 9–13 個）</t>
         </is>
       </c>
       <c r="F47" s="11" t="n"/>
@@ -2000,12 +2000,12 @@
     <row r="48" ht="88" customHeight="1">
       <c r="A48" s="13" t="inlineStr">
         <is>
-          <t>P2-01</t>
+          <t>R-03</t>
         </is>
       </c>
       <c r="B48" s="6" t="inlineStr">
         <is>
-          <t>修好後端測試環境</t>
+          <t>移除不用的 Deno／Cloudflare 後端與上游預設主機</t>
         </is>
       </c>
       <c r="C48" s="13" t="inlineStr">
@@ -2020,7 +2020,7 @@
       </c>
       <c r="E48" s="6" t="inlineStr">
         <is>
-          <t>cd server/fastapi &amp;&amp; .venv/bin/python -m pytest -q → 173 passed（原本 60 個 async 測試報「not natively supported」）；pyproject dev group 加 pytest&gt;=9,&lt;10、pytest-asyncio&gt;=1.4,&lt;2，asyncio_mode=auto；pip install --dry-run --group dev 可解析</t>
+          <t>① grep deno.dev|workers.dev|railway.app|VOICE_SERVER_DENO|VOICE_SERVER_CLOUDFLARE 全 repo → 只剩 seed.json 的任務描述本身 ② pio run 18 個 env 全 SUCCESS（S3 devkit/Waveshare/xmini-c3/Spotpear 各變體）③ FastAPI pytest 182 passed；另 tsc --noEmit 通過</t>
         </is>
       </c>
       <c r="F48" s="11" t="n"/>
@@ -2028,15 +2028,15 @@
       <c r="H48" s="11" t="n"/>
       <c r="I48" s="12" t="n"/>
     </row>
-    <row r="49" ht="60" customHeight="1">
+    <row r="49" ht="88" customHeight="1">
       <c r="A49" s="13" t="inlineStr">
         <is>
-          <t>P2-03</t>
+          <t>P2-01</t>
         </is>
       </c>
       <c r="B49" s="6" t="inlineStr">
         <is>
-          <t>提交目前未提交的改動</t>
+          <t>修好後端測試環境</t>
         </is>
       </c>
       <c r="C49" s="13" t="inlineStr">
@@ -2046,12 +2046,12 @@
       </c>
       <c r="D49" s="13" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="E49" s="6" t="inlineStr">
         <is>
-          <t>git status --short → 0 行；3bc7119..b322375 按主題拆成 5 個 commit（50 檔：xmini-c3 電量、facts 記憶層、日期時間天氣、BEAM 評測、進度追蹤）；git ls-remote mygithub main = HEAD = b322375</t>
+          <t>cd server/fastapi &amp;&amp; .venv/bin/python -m pytest -q → 173 passed（原本 60 個 async 測試報「not natively supported」）；pyproject dev group 加 pytest&gt;=9,&lt;10、pytest-asyncio&gt;=1.4,&lt;2，asyncio_mode=auto；pip install --dry-run --group dev 可解析</t>
         </is>
       </c>
       <c r="F49" s="11" t="n"/>
@@ -2059,50 +2059,58 @@
       <c r="H49" s="11" t="n"/>
       <c r="I49" s="12" t="n"/>
     </row>
-    <row r="51">
-      <c r="A51" s="10" t="inlineStr">
+    <row r="50" ht="60" customHeight="1">
+      <c r="A50" s="13" t="inlineStr">
+        <is>
+          <t>P2-03</t>
+        </is>
+      </c>
+      <c r="B50" s="6" t="inlineStr">
+        <is>
+          <t>提交目前未提交的改動</t>
+        </is>
+      </c>
+      <c r="C50" s="13" t="inlineStr">
+        <is>
+          <t>通過</t>
+        </is>
+      </c>
+      <c r="D50" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="E50" s="6" t="inlineStr">
+        <is>
+          <t>git status --short → 0 行；3bc7119..b322375 按主題拆成 5 個 commit（50 檔：xmini-c3 電量、facts 記憶層、日期時間天氣、BEAM 評測、進度追蹤）；git ls-remote mygithub main = HEAD = b322375</t>
+        </is>
+      </c>
+      <c r="F50" s="11" t="n"/>
+      <c r="G50" s="11" t="n"/>
+      <c r="H50" s="11" t="n"/>
+      <c r="I50" s="12" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="10" t="inlineStr">
         <is>
           <t>⏳ 等待依賴 / ⛔ 阻塞</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="4" t="inlineStr">
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
         <is>
           <t>編號</t>
         </is>
       </c>
-      <c r="B52" s="4" t="inlineStr">
+      <c r="B53" s="4" t="inlineStr">
         <is>
           <t>任務</t>
         </is>
       </c>
-      <c r="C52" s="4" t="inlineStr">
+      <c r="C53" s="4" t="inlineStr">
         <is>
           <t>在等什麼</t>
-        </is>
-      </c>
-      <c r="D52" s="11" t="n"/>
-      <c r="E52" s="11" t="n"/>
-      <c r="F52" s="11" t="n"/>
-      <c r="G52" s="11" t="n"/>
-      <c r="H52" s="11" t="n"/>
-      <c r="I52" s="12" t="n"/>
-    </row>
-    <row r="53" ht="60" customHeight="1">
-      <c r="A53" s="13" t="inlineStr">
-        <is>
-          <t>R-16</t>
-        </is>
-      </c>
-      <c r="B53" s="6" t="inlineStr">
-        <is>
-          <t>Spotpear 量產版加電池電壓檢測（GPIO0 分壓）</t>
-        </is>
-      </c>
-      <c r="C53" s="6" t="inlineStr">
-        <is>
-          <t>阻塞：[2026-10-07] 仍按 10/06 決定暫緩：等用戶做充滿再放電測試（與 R-17 同一次），看 VDD 低電提醒在關機前多久觸發；太遲或不觸發才向 Spotpear 提改板。已把分壓改板的問題一併放進給 Spotpear 的草稿，方便同一封發出</t>
         </is>
       </c>
       <c r="D53" s="11" t="n"/>
@@ -2112,20 +2120,20 @@
       <c r="H53" s="11" t="n"/>
       <c r="I53" s="12" t="n"/>
     </row>
-    <row r="54" ht="88" customHeight="1">
+    <row r="54" ht="60" customHeight="1">
       <c r="A54" s="13" t="inlineStr">
         <is>
-          <t>R-17</t>
+          <t>R-16</t>
         </is>
       </c>
       <c r="B54" s="6" t="inlineStr">
         <is>
-          <t>Spotpear 電池耗盡時插電能否正常開機（供電路徑）</t>
+          <t>Spotpear 量產版加電池電壓檢測（GPIO0 分壓）</t>
         </is>
       </c>
       <c r="C54" s="6" t="inlineStr">
         <is>
-          <t>阻塞：[2026-10-08] 2026-10-08 開發板 63:64 插著 USB 時兩次無法解釋的完全斷電重開：09:13:26（崩潰循環中）、10:44:33（閒置、用戶確認沒碰）。都是 USB 先斷線再以 ESP_RST_POWERON 開機，非 brownout；斷電前 6 秒 GPIO0 讀數 99.9% 參考值，屬突然切斷而非緩降（SupplyMonitor 取樣太疏抓不到瞬間）。韌體無法造成 POWERON，指向充電芯片/電池保護/供電路徑，應一併問 Spotpear；放電實測時留意插 USB 閒置時是否也會斷電</t>
+          <t>阻塞：[2026-10-07] 仍按 10/06 決定暫緩：等用戶做充滿再放電測試（與 R-17 同一次），看 VDD 低電提醒在關機前多久觸發；太遲或不觸發才向 Spotpear 提改板。已把分壓改板的問題一併放進給 Spotpear 的草稿，方便同一封發出</t>
         </is>
       </c>
       <c r="D54" s="11" t="n"/>
@@ -2135,20 +2143,20 @@
       <c r="H54" s="11" t="n"/>
       <c r="I54" s="12" t="n"/>
     </row>
-    <row r="55" ht="18" customHeight="1">
+    <row r="55" ht="88" customHeight="1">
       <c r="A55" s="13" t="inlineStr">
         <is>
-          <t>P0-07</t>
+          <t>R-17</t>
         </is>
       </c>
       <c r="B55" s="6" t="inlineStr">
         <is>
-          <t>輪換 JWT secret，作廢已發出的 token</t>
+          <t>Spotpear 電池耗盡時插電能否正常開機（供電路徑）</t>
         </is>
       </c>
       <c r="C55" s="6" t="inlineStr">
         <is>
-          <t>等 P0-06</t>
+          <t>阻塞：[2026-10-08] 2026-10-08 開發板 63:64 插著 USB 時兩次無法解釋的完全斷電重開：09:13:26（崩潰循環中）、10:44:33（閒置、用戶確認沒碰）。都是 USB 先斷線再以 ESP_RST_POWERON 開機，非 brownout；斷電前 6 秒 GPIO0 讀數 99.9% 參考值，屬突然切斷而非緩降（SupplyMonitor 取樣太疏抓不到瞬間）。韌體無法造成 POWERON，指向充電芯片/電池保護/供電路徑，應一併問 Spotpear；放電實測時留意插 USB 閒置時是否也會斷電</t>
         </is>
       </c>
       <c r="D55" s="11" t="n"/>
@@ -2161,12 +2169,12 @@
     <row r="56" ht="18" customHeight="1">
       <c r="A56" s="13" t="inlineStr">
         <is>
-          <t>P0-11</t>
+          <t>P0-07</t>
         </is>
       </c>
       <c r="B56" s="6" t="inlineStr">
         <is>
-          <t>設備認領要求持有證明</t>
+          <t>輪換 JWT secret，作廢已發出的 token</t>
         </is>
       </c>
       <c r="C56" s="6" t="inlineStr">
@@ -2184,17 +2192,17 @@
     <row r="57" ht="18" customHeight="1">
       <c r="A57" s="13" t="inlineStr">
         <is>
-          <t>P1-10</t>
+          <t>P0-11</t>
         </is>
       </c>
       <c r="B57" s="6" t="inlineStr">
         <is>
-          <t>管理操作審計記錄</t>
+          <t>設備認領要求持有證明</t>
         </is>
       </c>
       <c r="C57" s="6" t="inlineStr">
         <is>
-          <t>等 P0-12</t>
+          <t>等 P0-06</t>
         </is>
       </c>
       <c r="D57" s="11" t="n"/>
@@ -2207,17 +2215,17 @@
     <row r="58" ht="18" customHeight="1">
       <c r="A58" s="13" t="inlineStr">
         <is>
-          <t>R-05</t>
+          <t>P1-10</t>
         </is>
       </c>
       <c r="B58" s="6" t="inlineStr">
         <is>
-          <t>內測版外殼（3D 打印 20 台）</t>
+          <t>管理操作審計記錄</t>
         </is>
       </c>
       <c r="C58" s="6" t="inlineStr">
         <is>
-          <t>等 R-01</t>
+          <t>等 P0-12</t>
         </is>
       </c>
       <c r="D58" s="11" t="n"/>
@@ -2230,17 +2238,17 @@
     <row r="59" ht="18" customHeight="1">
       <c r="A59" s="13" t="inlineStr">
         <is>
-          <t>R-06</t>
+          <t>R-05</t>
         </is>
       </c>
       <c r="B59" s="6" t="inlineStr">
         <is>
-          <t>家長自助上手流程</t>
+          <t>內測版外殼（3D 打印 20 台）</t>
         </is>
       </c>
       <c r="C59" s="6" t="inlineStr">
         <is>
-          <t>等 P0-11</t>
+          <t>等 R-01</t>
         </is>
       </c>
       <c r="D59" s="11" t="n"/>
@@ -2250,20 +2258,20 @@
       <c r="H59" s="11" t="n"/>
       <c r="I59" s="12" t="n"/>
     </row>
-    <row r="60" ht="46" customHeight="1">
+    <row r="60" ht="18" customHeight="1">
       <c r="A60" s="13" t="inlineStr">
         <is>
-          <t>R-13</t>
+          <t>R-06</t>
         </is>
       </c>
       <c r="B60" s="6" t="inlineStr">
         <is>
-          <t>CP1 內測就緒檢查（10/30）</t>
+          <t>家長自助上手流程</t>
         </is>
       </c>
       <c r="C60" s="6" t="inlineStr">
         <is>
-          <t>等 P0-02、P0-03、P0-04、P0-05、P0-06、P0-07、P0-08、P0-09、P0-10、P0-11、P0-12、P0-13、P1-01、P1-02、P2-09、R-01、R-02、R-04、R-05、R-06、P0-15、P0-16、P1-09、P1-11</t>
+          <t>等 P0-11</t>
         </is>
       </c>
       <c r="D60" s="11" t="n"/>
@@ -2273,20 +2281,20 @@
       <c r="H60" s="11" t="n"/>
       <c r="I60" s="12" t="n"/>
     </row>
-    <row r="61" ht="18" customHeight="1">
+    <row r="61" ht="46" customHeight="1">
       <c r="A61" s="13" t="inlineStr">
         <is>
-          <t>P0-14</t>
+          <t>R-13</t>
         </is>
       </c>
       <c r="B61" s="6" t="inlineStr">
         <is>
-          <t>韌體簽章、Secure Boot 與 Flash 加密</t>
+          <t>CP1 內測就緒檢查（10/30）</t>
         </is>
       </c>
       <c r="C61" s="6" t="inlineStr">
         <is>
-          <t>等 P0-13、R-01</t>
+          <t>等 P0-02、P0-03、P0-04、P0-05、P0-06、P0-07、P0-08、P0-09、P0-10、P0-11、P0-12、P1-01、P1-02、P2-09、R-01、R-02、R-04、R-05、R-06、P0-15、P0-16、P1-09、P1-11</t>
         </is>
       </c>
       <c r="D61" s="11" t="n"/>
@@ -2296,20 +2304,20 @@
       <c r="H61" s="11" t="n"/>
       <c r="I61" s="12" t="n"/>
     </row>
-    <row r="62" ht="18" customHeight="1">
+    <row r="62" ht="32" customHeight="1">
       <c r="A62" s="13" t="inlineStr">
         <is>
-          <t>P1-06</t>
+          <t>R-18</t>
         </is>
       </c>
       <c r="B62" s="6" t="inlineStr">
         <is>
-          <t>處理 GPL-3.0 依賴（arduino-audio-tools）</t>
+          <t>長按 BOOT 重新配網（開 AIBuddy-XXXX 熱點）</t>
         </is>
       </c>
       <c r="C62" s="6" t="inlineStr">
         <is>
-          <t>等 Q3</t>
+          <t>等 R-01</t>
         </is>
       </c>
       <c r="D62" s="11" t="n"/>
@@ -2319,20 +2327,20 @@
       <c r="H62" s="11" t="n"/>
       <c r="I62" s="12" t="n"/>
     </row>
-    <row r="63" ht="18" customHeight="1">
+    <row r="63" ht="32" customHeight="1">
       <c r="A63" s="13" t="inlineStr">
         <is>
-          <t>P1-07</t>
+          <t>R-19</t>
         </is>
       </c>
       <c r="B63" s="6" t="inlineStr">
         <is>
-          <t>LGPL 合規與第三方授權聲明</t>
+          <t>外接按鈕：量產板加 I2C 擴展晶片（TCA9555）</t>
         </is>
       </c>
       <c r="C63" s="6" t="inlineStr">
         <is>
-          <t>等 Q3</t>
+          <t>等 R-01</t>
         </is>
       </c>
       <c r="D63" s="11" t="n"/>
@@ -2345,17 +2353,17 @@
     <row r="64" ht="18" customHeight="1">
       <c r="A64" s="13" t="inlineStr">
         <is>
-          <t>P1-08</t>
+          <t>R-20</t>
         </is>
       </c>
       <c r="B64" s="6" t="inlineStr">
         <is>
-          <t>硬件認證</t>
+          <t>孩子資料與角色改成每台設備一份</t>
         </is>
       </c>
       <c r="C64" s="6" t="inlineStr">
         <is>
-          <t>等 R-01、R-05</t>
+          <t>等 P1-12</t>
         </is>
       </c>
       <c r="D64" s="11" t="n"/>
@@ -2368,17 +2376,17 @@
     <row r="65" ht="18" customHeight="1">
       <c r="A65" s="13" t="inlineStr">
         <is>
-          <t>R-07</t>
+          <t>P0-14</t>
         </is>
       </c>
       <c r="B65" s="6" t="inlineStr">
         <is>
-          <t>20 個家庭封閉內測</t>
+          <t>韌體簽章、Secure Boot 與 Flash 加密</t>
         </is>
       </c>
       <c r="C65" s="6" t="inlineStr">
         <is>
-          <t>等 R-13</t>
+          <t>等 R-01</t>
         </is>
       </c>
       <c r="D65" s="11" t="n"/>
@@ -2391,17 +2399,17 @@
     <row r="66" ht="18" customHeight="1">
       <c r="A66" s="13" t="inlineStr">
         <is>
-          <t>R-08</t>
+          <t>P1-06</t>
         </is>
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
-          <t>第 8 週關卡決策</t>
+          <t>處理 GPL-3.0 依賴（arduino-audio-tools）</t>
         </is>
       </c>
       <c r="C66" s="6" t="inlineStr">
         <is>
-          <t>等 R-07、P2-09、P1-08</t>
+          <t>等 Q3</t>
         </is>
       </c>
       <c r="D66" s="11" t="n"/>
@@ -2414,17 +2422,17 @@
     <row r="67" ht="18" customHeight="1">
       <c r="A67" s="13" t="inlineStr">
         <is>
-          <t>R-14</t>
+          <t>P1-07</t>
         </is>
       </c>
       <c r="B67" s="6" t="inlineStr">
         <is>
-          <t>離線兒歌與故事</t>
+          <t>LGPL 合規與第三方授權聲明</t>
         </is>
       </c>
       <c r="C67" s="6" t="inlineStr">
         <is>
-          <t>等 R-01</t>
+          <t>等 Q3</t>
         </is>
       </c>
       <c r="D67" s="11" t="n"/>
@@ -2437,17 +2445,17 @@
     <row r="68" ht="18" customHeight="1">
       <c r="A68" s="13" t="inlineStr">
         <is>
-          <t>P2-05</t>
+          <t>P1-08</t>
         </is>
       </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t>拒絕未知設備並限制用量</t>
+          <t>硬件認證</t>
         </is>
       </c>
       <c r="C68" s="6" t="inlineStr">
         <is>
-          <t>等 P0-08</t>
+          <t>等 R-01、R-05</t>
         </is>
       </c>
       <c r="D68" s="11" t="n"/>
@@ -2460,17 +2468,17 @@
     <row r="69" ht="18" customHeight="1">
       <c r="A69" s="13" t="inlineStr">
         <is>
-          <t>R-09</t>
+          <t>R-07</t>
         </is>
       </c>
       <c r="B69" s="6" t="inlineStr">
         <is>
-          <t>量產外殼（真空複模）</t>
+          <t>20 個家庭封閉內測</t>
         </is>
       </c>
       <c r="C69" s="6" t="inlineStr">
         <is>
-          <t>等 R-08、R-05</t>
+          <t>等 R-13</t>
         </is>
       </c>
       <c r="D69" s="11" t="n"/>
@@ -2483,17 +2491,17 @@
     <row r="70" ht="18" customHeight="1">
       <c r="A70" s="13" t="inlineStr">
         <is>
-          <t>R-10</t>
+          <t>R-08</t>
         </is>
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>出廠流程</t>
+          <t>第 8 週關卡決策</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr">
         <is>
-          <t>等 P0-06、P0-14、R-01</t>
+          <t>等 R-07、P2-09、P1-08</t>
         </is>
       </c>
       <c r="D70" s="11" t="n"/>
@@ -2506,17 +2514,17 @@
     <row r="71" ht="18" customHeight="1">
       <c r="A71" s="13" t="inlineStr">
         <is>
-          <t>R-15</t>
+          <t>R-14</t>
         </is>
       </c>
       <c r="B71" s="6" t="inlineStr">
         <is>
-          <t>農曆新年前交付（生產 1/15、送達 1/29）</t>
+          <t>離線兒歌與故事</t>
         </is>
       </c>
       <c r="C71" s="6" t="inlineStr">
         <is>
-          <t>等 R-09、R-10</t>
+          <t>等 R-01</t>
         </is>
       </c>
       <c r="D71" s="11" t="n"/>
@@ -2526,27 +2534,66 @@
       <c r="H71" s="11" t="n"/>
       <c r="I71" s="12" t="n"/>
     </row>
-    <row r="73">
-      <c r="A73" s="10" t="inlineStr">
-        <is>
-          <t>❓ 待確認問題</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="4" t="inlineStr">
-        <is>
-          <t>編號</t>
-        </is>
-      </c>
-      <c r="B74" s="4" t="inlineStr">
-        <is>
-          <t>問題</t>
-        </is>
-      </c>
-      <c r="C74" s="4" t="inlineStr">
-        <is>
-          <t>影響的任務 / 為什麼重要</t>
+    <row r="72" ht="18" customHeight="1">
+      <c r="A72" s="13" t="inlineStr">
+        <is>
+          <t>P2-05</t>
+        </is>
+      </c>
+      <c r="B72" s="6" t="inlineStr">
+        <is>
+          <t>拒絕未知設備並限制用量</t>
+        </is>
+      </c>
+      <c r="C72" s="6" t="inlineStr">
+        <is>
+          <t>等 P0-08</t>
+        </is>
+      </c>
+      <c r="D72" s="11" t="n"/>
+      <c r="E72" s="11" t="n"/>
+      <c r="F72" s="11" t="n"/>
+      <c r="G72" s="11" t="n"/>
+      <c r="H72" s="11" t="n"/>
+      <c r="I72" s="12" t="n"/>
+    </row>
+    <row r="73" ht="18" customHeight="1">
+      <c r="A73" s="13" t="inlineStr">
+        <is>
+          <t>R-09</t>
+        </is>
+      </c>
+      <c r="B73" s="6" t="inlineStr">
+        <is>
+          <t>量產外殼（真空複模）</t>
+        </is>
+      </c>
+      <c r="C73" s="6" t="inlineStr">
+        <is>
+          <t>等 R-08、R-05</t>
+        </is>
+      </c>
+      <c r="D73" s="11" t="n"/>
+      <c r="E73" s="11" t="n"/>
+      <c r="F73" s="11" t="n"/>
+      <c r="G73" s="11" t="n"/>
+      <c r="H73" s="11" t="n"/>
+      <c r="I73" s="12" t="n"/>
+    </row>
+    <row r="74" ht="18" customHeight="1">
+      <c r="A74" s="13" t="inlineStr">
+        <is>
+          <t>R-10</t>
+        </is>
+      </c>
+      <c r="B74" s="6" t="inlineStr">
+        <is>
+          <t>出廠流程</t>
+        </is>
+      </c>
+      <c r="C74" s="6" t="inlineStr">
+        <is>
+          <t>等 P0-06、P0-14、R-01、P2-12</t>
         </is>
       </c>
       <c r="D74" s="11" t="n"/>
@@ -2559,17 +2606,17 @@
     <row r="75" ht="18" customHeight="1">
       <c r="A75" s="13" t="inlineStr">
         <is>
-          <t>Q3</t>
+          <t>R-15</t>
         </is>
       </c>
       <c r="B75" s="6" t="inlineStr">
         <is>
-          <t>韌體打算閉源商業銷售嗎？</t>
+          <t>農曆新年前交付（生產 1/15、送達 1/29）</t>
         </is>
       </c>
       <c r="C75" s="6" t="inlineStr">
         <is>
-          <t>P1-06, P1-07：決定 GPL／LGPL 依賴要開源還是替換。</t>
+          <t>等 R-09、R-10</t>
         </is>
       </c>
       <c r="D75" s="11" t="n"/>
@@ -2582,61 +2629,116 @@
     <row r="77">
       <c r="A77" s="10" t="inlineStr">
         <is>
+          <t>❓ 待確認問題</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="4" t="inlineStr">
+        <is>
+          <t>編號</t>
+        </is>
+      </c>
+      <c r="B78" s="4" t="inlineStr">
+        <is>
+          <t>問題</t>
+        </is>
+      </c>
+      <c r="C78" s="4" t="inlineStr">
+        <is>
+          <t>影響的任務 / 為什麼重要</t>
+        </is>
+      </c>
+      <c r="D78" s="11" t="n"/>
+      <c r="E78" s="11" t="n"/>
+      <c r="F78" s="11" t="n"/>
+      <c r="G78" s="11" t="n"/>
+      <c r="H78" s="11" t="n"/>
+      <c r="I78" s="12" t="n"/>
+    </row>
+    <row r="79" ht="18" customHeight="1">
+      <c r="A79" s="13" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="B79" s="6" t="inlineStr">
+        <is>
+          <t>韌體打算閉源商業銷售嗎？</t>
+        </is>
+      </c>
+      <c r="C79" s="6" t="inlineStr">
+        <is>
+          <t>P1-06, P1-07：決定 GPL／LGPL 依賴要開源還是替換。</t>
+        </is>
+      </c>
+      <c r="D79" s="11" t="n"/>
+      <c r="E79" s="11" t="n"/>
+      <c r="F79" s="11" t="n"/>
+      <c r="G79" s="11" t="n"/>
+      <c r="H79" s="11" t="n"/>
+      <c r="I79" s="12" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="10" t="inlineStr">
+        <is>
           <t>說明</t>
-        </is>
-      </c>
-    </row>
-    <row r="78" ht="32" customHeight="1">
-      <c r="A78" s="14" t="inlineStr">
-        <is>
-          <t>・狀態：未開始 → 進行中 → 已完成。只有測試真的跑過而且通過才算已完成；阻塞要在備註寫原因；不再需要的任務標不適用，不要刪。</t>
-        </is>
-      </c>
-    </row>
-    <row r="79" ht="18" customHeight="1">
-      <c r="A79" s="14" t="inlineStr">
-        <is>
-          <t>・測試結果：未測試 / 通過 / 失敗 / 部分通過。測試證據寫跑了什麼、看到什麼，完整歷史在「更新記錄」。</t>
-        </is>
-      </c>
-    </row>
-    <row r="80" ht="18" customHeight="1">
-      <c r="A80" s="14" t="inlineStr">
-        <is>
-          <t>・「接下來」按階段排序，同一階段內再按優先級；依賴還沒滿足的任務不會出現在「接下來」。</t>
-        </is>
-      </c>
-    </row>
-    <row r="81" ht="18" customHeight="1">
-      <c r="A81" s="14" t="inlineStr">
-        <is>
-          <t>・可以手動改：「任務清單」的狀態、測試結果、測試證據、Commit、備註，以及「待確認問題」的回答。其餘欄位和本頁由腳本維護。</t>
         </is>
       </c>
     </row>
     <row r="82" ht="32" customHeight="1">
       <c r="A82" s="14" t="inlineStr">
         <is>
+          <t>・狀態：未開始 → 進行中 → 已完成。只有測試真的跑過而且通過才算已完成；阻塞要在備註寫原因；不再需要的任務標不適用，不要刪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="18" customHeight="1">
+      <c r="A83" s="14" t="inlineStr">
+        <is>
+          <t>・測試結果：未測試 / 通過 / 失敗 / 部分通過。測試證據寫跑了什麼、看到什麼，完整歷史在「更新記錄」。</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="18" customHeight="1">
+      <c r="A84" s="14" t="inlineStr">
+        <is>
+          <t>・「接下來」按階段排序，同一階段內再按優先級；依賴還沒滿足的任務不會出現在「接下來」。</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="18" customHeight="1">
+      <c r="A85" s="14" t="inlineStr">
+        <is>
+          <t>・可以手動改：「任務清單」的狀態、測試結果、測試證據、Commit、備註，以及「待確認問題」的回答。其餘欄位和本頁由腳本維護。</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="32" customHeight="1">
+      <c r="A86" s="14" t="inlineStr">
+        <is>
           <t>・建議用法：在 Claude Code 對 Claude 說「P0-02 做完了」或輸入 /prod-readiness。Claude 會先跑測試再更新，並寫進「更新記錄」。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="63">
+  <mergeCells count="67">
     <mergeCell ref="E21:I21"/>
     <mergeCell ref="C61:I61"/>
-    <mergeCell ref="C52:I52"/>
+    <mergeCell ref="E50:I50"/>
     <mergeCell ref="C70:I70"/>
+    <mergeCell ref="A84:I84"/>
     <mergeCell ref="E24:I24"/>
     <mergeCell ref="E42:I42"/>
-    <mergeCell ref="A80:I80"/>
     <mergeCell ref="E33:I33"/>
     <mergeCell ref="A3:I3"/>
     <mergeCell ref="E23:I23"/>
+    <mergeCell ref="C72:I72"/>
     <mergeCell ref="E39:I39"/>
     <mergeCell ref="C67:I67"/>
     <mergeCell ref="E48:I48"/>
     <mergeCell ref="C57:I57"/>
+    <mergeCell ref="A86:I86"/>
     <mergeCell ref="C53:I53"/>
     <mergeCell ref="C66:I66"/>
     <mergeCell ref="A2:I2"/>
@@ -2645,19 +2747,24 @@
     <mergeCell ref="E20:I20"/>
     <mergeCell ref="E38:I38"/>
     <mergeCell ref="C69:I69"/>
+    <mergeCell ref="C78:I78"/>
+    <mergeCell ref="A85:I85"/>
     <mergeCell ref="E28:I28"/>
     <mergeCell ref="C62:I62"/>
     <mergeCell ref="C68:I68"/>
     <mergeCell ref="E31:I31"/>
     <mergeCell ref="E40:I40"/>
     <mergeCell ref="C58:I58"/>
+    <mergeCell ref="A52:I52"/>
     <mergeCell ref="E30:I30"/>
     <mergeCell ref="A81:I81"/>
     <mergeCell ref="E34:I34"/>
     <mergeCell ref="A19:I19"/>
     <mergeCell ref="C74:I74"/>
     <mergeCell ref="C64:I64"/>
+    <mergeCell ref="C79:I79"/>
     <mergeCell ref="E46:I46"/>
+    <mergeCell ref="C73:I73"/>
     <mergeCell ref="A44:I44"/>
     <mergeCell ref="E49:I49"/>
     <mergeCell ref="E27:I27"/>
@@ -2665,26 +2772,23 @@
     <mergeCell ref="C54:I54"/>
     <mergeCell ref="A77:I77"/>
     <mergeCell ref="E36:I36"/>
+    <mergeCell ref="A83:I83"/>
     <mergeCell ref="C63:I63"/>
     <mergeCell ref="C65:I65"/>
     <mergeCell ref="E26:I26"/>
     <mergeCell ref="C55:I55"/>
     <mergeCell ref="A82:I82"/>
     <mergeCell ref="C75:I75"/>
-    <mergeCell ref="A73:I73"/>
-    <mergeCell ref="A51:I51"/>
     <mergeCell ref="C56:I56"/>
     <mergeCell ref="E32:I32"/>
     <mergeCell ref="E25:I25"/>
     <mergeCell ref="C59:I59"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="E41:I41"/>
-    <mergeCell ref="A79:I79"/>
     <mergeCell ref="E37:I37"/>
     <mergeCell ref="C60:I60"/>
     <mergeCell ref="E22:I22"/>
     <mergeCell ref="E47:I47"/>
-    <mergeCell ref="A78:I78"/>
     <mergeCell ref="C71:I71"/>
   </mergeCells>
   <conditionalFormatting sqref="I6:I10">
@@ -2715,7 +2819,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P57"/>
+  <dimension ref="A1:P62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3756,7 +3860,7 @@
       </c>
       <c r="F14" s="13" t="inlineStr">
         <is>
-          <t>進行中</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="G14" s="13" t="inlineStr">
@@ -3764,7 +3868,11 @@
           <t>通過</t>
         </is>
       </c>
-      <c r="H14" s="13" t="n"/>
+      <c r="H14" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
       <c r="I14" s="6" t="inlineStr">
         <is>
           <t>OTA 的韌體 URL 與伺服器證書仍是佔位符：出貨後無法修補任何漏洞。</t>
@@ -3789,12 +3897,12 @@
       <c r="M14" s="13" t="n"/>
       <c r="N14" s="6" t="inlineStr">
         <is>
-          <t>實機開發板 63:64（localall，本機後端）：① 1.1.0→1.2.1 OTA 下載 14s、sha256 過、重啟到 app1 試用、連上語音伺服器後穩定 120s 才 confirmed、開場白播完、devices 記 1.2.1 ② 推開機 3s 崩潰的 1.2.2：安裝→崩潰→bootloader 1s 內回到 1.2.1『rolled back from 1.2.2』→上報 ota_failed_version=1.2.2→再重啟不再下載。過程中測出並修好 2 個 bug：收到 auth 即確認太早（1.0.2 確認後崩潰循環，887b769 改為穩定 2 分鐘）；millis()|1 計時繞回導致誤回滾（3a874dd）。API 16/16，pio 全 env 通過</t>
+          <t>生產雲端 HTTPS OTA（2026-10-09）：release_firmware.py publish spotpear-ai-toy --current → 1.0.1 現行；42:34 開機 1.0.0 → token 回應 Installing 1.0.1 (1655776 bytes) → 經 Cloudflare+nginx 下載 100% → 重啟到 app1 on probation → 連上語音伺服器 → 120s 後『Firmware 1.0.1 confirmed』。②崩潰回滾沿用 10-08 開發板實測（1.2.2/1.5.3 回滾、1.5.2 切回舊槽）；本機 63:64 1.5.1→1.6.1 亦確認</t>
         </is>
       </c>
       <c r="O14" s="13" t="inlineStr">
         <is>
-          <t>682f3b4</t>
+          <t>036c0f9</t>
         </is>
       </c>
       <c r="P14" s="6" t="inlineStr">
@@ -3802,7 +3910,8 @@
           <t>[2026-10-08] 2026-10-08 b27cc07（分支 p0-13-ota）。部署時要套 20261008100000_firmware_releases.sql，發佈要用 SUPABASE_URL+service key 跑 tools/release_firmware.py
 [2026-10-08] 2026-10-08 實機①②通過，未部署。上線要：套 20261008100000、部署前端、用 release_firmware.py 發佈正式 build；生產 HTTPS（同 CF CA）的 1.6MB 下載尚未在線上驗證。開發板現跑 1.2.1 localall。未做：已確認版本日後若崩潰循環不會自動切回舊槽，需 USB 救（可另立任務）
 [2026-10-08] 2026-10-08 OTA 檢查併入 /api/generate_auth_token（68b9550），開機回到一次 TLS 握手；/api/ota/check 移除。token 路徑 API 11/11（舊韌體無 ota、格式錯仍發 token、回滾版本不再提供）；實機 1.3.0→1.3.1 經 token 回應安裝、試用、播完開場白、120s 確認。第一次升級 1.3.1 被 async_tcp 任務看門狗觸發重啟並正確回滾——是既有韌體 bug，見新任務
-[2026-10-08] 2026-10-08 交板前強化（682f3b4）：① 確認後連續崩潰 3 次 → 切回另一槽位（每段崩潰期一次）、立即重新確認、上報失敗 ② 回滾按重啟原因判定：崩潰/看門狗即失敗，斷電等非崩潰原因可重試 2 次（R-17 會自己斷電）。實機 1.5.x：試用期內 EN 重啟 → 重試第 2 次並確認；1.5.2 確認後崩潰 3 次 → 回 1.5.1、重新確認、報失敗；1.5.3 試用期崩潰 → 回滾、reason 4 即報失敗。runbook 已加 20261008100000 與 OTA 檢查（3aa632a）。上線後須用開發板對雲端走一次 HTTPS OTA 再交板</t>
+[2026-10-08] 2026-10-08 交板前強化（682f3b4）：① 確認後連續崩潰 3 次 → 切回另一槽位（每段崩潰期一次）、立即重新確認、上報失敗 ② 回滾按重啟原因判定：崩潰/看門狗即失敗，斷電等非崩潰原因可重試 2 次（R-17 會自己斷電）。實機 1.5.x：試用期內 EN 重啟 → 重試第 2 次並確認；1.5.2 確認後崩潰 3 次 → 回 1.5.1、重新確認、報失敗；1.5.3 試用期崩潰 → 回滾、reason 4 即報失敗。runbook 已加 20261008100000 與 OTA 檢查（3aa632a）。上線後須用開發板對雲端走一次 HTTPS OTA 再交板
+[2026-10-09] 2026-10-09 上線前兩個阻礙已修：① Cloudflare 對 Python-urllib UA 回 403 error 1010 → release_firmware.py 自帶 User-Agent（036c0f9）② 主機 nginx /supabase-api/ 預設 1MB 上限 → 413，已在 /home/jackylee/nginx/conf.d/elatoai.conf 兩段 location 加 client_max_body_size 16m（備份 ~/nginx/elatoai.conf.2026-10-09.bak）。雲端此前沒有任何 Spotpear release。service key 只在伺服器 .env.production</t>
         </is>
       </c>
     </row>
@@ -4013,7 +4122,7 @@
       <c r="O17" s="13" t="n"/>
       <c r="P17" s="6" t="n"/>
     </row>
-    <row r="18" ht="32" customHeight="1">
+    <row r="18" ht="158" customHeight="1">
       <c r="A18" s="13" t="inlineStr">
         <is>
           <t>P1-03</t>
@@ -4074,7 +4183,12 @@
       <c r="M18" s="13" t="n"/>
       <c r="N18" s="6" t="n"/>
       <c r="O18" s="13" t="n"/>
-      <c r="P18" s="6" t="n"/>
+      <c r="P18" s="6" t="inlineStr">
+        <is>
+          <t>[2026-10-09] 解綁時選擇保留的記憶（P1-12）沒有設備綁定，也要納入保留期限，例如帳號沒有設備且 12 個月沒活動就清除。
+[2026-10-09] 補充（2026-10-09 晚）：記憶改成跟設備後，解綁時保留的記憶掛在已解綁的設備名下，家長在設定頁看不到也清不了；還有 device_id 為 NULL 的舊記憶（沒有設備的帳號）。兩者都要納入保留期限自動清理。</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="32" customHeight="1">
       <c r="A19" s="13" t="inlineStr">
@@ -5413,7 +5527,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="46" customHeight="1">
+    <row r="38" ht="116" customHeight="1">
       <c r="A38" s="13" t="inlineStr">
         <is>
           <t>R-06</t>
@@ -5478,7 +5592,11 @@
       </c>
       <c r="N38" s="6" t="n"/>
       <c r="O38" s="13" t="n"/>
-      <c r="P38" s="6" t="n"/>
+      <c r="P38" s="6" t="inlineStr">
+        <is>
+          <t>[2026-10-09] 2026-10-09 配網熱點由所有板同名的 ELATO-DEVICE 改為 AIBuddy-XXXX（STA MAC 尾 4 位，22ce0ae），App 的「找不到設備」提示同步改；雲端 1.0.1 已 OTA 推出。62:70 用手機連 AIBuddy-6270 配網成功。家長自助流程本身仍未找非團隊成員測試</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="102" customHeight="1">
       <c r="A39" s="13" t="inlineStr">
@@ -5751,14 +5869,14 @@
       </c>
       <c r="M42" s="13" t="inlineStr">
         <is>
-          <t>P0-06, P0-14, R-01</t>
+          <t>P0-06, P0-14, R-01, P2-12</t>
         </is>
       </c>
       <c r="N42" s="6" t="n"/>
       <c r="O42" s="13" t="n"/>
       <c r="P42" s="6" t="n"/>
     </row>
-    <row r="43" ht="46" customHeight="1">
+    <row r="43" ht="186" customHeight="1">
       <c r="A43" s="13" t="inlineStr">
         <is>
           <t>R-11</t>
@@ -5820,7 +5938,9 @@
       <c r="O43" s="13" t="n"/>
       <c r="P43" s="6" t="inlineStr">
         <is>
-          <t>[2026-09-30] v1 沒有客服角色，售後工具由超級管理員使用（Q9）</t>
+          <t>[2026-09-30] v1 沒有客服角色，售後工具由超級管理員使用（Q9）
+[2026-10-09] 換機時記憶不用搬：記憶跟帳號，同一帳號認領新設備就會繼續（P1-12 TC4）。
+[2026-10-09] 更正（2026-10-09 晚）：記憶改成跟設備（P1-12），換新設備會從空白開始。換機流程要加「把舊設備的記憶搬到新設備」：把 memory_facts、memory_segments、conversations 的 device_id 從舊機改成新機（同一 user_id），並由超級管理員執行。</t>
         </is>
       </c>
     </row>
@@ -6830,8 +6950,360 @@
         </is>
       </c>
     </row>
+    <row r="58" ht="60" customHeight="1">
+      <c r="A58" s="13" t="inlineStr">
+        <is>
+          <t>R-18</t>
+        </is>
+      </c>
+      <c r="B58" s="13" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="C58" s="13" t="inlineStr">
+        <is>
+          <t>2 內測準備</t>
+        </is>
+      </c>
+      <c r="D58" s="6" t="inlineStr">
+        <is>
+          <t>體驗</t>
+        </is>
+      </c>
+      <c r="E58" s="6" t="inlineStr">
+        <is>
+          <t>長按 BOOT 重新配網（開 AIBuddy-XXXX 熱點）</t>
+        </is>
+      </c>
+      <c r="F58" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="G58" s="13" t="inlineStr">
+        <is>
+          <t>未測試</t>
+        </is>
+      </c>
+      <c r="I58" s="6" t="inlineStr">
+        <is>
+          <t>Spotpear 只有 BOOT 一個鍵，韌體沒有重新配網的操作：舊 WiFi 仍在範圍內時，家長換路由器或改密碼後無法讓設備重新開熱點，只能用瀏覽器開 http://&lt;設備IP&gt;/wifi 或恢復出廠</t>
+        </is>
+      </c>
+      <c r="J58" s="6" t="inlineStr">
+        <is>
+          <t>firmware-arduino/src/main.cpp（按鍵處理、setupWiFi）；src/WifiManager.cpp runSoftAP()</t>
+        </is>
+      </c>
+      <c r="K58" s="6" t="inlineStr">
+        <is>
+          <t>長按 BOOT ≥5 秒：燈號提示、開出 AIBuddy-XXXX 熱點並保留已存 WiFi 直到新設定保存；短按行為不變；設備密鑰與綁定不受影響；隨 OTA 推出</t>
+        </is>
+      </c>
+      <c r="L58" s="6" t="inlineStr">
+        <is>
+          <t>Spotpear 實機：已連 WiFi 時長按 5 秒 → 手機見到 AIBuddy-XXXX → 配新 WiFi → 連上並能對話；長按 3 秒不觸發；配網中途放棄 → 120 秒後回到舊 WiFi；雲端 token 照常（不需重新綁定）</t>
+        </is>
+      </c>
+      <c r="M58" s="13" t="inlineStr">
+        <is>
+          <t>R-01</t>
+        </is>
+      </c>
+      <c r="P58" s="6" t="inlineStr">
+        <is>
+          <t>[2026-10-09] 新增</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="60" customHeight="1">
+      <c r="A59" s="13" t="inlineStr">
+        <is>
+          <t>P2-12</t>
+        </is>
+      </c>
+      <c r="B59" s="13" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C59" s="13" t="inlineStr">
+        <is>
+          <t>3 封閉內測</t>
+        </is>
+      </c>
+      <c r="D59" s="6" t="inlineStr">
+        <is>
+          <t>韌體</t>
+        </is>
+      </c>
+      <c r="E59" s="6" t="inlineStr">
+        <is>
+          <t>量產燒錄前加大 app 分區</t>
+        </is>
+      </c>
+      <c r="F59" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="G59" s="13" t="inlineStr">
+        <is>
+          <t>未測試</t>
+        </is>
+      </c>
+      <c r="I59" s="6" t="inlineStr">
+        <is>
+          <t>app0/app1 各 2MB，1.0.1 已用 1.66MB（約 79%，剩約 400KB）；分區表 OTA 改不了，韌體超過 2MB 後所有已出貨設備無法再 OTA。板上有 16MB flash，現分區只用約 7MB</t>
+        </is>
+      </c>
+      <c r="J59" s="6" t="inlineStr">
+        <is>
+          <t>firmware-arduino/partition.csv；R-10 出廠腳本</t>
+        </is>
+      </c>
+      <c r="K59" s="6" t="inlineStr">
+        <is>
+          <t>新分區表（例如 app0/app1 各 4MB，保留 nvs/otadata 位置）在出廠前定案並寫入出廠腳本；OTA 與回滾在新分區表上照常</t>
+        </is>
+      </c>
+      <c r="L59" s="6" t="inlineStr">
+        <is>
+          <t>用新分區表 USB 燒 Spotpear → 雲端 OTA 一次並確認 → 推崩潰版確認回滾；pio 全 env 編譯通過；release_firmware.py 發佈的映像大小 &lt; 新分區</t>
+        </is>
+      </c>
+      <c r="M59" s="13" t="n"/>
+      <c r="P59" s="6" t="inlineStr">
+        <is>
+          <t>[2026-10-09] 新增</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="74" customHeight="1">
+      <c r="A60" s="13" t="inlineStr">
+        <is>
+          <t>R-19</t>
+        </is>
+      </c>
+      <c r="B60" s="13" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="C60" s="13" t="inlineStr">
+        <is>
+          <t>2 內測準備</t>
+        </is>
+      </c>
+      <c r="D60" s="6" t="inlineStr">
+        <is>
+          <t>硬件</t>
+        </is>
+      </c>
+      <c r="E60" s="6" t="inlineStr">
+        <is>
+          <t>外接按鈕：量產板加 I2C 擴展晶片（TCA9555）</t>
+        </is>
+      </c>
+      <c r="F60" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="G60" s="13" t="inlineStr">
+        <is>
+          <t>未測試</t>
+        </is>
+      </c>
+      <c r="I60" s="6" t="inlineStr">
+        <is>
+          <t>後續要外接按鈕，但 Spotpear C3 已無空閒 GPIO（0 電壓檢測、1/20/21 屏幕、2 LED、3/4 I2C、5–8/10 I2S、9 BOOT、11 功放）；硬件出貨後 OTA 補不了，GPIO2/8/9 為開機模式腳不宜接按鈕。用戶不焊接，需 Spotpear 改板</t>
+        </is>
+      </c>
+      <c r="J60" s="6" t="inlineStr">
+        <is>
+          <t>Spotpear 改板（與 R-16 同一封詢問）；firmware-arduino/src/IoExpander.*、BoardConfig.h（Waveshare 已有 TCA9555 讀鍵程式）</t>
+        </is>
+      </c>
+      <c r="K60" s="6" t="inlineStr">
+        <is>
+          <t>確定按鈕數量與用途；Spotpear 量產版在 I2C（SDA3/SCL4）加 TCA9555 與按鈕接口並給出報價交期；韌體在 Spotpear 上經擴展晶片讀鍵，按鍵功能之後可經 OTA 調整</t>
+        </is>
+      </c>
+      <c r="L60" s="6" t="inlineStr">
+        <is>
+          <t>樣板：I2C 掃描見 0x18 與擴展晶片地址；每個按鈕短按/長按都在 log 出現且觸發對應功能；按住任一按鈕上電仍正常開機；連續對話 30 分鐘音訊無雜音</t>
+        </is>
+      </c>
+      <c r="M60" s="13" t="inlineStr">
+        <is>
+          <t>R-01</t>
+        </is>
+      </c>
+      <c r="P60" s="6" t="inlineStr">
+        <is>
+          <t>[2026-10-09] 新增</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="409" customHeight="1">
+      <c r="A61" s="13" t="inlineStr">
+        <is>
+          <t>P1-12</t>
+        </is>
+      </c>
+      <c r="B61" s="13" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C61" s="13" t="inlineStr">
+        <is>
+          <t>2 內測準備</t>
+        </is>
+      </c>
+      <c r="D61" s="6" t="inlineStr">
+        <is>
+          <t>私隱</t>
+        </is>
+      </c>
+      <c r="E61" s="6" t="inlineStr">
+        <is>
+          <t>設備解綁時的記憶處理：確認、預設保留、可選清除</t>
+        </is>
+      </c>
+      <c r="F61" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="G61" s="13" t="inlineStr">
+        <is>
+          <t>部分通過</t>
+        </is>
+      </c>
+      <c r="I61" s="6" t="inlineStr">
+        <is>
+          <t>解綁一按即生效，沒有確認；記憶在解綁時怎麼處理也沒有定義。家長排除故障時重綁可能誤刪孩子的記憶，想刪時又刪不乾淨（設定頁「清除全部」只刪 memory_facts／memory_segments，conversations 原始對話仍在）。</t>
+        </is>
+      </c>
+      <c r="J61" s="6" t="inlineStr">
+        <is>
+          <t>frontend-nextjs/app/components/Settings/AppSettings.tsx（handleUnbind）、app/actions.ts（unbindDeviceAction）、db/devices.ts（unbindDevice）、Settings/MemorySection.tsx 與 db/memories.ts（清除全部）、server/fastapi/memory/session.py（session 結束時的 consolidation）</t>
+        </is>
+      </c>
+      <c r="K61" s="6" t="inlineStr">
+        <is>
+          <t>① 按「解綁」先彈出確認對話框，取消則什麼都不改。② 對話框預設保留記憶；「同時清除記憶」要主動勾選，並寫明無法復原。③ 記憶跟設備：鍵是 (user_id, device_id, ip_key)。同一帳號的每台設備各自一份記憶；保留時，同帳號重綁同一台會接著用；換新設備從空白開始（搬記憶交給 R-11）。④ 清除在伺服器端一個交易完成：先刪該設備的 memory_facts、memory_segments、conversations（連帳號的舊 memories），再解綁；任何一步失敗就不解綁，並顯示錯誤。⑤ 其他帳號認領同一台設備，看不到舊記憶（靠 user_id 隔離，不靠刪除成功）。⑥ 設定頁按設備顯示記憶；「清除全部」只清所選設備，連 conversations 一起刪。⑦ 對話中清除，之後的寫入和 consolidation 不會把記憶寫回（devices.memories_revision + trigger）。⑧ 未認領的設備不能對話：/ws/esp32 查到設備沒有 user_id 就在 auth 前以 4401 關閉，即使 24 小時 token 未過期；韌體重新取 token 拿到 202，回到配對狀態。⑨ 解綁時立即中斷該設備正在進行的語音 session。⑩ 網頁語音（playground）沒有設備，不讀也不寫記憶。</t>
+        </is>
+      </c>
+      <c r="L61" s="6" t="inlineStr">
+        <is>
+          <t>TC1 取消：點解綁 → 對話框 → 取消 → devices.user_id 不變。
+TC2 預設保留：記下該設備 memory_facts／memory_segments／conversations 行數 → 不勾清除並解綁 → 行數不變。
+TC3 同機重綁：接 TC2，A 重新認領同一台 → 開始對話時 log『Loaded N fact(s)』的 N 等於解綁前；問玩具解綁前講過的事（例如寵物名），能答對。
+TC4 換機／多設備：A 認領第二台設備 → 第二台開始對話時是空白（starts cold），第一台的記憶不受影響；設定頁可切換兩台，各自顯示自己的記憶。
+TC5 轉讓隔離：A 解綁（保留）→ B 認領同一台 → B 的 session 載入 0 facts；用 B 的登入 token 查三張表拿不到 A 的行；A 的行仍在。
+TC6 勾選清除：A 勾選清除並解綁 → 該設備四張表都是 0 行；重綁後開始對話是空白。
+TC7 清除失敗不解綁：讓刪除報錯（例如暫時撤銷 service_role 對 conversations 的 DELETE）→ 介面顯示錯誤，devices.user_id 和 memories_revision 不變，記憶行數不變。
+TC8 設定頁清除全部：按「Clear all」→ 所選設備的四張表都是 0 行，代數遞增，設備仍綁定。
+TC9 越權：B 呼叫 unbind_device／clear_device_memory 對 A 的設備 → 回傳 NULL／報錯；A 的設備和記憶不受影響；anon、authenticated 沒有 EXECUTE 權限。
+TC10 對話中清除：玩具對話中勾選清除並解綁 → 對話被中斷 → 等 consolidation 跑完仍是 0 行；用 store 以舊代數寫入三張表 → 全部被資料庫拒絕（HTTP 400 P0001）。
+TC11 回歸：pytest server/fastapi/tests 全過；正常對話記憶照常寫入和載入。
+TC12 解綁後不重開機不能對話：設備手上有未過期的 token → 解綁 → 再連 /ws/esp32 → auth 前被 4401 拒絕；真機：串口顯示重新取 token 得到 202，回到配對狀態。
+TC13 對話中解綁立即中斷：對話中解綁（保留）→ 數秒內 websocket 被關閉（4001），記憶行數不變。
+TC14 網頁語音不開記憶：在 playground 對話 → 伺服器 log 顯示 No device … running without memory，三張表沒有新行。</t>
+        </is>
+      </c>
+      <c r="M61" s="13" t="n"/>
+      <c r="N61" s="6" t="inlineStr">
+        <is>
+          <t>本機（開發板 DEV636 身份的模擬裝置 + 網頁）：TC1/2/5/6/7/8/10/11/13 通過；TC3 重綁後 log『Loaded 2 fact(s)』；TC4 第二台 starts cold、設定頁可切換；TC9 DB 層 B 解綁回 NULL、清除報錯，anon/authenticated 無 EXECUTE；TC10 舊代數寫入三表皆 HTTP 400、清除後 40 秒仍 0 行；TC12 伺服器端 4401 通過；pytest 214 passed。未做：TC12 真機 202/配對、TC3 真機問答、TC14 網頁語音。</t>
+        </is>
+      </c>
+      <c r="O61" s="13" t="inlineStr">
+        <is>
+          <t>98faef9</t>
+        </is>
+      </c>
+      <c r="P61" s="6" t="inlineStr">
+        <is>
+          <t>[2026-10-09] 新增：決定（2026-10-09）：記憶跟帳號，不跟 device_id。目前一個帳號只有一個孩子、一台設備，user_id 就是孩子；以後支援一個家長多個孩子時，再加 child_profiles，devices.child_id 指向孩子，記憶鍵改 (child_id, ip_key)，一對一回填。解綁時保留下來的記憶，由 P1-03 的保留期限兜底清理。
+[2026-10-09] 補充 ⑧⑨ 和 TC12、TC13（2026-10-09）：現在 /ws/esp32 只驗 token 簽名，不查是否已認領；token 存在玩具 RAM 裡 24 小時不會重新檢查，所以解綁後不重開機仍能以預設角色、無記憶對話。要改 server/fastapi/server.py（/ws/esp32 與解綁時斷線）和 unbindDeviceAction（通知語音伺服器）。本機開發模式（NEXT_PUBLIC_SKIP_DEVICE_REGISTRATION=True）允許未認領設備對話，⑧ 要對這個模式保留同樣的例外。
+[2026-10-09] 決定改變（2026-10-09 晚）：用戶決定記憶跟設備，不跟帳號（一個帳號可綁多台，多數是一個孩子一台）。網頁語音不開記憶；舊資料歸到帳號最早認領的設備。分支 p1-12-unbind-memory（建在 multi-device-binding 9c8e106 上），commit 8bb9fb8 + 98faef9，未 push、未部署。</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="74" customHeight="1">
+      <c r="A62" s="13" t="inlineStr">
+        <is>
+          <t>R-20</t>
+        </is>
+      </c>
+      <c r="B62" s="13" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="C62" s="13" t="inlineStr">
+        <is>
+          <t>2 內測準備</t>
+        </is>
+      </c>
+      <c r="D62" s="6" t="inlineStr">
+        <is>
+          <t>產品</t>
+        </is>
+      </c>
+      <c r="E62" s="6" t="inlineStr">
+        <is>
+          <t>孩子資料與角色改成每台設備一份</t>
+        </is>
+      </c>
+      <c r="F62" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="G62" s="13" t="inlineStr">
+        <is>
+          <t>未測試</t>
+        </is>
+      </c>
+      <c r="I62" s="6" t="inlineStr">
+        <is>
+          <t>記憶已改成每台設備一份（P1-12），但孩子的名字、年齡、性格，以及角色，仍是每個帳號一份（users.supervisee_*、users.personality_id）。兄弟姊妹各一隻玩具時，其中一隻會叫錯名字、用錯年齡。</t>
+        </is>
+      </c>
+      <c r="J62" s="6" t="inlineStr">
+        <is>
+          <t>users.supervisee_name／supervisee_age／supervisee_persona／personality_id、server/fastapi/device_registry.py（_ACCOUNT_SELECT）、frontend-nextjs 設定頁的 My Info 與角色選擇</t>
+        </is>
+      </c>
+      <c r="K62" s="6" t="inlineStr">
+        <is>
+          <t>每台設備可以設定自己的孩子名字、年齡、性格和角色；沒設定時沿用帳號的預設值。語音伺服器按設備讀取。設定頁每台設備各自編輯。</t>
+        </is>
+      </c>
+      <c r="L62" s="6" t="inlineStr">
+        <is>
+          <t>① 帳號綁兩台設備，分別設孩子 A／B → 兩台開場時分別叫 A 和 B。② 只設一台時，另一台沿用帳號預設。③ 換角色只影響所選設備。</t>
+        </is>
+      </c>
+      <c r="M62" s="13" t="inlineStr">
+        <is>
+          <t>P1-12</t>
+        </is>
+      </c>
+      <c r="P62" s="6" t="inlineStr">
+        <is>
+          <t>[2026-10-09] 新增：2026-10-09 實作 P1-12 時發現；beta 家庭若有兄弟姊妹各一隻，要在 R-07 前完成。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P57"/>
+  <autoFilter ref="A1:P62"/>
   <conditionalFormatting sqref="F2:F1000">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"已完成"</formula>
@@ -7294,7 +7766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I128"/>
+  <dimension ref="A1:I144"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -11823,8 +12295,544 @@
         </is>
       </c>
     </row>
+    <row r="129" ht="172" customHeight="1">
+      <c r="A129" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-09 14:42</t>
+        </is>
+      </c>
+      <c r="B129" s="13" t="inlineStr">
+        <is>
+          <t>P0-13</t>
+        </is>
+      </c>
+      <c r="C129" s="6" t="inlineStr">
+        <is>
+          <t>讓 OTA 真正可用並能回滾</t>
+        </is>
+      </c>
+      <c r="D129" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="E129" s="13" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="F129" s="13" t="inlineStr">
+        <is>
+          <t>通過</t>
+        </is>
+      </c>
+      <c r="G129" s="6" t="inlineStr">
+        <is>
+          <t>生產雲端 HTTPS OTA（2026-10-09）：release_firmware.py publish spotpear-ai-toy --current → 1.0.1 現行；42:34 開機 1.0.0 → token 回應 Installing 1.0.1 (1655776 bytes) → 經 Cloudflare+nginx 下載 100% → 重啟到 app1 on probation → 連上語音伺服器 → 120s 後『Firmware 1.0.1 confirmed』。②崩潰回滾沿用 10-08 開發板實測（1.2.2/1.5.3 回滾、1.5.2 切回舊槽）；本機 63:64 1.5.1→1.6.1 亦確認</t>
+        </is>
+      </c>
+      <c r="H129" s="13" t="inlineStr">
+        <is>
+          <t>036c0f9</t>
+        </is>
+      </c>
+      <c r="I129" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-09 上線前兩個阻礙已修：① Cloudflare 對 Python-urllib UA 回 403 error 1010 → release_firmware.py 自帶 User-Agent（036c0f9）② 主機 nginx /supabase-api/ 預設 1MB 上限 → 413，已在 /home/jackylee/nginx/conf.d/elatoai.conf 兩段 location 加 client_max_body_size 16m（備份 ~/nginx/elatoai.conf.2026-10-09.bak）。雲端此前沒有任何 Spotpear release。service key 只在伺服器 .env.production</t>
+        </is>
+      </c>
+    </row>
+    <row r="130" ht="102" customHeight="1">
+      <c r="A130" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-09 16:03</t>
+        </is>
+      </c>
+      <c r="B130" s="13" t="inlineStr">
+        <is>
+          <t>R-06</t>
+        </is>
+      </c>
+      <c r="C130" s="6" t="inlineStr">
+        <is>
+          <t>家長自助上手流程</t>
+        </is>
+      </c>
+      <c r="D130" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E130" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="F130" s="13" t="n"/>
+      <c r="G130" s="6" t="n"/>
+      <c r="H130" s="13" t="n"/>
+      <c r="I130" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-09 配網熱點由所有板同名的 ELATO-DEVICE 改為 AIBuddy-XXXX（STA MAC 尾 4 位，22ce0ae），App 的「找不到設備」提示同步改；雲端 1.0.1 已 OTA 推出。62:70 用手機連 AIBuddy-6270 配網成功。家長自助流程本身仍未找非團隊成員測試</t>
+        </is>
+      </c>
+    </row>
+    <row r="131" ht="32" customHeight="1">
+      <c r="A131" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-09 16:03</t>
+        </is>
+      </c>
+      <c r="B131" s="13" t="inlineStr">
+        <is>
+          <t>R-18</t>
+        </is>
+      </c>
+      <c r="C131" s="6" t="inlineStr">
+        <is>
+          <t>長按 BOOT 重新配網（開 AIBuddy-XXXX 熱點）</t>
+        </is>
+      </c>
+      <c r="E131" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="I131" s="6" t="inlineStr">
+        <is>
+          <t>新增任務</t>
+        </is>
+      </c>
+    </row>
+    <row r="132" ht="32" customHeight="1">
+      <c r="A132" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-09 16:03</t>
+        </is>
+      </c>
+      <c r="B132" s="13" t="inlineStr">
+        <is>
+          <t>P2-12</t>
+        </is>
+      </c>
+      <c r="C132" s="6" t="inlineStr">
+        <is>
+          <t>量產燒錄前加大 app 分區</t>
+        </is>
+      </c>
+      <c r="E132" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="I132" s="6" t="inlineStr">
+        <is>
+          <t>新增任務</t>
+        </is>
+      </c>
+    </row>
+    <row r="133" ht="32" customHeight="1">
+      <c r="A133" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-09 16:03</t>
+        </is>
+      </c>
+      <c r="B133" s="13" t="inlineStr">
+        <is>
+          <t>R-19</t>
+        </is>
+      </c>
+      <c r="C133" s="6" t="inlineStr">
+        <is>
+          <t>外接按鈕：量產板加 I2C 擴展晶片（TCA9555）</t>
+        </is>
+      </c>
+      <c r="E133" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="I133" s="6" t="inlineStr">
+        <is>
+          <t>新增任務</t>
+        </is>
+      </c>
+    </row>
+    <row r="134" ht="32" customHeight="1">
+      <c r="A134" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-09 16:03</t>
+        </is>
+      </c>
+      <c r="B134" s="13" t="inlineStr">
+        <is>
+          <t>R-10</t>
+        </is>
+      </c>
+      <c r="C134" s="6" t="inlineStr">
+        <is>
+          <t>出廠流程</t>
+        </is>
+      </c>
+      <c r="D134" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E134" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="F134" s="13" t="n"/>
+      <c r="G134" s="6" t="n"/>
+      <c r="H134" s="13" t="n"/>
+      <c r="I134" s="6" t="inlineStr">
+        <is>
+          <t>修改了依賴→P0-06, P0-14, R-01, P2-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="135" ht="32" customHeight="1">
+      <c r="A135" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-09 20:46</t>
+        </is>
+      </c>
+      <c r="B135" s="13" t="inlineStr">
+        <is>
+          <t>P1-12</t>
+        </is>
+      </c>
+      <c r="C135" s="6" t="inlineStr">
+        <is>
+          <t>設備解綁時的記憶處理：確認、預設保留、可選清除</t>
+        </is>
+      </c>
+      <c r="E135" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="I135" s="6" t="inlineStr">
+        <is>
+          <t>新增任務</t>
+        </is>
+      </c>
+    </row>
+    <row r="136" ht="46" customHeight="1">
+      <c r="A136" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-09 20:46</t>
+        </is>
+      </c>
+      <c r="B136" s="13" t="inlineStr">
+        <is>
+          <t>P1-03</t>
+        </is>
+      </c>
+      <c r="C136" s="6" t="inlineStr">
+        <is>
+          <t>資料保留期限與自動清理</t>
+        </is>
+      </c>
+      <c r="D136" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E136" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="F136" s="13" t="n"/>
+      <c r="G136" s="6" t="n"/>
+      <c r="H136" s="13" t="n"/>
+      <c r="I136" s="6" t="inlineStr">
+        <is>
+          <t>解綁時選擇保留的記憶（P1-12）沒有設備綁定，也要納入保留期限，例如帳號沒有設備且 12 個月沒活動就清除。</t>
+        </is>
+      </c>
+    </row>
+    <row r="137" ht="46" customHeight="1">
+      <c r="A137" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-09 20:46</t>
+        </is>
+      </c>
+      <c r="B137" s="13" t="inlineStr">
+        <is>
+          <t>R-11</t>
+        </is>
+      </c>
+      <c r="C137" s="6" t="inlineStr">
+        <is>
+          <t>售後：客服、保修與換機</t>
+        </is>
+      </c>
+      <c r="D137" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E137" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="F137" s="13" t="n"/>
+      <c r="G137" s="6" t="n"/>
+      <c r="H137" s="13" t="n"/>
+      <c r="I137" s="6" t="inlineStr">
+        <is>
+          <t>換機時記憶不用搬：記憶跟帳號，同一帳號認領新設備就會繼續（P1-12 TC4）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="138" ht="172" customHeight="1">
+      <c r="A138" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-09 21:03</t>
+        </is>
+      </c>
+      <c r="B138" s="13" t="inlineStr">
+        <is>
+          <t>P1-12</t>
+        </is>
+      </c>
+      <c r="C138" s="6" t="inlineStr">
+        <is>
+          <t>設備解綁時的記憶處理：確認、預設保留、可選清除</t>
+        </is>
+      </c>
+      <c r="D138" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E138" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="F138" s="13" t="n"/>
+      <c r="G138" s="6" t="n"/>
+      <c r="H138" s="13" t="n"/>
+      <c r="I138" s="6" t="inlineStr">
+        <is>
+          <t>補充 ⑧⑨ 和 TC12、TC13（2026-10-09）：現在 /ws/esp32 只驗 token 簽名，不查是否已認領；token 存在玩具 RAM 裡 24 小時不會重新檢查，所以解綁後不重開機仍能以預設角色、無記憶對話。要改 server/fastapi/server.py（/ws/esp32 與解綁時斷線）和 unbindDeviceAction（通知語音伺服器）。本機開發模式（NEXT_PUBLIC_SKIP_DEVICE_REGISTRATION=True）允許未認領設備對話，⑧ 要對這個模式保留同樣的例外。；修改了驗收標準、測試方法</t>
+        </is>
+      </c>
+    </row>
+    <row r="139" ht="32" customHeight="1">
+      <c r="A139" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-09 21:04</t>
+        </is>
+      </c>
+      <c r="B139" s="13" t="inlineStr">
+        <is>
+          <t>P1-12</t>
+        </is>
+      </c>
+      <c r="C139" s="6" t="inlineStr">
+        <is>
+          <t>設備解綁時的記憶處理：確認、預設保留、可選清除</t>
+        </is>
+      </c>
+      <c r="D139" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E139" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F139" s="13" t="n"/>
+      <c r="G139" s="6" t="n"/>
+      <c r="H139" s="13" t="n"/>
+      <c r="I139" s="6" t="n"/>
+    </row>
+    <row r="140" ht="130" customHeight="1">
+      <c r="A140" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-09 21:53</t>
+        </is>
+      </c>
+      <c r="B140" s="13" t="inlineStr">
+        <is>
+          <t>P1-12</t>
+        </is>
+      </c>
+      <c r="C140" s="6" t="inlineStr">
+        <is>
+          <t>設備解綁時的記憶處理：確認、預設保留、可選清除</t>
+        </is>
+      </c>
+      <c r="D140" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="E140" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F140" s="13" t="n"/>
+      <c r="G140" s="6" t="n"/>
+      <c r="H140" s="13" t="n"/>
+      <c r="I140" s="6" t="inlineStr">
+        <is>
+          <t>決定改變（2026-10-09 晚）：用戶決定記憶跟設備，不跟帳號（一個帳號可綁多台，多數是一個孩子一台）。網頁語音不開記憶；舊資料歸到帳號最早認領的設備。分支 p1-12-unbind-memory（建在 multi-device-binding 9c8e106 上），commit 8bb9fb8 + 98faef9，未 push、未部署。；修改了驗收標準、測試方法</t>
+        </is>
+      </c>
+    </row>
+    <row r="141" ht="116" customHeight="1">
+      <c r="A141" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-09 21:53</t>
+        </is>
+      </c>
+      <c r="B141" s="13" t="inlineStr">
+        <is>
+          <t>P1-12</t>
+        </is>
+      </c>
+      <c r="C141" s="6" t="inlineStr">
+        <is>
+          <t>設備解綁時的記憶處理：確認、預設保留、可選清除</t>
+        </is>
+      </c>
+      <c r="D141" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="E141" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F141" s="13" t="inlineStr">
+        <is>
+          <t>部分通過</t>
+        </is>
+      </c>
+      <c r="G141" s="6" t="inlineStr">
+        <is>
+          <t>本機（開發板 DEV636 身份的模擬裝置 + 網頁）：TC1/2/5/6/7/8/10/11/13 通過；TC3 重綁後 log『Loaded 2 fact(s)』；TC4 第二台 starts cold、設定頁可切換；TC9 DB 層 B 解綁回 NULL、清除報錯，anon/authenticated 無 EXECUTE；TC10 舊代數寫入三表皆 HTTP 400、清除後 40 秒仍 0 行；TC12 伺服器端 4401 通過；pytest 214 passed。未做：TC12 真機 202/配對、TC3 真機問答、TC14 網頁語音。</t>
+        </is>
+      </c>
+      <c r="H141" s="13" t="inlineStr">
+        <is>
+          <t>98faef9</t>
+        </is>
+      </c>
+      <c r="I141" s="6" t="n"/>
+    </row>
+    <row r="142" ht="102" customHeight="1">
+      <c r="A142" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-09 21:54</t>
+        </is>
+      </c>
+      <c r="B142" s="13" t="inlineStr">
+        <is>
+          <t>R-11</t>
+        </is>
+      </c>
+      <c r="C142" s="6" t="inlineStr">
+        <is>
+          <t>售後：客服、保修與換機</t>
+        </is>
+      </c>
+      <c r="D142" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E142" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="F142" s="13" t="n"/>
+      <c r="G142" s="6" t="n"/>
+      <c r="H142" s="13" t="n"/>
+      <c r="I142" s="6" t="inlineStr">
+        <is>
+          <t>更正（2026-10-09 晚）：記憶改成跟設備（P1-12），換新設備會從空白開始。換機流程要加「把舊設備的記憶搬到新設備」：把 memory_facts、memory_segments、conversations 的 device_id 從舊機改成新機（同一 user_id），並由超級管理員執行。</t>
+        </is>
+      </c>
+    </row>
+    <row r="143" ht="88" customHeight="1">
+      <c r="A143" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-09 21:54</t>
+        </is>
+      </c>
+      <c r="B143" s="13" t="inlineStr">
+        <is>
+          <t>P1-03</t>
+        </is>
+      </c>
+      <c r="C143" s="6" t="inlineStr">
+        <is>
+          <t>資料保留期限與自動清理</t>
+        </is>
+      </c>
+      <c r="D143" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E143" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="F143" s="13" t="n"/>
+      <c r="G143" s="6" t="n"/>
+      <c r="H143" s="13" t="n"/>
+      <c r="I143" s="6" t="inlineStr">
+        <is>
+          <t>補充（2026-10-09 晚）：記憶改成跟設備後，解綁時保留的記憶掛在已解綁的設備名下，家長在設定頁看不到也清不了；還有 device_id 為 NULL 的舊記憶（沒有設備的帳號）。兩者都要納入保留期限自動清理。</t>
+        </is>
+      </c>
+    </row>
+    <row r="144" ht="32" customHeight="1">
+      <c r="A144" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-09 21:54</t>
+        </is>
+      </c>
+      <c r="B144" s="13" t="inlineStr">
+        <is>
+          <t>R-20</t>
+        </is>
+      </c>
+      <c r="C144" s="6" t="inlineStr">
+        <is>
+          <t>孩子資料與角色改成每台設備一份</t>
+        </is>
+      </c>
+      <c r="E144" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="I144" s="6" t="inlineStr">
+        <is>
+          <t>新增任務</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I128"/>
+  <autoFilter ref="A1:I144"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Track R-38: each toy is locked to the IP registered for its MAC at the factory.
Also updates the factory timeline draft (v0.6).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/production-readiness.xlsx
+++ b/docs/production-readiness.xlsx
@@ -13,9 +13,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="更新記錄" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'任務清單'!$A$1:$P$79</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'任務清單'!$A$1:$P$80</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'待確認問題'!$A$1:$G$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$223</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$227</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -641,7 +641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I90"/>
+  <dimension ref="A1:I92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -665,14 +665,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>最後更新：2026-10-13 14:30　·　本頁由 tracker.py 自動生成，請勿手動編輯</t>
+          <t>最後更新：2026-10-13 19:06　·　本頁由 tracker.py 自動生成，請勿手動編輯</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>總進度：17/75 已完成（23%）　·　目前階段：1 止血定案（10/5–10/16）</t>
+          <t>總進度：17/76 已完成（22%）　·　目前階段：1 止血定案（10/5–10/16）</t>
         </is>
       </c>
     </row>
@@ -856,7 +856,7 @@
       </c>
       <c r="C9" s="7">
         <f>COUNTIF('任務清單'!$B:$B,$A9)</f>
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D9" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A9,'任務清單'!$F:$F,D$5)</f>
@@ -864,7 +864,7 @@
       </c>
       <c r="E9" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A9,'任務清單'!$F:$F,E$5)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F9" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A9,'任務清單'!$F:$F,F$5)</f>
@@ -880,7 +880,7 @@
       </c>
       <c r="I9" s="8">
         <f>IFERROR(F9/(C9-H9),0)</f>
-        <v>0.02857142857142857</v>
+        <v>0.027777777777777776</v>
       </c>
     </row>
     <row r="10">
@@ -892,7 +892,7 @@
       <c r="B10" s="6" t="n"/>
       <c r="C10" s="5">
         <f>SUM(C6:C9)</f>
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D10" s="5">
         <f>SUM(D6:D9)</f>
@@ -900,7 +900,7 @@
       </c>
       <c r="E10" s="5">
         <f>SUM(E6:E9)</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F10" s="5">
         <f>SUM(F6:F9)</f>
@@ -916,7 +916,7 @@
       </c>
       <c r="I10" s="9">
         <f>IFERROR(F10/(C10-H10),0)</f>
-        <v>0.22666666666666666</v>
+        <v>0.2236842105263158</v>
       </c>
     </row>
     <row r="12">
@@ -1059,7 +1059,7 @@
       </c>
       <c r="C15" s="7">
         <f>COUNTIF('任務清單'!$C:$C,$A15)</f>
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D15" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A15,'任務清單'!$F:$F,D$12)</f>
@@ -1067,7 +1067,7 @@
       </c>
       <c r="E15" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A15,'任務清單'!$F:$F,E$12)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F15" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A15,'任務清單'!$F:$F,F$12)</f>
@@ -1135,7 +1135,7 @@
       <c r="B17" s="6" t="n"/>
       <c r="C17" s="5">
         <f>SUM(C13:C16)</f>
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D17" s="5">
         <f>SUM(D13:D16)</f>
@@ -1143,7 +1143,7 @@
       </c>
       <c r="E17" s="5">
         <f>SUM(E13:E16)</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F17" s="5">
         <f>SUM(F13:F16)</f>
@@ -1159,7 +1159,7 @@
       </c>
       <c r="I17" s="9">
         <f>IFERROR(F17/(C17-H17),0)</f>
-        <v>0.22666666666666666</v>
+        <v>0.2236842105263158</v>
       </c>
     </row>
     <row r="19">
@@ -1452,30 +1452,31 @@
       <c r="H28" s="11" t="n"/>
       <c r="I28" s="12" t="n"/>
     </row>
-    <row r="29" ht="60" customHeight="1">
+    <row r="29" ht="242" customHeight="1">
       <c r="A29" s="13" t="inlineStr">
         <is>
-          <t>P1-01</t>
+          <t>R-37</t>
         </is>
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>加入內容審核層（輸入與輸出）</t>
+          <t>網頁設定玩具的 Wi-Fi：查看、新增、刪除</t>
         </is>
       </c>
       <c r="C29" s="13" t="inlineStr">
         <is>
-          <t>2 內測準備</t>
+          <t>3 封閉內測</t>
         </is>
       </c>
       <c r="D29" s="13" t="inlineStr">
         <is>
-          <t>未開始</t>
+          <t>進行中</t>
         </is>
       </c>
       <c r="E29" s="6" t="inlineStr">
         <is>
-          <t>STT 文字與 LLM 輸出都經審核，尺度按 3–6 歲；命中時換成安全回覆並記錄事件，事件只記類別、時間、角色，不記原文（管理員不能看兒童內容，見 Q7）；首字延遲增加 ≤150ms。</t>
+          <t>上次測試：部分通過 — 模擬玩具經本機語音服務器＋網頁：status/scan/add/delete 正常；刪除目前 Wi-Fi → current 被拒；斷線 5 秒內頁面顯示睡著、按鈕停用；測試密碼在語音服務器日誌、網頁服務器日誌、資料庫均搜不到；用別人裝置 ID 重放 server action → forbidden；pytest 17 項通過（全套 230）；韌體 spotpear-ai-toy-localall 編譯通過（RAM 17.5%、Flash 75.9%）。未測：真機 ①② 及 OTA 推出
+① 設定頁顯示玩具在線／離線、目前 Wi-Fi 和訊號、已記住的 Wi-Fi 清單（只有名稱，不顯示密碼）② 在線時可新增 Wi-Fi（輸入或從玩具掃描到的清單選）、刪除 Wi-Fi；不能刪除正在使用的那個 ③ 經 /ws/esp32 轉送：伺服器先確認是設備主人；密碼不寫入資料庫、不寫入日誌 ④ 新增不切換網絡，目前 Wi-Fi 消失時才按訊號選；清單標示「連過／未連過」⑤ 上限 8 個 ⑥ 韌體改動經 OTA 推出</t>
         </is>
       </c>
       <c r="F29" s="11" t="n"/>
@@ -1483,15 +1484,15 @@
       <c r="H29" s="11" t="n"/>
       <c r="I29" s="12" t="n"/>
     </row>
-    <row r="30" ht="32" customHeight="1">
+    <row r="30" ht="60" customHeight="1">
       <c r="A30" s="13" t="inlineStr">
         <is>
-          <t>P1-02</t>
+          <t>P1-01</t>
         </is>
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>日誌移除兒童個人資料</t>
+          <t>加入內容審核層（輸入與輸出）</t>
         </is>
       </c>
       <c r="C30" s="13" t="inlineStr">
@@ -1506,7 +1507,7 @@
       </c>
       <c r="E30" s="6" t="inlineStr">
         <is>
-          <t>生產日誌只記 ID、長度、類別，不記內容；內容只在 DEBUG 等級輸出，生產不開 DEBUG。</t>
+          <t>STT 文字與 LLM 輸出都經審核，尺度按 3–6 歲；命中時換成安全回覆並記錄事件，事件只記類別、時間、角色，不記原文（管理員不能看兒童內容，見 Q7）；首字延遲增加 ≤150ms。</t>
         </is>
       </c>
       <c r="F30" s="11" t="n"/>
@@ -1514,15 +1515,15 @@
       <c r="H30" s="11" t="n"/>
       <c r="I30" s="12" t="n"/>
     </row>
-    <row r="31" ht="60" customHeight="1">
+    <row r="31" ht="32" customHeight="1">
       <c r="A31" s="13" t="inlineStr">
         <is>
-          <t>P1-10</t>
+          <t>P1-02</t>
         </is>
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>管理操作審計記錄</t>
+          <t>日誌移除兒童個人資料</t>
         </is>
       </c>
       <c r="C31" s="13" t="inlineStr">
@@ -1537,7 +1538,7 @@
       </c>
       <c r="E31" s="6" t="inlineStr">
         <is>
-          <t>每個管理操作寫一筆記錄：誰、什麼時間、什麼操作、對象、改之前與改之後的值；記錄只能新增，任何人（包括超級管理員）都不能修改或刪除；超級管理員能在管理端查看。</t>
+          <t>生產日誌只記 ID、長度、類別，不記內容；內容只在 DEBUG 等級輸出，生產不開 DEBUG。</t>
         </is>
       </c>
       <c r="F31" s="11" t="n"/>
@@ -1545,15 +1546,15 @@
       <c r="H31" s="11" t="n"/>
       <c r="I31" s="12" t="n"/>
     </row>
-    <row r="32" ht="46" customHeight="1">
+    <row r="32" ht="60" customHeight="1">
       <c r="A32" s="13" t="inlineStr">
         <is>
-          <t>P1-11</t>
+          <t>P1-10</t>
         </is>
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>伺服器與資料庫直接存取的管控</t>
+          <t>管理操作審計記錄</t>
         </is>
       </c>
       <c r="C32" s="13" t="inlineStr">
@@ -1568,7 +1569,7 @@
       </c>
       <c r="E32" s="6" t="inlineStr">
         <is>
-          <t>列出誰有 SSH 與資料庫直連權限（越少越好）；service_role key 只存在伺服器的 env；私隱政策寫明這類存取的範圍；每次直接查看生產資料都留記錄。</t>
+          <t>每個管理操作寫一筆記錄：誰、什麼時間、什麼操作、對象、改之前與改之後的值；記錄只能新增，任何人（包括超級管理員）都不能修改或刪除；超級管理員能在管理端查看。</t>
         </is>
       </c>
       <c r="F32" s="11" t="n"/>
@@ -1579,12 +1580,12 @@
     <row r="33" ht="46" customHeight="1">
       <c r="A33" s="13" t="inlineStr">
         <is>
-          <t>P2-02</t>
+          <t>P1-11</t>
         </is>
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>CI 跑測試與靜態檢查</t>
+          <t>伺服器與資料庫直接存取的管控</t>
         </is>
       </c>
       <c r="C33" s="13" t="inlineStr">
@@ -1599,7 +1600,7 @@
       </c>
       <c r="E33" s="6" t="inlineStr">
         <is>
-          <t>推送與 PR 時跑 pytest、ruff、pyright、next lint、tsc --noEmit、pio run；任何一項失敗就不發佈 image。</t>
+          <t>列出誰有 SSH 與資料庫直連權限（越少越好）；service_role key 只存在伺服器的 env；私隱政策寫明這類存取的範圍；每次直接查看生產資料都留記錄。</t>
         </is>
       </c>
       <c r="F33" s="11" t="n"/>
@@ -1607,15 +1608,15 @@
       <c r="H33" s="11" t="n"/>
       <c r="I33" s="12" t="n"/>
     </row>
-    <row r="34" ht="32" customHeight="1">
+    <row r="34" ht="46" customHeight="1">
       <c r="A34" s="13" t="inlineStr">
         <is>
-          <t>P2-04</t>
+          <t>P2-02</t>
         </is>
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>容器改用非 root 用戶</t>
+          <t>CI 跑測試與靜態檢查</t>
         </is>
       </c>
       <c r="C34" s="13" t="inlineStr">
@@ -1630,7 +1631,7 @@
       </c>
       <c r="E34" s="6" t="inlineStr">
         <is>
-          <t>兩個 Dockerfile 都設定非 root 的 USER。</t>
+          <t>推送與 PR 時跑 pytest、ruff、pyright、next lint、tsc --noEmit、pio run；任何一項失敗就不發佈 image。</t>
         </is>
       </c>
       <c r="F34" s="11" t="n"/>
@@ -1638,68 +1639,68 @@
       <c r="H34" s="11" t="n"/>
       <c r="I34" s="12" t="n"/>
     </row>
-    <row r="36">
-      <c r="A36" s="10" t="inlineStr">
+    <row r="35" ht="32" customHeight="1">
+      <c r="A35" s="13" t="inlineStr">
+        <is>
+          <t>P2-04</t>
+        </is>
+      </c>
+      <c r="B35" s="6" t="inlineStr">
+        <is>
+          <t>容器改用非 root 用戶</t>
+        </is>
+      </c>
+      <c r="C35" s="13" t="inlineStr">
+        <is>
+          <t>2 內測準備</t>
+        </is>
+      </c>
+      <c r="D35" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E35" s="6" t="inlineStr">
+        <is>
+          <t>兩個 Dockerfile 都設定非 root 的 USER。</t>
+        </is>
+      </c>
+      <c r="F35" s="11" t="n"/>
+      <c r="G35" s="11" t="n"/>
+      <c r="H35" s="11" t="n"/>
+      <c r="I35" s="12" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="10" t="inlineStr">
         <is>
           <t>✅ 最近完成與測試效果</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="4" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
         <is>
           <t>編號</t>
         </is>
       </c>
-      <c r="B37" s="4" t="inlineStr">
+      <c r="B38" s="4" t="inlineStr">
         <is>
           <t>任務</t>
         </is>
       </c>
-      <c r="C37" s="4" t="inlineStr">
+      <c r="C38" s="4" t="inlineStr">
         <is>
           <t>測試結果</t>
         </is>
       </c>
-      <c r="D37" s="4" t="inlineStr">
+      <c r="D38" s="4" t="inlineStr">
         <is>
           <t>完成日期</t>
         </is>
       </c>
-      <c r="E37" s="4" t="inlineStr">
+      <c r="E38" s="4" t="inlineStr">
         <is>
           <t>測試證據</t>
-        </is>
-      </c>
-      <c r="F37" s="11" t="n"/>
-      <c r="G37" s="11" t="n"/>
-      <c r="H37" s="11" t="n"/>
-      <c r="I37" s="12" t="n"/>
-    </row>
-    <row r="38" ht="102" customHeight="1">
-      <c r="A38" s="13" t="inlineStr">
-        <is>
-          <t>P0-12</t>
-        </is>
-      </c>
-      <c r="B38" s="6" t="inlineStr">
-        <is>
-          <t>收緊 Admin 權限與路由保護</t>
-        </is>
-      </c>
-      <c r="C38" s="13" t="inlineStr">
-        <is>
-          <t>通過</t>
-        </is>
-      </c>
-      <c r="D38" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-12</t>
-        </is>
-      </c>
-      <c r="E38" s="6" t="inlineStr">
-        <is>
-          <t>線上 2026-10-12（bac24e9）：runbook 10/08 檢查 未登入 /admin→/login、/api/admin→401、has_role() 只看角色、無管理員 policy 觸及 conversations/記憶表、超管≥1；未登入 /home、/admin→/login；用戶確認：家長帳號開 /admin 轉回 /home、管理員在 /admin 修改角色保存成功；角色細分權限沿用本機 61/61</t>
         </is>
       </c>
       <c r="F38" s="11" t="n"/>
@@ -1707,15 +1708,15 @@
       <c r="H38" s="11" t="n"/>
       <c r="I38" s="12" t="n"/>
     </row>
-    <row r="39" ht="88" customHeight="1">
+    <row r="39" ht="102" customHeight="1">
       <c r="A39" s="13" t="inlineStr">
         <is>
-          <t>P0-15</t>
+          <t>P0-12</t>
         </is>
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>角色表權限：只有內容管理員能發佈，關閉家長自建角色</t>
+          <t>收緊 Admin 權限與路由保護</t>
         </is>
       </c>
       <c r="C39" s="13" t="inlineStr">
@@ -1730,7 +1731,7 @@
       </c>
       <c r="E39" s="6" t="inlineStr">
         <is>
-          <t>線上 2026-10-12：② anon 只見 6 個已發佈 hk_ 內建，查隱藏/醫生/家長自建 → []，anon POST → 401；① authenticated 寫入權限由 20261007140000 REVOKE（runbook 10/08 已套用）；用戶確認：④ 家長登入後 /home/create 轉回 /home ③ 管理員在 /admin 修改角色保存成功</t>
+          <t>線上 2026-10-12（bac24e9）：runbook 10/08 檢查 未登入 /admin→/login、/api/admin→401、has_role() 只看角色、無管理員 policy 觸及 conversations/記憶表、超管≥1；未登入 /home、/admin→/login；用戶確認：家長帳號開 /admin 轉回 /home、管理員在 /admin 修改角色保存成功；角色細分權限沿用本機 61/61</t>
         </is>
       </c>
       <c r="F39" s="11" t="n"/>
@@ -1741,12 +1742,12 @@
     <row r="40" ht="88" customHeight="1">
       <c r="A40" s="13" t="inlineStr">
         <is>
-          <t>P0-16</t>
+          <t>P0-15</t>
         </is>
       </c>
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>移除「醫生」身份與寫死的通關碼</t>
+          <t>角色表權限：只有內容管理員能發佈，關閉家長自建角色</t>
         </is>
       </c>
       <c r="C40" s="13" t="inlineStr">
@@ -1761,7 +1762,7 @@
       </c>
       <c r="E40" s="6" t="inlineStr">
         <is>
-          <t>線上 2026-10-12：生產 commit bac24e9 git grep checkDoctorAction/kiwi-subtle-emu/=== "doctor"/isDoctor → 0；線上 13 個 JS（/、/login、/onboard）grep 通關碼/"doctor"/Santa/patient → 0；anon 讀角色只見 6 個 hk_ 角色、is_doctor 全 false；用戶今日線上登入及 playground 正常</t>
+          <t>線上 2026-10-12：② anon 只見 6 個已發佈 hk_ 內建，查隱藏/醫生/家長自建 → []，anon POST → 401；① authenticated 寫入權限由 20261007140000 REVOKE（runbook 10/08 已套用）；用戶確認：④ 家長登入後 /home/create 轉回 /home ③ 管理員在 /admin 修改角色保存成功</t>
         </is>
       </c>
       <c r="F40" s="11" t="n"/>
@@ -1769,15 +1770,15 @@
       <c r="H40" s="11" t="n"/>
       <c r="I40" s="12" t="n"/>
     </row>
-    <row r="41" ht="60" customHeight="1">
+    <row r="41" ht="88" customHeight="1">
       <c r="A41" s="13" t="inlineStr">
         <is>
-          <t>P0-09</t>
+          <t>P0-16</t>
         </is>
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>瀏覽器語音路由改用簽名 token（/ws/nextjs）</t>
+          <t>移除「醫生」身份與寫死的通關碼</t>
         </is>
       </c>
       <c r="C41" s="13" t="inlineStr">
@@ -1792,7 +1793,7 @@
       </c>
       <c r="E41" s="6" t="inlineStr">
         <is>
-          <t>線上 2026-10-12（bac24e9）：wss /fastapi/ws/nextjs 只帶 user_id 或 token=bogus → 4401；用戶確認：登入 elatoai.hkqft.com 後網頁 playground 可正常對話</t>
+          <t>線上 2026-10-12：生產 commit bac24e9 git grep checkDoctorAction/kiwi-subtle-emu/=== "doctor"/isDoctor → 0；線上 13 個 JS（/、/login、/onboard）grep 通關碼/"doctor"/Santa/patient → 0；anon 讀角色只見 6 個 hk_ 角色、is_doctor 全 false；用戶今日線上登入及 playground 正常</t>
         </is>
       </c>
       <c r="F41" s="11" t="n"/>
@@ -1803,12 +1804,12 @@
     <row r="42" ht="60" customHeight="1">
       <c r="A42" s="13" t="inlineStr">
         <is>
-          <t>P0-17</t>
+          <t>P0-09</t>
         </is>
       </c>
       <c r="B42" s="6" t="inlineStr">
         <is>
-          <t>前端的 anon key 必須是公開 key，不可是 secret／service_role</t>
+          <t>瀏覽器語音路由改用簽名 token（/ws/nextjs）</t>
         </is>
       </c>
       <c r="C42" s="13" t="inlineStr">
@@ -1823,7 +1824,7 @@
       </c>
       <c r="E42" s="6" t="inlineStr">
         <is>
-          <t>線上 2026-10-12（bac24e9）：/login 引用的 13 個 JS + HTML 無 sb_secret_，唯一 key 為 role=anon 的 JWT；② 用該 key GET /rest/v1/users → 42501；③ 本機 10/07 已換 publishable</t>
+          <t>線上 2026-10-12（bac24e9）：wss /fastapi/ws/nextjs 只帶 user_id 或 token=bogus → 4401；用戶確認：登入 elatoai.hkqft.com 後網頁 playground 可正常對話</t>
         </is>
       </c>
       <c r="F42" s="11" t="n"/>
@@ -1831,15 +1832,15 @@
       <c r="H42" s="11" t="n"/>
       <c r="I42" s="12" t="n"/>
     </row>
-    <row r="43" ht="46" customHeight="1">
+    <row r="43" ht="60" customHeight="1">
       <c r="A43" s="13" t="inlineStr">
         <is>
-          <t>P0-10</t>
+          <t>P0-17</t>
         </is>
       </c>
       <c r="B43" s="6" t="inlineStr">
         <is>
-          <t>生產環境關閉 /browser 測試頁與 /ws/browser</t>
+          <t>前端的 anon key 必須是公開 key，不可是 secret／service_role</t>
         </is>
       </c>
       <c r="C43" s="13" t="inlineStr">
@@ -1854,7 +1855,7 @@
       </c>
       <c r="E43" s="6" t="inlineStr">
         <is>
-          <t>線上 2026-10-12（bac24e9）：GET /fastapi/browser 404、/fastapi/ 404、/fastapi/healthz 200、wss /fastapi/ws/browser → HTTP 403</t>
+          <t>線上 2026-10-12（bac24e9）：/login 引用的 13 個 JS + HTML 無 sb_secret_，唯一 key 為 role=anon 的 JWT；② 用該 key GET /rest/v1/users → 42501；③ 本機 10/07 已換 publishable</t>
         </is>
       </c>
       <c r="F43" s="11" t="n"/>
@@ -1862,15 +1863,15 @@
       <c r="H43" s="11" t="n"/>
       <c r="I43" s="12" t="n"/>
     </row>
-    <row r="44" ht="60" customHeight="1">
+    <row r="44" ht="46" customHeight="1">
       <c r="A44" s="13" t="inlineStr">
         <is>
-          <t>P0-08</t>
+          <t>P0-10</t>
         </is>
       </c>
       <c r="B44" s="6" t="inlineStr">
         <is>
-          <t>語音伺服器驗證設備身份（/ws/esp32）</t>
+          <t>生產環境關閉 /browser 測試頁與 /ws/browser</t>
         </is>
       </c>
       <c r="C44" s="13" t="inlineStr">
@@ -1885,7 +1886,7 @@
       </c>
       <c r="E44" s="6" t="inlineStr">
         <is>
-          <t>線上 2026-10-12（bac24e9）：wss /fastapi/ws/esp32 不帶 token、偽造 token＋X-Device-Mac → 均 4401 invalid device token；42:34 以有效 token 連線對話正常（P0-13 10/09）</t>
+          <t>線上 2026-10-12（bac24e9）：GET /fastapi/browser 404、/fastapi/ 404、/fastapi/healthz 200、wss /fastapi/ws/browser → HTTP 403</t>
         </is>
       </c>
       <c r="F44" s="11" t="n"/>
@@ -1896,12 +1897,12 @@
     <row r="45" ht="60" customHeight="1">
       <c r="A45" s="13" t="inlineStr">
         <is>
-          <t>P0-06</t>
+          <t>P0-08</t>
         </is>
       </c>
       <c r="B45" s="6" t="inlineStr">
         <is>
-          <t>停止憑 MAC 發放永久用戶 JWT</t>
+          <t>語音伺服器驗證設備身份（/ws/esp32）</t>
         </is>
       </c>
       <c r="C45" s="13" t="inlineStr">
@@ -1916,7 +1917,7 @@
       </c>
       <c r="E45" s="6" t="inlineStr">
         <is>
-          <t>線上 2026-10-12（bac24e9）：POST /api/generate_auth_token 只帶 42:34 的 MAC → 401、帶錯誤密鑰 → 401、GET → 410；42:34 用 NVS 密鑰在線上換 token 並連上語音伺服器（P0-13 10/09 實測）</t>
+          <t>線上 2026-10-12（bac24e9）：wss /fastapi/ws/esp32 不帶 token、偽造 token＋X-Device-Mac → 均 4401 invalid device token；42:34 以有效 token 連線對話正常（P0-13 10/09）</t>
         </is>
       </c>
       <c r="F45" s="11" t="n"/>
@@ -1924,50 +1925,58 @@
       <c r="H45" s="11" t="n"/>
       <c r="I45" s="12" t="n"/>
     </row>
-    <row r="47">
-      <c r="A47" s="10" t="inlineStr">
+    <row r="46" ht="60" customHeight="1">
+      <c r="A46" s="13" t="inlineStr">
+        <is>
+          <t>P0-06</t>
+        </is>
+      </c>
+      <c r="B46" s="6" t="inlineStr">
+        <is>
+          <t>停止憑 MAC 發放永久用戶 JWT</t>
+        </is>
+      </c>
+      <c r="C46" s="13" t="inlineStr">
+        <is>
+          <t>通過</t>
+        </is>
+      </c>
+      <c r="D46" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="E46" s="6" t="inlineStr">
+        <is>
+          <t>線上 2026-10-12（bac24e9）：POST /api/generate_auth_token 只帶 42:34 的 MAC → 401、帶錯誤密鑰 → 401、GET → 410；42:34 用 NVS 密鑰在線上換 token 並連上語音伺服器（P0-13 10/09 實測）</t>
+        </is>
+      </c>
+      <c r="F46" s="11" t="n"/>
+      <c r="G46" s="11" t="n"/>
+      <c r="H46" s="11" t="n"/>
+      <c r="I46" s="12" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="10" t="inlineStr">
         <is>
           <t>⏳ 等待依賴 / ⛔ 阻塞</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="4" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
         <is>
           <t>編號</t>
         </is>
       </c>
-      <c r="B48" s="4" t="inlineStr">
+      <c r="B49" s="4" t="inlineStr">
         <is>
           <t>任務</t>
         </is>
       </c>
-      <c r="C48" s="4" t="inlineStr">
+      <c r="C49" s="4" t="inlineStr">
         <is>
           <t>在等什麼</t>
-        </is>
-      </c>
-      <c r="D48" s="11" t="n"/>
-      <c r="E48" s="11" t="n"/>
-      <c r="F48" s="11" t="n"/>
-      <c r="G48" s="11" t="n"/>
-      <c r="H48" s="11" t="n"/>
-      <c r="I48" s="12" t="n"/>
-    </row>
-    <row r="49" ht="60" customHeight="1">
-      <c r="A49" s="13" t="inlineStr">
-        <is>
-          <t>R-16</t>
-        </is>
-      </c>
-      <c r="B49" s="6" t="inlineStr">
-        <is>
-          <t>Spotpear 量產版加電池電壓檢測（GPIO0 分壓）</t>
-        </is>
-      </c>
-      <c r="C49" s="6" t="inlineStr">
-        <is>
-          <t>阻塞：[2026-10-07] 仍按 10/06 決定暫緩：等用戶做充滿再放電測試（與 R-17 同一次），看 VDD 低電提醒在關機前多久觸發；太遲或不觸發才向 Spotpear 提改板。已把分壓改板的問題一併放進給 Spotpear 的草稿，方便同一封發出</t>
         </is>
       </c>
       <c r="D49" s="11" t="n"/>
@@ -1977,20 +1986,20 @@
       <c r="H49" s="11" t="n"/>
       <c r="I49" s="12" t="n"/>
     </row>
-    <row r="50" ht="88" customHeight="1">
+    <row r="50" ht="60" customHeight="1">
       <c r="A50" s="13" t="inlineStr">
         <is>
-          <t>R-17</t>
+          <t>R-16</t>
         </is>
       </c>
       <c r="B50" s="6" t="inlineStr">
         <is>
-          <t>Spotpear 電池耗盡時插電能否正常開機（供電路徑）</t>
+          <t>Spotpear 量產版加電池電壓檢測（GPIO0 分壓）</t>
         </is>
       </c>
       <c r="C50" s="6" t="inlineStr">
         <is>
-          <t>阻塞：[2026-10-08] 2026-10-08 開發板 63:64 插著 USB 時兩次無法解釋的完全斷電重開：09:13:26（崩潰循環中）、10:44:33（閒置、用戶確認沒碰）。都是 USB 先斷線再以 ESP_RST_POWERON 開機，非 brownout；斷電前 6 秒 GPIO0 讀數 99.9% 參考值，屬突然切斷而非緩降（SupplyMonitor 取樣太疏抓不到瞬間）。韌體無法造成 POWERON，指向充電芯片/電池保護/供電路徑，應一併問 Spotpear；放電實測時留意插 USB 閒置時是否也會斷電</t>
+          <t>阻塞：[2026-10-07] 仍按 10/06 決定暫緩：等用戶做充滿再放電測試（與 R-17 同一次），看 VDD 低電提醒在關機前多久觸發；太遲或不觸發才向 Spotpear 提改板。已把分壓改板的問題一併放進給 Spotpear 的草稿，方便同一封發出</t>
         </is>
       </c>
       <c r="D50" s="11" t="n"/>
@@ -2000,20 +2009,20 @@
       <c r="H50" s="11" t="n"/>
       <c r="I50" s="12" t="n"/>
     </row>
-    <row r="51" ht="32" customHeight="1">
+    <row r="51" ht="88" customHeight="1">
       <c r="A51" s="13" t="inlineStr">
         <is>
-          <t>P1-09</t>
+          <t>R-17</t>
         </is>
       </c>
       <c r="B51" s="6" t="inlineStr">
         <is>
-          <t>家長鎖：孩子模式進設定要輸入 PIN</t>
+          <t>Spotpear 電池耗盡時插電能否正常開機（供電路徑）</t>
         </is>
       </c>
       <c r="C51" s="6" t="inlineStr">
         <is>
-          <t>阻塞：[2026-10-13] 2026-10-13 用戶決定：AI Buddy（品牌 C）延到 1/15 之後，本項不卡 1/15 出廠；AI Buddy 啟動時再開。</t>
+          <t>阻塞：[2026-10-08] 2026-10-08 開發板 63:64 插著 USB 時兩次無法解釋的完全斷電重開：09:13:26（崩潰循環中）、10:44:33（閒置、用戶確認沒碰）。都是 USB 先斷線再以 ESP_RST_POWERON 開機，非 brownout；斷電前 6 秒 GPIO0 讀數 99.9% 參考值，屬突然切斷而非緩降（SupplyMonitor 取樣太疏抓不到瞬間）。韌體無法造成 POWERON，指向充電芯片/電池保護/供電路徑，應一併問 Spotpear；放電實測時留意插 USB 閒置時是否也會斷電</t>
         </is>
       </c>
       <c r="D51" s="11" t="n"/>
@@ -2026,12 +2035,12 @@
     <row r="52" ht="32" customHeight="1">
       <c r="A52" s="13" t="inlineStr">
         <is>
-          <t>R-12</t>
+          <t>P1-09</t>
         </is>
       </c>
       <c r="B52" s="6" t="inlineStr">
         <is>
-          <t>家長控制：每日使用上限和休息時段</t>
+          <t>家長鎖：孩子模式進設定要輸入 PIN</t>
         </is>
       </c>
       <c r="C52" s="6" t="inlineStr">
@@ -2049,12 +2058,12 @@
     <row r="53" ht="32" customHeight="1">
       <c r="A53" s="13" t="inlineStr">
         <is>
-          <t>R-29</t>
+          <t>R-12</t>
         </is>
       </c>
       <c r="B53" s="6" t="inlineStr">
         <is>
-          <t>AI Buddy App（品牌 C）頁面</t>
+          <t>家長控制：每日使用上限和休息時段</t>
         </is>
       </c>
       <c r="C53" s="6" t="inlineStr">
@@ -2069,20 +2078,20 @@
       <c r="H53" s="11" t="n"/>
       <c r="I53" s="12" t="n"/>
     </row>
-    <row r="54" ht="18" customHeight="1">
+    <row r="54" ht="32" customHeight="1">
       <c r="A54" s="13" t="inlineStr">
         <is>
-          <t>R-05</t>
+          <t>R-29</t>
         </is>
       </c>
       <c r="B54" s="6" t="inlineStr">
         <is>
-          <t>內測版外殼（3D 打印 20 台）</t>
+          <t>AI Buddy App（品牌 C）頁面</t>
         </is>
       </c>
       <c r="C54" s="6" t="inlineStr">
         <is>
-          <t>等 R-01</t>
+          <t>阻塞：[2026-10-13] 2026-10-13 用戶決定：AI Buddy（品牌 C）延到 1/15 之後，本項不卡 1/15 出廠；AI Buddy 啟動時再開。</t>
         </is>
       </c>
       <c r="D54" s="11" t="n"/>
@@ -2095,17 +2104,17 @@
     <row r="55" ht="18" customHeight="1">
       <c r="A55" s="13" t="inlineStr">
         <is>
-          <t>R-06</t>
+          <t>R-05</t>
         </is>
       </c>
       <c r="B55" s="6" t="inlineStr">
         <is>
-          <t>家長自助上手流程</t>
+          <t>內測版外殼（3D 打印 20 台）</t>
         </is>
       </c>
       <c r="C55" s="6" t="inlineStr">
         <is>
-          <t>等 P0-11</t>
+          <t>等 R-01</t>
         </is>
       </c>
       <c r="D55" s="11" t="n"/>
@@ -2115,20 +2124,20 @@
       <c r="H55" s="11" t="n"/>
       <c r="I55" s="12" t="n"/>
     </row>
-    <row r="56" ht="32" customHeight="1">
+    <row r="56" ht="18" customHeight="1">
       <c r="A56" s="13" t="inlineStr">
         <is>
-          <t>R-13</t>
+          <t>R-06</t>
         </is>
       </c>
       <c r="B56" s="6" t="inlineStr">
         <is>
-          <t>CP1 內測就緒檢查（10/30）</t>
+          <t>家長自助上手流程</t>
         </is>
       </c>
       <c r="C56" s="6" t="inlineStr">
         <is>
-          <t>等 P0-07、P0-11、P1-01、P1-02、P2-09、R-01、R-02、R-04、R-05、R-06、P1-09、P1-11</t>
+          <t>等 P0-11</t>
         </is>
       </c>
       <c r="D56" s="11" t="n"/>
@@ -2141,17 +2150,17 @@
     <row r="57" ht="32" customHeight="1">
       <c r="A57" s="13" t="inlineStr">
         <is>
-          <t>R-18</t>
+          <t>R-13</t>
         </is>
       </c>
       <c r="B57" s="6" t="inlineStr">
         <is>
-          <t>長按 BOOT 重新配網（開 AIBuddy-XXXX 熱點）</t>
+          <t>CP1 內測就緒檢查（10/30）</t>
         </is>
       </c>
       <c r="C57" s="6" t="inlineStr">
         <is>
-          <t>等 R-01</t>
+          <t>等 P0-07、P0-11、P1-01、P1-02、P2-09、R-01、R-02、R-04、R-05、R-06、P1-09、P1-11</t>
         </is>
       </c>
       <c r="D57" s="11" t="n"/>
@@ -2164,12 +2173,12 @@
     <row r="58" ht="32" customHeight="1">
       <c r="A58" s="13" t="inlineStr">
         <is>
-          <t>R-19</t>
+          <t>R-18</t>
         </is>
       </c>
       <c r="B58" s="6" t="inlineStr">
         <is>
-          <t>外接按鈕：量產板加 I2C 擴展晶片（TCA9555）</t>
+          <t>長按 BOOT 重新配網（開 AIBuddy-XXXX 熱點）</t>
         </is>
       </c>
       <c r="C58" s="6" t="inlineStr">
@@ -2184,20 +2193,20 @@
       <c r="H58" s="11" t="n"/>
       <c r="I58" s="12" t="n"/>
     </row>
-    <row r="59" ht="18" customHeight="1">
+    <row r="59" ht="32" customHeight="1">
       <c r="A59" s="13" t="inlineStr">
         <is>
-          <t>R-20</t>
+          <t>R-19</t>
         </is>
       </c>
       <c r="B59" s="6" t="inlineStr">
         <is>
-          <t>孩子資料與角色改成每台設備一份</t>
+          <t>外接按鈕：量產板加 I2C 擴展晶片（TCA9555）</t>
         </is>
       </c>
       <c r="C59" s="6" t="inlineStr">
         <is>
-          <t>等 P1-12</t>
+          <t>等 R-01</t>
         </is>
       </c>
       <c r="D59" s="11" t="n"/>
@@ -2207,20 +2216,20 @@
       <c r="H59" s="11" t="n"/>
       <c r="I59" s="12" t="n"/>
     </row>
-    <row r="60" ht="32" customHeight="1">
+    <row r="60" ht="18" customHeight="1">
       <c r="A60" s="13" t="inlineStr">
         <is>
-          <t>R-27</t>
+          <t>R-20</t>
         </is>
       </c>
       <c r="B60" s="6" t="inlineStr">
         <is>
-          <t>App 內登入：驗證碼、原生社交登入、刪除帳號</t>
+          <t>孩子資料與角色改成每台設備一份</t>
         </is>
       </c>
       <c r="C60" s="6" t="inlineStr">
         <is>
-          <t>等 R-26</t>
+          <t>等 P1-12</t>
         </is>
       </c>
       <c r="D60" s="11" t="n"/>
@@ -2230,20 +2239,20 @@
       <c r="H60" s="11" t="n"/>
       <c r="I60" s="12" t="n"/>
     </row>
-    <row r="61" ht="18" customHeight="1">
+    <row r="61" ht="32" customHeight="1">
       <c r="A61" s="13" t="inlineStr">
         <is>
-          <t>P0-14</t>
+          <t>R-27</t>
         </is>
       </c>
       <c r="B61" s="6" t="inlineStr">
         <is>
-          <t>韌體簽章、Secure Boot 與 Flash 加密</t>
+          <t>App 內登入：驗證碼、原生社交登入、刪除帳號</t>
         </is>
       </c>
       <c r="C61" s="6" t="inlineStr">
         <is>
-          <t>等 R-01</t>
+          <t>等 R-26</t>
         </is>
       </c>
       <c r="D61" s="11" t="n"/>
@@ -2256,17 +2265,17 @@
     <row r="62" ht="18" customHeight="1">
       <c r="A62" s="13" t="inlineStr">
         <is>
-          <t>P1-06</t>
+          <t>P0-14</t>
         </is>
       </c>
       <c r="B62" s="6" t="inlineStr">
         <is>
-          <t>處理 GPL-3.0 依賴（arduino-audio-tools）</t>
+          <t>韌體簽章、Secure Boot 與 Flash 加密</t>
         </is>
       </c>
       <c r="C62" s="6" t="inlineStr">
         <is>
-          <t>等 Q3</t>
+          <t>等 R-01</t>
         </is>
       </c>
       <c r="D62" s="11" t="n"/>
@@ -2279,12 +2288,12 @@
     <row r="63" ht="18" customHeight="1">
       <c r="A63" s="13" t="inlineStr">
         <is>
-          <t>P1-07</t>
+          <t>P1-06</t>
         </is>
       </c>
       <c r="B63" s="6" t="inlineStr">
         <is>
-          <t>LGPL 合規與第三方授權聲明</t>
+          <t>處理 GPL-3.0 依賴（arduino-audio-tools）</t>
         </is>
       </c>
       <c r="C63" s="6" t="inlineStr">
@@ -2302,17 +2311,17 @@
     <row r="64" ht="18" customHeight="1">
       <c r="A64" s="13" t="inlineStr">
         <is>
-          <t>P1-08</t>
+          <t>P1-07</t>
         </is>
       </c>
       <c r="B64" s="6" t="inlineStr">
         <is>
-          <t>硬件認證</t>
+          <t>LGPL 合規與第三方授權聲明</t>
         </is>
       </c>
       <c r="C64" s="6" t="inlineStr">
         <is>
-          <t>等 R-01、R-05</t>
+          <t>等 Q3</t>
         </is>
       </c>
       <c r="D64" s="11" t="n"/>
@@ -2325,17 +2334,17 @@
     <row r="65" ht="18" customHeight="1">
       <c r="A65" s="13" t="inlineStr">
         <is>
-          <t>R-07</t>
+          <t>P1-08</t>
         </is>
       </c>
       <c r="B65" s="6" t="inlineStr">
         <is>
-          <t>20 個家庭封閉內測</t>
+          <t>硬件認證</t>
         </is>
       </c>
       <c r="C65" s="6" t="inlineStr">
         <is>
-          <t>等 R-13</t>
+          <t>等 R-01、R-05</t>
         </is>
       </c>
       <c r="D65" s="11" t="n"/>
@@ -2348,17 +2357,17 @@
     <row r="66" ht="18" customHeight="1">
       <c r="A66" s="13" t="inlineStr">
         <is>
-          <t>R-08</t>
+          <t>R-07</t>
         </is>
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
-          <t>第 8 週關卡決策</t>
+          <t>20 個家庭封閉內測</t>
         </is>
       </c>
       <c r="C66" s="6" t="inlineStr">
         <is>
-          <t>等 R-07、P2-09、P1-08</t>
+          <t>等 R-13</t>
         </is>
       </c>
       <c r="D66" s="11" t="n"/>
@@ -2371,17 +2380,17 @@
     <row r="67" ht="18" customHeight="1">
       <c r="A67" s="13" t="inlineStr">
         <is>
-          <t>R-14</t>
+          <t>R-08</t>
         </is>
       </c>
       <c r="B67" s="6" t="inlineStr">
         <is>
-          <t>離線兒歌與故事</t>
+          <t>第 8 週關卡決策</t>
         </is>
       </c>
       <c r="C67" s="6" t="inlineStr">
         <is>
-          <t>等 R-01</t>
+          <t>等 R-07、P2-09、P1-08</t>
         </is>
       </c>
       <c r="D67" s="11" t="n"/>
@@ -2394,17 +2403,17 @@
     <row r="68" ht="18" customHeight="1">
       <c r="A68" s="13" t="inlineStr">
         <is>
-          <t>R-24</t>
+          <t>R-14</t>
         </is>
       </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t>設備只能用自己品牌的角色</t>
+          <t>離線兒歌與故事</t>
         </is>
       </c>
       <c r="C68" s="6" t="inlineStr">
         <is>
-          <t>等 R-34</t>
+          <t>等 R-01</t>
         </is>
       </c>
       <c r="D68" s="11" t="n"/>
@@ -2417,17 +2426,17 @@
     <row r="69" ht="18" customHeight="1">
       <c r="A69" s="13" t="inlineStr">
         <is>
-          <t>R-28</t>
+          <t>R-24</t>
         </is>
       </c>
       <c r="B69" s="6" t="inlineStr">
         <is>
-          <t>三個 App 的殼：品牌版本與測試版</t>
+          <t>設備只能用自己品牌的角色</t>
         </is>
       </c>
       <c r="C69" s="6" t="inlineStr">
         <is>
-          <t>等 R-25、R-26</t>
+          <t>等 R-34</t>
         </is>
       </c>
       <c r="D69" s="11" t="n"/>
@@ -2440,17 +2449,17 @@
     <row r="70" ht="18" customHeight="1">
       <c r="A70" s="13" t="inlineStr">
         <is>
-          <t>R-30</t>
+          <t>R-28</t>
         </is>
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>快活 App（品牌 A）頁面</t>
+          <t>三個 App 的殼：品牌版本與測試版</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr">
         <is>
-          <t>等 R-25、R-34、Q12</t>
+          <t>等 R-25、R-26</t>
         </is>
       </c>
       <c r="D70" s="11" t="n"/>
@@ -2463,17 +2472,17 @@
     <row r="71" ht="18" customHeight="1">
       <c r="A71" s="13" t="inlineStr">
         <is>
-          <t>R-31</t>
+          <t>R-30</t>
         </is>
       </c>
       <c r="B71" s="6" t="inlineStr">
         <is>
-          <t>政協青年聯會版 App（品牌 B）頁面</t>
+          <t>快活 App（品牌 A）頁面</t>
         </is>
       </c>
       <c r="C71" s="6" t="inlineStr">
         <is>
-          <t>等 R-25、R-34、Q13</t>
+          <t>等 R-25、R-34、Q12</t>
         </is>
       </c>
       <c r="D71" s="11" t="n"/>
@@ -2486,17 +2495,17 @@
     <row r="72" ht="18" customHeight="1">
       <c r="A72" s="13" t="inlineStr">
         <is>
-          <t>R-35</t>
+          <t>R-31</t>
         </is>
       </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>韌體按品牌連線：伺服器網址在出廠時寫入</t>
+          <t>政協青年聯會版 App（品牌 B）頁面</t>
         </is>
       </c>
       <c r="C72" s="6" t="inlineStr">
         <is>
-          <t>等 R-34</t>
+          <t>等 R-25、R-34、Q13</t>
         </is>
       </c>
       <c r="D72" s="11" t="n"/>
@@ -2509,17 +2518,17 @@
     <row r="73" ht="18" customHeight="1">
       <c r="A73" s="13" t="inlineStr">
         <is>
-          <t>R-09</t>
+          <t>R-35</t>
         </is>
       </c>
       <c r="B73" s="6" t="inlineStr">
         <is>
-          <t>量產外殼（真空複模）</t>
+          <t>韌體按品牌連線：伺服器網址在出廠時寫入</t>
         </is>
       </c>
       <c r="C73" s="6" t="inlineStr">
         <is>
-          <t>等 R-08、R-05、Q11</t>
+          <t>等 R-34</t>
         </is>
       </c>
       <c r="D73" s="11" t="n"/>
@@ -2529,20 +2538,20 @@
       <c r="H73" s="11" t="n"/>
       <c r="I73" s="12" t="n"/>
     </row>
-    <row r="74" ht="18" customHeight="1">
+    <row r="74" ht="32" customHeight="1">
       <c r="A74" s="13" t="inlineStr">
         <is>
-          <t>R-10</t>
+          <t>R-38</t>
         </is>
       </c>
       <c r="B74" s="6" t="inlineStr">
         <is>
-          <t>出廠流程</t>
+          <t>公仔出廠鎖死所屬 IP，綁定時顯示該 IP 頭像</t>
         </is>
       </c>
       <c r="C74" s="6" t="inlineStr">
         <is>
-          <t>等 P0-14、R-01、P2-12、R-34、R-35</t>
+          <t>等 P0-11</t>
         </is>
       </c>
       <c r="D74" s="11" t="n"/>
@@ -2555,17 +2564,17 @@
     <row r="75" ht="18" customHeight="1">
       <c r="A75" s="13" t="inlineStr">
         <is>
-          <t>R-15</t>
+          <t>R-09</t>
         </is>
       </c>
       <c r="B75" s="6" t="inlineStr">
         <is>
-          <t>農曆新年前交付（生產 1/15、送達 1/29）</t>
+          <t>量產外殼（真空複模）</t>
         </is>
       </c>
       <c r="C75" s="6" t="inlineStr">
         <is>
-          <t>等 R-09、R-10</t>
+          <t>等 R-08、R-05、Q11</t>
         </is>
       </c>
       <c r="D75" s="11" t="n"/>
@@ -2578,17 +2587,17 @@
     <row r="76" ht="18" customHeight="1">
       <c r="A76" s="13" t="inlineStr">
         <is>
-          <t>R-33</t>
+          <t>R-10</t>
         </is>
       </c>
       <c r="B76" s="6" t="inlineStr">
         <is>
-          <t>三個 App 送審並通過</t>
+          <t>出廠流程</t>
         </is>
       </c>
       <c r="C76" s="6" t="inlineStr">
         <is>
-          <t>等 R-27、R-21、R-28、R-29、R-30、R-31、R-32</t>
+          <t>等 P0-14、R-01、P2-12、R-34、R-35、R-38</t>
         </is>
       </c>
       <c r="D76" s="11" t="n"/>
@@ -2598,73 +2607,73 @@
       <c r="H76" s="11" t="n"/>
       <c r="I76" s="12" t="n"/>
     </row>
-    <row r="78">
-      <c r="A78" s="10" t="inlineStr">
+    <row r="77" ht="18" customHeight="1">
+      <c r="A77" s="13" t="inlineStr">
+        <is>
+          <t>R-15</t>
+        </is>
+      </c>
+      <c r="B77" s="6" t="inlineStr">
+        <is>
+          <t>農曆新年前交付（生產 1/15、送達 1/29）</t>
+        </is>
+      </c>
+      <c r="C77" s="6" t="inlineStr">
+        <is>
+          <t>等 R-09、R-10</t>
+        </is>
+      </c>
+      <c r="D77" s="11" t="n"/>
+      <c r="E77" s="11" t="n"/>
+      <c r="F77" s="11" t="n"/>
+      <c r="G77" s="11" t="n"/>
+      <c r="H77" s="11" t="n"/>
+      <c r="I77" s="12" t="n"/>
+    </row>
+    <row r="78" ht="18" customHeight="1">
+      <c r="A78" s="13" t="inlineStr">
+        <is>
+          <t>R-33</t>
+        </is>
+      </c>
+      <c r="B78" s="6" t="inlineStr">
+        <is>
+          <t>三個 App 送審並通過</t>
+        </is>
+      </c>
+      <c r="C78" s="6" t="inlineStr">
+        <is>
+          <t>等 R-27、R-21、R-28、R-29、R-30、R-31、R-32</t>
+        </is>
+      </c>
+      <c r="D78" s="11" t="n"/>
+      <c r="E78" s="11" t="n"/>
+      <c r="F78" s="11" t="n"/>
+      <c r="G78" s="11" t="n"/>
+      <c r="H78" s="11" t="n"/>
+      <c r="I78" s="12" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="10" t="inlineStr">
         <is>
           <t>❓ 待確認問題</t>
         </is>
       </c>
     </row>
-    <row r="79">
-      <c r="A79" s="4" t="inlineStr">
+    <row r="81">
+      <c r="A81" s="4" t="inlineStr">
         <is>
           <t>編號</t>
         </is>
       </c>
-      <c r="B79" s="4" t="inlineStr">
+      <c r="B81" s="4" t="inlineStr">
         <is>
           <t>問題</t>
         </is>
       </c>
-      <c r="C79" s="4" t="inlineStr">
+      <c r="C81" s="4" t="inlineStr">
         <is>
           <t>影響的任務 / 為什麼重要</t>
-        </is>
-      </c>
-      <c r="D79" s="11" t="n"/>
-      <c r="E79" s="11" t="n"/>
-      <c r="F79" s="11" t="n"/>
-      <c r="G79" s="11" t="n"/>
-      <c r="H79" s="11" t="n"/>
-      <c r="I79" s="12" t="n"/>
-    </row>
-    <row r="80" ht="18" customHeight="1">
-      <c r="A80" s="13" t="inlineStr">
-        <is>
-          <t>Q3</t>
-        </is>
-      </c>
-      <c r="B80" s="6" t="inlineStr">
-        <is>
-          <t>韌體打算閉源商業銷售嗎？</t>
-        </is>
-      </c>
-      <c r="C80" s="6" t="inlineStr">
-        <is>
-          <t>P1-06, P1-07：決定 GPL／LGPL 依賴要開源還是替換。</t>
-        </is>
-      </c>
-      <c r="D80" s="11" t="n"/>
-      <c r="E80" s="11" t="n"/>
-      <c r="F80" s="11" t="n"/>
-      <c r="G80" s="11" t="n"/>
-      <c r="H80" s="11" t="n"/>
-      <c r="I80" s="12" t="n"/>
-    </row>
-    <row r="81" ht="32" customHeight="1">
-      <c r="A81" s="13" t="inlineStr">
-        <is>
-          <t>Q11</t>
-        </is>
-      </c>
-      <c r="B81" s="6" t="inlineStr">
-        <is>
-          <t>馬會快活的賽馬日版和新春版各多少隻（共 2,500）？</t>
-        </is>
-      </c>
-      <c r="C81" s="6" t="inlineStr">
-        <is>
-          <t>R-09, R-15：兩款的服裝和配件要分開訂料；11/20 前不知道，PP 樣和大貨單（11/27）會被拖慢。由馬會決定。</t>
         </is>
       </c>
       <c r="D81" s="11" t="n"/>
@@ -2674,20 +2683,20 @@
       <c r="H81" s="11" t="n"/>
       <c r="I81" s="12" t="n"/>
     </row>
-    <row r="82" ht="60" customHeight="1">
+    <row r="82" ht="18" customHeight="1">
       <c r="A82" s="13" t="inlineStr">
         <is>
-          <t>Q12</t>
+          <t>Q3</t>
         </is>
       </c>
       <c r="B82" s="6" t="inlineStr">
         <is>
-          <t>快活 App 的「會員綁定」是指甚麼：用我們自己的帳號（email 驗證碼），還是接馬會的會員帳號登入（SSO）？</t>
+          <t>韌體打算閉源商業銷售嗎？</t>
         </is>
       </c>
       <c r="C82" s="6" t="inlineStr">
         <is>
-          <t>P0-11, 快活 App（未入追蹤表）：接馬會 SSO 的話，登入、帳號刪除和資料歸屬都要按馬會的介面重做，工作量和排期要另估，而且 W5（11/9–11/13）就要做快活 App 的綁定；用我們的帳號則和其他品牌共用同一套流程。由馬會決定，要盡早問。</t>
+          <t>P1-06, P1-07：決定 GPL／LGPL 依賴要開源還是替換。</t>
         </is>
       </c>
       <c r="D82" s="11" t="n"/>
@@ -2697,20 +2706,20 @@
       <c r="H82" s="11" t="n"/>
       <c r="I82" s="12" t="n"/>
     </row>
-    <row r="83" ht="46" customHeight="1">
+    <row r="83" ht="32" customHeight="1">
       <c r="A83" s="13" t="inlineStr">
         <is>
-          <t>Q13</t>
+          <t>Q11</t>
         </is>
       </c>
       <c r="B83" s="6" t="inlineStr">
         <is>
-          <t>政協青年聯會版的角色、語言和內容由誰提供？什麼時候交？</t>
+          <t>馬會快活的賽馬日版和新春版各多少隻（共 2,500）？</t>
         </is>
       </c>
       <c r="C83" s="6" t="inlineStr">
         <is>
-          <t>品牌 B 的 App 頁面：品牌 B 的用戶是成人會員，但角色、說話語言、內容規則都還沒有。最遲 11/13 要拿到，才趕得及內部測試和 App 頁面（W6）。</t>
+          <t>R-09, R-15：兩款的服裝和配件要分開訂料；11/20 前不知道，PP 樣和大貨單（11/27）會被拖慢。由馬會決定。</t>
         </is>
       </c>
       <c r="D83" s="11" t="n"/>
@@ -2720,63 +2729,109 @@
       <c r="H83" s="11" t="n"/>
       <c r="I83" s="12" t="n"/>
     </row>
-    <row r="85">
-      <c r="A85" s="10" t="inlineStr">
+    <row r="84" ht="60" customHeight="1">
+      <c r="A84" s="13" t="inlineStr">
+        <is>
+          <t>Q12</t>
+        </is>
+      </c>
+      <c r="B84" s="6" t="inlineStr">
+        <is>
+          <t>快活 App 的「會員綁定」是指甚麼：用我們自己的帳號（email 驗證碼），還是接馬會的會員帳號登入（SSO）？</t>
+        </is>
+      </c>
+      <c r="C84" s="6" t="inlineStr">
+        <is>
+          <t>P0-11, 快活 App（未入追蹤表）：接馬會 SSO 的話，登入、帳號刪除和資料歸屬都要按馬會的介面重做，工作量和排期要另估，而且 W5（11/9–11/13）就要做快活 App 的綁定；用我們的帳號則和其他品牌共用同一套流程。由馬會決定，要盡早問。</t>
+        </is>
+      </c>
+      <c r="D84" s="11" t="n"/>
+      <c r="E84" s="11" t="n"/>
+      <c r="F84" s="11" t="n"/>
+      <c r="G84" s="11" t="n"/>
+      <c r="H84" s="11" t="n"/>
+      <c r="I84" s="12" t="n"/>
+    </row>
+    <row r="85" ht="46" customHeight="1">
+      <c r="A85" s="13" t="inlineStr">
+        <is>
+          <t>Q13</t>
+        </is>
+      </c>
+      <c r="B85" s="6" t="inlineStr">
+        <is>
+          <t>政協青年聯會版的角色、語言和內容由誰提供？什麼時候交？</t>
+        </is>
+      </c>
+      <c r="C85" s="6" t="inlineStr">
+        <is>
+          <t>品牌 B 的 App 頁面：品牌 B 的用戶是成人會員，但角色、說話語言、內容規則都還沒有。最遲 11/13 要拿到，才趕得及內部測試和 App 頁面（W6）。</t>
+        </is>
+      </c>
+      <c r="D85" s="11" t="n"/>
+      <c r="E85" s="11" t="n"/>
+      <c r="F85" s="11" t="n"/>
+      <c r="G85" s="11" t="n"/>
+      <c r="H85" s="11" t="n"/>
+      <c r="I85" s="12" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="10" t="inlineStr">
         <is>
           <t>說明</t>
         </is>
       </c>
     </row>
-    <row r="86" ht="32" customHeight="1">
-      <c r="A86" s="14" t="inlineStr">
+    <row r="88" ht="32" customHeight="1">
+      <c r="A88" s="14" t="inlineStr">
         <is>
           <t>・狀態：未開始 → 進行中 → 已完成。只有測試真的跑過而且通過才算已完成；阻塞要在備註寫原因；不再需要的任務標不適用，不要刪。</t>
-        </is>
-      </c>
-    </row>
-    <row r="87" ht="18" customHeight="1">
-      <c r="A87" s="14" t="inlineStr">
-        <is>
-          <t>・測試結果：未測試 / 通過 / 失敗 / 部分通過。測試證據寫跑了什麼、看到什麼，完整歷史在「更新記錄」。</t>
-        </is>
-      </c>
-    </row>
-    <row r="88" ht="18" customHeight="1">
-      <c r="A88" s="14" t="inlineStr">
-        <is>
-          <t>・「接下來」按階段排序，同一階段內再按優先級；依賴還沒滿足的任務不會出現在「接下來」。</t>
         </is>
       </c>
     </row>
     <row r="89" ht="18" customHeight="1">
       <c r="A89" s="14" t="inlineStr">
         <is>
+          <t>・測試結果：未測試 / 通過 / 失敗 / 部分通過。測試證據寫跑了什麼、看到什麼，完整歷史在「更新記錄」。</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="18" customHeight="1">
+      <c r="A90" s="14" t="inlineStr">
+        <is>
+          <t>・「接下來」按階段排序，同一階段內再按優先級；依賴還沒滿足的任務不會出現在「接下來」。</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="18" customHeight="1">
+      <c r="A91" s="14" t="inlineStr">
+        <is>
           <t>・可以手動改：「任務清單」的狀態、測試結果、測試證據、Commit、備註，以及「待確認問題」的回答。其餘欄位和本頁由腳本維護。</t>
         </is>
       </c>
     </row>
-    <row r="90" ht="32" customHeight="1">
-      <c r="A90" s="14" t="inlineStr">
+    <row r="92" ht="32" customHeight="1">
+      <c r="A92" s="14" t="inlineStr">
         <is>
           <t>・建議用法：在 Claude Code 對 Claude 說「P0-02 做完了」或輸入 /prod-readiness。Claude 會先跑測試再更新，並寫進「更新記錄」。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="71">
+  <mergeCells count="73">
     <mergeCell ref="E21:I21"/>
     <mergeCell ref="C61:I61"/>
     <mergeCell ref="E43:I43"/>
     <mergeCell ref="C52:I52"/>
     <mergeCell ref="C70:I70"/>
     <mergeCell ref="A90:I90"/>
-    <mergeCell ref="C48:I48"/>
+    <mergeCell ref="A37:I37"/>
     <mergeCell ref="E24:I24"/>
     <mergeCell ref="E42:I42"/>
     <mergeCell ref="C82:I82"/>
+    <mergeCell ref="A80:I80"/>
+    <mergeCell ref="E33:I33"/>
     <mergeCell ref="A89:I89"/>
-    <mergeCell ref="E33:I33"/>
-    <mergeCell ref="A78:I78"/>
     <mergeCell ref="A3:I3"/>
     <mergeCell ref="E23:I23"/>
     <mergeCell ref="C72:I72"/>
@@ -2784,22 +2839,23 @@
     <mergeCell ref="C67:I67"/>
     <mergeCell ref="C81:I81"/>
     <mergeCell ref="C57:I57"/>
-    <mergeCell ref="A86:I86"/>
     <mergeCell ref="C53:I53"/>
     <mergeCell ref="C66:I66"/>
     <mergeCell ref="E44:I44"/>
     <mergeCell ref="A2:I2"/>
     <mergeCell ref="E29:I29"/>
-    <mergeCell ref="C69:I69"/>
+    <mergeCell ref="E35:I35"/>
     <mergeCell ref="E20:I20"/>
     <mergeCell ref="E38:I38"/>
-    <mergeCell ref="A47:I47"/>
-    <mergeCell ref="A85:I85"/>
+    <mergeCell ref="C69:I69"/>
+    <mergeCell ref="C78:I78"/>
     <mergeCell ref="C49:I49"/>
     <mergeCell ref="E28:I28"/>
+    <mergeCell ref="C77:I77"/>
     <mergeCell ref="C83:I83"/>
     <mergeCell ref="C62:I62"/>
     <mergeCell ref="C68:I68"/>
+    <mergeCell ref="A91:I91"/>
     <mergeCell ref="E31:I31"/>
     <mergeCell ref="E40:I40"/>
     <mergeCell ref="C58:I58"/>
@@ -2808,27 +2864,28 @@
     <mergeCell ref="A19:I19"/>
     <mergeCell ref="C74:I74"/>
     <mergeCell ref="C64:I64"/>
-    <mergeCell ref="C79:I79"/>
+    <mergeCell ref="E46:I46"/>
     <mergeCell ref="C73:I73"/>
     <mergeCell ref="E27:I27"/>
     <mergeCell ref="E45:I45"/>
     <mergeCell ref="C54:I54"/>
+    <mergeCell ref="C85:I85"/>
     <mergeCell ref="C63:I63"/>
+    <mergeCell ref="A48:I48"/>
     <mergeCell ref="C65:I65"/>
     <mergeCell ref="E26:I26"/>
+    <mergeCell ref="A92:I92"/>
     <mergeCell ref="C55:I55"/>
     <mergeCell ref="C50:I50"/>
     <mergeCell ref="C75:I75"/>
-    <mergeCell ref="C80:I80"/>
+    <mergeCell ref="C84:I84"/>
     <mergeCell ref="C56:I56"/>
     <mergeCell ref="E32:I32"/>
-    <mergeCell ref="A36:I36"/>
     <mergeCell ref="E25:I25"/>
     <mergeCell ref="C59:I59"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="E41:I41"/>
     <mergeCell ref="A88:I88"/>
-    <mergeCell ref="E37:I37"/>
     <mergeCell ref="C60:I60"/>
     <mergeCell ref="E22:I22"/>
     <mergeCell ref="A87:I87"/>
@@ -2864,7 +2921,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P79"/>
+  <dimension ref="A1:P80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -5918,7 +5975,7 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="214" customHeight="1">
+    <row r="42" ht="270" customHeight="1">
       <c r="A42" s="13" t="inlineStr">
         <is>
           <t>R-10</t>
@@ -5969,17 +6026,17 @@
       </c>
       <c r="K42" s="6" t="inlineStr">
         <is>
-          <t>兩段式出廠流程：① Spotpear 出貨前燒共用出廠韌體（不含密鑰、不分品牌，含最終 bootloader、分區表、Secure Boot），附每片 MAC 清單 ② 玩具廠裝機芯盒工位用我方電腦和腳本：經序列埠寫入設備密鑰 → 選品牌和款式 → 自檢（喇叭、麥克風、按鍵、燈、電池、WiFi）→ 經 HTTPS 登記設備；每台留一行 QC 記錄；工廠工人照作業指導書即可操作，每台約 1.5 分鐘。</t>
+          <t>兩段式出廠流程：① Spotpear 出貨前燒共用出廠韌體（不含密鑰、不分品牌、不含某個 IP，含最終 bootloader、分區表、Secure Boot），附每片 MAC 清單 ② 玩具廠裝機芯盒工位用我方電腦和腳本：經序列埠寫入設備密鑰 → 選品牌和款式 → 自檢（喇叭、麥克風、按鍵、燈、電池、WiFi）→ 經 HTTPS 按 MAC 登記設備，寫入該公仔的 ip_key 和這個 IP 的預設角色（R-38）；每台留一行 QC 記錄；工廠工人照作業指導書即可操作，每台約 1.5 分鐘。</t>
         </is>
       </c>
       <c r="L42" s="6" t="inlineStr">
         <is>
-          <t>用 Spotpear 燒好的板連續處理 10 台，全部通過且記錄完整；混入一台壞板，自檢能攔下；混入一台未燒共用韌體的板，工位能識別並提示；登記失敗（例如斷網）時該台標為不合格、可重做，不會出現已寫密鑰但伺服器沒有記錄的設備。</t>
+          <t>用 Spotpear 燒好的板連續處理 10 台，其中至少兩種 IP，全部通過且記錄完整，devices.ip_key 與預設角色正確；混入一台壞板，自檢能攔下；混入一台未燒共用韌體的板，工位能識別並提示；登記失敗（例如斷網）時該台標為不合格、可重做，不會出現已寫密鑰但伺服器沒有記錄的設備。重燒 app 分區後 ip_key 仍在。</t>
         </is>
       </c>
       <c r="M42" s="13" t="inlineStr">
         <is>
-          <t>P0-06, P0-14, R-01, P2-12, Q10, R-34, R-35</t>
+          <t>P0-06, P0-14, R-01, P2-12, Q10, R-34, R-35, R-38</t>
         </is>
       </c>
       <c r="N42" s="6" t="n"/>
@@ -5988,7 +6045,8 @@
         <is>
           <t>[2026-10-12] 2026-10-12：燒錄地點未定（Q10），最遲 11/6。設備密鑰、品牌和款式都在出廠時寫入（三個品牌共用一個韌體）。
 [2026-10-12] 2026-10-12 Q10 已定（燒共用韌體）。Spotpear 出貨測試第一次通電就會開 Secure Boot 和 Flash 加密，所以 11/27 交 Spotpear 的映像必須是最終版（P0-14 要在 W5 前驗證）；app 之後經 OTA 更新。
-[2026-10-12] 2026-10-12：三個品牌分開部署後，出廠工位要把每台設備登記到該品牌那套的伺服器，並寫入該品牌的網址（R-35）。</t>
+[2026-10-12] 2026-10-12：三個品牌分開部署後，出廠工位要把每台設備登記到該品牌那套的伺服器，並寫入該品牌的網址（R-35）。
+[2026-10-13] 2026-10-13：工位登記要寫入該公仔的 ip_key 和預設角色（R-38）。IP 不編進共用韌體。</t>
         </is>
       </c>
     </row>
@@ -8506,7 +8564,7 @@
         </is>
       </c>
     </row>
-    <row r="79" ht="116" customHeight="1">
+    <row r="79" ht="270" customHeight="1">
       <c r="A79" s="13" t="inlineStr">
         <is>
           <t>R-37</t>
@@ -8534,43 +8592,123 @@
       </c>
       <c r="F79" s="13" t="inlineStr">
         <is>
-          <t>未開始</t>
+          <t>進行中</t>
         </is>
       </c>
       <c r="G79" s="13" t="inlineStr">
         <is>
+          <t>部分通過</t>
+        </is>
+      </c>
+      <c r="I79" s="6" t="inlineStr">
+        <is>
+          <t>玩具連上 Wi-Fi 後設定熱點就關閉，用戶沒有入口再加第二個 Wi-Fi（例如手機熱點、親戚家）；現在只能在同一網絡打開 http://&lt;板子IP&gt;/wifi，而且那一頁不用登入。用戶 2026-10-13 參考競品的 Network Management 頁，要在網頁做。</t>
+        </is>
+      </c>
+      <c r="J79" s="6" t="inlineStr">
+        <is>
+          <t>firmware-arduino/src/WifiManager.cpp、Audio.cpp（websocket 訊息）；server/fastapi/server.py（/ws/esp32 轉送）；frontend-nextjs 設定頁</t>
+        </is>
+      </c>
+      <c r="K79" s="6" t="inlineStr">
+        <is>
+          <t>① 設定頁顯示玩具在線／離線、目前 Wi-Fi 和訊號、已記住的 Wi-Fi 清單（只有名稱，不顯示密碼）② 在線時可新增 Wi-Fi（輸入或從玩具掃描到的清單選）、刪除 Wi-Fi；不能刪除正在使用的那個 ③ 經 /ws/esp32 轉送：伺服器先確認是設備主人；密碼不寫入資料庫、不寫入日誌 ④ 新增不切換網絡，目前 Wi-Fi 消失時才按訊號選；清單標示「連過／未連過」⑤ 上限 8 個 ⑥ 韌體改動經 OTA 推出</t>
+        </is>
+      </c>
+      <c r="L79" s="6" t="inlineStr">
+        <is>
+          <t>① 網頁新增 Wi-Fi B，關掉 A → 玩具自動改連 B ② B 密碼打錯 → 玩具留在 A，B 標示未連過 ③ 嘗試刪除目前 Wi-Fi → 被拒 ④ 另一帳號呼叫同一接口 → 403 ⑤ 搜尋資料庫和伺服器日誌，找不到測試密碼 ⑥ 玩具離線時頁面顯示離線，新增按鈕停用</t>
+        </is>
+      </c>
+      <c r="M79" s="13" t="n"/>
+      <c r="N79" s="6" t="inlineStr">
+        <is>
+          <t>模擬玩具經本機語音服務器＋網頁：status/scan/add/delete 正常；刪除目前 Wi-Fi → current 被拒；斷線 5 秒內頁面顯示睡著、按鈕停用；測試密碼在語音服務器日誌、網頁服務器日誌、資料庫均搜不到；用別人裝置 ID 重放 server action → forbidden；pytest 17 項通過（全套 230）；韌體 spotpear-ai-toy-localall 編譯通過（RAM 17.5%、Flash 75.9%）。未測：真機 ①② 及 OTA 推出</t>
+        </is>
+      </c>
+      <c r="P79" s="6" t="inlineStr">
+        <is>
+          <t>[2026-10-13] 新增：時間表（project-schedule.xlsx「Jacky 開發與測試」）排在 W4 11/2–11/6，和快活網頁核心一起；內部測試的家庭要加家裡的 Wi-Fi。
+[2026-10-13] 2026-10-13 應 Jacky 要求從 W4 提前開始。韌體：上限 8 個、NVS apOk%d 記錄連過、經 /ws/esp32 收 status/add/delete/scan、不刪不改目前 Wi-Fi、Wi-Fi 指令不印串口、修 delWifi 計數 bug。伺服器：device_wifi.py＋/internal/device_wifi（含 peek），密碼只轉送不留存。網頁：我 &gt; 裝置 &gt; Network &gt; Wi-Fi（Figma C4），deviceWifiAction 檢查擁有者。剩真機測試 ①②（需 62:70 刷 -localall＋兩個真實網絡）與 OTA。</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="298" customHeight="1">
+      <c r="A80" s="13" t="inlineStr">
+        <is>
+          <t>R-38</t>
+        </is>
+      </c>
+      <c r="B80" s="13" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="C80" s="13" t="inlineStr">
+        <is>
+          <t>3 封閉內測</t>
+        </is>
+      </c>
+      <c r="D80" s="6" t="inlineStr">
+        <is>
+          <t>產品</t>
+        </is>
+      </c>
+      <c r="E80" s="6" t="inlineStr">
+        <is>
+          <t>公仔出廠鎖死所屬 IP，綁定時顯示該 IP 頭像</t>
+        </is>
+      </c>
+      <c r="F80" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="G80" s="13" t="inlineStr">
+        <is>
           <t>未測試</t>
         </is>
       </c>
-      <c r="I79" s="6" t="inlineStr">
-        <is>
-          <t>玩具連上 Wi-Fi 後設定熱點就關閉，用戶沒有入口再加第二個 Wi-Fi（例如手機熱點、親戚家）；現在只能在同一網絡打開 http://&lt;板子IP&gt;/wifi，而且那一頁不用登入。用戶 2026-10-13 參考競品的 Network Management 頁，要在網頁做。</t>
-        </is>
-      </c>
-      <c r="J79" s="6" t="inlineStr">
-        <is>
-          <t>firmware-arduino/src/WifiManager.cpp、Audio.cpp（websocket 訊息）；server/fastapi/server.py（/ws/esp32 轉送）；frontend-nextjs 設定頁</t>
-        </is>
-      </c>
-      <c r="K79" s="6" t="inlineStr">
-        <is>
-          <t>① 設定頁顯示玩具在線／離線、目前 Wi-Fi 和訊號、已記住的 Wi-Fi 清單（只有名稱，不顯示密碼）② 在線時可新增 Wi-Fi（輸入或從玩具掃描到的清單選）、刪除 Wi-Fi；不能刪除正在使用的那個 ③ 經 /ws/esp32 轉送：伺服器先確認是設備主人；密碼不寫入資料庫、不寫入日誌 ④ 新增不切換網絡，目前 Wi-Fi 消失時才按訊號選；清單標示「連過／未連過」⑤ 上限 8 個 ⑥ 韌體改動經 OTA 推出</t>
-        </is>
-      </c>
-      <c r="L79" s="6" t="inlineStr">
-        <is>
-          <t>① 網頁新增 Wi-Fi B，關掉 A → 玩具自動改連 B ② B 密碼打錯 → 玩具留在 A，B 標示未連過 ③ 嘗試刪除目前 Wi-Fi → 被拒 ④ 另一帳號呼叫同一接口 → 403 ⑤ 搜尋資料庫和伺服器日誌，找不到測試密碼 ⑥ 玩具離線時頁面顯示離線，新增按鈕停用</t>
-        </is>
-      </c>
-      <c r="M79" s="13" t="n"/>
-      <c r="P79" s="6" t="inlineStr">
-        <is>
-          <t>[2026-10-13] 新增：時間表（project-schedule.xlsx「Jacky 開發與測試」）排在 W4 11/2–11/6，和快活網頁核心一起；內部測試的家庭要加家裡的 Wi-Fi。</t>
+      <c r="I80" s="6" t="inlineStr">
+        <is>
+          <t>同一個 App 會同時賣兩種以上鎖死的公仔。若 IP 只靠這套部署裡有哪些角色來區分，一個帳號上的兩隻公仔會共用同一個角色，其中一隻會說成另一個 IP 的人。</t>
+        </is>
+      </c>
+      <c r="J80" s="6" t="inlineStr">
+        <is>
+          <t>supabase：devices.ip_key、devices.personality_id\nserver/fastapi/device_registry.py\nfrontend-nextjs 認領、My Devices、Playground\nadmin 的 IP image_url\n出廠登記（R-10）</t>
+        </is>
+      </c>
+      <c r="K80" s="6" t="inlineStr">
+        <is>
+          <t>共用韌體映像不含某個 IP。出廠工位按 MAC 把 ip_key 和該 IP 的預設角色寫進 devices；板子不報 IP，解綁不清這欄，家長和 App 改不了。ip_key 為空的開發板維持現在的行為。認領前和 My Devices 用 ips.image_url 顯示這隻公仔的頭像；帳號上的 Current Character 仍是角色圖。角色在 devices.personality_id，資料庫拒絕把別的 IP 的角色寫到這台上。一個帳號可以同時綁兩種 IP 的公仔，各說各的角色；Playground 從某台進去，只列該 IP 的角色。語音伺服器讀這台自己的角色。孩子資料仍在帳號。記憶仍是（帳號、設備、ip_key），另一隻聽不到。</t>
+        </is>
+      </c>
+      <c r="L80" s="6" t="inlineStr">
+        <is>
+          <t>① 登記兩塊 MAC，分別寫入 IP-A、IP-B 和各自的預設角色。兩塊板燒的是同一份韌體。查 devices，ip_key 和 personality_id 正確。
+② 認領清單在按下認領前顯示該 IP 的名稱和 image_url；image_url 為空時用佔位圖。認領後 My Devices 卡片是這張圖，Current Character 仍是角色圖。
+③ 同一帳號再認領另一 IP 的板。兩台設備卡片各顯示自己的 IP 頭像。
+④ 用家長身份更新 devices.ip_key，被拒絕。把 personality_id 改成另一個 IP 的角色，被外鍵拒絕。
+⑤ 從 IP-A 的設備進 Playground，只看到 A 的角色，沒有換到 B 的入口。A 的板開 session，用的是 A 的角色；B 的板不受影響。
+⑥ 解綁 A 再被另一個帳號認領，ip_key 仍是 A，頭像不變。A 的記憶不會出現在 B 的 session。
+⑦ ip_key 為空的開發板仍可選任何角色，session 照現在的帳號角色走。
+⑧ 只更新韌體（OTA 或重燒 app），devices.ip_key 不變。</t>
+        </is>
+      </c>
+      <c r="M80" s="13" t="inlineStr">
+        <is>
+          <t>P0-11</t>
+        </is>
+      </c>
+      <c r="P80" s="6" t="inlineStr">
+        <is>
+          <t>[2026-10-13] 新增：2026-10-13 定案：同一個 App 裡兩種鎖死公仔是一定的。IP 在出廠登記時按 MAC 寫入，不編進韌體。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P79"/>
+  <autoFilter ref="A1:P80"/>
   <conditionalFormatting sqref="F2:F1000">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"已完成"</formula>
@@ -9151,7 +9289,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I223"/>
+  <dimension ref="A1:I227"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -16882,8 +17020,144 @@
         </is>
       </c>
     </row>
+    <row r="224" ht="32" customHeight="1">
+      <c r="A224" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-13 16:33</t>
+        </is>
+      </c>
+      <c r="B224" s="13" t="inlineStr">
+        <is>
+          <t>R-37</t>
+        </is>
+      </c>
+      <c r="C224" s="6" t="inlineStr">
+        <is>
+          <t>網頁設定玩具的 Wi-Fi：查看、新增、刪除</t>
+        </is>
+      </c>
+      <c r="D224" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E224" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F224" s="13" t="n"/>
+      <c r="G224" s="6" t="n"/>
+      <c r="H224" s="13" t="n"/>
+      <c r="I224" s="6" t="n"/>
+    </row>
+    <row r="225" ht="172" customHeight="1">
+      <c r="A225" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-13 16:33</t>
+        </is>
+      </c>
+      <c r="B225" s="13" t="inlineStr">
+        <is>
+          <t>R-37</t>
+        </is>
+      </c>
+      <c r="C225" s="6" t="inlineStr">
+        <is>
+          <t>網頁設定玩具的 Wi-Fi：查看、新增、刪除</t>
+        </is>
+      </c>
+      <c r="D225" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="E225" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F225" s="13" t="inlineStr">
+        <is>
+          <t>部分通過</t>
+        </is>
+      </c>
+      <c r="G225" s="6" t="inlineStr">
+        <is>
+          <t>模擬玩具經本機語音服務器＋網頁：status/scan/add/delete 正常；刪除目前 Wi-Fi → current 被拒；斷線 5 秒內頁面顯示睡著、按鈕停用；測試密碼在語音服務器日誌、網頁服務器日誌、資料庫均搜不到；用別人裝置 ID 重放 server action → forbidden；pytest 17 項通過（全套 230）；韌體 spotpear-ai-toy-localall 編譯通過（RAM 17.5%、Flash 75.9%）。未測：真機 ①② 及 OTA 推出</t>
+        </is>
+      </c>
+      <c r="H225" s="13" t="n"/>
+      <c r="I225" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-13 應 Jacky 要求從 W4 提前開始。韌體：上限 8 個、NVS apOk%d 記錄連過、經 /ws/esp32 收 status/add/delete/scan、不刪不改目前 Wi-Fi、Wi-Fi 指令不印串口、修 delWifi 計數 bug。伺服器：device_wifi.py＋/internal/device_wifi（含 peek），密碼只轉送不留存。網頁：我 &gt; 裝置 &gt; Network &gt; Wi-Fi（Figma C4），deviceWifiAction 檢查擁有者。剩真機測試 ①②（需 62:70 刷 -localall＋兩個真實網絡）與 OTA。</t>
+        </is>
+      </c>
+    </row>
+    <row r="226" ht="32" customHeight="1">
+      <c r="A226" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-13 19:05</t>
+        </is>
+      </c>
+      <c r="B226" s="13" t="inlineStr">
+        <is>
+          <t>R-38</t>
+        </is>
+      </c>
+      <c r="C226" s="6" t="inlineStr">
+        <is>
+          <t>公仔出廠鎖死所屬 IP，綁定時顯示該 IP 頭像</t>
+        </is>
+      </c>
+      <c r="E226" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="I226" s="6" t="inlineStr">
+        <is>
+          <t>新增任務</t>
+        </is>
+      </c>
+    </row>
+    <row r="227" ht="74" customHeight="1">
+      <c r="A227" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-13 19:06</t>
+        </is>
+      </c>
+      <c r="B227" s="13" t="inlineStr">
+        <is>
+          <t>R-10</t>
+        </is>
+      </c>
+      <c r="C227" s="6" t="inlineStr">
+        <is>
+          <t>出廠流程</t>
+        </is>
+      </c>
+      <c r="D227" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E227" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="F227" s="13" t="n"/>
+      <c r="G227" s="6" t="n"/>
+      <c r="H227" s="13" t="n"/>
+      <c r="I227" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-13：工位登記要寫入該公仔的 ip_key 和預設角色（R-38）。IP 不編進共用韌體。；修改了驗收標準、測試方法、依賴→P0-06, P0-14, R-01, P2-12, Q10, R-34, R-35, R-38</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I223"/>
+  <autoFilter ref="A1:I227"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record the fixed partition table and the UAT decision (P2-12).
UAT is the existing elatoai.hkqft.com stack until the two brand stacks
exist; P2-12 and R-10 carry the test results and the extra factory step.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/production-readiness.xlsx
+++ b/docs/production-readiness.xlsx
@@ -13,9 +13,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="更新記錄" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'任務清單'!$A$1:$P$80</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'任務清單'!$A$1:$P$88</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'待確認問題'!$A$1:$G$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$227</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$253</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -641,7 +641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I92"/>
+  <dimension ref="A1:I103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -665,14 +665,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>最後更新：2026-10-13 19:06　·　本頁由 tracker.py 自動生成，請勿手動編輯</t>
+          <t>最後更新：2026-10-14 11:03　·　本頁由 tracker.py 自動生成，請勿手動編輯</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>總進度：17/76 已完成（22%）　·　目前階段：1 止血定案（10/5–10/16）</t>
+          <t>總進度：17/83 已完成（20%）　·　目前階段：1 止血定案（10/5–10/16）</t>
         </is>
       </c>
     </row>
@@ -776,7 +776,7 @@
       </c>
       <c r="C7" s="7">
         <f>COUNTIF('任務清單'!$B:$B,$A7)</f>
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D7" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A7,'任務清單'!$F:$F,D$5)</f>
@@ -784,7 +784,7 @@
       </c>
       <c r="E7" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A7,'任務清單'!$F:$F,E$5)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F7" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A7,'任務清單'!$F:$F,F$5)</f>
@@ -796,7 +796,7 @@
       </c>
       <c r="H7" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A7,'任務清單'!$F:$F,H$5)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I7" s="8">
         <f>IFERROR(F7/(C7-H7),0)</f>
@@ -816,15 +816,15 @@
       </c>
       <c r="C8" s="7">
         <f>COUNTIF('任務清單'!$B:$B,$A8)</f>
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="D8" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A8,'任務清單'!$F:$F,D$5)</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E8" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A8,'任務清單'!$F:$F,E$5)</f>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F8" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A8,'任務清單'!$F:$F,F$5)</f>
@@ -840,7 +840,7 @@
       </c>
       <c r="I8" s="8">
         <f>IFERROR(F8/(C8-H8),0)</f>
-        <v>0.25</v>
+        <v>0.1875</v>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1">
@@ -856,11 +856,11 @@
       </c>
       <c r="C9" s="7">
         <f>COUNTIF('任務清單'!$B:$B,$A9)</f>
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D9" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A9,'任務清單'!$F:$F,D$5)</f>
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E9" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A9,'任務清單'!$F:$F,E$5)</f>
@@ -880,7 +880,7 @@
       </c>
       <c r="I9" s="8">
         <f>IFERROR(F9/(C9-H9),0)</f>
-        <v>0.027777777777777776</v>
+        <v>0.02631578947368421</v>
       </c>
     </row>
     <row r="10">
@@ -892,15 +892,15 @@
       <c r="B10" s="6" t="n"/>
       <c r="C10" s="5">
         <f>SUM(C6:C9)</f>
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="D10" s="5">
         <f>SUM(D6:D9)</f>
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="E10" s="5">
         <f>SUM(E6:E9)</f>
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="F10" s="5">
         <f>SUM(F6:F9)</f>
@@ -912,11 +912,11 @@
       </c>
       <c r="H10" s="5">
         <f>SUM(H6:H9)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I10" s="9">
         <f>IFERROR(F10/(C10-H10),0)</f>
-        <v>0.2236842105263158</v>
+        <v>0.20481927710843373</v>
       </c>
     </row>
     <row r="12">
@@ -1019,15 +1019,15 @@
       </c>
       <c r="C14" s="7">
         <f>COUNTIF('任務清單'!$C:$C,$A14)</f>
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="D14" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A14,'任務清單'!$F:$F,D$12)</f>
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E14" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A14,'任務清單'!$F:$F,E$12)</f>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F14" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A14,'任務清單'!$F:$F,F$12)</f>
@@ -1039,11 +1039,11 @@
       </c>
       <c r="H14" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A14,'任務清單'!$F:$F,H$12)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I14" s="8">
         <f>IFERROR(F14/(C14-H14),0)</f>
-        <v>0.08333333333333333</v>
+        <v>0.07692307692307693</v>
       </c>
     </row>
     <row r="15" ht="46" customHeight="1">
@@ -1059,15 +1059,15 @@
       </c>
       <c r="C15" s="7">
         <f>COUNTIF('任務清單'!$C:$C,$A15)</f>
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="D15" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A15,'任務清單'!$F:$F,D$12)</f>
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E15" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A15,'任務清單'!$F:$F,E$12)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F15" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A15,'任務清單'!$F:$F,F$12)</f>
@@ -1099,11 +1099,11 @@
       </c>
       <c r="C16" s="7">
         <f>COUNTIF('任務清單'!$C:$C,$A16)</f>
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D16" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A16,'任務清單'!$F:$F,D$12)</f>
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E16" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A16,'任務清單'!$F:$F,E$12)</f>
@@ -1135,15 +1135,15 @@
       <c r="B17" s="6" t="n"/>
       <c r="C17" s="5">
         <f>SUM(C13:C16)</f>
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="D17" s="5">
         <f>SUM(D13:D16)</f>
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="E17" s="5">
         <f>SUM(E13:E16)</f>
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="F17" s="5">
         <f>SUM(F13:F16)</f>
@@ -1155,11 +1155,11 @@
       </c>
       <c r="H17" s="5">
         <f>SUM(H13:H16)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I17" s="9">
         <f>IFERROR(F17/(C17-H17),0)</f>
-        <v>0.2236842105263158</v>
+        <v>0.20481927710843373</v>
       </c>
     </row>
     <row r="19">
@@ -1358,15 +1358,15 @@
       <c r="H25" s="11" t="n"/>
       <c r="I25" s="12" t="n"/>
     </row>
-    <row r="26" ht="409" customHeight="1">
+    <row r="26" ht="60" customHeight="1">
       <c r="A26" s="13" t="inlineStr">
         <is>
-          <t>P1-12</t>
+          <t>P1-10</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>設備解綁時的記憶處理：確認、預設保留、可選清除</t>
+          <t>管理操作審計記錄</t>
         </is>
       </c>
       <c r="C26" s="13" t="inlineStr">
@@ -1381,8 +1381,7 @@
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
-          <t>上次測試：部分通過 — 本機（開發板 DEV636 身份的模擬裝置 + 網頁）：TC1/2/5/6/7/8/10/11/13 通過；TC3 重綁後 log『Loaded 2 fact(s)』；TC4 第二台 starts cold、設定頁可切換；TC9 DB 層 B 解綁回 NULL、清除報錯，anon/authenticated 無 EXECUTE；TC10 舊代數寫入三表皆 HTTP 400、清除後 40 秒仍 0 行；TC12 伺服器端 4401 通過；pytest 214 passed。TC14（2026-10-12，rebase 到 main 後的 p1-12-rebased 8d4b9e2，本機 7861）：/ws/nextjs 以網頁 token 對話兩輪，波波熊有回應 → turn_metrics 0→3，memory_facts／memory_segments／conversations 皆 0→0；log 只有 NextJS websocket connected。真機 62:70（2026-10-12，localall 測試版 → 本機 7861/3014，p1-12-rebased）：按住 BOOT 對話 6 輪，conversations 記下『我隻狗叫豆豆…』；TC12：介面解綁（不勾清除）→ 16:06:51 即斷線，之後每次重連都在 auth 前被拒（device token refused），16:07:02 重新取 token 得 202 並顯示配對碼 UKDM7N；facts 1→1、conversations 14→14、segments 1→2（結束時的摘要）、revision 0。TC3：同帳號重綁 → log『Loaded 1 fact(s)』（有一隻3歲嘅狗叫豆豆）＋2 段摘要；真機問『我隻狗叫咩名』的回答未記錄（用戶決定直接部署）。發現：韌體拿到 202 後 websocket 仍每秒重連一次直到被認領，沒有真正停在配對狀態（不屬 P1-12 伺服器端，另開任務）。
-① 按「解綁」先彈出確認對話框，取消則什麼都不改。② 對話框預設保留記憶；「同時清除記憶」要主動勾選，並寫明無法復原。③ 記憶跟設備：鍵是 (user_id, device_id, ip_key)。同一帳號的每台設備各自一份記憶；保留時，同帳號重綁同一台會接著用；換新設備從空白開始（搬記憶交給 R-11）。④ 清除在伺服器端一個交易完成：先刪該設備的 memory_facts、memory_segments、conversations（連帳號的舊 memories），再解綁；任何一步失敗就不解綁，並顯示錯誤。⑤ 其他帳號認領同一台設備，看不到舊記憶（靠 user_id 隔離，不靠刪除成功）。⑥ 設定頁按設備顯示記憶；「清除全部」只清所選設備，連 conversations 一起刪。⑦ 對話中清除，之後的寫入和 consolidation 不會把記憶寫回（devices.memories_revision + trigger）。⑧ 未認領的設備不能對話：/ws/esp32 查到設備沒有 user_id 就在 auth 前以 4401 關閉，即使 24 小時 token 未過期；韌體重新取 token 拿到 202，回到配對狀態。⑨ 解綁時立即中斷該設備正在進行的語音 session。⑩ 網頁語音（playground）沒有設備，不讀也不寫記憶。</t>
+          <t>每個管理操作寫一筆記錄：誰、什麼時間、什麼操作、對象、改之前與改之後的值；記錄只能新增，任何人（包括超級管理員）都不能修改或刪除；超級管理員能在管理端查看。</t>
         </is>
       </c>
       <c r="F26" s="11" t="n"/>
@@ -1390,15 +1389,15 @@
       <c r="H26" s="11" t="n"/>
       <c r="I26" s="12" t="n"/>
     </row>
-    <row r="27" ht="200" customHeight="1">
+    <row r="27" ht="409" customHeight="1">
       <c r="A27" s="13" t="inlineStr">
         <is>
-          <t>R-21</t>
+          <t>P1-12</t>
         </is>
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>藍牙配網與綁定（取代熱點配網）</t>
+          <t>設備解綁時的記憶處理：確認、預設保留、可選清除</t>
         </is>
       </c>
       <c r="C27" s="13" t="inlineStr">
@@ -1413,7 +1412,8 @@
       </c>
       <c r="E27" s="6" t="inlineStr">
         <is>
-          <t>① 設備在「未配網、Wi-Fi 連不上、未綁定、長按 BOOT」時以 AIBuddy-XXXX 名稱廣播藍牙，廣播資料帶品牌，品牌 App 只列出自己品牌的設備。② 設備經藍牙回傳它掃描到的 2.4GHz Wi-Fi 清單，App 讓用戶選擇並填密碼。③ App 經藍牙把 SSID、密碼和綁定票（P0-11）一起交給設備；藍牙通道加密（ESP 標準配網協定 security 1/2 或同等）。④ 設備連上 Wi-Fi 後自己完成認領，App 顯示綁定成功或失敗原因（密碼錯、設備已有主人、票過期）。⑤ 配網期間不啟動音訊；完成後釋放藍牙記憶體再開語音（必要時重開機），對話中最低 heap 不比現在差。⑥ 解綁在 App 內完成（P1-12），解綁後設備進入藍牙待綁定狀態。⑦ SoftAP 熱點配網保留給開發和運維（隱藏觸發方式或編譯開關），量產用戶流程不出現。</t>
+          <t>上次測試：部分通過 — 本機（開發板 DEV636 身份的模擬裝置 + 網頁）：TC1/2/5/6/7/8/10/11/13 通過；TC3 重綁後 log『Loaded 2 fact(s)』；TC4 第二台 starts cold、設定頁可切換；TC9 DB 層 B 解綁回 NULL、清除報錯，anon/authenticated 無 EXECUTE；TC10 舊代數寫入三表皆 HTTP 400、清除後 40 秒仍 0 行；TC12 伺服器端 4401 通過；pytest 214 passed。TC14（2026-10-12，rebase 到 main 後的 p1-12-rebased 8d4b9e2，本機 7861）：/ws/nextjs 以網頁 token 對話兩輪，波波熊有回應 → turn_metrics 0→3，memory_facts／memory_segments／conversations 皆 0→0；log 只有 NextJS websocket connected。真機 62:70（2026-10-12，localall 測試版 → 本機 7861/3014，p1-12-rebased）：按住 BOOT 對話 6 輪，conversations 記下『我隻狗叫豆豆…』；TC12：介面解綁（不勾清除）→ 16:06:51 即斷線，之後每次重連都在 auth 前被拒（device token refused），16:07:02 重新取 token 得 202 並顯示配對碼 UKDM7N；facts 1→1、conversations 14→14、segments 1→2（結束時的摘要）、revision 0。TC3：同帳號重綁 → log『Loaded 1 fact(s)』（有一隻3歲嘅狗叫豆豆）＋2 段摘要；真機問『我隻狗叫咩名』的回答未記錄（用戶決定直接部署）。發現：韌體拿到 202 後 websocket 仍每秒重連一次直到被認領，沒有真正停在配對狀態（不屬 P1-12 伺服器端，另開任務）。
+① 按「解綁」先彈出確認對話框，取消則什麼都不改。② 對話框預設保留記憶；「同時清除記憶」要主動勾選，並寫明無法復原。③ 記憶跟設備：鍵是 (user_id, device_id, ip_key)。同一帳號的每台設備各自一份記憶；保留時，同帳號重綁同一台會接著用；換新設備從空白開始（搬記憶交給 R-11）。④ 清除在伺服器端一個交易完成：先刪該設備的 memory_facts、memory_segments、conversations（連帳號的舊 memories），再解綁；任何一步失敗就不解綁，並顯示錯誤。⑤ 其他帳號認領同一台設備，看不到舊記憶（靠 user_id 隔離，不靠刪除成功）。⑥ 設定頁按設備顯示記憶；「清除全部」只清所選設備，連 conversations 一起刪。⑦ 對話中清除，之後的寫入和 consolidation 不會把記憶寫回（devices.memories_revision + trigger）。⑧ 未認領的設備不能對話：/ws/esp32 查到設備沒有 user_id 就在 auth 前以 4401 關閉，即使 24 小時 token 未過期；韌體重新取 token 拿到 202，回到配對狀態。⑨ 解綁時立即中斷該設備正在進行的語音 session。⑩ 網頁語音（playground）沒有設備，不讀也不寫記憶。</t>
         </is>
       </c>
       <c r="F27" s="11" t="n"/>
@@ -1421,15 +1421,15 @@
       <c r="H27" s="11" t="n"/>
       <c r="I27" s="12" t="n"/>
     </row>
-    <row r="28" ht="116" customHeight="1">
+    <row r="28" ht="32" customHeight="1">
       <c r="A28" s="13" t="inlineStr">
         <is>
-          <t>R-36</t>
+          <t>P2-09</t>
         </is>
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>未認領的設備停在配對狀態，不再每秒重連 websocket</t>
+          <t>每台設備成本監控</t>
         </is>
       </c>
       <c r="C28" s="13" t="inlineStr">
@@ -1444,7 +1444,7 @@
       </c>
       <c r="E28" s="6" t="inlineStr">
         <is>
-          <t>① 拿到 202 或 websocket 被 4401 拒絕後，設備停掉 websocket 自動重連，進入待綁定狀態（燈號可分辨）。② 待綁定時只按退避（5 秒起、上限 PROVISION_BACKOFF_MAX）呼叫 generate_auth_token，不開 websocket。③ 被認領後下一次輪詢拿到 200，在 10 秒內（加退避）自動開 websocket 並能對話，不用重開機。④ 已綁定設備網絡斷線重連的行為不變。⑤ 隨 OTA 推出。</t>
+          <t>每個 session 記錄 STT 秒數、LLM token、TTS 字數並換算成本；admin 頁顯示每台設備的月成本。</t>
         </is>
       </c>
       <c r="F28" s="11" t="n"/>
@@ -1452,20 +1452,20 @@
       <c r="H28" s="11" t="n"/>
       <c r="I28" s="12" t="n"/>
     </row>
-    <row r="29" ht="242" customHeight="1">
+    <row r="29" ht="172" customHeight="1">
       <c r="A29" s="13" t="inlineStr">
         <is>
-          <t>R-37</t>
+          <t>P2-13</t>
         </is>
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>網頁設定玩具的 Wi-Fi：查看、新增、刪除</t>
+          <t>Admin 後台改成分組側欄（新頁面先用示例數據預覽）</t>
         </is>
       </c>
       <c r="C29" s="13" t="inlineStr">
         <is>
-          <t>3 封閉內測</t>
+          <t>2 內測準備</t>
         </is>
       </c>
       <c r="D29" s="13" t="inlineStr">
@@ -1475,8 +1475,8 @@
       </c>
       <c r="E29" s="6" t="inlineStr">
         <is>
-          <t>上次測試：部分通過 — 模擬玩具經本機語音服務器＋網頁：status/scan/add/delete 正常；刪除目前 Wi-Fi → current 被拒；斷線 5 秒內頁面顯示睡著、按鈕停用；測試密碼在語音服務器日誌、網頁服務器日誌、資料庫均搜不到；用別人裝置 ID 重放 server action → forbidden；pytest 17 項通過（全套 230）；韌體 spotpear-ai-toy-localall 編譯通過（RAM 17.5%、Flash 75.9%）。未測：真機 ①② 及 OTA 推出
-① 設定頁顯示玩具在線／離線、目前 Wi-Fi 和訊號、已記住的 Wi-Fi 清單（只有名稱，不顯示密碼）② 在線時可新增 Wi-Fi（輸入或從玩具掃描到的清單選）、刪除 Wi-Fi；不能刪除正在使用的那個 ③ 經 /ws/esp32 轉送：伺服器先確認是設備主人；密碼不寫入資料庫、不寫入日誌 ④ 新增不切換網絡，目前 Wi-Fi 消失時才按訊號選；清單標示「連過／未連過」⑤ 上限 8 個 ⑥ 韌體改動經 OTA 推出</t>
+          <t>上次測試：部分通過 — ① tsc --noEmit 通過 ② 略過登入的測試頁（另一份副本、獨立 .next）：超級管理員 15 頁、內容管理員只見 Characters／IPs；1360px 與 375px 均無橫向捲動（scrollWidth=clientWidth=375）；#audit 直接打開正確；③④ 未做：需真實帳號登入 /admin
+6 個現有分頁（Model、Latency、Characters、IPs、Accounts、Admins）在新側欄照常使用，讀寫真實數據；內容管理員只看到 Characters 和 IPs；預覽頁和規劃頁只有超級管理員看到，並有橫幅寫明示例數據、按鈕不能用；每頁有 #hash 可直接打開；手機寬度沒有橫向捲動。</t>
         </is>
       </c>
       <c r="F29" s="11" t="n"/>
@@ -1484,15 +1484,15 @@
       <c r="H29" s="11" t="n"/>
       <c r="I29" s="12" t="n"/>
     </row>
-    <row r="30" ht="60" customHeight="1">
+    <row r="30" ht="200" customHeight="1">
       <c r="A30" s="13" t="inlineStr">
         <is>
-          <t>P1-01</t>
+          <t>R-21</t>
         </is>
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>加入內容審核層（輸入與輸出）</t>
+          <t>藍牙配網與綁定（取代熱點配網）</t>
         </is>
       </c>
       <c r="C30" s="13" t="inlineStr">
@@ -1502,12 +1502,12 @@
       </c>
       <c r="D30" s="13" t="inlineStr">
         <is>
-          <t>未開始</t>
+          <t>進行中</t>
         </is>
       </c>
       <c r="E30" s="6" t="inlineStr">
         <is>
-          <t>STT 文字與 LLM 輸出都經審核，尺度按 3–6 歲；命中時換成安全回覆並記錄事件，事件只記類別、時間、角色，不記原文（管理員不能看兒童內容，見 Q7）；首字延遲增加 ≤150ms。</t>
+          <t>① 設備在「未配網、Wi-Fi 連不上、未綁定、長按 BOOT」時以 AIBuddy-XXXX 名稱廣播藍牙，廣播資料帶品牌，品牌 App 只列出自己品牌的設備。② 設備經藍牙回傳它掃描到的 2.4GHz Wi-Fi 清單，App 讓用戶選擇並填密碼。③ App 經藍牙把 SSID、密碼和綁定票（P0-11）一起交給設備；藍牙通道加密（ESP 標準配網協定 security 1/2 或同等）。④ 設備連上 Wi-Fi 後自己完成認領，App 顯示綁定成功或失敗原因（密碼錯、設備已有主人、票過期）。⑤ 配網期間不啟動音訊；完成後釋放藍牙記憶體再開語音（必要時重開機），對話中最低 heap 不比現在差。⑥ 解綁在 App 內完成（P1-12），解綁後設備進入藍牙待綁定狀態。⑦ SoftAP 熱點配網保留給開發和運維（隱藏觸發方式或編譯開關），量產用戶流程不出現。</t>
         </is>
       </c>
       <c r="F30" s="11" t="n"/>
@@ -1515,15 +1515,15 @@
       <c r="H30" s="11" t="n"/>
       <c r="I30" s="12" t="n"/>
     </row>
-    <row r="31" ht="32" customHeight="1">
+    <row r="31" ht="116" customHeight="1">
       <c r="A31" s="13" t="inlineStr">
         <is>
-          <t>P1-02</t>
+          <t>R-36</t>
         </is>
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>日誌移除兒童個人資料</t>
+          <t>未認領的設備停在配對狀態，不再每秒重連 websocket</t>
         </is>
       </c>
       <c r="C31" s="13" t="inlineStr">
@@ -1533,12 +1533,12 @@
       </c>
       <c r="D31" s="13" t="inlineStr">
         <is>
-          <t>未開始</t>
+          <t>進行中</t>
         </is>
       </c>
       <c r="E31" s="6" t="inlineStr">
         <is>
-          <t>生產日誌只記 ID、長度、類別，不記內容；內容只在 DEBUG 等級輸出，生產不開 DEBUG。</t>
+          <t>① 拿到 202 或 websocket 被 4401 拒絕後，設備停掉 websocket 自動重連，進入待綁定狀態（燈號可分辨）。② 待綁定時只按退避（5 秒起、上限 PROVISION_BACKOFF_MAX）呼叫 generate_auth_token，不開 websocket。③ 被認領後下一次輪詢拿到 200，在 10 秒內（加退避）自動開 websocket 並能對話，不用重開機。④ 已綁定設備網絡斷線重連的行為不變。⑤ 隨 OTA 推出。</t>
         </is>
       </c>
       <c r="F31" s="11" t="n"/>
@@ -1546,30 +1546,31 @@
       <c r="H31" s="11" t="n"/>
       <c r="I31" s="12" t="n"/>
     </row>
-    <row r="32" ht="60" customHeight="1">
+    <row r="32" ht="228" customHeight="1">
       <c r="A32" s="13" t="inlineStr">
         <is>
-          <t>P1-10</t>
+          <t>P2-12</t>
         </is>
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>管理操作審計記錄</t>
+          <t>量產燒錄前加大 app 分區</t>
         </is>
       </c>
       <c r="C32" s="13" t="inlineStr">
         <is>
-          <t>2 內測準備</t>
+          <t>3 封閉內測</t>
         </is>
       </c>
       <c r="D32" s="13" t="inlineStr">
         <is>
-          <t>未開始</t>
+          <t>進行中</t>
         </is>
       </c>
       <c r="E32" s="6" t="inlineStr">
         <is>
-          <t>每個管理操作寫一筆記錄：誰、什麼時間、什麼操作、對象、改之前與改之後的值；記錄只能新增，任何人（包括超級管理員）都不能修改或刪除；超級管理員能在管理端查看。</t>
+          <t>上次測試：部分通過 — 62:70（spotpear-ai-toy-p212 原型，現已併入 spotpear-ai-toy）：① 本機 OTA 1.6.1→1.6.2 寫入新 app1，120s 後 confirmed ② 3 秒 abort 的 1.6.3 → PANIC → 回到 1.6.2，ota_failed_version=1.6.3 ③ 崩潰寫入 coredump 14.8KB ④ 資源分區 9 個聲音 504KB/2MB，開機 CRC 63ms，OTA 後照常；損壞/清空 → 退回內建聲音無崩潰 ⑤ pio 全部 18 個 env 編譯通過，映像都在各自 app 槽內（Spotpear 4 個 1.59–1.60MB / 4MB；其他板仍 2MB 槽）；R-21 藍牙探針版 2,326,128 bytes &lt; 4MB ⑥ release_firmware.py 映像 &gt; app 槽即拒發。未做：雲端 OTA 一次（等上 UAT）、出廠腳本寫入資源包（R-10）
+新分區表（例如 app0/app1 各 4MB，保留 nvs/otadata 位置）在出廠前定案並寫入出廠腳本；OTA 與回滾在新分區表上照常</t>
         </is>
       </c>
       <c r="F32" s="11" t="n"/>
@@ -1577,30 +1578,31 @@
       <c r="H32" s="11" t="n"/>
       <c r="I32" s="12" t="n"/>
     </row>
-    <row r="33" ht="46" customHeight="1">
+    <row r="33" ht="242" customHeight="1">
       <c r="A33" s="13" t="inlineStr">
         <is>
-          <t>P1-11</t>
+          <t>R-37</t>
         </is>
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>伺服器與資料庫直接存取的管控</t>
+          <t>網頁設定玩具的 Wi-Fi：查看、新增、刪除</t>
         </is>
       </c>
       <c r="C33" s="13" t="inlineStr">
         <is>
-          <t>2 內測準備</t>
+          <t>3 封閉內測</t>
         </is>
       </c>
       <c r="D33" s="13" t="inlineStr">
         <is>
-          <t>未開始</t>
+          <t>進行中</t>
         </is>
       </c>
       <c r="E33" s="6" t="inlineStr">
         <is>
-          <t>列出誰有 SSH 與資料庫直連權限（越少越好）；service_role key 只存在伺服器的 env；私隱政策寫明這類存取的範圍；每次直接查看生產資料都留記錄。</t>
+          <t>上次測試：部分通過 — 模擬玩具經本機語音服務器＋網頁：status/scan/add/delete 正常；刪除目前 Wi-Fi → current 被拒；斷線 5 秒內頁面顯示睡著、按鈕停用；測試密碼在語音服務器日誌、網頁服務器日誌、資料庫均搜不到；用別人裝置 ID 重放 server action → forbidden；pytest 17 項通過（全套 230）；韌體 spotpear-ai-toy-localall 編譯通過（RAM 17.5%、Flash 75.9%）。未測：真機 ①② 及 OTA 推出
+① 設定頁顯示玩具在線／離線、目前 Wi-Fi 和訊號、已記住的 Wi-Fi 清單（只有名稱，不顯示密碼）② 在線時可新增 Wi-Fi（輸入或從玩具掃描到的清單選）、刪除 Wi-Fi；不能刪除正在使用的那個 ③ 經 /ws/esp32 轉送：伺服器先確認是設備主人；密碼不寫入資料庫、不寫入日誌 ④ 新增不切換網絡，目前 Wi-Fi 消失時才按訊號選；清單標示「連過／未連過」⑤ 上限 8 個 ⑥ 韌體改動經 OTA 推出</t>
         </is>
       </c>
       <c r="F33" s="11" t="n"/>
@@ -1608,15 +1610,15 @@
       <c r="H33" s="11" t="n"/>
       <c r="I33" s="12" t="n"/>
     </row>
-    <row r="34" ht="46" customHeight="1">
+    <row r="34" ht="60" customHeight="1">
       <c r="A34" s="13" t="inlineStr">
         <is>
-          <t>P2-02</t>
+          <t>P1-01</t>
         </is>
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>CI 跑測試與靜態檢查</t>
+          <t>加入內容審核層（輸入與輸出）</t>
         </is>
       </c>
       <c r="C34" s="13" t="inlineStr">
@@ -1631,7 +1633,7 @@
       </c>
       <c r="E34" s="6" t="inlineStr">
         <is>
-          <t>推送與 PR 時跑 pytest、ruff、pyright、next lint、tsc --noEmit、pio run；任何一項失敗就不發佈 image。</t>
+          <t>STT 文字與 LLM 輸出都經審核，尺度按 3–6 歲；命中時換成安全回覆並記錄事件，事件只記類別、時間、角色，不記原文（管理員不能看兒童內容，見 Q7）；首字延遲增加 ≤150ms。</t>
         </is>
       </c>
       <c r="F34" s="11" t="n"/>
@@ -1642,12 +1644,12 @@
     <row r="35" ht="32" customHeight="1">
       <c r="A35" s="13" t="inlineStr">
         <is>
-          <t>P2-04</t>
+          <t>P1-02</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>容器改用非 root 用戶</t>
+          <t>日誌移除兒童個人資料</t>
         </is>
       </c>
       <c r="C35" s="13" t="inlineStr">
@@ -1662,7 +1664,7 @@
       </c>
       <c r="E35" s="6" t="inlineStr">
         <is>
-          <t>兩個 Dockerfile 都設定非 root 的 USER。</t>
+          <t>生產日誌只記 ID、長度、類別，不記內容；內容只在 DEBUG 等級輸出，生產不開 DEBUG。</t>
         </is>
       </c>
       <c r="F35" s="11" t="n"/>
@@ -1670,37 +1672,92 @@
       <c r="H35" s="11" t="n"/>
       <c r="I35" s="12" t="n"/>
     </row>
-    <row r="37">
-      <c r="A37" s="10" t="inlineStr">
-        <is>
-          <t>✅ 最近完成與測試效果</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="4" t="inlineStr">
-        <is>
-          <t>編號</t>
-        </is>
-      </c>
-      <c r="B38" s="4" t="inlineStr">
-        <is>
-          <t>任務</t>
-        </is>
-      </c>
-      <c r="C38" s="4" t="inlineStr">
-        <is>
-          <t>測試結果</t>
-        </is>
-      </c>
-      <c r="D38" s="4" t="inlineStr">
-        <is>
-          <t>完成日期</t>
-        </is>
-      </c>
-      <c r="E38" s="4" t="inlineStr">
-        <is>
-          <t>測試證據</t>
+    <row r="36" ht="46" customHeight="1">
+      <c r="A36" s="13" t="inlineStr">
+        <is>
+          <t>P1-11</t>
+        </is>
+      </c>
+      <c r="B36" s="6" t="inlineStr">
+        <is>
+          <t>伺服器與資料庫直接存取的管控</t>
+        </is>
+      </c>
+      <c r="C36" s="13" t="inlineStr">
+        <is>
+          <t>2 內測準備</t>
+        </is>
+      </c>
+      <c r="D36" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E36" s="6" t="inlineStr">
+        <is>
+          <t>列出誰有 SSH 與資料庫直連權限（越少越好）；service_role key 只存在伺服器的 env；私隱政策寫明這類存取的範圍；每次直接查看生產資料都留記錄。</t>
+        </is>
+      </c>
+      <c r="F36" s="11" t="n"/>
+      <c r="G36" s="11" t="n"/>
+      <c r="H36" s="11" t="n"/>
+      <c r="I36" s="12" t="n"/>
+    </row>
+    <row r="37" ht="46" customHeight="1">
+      <c r="A37" s="13" t="inlineStr">
+        <is>
+          <t>P2-02</t>
+        </is>
+      </c>
+      <c r="B37" s="6" t="inlineStr">
+        <is>
+          <t>CI 跑測試與靜態檢查</t>
+        </is>
+      </c>
+      <c r="C37" s="13" t="inlineStr">
+        <is>
+          <t>2 內測準備</t>
+        </is>
+      </c>
+      <c r="D37" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E37" s="6" t="inlineStr">
+        <is>
+          <t>推送與 PR 時跑 pytest、ruff、pyright、next lint、tsc --noEmit、pio run；任何一項失敗就不發佈 image。</t>
+        </is>
+      </c>
+      <c r="F37" s="11" t="n"/>
+      <c r="G37" s="11" t="n"/>
+      <c r="H37" s="11" t="n"/>
+      <c r="I37" s="12" t="n"/>
+    </row>
+    <row r="38" ht="32" customHeight="1">
+      <c r="A38" s="13" t="inlineStr">
+        <is>
+          <t>P2-04</t>
+        </is>
+      </c>
+      <c r="B38" s="6" t="inlineStr">
+        <is>
+          <t>容器改用非 root 用戶</t>
+        </is>
+      </c>
+      <c r="C38" s="13" t="inlineStr">
+        <is>
+          <t>2 內測準備</t>
+        </is>
+      </c>
+      <c r="D38" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E38" s="6" t="inlineStr">
+        <is>
+          <t>兩個 Dockerfile 都設定非 root 的 USER。</t>
         </is>
       </c>
       <c r="F38" s="11" t="n"/>
@@ -1708,30 +1765,30 @@
       <c r="H38" s="11" t="n"/>
       <c r="I38" s="12" t="n"/>
     </row>
-    <row r="39" ht="102" customHeight="1">
+    <row r="39" ht="46" customHeight="1">
       <c r="A39" s="13" t="inlineStr">
         <is>
-          <t>P0-12</t>
+          <t>R-04</t>
         </is>
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>收緊 Admin 權限與路由保護</t>
+          <t>粵語質量評測</t>
         </is>
       </c>
       <c r="C39" s="13" t="inlineStr">
         <is>
-          <t>通過</t>
+          <t>2 內測準備</t>
         </is>
       </c>
       <c r="D39" s="13" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>未開始</t>
         </is>
       </c>
       <c r="E39" s="6" t="inlineStr">
         <is>
-          <t>線上 2026-10-12（bac24e9）：runbook 10/08 檢查 未登入 /admin→/login、/api/admin→401、has_role() 只看角色、無管理員 policy 觸及 conversations/記憶表、超管≥1；未登入 /home、/admin→/login；用戶確認：家長帳號開 /admin 轉回 /home、管理員在 /admin 修改角色保存成功；角色細分權限沿用本機 61/61</t>
+          <t>有一套粵語評測集（兒童錄音＋文字提示）；選定的 STT 與 LLM 達到門檻：兒童語音字錯率 ≤15%、口語粵語回覆 ≥90%、中英夾雜句能正確理解。</t>
         </is>
       </c>
       <c r="F39" s="11" t="n"/>
@@ -1739,92 +1796,37 @@
       <c r="H39" s="11" t="n"/>
       <c r="I39" s="12" t="n"/>
     </row>
-    <row r="40" ht="88" customHeight="1">
-      <c r="A40" s="13" t="inlineStr">
-        <is>
-          <t>P0-15</t>
-        </is>
-      </c>
-      <c r="B40" s="6" t="inlineStr">
-        <is>
-          <t>角色表權限：只有內容管理員能發佈，關閉家長自建角色</t>
-        </is>
-      </c>
-      <c r="C40" s="13" t="inlineStr">
-        <is>
-          <t>通過</t>
-        </is>
-      </c>
-      <c r="D40" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-12</t>
-        </is>
-      </c>
-      <c r="E40" s="6" t="inlineStr">
-        <is>
-          <t>線上 2026-10-12：② anon 只見 6 個已發佈 hk_ 內建，查隱藏/醫生/家長自建 → []，anon POST → 401；① authenticated 寫入權限由 20261007140000 REVOKE（runbook 10/08 已套用）；用戶確認：④ 家長登入後 /home/create 轉回 /home ③ 管理員在 /admin 修改角色保存成功</t>
-        </is>
-      </c>
-      <c r="F40" s="11" t="n"/>
-      <c r="G40" s="11" t="n"/>
-      <c r="H40" s="11" t="n"/>
-      <c r="I40" s="12" t="n"/>
-    </row>
-    <row r="41" ht="88" customHeight="1">
-      <c r="A41" s="13" t="inlineStr">
-        <is>
-          <t>P0-16</t>
-        </is>
-      </c>
-      <c r="B41" s="6" t="inlineStr">
-        <is>
-          <t>移除「醫生」身份與寫死的通關碼</t>
-        </is>
-      </c>
-      <c r="C41" s="13" t="inlineStr">
-        <is>
-          <t>通過</t>
-        </is>
-      </c>
-      <c r="D41" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-12</t>
-        </is>
-      </c>
-      <c r="E41" s="6" t="inlineStr">
-        <is>
-          <t>線上 2026-10-12：生產 commit bac24e9 git grep checkDoctorAction/kiwi-subtle-emu/=== "doctor"/isDoctor → 0；線上 13 個 JS（/、/login、/onboard）grep 通關碼/"doctor"/Santa/patient → 0；anon 讀角色只見 6 個 hk_ 角色、is_doctor 全 false；用戶今日線上登入及 playground 正常</t>
-        </is>
-      </c>
-      <c r="F41" s="11" t="n"/>
-      <c r="G41" s="11" t="n"/>
-      <c r="H41" s="11" t="n"/>
-      <c r="I41" s="12" t="n"/>
-    </row>
-    <row r="42" ht="60" customHeight="1">
-      <c r="A42" s="13" t="inlineStr">
-        <is>
-          <t>P0-09</t>
-        </is>
-      </c>
-      <c r="B42" s="6" t="inlineStr">
-        <is>
-          <t>瀏覽器語音路由改用簽名 token（/ws/nextjs）</t>
-        </is>
-      </c>
-      <c r="C42" s="13" t="inlineStr">
-        <is>
-          <t>通過</t>
-        </is>
-      </c>
-      <c r="D42" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-12</t>
-        </is>
-      </c>
-      <c r="E42" s="6" t="inlineStr">
-        <is>
-          <t>線上 2026-10-12（bac24e9）：wss /fastapi/ws/nextjs 只帶 user_id 或 token=bogus → 4401；用戶確認：登入 elatoai.hkqft.com 後網頁 playground 可正常對話</t>
+    <row r="41">
+      <c r="A41" s="10" t="inlineStr">
+        <is>
+          <t>✅ 最近完成與測試效果</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>編號</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>任務</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>測試結果</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>完成日期</t>
+        </is>
+      </c>
+      <c r="E42" s="4" t="inlineStr">
+        <is>
+          <t>測試證據</t>
         </is>
       </c>
       <c r="F42" s="11" t="n"/>
@@ -1832,15 +1834,15 @@
       <c r="H42" s="11" t="n"/>
       <c r="I42" s="12" t="n"/>
     </row>
-    <row r="43" ht="60" customHeight="1">
+    <row r="43" ht="102" customHeight="1">
       <c r="A43" s="13" t="inlineStr">
         <is>
-          <t>P0-17</t>
+          <t>P0-12</t>
         </is>
       </c>
       <c r="B43" s="6" t="inlineStr">
         <is>
-          <t>前端的 anon key 必須是公開 key，不可是 secret／service_role</t>
+          <t>收緊 Admin 權限與路由保護</t>
         </is>
       </c>
       <c r="C43" s="13" t="inlineStr">
@@ -1855,7 +1857,7 @@
       </c>
       <c r="E43" s="6" t="inlineStr">
         <is>
-          <t>線上 2026-10-12（bac24e9）：/login 引用的 13 個 JS + HTML 無 sb_secret_，唯一 key 為 role=anon 的 JWT；② 用該 key GET /rest/v1/users → 42501；③ 本機 10/07 已換 publishable</t>
+          <t>線上 2026-10-12（bac24e9）：runbook 10/08 檢查 未登入 /admin→/login、/api/admin→401、has_role() 只看角色、無管理員 policy 觸及 conversations/記憶表、超管≥1；未登入 /home、/admin→/login；用戶確認：家長帳號開 /admin 轉回 /home、管理員在 /admin 修改角色保存成功；角色細分權限沿用本機 61/61</t>
         </is>
       </c>
       <c r="F43" s="11" t="n"/>
@@ -1863,15 +1865,15 @@
       <c r="H43" s="11" t="n"/>
       <c r="I43" s="12" t="n"/>
     </row>
-    <row r="44" ht="46" customHeight="1">
+    <row r="44" ht="88" customHeight="1">
       <c r="A44" s="13" t="inlineStr">
         <is>
-          <t>P0-10</t>
+          <t>P0-15</t>
         </is>
       </c>
       <c r="B44" s="6" t="inlineStr">
         <is>
-          <t>生產環境關閉 /browser 測試頁與 /ws/browser</t>
+          <t>角色表權限：只有內容管理員能發佈，關閉家長自建角色</t>
         </is>
       </c>
       <c r="C44" s="13" t="inlineStr">
@@ -1886,7 +1888,7 @@
       </c>
       <c r="E44" s="6" t="inlineStr">
         <is>
-          <t>線上 2026-10-12（bac24e9）：GET /fastapi/browser 404、/fastapi/ 404、/fastapi/healthz 200、wss /fastapi/ws/browser → HTTP 403</t>
+          <t>線上 2026-10-12：② anon 只見 6 個已發佈 hk_ 內建，查隱藏/醫生/家長自建 → []，anon POST → 401；① authenticated 寫入權限由 20261007140000 REVOKE（runbook 10/08 已套用）；用戶確認：④ 家長登入後 /home/create 轉回 /home ③ 管理員在 /admin 修改角色保存成功</t>
         </is>
       </c>
       <c r="F44" s="11" t="n"/>
@@ -1894,15 +1896,15 @@
       <c r="H44" s="11" t="n"/>
       <c r="I44" s="12" t="n"/>
     </row>
-    <row r="45" ht="60" customHeight="1">
+    <row r="45" ht="88" customHeight="1">
       <c r="A45" s="13" t="inlineStr">
         <is>
-          <t>P0-08</t>
+          <t>P0-16</t>
         </is>
       </c>
       <c r="B45" s="6" t="inlineStr">
         <is>
-          <t>語音伺服器驗證設備身份（/ws/esp32）</t>
+          <t>移除「醫生」身份與寫死的通關碼</t>
         </is>
       </c>
       <c r="C45" s="13" t="inlineStr">
@@ -1917,7 +1919,7 @@
       </c>
       <c r="E45" s="6" t="inlineStr">
         <is>
-          <t>線上 2026-10-12（bac24e9）：wss /fastapi/ws/esp32 不帶 token、偽造 token＋X-Device-Mac → 均 4401 invalid device token；42:34 以有效 token 連線對話正常（P0-13 10/09）</t>
+          <t>線上 2026-10-12：生產 commit bac24e9 git grep checkDoctorAction/kiwi-subtle-emu/=== "doctor"/isDoctor → 0；線上 13 個 JS（/、/login、/onboard）grep 通關碼/"doctor"/Santa/patient → 0；anon 讀角色只見 6 個 hk_ 角色、is_doctor 全 false；用戶今日線上登入及 playground 正常</t>
         </is>
       </c>
       <c r="F45" s="11" t="n"/>
@@ -1928,12 +1930,12 @@
     <row r="46" ht="60" customHeight="1">
       <c r="A46" s="13" t="inlineStr">
         <is>
-          <t>P0-06</t>
+          <t>P0-09</t>
         </is>
       </c>
       <c r="B46" s="6" t="inlineStr">
         <is>
-          <t>停止憑 MAC 發放永久用戶 JWT</t>
+          <t>瀏覽器語音路由改用簽名 token（/ws/nextjs）</t>
         </is>
       </c>
       <c r="C46" s="13" t="inlineStr">
@@ -1948,7 +1950,7 @@
       </c>
       <c r="E46" s="6" t="inlineStr">
         <is>
-          <t>線上 2026-10-12（bac24e9）：POST /api/generate_auth_token 只帶 42:34 的 MAC → 401、帶錯誤密鑰 → 401、GET → 410；42:34 用 NVS 密鑰在線上換 token 並連上語音伺服器（P0-13 10/09 實測）</t>
+          <t>線上 2026-10-12（bac24e9）：wss /fastapi/ws/nextjs 只帶 user_id 或 token=bogus → 4401；用戶確認：登入 elatoai.hkqft.com 後網頁 playground 可正常對話</t>
         </is>
       </c>
       <c r="F46" s="11" t="n"/>
@@ -1956,31 +1958,94 @@
       <c r="H46" s="11" t="n"/>
       <c r="I46" s="12" t="n"/>
     </row>
-    <row r="48">
-      <c r="A48" s="10" t="inlineStr">
-        <is>
-          <t>⏳ 等待依賴 / ⛔ 阻塞</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="4" t="inlineStr">
-        <is>
-          <t>編號</t>
-        </is>
-      </c>
-      <c r="B49" s="4" t="inlineStr">
-        <is>
-          <t>任務</t>
-        </is>
-      </c>
-      <c r="C49" s="4" t="inlineStr">
-        <is>
-          <t>在等什麼</t>
-        </is>
-      </c>
-      <c r="D49" s="11" t="n"/>
-      <c r="E49" s="11" t="n"/>
+    <row r="47" ht="60" customHeight="1">
+      <c r="A47" s="13" t="inlineStr">
+        <is>
+          <t>P0-17</t>
+        </is>
+      </c>
+      <c r="B47" s="6" t="inlineStr">
+        <is>
+          <t>前端的 anon key 必須是公開 key，不可是 secret／service_role</t>
+        </is>
+      </c>
+      <c r="C47" s="13" t="inlineStr">
+        <is>
+          <t>通過</t>
+        </is>
+      </c>
+      <c r="D47" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="E47" s="6" t="inlineStr">
+        <is>
+          <t>線上 2026-10-12（bac24e9）：/login 引用的 13 個 JS + HTML 無 sb_secret_，唯一 key 為 role=anon 的 JWT；② 用該 key GET /rest/v1/users → 42501；③ 本機 10/07 已換 publishable</t>
+        </is>
+      </c>
+      <c r="F47" s="11" t="n"/>
+      <c r="G47" s="11" t="n"/>
+      <c r="H47" s="11" t="n"/>
+      <c r="I47" s="12" t="n"/>
+    </row>
+    <row r="48" ht="46" customHeight="1">
+      <c r="A48" s="13" t="inlineStr">
+        <is>
+          <t>P0-10</t>
+        </is>
+      </c>
+      <c r="B48" s="6" t="inlineStr">
+        <is>
+          <t>生產環境關閉 /browser 測試頁與 /ws/browser</t>
+        </is>
+      </c>
+      <c r="C48" s="13" t="inlineStr">
+        <is>
+          <t>通過</t>
+        </is>
+      </c>
+      <c r="D48" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="E48" s="6" t="inlineStr">
+        <is>
+          <t>線上 2026-10-12（bac24e9）：GET /fastapi/browser 404、/fastapi/ 404、/fastapi/healthz 200、wss /fastapi/ws/browser → HTTP 403</t>
+        </is>
+      </c>
+      <c r="F48" s="11" t="n"/>
+      <c r="G48" s="11" t="n"/>
+      <c r="H48" s="11" t="n"/>
+      <c r="I48" s="12" t="n"/>
+    </row>
+    <row r="49" ht="60" customHeight="1">
+      <c r="A49" s="13" t="inlineStr">
+        <is>
+          <t>P0-08</t>
+        </is>
+      </c>
+      <c r="B49" s="6" t="inlineStr">
+        <is>
+          <t>語音伺服器驗證設備身份（/ws/esp32）</t>
+        </is>
+      </c>
+      <c r="C49" s="13" t="inlineStr">
+        <is>
+          <t>通過</t>
+        </is>
+      </c>
+      <c r="D49" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="E49" s="6" t="inlineStr">
+        <is>
+          <t>線上 2026-10-12（bac24e9）：wss /fastapi/ws/esp32 不帶 token、偽造 token＋X-Device-Mac → 均 4401 invalid device token；42:34 以有效 token 連線對話正常（P0-13 10/09）</t>
+        </is>
+      </c>
       <c r="F49" s="11" t="n"/>
       <c r="G49" s="11" t="n"/>
       <c r="H49" s="11" t="n"/>
@@ -1989,86 +2054,55 @@
     <row r="50" ht="60" customHeight="1">
       <c r="A50" s="13" t="inlineStr">
         <is>
-          <t>R-16</t>
+          <t>P0-06</t>
         </is>
       </c>
       <c r="B50" s="6" t="inlineStr">
         <is>
-          <t>Spotpear 量產版加電池電壓檢測（GPIO0 分壓）</t>
-        </is>
-      </c>
-      <c r="C50" s="6" t="inlineStr">
-        <is>
-          <t>阻塞：[2026-10-07] 仍按 10/06 決定暫緩：等用戶做充滿再放電測試（與 R-17 同一次），看 VDD 低電提醒在關機前多久觸發；太遲或不觸發才向 Spotpear 提改板。已把分壓改板的問題一併放進給 Spotpear 的草稿，方便同一封發出</t>
-        </is>
-      </c>
-      <c r="D50" s="11" t="n"/>
-      <c r="E50" s="11" t="n"/>
+          <t>停止憑 MAC 發放永久用戶 JWT</t>
+        </is>
+      </c>
+      <c r="C50" s="13" t="inlineStr">
+        <is>
+          <t>通過</t>
+        </is>
+      </c>
+      <c r="D50" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="E50" s="6" t="inlineStr">
+        <is>
+          <t>線上 2026-10-12（bac24e9）：POST /api/generate_auth_token 只帶 42:34 的 MAC → 401、帶錯誤密鑰 → 401、GET → 410；42:34 用 NVS 密鑰在線上換 token 並連上語音伺服器（P0-13 10/09 實測）</t>
+        </is>
+      </c>
       <c r="F50" s="11" t="n"/>
       <c r="G50" s="11" t="n"/>
       <c r="H50" s="11" t="n"/>
       <c r="I50" s="12" t="n"/>
     </row>
-    <row r="51" ht="88" customHeight="1">
-      <c r="A51" s="13" t="inlineStr">
-        <is>
-          <t>R-17</t>
-        </is>
-      </c>
-      <c r="B51" s="6" t="inlineStr">
-        <is>
-          <t>Spotpear 電池耗盡時插電能否正常開機（供電路徑）</t>
-        </is>
-      </c>
-      <c r="C51" s="6" t="inlineStr">
-        <is>
-          <t>阻塞：[2026-10-08] 2026-10-08 開發板 63:64 插著 USB 時兩次無法解釋的完全斷電重開：09:13:26（崩潰循環中）、10:44:33（閒置、用戶確認沒碰）。都是 USB 先斷線再以 ESP_RST_POWERON 開機，非 brownout；斷電前 6 秒 GPIO0 讀數 99.9% 參考值，屬突然切斷而非緩降（SupplyMonitor 取樣太疏抓不到瞬間）。韌體無法造成 POWERON，指向充電芯片/電池保護/供電路徑，應一併問 Spotpear；放電實測時留意插 USB 閒置時是否也會斷電</t>
-        </is>
-      </c>
-      <c r="D51" s="11" t="n"/>
-      <c r="E51" s="11" t="n"/>
-      <c r="F51" s="11" t="n"/>
-      <c r="G51" s="11" t="n"/>
-      <c r="H51" s="11" t="n"/>
-      <c r="I51" s="12" t="n"/>
-    </row>
-    <row r="52" ht="32" customHeight="1">
-      <c r="A52" s="13" t="inlineStr">
-        <is>
-          <t>P1-09</t>
-        </is>
-      </c>
-      <c r="B52" s="6" t="inlineStr">
-        <is>
-          <t>家長鎖：孩子模式進設定要輸入 PIN</t>
-        </is>
-      </c>
-      <c r="C52" s="6" t="inlineStr">
-        <is>
-          <t>阻塞：[2026-10-13] 2026-10-13 用戶決定：AI Buddy（品牌 C）延到 1/15 之後，本項不卡 1/15 出廠；AI Buddy 啟動時再開。</t>
-        </is>
-      </c>
-      <c r="D52" s="11" t="n"/>
-      <c r="E52" s="11" t="n"/>
-      <c r="F52" s="11" t="n"/>
-      <c r="G52" s="11" t="n"/>
-      <c r="H52" s="11" t="n"/>
-      <c r="I52" s="12" t="n"/>
-    </row>
-    <row r="53" ht="32" customHeight="1">
-      <c r="A53" s="13" t="inlineStr">
-        <is>
-          <t>R-12</t>
-        </is>
-      </c>
-      <c r="B53" s="6" t="inlineStr">
-        <is>
-          <t>家長控制：每日使用上限和休息時段</t>
-        </is>
-      </c>
-      <c r="C53" s="6" t="inlineStr">
-        <is>
-          <t>阻塞：[2026-10-13] 2026-10-13 用戶決定：AI Buddy（品牌 C）延到 1/15 之後，本項不卡 1/15 出廠；AI Buddy 啟動時再開。</t>
+    <row r="52">
+      <c r="A52" s="10" t="inlineStr">
+        <is>
+          <t>⏳ 等待依賴 / ⛔ 阻塞</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>編號</t>
+        </is>
+      </c>
+      <c r="B53" s="4" t="inlineStr">
+        <is>
+          <t>任務</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="inlineStr">
+        <is>
+          <t>在等什麼</t>
         </is>
       </c>
       <c r="D53" s="11" t="n"/>
@@ -2078,20 +2112,20 @@
       <c r="H53" s="11" t="n"/>
       <c r="I53" s="12" t="n"/>
     </row>
-    <row r="54" ht="32" customHeight="1">
+    <row r="54" ht="60" customHeight="1">
       <c r="A54" s="13" t="inlineStr">
         <is>
-          <t>R-29</t>
+          <t>R-16</t>
         </is>
       </c>
       <c r="B54" s="6" t="inlineStr">
         <is>
-          <t>AI Buddy App（品牌 C）頁面</t>
+          <t>Spotpear 量產版加電池電壓檢測（GPIO0 分壓）</t>
         </is>
       </c>
       <c r="C54" s="6" t="inlineStr">
         <is>
-          <t>阻塞：[2026-10-13] 2026-10-13 用戶決定：AI Buddy（品牌 C）延到 1/15 之後，本項不卡 1/15 出廠；AI Buddy 啟動時再開。</t>
+          <t>阻塞：[2026-10-07] 仍按 10/06 決定暫緩：等用戶做充滿再放電測試（與 R-17 同一次），看 VDD 低電提醒在關機前多久觸發；太遲或不觸發才向 Spotpear 提改板。已把分壓改板的問題一併放進給 Spotpear 的草稿，方便同一封發出</t>
         </is>
       </c>
       <c r="D54" s="11" t="n"/>
@@ -2101,20 +2135,20 @@
       <c r="H54" s="11" t="n"/>
       <c r="I54" s="12" t="n"/>
     </row>
-    <row r="55" ht="18" customHeight="1">
+    <row r="55" ht="88" customHeight="1">
       <c r="A55" s="13" t="inlineStr">
         <is>
-          <t>R-05</t>
+          <t>R-17</t>
         </is>
       </c>
       <c r="B55" s="6" t="inlineStr">
         <is>
-          <t>內測版外殼（3D 打印 20 台）</t>
+          <t>Spotpear 電池耗盡時插電能否正常開機（供電路徑）</t>
         </is>
       </c>
       <c r="C55" s="6" t="inlineStr">
         <is>
-          <t>等 R-01</t>
+          <t>阻塞：[2026-10-08] 2026-10-08 開發板 63:64 插著 USB 時兩次無法解釋的完全斷電重開：09:13:26（崩潰循環中）、10:44:33（閒置、用戶確認沒碰）。都是 USB 先斷線再以 ESP_RST_POWERON 開機，非 brownout；斷電前 6 秒 GPIO0 讀數 99.9% 參考值，屬突然切斷而非緩降（SupplyMonitor 取樣太疏抓不到瞬間）。韌體無法造成 POWERON，指向充電芯片/電池保護/供電路徑，應一併問 Spotpear；放電實測時留意插 USB 閒置時是否也會斷電</t>
         </is>
       </c>
       <c r="D55" s="11" t="n"/>
@@ -2124,20 +2158,20 @@
       <c r="H55" s="11" t="n"/>
       <c r="I55" s="12" t="n"/>
     </row>
-    <row r="56" ht="18" customHeight="1">
+    <row r="56" ht="32" customHeight="1">
       <c r="A56" s="13" t="inlineStr">
         <is>
-          <t>R-06</t>
+          <t>P1-09</t>
         </is>
       </c>
       <c r="B56" s="6" t="inlineStr">
         <is>
-          <t>家長自助上手流程</t>
+          <t>家長鎖：孩子模式進設定要輸入 PIN</t>
         </is>
       </c>
       <c r="C56" s="6" t="inlineStr">
         <is>
-          <t>等 P0-11</t>
+          <t>阻塞：[2026-10-13] 2026-10-13 用戶決定：AI Buddy（品牌 C）延到 1/15 之後，本項不卡 1/15 出廠；AI Buddy 啟動時再開。</t>
         </is>
       </c>
       <c r="D56" s="11" t="n"/>
@@ -2150,17 +2184,17 @@
     <row r="57" ht="32" customHeight="1">
       <c r="A57" s="13" t="inlineStr">
         <is>
-          <t>R-13</t>
+          <t>R-12</t>
         </is>
       </c>
       <c r="B57" s="6" t="inlineStr">
         <is>
-          <t>CP1 內測就緒檢查（10/30）</t>
+          <t>家長控制：每日使用上限和休息時段</t>
         </is>
       </c>
       <c r="C57" s="6" t="inlineStr">
         <is>
-          <t>等 P0-07、P0-11、P1-01、P1-02、P2-09、R-01、R-02、R-04、R-05、R-06、P1-09、P1-11</t>
+          <t>阻塞：[2026-10-13] 2026-10-13 用戶決定：AI Buddy（品牌 C）延到 1/15 之後，本項不卡 1/15 出廠；AI Buddy 啟動時再開。</t>
         </is>
       </c>
       <c r="D57" s="11" t="n"/>
@@ -2173,17 +2207,17 @@
     <row r="58" ht="32" customHeight="1">
       <c r="A58" s="13" t="inlineStr">
         <is>
-          <t>R-18</t>
+          <t>R-29</t>
         </is>
       </c>
       <c r="B58" s="6" t="inlineStr">
         <is>
-          <t>長按 BOOT 重新配網（開 AIBuddy-XXXX 熱點）</t>
+          <t>AI Buddy App（品牌 C）頁面</t>
         </is>
       </c>
       <c r="C58" s="6" t="inlineStr">
         <is>
-          <t>等 R-01</t>
+          <t>阻塞：[2026-10-13] 2026-10-13 用戶決定：AI Buddy（品牌 C）延到 1/15 之後，本項不卡 1/15 出廠；AI Buddy 啟動時再開。</t>
         </is>
       </c>
       <c r="D58" s="11" t="n"/>
@@ -2196,17 +2230,17 @@
     <row r="59" ht="32" customHeight="1">
       <c r="A59" s="13" t="inlineStr">
         <is>
-          <t>R-19</t>
+          <t>P2-14</t>
         </is>
       </c>
       <c r="B59" s="6" t="inlineStr">
         <is>
-          <t>外接按鈕：量產板加 I2C 擴展晶片（TCA9555）</t>
+          <t>Admin 設備頁：每台玩具的狀態、韌體與基本操作</t>
         </is>
       </c>
       <c r="C59" s="6" t="inlineStr">
         <is>
-          <t>等 R-01</t>
+          <t>等 P1-10、P2-13</t>
         </is>
       </c>
       <c r="D59" s="11" t="n"/>
@@ -2219,17 +2253,17 @@
     <row r="60" ht="18" customHeight="1">
       <c r="A60" s="13" t="inlineStr">
         <is>
-          <t>R-20</t>
+          <t>R-05</t>
         </is>
       </c>
       <c r="B60" s="6" t="inlineStr">
         <is>
-          <t>孩子資料與角色改成每台設備一份</t>
+          <t>內測版外殼（3D 打印 20 台）</t>
         </is>
       </c>
       <c r="C60" s="6" t="inlineStr">
         <is>
-          <t>等 P1-12</t>
+          <t>等 R-01</t>
         </is>
       </c>
       <c r="D60" s="11" t="n"/>
@@ -2239,20 +2273,20 @@
       <c r="H60" s="11" t="n"/>
       <c r="I60" s="12" t="n"/>
     </row>
-    <row r="61" ht="32" customHeight="1">
+    <row r="61" ht="18" customHeight="1">
       <c r="A61" s="13" t="inlineStr">
         <is>
-          <t>R-27</t>
+          <t>R-06</t>
         </is>
       </c>
       <c r="B61" s="6" t="inlineStr">
         <is>
-          <t>App 內登入：驗證碼、原生社交登入、刪除帳號</t>
+          <t>家長自助上手流程</t>
         </is>
       </c>
       <c r="C61" s="6" t="inlineStr">
         <is>
-          <t>等 R-26</t>
+          <t>等 P0-11</t>
         </is>
       </c>
       <c r="D61" s="11" t="n"/>
@@ -2262,20 +2296,20 @@
       <c r="H61" s="11" t="n"/>
       <c r="I61" s="12" t="n"/>
     </row>
-    <row r="62" ht="18" customHeight="1">
+    <row r="62" ht="32" customHeight="1">
       <c r="A62" s="13" t="inlineStr">
         <is>
-          <t>P0-14</t>
+          <t>R-13</t>
         </is>
       </c>
       <c r="B62" s="6" t="inlineStr">
         <is>
-          <t>韌體簽章、Secure Boot 與 Flash 加密</t>
+          <t>CP1 內測就緒檢查（10/30）</t>
         </is>
       </c>
       <c r="C62" s="6" t="inlineStr">
         <is>
-          <t>等 R-01</t>
+          <t>等 P0-07、P0-11、P1-01、P1-02、P2-09、R-01、R-02、R-04、R-05、R-06、P1-09、P1-11</t>
         </is>
       </c>
       <c r="D62" s="11" t="n"/>
@@ -2285,20 +2319,20 @@
       <c r="H62" s="11" t="n"/>
       <c r="I62" s="12" t="n"/>
     </row>
-    <row r="63" ht="18" customHeight="1">
+    <row r="63" ht="32" customHeight="1">
       <c r="A63" s="13" t="inlineStr">
         <is>
-          <t>P1-06</t>
+          <t>R-18</t>
         </is>
       </c>
       <c r="B63" s="6" t="inlineStr">
         <is>
-          <t>處理 GPL-3.0 依賴（arduino-audio-tools）</t>
+          <t>長按 BOOT 重新配網（開 AIBuddy-XXXX 熱點）</t>
         </is>
       </c>
       <c r="C63" s="6" t="inlineStr">
         <is>
-          <t>等 Q3</t>
+          <t>等 R-01</t>
         </is>
       </c>
       <c r="D63" s="11" t="n"/>
@@ -2308,20 +2342,20 @@
       <c r="H63" s="11" t="n"/>
       <c r="I63" s="12" t="n"/>
     </row>
-    <row r="64" ht="18" customHeight="1">
+    <row r="64" ht="32" customHeight="1">
       <c r="A64" s="13" t="inlineStr">
         <is>
-          <t>P1-07</t>
+          <t>R-19</t>
         </is>
       </c>
       <c r="B64" s="6" t="inlineStr">
         <is>
-          <t>LGPL 合規與第三方授權聲明</t>
+          <t>外接按鈕：量產板加 I2C 擴展晶片（TCA9555）</t>
         </is>
       </c>
       <c r="C64" s="6" t="inlineStr">
         <is>
-          <t>等 Q3</t>
+          <t>等 R-01</t>
         </is>
       </c>
       <c r="D64" s="11" t="n"/>
@@ -2334,17 +2368,17 @@
     <row r="65" ht="18" customHeight="1">
       <c r="A65" s="13" t="inlineStr">
         <is>
-          <t>P1-08</t>
+          <t>R-20</t>
         </is>
       </c>
       <c r="B65" s="6" t="inlineStr">
         <is>
-          <t>硬件認證</t>
+          <t>孩子資料與角色改成每台設備一份</t>
         </is>
       </c>
       <c r="C65" s="6" t="inlineStr">
         <is>
-          <t>等 R-01、R-05</t>
+          <t>等 P1-12</t>
         </is>
       </c>
       <c r="D65" s="11" t="n"/>
@@ -2354,20 +2388,20 @@
       <c r="H65" s="11" t="n"/>
       <c r="I65" s="12" t="n"/>
     </row>
-    <row r="66" ht="18" customHeight="1">
+    <row r="66" ht="32" customHeight="1">
       <c r="A66" s="13" t="inlineStr">
         <is>
-          <t>R-07</t>
+          <t>R-27</t>
         </is>
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
-          <t>20 個家庭封閉內測</t>
+          <t>App 內登入：驗證碼、原生社交登入、刪除帳號</t>
         </is>
       </c>
       <c r="C66" s="6" t="inlineStr">
         <is>
-          <t>等 R-13</t>
+          <t>等 R-26</t>
         </is>
       </c>
       <c r="D66" s="11" t="n"/>
@@ -2380,17 +2414,17 @@
     <row r="67" ht="18" customHeight="1">
       <c r="A67" s="13" t="inlineStr">
         <is>
-          <t>R-08</t>
+          <t>P0-14</t>
         </is>
       </c>
       <c r="B67" s="6" t="inlineStr">
         <is>
-          <t>第 8 週關卡決策</t>
+          <t>韌體簽章、Secure Boot 與 Flash 加密</t>
         </is>
       </c>
       <c r="C67" s="6" t="inlineStr">
         <is>
-          <t>等 R-07、P2-09、P1-08</t>
+          <t>等 R-01</t>
         </is>
       </c>
       <c r="D67" s="11" t="n"/>
@@ -2403,17 +2437,17 @@
     <row r="68" ht="18" customHeight="1">
       <c r="A68" s="13" t="inlineStr">
         <is>
-          <t>R-14</t>
+          <t>P1-06</t>
         </is>
       </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t>離線兒歌與故事</t>
+          <t>處理 GPL-3.0 依賴（arduino-audio-tools）</t>
         </is>
       </c>
       <c r="C68" s="6" t="inlineStr">
         <is>
-          <t>等 R-01</t>
+          <t>等 Q3</t>
         </is>
       </c>
       <c r="D68" s="11" t="n"/>
@@ -2426,17 +2460,17 @@
     <row r="69" ht="18" customHeight="1">
       <c r="A69" s="13" t="inlineStr">
         <is>
-          <t>R-24</t>
+          <t>P1-07</t>
         </is>
       </c>
       <c r="B69" s="6" t="inlineStr">
         <is>
-          <t>設備只能用自己品牌的角色</t>
+          <t>LGPL 合規與第三方授權聲明</t>
         </is>
       </c>
       <c r="C69" s="6" t="inlineStr">
         <is>
-          <t>等 R-34</t>
+          <t>等 Q3</t>
         </is>
       </c>
       <c r="D69" s="11" t="n"/>
@@ -2449,17 +2483,17 @@
     <row r="70" ht="18" customHeight="1">
       <c r="A70" s="13" t="inlineStr">
         <is>
-          <t>R-28</t>
+          <t>P1-08</t>
         </is>
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>三個 App 的殼：品牌版本與測試版</t>
+          <t>硬件認證</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr">
         <is>
-          <t>等 R-25、R-26</t>
+          <t>等 R-01、R-05</t>
         </is>
       </c>
       <c r="D70" s="11" t="n"/>
@@ -2472,17 +2506,17 @@
     <row r="71" ht="18" customHeight="1">
       <c r="A71" s="13" t="inlineStr">
         <is>
-          <t>R-30</t>
+          <t>P1-14</t>
         </is>
       </c>
       <c r="B71" s="6" t="inlineStr">
         <is>
-          <t>快活 App（品牌 A）頁面</t>
+          <t>Admin 內容安全頁：審核事件只按類別統計</t>
         </is>
       </c>
       <c r="C71" s="6" t="inlineStr">
         <is>
-          <t>等 R-25、R-34、Q12</t>
+          <t>等 P1-01、P2-13</t>
         </is>
       </c>
       <c r="D71" s="11" t="n"/>
@@ -2492,20 +2526,20 @@
       <c r="H71" s="11" t="n"/>
       <c r="I71" s="12" t="n"/>
     </row>
-    <row r="72" ht="18" customHeight="1">
+    <row r="72" ht="32" customHeight="1">
       <c r="A72" s="13" t="inlineStr">
         <is>
-          <t>R-31</t>
+          <t>P2-15</t>
         </is>
       </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>政協青年聯會版 App（品牌 B）頁面</t>
+          <t>Admin 總覽頁：在線、用量、成本與待處理事項</t>
         </is>
       </c>
       <c r="C72" s="6" t="inlineStr">
         <is>
-          <t>等 R-25、R-34、Q13</t>
+          <t>等 P2-14、P2-09</t>
         </is>
       </c>
       <c r="D72" s="11" t="n"/>
@@ -2518,17 +2552,17 @@
     <row r="73" ht="18" customHeight="1">
       <c r="A73" s="13" t="inlineStr">
         <is>
-          <t>R-35</t>
+          <t>R-07</t>
         </is>
       </c>
       <c r="B73" s="6" t="inlineStr">
         <is>
-          <t>韌體按品牌連線：伺服器網址在出廠時寫入</t>
+          <t>20 個家庭封閉內測</t>
         </is>
       </c>
       <c r="C73" s="6" t="inlineStr">
         <is>
-          <t>等 R-34</t>
+          <t>等 R-13</t>
         </is>
       </c>
       <c r="D73" s="11" t="n"/>
@@ -2538,20 +2572,20 @@
       <c r="H73" s="11" t="n"/>
       <c r="I73" s="12" t="n"/>
     </row>
-    <row r="74" ht="32" customHeight="1">
+    <row r="74" ht="18" customHeight="1">
       <c r="A74" s="13" t="inlineStr">
         <is>
-          <t>R-38</t>
+          <t>R-08</t>
         </is>
       </c>
       <c r="B74" s="6" t="inlineStr">
         <is>
-          <t>公仔出廠鎖死所屬 IP，綁定時顯示該 IP 頭像</t>
+          <t>第 8 週關卡決策</t>
         </is>
       </c>
       <c r="C74" s="6" t="inlineStr">
         <is>
-          <t>等 P0-11</t>
+          <t>等 R-07、P2-09、P1-08</t>
         </is>
       </c>
       <c r="D74" s="11" t="n"/>
@@ -2564,17 +2598,17 @@
     <row r="75" ht="18" customHeight="1">
       <c r="A75" s="13" t="inlineStr">
         <is>
-          <t>R-09</t>
+          <t>R-14</t>
         </is>
       </c>
       <c r="B75" s="6" t="inlineStr">
         <is>
-          <t>量產外殼（真空複模）</t>
+          <t>離線兒歌與故事</t>
         </is>
       </c>
       <c r="C75" s="6" t="inlineStr">
         <is>
-          <t>等 R-08、R-05、Q11</t>
+          <t>等 R-01</t>
         </is>
       </c>
       <c r="D75" s="11" t="n"/>
@@ -2587,17 +2621,17 @@
     <row r="76" ht="18" customHeight="1">
       <c r="A76" s="13" t="inlineStr">
         <is>
-          <t>R-10</t>
+          <t>R-24</t>
         </is>
       </c>
       <c r="B76" s="6" t="inlineStr">
         <is>
-          <t>出廠流程</t>
+          <t>設備只能用自己品牌的角色</t>
         </is>
       </c>
       <c r="C76" s="6" t="inlineStr">
         <is>
-          <t>等 P0-14、R-01、P2-12、R-34、R-35、R-38</t>
+          <t>等 R-34</t>
         </is>
       </c>
       <c r="D76" s="11" t="n"/>
@@ -2610,17 +2644,17 @@
     <row r="77" ht="18" customHeight="1">
       <c r="A77" s="13" t="inlineStr">
         <is>
-          <t>R-15</t>
+          <t>R-28</t>
         </is>
       </c>
       <c r="B77" s="6" t="inlineStr">
         <is>
-          <t>農曆新年前交付（生產 1/15、送達 1/29）</t>
+          <t>三個 App 的殼：品牌版本與測試版</t>
         </is>
       </c>
       <c r="C77" s="6" t="inlineStr">
         <is>
-          <t>等 R-09、R-10</t>
+          <t>等 R-25、R-26</t>
         </is>
       </c>
       <c r="D77" s="11" t="n"/>
@@ -2633,17 +2667,17 @@
     <row r="78" ht="18" customHeight="1">
       <c r="A78" s="13" t="inlineStr">
         <is>
-          <t>R-33</t>
+          <t>R-30</t>
         </is>
       </c>
       <c r="B78" s="6" t="inlineStr">
         <is>
-          <t>三個 App 送審並通過</t>
+          <t>快活 App（品牌 A）頁面</t>
         </is>
       </c>
       <c r="C78" s="6" t="inlineStr">
         <is>
-          <t>等 R-27、R-21、R-28、R-29、R-30、R-31、R-32</t>
+          <t>等 R-25、R-34、Q12</t>
         </is>
       </c>
       <c r="D78" s="11" t="n"/>
@@ -2653,27 +2687,66 @@
       <c r="H78" s="11" t="n"/>
       <c r="I78" s="12" t="n"/>
     </row>
-    <row r="80">
-      <c r="A80" s="10" t="inlineStr">
-        <is>
-          <t>❓ 待確認問題</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" s="4" t="inlineStr">
-        <is>
-          <t>編號</t>
-        </is>
-      </c>
-      <c r="B81" s="4" t="inlineStr">
-        <is>
-          <t>問題</t>
-        </is>
-      </c>
-      <c r="C81" s="4" t="inlineStr">
-        <is>
-          <t>影響的任務 / 為什麼重要</t>
+    <row r="79" ht="18" customHeight="1">
+      <c r="A79" s="13" t="inlineStr">
+        <is>
+          <t>R-31</t>
+        </is>
+      </c>
+      <c r="B79" s="6" t="inlineStr">
+        <is>
+          <t>政協青年聯會版 App（品牌 B）頁面</t>
+        </is>
+      </c>
+      <c r="C79" s="6" t="inlineStr">
+        <is>
+          <t>等 R-25、R-34、Q13</t>
+        </is>
+      </c>
+      <c r="D79" s="11" t="n"/>
+      <c r="E79" s="11" t="n"/>
+      <c r="F79" s="11" t="n"/>
+      <c r="G79" s="11" t="n"/>
+      <c r="H79" s="11" t="n"/>
+      <c r="I79" s="12" t="n"/>
+    </row>
+    <row r="80" ht="18" customHeight="1">
+      <c r="A80" s="13" t="inlineStr">
+        <is>
+          <t>R-35</t>
+        </is>
+      </c>
+      <c r="B80" s="6" t="inlineStr">
+        <is>
+          <t>韌體按品牌連線：伺服器網址在出廠時寫入</t>
+        </is>
+      </c>
+      <c r="C80" s="6" t="inlineStr">
+        <is>
+          <t>等 R-34</t>
+        </is>
+      </c>
+      <c r="D80" s="11" t="n"/>
+      <c r="E80" s="11" t="n"/>
+      <c r="F80" s="11" t="n"/>
+      <c r="G80" s="11" t="n"/>
+      <c r="H80" s="11" t="n"/>
+      <c r="I80" s="12" t="n"/>
+    </row>
+    <row r="81" ht="32" customHeight="1">
+      <c r="A81" s="13" t="inlineStr">
+        <is>
+          <t>R-38</t>
+        </is>
+      </c>
+      <c r="B81" s="6" t="inlineStr">
+        <is>
+          <t>公仔出廠鎖死所屬 IP，綁定時顯示該 IP 頭像</t>
+        </is>
+      </c>
+      <c r="C81" s="6" t="inlineStr">
+        <is>
+          <t>等 P0-11</t>
         </is>
       </c>
       <c r="D81" s="11" t="n"/>
@@ -2683,20 +2756,20 @@
       <c r="H81" s="11" t="n"/>
       <c r="I81" s="12" t="n"/>
     </row>
-    <row r="82" ht="18" customHeight="1">
+    <row r="82" ht="32" customHeight="1">
       <c r="A82" s="13" t="inlineStr">
         <is>
-          <t>Q3</t>
+          <t>R-39</t>
         </is>
       </c>
       <c r="B82" s="6" t="inlineStr">
         <is>
-          <t>韌體打算閉源商業銷售嗎？</t>
+          <t>Admin 出廠登記頁：匯入 MAC 清單、指定公仔、查看自檢結果</t>
         </is>
       </c>
       <c r="C82" s="6" t="inlineStr">
         <is>
-          <t>P1-06, P1-07：決定 GPL／LGPL 依賴要開源還是替換。</t>
+          <t>等 R-38、P1-10</t>
         </is>
       </c>
       <c r="D82" s="11" t="n"/>
@@ -2706,20 +2779,20 @@
       <c r="H82" s="11" t="n"/>
       <c r="I82" s="12" t="n"/>
     </row>
-    <row r="83" ht="32" customHeight="1">
+    <row r="83" ht="18" customHeight="1">
       <c r="A83" s="13" t="inlineStr">
         <is>
-          <t>Q11</t>
+          <t>P2-16</t>
         </is>
       </c>
       <c r="B83" s="6" t="inlineStr">
         <is>
-          <t>馬會快活的賽馬日版和新春版各多少隻（共 2,500）？</t>
+          <t>OTA 分批推送與後台發佈頁</t>
         </is>
       </c>
       <c r="C83" s="6" t="inlineStr">
         <is>
-          <t>R-09, R-15：兩款的服裝和配件要分開訂料；11/20 前不知道，PP 樣和大貨單（11/27）會被拖慢。由馬會決定。</t>
+          <t>等 P2-14、P1-10</t>
         </is>
       </c>
       <c r="D83" s="11" t="n"/>
@@ -2729,20 +2802,20 @@
       <c r="H83" s="11" t="n"/>
       <c r="I83" s="12" t="n"/>
     </row>
-    <row r="84" ht="60" customHeight="1">
+    <row r="84" ht="18" customHeight="1">
       <c r="A84" s="13" t="inlineStr">
         <is>
-          <t>Q12</t>
+          <t>R-09</t>
         </is>
       </c>
       <c r="B84" s="6" t="inlineStr">
         <is>
-          <t>快活 App 的「會員綁定」是指甚麼：用我們自己的帳號（email 驗證碼），還是接馬會的會員帳號登入（SSO）？</t>
+          <t>量產外殼（真空複模）</t>
         </is>
       </c>
       <c r="C84" s="6" t="inlineStr">
         <is>
-          <t>P0-11, 快活 App（未入追蹤表）：接馬會 SSO 的話，登入、帳號刪除和資料歸屬都要按馬會的介面重做，工作量和排期要另估，而且 W5（11/9–11/13）就要做快活 App 的綁定；用我們的帳號則和其他品牌共用同一套流程。由馬會決定，要盡早問。</t>
+          <t>等 R-08、R-05、Q11</t>
         </is>
       </c>
       <c r="D84" s="11" t="n"/>
@@ -2752,20 +2825,20 @@
       <c r="H84" s="11" t="n"/>
       <c r="I84" s="12" t="n"/>
     </row>
-    <row r="85" ht="46" customHeight="1">
+    <row r="85" ht="18" customHeight="1">
       <c r="A85" s="13" t="inlineStr">
         <is>
-          <t>Q13</t>
+          <t>R-10</t>
         </is>
       </c>
       <c r="B85" s="6" t="inlineStr">
         <is>
-          <t>政協青年聯會版的角色、語言和內容由誰提供？什麼時候交？</t>
+          <t>出廠流程</t>
         </is>
       </c>
       <c r="C85" s="6" t="inlineStr">
         <is>
-          <t>品牌 B 的 App 頁面：品牌 B 的用戶是成人會員，但角色、說話語言、內容規則都還沒有。最遲 11/13 要拿到，才趕得及內部測試和 App 頁面（W6）。</t>
+          <t>等 P0-14、R-01、P2-12、R-34、R-35、R-38、R-39</t>
         </is>
       </c>
       <c r="D85" s="11" t="n"/>
@@ -2775,123 +2848,348 @@
       <c r="H85" s="11" t="n"/>
       <c r="I85" s="12" t="n"/>
     </row>
-    <row r="87">
-      <c r="A87" s="10" t="inlineStr">
+    <row r="86" ht="18" customHeight="1">
+      <c r="A86" s="13" t="inlineStr">
+        <is>
+          <t>R-11</t>
+        </is>
+      </c>
+      <c r="B86" s="6" t="inlineStr">
+        <is>
+          <t>售後：客服、保修與換機</t>
+        </is>
+      </c>
+      <c r="C86" s="6" t="inlineStr">
+        <is>
+          <t>等 P2-14、R-40</t>
+        </is>
+      </c>
+      <c r="D86" s="11" t="n"/>
+      <c r="E86" s="11" t="n"/>
+      <c r="F86" s="11" t="n"/>
+      <c r="G86" s="11" t="n"/>
+      <c r="H86" s="11" t="n"/>
+      <c r="I86" s="12" t="n"/>
+    </row>
+    <row r="87" ht="18" customHeight="1">
+      <c r="A87" s="13" t="inlineStr">
+        <is>
+          <t>R-15</t>
+        </is>
+      </c>
+      <c r="B87" s="6" t="inlineStr">
+        <is>
+          <t>農曆新年前交付（生產 1/15、送達 1/29）</t>
+        </is>
+      </c>
+      <c r="C87" s="6" t="inlineStr">
+        <is>
+          <t>等 R-09、R-10</t>
+        </is>
+      </c>
+      <c r="D87" s="11" t="n"/>
+      <c r="E87" s="11" t="n"/>
+      <c r="F87" s="11" t="n"/>
+      <c r="G87" s="11" t="n"/>
+      <c r="H87" s="11" t="n"/>
+      <c r="I87" s="12" t="n"/>
+    </row>
+    <row r="88" ht="18" customHeight="1">
+      <c r="A88" s="13" t="inlineStr">
+        <is>
+          <t>R-33</t>
+        </is>
+      </c>
+      <c r="B88" s="6" t="inlineStr">
+        <is>
+          <t>三個 App 送審並通過</t>
+        </is>
+      </c>
+      <c r="C88" s="6" t="inlineStr">
+        <is>
+          <t>等 R-27、R-21、R-28、R-29、R-30、R-31、R-32</t>
+        </is>
+      </c>
+      <c r="D88" s="11" t="n"/>
+      <c r="E88" s="11" t="n"/>
+      <c r="F88" s="11" t="n"/>
+      <c r="G88" s="11" t="n"/>
+      <c r="H88" s="11" t="n"/>
+      <c r="I88" s="12" t="n"/>
+    </row>
+    <row r="89" ht="32" customHeight="1">
+      <c r="A89" s="13" t="inlineStr">
+        <is>
+          <t>R-40</t>
+        </is>
+      </c>
+      <c r="B89" s="6" t="inlineStr">
+        <is>
+          <t>Admin 客服查詢頁：查帳號、名下設備與最近事件</t>
+        </is>
+      </c>
+      <c r="C89" s="6" t="inlineStr">
+        <is>
+          <t>等 P2-14、P1-10、P1-12</t>
+        </is>
+      </c>
+      <c r="D89" s="11" t="n"/>
+      <c r="E89" s="11" t="n"/>
+      <c r="F89" s="11" t="n"/>
+      <c r="G89" s="11" t="n"/>
+      <c r="H89" s="11" t="n"/>
+      <c r="I89" s="12" t="n"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="10" t="inlineStr">
+        <is>
+          <t>❓ 待確認問題</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="4" t="inlineStr">
+        <is>
+          <t>編號</t>
+        </is>
+      </c>
+      <c r="B92" s="4" t="inlineStr">
+        <is>
+          <t>問題</t>
+        </is>
+      </c>
+      <c r="C92" s="4" t="inlineStr">
+        <is>
+          <t>影響的任務 / 為什麼重要</t>
+        </is>
+      </c>
+      <c r="D92" s="11" t="n"/>
+      <c r="E92" s="11" t="n"/>
+      <c r="F92" s="11" t="n"/>
+      <c r="G92" s="11" t="n"/>
+      <c r="H92" s="11" t="n"/>
+      <c r="I92" s="12" t="n"/>
+    </row>
+    <row r="93" ht="18" customHeight="1">
+      <c r="A93" s="13" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="B93" s="6" t="inlineStr">
+        <is>
+          <t>韌體打算閉源商業銷售嗎？</t>
+        </is>
+      </c>
+      <c r="C93" s="6" t="inlineStr">
+        <is>
+          <t>P1-06, P1-07：決定 GPL／LGPL 依賴要開源還是替換。</t>
+        </is>
+      </c>
+      <c r="D93" s="11" t="n"/>
+      <c r="E93" s="11" t="n"/>
+      <c r="F93" s="11" t="n"/>
+      <c r="G93" s="11" t="n"/>
+      <c r="H93" s="11" t="n"/>
+      <c r="I93" s="12" t="n"/>
+    </row>
+    <row r="94" ht="32" customHeight="1">
+      <c r="A94" s="13" t="inlineStr">
+        <is>
+          <t>Q11</t>
+        </is>
+      </c>
+      <c r="B94" s="6" t="inlineStr">
+        <is>
+          <t>馬會快活的賽馬日版和新春版各多少隻（共 2,500）？</t>
+        </is>
+      </c>
+      <c r="C94" s="6" t="inlineStr">
+        <is>
+          <t>R-09, R-15：兩款的服裝和配件要分開訂料；11/20 前不知道，PP 樣和大貨單（11/27）會被拖慢。由馬會決定。</t>
+        </is>
+      </c>
+      <c r="D94" s="11" t="n"/>
+      <c r="E94" s="11" t="n"/>
+      <c r="F94" s="11" t="n"/>
+      <c r="G94" s="11" t="n"/>
+      <c r="H94" s="11" t="n"/>
+      <c r="I94" s="12" t="n"/>
+    </row>
+    <row r="95" ht="60" customHeight="1">
+      <c r="A95" s="13" t="inlineStr">
+        <is>
+          <t>Q12</t>
+        </is>
+      </c>
+      <c r="B95" s="6" t="inlineStr">
+        <is>
+          <t>快活 App 的「會員綁定」是指甚麼：用我們自己的帳號（email 驗證碼），還是接馬會的會員帳號登入（SSO）？</t>
+        </is>
+      </c>
+      <c r="C95" s="6" t="inlineStr">
+        <is>
+          <t>P0-11, 快活 App（未入追蹤表）：接馬會 SSO 的話，登入、帳號刪除和資料歸屬都要按馬會的介面重做，工作量和排期要另估，而且 W5（11/9–11/13）就要做快活 App 的綁定；用我們的帳號則和其他品牌共用同一套流程。由馬會決定，要盡早問。</t>
+        </is>
+      </c>
+      <c r="D95" s="11" t="n"/>
+      <c r="E95" s="11" t="n"/>
+      <c r="F95" s="11" t="n"/>
+      <c r="G95" s="11" t="n"/>
+      <c r="H95" s="11" t="n"/>
+      <c r="I95" s="12" t="n"/>
+    </row>
+    <row r="96" ht="46" customHeight="1">
+      <c r="A96" s="13" t="inlineStr">
+        <is>
+          <t>Q13</t>
+        </is>
+      </c>
+      <c r="B96" s="6" t="inlineStr">
+        <is>
+          <t>政協青年聯會版的角色、語言和內容由誰提供？什麼時候交？</t>
+        </is>
+      </c>
+      <c r="C96" s="6" t="inlineStr">
+        <is>
+          <t>品牌 B 的 App 頁面：品牌 B 的用戶是成人會員，但角色、說話語言、內容規則都還沒有。最遲 11/13 要拿到，才趕得及內部測試和 App 頁面（W6）。</t>
+        </is>
+      </c>
+      <c r="D96" s="11" t="n"/>
+      <c r="E96" s="11" t="n"/>
+      <c r="F96" s="11" t="n"/>
+      <c r="G96" s="11" t="n"/>
+      <c r="H96" s="11" t="n"/>
+      <c r="I96" s="12" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="10" t="inlineStr">
         <is>
           <t>說明</t>
         </is>
       </c>
     </row>
-    <row r="88" ht="32" customHeight="1">
-      <c r="A88" s="14" t="inlineStr">
+    <row r="99" ht="32" customHeight="1">
+      <c r="A99" s="14" t="inlineStr">
         <is>
           <t>・狀態：未開始 → 進行中 → 已完成。只有測試真的跑過而且通過才算已完成；阻塞要在備註寫原因；不再需要的任務標不適用，不要刪。</t>
         </is>
       </c>
     </row>
-    <row r="89" ht="18" customHeight="1">
-      <c r="A89" s="14" t="inlineStr">
+    <row r="100" ht="18" customHeight="1">
+      <c r="A100" s="14" t="inlineStr">
         <is>
           <t>・測試結果：未測試 / 通過 / 失敗 / 部分通過。測試證據寫跑了什麼、看到什麼，完整歷史在「更新記錄」。</t>
         </is>
       </c>
     </row>
-    <row r="90" ht="18" customHeight="1">
-      <c r="A90" s="14" t="inlineStr">
+    <row r="101" ht="18" customHeight="1">
+      <c r="A101" s="14" t="inlineStr">
         <is>
           <t>・「接下來」按階段排序，同一階段內再按優先級；依賴還沒滿足的任務不會出現在「接下來」。</t>
         </is>
       </c>
     </row>
-    <row r="91" ht="18" customHeight="1">
-      <c r="A91" s="14" t="inlineStr">
+    <row r="102" ht="18" customHeight="1">
+      <c r="A102" s="14" t="inlineStr">
         <is>
           <t>・可以手動改：「任務清單」的狀態、測試結果、測試證據、Commit、備註，以及「待確認問題」的回答。其餘欄位和本頁由腳本維護。</t>
         </is>
       </c>
     </row>
-    <row r="92" ht="32" customHeight="1">
-      <c r="A92" s="14" t="inlineStr">
+    <row r="103" ht="32" customHeight="1">
+      <c r="A103" s="14" t="inlineStr">
         <is>
           <t>・建議用法：在 Claude Code 對 Claude 說「P0-02 做完了」或輸入 /prod-readiness。Claude 會先跑測試再更新，並寫進「更新記錄」。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="73">
-    <mergeCell ref="E21:I21"/>
+  <mergeCells count="84">
+    <mergeCell ref="A41:I41"/>
+    <mergeCell ref="A99:I99"/>
+    <mergeCell ref="C82:I82"/>
+    <mergeCell ref="E39:I39"/>
+    <mergeCell ref="C67:I67"/>
+    <mergeCell ref="E48:I48"/>
+    <mergeCell ref="A101:I101"/>
+    <mergeCell ref="C53:I53"/>
+    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="E29:I29"/>
+    <mergeCell ref="E38:I38"/>
+    <mergeCell ref="C83:I83"/>
+    <mergeCell ref="C92:I92"/>
+    <mergeCell ref="E31:I31"/>
+    <mergeCell ref="A19:I19"/>
+    <mergeCell ref="E26:I26"/>
+    <mergeCell ref="A103:I103"/>
+    <mergeCell ref="E25:I25"/>
+    <mergeCell ref="C95:I95"/>
+    <mergeCell ref="C60:I60"/>
+    <mergeCell ref="C71:I71"/>
+    <mergeCell ref="E50:I50"/>
+    <mergeCell ref="E42:I42"/>
+    <mergeCell ref="C57:I57"/>
+    <mergeCell ref="C66:I66"/>
+    <mergeCell ref="E44:I44"/>
+    <mergeCell ref="E20:I20"/>
+    <mergeCell ref="E28:I28"/>
+    <mergeCell ref="C77:I77"/>
+    <mergeCell ref="C86:I86"/>
+    <mergeCell ref="C68:I68"/>
+    <mergeCell ref="A91:I91"/>
+    <mergeCell ref="A100:I100"/>
+    <mergeCell ref="C58:I58"/>
+    <mergeCell ref="A52:I52"/>
+    <mergeCell ref="E30:I30"/>
+    <mergeCell ref="E46:I46"/>
+    <mergeCell ref="A102:I102"/>
+    <mergeCell ref="C85:I85"/>
+    <mergeCell ref="C94:I94"/>
+    <mergeCell ref="C65:I65"/>
+    <mergeCell ref="C75:I75"/>
+    <mergeCell ref="C84:I84"/>
+    <mergeCell ref="C80:I80"/>
+    <mergeCell ref="E32:I32"/>
+    <mergeCell ref="C59:I59"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="E47:I47"/>
     <mergeCell ref="C61:I61"/>
     <mergeCell ref="E43:I43"/>
-    <mergeCell ref="C52:I52"/>
     <mergeCell ref="C70:I70"/>
-    <mergeCell ref="A90:I90"/>
-    <mergeCell ref="A37:I37"/>
     <mergeCell ref="E24:I24"/>
-    <mergeCell ref="E42:I42"/>
-    <mergeCell ref="C82:I82"/>
-    <mergeCell ref="A80:I80"/>
     <mergeCell ref="E33:I33"/>
-    <mergeCell ref="A89:I89"/>
     <mergeCell ref="A3:I3"/>
+    <mergeCell ref="E35:I35"/>
+    <mergeCell ref="C74:I74"/>
+    <mergeCell ref="C88:I88"/>
+    <mergeCell ref="E45:I45"/>
+    <mergeCell ref="C55:I55"/>
+    <mergeCell ref="E37:I37"/>
+    <mergeCell ref="E21:I21"/>
     <mergeCell ref="E23:I23"/>
     <mergeCell ref="C72:I72"/>
-    <mergeCell ref="E39:I39"/>
-    <mergeCell ref="C67:I67"/>
     <mergeCell ref="C81:I81"/>
-    <mergeCell ref="C57:I57"/>
-    <mergeCell ref="C53:I53"/>
-    <mergeCell ref="C66:I66"/>
-    <mergeCell ref="E44:I44"/>
-    <mergeCell ref="A2:I2"/>
-    <mergeCell ref="E29:I29"/>
-    <mergeCell ref="E35:I35"/>
-    <mergeCell ref="E20:I20"/>
-    <mergeCell ref="E38:I38"/>
     <mergeCell ref="C69:I69"/>
+    <mergeCell ref="C96:I96"/>
     <mergeCell ref="C78:I78"/>
-    <mergeCell ref="C49:I49"/>
-    <mergeCell ref="E28:I28"/>
-    <mergeCell ref="C77:I77"/>
-    <mergeCell ref="C83:I83"/>
+    <mergeCell ref="C87:I87"/>
     <mergeCell ref="C62:I62"/>
-    <mergeCell ref="C68:I68"/>
-    <mergeCell ref="A91:I91"/>
-    <mergeCell ref="E31:I31"/>
-    <mergeCell ref="E40:I40"/>
-    <mergeCell ref="C58:I58"/>
-    <mergeCell ref="E30:I30"/>
+    <mergeCell ref="C89:I89"/>
     <mergeCell ref="E34:I34"/>
-    <mergeCell ref="A19:I19"/>
-    <mergeCell ref="C74:I74"/>
     <mergeCell ref="C64:I64"/>
-    <mergeCell ref="E46:I46"/>
+    <mergeCell ref="C79:I79"/>
     <mergeCell ref="C73:I73"/>
+    <mergeCell ref="E49:I49"/>
     <mergeCell ref="E27:I27"/>
-    <mergeCell ref="E45:I45"/>
     <mergeCell ref="C54:I54"/>
-    <mergeCell ref="C85:I85"/>
+    <mergeCell ref="E36:I36"/>
     <mergeCell ref="C63:I63"/>
-    <mergeCell ref="A48:I48"/>
-    <mergeCell ref="C65:I65"/>
-    <mergeCell ref="E26:I26"/>
-    <mergeCell ref="A92:I92"/>
-    <mergeCell ref="C55:I55"/>
-    <mergeCell ref="C50:I50"/>
-    <mergeCell ref="C75:I75"/>
-    <mergeCell ref="C84:I84"/>
+    <mergeCell ref="C93:I93"/>
+    <mergeCell ref="A98:I98"/>
     <mergeCell ref="C56:I56"/>
-    <mergeCell ref="E32:I32"/>
-    <mergeCell ref="E25:I25"/>
-    <mergeCell ref="C59:I59"/>
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="E41:I41"/>
-    <mergeCell ref="A88:I88"/>
-    <mergeCell ref="C60:I60"/>
     <mergeCell ref="E22:I22"/>
-    <mergeCell ref="A87:I87"/>
-    <mergeCell ref="C51:I51"/>
     <mergeCell ref="C76:I76"/>
-    <mergeCell ref="C71:I71"/>
   </mergeCells>
   <conditionalFormatting sqref="I6:I10">
     <cfRule type="dataBar" priority="1">
@@ -2921,7 +3219,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P80"/>
+  <dimension ref="A1:P88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -4205,7 +4503,8 @@
       <c r="O16" s="13" t="n"/>
       <c r="P16" s="6" t="inlineStr">
         <is>
-          <t>[2026-09-30] Q5：3–6 歲；Q7：事件不記原文</t>
+          <t>[2026-09-30] Q5：3–6 歲；Q7：事件不記原文
+[2026-10-14] 2026-10-14：審核事件的後台頁拆成 P1-14，等本項完成後做。</t>
         </is>
       </c>
     </row>
@@ -5030,7 +5329,7 @@
       <c r="O28" s="13" t="n"/>
       <c r="P28" s="6" t="n"/>
     </row>
-    <row r="29" ht="46" customHeight="1">
+    <row r="29" ht="102" customHeight="1">
       <c r="A29" s="13" t="inlineStr">
         <is>
           <t>P2-06</t>
@@ -5092,7 +5391,8 @@
       <c r="O29" s="13" t="n"/>
       <c r="P29" s="6" t="inlineStr">
         <is>
-          <t>[2026-10-12] 2026-10-12：三套獨立部署（R-34），監控集中在一個面板，告警寫明品牌。</t>
+          <t>[2026-10-12] 2026-10-12：三套獨立部署（R-34），監控集中在一個面板，告警寫明品牌。
+[2026-10-14] 2026-10-14：admin 的「系統健康」頁只放摘要和外部監控連結，錯誤追蹤與告警用外部服務，不在後台自己做。</t>
         </is>
       </c>
     </row>
@@ -5230,7 +5530,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="32" customHeight="1">
+    <row r="32" ht="144" customHeight="1">
       <c r="A32" s="13" t="inlineStr">
         <is>
           <t>P2-09</t>
@@ -5258,7 +5558,7 @@
       </c>
       <c r="F32" s="13" t="inlineStr">
         <is>
-          <t>未開始</t>
+          <t>進行中</t>
         </is>
       </c>
       <c r="G32" s="13" t="inlineStr">
@@ -5291,7 +5591,11 @@
       <c r="M32" s="13" t="n"/>
       <c r="N32" s="6" t="n"/>
       <c r="O32" s="13" t="n"/>
-      <c r="P32" s="6" t="n"/>
+      <c r="P32" s="6" t="inlineStr">
+        <is>
+          <t>[2026-10-14] 2026-10-14：turn_metrics 目前只記 user_id 和 chat_group_id，沒有設備，也沒有 STT 秒數（只有 transcript_chars／response_chars），要改語音伺服器補上，並加單價表。頁面樣子在 preview/UsagePreview.tsx。內部測試每週要報每台每月成本（R-07），數據只能從開始記錄那天累積，建議 10/30 前做好。</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="409" customHeight="1">
       <c r="A33" s="13" t="inlineStr">
@@ -5975,7 +6279,7 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="270" customHeight="1">
+    <row r="42" ht="409" customHeight="1">
       <c r="A42" s="13" t="inlineStr">
         <is>
           <t>R-10</t>
@@ -6036,7 +6340,7 @@
       </c>
       <c r="M42" s="13" t="inlineStr">
         <is>
-          <t>P0-06, P0-14, R-01, P2-12, Q10, R-34, R-35, R-38</t>
+          <t>P0-06, P0-14, R-01, P2-12, Q10, R-34, R-35, R-38, R-39</t>
         </is>
       </c>
       <c r="N42" s="6" t="n"/>
@@ -6046,11 +6350,13 @@
           <t>[2026-10-12] 2026-10-12：燒錄地點未定（Q10），最遲 11/6。設備密鑰、品牌和款式都在出廠時寫入（三個品牌共用一個韌體）。
 [2026-10-12] 2026-10-12 Q10 已定（燒共用韌體）。Spotpear 出貨測試第一次通電就會開 Secure Boot 和 Flash 加密，所以 11/27 交 Spotpear 的映像必須是最終版（P0-14 要在 W5 前驗證）；app 之後經 OTA 更新。
 [2026-10-12] 2026-10-12：三個品牌分開部署後，出廠工位要把每台設備登記到該品牌那套的伺服器，並寫入該品牌的網址（R-35）。
-[2026-10-13] 2026-10-13：工位登記要寫入該公仔的 ip_key 和預設角色（R-38）。IP 不編進共用韌體。</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="186" customHeight="1">
+[2026-10-13] 2026-10-13：工位登記要寫入該公仔的 ip_key 和預設角色（R-38）。IP 不編進共用韌體。
+[2026-10-14] 2026-10-14：P2-12 定案後，工位多一步：按品牌寫入資源包（tools/build_assets.py --brand ... → esptool write_flash 0x810000），開機 log『Assets: brand ...crc ok』作自檢一項。
+[2026-10-14] 2026-10-14：後台的 MAC 清單匯入、整批指定公仔、QC 結果查看拆成 R-39，與工位腳本一起試產。</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="242" customHeight="1">
       <c r="A43" s="13" t="inlineStr">
         <is>
           <t>R-11</t>
@@ -6107,14 +6413,19 @@
           <t>演練一次：模擬家長報修 → 診斷 → 換機，全程有記錄。</t>
         </is>
       </c>
-      <c r="M43" s="13" t="n"/>
+      <c r="M43" s="13" t="inlineStr">
+        <is>
+          <t>P2-14, R-40</t>
+        </is>
+      </c>
       <c r="N43" s="6" t="n"/>
       <c r="O43" s="13" t="n"/>
       <c r="P43" s="6" t="inlineStr">
         <is>
           <t>[2026-09-30] v1 沒有客服角色，售後工具由超級管理員使用（Q9）
 [2026-10-09] 換機時記憶不用搬：記憶跟帳號，同一帳號認領新設備就會繼續（P1-12 TC4）。
-[2026-10-09] 更正（2026-10-09 晚）：記憶改成跟設備（P1-12），換新設備會從空白開始。換機流程要加「把舊設備的記憶搬到新設備」：把 memory_facts、memory_segments、conversations 的 device_id 從舊機改成新機（同一 user_id），並由超級管理員執行。</t>
+[2026-10-09] 更正（2026-10-09 晚）：記憶改成跟設備（P1-12），換新設備會從空白開始。換機流程要加「把舊設備的記憶搬到新設備」：把 memory_facts、memory_segments、conversations 的 device_id 從舊機改成新機（同一 user_id），並由超級管理員執行。
+[2026-10-14] 2026-10-14：admin 端的診斷靠設備頁（P2-14），報修、換機、刪帳號的工具在客服查詢頁（R-40）。</t>
         </is>
       </c>
     </row>
@@ -6436,7 +6747,7 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="60" customHeight="1">
+    <row r="48" ht="130" customHeight="1">
       <c r="A48" s="13" t="inlineStr">
         <is>
           <t>P1-10</t>
@@ -6464,7 +6775,7 @@
       </c>
       <c r="F48" s="13" t="inlineStr">
         <is>
-          <t>未開始</t>
+          <t>進行中</t>
         </is>
       </c>
       <c r="G48" s="13" t="inlineStr">
@@ -6504,7 +6815,8 @@
       <c r="O48" s="13" t="n"/>
       <c r="P48" s="6" t="inlineStr">
         <is>
-          <t>[2026-09-30] 新增</t>
+          <t>[2026-09-30] 新增
+[2026-10-14] 2026-10-14：admin 改側欄後（P2-13），actions.ts 在 frontend-nextjs/app/admin/actions.ts；審計記錄頁的樣子在 preview/AuditPreview.tsx。建議第一個做：設備頁、客服頁、OTA、出廠的每個動作都要寫審計，先有這張表就不用回頭改。</t>
         </is>
       </c>
     </row>
@@ -7208,7 +7520,7 @@
         </is>
       </c>
     </row>
-    <row r="59" ht="88" customHeight="1">
+    <row r="59" ht="354" customHeight="1">
       <c r="A59" s="13" t="inlineStr">
         <is>
           <t>P2-12</t>
@@ -7236,12 +7548,12 @@
       </c>
       <c r="F59" s="13" t="inlineStr">
         <is>
-          <t>未開始</t>
+          <t>進行中</t>
         </is>
       </c>
       <c r="G59" s="13" t="inlineStr">
         <is>
-          <t>未測試</t>
+          <t>部分通過</t>
         </is>
       </c>
       <c r="I59" s="6" t="inlineStr">
@@ -7265,10 +7577,22 @@
         </is>
       </c>
       <c r="M59" s="13" t="n"/>
+      <c r="N59" s="6" t="inlineStr">
+        <is>
+          <t>62:70（spotpear-ai-toy-p212 原型，現已併入 spotpear-ai-toy）：① 本機 OTA 1.6.1→1.6.2 寫入新 app1，120s 後 confirmed ② 3 秒 abort 的 1.6.3 → PANIC → 回到 1.6.2，ota_failed_version=1.6.3 ③ 崩潰寫入 coredump 14.8KB ④ 資源分區 9 個聲音 504KB/2MB，開機 CRC 63ms，OTA 後照常；損壞/清空 → 退回內建聲音無崩潰 ⑤ pio 全部 18 個 env 編譯通過，映像都在各自 app 槽內（Spotpear 4 個 1.59–1.60MB / 4MB；其他板仍 2MB 槽）；R-21 藍牙探針版 2,326,128 bytes &lt; 4MB ⑥ release_firmware.py 映像 &gt; app 槽即拒發。未做：雲端 OTA 一次（等上 UAT）、出廠腳本寫入資源包（R-10）</t>
+        </is>
+      </c>
+      <c r="O59" s="13" t="inlineStr">
+        <is>
+          <t>5e9ffce</t>
+        </is>
+      </c>
       <c r="P59" s="6" t="inlineStr">
         <is>
           <t>[2026-10-09] 新增
-[2026-10-12] 2026-10-12：藍牙配網（R-21）會令韌體大約多 300KB，2MB 分區不夠。新分區表要按 app 各 4MB 定，並在 11/13 凍結前把藍牙版本編譯一次確認大小。</t>
+[2026-10-12] 2026-10-12：藍牙配網（R-21）會令韌體大約多 300KB，2MB 分區不夠。新分區表要按 app 各 4MB 定，並在 11/13 凍結前把藍牙版本編譯一次確認大小。
+[2026-10-14] 2026-10-14：用戶要求把配網提示音放進韌體；7 句 16kHz PCM 約 420KB，編進 app 後映像 2,147,728 bytes 超過 2MB 槽，板子在 bootloader 循環重啟（pio 仍報 Flash 99% SUCCESS）。按路線圖改放品牌資源分區。分區表待用戶確認後才算定案。
+[2026-10-14] 2026-10-14 用戶定案 partition_16m.csv：nvs 0x9000/20K、otadata 0xe000/8K（不變）、app0 0x10000/4MB、app1 0x410000/4MB、assets 0x810000/2MB（品牌聲音）、nvs_keys 0xa10000/4K（P0-14）、coredump 0xa20000/64K、media 0xa30000/5.8MB（R-14）。spotpear-ai-toy 全部 env 改用此表；R-21 藍牙探針版映像 2,326,128 bytes，在 4MB 槽內。</t>
         </is>
       </c>
     </row>
@@ -8707,8 +9031,546 @@
         </is>
       </c>
     </row>
+    <row r="81" ht="102" customHeight="1">
+      <c r="A81" s="13" t="inlineStr">
+        <is>
+          <t>P2-13</t>
+        </is>
+      </c>
+      <c r="B81" s="13" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C81" s="13" t="inlineStr">
+        <is>
+          <t>2 內測準備</t>
+        </is>
+      </c>
+      <c r="D81" s="6" t="inlineStr">
+        <is>
+          <t>運維-後台</t>
+        </is>
+      </c>
+      <c r="E81" s="6" t="inlineStr">
+        <is>
+          <t>Admin 後台改成分組側欄（新頁面先用示例數據預覽）</t>
+        </is>
+      </c>
+      <c r="F81" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="G81" s="13" t="inlineStr">
+        <is>
+          <t>部分通過</t>
+        </is>
+      </c>
+      <c r="I81" s="6" t="inlineStr">
+        <is>
+          <t>原本頂部膠囊分頁只放得下 6 頁，之後要加設備、客服、OTA、出廠、用量、審計等頁面放不下；新頁面要先有固定位置和樣子，再逐頁接上真實數據。</t>
+        </is>
+      </c>
+      <c r="J81" s="6" t="inlineStr">
+        <is>
+          <t>frontend-nextjs/app/components/Admin/AdminDashboard.tsx
+frontend-nextjs/app/components/Admin/adminPages.ts
+frontend-nextjs/app/components/Admin/preview/（示例數據在 previewData.ts）</t>
+        </is>
+      </c>
+      <c r="K81" s="6" t="inlineStr">
+        <is>
+          <t>6 個現有分頁（Model、Latency、Characters、IPs、Accounts、Admins）在新側欄照常使用，讀寫真實數據；內容管理員只看到 Characters 和 IPs；預覽頁和規劃頁只有超級管理員看到，並有橫幅寫明示例數據、按鈕不能用；每頁有 #hash 可直接打開；手機寬度沒有橫向捲動。</t>
+        </is>
+      </c>
+      <c r="L81" s="6" t="inlineStr">
+        <is>
+          <t>① tsc 通過 ② 用略過登入的測試頁檢查超級管理員和內容管理員兩種視角、桌面和手機寬度、#hash 直接打開 ③ 用真實超級管理員帳號登入 /admin，逐頁確認讀到真實數據（Model 讀到 OpenRouter 模型目錄、Latency 有記錄、Characters 可編輯並保存）④ 用內容管理員帳號登入，側欄只有 Characters、IPs</t>
+        </is>
+      </c>
+      <c r="M81" s="13" t="n"/>
+      <c r="N81" s="6" t="inlineStr">
+        <is>
+          <t>① tsc --noEmit 通過 ② 略過登入的測試頁（另一份副本、獨立 .next）：超級管理員 15 頁、內容管理員只見 Characters／IPs；1360px 與 375px 均無橫向捲動（scrollWidth=clientWidth=375）；#audit 直接打開正確；③④ 未做：需真實帳號登入 /admin</t>
+        </is>
+      </c>
+      <c r="O81" s="13" t="inlineStr">
+        <is>
+          <t>77fc4f7</t>
+        </is>
+      </c>
+      <c r="P81" s="6" t="inlineStr">
+        <is>
+          <t>[2026-10-14] 新增</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="60" customHeight="1">
+      <c r="A82" s="13" t="inlineStr">
+        <is>
+          <t>P1-13</t>
+        </is>
+      </c>
+      <c r="B82" s="13" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C82" s="13" t="inlineStr">
+        <is>
+          <t>2 內測準備</t>
+        </is>
+      </c>
+      <c r="D82" s="6" t="inlineStr">
+        <is>
+          <t>安全-權限</t>
+        </is>
+      </c>
+      <c r="E82" s="6" t="inlineStr">
+        <is>
+          <t>PLACEHOLDER</t>
+        </is>
+      </c>
+      <c r="F82" s="13" t="inlineStr">
+        <is>
+          <t>不適用</t>
+        </is>
+      </c>
+      <c r="G82" s="13" t="inlineStr">
+        <is>
+          <t>未測試</t>
+        </is>
+      </c>
+      <c r="I82" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="J82" s="6" t="n"/>
+      <c r="K82" s="6" t="n"/>
+      <c r="L82" s="6" t="n"/>
+      <c r="M82" s="13" t="n"/>
+      <c r="P82" s="6" t="inlineStr">
+        <is>
+          <t>[2026-10-14] 新增
+[2026-10-14] 2026-10-14 新增任務時指令打錯而誤建的空白行，沒有內容，不代表任何工作。</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="102" customHeight="1">
+      <c r="A83" s="13" t="inlineStr">
+        <is>
+          <t>P2-14</t>
+        </is>
+      </c>
+      <c r="B83" s="13" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C83" s="13" t="inlineStr">
+        <is>
+          <t>2 內測準備</t>
+        </is>
+      </c>
+      <c r="D83" s="6" t="inlineStr">
+        <is>
+          <t>運維-後台</t>
+        </is>
+      </c>
+      <c r="E83" s="6" t="inlineStr">
+        <is>
+          <t>Admin 設備頁：每台玩具的狀態、韌體與基本操作</t>
+        </is>
+      </c>
+      <c r="F83" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="G83" s="13" t="inlineStr">
+        <is>
+          <t>未測試</t>
+        </is>
+      </c>
+      <c r="I83" s="6" t="inlineStr">
+        <is>
+          <t>內部測試有 20 台在外面，玩具連不上時只能直接查資料庫或靠家長描述；NVS 被清空後要手動刪 device_secrets 那一行。數據大多已在 devices 表（last_seen_at、firmware_version、ota_failed_*、claimed_at），只是沒有地方顯示。</t>
+        </is>
+      </c>
+      <c r="J83" s="6" t="inlineStr">
+        <is>
+          <t>frontend-nextjs/app/components/Admin/preview/DevicesPreview.tsx（換成真實數據）
+devices、device_secrets 表
+server/fastapi/server.py（在線狀態：device_wifi.snapshot 已有 online，需開一個只讀的內部接口）</t>
+        </is>
+      </c>
+      <c r="K83" s="6" t="inlineStr">
+        <is>
+          <t>列出全部設備，可按 MAC、設備名、家長 email 搜尋，按狀態和韌體篩選；顯示在線／離線（取自語音伺服器）、上次上線、韌體版本、OTA 失敗版本、綁定帳號與時間、出廠鎖定的 IP；單台詳情可做「重置設備密鑰」「強制解綁」，兩者都要填原因並寫入審計記錄（P1-10）；不顯示任何對話、記憶或孩子資料（Q7）；只有超級管理員能讀。</t>
+        </is>
+      </c>
+      <c r="L83" s="6" t="inlineStr">
+        <is>
+          <t>① 開發板 62:70 開機 → 1 分鐘內顯示在線；拔電 → 顯示離線 ② 對開發板「重置設備密鑰」→ device_secrets 該行刪除，板子重開後重新登記成功 ③「強制解綁」一台測試設備 → 設備回到配對狀態，審計表多一筆含原因 ④ 用內容管理員 JWT 讀 devices 管理接口被拒</t>
+        </is>
+      </c>
+      <c r="M83" s="13" t="inlineStr">
+        <is>
+          <t>P1-10, P2-13</t>
+        </is>
+      </c>
+      <c r="P83" s="6" t="inlineStr">
+        <is>
+          <t>[2026-10-14] 新增</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="88" customHeight="1">
+      <c r="A84" s="13" t="inlineStr">
+        <is>
+          <t>P2-15</t>
+        </is>
+      </c>
+      <c r="B84" s="13" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C84" s="13" t="inlineStr">
+        <is>
+          <t>3 封閉內測</t>
+        </is>
+      </c>
+      <c r="D84" s="6" t="inlineStr">
+        <is>
+          <t>運維-後台</t>
+        </is>
+      </c>
+      <c r="E84" s="6" t="inlineStr">
+        <is>
+          <t>Admin 總覽頁：在線、用量、成本與待處理事項</t>
+        </is>
+      </c>
+      <c r="F84" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="G84" s="13" t="inlineStr">
+        <is>
+          <t>未測試</t>
+        </is>
+      </c>
+      <c r="I84" s="6" t="inlineStr">
+        <is>
+          <t>每天要逐頁看才知道有沒有問題；內部測試期間需要一眼看到在線數、今日成本和要處理的設備。</t>
+        </is>
+      </c>
+      <c r="J84" s="6" t="inlineStr">
+        <is>
+          <t>frontend-nextjs/app/components/Admin/preview/OverviewPreview.tsx（換成真實數據）</t>
+        </is>
+      </c>
+      <c r="K84" s="6" t="inlineStr">
+        <is>
+          <t>顯示：在線玩具／已綁定、今日對話輪數、今日成本與每台成本、待處理數；近 14 天活躍設備與輪數趨勢；韌體版本分佈；待處理清單（OTA 回滾、用量異常、供應商錯誤率），每項可跳到對應頁；最近管理操作取自審計記錄。所有數字與設備頁、用量頁一致。</t>
+        </is>
+      </c>
+      <c r="L84" s="6" t="inlineStr">
+        <is>
+          <t>用 SQL 直接算同一天的在線數、輪數、成本和韌體分佈，與總覽頁數字逐項對照一致；製造一台 OTA 回滾（ota_failed_version）→ 出現在待處理並能跳到該設備</t>
+        </is>
+      </c>
+      <c r="M84" s="13" t="inlineStr">
+        <is>
+          <t>P2-14, P2-09</t>
+        </is>
+      </c>
+      <c r="P84" s="6" t="inlineStr">
+        <is>
+          <t>[2026-10-14] 新增</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="102" customHeight="1">
+      <c r="A85" s="13" t="inlineStr">
+        <is>
+          <t>P2-16</t>
+        </is>
+      </c>
+      <c r="B85" s="13" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C85" s="13" t="inlineStr">
+        <is>
+          <t>4 量產出貨</t>
+        </is>
+      </c>
+      <c r="D85" s="6" t="inlineStr">
+        <is>
+          <t>運維-OTA</t>
+        </is>
+      </c>
+      <c r="E85" s="6" t="inlineStr">
+        <is>
+          <t>OTA 分批推送與後台發佈頁</t>
+        </is>
+      </c>
+      <c r="F85" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="G85" s="13" t="inlineStr">
+        <is>
+          <t>未測試</t>
+        </is>
+      </c>
+      <c r="I85" s="6" t="inlineStr">
+        <is>
+          <t>現在設為 current 的版本會一次推給該板型的所有設備；3,000 台出貨後，一個壞版本會同時推給全部設備。發佈只能在 Mac 上用 release_firmware.py，要手動貼 service key。分批推送只改伺服器決定哪台收到 ota，不用改韌體，所以不受 11/27 韌體定版的時限限制，但必須在出貨後第一次 OTA 之前完成。</t>
+        </is>
+      </c>
+      <c r="J85" s="6" t="inlineStr">
+        <is>
+          <t>frontend-nextjs/app/components/Admin/preview/OtaPreview.tsx（換成真實數據）
+frontend-nextjs/app/api/generate_auth_token/route.ts（回傳 ota 的地方）
+firmware_releases 表、firmware-arduino/tools/release_firmware.py</t>
+        </is>
+      </c>
+      <c r="K85" s="6" t="inlineStr">
+        <is>
+          <t>後台可上傳韌體（伺服器算 SHA-256、寫 firmware_releases）、填說明、設為 current；推送分階段：白名單 MAC → 10% → 50% → 100%，按 MAC 雜湊穩定分組；回滾率超過 5% 或任一台在試用期內重啟 3 次即自動暫停；顯示每個版本已更新、回滾台數與回滾設備清單；顯示 app 分區用量（P2-12）；每個發佈操作寫入審計記錄。</t>
+        </is>
+      </c>
+      <c r="L85" s="6" t="inlineStr">
+        <is>
+          <t>本機 Supabase + 裝置模擬器（2bb6656）模擬 20 台：① 10% 階段只有約 2 台拿到 ota，重複請求結果不變 ② 讓 2 台回報 failed_version → 自動暫停，其餘不再拿到 ota ③ 推到 100% 全部拿到 ④ 開發板 62:70 實機走一次白名單階段並確認新版本 ⑤ 審計表有每次階段變更</t>
+        </is>
+      </c>
+      <c r="M85" s="13" t="inlineStr">
+        <is>
+          <t>P0-13, P2-14, P1-10</t>
+        </is>
+      </c>
+      <c r="P85" s="6" t="inlineStr">
+        <is>
+          <t>[2026-10-14] 新增</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="130" customHeight="1">
+      <c r="A86" s="13" t="inlineStr">
+        <is>
+          <t>R-39</t>
+        </is>
+      </c>
+      <c r="B86" s="13" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="C86" s="13" t="inlineStr">
+        <is>
+          <t>3 封閉內測</t>
+        </is>
+      </c>
+      <c r="D86" s="6" t="inlineStr">
+        <is>
+          <t>生產</t>
+        </is>
+      </c>
+      <c r="E86" s="6" t="inlineStr">
+        <is>
+          <t>Admin 出廠登記頁：匯入 MAC 清單、指定公仔、查看自檢結果</t>
+        </is>
+      </c>
+      <c r="F86" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="G86" s="13" t="inlineStr">
+        <is>
+          <t>未測試</t>
+        </is>
+      </c>
+      <c r="I86" s="6" t="inlineStr">
+        <is>
+          <t>3,000 台的 MAC、公仔和 IP 不可能逐台手動改資料庫；工位登記結果（R-10）要有地方看，才知道哪批哪台沒通過。要在 12/14 量產前跟工位腳本一起用小批量試產跑通。</t>
+        </is>
+      </c>
+      <c r="J86" s="6" t="inlineStr">
+        <is>
+          <t>frontend-nextjs/app/components/Admin/preview/FactoryPreview.tsx（換成真實數據）
+新表：出廠批次與每台 QC 記錄
+R-10 工位腳本的登記接口</t>
+        </is>
+      </c>
+      <c r="K86" s="6" t="inlineStr">
+        <is>
+          <t>可匯入 Spotpear 的 MAC 清單 CSV（MAC、批次、日期），重複或格式錯誤的行跳過並列出；每批顯示已匯入、已寫密鑰、自檢通過、自檢失敗、未開始的數量；可整批為未寫密鑰的板子指定公仔（IP）；顯示工位回傳的每台自檢結果（咪、喇叭、燈、按鍵、Wi-Fi）與失敗原因；寫入密鑰後公仔鎖定，只有超級管理員能在此改，家長端不能改（R-38）；可匯出失敗清單；只看到分配給本部署的板子；匯入和指定都寫入審計記錄。</t>
+        </is>
+      </c>
+      <c r="L86" s="6" t="inlineStr">
+        <is>
+          <t>① 匯入 300 行 CSV，其中 3 行重複、1 行格式錯 → 新增 296 行並列出 4 行 ② 為 20 台指定公仔後，工位腳本處理其中 10 台 → 進度與 QC 記錄正確，已寫密鑰的不能再改公仔 ③ 匯出失敗清單內容與 QC 記錄一致</t>
+        </is>
+      </c>
+      <c r="M86" s="13" t="inlineStr">
+        <is>
+          <t>R-38, P1-10</t>
+        </is>
+      </c>
+      <c r="P86" s="6" t="inlineStr">
+        <is>
+          <t>[2026-10-14] 新增</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="116" customHeight="1">
+      <c r="A87" s="13" t="inlineStr">
+        <is>
+          <t>R-40</t>
+        </is>
+      </c>
+      <c r="B87" s="13" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="C87" s="13" t="inlineStr">
+        <is>
+          <t>4 量產出貨</t>
+        </is>
+      </c>
+      <c r="D87" s="6" t="inlineStr">
+        <is>
+          <t>營運</t>
+        </is>
+      </c>
+      <c r="E87" s="6" t="inlineStr">
+        <is>
+          <t>Admin 客服查詢頁：查帳號、名下設備與最近事件</t>
+        </is>
+      </c>
+      <c r="F87" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="G87" s="13" t="inlineStr">
+        <is>
+          <t>未測試</t>
+        </is>
+      </c>
+      <c r="I87" s="6" t="inlineStr">
+        <is>
+          <t>家長來電時要能用一個搜尋找到帳號和玩具；R-11 要求的報修、診斷、換機流程現在沒有工具，只能直接改資料庫。</t>
+        </is>
+      </c>
+      <c r="J87" s="6" t="inlineStr">
+        <is>
+          <t>frontend-nextjs/app/components/Admin/preview/SupportPreview.tsx（換成真實數據）
+auth.users（service role，只在伺服器端讀）
+devices、users 表</t>
+        </is>
+      </c>
+      <c r="K87" s="6" t="inlineStr">
+        <is>
+          <t>可用 email、MAC 或設備名稱後四位查到帳號；顯示註冊時間、登入方式、家長鎖與使用上限設定、名下設備（狀態、韌體、上次上線）和最近的系統事件（連線失敗、OTA、綁定、Wi-Fi 變更）；動作：解綁、換機（解綁舊機、綁新機、記憶搬到新設備，按 P1-12 的定案）、重發登入驗證碼、刪除帳號及資料；每個動作要填原因並寫入審計記錄；不顯示對話、記憶、孩子的性格描述（Q7）。</t>
+        </is>
+      </c>
+      <c r="L87" s="6" t="inlineStr">
+        <is>
+          <t>按 R-11 演練一次：用測試帳號模擬家長報修 → 在客服頁找到帳號和設備、看到事件 → 換機到另一台測試設備，新設備保留記憶 → 審計表有每一步；刪除測試帳號後，其對話、記憶和綁定都已刪除</t>
+        </is>
+      </c>
+      <c r="M87" s="13" t="inlineStr">
+        <is>
+          <t>P2-14, P1-10, P1-12</t>
+        </is>
+      </c>
+      <c r="P87" s="6" t="inlineStr">
+        <is>
+          <t>[2026-10-14] 新增</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="74" customHeight="1">
+      <c r="A88" s="13" t="inlineStr">
+        <is>
+          <t>P1-14</t>
+        </is>
+      </c>
+      <c r="B88" s="13" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C88" s="13" t="inlineStr">
+        <is>
+          <t>3 封閉內測</t>
+        </is>
+      </c>
+      <c r="D88" s="6" t="inlineStr">
+        <is>
+          <t>兒童安全</t>
+        </is>
+      </c>
+      <c r="E88" s="6" t="inlineStr">
+        <is>
+          <t>Admin 內容安全頁：審核事件只按類別統計</t>
+        </is>
+      </c>
+      <c r="F88" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="G88" s="13" t="inlineStr">
+        <is>
+          <t>未測試</t>
+        </is>
+      </c>
+      <c r="I88" s="6" t="inlineStr">
+        <is>
+          <t>P1-01 審核層會記錄攔截事件，但沒有地方看；某台設備或某個角色攔截突然變多時沒人知道。</t>
+        </is>
+      </c>
+      <c r="J88" s="6" t="inlineStr">
+        <is>
+          <t>frontend-nextjs/app/components/Admin/adminPages.ts（目前是規劃頁 safety）
+P1-01 的審核事件表</t>
+        </is>
+      </c>
+      <c r="K88" s="6" t="inlineStr">
+        <is>
+          <t>按日顯示輸入和回覆被攔截的次數，只按類別（暴力、性、個人資料、自我傷害等），不顯示原文（Q7）；可按角色和設備看攔截率；單台設備單日攔截數超過門檻時出現在總覽的待處理；只有超級管理員能讀。</t>
+        </is>
+      </c>
+      <c r="L88" s="6" t="inlineStr">
+        <is>
+          <t>在測試設備上觸發每個類別各 3 次 → 頁面計數與審核事件表一致；資料庫和頁面回應中都找不到觸發用的原文</t>
+        </is>
+      </c>
+      <c r="M88" s="13" t="inlineStr">
+        <is>
+          <t>P1-01, P2-13</t>
+        </is>
+      </c>
+      <c r="P88" s="6" t="inlineStr">
+        <is>
+          <t>[2026-10-14] 新增</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P80"/>
+  <autoFilter ref="A1:P88"/>
   <conditionalFormatting sqref="F2:F1000">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"已完成"</formula>
@@ -9289,7 +10151,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I227"/>
+  <dimension ref="A1:I253"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -17156,8 +18018,862 @@
         </is>
       </c>
     </row>
+    <row r="228" ht="32" customHeight="1">
+      <c r="A228" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 10:25</t>
+        </is>
+      </c>
+      <c r="B228" s="13" t="inlineStr">
+        <is>
+          <t>P2-12</t>
+        </is>
+      </c>
+      <c r="C228" s="6" t="inlineStr">
+        <is>
+          <t>量產燒錄前加大 app 分區</t>
+        </is>
+      </c>
+      <c r="D228" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E228" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F228" s="13" t="n"/>
+      <c r="G228" s="6" t="n"/>
+      <c r="H228" s="13" t="n"/>
+      <c r="I228" s="6" t="n"/>
+    </row>
+    <row r="229" ht="200" customHeight="1">
+      <c r="A229" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 10:25</t>
+        </is>
+      </c>
+      <c r="B229" s="13" t="inlineStr">
+        <is>
+          <t>P2-12</t>
+        </is>
+      </c>
+      <c r="C229" s="6" t="inlineStr">
+        <is>
+          <t>量產燒錄前加大 app 分區</t>
+        </is>
+      </c>
+      <c r="D229" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="E229" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F229" s="13" t="inlineStr">
+        <is>
+          <t>部分通過</t>
+        </is>
+      </c>
+      <c r="G229" s="6" t="inlineStr">
+        <is>
+          <t>62:70（分支 p2-12-partitions，env spotpear-ai-toy-p212，partition_16m.csv：app0/app1 各 4MB、assets 2MB、nvs_keys、coredump、media 5.8MB；nvs/otadata 位置不變，USB 換表後 Wi-Fi 與設備密鑰保留）：① 本機 OTA 1.6.1→1.6.2 寫入新 app1，Voice server reached 後 120s『Firmware 1.6.2 confirmed』② 推 3 秒 abort 的 1.6.3 → PANIC → 回到 1.6.2，devices.ota_failed_version=1.6.3 ③ 崩潰寫入 coredump 分區 14.8KB ④ 資源分區 9 個聲音 504KB（25%），開機 CRC 63ms，OTA 後照常；損壞/清空 → 退回內建聲音無崩潰 ⑤ 映像 1,591,168 bytes &lt; 4MB；release_firmware.py 加映像 &gt; app 槽即拒發。未做：雲端 OTA、pio 全 env 編譯、R-21 藍牙版在新表上的大小、正式 env 改用新表、寫入出廠腳本（R-10）</t>
+        </is>
+      </c>
+      <c r="H229" s="13" t="inlineStr">
+        <is>
+          <t>99204e9</t>
+        </is>
+      </c>
+      <c r="I229" s="6" t="n"/>
+    </row>
+    <row r="230" ht="102" customHeight="1">
+      <c r="A230" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 10:25</t>
+        </is>
+      </c>
+      <c r="B230" s="13" t="inlineStr">
+        <is>
+          <t>P2-12</t>
+        </is>
+      </c>
+      <c r="C230" s="6" t="inlineStr">
+        <is>
+          <t>量產燒錄前加大 app 分區</t>
+        </is>
+      </c>
+      <c r="D230" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="E230" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F230" s="13" t="n"/>
+      <c r="G230" s="6" t="n"/>
+      <c r="H230" s="13" t="n"/>
+      <c r="I230" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-14：用戶要求把配網提示音放進韌體；7 句 16kHz PCM 約 420KB，編進 app 後映像 2,147,728 bytes 超過 2MB 槽，板子在 bootloader 循環重啟（pio 仍報 Flash 99% SUCCESS）。按路線圖改放品牌資源分區。分區表待用戶確認後才算定案。</t>
+        </is>
+      </c>
+    </row>
+    <row r="231" ht="144" customHeight="1">
+      <c r="A231" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 10:28</t>
+        </is>
+      </c>
+      <c r="B231" s="13" t="inlineStr">
+        <is>
+          <t>P2-12</t>
+        </is>
+      </c>
+      <c r="C231" s="6" t="inlineStr">
+        <is>
+          <t>量產燒錄前加大 app 分區</t>
+        </is>
+      </c>
+      <c r="D231" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="E231" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F231" s="13" t="n"/>
+      <c r="G231" s="6" t="n"/>
+      <c r="H231" s="13" t="n"/>
+      <c r="I231" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-14 用戶定案 partition_16m.csv：nvs 0x9000/20K、otadata 0xe000/8K（不變）、app0 0x10000/4MB、app1 0x410000/4MB、assets 0x810000/2MB（品牌聲音）、nvs_keys 0xa10000/4K（P0-14）、coredump 0xa20000/64K、media 0xa30000/5.8MB（R-14）。spotpear-ai-toy 全部 env 改用此表；R-21 藍牙探針版映像 2,326,128 bytes，在 4MB 槽內。</t>
+        </is>
+      </c>
+    </row>
+    <row r="232" ht="74" customHeight="1">
+      <c r="A232" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 10:29</t>
+        </is>
+      </c>
+      <c r="B232" s="13" t="inlineStr">
+        <is>
+          <t>R-10</t>
+        </is>
+      </c>
+      <c r="C232" s="6" t="inlineStr">
+        <is>
+          <t>出廠流程</t>
+        </is>
+      </c>
+      <c r="D232" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E232" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="F232" s="13" t="n"/>
+      <c r="G232" s="6" t="n"/>
+      <c r="H232" s="13" t="n"/>
+      <c r="I232" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-14：P2-12 定案後，工位多一步：按品牌寫入資源包（tools/build_assets.py --brand ... → esptool write_flash 0x810000），開機 log『Assets: brand ...crc ok』作自檢一項。</t>
+        </is>
+      </c>
+    </row>
+    <row r="233" ht="32" customHeight="1">
+      <c r="A233" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 10:33</t>
+        </is>
+      </c>
+      <c r="B233" s="13" t="inlineStr">
+        <is>
+          <t>P2-13</t>
+        </is>
+      </c>
+      <c r="C233" s="6" t="inlineStr">
+        <is>
+          <t>Admin 後台改成分組側欄（新頁面先用示例數據預覽）</t>
+        </is>
+      </c>
+      <c r="E233" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="I233" s="6" t="inlineStr">
+        <is>
+          <t>新增任務</t>
+        </is>
+      </c>
+    </row>
+    <row r="234" ht="32" customHeight="1">
+      <c r="A234" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 10:33</t>
+        </is>
+      </c>
+      <c r="B234" s="13" t="inlineStr">
+        <is>
+          <t>P1-13</t>
+        </is>
+      </c>
+      <c r="C234" s="6" t="inlineStr">
+        <is>
+          <t>PLACEHOLDER</t>
+        </is>
+      </c>
+      <c r="E234" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="I234" s="6" t="inlineStr">
+        <is>
+          <t>新增任務</t>
+        </is>
+      </c>
+    </row>
+    <row r="235" ht="46" customHeight="1">
+      <c r="A235" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 10:34</t>
+        </is>
+      </c>
+      <c r="B235" s="13" t="inlineStr">
+        <is>
+          <t>P1-13</t>
+        </is>
+      </c>
+      <c r="C235" s="6" t="inlineStr">
+        <is>
+          <t>PLACEHOLDER</t>
+        </is>
+      </c>
+      <c r="D235" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E235" s="13" t="inlineStr">
+        <is>
+          <t>不適用</t>
+        </is>
+      </c>
+      <c r="F235" s="13" t="n"/>
+      <c r="G235" s="6" t="n"/>
+      <c r="H235" s="13" t="n"/>
+      <c r="I235" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-14 新增任務時指令打錯而誤建的空白行，沒有內容，不代表任何工作。</t>
+        </is>
+      </c>
+    </row>
+    <row r="236" ht="32" customHeight="1">
+      <c r="A236" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 10:34</t>
+        </is>
+      </c>
+      <c r="B236" s="13" t="inlineStr">
+        <is>
+          <t>P2-14</t>
+        </is>
+      </c>
+      <c r="C236" s="6" t="inlineStr">
+        <is>
+          <t>Admin 設備頁：每台玩具的狀態、韌體與基本操作</t>
+        </is>
+      </c>
+      <c r="E236" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="I236" s="6" t="inlineStr">
+        <is>
+          <t>新增任務</t>
+        </is>
+      </c>
+    </row>
+    <row r="237" ht="32" customHeight="1">
+      <c r="A237" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 10:34</t>
+        </is>
+      </c>
+      <c r="B237" s="13" t="inlineStr">
+        <is>
+          <t>P2-15</t>
+        </is>
+      </c>
+      <c r="C237" s="6" t="inlineStr">
+        <is>
+          <t>Admin 總覽頁：在線、用量、成本與待處理事項</t>
+        </is>
+      </c>
+      <c r="E237" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="I237" s="6" t="inlineStr">
+        <is>
+          <t>新增任務</t>
+        </is>
+      </c>
+    </row>
+    <row r="238" ht="32" customHeight="1">
+      <c r="A238" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 10:35</t>
+        </is>
+      </c>
+      <c r="B238" s="13" t="inlineStr">
+        <is>
+          <t>P2-15</t>
+        </is>
+      </c>
+      <c r="C238" s="6" t="inlineStr">
+        <is>
+          <t>Admin 總覽頁：在線、用量、成本與待處理事項</t>
+        </is>
+      </c>
+      <c r="D238" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E238" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="F238" s="13" t="n"/>
+      <c r="G238" s="6" t="n"/>
+      <c r="H238" s="13" t="n"/>
+      <c r="I238" s="6" t="inlineStr">
+        <is>
+          <t>修改了依賴→P2-14, P2-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="239" ht="32" customHeight="1">
+      <c r="A239" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 10:35</t>
+        </is>
+      </c>
+      <c r="B239" s="13" t="inlineStr">
+        <is>
+          <t>P2-16</t>
+        </is>
+      </c>
+      <c r="C239" s="6" t="inlineStr">
+        <is>
+          <t>OTA 分批推送與後台發佈頁</t>
+        </is>
+      </c>
+      <c r="E239" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="I239" s="6" t="inlineStr">
+        <is>
+          <t>新增任務</t>
+        </is>
+      </c>
+    </row>
+    <row r="240" ht="32" customHeight="1">
+      <c r="A240" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 10:35</t>
+        </is>
+      </c>
+      <c r="B240" s="13" t="inlineStr">
+        <is>
+          <t>R-39</t>
+        </is>
+      </c>
+      <c r="C240" s="6" t="inlineStr">
+        <is>
+          <t>Admin 出廠登記頁：匯入 MAC 清單、指定公仔、查看自檢結果</t>
+        </is>
+      </c>
+      <c r="E240" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="I240" s="6" t="inlineStr">
+        <is>
+          <t>新增任務</t>
+        </is>
+      </c>
+    </row>
+    <row r="241" ht="32" customHeight="1">
+      <c r="A241" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 10:35</t>
+        </is>
+      </c>
+      <c r="B241" s="13" t="inlineStr">
+        <is>
+          <t>R-40</t>
+        </is>
+      </c>
+      <c r="C241" s="6" t="inlineStr">
+        <is>
+          <t>Admin 客服查詢頁：查帳號、名下設備與最近事件</t>
+        </is>
+      </c>
+      <c r="E241" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="I241" s="6" t="inlineStr">
+        <is>
+          <t>新增任務</t>
+        </is>
+      </c>
+    </row>
+    <row r="242" ht="32" customHeight="1">
+      <c r="A242" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 10:35</t>
+        </is>
+      </c>
+      <c r="B242" s="13" t="inlineStr">
+        <is>
+          <t>P1-14</t>
+        </is>
+      </c>
+      <c r="C242" s="6" t="inlineStr">
+        <is>
+          <t>Admin 內容安全頁：審核事件只按類別統計</t>
+        </is>
+      </c>
+      <c r="E242" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="I242" s="6" t="inlineStr">
+        <is>
+          <t>新增任務</t>
+        </is>
+      </c>
+    </row>
+    <row r="243" ht="74" customHeight="1">
+      <c r="A243" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 10:35</t>
+        </is>
+      </c>
+      <c r="B243" s="13" t="inlineStr">
+        <is>
+          <t>R-10</t>
+        </is>
+      </c>
+      <c r="C243" s="6" t="inlineStr">
+        <is>
+          <t>出廠流程</t>
+        </is>
+      </c>
+      <c r="D243" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E243" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="F243" s="13" t="n"/>
+      <c r="G243" s="6" t="n"/>
+      <c r="H243" s="13" t="n"/>
+      <c r="I243" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-14：後台的 MAC 清單匯入、整批指定公仔、QC 結果查看拆成 R-39，與工位腳本一起試產。；修改了依賴→P0-06, P0-14, R-01, P2-12, Q10, R-34, R-35, R-38, R-39</t>
+        </is>
+      </c>
+    </row>
+    <row r="244" ht="60" customHeight="1">
+      <c r="A244" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 10:35</t>
+        </is>
+      </c>
+      <c r="B244" s="13" t="inlineStr">
+        <is>
+          <t>R-11</t>
+        </is>
+      </c>
+      <c r="C244" s="6" t="inlineStr">
+        <is>
+          <t>售後：客服、保修與換機</t>
+        </is>
+      </c>
+      <c r="D244" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E244" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="F244" s="13" t="n"/>
+      <c r="G244" s="6" t="n"/>
+      <c r="H244" s="13" t="n"/>
+      <c r="I244" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-14：admin 端的診斷靠設備頁（P2-14），報修、換機、刪帳號的工具在客服查詢頁（R-40）。；修改了依賴→P2-14, R-40</t>
+        </is>
+      </c>
+    </row>
+    <row r="245" ht="102" customHeight="1">
+      <c r="A245" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 10:35</t>
+        </is>
+      </c>
+      <c r="B245" s="13" t="inlineStr">
+        <is>
+          <t>P1-10</t>
+        </is>
+      </c>
+      <c r="C245" s="6" t="inlineStr">
+        <is>
+          <t>管理操作審計記錄</t>
+        </is>
+      </c>
+      <c r="D245" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E245" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="F245" s="13" t="n"/>
+      <c r="G245" s="6" t="n"/>
+      <c r="H245" s="13" t="n"/>
+      <c r="I245" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-14：admin 改側欄後（P2-13），actions.ts 在 frontend-nextjs/app/admin/actions.ts；審計記錄頁的樣子在 preview/AuditPreview.tsx。建議第一個做：設備頁、客服頁、OTA、出廠的每個動作都要寫審計，先有這張表就不用回頭改。</t>
+        </is>
+      </c>
+    </row>
+    <row r="246" ht="130" customHeight="1">
+      <c r="A246" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 10:35</t>
+        </is>
+      </c>
+      <c r="B246" s="13" t="inlineStr">
+        <is>
+          <t>P2-09</t>
+        </is>
+      </c>
+      <c r="C246" s="6" t="inlineStr">
+        <is>
+          <t>每台設備成本監控</t>
+        </is>
+      </c>
+      <c r="D246" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E246" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="F246" s="13" t="n"/>
+      <c r="G246" s="6" t="n"/>
+      <c r="H246" s="13" t="n"/>
+      <c r="I246" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-14：turn_metrics 目前只記 user_id 和 chat_group_id，沒有設備，也沒有 STT 秒數（只有 transcript_chars／response_chars），要改語音伺服器補上，並加單價表。頁面樣子在 preview/UsagePreview.tsx。內部測試每週要報每台每月成本（R-07），數據只能從開始記錄那天累積，建議 10/30 前做好。</t>
+        </is>
+      </c>
+    </row>
+    <row r="247" ht="46" customHeight="1">
+      <c r="A247" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 10:35</t>
+        </is>
+      </c>
+      <c r="B247" s="13" t="inlineStr">
+        <is>
+          <t>P2-06</t>
+        </is>
+      </c>
+      <c r="C247" s="6" t="inlineStr">
+        <is>
+          <t>錯誤追蹤與告警</t>
+        </is>
+      </c>
+      <c r="D247" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E247" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="F247" s="13" t="n"/>
+      <c r="G247" s="6" t="n"/>
+      <c r="H247" s="13" t="n"/>
+      <c r="I247" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-14：admin 的「系統健康」頁只放摘要和外部監控連結，錯誤追蹤與告警用外部服務，不在後台自己做。</t>
+        </is>
+      </c>
+    </row>
+    <row r="248" ht="32" customHeight="1">
+      <c r="A248" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 10:35</t>
+        </is>
+      </c>
+      <c r="B248" s="13" t="inlineStr">
+        <is>
+          <t>P1-01</t>
+        </is>
+      </c>
+      <c r="C248" s="6" t="inlineStr">
+        <is>
+          <t>加入內容審核層（輸入與輸出）</t>
+        </is>
+      </c>
+      <c r="D248" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E248" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="F248" s="13" t="n"/>
+      <c r="G248" s="6" t="n"/>
+      <c r="H248" s="13" t="n"/>
+      <c r="I248" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-14：審核事件的後台頁拆成 P1-14，等本項完成後做。</t>
+        </is>
+      </c>
+    </row>
+    <row r="249" ht="32" customHeight="1">
+      <c r="A249" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 10:35</t>
+        </is>
+      </c>
+      <c r="B249" s="13" t="inlineStr">
+        <is>
+          <t>P2-13</t>
+        </is>
+      </c>
+      <c r="C249" s="6" t="inlineStr">
+        <is>
+          <t>Admin 後台改成分組側欄（新頁面先用示例數據預覽）</t>
+        </is>
+      </c>
+      <c r="D249" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E249" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F249" s="13" t="n"/>
+      <c r="G249" s="6" t="n"/>
+      <c r="H249" s="13" t="n"/>
+      <c r="I249" s="6" t="n"/>
+    </row>
+    <row r="250" ht="74" customHeight="1">
+      <c r="A250" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 10:35</t>
+        </is>
+      </c>
+      <c r="B250" s="13" t="inlineStr">
+        <is>
+          <t>P2-13</t>
+        </is>
+      </c>
+      <c r="C250" s="6" t="inlineStr">
+        <is>
+          <t>Admin 後台改成分組側欄（新頁面先用示例數據預覽）</t>
+        </is>
+      </c>
+      <c r="D250" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="E250" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F250" s="13" t="inlineStr">
+        <is>
+          <t>部分通過</t>
+        </is>
+      </c>
+      <c r="G250" s="6" t="inlineStr">
+        <is>
+          <t>① tsc --noEmit 通過 ② 略過登入的測試頁（另一份副本、獨立 .next）：超級管理員 15 頁、內容管理員只見 Characters／IPs；1360px 與 375px 均無橫向捲動（scrollWidth=clientWidth=375）；#audit 直接打開正確；③④ 未做：需真實帳號登入 /admin</t>
+        </is>
+      </c>
+      <c r="H250" s="13" t="inlineStr">
+        <is>
+          <t>77fc4f7</t>
+        </is>
+      </c>
+      <c r="I250" s="6" t="n"/>
+    </row>
+    <row r="251" ht="32" customHeight="1">
+      <c r="A251" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 10:42</t>
+        </is>
+      </c>
+      <c r="B251" s="13" t="inlineStr">
+        <is>
+          <t>P1-10</t>
+        </is>
+      </c>
+      <c r="C251" s="6" t="inlineStr">
+        <is>
+          <t>管理操作審計記錄</t>
+        </is>
+      </c>
+      <c r="D251" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E251" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F251" s="13" t="n"/>
+      <c r="G251" s="6" t="n"/>
+      <c r="H251" s="13" t="n"/>
+      <c r="I251" s="6" t="n"/>
+    </row>
+    <row r="252" ht="32" customHeight="1">
+      <c r="A252" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 10:42</t>
+        </is>
+      </c>
+      <c r="B252" s="13" t="inlineStr">
+        <is>
+          <t>P2-09</t>
+        </is>
+      </c>
+      <c r="C252" s="6" t="inlineStr">
+        <is>
+          <t>每台設備成本監控</t>
+        </is>
+      </c>
+      <c r="D252" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E252" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F252" s="13" t="n"/>
+      <c r="G252" s="6" t="n"/>
+      <c r="H252" s="13" t="n"/>
+      <c r="I252" s="6" t="n"/>
+    </row>
+    <row r="253" ht="172" customHeight="1">
+      <c r="A253" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 11:03</t>
+        </is>
+      </c>
+      <c r="B253" s="13" t="inlineStr">
+        <is>
+          <t>P2-12</t>
+        </is>
+      </c>
+      <c r="C253" s="6" t="inlineStr">
+        <is>
+          <t>量產燒錄前加大 app 分區</t>
+        </is>
+      </c>
+      <c r="D253" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="E253" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F253" s="13" t="inlineStr">
+        <is>
+          <t>部分通過</t>
+        </is>
+      </c>
+      <c r="G253" s="6" t="inlineStr">
+        <is>
+          <t>62:70（spotpear-ai-toy-p212 原型，現已併入 spotpear-ai-toy）：① 本機 OTA 1.6.1→1.6.2 寫入新 app1，120s 後 confirmed ② 3 秒 abort 的 1.6.3 → PANIC → 回到 1.6.2，ota_failed_version=1.6.3 ③ 崩潰寫入 coredump 14.8KB ④ 資源分區 9 個聲音 504KB/2MB，開機 CRC 63ms，OTA 後照常；損壞/清空 → 退回內建聲音無崩潰 ⑤ pio 全部 18 個 env 編譯通過，映像都在各自 app 槽內（Spotpear 4 個 1.59–1.60MB / 4MB；其他板仍 2MB 槽）；R-21 藍牙探針版 2,326,128 bytes &lt; 4MB ⑥ release_firmware.py 映像 &gt; app 槽即拒發。未做：雲端 OTA 一次（等上 UAT）、出廠腳本寫入資源包（R-10）</t>
+        </is>
+      </c>
+      <c r="H253" s="13" t="inlineStr">
+        <is>
+          <t>5e9ffce</t>
+        </is>
+      </c>
+      <c r="I253" s="6" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I227"/>
+  <autoFilter ref="A1:I253"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add the runbook for the audit log and usage release (P1-10, P2-09).
Takes production from 8db9d9c to dev: backup, the two additive
migrations, then the new voice server and web app, then checks. The voice
server must not start before the migrations, since it writes turn_metrics
columns the old table lacks. Checks run their probes in rolled-back
transactions, and step 6 confirms usage rows after a real board session.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/production-readiness.xlsx
+++ b/docs/production-readiness.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'任務清單'!$A$1:$P$88</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'待確認問題'!$A$1:$G$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$253</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$257</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -665,7 +665,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>最後更新：2026-10-14 11:03　·　本頁由 tracker.py 自動生成，請勿手動編輯</t>
+          <t>最後更新：2026-10-14 11:10　·　本頁由 tracker.py 自動生成，請勿手動編輯</t>
         </is>
       </c>
     </row>
@@ -1358,7 +1358,7 @@
       <c r="H25" s="11" t="n"/>
       <c r="I25" s="12" t="n"/>
     </row>
-    <row r="26" ht="60" customHeight="1">
+    <row r="26" ht="242" customHeight="1">
       <c r="A26" s="13" t="inlineStr">
         <is>
           <t>P1-10</t>
@@ -1381,7 +1381,8 @@
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
-          <t>每個管理操作寫一筆記錄：誰、什麼時間、什麼操作、對象、改之前與改之後的值；記錄只能新增，任何人（包括超級管理員）都不能修改或刪除；超級管理員能在管理端查看。</t>
+          <t>上次測試：部分通過 — 本機（分支 p1-10-p2-09-audit-usage，migration 已套用到本機 Supabase）：探測腳本 22/22，用 GoTrue 真實登入、只把 42501 當拒絕。① 超管改角色 short_description → 1 筆 update、before/after 只有該欄、actor=該管理員；改 voice_stack → 1 筆含新舊值；不改內容再存 → 0 筆 ② 超管 JWT UPDATE/DELETE → 42501；service role DELETE → 42501；postgres DELETE/TRUNCATE 被觸發器拒絕；內容管理員、家長讀 → []；anon → 42501。網頁實測：IP 加一個活動提示 → 只記 1 筆 ip_modes insert，原樣再存 → 0 筆，清除 → 1 筆 delete；Accounts 建帳號 → account.create（不含密碼）；改匯率 → 1 筆。未做：部署線上。
+每個管理操作寫一筆記錄：誰、什麼時間、什麼操作、對象、改之前與改之後的值；記錄只能新增，任何人（包括超級管理員）都不能修改或刪除；超級管理員能在管理端查看。</t>
         </is>
       </c>
       <c r="F26" s="11" t="n"/>
@@ -1421,7 +1422,7 @@
       <c r="H27" s="11" t="n"/>
       <c r="I27" s="12" t="n"/>
     </row>
-    <row r="28" ht="32" customHeight="1">
+    <row r="28" ht="200" customHeight="1">
       <c r="A28" s="13" t="inlineStr">
         <is>
           <t>P2-09</t>
@@ -1444,7 +1445,8 @@
       </c>
       <c r="E28" s="6" t="inlineStr">
         <is>
-          <t>每個 session 記錄 STT 秒數、LLM token、TTS 字數並換算成本；admin 頁顯示每台設備的月成本。</t>
+          <t>上次測試：部分通過 — 本機：pytest 239 passed（新增 8 項：STT/TTS 用量入行、遲到的用量帶到下一行、session 結束寫 usage 行、設備 ID、同一輪多次 LLM 相加、記憶整理的 token 即使回覆解析失敗也記錄並記到該設備）。模擬板子跑 2 輪（本機語音伺服器 7865）：送 2.24s 音訊 → stt_audio_ms=2242（兩輪皆是）；每輪有 tts_chars、token、device_id；session 結束的記憶整理寫成 memory 行（deepseek-v4-flash 946/10 token）。Usage 頁按設備與日期顯示 HK$，改費率即重算並進審計。未做：抽 10 個 session 與 Azure/MiniMax/OpenRouter 帳單對帳（需用戶提供帳單）、部署線上。
+每個 session 記錄 STT 秒數、LLM token、TTS 字數並換算成本；admin 頁顯示每台設備的月成本。</t>
         </is>
       </c>
       <c r="F28" s="11" t="n"/>
@@ -5530,7 +5532,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="144" customHeight="1">
+    <row r="32" ht="256" customHeight="1">
       <c r="A32" s="13" t="inlineStr">
         <is>
           <t>P2-09</t>
@@ -5563,7 +5565,7 @@
       </c>
       <c r="G32" s="13" t="inlineStr">
         <is>
-          <t>未測試</t>
+          <t>部分通過</t>
         </is>
       </c>
       <c r="H32" s="13" t="n"/>
@@ -5589,11 +5591,20 @@
         </is>
       </c>
       <c r="M32" s="13" t="n"/>
-      <c r="N32" s="6" t="n"/>
-      <c r="O32" s="13" t="n"/>
+      <c r="N32" s="6" t="inlineStr">
+        <is>
+          <t>本機：pytest 239 passed（新增 8 項：STT/TTS 用量入行、遲到的用量帶到下一行、session 結束寫 usage 行、設備 ID、同一輪多次 LLM 相加、記憶整理的 token 即使回覆解析失敗也記錄並記到該設備）。模擬板子跑 2 輪（本機語音伺服器 7865）：送 2.24s 音訊 → stt_audio_ms=2242（兩輪皆是）；每輪有 tts_chars、token、device_id；session 結束的記憶整理寫成 memory 行（deepseek-v4-flash 946/10 token）。Usage 頁按設備與日期顯示 HK$，改費率即重算並進審計。未做：抽 10 個 session 與 Azure/MiniMax/OpenRouter 帳單對帳（需用戶提供帳單）、部署線上。</t>
+        </is>
+      </c>
+      <c r="O32" s="13" t="inlineStr">
+        <is>
+          <t>8e3b2c5</t>
+        </is>
+      </c>
       <c r="P32" s="6" t="inlineStr">
         <is>
-          <t>[2026-10-14] 2026-10-14：turn_metrics 目前只記 user_id 和 chat_group_id，沒有設備，也沒有 STT 秒數（只有 transcript_chars／response_chars），要改語音伺服器補上，並加單價表。頁面樣子在 preview/UsagePreview.tsx。內部測試每週要報每台每月成本（R-07），數據只能從開始記錄那天累積，建議 10/30 前做好。</t>
+          <t>[2026-10-14] 2026-10-14：turn_metrics 目前只記 user_id 和 chat_group_id，沒有設備，也沒有 STT 秒數（只有 transcript_chars／response_chars），要改語音伺服器補上，並加單價表。頁面樣子在 preview/UsagePreview.tsx。內部測試每週要報每台每月成本（R-07），數據只能從開始記錄那天累積，建議 10/30 前做好。
+[2026-10-14] 2026-10-14：已合併進 dev（rebase 後 commit 8e3b2c5，原 e438bab）。部署用 docs/deploy/release-2026-10-14-audit-usage.sh：先套兩個 migration，再換語音伺服器和網頁映像；第 5 步自動檢查，第 6 步在跟已綁定的玩具對話後確認用量行。</t>
         </is>
       </c>
     </row>
@@ -6747,7 +6758,7 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="130" customHeight="1">
+    <row r="48" ht="242" customHeight="1">
       <c r="A48" s="13" t="inlineStr">
         <is>
           <t>P1-10</t>
@@ -6780,7 +6791,7 @@
       </c>
       <c r="G48" s="13" t="inlineStr">
         <is>
-          <t>未測試</t>
+          <t>部分通過</t>
         </is>
       </c>
       <c r="H48" s="13" t="n"/>
@@ -6811,12 +6822,21 @@
           <t>P0-12</t>
         </is>
       </c>
-      <c r="N48" s="6" t="n"/>
-      <c r="O48" s="13" t="n"/>
+      <c r="N48" s="6" t="inlineStr">
+        <is>
+          <t>本機（分支 p1-10-p2-09-audit-usage，migration 已套用到本機 Supabase）：探測腳本 22/22，用 GoTrue 真實登入、只把 42501 當拒絕。① 超管改角色 short_description → 1 筆 update、before/after 只有該欄、actor=該管理員；改 voice_stack → 1 筆含新舊值；不改內容再存 → 0 筆 ② 超管 JWT UPDATE/DELETE → 42501；service role DELETE → 42501；postgres DELETE/TRUNCATE 被觸發器拒絕；內容管理員、家長讀 → []；anon → 42501。網頁實測：IP 加一個活動提示 → 只記 1 筆 ip_modes insert，原樣再存 → 0 筆，清除 → 1 筆 delete；Accounts 建帳號 → account.create（不含密碼）；改匯率 → 1 筆。未做：部署線上。</t>
+        </is>
+      </c>
+      <c r="O48" s="13" t="inlineStr">
+        <is>
+          <t>8e3b2c5</t>
+        </is>
+      </c>
       <c r="P48" s="6" t="inlineStr">
         <is>
           <t>[2026-09-30] 新增
-[2026-10-14] 2026-10-14：admin 改側欄後（P2-13），actions.ts 在 frontend-nextjs/app/admin/actions.ts；審計記錄頁的樣子在 preview/AuditPreview.tsx。建議第一個做：設備頁、客服頁、OTA、出廠的每個動作都要寫審計，先有這張表就不用回頭改。</t>
+[2026-10-14] 2026-10-14：admin 改側欄後（P2-13），actions.ts 在 frontend-nextjs/app/admin/actions.ts；審計記錄頁的樣子在 preview/AuditPreview.tsx。建議第一個做：設備頁、客服頁、OTA、出廠的每個動作都要寫審計，先有這張表就不用回頭改。
+[2026-10-14] 2026-10-14：已合併進 dev（rebase 後 commit 8e3b2c5，原 e438bab）。部署用 docs/deploy/release-2026-10-14-audit-usage.sh：先套兩個 migration，再換語音伺服器和網頁映像；第 5 步自動檢查，第 6 步在跟已綁定的玩具對話後確認用量行。</t>
         </is>
       </c>
     </row>
@@ -10151,7 +10171,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I253"/>
+  <dimension ref="A1:I257"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -18872,8 +18892,172 @@
       </c>
       <c r="I253" s="6" t="n"/>
     </row>
+    <row r="254" ht="172" customHeight="1">
+      <c r="A254" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 11:06</t>
+        </is>
+      </c>
+      <c r="B254" s="13" t="inlineStr">
+        <is>
+          <t>P1-10</t>
+        </is>
+      </c>
+      <c r="C254" s="6" t="inlineStr">
+        <is>
+          <t>管理操作審計記錄</t>
+        </is>
+      </c>
+      <c r="D254" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="E254" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F254" s="13" t="inlineStr">
+        <is>
+          <t>部分通過</t>
+        </is>
+      </c>
+      <c r="G254" s="6" t="inlineStr">
+        <is>
+          <t>本機（分支 p1-10-p2-09-audit-usage，migration 已套用到本機 Supabase）：探測腳本 22/22，用 GoTrue 真實登入、只把 42501 當拒絕。① 超管改角色 short_description → 1 筆 update、before/after 只有該欄、actor=該管理員；改 voice_stack → 1 筆含新舊值；不改內容再存 → 0 筆 ② 超管 JWT UPDATE/DELETE → 42501；service role DELETE → 42501；postgres DELETE/TRUNCATE 被觸發器拒絕；內容管理員、家長讀 → []；anon → 42501。網頁實測：IP 加一個活動提示 → 只記 1 筆 ip_modes insert，原樣再存 → 0 筆，清除 → 1 筆 delete；Accounts 建帳號 → account.create（不含密碼）；改匯率 → 1 筆。未做：部署線上。</t>
+        </is>
+      </c>
+      <c r="H254" s="13" t="inlineStr">
+        <is>
+          <t>e438bab</t>
+        </is>
+      </c>
+      <c r="I254" s="6" t="n"/>
+    </row>
+    <row r="255" ht="158" customHeight="1">
+      <c r="A255" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 11:06</t>
+        </is>
+      </c>
+      <c r="B255" s="13" t="inlineStr">
+        <is>
+          <t>P2-09</t>
+        </is>
+      </c>
+      <c r="C255" s="6" t="inlineStr">
+        <is>
+          <t>每台設備成本監控</t>
+        </is>
+      </c>
+      <c r="D255" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="E255" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F255" s="13" t="inlineStr">
+        <is>
+          <t>部分通過</t>
+        </is>
+      </c>
+      <c r="G255" s="6" t="inlineStr">
+        <is>
+          <t>本機：pytest 239 passed（新增 8 項：STT/TTS 用量入行、遲到的用量帶到下一行、session 結束寫 usage 行、設備 ID、同一輪多次 LLM 相加、記憶整理的 token 即使回覆解析失敗也記錄並記到該設備）。模擬板子跑 2 輪（本機語音伺服器 7865）：送 2.24s 音訊 → stt_audio_ms=2242（兩輪皆是）；每輪有 tts_chars、token、device_id；session 結束的記憶整理寫成 memory 行（deepseek-v4-flash 946/10 token）。Usage 頁按設備與日期顯示 HK$，改費率即重算並進審計。未做：抽 10 個 session 與 Azure/MiniMax/OpenRouter 帳單對帳（需用戶提供帳單）、部署線上。</t>
+        </is>
+      </c>
+      <c r="H255" s="13" t="inlineStr">
+        <is>
+          <t>e438bab</t>
+        </is>
+      </c>
+      <c r="I255" s="6" t="n"/>
+    </row>
+    <row r="256" ht="102" customHeight="1">
+      <c r="A256" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 11:10</t>
+        </is>
+      </c>
+      <c r="B256" s="13" t="inlineStr">
+        <is>
+          <t>P1-10</t>
+        </is>
+      </c>
+      <c r="C256" s="6" t="inlineStr">
+        <is>
+          <t>管理操作審計記錄</t>
+        </is>
+      </c>
+      <c r="D256" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="E256" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F256" s="13" t="n"/>
+      <c r="G256" s="6" t="n"/>
+      <c r="H256" s="13" t="inlineStr">
+        <is>
+          <t>8e3b2c5</t>
+        </is>
+      </c>
+      <c r="I256" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-14：已合併進 dev（rebase 後 commit 8e3b2c5，原 e438bab）。部署用 docs/deploy/release-2026-10-14-audit-usage.sh：先套兩個 migration，再換語音伺服器和網頁映像；第 5 步自動檢查，第 6 步在跟已綁定的玩具對話後確認用量行。</t>
+        </is>
+      </c>
+    </row>
+    <row r="257" ht="102" customHeight="1">
+      <c r="A257" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 11:10</t>
+        </is>
+      </c>
+      <c r="B257" s="13" t="inlineStr">
+        <is>
+          <t>P2-09</t>
+        </is>
+      </c>
+      <c r="C257" s="6" t="inlineStr">
+        <is>
+          <t>每台設備成本監控</t>
+        </is>
+      </c>
+      <c r="D257" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="E257" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F257" s="13" t="n"/>
+      <c r="G257" s="6" t="n"/>
+      <c r="H257" s="13" t="inlineStr">
+        <is>
+          <t>8e3b2c5</t>
+        </is>
+      </c>
+      <c r="I257" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-14：已合併進 dev（rebase 後 commit 8e3b2c5，原 e438bab）。部署用 docs/deploy/release-2026-10-14-audit-usage.sh：先套兩個 migration，再換語音伺服器和網頁映像；第 5 步自動檢查，第 6 步在跟已綁定的玩具對話後確認用量行。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I253"/>
+  <autoFilter ref="A1:I257"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Track P1-02, P1-10 and P2-09 results and drop P1-09 from the CP1 gate.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/production-readiness.xlsx
+++ b/docs/production-readiness.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'任務清單'!$A$1:$P$88</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'待確認問題'!$A$1:$G$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$257</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$260</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -641,7 +641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I103"/>
+  <dimension ref="A1:I104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -665,7 +665,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>最後更新：2026-10-14 11:10　·　本頁由 tracker.py 自動生成，請勿手動編輯</t>
+          <t>最後更新：2026-10-14 11:28　·　本頁由 tracker.py 自動生成，請勿手動編輯</t>
         </is>
       </c>
     </row>
@@ -780,11 +780,11 @@
       </c>
       <c r="D7" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A7,'任務清單'!$F:$F,D$5)</f>
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E7" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A7,'任務清單'!$F:$F,E$5)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F7" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A7,'任務清單'!$F:$F,F$5)</f>
@@ -896,11 +896,11 @@
       </c>
       <c r="D10" s="5">
         <f>SUM(D6:D9)</f>
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E10" s="5">
         <f>SUM(E6:E9)</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F10" s="5">
         <f>SUM(F6:F9)</f>
@@ -1023,11 +1023,11 @@
       </c>
       <c r="D14" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A14,'任務清單'!$F:$F,D$12)</f>
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E14" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A14,'任務清單'!$F:$F,E$12)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F14" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A14,'任務清單'!$F:$F,F$12)</f>
@@ -1139,11 +1139,11 @@
       </c>
       <c r="D17" s="5">
         <f>SUM(D13:D16)</f>
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E17" s="5">
         <f>SUM(E13:E16)</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F17" s="5">
         <f>SUM(F13:F16)</f>
@@ -1358,15 +1358,15 @@
       <c r="H25" s="11" t="n"/>
       <c r="I25" s="12" t="n"/>
     </row>
-    <row r="26" ht="242" customHeight="1">
+    <row r="26" ht="172" customHeight="1">
       <c r="A26" s="13" t="inlineStr">
         <is>
-          <t>P1-10</t>
+          <t>P1-02</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>管理操作審計記錄</t>
+          <t>日誌移除兒童個人資料</t>
         </is>
       </c>
       <c r="C26" s="13" t="inlineStr">
@@ -1381,8 +1381,8 @@
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
-          <t>上次測試：部分通過 — 本機（分支 p1-10-p2-09-audit-usage，migration 已套用到本機 Supabase）：探測腳本 22/22，用 GoTrue 真實登入、只把 42501 當拒絕。① 超管改角色 short_description → 1 筆 update、before/after 只有該欄、actor=該管理員；改 voice_stack → 1 筆含新舊值；不改內容再存 → 0 筆 ② 超管 JWT UPDATE/DELETE → 42501；service role DELETE → 42501；postgres DELETE/TRUNCATE 被觸發器拒絕；內容管理員、家長讀 → []；anon → 42501。網頁實測：IP 加一個活動提示 → 只記 1 筆 ip_modes insert，原樣再存 → 0 筆，清除 → 1 筆 delete；Accounts 建帳號 → account.create（不含密碼）；改匯率 → 1 筆。未做：部署線上。
-每個管理操作寫一筆記錄：誰、什麼時間、什麼操作、對象、改之前與改之後的值；記錄只能新增，任何人（包括超級管理員）都不能修改或刪除；超級管理員能在管理端查看。</t>
+          <t>上次測試：部分通過 — 本機（分支 p1-02-log-pii）：模擬板子跑 3 輪，孩子名 PROBE小明、性格『鍾意恐龍』、記憶『佢有隻狗叫PROBE豆豆』；把對話、回覆、事實切成 47 段搜日誌 → 預設 INFO 0 段；同一流程 LOG_LEVEL=DEBUG → 27 段（證明搜尋有效）。INFO 日誌也無 token。pytest 245 passed（新增 test_log_privacy 6 項：事實/摘要、PostgREST details、OpenRouter flagged_input、非 JSON 回覆、預設 INFO 與 traceback 無變量值）。未做：部署線上並在生產日誌重跑。
+生產日誌只記 ID、長度、類別，不記內容；內容只在 DEBUG 等級輸出，生產不開 DEBUG。</t>
         </is>
       </c>
       <c r="F26" s="11" t="n"/>
@@ -1390,15 +1390,15 @@
       <c r="H26" s="11" t="n"/>
       <c r="I26" s="12" t="n"/>
     </row>
-    <row r="27" ht="409" customHeight="1">
+    <row r="27" ht="242" customHeight="1">
       <c r="A27" s="13" t="inlineStr">
         <is>
-          <t>P1-12</t>
+          <t>P1-10</t>
         </is>
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>設備解綁時的記憶處理：確認、預設保留、可選清除</t>
+          <t>管理操作審計記錄</t>
         </is>
       </c>
       <c r="C27" s="13" t="inlineStr">
@@ -1413,8 +1413,8 @@
       </c>
       <c r="E27" s="6" t="inlineStr">
         <is>
-          <t>上次測試：部分通過 — 本機（開發板 DEV636 身份的模擬裝置 + 網頁）：TC1/2/5/6/7/8/10/11/13 通過；TC3 重綁後 log『Loaded 2 fact(s)』；TC4 第二台 starts cold、設定頁可切換；TC9 DB 層 B 解綁回 NULL、清除報錯，anon/authenticated 無 EXECUTE；TC10 舊代數寫入三表皆 HTTP 400、清除後 40 秒仍 0 行；TC12 伺服器端 4401 通過；pytest 214 passed。TC14（2026-10-12，rebase 到 main 後的 p1-12-rebased 8d4b9e2，本機 7861）：/ws/nextjs 以網頁 token 對話兩輪，波波熊有回應 → turn_metrics 0→3，memory_facts／memory_segments／conversations 皆 0→0；log 只有 NextJS websocket connected。真機 62:70（2026-10-12，localall 測試版 → 本機 7861/3014，p1-12-rebased）：按住 BOOT 對話 6 輪，conversations 記下『我隻狗叫豆豆…』；TC12：介面解綁（不勾清除）→ 16:06:51 即斷線，之後每次重連都在 auth 前被拒（device token refused），16:07:02 重新取 token 得 202 並顯示配對碼 UKDM7N；facts 1→1、conversations 14→14、segments 1→2（結束時的摘要）、revision 0。TC3：同帳號重綁 → log『Loaded 1 fact(s)』（有一隻3歲嘅狗叫豆豆）＋2 段摘要；真機問『我隻狗叫咩名』的回答未記錄（用戶決定直接部署）。發現：韌體拿到 202 後 websocket 仍每秒重連一次直到被認領，沒有真正停在配對狀態（不屬 P1-12 伺服器端，另開任務）。
-① 按「解綁」先彈出確認對話框，取消則什麼都不改。② 對話框預設保留記憶；「同時清除記憶」要主動勾選，並寫明無法復原。③ 記憶跟設備：鍵是 (user_id, device_id, ip_key)。同一帳號的每台設備各自一份記憶；保留時，同帳號重綁同一台會接著用；換新設備從空白開始（搬記憶交給 R-11）。④ 清除在伺服器端一個交易完成：先刪該設備的 memory_facts、memory_segments、conversations（連帳號的舊 memories），再解綁；任何一步失敗就不解綁，並顯示錯誤。⑤ 其他帳號認領同一台設備，看不到舊記憶（靠 user_id 隔離，不靠刪除成功）。⑥ 設定頁按設備顯示記憶；「清除全部」只清所選設備，連 conversations 一起刪。⑦ 對話中清除，之後的寫入和 consolidation 不會把記憶寫回（devices.memories_revision + trigger）。⑧ 未認領的設備不能對話：/ws/esp32 查到設備沒有 user_id 就在 auth 前以 4401 關閉，即使 24 小時 token 未過期；韌體重新取 token 拿到 202，回到配對狀態。⑨ 解綁時立即中斷該設備正在進行的語音 session。⑩ 網頁語音（playground）沒有設備，不讀也不寫記憶。</t>
+          <t>上次測試：部分通過 — 本機（分支 p1-10-p2-09-audit-usage，migration 已套用到本機 Supabase）：探測腳本 22/22，用 GoTrue 真實登入、只把 42501 當拒絕。① 超管改角色 short_description → 1 筆 update、before/after 只有該欄、actor=該管理員；改 voice_stack → 1 筆含新舊值；不改內容再存 → 0 筆 ② 超管 JWT UPDATE/DELETE → 42501；service role DELETE → 42501；postgres DELETE/TRUNCATE 被觸發器拒絕；內容管理員、家長讀 → []；anon → 42501。網頁實測：IP 加一個活動提示 → 只記 1 筆 ip_modes insert，原樣再存 → 0 筆，清除 → 1 筆 delete；Accounts 建帳號 → account.create（不含密碼）；改匯率 → 1 筆。未做：部署線上。
+每個管理操作寫一筆記錄：誰、什麼時間、什麼操作、對象、改之前與改之後的值；記錄只能新增，任何人（包括超級管理員）都不能修改或刪除；超級管理員能在管理端查看。</t>
         </is>
       </c>
       <c r="F27" s="11" t="n"/>
@@ -1422,15 +1422,15 @@
       <c r="H27" s="11" t="n"/>
       <c r="I27" s="12" t="n"/>
     </row>
-    <row r="28" ht="200" customHeight="1">
+    <row r="28" ht="409" customHeight="1">
       <c r="A28" s="13" t="inlineStr">
         <is>
-          <t>P2-09</t>
+          <t>P1-12</t>
         </is>
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>每台設備成本監控</t>
+          <t>設備解綁時的記憶處理：確認、預設保留、可選清除</t>
         </is>
       </c>
       <c r="C28" s="13" t="inlineStr">
@@ -1445,8 +1445,8 @@
       </c>
       <c r="E28" s="6" t="inlineStr">
         <is>
-          <t>上次測試：部分通過 — 本機：pytest 239 passed（新增 8 項：STT/TTS 用量入行、遲到的用量帶到下一行、session 結束寫 usage 行、設備 ID、同一輪多次 LLM 相加、記憶整理的 token 即使回覆解析失敗也記錄並記到該設備）。模擬板子跑 2 輪（本機語音伺服器 7865）：送 2.24s 音訊 → stt_audio_ms=2242（兩輪皆是）；每輪有 tts_chars、token、device_id；session 結束的記憶整理寫成 memory 行（deepseek-v4-flash 946/10 token）。Usage 頁按設備與日期顯示 HK$，改費率即重算並進審計。未做：抽 10 個 session 與 Azure/MiniMax/OpenRouter 帳單對帳（需用戶提供帳單）、部署線上。
-每個 session 記錄 STT 秒數、LLM token、TTS 字數並換算成本；admin 頁顯示每台設備的月成本。</t>
+          <t>上次測試：部分通過 — 本機（開發板 DEV636 身份的模擬裝置 + 網頁）：TC1/2/5/6/7/8/10/11/13 通過；TC3 重綁後 log『Loaded 2 fact(s)』；TC4 第二台 starts cold、設定頁可切換；TC9 DB 層 B 解綁回 NULL、清除報錯，anon/authenticated 無 EXECUTE；TC10 舊代數寫入三表皆 HTTP 400、清除後 40 秒仍 0 行；TC12 伺服器端 4401 通過；pytest 214 passed。TC14（2026-10-12，rebase 到 main 後的 p1-12-rebased 8d4b9e2，本機 7861）：/ws/nextjs 以網頁 token 對話兩輪，波波熊有回應 → turn_metrics 0→3，memory_facts／memory_segments／conversations 皆 0→0；log 只有 NextJS websocket connected。真機 62:70（2026-10-12，localall 測試版 → 本機 7861/3014，p1-12-rebased）：按住 BOOT 對話 6 輪，conversations 記下『我隻狗叫豆豆…』；TC12：介面解綁（不勾清除）→ 16:06:51 即斷線，之後每次重連都在 auth 前被拒（device token refused），16:07:02 重新取 token 得 202 並顯示配對碼 UKDM7N；facts 1→1、conversations 14→14、segments 1→2（結束時的摘要）、revision 0。TC3：同帳號重綁 → log『Loaded 1 fact(s)』（有一隻3歲嘅狗叫豆豆）＋2 段摘要；真機問『我隻狗叫咩名』的回答未記錄（用戶決定直接部署）。發現：韌體拿到 202 後 websocket 仍每秒重連一次直到被認領，沒有真正停在配對狀態（不屬 P1-12 伺服器端，另開任務）。
+① 按「解綁」先彈出確認對話框，取消則什麼都不改。② 對話框預設保留記憶；「同時清除記憶」要主動勾選，並寫明無法復原。③ 記憶跟設備：鍵是 (user_id, device_id, ip_key)。同一帳號的每台設備各自一份記憶；保留時，同帳號重綁同一台會接著用；換新設備從空白開始（搬記憶交給 R-11）。④ 清除在伺服器端一個交易完成：先刪該設備的 memory_facts、memory_segments、conversations（連帳號的舊 memories），再解綁；任何一步失敗就不解綁，並顯示錯誤。⑤ 其他帳號認領同一台設備，看不到舊記憶（靠 user_id 隔離，不靠刪除成功）。⑥ 設定頁按設備顯示記憶；「清除全部」只清所選設備，連 conversations 一起刪。⑦ 對話中清除，之後的寫入和 consolidation 不會把記憶寫回（devices.memories_revision + trigger）。⑧ 未認領的設備不能對話：/ws/esp32 查到設備沒有 user_id 就在 auth 前以 4401 關閉，即使 24 小時 token 未過期；韌體重新取 token 拿到 202，回到配對狀態。⑨ 解綁時立即中斷該設備正在進行的語音 session。⑩ 網頁語音（playground）沒有設備，不讀也不寫記憶。</t>
         </is>
       </c>
       <c r="F28" s="11" t="n"/>
@@ -1454,15 +1454,15 @@
       <c r="H28" s="11" t="n"/>
       <c r="I28" s="12" t="n"/>
     </row>
-    <row r="29" ht="172" customHeight="1">
+    <row r="29" ht="200" customHeight="1">
       <c r="A29" s="13" t="inlineStr">
         <is>
-          <t>P2-13</t>
+          <t>P2-09</t>
         </is>
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>Admin 後台改成分組側欄（新頁面先用示例數據預覽）</t>
+          <t>每台設備成本監控</t>
         </is>
       </c>
       <c r="C29" s="13" t="inlineStr">
@@ -1477,8 +1477,8 @@
       </c>
       <c r="E29" s="6" t="inlineStr">
         <is>
-          <t>上次測試：部分通過 — ① tsc --noEmit 通過 ② 略過登入的測試頁（另一份副本、獨立 .next）：超級管理員 15 頁、內容管理員只見 Characters／IPs；1360px 與 375px 均無橫向捲動（scrollWidth=clientWidth=375）；#audit 直接打開正確；③④ 未做：需真實帳號登入 /admin
-6 個現有分頁（Model、Latency、Characters、IPs、Accounts、Admins）在新側欄照常使用，讀寫真實數據；內容管理員只看到 Characters 和 IPs；預覽頁和規劃頁只有超級管理員看到，並有橫幅寫明示例數據、按鈕不能用；每頁有 #hash 可直接打開；手機寬度沒有橫向捲動。</t>
+          <t>上次測試：部分通過 — 本機：pytest 239 passed（新增 8 項：STT/TTS 用量入行、遲到的用量帶到下一行、session 結束寫 usage 行、設備 ID、同一輪多次 LLM 相加、記憶整理的 token 即使回覆解析失敗也記錄並記到該設備）。模擬板子跑 2 輪（本機語音伺服器 7865）：送 2.24s 音訊 → stt_audio_ms=2242（兩輪皆是）；每輪有 tts_chars、token、device_id；session 結束的記憶整理寫成 memory 行（deepseek-v4-flash 946/10 token）。Usage 頁按設備與日期顯示 HK$，改費率即重算並進審計。未做：抽 10 個 session 與 Azure/MiniMax/OpenRouter 帳單對帳（需用戶提供帳單）、部署線上。
+每個 session 記錄 STT 秒數、LLM token、TTS 字數並換算成本；admin 頁顯示每台設備的月成本。</t>
         </is>
       </c>
       <c r="F29" s="11" t="n"/>
@@ -1486,15 +1486,15 @@
       <c r="H29" s="11" t="n"/>
       <c r="I29" s="12" t="n"/>
     </row>
-    <row r="30" ht="200" customHeight="1">
+    <row r="30" ht="172" customHeight="1">
       <c r="A30" s="13" t="inlineStr">
         <is>
-          <t>R-21</t>
+          <t>P2-13</t>
         </is>
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>藍牙配網與綁定（取代熱點配網）</t>
+          <t>Admin 後台改成分組側欄（新頁面先用示例數據預覽）</t>
         </is>
       </c>
       <c r="C30" s="13" t="inlineStr">
@@ -1509,7 +1509,8 @@
       </c>
       <c r="E30" s="6" t="inlineStr">
         <is>
-          <t>① 設備在「未配網、Wi-Fi 連不上、未綁定、長按 BOOT」時以 AIBuddy-XXXX 名稱廣播藍牙，廣播資料帶品牌，品牌 App 只列出自己品牌的設備。② 設備經藍牙回傳它掃描到的 2.4GHz Wi-Fi 清單，App 讓用戶選擇並填密碼。③ App 經藍牙把 SSID、密碼和綁定票（P0-11）一起交給設備；藍牙通道加密（ESP 標準配網協定 security 1/2 或同等）。④ 設備連上 Wi-Fi 後自己完成認領，App 顯示綁定成功或失敗原因（密碼錯、設備已有主人、票過期）。⑤ 配網期間不啟動音訊；完成後釋放藍牙記憶體再開語音（必要時重開機），對話中最低 heap 不比現在差。⑥ 解綁在 App 內完成（P1-12），解綁後設備進入藍牙待綁定狀態。⑦ SoftAP 熱點配網保留給開發和運維（隱藏觸發方式或編譯開關），量產用戶流程不出現。</t>
+          <t>上次測試：部分通過 — ① tsc --noEmit 通過 ② 略過登入的測試頁（另一份副本、獨立 .next）：超級管理員 15 頁、內容管理員只見 Characters／IPs；1360px 與 375px 均無橫向捲動（scrollWidth=clientWidth=375）；#audit 直接打開正確；③④ 未做：需真實帳號登入 /admin
+6 個現有分頁（Model、Latency、Characters、IPs、Accounts、Admins）在新側欄照常使用，讀寫真實數據；內容管理員只看到 Characters 和 IPs；預覽頁和規劃頁只有超級管理員看到，並有橫幅寫明示例數據、按鈕不能用；每頁有 #hash 可直接打開；手機寬度沒有橫向捲動。</t>
         </is>
       </c>
       <c r="F30" s="11" t="n"/>
@@ -1517,15 +1518,15 @@
       <c r="H30" s="11" t="n"/>
       <c r="I30" s="12" t="n"/>
     </row>
-    <row r="31" ht="116" customHeight="1">
+    <row r="31" ht="200" customHeight="1">
       <c r="A31" s="13" t="inlineStr">
         <is>
-          <t>R-36</t>
+          <t>R-21</t>
         </is>
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>未認領的設備停在配對狀態，不再每秒重連 websocket</t>
+          <t>藍牙配網與綁定（取代熱點配網）</t>
         </is>
       </c>
       <c r="C31" s="13" t="inlineStr">
@@ -1540,7 +1541,7 @@
       </c>
       <c r="E31" s="6" t="inlineStr">
         <is>
-          <t>① 拿到 202 或 websocket 被 4401 拒絕後，設備停掉 websocket 自動重連，進入待綁定狀態（燈號可分辨）。② 待綁定時只按退避（5 秒起、上限 PROVISION_BACKOFF_MAX）呼叫 generate_auth_token，不開 websocket。③ 被認領後下一次輪詢拿到 200，在 10 秒內（加退避）自動開 websocket 並能對話，不用重開機。④ 已綁定設備網絡斷線重連的行為不變。⑤ 隨 OTA 推出。</t>
+          <t>① 設備在「未配網、Wi-Fi 連不上、未綁定、長按 BOOT」時以 AIBuddy-XXXX 名稱廣播藍牙，廣播資料帶品牌，品牌 App 只列出自己品牌的設備。② 設備經藍牙回傳它掃描到的 2.4GHz Wi-Fi 清單，App 讓用戶選擇並填密碼。③ App 經藍牙把 SSID、密碼和綁定票（P0-11）一起交給設備；藍牙通道加密（ESP 標準配網協定 security 1/2 或同等）。④ 設備連上 Wi-Fi 後自己完成認領，App 顯示綁定成功或失敗原因（密碼錯、設備已有主人、票過期）。⑤ 配網期間不啟動音訊；完成後釋放藍牙記憶體再開語音（必要時重開機），對話中最低 heap 不比現在差。⑥ 解綁在 App 內完成（P1-12），解綁後設備進入藍牙待綁定狀態。⑦ SoftAP 熱點配網保留給開發和運維（隱藏觸發方式或編譯開關），量產用戶流程不出現。</t>
         </is>
       </c>
       <c r="F31" s="11" t="n"/>
@@ -1548,20 +1549,20 @@
       <c r="H31" s="11" t="n"/>
       <c r="I31" s="12" t="n"/>
     </row>
-    <row r="32" ht="228" customHeight="1">
+    <row r="32" ht="116" customHeight="1">
       <c r="A32" s="13" t="inlineStr">
         <is>
-          <t>P2-12</t>
+          <t>R-36</t>
         </is>
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>量產燒錄前加大 app 分區</t>
+          <t>未認領的設備停在配對狀態，不再每秒重連 websocket</t>
         </is>
       </c>
       <c r="C32" s="13" t="inlineStr">
         <is>
-          <t>3 封閉內測</t>
+          <t>2 內測準備</t>
         </is>
       </c>
       <c r="D32" s="13" t="inlineStr">
@@ -1571,8 +1572,7 @@
       </c>
       <c r="E32" s="6" t="inlineStr">
         <is>
-          <t>上次測試：部分通過 — 62:70（spotpear-ai-toy-p212 原型，現已併入 spotpear-ai-toy）：① 本機 OTA 1.6.1→1.6.2 寫入新 app1，120s 後 confirmed ② 3 秒 abort 的 1.6.3 → PANIC → 回到 1.6.2，ota_failed_version=1.6.3 ③ 崩潰寫入 coredump 14.8KB ④ 資源分區 9 個聲音 504KB/2MB，開機 CRC 63ms，OTA 後照常；損壞/清空 → 退回內建聲音無崩潰 ⑤ pio 全部 18 個 env 編譯通過，映像都在各自 app 槽內（Spotpear 4 個 1.59–1.60MB / 4MB；其他板仍 2MB 槽）；R-21 藍牙探針版 2,326,128 bytes &lt; 4MB ⑥ release_firmware.py 映像 &gt; app 槽即拒發。未做：雲端 OTA 一次（等上 UAT）、出廠腳本寫入資源包（R-10）
-新分區表（例如 app0/app1 各 4MB，保留 nvs/otadata 位置）在出廠前定案並寫入出廠腳本；OTA 與回滾在新分區表上照常</t>
+          <t>① 拿到 202 或 websocket 被 4401 拒絕後，設備停掉 websocket 自動重連，進入待綁定狀態（燈號可分辨）。② 待綁定時只按退避（5 秒起、上限 PROVISION_BACKOFF_MAX）呼叫 generate_auth_token，不開 websocket。③ 被認領後下一次輪詢拿到 200，在 10 秒內（加退避）自動開 websocket 並能對話，不用重開機。④ 已綁定設備網絡斷線重連的行為不變。⑤ 隨 OTA 推出。</t>
         </is>
       </c>
       <c r="F32" s="11" t="n"/>
@@ -1580,15 +1580,15 @@
       <c r="H32" s="11" t="n"/>
       <c r="I32" s="12" t="n"/>
     </row>
-    <row r="33" ht="242" customHeight="1">
+    <row r="33" ht="228" customHeight="1">
       <c r="A33" s="13" t="inlineStr">
         <is>
-          <t>R-37</t>
+          <t>P2-12</t>
         </is>
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>網頁設定玩具的 Wi-Fi：查看、新增、刪除</t>
+          <t>量產燒錄前加大 app 分區</t>
         </is>
       </c>
       <c r="C33" s="13" t="inlineStr">
@@ -1603,8 +1603,8 @@
       </c>
       <c r="E33" s="6" t="inlineStr">
         <is>
-          <t>上次測試：部分通過 — 模擬玩具經本機語音服務器＋網頁：status/scan/add/delete 正常；刪除目前 Wi-Fi → current 被拒；斷線 5 秒內頁面顯示睡著、按鈕停用；測試密碼在語音服務器日誌、網頁服務器日誌、資料庫均搜不到；用別人裝置 ID 重放 server action → forbidden；pytest 17 項通過（全套 230）；韌體 spotpear-ai-toy-localall 編譯通過（RAM 17.5%、Flash 75.9%）。未測：真機 ①② 及 OTA 推出
-① 設定頁顯示玩具在線／離線、目前 Wi-Fi 和訊號、已記住的 Wi-Fi 清單（只有名稱，不顯示密碼）② 在線時可新增 Wi-Fi（輸入或從玩具掃描到的清單選）、刪除 Wi-Fi；不能刪除正在使用的那個 ③ 經 /ws/esp32 轉送：伺服器先確認是設備主人；密碼不寫入資料庫、不寫入日誌 ④ 新增不切換網絡，目前 Wi-Fi 消失時才按訊號選；清單標示「連過／未連過」⑤ 上限 8 個 ⑥ 韌體改動經 OTA 推出</t>
+          <t>上次測試：部分通過 — 62:70（spotpear-ai-toy-p212 原型，現已併入 spotpear-ai-toy）：① 本機 OTA 1.6.1→1.6.2 寫入新 app1，120s 後 confirmed ② 3 秒 abort 的 1.6.3 → PANIC → 回到 1.6.2，ota_failed_version=1.6.3 ③ 崩潰寫入 coredump 14.8KB ④ 資源分區 9 個聲音 504KB/2MB，開機 CRC 63ms，OTA 後照常；損壞/清空 → 退回內建聲音無崩潰 ⑤ pio 全部 18 個 env 編譯通過，映像都在各自 app 槽內（Spotpear 4 個 1.59–1.60MB / 4MB；其他板仍 2MB 槽）；R-21 藍牙探針版 2,326,128 bytes &lt; 4MB ⑥ release_firmware.py 映像 &gt; app 槽即拒發。未做：雲端 OTA 一次（等上 UAT）、出廠腳本寫入資源包（R-10）
+新分區表（例如 app0/app1 各 4MB，保留 nvs/otadata 位置）在出廠前定案並寫入出廠腳本；OTA 與回滾在新分區表上照常</t>
         </is>
       </c>
       <c r="F33" s="11" t="n"/>
@@ -1612,30 +1612,31 @@
       <c r="H33" s="11" t="n"/>
       <c r="I33" s="12" t="n"/>
     </row>
-    <row r="34" ht="60" customHeight="1">
+    <row r="34" ht="242" customHeight="1">
       <c r="A34" s="13" t="inlineStr">
         <is>
-          <t>P1-01</t>
+          <t>R-37</t>
         </is>
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>加入內容審核層（輸入與輸出）</t>
+          <t>網頁設定玩具的 Wi-Fi：查看、新增、刪除</t>
         </is>
       </c>
       <c r="C34" s="13" t="inlineStr">
         <is>
-          <t>2 內測準備</t>
+          <t>3 封閉內測</t>
         </is>
       </c>
       <c r="D34" s="13" t="inlineStr">
         <is>
-          <t>未開始</t>
+          <t>進行中</t>
         </is>
       </c>
       <c r="E34" s="6" t="inlineStr">
         <is>
-          <t>STT 文字與 LLM 輸出都經審核，尺度按 3–6 歲；命中時換成安全回覆並記錄事件，事件只記類別、時間、角色，不記原文（管理員不能看兒童內容，見 Q7）；首字延遲增加 ≤150ms。</t>
+          <t>上次測試：部分通過 — 模擬玩具經本機語音服務器＋網頁：status/scan/add/delete 正常；刪除目前 Wi-Fi → current 被拒；斷線 5 秒內頁面顯示睡著、按鈕停用；測試密碼在語音服務器日誌、網頁服務器日誌、資料庫均搜不到；用別人裝置 ID 重放 server action → forbidden；pytest 17 項通過（全套 230）；韌體 spotpear-ai-toy-localall 編譯通過（RAM 17.5%、Flash 75.9%）。未測：真機 ①② 及 OTA 推出
+① 設定頁顯示玩具在線／離線、目前 Wi-Fi 和訊號、已記住的 Wi-Fi 清單（只有名稱，不顯示密碼）② 在線時可新增 Wi-Fi（輸入或從玩具掃描到的清單選）、刪除 Wi-Fi；不能刪除正在使用的那個 ③ 經 /ws/esp32 轉送：伺服器先確認是設備主人；密碼不寫入資料庫、不寫入日誌 ④ 新增不切換網絡，目前 Wi-Fi 消失時才按訊號選；清單標示「連過／未連過」⑤ 上限 8 個 ⑥ 韌體改動經 OTA 推出</t>
         </is>
       </c>
       <c r="F34" s="11" t="n"/>
@@ -1643,15 +1644,15 @@
       <c r="H34" s="11" t="n"/>
       <c r="I34" s="12" t="n"/>
     </row>
-    <row r="35" ht="32" customHeight="1">
+    <row r="35" ht="60" customHeight="1">
       <c r="A35" s="13" t="inlineStr">
         <is>
-          <t>P1-02</t>
+          <t>P1-01</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>日誌移除兒童個人資料</t>
+          <t>加入內容審核層（輸入與輸出）</t>
         </is>
       </c>
       <c r="C35" s="13" t="inlineStr">
@@ -1666,7 +1667,7 @@
       </c>
       <c r="E35" s="6" t="inlineStr">
         <is>
-          <t>生產日誌只記 ID、長度、類別，不記內容；內容只在 DEBUG 等級輸出，生產不開 DEBUG。</t>
+          <t>STT 文字與 LLM 輸出都經審核，尺度按 3–6 歲；命中時換成安全回覆並記錄事件，事件只記類別、時間、角色，不記原文（管理員不能看兒童內容，見 Q7）；首字延遲增加 ≤150ms。</t>
         </is>
       </c>
       <c r="F35" s="11" t="n"/>
@@ -1798,68 +1799,68 @@
       <c r="H39" s="11" t="n"/>
       <c r="I39" s="12" t="n"/>
     </row>
-    <row r="41">
-      <c r="A41" s="10" t="inlineStr">
+    <row r="40" ht="116" customHeight="1">
+      <c r="A40" s="13" t="inlineStr">
+        <is>
+          <t>R-25</t>
+        </is>
+      </c>
+      <c r="B40" s="6" t="inlineStr">
+        <is>
+          <t>網頁的品牌主題系統</t>
+        </is>
+      </c>
+      <c r="C40" s="13" t="inlineStr">
+        <is>
+          <t>2 內測準備</t>
+        </is>
+      </c>
+      <c r="D40" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E40" s="6" t="inlineStr">
+        <is>
+          <t>① 每個品牌一個資料夾：主題 token（顏色、字體、圓角）、logo 和圖示、文案、功能開關；首頁、上手流程、角色頁可以有品牌版本，其餘頁面共用 ② 由部署的環境變數選品牌（每套部署一個品牌，見 R-34），伺服器端渲染的第一屏就是對的主題，不閃爍 ③ 共用元件裡沒有品牌名稱和寫死的品牌顏色 ④ 加一個品牌只需要加資料夾、設定和一套部署，不用改共用元件</t>
+        </is>
+      </c>
+      <c r="F40" s="11" t="n"/>
+      <c r="G40" s="11" t="n"/>
+      <c r="H40" s="11" t="n"/>
+      <c r="I40" s="12" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="10" t="inlineStr">
         <is>
           <t>✅ 最近完成與測試效果</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="4" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
         <is>
           <t>編號</t>
         </is>
       </c>
-      <c r="B42" s="4" t="inlineStr">
+      <c r="B43" s="4" t="inlineStr">
         <is>
           <t>任務</t>
         </is>
       </c>
-      <c r="C42" s="4" t="inlineStr">
+      <c r="C43" s="4" t="inlineStr">
         <is>
           <t>測試結果</t>
         </is>
       </c>
-      <c r="D42" s="4" t="inlineStr">
+      <c r="D43" s="4" t="inlineStr">
         <is>
           <t>完成日期</t>
         </is>
       </c>
-      <c r="E42" s="4" t="inlineStr">
+      <c r="E43" s="4" t="inlineStr">
         <is>
           <t>測試證據</t>
-        </is>
-      </c>
-      <c r="F42" s="11" t="n"/>
-      <c r="G42" s="11" t="n"/>
-      <c r="H42" s="11" t="n"/>
-      <c r="I42" s="12" t="n"/>
-    </row>
-    <row r="43" ht="102" customHeight="1">
-      <c r="A43" s="13" t="inlineStr">
-        <is>
-          <t>P0-12</t>
-        </is>
-      </c>
-      <c r="B43" s="6" t="inlineStr">
-        <is>
-          <t>收緊 Admin 權限與路由保護</t>
-        </is>
-      </c>
-      <c r="C43" s="13" t="inlineStr">
-        <is>
-          <t>通過</t>
-        </is>
-      </c>
-      <c r="D43" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-12</t>
-        </is>
-      </c>
-      <c r="E43" s="6" t="inlineStr">
-        <is>
-          <t>線上 2026-10-12（bac24e9）：runbook 10/08 檢查 未登入 /admin→/login、/api/admin→401、has_role() 只看角色、無管理員 policy 觸及 conversations/記憶表、超管≥1；未登入 /home、/admin→/login；用戶確認：家長帳號開 /admin 轉回 /home、管理員在 /admin 修改角色保存成功；角色細分權限沿用本機 61/61</t>
         </is>
       </c>
       <c r="F43" s="11" t="n"/>
@@ -1867,15 +1868,15 @@
       <c r="H43" s="11" t="n"/>
       <c r="I43" s="12" t="n"/>
     </row>
-    <row r="44" ht="88" customHeight="1">
+    <row r="44" ht="102" customHeight="1">
       <c r="A44" s="13" t="inlineStr">
         <is>
-          <t>P0-15</t>
+          <t>P0-12</t>
         </is>
       </c>
       <c r="B44" s="6" t="inlineStr">
         <is>
-          <t>角色表權限：只有內容管理員能發佈，關閉家長自建角色</t>
+          <t>收緊 Admin 權限與路由保護</t>
         </is>
       </c>
       <c r="C44" s="13" t="inlineStr">
@@ -1890,7 +1891,7 @@
       </c>
       <c r="E44" s="6" t="inlineStr">
         <is>
-          <t>線上 2026-10-12：② anon 只見 6 個已發佈 hk_ 內建，查隱藏/醫生/家長自建 → []，anon POST → 401；① authenticated 寫入權限由 20261007140000 REVOKE（runbook 10/08 已套用）；用戶確認：④ 家長登入後 /home/create 轉回 /home ③ 管理員在 /admin 修改角色保存成功</t>
+          <t>線上 2026-10-12（bac24e9）：runbook 10/08 檢查 未登入 /admin→/login、/api/admin→401、has_role() 只看角色、無管理員 policy 觸及 conversations/記憶表、超管≥1；未登入 /home、/admin→/login；用戶確認：家長帳號開 /admin 轉回 /home、管理員在 /admin 修改角色保存成功；角色細分權限沿用本機 61/61</t>
         </is>
       </c>
       <c r="F44" s="11" t="n"/>
@@ -1901,12 +1902,12 @@
     <row r="45" ht="88" customHeight="1">
       <c r="A45" s="13" t="inlineStr">
         <is>
-          <t>P0-16</t>
+          <t>P0-15</t>
         </is>
       </c>
       <c r="B45" s="6" t="inlineStr">
         <is>
-          <t>移除「醫生」身份與寫死的通關碼</t>
+          <t>角色表權限：只有內容管理員能發佈，關閉家長自建角色</t>
         </is>
       </c>
       <c r="C45" s="13" t="inlineStr">
@@ -1921,7 +1922,7 @@
       </c>
       <c r="E45" s="6" t="inlineStr">
         <is>
-          <t>線上 2026-10-12：生產 commit bac24e9 git grep checkDoctorAction/kiwi-subtle-emu/=== "doctor"/isDoctor → 0；線上 13 個 JS（/、/login、/onboard）grep 通關碼/"doctor"/Santa/patient → 0；anon 讀角色只見 6 個 hk_ 角色、is_doctor 全 false；用戶今日線上登入及 playground 正常</t>
+          <t>線上 2026-10-12：② anon 只見 6 個已發佈 hk_ 內建，查隱藏/醫生/家長自建 → []，anon POST → 401；① authenticated 寫入權限由 20261007140000 REVOKE（runbook 10/08 已套用）；用戶確認：④ 家長登入後 /home/create 轉回 /home ③ 管理員在 /admin 修改角色保存成功</t>
         </is>
       </c>
       <c r="F45" s="11" t="n"/>
@@ -1929,15 +1930,15 @@
       <c r="H45" s="11" t="n"/>
       <c r="I45" s="12" t="n"/>
     </row>
-    <row r="46" ht="60" customHeight="1">
+    <row r="46" ht="88" customHeight="1">
       <c r="A46" s="13" t="inlineStr">
         <is>
-          <t>P0-09</t>
+          <t>P0-16</t>
         </is>
       </c>
       <c r="B46" s="6" t="inlineStr">
         <is>
-          <t>瀏覽器語音路由改用簽名 token（/ws/nextjs）</t>
+          <t>移除「醫生」身份與寫死的通關碼</t>
         </is>
       </c>
       <c r="C46" s="13" t="inlineStr">
@@ -1952,7 +1953,7 @@
       </c>
       <c r="E46" s="6" t="inlineStr">
         <is>
-          <t>線上 2026-10-12（bac24e9）：wss /fastapi/ws/nextjs 只帶 user_id 或 token=bogus → 4401；用戶確認：登入 elatoai.hkqft.com 後網頁 playground 可正常對話</t>
+          <t>線上 2026-10-12：生產 commit bac24e9 git grep checkDoctorAction/kiwi-subtle-emu/=== "doctor"/isDoctor → 0；線上 13 個 JS（/、/login、/onboard）grep 通關碼/"doctor"/Santa/patient → 0；anon 讀角色只見 6 個 hk_ 角色、is_doctor 全 false；用戶今日線上登入及 playground 正常</t>
         </is>
       </c>
       <c r="F46" s="11" t="n"/>
@@ -1963,12 +1964,12 @@
     <row r="47" ht="60" customHeight="1">
       <c r="A47" s="13" t="inlineStr">
         <is>
-          <t>P0-17</t>
+          <t>P0-09</t>
         </is>
       </c>
       <c r="B47" s="6" t="inlineStr">
         <is>
-          <t>前端的 anon key 必須是公開 key，不可是 secret／service_role</t>
+          <t>瀏覽器語音路由改用簽名 token（/ws/nextjs）</t>
         </is>
       </c>
       <c r="C47" s="13" t="inlineStr">
@@ -1983,7 +1984,7 @@
       </c>
       <c r="E47" s="6" t="inlineStr">
         <is>
-          <t>線上 2026-10-12（bac24e9）：/login 引用的 13 個 JS + HTML 無 sb_secret_，唯一 key 為 role=anon 的 JWT；② 用該 key GET /rest/v1/users → 42501；③ 本機 10/07 已換 publishable</t>
+          <t>線上 2026-10-12（bac24e9）：wss /fastapi/ws/nextjs 只帶 user_id 或 token=bogus → 4401；用戶確認：登入 elatoai.hkqft.com 後網頁 playground 可正常對話</t>
         </is>
       </c>
       <c r="F47" s="11" t="n"/>
@@ -1991,15 +1992,15 @@
       <c r="H47" s="11" t="n"/>
       <c r="I47" s="12" t="n"/>
     </row>
-    <row r="48" ht="46" customHeight="1">
+    <row r="48" ht="60" customHeight="1">
       <c r="A48" s="13" t="inlineStr">
         <is>
-          <t>P0-10</t>
+          <t>P0-17</t>
         </is>
       </c>
       <c r="B48" s="6" t="inlineStr">
         <is>
-          <t>生產環境關閉 /browser 測試頁與 /ws/browser</t>
+          <t>前端的 anon key 必須是公開 key，不可是 secret／service_role</t>
         </is>
       </c>
       <c r="C48" s="13" t="inlineStr">
@@ -2014,7 +2015,7 @@
       </c>
       <c r="E48" s="6" t="inlineStr">
         <is>
-          <t>線上 2026-10-12（bac24e9）：GET /fastapi/browser 404、/fastapi/ 404、/fastapi/healthz 200、wss /fastapi/ws/browser → HTTP 403</t>
+          <t>線上 2026-10-12（bac24e9）：/login 引用的 13 個 JS + HTML 無 sb_secret_，唯一 key 為 role=anon 的 JWT；② 用該 key GET /rest/v1/users → 42501；③ 本機 10/07 已換 publishable</t>
         </is>
       </c>
       <c r="F48" s="11" t="n"/>
@@ -2022,15 +2023,15 @@
       <c r="H48" s="11" t="n"/>
       <c r="I48" s="12" t="n"/>
     </row>
-    <row r="49" ht="60" customHeight="1">
+    <row r="49" ht="46" customHeight="1">
       <c r="A49" s="13" t="inlineStr">
         <is>
-          <t>P0-08</t>
+          <t>P0-10</t>
         </is>
       </c>
       <c r="B49" s="6" t="inlineStr">
         <is>
-          <t>語音伺服器驗證設備身份（/ws/esp32）</t>
+          <t>生產環境關閉 /browser 測試頁與 /ws/browser</t>
         </is>
       </c>
       <c r="C49" s="13" t="inlineStr">
@@ -2045,7 +2046,7 @@
       </c>
       <c r="E49" s="6" t="inlineStr">
         <is>
-          <t>線上 2026-10-12（bac24e9）：wss /fastapi/ws/esp32 不帶 token、偽造 token＋X-Device-Mac → 均 4401 invalid device token；42:34 以有效 token 連線對話正常（P0-13 10/09）</t>
+          <t>線上 2026-10-12（bac24e9）：GET /fastapi/browser 404、/fastapi/ 404、/fastapi/healthz 200、wss /fastapi/ws/browser → HTTP 403</t>
         </is>
       </c>
       <c r="F49" s="11" t="n"/>
@@ -2056,12 +2057,12 @@
     <row r="50" ht="60" customHeight="1">
       <c r="A50" s="13" t="inlineStr">
         <is>
-          <t>P0-06</t>
+          <t>P0-08</t>
         </is>
       </c>
       <c r="B50" s="6" t="inlineStr">
         <is>
-          <t>停止憑 MAC 發放永久用戶 JWT</t>
+          <t>語音伺服器驗證設備身份（/ws/esp32）</t>
         </is>
       </c>
       <c r="C50" s="13" t="inlineStr">
@@ -2076,7 +2077,7 @@
       </c>
       <c r="E50" s="6" t="inlineStr">
         <is>
-          <t>線上 2026-10-12（bac24e9）：POST /api/generate_auth_token 只帶 42:34 的 MAC → 401、帶錯誤密鑰 → 401、GET → 410；42:34 用 NVS 密鑰在線上換 token 並連上語音伺服器（P0-13 10/09 實測）</t>
+          <t>線上 2026-10-12（bac24e9）：wss /fastapi/ws/esp32 不帶 token、偽造 token＋X-Device-Mac → 均 4401 invalid device token；42:34 以有效 token 連線對話正常（P0-13 10/09）</t>
         </is>
       </c>
       <c r="F50" s="11" t="n"/>
@@ -2084,50 +2085,58 @@
       <c r="H50" s="11" t="n"/>
       <c r="I50" s="12" t="n"/>
     </row>
-    <row r="52">
-      <c r="A52" s="10" t="inlineStr">
+    <row r="51" ht="60" customHeight="1">
+      <c r="A51" s="13" t="inlineStr">
+        <is>
+          <t>P0-06</t>
+        </is>
+      </c>
+      <c r="B51" s="6" t="inlineStr">
+        <is>
+          <t>停止憑 MAC 發放永久用戶 JWT</t>
+        </is>
+      </c>
+      <c r="C51" s="13" t="inlineStr">
+        <is>
+          <t>通過</t>
+        </is>
+      </c>
+      <c r="D51" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="E51" s="6" t="inlineStr">
+        <is>
+          <t>線上 2026-10-12（bac24e9）：POST /api/generate_auth_token 只帶 42:34 的 MAC → 401、帶錯誤密鑰 → 401、GET → 410；42:34 用 NVS 密鑰在線上換 token 並連上語音伺服器（P0-13 10/09 實測）</t>
+        </is>
+      </c>
+      <c r="F51" s="11" t="n"/>
+      <c r="G51" s="11" t="n"/>
+      <c r="H51" s="11" t="n"/>
+      <c r="I51" s="12" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="10" t="inlineStr">
         <is>
           <t>⏳ 等待依賴 / ⛔ 阻塞</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="4" t="inlineStr">
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
         <is>
           <t>編號</t>
         </is>
       </c>
-      <c r="B53" s="4" t="inlineStr">
+      <c r="B54" s="4" t="inlineStr">
         <is>
           <t>任務</t>
         </is>
       </c>
-      <c r="C53" s="4" t="inlineStr">
+      <c r="C54" s="4" t="inlineStr">
         <is>
           <t>在等什麼</t>
-        </is>
-      </c>
-      <c r="D53" s="11" t="n"/>
-      <c r="E53" s="11" t="n"/>
-      <c r="F53" s="11" t="n"/>
-      <c r="G53" s="11" t="n"/>
-      <c r="H53" s="11" t="n"/>
-      <c r="I53" s="12" t="n"/>
-    </row>
-    <row r="54" ht="60" customHeight="1">
-      <c r="A54" s="13" t="inlineStr">
-        <is>
-          <t>R-16</t>
-        </is>
-      </c>
-      <c r="B54" s="6" t="inlineStr">
-        <is>
-          <t>Spotpear 量產版加電池電壓檢測（GPIO0 分壓）</t>
-        </is>
-      </c>
-      <c r="C54" s="6" t="inlineStr">
-        <is>
-          <t>阻塞：[2026-10-07] 仍按 10/06 決定暫緩：等用戶做充滿再放電測試（與 R-17 同一次），看 VDD 低電提醒在關機前多久觸發；太遲或不觸發才向 Spotpear 提改板。已把分壓改板的問題一併放進給 Spotpear 的草稿，方便同一封發出</t>
         </is>
       </c>
       <c r="D54" s="11" t="n"/>
@@ -2137,20 +2146,20 @@
       <c r="H54" s="11" t="n"/>
       <c r="I54" s="12" t="n"/>
     </row>
-    <row r="55" ht="88" customHeight="1">
+    <row r="55" ht="60" customHeight="1">
       <c r="A55" s="13" t="inlineStr">
         <is>
-          <t>R-17</t>
+          <t>R-16</t>
         </is>
       </c>
       <c r="B55" s="6" t="inlineStr">
         <is>
-          <t>Spotpear 電池耗盡時插電能否正常開機（供電路徑）</t>
+          <t>Spotpear 量產版加電池電壓檢測（GPIO0 分壓）</t>
         </is>
       </c>
       <c r="C55" s="6" t="inlineStr">
         <is>
-          <t>阻塞：[2026-10-08] 2026-10-08 開發板 63:64 插著 USB 時兩次無法解釋的完全斷電重開：09:13:26（崩潰循環中）、10:44:33（閒置、用戶確認沒碰）。都是 USB 先斷線再以 ESP_RST_POWERON 開機，非 brownout；斷電前 6 秒 GPIO0 讀數 99.9% 參考值，屬突然切斷而非緩降（SupplyMonitor 取樣太疏抓不到瞬間）。韌體無法造成 POWERON，指向充電芯片/電池保護/供電路徑，應一併問 Spotpear；放電實測時留意插 USB 閒置時是否也會斷電</t>
+          <t>阻塞：[2026-10-07] 仍按 10/06 決定暫緩：等用戶做充滿再放電測試（與 R-17 同一次），看 VDD 低電提醒在關機前多久觸發；太遲或不觸發才向 Spotpear 提改板。已把分壓改板的問題一併放進給 Spotpear 的草稿，方便同一封發出</t>
         </is>
       </c>
       <c r="D55" s="11" t="n"/>
@@ -2160,20 +2169,20 @@
       <c r="H55" s="11" t="n"/>
       <c r="I55" s="12" t="n"/>
     </row>
-    <row r="56" ht="32" customHeight="1">
+    <row r="56" ht="88" customHeight="1">
       <c r="A56" s="13" t="inlineStr">
         <is>
-          <t>P1-09</t>
+          <t>R-17</t>
         </is>
       </c>
       <c r="B56" s="6" t="inlineStr">
         <is>
-          <t>家長鎖：孩子模式進設定要輸入 PIN</t>
+          <t>Spotpear 電池耗盡時插電能否正常開機（供電路徑）</t>
         </is>
       </c>
       <c r="C56" s="6" t="inlineStr">
         <is>
-          <t>阻塞：[2026-10-13] 2026-10-13 用戶決定：AI Buddy（品牌 C）延到 1/15 之後，本項不卡 1/15 出廠；AI Buddy 啟動時再開。</t>
+          <t>阻塞：[2026-10-08] 2026-10-08 開發板 63:64 插著 USB 時兩次無法解釋的完全斷電重開：09:13:26（崩潰循環中）、10:44:33（閒置、用戶確認沒碰）。都是 USB 先斷線再以 ESP_RST_POWERON 開機，非 brownout；斷電前 6 秒 GPIO0 讀數 99.9% 參考值，屬突然切斷而非緩降（SupplyMonitor 取樣太疏抓不到瞬間）。韌體無法造成 POWERON，指向充電芯片/電池保護/供電路徑，應一併問 Spotpear；放電實測時留意插 USB 閒置時是否也會斷電</t>
         </is>
       </c>
       <c r="D56" s="11" t="n"/>
@@ -2186,12 +2195,12 @@
     <row r="57" ht="32" customHeight="1">
       <c r="A57" s="13" t="inlineStr">
         <is>
-          <t>R-12</t>
+          <t>P1-09</t>
         </is>
       </c>
       <c r="B57" s="6" t="inlineStr">
         <is>
-          <t>家長控制：每日使用上限和休息時段</t>
+          <t>家長鎖：孩子模式進設定要輸入 PIN</t>
         </is>
       </c>
       <c r="C57" s="6" t="inlineStr">
@@ -2209,12 +2218,12 @@
     <row r="58" ht="32" customHeight="1">
       <c r="A58" s="13" t="inlineStr">
         <is>
-          <t>R-29</t>
+          <t>R-12</t>
         </is>
       </c>
       <c r="B58" s="6" t="inlineStr">
         <is>
-          <t>AI Buddy App（品牌 C）頁面</t>
+          <t>家長控制：每日使用上限和休息時段</t>
         </is>
       </c>
       <c r="C58" s="6" t="inlineStr">
@@ -2232,17 +2241,17 @@
     <row r="59" ht="32" customHeight="1">
       <c r="A59" s="13" t="inlineStr">
         <is>
-          <t>P2-14</t>
+          <t>R-29</t>
         </is>
       </c>
       <c r="B59" s="6" t="inlineStr">
         <is>
-          <t>Admin 設備頁：每台玩具的狀態、韌體與基本操作</t>
+          <t>AI Buddy App（品牌 C）頁面</t>
         </is>
       </c>
       <c r="C59" s="6" t="inlineStr">
         <is>
-          <t>等 P1-10、P2-13</t>
+          <t>阻塞：[2026-10-13] 2026-10-13 用戶決定：AI Buddy（品牌 C）延到 1/15 之後，本項不卡 1/15 出廠；AI Buddy 啟動時再開。</t>
         </is>
       </c>
       <c r="D59" s="11" t="n"/>
@@ -2252,20 +2261,20 @@
       <c r="H59" s="11" t="n"/>
       <c r="I59" s="12" t="n"/>
     </row>
-    <row r="60" ht="18" customHeight="1">
+    <row r="60" ht="32" customHeight="1">
       <c r="A60" s="13" t="inlineStr">
         <is>
-          <t>R-05</t>
+          <t>P2-14</t>
         </is>
       </c>
       <c r="B60" s="6" t="inlineStr">
         <is>
-          <t>內測版外殼（3D 打印 20 台）</t>
+          <t>Admin 設備頁：每台玩具的狀態、韌體與基本操作</t>
         </is>
       </c>
       <c r="C60" s="6" t="inlineStr">
         <is>
-          <t>等 R-01</t>
+          <t>等 P1-10、P2-13</t>
         </is>
       </c>
       <c r="D60" s="11" t="n"/>
@@ -2278,17 +2287,17 @@
     <row r="61" ht="18" customHeight="1">
       <c r="A61" s="13" t="inlineStr">
         <is>
-          <t>R-06</t>
+          <t>R-05</t>
         </is>
       </c>
       <c r="B61" s="6" t="inlineStr">
         <is>
-          <t>家長自助上手流程</t>
+          <t>內測版外殼（3D 打印 20 台）</t>
         </is>
       </c>
       <c r="C61" s="6" t="inlineStr">
         <is>
-          <t>等 P0-11</t>
+          <t>等 R-01</t>
         </is>
       </c>
       <c r="D61" s="11" t="n"/>
@@ -2298,20 +2307,20 @@
       <c r="H61" s="11" t="n"/>
       <c r="I61" s="12" t="n"/>
     </row>
-    <row r="62" ht="32" customHeight="1">
+    <row r="62" ht="18" customHeight="1">
       <c r="A62" s="13" t="inlineStr">
         <is>
-          <t>R-13</t>
+          <t>R-06</t>
         </is>
       </c>
       <c r="B62" s="6" t="inlineStr">
         <is>
-          <t>CP1 內測就緒檢查（10/30）</t>
+          <t>家長自助上手流程</t>
         </is>
       </c>
       <c r="C62" s="6" t="inlineStr">
         <is>
-          <t>等 P0-07、P0-11、P1-01、P1-02、P2-09、R-01、R-02、R-04、R-05、R-06、P1-09、P1-11</t>
+          <t>等 P0-11</t>
         </is>
       </c>
       <c r="D62" s="11" t="n"/>
@@ -2324,17 +2333,17 @@
     <row r="63" ht="32" customHeight="1">
       <c r="A63" s="13" t="inlineStr">
         <is>
-          <t>R-18</t>
+          <t>R-13</t>
         </is>
       </c>
       <c r="B63" s="6" t="inlineStr">
         <is>
-          <t>長按 BOOT 重新配網（開 AIBuddy-XXXX 熱點）</t>
+          <t>CP1 內測就緒檢查（10/30）</t>
         </is>
       </c>
       <c r="C63" s="6" t="inlineStr">
         <is>
-          <t>等 R-01</t>
+          <t>等 P0-07、P0-11、P1-01、P1-02、P2-09、R-01、R-02、R-04、R-05、R-06、P1-11</t>
         </is>
       </c>
       <c r="D63" s="11" t="n"/>
@@ -2347,12 +2356,12 @@
     <row r="64" ht="32" customHeight="1">
       <c r="A64" s="13" t="inlineStr">
         <is>
-          <t>R-19</t>
+          <t>R-18</t>
         </is>
       </c>
       <c r="B64" s="6" t="inlineStr">
         <is>
-          <t>外接按鈕：量產板加 I2C 擴展晶片（TCA9555）</t>
+          <t>長按 BOOT 重新配網（開 AIBuddy-XXXX 熱點）</t>
         </is>
       </c>
       <c r="C64" s="6" t="inlineStr">
@@ -2367,20 +2376,20 @@
       <c r="H64" s="11" t="n"/>
       <c r="I64" s="12" t="n"/>
     </row>
-    <row r="65" ht="18" customHeight="1">
+    <row r="65" ht="32" customHeight="1">
       <c r="A65" s="13" t="inlineStr">
         <is>
-          <t>R-20</t>
+          <t>R-19</t>
         </is>
       </c>
       <c r="B65" s="6" t="inlineStr">
         <is>
-          <t>孩子資料與角色改成每台設備一份</t>
+          <t>外接按鈕：量產板加 I2C 擴展晶片（TCA9555）</t>
         </is>
       </c>
       <c r="C65" s="6" t="inlineStr">
         <is>
-          <t>等 P1-12</t>
+          <t>等 R-01</t>
         </is>
       </c>
       <c r="D65" s="11" t="n"/>
@@ -2390,20 +2399,20 @@
       <c r="H65" s="11" t="n"/>
       <c r="I65" s="12" t="n"/>
     </row>
-    <row r="66" ht="32" customHeight="1">
+    <row r="66" ht="18" customHeight="1">
       <c r="A66" s="13" t="inlineStr">
         <is>
-          <t>R-27</t>
+          <t>R-20</t>
         </is>
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
-          <t>App 內登入：驗證碼、原生社交登入、刪除帳號</t>
+          <t>孩子資料與角色改成每台設備一份</t>
         </is>
       </c>
       <c r="C66" s="6" t="inlineStr">
         <is>
-          <t>等 R-26</t>
+          <t>等 P1-12</t>
         </is>
       </c>
       <c r="D66" s="11" t="n"/>
@@ -2413,20 +2422,20 @@
       <c r="H66" s="11" t="n"/>
       <c r="I66" s="12" t="n"/>
     </row>
-    <row r="67" ht="18" customHeight="1">
+    <row r="67" ht="32" customHeight="1">
       <c r="A67" s="13" t="inlineStr">
         <is>
-          <t>P0-14</t>
+          <t>R-27</t>
         </is>
       </c>
       <c r="B67" s="6" t="inlineStr">
         <is>
-          <t>韌體簽章、Secure Boot 與 Flash 加密</t>
+          <t>App 內登入：驗證碼、原生社交登入、刪除帳號</t>
         </is>
       </c>
       <c r="C67" s="6" t="inlineStr">
         <is>
-          <t>等 R-01</t>
+          <t>等 R-26</t>
         </is>
       </c>
       <c r="D67" s="11" t="n"/>
@@ -2439,17 +2448,17 @@
     <row r="68" ht="18" customHeight="1">
       <c r="A68" s="13" t="inlineStr">
         <is>
-          <t>P1-06</t>
+          <t>P0-14</t>
         </is>
       </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t>處理 GPL-3.0 依賴（arduino-audio-tools）</t>
+          <t>韌體簽章、Secure Boot 與 Flash 加密</t>
         </is>
       </c>
       <c r="C68" s="6" t="inlineStr">
         <is>
-          <t>等 Q3</t>
+          <t>等 R-01</t>
         </is>
       </c>
       <c r="D68" s="11" t="n"/>
@@ -2462,12 +2471,12 @@
     <row r="69" ht="18" customHeight="1">
       <c r="A69" s="13" t="inlineStr">
         <is>
-          <t>P1-07</t>
+          <t>P1-06</t>
         </is>
       </c>
       <c r="B69" s="6" t="inlineStr">
         <is>
-          <t>LGPL 合規與第三方授權聲明</t>
+          <t>處理 GPL-3.0 依賴（arduino-audio-tools）</t>
         </is>
       </c>
       <c r="C69" s="6" t="inlineStr">
@@ -2485,17 +2494,17 @@
     <row r="70" ht="18" customHeight="1">
       <c r="A70" s="13" t="inlineStr">
         <is>
-          <t>P1-08</t>
+          <t>P1-07</t>
         </is>
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>硬件認證</t>
+          <t>LGPL 合規與第三方授權聲明</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr">
         <is>
-          <t>等 R-01、R-05</t>
+          <t>等 Q3</t>
         </is>
       </c>
       <c r="D70" s="11" t="n"/>
@@ -2508,17 +2517,17 @@
     <row r="71" ht="18" customHeight="1">
       <c r="A71" s="13" t="inlineStr">
         <is>
-          <t>P1-14</t>
+          <t>P1-08</t>
         </is>
       </c>
       <c r="B71" s="6" t="inlineStr">
         <is>
-          <t>Admin 內容安全頁：審核事件只按類別統計</t>
+          <t>硬件認證</t>
         </is>
       </c>
       <c r="C71" s="6" t="inlineStr">
         <is>
-          <t>等 P1-01、P2-13</t>
+          <t>等 R-01、R-05</t>
         </is>
       </c>
       <c r="D71" s="11" t="n"/>
@@ -2528,20 +2537,20 @@
       <c r="H71" s="11" t="n"/>
       <c r="I71" s="12" t="n"/>
     </row>
-    <row r="72" ht="32" customHeight="1">
+    <row r="72" ht="18" customHeight="1">
       <c r="A72" s="13" t="inlineStr">
         <is>
-          <t>P2-15</t>
+          <t>P1-14</t>
         </is>
       </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>Admin 總覽頁：在線、用量、成本與待處理事項</t>
+          <t>Admin 內容安全頁：審核事件只按類別統計</t>
         </is>
       </c>
       <c r="C72" s="6" t="inlineStr">
         <is>
-          <t>等 P2-14、P2-09</t>
+          <t>等 P1-01、P2-13</t>
         </is>
       </c>
       <c r="D72" s="11" t="n"/>
@@ -2551,20 +2560,20 @@
       <c r="H72" s="11" t="n"/>
       <c r="I72" s="12" t="n"/>
     </row>
-    <row r="73" ht="18" customHeight="1">
+    <row r="73" ht="32" customHeight="1">
       <c r="A73" s="13" t="inlineStr">
         <is>
-          <t>R-07</t>
+          <t>P2-15</t>
         </is>
       </c>
       <c r="B73" s="6" t="inlineStr">
         <is>
-          <t>20 個家庭封閉內測</t>
+          <t>Admin 總覽頁：在線、用量、成本與待處理事項</t>
         </is>
       </c>
       <c r="C73" s="6" t="inlineStr">
         <is>
-          <t>等 R-13</t>
+          <t>等 P2-14、P2-09</t>
         </is>
       </c>
       <c r="D73" s="11" t="n"/>
@@ -2577,17 +2586,17 @@
     <row r="74" ht="18" customHeight="1">
       <c r="A74" s="13" t="inlineStr">
         <is>
-          <t>R-08</t>
+          <t>R-07</t>
         </is>
       </c>
       <c r="B74" s="6" t="inlineStr">
         <is>
-          <t>第 8 週關卡決策</t>
+          <t>20 個家庭封閉內測</t>
         </is>
       </c>
       <c r="C74" s="6" t="inlineStr">
         <is>
-          <t>等 R-07、P2-09、P1-08</t>
+          <t>等 R-13</t>
         </is>
       </c>
       <c r="D74" s="11" t="n"/>
@@ -2600,17 +2609,17 @@
     <row r="75" ht="18" customHeight="1">
       <c r="A75" s="13" t="inlineStr">
         <is>
-          <t>R-14</t>
+          <t>R-08</t>
         </is>
       </c>
       <c r="B75" s="6" t="inlineStr">
         <is>
-          <t>離線兒歌與故事</t>
+          <t>第 8 週關卡決策</t>
         </is>
       </c>
       <c r="C75" s="6" t="inlineStr">
         <is>
-          <t>等 R-01</t>
+          <t>等 R-07、P2-09、P1-08</t>
         </is>
       </c>
       <c r="D75" s="11" t="n"/>
@@ -2623,17 +2632,17 @@
     <row r="76" ht="18" customHeight="1">
       <c r="A76" s="13" t="inlineStr">
         <is>
-          <t>R-24</t>
+          <t>R-14</t>
         </is>
       </c>
       <c r="B76" s="6" t="inlineStr">
         <is>
-          <t>設備只能用自己品牌的角色</t>
+          <t>離線兒歌與故事</t>
         </is>
       </c>
       <c r="C76" s="6" t="inlineStr">
         <is>
-          <t>等 R-34</t>
+          <t>等 R-01</t>
         </is>
       </c>
       <c r="D76" s="11" t="n"/>
@@ -2646,17 +2655,17 @@
     <row r="77" ht="18" customHeight="1">
       <c r="A77" s="13" t="inlineStr">
         <is>
-          <t>R-28</t>
+          <t>R-24</t>
         </is>
       </c>
       <c r="B77" s="6" t="inlineStr">
         <is>
-          <t>三個 App 的殼：品牌版本與測試版</t>
+          <t>設備只能用自己品牌的角色</t>
         </is>
       </c>
       <c r="C77" s="6" t="inlineStr">
         <is>
-          <t>等 R-25、R-26</t>
+          <t>等 R-34</t>
         </is>
       </c>
       <c r="D77" s="11" t="n"/>
@@ -2669,17 +2678,17 @@
     <row r="78" ht="18" customHeight="1">
       <c r="A78" s="13" t="inlineStr">
         <is>
-          <t>R-30</t>
+          <t>R-28</t>
         </is>
       </c>
       <c r="B78" s="6" t="inlineStr">
         <is>
-          <t>快活 App（品牌 A）頁面</t>
+          <t>三個 App 的殼：品牌版本與測試版</t>
         </is>
       </c>
       <c r="C78" s="6" t="inlineStr">
         <is>
-          <t>等 R-25、R-34、Q12</t>
+          <t>等 R-25、R-26</t>
         </is>
       </c>
       <c r="D78" s="11" t="n"/>
@@ -2692,17 +2701,17 @@
     <row r="79" ht="18" customHeight="1">
       <c r="A79" s="13" t="inlineStr">
         <is>
-          <t>R-31</t>
+          <t>R-30</t>
         </is>
       </c>
       <c r="B79" s="6" t="inlineStr">
         <is>
-          <t>政協青年聯會版 App（品牌 B）頁面</t>
+          <t>快活 App（品牌 A）頁面</t>
         </is>
       </c>
       <c r="C79" s="6" t="inlineStr">
         <is>
-          <t>等 R-25、R-34、Q13</t>
+          <t>等 R-25、R-34、Q12</t>
         </is>
       </c>
       <c r="D79" s="11" t="n"/>
@@ -2715,17 +2724,17 @@
     <row r="80" ht="18" customHeight="1">
       <c r="A80" s="13" t="inlineStr">
         <is>
-          <t>R-35</t>
+          <t>R-31</t>
         </is>
       </c>
       <c r="B80" s="6" t="inlineStr">
         <is>
-          <t>韌體按品牌連線：伺服器網址在出廠時寫入</t>
+          <t>政協青年聯會版 App（品牌 B）頁面</t>
         </is>
       </c>
       <c r="C80" s="6" t="inlineStr">
         <is>
-          <t>等 R-34</t>
+          <t>等 R-25、R-34、Q13</t>
         </is>
       </c>
       <c r="D80" s="11" t="n"/>
@@ -2735,20 +2744,20 @@
       <c r="H80" s="11" t="n"/>
       <c r="I80" s="12" t="n"/>
     </row>
-    <row r="81" ht="32" customHeight="1">
+    <row r="81" ht="18" customHeight="1">
       <c r="A81" s="13" t="inlineStr">
         <is>
-          <t>R-38</t>
+          <t>R-35</t>
         </is>
       </c>
       <c r="B81" s="6" t="inlineStr">
         <is>
-          <t>公仔出廠鎖死所屬 IP，綁定時顯示該 IP 頭像</t>
+          <t>韌體按品牌連線：伺服器網址在出廠時寫入</t>
         </is>
       </c>
       <c r="C81" s="6" t="inlineStr">
         <is>
-          <t>等 P0-11</t>
+          <t>等 R-34</t>
         </is>
       </c>
       <c r="D81" s="11" t="n"/>
@@ -2761,17 +2770,17 @@
     <row r="82" ht="32" customHeight="1">
       <c r="A82" s="13" t="inlineStr">
         <is>
-          <t>R-39</t>
+          <t>R-38</t>
         </is>
       </c>
       <c r="B82" s="6" t="inlineStr">
         <is>
-          <t>Admin 出廠登記頁：匯入 MAC 清單、指定公仔、查看自檢結果</t>
+          <t>公仔出廠鎖死所屬 IP，綁定時顯示該 IP 頭像</t>
         </is>
       </c>
       <c r="C82" s="6" t="inlineStr">
         <is>
-          <t>等 R-38、P1-10</t>
+          <t>等 P0-11</t>
         </is>
       </c>
       <c r="D82" s="11" t="n"/>
@@ -2781,20 +2790,20 @@
       <c r="H82" s="11" t="n"/>
       <c r="I82" s="12" t="n"/>
     </row>
-    <row r="83" ht="18" customHeight="1">
+    <row r="83" ht="32" customHeight="1">
       <c r="A83" s="13" t="inlineStr">
         <is>
-          <t>P2-16</t>
+          <t>R-39</t>
         </is>
       </c>
       <c r="B83" s="6" t="inlineStr">
         <is>
-          <t>OTA 分批推送與後台發佈頁</t>
+          <t>Admin 出廠登記頁：匯入 MAC 清單、指定公仔、查看自檢結果</t>
         </is>
       </c>
       <c r="C83" s="6" t="inlineStr">
         <is>
-          <t>等 P2-14、P1-10</t>
+          <t>等 R-38、P1-10</t>
         </is>
       </c>
       <c r="D83" s="11" t="n"/>
@@ -2807,17 +2816,17 @@
     <row r="84" ht="18" customHeight="1">
       <c r="A84" s="13" t="inlineStr">
         <is>
-          <t>R-09</t>
+          <t>P2-16</t>
         </is>
       </c>
       <c r="B84" s="6" t="inlineStr">
         <is>
-          <t>量產外殼（真空複模）</t>
+          <t>OTA 分批推送與後台發佈頁</t>
         </is>
       </c>
       <c r="C84" s="6" t="inlineStr">
         <is>
-          <t>等 R-08、R-05、Q11</t>
+          <t>等 P2-14、P1-10</t>
         </is>
       </c>
       <c r="D84" s="11" t="n"/>
@@ -2830,17 +2839,17 @@
     <row r="85" ht="18" customHeight="1">
       <c r="A85" s="13" t="inlineStr">
         <is>
-          <t>R-10</t>
+          <t>R-09</t>
         </is>
       </c>
       <c r="B85" s="6" t="inlineStr">
         <is>
-          <t>出廠流程</t>
+          <t>量產外殼（真空複模）</t>
         </is>
       </c>
       <c r="C85" s="6" t="inlineStr">
         <is>
-          <t>等 P0-14、R-01、P2-12、R-34、R-35、R-38、R-39</t>
+          <t>等 R-08、R-05、Q11</t>
         </is>
       </c>
       <c r="D85" s="11" t="n"/>
@@ -2853,17 +2862,17 @@
     <row r="86" ht="18" customHeight="1">
       <c r="A86" s="13" t="inlineStr">
         <is>
-          <t>R-11</t>
+          <t>R-10</t>
         </is>
       </c>
       <c r="B86" s="6" t="inlineStr">
         <is>
-          <t>售後：客服、保修與換機</t>
+          <t>出廠流程</t>
         </is>
       </c>
       <c r="C86" s="6" t="inlineStr">
         <is>
-          <t>等 P2-14、R-40</t>
+          <t>等 P0-14、R-01、P2-12、R-34、R-35、R-38、R-39</t>
         </is>
       </c>
       <c r="D86" s="11" t="n"/>
@@ -2876,17 +2885,17 @@
     <row r="87" ht="18" customHeight="1">
       <c r="A87" s="13" t="inlineStr">
         <is>
-          <t>R-15</t>
+          <t>R-11</t>
         </is>
       </c>
       <c r="B87" s="6" t="inlineStr">
         <is>
-          <t>農曆新年前交付（生產 1/15、送達 1/29）</t>
+          <t>售後：客服、保修與換機</t>
         </is>
       </c>
       <c r="C87" s="6" t="inlineStr">
         <is>
-          <t>等 R-09、R-10</t>
+          <t>等 P2-14、R-40</t>
         </is>
       </c>
       <c r="D87" s="11" t="n"/>
@@ -2899,17 +2908,17 @@
     <row r="88" ht="18" customHeight="1">
       <c r="A88" s="13" t="inlineStr">
         <is>
-          <t>R-33</t>
+          <t>R-15</t>
         </is>
       </c>
       <c r="B88" s="6" t="inlineStr">
         <is>
-          <t>三個 App 送審並通過</t>
+          <t>農曆新年前交付（生產 1/15、送達 1/29）</t>
         </is>
       </c>
       <c r="C88" s="6" t="inlineStr">
         <is>
-          <t>等 R-27、R-21、R-28、R-29、R-30、R-31、R-32</t>
+          <t>等 R-09、R-10</t>
         </is>
       </c>
       <c r="D88" s="11" t="n"/>
@@ -2919,20 +2928,20 @@
       <c r="H88" s="11" t="n"/>
       <c r="I88" s="12" t="n"/>
     </row>
-    <row r="89" ht="32" customHeight="1">
+    <row r="89" ht="18" customHeight="1">
       <c r="A89" s="13" t="inlineStr">
         <is>
-          <t>R-40</t>
+          <t>R-33</t>
         </is>
       </c>
       <c r="B89" s="6" t="inlineStr">
         <is>
-          <t>Admin 客服查詢頁：查帳號、名下設備與最近事件</t>
+          <t>三個 App 送審並通過</t>
         </is>
       </c>
       <c r="C89" s="6" t="inlineStr">
         <is>
-          <t>等 P2-14、P1-10、P1-12</t>
+          <t>等 R-27、R-21、R-28、R-29、R-30、R-31、R-32</t>
         </is>
       </c>
       <c r="D89" s="11" t="n"/>
@@ -2942,50 +2951,50 @@
       <c r="H89" s="11" t="n"/>
       <c r="I89" s="12" t="n"/>
     </row>
-    <row r="91">
-      <c r="A91" s="10" t="inlineStr">
+    <row r="90" ht="32" customHeight="1">
+      <c r="A90" s="13" t="inlineStr">
+        <is>
+          <t>R-40</t>
+        </is>
+      </c>
+      <c r="B90" s="6" t="inlineStr">
+        <is>
+          <t>Admin 客服查詢頁：查帳號、名下設備與最近事件</t>
+        </is>
+      </c>
+      <c r="C90" s="6" t="inlineStr">
+        <is>
+          <t>等 P2-14、P1-10、P1-12</t>
+        </is>
+      </c>
+      <c r="D90" s="11" t="n"/>
+      <c r="E90" s="11" t="n"/>
+      <c r="F90" s="11" t="n"/>
+      <c r="G90" s="11" t="n"/>
+      <c r="H90" s="11" t="n"/>
+      <c r="I90" s="12" t="n"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="10" t="inlineStr">
         <is>
           <t>❓ 待確認問題</t>
         </is>
       </c>
     </row>
-    <row r="92">
-      <c r="A92" s="4" t="inlineStr">
+    <row r="93">
+      <c r="A93" s="4" t="inlineStr">
         <is>
           <t>編號</t>
         </is>
       </c>
-      <c r="B92" s="4" t="inlineStr">
+      <c r="B93" s="4" t="inlineStr">
         <is>
           <t>問題</t>
         </is>
       </c>
-      <c r="C92" s="4" t="inlineStr">
+      <c r="C93" s="4" t="inlineStr">
         <is>
           <t>影響的任務 / 為什麼重要</t>
-        </is>
-      </c>
-      <c r="D92" s="11" t="n"/>
-      <c r="E92" s="11" t="n"/>
-      <c r="F92" s="11" t="n"/>
-      <c r="G92" s="11" t="n"/>
-      <c r="H92" s="11" t="n"/>
-      <c r="I92" s="12" t="n"/>
-    </row>
-    <row r="93" ht="18" customHeight="1">
-      <c r="A93" s="13" t="inlineStr">
-        <is>
-          <t>Q3</t>
-        </is>
-      </c>
-      <c r="B93" s="6" t="inlineStr">
-        <is>
-          <t>韌體打算閉源商業銷售嗎？</t>
-        </is>
-      </c>
-      <c r="C93" s="6" t="inlineStr">
-        <is>
-          <t>P1-06, P1-07：決定 GPL／LGPL 依賴要開源還是替換。</t>
         </is>
       </c>
       <c r="D93" s="11" t="n"/>
@@ -2995,20 +3004,20 @@
       <c r="H93" s="11" t="n"/>
       <c r="I93" s="12" t="n"/>
     </row>
-    <row r="94" ht="32" customHeight="1">
+    <row r="94" ht="18" customHeight="1">
       <c r="A94" s="13" t="inlineStr">
         <is>
-          <t>Q11</t>
+          <t>Q3</t>
         </is>
       </c>
       <c r="B94" s="6" t="inlineStr">
         <is>
-          <t>馬會快活的賽馬日版和新春版各多少隻（共 2,500）？</t>
+          <t>韌體打算閉源商業銷售嗎？</t>
         </is>
       </c>
       <c r="C94" s="6" t="inlineStr">
         <is>
-          <t>R-09, R-15：兩款的服裝和配件要分開訂料；11/20 前不知道，PP 樣和大貨單（11/27）會被拖慢。由馬會決定。</t>
+          <t>P1-06, P1-07：決定 GPL／LGPL 依賴要開源還是替換。</t>
         </is>
       </c>
       <c r="D94" s="11" t="n"/>
@@ -3018,20 +3027,20 @@
       <c r="H94" s="11" t="n"/>
       <c r="I94" s="12" t="n"/>
     </row>
-    <row r="95" ht="60" customHeight="1">
+    <row r="95" ht="32" customHeight="1">
       <c r="A95" s="13" t="inlineStr">
         <is>
-          <t>Q12</t>
+          <t>Q11</t>
         </is>
       </c>
       <c r="B95" s="6" t="inlineStr">
         <is>
-          <t>快活 App 的「會員綁定」是指甚麼：用我們自己的帳號（email 驗證碼），還是接馬會的會員帳號登入（SSO）？</t>
+          <t>馬會快活的賽馬日版和新春版各多少隻（共 2,500）？</t>
         </is>
       </c>
       <c r="C95" s="6" t="inlineStr">
         <is>
-          <t>P0-11, 快活 App（未入追蹤表）：接馬會 SSO 的話，登入、帳號刪除和資料歸屬都要按馬會的介面重做，工作量和排期要另估，而且 W5（11/9–11/13）就要做快活 App 的綁定；用我們的帳號則和其他品牌共用同一套流程。由馬會決定，要盡早問。</t>
+          <t>R-09, R-15：兩款的服裝和配件要分開訂料；11/20 前不知道，PP 樣和大貨單（11/27）會被拖慢。由馬會決定。</t>
         </is>
       </c>
       <c r="D95" s="11" t="n"/>
@@ -3041,20 +3050,20 @@
       <c r="H95" s="11" t="n"/>
       <c r="I95" s="12" t="n"/>
     </row>
-    <row r="96" ht="46" customHeight="1">
+    <row r="96" ht="60" customHeight="1">
       <c r="A96" s="13" t="inlineStr">
         <is>
-          <t>Q13</t>
+          <t>Q12</t>
         </is>
       </c>
       <c r="B96" s="6" t="inlineStr">
         <is>
-          <t>政協青年聯會版的角色、語言和內容由誰提供？什麼時候交？</t>
+          <t>快活 App 的「會員綁定」是指甚麼：用我們自己的帳號（email 驗證碼），還是接馬會的會員帳號登入（SSO）？</t>
         </is>
       </c>
       <c r="C96" s="6" t="inlineStr">
         <is>
-          <t>品牌 B 的 App 頁面：品牌 B 的用戶是成人會員，但角色、說話語言、內容規則都還沒有。最遲 11/13 要拿到，才趕得及內部測試和 App 頁面（W6）。</t>
+          <t>P0-11, 快活 App（未入追蹤表）：接馬會 SSO 的話，登入、帳號刪除和資料歸屬都要按馬會的介面重做，工作量和排期要另估，而且 W5（11/9–11/13）就要做快活 App 的綁定；用我們的帳號則和其他品牌共用同一套流程。由馬會決定，要盡早問。</t>
         </is>
       </c>
       <c r="D96" s="11" t="n"/>
@@ -3064,64 +3073,88 @@
       <c r="H96" s="11" t="n"/>
       <c r="I96" s="12" t="n"/>
     </row>
-    <row r="98">
-      <c r="A98" s="10" t="inlineStr">
+    <row r="97" ht="46" customHeight="1">
+      <c r="A97" s="13" t="inlineStr">
+        <is>
+          <t>Q13</t>
+        </is>
+      </c>
+      <c r="B97" s="6" t="inlineStr">
+        <is>
+          <t>政協青年聯會版的角色、語言和內容由誰提供？什麼時候交？</t>
+        </is>
+      </c>
+      <c r="C97" s="6" t="inlineStr">
+        <is>
+          <t>品牌 B 的 App 頁面：品牌 B 的用戶是成人會員，但角色、說話語言、內容規則都還沒有。最遲 11/13 要拿到，才趕得及內部測試和 App 頁面（W6）。</t>
+        </is>
+      </c>
+      <c r="D97" s="11" t="n"/>
+      <c r="E97" s="11" t="n"/>
+      <c r="F97" s="11" t="n"/>
+      <c r="G97" s="11" t="n"/>
+      <c r="H97" s="11" t="n"/>
+      <c r="I97" s="12" t="n"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="10" t="inlineStr">
         <is>
           <t>說明</t>
         </is>
       </c>
     </row>
-    <row r="99" ht="32" customHeight="1">
-      <c r="A99" s="14" t="inlineStr">
+    <row r="100" ht="32" customHeight="1">
+      <c r="A100" s="14" t="inlineStr">
         <is>
           <t>・狀態：未開始 → 進行中 → 已完成。只有測試真的跑過而且通過才算已完成；阻塞要在備註寫原因；不再需要的任務標不適用，不要刪。</t>
-        </is>
-      </c>
-    </row>
-    <row r="100" ht="18" customHeight="1">
-      <c r="A100" s="14" t="inlineStr">
-        <is>
-          <t>・測試結果：未測試 / 通過 / 失敗 / 部分通過。測試證據寫跑了什麼、看到什麼，完整歷史在「更新記錄」。</t>
         </is>
       </c>
     </row>
     <row r="101" ht="18" customHeight="1">
       <c r="A101" s="14" t="inlineStr">
         <is>
-          <t>・「接下來」按階段排序，同一階段內再按優先級；依賴還沒滿足的任務不會出現在「接下來」。</t>
+          <t>・測試結果：未測試 / 通過 / 失敗 / 部分通過。測試證據寫跑了什麼、看到什麼，完整歷史在「更新記錄」。</t>
         </is>
       </c>
     </row>
     <row r="102" ht="18" customHeight="1">
       <c r="A102" s="14" t="inlineStr">
         <is>
+          <t>・「接下來」按階段排序，同一階段內再按優先級；依賴還沒滿足的任務不會出現在「接下來」。</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" ht="18" customHeight="1">
+      <c r="A103" s="14" t="inlineStr">
+        <is>
           <t>・可以手動改：「任務清單」的狀態、測試結果、測試證據、Commit、備註，以及「待確認問題」的回答。其餘欄位和本頁由腳本維護。</t>
         </is>
       </c>
     </row>
-    <row r="103" ht="32" customHeight="1">
-      <c r="A103" s="14" t="inlineStr">
+    <row r="104" ht="32" customHeight="1">
+      <c r="A104" s="14" t="inlineStr">
         <is>
           <t>・建議用法：在 Claude Code 對 Claude 說「P0-02 做完了」或輸入 /prod-readiness。Claude 會先跑測試再更新，並寫進「更新記錄」。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="84">
-    <mergeCell ref="A41:I41"/>
+  <mergeCells count="85">
     <mergeCell ref="A99:I99"/>
     <mergeCell ref="C82:I82"/>
     <mergeCell ref="E39:I39"/>
     <mergeCell ref="C67:I67"/>
     <mergeCell ref="E48:I48"/>
     <mergeCell ref="A101:I101"/>
-    <mergeCell ref="C53:I53"/>
     <mergeCell ref="A2:I2"/>
     <mergeCell ref="E29:I29"/>
     <mergeCell ref="E38:I38"/>
+    <mergeCell ref="A42:I42"/>
     <mergeCell ref="C83:I83"/>
-    <mergeCell ref="C92:I92"/>
+    <mergeCell ref="A53:I53"/>
     <mergeCell ref="E31:I31"/>
+    <mergeCell ref="E40:I40"/>
+    <mergeCell ref="C97:I97"/>
     <mergeCell ref="A19:I19"/>
     <mergeCell ref="E26:I26"/>
     <mergeCell ref="A103:I103"/>
@@ -3130,7 +3163,6 @@
     <mergeCell ref="C60:I60"/>
     <mergeCell ref="C71:I71"/>
     <mergeCell ref="E50:I50"/>
-    <mergeCell ref="E42:I42"/>
     <mergeCell ref="C57:I57"/>
     <mergeCell ref="C66:I66"/>
     <mergeCell ref="E44:I44"/>
@@ -3139,16 +3171,15 @@
     <mergeCell ref="C77:I77"/>
     <mergeCell ref="C86:I86"/>
     <mergeCell ref="C68:I68"/>
-    <mergeCell ref="A91:I91"/>
     <mergeCell ref="A100:I100"/>
     <mergeCell ref="C58:I58"/>
-    <mergeCell ref="A52:I52"/>
     <mergeCell ref="E30:I30"/>
     <mergeCell ref="E46:I46"/>
     <mergeCell ref="A102:I102"/>
     <mergeCell ref="C85:I85"/>
     <mergeCell ref="C94:I94"/>
     <mergeCell ref="C65:I65"/>
+    <mergeCell ref="A92:I92"/>
     <mergeCell ref="C75:I75"/>
     <mergeCell ref="C84:I84"/>
     <mergeCell ref="C80:I80"/>
@@ -3162,6 +3193,7 @@
     <mergeCell ref="E24:I24"/>
     <mergeCell ref="E33:I33"/>
     <mergeCell ref="A3:I3"/>
+    <mergeCell ref="A104:I104"/>
     <mergeCell ref="E35:I35"/>
     <mergeCell ref="C74:I74"/>
     <mergeCell ref="C88:I88"/>
@@ -3173,6 +3205,7 @@
     <mergeCell ref="C72:I72"/>
     <mergeCell ref="C81:I81"/>
     <mergeCell ref="C69:I69"/>
+    <mergeCell ref="E51:I51"/>
     <mergeCell ref="C96:I96"/>
     <mergeCell ref="C78:I78"/>
     <mergeCell ref="C87:I87"/>
@@ -3188,8 +3221,8 @@
     <mergeCell ref="E36:I36"/>
     <mergeCell ref="C63:I63"/>
     <mergeCell ref="C93:I93"/>
-    <mergeCell ref="A98:I98"/>
     <mergeCell ref="C56:I56"/>
+    <mergeCell ref="C90:I90"/>
     <mergeCell ref="E22:I22"/>
     <mergeCell ref="C76:I76"/>
   </mergeCells>
@@ -4510,7 +4543,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="60" customHeight="1">
+    <row r="17" ht="144" customHeight="1">
       <c r="A17" s="13" t="inlineStr">
         <is>
           <t>P1-02</t>
@@ -4538,12 +4571,12 @@
       </c>
       <c r="F17" s="13" t="inlineStr">
         <is>
-          <t>未開始</t>
+          <t>進行中</t>
         </is>
       </c>
       <c r="G17" s="13" t="inlineStr">
         <is>
-          <t>未測試</t>
+          <t>部分通過</t>
         </is>
       </c>
       <c r="H17" s="13" t="n"/>
@@ -4569,8 +4602,16 @@
         </is>
       </c>
       <c r="M17" s="13" t="n"/>
-      <c r="N17" s="6" t="n"/>
-      <c r="O17" s="13" t="n"/>
+      <c r="N17" s="6" t="inlineStr">
+        <is>
+          <t>本機（分支 p1-02-log-pii）：模擬板子跑 3 輪，孩子名 PROBE小明、性格『鍾意恐龍』、記憶『佢有隻狗叫PROBE豆豆』；把對話、回覆、事實切成 47 段搜日誌 → 預設 INFO 0 段；同一流程 LOG_LEVEL=DEBUG → 27 段（證明搜尋有效）。INFO 日誌也無 token。pytest 245 passed（新增 test_log_privacy 6 項：事實/摘要、PostgREST details、OpenRouter flagged_input、非 JSON 回覆、預設 INFO 與 traceback 無變量值）。未做：部署線上並在生產日誌重跑。</t>
+        </is>
+      </c>
+      <c r="O17" s="13" t="inlineStr">
+        <is>
+          <t>4214b99</t>
+        </is>
+      </c>
       <c r="P17" s="6" t="n"/>
     </row>
     <row r="18" ht="158" customHeight="1">
@@ -6909,7 +6950,7 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="228" customHeight="1">
+    <row r="50" ht="214" customHeight="1">
       <c r="A50" s="13" t="inlineStr">
         <is>
           <t>R-13</t>
@@ -6967,12 +7008,13 @@
       </c>
       <c r="M50" s="13" t="inlineStr">
         <is>
-          <t>P0-02, P0-03, P0-04, P0-05, P0-06, P0-07, P0-08, P0-09, P0-10, P0-11, P0-12, P0-13, P1-01, P1-02, P2-09, R-01, R-02, R-04, R-05, R-06, P0-15, P0-16, P1-09, P1-11</t>
+          <t>P0-02, P0-03, P0-04, P0-05, P0-06, P0-07, P0-08, P0-09, P0-10, P0-11, P0-12, P0-13, P1-01, P1-02, P2-09, R-01, R-02, R-04, R-05, R-06, P0-15, P0-16, P1-11</t>
         </is>
       </c>
       <c r="P50" s="6" t="inlineStr">
         <is>
-          <t>[2026-10-05] 新增：2026-10-05 定：兩個 checkpoint 為 10/30（CP1）與 11/27（CP2＝R-08）；硬底線是農曆新年（2027-02-06）前交付。</t>
+          <t>[2026-10-05] 新增：2026-10-05 定：兩個 checkpoint 為 10/30（CP1）與 11/27（CP2＝R-08）；硬底線是農曆新年（2027-02-06）前交付。
+[2026-10-14] 2026-10-14 用戶決定：移除 P1-09（家長鎖）。品牌 C 已延到 1/15 之後，P1-09 阻塞，留在依賴裡 CP1 永遠過不了。</t>
         </is>
       </c>
     </row>
@@ -10171,7 +10213,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I257"/>
+  <dimension ref="A1:I260"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -19056,8 +19098,117 @@
         </is>
       </c>
     </row>
+    <row r="258" ht="116" customHeight="1">
+      <c r="A258" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 11:20</t>
+        </is>
+      </c>
+      <c r="B258" s="13" t="inlineStr">
+        <is>
+          <t>R-13</t>
+        </is>
+      </c>
+      <c r="C258" s="6" t="inlineStr">
+        <is>
+          <t>CP1 內測就緒檢查（10/30）</t>
+        </is>
+      </c>
+      <c r="D258" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E258" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="F258" s="13" t="n"/>
+      <c r="G258" s="6" t="n"/>
+      <c r="H258" s="13" t="n"/>
+      <c r="I258" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-14 用戶決定：移除 P1-09（家長鎖）。品牌 C 已延到 1/15 之後，P1-09 阻塞，留在依賴裡 CP1 永遠過不了。；修改了依賴→P0-02, P0-03, P0-04, P0-05, P0-06, P0-07, P0-08, P0-09, P0-10, P0-11, P0-12, P0-13, P1-01, P1-02, P2-09, R-01, R-02, R-04, R-05, R-06, P0-15, P0-16, P1-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="259" ht="32" customHeight="1">
+      <c r="A259" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 11:20</t>
+        </is>
+      </c>
+      <c r="B259" s="13" t="inlineStr">
+        <is>
+          <t>P1-02</t>
+        </is>
+      </c>
+      <c r="C259" s="6" t="inlineStr">
+        <is>
+          <t>日誌移除兒童個人資料</t>
+        </is>
+      </c>
+      <c r="D259" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E259" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F259" s="13" t="n"/>
+      <c r="G259" s="6" t="n"/>
+      <c r="H259" s="13" t="n"/>
+      <c r="I259" s="6" t="n"/>
+    </row>
+    <row r="260" ht="130" customHeight="1">
+      <c r="A260" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 11:28</t>
+        </is>
+      </c>
+      <c r="B260" s="13" t="inlineStr">
+        <is>
+          <t>P1-02</t>
+        </is>
+      </c>
+      <c r="C260" s="6" t="inlineStr">
+        <is>
+          <t>日誌移除兒童個人資料</t>
+        </is>
+      </c>
+      <c r="D260" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="E260" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F260" s="13" t="inlineStr">
+        <is>
+          <t>部分通過</t>
+        </is>
+      </c>
+      <c r="G260" s="6" t="inlineStr">
+        <is>
+          <t>本機（分支 p1-02-log-pii）：模擬板子跑 3 輪，孩子名 PROBE小明、性格『鍾意恐龍』、記憶『佢有隻狗叫PROBE豆豆』；把對話、回覆、事實切成 47 段搜日誌 → 預設 INFO 0 段；同一流程 LOG_LEVEL=DEBUG → 27 段（證明搜尋有效）。INFO 日誌也無 token。pytest 245 passed（新增 test_log_privacy 6 項：事實/摘要、PostgREST details、OpenRouter flagged_input、非 JSON 回覆、預設 INFO 與 traceback 無變量值）。未做：部署線上並在生產日誌重跑。</t>
+        </is>
+      </c>
+      <c r="H260" s="13" t="inlineStr">
+        <is>
+          <t>4214b99</t>
+        </is>
+      </c>
+      <c r="I260" s="6" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I257"/>
+  <autoFilter ref="A1:I260"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add the admin Devices page: every toy's state, firmware and binding (P2-14).
admin_list_devices() gives super admins each board's firmware, last call,
owner email and when its key was issued -- no pairing code, secret or child
data. Online comes from the voice server's new /internal/devices_presence,
polled every 15 s, with the Wi-Fi a board last reported. Two support
actions, each with a reason written to the audit log in the same
transaction: reset a board's device key, and force-unbind it from its
account. The tracker records P2-14 as partly tested on the local stack, and
R-41 as done.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/production-readiness.xlsx
+++ b/docs/production-readiness.xlsx
@@ -13,9 +13,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="更新記錄" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'任務清單'!$A$1:$P$88</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'任務清單'!$A$1:$P$89</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'待確認問題'!$A$1:$G$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$260</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$270</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -665,14 +665,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>最後更新：2026-10-14 11:28　·　本頁由 tracker.py 自動生成，請勿手動編輯</t>
+          <t>最後更新：2026-10-14 15:50　·　本頁由 tracker.py 自動生成，請勿手動編輯</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>總進度：17/83 已完成（20%）　·　目前階段：1 止血定案（10/5–10/16）</t>
+          <t>總進度：18/84 已完成（21%）　·　目前階段：1 止血定案（10/5–10/16）</t>
         </is>
       </c>
     </row>
@@ -780,7 +780,7 @@
       </c>
       <c r="D7" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A7,'任務清單'!$F:$F,D$5)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E7" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A7,'任務清單'!$F:$F,E$5)</f>
@@ -792,7 +792,7 @@
       </c>
       <c r="G7" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A7,'任務清單'!$F:$F,G$5)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H7" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A7,'任務清單'!$F:$F,H$5)</f>
@@ -820,11 +820,11 @@
       </c>
       <c r="D8" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A8,'任務清單'!$F:$F,D$5)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E8" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A8,'任務清單'!$F:$F,E$5)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F8" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A8,'任務清單'!$F:$F,F$5)</f>
@@ -856,11 +856,11 @@
       </c>
       <c r="C9" s="7">
         <f>COUNTIF('任務清單'!$B:$B,$A9)</f>
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D9" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A9,'任務清單'!$F:$F,D$5)</f>
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E9" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A9,'任務清單'!$F:$F,E$5)</f>
@@ -868,11 +868,11 @@
       </c>
       <c r="F9" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A9,'任務清單'!$F:$F,F$5)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G9" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A9,'任務清單'!$F:$F,G$5)</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H9" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A9,'任務清單'!$F:$F,H$5)</f>
@@ -880,7 +880,7 @@
       </c>
       <c r="I9" s="8">
         <f>IFERROR(F9/(C9-H9),0)</f>
-        <v>0.02631578947368421</v>
+        <v>0.05128205128205128</v>
       </c>
     </row>
     <row r="10">
@@ -892,19 +892,19 @@
       <c r="B10" s="6" t="n"/>
       <c r="C10" s="5">
         <f>SUM(C6:C9)</f>
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D10" s="5">
         <f>SUM(D6:D9)</f>
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E10" s="5">
         <f>SUM(E6:E9)</f>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F10" s="5">
         <f>SUM(F6:F9)</f>
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G10" s="5">
         <f>SUM(G6:G9)</f>
@@ -916,7 +916,7 @@
       </c>
       <c r="I10" s="9">
         <f>IFERROR(F10/(C10-H10),0)</f>
-        <v>0.20481927710843373</v>
+        <v>0.21428571428571427</v>
       </c>
     </row>
     <row r="12">
@@ -983,7 +983,7 @@
       </c>
       <c r="D13" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A13,'任務清單'!$F:$F,D$12)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E13" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A13,'任務清單'!$F:$F,E$12)</f>
@@ -995,7 +995,7 @@
       </c>
       <c r="G13" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A13,'任務清單'!$F:$F,G$12)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H13" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A13,'任務清單'!$F:$F,H$12)</f>
@@ -1019,23 +1019,23 @@
       </c>
       <c r="C14" s="7">
         <f>COUNTIF('任務清單'!$C:$C,$A14)</f>
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D14" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A14,'任務清單'!$F:$F,D$12)</f>
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="E14" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A14,'任務清單'!$F:$F,E$12)</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F14" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A14,'任務清單'!$F:$F,F$12)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G14" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A14,'任務清單'!$F:$F,G$12)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H14" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A14,'任務清單'!$F:$F,H$12)</f>
@@ -1043,7 +1043,7 @@
       </c>
       <c r="I14" s="8">
         <f>IFERROR(F14/(C14-H14),0)</f>
-        <v>0.07692307692307693</v>
+        <v>0.1111111111111111</v>
       </c>
     </row>
     <row r="15" ht="46" customHeight="1">
@@ -1135,19 +1135,19 @@
       <c r="B17" s="6" t="n"/>
       <c r="C17" s="5">
         <f>SUM(C13:C16)</f>
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D17" s="5">
         <f>SUM(D13:D16)</f>
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E17" s="5">
         <f>SUM(E13:E16)</f>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F17" s="5">
         <f>SUM(F13:F16)</f>
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G17" s="5">
         <f>SUM(G13:G16)</f>
@@ -1159,7 +1159,7 @@
       </c>
       <c r="I17" s="9">
         <f>IFERROR(F17/(C17-H17),0)</f>
-        <v>0.20481927710843373</v>
+        <v>0.21428571428571427</v>
       </c>
     </row>
     <row r="19">
@@ -1518,15 +1518,15 @@
       <c r="H30" s="11" t="n"/>
       <c r="I30" s="12" t="n"/>
     </row>
-    <row r="31" ht="200" customHeight="1">
+    <row r="31" ht="298" customHeight="1">
       <c r="A31" s="13" t="inlineStr">
         <is>
-          <t>R-21</t>
+          <t>P2-14</t>
         </is>
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>藍牙配網與綁定（取代熱點配網）</t>
+          <t>Admin 設備頁：每台玩具的狀態、韌體與基本操作</t>
         </is>
       </c>
       <c r="C31" s="13" t="inlineStr">
@@ -1541,7 +1541,8 @@
       </c>
       <c r="E31" s="6" t="inlineStr">
         <is>
-          <t>① 設備在「未配網、Wi-Fi 連不上、未綁定、長按 BOOT」時以 AIBuddy-XXXX 名稱廣播藍牙，廣播資料帶品牌，品牌 App 只列出自己品牌的設備。② 設備經藍牙回傳它掃描到的 2.4GHz Wi-Fi 清單，App 讓用戶選擇並填密碼。③ App 經藍牙把 SSID、密碼和綁定票（P0-11）一起交給設備；藍牙通道加密（ESP 標準配網協定 security 1/2 或同等）。④ 設備連上 Wi-Fi 後自己完成認領，App 顯示綁定成功或失敗原因（密碼錯、設備已有主人、票過期）。⑤ 配網期間不啟動音訊；完成後釋放藍牙記憶體再開語音（必要時重開機），對話中最低 heap 不比現在差。⑥ 解綁在 App 內完成（P1-12），解綁後設備進入藍牙待綁定狀態。⑦ SoftAP 熱點配網保留給開發和運維（隱藏觸發方式或編譯開關），量產用戶流程不出現。</t>
+          <t>上次測試：部分通過 — 本機（未 commit）：migration 20261014140000 套用兩次無錯。探測腳本用 GoTrue 真實登入：超管 admin_list_devices 200（不含 user_code）；④ 內容管理員 → 42501、anon → 42501；超管直接讀 device_secrets → 42501；空原因 → 22023；重置密鑰 → device_secrets 行刪除；解綁 → user_id/claimed_at 清空；兩者各寫 1 筆含原因與前後值的審計，超管改審計 → 403。網頁（獨立副本+獨立語音伺服器 7871）：模擬 62:70 連上 → 15 秒內不刷新顯示 Online、-52 dBm；斷線後下一次輪詢變 Offline；按 f214 搜尋、強制解綁、重置密鑰、審計頁都看到兩筆；375px 無橫向捲動。pytest 71 passed。未做：① ② ③ 需真板 62:70，且要用新代碼重啟 7860 語音伺服器
+列出全部設備，可按 MAC、設備名、家長 email 搜尋，按狀態和韌體篩選；顯示在線／離線（取自語音伺服器）、上次上線、韌體版本、OTA 失敗版本、綁定帳號與時間、出廠鎖定的 IP；單台詳情可做「重置設備密鑰」「強制解綁」，兩者都要填原因並寫入審計記錄（P1-10）；不顯示任何對話、記憶或孩子資料（Q7）；只有超級管理員能讀。</t>
         </is>
       </c>
       <c r="F31" s="11" t="n"/>
@@ -1549,15 +1550,15 @@
       <c r="H31" s="11" t="n"/>
       <c r="I31" s="12" t="n"/>
     </row>
-    <row r="32" ht="116" customHeight="1">
+    <row r="32" ht="200" customHeight="1">
       <c r="A32" s="13" t="inlineStr">
         <is>
-          <t>R-36</t>
+          <t>R-21</t>
         </is>
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>未認領的設備停在配對狀態，不再每秒重連 websocket</t>
+          <t>藍牙配網與綁定（取代熱點配網）</t>
         </is>
       </c>
       <c r="C32" s="13" t="inlineStr">
@@ -1572,7 +1573,7 @@
       </c>
       <c r="E32" s="6" t="inlineStr">
         <is>
-          <t>① 拿到 202 或 websocket 被 4401 拒絕後，設備停掉 websocket 自動重連，進入待綁定狀態（燈號可分辨）。② 待綁定時只按退避（5 秒起、上限 PROVISION_BACKOFF_MAX）呼叫 generate_auth_token，不開 websocket。③ 被認領後下一次輪詢拿到 200，在 10 秒內（加退避）自動開 websocket 並能對話，不用重開機。④ 已綁定設備網絡斷線重連的行為不變。⑤ 隨 OTA 推出。</t>
+          <t>① 設備在「未配網、Wi-Fi 連不上、未綁定、長按 BOOT」時以 AIBuddy-XXXX 名稱廣播藍牙，廣播資料帶品牌，品牌 App 只列出自己品牌的設備。② 設備經藍牙回傳它掃描到的 2.4GHz Wi-Fi 清單，App 讓用戶選擇並填密碼。③ App 經藍牙把 SSID、密碼和綁定票（P0-11）一起交給設備；藍牙通道加密（ESP 標準配網協定 security 1/2 或同等）。④ 設備連上 Wi-Fi 後自己完成認領，App 顯示綁定成功或失敗原因（密碼錯、設備已有主人、票過期）。⑤ 配網期間不啟動音訊；完成後釋放藍牙記憶體再開語音（必要時重開機），對話中最低 heap 不比現在差。⑥ 解綁在 App 內完成（P1-12），解綁後設備進入藍牙待綁定狀態。⑦ SoftAP 熱點配網保留給開發和運維（隱藏觸發方式或編譯開關），量產用戶流程不出現。</t>
         </is>
       </c>
       <c r="F32" s="11" t="n"/>
@@ -1580,20 +1581,20 @@
       <c r="H32" s="11" t="n"/>
       <c r="I32" s="12" t="n"/>
     </row>
-    <row r="33" ht="228" customHeight="1">
+    <row r="33" ht="116" customHeight="1">
       <c r="A33" s="13" t="inlineStr">
         <is>
-          <t>P2-12</t>
+          <t>R-36</t>
         </is>
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>量產燒錄前加大 app 分區</t>
+          <t>未認領的設備停在配對狀態，不再每秒重連 websocket</t>
         </is>
       </c>
       <c r="C33" s="13" t="inlineStr">
         <is>
-          <t>3 封閉內測</t>
+          <t>2 內測準備</t>
         </is>
       </c>
       <c r="D33" s="13" t="inlineStr">
@@ -1603,8 +1604,7 @@
       </c>
       <c r="E33" s="6" t="inlineStr">
         <is>
-          <t>上次測試：部分通過 — 62:70（spotpear-ai-toy-p212 原型，現已併入 spotpear-ai-toy）：① 本機 OTA 1.6.1→1.6.2 寫入新 app1，120s 後 confirmed ② 3 秒 abort 的 1.6.3 → PANIC → 回到 1.6.2，ota_failed_version=1.6.3 ③ 崩潰寫入 coredump 14.8KB ④ 資源分區 9 個聲音 504KB/2MB，開機 CRC 63ms，OTA 後照常；損壞/清空 → 退回內建聲音無崩潰 ⑤ pio 全部 18 個 env 編譯通過，映像都在各自 app 槽內（Spotpear 4 個 1.59–1.60MB / 4MB；其他板仍 2MB 槽）；R-21 藍牙探針版 2,326,128 bytes &lt; 4MB ⑥ release_firmware.py 映像 &gt; app 槽即拒發。未做：雲端 OTA 一次（等上 UAT）、出廠腳本寫入資源包（R-10）
-新分區表（例如 app0/app1 各 4MB，保留 nvs/otadata 位置）在出廠前定案並寫入出廠腳本；OTA 與回滾在新分區表上照常</t>
+          <t>① 拿到 202 或 websocket 被 4401 拒絕後，設備停掉 websocket 自動重連，進入待綁定狀態（燈號可分辨）。② 待綁定時只按退避（5 秒起、上限 PROVISION_BACKOFF_MAX）呼叫 generate_auth_token，不開 websocket。③ 被認領後下一次輪詢拿到 200，在 10 秒內（加退避）自動開 websocket 並能對話，不用重開機。④ 已綁定設備網絡斷線重連的行為不變。⑤ 隨 OTA 推出。</t>
         </is>
       </c>
       <c r="F33" s="11" t="n"/>
@@ -1612,15 +1612,15 @@
       <c r="H33" s="11" t="n"/>
       <c r="I33" s="12" t="n"/>
     </row>
-    <row r="34" ht="242" customHeight="1">
+    <row r="34" ht="228" customHeight="1">
       <c r="A34" s="13" t="inlineStr">
         <is>
-          <t>R-37</t>
+          <t>P2-12</t>
         </is>
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>網頁設定玩具的 Wi-Fi：查看、新增、刪除</t>
+          <t>量產燒錄前加大 app 分區</t>
         </is>
       </c>
       <c r="C34" s="13" t="inlineStr">
@@ -1635,8 +1635,8 @@
       </c>
       <c r="E34" s="6" t="inlineStr">
         <is>
-          <t>上次測試：部分通過 — 模擬玩具經本機語音服務器＋網頁：status/scan/add/delete 正常；刪除目前 Wi-Fi → current 被拒；斷線 5 秒內頁面顯示睡著、按鈕停用；測試密碼在語音服務器日誌、網頁服務器日誌、資料庫均搜不到；用別人裝置 ID 重放 server action → forbidden；pytest 17 項通過（全套 230）；韌體 spotpear-ai-toy-localall 編譯通過（RAM 17.5%、Flash 75.9%）。未測：真機 ①② 及 OTA 推出
-① 設定頁顯示玩具在線／離線、目前 Wi-Fi 和訊號、已記住的 Wi-Fi 清單（只有名稱，不顯示密碼）② 在線時可新增 Wi-Fi（輸入或從玩具掃描到的清單選）、刪除 Wi-Fi；不能刪除正在使用的那個 ③ 經 /ws/esp32 轉送：伺服器先確認是設備主人；密碼不寫入資料庫、不寫入日誌 ④ 新增不切換網絡，目前 Wi-Fi 消失時才按訊號選；清單標示「連過／未連過」⑤ 上限 8 個 ⑥ 韌體改動經 OTA 推出</t>
+          <t>上次測試：部分通過 — 62:70（spotpear-ai-toy-p212 原型，現已併入 spotpear-ai-toy）：① 本機 OTA 1.6.1→1.6.2 寫入新 app1，120s 後 confirmed ② 3 秒 abort 的 1.6.3 → PANIC → 回到 1.6.2，ota_failed_version=1.6.3 ③ 崩潰寫入 coredump 14.8KB ④ 資源分區 9 個聲音 504KB/2MB，開機 CRC 63ms，OTA 後照常；損壞/清空 → 退回內建聲音無崩潰 ⑤ pio 全部 18 個 env 編譯通過，映像都在各自 app 槽內（Spotpear 4 個 1.59–1.60MB / 4MB；其他板仍 2MB 槽）；R-21 藍牙探針版 2,326,128 bytes &lt; 4MB ⑥ release_firmware.py 映像 &gt; app 槽即拒發。未做：雲端 OTA 一次（等上 UAT）、出廠腳本寫入資源包（R-10）
+新分區表（例如 app0/app1 各 4MB，保留 nvs/otadata 位置）在出廠前定案並寫入出廠腳本；OTA 與回滾在新分區表上照常</t>
         </is>
       </c>
       <c r="F34" s="11" t="n"/>
@@ -1644,30 +1644,31 @@
       <c r="H34" s="11" t="n"/>
       <c r="I34" s="12" t="n"/>
     </row>
-    <row r="35" ht="60" customHeight="1">
+    <row r="35" ht="242" customHeight="1">
       <c r="A35" s="13" t="inlineStr">
         <is>
-          <t>P1-01</t>
+          <t>R-37</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>加入內容審核層（輸入與輸出）</t>
+          <t>網頁設定玩具的 Wi-Fi：查看、新增、刪除</t>
         </is>
       </c>
       <c r="C35" s="13" t="inlineStr">
         <is>
-          <t>2 內測準備</t>
+          <t>3 封閉內測</t>
         </is>
       </c>
       <c r="D35" s="13" t="inlineStr">
         <is>
-          <t>未開始</t>
+          <t>進行中</t>
         </is>
       </c>
       <c r="E35" s="6" t="inlineStr">
         <is>
-          <t>STT 文字與 LLM 輸出都經審核，尺度按 3–6 歲；命中時換成安全回覆並記錄事件，事件只記類別、時間、角色，不記原文（管理員不能看兒童內容，見 Q7）；首字延遲增加 ≤150ms。</t>
+          <t>上次測試：部分通過 — 模擬玩具經本機語音服務器＋網頁：status/scan/add/delete 正常；刪除目前 Wi-Fi → current 被拒；斷線 5 秒內頁面顯示睡著、按鈕停用；測試密碼在語音服務器日誌、網頁服務器日誌、資料庫均搜不到；用別人裝置 ID 重放 server action → forbidden；pytest 17 項通過（全套 230）；韌體 spotpear-ai-toy-localall 編譯通過（RAM 17.5%、Flash 75.9%）。未測：真機 ①② 及 OTA 推出
+① 設定頁顯示玩具在線／離線、目前 Wi-Fi 和訊號、已記住的 Wi-Fi 清單（只有名稱，不顯示密碼）② 在線時可新增 Wi-Fi（輸入或從玩具掃描到的清單選）、刪除 Wi-Fi；不能刪除正在使用的那個 ③ 經 /ws/esp32 轉送：伺服器先確認是設備主人；密碼不寫入資料庫、不寫入日誌 ④ 新增不切換網絡，目前 Wi-Fi 消失時才按訊號選；清單標示「連過／未連過」⑤ 上限 8 個 ⑥ 韌體改動經 OTA 推出</t>
         </is>
       </c>
       <c r="F35" s="11" t="n"/>
@@ -1675,20 +1676,20 @@
       <c r="H35" s="11" t="n"/>
       <c r="I35" s="12" t="n"/>
     </row>
-    <row r="36" ht="46" customHeight="1">
+    <row r="36" ht="102" customHeight="1">
       <c r="A36" s="13" t="inlineStr">
         <is>
-          <t>P1-11</t>
+          <t>R-16</t>
         </is>
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>伺服器與資料庫直接存取的管控</t>
+          <t>Spotpear 量產版加電池電壓檢測（GPIO0 分壓）</t>
         </is>
       </c>
       <c r="C36" s="13" t="inlineStr">
         <is>
-          <t>2 內測準備</t>
+          <t>1 止血定案</t>
         </is>
       </c>
       <c r="D36" s="13" t="inlineStr">
@@ -1698,7 +1699,7 @@
       </c>
       <c r="E36" s="6" t="inlineStr">
         <is>
-          <t>列出誰有 SSH 與資料庫直連權限（越少越好）；service_role key 只存在伺服器的 env；私隱政策寫明這類存取的範圍；每次直接查看生產資料都留記錄。</t>
+          <t>Spotpear 書面確認量產版：GPIO1（屏幕 DC；本版不接屏幕，可空出來）接電芯正極（保護 IC 之後）100k/100k 分壓、100nF 濾波，屏幕不接該腳；GPIO0 保留給現有的 VDD 低電提醒；最好另把充電芯片 CHRG 接到 GPIO12 或 13。樣板到手後，固件讀到的電芯電壓與萬用表相差 ≤50mV，App（R-41）顯示百分比與充電中。</t>
         </is>
       </c>
       <c r="F36" s="11" t="n"/>
@@ -1709,12 +1710,12 @@
     <row r="37" ht="46" customHeight="1">
       <c r="A37" s="13" t="inlineStr">
         <is>
-          <t>P2-02</t>
+          <t>P1-11</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>CI 跑測試與靜態檢查</t>
+          <t>伺服器與資料庫直接存取的管控</t>
         </is>
       </c>
       <c r="C37" s="13" t="inlineStr">
@@ -1729,7 +1730,7 @@
       </c>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>推送與 PR 時跑 pytest、ruff、pyright、next lint、tsc --noEmit、pio run；任何一項失敗就不發佈 image。</t>
+          <t>列出誰有 SSH 與資料庫直連權限（越少越好）；service_role key 只存在伺服器的 env；私隱政策寫明這類存取的範圍；每次直接查看生產資料都留記錄。</t>
         </is>
       </c>
       <c r="F37" s="11" t="n"/>
@@ -1737,15 +1738,15 @@
       <c r="H37" s="11" t="n"/>
       <c r="I37" s="12" t="n"/>
     </row>
-    <row r="38" ht="32" customHeight="1">
+    <row r="38" ht="46" customHeight="1">
       <c r="A38" s="13" t="inlineStr">
         <is>
-          <t>P2-04</t>
+          <t>P2-02</t>
         </is>
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>容器改用非 root 用戶</t>
+          <t>CI 跑測試與靜態檢查</t>
         </is>
       </c>
       <c r="C38" s="13" t="inlineStr">
@@ -1760,7 +1761,7 @@
       </c>
       <c r="E38" s="6" t="inlineStr">
         <is>
-          <t>兩個 Dockerfile 都設定非 root 的 USER。</t>
+          <t>推送與 PR 時跑 pytest、ruff、pyright、next lint、tsc --noEmit、pio run；任何一項失敗就不發佈 image。</t>
         </is>
       </c>
       <c r="F38" s="11" t="n"/>
@@ -1768,15 +1769,15 @@
       <c r="H38" s="11" t="n"/>
       <c r="I38" s="12" t="n"/>
     </row>
-    <row r="39" ht="46" customHeight="1">
+    <row r="39" ht="32" customHeight="1">
       <c r="A39" s="13" t="inlineStr">
         <is>
-          <t>R-04</t>
+          <t>P2-04</t>
         </is>
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>粵語質量評測</t>
+          <t>容器改用非 root 用戶</t>
         </is>
       </c>
       <c r="C39" s="13" t="inlineStr">
@@ -1791,7 +1792,7 @@
       </c>
       <c r="E39" s="6" t="inlineStr">
         <is>
-          <t>有一套粵語評測集（兒童錄音＋文字提示）；選定的 STT 與 LLM 達到門檻：兒童語音字錯率 ≤15%、口語粵語回覆 ≥90%、中英夾雜句能正確理解。</t>
+          <t>兩個 Dockerfile 都設定非 root 的 USER。</t>
         </is>
       </c>
       <c r="F39" s="11" t="n"/>
@@ -1799,15 +1800,15 @@
       <c r="H39" s="11" t="n"/>
       <c r="I39" s="12" t="n"/>
     </row>
-    <row r="40" ht="116" customHeight="1">
+    <row r="40" ht="46" customHeight="1">
       <c r="A40" s="13" t="inlineStr">
         <is>
-          <t>R-25</t>
+          <t>R-04</t>
         </is>
       </c>
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>網頁的品牌主題系統</t>
+          <t>粵語質量評測</t>
         </is>
       </c>
       <c r="C40" s="13" t="inlineStr">
@@ -1822,7 +1823,7 @@
       </c>
       <c r="E40" s="6" t="inlineStr">
         <is>
-          <t>① 每個品牌一個資料夾：主題 token（顏色、字體、圓角）、logo 和圖示、文案、功能開關；首頁、上手流程、角色頁可以有品牌版本，其餘頁面共用 ② 由部署的環境變數選品牌（每套部署一個品牌，見 R-34），伺服器端渲染的第一屏就是對的主題，不閃爍 ③ 共用元件裡沒有品牌名稱和寫死的品牌顏色 ④ 加一個品牌只需要加資料夾、設定和一套部署，不用改共用元件</t>
+          <t>有一套粵語評測集（兒童錄音＋文字提示）；選定的 STT 與 LLM 達到門檻：兒童語音字錯率 ≤15%、口語粵語回覆 ≥90%、中英夾雜句能正確理解。</t>
         </is>
       </c>
       <c r="F40" s="11" t="n"/>
@@ -1830,68 +1831,68 @@
       <c r="H40" s="11" t="n"/>
       <c r="I40" s="12" t="n"/>
     </row>
-    <row r="42">
-      <c r="A42" s="10" t="inlineStr">
+    <row r="41" ht="116" customHeight="1">
+      <c r="A41" s="13" t="inlineStr">
+        <is>
+          <t>R-25</t>
+        </is>
+      </c>
+      <c r="B41" s="6" t="inlineStr">
+        <is>
+          <t>網頁的品牌主題系統</t>
+        </is>
+      </c>
+      <c r="C41" s="13" t="inlineStr">
+        <is>
+          <t>2 內測準備</t>
+        </is>
+      </c>
+      <c r="D41" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E41" s="6" t="inlineStr">
+        <is>
+          <t>① 每個品牌一個資料夾：主題 token（顏色、字體、圓角）、logo 和圖示、文案、功能開關；首頁、上手流程、角色頁可以有品牌版本，其餘頁面共用 ② 由部署的環境變數選品牌（每套部署一個品牌，見 R-34），伺服器端渲染的第一屏就是對的主題，不閃爍 ③ 共用元件裡沒有品牌名稱和寫死的品牌顏色 ④ 加一個品牌只需要加資料夾、設定和一套部署，不用改共用元件</t>
+        </is>
+      </c>
+      <c r="F41" s="11" t="n"/>
+      <c r="G41" s="11" t="n"/>
+      <c r="H41" s="11" t="n"/>
+      <c r="I41" s="12" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="10" t="inlineStr">
         <is>
           <t>✅ 最近完成與測試效果</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="4" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
         <is>
           <t>編號</t>
         </is>
       </c>
-      <c r="B43" s="4" t="inlineStr">
+      <c r="B44" s="4" t="inlineStr">
         <is>
           <t>任務</t>
         </is>
       </c>
-      <c r="C43" s="4" t="inlineStr">
+      <c r="C44" s="4" t="inlineStr">
         <is>
           <t>測試結果</t>
         </is>
       </c>
-      <c r="D43" s="4" t="inlineStr">
+      <c r="D44" s="4" t="inlineStr">
         <is>
           <t>完成日期</t>
         </is>
       </c>
-      <c r="E43" s="4" t="inlineStr">
+      <c r="E44" s="4" t="inlineStr">
         <is>
           <t>測試證據</t>
-        </is>
-      </c>
-      <c r="F43" s="11" t="n"/>
-      <c r="G43" s="11" t="n"/>
-      <c r="H43" s="11" t="n"/>
-      <c r="I43" s="12" t="n"/>
-    </row>
-    <row r="44" ht="102" customHeight="1">
-      <c r="A44" s="13" t="inlineStr">
-        <is>
-          <t>P0-12</t>
-        </is>
-      </c>
-      <c r="B44" s="6" t="inlineStr">
-        <is>
-          <t>收緊 Admin 權限與路由保護</t>
-        </is>
-      </c>
-      <c r="C44" s="13" t="inlineStr">
-        <is>
-          <t>通過</t>
-        </is>
-      </c>
-      <c r="D44" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-12</t>
-        </is>
-      </c>
-      <c r="E44" s="6" t="inlineStr">
-        <is>
-          <t>線上 2026-10-12（bac24e9）：runbook 10/08 檢查 未登入 /admin→/login、/api/admin→401、has_role() 只看角色、無管理員 policy 觸及 conversations/記憶表、超管≥1；未登入 /home、/admin→/login；用戶確認：家長帳號開 /admin 轉回 /home、管理員在 /admin 修改角色保存成功；角色細分權限沿用本機 61/61</t>
         </is>
       </c>
       <c r="F44" s="11" t="n"/>
@@ -1899,15 +1900,15 @@
       <c r="H44" s="11" t="n"/>
       <c r="I44" s="12" t="n"/>
     </row>
-    <row r="45" ht="88" customHeight="1">
+    <row r="45" ht="116" customHeight="1">
       <c r="A45" s="13" t="inlineStr">
         <is>
-          <t>P0-15</t>
+          <t>R-41</t>
         </is>
       </c>
       <c r="B45" s="6" t="inlineStr">
         <is>
-          <t>角色表權限：只有內容管理員能發佈，關閉家長自建角色</t>
+          <t>App 顯示玩具電量狀態（低電量提示）</t>
         </is>
       </c>
       <c r="C45" s="13" t="inlineStr">
@@ -1917,12 +1918,12 @@
       </c>
       <c r="D45" s="13" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E45" s="6" t="inlineStr">
         <is>
-          <t>線上 2026-10-12：② anon 只見 6 個已發佈 hk_ 內建，查隱藏/醫生/家長自建 → []，anon POST → 401；① authenticated 寫入權限由 20261007140000 REVOKE（runbook 10/08 已套用）；用戶確認：④ 家長登入後 /home/create 轉回 /home ③ 管理員在 /admin 修改角色保存成功</t>
+          <t>① pytest 33 passed；真 PATCH 本地 Supabase ② 62:70 刷 p212+R-41 強制低電 build（SUPPLY_LOW_RATIO_OVERRIDE=1.05）→ 串口 [WSc] power low:true，本地 DB battery_low=t ③ 刷回正常 1.6.2 → low:false，DB=f ④ App 讀 DB：低電紅標+Please charge+更新時間、72% 充電中、未上報不顯示 ⑤ 他人帳號 0 行、authenticated UPDATE 被拒。62:70 已還原為原 p212 build</t>
         </is>
       </c>
       <c r="F45" s="11" t="n"/>
@@ -1930,15 +1931,15 @@
       <c r="H45" s="11" t="n"/>
       <c r="I45" s="12" t="n"/>
     </row>
-    <row r="46" ht="88" customHeight="1">
+    <row r="46" ht="102" customHeight="1">
       <c r="A46" s="13" t="inlineStr">
         <is>
-          <t>P0-16</t>
+          <t>P0-12</t>
         </is>
       </c>
       <c r="B46" s="6" t="inlineStr">
         <is>
-          <t>移除「醫生」身份與寫死的通關碼</t>
+          <t>收緊 Admin 權限與路由保護</t>
         </is>
       </c>
       <c r="C46" s="13" t="inlineStr">
@@ -1953,7 +1954,7 @@
       </c>
       <c r="E46" s="6" t="inlineStr">
         <is>
-          <t>線上 2026-10-12：生產 commit bac24e9 git grep checkDoctorAction/kiwi-subtle-emu/=== "doctor"/isDoctor → 0；線上 13 個 JS（/、/login、/onboard）grep 通關碼/"doctor"/Santa/patient → 0；anon 讀角色只見 6 個 hk_ 角色、is_doctor 全 false；用戶今日線上登入及 playground 正常</t>
+          <t>線上 2026-10-12（bac24e9）：runbook 10/08 檢查 未登入 /admin→/login、/api/admin→401、has_role() 只看角色、無管理員 policy 觸及 conversations/記憶表、超管≥1；未登入 /home、/admin→/login；用戶確認：家長帳號開 /admin 轉回 /home、管理員在 /admin 修改角色保存成功；角色細分權限沿用本機 61/61</t>
         </is>
       </c>
       <c r="F46" s="11" t="n"/>
@@ -1961,15 +1962,15 @@
       <c r="H46" s="11" t="n"/>
       <c r="I46" s="12" t="n"/>
     </row>
-    <row r="47" ht="60" customHeight="1">
+    <row r="47" ht="88" customHeight="1">
       <c r="A47" s="13" t="inlineStr">
         <is>
-          <t>P0-09</t>
+          <t>P0-15</t>
         </is>
       </c>
       <c r="B47" s="6" t="inlineStr">
         <is>
-          <t>瀏覽器語音路由改用簽名 token（/ws/nextjs）</t>
+          <t>角色表權限：只有內容管理員能發佈，關閉家長自建角色</t>
         </is>
       </c>
       <c r="C47" s="13" t="inlineStr">
@@ -1984,7 +1985,7 @@
       </c>
       <c r="E47" s="6" t="inlineStr">
         <is>
-          <t>線上 2026-10-12（bac24e9）：wss /fastapi/ws/nextjs 只帶 user_id 或 token=bogus → 4401；用戶確認：登入 elatoai.hkqft.com 後網頁 playground 可正常對話</t>
+          <t>線上 2026-10-12：② anon 只見 6 個已發佈 hk_ 內建，查隱藏/醫生/家長自建 → []，anon POST → 401；① authenticated 寫入權限由 20261007140000 REVOKE（runbook 10/08 已套用）；用戶確認：④ 家長登入後 /home/create 轉回 /home ③ 管理員在 /admin 修改角色保存成功</t>
         </is>
       </c>
       <c r="F47" s="11" t="n"/>
@@ -1992,15 +1993,15 @@
       <c r="H47" s="11" t="n"/>
       <c r="I47" s="12" t="n"/>
     </row>
-    <row r="48" ht="60" customHeight="1">
+    <row r="48" ht="88" customHeight="1">
       <c r="A48" s="13" t="inlineStr">
         <is>
-          <t>P0-17</t>
+          <t>P0-16</t>
         </is>
       </c>
       <c r="B48" s="6" t="inlineStr">
         <is>
-          <t>前端的 anon key 必須是公開 key，不可是 secret／service_role</t>
+          <t>移除「醫生」身份與寫死的通關碼</t>
         </is>
       </c>
       <c r="C48" s="13" t="inlineStr">
@@ -2015,7 +2016,7 @@
       </c>
       <c r="E48" s="6" t="inlineStr">
         <is>
-          <t>線上 2026-10-12（bac24e9）：/login 引用的 13 個 JS + HTML 無 sb_secret_，唯一 key 為 role=anon 的 JWT；② 用該 key GET /rest/v1/users → 42501；③ 本機 10/07 已換 publishable</t>
+          <t>線上 2026-10-12：生產 commit bac24e9 git grep checkDoctorAction/kiwi-subtle-emu/=== "doctor"/isDoctor → 0；線上 13 個 JS（/、/login、/onboard）grep 通關碼/"doctor"/Santa/patient → 0；anon 讀角色只見 6 個 hk_ 角色、is_doctor 全 false；用戶今日線上登入及 playground 正常</t>
         </is>
       </c>
       <c r="F48" s="11" t="n"/>
@@ -2023,15 +2024,15 @@
       <c r="H48" s="11" t="n"/>
       <c r="I48" s="12" t="n"/>
     </row>
-    <row r="49" ht="46" customHeight="1">
+    <row r="49" ht="60" customHeight="1">
       <c r="A49" s="13" t="inlineStr">
         <is>
-          <t>P0-10</t>
+          <t>P0-09</t>
         </is>
       </c>
       <c r="B49" s="6" t="inlineStr">
         <is>
-          <t>生產環境關閉 /browser 測試頁與 /ws/browser</t>
+          <t>瀏覽器語音路由改用簽名 token（/ws/nextjs）</t>
         </is>
       </c>
       <c r="C49" s="13" t="inlineStr">
@@ -2046,7 +2047,7 @@
       </c>
       <c r="E49" s="6" t="inlineStr">
         <is>
-          <t>線上 2026-10-12（bac24e9）：GET /fastapi/browser 404、/fastapi/ 404、/fastapi/healthz 200、wss /fastapi/ws/browser → HTTP 403</t>
+          <t>線上 2026-10-12（bac24e9）：wss /fastapi/ws/nextjs 只帶 user_id 或 token=bogus → 4401；用戶確認：登入 elatoai.hkqft.com 後網頁 playground 可正常對話</t>
         </is>
       </c>
       <c r="F49" s="11" t="n"/>
@@ -2057,12 +2058,12 @@
     <row r="50" ht="60" customHeight="1">
       <c r="A50" s="13" t="inlineStr">
         <is>
-          <t>P0-08</t>
+          <t>P0-17</t>
         </is>
       </c>
       <c r="B50" s="6" t="inlineStr">
         <is>
-          <t>語音伺服器驗證設備身份（/ws/esp32）</t>
+          <t>前端的 anon key 必須是公開 key，不可是 secret／service_role</t>
         </is>
       </c>
       <c r="C50" s="13" t="inlineStr">
@@ -2077,7 +2078,7 @@
       </c>
       <c r="E50" s="6" t="inlineStr">
         <is>
-          <t>線上 2026-10-12（bac24e9）：wss /fastapi/ws/esp32 不帶 token、偽造 token＋X-Device-Mac → 均 4401 invalid device token；42:34 以有效 token 連線對話正常（P0-13 10/09）</t>
+          <t>線上 2026-10-12（bac24e9）：/login 引用的 13 個 JS + HTML 無 sb_secret_，唯一 key 為 role=anon 的 JWT；② 用該 key GET /rest/v1/users → 42501；③ 本機 10/07 已換 publishable</t>
         </is>
       </c>
       <c r="F50" s="11" t="n"/>
@@ -2085,15 +2086,15 @@
       <c r="H50" s="11" t="n"/>
       <c r="I50" s="12" t="n"/>
     </row>
-    <row r="51" ht="60" customHeight="1">
+    <row r="51" ht="46" customHeight="1">
       <c r="A51" s="13" t="inlineStr">
         <is>
-          <t>P0-06</t>
+          <t>P0-10</t>
         </is>
       </c>
       <c r="B51" s="6" t="inlineStr">
         <is>
-          <t>停止憑 MAC 發放永久用戶 JWT</t>
+          <t>生產環境關閉 /browser 測試頁與 /ws/browser</t>
         </is>
       </c>
       <c r="C51" s="13" t="inlineStr">
@@ -2108,7 +2109,7 @@
       </c>
       <c r="E51" s="6" t="inlineStr">
         <is>
-          <t>線上 2026-10-12（bac24e9）：POST /api/generate_auth_token 只帶 42:34 的 MAC → 401、帶錯誤密鑰 → 401、GET → 410；42:34 用 NVS 密鑰在線上換 token 並連上語音伺服器（P0-13 10/09 實測）</t>
+          <t>線上 2026-10-12（bac24e9）：GET /fastapi/browser 404、/fastapi/ 404、/fastapi/healthz 200、wss /fastapi/ws/browser → HTTP 403</t>
         </is>
       </c>
       <c r="F51" s="11" t="n"/>
@@ -2116,50 +2117,58 @@
       <c r="H51" s="11" t="n"/>
       <c r="I51" s="12" t="n"/>
     </row>
-    <row r="53">
-      <c r="A53" s="10" t="inlineStr">
+    <row r="52" ht="60" customHeight="1">
+      <c r="A52" s="13" t="inlineStr">
+        <is>
+          <t>P0-08</t>
+        </is>
+      </c>
+      <c r="B52" s="6" t="inlineStr">
+        <is>
+          <t>語音伺服器驗證設備身份（/ws/esp32）</t>
+        </is>
+      </c>
+      <c r="C52" s="13" t="inlineStr">
+        <is>
+          <t>通過</t>
+        </is>
+      </c>
+      <c r="D52" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="E52" s="6" t="inlineStr">
+        <is>
+          <t>線上 2026-10-12（bac24e9）：wss /fastapi/ws/esp32 不帶 token、偽造 token＋X-Device-Mac → 均 4401 invalid device token；42:34 以有效 token 連線對話正常（P0-13 10/09）</t>
+        </is>
+      </c>
+      <c r="F52" s="11" t="n"/>
+      <c r="G52" s="11" t="n"/>
+      <c r="H52" s="11" t="n"/>
+      <c r="I52" s="12" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="10" t="inlineStr">
         <is>
           <t>⏳ 等待依賴 / ⛔ 阻塞</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="4" t="inlineStr">
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
         <is>
           <t>編號</t>
         </is>
       </c>
-      <c r="B54" s="4" t="inlineStr">
+      <c r="B55" s="4" t="inlineStr">
         <is>
           <t>任務</t>
         </is>
       </c>
-      <c r="C54" s="4" t="inlineStr">
+      <c r="C55" s="4" t="inlineStr">
         <is>
           <t>在等什麼</t>
-        </is>
-      </c>
-      <c r="D54" s="11" t="n"/>
-      <c r="E54" s="11" t="n"/>
-      <c r="F54" s="11" t="n"/>
-      <c r="G54" s="11" t="n"/>
-      <c r="H54" s="11" t="n"/>
-      <c r="I54" s="12" t="n"/>
-    </row>
-    <row r="55" ht="60" customHeight="1">
-      <c r="A55" s="13" t="inlineStr">
-        <is>
-          <t>R-16</t>
-        </is>
-      </c>
-      <c r="B55" s="6" t="inlineStr">
-        <is>
-          <t>Spotpear 量產版加電池電壓檢測（GPIO0 分壓）</t>
-        </is>
-      </c>
-      <c r="C55" s="6" t="inlineStr">
-        <is>
-          <t>阻塞：[2026-10-07] 仍按 10/06 決定暫緩：等用戶做充滿再放電測試（與 R-17 同一次），看 VDD 低電提醒在關機前多久觸發；太遲或不觸發才向 Spotpear 提改板。已把分壓改板的問題一併放進給 Spotpear 的草稿，方便同一封發出</t>
         </is>
       </c>
       <c r="D55" s="11" t="n"/>
@@ -2192,20 +2201,20 @@
       <c r="H56" s="11" t="n"/>
       <c r="I56" s="12" t="n"/>
     </row>
-    <row r="57" ht="32" customHeight="1">
+    <row r="57" ht="60" customHeight="1">
       <c r="A57" s="13" t="inlineStr">
         <is>
-          <t>P1-09</t>
+          <t>P1-01</t>
         </is>
       </c>
       <c r="B57" s="6" t="inlineStr">
         <is>
-          <t>家長鎖：孩子模式進設定要輸入 PIN</t>
+          <t>加入內容審核層（輸入與輸出）</t>
         </is>
       </c>
       <c r="C57" s="6" t="inlineStr">
         <is>
-          <t>阻塞：[2026-10-13] 2026-10-13 用戶決定：AI Buddy（品牌 C）延到 1/15 之後，本項不卡 1/15 出廠；AI Buddy 啟動時再開。</t>
+          <t>阻塞：[2026-10-14] 2026-10-14 用戶決定：先不定審核服務商，本項暫停。候選：Azure Content Safety（建議，香港區、可在每句回覆說出口前檢查）、OpenRouter 安全模型、OpenAI Moderation、只用本機字詞表。未寫任何程式。</t>
         </is>
       </c>
       <c r="D57" s="11" t="n"/>
@@ -2218,12 +2227,12 @@
     <row r="58" ht="32" customHeight="1">
       <c r="A58" s="13" t="inlineStr">
         <is>
-          <t>R-12</t>
+          <t>P1-09</t>
         </is>
       </c>
       <c r="B58" s="6" t="inlineStr">
         <is>
-          <t>家長控制：每日使用上限和休息時段</t>
+          <t>家長鎖：孩子模式進設定要輸入 PIN</t>
         </is>
       </c>
       <c r="C58" s="6" t="inlineStr">
@@ -2241,12 +2250,12 @@
     <row r="59" ht="32" customHeight="1">
       <c r="A59" s="13" t="inlineStr">
         <is>
-          <t>R-29</t>
+          <t>R-12</t>
         </is>
       </c>
       <c r="B59" s="6" t="inlineStr">
         <is>
-          <t>AI Buddy App（品牌 C）頁面</t>
+          <t>家長控制：每日使用上限和休息時段</t>
         </is>
       </c>
       <c r="C59" s="6" t="inlineStr">
@@ -2264,17 +2273,17 @@
     <row r="60" ht="32" customHeight="1">
       <c r="A60" s="13" t="inlineStr">
         <is>
-          <t>P2-14</t>
+          <t>R-29</t>
         </is>
       </c>
       <c r="B60" s="6" t="inlineStr">
         <is>
-          <t>Admin 設備頁：每台玩具的狀態、韌體與基本操作</t>
+          <t>AI Buddy App（品牌 C）頁面</t>
         </is>
       </c>
       <c r="C60" s="6" t="inlineStr">
         <is>
-          <t>等 P1-10、P2-13</t>
+          <t>阻塞：[2026-10-13] 2026-10-13 用戶決定：AI Buddy（品牌 C）延到 1/15 之後，本項不卡 1/15 出廠；AI Buddy 啟動時再開。</t>
         </is>
       </c>
       <c r="D60" s="11" t="n"/>
@@ -3142,6 +3151,7 @@
   <mergeCells count="85">
     <mergeCell ref="A99:I99"/>
     <mergeCell ref="C82:I82"/>
+    <mergeCell ref="E52:I52"/>
     <mergeCell ref="E39:I39"/>
     <mergeCell ref="C67:I67"/>
     <mergeCell ref="E48:I48"/>
@@ -3149,9 +3159,7 @@
     <mergeCell ref="A2:I2"/>
     <mergeCell ref="E29:I29"/>
     <mergeCell ref="E38:I38"/>
-    <mergeCell ref="A42:I42"/>
     <mergeCell ref="C83:I83"/>
-    <mergeCell ref="A53:I53"/>
     <mergeCell ref="E31:I31"/>
     <mergeCell ref="E40:I40"/>
     <mergeCell ref="C97:I97"/>
@@ -3186,15 +3194,16 @@
     <mergeCell ref="E32:I32"/>
     <mergeCell ref="C59:I59"/>
     <mergeCell ref="A1:I1"/>
+    <mergeCell ref="E41:I41"/>
     <mergeCell ref="E47:I47"/>
     <mergeCell ref="C61:I61"/>
-    <mergeCell ref="E43:I43"/>
     <mergeCell ref="C70:I70"/>
     <mergeCell ref="E24:I24"/>
     <mergeCell ref="E33:I33"/>
     <mergeCell ref="A3:I3"/>
     <mergeCell ref="A104:I104"/>
     <mergeCell ref="E35:I35"/>
+    <mergeCell ref="A43:I43"/>
     <mergeCell ref="C74:I74"/>
     <mergeCell ref="C88:I88"/>
     <mergeCell ref="E45:I45"/>
@@ -3217,7 +3226,6 @@
     <mergeCell ref="C73:I73"/>
     <mergeCell ref="E49:I49"/>
     <mergeCell ref="E27:I27"/>
-    <mergeCell ref="C54:I54"/>
     <mergeCell ref="E36:I36"/>
     <mergeCell ref="C63:I63"/>
     <mergeCell ref="C93:I93"/>
@@ -3225,6 +3233,7 @@
     <mergeCell ref="C90:I90"/>
     <mergeCell ref="E22:I22"/>
     <mergeCell ref="C76:I76"/>
+    <mergeCell ref="A54:I54"/>
   </mergeCells>
   <conditionalFormatting sqref="I6:I10">
     <cfRule type="dataBar" priority="1">
@@ -3254,7 +3263,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P88"/>
+  <dimension ref="A1:P89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -4471,7 +4480,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="74" customHeight="1">
+    <row r="16" ht="172" customHeight="1">
       <c r="A16" s="13" t="inlineStr">
         <is>
           <t>P1-01</t>
@@ -4499,7 +4508,7 @@
       </c>
       <c r="F16" s="13" t="inlineStr">
         <is>
-          <t>未開始</t>
+          <t>阻塞</t>
         </is>
       </c>
       <c r="G16" s="13" t="inlineStr">
@@ -4539,7 +4548,8 @@
       <c r="P16" s="6" t="inlineStr">
         <is>
           <t>[2026-09-30] Q5：3–6 歲；Q7：事件不記原文
-[2026-10-14] 2026-10-14：審核事件的後台頁拆成 P1-14，等本項完成後做。</t>
+[2026-10-14] 2026-10-14：審核事件的後台頁拆成 P1-14，等本項完成後做。
+[2026-10-14] 2026-10-14 用戶決定：先不定審核服務商，本項暫停。候選：Azure Content Safety（建議，香港區、可在每句回覆說出口前檢查）、OpenRouter 安全模型、OpenAI Moderation、只用本機字詞表。未寫任何程式。</t>
         </is>
       </c>
     </row>
@@ -7157,7 +7167,7 @@
         </is>
       </c>
     </row>
-    <row r="53" ht="270" customHeight="1">
+    <row r="53" ht="409" customHeight="1">
       <c r="A53" s="13" t="inlineStr">
         <is>
           <t>R-16</t>
@@ -7185,7 +7195,7 @@
       </c>
       <c r="F53" s="13" t="inlineStr">
         <is>
-          <t>阻塞</t>
+          <t>未開始</t>
         </is>
       </c>
       <c r="G53" s="13" t="inlineStr">
@@ -7205,7 +7215,7 @@
       </c>
       <c r="K53" s="6" t="inlineStr">
         <is>
-          <t>Spotpear 書面確認量產版：GPIO0（或 GPIO1）接電芯正極（保護 IC 之後）100k/100k 分壓、100nF 濾波，屏幕不接該腳；最好另把充電芯片 CHRG 接到 GPIO12 或 13。樣板到手後，固件讀到的電芯電壓與萬用表相差 ≤50mV。</t>
+          <t>Spotpear 書面確認量產版：GPIO1（屏幕 DC；本版不接屏幕，可空出來）接電芯正極（保護 IC 之後）100k/100k 分壓、100nF 濾波，屏幕不接該腳；GPIO0 保留給現有的 VDD 低電提醒；最好另把充電芯片 CHRG 接到 GPIO12 或 13。樣板到手後，固件讀到的電芯電壓與萬用表相差 ≤50mV，App（R-41）顯示百分比與充電中。</t>
         </is>
       </c>
       <c r="L53" s="6" t="inlineStr">
@@ -7218,7 +7228,8 @@
         <is>
           <t>[2026-10-05] 新增
 [2026-10-06] 2026-10-06：用戶表示不需要精確電量，快沒電時提醒即可，也無法自行焊接。改為軟件方案：讀芯片自身供電（GPIO0 內部上下拉分壓，SupplyMonitor.cpp），讀數跌破基準 95.5% 就亮紅燈並播廣東話提醒。已用強制低電量測試版驗證：提醒能播出、紅燈正常。本任務（硬件分壓）暫緩，等充滿再放電的實測：若提醒太遲或不觸發才向 Spotpear 提出。
-[2026-10-07] 仍按 10/06 決定暫緩：等用戶做充滿再放電測試（與 R-17 同一次），看 VDD 低電提醒在關機前多久觸發；太遲或不觸發才向 Spotpear 提改板。已把分壓改板的問題一併放進給 Spotpear 的草稿，方便同一封發出</t>
+[2026-10-07] 仍按 10/06 決定暫緩：等用戶做充滿再放電測試（與 R-17 同一次），看 VDD 低電提醒在關機前多久觸發；太遲或不觸發才向 Spotpear 提改板。已把分壓改板的問題一併放進給 Spotpear 的草稿，方便同一封發出
+[2026-10-14] 2026-10-14：用戶決定 App 要顯示電量，恢復本任務（方案 B），與 R-41（方案 A：先顯示高低兩態）並行。改用 GPIO1：GPIO0 已被 SupplyMonitor 的 VDD 檢測佔用（標題仍寫 GPIO0，以驗收標準為準）。R-41 的上報協議已預留 percent / charging，改板後只需改固件的 Battery 設定。量產板訂單是關鍵路徑，要盡快向 Spotpear 提出。</t>
         </is>
       </c>
     </row>
@@ -9220,7 +9231,7 @@
         </is>
       </c>
     </row>
-    <row r="83" ht="102" customHeight="1">
+    <row r="83" ht="214" customHeight="1">
       <c r="A83" s="13" t="inlineStr">
         <is>
           <t>P2-14</t>
@@ -9248,12 +9259,12 @@
       </c>
       <c r="F83" s="13" t="inlineStr">
         <is>
-          <t>未開始</t>
+          <t>進行中</t>
         </is>
       </c>
       <c r="G83" s="13" t="inlineStr">
         <is>
-          <t>未測試</t>
+          <t>部分通過</t>
         </is>
       </c>
       <c r="I83" s="6" t="inlineStr">
@@ -9283,9 +9294,15 @@
           <t>P1-10, P2-13</t>
         </is>
       </c>
+      <c r="N83" s="6" t="inlineStr">
+        <is>
+          <t>本機（未 commit）：migration 20261014140000 套用兩次無錯。探測腳本用 GoTrue 真實登入：超管 admin_list_devices 200（不含 user_code）；④ 內容管理員 → 42501、anon → 42501；超管直接讀 device_secrets → 42501；空原因 → 22023；重置密鑰 → device_secrets 行刪除；解綁 → user_id/claimed_at 清空；兩者各寫 1 筆含原因與前後值的審計，超管改審計 → 403。網頁（獨立副本+獨立語音伺服器 7871）：模擬 62:70 連上 → 15 秒內不刷新顯示 Online、-52 dBm；斷線後下一次輪詢變 Offline；按 f214 搜尋、強制解綁、重置密鑰、審計頁都看到兩筆；375px 無橫向捲動。pytest 71 passed。未做：① ② ③ 需真板 62:70，且要用新代碼重啟 7860 語音伺服器</t>
+        </is>
+      </c>
       <c r="P83" s="6" t="inlineStr">
         <is>
-          <t>[2026-10-14] 新增</t>
+          <t>[2026-10-14] 新增
+[2026-10-14] devices.ip_key 未有（R-38），IP 欄暫顯示「未鎖定」。部署要三件一起：migration、語音伺服器（/internal/devices_presence）、網頁。在線只代表有語音連線，睡眠和關機都算離線。</t>
         </is>
       </c>
     </row>
@@ -9631,8 +9648,87 @@
         </is>
       </c>
     </row>
+    <row r="89" ht="116" customHeight="1">
+      <c r="A89" s="13" t="inlineStr">
+        <is>
+          <t>R-41</t>
+        </is>
+      </c>
+      <c r="B89" s="13" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="C89" s="13" t="inlineStr">
+        <is>
+          <t>2 內測準備</t>
+        </is>
+      </c>
+      <c r="D89" s="6" t="inlineStr">
+        <is>
+          <t>產品</t>
+        </is>
+      </c>
+      <c r="E89" s="6" t="inlineStr">
+        <is>
+          <t>App 顯示玩具電量狀態（低電量提示）</t>
+        </is>
+      </c>
+      <c r="F89" s="13" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G89" s="13" t="inlineStr">
+        <is>
+          <t>通過</t>
+        </is>
+      </c>
+      <c r="H89" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="I89" s="6" t="inlineStr">
+        <is>
+          <t>家長在 App 看不到玩具快沒電，只能靠玩具自己播提醒；玩具多數時間休眠，伺服器記憶體裡的狀態一重啟就沒了。</t>
+        </is>
+      </c>
+      <c r="J89" s="6" t="inlineStr">
+        <is>
+          <t>firmware-arduino/src/Audio.cpp（reportPower）；server/fastapi/device_power.py；supabase/migrations（devices.battery_*）；frontend-nextjs 設備頁</t>
+        </is>
+      </c>
+      <c r="K89" s="6" t="inlineStr">
+        <is>
+          <t>玩具每次連上語音伺服器並收到 auth 後上報一次電量狀態，狀態改變時再報；伺服器寫入 devices.battery_low / battery_percent / battery_charging / battery_at；App 設備頁顯示「電量正常／電量低，請充電」和最後更新時間，玩具離線時仍顯示最後已知狀態；沒有電量檢測的板不顯示電量。Spotpear 板只有高低兩態（R-16 改板後才有百分比）。</t>
+        </is>
+      </c>
+      <c r="L89" s="6" t="inlineStr">
+        <is>
+          <t>① 單元測試：伺服器只接受 power 訊息的合法欄位並寫入對應 MAC 的 devices 行 ② 62:70 用 SUPPLY_LOW_RATIO_OVERRIDE 強制低電量：本地 DB battery_low=true、App 顯示電量低 ③ 改回正常固件重連：battery_low=false、App 顯示正常 ④ 玩具斷線後 App 仍顯示最後狀態和時間 ⑤ 其他用戶讀不到這幾欄（RLS）</t>
+        </is>
+      </c>
+      <c r="M89" s="13" t="n"/>
+      <c r="N89" s="6" t="inlineStr">
+        <is>
+          <t>① pytest 33 passed；真 PATCH 本地 Supabase ② 62:70 刷 p212+R-41 強制低電 build（SUPPLY_LOW_RATIO_OVERRIDE=1.05）→ 串口 [WSc] power low:true，本地 DB battery_low=t ③ 刷回正常 1.6.2 → low:false，DB=f ④ App 讀 DB：低電紅標+Please charge+更新時間、72% 充電中、未上報不顯示 ⑤ 他人帳號 0 行、authenticated UPDATE 被拒。62:70 已還原為原 p212 build</t>
+        </is>
+      </c>
+      <c r="O89" s="13" t="inlineStr">
+        <is>
+          <t>42b4437</t>
+        </is>
+      </c>
+      <c r="P89" s="6" t="inlineStr">
+        <is>
+          <t>[2026-10-14] 新增
+[2026-10-14] 2026-10-14：rebase 後合併入 dev（42b4437）。migration 改名 20261014153000_device_battery.sql，避開同時間戳的 admin_accounts；powerSent 重置改到收到 auth 時。未部署。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P88"/>
+  <autoFilter ref="A1:P89"/>
   <conditionalFormatting sqref="F2:F1000">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"已完成"</formula>
@@ -10213,7 +10309,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I260"/>
+  <dimension ref="A1:I270"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -19207,8 +19303,366 @@
       </c>
       <c r="I260" s="6" t="n"/>
     </row>
+    <row r="261" ht="32" customHeight="1">
+      <c r="A261" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 11:38</t>
+        </is>
+      </c>
+      <c r="B261" s="13" t="inlineStr">
+        <is>
+          <t>P1-01</t>
+        </is>
+      </c>
+      <c r="C261" s="6" t="inlineStr">
+        <is>
+          <t>加入內容審核層（輸入與輸出）</t>
+        </is>
+      </c>
+      <c r="D261" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E261" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F261" s="13" t="n"/>
+      <c r="G261" s="6" t="n"/>
+      <c r="H261" s="13" t="n"/>
+      <c r="I261" s="6" t="n"/>
+    </row>
+    <row r="262" ht="88" customHeight="1">
+      <c r="A262" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 11:47</t>
+        </is>
+      </c>
+      <c r="B262" s="13" t="inlineStr">
+        <is>
+          <t>P1-01</t>
+        </is>
+      </c>
+      <c r="C262" s="6" t="inlineStr">
+        <is>
+          <t>加入內容審核層（輸入與輸出）</t>
+        </is>
+      </c>
+      <c r="D262" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="E262" s="13" t="inlineStr">
+        <is>
+          <t>阻塞</t>
+        </is>
+      </c>
+      <c r="F262" s="13" t="n"/>
+      <c r="G262" s="6" t="n"/>
+      <c r="H262" s="13" t="n"/>
+      <c r="I262" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-14 用戶決定：先不定審核服務商，本項暫停。候選：Azure Content Safety（建議，香港區、可在每句回覆說出口前檢查）、OpenRouter 安全模型、OpenAI Moderation、只用本機字詞表。未寫任何程式。</t>
+        </is>
+      </c>
+    </row>
+    <row r="263" ht="32" customHeight="1">
+      <c r="A263" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 11:50</t>
+        </is>
+      </c>
+      <c r="B263" s="13" t="inlineStr">
+        <is>
+          <t>P2-14</t>
+        </is>
+      </c>
+      <c r="C263" s="6" t="inlineStr">
+        <is>
+          <t>Admin 設備頁：每台玩具的狀態、韌體與基本操作</t>
+        </is>
+      </c>
+      <c r="D263" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E263" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F263" s="13" t="n"/>
+      <c r="G263" s="6" t="n"/>
+      <c r="H263" s="13" t="n"/>
+      <c r="I263" s="6" t="n"/>
+    </row>
+    <row r="264" ht="186" customHeight="1">
+      <c r="A264" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 12:03</t>
+        </is>
+      </c>
+      <c r="B264" s="13" t="inlineStr">
+        <is>
+          <t>P2-14</t>
+        </is>
+      </c>
+      <c r="C264" s="6" t="inlineStr">
+        <is>
+          <t>Admin 設備頁：每台玩具的狀態、韌體與基本操作</t>
+        </is>
+      </c>
+      <c r="D264" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="E264" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F264" s="13" t="inlineStr">
+        <is>
+          <t>部分通過</t>
+        </is>
+      </c>
+      <c r="G264" s="6" t="inlineStr">
+        <is>
+          <t>本機（未 commit）：migration 20261014140000 套用兩次無錯。探測腳本用 GoTrue 真實登入：超管 admin_list_devices 200（不含 user_code）；④ 內容管理員 → 42501、anon → 42501；超管直接讀 device_secrets → 42501；空原因 → 22023；重置密鑰 → device_secrets 行刪除；解綁 → user_id/claimed_at 清空；兩者各寫 1 筆含原因與前後值的審計，超管改審計 → 403。網頁（獨立副本+獨立語音伺服器 7871）：模擬 62:70 連上 → 15 秒內不刷新顯示 Online、-52 dBm；斷線後下一次輪詢變 Offline；按 f214 搜尋、強制解綁、重置密鑰、審計頁都看到兩筆；375px 無橫向捲動。pytest 71 passed。未做：① ② ③ 需真板 62:70，且要用新代碼重啟 7860 語音伺服器</t>
+        </is>
+      </c>
+      <c r="H264" s="13" t="n"/>
+      <c r="I264" s="6" t="inlineStr">
+        <is>
+          <t>devices.ip_key 未有（R-38），IP 欄暫顯示「未鎖定」。部署要三件一起：migration、語音伺服器（/internal/devices_presence）、網頁。在線只代表有語音連線，睡眠和關機都算離線。</t>
+        </is>
+      </c>
+    </row>
+    <row r="265" ht="32" customHeight="1">
+      <c r="A265" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 12:10</t>
+        </is>
+      </c>
+      <c r="B265" s="13" t="inlineStr">
+        <is>
+          <t>R-41</t>
+        </is>
+      </c>
+      <c r="C265" s="6" t="inlineStr">
+        <is>
+          <t>App 顯示玩具電量狀態（低電量提示）</t>
+        </is>
+      </c>
+      <c r="E265" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="I265" s="6" t="inlineStr">
+        <is>
+          <t>新增任務</t>
+        </is>
+      </c>
+    </row>
+    <row r="266" ht="32" customHeight="1">
+      <c r="A266" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 12:10</t>
+        </is>
+      </c>
+      <c r="B266" s="13" t="inlineStr">
+        <is>
+          <t>R-41</t>
+        </is>
+      </c>
+      <c r="C266" s="6" t="inlineStr">
+        <is>
+          <t>App 顯示玩具電量狀態（低電量提示）</t>
+        </is>
+      </c>
+      <c r="D266" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E266" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F266" s="13" t="n"/>
+      <c r="G266" s="6" t="n"/>
+      <c r="H266" s="13" t="n"/>
+      <c r="I266" s="6" t="n"/>
+    </row>
+    <row r="267" ht="144" customHeight="1">
+      <c r="A267" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 12:10</t>
+        </is>
+      </c>
+      <c r="B267" s="13" t="inlineStr">
+        <is>
+          <t>R-16</t>
+        </is>
+      </c>
+      <c r="C267" s="6" t="inlineStr">
+        <is>
+          <t>Spotpear 量產版加電池電壓檢測（GPIO0 分壓）</t>
+        </is>
+      </c>
+      <c r="D267" s="13" t="inlineStr">
+        <is>
+          <t>阻塞</t>
+        </is>
+      </c>
+      <c r="E267" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="F267" s="13" t="n"/>
+      <c r="G267" s="6" t="n"/>
+      <c r="H267" s="13" t="n"/>
+      <c r="I267" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-14：用戶決定 App 要顯示電量，恢復本任務（方案 B），與 R-41（方案 A：先顯示高低兩態）並行。改用 GPIO1：GPIO0 已被 SupplyMonitor 的 VDD 檢測佔用（標題仍寫 GPIO0，以驗收標準為準）。R-41 的上報協議已預留 percent / charging，改板後只需改固件的 Battery 設定。量產板訂單是關鍵路徑，要盡快向 Spotpear 提出。；修改了驗收標準</t>
+        </is>
+      </c>
+    </row>
+    <row r="268" ht="116" customHeight="1">
+      <c r="A268" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 15:24</t>
+        </is>
+      </c>
+      <c r="B268" s="13" t="inlineStr">
+        <is>
+          <t>R-41</t>
+        </is>
+      </c>
+      <c r="C268" s="6" t="inlineStr">
+        <is>
+          <t>App 顯示玩具電量狀態（低電量提示）</t>
+        </is>
+      </c>
+      <c r="D268" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="E268" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F268" s="13" t="inlineStr">
+        <is>
+          <t>部分通過</t>
+        </is>
+      </c>
+      <c r="G268" s="6" t="inlineStr">
+        <is>
+          <t>① pytest test_device_power+test_device_wifi 33 passed；device_power.write() 真 PATCH 本地 Supabase → 62:70 行 battery_low=t ④ App（手機尺寸）低電：列表紅色 Low battery、設定頁 Low · Please charge + 更新時間；72% 充電中顯示 Charging · 72%；全空不顯示 Battery 行 ⑤ 他人帳號讀 0 行、authenticated UPDATE 被拒。固件 spotpear/xmini-c3/S3 編譯通過。未做：②③ 62:70 真機（強制低電 build）</t>
+        </is>
+      </c>
+      <c r="H268" s="13" t="inlineStr">
+        <is>
+          <t>db30823</t>
+        </is>
+      </c>
+      <c r="I268" s="6" t="n"/>
+    </row>
+    <row r="269" ht="116" customHeight="1">
+      <c r="A269" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 15:40</t>
+        </is>
+      </c>
+      <c r="B269" s="13" t="inlineStr">
+        <is>
+          <t>R-41</t>
+        </is>
+      </c>
+      <c r="C269" s="6" t="inlineStr">
+        <is>
+          <t>App 顯示玩具電量狀態（低電量提示）</t>
+        </is>
+      </c>
+      <c r="D269" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="E269" s="13" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="F269" s="13" t="inlineStr">
+        <is>
+          <t>通過</t>
+        </is>
+      </c>
+      <c r="G269" s="6" t="inlineStr">
+        <is>
+          <t>① pytest 33 passed；真 PATCH 本地 Supabase ② 62:70 刷 p212+R-41 強制低電 build（SUPPLY_LOW_RATIO_OVERRIDE=1.05）→ 串口 [WSc] power low:true，本地 DB battery_low=t ③ 刷回正常 1.6.2 → low:false，DB=f ④ App 讀 DB：低電紅標+Please charge+更新時間、72% 充電中、未上報不顯示 ⑤ 他人帳號 0 行、authenticated UPDATE 被拒。62:70 已還原為原 p212 build</t>
+        </is>
+      </c>
+      <c r="H269" s="13" t="inlineStr">
+        <is>
+          <t>db30823</t>
+        </is>
+      </c>
+      <c r="I269" s="6" t="n"/>
+    </row>
+    <row r="270" ht="74" customHeight="1">
+      <c r="A270" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 15:50</t>
+        </is>
+      </c>
+      <c r="B270" s="13" t="inlineStr">
+        <is>
+          <t>R-41</t>
+        </is>
+      </c>
+      <c r="C270" s="6" t="inlineStr">
+        <is>
+          <t>App 顯示玩具電量狀態（低電量提示）</t>
+        </is>
+      </c>
+      <c r="D270" s="13" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="E270" s="13" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="F270" s="13" t="n"/>
+      <c r="G270" s="6" t="n"/>
+      <c r="H270" s="13" t="inlineStr">
+        <is>
+          <t>42b4437</t>
+        </is>
+      </c>
+      <c r="I270" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-14：rebase 後合併入 dev（42b4437）。migration 改名 20261014153000_device_battery.sql，避開同時間戳的 admin_accounts；powerSent 重置改到收到 auth 時。未部署。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I260"/>
+  <autoFilter ref="A1:I270"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Split P2-16 (OTA staged rollout and admin release page) into five tracked sub-tasks.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/production-readiness.xlsx
+++ b/docs/production-readiness.xlsx
@@ -13,9 +13,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="更新記錄" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'任務清單'!$A$1:$P$89</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'任務清單'!$A$1:$P$94</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'待確認問題'!$A$1:$G$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$270</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$277</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -641,7 +641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I104"/>
+  <dimension ref="A1:I108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -665,14 +665,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>最後更新：2026-10-14 15:50　·　本頁由 tracker.py 自動生成，請勿手動編輯</t>
+          <t>最後更新：2026-10-14 20:27　·　本頁由 tracker.py 自動生成，請勿手動編輯</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>總進度：18/84 已完成（21%）　·　目前階段：1 止血定案（10/5–10/16）</t>
+          <t>總進度：18/89 已完成（20%）　·　目前階段：1 止血定案（10/5–10/16）</t>
         </is>
       </c>
     </row>
@@ -816,15 +816,15 @@
       </c>
       <c r="C8" s="7">
         <f>COUNTIF('任務清單'!$B:$B,$A8)</f>
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="D8" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A8,'任務清單'!$F:$F,D$5)</f>
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E8" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A8,'任務清單'!$F:$F,E$5)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F8" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A8,'任務清單'!$F:$F,F$5)</f>
@@ -840,7 +840,7 @@
       </c>
       <c r="I8" s="8">
         <f>IFERROR(F8/(C8-H8),0)</f>
-        <v>0.1875</v>
+        <v>0.14285714285714285</v>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1">
@@ -892,15 +892,15 @@
       <c r="B10" s="6" t="n"/>
       <c r="C10" s="5">
         <f>SUM(C6:C9)</f>
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="D10" s="5">
         <f>SUM(D6:D9)</f>
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="E10" s="5">
         <f>SUM(E6:E9)</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F10" s="5">
         <f>SUM(F6:F9)</f>
@@ -916,7 +916,7 @@
       </c>
       <c r="I10" s="9">
         <f>IFERROR(F10/(C10-H10),0)</f>
-        <v>0.21428571428571427</v>
+        <v>0.20224719101123595</v>
       </c>
     </row>
     <row r="12">
@@ -1099,15 +1099,15 @@
       </c>
       <c r="C16" s="7">
         <f>COUNTIF('任務清單'!$C:$C,$A16)</f>
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="D16" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A16,'任務清單'!$F:$F,D$12)</f>
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="E16" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A16,'任務清單'!$F:$F,E$12)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F16" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A16,'任務清單'!$F:$F,F$12)</f>
@@ -1135,15 +1135,15 @@
       <c r="B17" s="6" t="n"/>
       <c r="C17" s="5">
         <f>SUM(C13:C16)</f>
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="D17" s="5">
         <f>SUM(D13:D16)</f>
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="E17" s="5">
         <f>SUM(E13:E16)</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F17" s="5">
         <f>SUM(F13:F16)</f>
@@ -1159,7 +1159,7 @@
       </c>
       <c r="I17" s="9">
         <f>IFERROR(F17/(C17-H17),0)</f>
-        <v>0.21428571428571427</v>
+        <v>0.20224719101123595</v>
       </c>
     </row>
     <row r="19">
@@ -1679,27 +1679,27 @@
     <row r="36" ht="102" customHeight="1">
       <c r="A36" s="13" t="inlineStr">
         <is>
-          <t>R-16</t>
+          <t>P2-16</t>
         </is>
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>Spotpear 量產版加電池電壓檢測（GPIO0 分壓）</t>
+          <t>OTA 分批推送與後台發佈頁</t>
         </is>
       </c>
       <c r="C36" s="13" t="inlineStr">
         <is>
-          <t>1 止血定案</t>
+          <t>4 量產出貨</t>
         </is>
       </c>
       <c r="D36" s="13" t="inlineStr">
         <is>
-          <t>未開始</t>
+          <t>進行中</t>
         </is>
       </c>
       <c r="E36" s="6" t="inlineStr">
         <is>
-          <t>Spotpear 書面確認量產版：GPIO1（屏幕 DC；本版不接屏幕，可空出來）接電芯正極（保護 IC 之後）100k/100k 分壓、100nF 濾波，屏幕不接該腳；GPIO0 保留給現有的 VDD 低電提醒；最好另把充電芯片 CHRG 接到 GPIO12 或 13。樣板到手後，固件讀到的電芯電壓與萬用表相差 ≤50mV，App（R-41）顯示百分比與充電中。</t>
+          <t>後台可上傳韌體（伺服器算 SHA-256、寫 firmware_releases）、填說明、設為 current；推送分階段：白名單 MAC → 10% → 50% → 100%，按 MAC 雜湊穩定分組；回滾率超過 5% 或任一台在試用期內重啟 3 次即自動暫停；顯示每個版本已更新、回滾台數與回滾設備清單；顯示 app 分區用量（P2-12）；每個發佈操作寫入審計記錄。</t>
         </is>
       </c>
       <c r="F36" s="11" t="n"/>
@@ -1707,20 +1707,20 @@
       <c r="H36" s="11" t="n"/>
       <c r="I36" s="12" t="n"/>
     </row>
-    <row r="37" ht="46" customHeight="1">
+    <row r="37" ht="102" customHeight="1">
       <c r="A37" s="13" t="inlineStr">
         <is>
-          <t>P1-11</t>
+          <t>R-16</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>伺服器與資料庫直接存取的管控</t>
+          <t>Spotpear 量產版加電池電壓檢測（GPIO0 分壓）</t>
         </is>
       </c>
       <c r="C37" s="13" t="inlineStr">
         <is>
-          <t>2 內測準備</t>
+          <t>1 止血定案</t>
         </is>
       </c>
       <c r="D37" s="13" t="inlineStr">
@@ -1730,7 +1730,7 @@
       </c>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>列出誰有 SSH 與資料庫直連權限（越少越好）；service_role key 只存在伺服器的 env；私隱政策寫明這類存取的範圍；每次直接查看生產資料都留記錄。</t>
+          <t>Spotpear 書面確認量產版：GPIO1（屏幕 DC；本版不接屏幕，可空出來）接電芯正極（保護 IC 之後）100k/100k 分壓、100nF 濾波，屏幕不接該腳；GPIO0 保留給現有的 VDD 低電提醒；最好另把充電芯片 CHRG 接到 GPIO12 或 13。樣板到手後，固件讀到的電芯電壓與萬用表相差 ≤50mV，App（R-41）顯示百分比與充電中。</t>
         </is>
       </c>
       <c r="F37" s="11" t="n"/>
@@ -1741,12 +1741,12 @@
     <row r="38" ht="46" customHeight="1">
       <c r="A38" s="13" t="inlineStr">
         <is>
-          <t>P2-02</t>
+          <t>P1-11</t>
         </is>
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>CI 跑測試與靜態檢查</t>
+          <t>伺服器與資料庫直接存取的管控</t>
         </is>
       </c>
       <c r="C38" s="13" t="inlineStr">
@@ -1761,7 +1761,7 @@
       </c>
       <c r="E38" s="6" t="inlineStr">
         <is>
-          <t>推送與 PR 時跑 pytest、ruff、pyright、next lint、tsc --noEmit、pio run；任何一項失敗就不發佈 image。</t>
+          <t>列出誰有 SSH 與資料庫直連權限（越少越好）；service_role key 只存在伺服器的 env；私隱政策寫明這類存取的範圍；每次直接查看生產資料都留記錄。</t>
         </is>
       </c>
       <c r="F38" s="11" t="n"/>
@@ -1769,15 +1769,15 @@
       <c r="H38" s="11" t="n"/>
       <c r="I38" s="12" t="n"/>
     </row>
-    <row r="39" ht="32" customHeight="1">
+    <row r="39" ht="46" customHeight="1">
       <c r="A39" s="13" t="inlineStr">
         <is>
-          <t>P2-04</t>
+          <t>P2-02</t>
         </is>
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>容器改用非 root 用戶</t>
+          <t>CI 跑測試與靜態檢查</t>
         </is>
       </c>
       <c r="C39" s="13" t="inlineStr">
@@ -1792,7 +1792,7 @@
       </c>
       <c r="E39" s="6" t="inlineStr">
         <is>
-          <t>兩個 Dockerfile 都設定非 root 的 USER。</t>
+          <t>推送與 PR 時跑 pytest、ruff、pyright、next lint、tsc --noEmit、pio run；任何一項失敗就不發佈 image。</t>
         </is>
       </c>
       <c r="F39" s="11" t="n"/>
@@ -1800,15 +1800,15 @@
       <c r="H39" s="11" t="n"/>
       <c r="I39" s="12" t="n"/>
     </row>
-    <row r="40" ht="46" customHeight="1">
+    <row r="40" ht="32" customHeight="1">
       <c r="A40" s="13" t="inlineStr">
         <is>
-          <t>R-04</t>
+          <t>P2-04</t>
         </is>
       </c>
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>粵語質量評測</t>
+          <t>容器改用非 root 用戶</t>
         </is>
       </c>
       <c r="C40" s="13" t="inlineStr">
@@ -1823,7 +1823,7 @@
       </c>
       <c r="E40" s="6" t="inlineStr">
         <is>
-          <t>有一套粵語評測集（兒童錄音＋文字提示）；選定的 STT 與 LLM 達到門檻：兒童語音字錯率 ≤15%、口語粵語回覆 ≥90%、中英夾雜句能正確理解。</t>
+          <t>兩個 Dockerfile 都設定非 root 的 USER。</t>
         </is>
       </c>
       <c r="F40" s="11" t="n"/>
@@ -1831,15 +1831,15 @@
       <c r="H40" s="11" t="n"/>
       <c r="I40" s="12" t="n"/>
     </row>
-    <row r="41" ht="116" customHeight="1">
+    <row r="41" ht="46" customHeight="1">
       <c r="A41" s="13" t="inlineStr">
         <is>
-          <t>R-25</t>
+          <t>R-04</t>
         </is>
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>網頁的品牌主題系統</t>
+          <t>粵語質量評測</t>
         </is>
       </c>
       <c r="C41" s="13" t="inlineStr">
@@ -1854,7 +1854,7 @@
       </c>
       <c r="E41" s="6" t="inlineStr">
         <is>
-          <t>① 每個品牌一個資料夾：主題 token（顏色、字體、圓角）、logo 和圖示、文案、功能開關；首頁、上手流程、角色頁可以有品牌版本，其餘頁面共用 ② 由部署的環境變數選品牌（每套部署一個品牌，見 R-34），伺服器端渲染的第一屏就是對的主題，不閃爍 ③ 共用元件裡沒有品牌名稱和寫死的品牌顏色 ④ 加一個品牌只需要加資料夾、設定和一套部署，不用改共用元件</t>
+          <t>有一套粵語評測集（兒童錄音＋文字提示）；選定的 STT 與 LLM 達到門檻：兒童語音字錯率 ≤15%、口語粵語回覆 ≥90%、中英夾雜句能正確理解。</t>
         </is>
       </c>
       <c r="F41" s="11" t="n"/>
@@ -1862,68 +1862,68 @@
       <c r="H41" s="11" t="n"/>
       <c r="I41" s="12" t="n"/>
     </row>
-    <row r="43">
-      <c r="A43" s="10" t="inlineStr">
+    <row r="42" ht="116" customHeight="1">
+      <c r="A42" s="13" t="inlineStr">
+        <is>
+          <t>R-25</t>
+        </is>
+      </c>
+      <c r="B42" s="6" t="inlineStr">
+        <is>
+          <t>網頁的品牌主題系統</t>
+        </is>
+      </c>
+      <c r="C42" s="13" t="inlineStr">
+        <is>
+          <t>2 內測準備</t>
+        </is>
+      </c>
+      <c r="D42" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E42" s="6" t="inlineStr">
+        <is>
+          <t>① 每個品牌一個資料夾：主題 token（顏色、字體、圓角）、logo 和圖示、文案、功能開關；首頁、上手流程、角色頁可以有品牌版本，其餘頁面共用 ② 由部署的環境變數選品牌（每套部署一個品牌，見 R-34），伺服器端渲染的第一屏就是對的主題，不閃爍 ③ 共用元件裡沒有品牌名稱和寫死的品牌顏色 ④ 加一個品牌只需要加資料夾、設定和一套部署，不用改共用元件</t>
+        </is>
+      </c>
+      <c r="F42" s="11" t="n"/>
+      <c r="G42" s="11" t="n"/>
+      <c r="H42" s="11" t="n"/>
+      <c r="I42" s="12" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="10" t="inlineStr">
         <is>
           <t>✅ 最近完成與測試效果</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="4" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
         <is>
           <t>編號</t>
         </is>
       </c>
-      <c r="B44" s="4" t="inlineStr">
+      <c r="B45" s="4" t="inlineStr">
         <is>
           <t>任務</t>
         </is>
       </c>
-      <c r="C44" s="4" t="inlineStr">
+      <c r="C45" s="4" t="inlineStr">
         <is>
           <t>測試結果</t>
         </is>
       </c>
-      <c r="D44" s="4" t="inlineStr">
+      <c r="D45" s="4" t="inlineStr">
         <is>
           <t>完成日期</t>
         </is>
       </c>
-      <c r="E44" s="4" t="inlineStr">
+      <c r="E45" s="4" t="inlineStr">
         <is>
           <t>測試證據</t>
-        </is>
-      </c>
-      <c r="F44" s="11" t="n"/>
-      <c r="G44" s="11" t="n"/>
-      <c r="H44" s="11" t="n"/>
-      <c r="I44" s="12" t="n"/>
-    </row>
-    <row r="45" ht="116" customHeight="1">
-      <c r="A45" s="13" t="inlineStr">
-        <is>
-          <t>R-41</t>
-        </is>
-      </c>
-      <c r="B45" s="6" t="inlineStr">
-        <is>
-          <t>App 顯示玩具電量狀態（低電量提示）</t>
-        </is>
-      </c>
-      <c r="C45" s="13" t="inlineStr">
-        <is>
-          <t>通過</t>
-        </is>
-      </c>
-      <c r="D45" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="E45" s="6" t="inlineStr">
-        <is>
-          <t>① pytest 33 passed；真 PATCH 本地 Supabase ② 62:70 刷 p212+R-41 強制低電 build（SUPPLY_LOW_RATIO_OVERRIDE=1.05）→ 串口 [WSc] power low:true，本地 DB battery_low=t ③ 刷回正常 1.6.2 → low:false，DB=f ④ App 讀 DB：低電紅標+Please charge+更新時間、72% 充電中、未上報不顯示 ⑤ 他人帳號 0 行、authenticated UPDATE 被拒。62:70 已還原為原 p212 build</t>
         </is>
       </c>
       <c r="F45" s="11" t="n"/>
@@ -1931,15 +1931,15 @@
       <c r="H45" s="11" t="n"/>
       <c r="I45" s="12" t="n"/>
     </row>
-    <row r="46" ht="102" customHeight="1">
+    <row r="46" ht="116" customHeight="1">
       <c r="A46" s="13" t="inlineStr">
         <is>
-          <t>P0-12</t>
+          <t>R-41</t>
         </is>
       </c>
       <c r="B46" s="6" t="inlineStr">
         <is>
-          <t>收緊 Admin 權限與路由保護</t>
+          <t>App 顯示玩具電量狀態（低電量提示）</t>
         </is>
       </c>
       <c r="C46" s="13" t="inlineStr">
@@ -1949,12 +1949,12 @@
       </c>
       <c r="D46" s="13" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E46" s="6" t="inlineStr">
         <is>
-          <t>線上 2026-10-12（bac24e9）：runbook 10/08 檢查 未登入 /admin→/login、/api/admin→401、has_role() 只看角色、無管理員 policy 觸及 conversations/記憶表、超管≥1；未登入 /home、/admin→/login；用戶確認：家長帳號開 /admin 轉回 /home、管理員在 /admin 修改角色保存成功；角色細分權限沿用本機 61/61</t>
+          <t>① pytest 33 passed；真 PATCH 本地 Supabase ② 62:70 刷 p212+R-41 強制低電 build（SUPPLY_LOW_RATIO_OVERRIDE=1.05）→ 串口 [WSc] power low:true，本地 DB battery_low=t ③ 刷回正常 1.6.2 → low:false，DB=f ④ App 讀 DB：低電紅標+Please charge+更新時間、72% 充電中、未上報不顯示 ⑤ 他人帳號 0 行、authenticated UPDATE 被拒。62:70 已還原為原 p212 build</t>
         </is>
       </c>
       <c r="F46" s="11" t="n"/>
@@ -1962,15 +1962,15 @@
       <c r="H46" s="11" t="n"/>
       <c r="I46" s="12" t="n"/>
     </row>
-    <row r="47" ht="88" customHeight="1">
+    <row r="47" ht="102" customHeight="1">
       <c r="A47" s="13" t="inlineStr">
         <is>
-          <t>P0-15</t>
+          <t>P0-12</t>
         </is>
       </c>
       <c r="B47" s="6" t="inlineStr">
         <is>
-          <t>角色表權限：只有內容管理員能發佈，關閉家長自建角色</t>
+          <t>收緊 Admin 權限與路由保護</t>
         </is>
       </c>
       <c r="C47" s="13" t="inlineStr">
@@ -1985,7 +1985,7 @@
       </c>
       <c r="E47" s="6" t="inlineStr">
         <is>
-          <t>線上 2026-10-12：② anon 只見 6 個已發佈 hk_ 內建，查隱藏/醫生/家長自建 → []，anon POST → 401；① authenticated 寫入權限由 20261007140000 REVOKE（runbook 10/08 已套用）；用戶確認：④ 家長登入後 /home/create 轉回 /home ③ 管理員在 /admin 修改角色保存成功</t>
+          <t>線上 2026-10-12（bac24e9）：runbook 10/08 檢查 未登入 /admin→/login、/api/admin→401、has_role() 只看角色、無管理員 policy 觸及 conversations/記憶表、超管≥1；未登入 /home、/admin→/login；用戶確認：家長帳號開 /admin 轉回 /home、管理員在 /admin 修改角色保存成功；角色細分權限沿用本機 61/61</t>
         </is>
       </c>
       <c r="F47" s="11" t="n"/>
@@ -1996,12 +1996,12 @@
     <row r="48" ht="88" customHeight="1">
       <c r="A48" s="13" t="inlineStr">
         <is>
-          <t>P0-16</t>
+          <t>P0-15</t>
         </is>
       </c>
       <c r="B48" s="6" t="inlineStr">
         <is>
-          <t>移除「醫生」身份與寫死的通關碼</t>
+          <t>角色表權限：只有內容管理員能發佈，關閉家長自建角色</t>
         </is>
       </c>
       <c r="C48" s="13" t="inlineStr">
@@ -2016,7 +2016,7 @@
       </c>
       <c r="E48" s="6" t="inlineStr">
         <is>
-          <t>線上 2026-10-12：生產 commit bac24e9 git grep checkDoctorAction/kiwi-subtle-emu/=== "doctor"/isDoctor → 0；線上 13 個 JS（/、/login、/onboard）grep 通關碼/"doctor"/Santa/patient → 0；anon 讀角色只見 6 個 hk_ 角色、is_doctor 全 false；用戶今日線上登入及 playground 正常</t>
+          <t>線上 2026-10-12：② anon 只見 6 個已發佈 hk_ 內建，查隱藏/醫生/家長自建 → []，anon POST → 401；① authenticated 寫入權限由 20261007140000 REVOKE（runbook 10/08 已套用）；用戶確認：④ 家長登入後 /home/create 轉回 /home ③ 管理員在 /admin 修改角色保存成功</t>
         </is>
       </c>
       <c r="F48" s="11" t="n"/>
@@ -2024,15 +2024,15 @@
       <c r="H48" s="11" t="n"/>
       <c r="I48" s="12" t="n"/>
     </row>
-    <row r="49" ht="60" customHeight="1">
+    <row r="49" ht="88" customHeight="1">
       <c r="A49" s="13" t="inlineStr">
         <is>
-          <t>P0-09</t>
+          <t>P0-16</t>
         </is>
       </c>
       <c r="B49" s="6" t="inlineStr">
         <is>
-          <t>瀏覽器語音路由改用簽名 token（/ws/nextjs）</t>
+          <t>移除「醫生」身份與寫死的通關碼</t>
         </is>
       </c>
       <c r="C49" s="13" t="inlineStr">
@@ -2047,7 +2047,7 @@
       </c>
       <c r="E49" s="6" t="inlineStr">
         <is>
-          <t>線上 2026-10-12（bac24e9）：wss /fastapi/ws/nextjs 只帶 user_id 或 token=bogus → 4401；用戶確認：登入 elatoai.hkqft.com 後網頁 playground 可正常對話</t>
+          <t>線上 2026-10-12：生產 commit bac24e9 git grep checkDoctorAction/kiwi-subtle-emu/=== "doctor"/isDoctor → 0；線上 13 個 JS（/、/login、/onboard）grep 通關碼/"doctor"/Santa/patient → 0；anon 讀角色只見 6 個 hk_ 角色、is_doctor 全 false；用戶今日線上登入及 playground 正常</t>
         </is>
       </c>
       <c r="F49" s="11" t="n"/>
@@ -2058,12 +2058,12 @@
     <row r="50" ht="60" customHeight="1">
       <c r="A50" s="13" t="inlineStr">
         <is>
-          <t>P0-17</t>
+          <t>P0-09</t>
         </is>
       </c>
       <c r="B50" s="6" t="inlineStr">
         <is>
-          <t>前端的 anon key 必須是公開 key，不可是 secret／service_role</t>
+          <t>瀏覽器語音路由改用簽名 token（/ws/nextjs）</t>
         </is>
       </c>
       <c r="C50" s="13" t="inlineStr">
@@ -2078,7 +2078,7 @@
       </c>
       <c r="E50" s="6" t="inlineStr">
         <is>
-          <t>線上 2026-10-12（bac24e9）：/login 引用的 13 個 JS + HTML 無 sb_secret_，唯一 key 為 role=anon 的 JWT；② 用該 key GET /rest/v1/users → 42501；③ 本機 10/07 已換 publishable</t>
+          <t>線上 2026-10-12（bac24e9）：wss /fastapi/ws/nextjs 只帶 user_id 或 token=bogus → 4401；用戶確認：登入 elatoai.hkqft.com 後網頁 playground 可正常對話</t>
         </is>
       </c>
       <c r="F50" s="11" t="n"/>
@@ -2086,15 +2086,15 @@
       <c r="H50" s="11" t="n"/>
       <c r="I50" s="12" t="n"/>
     </row>
-    <row r="51" ht="46" customHeight="1">
+    <row r="51" ht="60" customHeight="1">
       <c r="A51" s="13" t="inlineStr">
         <is>
-          <t>P0-10</t>
+          <t>P0-17</t>
         </is>
       </c>
       <c r="B51" s="6" t="inlineStr">
         <is>
-          <t>生產環境關閉 /browser 測試頁與 /ws/browser</t>
+          <t>前端的 anon key 必須是公開 key，不可是 secret／service_role</t>
         </is>
       </c>
       <c r="C51" s="13" t="inlineStr">
@@ -2109,7 +2109,7 @@
       </c>
       <c r="E51" s="6" t="inlineStr">
         <is>
-          <t>線上 2026-10-12（bac24e9）：GET /fastapi/browser 404、/fastapi/ 404、/fastapi/healthz 200、wss /fastapi/ws/browser → HTTP 403</t>
+          <t>線上 2026-10-12（bac24e9）：/login 引用的 13 個 JS + HTML 無 sb_secret_，唯一 key 為 role=anon 的 JWT；② 用該 key GET /rest/v1/users → 42501；③ 本機 10/07 已換 publishable</t>
         </is>
       </c>
       <c r="F51" s="11" t="n"/>
@@ -2117,15 +2117,15 @@
       <c r="H51" s="11" t="n"/>
       <c r="I51" s="12" t="n"/>
     </row>
-    <row r="52" ht="60" customHeight="1">
+    <row r="52" ht="46" customHeight="1">
       <c r="A52" s="13" t="inlineStr">
         <is>
-          <t>P0-08</t>
+          <t>P0-10</t>
         </is>
       </c>
       <c r="B52" s="6" t="inlineStr">
         <is>
-          <t>語音伺服器驗證設備身份（/ws/esp32）</t>
+          <t>生產環境關閉 /browser 測試頁與 /ws/browser</t>
         </is>
       </c>
       <c r="C52" s="13" t="inlineStr">
@@ -2140,7 +2140,7 @@
       </c>
       <c r="E52" s="6" t="inlineStr">
         <is>
-          <t>線上 2026-10-12（bac24e9）：wss /fastapi/ws/esp32 不帶 token、偽造 token＋X-Device-Mac → 均 4401 invalid device token；42:34 以有效 token 連線對話正常（P0-13 10/09）</t>
+          <t>線上 2026-10-12（bac24e9）：GET /fastapi/browser 404、/fastapi/ 404、/fastapi/healthz 200、wss /fastapi/ws/browser → HTTP 403</t>
         </is>
       </c>
       <c r="F52" s="11" t="n"/>
@@ -2148,50 +2148,58 @@
       <c r="H52" s="11" t="n"/>
       <c r="I52" s="12" t="n"/>
     </row>
-    <row r="54">
-      <c r="A54" s="10" t="inlineStr">
+    <row r="53" ht="60" customHeight="1">
+      <c r="A53" s="13" t="inlineStr">
+        <is>
+          <t>P0-08</t>
+        </is>
+      </c>
+      <c r="B53" s="6" t="inlineStr">
+        <is>
+          <t>語音伺服器驗證設備身份（/ws/esp32）</t>
+        </is>
+      </c>
+      <c r="C53" s="13" t="inlineStr">
+        <is>
+          <t>通過</t>
+        </is>
+      </c>
+      <c r="D53" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="E53" s="6" t="inlineStr">
+        <is>
+          <t>線上 2026-10-12（bac24e9）：wss /fastapi/ws/esp32 不帶 token、偽造 token＋X-Device-Mac → 均 4401 invalid device token；42:34 以有效 token 連線對話正常（P0-13 10/09）</t>
+        </is>
+      </c>
+      <c r="F53" s="11" t="n"/>
+      <c r="G53" s="11" t="n"/>
+      <c r="H53" s="11" t="n"/>
+      <c r="I53" s="12" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="10" t="inlineStr">
         <is>
           <t>⏳ 等待依賴 / ⛔ 阻塞</t>
         </is>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="4" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
         <is>
           <t>編號</t>
         </is>
       </c>
-      <c r="B55" s="4" t="inlineStr">
+      <c r="B56" s="4" t="inlineStr">
         <is>
           <t>任務</t>
         </is>
       </c>
-      <c r="C55" s="4" t="inlineStr">
+      <c r="C56" s="4" t="inlineStr">
         <is>
           <t>在等什麼</t>
-        </is>
-      </c>
-      <c r="D55" s="11" t="n"/>
-      <c r="E55" s="11" t="n"/>
-      <c r="F55" s="11" t="n"/>
-      <c r="G55" s="11" t="n"/>
-      <c r="H55" s="11" t="n"/>
-      <c r="I55" s="12" t="n"/>
-    </row>
-    <row r="56" ht="88" customHeight="1">
-      <c r="A56" s="13" t="inlineStr">
-        <is>
-          <t>R-17</t>
-        </is>
-      </c>
-      <c r="B56" s="6" t="inlineStr">
-        <is>
-          <t>Spotpear 電池耗盡時插電能否正常開機（供電路徑）</t>
-        </is>
-      </c>
-      <c r="C56" s="6" t="inlineStr">
-        <is>
-          <t>阻塞：[2026-10-08] 2026-10-08 開發板 63:64 插著 USB 時兩次無法解釋的完全斷電重開：09:13:26（崩潰循環中）、10:44:33（閒置、用戶確認沒碰）。都是 USB 先斷線再以 ESP_RST_POWERON 開機，非 brownout；斷電前 6 秒 GPIO0 讀數 99.9% 參考值，屬突然切斷而非緩降（SupplyMonitor 取樣太疏抓不到瞬間）。韌體無法造成 POWERON，指向充電芯片/電池保護/供電路徑，應一併問 Spotpear；放電實測時留意插 USB 閒置時是否也會斷電</t>
         </is>
       </c>
       <c r="D56" s="11" t="n"/>
@@ -2201,20 +2209,20 @@
       <c r="H56" s="11" t="n"/>
       <c r="I56" s="12" t="n"/>
     </row>
-    <row r="57" ht="60" customHeight="1">
+    <row r="57" ht="88" customHeight="1">
       <c r="A57" s="13" t="inlineStr">
         <is>
-          <t>P1-01</t>
+          <t>R-17</t>
         </is>
       </c>
       <c r="B57" s="6" t="inlineStr">
         <is>
-          <t>加入內容審核層（輸入與輸出）</t>
+          <t>Spotpear 電池耗盡時插電能否正常開機（供電路徑）</t>
         </is>
       </c>
       <c r="C57" s="6" t="inlineStr">
         <is>
-          <t>阻塞：[2026-10-14] 2026-10-14 用戶決定：先不定審核服務商，本項暫停。候選：Azure Content Safety（建議，香港區、可在每句回覆說出口前檢查）、OpenRouter 安全模型、OpenAI Moderation、只用本機字詞表。未寫任何程式。</t>
+          <t>阻塞：[2026-10-08] 2026-10-08 開發板 63:64 插著 USB 時兩次無法解釋的完全斷電重開：09:13:26（崩潰循環中）、10:44:33（閒置、用戶確認沒碰）。都是 USB 先斷線再以 ESP_RST_POWERON 開機，非 brownout；斷電前 6 秒 GPIO0 讀數 99.9% 參考值，屬突然切斷而非緩降（SupplyMonitor 取樣太疏抓不到瞬間）。韌體無法造成 POWERON，指向充電芯片/電池保護/供電路徑，應一併問 Spotpear；放電實測時留意插 USB 閒置時是否也會斷電</t>
         </is>
       </c>
       <c r="D57" s="11" t="n"/>
@@ -2224,20 +2232,20 @@
       <c r="H57" s="11" t="n"/>
       <c r="I57" s="12" t="n"/>
     </row>
-    <row r="58" ht="32" customHeight="1">
+    <row r="58" ht="60" customHeight="1">
       <c r="A58" s="13" t="inlineStr">
         <is>
-          <t>P1-09</t>
+          <t>P1-01</t>
         </is>
       </c>
       <c r="B58" s="6" t="inlineStr">
         <is>
-          <t>家長鎖：孩子模式進設定要輸入 PIN</t>
+          <t>加入內容審核層（輸入與輸出）</t>
         </is>
       </c>
       <c r="C58" s="6" t="inlineStr">
         <is>
-          <t>阻塞：[2026-10-13] 2026-10-13 用戶決定：AI Buddy（品牌 C）延到 1/15 之後，本項不卡 1/15 出廠；AI Buddy 啟動時再開。</t>
+          <t>阻塞：[2026-10-14] 2026-10-14 用戶決定：先不定審核服務商，本項暫停。候選：Azure Content Safety（建議，香港區、可在每句回覆說出口前檢查）、OpenRouter 安全模型、OpenAI Moderation、只用本機字詞表。未寫任何程式。</t>
         </is>
       </c>
       <c r="D58" s="11" t="n"/>
@@ -2250,12 +2258,12 @@
     <row r="59" ht="32" customHeight="1">
       <c r="A59" s="13" t="inlineStr">
         <is>
-          <t>R-12</t>
+          <t>P1-09</t>
         </is>
       </c>
       <c r="B59" s="6" t="inlineStr">
         <is>
-          <t>家長控制：每日使用上限和休息時段</t>
+          <t>家長鎖：孩子模式進設定要輸入 PIN</t>
         </is>
       </c>
       <c r="C59" s="6" t="inlineStr">
@@ -2273,12 +2281,12 @@
     <row r="60" ht="32" customHeight="1">
       <c r="A60" s="13" t="inlineStr">
         <is>
-          <t>R-29</t>
+          <t>R-12</t>
         </is>
       </c>
       <c r="B60" s="6" t="inlineStr">
         <is>
-          <t>AI Buddy App（品牌 C）頁面</t>
+          <t>家長控制：每日使用上限和休息時段</t>
         </is>
       </c>
       <c r="C60" s="6" t="inlineStr">
@@ -2293,20 +2301,20 @@
       <c r="H60" s="11" t="n"/>
       <c r="I60" s="12" t="n"/>
     </row>
-    <row r="61" ht="18" customHeight="1">
+    <row r="61" ht="32" customHeight="1">
       <c r="A61" s="13" t="inlineStr">
         <is>
-          <t>R-05</t>
+          <t>R-29</t>
         </is>
       </c>
       <c r="B61" s="6" t="inlineStr">
         <is>
-          <t>內測版外殼（3D 打印 20 台）</t>
+          <t>AI Buddy App（品牌 C）頁面</t>
         </is>
       </c>
       <c r="C61" s="6" t="inlineStr">
         <is>
-          <t>等 R-01</t>
+          <t>阻塞：[2026-10-13] 2026-10-13 用戶決定：AI Buddy（品牌 C）延到 1/15 之後，本項不卡 1/15 出廠；AI Buddy 啟動時再開。</t>
         </is>
       </c>
       <c r="D61" s="11" t="n"/>
@@ -2319,17 +2327,17 @@
     <row r="62" ht="18" customHeight="1">
       <c r="A62" s="13" t="inlineStr">
         <is>
-          <t>R-06</t>
+          <t>R-05</t>
         </is>
       </c>
       <c r="B62" s="6" t="inlineStr">
         <is>
-          <t>家長自助上手流程</t>
+          <t>內測版外殼（3D 打印 20 台）</t>
         </is>
       </c>
       <c r="C62" s="6" t="inlineStr">
         <is>
-          <t>等 P0-11</t>
+          <t>等 R-01</t>
         </is>
       </c>
       <c r="D62" s="11" t="n"/>
@@ -2339,20 +2347,20 @@
       <c r="H62" s="11" t="n"/>
       <c r="I62" s="12" t="n"/>
     </row>
-    <row r="63" ht="32" customHeight="1">
+    <row r="63" ht="18" customHeight="1">
       <c r="A63" s="13" t="inlineStr">
         <is>
-          <t>R-13</t>
+          <t>R-06</t>
         </is>
       </c>
       <c r="B63" s="6" t="inlineStr">
         <is>
-          <t>CP1 內測就緒檢查（10/30）</t>
+          <t>家長自助上手流程</t>
         </is>
       </c>
       <c r="C63" s="6" t="inlineStr">
         <is>
-          <t>等 P0-07、P0-11、P1-01、P1-02、P2-09、R-01、R-02、R-04、R-05、R-06、P1-11</t>
+          <t>等 P0-11</t>
         </is>
       </c>
       <c r="D63" s="11" t="n"/>
@@ -2365,17 +2373,17 @@
     <row r="64" ht="32" customHeight="1">
       <c r="A64" s="13" t="inlineStr">
         <is>
-          <t>R-18</t>
+          <t>R-13</t>
         </is>
       </c>
       <c r="B64" s="6" t="inlineStr">
         <is>
-          <t>長按 BOOT 重新配網（開 AIBuddy-XXXX 熱點）</t>
+          <t>CP1 內測就緒檢查（10/30）</t>
         </is>
       </c>
       <c r="C64" s="6" t="inlineStr">
         <is>
-          <t>等 R-01</t>
+          <t>等 P0-07、P0-11、P1-01、P1-02、P2-09、R-01、R-02、R-04、R-05、R-06、P1-11</t>
         </is>
       </c>
       <c r="D64" s="11" t="n"/>
@@ -2388,12 +2396,12 @@
     <row r="65" ht="32" customHeight="1">
       <c r="A65" s="13" t="inlineStr">
         <is>
-          <t>R-19</t>
+          <t>R-18</t>
         </is>
       </c>
       <c r="B65" s="6" t="inlineStr">
         <is>
-          <t>外接按鈕：量產板加 I2C 擴展晶片（TCA9555）</t>
+          <t>長按 BOOT 重新配網（開 AIBuddy-XXXX 熱點）</t>
         </is>
       </c>
       <c r="C65" s="6" t="inlineStr">
@@ -2408,20 +2416,20 @@
       <c r="H65" s="11" t="n"/>
       <c r="I65" s="12" t="n"/>
     </row>
-    <row r="66" ht="18" customHeight="1">
+    <row r="66" ht="32" customHeight="1">
       <c r="A66" s="13" t="inlineStr">
         <is>
-          <t>R-20</t>
+          <t>R-19</t>
         </is>
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
-          <t>孩子資料與角色改成每台設備一份</t>
+          <t>外接按鈕：量產板加 I2C 擴展晶片（TCA9555）</t>
         </is>
       </c>
       <c r="C66" s="6" t="inlineStr">
         <is>
-          <t>等 P1-12</t>
+          <t>等 R-01</t>
         </is>
       </c>
       <c r="D66" s="11" t="n"/>
@@ -2431,20 +2439,20 @@
       <c r="H66" s="11" t="n"/>
       <c r="I66" s="12" t="n"/>
     </row>
-    <row r="67" ht="32" customHeight="1">
+    <row r="67" ht="18" customHeight="1">
       <c r="A67" s="13" t="inlineStr">
         <is>
-          <t>R-27</t>
+          <t>R-20</t>
         </is>
       </c>
       <c r="B67" s="6" t="inlineStr">
         <is>
-          <t>App 內登入：驗證碼、原生社交登入、刪除帳號</t>
+          <t>孩子資料與角色改成每台設備一份</t>
         </is>
       </c>
       <c r="C67" s="6" t="inlineStr">
         <is>
-          <t>等 R-26</t>
+          <t>等 P1-12</t>
         </is>
       </c>
       <c r="D67" s="11" t="n"/>
@@ -2454,20 +2462,20 @@
       <c r="H67" s="11" t="n"/>
       <c r="I67" s="12" t="n"/>
     </row>
-    <row r="68" ht="18" customHeight="1">
+    <row r="68" ht="32" customHeight="1">
       <c r="A68" s="13" t="inlineStr">
         <is>
-          <t>P0-14</t>
+          <t>R-27</t>
         </is>
       </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t>韌體簽章、Secure Boot 與 Flash 加密</t>
+          <t>App 內登入：驗證碼、原生社交登入、刪除帳號</t>
         </is>
       </c>
       <c r="C68" s="6" t="inlineStr">
         <is>
-          <t>等 R-01</t>
+          <t>等 R-26</t>
         </is>
       </c>
       <c r="D68" s="11" t="n"/>
@@ -2480,17 +2488,17 @@
     <row r="69" ht="18" customHeight="1">
       <c r="A69" s="13" t="inlineStr">
         <is>
-          <t>P1-06</t>
+          <t>P0-14</t>
         </is>
       </c>
       <c r="B69" s="6" t="inlineStr">
         <is>
-          <t>處理 GPL-3.0 依賴（arduino-audio-tools）</t>
+          <t>韌體簽章、Secure Boot 與 Flash 加密</t>
         </is>
       </c>
       <c r="C69" s="6" t="inlineStr">
         <is>
-          <t>等 Q3</t>
+          <t>等 R-01</t>
         </is>
       </c>
       <c r="D69" s="11" t="n"/>
@@ -2503,12 +2511,12 @@
     <row r="70" ht="18" customHeight="1">
       <c r="A70" s="13" t="inlineStr">
         <is>
-          <t>P1-07</t>
+          <t>P1-06</t>
         </is>
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>LGPL 合規與第三方授權聲明</t>
+          <t>處理 GPL-3.0 依賴（arduino-audio-tools）</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr">
@@ -2526,17 +2534,17 @@
     <row r="71" ht="18" customHeight="1">
       <c r="A71" s="13" t="inlineStr">
         <is>
-          <t>P1-08</t>
+          <t>P1-07</t>
         </is>
       </c>
       <c r="B71" s="6" t="inlineStr">
         <is>
-          <t>硬件認證</t>
+          <t>LGPL 合規與第三方授權聲明</t>
         </is>
       </c>
       <c r="C71" s="6" t="inlineStr">
         <is>
-          <t>等 R-01、R-05</t>
+          <t>等 Q3</t>
         </is>
       </c>
       <c r="D71" s="11" t="n"/>
@@ -2549,17 +2557,17 @@
     <row r="72" ht="18" customHeight="1">
       <c r="A72" s="13" t="inlineStr">
         <is>
-          <t>P1-14</t>
+          <t>P1-08</t>
         </is>
       </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>Admin 內容安全頁：審核事件只按類別統計</t>
+          <t>硬件認證</t>
         </is>
       </c>
       <c r="C72" s="6" t="inlineStr">
         <is>
-          <t>等 P1-01、P2-13</t>
+          <t>等 R-01、R-05</t>
         </is>
       </c>
       <c r="D72" s="11" t="n"/>
@@ -2569,20 +2577,20 @@
       <c r="H72" s="11" t="n"/>
       <c r="I72" s="12" t="n"/>
     </row>
-    <row r="73" ht="32" customHeight="1">
+    <row r="73" ht="18" customHeight="1">
       <c r="A73" s="13" t="inlineStr">
         <is>
-          <t>P2-15</t>
+          <t>P1-14</t>
         </is>
       </c>
       <c r="B73" s="6" t="inlineStr">
         <is>
-          <t>Admin 總覽頁：在線、用量、成本與待處理事項</t>
+          <t>Admin 內容安全頁：審核事件只按類別統計</t>
         </is>
       </c>
       <c r="C73" s="6" t="inlineStr">
         <is>
-          <t>等 P2-14、P2-09</t>
+          <t>等 P1-01、P2-13</t>
         </is>
       </c>
       <c r="D73" s="11" t="n"/>
@@ -2592,20 +2600,20 @@
       <c r="H73" s="11" t="n"/>
       <c r="I73" s="12" t="n"/>
     </row>
-    <row r="74" ht="18" customHeight="1">
+    <row r="74" ht="32" customHeight="1">
       <c r="A74" s="13" t="inlineStr">
         <is>
-          <t>R-07</t>
+          <t>P2-15</t>
         </is>
       </c>
       <c r="B74" s="6" t="inlineStr">
         <is>
-          <t>20 個家庭封閉內測</t>
+          <t>Admin 總覽頁：在線、用量、成本與待處理事項</t>
         </is>
       </c>
       <c r="C74" s="6" t="inlineStr">
         <is>
-          <t>等 R-13</t>
+          <t>等 P2-14、P2-09</t>
         </is>
       </c>
       <c r="D74" s="11" t="n"/>
@@ -2618,17 +2626,17 @@
     <row r="75" ht="18" customHeight="1">
       <c r="A75" s="13" t="inlineStr">
         <is>
-          <t>R-08</t>
+          <t>R-07</t>
         </is>
       </c>
       <c r="B75" s="6" t="inlineStr">
         <is>
-          <t>第 8 週關卡決策</t>
+          <t>20 個家庭封閉內測</t>
         </is>
       </c>
       <c r="C75" s="6" t="inlineStr">
         <is>
-          <t>等 R-07、P2-09、P1-08</t>
+          <t>等 R-13</t>
         </is>
       </c>
       <c r="D75" s="11" t="n"/>
@@ -2641,17 +2649,17 @@
     <row r="76" ht="18" customHeight="1">
       <c r="A76" s="13" t="inlineStr">
         <is>
-          <t>R-14</t>
+          <t>R-08</t>
         </is>
       </c>
       <c r="B76" s="6" t="inlineStr">
         <is>
-          <t>離線兒歌與故事</t>
+          <t>第 8 週關卡決策</t>
         </is>
       </c>
       <c r="C76" s="6" t="inlineStr">
         <is>
-          <t>等 R-01</t>
+          <t>等 R-07、P2-09、P1-08</t>
         </is>
       </c>
       <c r="D76" s="11" t="n"/>
@@ -2664,17 +2672,17 @@
     <row r="77" ht="18" customHeight="1">
       <c r="A77" s="13" t="inlineStr">
         <is>
-          <t>R-24</t>
+          <t>R-14</t>
         </is>
       </c>
       <c r="B77" s="6" t="inlineStr">
         <is>
-          <t>設備只能用自己品牌的角色</t>
+          <t>離線兒歌與故事</t>
         </is>
       </c>
       <c r="C77" s="6" t="inlineStr">
         <is>
-          <t>等 R-34</t>
+          <t>等 R-01</t>
         </is>
       </c>
       <c r="D77" s="11" t="n"/>
@@ -2687,17 +2695,17 @@
     <row r="78" ht="18" customHeight="1">
       <c r="A78" s="13" t="inlineStr">
         <is>
-          <t>R-28</t>
+          <t>R-24</t>
         </is>
       </c>
       <c r="B78" s="6" t="inlineStr">
         <is>
-          <t>三個 App 的殼：品牌版本與測試版</t>
+          <t>設備只能用自己品牌的角色</t>
         </is>
       </c>
       <c r="C78" s="6" t="inlineStr">
         <is>
-          <t>等 R-25、R-26</t>
+          <t>等 R-34</t>
         </is>
       </c>
       <c r="D78" s="11" t="n"/>
@@ -2710,17 +2718,17 @@
     <row r="79" ht="18" customHeight="1">
       <c r="A79" s="13" t="inlineStr">
         <is>
-          <t>R-30</t>
+          <t>R-28</t>
         </is>
       </c>
       <c r="B79" s="6" t="inlineStr">
         <is>
-          <t>快活 App（品牌 A）頁面</t>
+          <t>三個 App 的殼：品牌版本與測試版</t>
         </is>
       </c>
       <c r="C79" s="6" t="inlineStr">
         <is>
-          <t>等 R-25、R-34、Q12</t>
+          <t>等 R-25、R-26</t>
         </is>
       </c>
       <c r="D79" s="11" t="n"/>
@@ -2733,17 +2741,17 @@
     <row r="80" ht="18" customHeight="1">
       <c r="A80" s="13" t="inlineStr">
         <is>
-          <t>R-31</t>
+          <t>R-30</t>
         </is>
       </c>
       <c r="B80" s="6" t="inlineStr">
         <is>
-          <t>政協青年聯會版 App（品牌 B）頁面</t>
+          <t>快活 App（品牌 A）頁面</t>
         </is>
       </c>
       <c r="C80" s="6" t="inlineStr">
         <is>
-          <t>等 R-25、R-34、Q13</t>
+          <t>等 R-25、R-34、Q12</t>
         </is>
       </c>
       <c r="D80" s="11" t="n"/>
@@ -2756,17 +2764,17 @@
     <row r="81" ht="18" customHeight="1">
       <c r="A81" s="13" t="inlineStr">
         <is>
-          <t>R-35</t>
+          <t>R-31</t>
         </is>
       </c>
       <c r="B81" s="6" t="inlineStr">
         <is>
-          <t>韌體按品牌連線：伺服器網址在出廠時寫入</t>
+          <t>政協青年聯會版 App（品牌 B）頁面</t>
         </is>
       </c>
       <c r="C81" s="6" t="inlineStr">
         <is>
-          <t>等 R-34</t>
+          <t>等 R-25、R-34、Q13</t>
         </is>
       </c>
       <c r="D81" s="11" t="n"/>
@@ -2776,20 +2784,20 @@
       <c r="H81" s="11" t="n"/>
       <c r="I81" s="12" t="n"/>
     </row>
-    <row r="82" ht="32" customHeight="1">
+    <row r="82" ht="18" customHeight="1">
       <c r="A82" s="13" t="inlineStr">
         <is>
-          <t>R-38</t>
+          <t>R-35</t>
         </is>
       </c>
       <c r="B82" s="6" t="inlineStr">
         <is>
-          <t>公仔出廠鎖死所屬 IP，綁定時顯示該 IP 頭像</t>
+          <t>韌體按品牌連線：伺服器網址在出廠時寫入</t>
         </is>
       </c>
       <c r="C82" s="6" t="inlineStr">
         <is>
-          <t>等 P0-11</t>
+          <t>等 R-34</t>
         </is>
       </c>
       <c r="D82" s="11" t="n"/>
@@ -2802,17 +2810,17 @@
     <row r="83" ht="32" customHeight="1">
       <c r="A83" s="13" t="inlineStr">
         <is>
-          <t>R-39</t>
+          <t>R-38</t>
         </is>
       </c>
       <c r="B83" s="6" t="inlineStr">
         <is>
-          <t>Admin 出廠登記頁：匯入 MAC 清單、指定公仔、查看自檢結果</t>
+          <t>公仔出廠鎖死所屬 IP，綁定時顯示該 IP 頭像</t>
         </is>
       </c>
       <c r="C83" s="6" t="inlineStr">
         <is>
-          <t>等 R-38、P1-10</t>
+          <t>等 P0-11</t>
         </is>
       </c>
       <c r="D83" s="11" t="n"/>
@@ -2822,20 +2830,20 @@
       <c r="H83" s="11" t="n"/>
       <c r="I83" s="12" t="n"/>
     </row>
-    <row r="84" ht="18" customHeight="1">
+    <row r="84" ht="32" customHeight="1">
       <c r="A84" s="13" t="inlineStr">
         <is>
-          <t>P2-16</t>
+          <t>R-39</t>
         </is>
       </c>
       <c r="B84" s="6" t="inlineStr">
         <is>
-          <t>OTA 分批推送與後台發佈頁</t>
+          <t>Admin 出廠登記頁：匯入 MAC 清單、指定公仔、查看自檢結果</t>
         </is>
       </c>
       <c r="C84" s="6" t="inlineStr">
         <is>
-          <t>等 P2-14、P1-10</t>
+          <t>等 R-38、P1-10</t>
         </is>
       </c>
       <c r="D84" s="11" t="n"/>
@@ -2845,20 +2853,20 @@
       <c r="H84" s="11" t="n"/>
       <c r="I84" s="12" t="n"/>
     </row>
-    <row r="85" ht="18" customHeight="1">
+    <row r="85" ht="32" customHeight="1">
       <c r="A85" s="13" t="inlineStr">
         <is>
-          <t>R-09</t>
+          <t>P2-18</t>
         </is>
       </c>
       <c r="B85" s="6" t="inlineStr">
         <is>
-          <t>量產外殼（真空複模）</t>
+          <t>P2-16 ② 按 MAC 雜湊穩定分組決定哪台收到 ota</t>
         </is>
       </c>
       <c r="C85" s="6" t="inlineStr">
         <is>
-          <t>等 R-08、R-05、Q11</t>
+          <t>等 P2-17</t>
         </is>
       </c>
       <c r="D85" s="11" t="n"/>
@@ -2871,17 +2879,17 @@
     <row r="86" ht="18" customHeight="1">
       <c r="A86" s="13" t="inlineStr">
         <is>
-          <t>R-10</t>
+          <t>P2-19</t>
         </is>
       </c>
       <c r="B86" s="6" t="inlineStr">
         <is>
-          <t>出廠流程</t>
+          <t>P2-16 ③ 回滾過多時自動暫停推送</t>
         </is>
       </c>
       <c r="C86" s="6" t="inlineStr">
         <is>
-          <t>等 P0-14、R-01、P2-12、R-34、R-35、R-38、R-39</t>
+          <t>等 P2-18</t>
         </is>
       </c>
       <c r="D86" s="11" t="n"/>
@@ -2891,20 +2899,20 @@
       <c r="H86" s="11" t="n"/>
       <c r="I86" s="12" t="n"/>
     </row>
-    <row r="87" ht="18" customHeight="1">
+    <row r="87" ht="32" customHeight="1">
       <c r="A87" s="13" t="inlineStr">
         <is>
-          <t>R-11</t>
+          <t>P2-20</t>
         </is>
       </c>
       <c r="B87" s="6" t="inlineStr">
         <is>
-          <t>售後：客服、保修與換機</t>
+          <t>P2-16 ④ 從後台上傳與發佈韌體（取代手貼 service key）</t>
         </is>
       </c>
       <c r="C87" s="6" t="inlineStr">
         <is>
-          <t>等 P2-14、R-40</t>
+          <t>等 P2-17、P1-10</t>
         </is>
       </c>
       <c r="D87" s="11" t="n"/>
@@ -2917,17 +2925,17 @@
     <row r="88" ht="18" customHeight="1">
       <c r="A88" s="13" t="inlineStr">
         <is>
-          <t>R-15</t>
+          <t>P2-21</t>
         </is>
       </c>
       <c r="B88" s="6" t="inlineStr">
         <is>
-          <t>農曆新年前交付（生產 1/15、送達 1/29）</t>
+          <t>P2-16 ⑤ 後台 OTA 頁換成真實數據與操作</t>
         </is>
       </c>
       <c r="C88" s="6" t="inlineStr">
         <is>
-          <t>等 R-09、R-10</t>
+          <t>等 P2-18、P2-19、P2-20、P2-14</t>
         </is>
       </c>
       <c r="D88" s="11" t="n"/>
@@ -2940,17 +2948,17 @@
     <row r="89" ht="18" customHeight="1">
       <c r="A89" s="13" t="inlineStr">
         <is>
-          <t>R-33</t>
+          <t>R-09</t>
         </is>
       </c>
       <c r="B89" s="6" t="inlineStr">
         <is>
-          <t>三個 App 送審並通過</t>
+          <t>量產外殼（真空複模）</t>
         </is>
       </c>
       <c r="C89" s="6" t="inlineStr">
         <is>
-          <t>等 R-27、R-21、R-28、R-29、R-30、R-31、R-32</t>
+          <t>等 R-08、R-05、Q11</t>
         </is>
       </c>
       <c r="D89" s="11" t="n"/>
@@ -2960,20 +2968,20 @@
       <c r="H89" s="11" t="n"/>
       <c r="I89" s="12" t="n"/>
     </row>
-    <row r="90" ht="32" customHeight="1">
+    <row r="90" ht="18" customHeight="1">
       <c r="A90" s="13" t="inlineStr">
         <is>
-          <t>R-40</t>
+          <t>R-10</t>
         </is>
       </c>
       <c r="B90" s="6" t="inlineStr">
         <is>
-          <t>Admin 客服查詢頁：查帳號、名下設備與最近事件</t>
+          <t>出廠流程</t>
         </is>
       </c>
       <c r="C90" s="6" t="inlineStr">
         <is>
-          <t>等 P2-14、P1-10、P1-12</t>
+          <t>等 P0-14、R-01、P2-12、R-34、R-35、R-38、R-39</t>
         </is>
       </c>
       <c r="D90" s="11" t="n"/>
@@ -2983,27 +2991,66 @@
       <c r="H90" s="11" t="n"/>
       <c r="I90" s="12" t="n"/>
     </row>
-    <row r="92">
-      <c r="A92" s="10" t="inlineStr">
-        <is>
-          <t>❓ 待確認問題</t>
-        </is>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" s="4" t="inlineStr">
-        <is>
-          <t>編號</t>
-        </is>
-      </c>
-      <c r="B93" s="4" t="inlineStr">
-        <is>
-          <t>問題</t>
-        </is>
-      </c>
-      <c r="C93" s="4" t="inlineStr">
-        <is>
-          <t>影響的任務 / 為什麼重要</t>
+    <row r="91" ht="18" customHeight="1">
+      <c r="A91" s="13" t="inlineStr">
+        <is>
+          <t>R-11</t>
+        </is>
+      </c>
+      <c r="B91" s="6" t="inlineStr">
+        <is>
+          <t>售後：客服、保修與換機</t>
+        </is>
+      </c>
+      <c r="C91" s="6" t="inlineStr">
+        <is>
+          <t>等 P2-14、R-40</t>
+        </is>
+      </c>
+      <c r="D91" s="11" t="n"/>
+      <c r="E91" s="11" t="n"/>
+      <c r="F91" s="11" t="n"/>
+      <c r="G91" s="11" t="n"/>
+      <c r="H91" s="11" t="n"/>
+      <c r="I91" s="12" t="n"/>
+    </row>
+    <row r="92" ht="18" customHeight="1">
+      <c r="A92" s="13" t="inlineStr">
+        <is>
+          <t>R-15</t>
+        </is>
+      </c>
+      <c r="B92" s="6" t="inlineStr">
+        <is>
+          <t>農曆新年前交付（生產 1/15、送達 1/29）</t>
+        </is>
+      </c>
+      <c r="C92" s="6" t="inlineStr">
+        <is>
+          <t>等 R-09、R-10</t>
+        </is>
+      </c>
+      <c r="D92" s="11" t="n"/>
+      <c r="E92" s="11" t="n"/>
+      <c r="F92" s="11" t="n"/>
+      <c r="G92" s="11" t="n"/>
+      <c r="H92" s="11" t="n"/>
+      <c r="I92" s="12" t="n"/>
+    </row>
+    <row r="93" ht="18" customHeight="1">
+      <c r="A93" s="13" t="inlineStr">
+        <is>
+          <t>R-33</t>
+        </is>
+      </c>
+      <c r="B93" s="6" t="inlineStr">
+        <is>
+          <t>三個 App 送審並通過</t>
+        </is>
+      </c>
+      <c r="C93" s="6" t="inlineStr">
+        <is>
+          <t>等 R-27、R-21、R-28、R-29、R-30、R-31、R-32</t>
         </is>
       </c>
       <c r="D93" s="11" t="n"/>
@@ -3013,20 +3060,20 @@
       <c r="H93" s="11" t="n"/>
       <c r="I93" s="12" t="n"/>
     </row>
-    <row r="94" ht="18" customHeight="1">
+    <row r="94" ht="32" customHeight="1">
       <c r="A94" s="13" t="inlineStr">
         <is>
-          <t>Q3</t>
+          <t>R-40</t>
         </is>
       </c>
       <c r="B94" s="6" t="inlineStr">
         <is>
-          <t>韌體打算閉源商業銷售嗎？</t>
+          <t>Admin 客服查詢頁：查帳號、名下設備與最近事件</t>
         </is>
       </c>
       <c r="C94" s="6" t="inlineStr">
         <is>
-          <t>P1-06, P1-07：決定 GPL／LGPL 依賴要開源還是替換。</t>
+          <t>等 P2-14、P1-10、P1-12</t>
         </is>
       </c>
       <c r="D94" s="11" t="n"/>
@@ -3036,66 +3083,27 @@
       <c r="H94" s="11" t="n"/>
       <c r="I94" s="12" t="n"/>
     </row>
-    <row r="95" ht="32" customHeight="1">
-      <c r="A95" s="13" t="inlineStr">
-        <is>
-          <t>Q11</t>
-        </is>
-      </c>
-      <c r="B95" s="6" t="inlineStr">
-        <is>
-          <t>馬會快活的賽馬日版和新春版各多少隻（共 2,500）？</t>
-        </is>
-      </c>
-      <c r="C95" s="6" t="inlineStr">
-        <is>
-          <t>R-09, R-15：兩款的服裝和配件要分開訂料；11/20 前不知道，PP 樣和大貨單（11/27）會被拖慢。由馬會決定。</t>
-        </is>
-      </c>
-      <c r="D95" s="11" t="n"/>
-      <c r="E95" s="11" t="n"/>
-      <c r="F95" s="11" t="n"/>
-      <c r="G95" s="11" t="n"/>
-      <c r="H95" s="11" t="n"/>
-      <c r="I95" s="12" t="n"/>
-    </row>
-    <row r="96" ht="60" customHeight="1">
-      <c r="A96" s="13" t="inlineStr">
-        <is>
-          <t>Q12</t>
-        </is>
-      </c>
-      <c r="B96" s="6" t="inlineStr">
-        <is>
-          <t>快活 App 的「會員綁定」是指甚麼：用我們自己的帳號（email 驗證碼），還是接馬會的會員帳號登入（SSO）？</t>
-        </is>
-      </c>
-      <c r="C96" s="6" t="inlineStr">
-        <is>
-          <t>P0-11, 快活 App（未入追蹤表）：接馬會 SSO 的話，登入、帳號刪除和資料歸屬都要按馬會的介面重做，工作量和排期要另估，而且 W5（11/9–11/13）就要做快活 App 的綁定；用我們的帳號則和其他品牌共用同一套流程。由馬會決定，要盡早問。</t>
-        </is>
-      </c>
-      <c r="D96" s="11" t="n"/>
-      <c r="E96" s="11" t="n"/>
-      <c r="F96" s="11" t="n"/>
-      <c r="G96" s="11" t="n"/>
-      <c r="H96" s="11" t="n"/>
-      <c r="I96" s="12" t="n"/>
-    </row>
-    <row r="97" ht="46" customHeight="1">
-      <c r="A97" s="13" t="inlineStr">
-        <is>
-          <t>Q13</t>
-        </is>
-      </c>
-      <c r="B97" s="6" t="inlineStr">
-        <is>
-          <t>政協青年聯會版的角色、語言和內容由誰提供？什麼時候交？</t>
-        </is>
-      </c>
-      <c r="C97" s="6" t="inlineStr">
-        <is>
-          <t>品牌 B 的 App 頁面：品牌 B 的用戶是成人會員，但角色、說話語言、內容規則都還沒有。最遲 11/13 要拿到，才趕得及內部測試和 App 頁面（W6）。</t>
+    <row r="96">
+      <c r="A96" s="10" t="inlineStr">
+        <is>
+          <t>❓ 待確認問題</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="4" t="inlineStr">
+        <is>
+          <t>編號</t>
+        </is>
+      </c>
+      <c r="B97" s="4" t="inlineStr">
+        <is>
+          <t>問題</t>
+        </is>
+      </c>
+      <c r="C97" s="4" t="inlineStr">
+        <is>
+          <t>影響的任務 / 為什麼重要</t>
         </is>
       </c>
       <c r="D97" s="11" t="n"/>
@@ -3105,61 +3113,153 @@
       <c r="H97" s="11" t="n"/>
       <c r="I97" s="12" t="n"/>
     </row>
-    <row r="99">
-      <c r="A99" s="10" t="inlineStr">
+    <row r="98" ht="18" customHeight="1">
+      <c r="A98" s="13" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="B98" s="6" t="inlineStr">
+        <is>
+          <t>韌體打算閉源商業銷售嗎？</t>
+        </is>
+      </c>
+      <c r="C98" s="6" t="inlineStr">
+        <is>
+          <t>P1-06, P1-07：決定 GPL／LGPL 依賴要開源還是替換。</t>
+        </is>
+      </c>
+      <c r="D98" s="11" t="n"/>
+      <c r="E98" s="11" t="n"/>
+      <c r="F98" s="11" t="n"/>
+      <c r="G98" s="11" t="n"/>
+      <c r="H98" s="11" t="n"/>
+      <c r="I98" s="12" t="n"/>
+    </row>
+    <row r="99" ht="32" customHeight="1">
+      <c r="A99" s="13" t="inlineStr">
+        <is>
+          <t>Q11</t>
+        </is>
+      </c>
+      <c r="B99" s="6" t="inlineStr">
+        <is>
+          <t>馬會快活的賽馬日版和新春版各多少隻（共 2,500）？</t>
+        </is>
+      </c>
+      <c r="C99" s="6" t="inlineStr">
+        <is>
+          <t>R-09, R-15：兩款的服裝和配件要分開訂料；11/20 前不知道，PP 樣和大貨單（11/27）會被拖慢。由馬會決定。</t>
+        </is>
+      </c>
+      <c r="D99" s="11" t="n"/>
+      <c r="E99" s="11" t="n"/>
+      <c r="F99" s="11" t="n"/>
+      <c r="G99" s="11" t="n"/>
+      <c r="H99" s="11" t="n"/>
+      <c r="I99" s="12" t="n"/>
+    </row>
+    <row r="100" ht="60" customHeight="1">
+      <c r="A100" s="13" t="inlineStr">
+        <is>
+          <t>Q12</t>
+        </is>
+      </c>
+      <c r="B100" s="6" t="inlineStr">
+        <is>
+          <t>快活 App 的「會員綁定」是指甚麼：用我們自己的帳號（email 驗證碼），還是接馬會的會員帳號登入（SSO）？</t>
+        </is>
+      </c>
+      <c r="C100" s="6" t="inlineStr">
+        <is>
+          <t>P0-11, 快活 App（未入追蹤表）：接馬會 SSO 的話，登入、帳號刪除和資料歸屬都要按馬會的介面重做，工作量和排期要另估，而且 W5（11/9–11/13）就要做快活 App 的綁定；用我們的帳號則和其他品牌共用同一套流程。由馬會決定，要盡早問。</t>
+        </is>
+      </c>
+      <c r="D100" s="11" t="n"/>
+      <c r="E100" s="11" t="n"/>
+      <c r="F100" s="11" t="n"/>
+      <c r="G100" s="11" t="n"/>
+      <c r="H100" s="11" t="n"/>
+      <c r="I100" s="12" t="n"/>
+    </row>
+    <row r="101" ht="46" customHeight="1">
+      <c r="A101" s="13" t="inlineStr">
+        <is>
+          <t>Q13</t>
+        </is>
+      </c>
+      <c r="B101" s="6" t="inlineStr">
+        <is>
+          <t>政協青年聯會版的角色、語言和內容由誰提供？什麼時候交？</t>
+        </is>
+      </c>
+      <c r="C101" s="6" t="inlineStr">
+        <is>
+          <t>品牌 B 的 App 頁面：品牌 B 的用戶是成人會員，但角色、說話語言、內容規則都還沒有。最遲 11/13 要拿到，才趕得及內部測試和 App 頁面（W6）。</t>
+        </is>
+      </c>
+      <c r="D101" s="11" t="n"/>
+      <c r="E101" s="11" t="n"/>
+      <c r="F101" s="11" t="n"/>
+      <c r="G101" s="11" t="n"/>
+      <c r="H101" s="11" t="n"/>
+      <c r="I101" s="12" t="n"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="10" t="inlineStr">
         <is>
           <t>說明</t>
-        </is>
-      </c>
-    </row>
-    <row r="100" ht="32" customHeight="1">
-      <c r="A100" s="14" t="inlineStr">
-        <is>
-          <t>・狀態：未開始 → 進行中 → 已完成。只有測試真的跑過而且通過才算已完成；阻塞要在備註寫原因；不再需要的任務標不適用，不要刪。</t>
-        </is>
-      </c>
-    </row>
-    <row r="101" ht="18" customHeight="1">
-      <c r="A101" s="14" t="inlineStr">
-        <is>
-          <t>・測試結果：未測試 / 通過 / 失敗 / 部分通過。測試證據寫跑了什麼、看到什麼，完整歷史在「更新記錄」。</t>
-        </is>
-      </c>
-    </row>
-    <row r="102" ht="18" customHeight="1">
-      <c r="A102" s="14" t="inlineStr">
-        <is>
-          <t>・「接下來」按階段排序，同一階段內再按優先級；依賴還沒滿足的任務不會出現在「接下來」。</t>
-        </is>
-      </c>
-    </row>
-    <row r="103" ht="18" customHeight="1">
-      <c r="A103" s="14" t="inlineStr">
-        <is>
-          <t>・可以手動改：「任務清單」的狀態、測試結果、測試證據、Commit、備註，以及「待確認問題」的回答。其餘欄位和本頁由腳本維護。</t>
         </is>
       </c>
     </row>
     <row r="104" ht="32" customHeight="1">
       <c r="A104" s="14" t="inlineStr">
         <is>
+          <t>・狀態：未開始 → 進行中 → 已完成。只有測試真的跑過而且通過才算已完成；阻塞要在備註寫原因；不再需要的任務標不適用，不要刪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" ht="18" customHeight="1">
+      <c r="A105" s="14" t="inlineStr">
+        <is>
+          <t>・測試結果：未測試 / 通過 / 失敗 / 部分通過。測試證據寫跑了什麼、看到什麼，完整歷史在「更新記錄」。</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="18" customHeight="1">
+      <c r="A106" s="14" t="inlineStr">
+        <is>
+          <t>・「接下來」按階段排序，同一階段內再按優先級；依賴還沒滿足的任務不會出現在「接下來」。</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" ht="18" customHeight="1">
+      <c r="A107" s="14" t="inlineStr">
+        <is>
+          <t>・可以手動改：「任務清單」的狀態、測試結果、測試證據、Commit、備註，以及「待確認問題」的回答。其餘欄位和本頁由腳本維護。</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" ht="32" customHeight="1">
+      <c r="A108" s="14" t="inlineStr">
+        <is>
           <t>・建議用法：在 Claude Code 對 Claude 說「P0-02 做完了」或輸入 /prod-readiness。Claude 會先跑測試再更新，並寫進「更新記錄」。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="85">
-    <mergeCell ref="A99:I99"/>
+  <mergeCells count="89">
+    <mergeCell ref="A108:I108"/>
     <mergeCell ref="C82:I82"/>
     <mergeCell ref="E52:I52"/>
     <mergeCell ref="E39:I39"/>
     <mergeCell ref="C67:I67"/>
     <mergeCell ref="E48:I48"/>
-    <mergeCell ref="A101:I101"/>
     <mergeCell ref="A2:I2"/>
     <mergeCell ref="E29:I29"/>
     <mergeCell ref="E38:I38"/>
     <mergeCell ref="C83:I83"/>
+    <mergeCell ref="C92:I92"/>
     <mergeCell ref="E31:I31"/>
     <mergeCell ref="E40:I40"/>
     <mergeCell ref="C97:I97"/>
@@ -3167,27 +3267,27 @@
     <mergeCell ref="E26:I26"/>
     <mergeCell ref="A103:I103"/>
     <mergeCell ref="E25:I25"/>
-    <mergeCell ref="C95:I95"/>
     <mergeCell ref="C60:I60"/>
     <mergeCell ref="C71:I71"/>
     <mergeCell ref="E50:I50"/>
+    <mergeCell ref="E42:I42"/>
+    <mergeCell ref="C91:I91"/>
+    <mergeCell ref="A105:I105"/>
     <mergeCell ref="C57:I57"/>
     <mergeCell ref="C66:I66"/>
-    <mergeCell ref="E44:I44"/>
     <mergeCell ref="E20:I20"/>
     <mergeCell ref="E28:I28"/>
     <mergeCell ref="C77:I77"/>
     <mergeCell ref="C86:I86"/>
     <mergeCell ref="C68:I68"/>
-    <mergeCell ref="A100:I100"/>
     <mergeCell ref="C58:I58"/>
     <mergeCell ref="E30:I30"/>
+    <mergeCell ref="E22:I22"/>
     <mergeCell ref="E46:I46"/>
-    <mergeCell ref="A102:I102"/>
     <mergeCell ref="C85:I85"/>
+    <mergeCell ref="C100:I100"/>
     <mergeCell ref="C94:I94"/>
     <mergeCell ref="C65:I65"/>
-    <mergeCell ref="A92:I92"/>
     <mergeCell ref="C75:I75"/>
     <mergeCell ref="C84:I84"/>
     <mergeCell ref="C80:I80"/>
@@ -3201,13 +3301,16 @@
     <mergeCell ref="E24:I24"/>
     <mergeCell ref="E33:I33"/>
     <mergeCell ref="A3:I3"/>
+    <mergeCell ref="A55:I55"/>
     <mergeCell ref="A104:I104"/>
     <mergeCell ref="E35:I35"/>
-    <mergeCell ref="A43:I43"/>
+    <mergeCell ref="C101:I101"/>
+    <mergeCell ref="A106:I106"/>
+    <mergeCell ref="A96:I96"/>
     <mergeCell ref="C74:I74"/>
     <mergeCell ref="C88:I88"/>
     <mergeCell ref="E45:I45"/>
-    <mergeCell ref="C55:I55"/>
+    <mergeCell ref="C99:I99"/>
     <mergeCell ref="E37:I37"/>
     <mergeCell ref="E21:I21"/>
     <mergeCell ref="E23:I23"/>
@@ -3215,25 +3318,26 @@
     <mergeCell ref="C81:I81"/>
     <mergeCell ref="C69:I69"/>
     <mergeCell ref="E51:I51"/>
-    <mergeCell ref="C96:I96"/>
     <mergeCell ref="C78:I78"/>
     <mergeCell ref="C87:I87"/>
     <mergeCell ref="C62:I62"/>
+    <mergeCell ref="C98:I98"/>
     <mergeCell ref="C89:I89"/>
     <mergeCell ref="E34:I34"/>
     <mergeCell ref="C64:I64"/>
     <mergeCell ref="C79:I79"/>
     <mergeCell ref="C73:I73"/>
+    <mergeCell ref="A44:I44"/>
     <mergeCell ref="E49:I49"/>
     <mergeCell ref="E27:I27"/>
     <mergeCell ref="E36:I36"/>
     <mergeCell ref="C63:I63"/>
     <mergeCell ref="C93:I93"/>
+    <mergeCell ref="A107:I107"/>
     <mergeCell ref="C56:I56"/>
     <mergeCell ref="C90:I90"/>
-    <mergeCell ref="E22:I22"/>
+    <mergeCell ref="E53:I53"/>
     <mergeCell ref="C76:I76"/>
-    <mergeCell ref="A54:I54"/>
   </mergeCells>
   <conditionalFormatting sqref="I6:I10">
     <cfRule type="dataBar" priority="1">
@@ -3263,7 +3367,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P89"/>
+  <dimension ref="A1:P94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -9401,7 +9505,7 @@
       </c>
       <c r="F85" s="13" t="inlineStr">
         <is>
-          <t>未開始</t>
+          <t>進行中</t>
         </is>
       </c>
       <c r="G85" s="13" t="inlineStr">
@@ -9433,12 +9537,13 @@
       </c>
       <c r="M85" s="13" t="inlineStr">
         <is>
-          <t>P0-13, P2-14, P1-10</t>
+          <t>P0-13, P2-14, P1-10, P2-17, P2-18, P2-19, P2-20, P2-21</t>
         </is>
       </c>
       <c r="P85" s="6" t="inlineStr">
         <is>
-          <t>[2026-10-14] 新增</t>
+          <t>[2026-10-14] 新增
+[2026-10-14] 2026-10-14 開分支 p2-16-ota-rollout（worktree ../aibuddy-p216，從 dev cac98aa）；拆成 P2-17～P2-21 五項子任務，本項的測試方法即整體驗收（含 62:70 實機白名單）。</t>
         </is>
       </c>
     </row>
@@ -9727,8 +9832,343 @@
         </is>
       </c>
     </row>
+    <row r="90" ht="102" customHeight="1">
+      <c r="A90" s="13" t="inlineStr">
+        <is>
+          <t>P2-17</t>
+        </is>
+      </c>
+      <c r="B90" s="13" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C90" s="13" t="inlineStr">
+        <is>
+          <t>4 量產出貨</t>
+        </is>
+      </c>
+      <c r="D90" s="6" t="inlineStr">
+        <is>
+          <t>運維-OTA</t>
+        </is>
+      </c>
+      <c r="E90" s="6" t="inlineStr">
+        <is>
+          <t>P2-16 ① 分批推送的數據表：推送階段、白名單、每台安裝結果</t>
+        </is>
+      </c>
+      <c r="F90" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="G90" s="13" t="inlineStr">
+        <is>
+          <t>未測試</t>
+        </is>
+      </c>
+      <c r="I90" s="6" t="inlineStr">
+        <is>
+          <t>firmware_releases 只有 is_current 一個開關，沒地方記推到哪個階段、是否暫停，也沒有每台對每個版本的安裝記錄，自動暫停和後台統計都無從算起。</t>
+        </is>
+      </c>
+      <c r="J90" s="6" t="inlineStr">
+        <is>
+          <t>supabase/migrations/（新 migration）、firmware_releases、devices</t>
+        </is>
+      </c>
+      <c r="K90" s="6" t="inlineStr">
+        <is>
+          <t>firmware_releases 加推送狀態（階段：白名單／10%／50%／100%、白名單 MAC、暫停與原因、階段變更時間）；新表記錄每台對每個版本：首次下發、下發次數、確認（回報版本＝該版）、回滾（failed_version＝該版）；只有超級管理員能讀，寫入只經 service role 或帶審計的 admin RPC；舊的 is_current 發佈照常可用（視為 100%）。</t>
+        </is>
+      </c>
+      <c r="L90" s="6" t="inlineStr">
+        <is>
+          <t>本機 Supabase BEGIN/ROLLBACK 套用兩次無錯；內容管理員、anon 讀新表 → 42501；現有 release_firmware.py promote 後 1.0.1 仍照常下發（token 路徑 API 測試不變）</t>
+        </is>
+      </c>
+      <c r="M90" s="13" t="inlineStr">
+        <is>
+          <t>P0-13</t>
+        </is>
+      </c>
+      <c r="P90" s="6" t="inlineStr">
+        <is>
+          <t>[2026-10-14] 新增：2026-10-14 分支 p2-16-ota-rollout（worktree ../aibuddy-p216）</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="74" customHeight="1">
+      <c r="A91" s="13" t="inlineStr">
+        <is>
+          <t>P2-18</t>
+        </is>
+      </c>
+      <c r="B91" s="13" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C91" s="13" t="inlineStr">
+        <is>
+          <t>4 量產出貨</t>
+        </is>
+      </c>
+      <c r="D91" s="6" t="inlineStr">
+        <is>
+          <t>運維-OTA</t>
+        </is>
+      </c>
+      <c r="E91" s="6" t="inlineStr">
+        <is>
+          <t>P2-16 ② 按 MAC 雜湊穩定分組決定哪台收到 ota</t>
+        </is>
+      </c>
+      <c r="F91" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="G91" s="13" t="inlineStr">
+        <is>
+          <t>未測試</t>
+        </is>
+      </c>
+      <c r="I91" s="6" t="inlineStr">
+        <is>
+          <t>現在 current 版本一次推給同板型全部設備，3,000 台出貨後一個壞版本會同時打到所有人。</t>
+        </is>
+      </c>
+      <c r="J91" s="6" t="inlineStr">
+        <is>
+          <t>frontend-nextjs/lib/ota.ts（recordReportAndDecide）、frontend-nextjs/app/api/generate_auth_token/route.ts</t>
+        </is>
+      </c>
+      <c r="K91" s="6" t="inlineStr">
+        <is>
+          <t>白名單階段只有名單內 MAC 拿到 ota；10%／50%／100% 按 MAC 雜湊（加版本作鹽）穩定分組，同一台重複請求結果不變，升階段時已在組內的不會掉出；暫停時一律不下發；每次下發與結果寫入 ① 的記錄；不用改韌體。</t>
+        </is>
+      </c>
+      <c r="L91" s="6" t="inlineStr">
+        <is>
+          <t>單元測試：10,000 個隨機 MAC 在 10%／50% 的比例誤差 &lt; 1 個百分點，同 MAC 重複呼叫結果一致；本機腳本模擬 20 台 POST /api/generate_auth_token：10% 階段約 2 台拿到 ota，重複請求名單不變，100% 全部拿到</t>
+        </is>
+      </c>
+      <c r="M91" s="13" t="inlineStr">
+        <is>
+          <t>P2-17</t>
+        </is>
+      </c>
+      <c r="P91" s="6" t="inlineStr">
+        <is>
+          <t>[2026-10-14] 新增</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="74" customHeight="1">
+      <c r="A92" s="13" t="inlineStr">
+        <is>
+          <t>P2-19</t>
+        </is>
+      </c>
+      <c r="B92" s="13" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C92" s="13" t="inlineStr">
+        <is>
+          <t>4 量產出貨</t>
+        </is>
+      </c>
+      <c r="D92" s="6" t="inlineStr">
+        <is>
+          <t>運維-OTA</t>
+        </is>
+      </c>
+      <c r="E92" s="6" t="inlineStr">
+        <is>
+          <t>P2-16 ③ 回滾過多時自動暫停推送</t>
+        </is>
+      </c>
+      <c r="F92" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="G92" s="13" t="inlineStr">
+        <is>
+          <t>未測試</t>
+        </is>
+      </c>
+      <c r="I92" s="6" t="inlineStr">
+        <is>
+          <t>壞版本推到 10% 後沒人盯著就會繼續推；板子在試用期內斷電重啟會重試安裝（最多 2 次），伺服器要從同一台反覆下發看出問題。</t>
+        </is>
+      </c>
+      <c r="J92" s="6" t="inlineStr">
+        <is>
+          <t>frontend-nextjs/lib/ota.ts、① 的每台記錄</t>
+        </is>
+      </c>
+      <c r="K92" s="6" t="inlineStr">
+        <is>
+          <t>已下發的設備中回滾率 &gt; 5%，或任一台對同一版本被下發 3 次仍未確認，即自動暫停該版本並記下原因；暫停後其餘設備不再拿到 ota；已確認的設備不受影響；自動暫停寫入審計記錄（操作者記為系統）；只能由超級管理員在後台恢復。</t>
+        </is>
+      </c>
+      <c r="L92" s="6" t="inlineStr">
+        <is>
+          <t>本機模擬 20 台、100% 階段：讓 2 台回報 failed_version → 該版本變暫停、原因含回滾率，其餘 18 台下一次請求不再拿到 ota；另讓 1 台連續 3 次拿到 ota 不確認 → 暫停；審計表各多一筆</t>
+        </is>
+      </c>
+      <c r="M92" s="13" t="inlineStr">
+        <is>
+          <t>P2-18</t>
+        </is>
+      </c>
+      <c r="P92" s="6" t="inlineStr">
+        <is>
+          <t>[2026-10-14] 新增</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="102" customHeight="1">
+      <c r="A93" s="13" t="inlineStr">
+        <is>
+          <t>P2-20</t>
+        </is>
+      </c>
+      <c r="B93" s="13" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C93" s="13" t="inlineStr">
+        <is>
+          <t>4 量產出貨</t>
+        </is>
+      </c>
+      <c r="D93" s="6" t="inlineStr">
+        <is>
+          <t>運維-OTA</t>
+        </is>
+      </c>
+      <c r="E93" s="6" t="inlineStr">
+        <is>
+          <t>P2-16 ④ 從後台上傳與發佈韌體（取代手貼 service key）</t>
+        </is>
+      </c>
+      <c r="F93" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="G93" s="13" t="inlineStr">
+        <is>
+          <t>未測試</t>
+        </is>
+      </c>
+      <c r="I93" s="6" t="inlineStr">
+        <is>
+          <t>發佈只能在 Mac 上跑 release_firmware.py，還要在 Terminal 貼伺服器上的 service key；多品牌後每套各要一次。</t>
+        </is>
+      </c>
+      <c r="J93" s="6" t="inlineStr">
+        <is>
+          <t>frontend-nextjs/app/api/admin/（新的上傳 route）、firmware storage bucket、firmware-arduino/tools/release_firmware.py</t>
+        </is>
+      </c>
+      <c r="K93" s="6" t="inlineStr">
+        <is>
+          <t>只有超級管理員能上傳；伺服器自己算 SHA-256 與大小，檢查是 ESP32 映像、大小不超過 app 分區（P2-12）、版本號沒發佈過、不是開發版；寫入 firmware storage 和 firmware_releases（含說明），上傳後狀態為草稿，不會下發；上傳、刪除草稿都寫審計記錄；release_firmware.py 照常可用。</t>
+        </is>
+      </c>
+      <c r="L93" s="6" t="inlineStr">
+        <is>
+          <t>本機：超管上傳 spotpear-ai-toy build → firmware_releases 新行 SHA-256 與本地 shasum -a 256 一致，任何設備都還拿不到 ota；重複版本、超出分區、非 ESP32 檔、localall build 各被拒；內容管理員上傳 → 403；審計表有上傳記錄</t>
+        </is>
+      </c>
+      <c r="M93" s="13" t="inlineStr">
+        <is>
+          <t>P2-17, P1-10</t>
+        </is>
+      </c>
+      <c r="P93" s="6" t="inlineStr">
+        <is>
+          <t>[2026-10-14] 新增</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="102" customHeight="1">
+      <c r="A94" s="13" t="inlineStr">
+        <is>
+          <t>P2-21</t>
+        </is>
+      </c>
+      <c r="B94" s="13" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C94" s="13" t="inlineStr">
+        <is>
+          <t>4 量產出貨</t>
+        </is>
+      </c>
+      <c r="D94" s="6" t="inlineStr">
+        <is>
+          <t>運維-OTA</t>
+        </is>
+      </c>
+      <c r="E94" s="6" t="inlineStr">
+        <is>
+          <t>P2-16 ⑤ 後台 OTA 頁換成真實數據與操作</t>
+        </is>
+      </c>
+      <c r="F94" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="G94" s="13" t="inlineStr">
+        <is>
+          <t>未測試</t>
+        </is>
+      </c>
+      <c r="I94" s="6" t="inlineStr">
+        <is>
+          <t>OTA 頁現在是示例數據（OtaPreview），看不到哪個版本推到哪、誰回滾了。</t>
+        </is>
+      </c>
+      <c r="J94" s="6" t="inlineStr">
+        <is>
+          <t>frontend-nextjs/app/components/Admin/preview/OtaPreview.tsx → 新的 OtaTab.tsx、adminPages.ts（ota 改為 live）</t>
+        </is>
+      </c>
+      <c r="K94" s="6" t="inlineStr">
+        <is>
+          <t>按板型列出版本：狀態（草稿／推送中＋階段／暫停＋原因／現行／舊版）、已更新／目標台數、回滾台數、大小、發佈時間、說明；單一版本可編輯白名單、推進下一階段、暫停／恢復、撤下；回滾設備清單可點進設備頁；顯示 app 分區用量（P2-12）；每個操作要確認並寫審計記錄；只有超級管理員可見；375px 無橫向捲動。</t>
+        </is>
+      </c>
+      <c r="L94" s="6" t="inlineStr">
+        <is>
+          <t>本機瀏覽器：上傳 → 白名單加 62:70 → 推進 10% → 50% → 100%，每步台數和模擬 20 台的結果一致；③ 觸發暫停後頁面顯示原因並可恢復；審計頁看到每次階段變更；內容管理員看不到該頁</t>
+        </is>
+      </c>
+      <c r="M94" s="13" t="inlineStr">
+        <is>
+          <t>P2-18, P2-19, P2-20, P2-14</t>
+        </is>
+      </c>
+      <c r="P94" s="6" t="inlineStr">
+        <is>
+          <t>[2026-10-14] 新增</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P89"/>
+  <autoFilter ref="A1:P94"/>
   <conditionalFormatting sqref="F2:F1000">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"已完成"</formula>
@@ -10309,7 +10749,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I270"/>
+  <dimension ref="A1:I277"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -19661,8 +20101,209 @@
         </is>
       </c>
     </row>
+    <row r="271" ht="32" customHeight="1">
+      <c r="A271" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 20:27</t>
+        </is>
+      </c>
+      <c r="B271" s="13" t="inlineStr">
+        <is>
+          <t>P2-17</t>
+        </is>
+      </c>
+      <c r="C271" s="6" t="inlineStr">
+        <is>
+          <t>P2-16 ① 分批推送的數據表：推送階段、白名單、每台安裝結果</t>
+        </is>
+      </c>
+      <c r="E271" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="I271" s="6" t="inlineStr">
+        <is>
+          <t>新增任務</t>
+        </is>
+      </c>
+    </row>
+    <row r="272" ht="32" customHeight="1">
+      <c r="A272" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 20:27</t>
+        </is>
+      </c>
+      <c r="B272" s="13" t="inlineStr">
+        <is>
+          <t>P2-18</t>
+        </is>
+      </c>
+      <c r="C272" s="6" t="inlineStr">
+        <is>
+          <t>P2-16 ② 按 MAC 雜湊穩定分組決定哪台收到 ota</t>
+        </is>
+      </c>
+      <c r="E272" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="I272" s="6" t="inlineStr">
+        <is>
+          <t>新增任務</t>
+        </is>
+      </c>
+    </row>
+    <row r="273" ht="32" customHeight="1">
+      <c r="A273" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 20:27</t>
+        </is>
+      </c>
+      <c r="B273" s="13" t="inlineStr">
+        <is>
+          <t>P2-19</t>
+        </is>
+      </c>
+      <c r="C273" s="6" t="inlineStr">
+        <is>
+          <t>P2-16 ③ 回滾過多時自動暫停推送</t>
+        </is>
+      </c>
+      <c r="E273" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="I273" s="6" t="inlineStr">
+        <is>
+          <t>新增任務</t>
+        </is>
+      </c>
+    </row>
+    <row r="274" ht="32" customHeight="1">
+      <c r="A274" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 20:27</t>
+        </is>
+      </c>
+      <c r="B274" s="13" t="inlineStr">
+        <is>
+          <t>P2-20</t>
+        </is>
+      </c>
+      <c r="C274" s="6" t="inlineStr">
+        <is>
+          <t>P2-16 ④ 從後台上傳與發佈韌體（取代手貼 service key）</t>
+        </is>
+      </c>
+      <c r="E274" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="I274" s="6" t="inlineStr">
+        <is>
+          <t>新增任務</t>
+        </is>
+      </c>
+    </row>
+    <row r="275" ht="32" customHeight="1">
+      <c r="A275" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 20:27</t>
+        </is>
+      </c>
+      <c r="B275" s="13" t="inlineStr">
+        <is>
+          <t>P2-21</t>
+        </is>
+      </c>
+      <c r="C275" s="6" t="inlineStr">
+        <is>
+          <t>P2-16 ⑤ 後台 OTA 頁換成真實數據與操作</t>
+        </is>
+      </c>
+      <c r="E275" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="I275" s="6" t="inlineStr">
+        <is>
+          <t>新增任務</t>
+        </is>
+      </c>
+    </row>
+    <row r="276" ht="102" customHeight="1">
+      <c r="A276" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 20:27</t>
+        </is>
+      </c>
+      <c r="B276" s="13" t="inlineStr">
+        <is>
+          <t>P2-16</t>
+        </is>
+      </c>
+      <c r="C276" s="6" t="inlineStr">
+        <is>
+          <t>OTA 分批推送與後台發佈頁</t>
+        </is>
+      </c>
+      <c r="D276" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E276" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="F276" s="13" t="n"/>
+      <c r="G276" s="6" t="n"/>
+      <c r="H276" s="13" t="n"/>
+      <c r="I276" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-14 開分支 p2-16-ota-rollout（worktree ../aibuddy-p216，從 dev cac98aa）；拆成 P2-17～P2-21 五項子任務，本項的測試方法即整體驗收（含 62:70 實機白名單）。；修改了依賴→P0-13, P2-14, P1-10, P2-17, P2-18, P2-19, P2-20, P2-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="277" ht="32" customHeight="1">
+      <c r="A277" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 20:27</t>
+        </is>
+      </c>
+      <c r="B277" s="13" t="inlineStr">
+        <is>
+          <t>P2-16</t>
+        </is>
+      </c>
+      <c r="C277" s="6" t="inlineStr">
+        <is>
+          <t>OTA 分批推送與後台發佈頁</t>
+        </is>
+      </c>
+      <c r="D277" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E277" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F277" s="13" t="n"/>
+      <c r="G277" s="6" t="n"/>
+      <c r="H277" s="13" t="n"/>
+      <c r="I277" s="6" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I270"/>
+  <autoFilter ref="A1:I277"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Move P2-16 and its sub-tasks to phase 2 and start P2-17.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/production-readiness.xlsx
+++ b/docs/production-readiness.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'任務清單'!$A$1:$P$94</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'待確認問題'!$A$1:$G$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$277</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$284</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -641,7 +641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I108"/>
+  <dimension ref="A1:I109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -665,7 +665,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>最後更新：2026-10-14 20:27　·　本頁由 tracker.py 自動生成，請勿手動編輯</t>
+          <t>最後更新：2026-10-14 20:41　·　本頁由 tracker.py 自動生成，請勿手動編輯</t>
         </is>
       </c>
     </row>
@@ -820,11 +820,11 @@
       </c>
       <c r="D8" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A8,'任務清單'!$F:$F,D$5)</f>
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E8" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A8,'任務清單'!$F:$F,E$5)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F8" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A8,'任務清單'!$F:$F,F$5)</f>
@@ -896,11 +896,11 @@
       </c>
       <c r="D10" s="5">
         <f>SUM(D6:D9)</f>
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E10" s="5">
         <f>SUM(E6:E9)</f>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F10" s="5">
         <f>SUM(F6:F9)</f>
@@ -1019,15 +1019,15 @@
       </c>
       <c r="C14" s="7">
         <f>COUNTIF('任務清單'!$C:$C,$A14)</f>
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="D14" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A14,'任務清單'!$F:$F,D$12)</f>
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="E14" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A14,'任務清單'!$F:$F,E$12)</f>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F14" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A14,'任務清單'!$F:$F,F$12)</f>
@@ -1043,7 +1043,7 @@
       </c>
       <c r="I14" s="8">
         <f>IFERROR(F14/(C14-H14),0)</f>
-        <v>0.1111111111111111</v>
+        <v>0.09090909090909091</v>
       </c>
     </row>
     <row r="15" ht="46" customHeight="1">
@@ -1099,15 +1099,15 @@
       </c>
       <c r="C16" s="7">
         <f>COUNTIF('任務清單'!$C:$C,$A16)</f>
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="D16" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A16,'任務清單'!$F:$F,D$12)</f>
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="E16" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A16,'任務清單'!$F:$F,E$12)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F16" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A16,'任務清單'!$F:$F,F$12)</f>
@@ -1139,11 +1139,11 @@
       </c>
       <c r="D17" s="5">
         <f>SUM(D13:D16)</f>
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E17" s="5">
         <f>SUM(E13:E16)</f>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F17" s="5">
         <f>SUM(F13:F16)</f>
@@ -1550,15 +1550,15 @@
       <c r="H31" s="11" t="n"/>
       <c r="I31" s="12" t="n"/>
     </row>
-    <row r="32" ht="200" customHeight="1">
+    <row r="32" ht="102" customHeight="1">
       <c r="A32" s="13" t="inlineStr">
         <is>
-          <t>R-21</t>
+          <t>P2-16</t>
         </is>
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>藍牙配網與綁定（取代熱點配網）</t>
+          <t>OTA 分批推送與後台發佈頁</t>
         </is>
       </c>
       <c r="C32" s="13" t="inlineStr">
@@ -1573,7 +1573,7 @@
       </c>
       <c r="E32" s="6" t="inlineStr">
         <is>
-          <t>① 設備在「未配網、Wi-Fi 連不上、未綁定、長按 BOOT」時以 AIBuddy-XXXX 名稱廣播藍牙，廣播資料帶品牌，品牌 App 只列出自己品牌的設備。② 設備經藍牙回傳它掃描到的 2.4GHz Wi-Fi 清單，App 讓用戶選擇並填密碼。③ App 經藍牙把 SSID、密碼和綁定票（P0-11）一起交給設備；藍牙通道加密（ESP 標準配網協定 security 1/2 或同等）。④ 設備連上 Wi-Fi 後自己完成認領，App 顯示綁定成功或失敗原因（密碼錯、設備已有主人、票過期）。⑤ 配網期間不啟動音訊；完成後釋放藍牙記憶體再開語音（必要時重開機），對話中最低 heap 不比現在差。⑥ 解綁在 App 內完成（P1-12），解綁後設備進入藍牙待綁定狀態。⑦ SoftAP 熱點配網保留給開發和運維（隱藏觸發方式或編譯開關），量產用戶流程不出現。</t>
+          <t>後台可上傳韌體（伺服器算 SHA-256、寫 firmware_releases）、填說明、設為 current；推送分階段：白名單 MAC → 10% → 50% → 100%，按 MAC 雜湊穩定分組；回滾率超過 5% 或任一台在試用期內重啟 3 次即自動暫停；顯示每個版本已更新、回滾台數與回滾設備清單；顯示 app 分區用量（P2-12）；每個發佈操作寫入審計記錄。</t>
         </is>
       </c>
       <c r="F32" s="11" t="n"/>
@@ -1581,15 +1581,15 @@
       <c r="H32" s="11" t="n"/>
       <c r="I32" s="12" t="n"/>
     </row>
-    <row r="33" ht="116" customHeight="1">
+    <row r="33" ht="102" customHeight="1">
       <c r="A33" s="13" t="inlineStr">
         <is>
-          <t>R-36</t>
+          <t>P2-17</t>
         </is>
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>未認領的設備停在配對狀態，不再每秒重連 websocket</t>
+          <t>P2-16 ① 分批推送的數據表：推送階段、白名單、每台安裝結果</t>
         </is>
       </c>
       <c r="C33" s="13" t="inlineStr">
@@ -1604,7 +1604,7 @@
       </c>
       <c r="E33" s="6" t="inlineStr">
         <is>
-          <t>① 拿到 202 或 websocket 被 4401 拒絕後，設備停掉 websocket 自動重連，進入待綁定狀態（燈號可分辨）。② 待綁定時只按退避（5 秒起、上限 PROVISION_BACKOFF_MAX）呼叫 generate_auth_token，不開 websocket。③ 被認領後下一次輪詢拿到 200，在 10 秒內（加退避）自動開 websocket 並能對話，不用重開機。④ 已綁定設備網絡斷線重連的行為不變。⑤ 隨 OTA 推出。</t>
+          <t>firmware_releases 加推送狀態（階段：白名單／10%／50%／100%、白名單 MAC、暫停與原因、階段變更時間）；新表記錄每台對每個版本：首次下發、下發次數、確認（回報版本＝該版）、回滾（failed_version＝該版）；只有超級管理員能讀，寫入只經 service role 或帶審計的 admin RPC；舊的 is_current 發佈照常可用（視為 100%）。</t>
         </is>
       </c>
       <c r="F33" s="11" t="n"/>
@@ -1612,20 +1612,20 @@
       <c r="H33" s="11" t="n"/>
       <c r="I33" s="12" t="n"/>
     </row>
-    <row r="34" ht="228" customHeight="1">
+    <row r="34" ht="200" customHeight="1">
       <c r="A34" s="13" t="inlineStr">
         <is>
-          <t>P2-12</t>
+          <t>R-21</t>
         </is>
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>量產燒錄前加大 app 分區</t>
+          <t>藍牙配網與綁定（取代熱點配網）</t>
         </is>
       </c>
       <c r="C34" s="13" t="inlineStr">
         <is>
-          <t>3 封閉內測</t>
+          <t>2 內測準備</t>
         </is>
       </c>
       <c r="D34" s="13" t="inlineStr">
@@ -1635,8 +1635,7 @@
       </c>
       <c r="E34" s="6" t="inlineStr">
         <is>
-          <t>上次測試：部分通過 — 62:70（spotpear-ai-toy-p212 原型，現已併入 spotpear-ai-toy）：① 本機 OTA 1.6.1→1.6.2 寫入新 app1，120s 後 confirmed ② 3 秒 abort 的 1.6.3 → PANIC → 回到 1.6.2，ota_failed_version=1.6.3 ③ 崩潰寫入 coredump 14.8KB ④ 資源分區 9 個聲音 504KB/2MB，開機 CRC 63ms，OTA 後照常；損壞/清空 → 退回內建聲音無崩潰 ⑤ pio 全部 18 個 env 編譯通過，映像都在各自 app 槽內（Spotpear 4 個 1.59–1.60MB / 4MB；其他板仍 2MB 槽）；R-21 藍牙探針版 2,326,128 bytes &lt; 4MB ⑥ release_firmware.py 映像 &gt; app 槽即拒發。未做：雲端 OTA 一次（等上 UAT）、出廠腳本寫入資源包（R-10）
-新分區表（例如 app0/app1 各 4MB，保留 nvs/otadata 位置）在出廠前定案並寫入出廠腳本；OTA 與回滾在新分區表上照常</t>
+          <t>① 設備在「未配網、Wi-Fi 連不上、未綁定、長按 BOOT」時以 AIBuddy-XXXX 名稱廣播藍牙，廣播資料帶品牌，品牌 App 只列出自己品牌的設備。② 設備經藍牙回傳它掃描到的 2.4GHz Wi-Fi 清單，App 讓用戶選擇並填密碼。③ App 經藍牙把 SSID、密碼和綁定票（P0-11）一起交給設備；藍牙通道加密（ESP 標準配網協定 security 1/2 或同等）。④ 設備連上 Wi-Fi 後自己完成認領，App 顯示綁定成功或失敗原因（密碼錯、設備已有主人、票過期）。⑤ 配網期間不啟動音訊；完成後釋放藍牙記憶體再開語音（必要時重開機），對話中最低 heap 不比現在差。⑥ 解綁在 App 內完成（P1-12），解綁後設備進入藍牙待綁定狀態。⑦ SoftAP 熱點配網保留給開發和運維（隱藏觸發方式或編譯開關），量產用戶流程不出現。</t>
         </is>
       </c>
       <c r="F34" s="11" t="n"/>
@@ -1644,20 +1643,20 @@
       <c r="H34" s="11" t="n"/>
       <c r="I34" s="12" t="n"/>
     </row>
-    <row r="35" ht="242" customHeight="1">
+    <row r="35" ht="116" customHeight="1">
       <c r="A35" s="13" t="inlineStr">
         <is>
-          <t>R-37</t>
+          <t>R-36</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>網頁設定玩具的 Wi-Fi：查看、新增、刪除</t>
+          <t>未認領的設備停在配對狀態，不再每秒重連 websocket</t>
         </is>
       </c>
       <c r="C35" s="13" t="inlineStr">
         <is>
-          <t>3 封閉內測</t>
+          <t>2 內測準備</t>
         </is>
       </c>
       <c r="D35" s="13" t="inlineStr">
@@ -1667,8 +1666,7 @@
       </c>
       <c r="E35" s="6" t="inlineStr">
         <is>
-          <t>上次測試：部分通過 — 模擬玩具經本機語音服務器＋網頁：status/scan/add/delete 正常；刪除目前 Wi-Fi → current 被拒；斷線 5 秒內頁面顯示睡著、按鈕停用；測試密碼在語音服務器日誌、網頁服務器日誌、資料庫均搜不到；用別人裝置 ID 重放 server action → forbidden；pytest 17 項通過（全套 230）；韌體 spotpear-ai-toy-localall 編譯通過（RAM 17.5%、Flash 75.9%）。未測：真機 ①② 及 OTA 推出
-① 設定頁顯示玩具在線／離線、目前 Wi-Fi 和訊號、已記住的 Wi-Fi 清單（只有名稱，不顯示密碼）② 在線時可新增 Wi-Fi（輸入或從玩具掃描到的清單選）、刪除 Wi-Fi；不能刪除正在使用的那個 ③ 經 /ws/esp32 轉送：伺服器先確認是設備主人；密碼不寫入資料庫、不寫入日誌 ④ 新增不切換網絡，目前 Wi-Fi 消失時才按訊號選；清單標示「連過／未連過」⑤ 上限 8 個 ⑥ 韌體改動經 OTA 推出</t>
+          <t>① 拿到 202 或 websocket 被 4401 拒絕後，設備停掉 websocket 自動重連，進入待綁定狀態（燈號可分辨）。② 待綁定時只按退避（5 秒起、上限 PROVISION_BACKOFF_MAX）呼叫 generate_auth_token，不開 websocket。③ 被認領後下一次輪詢拿到 200，在 10 秒內（加退避）自動開 websocket 並能對話，不用重開機。④ 已綁定設備網絡斷線重連的行為不變。⑤ 隨 OTA 推出。</t>
         </is>
       </c>
       <c r="F35" s="11" t="n"/>
@@ -1676,20 +1674,20 @@
       <c r="H35" s="11" t="n"/>
       <c r="I35" s="12" t="n"/>
     </row>
-    <row r="36" ht="102" customHeight="1">
+    <row r="36" ht="228" customHeight="1">
       <c r="A36" s="13" t="inlineStr">
         <is>
-          <t>P2-16</t>
+          <t>P2-12</t>
         </is>
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>OTA 分批推送與後台發佈頁</t>
+          <t>量產燒錄前加大 app 分區</t>
         </is>
       </c>
       <c r="C36" s="13" t="inlineStr">
         <is>
-          <t>4 量產出貨</t>
+          <t>3 封閉內測</t>
         </is>
       </c>
       <c r="D36" s="13" t="inlineStr">
@@ -1699,7 +1697,8 @@
       </c>
       <c r="E36" s="6" t="inlineStr">
         <is>
-          <t>後台可上傳韌體（伺服器算 SHA-256、寫 firmware_releases）、填說明、設為 current；推送分階段：白名單 MAC → 10% → 50% → 100%，按 MAC 雜湊穩定分組；回滾率超過 5% 或任一台在試用期內重啟 3 次即自動暫停；顯示每個版本已更新、回滾台數與回滾設備清單；顯示 app 分區用量（P2-12）；每個發佈操作寫入審計記錄。</t>
+          <t>上次測試：部分通過 — 62:70（spotpear-ai-toy-p212 原型，現已併入 spotpear-ai-toy）：① 本機 OTA 1.6.1→1.6.2 寫入新 app1，120s 後 confirmed ② 3 秒 abort 的 1.6.3 → PANIC → 回到 1.6.2，ota_failed_version=1.6.3 ③ 崩潰寫入 coredump 14.8KB ④ 資源分區 9 個聲音 504KB/2MB，開機 CRC 63ms，OTA 後照常；損壞/清空 → 退回內建聲音無崩潰 ⑤ pio 全部 18 個 env 編譯通過，映像都在各自 app 槽內（Spotpear 4 個 1.59–1.60MB / 4MB；其他板仍 2MB 槽）；R-21 藍牙探針版 2,326,128 bytes &lt; 4MB ⑥ release_firmware.py 映像 &gt; app 槽即拒發。未做：雲端 OTA 一次（等上 UAT）、出廠腳本寫入資源包（R-10）
+新分區表（例如 app0/app1 各 4MB，保留 nvs/otadata 位置）在出廠前定案並寫入出廠腳本；OTA 與回滾在新分區表上照常</t>
         </is>
       </c>
       <c r="F36" s="11" t="n"/>
@@ -1707,30 +1706,31 @@
       <c r="H36" s="11" t="n"/>
       <c r="I36" s="12" t="n"/>
     </row>
-    <row r="37" ht="102" customHeight="1">
+    <row r="37" ht="242" customHeight="1">
       <c r="A37" s="13" t="inlineStr">
         <is>
-          <t>R-16</t>
+          <t>R-37</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>Spotpear 量產版加電池電壓檢測（GPIO0 分壓）</t>
+          <t>網頁設定玩具的 Wi-Fi：查看、新增、刪除</t>
         </is>
       </c>
       <c r="C37" s="13" t="inlineStr">
         <is>
-          <t>1 止血定案</t>
+          <t>3 封閉內測</t>
         </is>
       </c>
       <c r="D37" s="13" t="inlineStr">
         <is>
-          <t>未開始</t>
+          <t>進行中</t>
         </is>
       </c>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>Spotpear 書面確認量產版：GPIO1（屏幕 DC；本版不接屏幕，可空出來）接電芯正極（保護 IC 之後）100k/100k 分壓、100nF 濾波，屏幕不接該腳；GPIO0 保留給現有的 VDD 低電提醒；最好另把充電芯片 CHRG 接到 GPIO12 或 13。樣板到手後，固件讀到的電芯電壓與萬用表相差 ≤50mV，App（R-41）顯示百分比與充電中。</t>
+          <t>上次測試：部分通過 — 模擬玩具經本機語音服務器＋網頁：status/scan/add/delete 正常；刪除目前 Wi-Fi → current 被拒；斷線 5 秒內頁面顯示睡著、按鈕停用；測試密碼在語音服務器日誌、網頁服務器日誌、資料庫均搜不到；用別人裝置 ID 重放 server action → forbidden；pytest 17 項通過（全套 230）；韌體 spotpear-ai-toy-localall 編譯通過（RAM 17.5%、Flash 75.9%）。未測：真機 ①② 及 OTA 推出
+① 設定頁顯示玩具在線／離線、目前 Wi-Fi 和訊號、已記住的 Wi-Fi 清單（只有名稱，不顯示密碼）② 在線時可新增 Wi-Fi（輸入或從玩具掃描到的清單選）、刪除 Wi-Fi；不能刪除正在使用的那個 ③ 經 /ws/esp32 轉送：伺服器先確認是設備主人；密碼不寫入資料庫、不寫入日誌 ④ 新增不切換網絡，目前 Wi-Fi 消失時才按訊號選；清單標示「連過／未連過」⑤ 上限 8 個 ⑥ 韌體改動經 OTA 推出</t>
         </is>
       </c>
       <c r="F37" s="11" t="n"/>
@@ -1738,20 +1738,20 @@
       <c r="H37" s="11" t="n"/>
       <c r="I37" s="12" t="n"/>
     </row>
-    <row r="38" ht="46" customHeight="1">
+    <row r="38" ht="102" customHeight="1">
       <c r="A38" s="13" t="inlineStr">
         <is>
-          <t>P1-11</t>
+          <t>R-16</t>
         </is>
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>伺服器與資料庫直接存取的管控</t>
+          <t>Spotpear 量產版加電池電壓檢測（GPIO0 分壓）</t>
         </is>
       </c>
       <c r="C38" s="13" t="inlineStr">
         <is>
-          <t>2 內測準備</t>
+          <t>1 止血定案</t>
         </is>
       </c>
       <c r="D38" s="13" t="inlineStr">
@@ -1761,7 +1761,7 @@
       </c>
       <c r="E38" s="6" t="inlineStr">
         <is>
-          <t>列出誰有 SSH 與資料庫直連權限（越少越好）；service_role key 只存在伺服器的 env；私隱政策寫明這類存取的範圍；每次直接查看生產資料都留記錄。</t>
+          <t>Spotpear 書面確認量產版：GPIO1（屏幕 DC；本版不接屏幕，可空出來）接電芯正極（保護 IC 之後）100k/100k 分壓、100nF 濾波，屏幕不接該腳；GPIO0 保留給現有的 VDD 低電提醒；最好另把充電芯片 CHRG 接到 GPIO12 或 13。樣板到手後，固件讀到的電芯電壓與萬用表相差 ≤50mV，App（R-41）顯示百分比與充電中。</t>
         </is>
       </c>
       <c r="F38" s="11" t="n"/>
@@ -1772,12 +1772,12 @@
     <row r="39" ht="46" customHeight="1">
       <c r="A39" s="13" t="inlineStr">
         <is>
-          <t>P2-02</t>
+          <t>P1-11</t>
         </is>
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>CI 跑測試與靜態檢查</t>
+          <t>伺服器與資料庫直接存取的管控</t>
         </is>
       </c>
       <c r="C39" s="13" t="inlineStr">
@@ -1792,7 +1792,7 @@
       </c>
       <c r="E39" s="6" t="inlineStr">
         <is>
-          <t>推送與 PR 時跑 pytest、ruff、pyright、next lint、tsc --noEmit、pio run；任何一項失敗就不發佈 image。</t>
+          <t>列出誰有 SSH 與資料庫直連權限（越少越好）；service_role key 只存在伺服器的 env；私隱政策寫明這類存取的範圍；每次直接查看生產資料都留記錄。</t>
         </is>
       </c>
       <c r="F39" s="11" t="n"/>
@@ -1800,15 +1800,15 @@
       <c r="H39" s="11" t="n"/>
       <c r="I39" s="12" t="n"/>
     </row>
-    <row r="40" ht="32" customHeight="1">
+    <row r="40" ht="46" customHeight="1">
       <c r="A40" s="13" t="inlineStr">
         <is>
-          <t>P2-04</t>
+          <t>P2-02</t>
         </is>
       </c>
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>容器改用非 root 用戶</t>
+          <t>CI 跑測試與靜態檢查</t>
         </is>
       </c>
       <c r="C40" s="13" t="inlineStr">
@@ -1823,7 +1823,7 @@
       </c>
       <c r="E40" s="6" t="inlineStr">
         <is>
-          <t>兩個 Dockerfile 都設定非 root 的 USER。</t>
+          <t>推送與 PR 時跑 pytest、ruff、pyright、next lint、tsc --noEmit、pio run；任何一項失敗就不發佈 image。</t>
         </is>
       </c>
       <c r="F40" s="11" t="n"/>
@@ -1831,15 +1831,15 @@
       <c r="H40" s="11" t="n"/>
       <c r="I40" s="12" t="n"/>
     </row>
-    <row r="41" ht="46" customHeight="1">
+    <row r="41" ht="32" customHeight="1">
       <c r="A41" s="13" t="inlineStr">
         <is>
-          <t>R-04</t>
+          <t>P2-04</t>
         </is>
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>粵語質量評測</t>
+          <t>容器改用非 root 用戶</t>
         </is>
       </c>
       <c r="C41" s="13" t="inlineStr">
@@ -1854,7 +1854,7 @@
       </c>
       <c r="E41" s="6" t="inlineStr">
         <is>
-          <t>有一套粵語評測集（兒童錄音＋文字提示）；選定的 STT 與 LLM 達到門檻：兒童語音字錯率 ≤15%、口語粵語回覆 ≥90%、中英夾雜句能正確理解。</t>
+          <t>兩個 Dockerfile 都設定非 root 的 USER。</t>
         </is>
       </c>
       <c r="F41" s="11" t="n"/>
@@ -1862,15 +1862,15 @@
       <c r="H41" s="11" t="n"/>
       <c r="I41" s="12" t="n"/>
     </row>
-    <row r="42" ht="116" customHeight="1">
+    <row r="42" ht="46" customHeight="1">
       <c r="A42" s="13" t="inlineStr">
         <is>
-          <t>R-25</t>
+          <t>R-04</t>
         </is>
       </c>
       <c r="B42" s="6" t="inlineStr">
         <is>
-          <t>網頁的品牌主題系統</t>
+          <t>粵語質量評測</t>
         </is>
       </c>
       <c r="C42" s="13" t="inlineStr">
@@ -1885,7 +1885,7 @@
       </c>
       <c r="E42" s="6" t="inlineStr">
         <is>
-          <t>① 每個品牌一個資料夾：主題 token（顏色、字體、圓角）、logo 和圖示、文案、功能開關；首頁、上手流程、角色頁可以有品牌版本，其餘頁面共用 ② 由部署的環境變數選品牌（每套部署一個品牌，見 R-34），伺服器端渲染的第一屏就是對的主題，不閃爍 ③ 共用元件裡沒有品牌名稱和寫死的品牌顏色 ④ 加一個品牌只需要加資料夾、設定和一套部署，不用改共用元件</t>
+          <t>有一套粵語評測集（兒童錄音＋文字提示）；選定的 STT 與 LLM 達到門檻：兒童語音字錯率 ≤15%、口語粵語回覆 ≥90%、中英夾雜句能正確理解。</t>
         </is>
       </c>
       <c r="F42" s="11" t="n"/>
@@ -1893,68 +1893,68 @@
       <c r="H42" s="11" t="n"/>
       <c r="I42" s="12" t="n"/>
     </row>
-    <row r="44">
-      <c r="A44" s="10" t="inlineStr">
+    <row r="43" ht="116" customHeight="1">
+      <c r="A43" s="13" t="inlineStr">
+        <is>
+          <t>R-25</t>
+        </is>
+      </c>
+      <c r="B43" s="6" t="inlineStr">
+        <is>
+          <t>網頁的品牌主題系統</t>
+        </is>
+      </c>
+      <c r="C43" s="13" t="inlineStr">
+        <is>
+          <t>2 內測準備</t>
+        </is>
+      </c>
+      <c r="D43" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E43" s="6" t="inlineStr">
+        <is>
+          <t>① 每個品牌一個資料夾：主題 token（顏色、字體、圓角）、logo 和圖示、文案、功能開關；首頁、上手流程、角色頁可以有品牌版本，其餘頁面共用 ② 由部署的環境變數選品牌（每套部署一個品牌，見 R-34），伺服器端渲染的第一屏就是對的主題，不閃爍 ③ 共用元件裡沒有品牌名稱和寫死的品牌顏色 ④ 加一個品牌只需要加資料夾、設定和一套部署，不用改共用元件</t>
+        </is>
+      </c>
+      <c r="F43" s="11" t="n"/>
+      <c r="G43" s="11" t="n"/>
+      <c r="H43" s="11" t="n"/>
+      <c r="I43" s="12" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="10" t="inlineStr">
         <is>
           <t>✅ 最近完成與測試效果</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="4" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
         <is>
           <t>編號</t>
         </is>
       </c>
-      <c r="B45" s="4" t="inlineStr">
+      <c r="B46" s="4" t="inlineStr">
         <is>
           <t>任務</t>
         </is>
       </c>
-      <c r="C45" s="4" t="inlineStr">
+      <c r="C46" s="4" t="inlineStr">
         <is>
           <t>測試結果</t>
         </is>
       </c>
-      <c r="D45" s="4" t="inlineStr">
+      <c r="D46" s="4" t="inlineStr">
         <is>
           <t>完成日期</t>
         </is>
       </c>
-      <c r="E45" s="4" t="inlineStr">
+      <c r="E46" s="4" t="inlineStr">
         <is>
           <t>測試證據</t>
-        </is>
-      </c>
-      <c r="F45" s="11" t="n"/>
-      <c r="G45" s="11" t="n"/>
-      <c r="H45" s="11" t="n"/>
-      <c r="I45" s="12" t="n"/>
-    </row>
-    <row r="46" ht="116" customHeight="1">
-      <c r="A46" s="13" t="inlineStr">
-        <is>
-          <t>R-41</t>
-        </is>
-      </c>
-      <c r="B46" s="6" t="inlineStr">
-        <is>
-          <t>App 顯示玩具電量狀態（低電量提示）</t>
-        </is>
-      </c>
-      <c r="C46" s="13" t="inlineStr">
-        <is>
-          <t>通過</t>
-        </is>
-      </c>
-      <c r="D46" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="E46" s="6" t="inlineStr">
-        <is>
-          <t>① pytest 33 passed；真 PATCH 本地 Supabase ② 62:70 刷 p212+R-41 強制低電 build（SUPPLY_LOW_RATIO_OVERRIDE=1.05）→ 串口 [WSc] power low:true，本地 DB battery_low=t ③ 刷回正常 1.6.2 → low:false，DB=f ④ App 讀 DB：低電紅標+Please charge+更新時間、72% 充電中、未上報不顯示 ⑤ 他人帳號 0 行、authenticated UPDATE 被拒。62:70 已還原為原 p212 build</t>
         </is>
       </c>
       <c r="F46" s="11" t="n"/>
@@ -1962,15 +1962,15 @@
       <c r="H46" s="11" t="n"/>
       <c r="I46" s="12" t="n"/>
     </row>
-    <row r="47" ht="102" customHeight="1">
+    <row r="47" ht="116" customHeight="1">
       <c r="A47" s="13" t="inlineStr">
         <is>
-          <t>P0-12</t>
+          <t>R-41</t>
         </is>
       </c>
       <c r="B47" s="6" t="inlineStr">
         <is>
-          <t>收緊 Admin 權限與路由保護</t>
+          <t>App 顯示玩具電量狀態（低電量提示）</t>
         </is>
       </c>
       <c r="C47" s="13" t="inlineStr">
@@ -1980,12 +1980,12 @@
       </c>
       <c r="D47" s="13" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E47" s="6" t="inlineStr">
         <is>
-          <t>線上 2026-10-12（bac24e9）：runbook 10/08 檢查 未登入 /admin→/login、/api/admin→401、has_role() 只看角色、無管理員 policy 觸及 conversations/記憶表、超管≥1；未登入 /home、/admin→/login；用戶確認：家長帳號開 /admin 轉回 /home、管理員在 /admin 修改角色保存成功；角色細分權限沿用本機 61/61</t>
+          <t>① pytest 33 passed；真 PATCH 本地 Supabase ② 62:70 刷 p212+R-41 強制低電 build（SUPPLY_LOW_RATIO_OVERRIDE=1.05）→ 串口 [WSc] power low:true，本地 DB battery_low=t ③ 刷回正常 1.6.2 → low:false，DB=f ④ App 讀 DB：低電紅標+Please charge+更新時間、72% 充電中、未上報不顯示 ⑤ 他人帳號 0 行、authenticated UPDATE 被拒。62:70 已還原為原 p212 build</t>
         </is>
       </c>
       <c r="F47" s="11" t="n"/>
@@ -1993,15 +1993,15 @@
       <c r="H47" s="11" t="n"/>
       <c r="I47" s="12" t="n"/>
     </row>
-    <row r="48" ht="88" customHeight="1">
+    <row r="48" ht="102" customHeight="1">
       <c r="A48" s="13" t="inlineStr">
         <is>
-          <t>P0-15</t>
+          <t>P0-12</t>
         </is>
       </c>
       <c r="B48" s="6" t="inlineStr">
         <is>
-          <t>角色表權限：只有內容管理員能發佈，關閉家長自建角色</t>
+          <t>收緊 Admin 權限與路由保護</t>
         </is>
       </c>
       <c r="C48" s="13" t="inlineStr">
@@ -2016,7 +2016,7 @@
       </c>
       <c r="E48" s="6" t="inlineStr">
         <is>
-          <t>線上 2026-10-12：② anon 只見 6 個已發佈 hk_ 內建，查隱藏/醫生/家長自建 → []，anon POST → 401；① authenticated 寫入權限由 20261007140000 REVOKE（runbook 10/08 已套用）；用戶確認：④ 家長登入後 /home/create 轉回 /home ③ 管理員在 /admin 修改角色保存成功</t>
+          <t>線上 2026-10-12（bac24e9）：runbook 10/08 檢查 未登入 /admin→/login、/api/admin→401、has_role() 只看角色、無管理員 policy 觸及 conversations/記憶表、超管≥1；未登入 /home、/admin→/login；用戶確認：家長帳號開 /admin 轉回 /home、管理員在 /admin 修改角色保存成功；角色細分權限沿用本機 61/61</t>
         </is>
       </c>
       <c r="F48" s="11" t="n"/>
@@ -2027,12 +2027,12 @@
     <row r="49" ht="88" customHeight="1">
       <c r="A49" s="13" t="inlineStr">
         <is>
-          <t>P0-16</t>
+          <t>P0-15</t>
         </is>
       </c>
       <c r="B49" s="6" t="inlineStr">
         <is>
-          <t>移除「醫生」身份與寫死的通關碼</t>
+          <t>角色表權限：只有內容管理員能發佈，關閉家長自建角色</t>
         </is>
       </c>
       <c r="C49" s="13" t="inlineStr">
@@ -2047,7 +2047,7 @@
       </c>
       <c r="E49" s="6" t="inlineStr">
         <is>
-          <t>線上 2026-10-12：生產 commit bac24e9 git grep checkDoctorAction/kiwi-subtle-emu/=== "doctor"/isDoctor → 0；線上 13 個 JS（/、/login、/onboard）grep 通關碼/"doctor"/Santa/patient → 0；anon 讀角色只見 6 個 hk_ 角色、is_doctor 全 false；用戶今日線上登入及 playground 正常</t>
+          <t>線上 2026-10-12：② anon 只見 6 個已發佈 hk_ 內建，查隱藏/醫生/家長自建 → []，anon POST → 401；① authenticated 寫入權限由 20261007140000 REVOKE（runbook 10/08 已套用）；用戶確認：④ 家長登入後 /home/create 轉回 /home ③ 管理員在 /admin 修改角色保存成功</t>
         </is>
       </c>
       <c r="F49" s="11" t="n"/>
@@ -2055,15 +2055,15 @@
       <c r="H49" s="11" t="n"/>
       <c r="I49" s="12" t="n"/>
     </row>
-    <row r="50" ht="60" customHeight="1">
+    <row r="50" ht="88" customHeight="1">
       <c r="A50" s="13" t="inlineStr">
         <is>
-          <t>P0-09</t>
+          <t>P0-16</t>
         </is>
       </c>
       <c r="B50" s="6" t="inlineStr">
         <is>
-          <t>瀏覽器語音路由改用簽名 token（/ws/nextjs）</t>
+          <t>移除「醫生」身份與寫死的通關碼</t>
         </is>
       </c>
       <c r="C50" s="13" t="inlineStr">
@@ -2078,7 +2078,7 @@
       </c>
       <c r="E50" s="6" t="inlineStr">
         <is>
-          <t>線上 2026-10-12（bac24e9）：wss /fastapi/ws/nextjs 只帶 user_id 或 token=bogus → 4401；用戶確認：登入 elatoai.hkqft.com 後網頁 playground 可正常對話</t>
+          <t>線上 2026-10-12：生產 commit bac24e9 git grep checkDoctorAction/kiwi-subtle-emu/=== "doctor"/isDoctor → 0；線上 13 個 JS（/、/login、/onboard）grep 通關碼/"doctor"/Santa/patient → 0；anon 讀角色只見 6 個 hk_ 角色、is_doctor 全 false；用戶今日線上登入及 playground 正常</t>
         </is>
       </c>
       <c r="F50" s="11" t="n"/>
@@ -2089,12 +2089,12 @@
     <row r="51" ht="60" customHeight="1">
       <c r="A51" s="13" t="inlineStr">
         <is>
-          <t>P0-17</t>
+          <t>P0-09</t>
         </is>
       </c>
       <c r="B51" s="6" t="inlineStr">
         <is>
-          <t>前端的 anon key 必須是公開 key，不可是 secret／service_role</t>
+          <t>瀏覽器語音路由改用簽名 token（/ws/nextjs）</t>
         </is>
       </c>
       <c r="C51" s="13" t="inlineStr">
@@ -2109,7 +2109,7 @@
       </c>
       <c r="E51" s="6" t="inlineStr">
         <is>
-          <t>線上 2026-10-12（bac24e9）：/login 引用的 13 個 JS + HTML 無 sb_secret_，唯一 key 為 role=anon 的 JWT；② 用該 key GET /rest/v1/users → 42501；③ 本機 10/07 已換 publishable</t>
+          <t>線上 2026-10-12（bac24e9）：wss /fastapi/ws/nextjs 只帶 user_id 或 token=bogus → 4401；用戶確認：登入 elatoai.hkqft.com 後網頁 playground 可正常對話</t>
         </is>
       </c>
       <c r="F51" s="11" t="n"/>
@@ -2117,15 +2117,15 @@
       <c r="H51" s="11" t="n"/>
       <c r="I51" s="12" t="n"/>
     </row>
-    <row r="52" ht="46" customHeight="1">
+    <row r="52" ht="60" customHeight="1">
       <c r="A52" s="13" t="inlineStr">
         <is>
-          <t>P0-10</t>
+          <t>P0-17</t>
         </is>
       </c>
       <c r="B52" s="6" t="inlineStr">
         <is>
-          <t>生產環境關閉 /browser 測試頁與 /ws/browser</t>
+          <t>前端的 anon key 必須是公開 key，不可是 secret／service_role</t>
         </is>
       </c>
       <c r="C52" s="13" t="inlineStr">
@@ -2140,7 +2140,7 @@
       </c>
       <c r="E52" s="6" t="inlineStr">
         <is>
-          <t>線上 2026-10-12（bac24e9）：GET /fastapi/browser 404、/fastapi/ 404、/fastapi/healthz 200、wss /fastapi/ws/browser → HTTP 403</t>
+          <t>線上 2026-10-12（bac24e9）：/login 引用的 13 個 JS + HTML 無 sb_secret_，唯一 key 為 role=anon 的 JWT；② 用該 key GET /rest/v1/users → 42501；③ 本機 10/07 已換 publishable</t>
         </is>
       </c>
       <c r="F52" s="11" t="n"/>
@@ -2148,15 +2148,15 @@
       <c r="H52" s="11" t="n"/>
       <c r="I52" s="12" t="n"/>
     </row>
-    <row r="53" ht="60" customHeight="1">
+    <row r="53" ht="46" customHeight="1">
       <c r="A53" s="13" t="inlineStr">
         <is>
-          <t>P0-08</t>
+          <t>P0-10</t>
         </is>
       </c>
       <c r="B53" s="6" t="inlineStr">
         <is>
-          <t>語音伺服器驗證設備身份（/ws/esp32）</t>
+          <t>生產環境關閉 /browser 測試頁與 /ws/browser</t>
         </is>
       </c>
       <c r="C53" s="13" t="inlineStr">
@@ -2171,7 +2171,7 @@
       </c>
       <c r="E53" s="6" t="inlineStr">
         <is>
-          <t>線上 2026-10-12（bac24e9）：wss /fastapi/ws/esp32 不帶 token、偽造 token＋X-Device-Mac → 均 4401 invalid device token；42:34 以有效 token 連線對話正常（P0-13 10/09）</t>
+          <t>線上 2026-10-12（bac24e9）：GET /fastapi/browser 404、/fastapi/ 404、/fastapi/healthz 200、wss /fastapi/ws/browser → HTTP 403</t>
         </is>
       </c>
       <c r="F53" s="11" t="n"/>
@@ -2179,50 +2179,58 @@
       <c r="H53" s="11" t="n"/>
       <c r="I53" s="12" t="n"/>
     </row>
-    <row r="55">
-      <c r="A55" s="10" t="inlineStr">
+    <row r="54" ht="60" customHeight="1">
+      <c r="A54" s="13" t="inlineStr">
+        <is>
+          <t>P0-08</t>
+        </is>
+      </c>
+      <c r="B54" s="6" t="inlineStr">
+        <is>
+          <t>語音伺服器驗證設備身份（/ws/esp32）</t>
+        </is>
+      </c>
+      <c r="C54" s="13" t="inlineStr">
+        <is>
+          <t>通過</t>
+        </is>
+      </c>
+      <c r="D54" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="E54" s="6" t="inlineStr">
+        <is>
+          <t>線上 2026-10-12（bac24e9）：wss /fastapi/ws/esp32 不帶 token、偽造 token＋X-Device-Mac → 均 4401 invalid device token；42:34 以有效 token 連線對話正常（P0-13 10/09）</t>
+        </is>
+      </c>
+      <c r="F54" s="11" t="n"/>
+      <c r="G54" s="11" t="n"/>
+      <c r="H54" s="11" t="n"/>
+      <c r="I54" s="12" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="10" t="inlineStr">
         <is>
           <t>⏳ 等待依賴 / ⛔ 阻塞</t>
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="4" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
         <is>
           <t>編號</t>
         </is>
       </c>
-      <c r="B56" s="4" t="inlineStr">
+      <c r="B57" s="4" t="inlineStr">
         <is>
           <t>任務</t>
         </is>
       </c>
-      <c r="C56" s="4" t="inlineStr">
+      <c r="C57" s="4" t="inlineStr">
         <is>
           <t>在等什麼</t>
-        </is>
-      </c>
-      <c r="D56" s="11" t="n"/>
-      <c r="E56" s="11" t="n"/>
-      <c r="F56" s="11" t="n"/>
-      <c r="G56" s="11" t="n"/>
-      <c r="H56" s="11" t="n"/>
-      <c r="I56" s="12" t="n"/>
-    </row>
-    <row r="57" ht="88" customHeight="1">
-      <c r="A57" s="13" t="inlineStr">
-        <is>
-          <t>R-17</t>
-        </is>
-      </c>
-      <c r="B57" s="6" t="inlineStr">
-        <is>
-          <t>Spotpear 電池耗盡時插電能否正常開機（供電路徑）</t>
-        </is>
-      </c>
-      <c r="C57" s="6" t="inlineStr">
-        <is>
-          <t>阻塞：[2026-10-08] 2026-10-08 開發板 63:64 插著 USB 時兩次無法解釋的完全斷電重開：09:13:26（崩潰循環中）、10:44:33（閒置、用戶確認沒碰）。都是 USB 先斷線再以 ESP_RST_POWERON 開機，非 brownout；斷電前 6 秒 GPIO0 讀數 99.9% 參考值，屬突然切斷而非緩降（SupplyMonitor 取樣太疏抓不到瞬間）。韌體無法造成 POWERON，指向充電芯片/電池保護/供電路徑，應一併問 Spotpear；放電實測時留意插 USB 閒置時是否也會斷電</t>
         </is>
       </c>
       <c r="D57" s="11" t="n"/>
@@ -2232,20 +2240,20 @@
       <c r="H57" s="11" t="n"/>
       <c r="I57" s="12" t="n"/>
     </row>
-    <row r="58" ht="60" customHeight="1">
+    <row r="58" ht="88" customHeight="1">
       <c r="A58" s="13" t="inlineStr">
         <is>
-          <t>P1-01</t>
+          <t>R-17</t>
         </is>
       </c>
       <c r="B58" s="6" t="inlineStr">
         <is>
-          <t>加入內容審核層（輸入與輸出）</t>
+          <t>Spotpear 電池耗盡時插電能否正常開機（供電路徑）</t>
         </is>
       </c>
       <c r="C58" s="6" t="inlineStr">
         <is>
-          <t>阻塞：[2026-10-14] 2026-10-14 用戶決定：先不定審核服務商，本項暫停。候選：Azure Content Safety（建議，香港區、可在每句回覆說出口前檢查）、OpenRouter 安全模型、OpenAI Moderation、只用本機字詞表。未寫任何程式。</t>
+          <t>阻塞：[2026-10-08] 2026-10-08 開發板 63:64 插著 USB 時兩次無法解釋的完全斷電重開：09:13:26（崩潰循環中）、10:44:33（閒置、用戶確認沒碰）。都是 USB 先斷線再以 ESP_RST_POWERON 開機，非 brownout；斷電前 6 秒 GPIO0 讀數 99.9% 參考值，屬突然切斷而非緩降（SupplyMonitor 取樣太疏抓不到瞬間）。韌體無法造成 POWERON，指向充電芯片/電池保護/供電路徑，應一併問 Spotpear；放電實測時留意插 USB 閒置時是否也會斷電</t>
         </is>
       </c>
       <c r="D58" s="11" t="n"/>
@@ -2255,20 +2263,20 @@
       <c r="H58" s="11" t="n"/>
       <c r="I58" s="12" t="n"/>
     </row>
-    <row r="59" ht="32" customHeight="1">
+    <row r="59" ht="60" customHeight="1">
       <c r="A59" s="13" t="inlineStr">
         <is>
-          <t>P1-09</t>
+          <t>P1-01</t>
         </is>
       </c>
       <c r="B59" s="6" t="inlineStr">
         <is>
-          <t>家長鎖：孩子模式進設定要輸入 PIN</t>
+          <t>加入內容審核層（輸入與輸出）</t>
         </is>
       </c>
       <c r="C59" s="6" t="inlineStr">
         <is>
-          <t>阻塞：[2026-10-13] 2026-10-13 用戶決定：AI Buddy（品牌 C）延到 1/15 之後，本項不卡 1/15 出廠；AI Buddy 啟動時再開。</t>
+          <t>阻塞：[2026-10-14] 2026-10-14 用戶決定：先不定審核服務商，本項暫停。候選：Azure Content Safety（建議，香港區、可在每句回覆說出口前檢查）、OpenRouter 安全模型、OpenAI Moderation、只用本機字詞表。未寫任何程式。</t>
         </is>
       </c>
       <c r="D59" s="11" t="n"/>
@@ -2281,12 +2289,12 @@
     <row r="60" ht="32" customHeight="1">
       <c r="A60" s="13" t="inlineStr">
         <is>
-          <t>R-12</t>
+          <t>P1-09</t>
         </is>
       </c>
       <c r="B60" s="6" t="inlineStr">
         <is>
-          <t>家長控制：每日使用上限和休息時段</t>
+          <t>家長鎖：孩子模式進設定要輸入 PIN</t>
         </is>
       </c>
       <c r="C60" s="6" t="inlineStr">
@@ -2304,12 +2312,12 @@
     <row r="61" ht="32" customHeight="1">
       <c r="A61" s="13" t="inlineStr">
         <is>
-          <t>R-29</t>
+          <t>R-12</t>
         </is>
       </c>
       <c r="B61" s="6" t="inlineStr">
         <is>
-          <t>AI Buddy App（品牌 C）頁面</t>
+          <t>家長控制：每日使用上限和休息時段</t>
         </is>
       </c>
       <c r="C61" s="6" t="inlineStr">
@@ -2324,20 +2332,20 @@
       <c r="H61" s="11" t="n"/>
       <c r="I61" s="12" t="n"/>
     </row>
-    <row r="62" ht="18" customHeight="1">
+    <row r="62" ht="32" customHeight="1">
       <c r="A62" s="13" t="inlineStr">
         <is>
-          <t>R-05</t>
+          <t>R-29</t>
         </is>
       </c>
       <c r="B62" s="6" t="inlineStr">
         <is>
-          <t>內測版外殼（3D 打印 20 台）</t>
+          <t>AI Buddy App（品牌 C）頁面</t>
         </is>
       </c>
       <c r="C62" s="6" t="inlineStr">
         <is>
-          <t>等 R-01</t>
+          <t>阻塞：[2026-10-13] 2026-10-13 用戶決定：AI Buddy（品牌 C）延到 1/15 之後，本項不卡 1/15 出廠；AI Buddy 啟動時再開。</t>
         </is>
       </c>
       <c r="D62" s="11" t="n"/>
@@ -2347,20 +2355,20 @@
       <c r="H62" s="11" t="n"/>
       <c r="I62" s="12" t="n"/>
     </row>
-    <row r="63" ht="18" customHeight="1">
+    <row r="63" ht="32" customHeight="1">
       <c r="A63" s="13" t="inlineStr">
         <is>
-          <t>R-06</t>
+          <t>P2-18</t>
         </is>
       </c>
       <c r="B63" s="6" t="inlineStr">
         <is>
-          <t>家長自助上手流程</t>
+          <t>P2-16 ② 按 MAC 雜湊穩定分組決定哪台收到 ota</t>
         </is>
       </c>
       <c r="C63" s="6" t="inlineStr">
         <is>
-          <t>等 P0-11</t>
+          <t>等 P2-17</t>
         </is>
       </c>
       <c r="D63" s="11" t="n"/>
@@ -2370,20 +2378,20 @@
       <c r="H63" s="11" t="n"/>
       <c r="I63" s="12" t="n"/>
     </row>
-    <row r="64" ht="32" customHeight="1">
+    <row r="64" ht="18" customHeight="1">
       <c r="A64" s="13" t="inlineStr">
         <is>
-          <t>R-13</t>
+          <t>P2-19</t>
         </is>
       </c>
       <c r="B64" s="6" t="inlineStr">
         <is>
-          <t>CP1 內測就緒檢查（10/30）</t>
+          <t>P2-16 ③ 回滾過多時自動暫停推送</t>
         </is>
       </c>
       <c r="C64" s="6" t="inlineStr">
         <is>
-          <t>等 P0-07、P0-11、P1-01、P1-02、P2-09、R-01、R-02、R-04、R-05、R-06、P1-11</t>
+          <t>等 P2-18</t>
         </is>
       </c>
       <c r="D64" s="11" t="n"/>
@@ -2396,17 +2404,17 @@
     <row r="65" ht="32" customHeight="1">
       <c r="A65" s="13" t="inlineStr">
         <is>
-          <t>R-18</t>
+          <t>P2-20</t>
         </is>
       </c>
       <c r="B65" s="6" t="inlineStr">
         <is>
-          <t>長按 BOOT 重新配網（開 AIBuddy-XXXX 熱點）</t>
+          <t>P2-16 ④ 從後台上傳與發佈韌體（取代手貼 service key）</t>
         </is>
       </c>
       <c r="C65" s="6" t="inlineStr">
         <is>
-          <t>等 R-01</t>
+          <t>等 P2-17、P1-10</t>
         </is>
       </c>
       <c r="D65" s="11" t="n"/>
@@ -2416,20 +2424,20 @@
       <c r="H65" s="11" t="n"/>
       <c r="I65" s="12" t="n"/>
     </row>
-    <row r="66" ht="32" customHeight="1">
+    <row r="66" ht="18" customHeight="1">
       <c r="A66" s="13" t="inlineStr">
         <is>
-          <t>R-19</t>
+          <t>P2-21</t>
         </is>
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
-          <t>外接按鈕：量產板加 I2C 擴展晶片（TCA9555）</t>
+          <t>P2-16 ⑤ 後台 OTA 頁換成真實數據與操作</t>
         </is>
       </c>
       <c r="C66" s="6" t="inlineStr">
         <is>
-          <t>等 R-01</t>
+          <t>等 P2-18、P2-19、P2-20、P2-14</t>
         </is>
       </c>
       <c r="D66" s="11" t="n"/>
@@ -2442,17 +2450,17 @@
     <row r="67" ht="18" customHeight="1">
       <c r="A67" s="13" t="inlineStr">
         <is>
-          <t>R-20</t>
+          <t>R-05</t>
         </is>
       </c>
       <c r="B67" s="6" t="inlineStr">
         <is>
-          <t>孩子資料與角色改成每台設備一份</t>
+          <t>內測版外殼（3D 打印 20 台）</t>
         </is>
       </c>
       <c r="C67" s="6" t="inlineStr">
         <is>
-          <t>等 P1-12</t>
+          <t>等 R-01</t>
         </is>
       </c>
       <c r="D67" s="11" t="n"/>
@@ -2462,20 +2470,20 @@
       <c r="H67" s="11" t="n"/>
       <c r="I67" s="12" t="n"/>
     </row>
-    <row r="68" ht="32" customHeight="1">
+    <row r="68" ht="18" customHeight="1">
       <c r="A68" s="13" t="inlineStr">
         <is>
-          <t>R-27</t>
+          <t>R-06</t>
         </is>
       </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t>App 內登入：驗證碼、原生社交登入、刪除帳號</t>
+          <t>家長自助上手流程</t>
         </is>
       </c>
       <c r="C68" s="6" t="inlineStr">
         <is>
-          <t>等 R-26</t>
+          <t>等 P0-11</t>
         </is>
       </c>
       <c r="D68" s="11" t="n"/>
@@ -2485,20 +2493,20 @@
       <c r="H68" s="11" t="n"/>
       <c r="I68" s="12" t="n"/>
     </row>
-    <row r="69" ht="18" customHeight="1">
+    <row r="69" ht="32" customHeight="1">
       <c r="A69" s="13" t="inlineStr">
         <is>
-          <t>P0-14</t>
+          <t>R-13</t>
         </is>
       </c>
       <c r="B69" s="6" t="inlineStr">
         <is>
-          <t>韌體簽章、Secure Boot 與 Flash 加密</t>
+          <t>CP1 內測就緒檢查（10/30）</t>
         </is>
       </c>
       <c r="C69" s="6" t="inlineStr">
         <is>
-          <t>等 R-01</t>
+          <t>等 P0-07、P0-11、P1-01、P1-02、P2-09、R-01、R-02、R-04、R-05、R-06、P1-11</t>
         </is>
       </c>
       <c r="D69" s="11" t="n"/>
@@ -2508,20 +2516,20 @@
       <c r="H69" s="11" t="n"/>
       <c r="I69" s="12" t="n"/>
     </row>
-    <row r="70" ht="18" customHeight="1">
+    <row r="70" ht="32" customHeight="1">
       <c r="A70" s="13" t="inlineStr">
         <is>
-          <t>P1-06</t>
+          <t>R-18</t>
         </is>
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>處理 GPL-3.0 依賴（arduino-audio-tools）</t>
+          <t>長按 BOOT 重新配網（開 AIBuddy-XXXX 熱點）</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr">
         <is>
-          <t>等 Q3</t>
+          <t>等 R-01</t>
         </is>
       </c>
       <c r="D70" s="11" t="n"/>
@@ -2531,20 +2539,20 @@
       <c r="H70" s="11" t="n"/>
       <c r="I70" s="12" t="n"/>
     </row>
-    <row r="71" ht="18" customHeight="1">
+    <row r="71" ht="32" customHeight="1">
       <c r="A71" s="13" t="inlineStr">
         <is>
-          <t>P1-07</t>
+          <t>R-19</t>
         </is>
       </c>
       <c r="B71" s="6" t="inlineStr">
         <is>
-          <t>LGPL 合規與第三方授權聲明</t>
+          <t>外接按鈕：量產板加 I2C 擴展晶片（TCA9555）</t>
         </is>
       </c>
       <c r="C71" s="6" t="inlineStr">
         <is>
-          <t>等 Q3</t>
+          <t>等 R-01</t>
         </is>
       </c>
       <c r="D71" s="11" t="n"/>
@@ -2557,17 +2565,17 @@
     <row r="72" ht="18" customHeight="1">
       <c r="A72" s="13" t="inlineStr">
         <is>
-          <t>P1-08</t>
+          <t>R-20</t>
         </is>
       </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>硬件認證</t>
+          <t>孩子資料與角色改成每台設備一份</t>
         </is>
       </c>
       <c r="C72" s="6" t="inlineStr">
         <is>
-          <t>等 R-01、R-05</t>
+          <t>等 P1-12</t>
         </is>
       </c>
       <c r="D72" s="11" t="n"/>
@@ -2577,20 +2585,20 @@
       <c r="H72" s="11" t="n"/>
       <c r="I72" s="12" t="n"/>
     </row>
-    <row r="73" ht="18" customHeight="1">
+    <row r="73" ht="32" customHeight="1">
       <c r="A73" s="13" t="inlineStr">
         <is>
-          <t>P1-14</t>
+          <t>R-27</t>
         </is>
       </c>
       <c r="B73" s="6" t="inlineStr">
         <is>
-          <t>Admin 內容安全頁：審核事件只按類別統計</t>
+          <t>App 內登入：驗證碼、原生社交登入、刪除帳號</t>
         </is>
       </c>
       <c r="C73" s="6" t="inlineStr">
         <is>
-          <t>等 P1-01、P2-13</t>
+          <t>等 R-26</t>
         </is>
       </c>
       <c r="D73" s="11" t="n"/>
@@ -2600,20 +2608,20 @@
       <c r="H73" s="11" t="n"/>
       <c r="I73" s="12" t="n"/>
     </row>
-    <row r="74" ht="32" customHeight="1">
+    <row r="74" ht="18" customHeight="1">
       <c r="A74" s="13" t="inlineStr">
         <is>
-          <t>P2-15</t>
+          <t>P0-14</t>
         </is>
       </c>
       <c r="B74" s="6" t="inlineStr">
         <is>
-          <t>Admin 總覽頁：在線、用量、成本與待處理事項</t>
+          <t>韌體簽章、Secure Boot 與 Flash 加密</t>
         </is>
       </c>
       <c r="C74" s="6" t="inlineStr">
         <is>
-          <t>等 P2-14、P2-09</t>
+          <t>等 R-01</t>
         </is>
       </c>
       <c r="D74" s="11" t="n"/>
@@ -2626,17 +2634,17 @@
     <row r="75" ht="18" customHeight="1">
       <c r="A75" s="13" t="inlineStr">
         <is>
-          <t>R-07</t>
+          <t>P1-06</t>
         </is>
       </c>
       <c r="B75" s="6" t="inlineStr">
         <is>
-          <t>20 個家庭封閉內測</t>
+          <t>處理 GPL-3.0 依賴（arduino-audio-tools）</t>
         </is>
       </c>
       <c r="C75" s="6" t="inlineStr">
         <is>
-          <t>等 R-13</t>
+          <t>等 Q3</t>
         </is>
       </c>
       <c r="D75" s="11" t="n"/>
@@ -2649,17 +2657,17 @@
     <row r="76" ht="18" customHeight="1">
       <c r="A76" s="13" t="inlineStr">
         <is>
-          <t>R-08</t>
+          <t>P1-07</t>
         </is>
       </c>
       <c r="B76" s="6" t="inlineStr">
         <is>
-          <t>第 8 週關卡決策</t>
+          <t>LGPL 合規與第三方授權聲明</t>
         </is>
       </c>
       <c r="C76" s="6" t="inlineStr">
         <is>
-          <t>等 R-07、P2-09、P1-08</t>
+          <t>等 Q3</t>
         </is>
       </c>
       <c r="D76" s="11" t="n"/>
@@ -2672,17 +2680,17 @@
     <row r="77" ht="18" customHeight="1">
       <c r="A77" s="13" t="inlineStr">
         <is>
-          <t>R-14</t>
+          <t>P1-08</t>
         </is>
       </c>
       <c r="B77" s="6" t="inlineStr">
         <is>
-          <t>離線兒歌與故事</t>
+          <t>硬件認證</t>
         </is>
       </c>
       <c r="C77" s="6" t="inlineStr">
         <is>
-          <t>等 R-01</t>
+          <t>等 R-01、R-05</t>
         </is>
       </c>
       <c r="D77" s="11" t="n"/>
@@ -2695,17 +2703,17 @@
     <row r="78" ht="18" customHeight="1">
       <c r="A78" s="13" t="inlineStr">
         <is>
-          <t>R-24</t>
+          <t>P1-14</t>
         </is>
       </c>
       <c r="B78" s="6" t="inlineStr">
         <is>
-          <t>設備只能用自己品牌的角色</t>
+          <t>Admin 內容安全頁：審核事件只按類別統計</t>
         </is>
       </c>
       <c r="C78" s="6" t="inlineStr">
         <is>
-          <t>等 R-34</t>
+          <t>等 P1-01、P2-13</t>
         </is>
       </c>
       <c r="D78" s="11" t="n"/>
@@ -2715,20 +2723,20 @@
       <c r="H78" s="11" t="n"/>
       <c r="I78" s="12" t="n"/>
     </row>
-    <row r="79" ht="18" customHeight="1">
+    <row r="79" ht="32" customHeight="1">
       <c r="A79" s="13" t="inlineStr">
         <is>
-          <t>R-28</t>
+          <t>P2-15</t>
         </is>
       </c>
       <c r="B79" s="6" t="inlineStr">
         <is>
-          <t>三個 App 的殼：品牌版本與測試版</t>
+          <t>Admin 總覽頁：在線、用量、成本與待處理事項</t>
         </is>
       </c>
       <c r="C79" s="6" t="inlineStr">
         <is>
-          <t>等 R-25、R-26</t>
+          <t>等 P2-14、P2-09</t>
         </is>
       </c>
       <c r="D79" s="11" t="n"/>
@@ -2741,17 +2749,17 @@
     <row r="80" ht="18" customHeight="1">
       <c r="A80" s="13" t="inlineStr">
         <is>
-          <t>R-30</t>
+          <t>R-07</t>
         </is>
       </c>
       <c r="B80" s="6" t="inlineStr">
         <is>
-          <t>快活 App（品牌 A）頁面</t>
+          <t>20 個家庭封閉內測</t>
         </is>
       </c>
       <c r="C80" s="6" t="inlineStr">
         <is>
-          <t>等 R-25、R-34、Q12</t>
+          <t>等 R-13</t>
         </is>
       </c>
       <c r="D80" s="11" t="n"/>
@@ -2764,17 +2772,17 @@
     <row r="81" ht="18" customHeight="1">
       <c r="A81" s="13" t="inlineStr">
         <is>
-          <t>R-31</t>
+          <t>R-08</t>
         </is>
       </c>
       <c r="B81" s="6" t="inlineStr">
         <is>
-          <t>政協青年聯會版 App（品牌 B）頁面</t>
+          <t>第 8 週關卡決策</t>
         </is>
       </c>
       <c r="C81" s="6" t="inlineStr">
         <is>
-          <t>等 R-25、R-34、Q13</t>
+          <t>等 R-07、P2-09、P1-08</t>
         </is>
       </c>
       <c r="D81" s="11" t="n"/>
@@ -2787,17 +2795,17 @@
     <row r="82" ht="18" customHeight="1">
       <c r="A82" s="13" t="inlineStr">
         <is>
-          <t>R-35</t>
+          <t>R-14</t>
         </is>
       </c>
       <c r="B82" s="6" t="inlineStr">
         <is>
-          <t>韌體按品牌連線：伺服器網址在出廠時寫入</t>
+          <t>離線兒歌與故事</t>
         </is>
       </c>
       <c r="C82" s="6" t="inlineStr">
         <is>
-          <t>等 R-34</t>
+          <t>等 R-01</t>
         </is>
       </c>
       <c r="D82" s="11" t="n"/>
@@ -2807,20 +2815,20 @@
       <c r="H82" s="11" t="n"/>
       <c r="I82" s="12" t="n"/>
     </row>
-    <row r="83" ht="32" customHeight="1">
+    <row r="83" ht="18" customHeight="1">
       <c r="A83" s="13" t="inlineStr">
         <is>
-          <t>R-38</t>
+          <t>R-24</t>
         </is>
       </c>
       <c r="B83" s="6" t="inlineStr">
         <is>
-          <t>公仔出廠鎖死所屬 IP，綁定時顯示該 IP 頭像</t>
+          <t>設備只能用自己品牌的角色</t>
         </is>
       </c>
       <c r="C83" s="6" t="inlineStr">
         <is>
-          <t>等 P0-11</t>
+          <t>等 R-34</t>
         </is>
       </c>
       <c r="D83" s="11" t="n"/>
@@ -2830,20 +2838,20 @@
       <c r="H83" s="11" t="n"/>
       <c r="I83" s="12" t="n"/>
     </row>
-    <row r="84" ht="32" customHeight="1">
+    <row r="84" ht="18" customHeight="1">
       <c r="A84" s="13" t="inlineStr">
         <is>
-          <t>R-39</t>
+          <t>R-28</t>
         </is>
       </c>
       <c r="B84" s="6" t="inlineStr">
         <is>
-          <t>Admin 出廠登記頁：匯入 MAC 清單、指定公仔、查看自檢結果</t>
+          <t>三個 App 的殼：品牌版本與測試版</t>
         </is>
       </c>
       <c r="C84" s="6" t="inlineStr">
         <is>
-          <t>等 R-38、P1-10</t>
+          <t>等 R-25、R-26</t>
         </is>
       </c>
       <c r="D84" s="11" t="n"/>
@@ -2853,20 +2861,20 @@
       <c r="H84" s="11" t="n"/>
       <c r="I84" s="12" t="n"/>
     </row>
-    <row r="85" ht="32" customHeight="1">
+    <row r="85" ht="18" customHeight="1">
       <c r="A85" s="13" t="inlineStr">
         <is>
-          <t>P2-18</t>
+          <t>R-30</t>
         </is>
       </c>
       <c r="B85" s="6" t="inlineStr">
         <is>
-          <t>P2-16 ② 按 MAC 雜湊穩定分組決定哪台收到 ota</t>
+          <t>快活 App（品牌 A）頁面</t>
         </is>
       </c>
       <c r="C85" s="6" t="inlineStr">
         <is>
-          <t>等 P2-17</t>
+          <t>等 R-25、R-34、Q12</t>
         </is>
       </c>
       <c r="D85" s="11" t="n"/>
@@ -2879,17 +2887,17 @@
     <row r="86" ht="18" customHeight="1">
       <c r="A86" s="13" t="inlineStr">
         <is>
-          <t>P2-19</t>
+          <t>R-31</t>
         </is>
       </c>
       <c r="B86" s="6" t="inlineStr">
         <is>
-          <t>P2-16 ③ 回滾過多時自動暫停推送</t>
+          <t>政協青年聯會版 App（品牌 B）頁面</t>
         </is>
       </c>
       <c r="C86" s="6" t="inlineStr">
         <is>
-          <t>等 P2-18</t>
+          <t>等 R-25、R-34、Q13</t>
         </is>
       </c>
       <c r="D86" s="11" t="n"/>
@@ -2899,20 +2907,20 @@
       <c r="H86" s="11" t="n"/>
       <c r="I86" s="12" t="n"/>
     </row>
-    <row r="87" ht="32" customHeight="1">
+    <row r="87" ht="18" customHeight="1">
       <c r="A87" s="13" t="inlineStr">
         <is>
-          <t>P2-20</t>
+          <t>R-35</t>
         </is>
       </c>
       <c r="B87" s="6" t="inlineStr">
         <is>
-          <t>P2-16 ④ 從後台上傳與發佈韌體（取代手貼 service key）</t>
+          <t>韌體按品牌連線：伺服器網址在出廠時寫入</t>
         </is>
       </c>
       <c r="C87" s="6" t="inlineStr">
         <is>
-          <t>等 P2-17、P1-10</t>
+          <t>等 R-34</t>
         </is>
       </c>
       <c r="D87" s="11" t="n"/>
@@ -2922,20 +2930,20 @@
       <c r="H87" s="11" t="n"/>
       <c r="I87" s="12" t="n"/>
     </row>
-    <row r="88" ht="18" customHeight="1">
+    <row r="88" ht="32" customHeight="1">
       <c r="A88" s="13" t="inlineStr">
         <is>
-          <t>P2-21</t>
+          <t>R-38</t>
         </is>
       </c>
       <c r="B88" s="6" t="inlineStr">
         <is>
-          <t>P2-16 ⑤ 後台 OTA 頁換成真實數據與操作</t>
+          <t>公仔出廠鎖死所屬 IP，綁定時顯示該 IP 頭像</t>
         </is>
       </c>
       <c r="C88" s="6" t="inlineStr">
         <is>
-          <t>等 P2-18、P2-19、P2-20、P2-14</t>
+          <t>等 P0-11</t>
         </is>
       </c>
       <c r="D88" s="11" t="n"/>
@@ -2945,20 +2953,20 @@
       <c r="H88" s="11" t="n"/>
       <c r="I88" s="12" t="n"/>
     </row>
-    <row r="89" ht="18" customHeight="1">
+    <row r="89" ht="32" customHeight="1">
       <c r="A89" s="13" t="inlineStr">
         <is>
-          <t>R-09</t>
+          <t>R-39</t>
         </is>
       </c>
       <c r="B89" s="6" t="inlineStr">
         <is>
-          <t>量產外殼（真空複模）</t>
+          <t>Admin 出廠登記頁：匯入 MAC 清單、指定公仔、查看自檢結果</t>
         </is>
       </c>
       <c r="C89" s="6" t="inlineStr">
         <is>
-          <t>等 R-08、R-05、Q11</t>
+          <t>等 R-38、P1-10</t>
         </is>
       </c>
       <c r="D89" s="11" t="n"/>
@@ -2971,17 +2979,17 @@
     <row r="90" ht="18" customHeight="1">
       <c r="A90" s="13" t="inlineStr">
         <is>
-          <t>R-10</t>
+          <t>R-09</t>
         </is>
       </c>
       <c r="B90" s="6" t="inlineStr">
         <is>
-          <t>出廠流程</t>
+          <t>量產外殼（真空複模）</t>
         </is>
       </c>
       <c r="C90" s="6" t="inlineStr">
         <is>
-          <t>等 P0-14、R-01、P2-12、R-34、R-35、R-38、R-39</t>
+          <t>等 R-08、R-05、Q11</t>
         </is>
       </c>
       <c r="D90" s="11" t="n"/>
@@ -2994,17 +3002,17 @@
     <row r="91" ht="18" customHeight="1">
       <c r="A91" s="13" t="inlineStr">
         <is>
-          <t>R-11</t>
+          <t>R-10</t>
         </is>
       </c>
       <c r="B91" s="6" t="inlineStr">
         <is>
-          <t>售後：客服、保修與換機</t>
+          <t>出廠流程</t>
         </is>
       </c>
       <c r="C91" s="6" t="inlineStr">
         <is>
-          <t>等 P2-14、R-40</t>
+          <t>等 P0-14、R-01、P2-12、R-34、R-35、R-38、R-39</t>
         </is>
       </c>
       <c r="D91" s="11" t="n"/>
@@ -3017,17 +3025,17 @@
     <row r="92" ht="18" customHeight="1">
       <c r="A92" s="13" t="inlineStr">
         <is>
-          <t>R-15</t>
+          <t>R-11</t>
         </is>
       </c>
       <c r="B92" s="6" t="inlineStr">
         <is>
-          <t>農曆新年前交付（生產 1/15、送達 1/29）</t>
+          <t>售後：客服、保修與換機</t>
         </is>
       </c>
       <c r="C92" s="6" t="inlineStr">
         <is>
-          <t>等 R-09、R-10</t>
+          <t>等 P2-14、R-40</t>
         </is>
       </c>
       <c r="D92" s="11" t="n"/>
@@ -3040,17 +3048,17 @@
     <row r="93" ht="18" customHeight="1">
       <c r="A93" s="13" t="inlineStr">
         <is>
-          <t>R-33</t>
+          <t>R-15</t>
         </is>
       </c>
       <c r="B93" s="6" t="inlineStr">
         <is>
-          <t>三個 App 送審並通過</t>
+          <t>農曆新年前交付（生產 1/15、送達 1/29）</t>
         </is>
       </c>
       <c r="C93" s="6" t="inlineStr">
         <is>
-          <t>等 R-27、R-21、R-28、R-29、R-30、R-31、R-32</t>
+          <t>等 R-09、R-10</t>
         </is>
       </c>
       <c r="D93" s="11" t="n"/>
@@ -3060,20 +3068,20 @@
       <c r="H93" s="11" t="n"/>
       <c r="I93" s="12" t="n"/>
     </row>
-    <row r="94" ht="32" customHeight="1">
+    <row r="94" ht="18" customHeight="1">
       <c r="A94" s="13" t="inlineStr">
         <is>
-          <t>R-40</t>
+          <t>R-33</t>
         </is>
       </c>
       <c r="B94" s="6" t="inlineStr">
         <is>
-          <t>Admin 客服查詢頁：查帳號、名下設備與最近事件</t>
+          <t>三個 App 送審並通過</t>
         </is>
       </c>
       <c r="C94" s="6" t="inlineStr">
         <is>
-          <t>等 P2-14、P1-10、P1-12</t>
+          <t>等 R-27、R-21、R-28、R-29、R-30、R-31、R-32</t>
         </is>
       </c>
       <c r="D94" s="11" t="n"/>
@@ -3083,50 +3091,50 @@
       <c r="H94" s="11" t="n"/>
       <c r="I94" s="12" t="n"/>
     </row>
-    <row r="96">
-      <c r="A96" s="10" t="inlineStr">
+    <row r="95" ht="32" customHeight="1">
+      <c r="A95" s="13" t="inlineStr">
+        <is>
+          <t>R-40</t>
+        </is>
+      </c>
+      <c r="B95" s="6" t="inlineStr">
+        <is>
+          <t>Admin 客服查詢頁：查帳號、名下設備與最近事件</t>
+        </is>
+      </c>
+      <c r="C95" s="6" t="inlineStr">
+        <is>
+          <t>等 P2-14、P1-10、P1-12</t>
+        </is>
+      </c>
+      <c r="D95" s="11" t="n"/>
+      <c r="E95" s="11" t="n"/>
+      <c r="F95" s="11" t="n"/>
+      <c r="G95" s="11" t="n"/>
+      <c r="H95" s="11" t="n"/>
+      <c r="I95" s="12" t="n"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="10" t="inlineStr">
         <is>
           <t>❓ 待確認問題</t>
         </is>
       </c>
     </row>
-    <row r="97">
-      <c r="A97" s="4" t="inlineStr">
+    <row r="98">
+      <c r="A98" s="4" t="inlineStr">
         <is>
           <t>編號</t>
         </is>
       </c>
-      <c r="B97" s="4" t="inlineStr">
+      <c r="B98" s="4" t="inlineStr">
         <is>
           <t>問題</t>
         </is>
       </c>
-      <c r="C97" s="4" t="inlineStr">
+      <c r="C98" s="4" t="inlineStr">
         <is>
           <t>影響的任務 / 為什麼重要</t>
-        </is>
-      </c>
-      <c r="D97" s="11" t="n"/>
-      <c r="E97" s="11" t="n"/>
-      <c r="F97" s="11" t="n"/>
-      <c r="G97" s="11" t="n"/>
-      <c r="H97" s="11" t="n"/>
-      <c r="I97" s="12" t="n"/>
-    </row>
-    <row r="98" ht="18" customHeight="1">
-      <c r="A98" s="13" t="inlineStr">
-        <is>
-          <t>Q3</t>
-        </is>
-      </c>
-      <c r="B98" s="6" t="inlineStr">
-        <is>
-          <t>韌體打算閉源商業銷售嗎？</t>
-        </is>
-      </c>
-      <c r="C98" s="6" t="inlineStr">
-        <is>
-          <t>P1-06, P1-07：決定 GPL／LGPL 依賴要開源還是替換。</t>
         </is>
       </c>
       <c r="D98" s="11" t="n"/>
@@ -3136,20 +3144,20 @@
       <c r="H98" s="11" t="n"/>
       <c r="I98" s="12" t="n"/>
     </row>
-    <row r="99" ht="32" customHeight="1">
+    <row r="99" ht="18" customHeight="1">
       <c r="A99" s="13" t="inlineStr">
         <is>
-          <t>Q11</t>
+          <t>Q3</t>
         </is>
       </c>
       <c r="B99" s="6" t="inlineStr">
         <is>
-          <t>馬會快活的賽馬日版和新春版各多少隻（共 2,500）？</t>
+          <t>韌體打算閉源商業銷售嗎？</t>
         </is>
       </c>
       <c r="C99" s="6" t="inlineStr">
         <is>
-          <t>R-09, R-15：兩款的服裝和配件要分開訂料；11/20 前不知道，PP 樣和大貨單（11/27）會被拖慢。由馬會決定。</t>
+          <t>P1-06, P1-07：決定 GPL／LGPL 依賴要開源還是替換。</t>
         </is>
       </c>
       <c r="D99" s="11" t="n"/>
@@ -3159,20 +3167,20 @@
       <c r="H99" s="11" t="n"/>
       <c r="I99" s="12" t="n"/>
     </row>
-    <row r="100" ht="60" customHeight="1">
+    <row r="100" ht="32" customHeight="1">
       <c r="A100" s="13" t="inlineStr">
         <is>
-          <t>Q12</t>
+          <t>Q11</t>
         </is>
       </c>
       <c r="B100" s="6" t="inlineStr">
         <is>
-          <t>快活 App 的「會員綁定」是指甚麼：用我們自己的帳號（email 驗證碼），還是接馬會的會員帳號登入（SSO）？</t>
+          <t>馬會快活的賽馬日版和新春版各多少隻（共 2,500）？</t>
         </is>
       </c>
       <c r="C100" s="6" t="inlineStr">
         <is>
-          <t>P0-11, 快活 App（未入追蹤表）：接馬會 SSO 的話，登入、帳號刪除和資料歸屬都要按馬會的介面重做，工作量和排期要另估，而且 W5（11/9–11/13）就要做快活 App 的綁定；用我們的帳號則和其他品牌共用同一套流程。由馬會決定，要盡早問。</t>
+          <t>R-09, R-15：兩款的服裝和配件要分開訂料；11/20 前不知道，PP 樣和大貨單（11/27）會被拖慢。由馬會決定。</t>
         </is>
       </c>
       <c r="D100" s="11" t="n"/>
@@ -3182,20 +3190,20 @@
       <c r="H100" s="11" t="n"/>
       <c r="I100" s="12" t="n"/>
     </row>
-    <row r="101" ht="46" customHeight="1">
+    <row r="101" ht="60" customHeight="1">
       <c r="A101" s="13" t="inlineStr">
         <is>
-          <t>Q13</t>
+          <t>Q12</t>
         </is>
       </c>
       <c r="B101" s="6" t="inlineStr">
         <is>
-          <t>政協青年聯會版的角色、語言和內容由誰提供？什麼時候交？</t>
+          <t>快活 App 的「會員綁定」是指甚麼：用我們自己的帳號（email 驗證碼），還是接馬會的會員帳號登入（SSO）？</t>
         </is>
       </c>
       <c r="C101" s="6" t="inlineStr">
         <is>
-          <t>品牌 B 的 App 頁面：品牌 B 的用戶是成人會員，但角色、說話語言、內容規則都還沒有。最遲 11/13 要拿到，才趕得及內部測試和 App 頁面（W6）。</t>
+          <t>P0-11, 快活 App（未入追蹤表）：接馬會 SSO 的話，登入、帳號刪除和資料歸屬都要按馬會的介面重做，工作量和排期要另估，而且 W5（11/9–11/13）就要做快活 App 的綁定；用我們的帳號則和其他品牌共用同一套流程。由馬會決定，要盡早問。</t>
         </is>
       </c>
       <c r="D101" s="11" t="n"/>
@@ -3205,53 +3213,77 @@
       <c r="H101" s="11" t="n"/>
       <c r="I101" s="12" t="n"/>
     </row>
-    <row r="103">
-      <c r="A103" s="10" t="inlineStr">
+    <row r="102" ht="46" customHeight="1">
+      <c r="A102" s="13" t="inlineStr">
+        <is>
+          <t>Q13</t>
+        </is>
+      </c>
+      <c r="B102" s="6" t="inlineStr">
+        <is>
+          <t>政協青年聯會版的角色、語言和內容由誰提供？什麼時候交？</t>
+        </is>
+      </c>
+      <c r="C102" s="6" t="inlineStr">
+        <is>
+          <t>品牌 B 的 App 頁面：品牌 B 的用戶是成人會員，但角色、說話語言、內容規則都還沒有。最遲 11/13 要拿到，才趕得及內部測試和 App 頁面（W6）。</t>
+        </is>
+      </c>
+      <c r="D102" s="11" t="n"/>
+      <c r="E102" s="11" t="n"/>
+      <c r="F102" s="11" t="n"/>
+      <c r="G102" s="11" t="n"/>
+      <c r="H102" s="11" t="n"/>
+      <c r="I102" s="12" t="n"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="10" t="inlineStr">
         <is>
           <t>說明</t>
         </is>
       </c>
     </row>
-    <row r="104" ht="32" customHeight="1">
-      <c r="A104" s="14" t="inlineStr">
+    <row r="105" ht="32" customHeight="1">
+      <c r="A105" s="14" t="inlineStr">
         <is>
           <t>・狀態：未開始 → 進行中 → 已完成。只有測試真的跑過而且通過才算已完成；阻塞要在備註寫原因；不再需要的任務標不適用，不要刪。</t>
-        </is>
-      </c>
-    </row>
-    <row r="105" ht="18" customHeight="1">
-      <c r="A105" s="14" t="inlineStr">
-        <is>
-          <t>・測試結果：未測試 / 通過 / 失敗 / 部分通過。測試證據寫跑了什麼、看到什麼，完整歷史在「更新記錄」。</t>
         </is>
       </c>
     </row>
     <row r="106" ht="18" customHeight="1">
       <c r="A106" s="14" t="inlineStr">
         <is>
-          <t>・「接下來」按階段排序，同一階段內再按優先級；依賴還沒滿足的任務不會出現在「接下來」。</t>
+          <t>・測試結果：未測試 / 通過 / 失敗 / 部分通過。測試證據寫跑了什麼、看到什麼，完整歷史在「更新記錄」。</t>
         </is>
       </c>
     </row>
     <row r="107" ht="18" customHeight="1">
       <c r="A107" s="14" t="inlineStr">
         <is>
+          <t>・「接下來」按階段排序，同一階段內再按優先級；依賴還沒滿足的任務不會出現在「接下來」。</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" ht="18" customHeight="1">
+      <c r="A108" s="14" t="inlineStr">
+        <is>
           <t>・可以手動改：「任務清單」的狀態、測試結果、測試證據、Commit、備註，以及「待確認問題」的回答。其餘欄位和本頁由腳本維護。</t>
         </is>
       </c>
     </row>
-    <row r="108" ht="32" customHeight="1">
-      <c r="A108" s="14" t="inlineStr">
+    <row r="109" ht="32" customHeight="1">
+      <c r="A109" s="14" t="inlineStr">
         <is>
           <t>・建議用法：在 Claude Code 對 Claude 說「P0-02 做完了」或輸入 /prod-readiness。Claude 會先跑測試再更新，並寫進「更新記錄」。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="89">
+  <mergeCells count="90">
     <mergeCell ref="A108:I108"/>
     <mergeCell ref="C82:I82"/>
     <mergeCell ref="E52:I52"/>
+    <mergeCell ref="A56:I56"/>
     <mergeCell ref="E39:I39"/>
     <mergeCell ref="C67:I67"/>
     <mergeCell ref="E48:I48"/>
@@ -3260,13 +3292,13 @@
     <mergeCell ref="E38:I38"/>
     <mergeCell ref="C83:I83"/>
     <mergeCell ref="C92:I92"/>
+    <mergeCell ref="A109:I109"/>
     <mergeCell ref="E31:I31"/>
     <mergeCell ref="E40:I40"/>
-    <mergeCell ref="C97:I97"/>
     <mergeCell ref="A19:I19"/>
     <mergeCell ref="E26:I26"/>
-    <mergeCell ref="A103:I103"/>
     <mergeCell ref="E25:I25"/>
+    <mergeCell ref="C95:I95"/>
     <mergeCell ref="C60:I60"/>
     <mergeCell ref="C71:I71"/>
     <mergeCell ref="E50:I50"/>
@@ -3275,6 +3307,7 @@
     <mergeCell ref="A105:I105"/>
     <mergeCell ref="C57:I57"/>
     <mergeCell ref="C66:I66"/>
+    <mergeCell ref="C102:I102"/>
     <mergeCell ref="E20:I20"/>
     <mergeCell ref="E28:I28"/>
     <mergeCell ref="C77:I77"/>
@@ -3291,25 +3324,25 @@
     <mergeCell ref="C75:I75"/>
     <mergeCell ref="C84:I84"/>
     <mergeCell ref="C80:I80"/>
+    <mergeCell ref="E54:I54"/>
     <mergeCell ref="E32:I32"/>
     <mergeCell ref="C59:I59"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="E41:I41"/>
+    <mergeCell ref="A45:I45"/>
     <mergeCell ref="E47:I47"/>
     <mergeCell ref="C61:I61"/>
+    <mergeCell ref="E43:I43"/>
     <mergeCell ref="C70:I70"/>
     <mergeCell ref="E24:I24"/>
     <mergeCell ref="E33:I33"/>
     <mergeCell ref="A3:I3"/>
-    <mergeCell ref="A55:I55"/>
     <mergeCell ref="A104:I104"/>
     <mergeCell ref="E35:I35"/>
     <mergeCell ref="C101:I101"/>
     <mergeCell ref="A106:I106"/>
-    <mergeCell ref="A96:I96"/>
     <mergeCell ref="C74:I74"/>
     <mergeCell ref="C88:I88"/>
-    <mergeCell ref="E45:I45"/>
     <mergeCell ref="C99:I99"/>
     <mergeCell ref="E37:I37"/>
     <mergeCell ref="E21:I21"/>
@@ -3321,20 +3354,19 @@
     <mergeCell ref="C78:I78"/>
     <mergeCell ref="C87:I87"/>
     <mergeCell ref="C62:I62"/>
+    <mergeCell ref="A97:I97"/>
     <mergeCell ref="C98:I98"/>
     <mergeCell ref="C89:I89"/>
     <mergeCell ref="E34:I34"/>
     <mergeCell ref="C64:I64"/>
     <mergeCell ref="C79:I79"/>
     <mergeCell ref="C73:I73"/>
-    <mergeCell ref="A44:I44"/>
     <mergeCell ref="E49:I49"/>
     <mergeCell ref="E27:I27"/>
     <mergeCell ref="E36:I36"/>
     <mergeCell ref="C63:I63"/>
     <mergeCell ref="C93:I93"/>
     <mergeCell ref="A107:I107"/>
-    <mergeCell ref="C56:I56"/>
     <mergeCell ref="C90:I90"/>
     <mergeCell ref="E53:I53"/>
     <mergeCell ref="C76:I76"/>
@@ -9477,7 +9509,7 @@
         </is>
       </c>
     </row>
-    <row r="85" ht="102" customHeight="1">
+    <row r="85" ht="130" customHeight="1">
       <c r="A85" s="13" t="inlineStr">
         <is>
           <t>P2-16</t>
@@ -9490,7 +9522,7 @@
       </c>
       <c r="C85" s="13" t="inlineStr">
         <is>
-          <t>4 量產出貨</t>
+          <t>2 內測準備</t>
         </is>
       </c>
       <c r="D85" s="6" t="inlineStr">
@@ -9543,7 +9575,8 @@
       <c r="P85" s="6" t="inlineStr">
         <is>
           <t>[2026-10-14] 新增
-[2026-10-14] 2026-10-14 開分支 p2-16-ota-rollout（worktree ../aibuddy-p216，從 dev cac98aa）；拆成 P2-17～P2-21 五項子任務，本項的測試方法即整體驗收（含 62:70 實機白名單）。</t>
+[2026-10-14] 2026-10-14 開分支 p2-16-ota-rollout（worktree ../aibuddy-p216，從 dev cac98aa）；拆成 P2-17～P2-21 五項子任務，本項的測試方法即整體驗收（含 62:70 實機白名單）。
+[2026-10-14] 2026-10-14 用戶決定提前到第 2 階段，現在開始做</t>
         </is>
       </c>
     </row>
@@ -9845,7 +9878,7 @@
       </c>
       <c r="C90" s="13" t="inlineStr">
         <is>
-          <t>4 量產出貨</t>
+          <t>2 內測準備</t>
         </is>
       </c>
       <c r="D90" s="6" t="inlineStr">
@@ -9860,7 +9893,7 @@
       </c>
       <c r="F90" s="13" t="inlineStr">
         <is>
-          <t>未開始</t>
+          <t>進行中</t>
         </is>
       </c>
       <c r="G90" s="13" t="inlineStr">
@@ -9895,7 +9928,8 @@
       </c>
       <c r="P90" s="6" t="inlineStr">
         <is>
-          <t>[2026-10-14] 新增：2026-10-14 分支 p2-16-ota-rollout（worktree ../aibuddy-p216）</t>
+          <t>[2026-10-14] 新增：2026-10-14 分支 p2-16-ota-rollout（worktree ../aibuddy-p216）
+[2026-10-14] 2026-10-14 用戶決定提前到第 2 階段，現在開始做</t>
         </is>
       </c>
     </row>
@@ -9912,7 +9946,7 @@
       </c>
       <c r="C91" s="13" t="inlineStr">
         <is>
-          <t>4 量產出貨</t>
+          <t>2 內測準備</t>
         </is>
       </c>
       <c r="D91" s="6" t="inlineStr">
@@ -9962,7 +9996,8 @@
       </c>
       <c r="P91" s="6" t="inlineStr">
         <is>
-          <t>[2026-10-14] 新增</t>
+          <t>[2026-10-14] 新增
+[2026-10-14] 2026-10-14 用戶決定提前到第 2 階段，現在開始做</t>
         </is>
       </c>
     </row>
@@ -9979,7 +10014,7 @@
       </c>
       <c r="C92" s="13" t="inlineStr">
         <is>
-          <t>4 量產出貨</t>
+          <t>2 內測準備</t>
         </is>
       </c>
       <c r="D92" s="6" t="inlineStr">
@@ -10029,7 +10064,8 @@
       </c>
       <c r="P92" s="6" t="inlineStr">
         <is>
-          <t>[2026-10-14] 新增</t>
+          <t>[2026-10-14] 新增
+[2026-10-14] 2026-10-14 用戶決定提前到第 2 階段，現在開始做</t>
         </is>
       </c>
     </row>
@@ -10046,7 +10082,7 @@
       </c>
       <c r="C93" s="13" t="inlineStr">
         <is>
-          <t>4 量產出貨</t>
+          <t>2 內測準備</t>
         </is>
       </c>
       <c r="D93" s="6" t="inlineStr">
@@ -10096,7 +10132,8 @@
       </c>
       <c r="P93" s="6" t="inlineStr">
         <is>
-          <t>[2026-10-14] 新增</t>
+          <t>[2026-10-14] 新增
+[2026-10-14] 2026-10-14 用戶決定提前到第 2 階段，現在開始做</t>
         </is>
       </c>
     </row>
@@ -10113,7 +10150,7 @@
       </c>
       <c r="C94" s="13" t="inlineStr">
         <is>
-          <t>4 量產出貨</t>
+          <t>2 內測準備</t>
         </is>
       </c>
       <c r="D94" s="6" t="inlineStr">
@@ -10163,7 +10200,8 @@
       </c>
       <c r="P94" s="6" t="inlineStr">
         <is>
-          <t>[2026-10-14] 新增</t>
+          <t>[2026-10-14] 新增
+[2026-10-14] 2026-10-14 用戶決定提前到第 2 階段，現在開始做</t>
         </is>
       </c>
     </row>
@@ -10749,7 +10787,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I277"/>
+  <dimension ref="A1:I284"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -20302,8 +20340,249 @@
       <c r="H277" s="13" t="n"/>
       <c r="I277" s="6" t="n"/>
     </row>
+    <row r="278" ht="32" customHeight="1">
+      <c r="A278" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 20:41</t>
+        </is>
+      </c>
+      <c r="B278" s="13" t="inlineStr">
+        <is>
+          <t>P2-16</t>
+        </is>
+      </c>
+      <c r="C278" s="6" t="inlineStr">
+        <is>
+          <t>OTA 分批推送與後台發佈頁</t>
+        </is>
+      </c>
+      <c r="D278" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="E278" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F278" s="13" t="n"/>
+      <c r="G278" s="6" t="n"/>
+      <c r="H278" s="13" t="n"/>
+      <c r="I278" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-14 用戶決定提前到第 2 階段，現在開始做；修改了階段→2 內測準備</t>
+        </is>
+      </c>
+    </row>
+    <row r="279" ht="32" customHeight="1">
+      <c r="A279" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 20:41</t>
+        </is>
+      </c>
+      <c r="B279" s="13" t="inlineStr">
+        <is>
+          <t>P2-17</t>
+        </is>
+      </c>
+      <c r="C279" s="6" t="inlineStr">
+        <is>
+          <t>P2-16 ① 分批推送的數據表：推送階段、白名單、每台安裝結果</t>
+        </is>
+      </c>
+      <c r="D279" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E279" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="F279" s="13" t="n"/>
+      <c r="G279" s="6" t="n"/>
+      <c r="H279" s="13" t="n"/>
+      <c r="I279" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-14 用戶決定提前到第 2 階段，現在開始做；修改了階段→2 內測準備</t>
+        </is>
+      </c>
+    </row>
+    <row r="280" ht="32" customHeight="1">
+      <c r="A280" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 20:41</t>
+        </is>
+      </c>
+      <c r="B280" s="13" t="inlineStr">
+        <is>
+          <t>P2-18</t>
+        </is>
+      </c>
+      <c r="C280" s="6" t="inlineStr">
+        <is>
+          <t>P2-16 ② 按 MAC 雜湊穩定分組決定哪台收到 ota</t>
+        </is>
+      </c>
+      <c r="D280" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E280" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="F280" s="13" t="n"/>
+      <c r="G280" s="6" t="n"/>
+      <c r="H280" s="13" t="n"/>
+      <c r="I280" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-14 用戶決定提前到第 2 階段，現在開始做；修改了階段→2 內測準備</t>
+        </is>
+      </c>
+    </row>
+    <row r="281" ht="32" customHeight="1">
+      <c r="A281" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 20:41</t>
+        </is>
+      </c>
+      <c r="B281" s="13" t="inlineStr">
+        <is>
+          <t>P2-19</t>
+        </is>
+      </c>
+      <c r="C281" s="6" t="inlineStr">
+        <is>
+          <t>P2-16 ③ 回滾過多時自動暫停推送</t>
+        </is>
+      </c>
+      <c r="D281" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E281" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="F281" s="13" t="n"/>
+      <c r="G281" s="6" t="n"/>
+      <c r="H281" s="13" t="n"/>
+      <c r="I281" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-14 用戶決定提前到第 2 階段，現在開始做；修改了階段→2 內測準備</t>
+        </is>
+      </c>
+    </row>
+    <row r="282" ht="32" customHeight="1">
+      <c r="A282" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 20:41</t>
+        </is>
+      </c>
+      <c r="B282" s="13" t="inlineStr">
+        <is>
+          <t>P2-20</t>
+        </is>
+      </c>
+      <c r="C282" s="6" t="inlineStr">
+        <is>
+          <t>P2-16 ④ 從後台上傳與發佈韌體（取代手貼 service key）</t>
+        </is>
+      </c>
+      <c r="D282" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E282" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="F282" s="13" t="n"/>
+      <c r="G282" s="6" t="n"/>
+      <c r="H282" s="13" t="n"/>
+      <c r="I282" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-14 用戶決定提前到第 2 階段，現在開始做；修改了階段→2 內測準備</t>
+        </is>
+      </c>
+    </row>
+    <row r="283" ht="32" customHeight="1">
+      <c r="A283" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 20:41</t>
+        </is>
+      </c>
+      <c r="B283" s="13" t="inlineStr">
+        <is>
+          <t>P2-21</t>
+        </is>
+      </c>
+      <c r="C283" s="6" t="inlineStr">
+        <is>
+          <t>P2-16 ⑤ 後台 OTA 頁換成真實數據與操作</t>
+        </is>
+      </c>
+      <c r="D283" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E283" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="F283" s="13" t="n"/>
+      <c r="G283" s="6" t="n"/>
+      <c r="H283" s="13" t="n"/>
+      <c r="I283" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-14 用戶決定提前到第 2 階段，現在開始做；修改了階段→2 內測準備</t>
+        </is>
+      </c>
+    </row>
+    <row r="284" ht="32" customHeight="1">
+      <c r="A284" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 20:41</t>
+        </is>
+      </c>
+      <c r="B284" s="13" t="inlineStr">
+        <is>
+          <t>P2-17</t>
+        </is>
+      </c>
+      <c r="C284" s="6" t="inlineStr">
+        <is>
+          <t>P2-16 ① 分批推送的數據表：推送階段、白名單、每台安裝結果</t>
+        </is>
+      </c>
+      <c r="D284" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E284" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F284" s="13" t="n"/>
+      <c r="G284" s="6" t="n"/>
+      <c r="H284" s="13" t="n"/>
+      <c r="I284" s="6" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I277"/>
+  <autoFilter ref="A1:I284"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Track P2-17 (staged-rollout tables) as passed.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/production-readiness.xlsx
+++ b/docs/production-readiness.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'任務清單'!$A$1:$P$94</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'待確認問題'!$A$1:$G$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$284</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$286</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -641,7 +641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I109"/>
+  <dimension ref="A1:I107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -665,14 +665,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>最後更新：2026-10-14 20:41　·　本頁由 tracker.py 自動生成，請勿手動編輯</t>
+          <t>最後更新：2026-10-14 20:45　·　本頁由 tracker.py 自動生成，請勿手動編輯</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>總進度：18/89 已完成（20%）　·　目前階段：1 止血定案（10/5–10/16）</t>
+          <t>總進度：19/89 已完成（21%）　·　目前階段：1 止血定案（10/5–10/16）</t>
         </is>
       </c>
     </row>
@@ -824,11 +824,11 @@
       </c>
       <c r="E8" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A8,'任務清單'!$F:$F,E$5)</f>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F8" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A8,'任務清單'!$F:$F,F$5)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G8" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A8,'任務清單'!$F:$F,G$5)</f>
@@ -840,7 +840,7 @@
       </c>
       <c r="I8" s="8">
         <f>IFERROR(F8/(C8-H8),0)</f>
-        <v>0.14285714285714285</v>
+        <v>0.19047619047619047</v>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1">
@@ -900,11 +900,11 @@
       </c>
       <c r="E10" s="5">
         <f>SUM(E6:E9)</f>
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F10" s="5">
         <f>SUM(F6:F9)</f>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="G10" s="5">
         <f>SUM(G6:G9)</f>
@@ -916,7 +916,7 @@
       </c>
       <c r="I10" s="9">
         <f>IFERROR(F10/(C10-H10),0)</f>
-        <v>0.20224719101123595</v>
+        <v>0.21348314606741572</v>
       </c>
     </row>
     <row r="12">
@@ -1027,11 +1027,11 @@
       </c>
       <c r="E14" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A14,'任務清單'!$F:$F,E$12)</f>
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F14" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A14,'任務清單'!$F:$F,F$12)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G14" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A14,'任務清單'!$F:$F,G$12)</f>
@@ -1043,7 +1043,7 @@
       </c>
       <c r="I14" s="8">
         <f>IFERROR(F14/(C14-H14),0)</f>
-        <v>0.09090909090909091</v>
+        <v>0.12121212121212122</v>
       </c>
     </row>
     <row r="15" ht="46" customHeight="1">
@@ -1143,11 +1143,11 @@
       </c>
       <c r="E17" s="5">
         <f>SUM(E13:E16)</f>
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F17" s="5">
         <f>SUM(F13:F16)</f>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="G17" s="5">
         <f>SUM(G13:G16)</f>
@@ -1159,7 +1159,7 @@
       </c>
       <c r="I17" s="9">
         <f>IFERROR(F17/(C17-H17),0)</f>
-        <v>0.20224719101123595</v>
+        <v>0.21348314606741572</v>
       </c>
     </row>
     <row r="19">
@@ -1581,15 +1581,15 @@
       <c r="H32" s="11" t="n"/>
       <c r="I32" s="12" t="n"/>
     </row>
-    <row r="33" ht="102" customHeight="1">
+    <row r="33" ht="200" customHeight="1">
       <c r="A33" s="13" t="inlineStr">
         <is>
-          <t>P2-17</t>
+          <t>R-21</t>
         </is>
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>P2-16 ① 分批推送的數據表：推送階段、白名單、每台安裝結果</t>
+          <t>藍牙配網與綁定（取代熱點配網）</t>
         </is>
       </c>
       <c r="C33" s="13" t="inlineStr">
@@ -1604,7 +1604,7 @@
       </c>
       <c r="E33" s="6" t="inlineStr">
         <is>
-          <t>firmware_releases 加推送狀態（階段：白名單／10%／50%／100%、白名單 MAC、暫停與原因、階段變更時間）；新表記錄每台對每個版本：首次下發、下發次數、確認（回報版本＝該版）、回滾（failed_version＝該版）；只有超級管理員能讀，寫入只經 service role 或帶審計的 admin RPC；舊的 is_current 發佈照常可用（視為 100%）。</t>
+          <t>① 設備在「未配網、Wi-Fi 連不上、未綁定、長按 BOOT」時以 AIBuddy-XXXX 名稱廣播藍牙，廣播資料帶品牌，品牌 App 只列出自己品牌的設備。② 設備經藍牙回傳它掃描到的 2.4GHz Wi-Fi 清單，App 讓用戶選擇並填密碼。③ App 經藍牙把 SSID、密碼和綁定票（P0-11）一起交給設備；藍牙通道加密（ESP 標準配網協定 security 1/2 或同等）。④ 設備連上 Wi-Fi 後自己完成認領，App 顯示綁定成功或失敗原因（密碼錯、設備已有主人、票過期）。⑤ 配網期間不啟動音訊；完成後釋放藍牙記憶體再開語音（必要時重開機），對話中最低 heap 不比現在差。⑥ 解綁在 App 內完成（P1-12），解綁後設備進入藍牙待綁定狀態。⑦ SoftAP 熱點配網保留給開發和運維（隱藏觸發方式或編譯開關），量產用戶流程不出現。</t>
         </is>
       </c>
       <c r="F33" s="11" t="n"/>
@@ -1612,15 +1612,15 @@
       <c r="H33" s="11" t="n"/>
       <c r="I33" s="12" t="n"/>
     </row>
-    <row r="34" ht="200" customHeight="1">
+    <row r="34" ht="116" customHeight="1">
       <c r="A34" s="13" t="inlineStr">
         <is>
-          <t>R-21</t>
+          <t>R-36</t>
         </is>
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>藍牙配網與綁定（取代熱點配網）</t>
+          <t>未認領的設備停在配對狀態，不再每秒重連 websocket</t>
         </is>
       </c>
       <c r="C34" s="13" t="inlineStr">
@@ -1635,7 +1635,7 @@
       </c>
       <c r="E34" s="6" t="inlineStr">
         <is>
-          <t>① 設備在「未配網、Wi-Fi 連不上、未綁定、長按 BOOT」時以 AIBuddy-XXXX 名稱廣播藍牙，廣播資料帶品牌，品牌 App 只列出自己品牌的設備。② 設備經藍牙回傳它掃描到的 2.4GHz Wi-Fi 清單，App 讓用戶選擇並填密碼。③ App 經藍牙把 SSID、密碼和綁定票（P0-11）一起交給設備；藍牙通道加密（ESP 標準配網協定 security 1/2 或同等）。④ 設備連上 Wi-Fi 後自己完成認領，App 顯示綁定成功或失敗原因（密碼錯、設備已有主人、票過期）。⑤ 配網期間不啟動音訊；完成後釋放藍牙記憶體再開語音（必要時重開機），對話中最低 heap 不比現在差。⑥ 解綁在 App 內完成（P1-12），解綁後設備進入藍牙待綁定狀態。⑦ SoftAP 熱點配網保留給開發和運維（隱藏觸發方式或編譯開關），量產用戶流程不出現。</t>
+          <t>① 拿到 202 或 websocket 被 4401 拒絕後，設備停掉 websocket 自動重連，進入待綁定狀態（燈號可分辨）。② 待綁定時只按退避（5 秒起、上限 PROVISION_BACKOFF_MAX）呼叫 generate_auth_token，不開 websocket。③ 被認領後下一次輪詢拿到 200，在 10 秒內（加退避）自動開 websocket 並能對話，不用重開機。④ 已綁定設備網絡斷線重連的行為不變。⑤ 隨 OTA 推出。</t>
         </is>
       </c>
       <c r="F34" s="11" t="n"/>
@@ -1643,20 +1643,20 @@
       <c r="H34" s="11" t="n"/>
       <c r="I34" s="12" t="n"/>
     </row>
-    <row r="35" ht="116" customHeight="1">
+    <row r="35" ht="228" customHeight="1">
       <c r="A35" s="13" t="inlineStr">
         <is>
-          <t>R-36</t>
+          <t>P2-12</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>未認領的設備停在配對狀態，不再每秒重連 websocket</t>
+          <t>量產燒錄前加大 app 分區</t>
         </is>
       </c>
       <c r="C35" s="13" t="inlineStr">
         <is>
-          <t>2 內測準備</t>
+          <t>3 封閉內測</t>
         </is>
       </c>
       <c r="D35" s="13" t="inlineStr">
@@ -1666,7 +1666,8 @@
       </c>
       <c r="E35" s="6" t="inlineStr">
         <is>
-          <t>① 拿到 202 或 websocket 被 4401 拒絕後，設備停掉 websocket 自動重連，進入待綁定狀態（燈號可分辨）。② 待綁定時只按退避（5 秒起、上限 PROVISION_BACKOFF_MAX）呼叫 generate_auth_token，不開 websocket。③ 被認領後下一次輪詢拿到 200，在 10 秒內（加退避）自動開 websocket 並能對話，不用重開機。④ 已綁定設備網絡斷線重連的行為不變。⑤ 隨 OTA 推出。</t>
+          <t>上次測試：部分通過 — 62:70（spotpear-ai-toy-p212 原型，現已併入 spotpear-ai-toy）：① 本機 OTA 1.6.1→1.6.2 寫入新 app1，120s 後 confirmed ② 3 秒 abort 的 1.6.3 → PANIC → 回到 1.6.2，ota_failed_version=1.6.3 ③ 崩潰寫入 coredump 14.8KB ④ 資源分區 9 個聲音 504KB/2MB，開機 CRC 63ms，OTA 後照常；損壞/清空 → 退回內建聲音無崩潰 ⑤ pio 全部 18 個 env 編譯通過，映像都在各自 app 槽內（Spotpear 4 個 1.59–1.60MB / 4MB；其他板仍 2MB 槽）；R-21 藍牙探針版 2,326,128 bytes &lt; 4MB ⑥ release_firmware.py 映像 &gt; app 槽即拒發。未做：雲端 OTA 一次（等上 UAT）、出廠腳本寫入資源包（R-10）
+新分區表（例如 app0/app1 各 4MB，保留 nvs/otadata 位置）在出廠前定案並寫入出廠腳本；OTA 與回滾在新分區表上照常</t>
         </is>
       </c>
       <c r="F35" s="11" t="n"/>
@@ -1674,15 +1675,15 @@
       <c r="H35" s="11" t="n"/>
       <c r="I35" s="12" t="n"/>
     </row>
-    <row r="36" ht="228" customHeight="1">
+    <row r="36" ht="242" customHeight="1">
       <c r="A36" s="13" t="inlineStr">
         <is>
-          <t>P2-12</t>
+          <t>R-37</t>
         </is>
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>量產燒錄前加大 app 分區</t>
+          <t>網頁設定玩具的 Wi-Fi：查看、新增、刪除</t>
         </is>
       </c>
       <c r="C36" s="13" t="inlineStr">
@@ -1697,8 +1698,8 @@
       </c>
       <c r="E36" s="6" t="inlineStr">
         <is>
-          <t>上次測試：部分通過 — 62:70（spotpear-ai-toy-p212 原型，現已併入 spotpear-ai-toy）：① 本機 OTA 1.6.1→1.6.2 寫入新 app1，120s 後 confirmed ② 3 秒 abort 的 1.6.3 → PANIC → 回到 1.6.2，ota_failed_version=1.6.3 ③ 崩潰寫入 coredump 14.8KB ④ 資源分區 9 個聲音 504KB/2MB，開機 CRC 63ms，OTA 後照常；損壞/清空 → 退回內建聲音無崩潰 ⑤ pio 全部 18 個 env 編譯通過，映像都在各自 app 槽內（Spotpear 4 個 1.59–1.60MB / 4MB；其他板仍 2MB 槽）；R-21 藍牙探針版 2,326,128 bytes &lt; 4MB ⑥ release_firmware.py 映像 &gt; app 槽即拒發。未做：雲端 OTA 一次（等上 UAT）、出廠腳本寫入資源包（R-10）
-新分區表（例如 app0/app1 各 4MB，保留 nvs/otadata 位置）在出廠前定案並寫入出廠腳本；OTA 與回滾在新分區表上照常</t>
+          <t>上次測試：部分通過 — 模擬玩具經本機語音服務器＋網頁：status/scan/add/delete 正常；刪除目前 Wi-Fi → current 被拒；斷線 5 秒內頁面顯示睡著、按鈕停用；測試密碼在語音服務器日誌、網頁服務器日誌、資料庫均搜不到；用別人裝置 ID 重放 server action → forbidden；pytest 17 項通過（全套 230）；韌體 spotpear-ai-toy-localall 編譯通過（RAM 17.5%、Flash 75.9%）。未測：真機 ①② 及 OTA 推出
+① 設定頁顯示玩具在線／離線、目前 Wi-Fi 和訊號、已記住的 Wi-Fi 清單（只有名稱，不顯示密碼）② 在線時可新增 Wi-Fi（輸入或從玩具掃描到的清單選）、刪除 Wi-Fi；不能刪除正在使用的那個 ③ 經 /ws/esp32 轉送：伺服器先確認是設備主人；密碼不寫入資料庫、不寫入日誌 ④ 新增不切換網絡，目前 Wi-Fi 消失時才按訊號選；清單標示「連過／未連過」⑤ 上限 8 個 ⑥ 韌體改動經 OTA 推出</t>
         </is>
       </c>
       <c r="F36" s="11" t="n"/>
@@ -1706,31 +1707,30 @@
       <c r="H36" s="11" t="n"/>
       <c r="I36" s="12" t="n"/>
     </row>
-    <row r="37" ht="242" customHeight="1">
+    <row r="37" ht="102" customHeight="1">
       <c r="A37" s="13" t="inlineStr">
         <is>
-          <t>R-37</t>
+          <t>R-16</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>網頁設定玩具的 Wi-Fi：查看、新增、刪除</t>
+          <t>Spotpear 量產版加電池電壓檢測（GPIO0 分壓）</t>
         </is>
       </c>
       <c r="C37" s="13" t="inlineStr">
         <is>
-          <t>3 封閉內測</t>
+          <t>1 止血定案</t>
         </is>
       </c>
       <c r="D37" s="13" t="inlineStr">
         <is>
-          <t>進行中</t>
+          <t>未開始</t>
         </is>
       </c>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>上次測試：部分通過 — 模擬玩具經本機語音服務器＋網頁：status/scan/add/delete 正常；刪除目前 Wi-Fi → current 被拒；斷線 5 秒內頁面顯示睡著、按鈕停用；測試密碼在語音服務器日誌、網頁服務器日誌、資料庫均搜不到；用別人裝置 ID 重放 server action → forbidden；pytest 17 項通過（全套 230）；韌體 spotpear-ai-toy-localall 編譯通過（RAM 17.5%、Flash 75.9%）。未測：真機 ①② 及 OTA 推出
-① 設定頁顯示玩具在線／離線、目前 Wi-Fi 和訊號、已記住的 Wi-Fi 清單（只有名稱，不顯示密碼）② 在線時可新增 Wi-Fi（輸入或從玩具掃描到的清單選）、刪除 Wi-Fi；不能刪除正在使用的那個 ③ 經 /ws/esp32 轉送：伺服器先確認是設備主人；密碼不寫入資料庫、不寫入日誌 ④ 新增不切換網絡，目前 Wi-Fi 消失時才按訊號選；清單標示「連過／未連過」⑤ 上限 8 個 ⑥ 韌體改動經 OTA 推出</t>
+          <t>Spotpear 書面確認量產版：GPIO1（屏幕 DC；本版不接屏幕，可空出來）接電芯正極（保護 IC 之後）100k/100k 分壓、100nF 濾波，屏幕不接該腳；GPIO0 保留給現有的 VDD 低電提醒；最好另把充電芯片 CHRG 接到 GPIO12 或 13。樣板到手後，固件讀到的電芯電壓與萬用表相差 ≤50mV，App（R-41）顯示百分比與充電中。</t>
         </is>
       </c>
       <c r="F37" s="11" t="n"/>
@@ -1738,20 +1738,20 @@
       <c r="H37" s="11" t="n"/>
       <c r="I37" s="12" t="n"/>
     </row>
-    <row r="38" ht="102" customHeight="1">
+    <row r="38" ht="46" customHeight="1">
       <c r="A38" s="13" t="inlineStr">
         <is>
-          <t>R-16</t>
+          <t>P1-11</t>
         </is>
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>Spotpear 量產版加電池電壓檢測（GPIO0 分壓）</t>
+          <t>伺服器與資料庫直接存取的管控</t>
         </is>
       </c>
       <c r="C38" s="13" t="inlineStr">
         <is>
-          <t>1 止血定案</t>
+          <t>2 內測準備</t>
         </is>
       </c>
       <c r="D38" s="13" t="inlineStr">
@@ -1761,7 +1761,7 @@
       </c>
       <c r="E38" s="6" t="inlineStr">
         <is>
-          <t>Spotpear 書面確認量產版：GPIO1（屏幕 DC；本版不接屏幕，可空出來）接電芯正極（保護 IC 之後）100k/100k 分壓、100nF 濾波，屏幕不接該腳；GPIO0 保留給現有的 VDD 低電提醒；最好另把充電芯片 CHRG 接到 GPIO12 或 13。樣板到手後，固件讀到的電芯電壓與萬用表相差 ≤50mV，App（R-41）顯示百分比與充電中。</t>
+          <t>列出誰有 SSH 與資料庫直連權限（越少越好）；service_role key 只存在伺服器的 env；私隱政策寫明這類存取的範圍；每次直接查看生產資料都留記錄。</t>
         </is>
       </c>
       <c r="F38" s="11" t="n"/>
@@ -1772,12 +1772,12 @@
     <row r="39" ht="46" customHeight="1">
       <c r="A39" s="13" t="inlineStr">
         <is>
-          <t>P1-11</t>
+          <t>P2-02</t>
         </is>
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>伺服器與資料庫直接存取的管控</t>
+          <t>CI 跑測試與靜態檢查</t>
         </is>
       </c>
       <c r="C39" s="13" t="inlineStr">
@@ -1792,7 +1792,7 @@
       </c>
       <c r="E39" s="6" t="inlineStr">
         <is>
-          <t>列出誰有 SSH 與資料庫直連權限（越少越好）；service_role key 只存在伺服器的 env；私隱政策寫明這類存取的範圍；每次直接查看生產資料都留記錄。</t>
+          <t>推送與 PR 時跑 pytest、ruff、pyright、next lint、tsc --noEmit、pio run；任何一項失敗就不發佈 image。</t>
         </is>
       </c>
       <c r="F39" s="11" t="n"/>
@@ -1800,15 +1800,15 @@
       <c r="H39" s="11" t="n"/>
       <c r="I39" s="12" t="n"/>
     </row>
-    <row r="40" ht="46" customHeight="1">
+    <row r="40" ht="32" customHeight="1">
       <c r="A40" s="13" t="inlineStr">
         <is>
-          <t>P2-02</t>
+          <t>P2-04</t>
         </is>
       </c>
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>CI 跑測試與靜態檢查</t>
+          <t>容器改用非 root 用戶</t>
         </is>
       </c>
       <c r="C40" s="13" t="inlineStr">
@@ -1823,7 +1823,7 @@
       </c>
       <c r="E40" s="6" t="inlineStr">
         <is>
-          <t>推送與 PR 時跑 pytest、ruff、pyright、next lint、tsc --noEmit、pio run；任何一項失敗就不發佈 image。</t>
+          <t>兩個 Dockerfile 都設定非 root 的 USER。</t>
         </is>
       </c>
       <c r="F40" s="11" t="n"/>
@@ -1831,15 +1831,15 @@
       <c r="H40" s="11" t="n"/>
       <c r="I40" s="12" t="n"/>
     </row>
-    <row r="41" ht="32" customHeight="1">
+    <row r="41" ht="74" customHeight="1">
       <c r="A41" s="13" t="inlineStr">
         <is>
-          <t>P2-04</t>
+          <t>P2-18</t>
         </is>
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>容器改用非 root 用戶</t>
+          <t>P2-16 ② 按 MAC 雜湊穩定分組決定哪台收到 ota</t>
         </is>
       </c>
       <c r="C41" s="13" t="inlineStr">
@@ -1854,7 +1854,7 @@
       </c>
       <c r="E41" s="6" t="inlineStr">
         <is>
-          <t>兩個 Dockerfile 都設定非 root 的 USER。</t>
+          <t>白名單階段只有名單內 MAC 拿到 ota；10%／50%／100% 按 MAC 雜湊（加版本作鹽）穩定分組，同一台重複請求結果不變，升階段時已在組內的不會掉出；暫停時一律不下發；每次下發與結果寫入 ① 的記錄；不用改韌體。</t>
         </is>
       </c>
       <c r="F41" s="11" t="n"/>
@@ -1893,68 +1893,68 @@
       <c r="H42" s="11" t="n"/>
       <c r="I42" s="12" t="n"/>
     </row>
-    <row r="43" ht="116" customHeight="1">
-      <c r="A43" s="13" t="inlineStr">
-        <is>
-          <t>R-25</t>
-        </is>
-      </c>
-      <c r="B43" s="6" t="inlineStr">
-        <is>
-          <t>網頁的品牌主題系統</t>
-        </is>
-      </c>
-      <c r="C43" s="13" t="inlineStr">
-        <is>
-          <t>2 內測準備</t>
-        </is>
-      </c>
-      <c r="D43" s="13" t="inlineStr">
-        <is>
-          <t>未開始</t>
-        </is>
-      </c>
-      <c r="E43" s="6" t="inlineStr">
-        <is>
-          <t>① 每個品牌一個資料夾：主題 token（顏色、字體、圓角）、logo 和圖示、文案、功能開關；首頁、上手流程、角色頁可以有品牌版本，其餘頁面共用 ② 由部署的環境變數選品牌（每套部署一個品牌，見 R-34），伺服器端渲染的第一屏就是對的主題，不閃爍 ③ 共用元件裡沒有品牌名稱和寫死的品牌顏色 ④ 加一個品牌只需要加資料夾、設定和一套部署，不用改共用元件</t>
-        </is>
-      </c>
-      <c r="F43" s="11" t="n"/>
-      <c r="G43" s="11" t="n"/>
-      <c r="H43" s="11" t="n"/>
-      <c r="I43" s="12" t="n"/>
+    <row r="44">
+      <c r="A44" s="10" t="inlineStr">
+        <is>
+          <t>✅ 最近完成與測試效果</t>
+        </is>
+      </c>
     </row>
     <row r="45">
-      <c r="A45" s="10" t="inlineStr">
-        <is>
-          <t>✅ 最近完成與測試效果</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="4" t="inlineStr">
+      <c r="A45" s="4" t="inlineStr">
         <is>
           <t>編號</t>
         </is>
       </c>
-      <c r="B46" s="4" t="inlineStr">
+      <c r="B45" s="4" t="inlineStr">
         <is>
           <t>任務</t>
         </is>
       </c>
-      <c r="C46" s="4" t="inlineStr">
+      <c r="C45" s="4" t="inlineStr">
         <is>
           <t>測試結果</t>
         </is>
       </c>
-      <c r="D46" s="4" t="inlineStr">
+      <c r="D45" s="4" t="inlineStr">
         <is>
           <t>完成日期</t>
         </is>
       </c>
-      <c r="E46" s="4" t="inlineStr">
+      <c r="E45" s="4" t="inlineStr">
         <is>
           <t>測試證據</t>
+        </is>
+      </c>
+      <c r="F45" s="11" t="n"/>
+      <c r="G45" s="11" t="n"/>
+      <c r="H45" s="11" t="n"/>
+      <c r="I45" s="12" t="n"/>
+    </row>
+    <row r="46" ht="172" customHeight="1">
+      <c r="A46" s="13" t="inlineStr">
+        <is>
+          <t>P2-17</t>
+        </is>
+      </c>
+      <c r="B46" s="6" t="inlineStr">
+        <is>
+          <t>P2-16 ① 分批推送的數據表：推送階段、白名單、每台安裝結果</t>
+        </is>
+      </c>
+      <c r="C46" s="13" t="inlineStr">
+        <is>
+          <t>通過</t>
+        </is>
+      </c>
+      <c r="D46" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="E46" s="6" t="inlineStr">
+        <is>
+          <t>migration 20261014190000 BEGIN/ROLLBACK 套用兩次無錯並已套用本機；行為：預設 100%、promote 記 stage_changed_at，7 種壞值（25%、小寫/空字串/NULL MAC、暫停缺原因等）全被 check 擋；ota_note_offer 1→2→3，report 正確標 running/failed、別板型不影響，刪發佈連帶刪記錄；審計 5 筆含 'test-board 9.9.9' 標籤。REST 13/13：超管可讀、內容管理員 0 行、anon 42501，三種身份寫入/改階段/呼叫 ota_note_offer 皆 42501。release_firmware.py promote spotpear-ai-toy 1.6.2 成功，token 查詢仍選 1.6.2，審計記 2 筆（actor 空＝service role）</t>
         </is>
       </c>
       <c r="F46" s="11" t="n"/>
@@ -2179,58 +2179,50 @@
       <c r="H53" s="11" t="n"/>
       <c r="I53" s="12" t="n"/>
     </row>
-    <row r="54" ht="60" customHeight="1">
-      <c r="A54" s="13" t="inlineStr">
-        <is>
-          <t>P0-08</t>
-        </is>
-      </c>
-      <c r="B54" s="6" t="inlineStr">
-        <is>
-          <t>語音伺服器驗證設備身份（/ws/esp32）</t>
-        </is>
-      </c>
-      <c r="C54" s="13" t="inlineStr">
-        <is>
-          <t>通過</t>
-        </is>
-      </c>
-      <c r="D54" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-12</t>
-        </is>
-      </c>
-      <c r="E54" s="6" t="inlineStr">
-        <is>
-          <t>線上 2026-10-12（bac24e9）：wss /fastapi/ws/esp32 不帶 token、偽造 token＋X-Device-Mac → 均 4401 invalid device token；42:34 以有效 token 連線對話正常（P0-13 10/09）</t>
-        </is>
-      </c>
-      <c r="F54" s="11" t="n"/>
-      <c r="G54" s="11" t="n"/>
-      <c r="H54" s="11" t="n"/>
-      <c r="I54" s="12" t="n"/>
+    <row r="55">
+      <c r="A55" s="10" t="inlineStr">
+        <is>
+          <t>⏳ 等待依賴 / ⛔ 阻塞</t>
+        </is>
+      </c>
     </row>
     <row r="56">
-      <c r="A56" s="10" t="inlineStr">
-        <is>
-          <t>⏳ 等待依賴 / ⛔ 阻塞</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="4" t="inlineStr">
+      <c r="A56" s="4" t="inlineStr">
         <is>
           <t>編號</t>
         </is>
       </c>
-      <c r="B57" s="4" t="inlineStr">
+      <c r="B56" s="4" t="inlineStr">
         <is>
           <t>任務</t>
         </is>
       </c>
-      <c r="C57" s="4" t="inlineStr">
+      <c r="C56" s="4" t="inlineStr">
         <is>
           <t>在等什麼</t>
+        </is>
+      </c>
+      <c r="D56" s="11" t="n"/>
+      <c r="E56" s="11" t="n"/>
+      <c r="F56" s="11" t="n"/>
+      <c r="G56" s="11" t="n"/>
+      <c r="H56" s="11" t="n"/>
+      <c r="I56" s="12" t="n"/>
+    </row>
+    <row r="57" ht="88" customHeight="1">
+      <c r="A57" s="13" t="inlineStr">
+        <is>
+          <t>R-17</t>
+        </is>
+      </c>
+      <c r="B57" s="6" t="inlineStr">
+        <is>
+          <t>Spotpear 電池耗盡時插電能否正常開機（供電路徑）</t>
+        </is>
+      </c>
+      <c r="C57" s="6" t="inlineStr">
+        <is>
+          <t>阻塞：[2026-10-08] 2026-10-08 開發板 63:64 插著 USB 時兩次無法解釋的完全斷電重開：09:13:26（崩潰循環中）、10:44:33（閒置、用戶確認沒碰）。都是 USB 先斷線再以 ESP_RST_POWERON 開機，非 brownout；斷電前 6 秒 GPIO0 讀數 99.9% 參考值，屬突然切斷而非緩降（SupplyMonitor 取樣太疏抓不到瞬間）。韌體無法造成 POWERON，指向充電芯片/電池保護/供電路徑，應一併問 Spotpear；放電實測時留意插 USB 閒置時是否也會斷電</t>
         </is>
       </c>
       <c r="D57" s="11" t="n"/>
@@ -2240,20 +2232,20 @@
       <c r="H57" s="11" t="n"/>
       <c r="I57" s="12" t="n"/>
     </row>
-    <row r="58" ht="88" customHeight="1">
+    <row r="58" ht="60" customHeight="1">
       <c r="A58" s="13" t="inlineStr">
         <is>
-          <t>R-17</t>
+          <t>P1-01</t>
         </is>
       </c>
       <c r="B58" s="6" t="inlineStr">
         <is>
-          <t>Spotpear 電池耗盡時插電能否正常開機（供電路徑）</t>
+          <t>加入內容審核層（輸入與輸出）</t>
         </is>
       </c>
       <c r="C58" s="6" t="inlineStr">
         <is>
-          <t>阻塞：[2026-10-08] 2026-10-08 開發板 63:64 插著 USB 時兩次無法解釋的完全斷電重開：09:13:26（崩潰循環中）、10:44:33（閒置、用戶確認沒碰）。都是 USB 先斷線再以 ESP_RST_POWERON 開機，非 brownout；斷電前 6 秒 GPIO0 讀數 99.9% 參考值，屬突然切斷而非緩降（SupplyMonitor 取樣太疏抓不到瞬間）。韌體無法造成 POWERON，指向充電芯片/電池保護/供電路徑，應一併問 Spotpear；放電實測時留意插 USB 閒置時是否也會斷電</t>
+          <t>阻塞：[2026-10-14] 2026-10-14 用戶決定：先不定審核服務商，本項暫停。候選：Azure Content Safety（建議，香港區、可在每句回覆說出口前檢查）、OpenRouter 安全模型、OpenAI Moderation、只用本機字詞表。未寫任何程式。</t>
         </is>
       </c>
       <c r="D58" s="11" t="n"/>
@@ -2263,20 +2255,20 @@
       <c r="H58" s="11" t="n"/>
       <c r="I58" s="12" t="n"/>
     </row>
-    <row r="59" ht="60" customHeight="1">
+    <row r="59" ht="32" customHeight="1">
       <c r="A59" s="13" t="inlineStr">
         <is>
-          <t>P1-01</t>
+          <t>P1-09</t>
         </is>
       </c>
       <c r="B59" s="6" t="inlineStr">
         <is>
-          <t>加入內容審核層（輸入與輸出）</t>
+          <t>家長鎖：孩子模式進設定要輸入 PIN</t>
         </is>
       </c>
       <c r="C59" s="6" t="inlineStr">
         <is>
-          <t>阻塞：[2026-10-14] 2026-10-14 用戶決定：先不定審核服務商，本項暫停。候選：Azure Content Safety（建議，香港區、可在每句回覆說出口前檢查）、OpenRouter 安全模型、OpenAI Moderation、只用本機字詞表。未寫任何程式。</t>
+          <t>阻塞：[2026-10-13] 2026-10-13 用戶決定：AI Buddy（品牌 C）延到 1/15 之後，本項不卡 1/15 出廠；AI Buddy 啟動時再開。</t>
         </is>
       </c>
       <c r="D59" s="11" t="n"/>
@@ -2289,12 +2281,12 @@
     <row r="60" ht="32" customHeight="1">
       <c r="A60" s="13" t="inlineStr">
         <is>
-          <t>P1-09</t>
+          <t>R-12</t>
         </is>
       </c>
       <c r="B60" s="6" t="inlineStr">
         <is>
-          <t>家長鎖：孩子模式進設定要輸入 PIN</t>
+          <t>家長控制：每日使用上限和休息時段</t>
         </is>
       </c>
       <c r="C60" s="6" t="inlineStr">
@@ -2312,12 +2304,12 @@
     <row r="61" ht="32" customHeight="1">
       <c r="A61" s="13" t="inlineStr">
         <is>
-          <t>R-12</t>
+          <t>R-29</t>
         </is>
       </c>
       <c r="B61" s="6" t="inlineStr">
         <is>
-          <t>家長控制：每日使用上限和休息時段</t>
+          <t>AI Buddy App（品牌 C）頁面</t>
         </is>
       </c>
       <c r="C61" s="6" t="inlineStr">
@@ -2332,20 +2324,20 @@
       <c r="H61" s="11" t="n"/>
       <c r="I61" s="12" t="n"/>
     </row>
-    <row r="62" ht="32" customHeight="1">
+    <row r="62" ht="18" customHeight="1">
       <c r="A62" s="13" t="inlineStr">
         <is>
-          <t>R-29</t>
+          <t>P2-19</t>
         </is>
       </c>
       <c r="B62" s="6" t="inlineStr">
         <is>
-          <t>AI Buddy App（品牌 C）頁面</t>
+          <t>P2-16 ③ 回滾過多時自動暫停推送</t>
         </is>
       </c>
       <c r="C62" s="6" t="inlineStr">
         <is>
-          <t>阻塞：[2026-10-13] 2026-10-13 用戶決定：AI Buddy（品牌 C）延到 1/15 之後，本項不卡 1/15 出廠；AI Buddy 啟動時再開。</t>
+          <t>等 P2-18</t>
         </is>
       </c>
       <c r="D62" s="11" t="n"/>
@@ -2358,17 +2350,17 @@
     <row r="63" ht="32" customHeight="1">
       <c r="A63" s="13" t="inlineStr">
         <is>
-          <t>P2-18</t>
+          <t>P2-20</t>
         </is>
       </c>
       <c r="B63" s="6" t="inlineStr">
         <is>
-          <t>P2-16 ② 按 MAC 雜湊穩定分組決定哪台收到 ota</t>
+          <t>P2-16 ④ 從後台上傳與發佈韌體（取代手貼 service key）</t>
         </is>
       </c>
       <c r="C63" s="6" t="inlineStr">
         <is>
-          <t>等 P2-17</t>
+          <t>等 P1-10</t>
         </is>
       </c>
       <c r="D63" s="11" t="n"/>
@@ -2381,17 +2373,17 @@
     <row r="64" ht="18" customHeight="1">
       <c r="A64" s="13" t="inlineStr">
         <is>
-          <t>P2-19</t>
+          <t>P2-21</t>
         </is>
       </c>
       <c r="B64" s="6" t="inlineStr">
         <is>
-          <t>P2-16 ③ 回滾過多時自動暫停推送</t>
+          <t>P2-16 ⑤ 後台 OTA 頁換成真實數據與操作</t>
         </is>
       </c>
       <c r="C64" s="6" t="inlineStr">
         <is>
-          <t>等 P2-18</t>
+          <t>等 P2-18、P2-19、P2-20、P2-14</t>
         </is>
       </c>
       <c r="D64" s="11" t="n"/>
@@ -2401,20 +2393,20 @@
       <c r="H64" s="11" t="n"/>
       <c r="I64" s="12" t="n"/>
     </row>
-    <row r="65" ht="32" customHeight="1">
+    <row r="65" ht="18" customHeight="1">
       <c r="A65" s="13" t="inlineStr">
         <is>
-          <t>P2-20</t>
+          <t>R-05</t>
         </is>
       </c>
       <c r="B65" s="6" t="inlineStr">
         <is>
-          <t>P2-16 ④ 從後台上傳與發佈韌體（取代手貼 service key）</t>
+          <t>內測版外殼（3D 打印 20 台）</t>
         </is>
       </c>
       <c r="C65" s="6" t="inlineStr">
         <is>
-          <t>等 P2-17、P1-10</t>
+          <t>等 R-01</t>
         </is>
       </c>
       <c r="D65" s="11" t="n"/>
@@ -2427,17 +2419,17 @@
     <row r="66" ht="18" customHeight="1">
       <c r="A66" s="13" t="inlineStr">
         <is>
-          <t>P2-21</t>
+          <t>R-06</t>
         </is>
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
-          <t>P2-16 ⑤ 後台 OTA 頁換成真實數據與操作</t>
+          <t>家長自助上手流程</t>
         </is>
       </c>
       <c r="C66" s="6" t="inlineStr">
         <is>
-          <t>等 P2-18、P2-19、P2-20、P2-14</t>
+          <t>等 P0-11</t>
         </is>
       </c>
       <c r="D66" s="11" t="n"/>
@@ -2447,20 +2439,20 @@
       <c r="H66" s="11" t="n"/>
       <c r="I66" s="12" t="n"/>
     </row>
-    <row r="67" ht="18" customHeight="1">
+    <row r="67" ht="32" customHeight="1">
       <c r="A67" s="13" t="inlineStr">
         <is>
-          <t>R-05</t>
+          <t>R-13</t>
         </is>
       </c>
       <c r="B67" s="6" t="inlineStr">
         <is>
-          <t>內測版外殼（3D 打印 20 台）</t>
+          <t>CP1 內測就緒檢查（10/30）</t>
         </is>
       </c>
       <c r="C67" s="6" t="inlineStr">
         <is>
-          <t>等 R-01</t>
+          <t>等 P0-07、P0-11、P1-01、P1-02、P2-09、R-01、R-02、R-04、R-05、R-06、P1-11</t>
         </is>
       </c>
       <c r="D67" s="11" t="n"/>
@@ -2470,20 +2462,20 @@
       <c r="H67" s="11" t="n"/>
       <c r="I67" s="12" t="n"/>
     </row>
-    <row r="68" ht="18" customHeight="1">
+    <row r="68" ht="32" customHeight="1">
       <c r="A68" s="13" t="inlineStr">
         <is>
-          <t>R-06</t>
+          <t>R-18</t>
         </is>
       </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t>家長自助上手流程</t>
+          <t>長按 BOOT 重新配網（開 AIBuddy-XXXX 熱點）</t>
         </is>
       </c>
       <c r="C68" s="6" t="inlineStr">
         <is>
-          <t>等 P0-11</t>
+          <t>等 R-01</t>
         </is>
       </c>
       <c r="D68" s="11" t="n"/>
@@ -2496,17 +2488,17 @@
     <row r="69" ht="32" customHeight="1">
       <c r="A69" s="13" t="inlineStr">
         <is>
-          <t>R-13</t>
+          <t>R-19</t>
         </is>
       </c>
       <c r="B69" s="6" t="inlineStr">
         <is>
-          <t>CP1 內測就緒檢查（10/30）</t>
+          <t>外接按鈕：量產板加 I2C 擴展晶片（TCA9555）</t>
         </is>
       </c>
       <c r="C69" s="6" t="inlineStr">
         <is>
-          <t>等 P0-07、P0-11、P1-01、P1-02、P2-09、R-01、R-02、R-04、R-05、R-06、P1-11</t>
+          <t>等 R-01</t>
         </is>
       </c>
       <c r="D69" s="11" t="n"/>
@@ -2516,20 +2508,20 @@
       <c r="H69" s="11" t="n"/>
       <c r="I69" s="12" t="n"/>
     </row>
-    <row r="70" ht="32" customHeight="1">
+    <row r="70" ht="18" customHeight="1">
       <c r="A70" s="13" t="inlineStr">
         <is>
-          <t>R-18</t>
+          <t>R-20</t>
         </is>
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>長按 BOOT 重新配網（開 AIBuddy-XXXX 熱點）</t>
+          <t>孩子資料與角色改成每台設備一份</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr">
         <is>
-          <t>等 R-01</t>
+          <t>等 P1-12</t>
         </is>
       </c>
       <c r="D70" s="11" t="n"/>
@@ -2542,17 +2534,17 @@
     <row r="71" ht="32" customHeight="1">
       <c r="A71" s="13" t="inlineStr">
         <is>
-          <t>R-19</t>
+          <t>R-27</t>
         </is>
       </c>
       <c r="B71" s="6" t="inlineStr">
         <is>
-          <t>外接按鈕：量產板加 I2C 擴展晶片（TCA9555）</t>
+          <t>App 內登入：驗證碼、原生社交登入、刪除帳號</t>
         </is>
       </c>
       <c r="C71" s="6" t="inlineStr">
         <is>
-          <t>等 R-01</t>
+          <t>等 R-26</t>
         </is>
       </c>
       <c r="D71" s="11" t="n"/>
@@ -2565,17 +2557,17 @@
     <row r="72" ht="18" customHeight="1">
       <c r="A72" s="13" t="inlineStr">
         <is>
-          <t>R-20</t>
+          <t>P0-14</t>
         </is>
       </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>孩子資料與角色改成每台設備一份</t>
+          <t>韌體簽章、Secure Boot 與 Flash 加密</t>
         </is>
       </c>
       <c r="C72" s="6" t="inlineStr">
         <is>
-          <t>等 P1-12</t>
+          <t>等 R-01</t>
         </is>
       </c>
       <c r="D72" s="11" t="n"/>
@@ -2585,20 +2577,20 @@
       <c r="H72" s="11" t="n"/>
       <c r="I72" s="12" t="n"/>
     </row>
-    <row r="73" ht="32" customHeight="1">
+    <row r="73" ht="18" customHeight="1">
       <c r="A73" s="13" t="inlineStr">
         <is>
-          <t>R-27</t>
+          <t>P1-06</t>
         </is>
       </c>
       <c r="B73" s="6" t="inlineStr">
         <is>
-          <t>App 內登入：驗證碼、原生社交登入、刪除帳號</t>
+          <t>處理 GPL-3.0 依賴（arduino-audio-tools）</t>
         </is>
       </c>
       <c r="C73" s="6" t="inlineStr">
         <is>
-          <t>等 R-26</t>
+          <t>等 Q3</t>
         </is>
       </c>
       <c r="D73" s="11" t="n"/>
@@ -2611,17 +2603,17 @@
     <row r="74" ht="18" customHeight="1">
       <c r="A74" s="13" t="inlineStr">
         <is>
-          <t>P0-14</t>
+          <t>P1-07</t>
         </is>
       </c>
       <c r="B74" s="6" t="inlineStr">
         <is>
-          <t>韌體簽章、Secure Boot 與 Flash 加密</t>
+          <t>LGPL 合規與第三方授權聲明</t>
         </is>
       </c>
       <c r="C74" s="6" t="inlineStr">
         <is>
-          <t>等 R-01</t>
+          <t>等 Q3</t>
         </is>
       </c>
       <c r="D74" s="11" t="n"/>
@@ -2634,17 +2626,17 @@
     <row r="75" ht="18" customHeight="1">
       <c r="A75" s="13" t="inlineStr">
         <is>
-          <t>P1-06</t>
+          <t>P1-08</t>
         </is>
       </c>
       <c r="B75" s="6" t="inlineStr">
         <is>
-          <t>處理 GPL-3.0 依賴（arduino-audio-tools）</t>
+          <t>硬件認證</t>
         </is>
       </c>
       <c r="C75" s="6" t="inlineStr">
         <is>
-          <t>等 Q3</t>
+          <t>等 R-01、R-05</t>
         </is>
       </c>
       <c r="D75" s="11" t="n"/>
@@ -2657,17 +2649,17 @@
     <row r="76" ht="18" customHeight="1">
       <c r="A76" s="13" t="inlineStr">
         <is>
-          <t>P1-07</t>
+          <t>P1-14</t>
         </is>
       </c>
       <c r="B76" s="6" t="inlineStr">
         <is>
-          <t>LGPL 合規與第三方授權聲明</t>
+          <t>Admin 內容安全頁：審核事件只按類別統計</t>
         </is>
       </c>
       <c r="C76" s="6" t="inlineStr">
         <is>
-          <t>等 Q3</t>
+          <t>等 P1-01、P2-13</t>
         </is>
       </c>
       <c r="D76" s="11" t="n"/>
@@ -2677,20 +2669,20 @@
       <c r="H76" s="11" t="n"/>
       <c r="I76" s="12" t="n"/>
     </row>
-    <row r="77" ht="18" customHeight="1">
+    <row r="77" ht="32" customHeight="1">
       <c r="A77" s="13" t="inlineStr">
         <is>
-          <t>P1-08</t>
+          <t>P2-15</t>
         </is>
       </c>
       <c r="B77" s="6" t="inlineStr">
         <is>
-          <t>硬件認證</t>
+          <t>Admin 總覽頁：在線、用量、成本與待處理事項</t>
         </is>
       </c>
       <c r="C77" s="6" t="inlineStr">
         <is>
-          <t>等 R-01、R-05</t>
+          <t>等 P2-14、P2-09</t>
         </is>
       </c>
       <c r="D77" s="11" t="n"/>
@@ -2703,17 +2695,17 @@
     <row r="78" ht="18" customHeight="1">
       <c r="A78" s="13" t="inlineStr">
         <is>
-          <t>P1-14</t>
+          <t>R-07</t>
         </is>
       </c>
       <c r="B78" s="6" t="inlineStr">
         <is>
-          <t>Admin 內容安全頁：審核事件只按類別統計</t>
+          <t>20 個家庭封閉內測</t>
         </is>
       </c>
       <c r="C78" s="6" t="inlineStr">
         <is>
-          <t>等 P1-01、P2-13</t>
+          <t>等 R-13</t>
         </is>
       </c>
       <c r="D78" s="11" t="n"/>
@@ -2723,20 +2715,20 @@
       <c r="H78" s="11" t="n"/>
       <c r="I78" s="12" t="n"/>
     </row>
-    <row r="79" ht="32" customHeight="1">
+    <row r="79" ht="18" customHeight="1">
       <c r="A79" s="13" t="inlineStr">
         <is>
-          <t>P2-15</t>
+          <t>R-08</t>
         </is>
       </c>
       <c r="B79" s="6" t="inlineStr">
         <is>
-          <t>Admin 總覽頁：在線、用量、成本與待處理事項</t>
+          <t>第 8 週關卡決策</t>
         </is>
       </c>
       <c r="C79" s="6" t="inlineStr">
         <is>
-          <t>等 P2-14、P2-09</t>
+          <t>等 R-07、P2-09、P1-08</t>
         </is>
       </c>
       <c r="D79" s="11" t="n"/>
@@ -2749,17 +2741,17 @@
     <row r="80" ht="18" customHeight="1">
       <c r="A80" s="13" t="inlineStr">
         <is>
-          <t>R-07</t>
+          <t>R-14</t>
         </is>
       </c>
       <c r="B80" s="6" t="inlineStr">
         <is>
-          <t>20 個家庭封閉內測</t>
+          <t>離線兒歌與故事</t>
         </is>
       </c>
       <c r="C80" s="6" t="inlineStr">
         <is>
-          <t>等 R-13</t>
+          <t>等 R-01</t>
         </is>
       </c>
       <c r="D80" s="11" t="n"/>
@@ -2772,17 +2764,17 @@
     <row r="81" ht="18" customHeight="1">
       <c r="A81" s="13" t="inlineStr">
         <is>
-          <t>R-08</t>
+          <t>R-24</t>
         </is>
       </c>
       <c r="B81" s="6" t="inlineStr">
         <is>
-          <t>第 8 週關卡決策</t>
+          <t>設備只能用自己品牌的角色</t>
         </is>
       </c>
       <c r="C81" s="6" t="inlineStr">
         <is>
-          <t>等 R-07、P2-09、P1-08</t>
+          <t>等 R-34</t>
         </is>
       </c>
       <c r="D81" s="11" t="n"/>
@@ -2795,17 +2787,17 @@
     <row r="82" ht="18" customHeight="1">
       <c r="A82" s="13" t="inlineStr">
         <is>
-          <t>R-14</t>
+          <t>R-28</t>
         </is>
       </c>
       <c r="B82" s="6" t="inlineStr">
         <is>
-          <t>離線兒歌與故事</t>
+          <t>三個 App 的殼：品牌版本與測試版</t>
         </is>
       </c>
       <c r="C82" s="6" t="inlineStr">
         <is>
-          <t>等 R-01</t>
+          <t>等 R-25、R-26</t>
         </is>
       </c>
       <c r="D82" s="11" t="n"/>
@@ -2818,17 +2810,17 @@
     <row r="83" ht="18" customHeight="1">
       <c r="A83" s="13" t="inlineStr">
         <is>
-          <t>R-24</t>
+          <t>R-30</t>
         </is>
       </c>
       <c r="B83" s="6" t="inlineStr">
         <is>
-          <t>設備只能用自己品牌的角色</t>
+          <t>快活 App（品牌 A）頁面</t>
         </is>
       </c>
       <c r="C83" s="6" t="inlineStr">
         <is>
-          <t>等 R-34</t>
+          <t>等 R-25、R-34、Q12</t>
         </is>
       </c>
       <c r="D83" s="11" t="n"/>
@@ -2841,17 +2833,17 @@
     <row r="84" ht="18" customHeight="1">
       <c r="A84" s="13" t="inlineStr">
         <is>
-          <t>R-28</t>
+          <t>R-31</t>
         </is>
       </c>
       <c r="B84" s="6" t="inlineStr">
         <is>
-          <t>三個 App 的殼：品牌版本與測試版</t>
+          <t>政協青年聯會版 App（品牌 B）頁面</t>
         </is>
       </c>
       <c r="C84" s="6" t="inlineStr">
         <is>
-          <t>等 R-25、R-26</t>
+          <t>等 R-25、R-34、Q13</t>
         </is>
       </c>
       <c r="D84" s="11" t="n"/>
@@ -2864,17 +2856,17 @@
     <row r="85" ht="18" customHeight="1">
       <c r="A85" s="13" t="inlineStr">
         <is>
-          <t>R-30</t>
+          <t>R-35</t>
         </is>
       </c>
       <c r="B85" s="6" t="inlineStr">
         <is>
-          <t>快活 App（品牌 A）頁面</t>
+          <t>韌體按品牌連線：伺服器網址在出廠時寫入</t>
         </is>
       </c>
       <c r="C85" s="6" t="inlineStr">
         <is>
-          <t>等 R-25、R-34、Q12</t>
+          <t>等 R-34</t>
         </is>
       </c>
       <c r="D85" s="11" t="n"/>
@@ -2884,20 +2876,20 @@
       <c r="H85" s="11" t="n"/>
       <c r="I85" s="12" t="n"/>
     </row>
-    <row r="86" ht="18" customHeight="1">
+    <row r="86" ht="32" customHeight="1">
       <c r="A86" s="13" t="inlineStr">
         <is>
-          <t>R-31</t>
+          <t>R-38</t>
         </is>
       </c>
       <c r="B86" s="6" t="inlineStr">
         <is>
-          <t>政協青年聯會版 App（品牌 B）頁面</t>
+          <t>公仔出廠鎖死所屬 IP，綁定時顯示該 IP 頭像</t>
         </is>
       </c>
       <c r="C86" s="6" t="inlineStr">
         <is>
-          <t>等 R-25、R-34、Q13</t>
+          <t>等 P0-11</t>
         </is>
       </c>
       <c r="D86" s="11" t="n"/>
@@ -2907,20 +2899,20 @@
       <c r="H86" s="11" t="n"/>
       <c r="I86" s="12" t="n"/>
     </row>
-    <row r="87" ht="18" customHeight="1">
+    <row r="87" ht="32" customHeight="1">
       <c r="A87" s="13" t="inlineStr">
         <is>
-          <t>R-35</t>
+          <t>R-39</t>
         </is>
       </c>
       <c r="B87" s="6" t="inlineStr">
         <is>
-          <t>韌體按品牌連線：伺服器網址在出廠時寫入</t>
+          <t>Admin 出廠登記頁：匯入 MAC 清單、指定公仔、查看自檢結果</t>
         </is>
       </c>
       <c r="C87" s="6" t="inlineStr">
         <is>
-          <t>等 R-34</t>
+          <t>等 R-38、P1-10</t>
         </is>
       </c>
       <c r="D87" s="11" t="n"/>
@@ -2930,20 +2922,20 @@
       <c r="H87" s="11" t="n"/>
       <c r="I87" s="12" t="n"/>
     </row>
-    <row r="88" ht="32" customHeight="1">
+    <row r="88" ht="18" customHeight="1">
       <c r="A88" s="13" t="inlineStr">
         <is>
-          <t>R-38</t>
+          <t>R-09</t>
         </is>
       </c>
       <c r="B88" s="6" t="inlineStr">
         <is>
-          <t>公仔出廠鎖死所屬 IP，綁定時顯示該 IP 頭像</t>
+          <t>量產外殼（真空複模）</t>
         </is>
       </c>
       <c r="C88" s="6" t="inlineStr">
         <is>
-          <t>等 P0-11</t>
+          <t>等 R-08、R-05、Q11</t>
         </is>
       </c>
       <c r="D88" s="11" t="n"/>
@@ -2953,20 +2945,20 @@
       <c r="H88" s="11" t="n"/>
       <c r="I88" s="12" t="n"/>
     </row>
-    <row r="89" ht="32" customHeight="1">
+    <row r="89" ht="18" customHeight="1">
       <c r="A89" s="13" t="inlineStr">
         <is>
-          <t>R-39</t>
+          <t>R-10</t>
         </is>
       </c>
       <c r="B89" s="6" t="inlineStr">
         <is>
-          <t>Admin 出廠登記頁：匯入 MAC 清單、指定公仔、查看自檢結果</t>
+          <t>出廠流程</t>
         </is>
       </c>
       <c r="C89" s="6" t="inlineStr">
         <is>
-          <t>等 R-38、P1-10</t>
+          <t>等 P0-14、R-01、P2-12、R-34、R-35、R-38、R-39</t>
         </is>
       </c>
       <c r="D89" s="11" t="n"/>
@@ -2979,17 +2971,17 @@
     <row r="90" ht="18" customHeight="1">
       <c r="A90" s="13" t="inlineStr">
         <is>
-          <t>R-09</t>
+          <t>R-11</t>
         </is>
       </c>
       <c r="B90" s="6" t="inlineStr">
         <is>
-          <t>量產外殼（真空複模）</t>
+          <t>售後：客服、保修與換機</t>
         </is>
       </c>
       <c r="C90" s="6" t="inlineStr">
         <is>
-          <t>等 R-08、R-05、Q11</t>
+          <t>等 P2-14、R-40</t>
         </is>
       </c>
       <c r="D90" s="11" t="n"/>
@@ -3002,17 +2994,17 @@
     <row r="91" ht="18" customHeight="1">
       <c r="A91" s="13" t="inlineStr">
         <is>
-          <t>R-10</t>
+          <t>R-15</t>
         </is>
       </c>
       <c r="B91" s="6" t="inlineStr">
         <is>
-          <t>出廠流程</t>
+          <t>農曆新年前交付（生產 1/15、送達 1/29）</t>
         </is>
       </c>
       <c r="C91" s="6" t="inlineStr">
         <is>
-          <t>等 P0-14、R-01、P2-12、R-34、R-35、R-38、R-39</t>
+          <t>等 R-09、R-10</t>
         </is>
       </c>
       <c r="D91" s="11" t="n"/>
@@ -3025,17 +3017,17 @@
     <row r="92" ht="18" customHeight="1">
       <c r="A92" s="13" t="inlineStr">
         <is>
-          <t>R-11</t>
+          <t>R-33</t>
         </is>
       </c>
       <c r="B92" s="6" t="inlineStr">
         <is>
-          <t>售後：客服、保修與換機</t>
+          <t>三個 App 送審並通過</t>
         </is>
       </c>
       <c r="C92" s="6" t="inlineStr">
         <is>
-          <t>等 P2-14、R-40</t>
+          <t>等 R-27、R-21、R-28、R-29、R-30、R-31、R-32</t>
         </is>
       </c>
       <c r="D92" s="11" t="n"/>
@@ -3045,20 +3037,20 @@
       <c r="H92" s="11" t="n"/>
       <c r="I92" s="12" t="n"/>
     </row>
-    <row r="93" ht="18" customHeight="1">
+    <row r="93" ht="32" customHeight="1">
       <c r="A93" s="13" t="inlineStr">
         <is>
-          <t>R-15</t>
+          <t>R-40</t>
         </is>
       </c>
       <c r="B93" s="6" t="inlineStr">
         <is>
-          <t>農曆新年前交付（生產 1/15、送達 1/29）</t>
+          <t>Admin 客服查詢頁：查帳號、名下設備與最近事件</t>
         </is>
       </c>
       <c r="C93" s="6" t="inlineStr">
         <is>
-          <t>等 R-09、R-10</t>
+          <t>等 P2-14、P1-10、P1-12</t>
         </is>
       </c>
       <c r="D93" s="11" t="n"/>
@@ -3068,73 +3060,73 @@
       <c r="H93" s="11" t="n"/>
       <c r="I93" s="12" t="n"/>
     </row>
-    <row r="94" ht="18" customHeight="1">
-      <c r="A94" s="13" t="inlineStr">
-        <is>
-          <t>R-33</t>
-        </is>
-      </c>
-      <c r="B94" s="6" t="inlineStr">
-        <is>
-          <t>三個 App 送審並通過</t>
-        </is>
-      </c>
-      <c r="C94" s="6" t="inlineStr">
-        <is>
-          <t>等 R-27、R-21、R-28、R-29、R-30、R-31、R-32</t>
-        </is>
-      </c>
-      <c r="D94" s="11" t="n"/>
-      <c r="E94" s="11" t="n"/>
-      <c r="F94" s="11" t="n"/>
-      <c r="G94" s="11" t="n"/>
-      <c r="H94" s="11" t="n"/>
-      <c r="I94" s="12" t="n"/>
-    </row>
-    <row r="95" ht="32" customHeight="1">
-      <c r="A95" s="13" t="inlineStr">
-        <is>
-          <t>R-40</t>
-        </is>
-      </c>
-      <c r="B95" s="6" t="inlineStr">
-        <is>
-          <t>Admin 客服查詢頁：查帳號、名下設備與最近事件</t>
-        </is>
-      </c>
-      <c r="C95" s="6" t="inlineStr">
-        <is>
-          <t>等 P2-14、P1-10、P1-12</t>
-        </is>
-      </c>
-      <c r="D95" s="11" t="n"/>
-      <c r="E95" s="11" t="n"/>
-      <c r="F95" s="11" t="n"/>
-      <c r="G95" s="11" t="n"/>
-      <c r="H95" s="11" t="n"/>
-      <c r="I95" s="12" t="n"/>
-    </row>
-    <row r="97">
-      <c r="A97" s="10" t="inlineStr">
+    <row r="95">
+      <c r="A95" s="10" t="inlineStr">
         <is>
           <t>❓ 待確認問題</t>
         </is>
       </c>
     </row>
-    <row r="98">
-      <c r="A98" s="4" t="inlineStr">
+    <row r="96">
+      <c r="A96" s="4" t="inlineStr">
         <is>
           <t>編號</t>
         </is>
       </c>
-      <c r="B98" s="4" t="inlineStr">
+      <c r="B96" s="4" t="inlineStr">
         <is>
           <t>問題</t>
         </is>
       </c>
-      <c r="C98" s="4" t="inlineStr">
+      <c r="C96" s="4" t="inlineStr">
         <is>
           <t>影響的任務 / 為什麼重要</t>
+        </is>
+      </c>
+      <c r="D96" s="11" t="n"/>
+      <c r="E96" s="11" t="n"/>
+      <c r="F96" s="11" t="n"/>
+      <c r="G96" s="11" t="n"/>
+      <c r="H96" s="11" t="n"/>
+      <c r="I96" s="12" t="n"/>
+    </row>
+    <row r="97" ht="18" customHeight="1">
+      <c r="A97" s="13" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="B97" s="6" t="inlineStr">
+        <is>
+          <t>韌體打算閉源商業銷售嗎？</t>
+        </is>
+      </c>
+      <c r="C97" s="6" t="inlineStr">
+        <is>
+          <t>P1-06, P1-07：決定 GPL／LGPL 依賴要開源還是替換。</t>
+        </is>
+      </c>
+      <c r="D97" s="11" t="n"/>
+      <c r="E97" s="11" t="n"/>
+      <c r="F97" s="11" t="n"/>
+      <c r="G97" s="11" t="n"/>
+      <c r="H97" s="11" t="n"/>
+      <c r="I97" s="12" t="n"/>
+    </row>
+    <row r="98" ht="32" customHeight="1">
+      <c r="A98" s="13" t="inlineStr">
+        <is>
+          <t>Q11</t>
+        </is>
+      </c>
+      <c r="B98" s="6" t="inlineStr">
+        <is>
+          <t>馬會快活的賽馬日版和新春版各多少隻（共 2,500）？</t>
+        </is>
+      </c>
+      <c r="C98" s="6" t="inlineStr">
+        <is>
+          <t>R-09, R-15：兩款的服裝和配件要分開訂料；11/20 前不知道，PP 樣和大貨單（11/27）會被拖慢。由馬會決定。</t>
         </is>
       </c>
       <c r="D98" s="11" t="n"/>
@@ -3144,20 +3136,20 @@
       <c r="H98" s="11" t="n"/>
       <c r="I98" s="12" t="n"/>
     </row>
-    <row r="99" ht="18" customHeight="1">
+    <row r="99" ht="60" customHeight="1">
       <c r="A99" s="13" t="inlineStr">
         <is>
-          <t>Q3</t>
+          <t>Q12</t>
         </is>
       </c>
       <c r="B99" s="6" t="inlineStr">
         <is>
-          <t>韌體打算閉源商業銷售嗎？</t>
+          <t>快活 App 的「會員綁定」是指甚麼：用我們自己的帳號（email 驗證碼），還是接馬會的會員帳號登入（SSO）？</t>
         </is>
       </c>
       <c r="C99" s="6" t="inlineStr">
         <is>
-          <t>P1-06, P1-07：決定 GPL／LGPL 依賴要開源還是替換。</t>
+          <t>P0-11, 快活 App（未入追蹤表）：接馬會 SSO 的話，登入、帳號刪除和資料歸屬都要按馬會的介面重做，工作量和排期要另估，而且 W5（11/9–11/13）就要做快活 App 的綁定；用我們的帳號則和其他品牌共用同一套流程。由馬會決定，要盡早問。</t>
         </is>
       </c>
       <c r="D99" s="11" t="n"/>
@@ -3167,20 +3159,20 @@
       <c r="H99" s="11" t="n"/>
       <c r="I99" s="12" t="n"/>
     </row>
-    <row r="100" ht="32" customHeight="1">
+    <row r="100" ht="46" customHeight="1">
       <c r="A100" s="13" t="inlineStr">
         <is>
-          <t>Q11</t>
+          <t>Q13</t>
         </is>
       </c>
       <c r="B100" s="6" t="inlineStr">
         <is>
-          <t>馬會快活的賽馬日版和新春版各多少隻（共 2,500）？</t>
+          <t>政協青年聯會版的角色、語言和內容由誰提供？什麼時候交？</t>
         </is>
       </c>
       <c r="C100" s="6" t="inlineStr">
         <is>
-          <t>R-09, R-15：兩款的服裝和配件要分開訂料；11/20 前不知道，PP 樣和大貨單（11/27）會被拖慢。由馬會決定。</t>
+          <t>品牌 B 的 App 頁面：品牌 B 的用戶是成人會員，但角色、說話語言、內容規則都還沒有。最遲 11/13 要拿到，才趕得及內部測試和 App 頁面（W6）。</t>
         </is>
       </c>
       <c r="D100" s="11" t="n"/>
@@ -3190,100 +3182,52 @@
       <c r="H100" s="11" t="n"/>
       <c r="I100" s="12" t="n"/>
     </row>
-    <row r="101" ht="60" customHeight="1">
-      <c r="A101" s="13" t="inlineStr">
-        <is>
-          <t>Q12</t>
-        </is>
-      </c>
-      <c r="B101" s="6" t="inlineStr">
-        <is>
-          <t>快活 App 的「會員綁定」是指甚麼：用我們自己的帳號（email 驗證碼），還是接馬會的會員帳號登入（SSO）？</t>
-        </is>
-      </c>
-      <c r="C101" s="6" t="inlineStr">
-        <is>
-          <t>P0-11, 快活 App（未入追蹤表）：接馬會 SSO 的話，登入、帳號刪除和資料歸屬都要按馬會的介面重做，工作量和排期要另估，而且 W5（11/9–11/13）就要做快活 App 的綁定；用我們的帳號則和其他品牌共用同一套流程。由馬會決定，要盡早問。</t>
-        </is>
-      </c>
-      <c r="D101" s="11" t="n"/>
-      <c r="E101" s="11" t="n"/>
-      <c r="F101" s="11" t="n"/>
-      <c r="G101" s="11" t="n"/>
-      <c r="H101" s="11" t="n"/>
-      <c r="I101" s="12" t="n"/>
-    </row>
-    <row r="102" ht="46" customHeight="1">
-      <c r="A102" s="13" t="inlineStr">
-        <is>
-          <t>Q13</t>
-        </is>
-      </c>
-      <c r="B102" s="6" t="inlineStr">
-        <is>
-          <t>政協青年聯會版的角色、語言和內容由誰提供？什麼時候交？</t>
-        </is>
-      </c>
-      <c r="C102" s="6" t="inlineStr">
-        <is>
-          <t>品牌 B 的 App 頁面：品牌 B 的用戶是成人會員，但角色、說話語言、內容規則都還沒有。最遲 11/13 要拿到，才趕得及內部測試和 App 頁面（W6）。</t>
-        </is>
-      </c>
-      <c r="D102" s="11" t="n"/>
-      <c r="E102" s="11" t="n"/>
-      <c r="F102" s="11" t="n"/>
-      <c r="G102" s="11" t="n"/>
-      <c r="H102" s="11" t="n"/>
-      <c r="I102" s="12" t="n"/>
-    </row>
-    <row r="104">
-      <c r="A104" s="10" t="inlineStr">
+    <row r="102">
+      <c r="A102" s="10" t="inlineStr">
         <is>
           <t>說明</t>
         </is>
       </c>
     </row>
-    <row r="105" ht="32" customHeight="1">
+    <row r="103" ht="32" customHeight="1">
+      <c r="A103" s="14" t="inlineStr">
+        <is>
+          <t>・狀態：未開始 → 進行中 → 已完成。只有測試真的跑過而且通過才算已完成；阻塞要在備註寫原因；不再需要的任務標不適用，不要刪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" ht="18" customHeight="1">
+      <c r="A104" s="14" t="inlineStr">
+        <is>
+          <t>・測試結果：未測試 / 通過 / 失敗 / 部分通過。測試證據寫跑了什麼、看到什麼，完整歷史在「更新記錄」。</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" ht="18" customHeight="1">
       <c r="A105" s="14" t="inlineStr">
         <is>
-          <t>・狀態：未開始 → 進行中 → 已完成。只有測試真的跑過而且通過才算已完成；阻塞要在備註寫原因；不再需要的任務標不適用，不要刪。</t>
+          <t>・「接下來」按階段排序，同一階段內再按優先級；依賴還沒滿足的任務不會出現在「接下來」。</t>
         </is>
       </c>
     </row>
     <row r="106" ht="18" customHeight="1">
       <c r="A106" s="14" t="inlineStr">
         <is>
-          <t>・測試結果：未測試 / 通過 / 失敗 / 部分通過。測試證據寫跑了什麼、看到什麼，完整歷史在「更新記錄」。</t>
-        </is>
-      </c>
-    </row>
-    <row r="107" ht="18" customHeight="1">
+          <t>・可以手動改：「任務清單」的狀態、測試結果、測試證據、Commit、備註，以及「待確認問題」的回答。其餘欄位和本頁由腳本維護。</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" ht="32" customHeight="1">
       <c r="A107" s="14" t="inlineStr">
         <is>
-          <t>・「接下來」按階段排序，同一階段內再按優先級；依賴還沒滿足的任務不會出現在「接下來」。</t>
-        </is>
-      </c>
-    </row>
-    <row r="108" ht="18" customHeight="1">
-      <c r="A108" s="14" t="inlineStr">
-        <is>
-          <t>・可以手動改：「任務清單」的狀態、測試結果、測試證據、Commit、備註，以及「待確認問題」的回答。其餘欄位和本頁由腳本維護。</t>
-        </is>
-      </c>
-    </row>
-    <row r="109" ht="32" customHeight="1">
-      <c r="A109" s="14" t="inlineStr">
-        <is>
           <t>・建議用法：在 Claude Code 對 Claude 說「P0-02 做完了」或輸入 /prod-readiness。Claude 會先跑測試再更新，並寫進「更新記錄」。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="90">
-    <mergeCell ref="A108:I108"/>
+  <mergeCells count="88">
     <mergeCell ref="C82:I82"/>
     <mergeCell ref="E52:I52"/>
-    <mergeCell ref="A56:I56"/>
     <mergeCell ref="E39:I39"/>
     <mergeCell ref="C67:I67"/>
     <mergeCell ref="E48:I48"/>
@@ -3292,13 +3236,13 @@
     <mergeCell ref="E38:I38"/>
     <mergeCell ref="C83:I83"/>
     <mergeCell ref="C92:I92"/>
-    <mergeCell ref="A109:I109"/>
     <mergeCell ref="E31:I31"/>
     <mergeCell ref="E40:I40"/>
+    <mergeCell ref="C97:I97"/>
     <mergeCell ref="A19:I19"/>
     <mergeCell ref="E26:I26"/>
+    <mergeCell ref="A103:I103"/>
     <mergeCell ref="E25:I25"/>
-    <mergeCell ref="C95:I95"/>
     <mergeCell ref="C60:I60"/>
     <mergeCell ref="C71:I71"/>
     <mergeCell ref="E50:I50"/>
@@ -3307,7 +3251,6 @@
     <mergeCell ref="A105:I105"/>
     <mergeCell ref="C57:I57"/>
     <mergeCell ref="C66:I66"/>
-    <mergeCell ref="C102:I102"/>
     <mergeCell ref="E20:I20"/>
     <mergeCell ref="E28:I28"/>
     <mergeCell ref="C77:I77"/>
@@ -3317,56 +3260,57 @@
     <mergeCell ref="E30:I30"/>
     <mergeCell ref="E22:I22"/>
     <mergeCell ref="E46:I46"/>
+    <mergeCell ref="A102:I102"/>
     <mergeCell ref="C85:I85"/>
     <mergeCell ref="C100:I100"/>
-    <mergeCell ref="C94:I94"/>
     <mergeCell ref="C65:I65"/>
     <mergeCell ref="C75:I75"/>
     <mergeCell ref="C84:I84"/>
     <mergeCell ref="C80:I80"/>
-    <mergeCell ref="E54:I54"/>
     <mergeCell ref="E32:I32"/>
     <mergeCell ref="C59:I59"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="E41:I41"/>
-    <mergeCell ref="A45:I45"/>
     <mergeCell ref="E47:I47"/>
     <mergeCell ref="C61:I61"/>
-    <mergeCell ref="E43:I43"/>
     <mergeCell ref="C70:I70"/>
     <mergeCell ref="E24:I24"/>
     <mergeCell ref="E33:I33"/>
     <mergeCell ref="A3:I3"/>
+    <mergeCell ref="A55:I55"/>
     <mergeCell ref="A104:I104"/>
     <mergeCell ref="E35:I35"/>
-    <mergeCell ref="C101:I101"/>
     <mergeCell ref="A106:I106"/>
     <mergeCell ref="C74:I74"/>
     <mergeCell ref="C88:I88"/>
+    <mergeCell ref="E45:I45"/>
     <mergeCell ref="C99:I99"/>
     <mergeCell ref="E37:I37"/>
     <mergeCell ref="E21:I21"/>
     <mergeCell ref="E23:I23"/>
     <mergeCell ref="C72:I72"/>
     <mergeCell ref="C81:I81"/>
+    <mergeCell ref="A95:I95"/>
     <mergeCell ref="C69:I69"/>
     <mergeCell ref="E51:I51"/>
+    <mergeCell ref="C96:I96"/>
     <mergeCell ref="C78:I78"/>
     <mergeCell ref="C87:I87"/>
     <mergeCell ref="C62:I62"/>
-    <mergeCell ref="A97:I97"/>
     <mergeCell ref="C98:I98"/>
     <mergeCell ref="C89:I89"/>
     <mergeCell ref="E34:I34"/>
     <mergeCell ref="C64:I64"/>
     <mergeCell ref="C79:I79"/>
     <mergeCell ref="C73:I73"/>
+    <mergeCell ref="A44:I44"/>
     <mergeCell ref="E49:I49"/>
     <mergeCell ref="E27:I27"/>
     <mergeCell ref="E36:I36"/>
     <mergeCell ref="C63:I63"/>
     <mergeCell ref="C93:I93"/>
     <mergeCell ref="A107:I107"/>
+    <mergeCell ref="C56:I56"/>
     <mergeCell ref="C90:I90"/>
     <mergeCell ref="E53:I53"/>
     <mergeCell ref="C76:I76"/>
@@ -9865,7 +9809,7 @@
         </is>
       </c>
     </row>
-    <row r="90" ht="102" customHeight="1">
+    <row r="90" ht="186" customHeight="1">
       <c r="A90" s="13" t="inlineStr">
         <is>
           <t>P2-17</t>
@@ -9893,12 +9837,17 @@
       </c>
       <c r="F90" s="13" t="inlineStr">
         <is>
-          <t>進行中</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="G90" s="13" t="inlineStr">
         <is>
-          <t>未測試</t>
+          <t>通過</t>
+        </is>
+      </c>
+      <c r="H90" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="I90" s="6" t="inlineStr">
@@ -9918,7 +9867,7 @@
       </c>
       <c r="L90" s="6" t="inlineStr">
         <is>
-          <t>本機 Supabase BEGIN/ROLLBACK 套用兩次無錯；內容管理員、anon 讀新表 → 42501；現有 release_firmware.py promote 後 1.0.1 仍照常下發（token 路徑 API 測試不變）</t>
+          <t>本機 Supabase BEGIN/ROLLBACK 套用兩次無錯；經 REST 用 GoTrue 真實登入：anon 讀新表 → 42501，內容管理員讀新表 → 0 行（RLS，與 firmware_releases 一致），anon／內容管理員／超管寫新表、改發佈階段、呼叫 ota_note_* → 42501，超管可讀；現有 release_firmware.py promote 後 current 版本照常被 token 路徑的查詢選中</t>
         </is>
       </c>
       <c r="M90" s="13" t="inlineStr">
@@ -9926,10 +9875,21 @@
           <t>P0-13</t>
         </is>
       </c>
+      <c r="N90" s="6" t="inlineStr">
+        <is>
+          <t>migration 20261014190000 BEGIN/ROLLBACK 套用兩次無錯並已套用本機；行為：預設 100%、promote 記 stage_changed_at，7 種壞值（25%、小寫/空字串/NULL MAC、暫停缺原因等）全被 check 擋；ota_note_offer 1→2→3，report 正確標 running/failed、別板型不影響，刪發佈連帶刪記錄；審計 5 筆含 'test-board 9.9.9' 標籤。REST 13/13：超管可讀、內容管理員 0 行、anon 42501，三種身份寫入/改階段/呼叫 ota_note_offer 皆 42501。release_firmware.py promote spotpear-ai-toy 1.6.2 成功，token 查詢仍選 1.6.2，審計記 2 筆（actor 空＝service role）</t>
+        </is>
+      </c>
+      <c r="O90" s="13" t="inlineStr">
+        <is>
+          <t>9f44e32</t>
+        </is>
+      </c>
       <c r="P90" s="6" t="inlineStr">
         <is>
           <t>[2026-10-14] 新增：2026-10-14 分支 p2-16-ota-rollout（worktree ../aibuddy-p216）
-[2026-10-14] 2026-10-14 用戶決定提前到第 2 階段，現在開始做</t>
+[2026-10-14] 2026-10-14 用戶決定提前到第 2 階段，現在開始做
+[2026-10-14] 測試方法修正：內容管理員讀取在 RLS 下是 200 + 0 行而非 42501，保護效果相同（看不到任何行），寫入一律 42501</t>
         </is>
       </c>
     </row>
@@ -10787,7 +10747,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I284"/>
+  <dimension ref="A1:I286"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -20581,8 +20541,86 @@
       <c r="H284" s="13" t="n"/>
       <c r="I284" s="6" t="n"/>
     </row>
+    <row r="285" ht="60" customHeight="1">
+      <c r="A285" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 20:45</t>
+        </is>
+      </c>
+      <c r="B285" s="13" t="inlineStr">
+        <is>
+          <t>P2-17</t>
+        </is>
+      </c>
+      <c r="C285" s="6" t="inlineStr">
+        <is>
+          <t>P2-16 ① 分批推送的數據表：推送階段、白名單、每台安裝結果</t>
+        </is>
+      </c>
+      <c r="D285" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="E285" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F285" s="13" t="n"/>
+      <c r="G285" s="6" t="n"/>
+      <c r="H285" s="13" t="n"/>
+      <c r="I285" s="6" t="inlineStr">
+        <is>
+          <t>測試方法修正：內容管理員讀取在 RLS 下是 200 + 0 行而非 42501，保護效果相同（看不到任何行），寫入一律 42501；修改了測試方法</t>
+        </is>
+      </c>
+    </row>
+    <row r="286" ht="158" customHeight="1">
+      <c r="A286" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 20:45</t>
+        </is>
+      </c>
+      <c r="B286" s="13" t="inlineStr">
+        <is>
+          <t>P2-17</t>
+        </is>
+      </c>
+      <c r="C286" s="6" t="inlineStr">
+        <is>
+          <t>P2-16 ① 分批推送的數據表：推送階段、白名單、每台安裝結果</t>
+        </is>
+      </c>
+      <c r="D286" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="E286" s="13" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="F286" s="13" t="inlineStr">
+        <is>
+          <t>通過</t>
+        </is>
+      </c>
+      <c r="G286" s="6" t="inlineStr">
+        <is>
+          <t>migration 20261014190000 BEGIN/ROLLBACK 套用兩次無錯並已套用本機；行為：預設 100%、promote 記 stage_changed_at，7 種壞值（25%、小寫/空字串/NULL MAC、暫停缺原因等）全被 check 擋；ota_note_offer 1→2→3，report 正確標 running/failed、別板型不影響，刪發佈連帶刪記錄；審計 5 筆含 'test-board 9.9.9' 標籤。REST 13/13：超管可讀、內容管理員 0 行、anon 42501，三種身份寫入/改階段/呼叫 ota_note_offer 皆 42501。release_firmware.py promote spotpear-ai-toy 1.6.2 成功，token 查詢仍選 1.6.2，審計記 2 筆（actor 空＝service role）</t>
+        </is>
+      </c>
+      <c r="H286" s="13" t="inlineStr">
+        <is>
+          <t>9f44e32</t>
+        </is>
+      </c>
+      <c r="I286" s="6" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I284"/>
+  <autoFilter ref="A1:I286"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Point P2-17 at its rebased commit.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/production-readiness.xlsx
+++ b/docs/production-readiness.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'任務清單'!$A$1:$P$94</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'待確認問題'!$A$1:$G$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$286</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$287</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -9882,14 +9882,15 @@
       </c>
       <c r="O90" s="13" t="inlineStr">
         <is>
-          <t>9f44e32</t>
+          <t>8675970</t>
         </is>
       </c>
       <c r="P90" s="6" t="inlineStr">
         <is>
           <t>[2026-10-14] 新增：2026-10-14 分支 p2-16-ota-rollout（worktree ../aibuddy-p216）
 [2026-10-14] 2026-10-14 用戶決定提前到第 2 階段，現在開始做
-[2026-10-14] 測試方法修正：內容管理員讀取在 RLS 下是 200 + 0 行而非 42501，保護效果相同（看不到任何行），寫入一律 42501</t>
+[2026-10-14] 測試方法修正：內容管理員讀取在 RLS 下是 200 + 0 行而非 42501，保護效果相同（看不到任何行），寫入一律 42501
+[2026-10-14] commit 在分支 p2-16-ota-rollout（rebase 後 9f44e32 → 8675970），未合併到 dev、未部署</t>
         </is>
       </c>
     </row>
@@ -10747,7 +10748,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I286"/>
+  <dimension ref="A1:I287"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -20619,8 +20620,47 @@
       </c>
       <c r="I286" s="6" t="n"/>
     </row>
+    <row r="287" ht="46" customHeight="1">
+      <c r="A287" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 20:45</t>
+        </is>
+      </c>
+      <c r="B287" s="13" t="inlineStr">
+        <is>
+          <t>P2-17</t>
+        </is>
+      </c>
+      <c r="C287" s="6" t="inlineStr">
+        <is>
+          <t>P2-16 ① 分批推送的數據表：推送階段、白名單、每台安裝結果</t>
+        </is>
+      </c>
+      <c r="D287" s="13" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="E287" s="13" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="F287" s="13" t="n"/>
+      <c r="G287" s="6" t="n"/>
+      <c r="H287" s="13" t="inlineStr">
+        <is>
+          <t>8675970</t>
+        </is>
+      </c>
+      <c r="I287" s="6" t="inlineStr">
+        <is>
+          <t>commit 在分支 p2-16-ota-rollout（rebase 後 9f44e32 → 8675970），未合併到 dev、未部署</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I286"/>
+  <autoFilter ref="A1:I287"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Track P2-18 (staged rollout in the token route) as passed.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/production-readiness.xlsx
+++ b/docs/production-readiness.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'任務清單'!$A$1:$P$94</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'待確認問題'!$A$1:$G$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$287</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$290</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -641,7 +641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I107"/>
+  <dimension ref="A1:I106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -665,14 +665,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>最後更新：2026-10-14 20:45　·　本頁由 tracker.py 自動生成，請勿手動編輯</t>
+          <t>最後更新：2026-10-14 20:50　·　本頁由 tracker.py 自動生成，請勿手動編輯</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>總進度：19/89 已完成（21%）　·　目前階段：1 止血定案（10/5–10/16）</t>
+          <t>總進度：20/89 已完成（22%）　·　目前階段：1 止血定案（10/5–10/16）</t>
         </is>
       </c>
     </row>
@@ -820,7 +820,7 @@
       </c>
       <c r="D8" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A8,'任務清單'!$F:$F,D$5)</f>
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E8" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A8,'任務清單'!$F:$F,E$5)</f>
@@ -828,7 +828,7 @@
       </c>
       <c r="F8" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A8,'任務清單'!$F:$F,F$5)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G8" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A8,'任務清單'!$F:$F,G$5)</f>
@@ -840,7 +840,7 @@
       </c>
       <c r="I8" s="8">
         <f>IFERROR(F8/(C8-H8),0)</f>
-        <v>0.19047619047619047</v>
+        <v>0.23809523809523808</v>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1">
@@ -896,7 +896,7 @@
       </c>
       <c r="D10" s="5">
         <f>SUM(D6:D9)</f>
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E10" s="5">
         <f>SUM(E6:E9)</f>
@@ -904,7 +904,7 @@
       </c>
       <c r="F10" s="5">
         <f>SUM(F6:F9)</f>
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G10" s="5">
         <f>SUM(G6:G9)</f>
@@ -916,7 +916,7 @@
       </c>
       <c r="I10" s="9">
         <f>IFERROR(F10/(C10-H10),0)</f>
-        <v>0.21348314606741572</v>
+        <v>0.2247191011235955</v>
       </c>
     </row>
     <row r="12">
@@ -1023,7 +1023,7 @@
       </c>
       <c r="D14" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A14,'任務清單'!$F:$F,D$12)</f>
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E14" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A14,'任務清單'!$F:$F,E$12)</f>
@@ -1031,7 +1031,7 @@
       </c>
       <c r="F14" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A14,'任務清單'!$F:$F,F$12)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G14" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A14,'任務清單'!$F:$F,G$12)</f>
@@ -1043,7 +1043,7 @@
       </c>
       <c r="I14" s="8">
         <f>IFERROR(F14/(C14-H14),0)</f>
-        <v>0.12121212121212122</v>
+        <v>0.15151515151515152</v>
       </c>
     </row>
     <row r="15" ht="46" customHeight="1">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="D17" s="5">
         <f>SUM(D13:D16)</f>
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E17" s="5">
         <f>SUM(E13:E16)</f>
@@ -1147,7 +1147,7 @@
       </c>
       <c r="F17" s="5">
         <f>SUM(F13:F16)</f>
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G17" s="5">
         <f>SUM(G13:G16)</f>
@@ -1159,7 +1159,7 @@
       </c>
       <c r="I17" s="9">
         <f>IFERROR(F17/(C17-H17),0)</f>
-        <v>0.21348314606741572</v>
+        <v>0.2247191011235955</v>
       </c>
     </row>
     <row r="19">
@@ -1834,12 +1834,12 @@
     <row r="41" ht="74" customHeight="1">
       <c r="A41" s="13" t="inlineStr">
         <is>
-          <t>P2-18</t>
+          <t>P2-19</t>
         </is>
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>P2-16 ② 按 MAC 雜湊穩定分組決定哪台收到 ota</t>
+          <t>P2-16 ③ 回滾過多時自動暫停推送</t>
         </is>
       </c>
       <c r="C41" s="13" t="inlineStr">
@@ -1854,7 +1854,7 @@
       </c>
       <c r="E41" s="6" t="inlineStr">
         <is>
-          <t>白名單階段只有名單內 MAC 拿到 ota；10%／50%／100% 按 MAC 雜湊（加版本作鹽）穩定分組，同一台重複請求結果不變，升階段時已在組內的不會掉出；暫停時一律不下發；每次下發與結果寫入 ① 的記錄；不用改韌體。</t>
+          <t>已下發的設備中回滾率 &gt; 5%，或任一台對同一版本被下發 3 次仍未確認，即自動暫停該版本並記下原因；暫停後其餘設備不再拿到 ota；已確認的設備不受影響；自動暫停寫入審計記錄（操作者記為系統）；只能由超級管理員在後台恢復。</t>
         </is>
       </c>
       <c r="F41" s="11" t="n"/>
@@ -1931,15 +1931,15 @@
       <c r="H45" s="11" t="n"/>
       <c r="I45" s="12" t="n"/>
     </row>
-    <row r="46" ht="172" customHeight="1">
+    <row r="46" ht="200" customHeight="1">
       <c r="A46" s="13" t="inlineStr">
         <is>
-          <t>P2-17</t>
+          <t>P2-18</t>
         </is>
       </c>
       <c r="B46" s="6" t="inlineStr">
         <is>
-          <t>P2-16 ① 分批推送的數據表：推送階段、白名單、每台安裝結果</t>
+          <t>P2-16 ② 按 MAC 雜湊穩定分組決定哪台收到 ota</t>
         </is>
       </c>
       <c r="C46" s="13" t="inlineStr">
@@ -1954,7 +1954,7 @@
       </c>
       <c r="E46" s="6" t="inlineStr">
         <is>
-          <t>migration 20261014190000 BEGIN/ROLLBACK 套用兩次無錯並已套用本機；行為：預設 100%、promote 記 stage_changed_at，7 種壞值（25%、小寫/空字串/NULL MAC、暫停缺原因等）全被 check 擋；ota_note_offer 1→2→3，report 正確標 running/failed、別板型不影響，刪發佈連帶刪記錄；審計 5 筆含 'test-board 9.9.9' 標籤。REST 13/13：超管可讀、內容管理員 0 行、anon 42501，三種身份寫入/改階段/呼叫 ota_note_offer 皆 42501。release_firmware.py promote spotpear-ai-toy 1.6.2 成功，token 查詢仍選 1.6.2，審計記 2 筆（actor 空＝service role）</t>
+          <t>node --test lib/otaRollout.test.mjs 6/6：10,000 隨機 MAC 在 10%/50% 誤差 &lt; 1 個百分點、同 MAC（含大小寫/空白）結果一致、升階段只增不減、白名單各階段都在、不同版本選不同的 10%。tsc --noEmit 通過。分支 dev server（3216）+ 本機 Supabase 模擬 20 台（板型 p218-sim，連跑兩次 9/9）：白名單階段只有 1 台、重複不變；10% 拿到的正是雜湊預測的那組（2–5 台含白名單），重複不變；50% 包含 10% 全部；暫停 → 0 台且下載映像 404，恢復 → 200；100% → 除已更新和已回滾的 2 台外 18 台；每台下發次數與記錄一致；運行中/已回滾正確標記；審計 6 筆對應 6 次變更。真 spotpear-ai-toy（預設 100%）回報 1.6.1 → 仍拿到 1.6.2。測試數據已清除</t>
         </is>
       </c>
       <c r="F46" s="11" t="n"/>
@@ -1962,15 +1962,15 @@
       <c r="H46" s="11" t="n"/>
       <c r="I46" s="12" t="n"/>
     </row>
-    <row r="47" ht="116" customHeight="1">
+    <row r="47" ht="172" customHeight="1">
       <c r="A47" s="13" t="inlineStr">
         <is>
-          <t>R-41</t>
+          <t>P2-17</t>
         </is>
       </c>
       <c r="B47" s="6" t="inlineStr">
         <is>
-          <t>App 顯示玩具電量狀態（低電量提示）</t>
+          <t>P2-16 ① 分批推送的數據表：推送階段、白名單、每台安裝結果</t>
         </is>
       </c>
       <c r="C47" s="13" t="inlineStr">
@@ -1985,7 +1985,7 @@
       </c>
       <c r="E47" s="6" t="inlineStr">
         <is>
-          <t>① pytest 33 passed；真 PATCH 本地 Supabase ② 62:70 刷 p212+R-41 強制低電 build（SUPPLY_LOW_RATIO_OVERRIDE=1.05）→ 串口 [WSc] power low:true，本地 DB battery_low=t ③ 刷回正常 1.6.2 → low:false，DB=f ④ App 讀 DB：低電紅標+Please charge+更新時間、72% 充電中、未上報不顯示 ⑤ 他人帳號 0 行、authenticated UPDATE 被拒。62:70 已還原為原 p212 build</t>
+          <t>migration 20261014190000 BEGIN/ROLLBACK 套用兩次無錯並已套用本機；行為：預設 100%、promote 記 stage_changed_at，7 種壞值（25%、小寫/空字串/NULL MAC、暫停缺原因等）全被 check 擋；ota_note_offer 1→2→3，report 正確標 running/failed、別板型不影響，刪發佈連帶刪記錄；審計 5 筆含 'test-board 9.9.9' 標籤。REST 13/13：超管可讀、內容管理員 0 行、anon 42501，三種身份寫入/改階段/呼叫 ota_note_offer 皆 42501。release_firmware.py promote spotpear-ai-toy 1.6.2 成功，token 查詢仍選 1.6.2，審計記 2 筆（actor 空＝service role）</t>
         </is>
       </c>
       <c r="F47" s="11" t="n"/>
@@ -1993,15 +1993,15 @@
       <c r="H47" s="11" t="n"/>
       <c r="I47" s="12" t="n"/>
     </row>
-    <row r="48" ht="102" customHeight="1">
+    <row r="48" ht="116" customHeight="1">
       <c r="A48" s="13" t="inlineStr">
         <is>
-          <t>P0-12</t>
+          <t>R-41</t>
         </is>
       </c>
       <c r="B48" s="6" t="inlineStr">
         <is>
-          <t>收緊 Admin 權限與路由保護</t>
+          <t>App 顯示玩具電量狀態（低電量提示）</t>
         </is>
       </c>
       <c r="C48" s="13" t="inlineStr">
@@ -2011,12 +2011,12 @@
       </c>
       <c r="D48" s="13" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E48" s="6" t="inlineStr">
         <is>
-          <t>線上 2026-10-12（bac24e9）：runbook 10/08 檢查 未登入 /admin→/login、/api/admin→401、has_role() 只看角色、無管理員 policy 觸及 conversations/記憶表、超管≥1；未登入 /home、/admin→/login；用戶確認：家長帳號開 /admin 轉回 /home、管理員在 /admin 修改角色保存成功；角色細分權限沿用本機 61/61</t>
+          <t>① pytest 33 passed；真 PATCH 本地 Supabase ② 62:70 刷 p212+R-41 強制低電 build（SUPPLY_LOW_RATIO_OVERRIDE=1.05）→ 串口 [WSc] power low:true，本地 DB battery_low=t ③ 刷回正常 1.6.2 → low:false，DB=f ④ App 讀 DB：低電紅標+Please charge+更新時間、72% 充電中、未上報不顯示 ⑤ 他人帳號 0 行、authenticated UPDATE 被拒。62:70 已還原為原 p212 build</t>
         </is>
       </c>
       <c r="F48" s="11" t="n"/>
@@ -2024,15 +2024,15 @@
       <c r="H48" s="11" t="n"/>
       <c r="I48" s="12" t="n"/>
     </row>
-    <row r="49" ht="88" customHeight="1">
+    <row r="49" ht="102" customHeight="1">
       <c r="A49" s="13" t="inlineStr">
         <is>
-          <t>P0-15</t>
+          <t>P0-12</t>
         </is>
       </c>
       <c r="B49" s="6" t="inlineStr">
         <is>
-          <t>角色表權限：只有內容管理員能發佈，關閉家長自建角色</t>
+          <t>收緊 Admin 權限與路由保護</t>
         </is>
       </c>
       <c r="C49" s="13" t="inlineStr">
@@ -2047,7 +2047,7 @@
       </c>
       <c r="E49" s="6" t="inlineStr">
         <is>
-          <t>線上 2026-10-12：② anon 只見 6 個已發佈 hk_ 內建，查隱藏/醫生/家長自建 → []，anon POST → 401；① authenticated 寫入權限由 20261007140000 REVOKE（runbook 10/08 已套用）；用戶確認：④ 家長登入後 /home/create 轉回 /home ③ 管理員在 /admin 修改角色保存成功</t>
+          <t>線上 2026-10-12（bac24e9）：runbook 10/08 檢查 未登入 /admin→/login、/api/admin→401、has_role() 只看角色、無管理員 policy 觸及 conversations/記憶表、超管≥1；未登入 /home、/admin→/login；用戶確認：家長帳號開 /admin 轉回 /home、管理員在 /admin 修改角色保存成功；角色細分權限沿用本機 61/61</t>
         </is>
       </c>
       <c r="F49" s="11" t="n"/>
@@ -2058,12 +2058,12 @@
     <row r="50" ht="88" customHeight="1">
       <c r="A50" s="13" t="inlineStr">
         <is>
-          <t>P0-16</t>
+          <t>P0-15</t>
         </is>
       </c>
       <c r="B50" s="6" t="inlineStr">
         <is>
-          <t>移除「醫生」身份與寫死的通關碼</t>
+          <t>角色表權限：只有內容管理員能發佈，關閉家長自建角色</t>
         </is>
       </c>
       <c r="C50" s="13" t="inlineStr">
@@ -2078,7 +2078,7 @@
       </c>
       <c r="E50" s="6" t="inlineStr">
         <is>
-          <t>線上 2026-10-12：生產 commit bac24e9 git grep checkDoctorAction/kiwi-subtle-emu/=== "doctor"/isDoctor → 0；線上 13 個 JS（/、/login、/onboard）grep 通關碼/"doctor"/Santa/patient → 0；anon 讀角色只見 6 個 hk_ 角色、is_doctor 全 false；用戶今日線上登入及 playground 正常</t>
+          <t>線上 2026-10-12：② anon 只見 6 個已發佈 hk_ 內建，查隱藏/醫生/家長自建 → []，anon POST → 401；① authenticated 寫入權限由 20261007140000 REVOKE（runbook 10/08 已套用）；用戶確認：④ 家長登入後 /home/create 轉回 /home ③ 管理員在 /admin 修改角色保存成功</t>
         </is>
       </c>
       <c r="F50" s="11" t="n"/>
@@ -2086,15 +2086,15 @@
       <c r="H50" s="11" t="n"/>
       <c r="I50" s="12" t="n"/>
     </row>
-    <row r="51" ht="60" customHeight="1">
+    <row r="51" ht="88" customHeight="1">
       <c r="A51" s="13" t="inlineStr">
         <is>
-          <t>P0-09</t>
+          <t>P0-16</t>
         </is>
       </c>
       <c r="B51" s="6" t="inlineStr">
         <is>
-          <t>瀏覽器語音路由改用簽名 token（/ws/nextjs）</t>
+          <t>移除「醫生」身份與寫死的通關碼</t>
         </is>
       </c>
       <c r="C51" s="13" t="inlineStr">
@@ -2109,7 +2109,7 @@
       </c>
       <c r="E51" s="6" t="inlineStr">
         <is>
-          <t>線上 2026-10-12（bac24e9）：wss /fastapi/ws/nextjs 只帶 user_id 或 token=bogus → 4401；用戶確認：登入 elatoai.hkqft.com 後網頁 playground 可正常對話</t>
+          <t>線上 2026-10-12：生產 commit bac24e9 git grep checkDoctorAction/kiwi-subtle-emu/=== "doctor"/isDoctor → 0；線上 13 個 JS（/、/login、/onboard）grep 通關碼/"doctor"/Santa/patient → 0；anon 讀角色只見 6 個 hk_ 角色、is_doctor 全 false；用戶今日線上登入及 playground 正常</t>
         </is>
       </c>
       <c r="F51" s="11" t="n"/>
@@ -2120,12 +2120,12 @@
     <row r="52" ht="60" customHeight="1">
       <c r="A52" s="13" t="inlineStr">
         <is>
-          <t>P0-17</t>
+          <t>P0-09</t>
         </is>
       </c>
       <c r="B52" s="6" t="inlineStr">
         <is>
-          <t>前端的 anon key 必須是公開 key，不可是 secret／service_role</t>
+          <t>瀏覽器語音路由改用簽名 token（/ws/nextjs）</t>
         </is>
       </c>
       <c r="C52" s="13" t="inlineStr">
@@ -2140,7 +2140,7 @@
       </c>
       <c r="E52" s="6" t="inlineStr">
         <is>
-          <t>線上 2026-10-12（bac24e9）：/login 引用的 13 個 JS + HTML 無 sb_secret_，唯一 key 為 role=anon 的 JWT；② 用該 key GET /rest/v1/users → 42501；③ 本機 10/07 已換 publishable</t>
+          <t>線上 2026-10-12（bac24e9）：wss /fastapi/ws/nextjs 只帶 user_id 或 token=bogus → 4401；用戶確認：登入 elatoai.hkqft.com 後網頁 playground 可正常對話</t>
         </is>
       </c>
       <c r="F52" s="11" t="n"/>
@@ -2148,15 +2148,15 @@
       <c r="H52" s="11" t="n"/>
       <c r="I52" s="12" t="n"/>
     </row>
-    <row r="53" ht="46" customHeight="1">
+    <row r="53" ht="60" customHeight="1">
       <c r="A53" s="13" t="inlineStr">
         <is>
-          <t>P0-10</t>
+          <t>P0-17</t>
         </is>
       </c>
       <c r="B53" s="6" t="inlineStr">
         <is>
-          <t>生產環境關閉 /browser 測試頁與 /ws/browser</t>
+          <t>前端的 anon key 必須是公開 key，不可是 secret／service_role</t>
         </is>
       </c>
       <c r="C53" s="13" t="inlineStr">
@@ -2171,7 +2171,7 @@
       </c>
       <c r="E53" s="6" t="inlineStr">
         <is>
-          <t>線上 2026-10-12（bac24e9）：GET /fastapi/browser 404、/fastapi/ 404、/fastapi/healthz 200、wss /fastapi/ws/browser → HTTP 403</t>
+          <t>線上 2026-10-12（bac24e9）：/login 引用的 13 個 JS + HTML 無 sb_secret_，唯一 key 為 role=anon 的 JWT；② 用該 key GET /rest/v1/users → 42501；③ 本機 10/07 已換 publishable</t>
         </is>
       </c>
       <c r="F53" s="11" t="n"/>
@@ -2324,20 +2324,20 @@
       <c r="H61" s="11" t="n"/>
       <c r="I61" s="12" t="n"/>
     </row>
-    <row r="62" ht="18" customHeight="1">
+    <row r="62" ht="32" customHeight="1">
       <c r="A62" s="13" t="inlineStr">
         <is>
-          <t>P2-19</t>
+          <t>P2-20</t>
         </is>
       </c>
       <c r="B62" s="6" t="inlineStr">
         <is>
-          <t>P2-16 ③ 回滾過多時自動暫停推送</t>
+          <t>P2-16 ④ 從後台上傳與發佈韌體（取代手貼 service key）</t>
         </is>
       </c>
       <c r="C62" s="6" t="inlineStr">
         <is>
-          <t>等 P2-18</t>
+          <t>等 P1-10</t>
         </is>
       </c>
       <c r="D62" s="11" t="n"/>
@@ -2347,20 +2347,20 @@
       <c r="H62" s="11" t="n"/>
       <c r="I62" s="12" t="n"/>
     </row>
-    <row r="63" ht="32" customHeight="1">
+    <row r="63" ht="18" customHeight="1">
       <c r="A63" s="13" t="inlineStr">
         <is>
-          <t>P2-20</t>
+          <t>P2-21</t>
         </is>
       </c>
       <c r="B63" s="6" t="inlineStr">
         <is>
-          <t>P2-16 ④ 從後台上傳與發佈韌體（取代手貼 service key）</t>
+          <t>P2-16 ⑤ 後台 OTA 頁換成真實數據與操作</t>
         </is>
       </c>
       <c r="C63" s="6" t="inlineStr">
         <is>
-          <t>等 P1-10</t>
+          <t>等 P2-19、P2-20、P2-14</t>
         </is>
       </c>
       <c r="D63" s="11" t="n"/>
@@ -2373,17 +2373,17 @@
     <row r="64" ht="18" customHeight="1">
       <c r="A64" s="13" t="inlineStr">
         <is>
-          <t>P2-21</t>
+          <t>R-05</t>
         </is>
       </c>
       <c r="B64" s="6" t="inlineStr">
         <is>
-          <t>P2-16 ⑤ 後台 OTA 頁換成真實數據與操作</t>
+          <t>內測版外殼（3D 打印 20 台）</t>
         </is>
       </c>
       <c r="C64" s="6" t="inlineStr">
         <is>
-          <t>等 P2-18、P2-19、P2-20、P2-14</t>
+          <t>等 R-01</t>
         </is>
       </c>
       <c r="D64" s="11" t="n"/>
@@ -2396,17 +2396,17 @@
     <row r="65" ht="18" customHeight="1">
       <c r="A65" s="13" t="inlineStr">
         <is>
-          <t>R-05</t>
+          <t>R-06</t>
         </is>
       </c>
       <c r="B65" s="6" t="inlineStr">
         <is>
-          <t>內測版外殼（3D 打印 20 台）</t>
+          <t>家長自助上手流程</t>
         </is>
       </c>
       <c r="C65" s="6" t="inlineStr">
         <is>
-          <t>等 R-01</t>
+          <t>等 P0-11</t>
         </is>
       </c>
       <c r="D65" s="11" t="n"/>
@@ -2416,20 +2416,20 @@
       <c r="H65" s="11" t="n"/>
       <c r="I65" s="12" t="n"/>
     </row>
-    <row r="66" ht="18" customHeight="1">
+    <row r="66" ht="32" customHeight="1">
       <c r="A66" s="13" t="inlineStr">
         <is>
-          <t>R-06</t>
+          <t>R-13</t>
         </is>
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
-          <t>家長自助上手流程</t>
+          <t>CP1 內測就緒檢查（10/30）</t>
         </is>
       </c>
       <c r="C66" s="6" t="inlineStr">
         <is>
-          <t>等 P0-11</t>
+          <t>等 P0-07、P0-11、P1-01、P1-02、P2-09、R-01、R-02、R-04、R-05、R-06、P1-11</t>
         </is>
       </c>
       <c r="D66" s="11" t="n"/>
@@ -2442,17 +2442,17 @@
     <row r="67" ht="32" customHeight="1">
       <c r="A67" s="13" t="inlineStr">
         <is>
-          <t>R-13</t>
+          <t>R-18</t>
         </is>
       </c>
       <c r="B67" s="6" t="inlineStr">
         <is>
-          <t>CP1 內測就緒檢查（10/30）</t>
+          <t>長按 BOOT 重新配網（開 AIBuddy-XXXX 熱點）</t>
         </is>
       </c>
       <c r="C67" s="6" t="inlineStr">
         <is>
-          <t>等 P0-07、P0-11、P1-01、P1-02、P2-09、R-01、R-02、R-04、R-05、R-06、P1-11</t>
+          <t>等 R-01</t>
         </is>
       </c>
       <c r="D67" s="11" t="n"/>
@@ -2465,12 +2465,12 @@
     <row r="68" ht="32" customHeight="1">
       <c r="A68" s="13" t="inlineStr">
         <is>
-          <t>R-18</t>
+          <t>R-19</t>
         </is>
       </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t>長按 BOOT 重新配網（開 AIBuddy-XXXX 熱點）</t>
+          <t>外接按鈕：量產板加 I2C 擴展晶片（TCA9555）</t>
         </is>
       </c>
       <c r="C68" s="6" t="inlineStr">
@@ -2485,20 +2485,20 @@
       <c r="H68" s="11" t="n"/>
       <c r="I68" s="12" t="n"/>
     </row>
-    <row r="69" ht="32" customHeight="1">
+    <row r="69" ht="18" customHeight="1">
       <c r="A69" s="13" t="inlineStr">
         <is>
-          <t>R-19</t>
+          <t>R-20</t>
         </is>
       </c>
       <c r="B69" s="6" t="inlineStr">
         <is>
-          <t>外接按鈕：量產板加 I2C 擴展晶片（TCA9555）</t>
+          <t>孩子資料與角色改成每台設備一份</t>
         </is>
       </c>
       <c r="C69" s="6" t="inlineStr">
         <is>
-          <t>等 R-01</t>
+          <t>等 P1-12</t>
         </is>
       </c>
       <c r="D69" s="11" t="n"/>
@@ -2508,20 +2508,20 @@
       <c r="H69" s="11" t="n"/>
       <c r="I69" s="12" t="n"/>
     </row>
-    <row r="70" ht="18" customHeight="1">
+    <row r="70" ht="32" customHeight="1">
       <c r="A70" s="13" t="inlineStr">
         <is>
-          <t>R-20</t>
+          <t>R-27</t>
         </is>
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>孩子資料與角色改成每台設備一份</t>
+          <t>App 內登入：驗證碼、原生社交登入、刪除帳號</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr">
         <is>
-          <t>等 P1-12</t>
+          <t>等 R-26</t>
         </is>
       </c>
       <c r="D70" s="11" t="n"/>
@@ -2531,20 +2531,20 @@
       <c r="H70" s="11" t="n"/>
       <c r="I70" s="12" t="n"/>
     </row>
-    <row r="71" ht="32" customHeight="1">
+    <row r="71" ht="18" customHeight="1">
       <c r="A71" s="13" t="inlineStr">
         <is>
-          <t>R-27</t>
+          <t>P0-14</t>
         </is>
       </c>
       <c r="B71" s="6" t="inlineStr">
         <is>
-          <t>App 內登入：驗證碼、原生社交登入、刪除帳號</t>
+          <t>韌體簽章、Secure Boot 與 Flash 加密</t>
         </is>
       </c>
       <c r="C71" s="6" t="inlineStr">
         <is>
-          <t>等 R-26</t>
+          <t>等 R-01</t>
         </is>
       </c>
       <c r="D71" s="11" t="n"/>
@@ -2557,17 +2557,17 @@
     <row r="72" ht="18" customHeight="1">
       <c r="A72" s="13" t="inlineStr">
         <is>
-          <t>P0-14</t>
+          <t>P1-06</t>
         </is>
       </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>韌體簽章、Secure Boot 與 Flash 加密</t>
+          <t>處理 GPL-3.0 依賴（arduino-audio-tools）</t>
         </is>
       </c>
       <c r="C72" s="6" t="inlineStr">
         <is>
-          <t>等 R-01</t>
+          <t>等 Q3</t>
         </is>
       </c>
       <c r="D72" s="11" t="n"/>
@@ -2580,12 +2580,12 @@
     <row r="73" ht="18" customHeight="1">
       <c r="A73" s="13" t="inlineStr">
         <is>
-          <t>P1-06</t>
+          <t>P1-07</t>
         </is>
       </c>
       <c r="B73" s="6" t="inlineStr">
         <is>
-          <t>處理 GPL-3.0 依賴（arduino-audio-tools）</t>
+          <t>LGPL 合規與第三方授權聲明</t>
         </is>
       </c>
       <c r="C73" s="6" t="inlineStr">
@@ -2603,17 +2603,17 @@
     <row r="74" ht="18" customHeight="1">
       <c r="A74" s="13" t="inlineStr">
         <is>
-          <t>P1-07</t>
+          <t>P1-08</t>
         </is>
       </c>
       <c r="B74" s="6" t="inlineStr">
         <is>
-          <t>LGPL 合規與第三方授權聲明</t>
+          <t>硬件認證</t>
         </is>
       </c>
       <c r="C74" s="6" t="inlineStr">
         <is>
-          <t>等 Q3</t>
+          <t>等 R-01、R-05</t>
         </is>
       </c>
       <c r="D74" s="11" t="n"/>
@@ -2626,17 +2626,17 @@
     <row r="75" ht="18" customHeight="1">
       <c r="A75" s="13" t="inlineStr">
         <is>
-          <t>P1-08</t>
+          <t>P1-14</t>
         </is>
       </c>
       <c r="B75" s="6" t="inlineStr">
         <is>
-          <t>硬件認證</t>
+          <t>Admin 內容安全頁：審核事件只按類別統計</t>
         </is>
       </c>
       <c r="C75" s="6" t="inlineStr">
         <is>
-          <t>等 R-01、R-05</t>
+          <t>等 P1-01、P2-13</t>
         </is>
       </c>
       <c r="D75" s="11" t="n"/>
@@ -2646,20 +2646,20 @@
       <c r="H75" s="11" t="n"/>
       <c r="I75" s="12" t="n"/>
     </row>
-    <row r="76" ht="18" customHeight="1">
+    <row r="76" ht="32" customHeight="1">
       <c r="A76" s="13" t="inlineStr">
         <is>
-          <t>P1-14</t>
+          <t>P2-15</t>
         </is>
       </c>
       <c r="B76" s="6" t="inlineStr">
         <is>
-          <t>Admin 內容安全頁：審核事件只按類別統計</t>
+          <t>Admin 總覽頁：在線、用量、成本與待處理事項</t>
         </is>
       </c>
       <c r="C76" s="6" t="inlineStr">
         <is>
-          <t>等 P1-01、P2-13</t>
+          <t>等 P2-14、P2-09</t>
         </is>
       </c>
       <c r="D76" s="11" t="n"/>
@@ -2669,20 +2669,20 @@
       <c r="H76" s="11" t="n"/>
       <c r="I76" s="12" t="n"/>
     </row>
-    <row r="77" ht="32" customHeight="1">
+    <row r="77" ht="18" customHeight="1">
       <c r="A77" s="13" t="inlineStr">
         <is>
-          <t>P2-15</t>
+          <t>R-07</t>
         </is>
       </c>
       <c r="B77" s="6" t="inlineStr">
         <is>
-          <t>Admin 總覽頁：在線、用量、成本與待處理事項</t>
+          <t>20 個家庭封閉內測</t>
         </is>
       </c>
       <c r="C77" s="6" t="inlineStr">
         <is>
-          <t>等 P2-14、P2-09</t>
+          <t>等 R-13</t>
         </is>
       </c>
       <c r="D77" s="11" t="n"/>
@@ -2695,17 +2695,17 @@
     <row r="78" ht="18" customHeight="1">
       <c r="A78" s="13" t="inlineStr">
         <is>
-          <t>R-07</t>
+          <t>R-08</t>
         </is>
       </c>
       <c r="B78" s="6" t="inlineStr">
         <is>
-          <t>20 個家庭封閉內測</t>
+          <t>第 8 週關卡決策</t>
         </is>
       </c>
       <c r="C78" s="6" t="inlineStr">
         <is>
-          <t>等 R-13</t>
+          <t>等 R-07、P2-09、P1-08</t>
         </is>
       </c>
       <c r="D78" s="11" t="n"/>
@@ -2718,17 +2718,17 @@
     <row r="79" ht="18" customHeight="1">
       <c r="A79" s="13" t="inlineStr">
         <is>
-          <t>R-08</t>
+          <t>R-14</t>
         </is>
       </c>
       <c r="B79" s="6" t="inlineStr">
         <is>
-          <t>第 8 週關卡決策</t>
+          <t>離線兒歌與故事</t>
         </is>
       </c>
       <c r="C79" s="6" t="inlineStr">
         <is>
-          <t>等 R-07、P2-09、P1-08</t>
+          <t>等 R-01</t>
         </is>
       </c>
       <c r="D79" s="11" t="n"/>
@@ -2741,17 +2741,17 @@
     <row r="80" ht="18" customHeight="1">
       <c r="A80" s="13" t="inlineStr">
         <is>
-          <t>R-14</t>
+          <t>R-24</t>
         </is>
       </c>
       <c r="B80" s="6" t="inlineStr">
         <is>
-          <t>離線兒歌與故事</t>
+          <t>設備只能用自己品牌的角色</t>
         </is>
       </c>
       <c r="C80" s="6" t="inlineStr">
         <is>
-          <t>等 R-01</t>
+          <t>等 R-34</t>
         </is>
       </c>
       <c r="D80" s="11" t="n"/>
@@ -2764,17 +2764,17 @@
     <row r="81" ht="18" customHeight="1">
       <c r="A81" s="13" t="inlineStr">
         <is>
-          <t>R-24</t>
+          <t>R-28</t>
         </is>
       </c>
       <c r="B81" s="6" t="inlineStr">
         <is>
-          <t>設備只能用自己品牌的角色</t>
+          <t>三個 App 的殼：品牌版本與測試版</t>
         </is>
       </c>
       <c r="C81" s="6" t="inlineStr">
         <is>
-          <t>等 R-34</t>
+          <t>等 R-25、R-26</t>
         </is>
       </c>
       <c r="D81" s="11" t="n"/>
@@ -2787,17 +2787,17 @@
     <row r="82" ht="18" customHeight="1">
       <c r="A82" s="13" t="inlineStr">
         <is>
-          <t>R-28</t>
+          <t>R-30</t>
         </is>
       </c>
       <c r="B82" s="6" t="inlineStr">
         <is>
-          <t>三個 App 的殼：品牌版本與測試版</t>
+          <t>快活 App（品牌 A）頁面</t>
         </is>
       </c>
       <c r="C82" s="6" t="inlineStr">
         <is>
-          <t>等 R-25、R-26</t>
+          <t>等 R-25、R-34、Q12</t>
         </is>
       </c>
       <c r="D82" s="11" t="n"/>
@@ -2810,17 +2810,17 @@
     <row r="83" ht="18" customHeight="1">
       <c r="A83" s="13" t="inlineStr">
         <is>
-          <t>R-30</t>
+          <t>R-31</t>
         </is>
       </c>
       <c r="B83" s="6" t="inlineStr">
         <is>
-          <t>快活 App（品牌 A）頁面</t>
+          <t>政協青年聯會版 App（品牌 B）頁面</t>
         </is>
       </c>
       <c r="C83" s="6" t="inlineStr">
         <is>
-          <t>等 R-25、R-34、Q12</t>
+          <t>等 R-25、R-34、Q13</t>
         </is>
       </c>
       <c r="D83" s="11" t="n"/>
@@ -2833,17 +2833,17 @@
     <row r="84" ht="18" customHeight="1">
       <c r="A84" s="13" t="inlineStr">
         <is>
-          <t>R-31</t>
+          <t>R-35</t>
         </is>
       </c>
       <c r="B84" s="6" t="inlineStr">
         <is>
-          <t>政協青年聯會版 App（品牌 B）頁面</t>
+          <t>韌體按品牌連線：伺服器網址在出廠時寫入</t>
         </is>
       </c>
       <c r="C84" s="6" t="inlineStr">
         <is>
-          <t>等 R-25、R-34、Q13</t>
+          <t>等 R-34</t>
         </is>
       </c>
       <c r="D84" s="11" t="n"/>
@@ -2853,20 +2853,20 @@
       <c r="H84" s="11" t="n"/>
       <c r="I84" s="12" t="n"/>
     </row>
-    <row r="85" ht="18" customHeight="1">
+    <row r="85" ht="32" customHeight="1">
       <c r="A85" s="13" t="inlineStr">
         <is>
-          <t>R-35</t>
+          <t>R-38</t>
         </is>
       </c>
       <c r="B85" s="6" t="inlineStr">
         <is>
-          <t>韌體按品牌連線：伺服器網址在出廠時寫入</t>
+          <t>公仔出廠鎖死所屬 IP，綁定時顯示該 IP 頭像</t>
         </is>
       </c>
       <c r="C85" s="6" t="inlineStr">
         <is>
-          <t>等 R-34</t>
+          <t>等 P0-11</t>
         </is>
       </c>
       <c r="D85" s="11" t="n"/>
@@ -2879,17 +2879,17 @@
     <row r="86" ht="32" customHeight="1">
       <c r="A86" s="13" t="inlineStr">
         <is>
-          <t>R-38</t>
+          <t>R-39</t>
         </is>
       </c>
       <c r="B86" s="6" t="inlineStr">
         <is>
-          <t>公仔出廠鎖死所屬 IP，綁定時顯示該 IP 頭像</t>
+          <t>Admin 出廠登記頁：匯入 MAC 清單、指定公仔、查看自檢結果</t>
         </is>
       </c>
       <c r="C86" s="6" t="inlineStr">
         <is>
-          <t>等 P0-11</t>
+          <t>等 R-38、P1-10</t>
         </is>
       </c>
       <c r="D86" s="11" t="n"/>
@@ -2899,20 +2899,20 @@
       <c r="H86" s="11" t="n"/>
       <c r="I86" s="12" t="n"/>
     </row>
-    <row r="87" ht="32" customHeight="1">
+    <row r="87" ht="18" customHeight="1">
       <c r="A87" s="13" t="inlineStr">
         <is>
-          <t>R-39</t>
+          <t>R-09</t>
         </is>
       </c>
       <c r="B87" s="6" t="inlineStr">
         <is>
-          <t>Admin 出廠登記頁：匯入 MAC 清單、指定公仔、查看自檢結果</t>
+          <t>量產外殼（真空複模）</t>
         </is>
       </c>
       <c r="C87" s="6" t="inlineStr">
         <is>
-          <t>等 R-38、P1-10</t>
+          <t>等 R-08、R-05、Q11</t>
         </is>
       </c>
       <c r="D87" s="11" t="n"/>
@@ -2925,17 +2925,17 @@
     <row r="88" ht="18" customHeight="1">
       <c r="A88" s="13" t="inlineStr">
         <is>
-          <t>R-09</t>
+          <t>R-10</t>
         </is>
       </c>
       <c r="B88" s="6" t="inlineStr">
         <is>
-          <t>量產外殼（真空複模）</t>
+          <t>出廠流程</t>
         </is>
       </c>
       <c r="C88" s="6" t="inlineStr">
         <is>
-          <t>等 R-08、R-05、Q11</t>
+          <t>等 P0-14、R-01、P2-12、R-34、R-35、R-38、R-39</t>
         </is>
       </c>
       <c r="D88" s="11" t="n"/>
@@ -2948,17 +2948,17 @@
     <row r="89" ht="18" customHeight="1">
       <c r="A89" s="13" t="inlineStr">
         <is>
-          <t>R-10</t>
+          <t>R-11</t>
         </is>
       </c>
       <c r="B89" s="6" t="inlineStr">
         <is>
-          <t>出廠流程</t>
+          <t>售後：客服、保修與換機</t>
         </is>
       </c>
       <c r="C89" s="6" t="inlineStr">
         <is>
-          <t>等 P0-14、R-01、P2-12、R-34、R-35、R-38、R-39</t>
+          <t>等 P2-14、R-40</t>
         </is>
       </c>
       <c r="D89" s="11" t="n"/>
@@ -2971,17 +2971,17 @@
     <row r="90" ht="18" customHeight="1">
       <c r="A90" s="13" t="inlineStr">
         <is>
-          <t>R-11</t>
+          <t>R-15</t>
         </is>
       </c>
       <c r="B90" s="6" t="inlineStr">
         <is>
-          <t>售後：客服、保修與換機</t>
+          <t>農曆新年前交付（生產 1/15、送達 1/29）</t>
         </is>
       </c>
       <c r="C90" s="6" t="inlineStr">
         <is>
-          <t>等 P2-14、R-40</t>
+          <t>等 R-09、R-10</t>
         </is>
       </c>
       <c r="D90" s="11" t="n"/>
@@ -2994,17 +2994,17 @@
     <row r="91" ht="18" customHeight="1">
       <c r="A91" s="13" t="inlineStr">
         <is>
-          <t>R-15</t>
+          <t>R-33</t>
         </is>
       </c>
       <c r="B91" s="6" t="inlineStr">
         <is>
-          <t>農曆新年前交付（生產 1/15、送達 1/29）</t>
+          <t>三個 App 送審並通過</t>
         </is>
       </c>
       <c r="C91" s="6" t="inlineStr">
         <is>
-          <t>等 R-09、R-10</t>
+          <t>等 R-27、R-21、R-28、R-29、R-30、R-31、R-32</t>
         </is>
       </c>
       <c r="D91" s="11" t="n"/>
@@ -3014,20 +3014,20 @@
       <c r="H91" s="11" t="n"/>
       <c r="I91" s="12" t="n"/>
     </row>
-    <row r="92" ht="18" customHeight="1">
+    <row r="92" ht="32" customHeight="1">
       <c r="A92" s="13" t="inlineStr">
         <is>
-          <t>R-33</t>
+          <t>R-40</t>
         </is>
       </c>
       <c r="B92" s="6" t="inlineStr">
         <is>
-          <t>三個 App 送審並通過</t>
+          <t>Admin 客服查詢頁：查帳號、名下設備與最近事件</t>
         </is>
       </c>
       <c r="C92" s="6" t="inlineStr">
         <is>
-          <t>等 R-27、R-21、R-28、R-29、R-30、R-31、R-32</t>
+          <t>等 P2-14、P1-10、P1-12</t>
         </is>
       </c>
       <c r="D92" s="11" t="n"/>
@@ -3037,50 +3037,50 @@
       <c r="H92" s="11" t="n"/>
       <c r="I92" s="12" t="n"/>
     </row>
-    <row r="93" ht="32" customHeight="1">
-      <c r="A93" s="13" t="inlineStr">
-        <is>
-          <t>R-40</t>
-        </is>
-      </c>
-      <c r="B93" s="6" t="inlineStr">
-        <is>
-          <t>Admin 客服查詢頁：查帳號、名下設備與最近事件</t>
-        </is>
-      </c>
-      <c r="C93" s="6" t="inlineStr">
-        <is>
-          <t>等 P2-14、P1-10、P1-12</t>
-        </is>
-      </c>
-      <c r="D93" s="11" t="n"/>
-      <c r="E93" s="11" t="n"/>
-      <c r="F93" s="11" t="n"/>
-      <c r="G93" s="11" t="n"/>
-      <c r="H93" s="11" t="n"/>
-      <c r="I93" s="12" t="n"/>
+    <row r="94">
+      <c r="A94" s="10" t="inlineStr">
+        <is>
+          <t>❓ 待確認問題</t>
+        </is>
+      </c>
     </row>
     <row r="95">
-      <c r="A95" s="10" t="inlineStr">
-        <is>
-          <t>❓ 待確認問題</t>
-        </is>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" s="4" t="inlineStr">
+      <c r="A95" s="4" t="inlineStr">
         <is>
           <t>編號</t>
         </is>
       </c>
-      <c r="B96" s="4" t="inlineStr">
+      <c r="B95" s="4" t="inlineStr">
         <is>
           <t>問題</t>
         </is>
       </c>
-      <c r="C96" s="4" t="inlineStr">
+      <c r="C95" s="4" t="inlineStr">
         <is>
           <t>影響的任務 / 為什麼重要</t>
+        </is>
+      </c>
+      <c r="D95" s="11" t="n"/>
+      <c r="E95" s="11" t="n"/>
+      <c r="F95" s="11" t="n"/>
+      <c r="G95" s="11" t="n"/>
+      <c r="H95" s="11" t="n"/>
+      <c r="I95" s="12" t="n"/>
+    </row>
+    <row r="96" ht="18" customHeight="1">
+      <c r="A96" s="13" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="B96" s="6" t="inlineStr">
+        <is>
+          <t>韌體打算閉源商業銷售嗎？</t>
+        </is>
+      </c>
+      <c r="C96" s="6" t="inlineStr">
+        <is>
+          <t>P1-06, P1-07：決定 GPL／LGPL 依賴要開源還是替換。</t>
         </is>
       </c>
       <c r="D96" s="11" t="n"/>
@@ -3090,20 +3090,20 @@
       <c r="H96" s="11" t="n"/>
       <c r="I96" s="12" t="n"/>
     </row>
-    <row r="97" ht="18" customHeight="1">
+    <row r="97" ht="32" customHeight="1">
       <c r="A97" s="13" t="inlineStr">
         <is>
-          <t>Q3</t>
+          <t>Q11</t>
         </is>
       </c>
       <c r="B97" s="6" t="inlineStr">
         <is>
-          <t>韌體打算閉源商業銷售嗎？</t>
+          <t>馬會快活的賽馬日版和新春版各多少隻（共 2,500）？</t>
         </is>
       </c>
       <c r="C97" s="6" t="inlineStr">
         <is>
-          <t>P1-06, P1-07：決定 GPL／LGPL 依賴要開源還是替換。</t>
+          <t>R-09, R-15：兩款的服裝和配件要分開訂料；11/20 前不知道，PP 樣和大貨單（11/27）會被拖慢。由馬會決定。</t>
         </is>
       </c>
       <c r="D97" s="11" t="n"/>
@@ -3113,20 +3113,20 @@
       <c r="H97" s="11" t="n"/>
       <c r="I97" s="12" t="n"/>
     </row>
-    <row r="98" ht="32" customHeight="1">
+    <row r="98" ht="60" customHeight="1">
       <c r="A98" s="13" t="inlineStr">
         <is>
-          <t>Q11</t>
+          <t>Q12</t>
         </is>
       </c>
       <c r="B98" s="6" t="inlineStr">
         <is>
-          <t>馬會快活的賽馬日版和新春版各多少隻（共 2,500）？</t>
+          <t>快活 App 的「會員綁定」是指甚麼：用我們自己的帳號（email 驗證碼），還是接馬會的會員帳號登入（SSO）？</t>
         </is>
       </c>
       <c r="C98" s="6" t="inlineStr">
         <is>
-          <t>R-09, R-15：兩款的服裝和配件要分開訂料；11/20 前不知道，PP 樣和大貨單（11/27）會被拖慢。由馬會決定。</t>
+          <t>P0-11, 快活 App（未入追蹤表）：接馬會 SSO 的話，登入、帳號刪除和資料歸屬都要按馬會的介面重做，工作量和排期要另估，而且 W5（11/9–11/13）就要做快活 App 的綁定；用我們的帳號則和其他品牌共用同一套流程。由馬會決定，要盡早問。</t>
         </is>
       </c>
       <c r="D98" s="11" t="n"/>
@@ -3136,20 +3136,20 @@
       <c r="H98" s="11" t="n"/>
       <c r="I98" s="12" t="n"/>
     </row>
-    <row r="99" ht="60" customHeight="1">
+    <row r="99" ht="46" customHeight="1">
       <c r="A99" s="13" t="inlineStr">
         <is>
-          <t>Q12</t>
+          <t>Q13</t>
         </is>
       </c>
       <c r="B99" s="6" t="inlineStr">
         <is>
-          <t>快活 App 的「會員綁定」是指甚麼：用我們自己的帳號（email 驗證碼），還是接馬會的會員帳號登入（SSO）？</t>
+          <t>政協青年聯會版的角色、語言和內容由誰提供？什麼時候交？</t>
         </is>
       </c>
       <c r="C99" s="6" t="inlineStr">
         <is>
-          <t>P0-11, 快活 App（未入追蹤表）：接馬會 SSO 的話，登入、帳號刪除和資料歸屬都要按馬會的介面重做，工作量和排期要另估，而且 W5（11/9–11/13）就要做快活 App 的綁定；用我們的帳號則和其他品牌共用同一套流程。由馬會決定，要盡早問。</t>
+          <t>品牌 B 的 App 頁面：品牌 B 的用戶是成人會員，但角色、說話語言、內容規則都還沒有。最遲 11/13 要拿到，才趕得及內部測試和 App 頁面（W6）。</t>
         </is>
       </c>
       <c r="D99" s="11" t="n"/>
@@ -3159,78 +3159,56 @@
       <c r="H99" s="11" t="n"/>
       <c r="I99" s="12" t="n"/>
     </row>
-    <row r="100" ht="46" customHeight="1">
-      <c r="A100" s="13" t="inlineStr">
-        <is>
-          <t>Q13</t>
-        </is>
-      </c>
-      <c r="B100" s="6" t="inlineStr">
-        <is>
-          <t>政協青年聯會版的角色、語言和內容由誰提供？什麼時候交？</t>
-        </is>
-      </c>
-      <c r="C100" s="6" t="inlineStr">
-        <is>
-          <t>品牌 B 的 App 頁面：品牌 B 的用戶是成人會員，但角色、說話語言、內容規則都還沒有。最遲 11/13 要拿到，才趕得及內部測試和 App 頁面（W6）。</t>
-        </is>
-      </c>
-      <c r="D100" s="11" t="n"/>
-      <c r="E100" s="11" t="n"/>
-      <c r="F100" s="11" t="n"/>
-      <c r="G100" s="11" t="n"/>
-      <c r="H100" s="11" t="n"/>
-      <c r="I100" s="12" t="n"/>
-    </row>
-    <row r="102">
-      <c r="A102" s="10" t="inlineStr">
+    <row r="101">
+      <c r="A101" s="10" t="inlineStr">
         <is>
           <t>說明</t>
         </is>
       </c>
     </row>
-    <row r="103" ht="32" customHeight="1">
+    <row r="102" ht="32" customHeight="1">
+      <c r="A102" s="14" t="inlineStr">
+        <is>
+          <t>・狀態：未開始 → 進行中 → 已完成。只有測試真的跑過而且通過才算已完成；阻塞要在備註寫原因；不再需要的任務標不適用，不要刪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" ht="18" customHeight="1">
       <c r="A103" s="14" t="inlineStr">
         <is>
-          <t>・狀態：未開始 → 進行中 → 已完成。只有測試真的跑過而且通過才算已完成；阻塞要在備註寫原因；不再需要的任務標不適用，不要刪。</t>
+          <t>・測試結果：未測試 / 通過 / 失敗 / 部分通過。測試證據寫跑了什麼、看到什麼，完整歷史在「更新記錄」。</t>
         </is>
       </c>
     </row>
     <row r="104" ht="18" customHeight="1">
       <c r="A104" s="14" t="inlineStr">
         <is>
-          <t>・測試結果：未測試 / 通過 / 失敗 / 部分通過。測試證據寫跑了什麼、看到什麼，完整歷史在「更新記錄」。</t>
+          <t>・「接下來」按階段排序，同一階段內再按優先級；依賴還沒滿足的任務不會出現在「接下來」。</t>
         </is>
       </c>
     </row>
     <row r="105" ht="18" customHeight="1">
       <c r="A105" s="14" t="inlineStr">
         <is>
-          <t>・「接下來」按階段排序，同一階段內再按優先級；依賴還沒滿足的任務不會出現在「接下來」。</t>
-        </is>
-      </c>
-    </row>
-    <row r="106" ht="18" customHeight="1">
+          <t>・可以手動改：「任務清單」的狀態、測試結果、測試證據、Commit、備註，以及「待確認問題」的回答。其餘欄位和本頁由腳本維護。</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="32" customHeight="1">
       <c r="A106" s="14" t="inlineStr">
         <is>
-          <t>・可以手動改：「任務清單」的狀態、測試結果、測試證據、Commit、備註，以及「待確認問題」的回答。其餘欄位和本頁由腳本維護。</t>
-        </is>
-      </c>
-    </row>
-    <row r="107" ht="32" customHeight="1">
-      <c r="A107" s="14" t="inlineStr">
-        <is>
           <t>・建議用法：在 Claude Code 對 Claude 說「P0-02 做完了」或輸入 /prod-readiness。Claude 會先跑測試再更新，並寫進「更新記錄」。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="88">
+  <mergeCells count="87">
     <mergeCell ref="C82:I82"/>
     <mergeCell ref="E52:I52"/>
     <mergeCell ref="E39:I39"/>
     <mergeCell ref="C67:I67"/>
     <mergeCell ref="E48:I48"/>
+    <mergeCell ref="A101:I101"/>
     <mergeCell ref="A2:I2"/>
     <mergeCell ref="E29:I29"/>
     <mergeCell ref="E38:I38"/>
@@ -3243,6 +3221,7 @@
     <mergeCell ref="E26:I26"/>
     <mergeCell ref="A103:I103"/>
     <mergeCell ref="E25:I25"/>
+    <mergeCell ref="C95:I95"/>
     <mergeCell ref="C60:I60"/>
     <mergeCell ref="C71:I71"/>
     <mergeCell ref="E50:I50"/>
@@ -3262,7 +3241,6 @@
     <mergeCell ref="E46:I46"/>
     <mergeCell ref="A102:I102"/>
     <mergeCell ref="C85:I85"/>
-    <mergeCell ref="C100:I100"/>
     <mergeCell ref="C65:I65"/>
     <mergeCell ref="C75:I75"/>
     <mergeCell ref="C84:I84"/>
@@ -3271,6 +3249,7 @@
     <mergeCell ref="C59:I59"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="E41:I41"/>
+    <mergeCell ref="A94:I94"/>
     <mergeCell ref="E47:I47"/>
     <mergeCell ref="C61:I61"/>
     <mergeCell ref="C70:I70"/>
@@ -3290,7 +3269,6 @@
     <mergeCell ref="E23:I23"/>
     <mergeCell ref="C72:I72"/>
     <mergeCell ref="C81:I81"/>
-    <mergeCell ref="A95:I95"/>
     <mergeCell ref="C69:I69"/>
     <mergeCell ref="E51:I51"/>
     <mergeCell ref="C96:I96"/>
@@ -3308,8 +3286,6 @@
     <mergeCell ref="E27:I27"/>
     <mergeCell ref="E36:I36"/>
     <mergeCell ref="C63:I63"/>
-    <mergeCell ref="C93:I93"/>
-    <mergeCell ref="A107:I107"/>
     <mergeCell ref="C56:I56"/>
     <mergeCell ref="C90:I90"/>
     <mergeCell ref="E53:I53"/>
@@ -9809,7 +9785,7 @@
         </is>
       </c>
     </row>
-    <row r="90" ht="186" customHeight="1">
+    <row r="90" ht="256" customHeight="1">
       <c r="A90" s="13" t="inlineStr">
         <is>
           <t>P2-17</t>
@@ -9882,7 +9858,7 @@
       </c>
       <c r="O90" s="13" t="inlineStr">
         <is>
-          <t>8675970</t>
+          <t>c510e02</t>
         </is>
       </c>
       <c r="P90" s="6" t="inlineStr">
@@ -9890,11 +9866,12 @@
           <t>[2026-10-14] 新增：2026-10-14 分支 p2-16-ota-rollout（worktree ../aibuddy-p216）
 [2026-10-14] 2026-10-14 用戶決定提前到第 2 階段，現在開始做
 [2026-10-14] 測試方法修正：內容管理員讀取在 RLS 下是 200 + 0 行而非 42501，保護效果相同（看不到任何行），寫入一律 42501
-[2026-10-14] commit 在分支 p2-16-ota-rollout（rebase 後 9f44e32 → 8675970），未合併到 dev、未部署</t>
-        </is>
-      </c>
-    </row>
-    <row r="91" ht="74" customHeight="1">
+[2026-10-14] commit 在分支 p2-16-ota-rollout（rebase 後 9f44e32 → 8675970），未合併到 dev、未部署
+[2026-10-14] commit 再次 rebase 後為 c510e02（分支 p2-16-ota-rollout）。之後分支不再為追蹤表 commit rebase，hash 到合併時才會變</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="214" customHeight="1">
       <c r="A91" s="13" t="inlineStr">
         <is>
           <t>P2-18</t>
@@ -9922,12 +9899,17 @@
       </c>
       <c r="F91" s="13" t="inlineStr">
         <is>
-          <t>未開始</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="G91" s="13" t="inlineStr">
         <is>
-          <t>未測試</t>
+          <t>通過</t>
+        </is>
+      </c>
+      <c r="H91" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="I91" s="6" t="inlineStr">
@@ -9953,6 +9935,16 @@
       <c r="M91" s="13" t="inlineStr">
         <is>
           <t>P2-17</t>
+        </is>
+      </c>
+      <c r="N91" s="6" t="inlineStr">
+        <is>
+          <t>node --test lib/otaRollout.test.mjs 6/6：10,000 隨機 MAC 在 10%/50% 誤差 &lt; 1 個百分點、同 MAC（含大小寫/空白）結果一致、升階段只增不減、白名單各階段都在、不同版本選不同的 10%。tsc --noEmit 通過。分支 dev server（3216）+ 本機 Supabase 模擬 20 台（板型 p218-sim，連跑兩次 9/9）：白名單階段只有 1 台、重複不變；10% 拿到的正是雜湊預測的那組（2–5 台含白名單），重複不變；50% 包含 10% 全部；暫停 → 0 台且下載映像 404，恢復 → 200；100% → 除已更新和已回滾的 2 台外 18 台；每台下發次數與記錄一致；運行中/已回滾正確標記；審計 6 筆對應 6 次變更。真 spotpear-ai-toy（預設 100%）回報 1.6.1 → 仍拿到 1.6.2。測試數據已清除</t>
+        </is>
+      </c>
+      <c r="O91" s="13" t="inlineStr">
+        <is>
+          <t>e57529d</t>
         </is>
       </c>
       <c r="P91" s="6" t="inlineStr">
@@ -10748,7 +10740,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I287"/>
+  <dimension ref="A1:I290"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -20659,8 +20651,121 @@
         </is>
       </c>
     </row>
+    <row r="288" ht="32" customHeight="1">
+      <c r="A288" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 20:46</t>
+        </is>
+      </c>
+      <c r="B288" s="13" t="inlineStr">
+        <is>
+          <t>P2-18</t>
+        </is>
+      </c>
+      <c r="C288" s="6" t="inlineStr">
+        <is>
+          <t>P2-16 ② 按 MAC 雜湊穩定分組決定哪台收到 ota</t>
+        </is>
+      </c>
+      <c r="D288" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E288" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F288" s="13" t="n"/>
+      <c r="G288" s="6" t="n"/>
+      <c r="H288" s="13" t="n"/>
+      <c r="I288" s="6" t="n"/>
+    </row>
+    <row r="289" ht="60" customHeight="1">
+      <c r="A289" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 20:50</t>
+        </is>
+      </c>
+      <c r="B289" s="13" t="inlineStr">
+        <is>
+          <t>P2-17</t>
+        </is>
+      </c>
+      <c r="C289" s="6" t="inlineStr">
+        <is>
+          <t>P2-16 ① 分批推送的數據表：推送階段、白名單、每台安裝結果</t>
+        </is>
+      </c>
+      <c r="D289" s="13" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="E289" s="13" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="F289" s="13" t="n"/>
+      <c r="G289" s="6" t="n"/>
+      <c r="H289" s="13" t="inlineStr">
+        <is>
+          <t>c510e02</t>
+        </is>
+      </c>
+      <c r="I289" s="6" t="inlineStr">
+        <is>
+          <t>commit 再次 rebase 後為 c510e02（分支 p2-16-ota-rollout）。之後分支不再為追蹤表 commit rebase，hash 到合併時才會變</t>
+        </is>
+      </c>
+    </row>
+    <row r="290" ht="186" customHeight="1">
+      <c r="A290" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 20:50</t>
+        </is>
+      </c>
+      <c r="B290" s="13" t="inlineStr">
+        <is>
+          <t>P2-18</t>
+        </is>
+      </c>
+      <c r="C290" s="6" t="inlineStr">
+        <is>
+          <t>P2-16 ② 按 MAC 雜湊穩定分組決定哪台收到 ota</t>
+        </is>
+      </c>
+      <c r="D290" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="E290" s="13" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="F290" s="13" t="inlineStr">
+        <is>
+          <t>通過</t>
+        </is>
+      </c>
+      <c r="G290" s="6" t="inlineStr">
+        <is>
+          <t>node --test lib/otaRollout.test.mjs 6/6：10,000 隨機 MAC 在 10%/50% 誤差 &lt; 1 個百分點、同 MAC（含大小寫/空白）結果一致、升階段只增不減、白名單各階段都在、不同版本選不同的 10%。tsc --noEmit 通過。分支 dev server（3216）+ 本機 Supabase 模擬 20 台（板型 p218-sim，連跑兩次 9/9）：白名單階段只有 1 台、重複不變；10% 拿到的正是雜湊預測的那組（2–5 台含白名單），重複不變；50% 包含 10% 全部；暫停 → 0 台且下載映像 404，恢復 → 200；100% → 除已更新和已回滾的 2 台外 18 台；每台下發次數與記錄一致；運行中/已回滾正確標記；審計 6 筆對應 6 次變更。真 spotpear-ai-toy（預設 100%）回報 1.6.1 → 仍拿到 1.6.2。測試數據已清除</t>
+        </is>
+      </c>
+      <c r="H290" s="13" t="inlineStr">
+        <is>
+          <t>e57529d</t>
+        </is>
+      </c>
+      <c r="I290" s="6" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I287"/>
+  <autoFilter ref="A1:I290"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Track P2-19 (auto-pause on rollbacks) as passed, without the repeated-install rule.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/production-readiness.xlsx
+++ b/docs/production-readiness.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'任務清單'!$A$1:$P$94</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'待確認問題'!$A$1:$G$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$290</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$294</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -665,14 +665,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>最後更新：2026-10-14 20:50　·　本頁由 tracker.py 自動生成，請勿手動編輯</t>
+          <t>最後更新：2026-10-14 20:58　·　本頁由 tracker.py 自動生成，請勿手動編輯</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>總進度：20/89 已完成（22%）　·　目前階段：1 止血定案（10/5–10/16）</t>
+          <t>總進度：21/89 已完成（24%）　·　目前階段：1 止血定案（10/5–10/16）</t>
         </is>
       </c>
     </row>
@@ -820,7 +820,7 @@
       </c>
       <c r="D8" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A8,'任務清單'!$F:$F,D$5)</f>
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E8" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A8,'任務清單'!$F:$F,E$5)</f>
@@ -828,7 +828,7 @@
       </c>
       <c r="F8" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A8,'任務清單'!$F:$F,F$5)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G8" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A8,'任務清單'!$F:$F,G$5)</f>
@@ -840,7 +840,7 @@
       </c>
       <c r="I8" s="8">
         <f>IFERROR(F8/(C8-H8),0)</f>
-        <v>0.23809523809523808</v>
+        <v>0.2857142857142857</v>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1">
@@ -896,7 +896,7 @@
       </c>
       <c r="D10" s="5">
         <f>SUM(D6:D9)</f>
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E10" s="5">
         <f>SUM(E6:E9)</f>
@@ -904,7 +904,7 @@
       </c>
       <c r="F10" s="5">
         <f>SUM(F6:F9)</f>
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G10" s="5">
         <f>SUM(G6:G9)</f>
@@ -916,7 +916,7 @@
       </c>
       <c r="I10" s="9">
         <f>IFERROR(F10/(C10-H10),0)</f>
-        <v>0.2247191011235955</v>
+        <v>0.23595505617977527</v>
       </c>
     </row>
     <row r="12">
@@ -1023,7 +1023,7 @@
       </c>
       <c r="D14" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A14,'任務清單'!$F:$F,D$12)</f>
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E14" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A14,'任務清單'!$F:$F,E$12)</f>
@@ -1031,7 +1031,7 @@
       </c>
       <c r="F14" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A14,'任務清單'!$F:$F,F$12)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G14" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A14,'任務清單'!$F:$F,G$12)</f>
@@ -1043,7 +1043,7 @@
       </c>
       <c r="I14" s="8">
         <f>IFERROR(F14/(C14-H14),0)</f>
-        <v>0.15151515151515152</v>
+        <v>0.18181818181818182</v>
       </c>
     </row>
     <row r="15" ht="46" customHeight="1">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="D17" s="5">
         <f>SUM(D13:D16)</f>
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E17" s="5">
         <f>SUM(E13:E16)</f>
@@ -1147,7 +1147,7 @@
       </c>
       <c r="F17" s="5">
         <f>SUM(F13:F16)</f>
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G17" s="5">
         <f>SUM(G13:G16)</f>
@@ -1159,7 +1159,7 @@
       </c>
       <c r="I17" s="9">
         <f>IFERROR(F17/(C17-H17),0)</f>
-        <v>0.2247191011235955</v>
+        <v>0.23595505617977527</v>
       </c>
     </row>
     <row r="19">
@@ -1573,7 +1573,7 @@
       </c>
       <c r="E32" s="6" t="inlineStr">
         <is>
-          <t>後台可上傳韌體（伺服器算 SHA-256、寫 firmware_releases）、填說明、設為 current；推送分階段：白名單 MAC → 10% → 50% → 100%，按 MAC 雜湊穩定分組；回滾率超過 5% 或任一台在試用期內重啟 3 次即自動暫停；顯示每個版本已更新、回滾台數與回滾設備清單；顯示 app 分區用量（P2-12）；每個發佈操作寫入審計記錄。</t>
+          <t>後台可上傳韌體（伺服器算 SHA-256、寫 firmware_releases）、填說明、設為 current；推送分階段：白名單 MAC → 10% → 50% → 100%，按 MAC 雜湊穩定分組；回滾率超過 5% 即自動暫停（2026-10-14 拿走「同一台重啟 3 次」，見 P2-19）；顯示每個版本已更新、回滾台數與回滾設備清單；顯示 app 分區用量（P2-12）；每個發佈操作寫入審計記錄。</t>
         </is>
       </c>
       <c r="F32" s="11" t="n"/>
@@ -1831,15 +1831,15 @@
       <c r="H40" s="11" t="n"/>
       <c r="I40" s="12" t="n"/>
     </row>
-    <row r="41" ht="74" customHeight="1">
+    <row r="41" ht="46" customHeight="1">
       <c r="A41" s="13" t="inlineStr">
         <is>
-          <t>P2-19</t>
+          <t>R-04</t>
         </is>
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>P2-16 ③ 回滾過多時自動暫停推送</t>
+          <t>粵語質量評測</t>
         </is>
       </c>
       <c r="C41" s="13" t="inlineStr">
@@ -1854,7 +1854,7 @@
       </c>
       <c r="E41" s="6" t="inlineStr">
         <is>
-          <t>已下發的設備中回滾率 &gt; 5%，或任一台對同一版本被下發 3 次仍未確認，即自動暫停該版本並記下原因；暫停後其餘設備不再拿到 ota；已確認的設備不受影響；自動暫停寫入審計記錄（操作者記為系統）；只能由超級管理員在後台恢復。</t>
+          <t>有一套粵語評測集（兒童錄音＋文字提示）；選定的 STT 與 LLM 達到門檻：兒童語音字錯率 ≤15%、口語粵語回覆 ≥90%、中英夾雜句能正確理解。</t>
         </is>
       </c>
       <c r="F41" s="11" t="n"/>
@@ -1862,15 +1862,15 @@
       <c r="H41" s="11" t="n"/>
       <c r="I41" s="12" t="n"/>
     </row>
-    <row r="42" ht="46" customHeight="1">
+    <row r="42" ht="116" customHeight="1">
       <c r="A42" s="13" t="inlineStr">
         <is>
-          <t>R-04</t>
+          <t>R-25</t>
         </is>
       </c>
       <c r="B42" s="6" t="inlineStr">
         <is>
-          <t>粵語質量評測</t>
+          <t>網頁的品牌主題系統</t>
         </is>
       </c>
       <c r="C42" s="13" t="inlineStr">
@@ -1885,7 +1885,7 @@
       </c>
       <c r="E42" s="6" t="inlineStr">
         <is>
-          <t>有一套粵語評測集（兒童錄音＋文字提示）；選定的 STT 與 LLM 達到門檻：兒童語音字錯率 ≤15%、口語粵語回覆 ≥90%、中英夾雜句能正確理解。</t>
+          <t>① 每個品牌一個資料夾：主題 token（顏色、字體、圓角）、logo 和圖示、文案、功能開關；首頁、上手流程、角色頁可以有品牌版本，其餘頁面共用 ② 由部署的環境變數選品牌（每套部署一個品牌，見 R-34），伺服器端渲染的第一屏就是對的主題，不閃爍 ③ 共用元件裡沒有品牌名稱和寫死的品牌顏色 ④ 加一個品牌只需要加資料夾、設定和一套部署，不用改共用元件</t>
         </is>
       </c>
       <c r="F42" s="11" t="n"/>
@@ -1931,15 +1931,15 @@
       <c r="H45" s="11" t="n"/>
       <c r="I45" s="12" t="n"/>
     </row>
-    <row r="46" ht="200" customHeight="1">
+    <row r="46" ht="158" customHeight="1">
       <c r="A46" s="13" t="inlineStr">
         <is>
-          <t>P2-18</t>
+          <t>P2-19</t>
         </is>
       </c>
       <c r="B46" s="6" t="inlineStr">
         <is>
-          <t>P2-16 ② 按 MAC 雜湊穩定分組決定哪台收到 ota</t>
+          <t>P2-16 ③ 回滾過多時自動暫停推送</t>
         </is>
       </c>
       <c r="C46" s="13" t="inlineStr">
@@ -1954,7 +1954,7 @@
       </c>
       <c r="E46" s="6" t="inlineStr">
         <is>
-          <t>node --test lib/otaRollout.test.mjs 6/6：10,000 隨機 MAC 在 10%/50% 誤差 &lt; 1 個百分點、同 MAC（含大小寫/空白）結果一致、升階段只增不減、白名單各階段都在、不同版本選不同的 10%。tsc --noEmit 通過。分支 dev server（3216）+ 本機 Supabase 模擬 20 台（板型 p218-sim，連跑兩次 9/9）：白名單階段只有 1 台、重複不變；10% 拿到的正是雜湊預測的那組（2–5 台含白名單），重複不變；50% 包含 10% 全部；暫停 → 0 台且下載映像 404，恢復 → 200；100% → 除已更新和已回滾的 2 台外 18 台；每台下發次數與記錄一致；運行中/已回滾正確標記；審計 6 筆對應 6 次變更。真 spotpear-ai-toy（預設 100%）回報 1.6.1 → 仍拿到 1.6.2。測試數據已清除</t>
+          <t>migration 20261014200000 BEGIN/ROLLBACK 套用兩次無錯並已套用本機。模擬 20 台連跑兩次 12/12：1/20 回滾不暫停、其餘 18 台照常；2/20 → 'Auto-paused: 2 of 20 boards rolled back (10%)'，其餘 0 台拿到 ota；已運行的設備記為 running 且不再下發；審計 1 筆 actor 空；恢復後 17 台拿到、保持恢復，第 3 台回滾 → 'Auto-paused: 3 of 20 (15%)'；白名單 2 台中 1 台回滾 → 50% 立即暫停、另一台不再下發；anon 呼叫 ota_maybe_pause → 401/42501。測試數據已清除，spotpear-ai-toy 1.6.2 仍 100% 未暫停</t>
         </is>
       </c>
       <c r="F46" s="11" t="n"/>
@@ -1962,15 +1962,15 @@
       <c r="H46" s="11" t="n"/>
       <c r="I46" s="12" t="n"/>
     </row>
-    <row r="47" ht="172" customHeight="1">
+    <row r="47" ht="200" customHeight="1">
       <c r="A47" s="13" t="inlineStr">
         <is>
-          <t>P2-17</t>
+          <t>P2-18</t>
         </is>
       </c>
       <c r="B47" s="6" t="inlineStr">
         <is>
-          <t>P2-16 ① 分批推送的數據表：推送階段、白名單、每台安裝結果</t>
+          <t>P2-16 ② 按 MAC 雜湊穩定分組決定哪台收到 ota</t>
         </is>
       </c>
       <c r="C47" s="13" t="inlineStr">
@@ -1985,7 +1985,7 @@
       </c>
       <c r="E47" s="6" t="inlineStr">
         <is>
-          <t>migration 20261014190000 BEGIN/ROLLBACK 套用兩次無錯並已套用本機；行為：預設 100%、promote 記 stage_changed_at，7 種壞值（25%、小寫/空字串/NULL MAC、暫停缺原因等）全被 check 擋；ota_note_offer 1→2→3，report 正確標 running/failed、別板型不影響，刪發佈連帶刪記錄；審計 5 筆含 'test-board 9.9.9' 標籤。REST 13/13：超管可讀、內容管理員 0 行、anon 42501，三種身份寫入/改階段/呼叫 ota_note_offer 皆 42501。release_firmware.py promote spotpear-ai-toy 1.6.2 成功，token 查詢仍選 1.6.2，審計記 2 筆（actor 空＝service role）</t>
+          <t>node --test lib/otaRollout.test.mjs 6/6：10,000 隨機 MAC 在 10%/50% 誤差 &lt; 1 個百分點、同 MAC（含大小寫/空白）結果一致、升階段只增不減、白名單各階段都在、不同版本選不同的 10%。tsc --noEmit 通過。分支 dev server（3216）+ 本機 Supabase 模擬 20 台（板型 p218-sim，連跑兩次 9/9）：白名單階段只有 1 台、重複不變；10% 拿到的正是雜湊預測的那組（2–5 台含白名單），重複不變；50% 包含 10% 全部；暫停 → 0 台且下載映像 404，恢復 → 200；100% → 除已更新和已回滾的 2 台外 18 台；每台下發次數與記錄一致；運行中/已回滾正確標記；審計 6 筆對應 6 次變更。真 spotpear-ai-toy（預設 100%）回報 1.6.1 → 仍拿到 1.6.2。測試數據已清除</t>
         </is>
       </c>
       <c r="F47" s="11" t="n"/>
@@ -1993,15 +1993,15 @@
       <c r="H47" s="11" t="n"/>
       <c r="I47" s="12" t="n"/>
     </row>
-    <row r="48" ht="116" customHeight="1">
+    <row r="48" ht="172" customHeight="1">
       <c r="A48" s="13" t="inlineStr">
         <is>
-          <t>R-41</t>
+          <t>P2-17</t>
         </is>
       </c>
       <c r="B48" s="6" t="inlineStr">
         <is>
-          <t>App 顯示玩具電量狀態（低電量提示）</t>
+          <t>P2-16 ① 分批推送的數據表：推送階段、白名單、每台安裝結果</t>
         </is>
       </c>
       <c r="C48" s="13" t="inlineStr">
@@ -2016,7 +2016,7 @@
       </c>
       <c r="E48" s="6" t="inlineStr">
         <is>
-          <t>① pytest 33 passed；真 PATCH 本地 Supabase ② 62:70 刷 p212+R-41 強制低電 build（SUPPLY_LOW_RATIO_OVERRIDE=1.05）→ 串口 [WSc] power low:true，本地 DB battery_low=t ③ 刷回正常 1.6.2 → low:false，DB=f ④ App 讀 DB：低電紅標+Please charge+更新時間、72% 充電中、未上報不顯示 ⑤ 他人帳號 0 行、authenticated UPDATE 被拒。62:70 已還原為原 p212 build</t>
+          <t>migration 20261014190000 BEGIN/ROLLBACK 套用兩次無錯並已套用本機；行為：預設 100%、promote 記 stage_changed_at，7 種壞值（25%、小寫/空字串/NULL MAC、暫停缺原因等）全被 check 擋；ota_note_offer 1→2→3，report 正確標 running/failed、別板型不影響，刪發佈連帶刪記錄；審計 5 筆含 'test-board 9.9.9' 標籤。REST 13/13：超管可讀、內容管理員 0 行、anon 42501，三種身份寫入/改階段/呼叫 ota_note_offer 皆 42501。release_firmware.py promote spotpear-ai-toy 1.6.2 成功，token 查詢仍選 1.6.2，審計記 2 筆（actor 空＝service role）</t>
         </is>
       </c>
       <c r="F48" s="11" t="n"/>
@@ -2024,15 +2024,15 @@
       <c r="H48" s="11" t="n"/>
       <c r="I48" s="12" t="n"/>
     </row>
-    <row r="49" ht="102" customHeight="1">
+    <row r="49" ht="116" customHeight="1">
       <c r="A49" s="13" t="inlineStr">
         <is>
-          <t>P0-12</t>
+          <t>R-41</t>
         </is>
       </c>
       <c r="B49" s="6" t="inlineStr">
         <is>
-          <t>收緊 Admin 權限與路由保護</t>
+          <t>App 顯示玩具電量狀態（低電量提示）</t>
         </is>
       </c>
       <c r="C49" s="13" t="inlineStr">
@@ -2042,12 +2042,12 @@
       </c>
       <c r="D49" s="13" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E49" s="6" t="inlineStr">
         <is>
-          <t>線上 2026-10-12（bac24e9）：runbook 10/08 檢查 未登入 /admin→/login、/api/admin→401、has_role() 只看角色、無管理員 policy 觸及 conversations/記憶表、超管≥1；未登入 /home、/admin→/login；用戶確認：家長帳號開 /admin 轉回 /home、管理員在 /admin 修改角色保存成功；角色細分權限沿用本機 61/61</t>
+          <t>① pytest 33 passed；真 PATCH 本地 Supabase ② 62:70 刷 p212+R-41 強制低電 build（SUPPLY_LOW_RATIO_OVERRIDE=1.05）→ 串口 [WSc] power low:true，本地 DB battery_low=t ③ 刷回正常 1.6.2 → low:false，DB=f ④ App 讀 DB：低電紅標+Please charge+更新時間、72% 充電中、未上報不顯示 ⑤ 他人帳號 0 行、authenticated UPDATE 被拒。62:70 已還原為原 p212 build</t>
         </is>
       </c>
       <c r="F49" s="11" t="n"/>
@@ -2055,15 +2055,15 @@
       <c r="H49" s="11" t="n"/>
       <c r="I49" s="12" t="n"/>
     </row>
-    <row r="50" ht="88" customHeight="1">
+    <row r="50" ht="102" customHeight="1">
       <c r="A50" s="13" t="inlineStr">
         <is>
-          <t>P0-15</t>
+          <t>P0-12</t>
         </is>
       </c>
       <c r="B50" s="6" t="inlineStr">
         <is>
-          <t>角色表權限：只有內容管理員能發佈，關閉家長自建角色</t>
+          <t>收緊 Admin 權限與路由保護</t>
         </is>
       </c>
       <c r="C50" s="13" t="inlineStr">
@@ -2078,7 +2078,7 @@
       </c>
       <c r="E50" s="6" t="inlineStr">
         <is>
-          <t>線上 2026-10-12：② anon 只見 6 個已發佈 hk_ 內建，查隱藏/醫生/家長自建 → []，anon POST → 401；① authenticated 寫入權限由 20261007140000 REVOKE（runbook 10/08 已套用）；用戶確認：④ 家長登入後 /home/create 轉回 /home ③ 管理員在 /admin 修改角色保存成功</t>
+          <t>線上 2026-10-12（bac24e9）：runbook 10/08 檢查 未登入 /admin→/login、/api/admin→401、has_role() 只看角色、無管理員 policy 觸及 conversations/記憶表、超管≥1；未登入 /home、/admin→/login；用戶確認：家長帳號開 /admin 轉回 /home、管理員在 /admin 修改角色保存成功；角色細分權限沿用本機 61/61</t>
         </is>
       </c>
       <c r="F50" s="11" t="n"/>
@@ -2089,12 +2089,12 @@
     <row r="51" ht="88" customHeight="1">
       <c r="A51" s="13" t="inlineStr">
         <is>
-          <t>P0-16</t>
+          <t>P0-15</t>
         </is>
       </c>
       <c r="B51" s="6" t="inlineStr">
         <is>
-          <t>移除「醫生」身份與寫死的通關碼</t>
+          <t>角色表權限：只有內容管理員能發佈，關閉家長自建角色</t>
         </is>
       </c>
       <c r="C51" s="13" t="inlineStr">
@@ -2109,7 +2109,7 @@
       </c>
       <c r="E51" s="6" t="inlineStr">
         <is>
-          <t>線上 2026-10-12：生產 commit bac24e9 git grep checkDoctorAction/kiwi-subtle-emu/=== "doctor"/isDoctor → 0；線上 13 個 JS（/、/login、/onboard）grep 通關碼/"doctor"/Santa/patient → 0；anon 讀角色只見 6 個 hk_ 角色、is_doctor 全 false；用戶今日線上登入及 playground 正常</t>
+          <t>線上 2026-10-12：② anon 只見 6 個已發佈 hk_ 內建，查隱藏/醫生/家長自建 → []，anon POST → 401；① authenticated 寫入權限由 20261007140000 REVOKE（runbook 10/08 已套用）；用戶確認：④ 家長登入後 /home/create 轉回 /home ③ 管理員在 /admin 修改角色保存成功</t>
         </is>
       </c>
       <c r="F51" s="11" t="n"/>
@@ -2117,15 +2117,15 @@
       <c r="H51" s="11" t="n"/>
       <c r="I51" s="12" t="n"/>
     </row>
-    <row r="52" ht="60" customHeight="1">
+    <row r="52" ht="88" customHeight="1">
       <c r="A52" s="13" t="inlineStr">
         <is>
-          <t>P0-09</t>
+          <t>P0-16</t>
         </is>
       </c>
       <c r="B52" s="6" t="inlineStr">
         <is>
-          <t>瀏覽器語音路由改用簽名 token（/ws/nextjs）</t>
+          <t>移除「醫生」身份與寫死的通關碼</t>
         </is>
       </c>
       <c r="C52" s="13" t="inlineStr">
@@ -2140,7 +2140,7 @@
       </c>
       <c r="E52" s="6" t="inlineStr">
         <is>
-          <t>線上 2026-10-12（bac24e9）：wss /fastapi/ws/nextjs 只帶 user_id 或 token=bogus → 4401；用戶確認：登入 elatoai.hkqft.com 後網頁 playground 可正常對話</t>
+          <t>線上 2026-10-12：生產 commit bac24e9 git grep checkDoctorAction/kiwi-subtle-emu/=== "doctor"/isDoctor → 0；線上 13 個 JS（/、/login、/onboard）grep 通關碼/"doctor"/Santa/patient → 0；anon 讀角色只見 6 個 hk_ 角色、is_doctor 全 false；用戶今日線上登入及 playground 正常</t>
         </is>
       </c>
       <c r="F52" s="11" t="n"/>
@@ -2151,12 +2151,12 @@
     <row r="53" ht="60" customHeight="1">
       <c r="A53" s="13" t="inlineStr">
         <is>
-          <t>P0-17</t>
+          <t>P0-09</t>
         </is>
       </c>
       <c r="B53" s="6" t="inlineStr">
         <is>
-          <t>前端的 anon key 必須是公開 key，不可是 secret／service_role</t>
+          <t>瀏覽器語音路由改用簽名 token（/ws/nextjs）</t>
         </is>
       </c>
       <c r="C53" s="13" t="inlineStr">
@@ -2171,7 +2171,7 @@
       </c>
       <c r="E53" s="6" t="inlineStr">
         <is>
-          <t>線上 2026-10-12（bac24e9）：/login 引用的 13 個 JS + HTML 無 sb_secret_，唯一 key 為 role=anon 的 JWT；② 用該 key GET /rest/v1/users → 42501；③ 本機 10/07 已換 publishable</t>
+          <t>線上 2026-10-12（bac24e9）：wss /fastapi/ws/nextjs 只帶 user_id 或 token=bogus → 4401；用戶確認：登入 elatoai.hkqft.com 後網頁 playground 可正常對話</t>
         </is>
       </c>
       <c r="F53" s="11" t="n"/>
@@ -2360,7 +2360,7 @@
       </c>
       <c r="C63" s="6" t="inlineStr">
         <is>
-          <t>等 P2-19、P2-20、P2-14</t>
+          <t>等 P2-20、P2-14</t>
         </is>
       </c>
       <c r="D63" s="11" t="n"/>
@@ -9429,7 +9429,7 @@
         </is>
       </c>
     </row>
-    <row r="85" ht="130" customHeight="1">
+    <row r="85" ht="172" customHeight="1">
       <c r="A85" s="13" t="inlineStr">
         <is>
           <t>P2-16</t>
@@ -9479,12 +9479,12 @@
       </c>
       <c r="K85" s="6" t="inlineStr">
         <is>
-          <t>後台可上傳韌體（伺服器算 SHA-256、寫 firmware_releases）、填說明、設為 current；推送分階段：白名單 MAC → 10% → 50% → 100%，按 MAC 雜湊穩定分組；回滾率超過 5% 或任一台在試用期內重啟 3 次即自動暫停；顯示每個版本已更新、回滾台數與回滾設備清單；顯示 app 分區用量（P2-12）；每個發佈操作寫入審計記錄。</t>
+          <t>後台可上傳韌體（伺服器算 SHA-256、寫 firmware_releases）、填說明、設為 current；推送分階段：白名單 MAC → 10% → 50% → 100%，按 MAC 雜湊穩定分組；回滾率超過 5% 即自動暫停（2026-10-14 拿走「同一台重啟 3 次」，見 P2-19）；顯示每個版本已更新、回滾台數與回滾設備清單；顯示 app 分區用量（P2-12）；每個發佈操作寫入審計記錄。</t>
         </is>
       </c>
       <c r="L85" s="6" t="inlineStr">
         <is>
-          <t>本機 Supabase + 裝置模擬器（2bb6656）模擬 20 台：① 10% 階段只有約 2 台拿到 ota，重複請求結果不變 ② 讓 2 台回報 failed_version → 自動暫停，其餘不再拿到 ota ③ 推到 100% 全部拿到 ④ 開發板 62:70 實機走一次白名單階段並確認新版本 ⑤ 審計表有每次階段變更</t>
+          <t>本機 Supabase 模擬 20 台：① 10% 階段只有約 2 台拿到 ota，重複請求結果不變 ② 讓 2 台回報 failed_version → 自動暫停，其餘不再拿到 ota ③ 推到 100% 全部拿到 ④ 開發板 62:70 實機走一次白名單階段並確認新版本 ⑤ 審計表有每次階段變更</t>
         </is>
       </c>
       <c r="M85" s="13" t="inlineStr">
@@ -9496,7 +9496,8 @@
         <is>
           <t>[2026-10-14] 新增
 [2026-10-14] 2026-10-14 開分支 p2-16-ota-rollout（worktree ../aibuddy-p216，從 dev cac98aa）；拆成 P2-17～P2-21 五項子任務，本項的測試方法即整體驗收（含 62:70 實機白名單）。
-[2026-10-14] 2026-10-14 用戶決定提前到第 2 階段，現在開始做</t>
+[2026-10-14] 2026-10-14 用戶決定提前到第 2 階段，現在開始做
+[2026-10-14] 2026-10-14 用戶決定拿走「同一台重啟 3 次即暫停」，原因見 P2-19</t>
         </is>
       </c>
     </row>
@@ -9954,7 +9955,7 @@
         </is>
       </c>
     </row>
-    <row r="92" ht="74" customHeight="1">
+    <row r="92" ht="214" customHeight="1">
       <c r="A92" s="13" t="inlineStr">
         <is>
           <t>P2-19</t>
@@ -9982,12 +9983,17 @@
       </c>
       <c r="F92" s="13" t="inlineStr">
         <is>
-          <t>未開始</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="G92" s="13" t="inlineStr">
         <is>
-          <t>未測試</t>
+          <t>通過</t>
+        </is>
+      </c>
+      <c r="H92" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="I92" s="6" t="inlineStr">
@@ -10002,12 +10008,12 @@
       </c>
       <c r="K92" s="6" t="inlineStr">
         <is>
-          <t>已下發的設備中回滾率 &gt; 5%，或任一台對同一版本被下發 3 次仍未確認，即自動暫停該版本並記下原因；暫停後其餘設備不再拿到 ota；已確認的設備不受影響；自動暫停寫入審計記錄（操作者記為系統）；只能由超級管理員在後台恢復。</t>
+          <t>已下發的設備中回滾率 &gt; 5% 即自動暫停該版本並記下原因（台數少的階段第一台回滾就暫停）；暫停後其餘設備不再拿到 ota、映像不再提供下載；已在運行該版本的設備不受影響；自動暫停寫入審計記錄（操作者為空、paused_by 為空、原因以 Auto-paused 開頭）；只能由超級管理員恢復，恢復後要有新的回滾才會再判斷。</t>
         </is>
       </c>
       <c r="L92" s="6" t="inlineStr">
         <is>
-          <t>本機模擬 20 台、100% 階段：讓 2 台回報 failed_version → 該版本變暫停、原因含回滾率，其餘 18 台下一次請求不再拿到 ota；另讓 1 台連續 3 次拿到 ota 不確認 → 暫停；審計表各多一筆</t>
+          <t>本機模擬 20 台（分支 dev server + 本機 Supabase）：100% 階段 1 台回滾（5%）不暫停；第 2 台回滾（10%）→ 暫停、原因含回滾率，其餘 18 台不再拿到 ota；已運行新版的設備照常；審計多一筆、actor 為空；恢復後保持恢復，第 3 台回滾再暫停；白名單 2 台中 1 台回滾 → 立即暫停；anon 呼叫 ota_maybe_pause → 42501</t>
         </is>
       </c>
       <c r="M92" s="13" t="inlineStr">
@@ -10015,10 +10021,21 @@
           <t>P2-18</t>
         </is>
       </c>
+      <c r="N92" s="6" t="inlineStr">
+        <is>
+          <t>migration 20261014200000 BEGIN/ROLLBACK 套用兩次無錯並已套用本機。模擬 20 台連跑兩次 12/12：1/20 回滾不暫停、其餘 18 台照常；2/20 → 'Auto-paused: 2 of 20 boards rolled back (10%)'，其餘 0 台拿到 ota；已運行的設備記為 running 且不再下發；審計 1 筆 actor 空；恢復後 17 台拿到、保持恢復，第 3 台回滾 → 'Auto-paused: 3 of 20 (15%)'；白名單 2 台中 1 台回滾 → 50% 立即暫停、另一台不再下發；anon 呼叫 ota_maybe_pause → 401/42501。測試數據已清除，spotpear-ai-toy 1.6.2 仍 100% 未暫停</t>
+        </is>
+      </c>
+      <c r="O92" s="13" t="inlineStr">
+        <is>
+          <t>9500d50</t>
+        </is>
+      </c>
       <c r="P92" s="6" t="inlineStr">
         <is>
           <t>[2026-10-14] 新增
-[2026-10-14] 2026-10-14 用戶決定提前到第 2 階段，現在開始做</t>
+[2026-10-14] 2026-10-14 用戶決定提前到第 2 階段，現在開始做
+[2026-10-14] 2026-10-14 用戶決定拿走「同一台下發/下載 3 次未確認即暫停」：實測中途斷開的下載 3 次有 1 次被當成完整下載（伺服器只知道寫進緩衝區），線上映像經 nginx 和 Cloudflare 會被整個先收下，伺服器永遠看到下載完成；按下發次數計會把網絡不穩（C3 TLS）誤判成壞版本。韌體已把崩潰和試用期內斷電重裝 2 次（OTA_MAX_TRIES）都回報成回滾，由回滾率規則處理。</t>
         </is>
       </c>
     </row>
@@ -10740,7 +10757,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I290"/>
+  <dimension ref="A1:I294"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -20764,8 +20781,152 @@
       </c>
       <c r="I290" s="6" t="n"/>
     </row>
+    <row r="291" ht="32" customHeight="1">
+      <c r="A291" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 20:51</t>
+        </is>
+      </c>
+      <c r="B291" s="13" t="inlineStr">
+        <is>
+          <t>P2-19</t>
+        </is>
+      </c>
+      <c r="C291" s="6" t="inlineStr">
+        <is>
+          <t>P2-16 ③ 回滾過多時自動暫停推送</t>
+        </is>
+      </c>
+      <c r="D291" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E291" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F291" s="13" t="n"/>
+      <c r="G291" s="6" t="n"/>
+      <c r="H291" s="13" t="n"/>
+      <c r="I291" s="6" t="n"/>
+    </row>
+    <row r="292" ht="158" customHeight="1">
+      <c r="A292" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 20:58</t>
+        </is>
+      </c>
+      <c r="B292" s="13" t="inlineStr">
+        <is>
+          <t>P2-19</t>
+        </is>
+      </c>
+      <c r="C292" s="6" t="inlineStr">
+        <is>
+          <t>P2-16 ③ 回滾過多時自動暫停推送</t>
+        </is>
+      </c>
+      <c r="D292" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="E292" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F292" s="13" t="n"/>
+      <c r="G292" s="6" t="n"/>
+      <c r="H292" s="13" t="n"/>
+      <c r="I292" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-14 用戶決定拿走「同一台下發/下載 3 次未確認即暫停」：實測中途斷開的下載 3 次有 1 次被當成完整下載（伺服器只知道寫進緩衝區），線上映像經 nginx 和 Cloudflare 會被整個先收下，伺服器永遠看到下載完成；按下發次數計會把網絡不穩（C3 TLS）誤判成壞版本。韌體已把崩潰和試用期內斷電重裝 2 次（OTA_MAX_TRIES）都回報成回滾，由回滾率規則處理。；修改了驗收標準、測試方法</t>
+        </is>
+      </c>
+    </row>
+    <row r="293" ht="144" customHeight="1">
+      <c r="A293" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 20:58</t>
+        </is>
+      </c>
+      <c r="B293" s="13" t="inlineStr">
+        <is>
+          <t>P2-19</t>
+        </is>
+      </c>
+      <c r="C293" s="6" t="inlineStr">
+        <is>
+          <t>P2-16 ③ 回滾過多時自動暫停推送</t>
+        </is>
+      </c>
+      <c r="D293" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="E293" s="13" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="F293" s="13" t="inlineStr">
+        <is>
+          <t>通過</t>
+        </is>
+      </c>
+      <c r="G293" s="6" t="inlineStr">
+        <is>
+          <t>migration 20261014200000 BEGIN/ROLLBACK 套用兩次無錯並已套用本機。模擬 20 台連跑兩次 12/12：1/20 回滾不暫停、其餘 18 台照常；2/20 → 'Auto-paused: 2 of 20 boards rolled back (10%)'，其餘 0 台拿到 ota；已運行的設備記為 running 且不再下發；審計 1 筆 actor 空；恢復後 17 台拿到、保持恢復，第 3 台回滾 → 'Auto-paused: 3 of 20 (15%)'；白名單 2 台中 1 台回滾 → 50% 立即暫停、另一台不再下發；anon 呼叫 ota_maybe_pause → 401/42501。測試數據已清除，spotpear-ai-toy 1.6.2 仍 100% 未暫停</t>
+        </is>
+      </c>
+      <c r="H293" s="13" t="inlineStr">
+        <is>
+          <t>9500d50</t>
+        </is>
+      </c>
+      <c r="I293" s="6" t="n"/>
+    </row>
+    <row r="294" ht="46" customHeight="1">
+      <c r="A294" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 20:58</t>
+        </is>
+      </c>
+      <c r="B294" s="13" t="inlineStr">
+        <is>
+          <t>P2-16</t>
+        </is>
+      </c>
+      <c r="C294" s="6" t="inlineStr">
+        <is>
+          <t>OTA 分批推送與後台發佈頁</t>
+        </is>
+      </c>
+      <c r="D294" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="E294" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F294" s="13" t="n"/>
+      <c r="G294" s="6" t="n"/>
+      <c r="H294" s="13" t="n"/>
+      <c r="I294" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-14 用戶決定拿走「同一台重啟 3 次即暫停」，原因見 P2-19；修改了驗收標準、測試方法</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I290"/>
+  <autoFilter ref="A1:I294"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Track P2-20 (admin firmware upload) as passed.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/production-readiness.xlsx
+++ b/docs/production-readiness.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'任務清單'!$A$1:$P$94</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'待確認問題'!$A$1:$G$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$294</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$296</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -641,7 +641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I106"/>
+  <dimension ref="A1:I105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -665,14 +665,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>最後更新：2026-10-14 20:58　·　本頁由 tracker.py 自動生成，請勿手動編輯</t>
+          <t>最後更新：2026-10-14 21:10　·　本頁由 tracker.py 自動生成，請勿手動編輯</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>總進度：21/89 已完成（24%）　·　目前階段：1 止血定案（10/5–10/16）</t>
+          <t>總進度：22/89 已完成（25%）　·　目前階段：1 止血定案（10/5–10/16）</t>
         </is>
       </c>
     </row>
@@ -820,7 +820,7 @@
       </c>
       <c r="D8" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A8,'任務清單'!$F:$F,D$5)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E8" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A8,'任務清單'!$F:$F,E$5)</f>
@@ -828,7 +828,7 @@
       </c>
       <c r="F8" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A8,'任務清單'!$F:$F,F$5)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G8" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A8,'任務清單'!$F:$F,G$5)</f>
@@ -840,7 +840,7 @@
       </c>
       <c r="I8" s="8">
         <f>IFERROR(F8/(C8-H8),0)</f>
-        <v>0.2857142857142857</v>
+        <v>0.3333333333333333</v>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1">
@@ -896,7 +896,7 @@
       </c>
       <c r="D10" s="5">
         <f>SUM(D6:D9)</f>
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E10" s="5">
         <f>SUM(E6:E9)</f>
@@ -904,7 +904,7 @@
       </c>
       <c r="F10" s="5">
         <f>SUM(F6:F9)</f>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G10" s="5">
         <f>SUM(G6:G9)</f>
@@ -916,7 +916,7 @@
       </c>
       <c r="I10" s="9">
         <f>IFERROR(F10/(C10-H10),0)</f>
-        <v>0.23595505617977527</v>
+        <v>0.24719101123595505</v>
       </c>
     </row>
     <row r="12">
@@ -1023,7 +1023,7 @@
       </c>
       <c r="D14" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A14,'任務清單'!$F:$F,D$12)</f>
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E14" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A14,'任務清單'!$F:$F,E$12)</f>
@@ -1031,7 +1031,7 @@
       </c>
       <c r="F14" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A14,'任務清單'!$F:$F,F$12)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G14" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A14,'任務清單'!$F:$F,G$12)</f>
@@ -1043,7 +1043,7 @@
       </c>
       <c r="I14" s="8">
         <f>IFERROR(F14/(C14-H14),0)</f>
-        <v>0.18181818181818182</v>
+        <v>0.21212121212121213</v>
       </c>
     </row>
     <row r="15" ht="46" customHeight="1">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="D17" s="5">
         <f>SUM(D13:D16)</f>
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E17" s="5">
         <f>SUM(E13:E16)</f>
@@ -1147,7 +1147,7 @@
       </c>
       <c r="F17" s="5">
         <f>SUM(F13:F16)</f>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G17" s="5">
         <f>SUM(G13:G16)</f>
@@ -1159,7 +1159,7 @@
       </c>
       <c r="I17" s="9">
         <f>IFERROR(F17/(C17-H17),0)</f>
-        <v>0.23595505617977527</v>
+        <v>0.24719101123595505</v>
       </c>
     </row>
     <row r="19">
@@ -1931,15 +1931,15 @@
       <c r="H45" s="11" t="n"/>
       <c r="I45" s="12" t="n"/>
     </row>
-    <row r="46" ht="158" customHeight="1">
+    <row r="46" ht="214" customHeight="1">
       <c r="A46" s="13" t="inlineStr">
         <is>
-          <t>P2-19</t>
+          <t>P2-20</t>
         </is>
       </c>
       <c r="B46" s="6" t="inlineStr">
         <is>
-          <t>P2-16 ③ 回滾過多時自動暫停推送</t>
+          <t>P2-16 ④ 從後台上傳與發佈韌體（取代手貼 service key）</t>
         </is>
       </c>
       <c r="C46" s="13" t="inlineStr">
@@ -1954,7 +1954,7 @@
       </c>
       <c r="E46" s="6" t="inlineStr">
         <is>
-          <t>migration 20261014200000 BEGIN/ROLLBACK 套用兩次無錯並已套用本機。模擬 20 台連跑兩次 12/12：1/20 回滾不暫停、其餘 18 台照常；2/20 → 'Auto-paused: 2 of 20 boards rolled back (10%)'，其餘 0 台拿到 ota；已運行的設備記為 running 且不再下發；審計 1 筆 actor 空；恢復後 17 台拿到、保持恢復，第 3 台回滾 → 'Auto-paused: 3 of 20 (15%)'；白名單 2 台中 1 台回滾 → 50% 立即暫停、另一台不再下發；anon 呼叫 ota_maybe_pause → 401/42501。測試數據已清除，spotpear-ai-toy 1.6.2 仍 100% 未暫停</t>
+          <t>node --test lib/firmwareImage.test.mjs 8/8（合成映像：dev build、無標記、未知板、晶片不符、非映像、截斷/損壞、超 4MB 拒；超 2MB 只警告）。分支 dev server + 本機 Supabase 端到端 16/16（GoTrue 真實登入的 cookie）：超管上傳 9.9.0 release build → 201 草稿（is_current f、rollout 0%），DB SHA-256 = 檔案、storage 原樣；審計 insert 記該超管；設備仍只拿到 current 1.6.2；已有 1.0.2 → 409；localall → 422 dev build；4MB+16 → 422；9MB → 413；PNG → 422；舊 1.6.1 映像（無標記）→ 422 指向 release_firmware.py；內容管理員上傳/刪除 → 403；未登入 → 401；刪 current → 409；超管刪草稿 → 行和映像都刪、審計 delete 記該超管。release_firmware.py list 照常。測試帳號與數據已清除</t>
         </is>
       </c>
       <c r="F46" s="11" t="n"/>
@@ -1962,15 +1962,15 @@
       <c r="H46" s="11" t="n"/>
       <c r="I46" s="12" t="n"/>
     </row>
-    <row r="47" ht="200" customHeight="1">
+    <row r="47" ht="158" customHeight="1">
       <c r="A47" s="13" t="inlineStr">
         <is>
-          <t>P2-18</t>
+          <t>P2-19</t>
         </is>
       </c>
       <c r="B47" s="6" t="inlineStr">
         <is>
-          <t>P2-16 ② 按 MAC 雜湊穩定分組決定哪台收到 ota</t>
+          <t>P2-16 ③ 回滾過多時自動暫停推送</t>
         </is>
       </c>
       <c r="C47" s="13" t="inlineStr">
@@ -1985,7 +1985,7 @@
       </c>
       <c r="E47" s="6" t="inlineStr">
         <is>
-          <t>node --test lib/otaRollout.test.mjs 6/6：10,000 隨機 MAC 在 10%/50% 誤差 &lt; 1 個百分點、同 MAC（含大小寫/空白）結果一致、升階段只增不減、白名單各階段都在、不同版本選不同的 10%。tsc --noEmit 通過。分支 dev server（3216）+ 本機 Supabase 模擬 20 台（板型 p218-sim，連跑兩次 9/9）：白名單階段只有 1 台、重複不變；10% 拿到的正是雜湊預測的那組（2–5 台含白名單），重複不變；50% 包含 10% 全部；暫停 → 0 台且下載映像 404，恢復 → 200；100% → 除已更新和已回滾的 2 台外 18 台；每台下發次數與記錄一致；運行中/已回滾正確標記；審計 6 筆對應 6 次變更。真 spotpear-ai-toy（預設 100%）回報 1.6.1 → 仍拿到 1.6.2。測試數據已清除</t>
+          <t>migration 20261014200000 BEGIN/ROLLBACK 套用兩次無錯並已套用本機。模擬 20 台連跑兩次 12/12：1/20 回滾不暫停、其餘 18 台照常；2/20 → 'Auto-paused: 2 of 20 boards rolled back (10%)'，其餘 0 台拿到 ota；已運行的設備記為 running 且不再下發；審計 1 筆 actor 空；恢復後 17 台拿到、保持恢復，第 3 台回滾 → 'Auto-paused: 3 of 20 (15%)'；白名單 2 台中 1 台回滾 → 50% 立即暫停、另一台不再下發；anon 呼叫 ota_maybe_pause → 401/42501。測試數據已清除，spotpear-ai-toy 1.6.2 仍 100% 未暫停</t>
         </is>
       </c>
       <c r="F47" s="11" t="n"/>
@@ -1993,15 +1993,15 @@
       <c r="H47" s="11" t="n"/>
       <c r="I47" s="12" t="n"/>
     </row>
-    <row r="48" ht="172" customHeight="1">
+    <row r="48" ht="200" customHeight="1">
       <c r="A48" s="13" t="inlineStr">
         <is>
-          <t>P2-17</t>
+          <t>P2-18</t>
         </is>
       </c>
       <c r="B48" s="6" t="inlineStr">
         <is>
-          <t>P2-16 ① 分批推送的數據表：推送階段、白名單、每台安裝結果</t>
+          <t>P2-16 ② 按 MAC 雜湊穩定分組決定哪台收到 ota</t>
         </is>
       </c>
       <c r="C48" s="13" t="inlineStr">
@@ -2016,7 +2016,7 @@
       </c>
       <c r="E48" s="6" t="inlineStr">
         <is>
-          <t>migration 20261014190000 BEGIN/ROLLBACK 套用兩次無錯並已套用本機；行為：預設 100%、promote 記 stage_changed_at，7 種壞值（25%、小寫/空字串/NULL MAC、暫停缺原因等）全被 check 擋；ota_note_offer 1→2→3，report 正確標 running/failed、別板型不影響，刪發佈連帶刪記錄；審計 5 筆含 'test-board 9.9.9' 標籤。REST 13/13：超管可讀、內容管理員 0 行、anon 42501，三種身份寫入/改階段/呼叫 ota_note_offer 皆 42501。release_firmware.py promote spotpear-ai-toy 1.6.2 成功，token 查詢仍選 1.6.2，審計記 2 筆（actor 空＝service role）</t>
+          <t>node --test lib/otaRollout.test.mjs 6/6：10,000 隨機 MAC 在 10%/50% 誤差 &lt; 1 個百分點、同 MAC（含大小寫/空白）結果一致、升階段只增不減、白名單各階段都在、不同版本選不同的 10%。tsc --noEmit 通過。分支 dev server（3216）+ 本機 Supabase 模擬 20 台（板型 p218-sim，連跑兩次 9/9）：白名單階段只有 1 台、重複不變；10% 拿到的正是雜湊預測的那組（2–5 台含白名單），重複不變；50% 包含 10% 全部；暫停 → 0 台且下載映像 404，恢復 → 200；100% → 除已更新和已回滾的 2 台外 18 台；每台下發次數與記錄一致；運行中/已回滾正確標記；審計 6 筆對應 6 次變更。真 spotpear-ai-toy（預設 100%）回報 1.6.1 → 仍拿到 1.6.2。測試數據已清除</t>
         </is>
       </c>
       <c r="F48" s="11" t="n"/>
@@ -2024,15 +2024,15 @@
       <c r="H48" s="11" t="n"/>
       <c r="I48" s="12" t="n"/>
     </row>
-    <row r="49" ht="116" customHeight="1">
+    <row r="49" ht="172" customHeight="1">
       <c r="A49" s="13" t="inlineStr">
         <is>
-          <t>R-41</t>
+          <t>P2-17</t>
         </is>
       </c>
       <c r="B49" s="6" t="inlineStr">
         <is>
-          <t>App 顯示玩具電量狀態（低電量提示）</t>
+          <t>P2-16 ① 分批推送的數據表：推送階段、白名單、每台安裝結果</t>
         </is>
       </c>
       <c r="C49" s="13" t="inlineStr">
@@ -2047,7 +2047,7 @@
       </c>
       <c r="E49" s="6" t="inlineStr">
         <is>
-          <t>① pytest 33 passed；真 PATCH 本地 Supabase ② 62:70 刷 p212+R-41 強制低電 build（SUPPLY_LOW_RATIO_OVERRIDE=1.05）→ 串口 [WSc] power low:true，本地 DB battery_low=t ③ 刷回正常 1.6.2 → low:false，DB=f ④ App 讀 DB：低電紅標+Please charge+更新時間、72% 充電中、未上報不顯示 ⑤ 他人帳號 0 行、authenticated UPDATE 被拒。62:70 已還原為原 p212 build</t>
+          <t>migration 20261014190000 BEGIN/ROLLBACK 套用兩次無錯並已套用本機；行為：預設 100%、promote 記 stage_changed_at，7 種壞值（25%、小寫/空字串/NULL MAC、暫停缺原因等）全被 check 擋；ota_note_offer 1→2→3，report 正確標 running/failed、別板型不影響，刪發佈連帶刪記錄；審計 5 筆含 'test-board 9.9.9' 標籤。REST 13/13：超管可讀、內容管理員 0 行、anon 42501，三種身份寫入/改階段/呼叫 ota_note_offer 皆 42501。release_firmware.py promote spotpear-ai-toy 1.6.2 成功，token 查詢仍選 1.6.2，審計記 2 筆（actor 空＝service role）</t>
         </is>
       </c>
       <c r="F49" s="11" t="n"/>
@@ -2055,15 +2055,15 @@
       <c r="H49" s="11" t="n"/>
       <c r="I49" s="12" t="n"/>
     </row>
-    <row r="50" ht="102" customHeight="1">
+    <row r="50" ht="116" customHeight="1">
       <c r="A50" s="13" t="inlineStr">
         <is>
-          <t>P0-12</t>
+          <t>R-41</t>
         </is>
       </c>
       <c r="B50" s="6" t="inlineStr">
         <is>
-          <t>收緊 Admin 權限與路由保護</t>
+          <t>App 顯示玩具電量狀態（低電量提示）</t>
         </is>
       </c>
       <c r="C50" s="13" t="inlineStr">
@@ -2073,12 +2073,12 @@
       </c>
       <c r="D50" s="13" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E50" s="6" t="inlineStr">
         <is>
-          <t>線上 2026-10-12（bac24e9）：runbook 10/08 檢查 未登入 /admin→/login、/api/admin→401、has_role() 只看角色、無管理員 policy 觸及 conversations/記憶表、超管≥1；未登入 /home、/admin→/login；用戶確認：家長帳號開 /admin 轉回 /home、管理員在 /admin 修改角色保存成功；角色細分權限沿用本機 61/61</t>
+          <t>① pytest 33 passed；真 PATCH 本地 Supabase ② 62:70 刷 p212+R-41 強制低電 build（SUPPLY_LOW_RATIO_OVERRIDE=1.05）→ 串口 [WSc] power low:true，本地 DB battery_low=t ③ 刷回正常 1.6.2 → low:false，DB=f ④ App 讀 DB：低電紅標+Please charge+更新時間、72% 充電中、未上報不顯示 ⑤ 他人帳號 0 行、authenticated UPDATE 被拒。62:70 已還原為原 p212 build</t>
         </is>
       </c>
       <c r="F50" s="11" t="n"/>
@@ -2086,15 +2086,15 @@
       <c r="H50" s="11" t="n"/>
       <c r="I50" s="12" t="n"/>
     </row>
-    <row r="51" ht="88" customHeight="1">
+    <row r="51" ht="102" customHeight="1">
       <c r="A51" s="13" t="inlineStr">
         <is>
-          <t>P0-15</t>
+          <t>P0-12</t>
         </is>
       </c>
       <c r="B51" s="6" t="inlineStr">
         <is>
-          <t>角色表權限：只有內容管理員能發佈，關閉家長自建角色</t>
+          <t>收緊 Admin 權限與路由保護</t>
         </is>
       </c>
       <c r="C51" s="13" t="inlineStr">
@@ -2109,7 +2109,7 @@
       </c>
       <c r="E51" s="6" t="inlineStr">
         <is>
-          <t>線上 2026-10-12：② anon 只見 6 個已發佈 hk_ 內建，查隱藏/醫生/家長自建 → []，anon POST → 401；① authenticated 寫入權限由 20261007140000 REVOKE（runbook 10/08 已套用）；用戶確認：④ 家長登入後 /home/create 轉回 /home ③ 管理員在 /admin 修改角色保存成功</t>
+          <t>線上 2026-10-12（bac24e9）：runbook 10/08 檢查 未登入 /admin→/login、/api/admin→401、has_role() 只看角色、無管理員 policy 觸及 conversations/記憶表、超管≥1；未登入 /home、/admin→/login；用戶確認：家長帳號開 /admin 轉回 /home、管理員在 /admin 修改角色保存成功；角色細分權限沿用本機 61/61</t>
         </is>
       </c>
       <c r="F51" s="11" t="n"/>
@@ -2120,12 +2120,12 @@
     <row r="52" ht="88" customHeight="1">
       <c r="A52" s="13" t="inlineStr">
         <is>
-          <t>P0-16</t>
+          <t>P0-15</t>
         </is>
       </c>
       <c r="B52" s="6" t="inlineStr">
         <is>
-          <t>移除「醫生」身份與寫死的通關碼</t>
+          <t>角色表權限：只有內容管理員能發佈，關閉家長自建角色</t>
         </is>
       </c>
       <c r="C52" s="13" t="inlineStr">
@@ -2140,7 +2140,7 @@
       </c>
       <c r="E52" s="6" t="inlineStr">
         <is>
-          <t>線上 2026-10-12：生產 commit bac24e9 git grep checkDoctorAction/kiwi-subtle-emu/=== "doctor"/isDoctor → 0；線上 13 個 JS（/、/login、/onboard）grep 通關碼/"doctor"/Santa/patient → 0；anon 讀角色只見 6 個 hk_ 角色、is_doctor 全 false；用戶今日線上登入及 playground 正常</t>
+          <t>線上 2026-10-12：② anon 只見 6 個已發佈 hk_ 內建，查隱藏/醫生/家長自建 → []，anon POST → 401；① authenticated 寫入權限由 20261007140000 REVOKE（runbook 10/08 已套用）；用戶確認：④ 家長登入後 /home/create 轉回 /home ③ 管理員在 /admin 修改角色保存成功</t>
         </is>
       </c>
       <c r="F52" s="11" t="n"/>
@@ -2148,15 +2148,15 @@
       <c r="H52" s="11" t="n"/>
       <c r="I52" s="12" t="n"/>
     </row>
-    <row r="53" ht="60" customHeight="1">
+    <row r="53" ht="88" customHeight="1">
       <c r="A53" s="13" t="inlineStr">
         <is>
-          <t>P0-09</t>
+          <t>P0-16</t>
         </is>
       </c>
       <c r="B53" s="6" t="inlineStr">
         <is>
-          <t>瀏覽器語音路由改用簽名 token（/ws/nextjs）</t>
+          <t>移除「醫生」身份與寫死的通關碼</t>
         </is>
       </c>
       <c r="C53" s="13" t="inlineStr">
@@ -2171,7 +2171,7 @@
       </c>
       <c r="E53" s="6" t="inlineStr">
         <is>
-          <t>線上 2026-10-12（bac24e9）：wss /fastapi/ws/nextjs 只帶 user_id 或 token=bogus → 4401；用戶確認：登入 elatoai.hkqft.com 後網頁 playground 可正常對話</t>
+          <t>線上 2026-10-12：生產 commit bac24e9 git grep checkDoctorAction/kiwi-subtle-emu/=== "doctor"/isDoctor → 0；線上 13 個 JS（/、/login、/onboard）grep 通關碼/"doctor"/Santa/patient → 0；anon 讀角色只見 6 個 hk_ 角色、is_doctor 全 false；用戶今日線上登入及 playground 正常</t>
         </is>
       </c>
       <c r="F53" s="11" t="n"/>
@@ -2324,20 +2324,20 @@
       <c r="H61" s="11" t="n"/>
       <c r="I61" s="12" t="n"/>
     </row>
-    <row r="62" ht="32" customHeight="1">
+    <row r="62" ht="18" customHeight="1">
       <c r="A62" s="13" t="inlineStr">
         <is>
-          <t>P2-20</t>
+          <t>P2-21</t>
         </is>
       </c>
       <c r="B62" s="6" t="inlineStr">
         <is>
-          <t>P2-16 ④ 從後台上傳與發佈韌體（取代手貼 service key）</t>
+          <t>P2-16 ⑤ 後台 OTA 頁換成真實數據與操作</t>
         </is>
       </c>
       <c r="C62" s="6" t="inlineStr">
         <is>
-          <t>等 P1-10</t>
+          <t>等 P2-14</t>
         </is>
       </c>
       <c r="D62" s="11" t="n"/>
@@ -2350,17 +2350,17 @@
     <row r="63" ht="18" customHeight="1">
       <c r="A63" s="13" t="inlineStr">
         <is>
-          <t>P2-21</t>
+          <t>R-05</t>
         </is>
       </c>
       <c r="B63" s="6" t="inlineStr">
         <is>
-          <t>P2-16 ⑤ 後台 OTA 頁換成真實數據與操作</t>
+          <t>內測版外殼（3D 打印 20 台）</t>
         </is>
       </c>
       <c r="C63" s="6" t="inlineStr">
         <is>
-          <t>等 P2-20、P2-14</t>
+          <t>等 R-01</t>
         </is>
       </c>
       <c r="D63" s="11" t="n"/>
@@ -2373,17 +2373,17 @@
     <row r="64" ht="18" customHeight="1">
       <c r="A64" s="13" t="inlineStr">
         <is>
-          <t>R-05</t>
+          <t>R-06</t>
         </is>
       </c>
       <c r="B64" s="6" t="inlineStr">
         <is>
-          <t>內測版外殼（3D 打印 20 台）</t>
+          <t>家長自助上手流程</t>
         </is>
       </c>
       <c r="C64" s="6" t="inlineStr">
         <is>
-          <t>等 R-01</t>
+          <t>等 P0-11</t>
         </is>
       </c>
       <c r="D64" s="11" t="n"/>
@@ -2393,20 +2393,20 @@
       <c r="H64" s="11" t="n"/>
       <c r="I64" s="12" t="n"/>
     </row>
-    <row r="65" ht="18" customHeight="1">
+    <row r="65" ht="32" customHeight="1">
       <c r="A65" s="13" t="inlineStr">
         <is>
-          <t>R-06</t>
+          <t>R-13</t>
         </is>
       </c>
       <c r="B65" s="6" t="inlineStr">
         <is>
-          <t>家長自助上手流程</t>
+          <t>CP1 內測就緒檢查（10/30）</t>
         </is>
       </c>
       <c r="C65" s="6" t="inlineStr">
         <is>
-          <t>等 P0-11</t>
+          <t>等 P0-07、P0-11、P1-01、P1-02、P2-09、R-01、R-02、R-04、R-05、R-06、P1-11</t>
         </is>
       </c>
       <c r="D65" s="11" t="n"/>
@@ -2419,17 +2419,17 @@
     <row r="66" ht="32" customHeight="1">
       <c r="A66" s="13" t="inlineStr">
         <is>
-          <t>R-13</t>
+          <t>R-18</t>
         </is>
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
-          <t>CP1 內測就緒檢查（10/30）</t>
+          <t>長按 BOOT 重新配網（開 AIBuddy-XXXX 熱點）</t>
         </is>
       </c>
       <c r="C66" s="6" t="inlineStr">
         <is>
-          <t>等 P0-07、P0-11、P1-01、P1-02、P2-09、R-01、R-02、R-04、R-05、R-06、P1-11</t>
+          <t>等 R-01</t>
         </is>
       </c>
       <c r="D66" s="11" t="n"/>
@@ -2442,12 +2442,12 @@
     <row r="67" ht="32" customHeight="1">
       <c r="A67" s="13" t="inlineStr">
         <is>
-          <t>R-18</t>
+          <t>R-19</t>
         </is>
       </c>
       <c r="B67" s="6" t="inlineStr">
         <is>
-          <t>長按 BOOT 重新配網（開 AIBuddy-XXXX 熱點）</t>
+          <t>外接按鈕：量產板加 I2C 擴展晶片（TCA9555）</t>
         </is>
       </c>
       <c r="C67" s="6" t="inlineStr">
@@ -2462,20 +2462,20 @@
       <c r="H67" s="11" t="n"/>
       <c r="I67" s="12" t="n"/>
     </row>
-    <row r="68" ht="32" customHeight="1">
+    <row r="68" ht="18" customHeight="1">
       <c r="A68" s="13" t="inlineStr">
         <is>
-          <t>R-19</t>
+          <t>R-20</t>
         </is>
       </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t>外接按鈕：量產板加 I2C 擴展晶片（TCA9555）</t>
+          <t>孩子資料與角色改成每台設備一份</t>
         </is>
       </c>
       <c r="C68" s="6" t="inlineStr">
         <is>
-          <t>等 R-01</t>
+          <t>等 P1-12</t>
         </is>
       </c>
       <c r="D68" s="11" t="n"/>
@@ -2485,20 +2485,20 @@
       <c r="H68" s="11" t="n"/>
       <c r="I68" s="12" t="n"/>
     </row>
-    <row r="69" ht="18" customHeight="1">
+    <row r="69" ht="32" customHeight="1">
       <c r="A69" s="13" t="inlineStr">
         <is>
-          <t>R-20</t>
+          <t>R-27</t>
         </is>
       </c>
       <c r="B69" s="6" t="inlineStr">
         <is>
-          <t>孩子資料與角色改成每台設備一份</t>
+          <t>App 內登入：驗證碼、原生社交登入、刪除帳號</t>
         </is>
       </c>
       <c r="C69" s="6" t="inlineStr">
         <is>
-          <t>等 P1-12</t>
+          <t>等 R-26</t>
         </is>
       </c>
       <c r="D69" s="11" t="n"/>
@@ -2508,20 +2508,20 @@
       <c r="H69" s="11" t="n"/>
       <c r="I69" s="12" t="n"/>
     </row>
-    <row r="70" ht="32" customHeight="1">
+    <row r="70" ht="18" customHeight="1">
       <c r="A70" s="13" t="inlineStr">
         <is>
-          <t>R-27</t>
+          <t>P0-14</t>
         </is>
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>App 內登入：驗證碼、原生社交登入、刪除帳號</t>
+          <t>韌體簽章、Secure Boot 與 Flash 加密</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr">
         <is>
-          <t>等 R-26</t>
+          <t>等 R-01</t>
         </is>
       </c>
       <c r="D70" s="11" t="n"/>
@@ -2534,17 +2534,17 @@
     <row r="71" ht="18" customHeight="1">
       <c r="A71" s="13" t="inlineStr">
         <is>
-          <t>P0-14</t>
+          <t>P1-06</t>
         </is>
       </c>
       <c r="B71" s="6" t="inlineStr">
         <is>
-          <t>韌體簽章、Secure Boot 與 Flash 加密</t>
+          <t>處理 GPL-3.0 依賴（arduino-audio-tools）</t>
         </is>
       </c>
       <c r="C71" s="6" t="inlineStr">
         <is>
-          <t>等 R-01</t>
+          <t>等 Q3</t>
         </is>
       </c>
       <c r="D71" s="11" t="n"/>
@@ -2557,12 +2557,12 @@
     <row r="72" ht="18" customHeight="1">
       <c r="A72" s="13" t="inlineStr">
         <is>
-          <t>P1-06</t>
+          <t>P1-07</t>
         </is>
       </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>處理 GPL-3.0 依賴（arduino-audio-tools）</t>
+          <t>LGPL 合規與第三方授權聲明</t>
         </is>
       </c>
       <c r="C72" s="6" t="inlineStr">
@@ -2580,17 +2580,17 @@
     <row r="73" ht="18" customHeight="1">
       <c r="A73" s="13" t="inlineStr">
         <is>
-          <t>P1-07</t>
+          <t>P1-08</t>
         </is>
       </c>
       <c r="B73" s="6" t="inlineStr">
         <is>
-          <t>LGPL 合規與第三方授權聲明</t>
+          <t>硬件認證</t>
         </is>
       </c>
       <c r="C73" s="6" t="inlineStr">
         <is>
-          <t>等 Q3</t>
+          <t>等 R-01、R-05</t>
         </is>
       </c>
       <c r="D73" s="11" t="n"/>
@@ -2603,17 +2603,17 @@
     <row r="74" ht="18" customHeight="1">
       <c r="A74" s="13" t="inlineStr">
         <is>
-          <t>P1-08</t>
+          <t>P1-14</t>
         </is>
       </c>
       <c r="B74" s="6" t="inlineStr">
         <is>
-          <t>硬件認證</t>
+          <t>Admin 內容安全頁：審核事件只按類別統計</t>
         </is>
       </c>
       <c r="C74" s="6" t="inlineStr">
         <is>
-          <t>等 R-01、R-05</t>
+          <t>等 P1-01、P2-13</t>
         </is>
       </c>
       <c r="D74" s="11" t="n"/>
@@ -2623,20 +2623,20 @@
       <c r="H74" s="11" t="n"/>
       <c r="I74" s="12" t="n"/>
     </row>
-    <row r="75" ht="18" customHeight="1">
+    <row r="75" ht="32" customHeight="1">
       <c r="A75" s="13" t="inlineStr">
         <is>
-          <t>P1-14</t>
+          <t>P2-15</t>
         </is>
       </c>
       <c r="B75" s="6" t="inlineStr">
         <is>
-          <t>Admin 內容安全頁：審核事件只按類別統計</t>
+          <t>Admin 總覽頁：在線、用量、成本與待處理事項</t>
         </is>
       </c>
       <c r="C75" s="6" t="inlineStr">
         <is>
-          <t>等 P1-01、P2-13</t>
+          <t>等 P2-14、P2-09</t>
         </is>
       </c>
       <c r="D75" s="11" t="n"/>
@@ -2646,20 +2646,20 @@
       <c r="H75" s="11" t="n"/>
       <c r="I75" s="12" t="n"/>
     </row>
-    <row r="76" ht="32" customHeight="1">
+    <row r="76" ht="18" customHeight="1">
       <c r="A76" s="13" t="inlineStr">
         <is>
-          <t>P2-15</t>
+          <t>R-07</t>
         </is>
       </c>
       <c r="B76" s="6" t="inlineStr">
         <is>
-          <t>Admin 總覽頁：在線、用量、成本與待處理事項</t>
+          <t>20 個家庭封閉內測</t>
         </is>
       </c>
       <c r="C76" s="6" t="inlineStr">
         <is>
-          <t>等 P2-14、P2-09</t>
+          <t>等 R-13</t>
         </is>
       </c>
       <c r="D76" s="11" t="n"/>
@@ -2672,17 +2672,17 @@
     <row r="77" ht="18" customHeight="1">
       <c r="A77" s="13" t="inlineStr">
         <is>
-          <t>R-07</t>
+          <t>R-08</t>
         </is>
       </c>
       <c r="B77" s="6" t="inlineStr">
         <is>
-          <t>20 個家庭封閉內測</t>
+          <t>第 8 週關卡決策</t>
         </is>
       </c>
       <c r="C77" s="6" t="inlineStr">
         <is>
-          <t>等 R-13</t>
+          <t>等 R-07、P2-09、P1-08</t>
         </is>
       </c>
       <c r="D77" s="11" t="n"/>
@@ -2695,17 +2695,17 @@
     <row r="78" ht="18" customHeight="1">
       <c r="A78" s="13" t="inlineStr">
         <is>
-          <t>R-08</t>
+          <t>R-14</t>
         </is>
       </c>
       <c r="B78" s="6" t="inlineStr">
         <is>
-          <t>第 8 週關卡決策</t>
+          <t>離線兒歌與故事</t>
         </is>
       </c>
       <c r="C78" s="6" t="inlineStr">
         <is>
-          <t>等 R-07、P2-09、P1-08</t>
+          <t>等 R-01</t>
         </is>
       </c>
       <c r="D78" s="11" t="n"/>
@@ -2718,17 +2718,17 @@
     <row r="79" ht="18" customHeight="1">
       <c r="A79" s="13" t="inlineStr">
         <is>
-          <t>R-14</t>
+          <t>R-24</t>
         </is>
       </c>
       <c r="B79" s="6" t="inlineStr">
         <is>
-          <t>離線兒歌與故事</t>
+          <t>設備只能用自己品牌的角色</t>
         </is>
       </c>
       <c r="C79" s="6" t="inlineStr">
         <is>
-          <t>等 R-01</t>
+          <t>等 R-34</t>
         </is>
       </c>
       <c r="D79" s="11" t="n"/>
@@ -2741,17 +2741,17 @@
     <row r="80" ht="18" customHeight="1">
       <c r="A80" s="13" t="inlineStr">
         <is>
-          <t>R-24</t>
+          <t>R-28</t>
         </is>
       </c>
       <c r="B80" s="6" t="inlineStr">
         <is>
-          <t>設備只能用自己品牌的角色</t>
+          <t>三個 App 的殼：品牌版本與測試版</t>
         </is>
       </c>
       <c r="C80" s="6" t="inlineStr">
         <is>
-          <t>等 R-34</t>
+          <t>等 R-25、R-26</t>
         </is>
       </c>
       <c r="D80" s="11" t="n"/>
@@ -2764,17 +2764,17 @@
     <row r="81" ht="18" customHeight="1">
       <c r="A81" s="13" t="inlineStr">
         <is>
-          <t>R-28</t>
+          <t>R-30</t>
         </is>
       </c>
       <c r="B81" s="6" t="inlineStr">
         <is>
-          <t>三個 App 的殼：品牌版本與測試版</t>
+          <t>快活 App（品牌 A）頁面</t>
         </is>
       </c>
       <c r="C81" s="6" t="inlineStr">
         <is>
-          <t>等 R-25、R-26</t>
+          <t>等 R-25、R-34、Q12</t>
         </is>
       </c>
       <c r="D81" s="11" t="n"/>
@@ -2787,17 +2787,17 @@
     <row r="82" ht="18" customHeight="1">
       <c r="A82" s="13" t="inlineStr">
         <is>
-          <t>R-30</t>
+          <t>R-31</t>
         </is>
       </c>
       <c r="B82" s="6" t="inlineStr">
         <is>
-          <t>快活 App（品牌 A）頁面</t>
+          <t>政協青年聯會版 App（品牌 B）頁面</t>
         </is>
       </c>
       <c r="C82" s="6" t="inlineStr">
         <is>
-          <t>等 R-25、R-34、Q12</t>
+          <t>等 R-25、R-34、Q13</t>
         </is>
       </c>
       <c r="D82" s="11" t="n"/>
@@ -2810,17 +2810,17 @@
     <row r="83" ht="18" customHeight="1">
       <c r="A83" s="13" t="inlineStr">
         <is>
-          <t>R-31</t>
+          <t>R-35</t>
         </is>
       </c>
       <c r="B83" s="6" t="inlineStr">
         <is>
-          <t>政協青年聯會版 App（品牌 B）頁面</t>
+          <t>韌體按品牌連線：伺服器網址在出廠時寫入</t>
         </is>
       </c>
       <c r="C83" s="6" t="inlineStr">
         <is>
-          <t>等 R-25、R-34、Q13</t>
+          <t>等 R-34</t>
         </is>
       </c>
       <c r="D83" s="11" t="n"/>
@@ -2830,20 +2830,20 @@
       <c r="H83" s="11" t="n"/>
       <c r="I83" s="12" t="n"/>
     </row>
-    <row r="84" ht="18" customHeight="1">
+    <row r="84" ht="32" customHeight="1">
       <c r="A84" s="13" t="inlineStr">
         <is>
-          <t>R-35</t>
+          <t>R-38</t>
         </is>
       </c>
       <c r="B84" s="6" t="inlineStr">
         <is>
-          <t>韌體按品牌連線：伺服器網址在出廠時寫入</t>
+          <t>公仔出廠鎖死所屬 IP，綁定時顯示該 IP 頭像</t>
         </is>
       </c>
       <c r="C84" s="6" t="inlineStr">
         <is>
-          <t>等 R-34</t>
+          <t>等 P0-11</t>
         </is>
       </c>
       <c r="D84" s="11" t="n"/>
@@ -2856,17 +2856,17 @@
     <row r="85" ht="32" customHeight="1">
       <c r="A85" s="13" t="inlineStr">
         <is>
-          <t>R-38</t>
+          <t>R-39</t>
         </is>
       </c>
       <c r="B85" s="6" t="inlineStr">
         <is>
-          <t>公仔出廠鎖死所屬 IP，綁定時顯示該 IP 頭像</t>
+          <t>Admin 出廠登記頁：匯入 MAC 清單、指定公仔、查看自檢結果</t>
         </is>
       </c>
       <c r="C85" s="6" t="inlineStr">
         <is>
-          <t>等 P0-11</t>
+          <t>等 R-38、P1-10</t>
         </is>
       </c>
       <c r="D85" s="11" t="n"/>
@@ -2876,20 +2876,20 @@
       <c r="H85" s="11" t="n"/>
       <c r="I85" s="12" t="n"/>
     </row>
-    <row r="86" ht="32" customHeight="1">
+    <row r="86" ht="18" customHeight="1">
       <c r="A86" s="13" t="inlineStr">
         <is>
-          <t>R-39</t>
+          <t>R-09</t>
         </is>
       </c>
       <c r="B86" s="6" t="inlineStr">
         <is>
-          <t>Admin 出廠登記頁：匯入 MAC 清單、指定公仔、查看自檢結果</t>
+          <t>量產外殼（真空複模）</t>
         </is>
       </c>
       <c r="C86" s="6" t="inlineStr">
         <is>
-          <t>等 R-38、P1-10</t>
+          <t>等 R-08、R-05、Q11</t>
         </is>
       </c>
       <c r="D86" s="11" t="n"/>
@@ -2902,17 +2902,17 @@
     <row r="87" ht="18" customHeight="1">
       <c r="A87" s="13" t="inlineStr">
         <is>
-          <t>R-09</t>
+          <t>R-10</t>
         </is>
       </c>
       <c r="B87" s="6" t="inlineStr">
         <is>
-          <t>量產外殼（真空複模）</t>
+          <t>出廠流程</t>
         </is>
       </c>
       <c r="C87" s="6" t="inlineStr">
         <is>
-          <t>等 R-08、R-05、Q11</t>
+          <t>等 P0-14、R-01、P2-12、R-34、R-35、R-38、R-39</t>
         </is>
       </c>
       <c r="D87" s="11" t="n"/>
@@ -2925,17 +2925,17 @@
     <row r="88" ht="18" customHeight="1">
       <c r="A88" s="13" t="inlineStr">
         <is>
-          <t>R-10</t>
+          <t>R-11</t>
         </is>
       </c>
       <c r="B88" s="6" t="inlineStr">
         <is>
-          <t>出廠流程</t>
+          <t>售後：客服、保修與換機</t>
         </is>
       </c>
       <c r="C88" s="6" t="inlineStr">
         <is>
-          <t>等 P0-14、R-01、P2-12、R-34、R-35、R-38、R-39</t>
+          <t>等 P2-14、R-40</t>
         </is>
       </c>
       <c r="D88" s="11" t="n"/>
@@ -2948,17 +2948,17 @@
     <row r="89" ht="18" customHeight="1">
       <c r="A89" s="13" t="inlineStr">
         <is>
-          <t>R-11</t>
+          <t>R-15</t>
         </is>
       </c>
       <c r="B89" s="6" t="inlineStr">
         <is>
-          <t>售後：客服、保修與換機</t>
+          <t>農曆新年前交付（生產 1/15、送達 1/29）</t>
         </is>
       </c>
       <c r="C89" s="6" t="inlineStr">
         <is>
-          <t>等 P2-14、R-40</t>
+          <t>等 R-09、R-10</t>
         </is>
       </c>
       <c r="D89" s="11" t="n"/>
@@ -2971,17 +2971,17 @@
     <row r="90" ht="18" customHeight="1">
       <c r="A90" s="13" t="inlineStr">
         <is>
-          <t>R-15</t>
+          <t>R-33</t>
         </is>
       </c>
       <c r="B90" s="6" t="inlineStr">
         <is>
-          <t>農曆新年前交付（生產 1/15、送達 1/29）</t>
+          <t>三個 App 送審並通過</t>
         </is>
       </c>
       <c r="C90" s="6" t="inlineStr">
         <is>
-          <t>等 R-09、R-10</t>
+          <t>等 R-27、R-21、R-28、R-29、R-30、R-31、R-32</t>
         </is>
       </c>
       <c r="D90" s="11" t="n"/>
@@ -2991,20 +2991,20 @@
       <c r="H90" s="11" t="n"/>
       <c r="I90" s="12" t="n"/>
     </row>
-    <row r="91" ht="18" customHeight="1">
+    <row r="91" ht="32" customHeight="1">
       <c r="A91" s="13" t="inlineStr">
         <is>
-          <t>R-33</t>
+          <t>R-40</t>
         </is>
       </c>
       <c r="B91" s="6" t="inlineStr">
         <is>
-          <t>三個 App 送審並通過</t>
+          <t>Admin 客服查詢頁：查帳號、名下設備與最近事件</t>
         </is>
       </c>
       <c r="C91" s="6" t="inlineStr">
         <is>
-          <t>等 R-27、R-21、R-28、R-29、R-30、R-31、R-32</t>
+          <t>等 P2-14、P1-10、P1-12</t>
         </is>
       </c>
       <c r="D91" s="11" t="n"/>
@@ -3014,50 +3014,50 @@
       <c r="H91" s="11" t="n"/>
       <c r="I91" s="12" t="n"/>
     </row>
-    <row r="92" ht="32" customHeight="1">
-      <c r="A92" s="13" t="inlineStr">
-        <is>
-          <t>R-40</t>
-        </is>
-      </c>
-      <c r="B92" s="6" t="inlineStr">
-        <is>
-          <t>Admin 客服查詢頁：查帳號、名下設備與最近事件</t>
-        </is>
-      </c>
-      <c r="C92" s="6" t="inlineStr">
-        <is>
-          <t>等 P2-14、P1-10、P1-12</t>
-        </is>
-      </c>
-      <c r="D92" s="11" t="n"/>
-      <c r="E92" s="11" t="n"/>
-      <c r="F92" s="11" t="n"/>
-      <c r="G92" s="11" t="n"/>
-      <c r="H92" s="11" t="n"/>
-      <c r="I92" s="12" t="n"/>
+    <row r="93">
+      <c r="A93" s="10" t="inlineStr">
+        <is>
+          <t>❓ 待確認問題</t>
+        </is>
+      </c>
     </row>
     <row r="94">
-      <c r="A94" s="10" t="inlineStr">
-        <is>
-          <t>❓ 待確認問題</t>
-        </is>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" s="4" t="inlineStr">
+      <c r="A94" s="4" t="inlineStr">
         <is>
           <t>編號</t>
         </is>
       </c>
-      <c r="B95" s="4" t="inlineStr">
+      <c r="B94" s="4" t="inlineStr">
         <is>
           <t>問題</t>
         </is>
       </c>
-      <c r="C95" s="4" t="inlineStr">
+      <c r="C94" s="4" t="inlineStr">
         <is>
           <t>影響的任務 / 為什麼重要</t>
+        </is>
+      </c>
+      <c r="D94" s="11" t="n"/>
+      <c r="E94" s="11" t="n"/>
+      <c r="F94" s="11" t="n"/>
+      <c r="G94" s="11" t="n"/>
+      <c r="H94" s="11" t="n"/>
+      <c r="I94" s="12" t="n"/>
+    </row>
+    <row r="95" ht="18" customHeight="1">
+      <c r="A95" s="13" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="B95" s="6" t="inlineStr">
+        <is>
+          <t>韌體打算閉源商業銷售嗎？</t>
+        </is>
+      </c>
+      <c r="C95" s="6" t="inlineStr">
+        <is>
+          <t>P1-06, P1-07：決定 GPL／LGPL 依賴要開源還是替換。</t>
         </is>
       </c>
       <c r="D95" s="11" t="n"/>
@@ -3067,20 +3067,20 @@
       <c r="H95" s="11" t="n"/>
       <c r="I95" s="12" t="n"/>
     </row>
-    <row r="96" ht="18" customHeight="1">
+    <row r="96" ht="32" customHeight="1">
       <c r="A96" s="13" t="inlineStr">
         <is>
-          <t>Q3</t>
+          <t>Q11</t>
         </is>
       </c>
       <c r="B96" s="6" t="inlineStr">
         <is>
-          <t>韌體打算閉源商業銷售嗎？</t>
+          <t>馬會快活的賽馬日版和新春版各多少隻（共 2,500）？</t>
         </is>
       </c>
       <c r="C96" s="6" t="inlineStr">
         <is>
-          <t>P1-06, P1-07：決定 GPL／LGPL 依賴要開源還是替換。</t>
+          <t>R-09, R-15：兩款的服裝和配件要分開訂料；11/20 前不知道，PP 樣和大貨單（11/27）會被拖慢。由馬會決定。</t>
         </is>
       </c>
       <c r="D96" s="11" t="n"/>
@@ -3090,20 +3090,20 @@
       <c r="H96" s="11" t="n"/>
       <c r="I96" s="12" t="n"/>
     </row>
-    <row r="97" ht="32" customHeight="1">
+    <row r="97" ht="60" customHeight="1">
       <c r="A97" s="13" t="inlineStr">
         <is>
-          <t>Q11</t>
+          <t>Q12</t>
         </is>
       </c>
       <c r="B97" s="6" t="inlineStr">
         <is>
-          <t>馬會快活的賽馬日版和新春版各多少隻（共 2,500）？</t>
+          <t>快活 App 的「會員綁定」是指甚麼：用我們自己的帳號（email 驗證碼），還是接馬會的會員帳號登入（SSO）？</t>
         </is>
       </c>
       <c r="C97" s="6" t="inlineStr">
         <is>
-          <t>R-09, R-15：兩款的服裝和配件要分開訂料；11/20 前不知道，PP 樣和大貨單（11/27）會被拖慢。由馬會決定。</t>
+          <t>P0-11, 快活 App（未入追蹤表）：接馬會 SSO 的話，登入、帳號刪除和資料歸屬都要按馬會的介面重做，工作量和排期要另估，而且 W5（11/9–11/13）就要做快活 App 的綁定；用我們的帳號則和其他品牌共用同一套流程。由馬會決定，要盡早問。</t>
         </is>
       </c>
       <c r="D97" s="11" t="n"/>
@@ -3113,20 +3113,20 @@
       <c r="H97" s="11" t="n"/>
       <c r="I97" s="12" t="n"/>
     </row>
-    <row r="98" ht="60" customHeight="1">
+    <row r="98" ht="46" customHeight="1">
       <c r="A98" s="13" t="inlineStr">
         <is>
-          <t>Q12</t>
+          <t>Q13</t>
         </is>
       </c>
       <c r="B98" s="6" t="inlineStr">
         <is>
-          <t>快活 App 的「會員綁定」是指甚麼：用我們自己的帳號（email 驗證碼），還是接馬會的會員帳號登入（SSO）？</t>
+          <t>政協青年聯會版的角色、語言和內容由誰提供？什麼時候交？</t>
         </is>
       </c>
       <c r="C98" s="6" t="inlineStr">
         <is>
-          <t>P0-11, 快活 App（未入追蹤表）：接馬會 SSO 的話，登入、帳號刪除和資料歸屬都要按馬會的介面重做，工作量和排期要另估，而且 W5（11/9–11/13）就要做快活 App 的綁定；用我們的帳號則和其他品牌共用同一套流程。由馬會決定，要盡早問。</t>
+          <t>品牌 B 的 App 頁面：品牌 B 的用戶是成人會員，但角色、說話語言、內容規則都還沒有。最遲 11/13 要拿到，才趕得及內部測試和 App 頁面（W6）。</t>
         </is>
       </c>
       <c r="D98" s="11" t="n"/>
@@ -3136,73 +3136,50 @@
       <c r="H98" s="11" t="n"/>
       <c r="I98" s="12" t="n"/>
     </row>
-    <row r="99" ht="46" customHeight="1">
-      <c r="A99" s="13" t="inlineStr">
-        <is>
-          <t>Q13</t>
-        </is>
-      </c>
-      <c r="B99" s="6" t="inlineStr">
-        <is>
-          <t>政協青年聯會版的角色、語言和內容由誰提供？什麼時候交？</t>
-        </is>
-      </c>
-      <c r="C99" s="6" t="inlineStr">
-        <is>
-          <t>品牌 B 的 App 頁面：品牌 B 的用戶是成人會員，但角色、說話語言、內容規則都還沒有。最遲 11/13 要拿到，才趕得及內部測試和 App 頁面（W6）。</t>
-        </is>
-      </c>
-      <c r="D99" s="11" t="n"/>
-      <c r="E99" s="11" t="n"/>
-      <c r="F99" s="11" t="n"/>
-      <c r="G99" s="11" t="n"/>
-      <c r="H99" s="11" t="n"/>
-      <c r="I99" s="12" t="n"/>
-    </row>
-    <row r="101">
-      <c r="A101" s="10" t="inlineStr">
+    <row r="100">
+      <c r="A100" s="10" t="inlineStr">
         <is>
           <t>說明</t>
         </is>
       </c>
     </row>
-    <row r="102" ht="32" customHeight="1">
+    <row r="101" ht="32" customHeight="1">
+      <c r="A101" s="14" t="inlineStr">
+        <is>
+          <t>・狀態：未開始 → 進行中 → 已完成。只有測試真的跑過而且通過才算已完成；阻塞要在備註寫原因；不再需要的任務標不適用，不要刪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="18" customHeight="1">
       <c r="A102" s="14" t="inlineStr">
         <is>
-          <t>・狀態：未開始 → 進行中 → 已完成。只有測試真的跑過而且通過才算已完成；阻塞要在備註寫原因；不再需要的任務標不適用，不要刪。</t>
+          <t>・測試結果：未測試 / 通過 / 失敗 / 部分通過。測試證據寫跑了什麼、看到什麼，完整歷史在「更新記錄」。</t>
         </is>
       </c>
     </row>
     <row r="103" ht="18" customHeight="1">
       <c r="A103" s="14" t="inlineStr">
         <is>
-          <t>・測試結果：未測試 / 通過 / 失敗 / 部分通過。測試證據寫跑了什麼、看到什麼，完整歷史在「更新記錄」。</t>
+          <t>・「接下來」按階段排序，同一階段內再按優先級；依賴還沒滿足的任務不會出現在「接下來」。</t>
         </is>
       </c>
     </row>
     <row r="104" ht="18" customHeight="1">
       <c r="A104" s="14" t="inlineStr">
         <is>
-          <t>・「接下來」按階段排序，同一階段內再按優先級；依賴還沒滿足的任務不會出現在「接下來」。</t>
-        </is>
-      </c>
-    </row>
-    <row r="105" ht="18" customHeight="1">
+          <t>・可以手動改：「任務清單」的狀態、測試結果、測試證據、Commit、備註，以及「待確認問題」的回答。其餘欄位和本頁由腳本維護。</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" ht="32" customHeight="1">
       <c r="A105" s="14" t="inlineStr">
         <is>
-          <t>・可以手動改：「任務清單」的狀態、測試結果、測試證據、Commit、備註，以及「待確認問題」的回答。其餘欄位和本頁由腳本維護。</t>
-        </is>
-      </c>
-    </row>
-    <row r="106" ht="32" customHeight="1">
-      <c r="A106" s="14" t="inlineStr">
-        <is>
           <t>・建議用法：在 Claude Code 對 Claude 說「P0-02 做完了」或輸入 /prod-readiness。Claude 會先跑測試再更新，並寫進「更新記錄」。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="87">
+  <mergeCells count="86">
     <mergeCell ref="C82:I82"/>
     <mergeCell ref="E52:I52"/>
     <mergeCell ref="E39:I39"/>
@@ -3213,7 +3190,6 @@
     <mergeCell ref="E29:I29"/>
     <mergeCell ref="E38:I38"/>
     <mergeCell ref="C83:I83"/>
-    <mergeCell ref="C92:I92"/>
     <mergeCell ref="E31:I31"/>
     <mergeCell ref="E40:I40"/>
     <mergeCell ref="C97:I97"/>
@@ -3235,12 +3211,15 @@
     <mergeCell ref="C77:I77"/>
     <mergeCell ref="C86:I86"/>
     <mergeCell ref="C68:I68"/>
+    <mergeCell ref="A100:I100"/>
     <mergeCell ref="C58:I58"/>
     <mergeCell ref="E30:I30"/>
     <mergeCell ref="E22:I22"/>
+    <mergeCell ref="A93:I93"/>
     <mergeCell ref="E46:I46"/>
     <mergeCell ref="A102:I102"/>
     <mergeCell ref="C85:I85"/>
+    <mergeCell ref="C94:I94"/>
     <mergeCell ref="C65:I65"/>
     <mergeCell ref="C75:I75"/>
     <mergeCell ref="C84:I84"/>
@@ -3249,7 +3228,6 @@
     <mergeCell ref="C59:I59"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="E41:I41"/>
-    <mergeCell ref="A94:I94"/>
     <mergeCell ref="E47:I47"/>
     <mergeCell ref="C61:I61"/>
     <mergeCell ref="C70:I70"/>
@@ -3259,11 +3237,9 @@
     <mergeCell ref="A55:I55"/>
     <mergeCell ref="A104:I104"/>
     <mergeCell ref="E35:I35"/>
-    <mergeCell ref="A106:I106"/>
     <mergeCell ref="C74:I74"/>
     <mergeCell ref="C88:I88"/>
     <mergeCell ref="E45:I45"/>
-    <mergeCell ref="C99:I99"/>
     <mergeCell ref="E37:I37"/>
     <mergeCell ref="E21:I21"/>
     <mergeCell ref="E23:I23"/>
@@ -10039,7 +10015,7 @@
         </is>
       </c>
     </row>
-    <row r="93" ht="102" customHeight="1">
+    <row r="93" ht="270" customHeight="1">
       <c r="A93" s="13" t="inlineStr">
         <is>
           <t>P2-20</t>
@@ -10067,12 +10043,17 @@
       </c>
       <c r="F93" s="13" t="inlineStr">
         <is>
-          <t>未開始</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="G93" s="13" t="inlineStr">
         <is>
-          <t>未測試</t>
+          <t>通過</t>
+        </is>
+      </c>
+      <c r="H93" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="I93" s="6" t="inlineStr">
@@ -10100,10 +10081,21 @@
           <t>P2-17, P1-10</t>
         </is>
       </c>
+      <c r="N93" s="6" t="inlineStr">
+        <is>
+          <t>node --test lib/firmwareImage.test.mjs 8/8（合成映像：dev build、無標記、未知板、晶片不符、非映像、截斷/損壞、超 4MB 拒；超 2MB 只警告）。分支 dev server + 本機 Supabase 端到端 16/16（GoTrue 真實登入的 cookie）：超管上傳 9.9.0 release build → 201 草稿（is_current f、rollout 0%），DB SHA-256 = 檔案、storage 原樣；審計 insert 記該超管；設備仍只拿到 current 1.6.2；已有 1.0.2 → 409；localall → 422 dev build；4MB+16 → 422；9MB → 413；PNG → 422；舊 1.6.1 映像（無標記）→ 422 指向 release_firmware.py；內容管理員上傳/刪除 → 403；未登入 → 401；刪 current → 409；超管刪草稿 → 行和映像都刪、審計 delete 記該超管。release_firmware.py list 照常。測試帳號與數據已清除</t>
+        </is>
+      </c>
+      <c r="O93" s="13" t="inlineStr">
+        <is>
+          <t>ebe8dc9</t>
+        </is>
+      </c>
       <c r="P93" s="6" t="inlineStr">
         <is>
           <t>[2026-10-14] 新增
-[2026-10-14] 2026-10-14 用戶決定提前到第 2 階段，現在開始做</t>
+[2026-10-14] 2026-10-14 用戶決定提前到第 2 階段，現在開始做
+[2026-10-14] 做法：韌體 OTA.cpp 加 BUILD_INFO 字串（kind=release/dev;board;version），伺服器從映像讀板型和版本，不用手填；DEV_MODE/LOCAL_WS_HOST/LOCAL_BACKEND_HOST/AUDIO_SELFTEST 為 dev。只有加了標記之後編譯的韌體能從後台上傳，之前的仍用 release_firmware.py。部署注意：① 網頁的 nginx location 很可能仍是預設 1MB 上限（/supabase-api/ 已改 16m），上傳 1.6MB 映像會 413，部署時要加 client_max_body_size 16m 並用 curl 驗證 ② 依賴 P1-10 的審計表（本機已有，線上隨 10-14 release 部署）</t>
         </is>
       </c>
     </row>
@@ -10757,7 +10749,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I294"/>
+  <dimension ref="A1:I296"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -20925,8 +20917,86 @@
         </is>
       </c>
     </row>
+    <row r="295" ht="32" customHeight="1">
+      <c r="A295" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 21:00</t>
+        </is>
+      </c>
+      <c r="B295" s="13" t="inlineStr">
+        <is>
+          <t>P2-20</t>
+        </is>
+      </c>
+      <c r="C295" s="6" t="inlineStr">
+        <is>
+          <t>P2-16 ④ 從後台上傳與發佈韌體（取代手貼 service key）</t>
+        </is>
+      </c>
+      <c r="D295" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E295" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F295" s="13" t="n"/>
+      <c r="G295" s="6" t="n"/>
+      <c r="H295" s="13" t="n"/>
+      <c r="I295" s="6" t="n"/>
+    </row>
+    <row r="296" ht="200" customHeight="1">
+      <c r="A296" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 21:10</t>
+        </is>
+      </c>
+      <c r="B296" s="13" t="inlineStr">
+        <is>
+          <t>P2-20</t>
+        </is>
+      </c>
+      <c r="C296" s="6" t="inlineStr">
+        <is>
+          <t>P2-16 ④ 從後台上傳與發佈韌體（取代手貼 service key）</t>
+        </is>
+      </c>
+      <c r="D296" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="E296" s="13" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="F296" s="13" t="inlineStr">
+        <is>
+          <t>通過</t>
+        </is>
+      </c>
+      <c r="G296" s="6" t="inlineStr">
+        <is>
+          <t>node --test lib/firmwareImage.test.mjs 8/8（合成映像：dev build、無標記、未知板、晶片不符、非映像、截斷/損壞、超 4MB 拒；超 2MB 只警告）。分支 dev server + 本機 Supabase 端到端 16/16（GoTrue 真實登入的 cookie）：超管上傳 9.9.0 release build → 201 草稿（is_current f、rollout 0%），DB SHA-256 = 檔案、storage 原樣；審計 insert 記該超管；設備仍只拿到 current 1.6.2；已有 1.0.2 → 409；localall → 422 dev build；4MB+16 → 422；9MB → 413；PNG → 422；舊 1.6.1 映像（無標記）→ 422 指向 release_firmware.py；內容管理員上傳/刪除 → 403；未登入 → 401；刪 current → 409；超管刪草稿 → 行和映像都刪、審計 delete 記該超管。release_firmware.py list 照常。測試帳號與數據已清除</t>
+        </is>
+      </c>
+      <c r="H296" s="13" t="inlineStr">
+        <is>
+          <t>ebe8dc9</t>
+        </is>
+      </c>
+      <c r="I296" s="6" t="inlineStr">
+        <is>
+          <t>做法：韌體 OTA.cpp 加 BUILD_INFO 字串（kind=release/dev;board;version），伺服器從映像讀板型和版本，不用手填；DEV_MODE/LOCAL_WS_HOST/LOCAL_BACKEND_HOST/AUDIO_SELFTEST 為 dev。只有加了標記之後編譯的韌體能從後台上傳，之前的仍用 release_firmware.py。部署注意：① 網頁的 nginx location 很可能仍是預設 1MB 上限（/supabase-api/ 已改 16m），上傳 1.6MB 映像會 413，部署時要加 client_max_body_size 16m 並用 curl 驗證 ② 依賴 P1-10 的審計表（本機已有，線上隨 10-14 release 部署）</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I294"/>
+  <autoFilter ref="A1:I296"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Track P2-21 (admin OTA page) and P2-16 as partly passed: the dev-board run is left.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/production-readiness.xlsx
+++ b/docs/production-readiness.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'任務清單'!$A$1:$P$94</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'待確認問題'!$A$1:$G$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$296</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$299</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -665,7 +665,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>最後更新：2026-10-14 21:10　·　本頁由 tracker.py 自動生成，請勿手動編輯</t>
+          <t>最後更新：2026-10-14 21:59　·　本頁由 tracker.py 自動生成，請勿手動編輯</t>
         </is>
       </c>
     </row>
@@ -820,11 +820,11 @@
       </c>
       <c r="D8" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A8,'任務清單'!$F:$F,D$5)</f>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E8" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A8,'任務清單'!$F:$F,E$5)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F8" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A8,'任務清單'!$F:$F,F$5)</f>
@@ -896,11 +896,11 @@
       </c>
       <c r="D10" s="5">
         <f>SUM(D6:D9)</f>
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E10" s="5">
         <f>SUM(E6:E9)</f>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F10" s="5">
         <f>SUM(F6:F9)</f>
@@ -1023,11 +1023,11 @@
       </c>
       <c r="D14" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A14,'任務清單'!$F:$F,D$12)</f>
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E14" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A14,'任務清單'!$F:$F,E$12)</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F14" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A14,'任務清單'!$F:$F,F$12)</f>
@@ -1139,11 +1139,11 @@
       </c>
       <c r="D17" s="5">
         <f>SUM(D13:D16)</f>
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E17" s="5">
         <f>SUM(E13:E16)</f>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F17" s="5">
         <f>SUM(F13:F16)</f>
@@ -1550,7 +1550,7 @@
       <c r="H31" s="11" t="n"/>
       <c r="I31" s="12" t="n"/>
     </row>
-    <row r="32" ht="102" customHeight="1">
+    <row r="32" ht="214" customHeight="1">
       <c r="A32" s="13" t="inlineStr">
         <is>
           <t>P2-16</t>
@@ -1573,7 +1573,8 @@
       </c>
       <c r="E32" s="6" t="inlineStr">
         <is>
-          <t>後台可上傳韌體（伺服器算 SHA-256、寫 firmware_releases）、填說明、設為 current；推送分階段：白名單 MAC → 10% → 50% → 100%，按 MAC 雜湊穩定分組；回滾率超過 5% 即自動暫停（2026-10-14 拿走「同一台重啟 3 次」，見 P2-19）；顯示每個版本已更新、回滾台數與回滾設備清單；顯示 app 分區用量（P2-12）；每個發佈操作寫入審計記錄。</t>
+          <t>上次測試：部分通過 — 子任務 P2-17～P2-20 通過、P2-21 部分通過（等 P2-14）。① 10% 階段只有雜湊預測的那組拿到、重複不變（P2-18、P2-21）② 2 台回滾 → 自動暫停、其餘不再拿到（P2-19、P2-21）③ 100% 全部拿到 ⑤ 審計表有每次階段變更（P2-21 9 筆）。未做：④ 開發板 62:70 實機走一次白名單階段（用戶目前手上沒有板子），同時驗證新韌體開機印出 BUILD_INFO
+後台可上傳韌體（伺服器算 SHA-256、寫 firmware_releases）、填說明、設為 current；推送分階段：白名單 MAC → 10% → 50% → 100%，按 MAC 雜湊穩定分組；回滾率超過 5% 即自動暫停（2026-10-14 拿走「同一台重啟 3 次」，見 P2-19）；顯示每個版本已更新、回滾台數與回滾設備清單；顯示 app 分區用量（P2-12）；每個發佈操作寫入審計記錄。</t>
         </is>
       </c>
       <c r="F32" s="11" t="n"/>
@@ -1581,15 +1582,15 @@
       <c r="H32" s="11" t="n"/>
       <c r="I32" s="12" t="n"/>
     </row>
-    <row r="33" ht="200" customHeight="1">
+    <row r="33" ht="382" customHeight="1">
       <c r="A33" s="13" t="inlineStr">
         <is>
-          <t>R-21</t>
+          <t>P2-21</t>
         </is>
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>藍牙配網與綁定（取代熱點配網）</t>
+          <t>P2-16 ⑤ 後台 OTA 頁換成真實數據與操作</t>
         </is>
       </c>
       <c r="C33" s="13" t="inlineStr">
@@ -1604,7 +1605,8 @@
       </c>
       <c r="E33" s="6" t="inlineStr">
         <is>
-          <t>① 設備在「未配網、Wi-Fi 連不上、未綁定、長按 BOOT」時以 AIBuddy-XXXX 名稱廣播藍牙，廣播資料帶品牌，品牌 App 只列出自己品牌的設備。② 設備經藍牙回傳它掃描到的 2.4GHz Wi-Fi 清單，App 讓用戶選擇並填密碼。③ App 經藍牙把 SSID、密碼和綁定票（P0-11）一起交給設備；藍牙通道加密（ESP 標準配網協定 security 1/2 或同等）。④ 設備連上 Wi-Fi 後自己完成認領，App 顯示綁定成功或失敗原因（密碼錯、設備已有主人、票過期）。⑤ 配網期間不啟動音訊；完成後釋放藍牙記憶體再開語音（必要時重開機），對話中最低 heap 不比現在差。⑥ 解綁在 App 內完成（P1-12），解綁後設備進入藍牙待綁定狀態。⑦ SoftAP 熱點配網保留給開發和運維（隱藏觸發方式或編譯開關），量產用戶流程不出現。</t>
+          <t>上次測試：部分通過 — 本機（分支 dev server 3216 + 本機 Supabase，GoTrue 真實登入的超管 cookie），用 xmini-c3 板型 + 20 台模擬設備以免碰到真開發板：頁面上傳 9.9.0 → 草稿；白名單加 1 台（UI 選單）→ 存檔；設為 current → 頁面預測 1 台、模擬 1 台；推進 10% → 預測 4、實得 4（重複不變）；50% → 預測 9、實得 9 且包含 10% 全部；100% → 20/20。2 台回滾 → 頁面顯示 'Paused … by the server: Auto-paused: 2 of 20 boards rolled back (10%)' 與回滾清單 2 台；點回滾設備 → 設備頁已帶 MAC 搜尋；恢復 → 其餘 18 台再拿到、回滾的 2 台不再下發；手動暫停未填原因不能確認、填後顯示 'by an admin'。審計頁 9 筆（上傳、白名單、current、10/50/100%、系統暫停、恢復、手動暫停），系統暫停顯示 System。375px scrollWidth=375。內容管理員側欄只有 Characters/IPs、#ota 退回 Characters、頁面無 OTA 數據，直接呼叫 admin_change_firmware_rollout → 403/42501。測試中發現並修正：舊版本（含 63:64 仍在跑的 1.6.1）被當成可刪除的草稿（6c2dc9d）。測試數據已清除
+按板型列出版本：狀態（草稿／推送中＋階段／暫停＋原因／現行／舊版）、已更新／目標台數、回滾台數、大小、發佈時間、說明；單一版本可編輯白名單、推進下一階段、暫停／恢復、撤下；回滾設備清單可點進設備頁；顯示 app 分區用量（P2-12）；每個操作要確認並寫審計記錄；只有超級管理員可見；375px 無橫向捲動。</t>
         </is>
       </c>
       <c r="F33" s="11" t="n"/>
@@ -1612,15 +1614,15 @@
       <c r="H33" s="11" t="n"/>
       <c r="I33" s="12" t="n"/>
     </row>
-    <row r="34" ht="116" customHeight="1">
+    <row r="34" ht="200" customHeight="1">
       <c r="A34" s="13" t="inlineStr">
         <is>
-          <t>R-36</t>
+          <t>R-21</t>
         </is>
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>未認領的設備停在配對狀態，不再每秒重連 websocket</t>
+          <t>藍牙配網與綁定（取代熱點配網）</t>
         </is>
       </c>
       <c r="C34" s="13" t="inlineStr">
@@ -1635,7 +1637,7 @@
       </c>
       <c r="E34" s="6" t="inlineStr">
         <is>
-          <t>① 拿到 202 或 websocket 被 4401 拒絕後，設備停掉 websocket 自動重連，進入待綁定狀態（燈號可分辨）。② 待綁定時只按退避（5 秒起、上限 PROVISION_BACKOFF_MAX）呼叫 generate_auth_token，不開 websocket。③ 被認領後下一次輪詢拿到 200，在 10 秒內（加退避）自動開 websocket 並能對話，不用重開機。④ 已綁定設備網絡斷線重連的行為不變。⑤ 隨 OTA 推出。</t>
+          <t>① 設備在「未配網、Wi-Fi 連不上、未綁定、長按 BOOT」時以 AIBuddy-XXXX 名稱廣播藍牙，廣播資料帶品牌，品牌 App 只列出自己品牌的設備。② 設備經藍牙回傳它掃描到的 2.4GHz Wi-Fi 清單，App 讓用戶選擇並填密碼。③ App 經藍牙把 SSID、密碼和綁定票（P0-11）一起交給設備；藍牙通道加密（ESP 標準配網協定 security 1/2 或同等）。④ 設備連上 Wi-Fi 後自己完成認領，App 顯示綁定成功或失敗原因（密碼錯、設備已有主人、票過期）。⑤ 配網期間不啟動音訊；完成後釋放藍牙記憶體再開語音（必要時重開機），對話中最低 heap 不比現在差。⑥ 解綁在 App 內完成（P1-12），解綁後設備進入藍牙待綁定狀態。⑦ SoftAP 熱點配網保留給開發和運維（隱藏觸發方式或編譯開關），量產用戶流程不出現。</t>
         </is>
       </c>
       <c r="F34" s="11" t="n"/>
@@ -1643,20 +1645,20 @@
       <c r="H34" s="11" t="n"/>
       <c r="I34" s="12" t="n"/>
     </row>
-    <row r="35" ht="228" customHeight="1">
+    <row r="35" ht="116" customHeight="1">
       <c r="A35" s="13" t="inlineStr">
         <is>
-          <t>P2-12</t>
+          <t>R-36</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>量產燒錄前加大 app 分區</t>
+          <t>未認領的設備停在配對狀態，不再每秒重連 websocket</t>
         </is>
       </c>
       <c r="C35" s="13" t="inlineStr">
         <is>
-          <t>3 封閉內測</t>
+          <t>2 內測準備</t>
         </is>
       </c>
       <c r="D35" s="13" t="inlineStr">
@@ -1666,8 +1668,7 @@
       </c>
       <c r="E35" s="6" t="inlineStr">
         <is>
-          <t>上次測試：部分通過 — 62:70（spotpear-ai-toy-p212 原型，現已併入 spotpear-ai-toy）：① 本機 OTA 1.6.1→1.6.2 寫入新 app1，120s 後 confirmed ② 3 秒 abort 的 1.6.3 → PANIC → 回到 1.6.2，ota_failed_version=1.6.3 ③ 崩潰寫入 coredump 14.8KB ④ 資源分區 9 個聲音 504KB/2MB，開機 CRC 63ms，OTA 後照常；損壞/清空 → 退回內建聲音無崩潰 ⑤ pio 全部 18 個 env 編譯通過，映像都在各自 app 槽內（Spotpear 4 個 1.59–1.60MB / 4MB；其他板仍 2MB 槽）；R-21 藍牙探針版 2,326,128 bytes &lt; 4MB ⑥ release_firmware.py 映像 &gt; app 槽即拒發。未做：雲端 OTA 一次（等上 UAT）、出廠腳本寫入資源包（R-10）
-新分區表（例如 app0/app1 各 4MB，保留 nvs/otadata 位置）在出廠前定案並寫入出廠腳本；OTA 與回滾在新分區表上照常</t>
+          <t>① 拿到 202 或 websocket 被 4401 拒絕後，設備停掉 websocket 自動重連，進入待綁定狀態（燈號可分辨）。② 待綁定時只按退避（5 秒起、上限 PROVISION_BACKOFF_MAX）呼叫 generate_auth_token，不開 websocket。③ 被認領後下一次輪詢拿到 200，在 10 秒內（加退避）自動開 websocket 並能對話，不用重開機。④ 已綁定設備網絡斷線重連的行為不變。⑤ 隨 OTA 推出。</t>
         </is>
       </c>
       <c r="F35" s="11" t="n"/>
@@ -1675,15 +1676,15 @@
       <c r="H35" s="11" t="n"/>
       <c r="I35" s="12" t="n"/>
     </row>
-    <row r="36" ht="242" customHeight="1">
+    <row r="36" ht="228" customHeight="1">
       <c r="A36" s="13" t="inlineStr">
         <is>
-          <t>R-37</t>
+          <t>P2-12</t>
         </is>
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>網頁設定玩具的 Wi-Fi：查看、新增、刪除</t>
+          <t>量產燒錄前加大 app 分區</t>
         </is>
       </c>
       <c r="C36" s="13" t="inlineStr">
@@ -1698,8 +1699,8 @@
       </c>
       <c r="E36" s="6" t="inlineStr">
         <is>
-          <t>上次測試：部分通過 — 模擬玩具經本機語音服務器＋網頁：status/scan/add/delete 正常；刪除目前 Wi-Fi → current 被拒；斷線 5 秒內頁面顯示睡著、按鈕停用；測試密碼在語音服務器日誌、網頁服務器日誌、資料庫均搜不到；用別人裝置 ID 重放 server action → forbidden；pytest 17 項通過（全套 230）；韌體 spotpear-ai-toy-localall 編譯通過（RAM 17.5%、Flash 75.9%）。未測：真機 ①② 及 OTA 推出
-① 設定頁顯示玩具在線／離線、目前 Wi-Fi 和訊號、已記住的 Wi-Fi 清單（只有名稱，不顯示密碼）② 在線時可新增 Wi-Fi（輸入或從玩具掃描到的清單選）、刪除 Wi-Fi；不能刪除正在使用的那個 ③ 經 /ws/esp32 轉送：伺服器先確認是設備主人；密碼不寫入資料庫、不寫入日誌 ④ 新增不切換網絡，目前 Wi-Fi 消失時才按訊號選；清單標示「連過／未連過」⑤ 上限 8 個 ⑥ 韌體改動經 OTA 推出</t>
+          <t>上次測試：部分通過 — 62:70（spotpear-ai-toy-p212 原型，現已併入 spotpear-ai-toy）：① 本機 OTA 1.6.1→1.6.2 寫入新 app1，120s 後 confirmed ② 3 秒 abort 的 1.6.3 → PANIC → 回到 1.6.2，ota_failed_version=1.6.3 ③ 崩潰寫入 coredump 14.8KB ④ 資源分區 9 個聲音 504KB/2MB，開機 CRC 63ms，OTA 後照常；損壞/清空 → 退回內建聲音無崩潰 ⑤ pio 全部 18 個 env 編譯通過，映像都在各自 app 槽內（Spotpear 4 個 1.59–1.60MB / 4MB；其他板仍 2MB 槽）；R-21 藍牙探針版 2,326,128 bytes &lt; 4MB ⑥ release_firmware.py 映像 &gt; app 槽即拒發。未做：雲端 OTA 一次（等上 UAT）、出廠腳本寫入資源包（R-10）
+新分區表（例如 app0/app1 各 4MB，保留 nvs/otadata 位置）在出廠前定案並寫入出廠腳本；OTA 與回滾在新分區表上照常</t>
         </is>
       </c>
       <c r="F36" s="11" t="n"/>
@@ -1707,30 +1708,31 @@
       <c r="H36" s="11" t="n"/>
       <c r="I36" s="12" t="n"/>
     </row>
-    <row r="37" ht="102" customHeight="1">
+    <row r="37" ht="242" customHeight="1">
       <c r="A37" s="13" t="inlineStr">
         <is>
-          <t>R-16</t>
+          <t>R-37</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>Spotpear 量產版加電池電壓檢測（GPIO0 分壓）</t>
+          <t>網頁設定玩具的 Wi-Fi：查看、新增、刪除</t>
         </is>
       </c>
       <c r="C37" s="13" t="inlineStr">
         <is>
-          <t>1 止血定案</t>
+          <t>3 封閉內測</t>
         </is>
       </c>
       <c r="D37" s="13" t="inlineStr">
         <is>
-          <t>未開始</t>
+          <t>進行中</t>
         </is>
       </c>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>Spotpear 書面確認量產版：GPIO1（屏幕 DC；本版不接屏幕，可空出來）接電芯正極（保護 IC 之後）100k/100k 分壓、100nF 濾波，屏幕不接該腳；GPIO0 保留給現有的 VDD 低電提醒；最好另把充電芯片 CHRG 接到 GPIO12 或 13。樣板到手後，固件讀到的電芯電壓與萬用表相差 ≤50mV，App（R-41）顯示百分比與充電中。</t>
+          <t>上次測試：部分通過 — 模擬玩具經本機語音服務器＋網頁：status/scan/add/delete 正常；刪除目前 Wi-Fi → current 被拒；斷線 5 秒內頁面顯示睡著、按鈕停用；測試密碼在語音服務器日誌、網頁服務器日誌、資料庫均搜不到；用別人裝置 ID 重放 server action → forbidden；pytest 17 項通過（全套 230）；韌體 spotpear-ai-toy-localall 編譯通過（RAM 17.5%、Flash 75.9%）。未測：真機 ①② 及 OTA 推出
+① 設定頁顯示玩具在線／離線、目前 Wi-Fi 和訊號、已記住的 Wi-Fi 清單（只有名稱，不顯示密碼）② 在線時可新增 Wi-Fi（輸入或從玩具掃描到的清單選）、刪除 Wi-Fi；不能刪除正在使用的那個 ③ 經 /ws/esp32 轉送：伺服器先確認是設備主人；密碼不寫入資料庫、不寫入日誌 ④ 新增不切換網絡，目前 Wi-Fi 消失時才按訊號選；清單標示「連過／未連過」⑤ 上限 8 個 ⑥ 韌體改動經 OTA 推出</t>
         </is>
       </c>
       <c r="F37" s="11" t="n"/>
@@ -1738,20 +1740,20 @@
       <c r="H37" s="11" t="n"/>
       <c r="I37" s="12" t="n"/>
     </row>
-    <row r="38" ht="46" customHeight="1">
+    <row r="38" ht="102" customHeight="1">
       <c r="A38" s="13" t="inlineStr">
         <is>
-          <t>P1-11</t>
+          <t>R-16</t>
         </is>
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>伺服器與資料庫直接存取的管控</t>
+          <t>Spotpear 量產版加電池電壓檢測（GPIO0 分壓）</t>
         </is>
       </c>
       <c r="C38" s="13" t="inlineStr">
         <is>
-          <t>2 內測準備</t>
+          <t>1 止血定案</t>
         </is>
       </c>
       <c r="D38" s="13" t="inlineStr">
@@ -1761,7 +1763,7 @@
       </c>
       <c r="E38" s="6" t="inlineStr">
         <is>
-          <t>列出誰有 SSH 與資料庫直連權限（越少越好）；service_role key 只存在伺服器的 env；私隱政策寫明這類存取的範圍；每次直接查看生產資料都留記錄。</t>
+          <t>Spotpear 書面確認量產版：GPIO1（屏幕 DC；本版不接屏幕，可空出來）接電芯正極（保護 IC 之後）100k/100k 分壓、100nF 濾波，屏幕不接該腳；GPIO0 保留給現有的 VDD 低電提醒；最好另把充電芯片 CHRG 接到 GPIO12 或 13。樣板到手後，固件讀到的電芯電壓與萬用表相差 ≤50mV，App（R-41）顯示百分比與充電中。</t>
         </is>
       </c>
       <c r="F38" s="11" t="n"/>
@@ -1772,12 +1774,12 @@
     <row r="39" ht="46" customHeight="1">
       <c r="A39" s="13" t="inlineStr">
         <is>
-          <t>P2-02</t>
+          <t>P1-11</t>
         </is>
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>CI 跑測試與靜態檢查</t>
+          <t>伺服器與資料庫直接存取的管控</t>
         </is>
       </c>
       <c r="C39" s="13" t="inlineStr">
@@ -1792,7 +1794,7 @@
       </c>
       <c r="E39" s="6" t="inlineStr">
         <is>
-          <t>推送與 PR 時跑 pytest、ruff、pyright、next lint、tsc --noEmit、pio run；任何一項失敗就不發佈 image。</t>
+          <t>列出誰有 SSH 與資料庫直連權限（越少越好）；service_role key 只存在伺服器的 env；私隱政策寫明這類存取的範圍；每次直接查看生產資料都留記錄。</t>
         </is>
       </c>
       <c r="F39" s="11" t="n"/>
@@ -1800,15 +1802,15 @@
       <c r="H39" s="11" t="n"/>
       <c r="I39" s="12" t="n"/>
     </row>
-    <row r="40" ht="32" customHeight="1">
+    <row r="40" ht="46" customHeight="1">
       <c r="A40" s="13" t="inlineStr">
         <is>
-          <t>P2-04</t>
+          <t>P2-02</t>
         </is>
       </c>
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>容器改用非 root 用戶</t>
+          <t>CI 跑測試與靜態檢查</t>
         </is>
       </c>
       <c r="C40" s="13" t="inlineStr">
@@ -1823,7 +1825,7 @@
       </c>
       <c r="E40" s="6" t="inlineStr">
         <is>
-          <t>兩個 Dockerfile 都設定非 root 的 USER。</t>
+          <t>推送與 PR 時跑 pytest、ruff、pyright、next lint、tsc --noEmit、pio run；任何一項失敗就不發佈 image。</t>
         </is>
       </c>
       <c r="F40" s="11" t="n"/>
@@ -1831,15 +1833,15 @@
       <c r="H40" s="11" t="n"/>
       <c r="I40" s="12" t="n"/>
     </row>
-    <row r="41" ht="46" customHeight="1">
+    <row r="41" ht="32" customHeight="1">
       <c r="A41" s="13" t="inlineStr">
         <is>
-          <t>R-04</t>
+          <t>P2-04</t>
         </is>
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>粵語質量評測</t>
+          <t>容器改用非 root 用戶</t>
         </is>
       </c>
       <c r="C41" s="13" t="inlineStr">
@@ -1854,7 +1856,7 @@
       </c>
       <c r="E41" s="6" t="inlineStr">
         <is>
-          <t>有一套粵語評測集（兒童錄音＋文字提示）；選定的 STT 與 LLM 達到門檻：兒童語音字錯率 ≤15%、口語粵語回覆 ≥90%、中英夾雜句能正確理解。</t>
+          <t>兩個 Dockerfile 都設定非 root 的 USER。</t>
         </is>
       </c>
       <c r="F41" s="11" t="n"/>
@@ -1862,15 +1864,15 @@
       <c r="H41" s="11" t="n"/>
       <c r="I41" s="12" t="n"/>
     </row>
-    <row r="42" ht="116" customHeight="1">
+    <row r="42" ht="46" customHeight="1">
       <c r="A42" s="13" t="inlineStr">
         <is>
-          <t>R-25</t>
+          <t>R-04</t>
         </is>
       </c>
       <c r="B42" s="6" t="inlineStr">
         <is>
-          <t>網頁的品牌主題系統</t>
+          <t>粵語質量評測</t>
         </is>
       </c>
       <c r="C42" s="13" t="inlineStr">
@@ -1885,7 +1887,7 @@
       </c>
       <c r="E42" s="6" t="inlineStr">
         <is>
-          <t>① 每個品牌一個資料夾：主題 token（顏色、字體、圓角）、logo 和圖示、文案、功能開關；首頁、上手流程、角色頁可以有品牌版本，其餘頁面共用 ② 由部署的環境變數選品牌（每套部署一個品牌，見 R-34），伺服器端渲染的第一屏就是對的主題，不閃爍 ③ 共用元件裡沒有品牌名稱和寫死的品牌顏色 ④ 加一個品牌只需要加資料夾、設定和一套部署，不用改共用元件</t>
+          <t>有一套粵語評測集（兒童錄音＋文字提示）；選定的 STT 與 LLM 達到門檻：兒童語音字錯率 ≤15%、口語粵語回覆 ≥90%、中英夾雜句能正確理解。</t>
         </is>
       </c>
       <c r="F42" s="11" t="n"/>
@@ -1893,68 +1895,68 @@
       <c r="H42" s="11" t="n"/>
       <c r="I42" s="12" t="n"/>
     </row>
-    <row r="44">
-      <c r="A44" s="10" t="inlineStr">
+    <row r="43" ht="116" customHeight="1">
+      <c r="A43" s="13" t="inlineStr">
+        <is>
+          <t>R-25</t>
+        </is>
+      </c>
+      <c r="B43" s="6" t="inlineStr">
+        <is>
+          <t>網頁的品牌主題系統</t>
+        </is>
+      </c>
+      <c r="C43" s="13" t="inlineStr">
+        <is>
+          <t>2 內測準備</t>
+        </is>
+      </c>
+      <c r="D43" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E43" s="6" t="inlineStr">
+        <is>
+          <t>① 每個品牌一個資料夾：主題 token（顏色、字體、圓角）、logo 和圖示、文案、功能開關；首頁、上手流程、角色頁可以有品牌版本，其餘頁面共用 ② 由部署的環境變數選品牌（每套部署一個品牌，見 R-34），伺服器端渲染的第一屏就是對的主題，不閃爍 ③ 共用元件裡沒有品牌名稱和寫死的品牌顏色 ④ 加一個品牌只需要加資料夾、設定和一套部署，不用改共用元件</t>
+        </is>
+      </c>
+      <c r="F43" s="11" t="n"/>
+      <c r="G43" s="11" t="n"/>
+      <c r="H43" s="11" t="n"/>
+      <c r="I43" s="12" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="10" t="inlineStr">
         <is>
           <t>✅ 最近完成與測試效果</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="4" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
         <is>
           <t>編號</t>
         </is>
       </c>
-      <c r="B45" s="4" t="inlineStr">
+      <c r="B46" s="4" t="inlineStr">
         <is>
           <t>任務</t>
         </is>
       </c>
-      <c r="C45" s="4" t="inlineStr">
+      <c r="C46" s="4" t="inlineStr">
         <is>
           <t>測試結果</t>
         </is>
       </c>
-      <c r="D45" s="4" t="inlineStr">
+      <c r="D46" s="4" t="inlineStr">
         <is>
           <t>完成日期</t>
         </is>
       </c>
-      <c r="E45" s="4" t="inlineStr">
+      <c r="E46" s="4" t="inlineStr">
         <is>
           <t>測試證據</t>
-        </is>
-      </c>
-      <c r="F45" s="11" t="n"/>
-      <c r="G45" s="11" t="n"/>
-      <c r="H45" s="11" t="n"/>
-      <c r="I45" s="12" t="n"/>
-    </row>
-    <row r="46" ht="214" customHeight="1">
-      <c r="A46" s="13" t="inlineStr">
-        <is>
-          <t>P2-20</t>
-        </is>
-      </c>
-      <c r="B46" s="6" t="inlineStr">
-        <is>
-          <t>P2-16 ④ 從後台上傳與發佈韌體（取代手貼 service key）</t>
-        </is>
-      </c>
-      <c r="C46" s="13" t="inlineStr">
-        <is>
-          <t>通過</t>
-        </is>
-      </c>
-      <c r="D46" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="E46" s="6" t="inlineStr">
-        <is>
-          <t>node --test lib/firmwareImage.test.mjs 8/8（合成映像：dev build、無標記、未知板、晶片不符、非映像、截斷/損壞、超 4MB 拒；超 2MB 只警告）。分支 dev server + 本機 Supabase 端到端 16/16（GoTrue 真實登入的 cookie）：超管上傳 9.9.0 release build → 201 草稿（is_current f、rollout 0%），DB SHA-256 = 檔案、storage 原樣；審計 insert 記該超管；設備仍只拿到 current 1.6.2；已有 1.0.2 → 409；localall → 422 dev build；4MB+16 → 422；9MB → 413；PNG → 422；舊 1.6.1 映像（無標記）→ 422 指向 release_firmware.py；內容管理員上傳/刪除 → 403；未登入 → 401；刪 current → 409；超管刪草稿 → 行和映像都刪、審計 delete 記該超管。release_firmware.py list 照常。測試帳號與數據已清除</t>
         </is>
       </c>
       <c r="F46" s="11" t="n"/>
@@ -1962,15 +1964,15 @@
       <c r="H46" s="11" t="n"/>
       <c r="I46" s="12" t="n"/>
     </row>
-    <row r="47" ht="158" customHeight="1">
+    <row r="47" ht="214" customHeight="1">
       <c r="A47" s="13" t="inlineStr">
         <is>
-          <t>P2-19</t>
+          <t>P2-20</t>
         </is>
       </c>
       <c r="B47" s="6" t="inlineStr">
         <is>
-          <t>P2-16 ③ 回滾過多時自動暫停推送</t>
+          <t>P2-16 ④ 從後台上傳與發佈韌體（取代手貼 service key）</t>
         </is>
       </c>
       <c r="C47" s="13" t="inlineStr">
@@ -1985,7 +1987,7 @@
       </c>
       <c r="E47" s="6" t="inlineStr">
         <is>
-          <t>migration 20261014200000 BEGIN/ROLLBACK 套用兩次無錯並已套用本機。模擬 20 台連跑兩次 12/12：1/20 回滾不暫停、其餘 18 台照常；2/20 → 'Auto-paused: 2 of 20 boards rolled back (10%)'，其餘 0 台拿到 ota；已運行的設備記為 running 且不再下發；審計 1 筆 actor 空；恢復後 17 台拿到、保持恢復，第 3 台回滾 → 'Auto-paused: 3 of 20 (15%)'；白名單 2 台中 1 台回滾 → 50% 立即暫停、另一台不再下發；anon 呼叫 ota_maybe_pause → 401/42501。測試數據已清除，spotpear-ai-toy 1.6.2 仍 100% 未暫停</t>
+          <t>node --test lib/firmwareImage.test.mjs 8/8（合成映像：dev build、無標記、未知板、晶片不符、非映像、截斷/損壞、超 4MB 拒；超 2MB 只警告）。分支 dev server + 本機 Supabase 端到端 16/16（GoTrue 真實登入的 cookie）：超管上傳 9.9.0 release build → 201 草稿（is_current f、rollout 0%），DB SHA-256 = 檔案、storage 原樣；審計 insert 記該超管；設備仍只拿到 current 1.6.2；已有 1.0.2 → 409；localall → 422 dev build；4MB+16 → 422；9MB → 413；PNG → 422；舊 1.6.1 映像（無標記）→ 422 指向 release_firmware.py；內容管理員上傳/刪除 → 403；未登入 → 401；刪 current → 409；超管刪草稿 → 行和映像都刪、審計 delete 記該超管。release_firmware.py list 照常。測試帳號與數據已清除</t>
         </is>
       </c>
       <c r="F47" s="11" t="n"/>
@@ -1993,15 +1995,15 @@
       <c r="H47" s="11" t="n"/>
       <c r="I47" s="12" t="n"/>
     </row>
-    <row r="48" ht="200" customHeight="1">
+    <row r="48" ht="158" customHeight="1">
       <c r="A48" s="13" t="inlineStr">
         <is>
-          <t>P2-18</t>
+          <t>P2-19</t>
         </is>
       </c>
       <c r="B48" s="6" t="inlineStr">
         <is>
-          <t>P2-16 ② 按 MAC 雜湊穩定分組決定哪台收到 ota</t>
+          <t>P2-16 ③ 回滾過多時自動暫停推送</t>
         </is>
       </c>
       <c r="C48" s="13" t="inlineStr">
@@ -2016,7 +2018,7 @@
       </c>
       <c r="E48" s="6" t="inlineStr">
         <is>
-          <t>node --test lib/otaRollout.test.mjs 6/6：10,000 隨機 MAC 在 10%/50% 誤差 &lt; 1 個百分點、同 MAC（含大小寫/空白）結果一致、升階段只增不減、白名單各階段都在、不同版本選不同的 10%。tsc --noEmit 通過。分支 dev server（3216）+ 本機 Supabase 模擬 20 台（板型 p218-sim，連跑兩次 9/9）：白名單階段只有 1 台、重複不變；10% 拿到的正是雜湊預測的那組（2–5 台含白名單），重複不變；50% 包含 10% 全部；暫停 → 0 台且下載映像 404，恢復 → 200；100% → 除已更新和已回滾的 2 台外 18 台；每台下發次數與記錄一致；運行中/已回滾正確標記；審計 6 筆對應 6 次變更。真 spotpear-ai-toy（預設 100%）回報 1.6.1 → 仍拿到 1.6.2。測試數據已清除</t>
+          <t>migration 20261014200000 BEGIN/ROLLBACK 套用兩次無錯並已套用本機。模擬 20 台連跑兩次 12/12：1/20 回滾不暫停、其餘 18 台照常；2/20 → 'Auto-paused: 2 of 20 boards rolled back (10%)'，其餘 0 台拿到 ota；已運行的設備記為 running 且不再下發；審計 1 筆 actor 空；恢復後 17 台拿到、保持恢復，第 3 台回滾 → 'Auto-paused: 3 of 20 (15%)'；白名單 2 台中 1 台回滾 → 50% 立即暫停、另一台不再下發；anon 呼叫 ota_maybe_pause → 401/42501。測試數據已清除，spotpear-ai-toy 1.6.2 仍 100% 未暫停</t>
         </is>
       </c>
       <c r="F48" s="11" t="n"/>
@@ -2024,15 +2026,15 @@
       <c r="H48" s="11" t="n"/>
       <c r="I48" s="12" t="n"/>
     </row>
-    <row r="49" ht="172" customHeight="1">
+    <row r="49" ht="200" customHeight="1">
       <c r="A49" s="13" t="inlineStr">
         <is>
-          <t>P2-17</t>
+          <t>P2-18</t>
         </is>
       </c>
       <c r="B49" s="6" t="inlineStr">
         <is>
-          <t>P2-16 ① 分批推送的數據表：推送階段、白名單、每台安裝結果</t>
+          <t>P2-16 ② 按 MAC 雜湊穩定分組決定哪台收到 ota</t>
         </is>
       </c>
       <c r="C49" s="13" t="inlineStr">
@@ -2047,7 +2049,7 @@
       </c>
       <c r="E49" s="6" t="inlineStr">
         <is>
-          <t>migration 20261014190000 BEGIN/ROLLBACK 套用兩次無錯並已套用本機；行為：預設 100%、promote 記 stage_changed_at，7 種壞值（25%、小寫/空字串/NULL MAC、暫停缺原因等）全被 check 擋；ota_note_offer 1→2→3，report 正確標 running/failed、別板型不影響，刪發佈連帶刪記錄；審計 5 筆含 'test-board 9.9.9' 標籤。REST 13/13：超管可讀、內容管理員 0 行、anon 42501，三種身份寫入/改階段/呼叫 ota_note_offer 皆 42501。release_firmware.py promote spotpear-ai-toy 1.6.2 成功，token 查詢仍選 1.6.2，審計記 2 筆（actor 空＝service role）</t>
+          <t>node --test lib/otaRollout.test.mjs 6/6：10,000 隨機 MAC 在 10%/50% 誤差 &lt; 1 個百分點、同 MAC（含大小寫/空白）結果一致、升階段只增不減、白名單各階段都在、不同版本選不同的 10%。tsc --noEmit 通過。分支 dev server（3216）+ 本機 Supabase 模擬 20 台（板型 p218-sim，連跑兩次 9/9）：白名單階段只有 1 台、重複不變；10% 拿到的正是雜湊預測的那組（2–5 台含白名單），重複不變；50% 包含 10% 全部；暫停 → 0 台且下載映像 404，恢復 → 200；100% → 除已更新和已回滾的 2 台外 18 台；每台下發次數與記錄一致；運行中/已回滾正確標記；審計 6 筆對應 6 次變更。真 spotpear-ai-toy（預設 100%）回報 1.6.1 → 仍拿到 1.6.2。測試數據已清除</t>
         </is>
       </c>
       <c r="F49" s="11" t="n"/>
@@ -2055,15 +2057,15 @@
       <c r="H49" s="11" t="n"/>
       <c r="I49" s="12" t="n"/>
     </row>
-    <row r="50" ht="116" customHeight="1">
+    <row r="50" ht="172" customHeight="1">
       <c r="A50" s="13" t="inlineStr">
         <is>
-          <t>R-41</t>
+          <t>P2-17</t>
         </is>
       </c>
       <c r="B50" s="6" t="inlineStr">
         <is>
-          <t>App 顯示玩具電量狀態（低電量提示）</t>
+          <t>P2-16 ① 分批推送的數據表：推送階段、白名單、每台安裝結果</t>
         </is>
       </c>
       <c r="C50" s="13" t="inlineStr">
@@ -2078,7 +2080,7 @@
       </c>
       <c r="E50" s="6" t="inlineStr">
         <is>
-          <t>① pytest 33 passed；真 PATCH 本地 Supabase ② 62:70 刷 p212+R-41 強制低電 build（SUPPLY_LOW_RATIO_OVERRIDE=1.05）→ 串口 [WSc] power low:true，本地 DB battery_low=t ③ 刷回正常 1.6.2 → low:false，DB=f ④ App 讀 DB：低電紅標+Please charge+更新時間、72% 充電中、未上報不顯示 ⑤ 他人帳號 0 行、authenticated UPDATE 被拒。62:70 已還原為原 p212 build</t>
+          <t>migration 20261014190000 BEGIN/ROLLBACK 套用兩次無錯並已套用本機；行為：預設 100%、promote 記 stage_changed_at，7 種壞值（25%、小寫/空字串/NULL MAC、暫停缺原因等）全被 check 擋；ota_note_offer 1→2→3，report 正確標 running/failed、別板型不影響，刪發佈連帶刪記錄；審計 5 筆含 'test-board 9.9.9' 標籤。REST 13/13：超管可讀、內容管理員 0 行、anon 42501，三種身份寫入/改階段/呼叫 ota_note_offer 皆 42501。release_firmware.py promote spotpear-ai-toy 1.6.2 成功，token 查詢仍選 1.6.2，審計記 2 筆（actor 空＝service role）</t>
         </is>
       </c>
       <c r="F50" s="11" t="n"/>
@@ -2086,15 +2088,15 @@
       <c r="H50" s="11" t="n"/>
       <c r="I50" s="12" t="n"/>
     </row>
-    <row r="51" ht="102" customHeight="1">
+    <row r="51" ht="116" customHeight="1">
       <c r="A51" s="13" t="inlineStr">
         <is>
-          <t>P0-12</t>
+          <t>R-41</t>
         </is>
       </c>
       <c r="B51" s="6" t="inlineStr">
         <is>
-          <t>收緊 Admin 權限與路由保護</t>
+          <t>App 顯示玩具電量狀態（低電量提示）</t>
         </is>
       </c>
       <c r="C51" s="13" t="inlineStr">
@@ -2104,12 +2106,12 @@
       </c>
       <c r="D51" s="13" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E51" s="6" t="inlineStr">
         <is>
-          <t>線上 2026-10-12（bac24e9）：runbook 10/08 檢查 未登入 /admin→/login、/api/admin→401、has_role() 只看角色、無管理員 policy 觸及 conversations/記憶表、超管≥1；未登入 /home、/admin→/login；用戶確認：家長帳號開 /admin 轉回 /home、管理員在 /admin 修改角色保存成功；角色細分權限沿用本機 61/61</t>
+          <t>① pytest 33 passed；真 PATCH 本地 Supabase ② 62:70 刷 p212+R-41 強制低電 build（SUPPLY_LOW_RATIO_OVERRIDE=1.05）→ 串口 [WSc] power low:true，本地 DB battery_low=t ③ 刷回正常 1.6.2 → low:false，DB=f ④ App 讀 DB：低電紅標+Please charge+更新時間、72% 充電中、未上報不顯示 ⑤ 他人帳號 0 行、authenticated UPDATE 被拒。62:70 已還原為原 p212 build</t>
         </is>
       </c>
       <c r="F51" s="11" t="n"/>
@@ -2117,15 +2119,15 @@
       <c r="H51" s="11" t="n"/>
       <c r="I51" s="12" t="n"/>
     </row>
-    <row r="52" ht="88" customHeight="1">
+    <row r="52" ht="102" customHeight="1">
       <c r="A52" s="13" t="inlineStr">
         <is>
-          <t>P0-15</t>
+          <t>P0-12</t>
         </is>
       </c>
       <c r="B52" s="6" t="inlineStr">
         <is>
-          <t>角色表權限：只有內容管理員能發佈，關閉家長自建角色</t>
+          <t>收緊 Admin 權限與路由保護</t>
         </is>
       </c>
       <c r="C52" s="13" t="inlineStr">
@@ -2140,7 +2142,7 @@
       </c>
       <c r="E52" s="6" t="inlineStr">
         <is>
-          <t>線上 2026-10-12：② anon 只見 6 個已發佈 hk_ 內建，查隱藏/醫生/家長自建 → []，anon POST → 401；① authenticated 寫入權限由 20261007140000 REVOKE（runbook 10/08 已套用）；用戶確認：④ 家長登入後 /home/create 轉回 /home ③ 管理員在 /admin 修改角色保存成功</t>
+          <t>線上 2026-10-12（bac24e9）：runbook 10/08 檢查 未登入 /admin→/login、/api/admin→401、has_role() 只看角色、無管理員 policy 觸及 conversations/記憶表、超管≥1；未登入 /home、/admin→/login；用戶確認：家長帳號開 /admin 轉回 /home、管理員在 /admin 修改角色保存成功；角色細分權限沿用本機 61/61</t>
         </is>
       </c>
       <c r="F52" s="11" t="n"/>
@@ -2151,12 +2153,12 @@
     <row r="53" ht="88" customHeight="1">
       <c r="A53" s="13" t="inlineStr">
         <is>
-          <t>P0-16</t>
+          <t>P0-15</t>
         </is>
       </c>
       <c r="B53" s="6" t="inlineStr">
         <is>
-          <t>移除「醫生」身份與寫死的通關碼</t>
+          <t>角色表權限：只有內容管理員能發佈，關閉家長自建角色</t>
         </is>
       </c>
       <c r="C53" s="13" t="inlineStr">
@@ -2171,7 +2173,7 @@
       </c>
       <c r="E53" s="6" t="inlineStr">
         <is>
-          <t>線上 2026-10-12：生產 commit bac24e9 git grep checkDoctorAction/kiwi-subtle-emu/=== "doctor"/isDoctor → 0；線上 13 個 JS（/、/login、/onboard）grep 通關碼/"doctor"/Santa/patient → 0；anon 讀角色只見 6 個 hk_ 角色、is_doctor 全 false；用戶今日線上登入及 playground 正常</t>
+          <t>線上 2026-10-12：② anon 只見 6 個已發佈 hk_ 內建，查隱藏/醫生/家長自建 → []，anon POST → 401；① authenticated 寫入權限由 20261007140000 REVOKE（runbook 10/08 已套用）；用戶確認：④ 家長登入後 /home/create 轉回 /home ③ 管理員在 /admin 修改角色保存成功</t>
         </is>
       </c>
       <c r="F53" s="11" t="n"/>
@@ -2179,50 +2181,58 @@
       <c r="H53" s="11" t="n"/>
       <c r="I53" s="12" t="n"/>
     </row>
-    <row r="55">
-      <c r="A55" s="10" t="inlineStr">
+    <row r="54" ht="88" customHeight="1">
+      <c r="A54" s="13" t="inlineStr">
+        <is>
+          <t>P0-16</t>
+        </is>
+      </c>
+      <c r="B54" s="6" t="inlineStr">
+        <is>
+          <t>移除「醫生」身份與寫死的通關碼</t>
+        </is>
+      </c>
+      <c r="C54" s="13" t="inlineStr">
+        <is>
+          <t>通過</t>
+        </is>
+      </c>
+      <c r="D54" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="E54" s="6" t="inlineStr">
+        <is>
+          <t>線上 2026-10-12：生產 commit bac24e9 git grep checkDoctorAction/kiwi-subtle-emu/=== "doctor"/isDoctor → 0；線上 13 個 JS（/、/login、/onboard）grep 通關碼/"doctor"/Santa/patient → 0；anon 讀角色只見 6 個 hk_ 角色、is_doctor 全 false；用戶今日線上登入及 playground 正常</t>
+        </is>
+      </c>
+      <c r="F54" s="11" t="n"/>
+      <c r="G54" s="11" t="n"/>
+      <c r="H54" s="11" t="n"/>
+      <c r="I54" s="12" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="10" t="inlineStr">
         <is>
           <t>⏳ 等待依賴 / ⛔ 阻塞</t>
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="4" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
         <is>
           <t>編號</t>
         </is>
       </c>
-      <c r="B56" s="4" t="inlineStr">
+      <c r="B57" s="4" t="inlineStr">
         <is>
           <t>任務</t>
         </is>
       </c>
-      <c r="C56" s="4" t="inlineStr">
+      <c r="C57" s="4" t="inlineStr">
         <is>
           <t>在等什麼</t>
-        </is>
-      </c>
-      <c r="D56" s="11" t="n"/>
-      <c r="E56" s="11" t="n"/>
-      <c r="F56" s="11" t="n"/>
-      <c r="G56" s="11" t="n"/>
-      <c r="H56" s="11" t="n"/>
-      <c r="I56" s="12" t="n"/>
-    </row>
-    <row r="57" ht="88" customHeight="1">
-      <c r="A57" s="13" t="inlineStr">
-        <is>
-          <t>R-17</t>
-        </is>
-      </c>
-      <c r="B57" s="6" t="inlineStr">
-        <is>
-          <t>Spotpear 電池耗盡時插電能否正常開機（供電路徑）</t>
-        </is>
-      </c>
-      <c r="C57" s="6" t="inlineStr">
-        <is>
-          <t>阻塞：[2026-10-08] 2026-10-08 開發板 63:64 插著 USB 時兩次無法解釋的完全斷電重開：09:13:26（崩潰循環中）、10:44:33（閒置、用戶確認沒碰）。都是 USB 先斷線再以 ESP_RST_POWERON 開機，非 brownout；斷電前 6 秒 GPIO0 讀數 99.9% 參考值，屬突然切斷而非緩降（SupplyMonitor 取樣太疏抓不到瞬間）。韌體無法造成 POWERON，指向充電芯片/電池保護/供電路徑，應一併問 Spotpear；放電實測時留意插 USB 閒置時是否也會斷電</t>
         </is>
       </c>
       <c r="D57" s="11" t="n"/>
@@ -2232,20 +2242,20 @@
       <c r="H57" s="11" t="n"/>
       <c r="I57" s="12" t="n"/>
     </row>
-    <row r="58" ht="60" customHeight="1">
+    <row r="58" ht="88" customHeight="1">
       <c r="A58" s="13" t="inlineStr">
         <is>
-          <t>P1-01</t>
+          <t>R-17</t>
         </is>
       </c>
       <c r="B58" s="6" t="inlineStr">
         <is>
-          <t>加入內容審核層（輸入與輸出）</t>
+          <t>Spotpear 電池耗盡時插電能否正常開機（供電路徑）</t>
         </is>
       </c>
       <c r="C58" s="6" t="inlineStr">
         <is>
-          <t>阻塞：[2026-10-14] 2026-10-14 用戶決定：先不定審核服務商，本項暫停。候選：Azure Content Safety（建議，香港區、可在每句回覆說出口前檢查）、OpenRouter 安全模型、OpenAI Moderation、只用本機字詞表。未寫任何程式。</t>
+          <t>阻塞：[2026-10-08] 2026-10-08 開發板 63:64 插著 USB 時兩次無法解釋的完全斷電重開：09:13:26（崩潰循環中）、10:44:33（閒置、用戶確認沒碰）。都是 USB 先斷線再以 ESP_RST_POWERON 開機，非 brownout；斷電前 6 秒 GPIO0 讀數 99.9% 參考值，屬突然切斷而非緩降（SupplyMonitor 取樣太疏抓不到瞬間）。韌體無法造成 POWERON，指向充電芯片/電池保護/供電路徑，應一併問 Spotpear；放電實測時留意插 USB 閒置時是否也會斷電</t>
         </is>
       </c>
       <c r="D58" s="11" t="n"/>
@@ -2255,20 +2265,20 @@
       <c r="H58" s="11" t="n"/>
       <c r="I58" s="12" t="n"/>
     </row>
-    <row r="59" ht="32" customHeight="1">
+    <row r="59" ht="60" customHeight="1">
       <c r="A59" s="13" t="inlineStr">
         <is>
-          <t>P1-09</t>
+          <t>P1-01</t>
         </is>
       </c>
       <c r="B59" s="6" t="inlineStr">
         <is>
-          <t>家長鎖：孩子模式進設定要輸入 PIN</t>
+          <t>加入內容審核層（輸入與輸出）</t>
         </is>
       </c>
       <c r="C59" s="6" t="inlineStr">
         <is>
-          <t>阻塞：[2026-10-13] 2026-10-13 用戶決定：AI Buddy（品牌 C）延到 1/15 之後，本項不卡 1/15 出廠；AI Buddy 啟動時再開。</t>
+          <t>阻塞：[2026-10-14] 2026-10-14 用戶決定：先不定審核服務商，本項暫停。候選：Azure Content Safety（建議，香港區、可在每句回覆說出口前檢查）、OpenRouter 安全模型、OpenAI Moderation、只用本機字詞表。未寫任何程式。</t>
         </is>
       </c>
       <c r="D59" s="11" t="n"/>
@@ -2281,12 +2291,12 @@
     <row r="60" ht="32" customHeight="1">
       <c r="A60" s="13" t="inlineStr">
         <is>
-          <t>R-12</t>
+          <t>P1-09</t>
         </is>
       </c>
       <c r="B60" s="6" t="inlineStr">
         <is>
-          <t>家長控制：每日使用上限和休息時段</t>
+          <t>家長鎖：孩子模式進設定要輸入 PIN</t>
         </is>
       </c>
       <c r="C60" s="6" t="inlineStr">
@@ -2304,12 +2314,12 @@
     <row r="61" ht="32" customHeight="1">
       <c r="A61" s="13" t="inlineStr">
         <is>
-          <t>R-29</t>
+          <t>R-12</t>
         </is>
       </c>
       <c r="B61" s="6" t="inlineStr">
         <is>
-          <t>AI Buddy App（品牌 C）頁面</t>
+          <t>家長控制：每日使用上限和休息時段</t>
         </is>
       </c>
       <c r="C61" s="6" t="inlineStr">
@@ -2324,20 +2334,20 @@
       <c r="H61" s="11" t="n"/>
       <c r="I61" s="12" t="n"/>
     </row>
-    <row r="62" ht="18" customHeight="1">
+    <row r="62" ht="32" customHeight="1">
       <c r="A62" s="13" t="inlineStr">
         <is>
-          <t>P2-21</t>
+          <t>R-29</t>
         </is>
       </c>
       <c r="B62" s="6" t="inlineStr">
         <is>
-          <t>P2-16 ⑤ 後台 OTA 頁換成真實數據與操作</t>
+          <t>AI Buddy App（品牌 C）頁面</t>
         </is>
       </c>
       <c r="C62" s="6" t="inlineStr">
         <is>
-          <t>等 P2-14</t>
+          <t>阻塞：[2026-10-13] 2026-10-13 用戶決定：AI Buddy（品牌 C）延到 1/15 之後，本項不卡 1/15 出廠；AI Buddy 啟動時再開。</t>
         </is>
       </c>
       <c r="D62" s="11" t="n"/>
@@ -3182,6 +3192,7 @@
   <mergeCells count="86">
     <mergeCell ref="C82:I82"/>
     <mergeCell ref="E52:I52"/>
+    <mergeCell ref="A56:I56"/>
     <mergeCell ref="E39:I39"/>
     <mergeCell ref="C67:I67"/>
     <mergeCell ref="E48:I48"/>
@@ -3224,22 +3235,23 @@
     <mergeCell ref="C75:I75"/>
     <mergeCell ref="C84:I84"/>
     <mergeCell ref="C80:I80"/>
+    <mergeCell ref="E54:I54"/>
     <mergeCell ref="E32:I32"/>
     <mergeCell ref="C59:I59"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="E41:I41"/>
+    <mergeCell ref="A45:I45"/>
     <mergeCell ref="E47:I47"/>
     <mergeCell ref="C61:I61"/>
+    <mergeCell ref="E43:I43"/>
     <mergeCell ref="C70:I70"/>
     <mergeCell ref="E24:I24"/>
     <mergeCell ref="E33:I33"/>
     <mergeCell ref="A3:I3"/>
-    <mergeCell ref="A55:I55"/>
     <mergeCell ref="A104:I104"/>
     <mergeCell ref="E35:I35"/>
     <mergeCell ref="C74:I74"/>
     <mergeCell ref="C88:I88"/>
-    <mergeCell ref="E45:I45"/>
     <mergeCell ref="E37:I37"/>
     <mergeCell ref="E21:I21"/>
     <mergeCell ref="E23:I23"/>
@@ -3257,12 +3269,10 @@
     <mergeCell ref="C64:I64"/>
     <mergeCell ref="C79:I79"/>
     <mergeCell ref="C73:I73"/>
-    <mergeCell ref="A44:I44"/>
     <mergeCell ref="E49:I49"/>
     <mergeCell ref="E27:I27"/>
     <mergeCell ref="E36:I36"/>
     <mergeCell ref="C63:I63"/>
-    <mergeCell ref="C56:I56"/>
     <mergeCell ref="C90:I90"/>
     <mergeCell ref="E53:I53"/>
     <mergeCell ref="C76:I76"/>
@@ -9405,7 +9415,7 @@
         </is>
       </c>
     </row>
-    <row r="85" ht="172" customHeight="1">
+    <row r="85" ht="326" customHeight="1">
       <c r="A85" s="13" t="inlineStr">
         <is>
           <t>P2-16</t>
@@ -9438,7 +9448,7 @@
       </c>
       <c r="G85" s="13" t="inlineStr">
         <is>
-          <t>未測試</t>
+          <t>部分通過</t>
         </is>
       </c>
       <c r="I85" s="6" t="inlineStr">
@@ -9468,12 +9478,18 @@
           <t>P0-13, P2-14, P1-10, P2-17, P2-18, P2-19, P2-20, P2-21</t>
         </is>
       </c>
+      <c r="N85" s="6" t="inlineStr">
+        <is>
+          <t>子任務 P2-17～P2-20 通過、P2-21 部分通過（等 P2-14）。① 10% 階段只有雜湊預測的那組拿到、重複不變（P2-18、P2-21）② 2 台回滾 → 自動暫停、其餘不再拿到（P2-19、P2-21）③ 100% 全部拿到 ⑤ 審計表有每次階段變更（P2-21 9 筆）。未做：④ 開發板 62:70 實機走一次白名單階段（用戶目前手上沒有板子），同時驗證新韌體開機印出 BUILD_INFO</t>
+        </is>
+      </c>
       <c r="P85" s="6" t="inlineStr">
         <is>
           <t>[2026-10-14] 新增
 [2026-10-14] 2026-10-14 開分支 p2-16-ota-rollout（worktree ../aibuddy-p216，從 dev cac98aa）；拆成 P2-17～P2-21 五項子任務，本項的測試方法即整體驗收（含 62:70 實機白名單）。
 [2026-10-14] 2026-10-14 用戶決定提前到第 2 階段，現在開始做
-[2026-10-14] 2026-10-14 用戶決定拿走「同一台重啟 3 次即暫停」，原因見 P2-19</t>
+[2026-10-14] 2026-10-14 用戶決定拿走「同一台重啟 3 次即暫停」，原因見 P2-19
+[2026-10-14] 部署清單：① migrations 20261014190000、200000、210000、220000（依序，在 10-14 release 的 7 個之後）② 網頁 image ③ nginx 網頁 location 加 client_max_body_size 16m，curl 上傳 2MB 不得 413 ④ 韌體 BUILD_INFO 隨下一版韌體出，之前的版本仍用 release_firmware.py 發佈。分支 p2-16-ota-rollout 6 個 commit，未合併 dev、未推送</t>
         </is>
       </c>
     </row>
@@ -10099,7 +10115,7 @@
         </is>
       </c>
     </row>
-    <row r="94" ht="102" customHeight="1">
+    <row r="94" ht="312" customHeight="1">
       <c r="A94" s="13" t="inlineStr">
         <is>
           <t>P2-21</t>
@@ -10127,12 +10143,12 @@
       </c>
       <c r="F94" s="13" t="inlineStr">
         <is>
-          <t>未開始</t>
+          <t>進行中</t>
         </is>
       </c>
       <c r="G94" s="13" t="inlineStr">
         <is>
-          <t>未測試</t>
+          <t>部分通過</t>
         </is>
       </c>
       <c r="I94" s="6" t="inlineStr">
@@ -10160,10 +10176,21 @@
           <t>P2-18, P2-19, P2-20, P2-14</t>
         </is>
       </c>
+      <c r="N94" s="6" t="inlineStr">
+        <is>
+          <t>本機（分支 dev server 3216 + 本機 Supabase，GoTrue 真實登入的超管 cookie），用 xmini-c3 板型 + 20 台模擬設備以免碰到真開發板：頁面上傳 9.9.0 → 草稿；白名單加 1 台（UI 選單）→ 存檔；設為 current → 頁面預測 1 台、模擬 1 台；推進 10% → 預測 4、實得 4（重複不變）；50% → 預測 9、實得 9 且包含 10% 全部；100% → 20/20。2 台回滾 → 頁面顯示 'Paused … by the server: Auto-paused: 2 of 20 boards rolled back (10%)' 與回滾清單 2 台；點回滾設備 → 設備頁已帶 MAC 搜尋；恢復 → 其餘 18 台再拿到、回滾的 2 台不再下發；手動暫停未填原因不能確認、填後顯示 'by an admin'。審計頁 9 筆（上傳、白名單、current、10/50/100%、系統暫停、恢復、手動暫停），系統暫停顯示 System。375px scrollWidth=375。內容管理員側欄只有 Characters/IPs、#ota 退回 Characters、頁面無 OTA 數據，直接呼叫 admin_change_firmware_rollout → 403/42501。測試中發現並修正：舊版本（含 63:64 仍在跑的 1.6.1）被當成可刪除的草稿（6c2dc9d）。測試數據已清除</t>
+        </is>
+      </c>
+      <c r="O94" s="13" t="inlineStr">
+        <is>
+          <t>e0d7ac6</t>
+        </is>
+      </c>
       <c r="P94" s="6" t="inlineStr">
         <is>
           <t>[2026-10-14] 新增
-[2026-10-14] 2026-10-14 用戶決定提前到第 2 階段，現在開始做</t>
+[2026-10-14] 2026-10-14 用戶決定提前到第 2 階段，現在開始做
+[2026-10-14] 未完成：依賴 P2-14 的真板測試未做；測試方法中『白名單加 62:70』以模擬設備代替，實機一步歸 P2-16 ④，等板子到手一起做</t>
         </is>
       </c>
     </row>
@@ -10749,7 +10776,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I296"/>
+  <dimension ref="A1:I299"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -20995,8 +21022,129 @@
         </is>
       </c>
     </row>
+    <row r="297" ht="32" customHeight="1">
+      <c r="A297" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 21:47</t>
+        </is>
+      </c>
+      <c r="B297" s="13" t="inlineStr">
+        <is>
+          <t>P2-21</t>
+        </is>
+      </c>
+      <c r="C297" s="6" t="inlineStr">
+        <is>
+          <t>P2-16 ⑤ 後台 OTA 頁換成真實數據與操作</t>
+        </is>
+      </c>
+      <c r="D297" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E297" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F297" s="13" t="n"/>
+      <c r="G297" s="6" t="n"/>
+      <c r="H297" s="13" t="n"/>
+      <c r="I297" s="6" t="n"/>
+    </row>
+    <row r="298" ht="270" customHeight="1">
+      <c r="A298" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 21:59</t>
+        </is>
+      </c>
+      <c r="B298" s="13" t="inlineStr">
+        <is>
+          <t>P2-21</t>
+        </is>
+      </c>
+      <c r="C298" s="6" t="inlineStr">
+        <is>
+          <t>P2-16 ⑤ 後台 OTA 頁換成真實數據與操作</t>
+        </is>
+      </c>
+      <c r="D298" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="E298" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F298" s="13" t="inlineStr">
+        <is>
+          <t>部分通過</t>
+        </is>
+      </c>
+      <c r="G298" s="6" t="inlineStr">
+        <is>
+          <t>本機（分支 dev server 3216 + 本機 Supabase，GoTrue 真實登入的超管 cookie），用 xmini-c3 板型 + 20 台模擬設備以免碰到真開發板：頁面上傳 9.9.0 → 草稿；白名單加 1 台（UI 選單）→ 存檔；設為 current → 頁面預測 1 台、模擬 1 台；推進 10% → 預測 4、實得 4（重複不變）；50% → 預測 9、實得 9 且包含 10% 全部；100% → 20/20。2 台回滾 → 頁面顯示 'Paused … by the server: Auto-paused: 2 of 20 boards rolled back (10%)' 與回滾清單 2 台；點回滾設備 → 設備頁已帶 MAC 搜尋；恢復 → 其餘 18 台再拿到、回滾的 2 台不再下發；手動暫停未填原因不能確認、填後顯示 'by an admin'。審計頁 9 筆（上傳、白名單、current、10/50/100%、系統暫停、恢復、手動暫停），系統暫停顯示 System。375px scrollWidth=375。內容管理員側欄只有 Characters/IPs、#ota 退回 Characters、頁面無 OTA 數據，直接呼叫 admin_change_firmware_rollout → 403/42501。測試中發現並修正：舊版本（含 63:64 仍在跑的 1.6.1）被當成可刪除的草稿（6c2dc9d）。測試數據已清除</t>
+        </is>
+      </c>
+      <c r="H298" s="13" t="inlineStr">
+        <is>
+          <t>e0d7ac6</t>
+        </is>
+      </c>
+      <c r="I298" s="6" t="inlineStr">
+        <is>
+          <t>未完成：依賴 P2-14 的真板測試未做；測試方法中『白名單加 62:70』以模擬設備代替，實機一步歸 P2-16 ④，等板子到手一起做</t>
+        </is>
+      </c>
+    </row>
+    <row r="299" ht="144" customHeight="1">
+      <c r="A299" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 21:59</t>
+        </is>
+      </c>
+      <c r="B299" s="13" t="inlineStr">
+        <is>
+          <t>P2-16</t>
+        </is>
+      </c>
+      <c r="C299" s="6" t="inlineStr">
+        <is>
+          <t>OTA 分批推送與後台發佈頁</t>
+        </is>
+      </c>
+      <c r="D299" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="E299" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F299" s="13" t="inlineStr">
+        <is>
+          <t>部分通過</t>
+        </is>
+      </c>
+      <c r="G299" s="6" t="inlineStr">
+        <is>
+          <t>子任務 P2-17～P2-20 通過、P2-21 部分通過（等 P2-14）。① 10% 階段只有雜湊預測的那組拿到、重複不變（P2-18、P2-21）② 2 台回滾 → 自動暫停、其餘不再拿到（P2-19、P2-21）③ 100% 全部拿到 ⑤ 審計表有每次階段變更（P2-21 9 筆）。未做：④ 開發板 62:70 實機走一次白名單階段（用戶目前手上沒有板子），同時驗證新韌體開機印出 BUILD_INFO</t>
+        </is>
+      </c>
+      <c r="H299" s="13" t="n"/>
+      <c r="I299" s="6" t="inlineStr">
+        <is>
+          <t>部署清單：① migrations 20261014190000、200000、210000、220000（依序，在 10-14 release 的 7 個之後）② 網頁 image ③ nginx 網頁 location 加 client_max_body_size 16m，curl 上傳 2MB 不得 413 ④ 韌體 BUILD_INFO 隨下一版韌體出，之前的版本仍用 release_firmware.py 發佈。分支 p2-16-ota-rollout 6 個 commit，未合併 dev、未推送</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I296"/>
+  <autoFilter ref="A1:I299"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Track P2-22: survive server URL changes without losing OTA.
The voice URL comes from the token answer, the backend URL can migrate,
and a confirmed image that cannot reach the server for days falls back
to the other slot.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/production-readiness.xlsx
+++ b/docs/production-readiness.xlsx
@@ -13,9 +13,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="更新記錄" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'任務清單'!$A$1:$P$94</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'任務清單'!$A$1:$P$95</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'待確認問題'!$A$1:$G$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$299</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$301</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -641,7 +641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I105"/>
+  <dimension ref="A1:I106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -665,14 +665,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>最後更新：2026-10-14 21:59　·　本頁由 tracker.py 自動生成，請勿手動編輯</t>
+          <t>最後更新：2026-10-14 22:19　·　本頁由 tracker.py 自動生成，請勿手動編輯</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>總進度：22/89 已完成（25%）　·　目前階段：1 止血定案（10/5–10/16）</t>
+          <t>總進度：22/90 已完成（24%）　·　目前階段：1 止血定案（10/5–10/16）</t>
         </is>
       </c>
     </row>
@@ -816,11 +816,11 @@
       </c>
       <c r="C8" s="7">
         <f>COUNTIF('任務清單'!$B:$B,$A8)</f>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D8" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A8,'任務清單'!$F:$F,D$5)</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E8" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A8,'任務清單'!$F:$F,E$5)</f>
@@ -840,7 +840,7 @@
       </c>
       <c r="I8" s="8">
         <f>IFERROR(F8/(C8-H8),0)</f>
-        <v>0.3333333333333333</v>
+        <v>0.3181818181818182</v>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1">
@@ -892,11 +892,11 @@
       <c r="B10" s="6" t="n"/>
       <c r="C10" s="5">
         <f>SUM(C6:C9)</f>
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D10" s="5">
         <f>SUM(D6:D9)</f>
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E10" s="5">
         <f>SUM(E6:E9)</f>
@@ -916,7 +916,7 @@
       </c>
       <c r="I10" s="9">
         <f>IFERROR(F10/(C10-H10),0)</f>
-        <v>0.24719101123595505</v>
+        <v>0.24444444444444444</v>
       </c>
     </row>
     <row r="12">
@@ -1059,11 +1059,11 @@
       </c>
       <c r="C15" s="7">
         <f>COUNTIF('任務清單'!$C:$C,$A15)</f>
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D15" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A15,'任務清單'!$F:$F,D$12)</f>
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E15" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A15,'任務清單'!$F:$F,E$12)</f>
@@ -1135,11 +1135,11 @@
       <c r="B17" s="6" t="n"/>
       <c r="C17" s="5">
         <f>SUM(C13:C16)</f>
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D17" s="5">
         <f>SUM(D13:D16)</f>
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E17" s="5">
         <f>SUM(E13:E16)</f>
@@ -1159,7 +1159,7 @@
       </c>
       <c r="I17" s="9">
         <f>IFERROR(F17/(C17-H17),0)</f>
-        <v>0.24719101123595505</v>
+        <v>0.24444444444444444</v>
       </c>
     </row>
     <row r="19">
@@ -2656,20 +2656,20 @@
       <c r="H75" s="11" t="n"/>
       <c r="I75" s="12" t="n"/>
     </row>
-    <row r="76" ht="18" customHeight="1">
+    <row r="76" ht="46" customHeight="1">
       <c r="A76" s="13" t="inlineStr">
         <is>
-          <t>R-07</t>
+          <t>P2-22</t>
         </is>
       </c>
       <c r="B76" s="6" t="inlineStr">
         <is>
-          <t>20 個家庭封閉內測</t>
+          <t>改服務器網址也不失聯：語音網址由後端下發、後端網址可遷移、已確認韌體長期連不上時自救</t>
         </is>
       </c>
       <c r="C76" s="6" t="inlineStr">
         <is>
-          <t>等 R-13</t>
+          <t>等 R-35</t>
         </is>
       </c>
       <c r="D76" s="11" t="n"/>
@@ -2682,17 +2682,17 @@
     <row r="77" ht="18" customHeight="1">
       <c r="A77" s="13" t="inlineStr">
         <is>
-          <t>R-08</t>
+          <t>R-07</t>
         </is>
       </c>
       <c r="B77" s="6" t="inlineStr">
         <is>
-          <t>第 8 週關卡決策</t>
+          <t>20 個家庭封閉內測</t>
         </is>
       </c>
       <c r="C77" s="6" t="inlineStr">
         <is>
-          <t>等 R-07、P2-09、P1-08</t>
+          <t>等 R-13</t>
         </is>
       </c>
       <c r="D77" s="11" t="n"/>
@@ -2705,17 +2705,17 @@
     <row r="78" ht="18" customHeight="1">
       <c r="A78" s="13" t="inlineStr">
         <is>
-          <t>R-14</t>
+          <t>R-08</t>
         </is>
       </c>
       <c r="B78" s="6" t="inlineStr">
         <is>
-          <t>離線兒歌與故事</t>
+          <t>第 8 週關卡決策</t>
         </is>
       </c>
       <c r="C78" s="6" t="inlineStr">
         <is>
-          <t>等 R-01</t>
+          <t>等 R-07、P2-09、P1-08</t>
         </is>
       </c>
       <c r="D78" s="11" t="n"/>
@@ -2728,17 +2728,17 @@
     <row r="79" ht="18" customHeight="1">
       <c r="A79" s="13" t="inlineStr">
         <is>
-          <t>R-24</t>
+          <t>R-14</t>
         </is>
       </c>
       <c r="B79" s="6" t="inlineStr">
         <is>
-          <t>設備只能用自己品牌的角色</t>
+          <t>離線兒歌與故事</t>
         </is>
       </c>
       <c r="C79" s="6" t="inlineStr">
         <is>
-          <t>等 R-34</t>
+          <t>等 R-01</t>
         </is>
       </c>
       <c r="D79" s="11" t="n"/>
@@ -2751,17 +2751,17 @@
     <row r="80" ht="18" customHeight="1">
       <c r="A80" s="13" t="inlineStr">
         <is>
-          <t>R-28</t>
+          <t>R-24</t>
         </is>
       </c>
       <c r="B80" s="6" t="inlineStr">
         <is>
-          <t>三個 App 的殼：品牌版本與測試版</t>
+          <t>設備只能用自己品牌的角色</t>
         </is>
       </c>
       <c r="C80" s="6" t="inlineStr">
         <is>
-          <t>等 R-25、R-26</t>
+          <t>等 R-34</t>
         </is>
       </c>
       <c r="D80" s="11" t="n"/>
@@ -2774,17 +2774,17 @@
     <row r="81" ht="18" customHeight="1">
       <c r="A81" s="13" t="inlineStr">
         <is>
-          <t>R-30</t>
+          <t>R-28</t>
         </is>
       </c>
       <c r="B81" s="6" t="inlineStr">
         <is>
-          <t>快活 App（品牌 A）頁面</t>
+          <t>三個 App 的殼：品牌版本與測試版</t>
         </is>
       </c>
       <c r="C81" s="6" t="inlineStr">
         <is>
-          <t>等 R-25、R-34、Q12</t>
+          <t>等 R-25、R-26</t>
         </is>
       </c>
       <c r="D81" s="11" t="n"/>
@@ -2797,17 +2797,17 @@
     <row r="82" ht="18" customHeight="1">
       <c r="A82" s="13" t="inlineStr">
         <is>
-          <t>R-31</t>
+          <t>R-30</t>
         </is>
       </c>
       <c r="B82" s="6" t="inlineStr">
         <is>
-          <t>政協青年聯會版 App（品牌 B）頁面</t>
+          <t>快活 App（品牌 A）頁面</t>
         </is>
       </c>
       <c r="C82" s="6" t="inlineStr">
         <is>
-          <t>等 R-25、R-34、Q13</t>
+          <t>等 R-25、R-34、Q12</t>
         </is>
       </c>
       <c r="D82" s="11" t="n"/>
@@ -2820,17 +2820,17 @@
     <row r="83" ht="18" customHeight="1">
       <c r="A83" s="13" t="inlineStr">
         <is>
-          <t>R-35</t>
+          <t>R-31</t>
         </is>
       </c>
       <c r="B83" s="6" t="inlineStr">
         <is>
-          <t>韌體按品牌連線：伺服器網址在出廠時寫入</t>
+          <t>政協青年聯會版 App（品牌 B）頁面</t>
         </is>
       </c>
       <c r="C83" s="6" t="inlineStr">
         <is>
-          <t>等 R-34</t>
+          <t>等 R-25、R-34、Q13</t>
         </is>
       </c>
       <c r="D83" s="11" t="n"/>
@@ -2840,20 +2840,20 @@
       <c r="H83" s="11" t="n"/>
       <c r="I83" s="12" t="n"/>
     </row>
-    <row r="84" ht="32" customHeight="1">
+    <row r="84" ht="18" customHeight="1">
       <c r="A84" s="13" t="inlineStr">
         <is>
-          <t>R-38</t>
+          <t>R-35</t>
         </is>
       </c>
       <c r="B84" s="6" t="inlineStr">
         <is>
-          <t>公仔出廠鎖死所屬 IP，綁定時顯示該 IP 頭像</t>
+          <t>韌體按品牌連線：伺服器網址在出廠時寫入</t>
         </is>
       </c>
       <c r="C84" s="6" t="inlineStr">
         <is>
-          <t>等 P0-11</t>
+          <t>等 R-34</t>
         </is>
       </c>
       <c r="D84" s="11" t="n"/>
@@ -2866,17 +2866,17 @@
     <row r="85" ht="32" customHeight="1">
       <c r="A85" s="13" t="inlineStr">
         <is>
-          <t>R-39</t>
+          <t>R-38</t>
         </is>
       </c>
       <c r="B85" s="6" t="inlineStr">
         <is>
-          <t>Admin 出廠登記頁：匯入 MAC 清單、指定公仔、查看自檢結果</t>
+          <t>公仔出廠鎖死所屬 IP，綁定時顯示該 IP 頭像</t>
         </is>
       </c>
       <c r="C85" s="6" t="inlineStr">
         <is>
-          <t>等 R-38、P1-10</t>
+          <t>等 P0-11</t>
         </is>
       </c>
       <c r="D85" s="11" t="n"/>
@@ -2886,20 +2886,20 @@
       <c r="H85" s="11" t="n"/>
       <c r="I85" s="12" t="n"/>
     </row>
-    <row r="86" ht="18" customHeight="1">
+    <row r="86" ht="32" customHeight="1">
       <c r="A86" s="13" t="inlineStr">
         <is>
-          <t>R-09</t>
+          <t>R-39</t>
         </is>
       </c>
       <c r="B86" s="6" t="inlineStr">
         <is>
-          <t>量產外殼（真空複模）</t>
+          <t>Admin 出廠登記頁：匯入 MAC 清單、指定公仔、查看自檢結果</t>
         </is>
       </c>
       <c r="C86" s="6" t="inlineStr">
         <is>
-          <t>等 R-08、R-05、Q11</t>
+          <t>等 R-38、P1-10</t>
         </is>
       </c>
       <c r="D86" s="11" t="n"/>
@@ -2912,17 +2912,17 @@
     <row r="87" ht="18" customHeight="1">
       <c r="A87" s="13" t="inlineStr">
         <is>
-          <t>R-10</t>
+          <t>R-09</t>
         </is>
       </c>
       <c r="B87" s="6" t="inlineStr">
         <is>
-          <t>出廠流程</t>
+          <t>量產外殼（真空複模）</t>
         </is>
       </c>
       <c r="C87" s="6" t="inlineStr">
         <is>
-          <t>等 P0-14、R-01、P2-12、R-34、R-35、R-38、R-39</t>
+          <t>等 R-08、R-05、Q11</t>
         </is>
       </c>
       <c r="D87" s="11" t="n"/>
@@ -2935,17 +2935,17 @@
     <row r="88" ht="18" customHeight="1">
       <c r="A88" s="13" t="inlineStr">
         <is>
-          <t>R-11</t>
+          <t>R-10</t>
         </is>
       </c>
       <c r="B88" s="6" t="inlineStr">
         <is>
-          <t>售後：客服、保修與換機</t>
+          <t>出廠流程</t>
         </is>
       </c>
       <c r="C88" s="6" t="inlineStr">
         <is>
-          <t>等 P2-14、R-40</t>
+          <t>等 P0-14、R-01、P2-12、R-34、R-35、R-38、R-39</t>
         </is>
       </c>
       <c r="D88" s="11" t="n"/>
@@ -2958,17 +2958,17 @@
     <row r="89" ht="18" customHeight="1">
       <c r="A89" s="13" t="inlineStr">
         <is>
-          <t>R-15</t>
+          <t>R-11</t>
         </is>
       </c>
       <c r="B89" s="6" t="inlineStr">
         <is>
-          <t>農曆新年前交付（生產 1/15、送達 1/29）</t>
+          <t>售後：客服、保修與換機</t>
         </is>
       </c>
       <c r="C89" s="6" t="inlineStr">
         <is>
-          <t>等 R-09、R-10</t>
+          <t>等 P2-14、R-40</t>
         </is>
       </c>
       <c r="D89" s="11" t="n"/>
@@ -2981,17 +2981,17 @@
     <row r="90" ht="18" customHeight="1">
       <c r="A90" s="13" t="inlineStr">
         <is>
-          <t>R-33</t>
+          <t>R-15</t>
         </is>
       </c>
       <c r="B90" s="6" t="inlineStr">
         <is>
-          <t>三個 App 送審並通過</t>
+          <t>農曆新年前交付（生產 1/15、送達 1/29）</t>
         </is>
       </c>
       <c r="C90" s="6" t="inlineStr">
         <is>
-          <t>等 R-27、R-21、R-28、R-29、R-30、R-31、R-32</t>
+          <t>等 R-09、R-10</t>
         </is>
       </c>
       <c r="D90" s="11" t="n"/>
@@ -3001,20 +3001,20 @@
       <c r="H90" s="11" t="n"/>
       <c r="I90" s="12" t="n"/>
     </row>
-    <row r="91" ht="32" customHeight="1">
+    <row r="91" ht="18" customHeight="1">
       <c r="A91" s="13" t="inlineStr">
         <is>
-          <t>R-40</t>
+          <t>R-33</t>
         </is>
       </c>
       <c r="B91" s="6" t="inlineStr">
         <is>
-          <t>Admin 客服查詢頁：查帳號、名下設備與最近事件</t>
+          <t>三個 App 送審並通過</t>
         </is>
       </c>
       <c r="C91" s="6" t="inlineStr">
         <is>
-          <t>等 P2-14、P1-10、P1-12</t>
+          <t>等 R-27、R-21、R-28、R-29、R-30、R-31、R-32</t>
         </is>
       </c>
       <c r="D91" s="11" t="n"/>
@@ -3024,50 +3024,50 @@
       <c r="H91" s="11" t="n"/>
       <c r="I91" s="12" t="n"/>
     </row>
-    <row r="93">
-      <c r="A93" s="10" t="inlineStr">
+    <row r="92" ht="32" customHeight="1">
+      <c r="A92" s="13" t="inlineStr">
+        <is>
+          <t>R-40</t>
+        </is>
+      </c>
+      <c r="B92" s="6" t="inlineStr">
+        <is>
+          <t>Admin 客服查詢頁：查帳號、名下設備與最近事件</t>
+        </is>
+      </c>
+      <c r="C92" s="6" t="inlineStr">
+        <is>
+          <t>等 P2-14、P1-10、P1-12</t>
+        </is>
+      </c>
+      <c r="D92" s="11" t="n"/>
+      <c r="E92" s="11" t="n"/>
+      <c r="F92" s="11" t="n"/>
+      <c r="G92" s="11" t="n"/>
+      <c r="H92" s="11" t="n"/>
+      <c r="I92" s="12" t="n"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="10" t="inlineStr">
         <is>
           <t>❓ 待確認問題</t>
         </is>
       </c>
     </row>
-    <row r="94">
-      <c r="A94" s="4" t="inlineStr">
+    <row r="95">
+      <c r="A95" s="4" t="inlineStr">
         <is>
           <t>編號</t>
         </is>
       </c>
-      <c r="B94" s="4" t="inlineStr">
+      <c r="B95" s="4" t="inlineStr">
         <is>
           <t>問題</t>
         </is>
       </c>
-      <c r="C94" s="4" t="inlineStr">
+      <c r="C95" s="4" t="inlineStr">
         <is>
           <t>影響的任務 / 為什麼重要</t>
-        </is>
-      </c>
-      <c r="D94" s="11" t="n"/>
-      <c r="E94" s="11" t="n"/>
-      <c r="F94" s="11" t="n"/>
-      <c r="G94" s="11" t="n"/>
-      <c r="H94" s="11" t="n"/>
-      <c r="I94" s="12" t="n"/>
-    </row>
-    <row r="95" ht="18" customHeight="1">
-      <c r="A95" s="13" t="inlineStr">
-        <is>
-          <t>Q3</t>
-        </is>
-      </c>
-      <c r="B95" s="6" t="inlineStr">
-        <is>
-          <t>韌體打算閉源商業銷售嗎？</t>
-        </is>
-      </c>
-      <c r="C95" s="6" t="inlineStr">
-        <is>
-          <t>P1-06, P1-07：決定 GPL／LGPL 依賴要開源還是替換。</t>
         </is>
       </c>
       <c r="D95" s="11" t="n"/>
@@ -3077,20 +3077,20 @@
       <c r="H95" s="11" t="n"/>
       <c r="I95" s="12" t="n"/>
     </row>
-    <row r="96" ht="32" customHeight="1">
+    <row r="96" ht="18" customHeight="1">
       <c r="A96" s="13" t="inlineStr">
         <is>
-          <t>Q11</t>
+          <t>Q3</t>
         </is>
       </c>
       <c r="B96" s="6" t="inlineStr">
         <is>
-          <t>馬會快活的賽馬日版和新春版各多少隻（共 2,500）？</t>
+          <t>韌體打算閉源商業銷售嗎？</t>
         </is>
       </c>
       <c r="C96" s="6" t="inlineStr">
         <is>
-          <t>R-09, R-15：兩款的服裝和配件要分開訂料；11/20 前不知道，PP 樣和大貨單（11/27）會被拖慢。由馬會決定。</t>
+          <t>P1-06, P1-07：決定 GPL／LGPL 依賴要開源還是替換。</t>
         </is>
       </c>
       <c r="D96" s="11" t="n"/>
@@ -3100,20 +3100,20 @@
       <c r="H96" s="11" t="n"/>
       <c r="I96" s="12" t="n"/>
     </row>
-    <row r="97" ht="60" customHeight="1">
+    <row r="97" ht="32" customHeight="1">
       <c r="A97" s="13" t="inlineStr">
         <is>
-          <t>Q12</t>
+          <t>Q11</t>
         </is>
       </c>
       <c r="B97" s="6" t="inlineStr">
         <is>
-          <t>快活 App 的「會員綁定」是指甚麼：用我們自己的帳號（email 驗證碼），還是接馬會的會員帳號登入（SSO）？</t>
+          <t>馬會快活的賽馬日版和新春版各多少隻（共 2,500）？</t>
         </is>
       </c>
       <c r="C97" s="6" t="inlineStr">
         <is>
-          <t>P0-11, 快活 App（未入追蹤表）：接馬會 SSO 的話，登入、帳號刪除和資料歸屬都要按馬會的介面重做，工作量和排期要另估，而且 W5（11/9–11/13）就要做快活 App 的綁定；用我們的帳號則和其他品牌共用同一套流程。由馬會決定，要盡早問。</t>
+          <t>R-09, R-15：兩款的服裝和配件要分開訂料；11/20 前不知道，PP 樣和大貨單（11/27）會被拖慢。由馬會決定。</t>
         </is>
       </c>
       <c r="D97" s="11" t="n"/>
@@ -3123,20 +3123,20 @@
       <c r="H97" s="11" t="n"/>
       <c r="I97" s="12" t="n"/>
     </row>
-    <row r="98" ht="46" customHeight="1">
+    <row r="98" ht="60" customHeight="1">
       <c r="A98" s="13" t="inlineStr">
         <is>
-          <t>Q13</t>
+          <t>Q12</t>
         </is>
       </c>
       <c r="B98" s="6" t="inlineStr">
         <is>
-          <t>政協青年聯會版的角色、語言和內容由誰提供？什麼時候交？</t>
+          <t>快活 App 的「會員綁定」是指甚麼：用我們自己的帳號（email 驗證碼），還是接馬會的會員帳號登入（SSO）？</t>
         </is>
       </c>
       <c r="C98" s="6" t="inlineStr">
         <is>
-          <t>品牌 B 的 App 頁面：品牌 B 的用戶是成人會員，但角色、說話語言、內容規則都還沒有。最遲 11/13 要拿到，才趕得及內部測試和 App 頁面（W6）。</t>
+          <t>P0-11, 快活 App（未入追蹤表）：接馬會 SSO 的話，登入、帳號刪除和資料歸屬都要按馬會的介面重做，工作量和排期要另估，而且 W5（11/9–11/13）就要做快活 App 的綁定；用我們的帳號則和其他品牌共用同一套流程。由馬會決定，要盡早問。</t>
         </is>
       </c>
       <c r="D98" s="11" t="n"/>
@@ -3146,50 +3146,73 @@
       <c r="H98" s="11" t="n"/>
       <c r="I98" s="12" t="n"/>
     </row>
-    <row r="100">
-      <c r="A100" s="10" t="inlineStr">
+    <row r="99" ht="46" customHeight="1">
+      <c r="A99" s="13" t="inlineStr">
+        <is>
+          <t>Q13</t>
+        </is>
+      </c>
+      <c r="B99" s="6" t="inlineStr">
+        <is>
+          <t>政協青年聯會版的角色、語言和內容由誰提供？什麼時候交？</t>
+        </is>
+      </c>
+      <c r="C99" s="6" t="inlineStr">
+        <is>
+          <t>品牌 B 的 App 頁面：品牌 B 的用戶是成人會員，但角色、說話語言、內容規則都還沒有。最遲 11/13 要拿到，才趕得及內部測試和 App 頁面（W6）。</t>
+        </is>
+      </c>
+      <c r="D99" s="11" t="n"/>
+      <c r="E99" s="11" t="n"/>
+      <c r="F99" s="11" t="n"/>
+      <c r="G99" s="11" t="n"/>
+      <c r="H99" s="11" t="n"/>
+      <c r="I99" s="12" t="n"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="10" t="inlineStr">
         <is>
           <t>說明</t>
         </is>
       </c>
     </row>
-    <row r="101" ht="32" customHeight="1">
-      <c r="A101" s="14" t="inlineStr">
+    <row r="102" ht="32" customHeight="1">
+      <c r="A102" s="14" t="inlineStr">
         <is>
           <t>・狀態：未開始 → 進行中 → 已完成。只有測試真的跑過而且通過才算已完成；阻塞要在備註寫原因；不再需要的任務標不適用，不要刪。</t>
-        </is>
-      </c>
-    </row>
-    <row r="102" ht="18" customHeight="1">
-      <c r="A102" s="14" t="inlineStr">
-        <is>
-          <t>・測試結果：未測試 / 通過 / 失敗 / 部分通過。測試證據寫跑了什麼、看到什麼，完整歷史在「更新記錄」。</t>
         </is>
       </c>
     </row>
     <row r="103" ht="18" customHeight="1">
       <c r="A103" s="14" t="inlineStr">
         <is>
-          <t>・「接下來」按階段排序，同一階段內再按優先級；依賴還沒滿足的任務不會出現在「接下來」。</t>
+          <t>・測試結果：未測試 / 通過 / 失敗 / 部分通過。測試證據寫跑了什麼、看到什麼，完整歷史在「更新記錄」。</t>
         </is>
       </c>
     </row>
     <row r="104" ht="18" customHeight="1">
       <c r="A104" s="14" t="inlineStr">
         <is>
+          <t>・「接下來」按階段排序，同一階段內再按優先級；依賴還沒滿足的任務不會出現在「接下來」。</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" ht="18" customHeight="1">
+      <c r="A105" s="14" t="inlineStr">
+        <is>
           <t>・可以手動改：「任務清單」的狀態、測試結果、測試證據、Commit、備註，以及「待確認問題」的回答。其餘欄位和本頁由腳本維護。</t>
         </is>
       </c>
     </row>
-    <row r="105" ht="32" customHeight="1">
-      <c r="A105" s="14" t="inlineStr">
+    <row r="106" ht="32" customHeight="1">
+      <c r="A106" s="14" t="inlineStr">
         <is>
           <t>・建議用法：在 Claude Code 對 Claude 說「P0-02 做完了」或輸入 /prod-readiness。Claude 會先跑測試再更新，並寫進「更新記錄」。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="86">
+  <mergeCells count="87">
     <mergeCell ref="C82:I82"/>
     <mergeCell ref="E52:I52"/>
     <mergeCell ref="A56:I56"/>
@@ -3201,6 +3224,7 @@
     <mergeCell ref="E29:I29"/>
     <mergeCell ref="E38:I38"/>
     <mergeCell ref="C83:I83"/>
+    <mergeCell ref="C92:I92"/>
     <mergeCell ref="E31:I31"/>
     <mergeCell ref="E40:I40"/>
     <mergeCell ref="C97:I97"/>
@@ -3222,15 +3246,12 @@
     <mergeCell ref="C77:I77"/>
     <mergeCell ref="C86:I86"/>
     <mergeCell ref="C68:I68"/>
-    <mergeCell ref="A100:I100"/>
     <mergeCell ref="C58:I58"/>
     <mergeCell ref="E30:I30"/>
     <mergeCell ref="E22:I22"/>
-    <mergeCell ref="A93:I93"/>
     <mergeCell ref="E46:I46"/>
     <mergeCell ref="A102:I102"/>
     <mergeCell ref="C85:I85"/>
-    <mergeCell ref="C94:I94"/>
     <mergeCell ref="C65:I65"/>
     <mergeCell ref="C75:I75"/>
     <mergeCell ref="C84:I84"/>
@@ -3241,6 +3262,7 @@
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="E41:I41"/>
     <mergeCell ref="A45:I45"/>
+    <mergeCell ref="A94:I94"/>
     <mergeCell ref="E47:I47"/>
     <mergeCell ref="C61:I61"/>
     <mergeCell ref="E43:I43"/>
@@ -3250,8 +3272,10 @@
     <mergeCell ref="A3:I3"/>
     <mergeCell ref="A104:I104"/>
     <mergeCell ref="E35:I35"/>
+    <mergeCell ref="A106:I106"/>
     <mergeCell ref="C74:I74"/>
     <mergeCell ref="C88:I88"/>
+    <mergeCell ref="C99:I99"/>
     <mergeCell ref="E37:I37"/>
     <mergeCell ref="E21:I21"/>
     <mergeCell ref="E23:I23"/>
@@ -3305,7 +3329,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P94"/>
+  <dimension ref="A1:P95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -10194,8 +10218,76 @@
         </is>
       </c>
     </row>
+    <row r="95" ht="298" customHeight="1">
+      <c r="A95" s="13" t="inlineStr">
+        <is>
+          <t>P2-22</t>
+        </is>
+      </c>
+      <c r="B95" s="13" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C95" s="13" t="inlineStr">
+        <is>
+          <t>3 封閉內測</t>
+        </is>
+      </c>
+      <c r="D95" s="6" t="inlineStr">
+        <is>
+          <t>OTA/韌體</t>
+        </is>
+      </c>
+      <c r="E95" s="6" t="inlineStr">
+        <is>
+          <t>改服務器網址也不失聯：語音網址由後端下發、後端網址可遷移、已確認韌體長期連不上時自救</t>
+        </is>
+      </c>
+      <c r="F95" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="G95" s="13" t="inlineStr">
+        <is>
+          <t>未測試</t>
+        </is>
+      </c>
+      <c r="I95" s="6" t="inlineStr">
+        <is>
+          <t>OTA 和取 token 都走後端（backend_server），語音伺服器網址（ws_server/ws_path，現為 elatoai.hkqft.com/fastapi/ws/esp32）寫死在韌體裡。日後改 FastAPI 網址就要先推新韌體，而新韌體在試用期內連不上新網址會被回滾；後端網址一改，現有板子連 OTA 都收不到，只能 USB 救。另一個缺口：已確認（過了試用期）的韌體如果之後一直連不上服務器但不崩潰，682f3b4 的連續崩溃切槽不會觸發，板子收不到修復。</t>
+        </is>
+      </c>
+      <c r="J95" s="6" t="inlineStr">
+        <is>
+          <t>firmware-arduino/src/Config.cpp（ws_server、ws_port、ws_path、backend_server、CF_CA_bundle）、src/OTA.cpp（otaBootCheck、usableOtherSlot）、取 token 的流程；frontend-nextjs 的 /api/generate_auth_token（回應加 voice_url / backend_url）；R-35 的 NVS 網址</t>
+        </is>
+      </c>
+      <c r="K95" s="6" t="inlineStr">
+        <is>
+          <t>① /api/generate_auth_token 的回應帶 voice_url（wss 主機＋端口＋路徑，來自後端環境變數）；韌體用它連 /ws，並把最後一次成功的值存進 NVS；改 FastAPI 網址只改伺服器設定，不需新韌體 ② 回應沒有 voice_url（舊後端）或新網址連不上時，退回 NVS 上次成功的值，再退回出廠／編譯時的預設值 ③ 後端網址可遷移：回應可帶 backend_url；韌體先存為候選，下次開機用新網址取 token 成功才正式替換，失敗就繼續用舊網址；舊網址在遷移期內保持可用（runbook 寫明保留多久） ④ 已確認的韌體若連續 N 次開機（預設 10 次、跨度至少 24 小時，計數存 NVS）Wi-Fi 已拿到 IP 卻取不到 token：先依次試 NVS、出廠的後端網址；仍失敗且另一個槽可用，就切到另一個槽一次，並在下次連上時把本版本報為失敗 ⑤ 純斷網（拿不到 IP、路由器沒外網）不計入 ④ ⑥ 新網址的證書必須鏈到 CF_CA_bundle 裡的根（GTS Root R4、ISRG Root X1）；換主機或離開 Cloudflare 前先查證書鏈，runbook 寫明 ⑦ 只接受 https 的 backend_url 和 wss 的 voice_url，主機須在韌體內允許的網域後綴之下，防止後端被冒充時把板子引去別處</t>
+        </is>
+      </c>
+      <c r="L95" s="6" t="inlineStr">
+        <is>
+          <t>① 62:70（-localall）：後端環境變數把 voice_url 改到另一個端口的語音伺服器，重開機 → 連上新的，不需刷機 ② 把 voice_url 改成連不上的地址 → 退回 NVS 上次成功的值，照常對話 ③ backend_url 指向第二個本地後端 → 下次開機在新後端取 token 成功並替換；指向不存在的地址 → 繼續用舊的，對話不中斷 ④ 停掉後端、保留 Wi-Fi，把 N 臨時調小（例如 3 次、跨度 0）→ 第 N 次開機切到另一個槽，恢復後端後該版本被記為失敗 ⑤ 路由器拔掉外網線重開 N 次 → 不切槽 ⑥ 一塊雲端板上用同樣流程驗證 ①（改 elatoai 那套的 voice_url）⑦ 下發不在允許網域後綴之下的網址 → 韌體拒用並在序列埠提示</t>
+        </is>
+      </c>
+      <c r="M95" s="13" t="inlineStr">
+        <is>
+          <t>R-35</t>
+        </is>
+      </c>
+      <c r="P95" s="6" t="inlineStr">
+        <is>
+          <t>[2026-10-14] 新增
+[2026-10-14] 2026-10-14 用戶要求：日後改 FastAPI 網址，板子仍要能 OTA 並連上。① 後端改動可隨時部署；②–⑦ 的韌體部分必須在 11/27 交 Spotpear 的出廠映像之前完成，出廠後才加的話，已出貨的板子靠 OTA 也能拿到，但前提是當時的網址還連得上。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P94"/>
+  <autoFilter ref="A1:P95"/>
   <conditionalFormatting sqref="F2:F1000">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"已完成"</formula>
@@ -10776,7 +10868,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I299"/>
+  <dimension ref="A1:I301"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -21143,8 +21235,70 @@
         </is>
       </c>
     </row>
+    <row r="300" ht="46" customHeight="1">
+      <c r="A300" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 22:19</t>
+        </is>
+      </c>
+      <c r="B300" s="13" t="inlineStr">
+        <is>
+          <t>P2-22</t>
+        </is>
+      </c>
+      <c r="C300" s="6" t="inlineStr">
+        <is>
+          <t>改服務器網址也不失聯：語音網址由後端下發、後端網址可遷移、已確認韌體長期連不上時自救</t>
+        </is>
+      </c>
+      <c r="E300" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="I300" s="6" t="inlineStr">
+        <is>
+          <t>新增任務</t>
+        </is>
+      </c>
+    </row>
+    <row r="301" ht="102" customHeight="1">
+      <c r="A301" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14 22:19</t>
+        </is>
+      </c>
+      <c r="B301" s="13" t="inlineStr">
+        <is>
+          <t>P2-22</t>
+        </is>
+      </c>
+      <c r="C301" s="6" t="inlineStr">
+        <is>
+          <t>改服務器網址也不失聯：語音網址由後端下發、後端網址可遷移、已確認韌體長期連不上時自救</t>
+        </is>
+      </c>
+      <c r="D301" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E301" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="F301" s="13" t="n"/>
+      <c r="G301" s="6" t="n"/>
+      <c r="H301" s="13" t="n"/>
+      <c r="I301" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-14 用戶要求：日後改 FastAPI 網址，板子仍要能 OTA 並連上。① 後端改動可隨時部署；②–⑦ 的韌體部分必須在 11/27 交 Spotpear 的出廠映像之前完成，出廠後才加的話，已出貨的板子靠 OTA 也能拿到，但前提是當時的網址還連得上。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I299"/>
+  <autoFilter ref="A1:I301"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Track P2-22 as started: backend part passes, firmware part to do.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/production-readiness.xlsx
+++ b/docs/production-readiness.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'任務清單'!$A$1:$P$95</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'待確認問題'!$A$1:$G$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$301</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$303</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -665,7 +665,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>最後更新：2026-10-14 22:19　·　本頁由 tracker.py 自動生成，請勿手動編輯</t>
+          <t>最後更新：2026-10-15 09:15　·　本頁由 tracker.py 自動生成，請勿手動編輯</t>
         </is>
       </c>
     </row>
@@ -820,11 +820,11 @@
       </c>
       <c r="D8" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A8,'任務清單'!$F:$F,D$5)</f>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E8" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A8,'任務清單'!$F:$F,E$5)</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F8" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A8,'任務清單'!$F:$F,F$5)</f>
@@ -896,11 +896,11 @@
       </c>
       <c r="D10" s="5">
         <f>SUM(D6:D9)</f>
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E10" s="5">
         <f>SUM(E6:E9)</f>
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F10" s="5">
         <f>SUM(F6:F9)</f>
@@ -1063,11 +1063,11 @@
       </c>
       <c r="D15" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A15,'任務清單'!$F:$F,D$12)</f>
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E15" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A15,'任務清單'!$F:$F,E$12)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F15" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A15,'任務清單'!$F:$F,F$12)</f>
@@ -1139,11 +1139,11 @@
       </c>
       <c r="D17" s="5">
         <f>SUM(D13:D16)</f>
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E17" s="5">
         <f>SUM(E13:E16)</f>
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F17" s="5">
         <f>SUM(F13:F16)</f>
@@ -1708,15 +1708,15 @@
       <c r="H36" s="11" t="n"/>
       <c r="I36" s="12" t="n"/>
     </row>
-    <row r="37" ht="242" customHeight="1">
+    <row r="37" ht="409" customHeight="1">
       <c r="A37" s="13" t="inlineStr">
         <is>
-          <t>R-37</t>
+          <t>P2-22</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>網頁設定玩具的 Wi-Fi：查看、新增、刪除</t>
+          <t>改服務器網址也不失聯：語音網址由後端下發、後端網址可遷移、已確認韌體長期連不上時自救</t>
         </is>
       </c>
       <c r="C37" s="13" t="inlineStr">
@@ -1731,8 +1731,8 @@
       </c>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>上次測試：部分通過 — 模擬玩具經本機語音服務器＋網頁：status/scan/add/delete 正常；刪除目前 Wi-Fi → current 被拒；斷線 5 秒內頁面顯示睡著、按鈕停用；測試密碼在語音服務器日誌、網頁服務器日誌、資料庫均搜不到；用別人裝置 ID 重放 server action → forbidden；pytest 17 項通過（全套 230）；韌體 spotpear-ai-toy-localall 編譯通過（RAM 17.5%、Flash 75.9%）。未測：真機 ①② 及 OTA 推出
-① 設定頁顯示玩具在線／離線、目前 Wi-Fi 和訊號、已記住的 Wi-Fi 清單（只有名稱，不顯示密碼）② 在線時可新增 Wi-Fi（輸入或從玩具掃描到的清單選）、刪除 Wi-Fi；不能刪除正在使用的那個 ③ 經 /ws/esp32 轉送：伺服器先確認是設備主人；密碼不寫入資料庫、不寫入日誌 ④ 新增不切換網絡，目前 Wi-Fi 消失時才按訊號選；清單標示「連過／未連過」⑤ 上限 8 個 ⑥ 韌體改動經 OTA 推出</t>
+          <t>上次測試：部分通過 — 後端部分（分支 p2-22-server-urls）：node --test lib/deviceServerUrls.test.mjs 5/5、tsc 0 錯誤。worktree dev server 3222 + 本機 Supabase，兩塊假板（02:22:…:01/02）：已認領 200 帶 voice_url + backend_url；未認領 202 只帶 backend_url；DEVICE_VOICE_URL=ws://fastapi:7860/… → 不發、日誌記錯誤；兩個變數都不設 → 兩個欄位都不帶；生產值 → wss://elatoai.hkqft.com/fastapi/ws/esp32、https://elatoai.hkqft.com。測試數據已清除
+① /api/generate_auth_token 的回應帶 voice_url（wss 主機＋端口＋路徑，來自後端環境變數）；韌體用它連 /ws，並把最後一次成功的值存進 NVS；改 FastAPI 網址只改伺服器設定，不需新韌體 ② 回應沒有 voice_url（舊後端）或新網址連不上時，退回 NVS 上次成功的值，再退回出廠／編譯時的預設值 ③ 後端網址可遷移：回應可帶 backend_url；韌體先存為候選，下次開機用新網址取 token 成功才正式替換，失敗就繼續用舊網址；舊網址在遷移期內保持可用（runbook 寫明保留多久） ④ 已確認的韌體若連續 N 次開機（預設 10 次、跨度至少 24 小時，計數存 NVS）Wi-Fi 已拿到 IP 卻取不到 token：先依次試 NVS、出廠的後端網址；仍失敗且另一個槽可用，就切到另一個槽一次，並在下次連上時把本版本報為失敗 ⑤ 純斷網（拿不到 IP、路由器沒外網）不計入 ④ ⑥ 新網址的證書必須鏈到 CF_CA_bundle 裡的根（GTS Root R4、ISRG Root X1）；換主機或離開 Cloudflare 前先查證書鏈，runbook 寫明 ⑦ 只接受 https 的 backend_url 和 wss 的 voice_url，主機須在韌體內允許的網域後綴之下，防止後端被冒充時把板子引去別處</t>
         </is>
       </c>
       <c r="F37" s="11" t="n"/>
@@ -1740,30 +1740,31 @@
       <c r="H37" s="11" t="n"/>
       <c r="I37" s="12" t="n"/>
     </row>
-    <row r="38" ht="102" customHeight="1">
+    <row r="38" ht="242" customHeight="1">
       <c r="A38" s="13" t="inlineStr">
         <is>
-          <t>R-16</t>
+          <t>R-37</t>
         </is>
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>Spotpear 量產版加電池電壓檢測（GPIO0 分壓）</t>
+          <t>網頁設定玩具的 Wi-Fi：查看、新增、刪除</t>
         </is>
       </c>
       <c r="C38" s="13" t="inlineStr">
         <is>
-          <t>1 止血定案</t>
+          <t>3 封閉內測</t>
         </is>
       </c>
       <c r="D38" s="13" t="inlineStr">
         <is>
-          <t>未開始</t>
+          <t>進行中</t>
         </is>
       </c>
       <c r="E38" s="6" t="inlineStr">
         <is>
-          <t>Spotpear 書面確認量產版：GPIO1（屏幕 DC；本版不接屏幕，可空出來）接電芯正極（保護 IC 之後）100k/100k 分壓、100nF 濾波，屏幕不接該腳；GPIO0 保留給現有的 VDD 低電提醒；最好另把充電芯片 CHRG 接到 GPIO12 或 13。樣板到手後，固件讀到的電芯電壓與萬用表相差 ≤50mV，App（R-41）顯示百分比與充電中。</t>
+          <t>上次測試：部分通過 — 模擬玩具經本機語音服務器＋網頁：status/scan/add/delete 正常；刪除目前 Wi-Fi → current 被拒；斷線 5 秒內頁面顯示睡著、按鈕停用；測試密碼在語音服務器日誌、網頁服務器日誌、資料庫均搜不到；用別人裝置 ID 重放 server action → forbidden；pytest 17 項通過（全套 230）；韌體 spotpear-ai-toy-localall 編譯通過（RAM 17.5%、Flash 75.9%）。未測：真機 ①② 及 OTA 推出
+① 設定頁顯示玩具在線／離線、目前 Wi-Fi 和訊號、已記住的 Wi-Fi 清單（只有名稱，不顯示密碼）② 在線時可新增 Wi-Fi（輸入或從玩具掃描到的清單選）、刪除 Wi-Fi；不能刪除正在使用的那個 ③ 經 /ws/esp32 轉送：伺服器先確認是設備主人；密碼不寫入資料庫、不寫入日誌 ④ 新增不切換網絡，目前 Wi-Fi 消失時才按訊號選；清單標示「連過／未連過」⑤ 上限 8 個 ⑥ 韌體改動經 OTA 推出</t>
         </is>
       </c>
       <c r="F38" s="11" t="n"/>
@@ -1771,20 +1772,20 @@
       <c r="H38" s="11" t="n"/>
       <c r="I38" s="12" t="n"/>
     </row>
-    <row r="39" ht="46" customHeight="1">
+    <row r="39" ht="102" customHeight="1">
       <c r="A39" s="13" t="inlineStr">
         <is>
-          <t>P1-11</t>
+          <t>R-16</t>
         </is>
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>伺服器與資料庫直接存取的管控</t>
+          <t>Spotpear 量產版加電池電壓檢測（GPIO0 分壓）</t>
         </is>
       </c>
       <c r="C39" s="13" t="inlineStr">
         <is>
-          <t>2 內測準備</t>
+          <t>1 止血定案</t>
         </is>
       </c>
       <c r="D39" s="13" t="inlineStr">
@@ -1794,7 +1795,7 @@
       </c>
       <c r="E39" s="6" t="inlineStr">
         <is>
-          <t>列出誰有 SSH 與資料庫直連權限（越少越好）；service_role key 只存在伺服器的 env；私隱政策寫明這類存取的範圍；每次直接查看生產資料都留記錄。</t>
+          <t>Spotpear 書面確認量產版：GPIO1（屏幕 DC；本版不接屏幕，可空出來）接電芯正極（保護 IC 之後）100k/100k 分壓、100nF 濾波，屏幕不接該腳；GPIO0 保留給現有的 VDD 低電提醒；最好另把充電芯片 CHRG 接到 GPIO12 或 13。樣板到手後，固件讀到的電芯電壓與萬用表相差 ≤50mV，App（R-41）顯示百分比與充電中。</t>
         </is>
       </c>
       <c r="F39" s="11" t="n"/>
@@ -1805,12 +1806,12 @@
     <row r="40" ht="46" customHeight="1">
       <c r="A40" s="13" t="inlineStr">
         <is>
-          <t>P2-02</t>
+          <t>P1-11</t>
         </is>
       </c>
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>CI 跑測試與靜態檢查</t>
+          <t>伺服器與資料庫直接存取的管控</t>
         </is>
       </c>
       <c r="C40" s="13" t="inlineStr">
@@ -1825,7 +1826,7 @@
       </c>
       <c r="E40" s="6" t="inlineStr">
         <is>
-          <t>推送與 PR 時跑 pytest、ruff、pyright、next lint、tsc --noEmit、pio run；任何一項失敗就不發佈 image。</t>
+          <t>列出誰有 SSH 與資料庫直連權限（越少越好）；service_role key 只存在伺服器的 env；私隱政策寫明這類存取的範圍；每次直接查看生產資料都留記錄。</t>
         </is>
       </c>
       <c r="F40" s="11" t="n"/>
@@ -1833,15 +1834,15 @@
       <c r="H40" s="11" t="n"/>
       <c r="I40" s="12" t="n"/>
     </row>
-    <row r="41" ht="32" customHeight="1">
+    <row r="41" ht="46" customHeight="1">
       <c r="A41" s="13" t="inlineStr">
         <is>
-          <t>P2-04</t>
+          <t>P2-02</t>
         </is>
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>容器改用非 root 用戶</t>
+          <t>CI 跑測試與靜態檢查</t>
         </is>
       </c>
       <c r="C41" s="13" t="inlineStr">
@@ -1856,7 +1857,7 @@
       </c>
       <c r="E41" s="6" t="inlineStr">
         <is>
-          <t>兩個 Dockerfile 都設定非 root 的 USER。</t>
+          <t>推送與 PR 時跑 pytest、ruff、pyright、next lint、tsc --noEmit、pio run；任何一項失敗就不發佈 image。</t>
         </is>
       </c>
       <c r="F41" s="11" t="n"/>
@@ -1864,15 +1865,15 @@
       <c r="H41" s="11" t="n"/>
       <c r="I41" s="12" t="n"/>
     </row>
-    <row r="42" ht="46" customHeight="1">
+    <row r="42" ht="32" customHeight="1">
       <c r="A42" s="13" t="inlineStr">
         <is>
-          <t>R-04</t>
+          <t>P2-04</t>
         </is>
       </c>
       <c r="B42" s="6" t="inlineStr">
         <is>
-          <t>粵語質量評測</t>
+          <t>容器改用非 root 用戶</t>
         </is>
       </c>
       <c r="C42" s="13" t="inlineStr">
@@ -1887,7 +1888,7 @@
       </c>
       <c r="E42" s="6" t="inlineStr">
         <is>
-          <t>有一套粵語評測集（兒童錄音＋文字提示）；選定的 STT 與 LLM 達到門檻：兒童語音字錯率 ≤15%、口語粵語回覆 ≥90%、中英夾雜句能正確理解。</t>
+          <t>兩個 Dockerfile 都設定非 root 的 USER。</t>
         </is>
       </c>
       <c r="F42" s="11" t="n"/>
@@ -1895,15 +1896,15 @@
       <c r="H42" s="11" t="n"/>
       <c r="I42" s="12" t="n"/>
     </row>
-    <row r="43" ht="116" customHeight="1">
+    <row r="43" ht="46" customHeight="1">
       <c r="A43" s="13" t="inlineStr">
         <is>
-          <t>R-25</t>
+          <t>R-04</t>
         </is>
       </c>
       <c r="B43" s="6" t="inlineStr">
         <is>
-          <t>網頁的品牌主題系統</t>
+          <t>粵語質量評測</t>
         </is>
       </c>
       <c r="C43" s="13" t="inlineStr">
@@ -1918,7 +1919,7 @@
       </c>
       <c r="E43" s="6" t="inlineStr">
         <is>
-          <t>① 每個品牌一個資料夾：主題 token（顏色、字體、圓角）、logo 和圖示、文案、功能開關；首頁、上手流程、角色頁可以有品牌版本，其餘頁面共用 ② 由部署的環境變數選品牌（每套部署一個品牌，見 R-34），伺服器端渲染的第一屏就是對的主題，不閃爍 ③ 共用元件裡沒有品牌名稱和寫死的品牌顏色 ④ 加一個品牌只需要加資料夾、設定和一套部署，不用改共用元件</t>
+          <t>有一套粵語評測集（兒童錄音＋文字提示）；選定的 STT 與 LLM 達到門檻：兒童語音字錯率 ≤15%、口語粵語回覆 ≥90%、中英夾雜句能正確理解。</t>
         </is>
       </c>
       <c r="F43" s="11" t="n"/>
@@ -1926,68 +1927,68 @@
       <c r="H43" s="11" t="n"/>
       <c r="I43" s="12" t="n"/>
     </row>
-    <row r="45">
-      <c r="A45" s="10" t="inlineStr">
+    <row r="44" ht="116" customHeight="1">
+      <c r="A44" s="13" t="inlineStr">
+        <is>
+          <t>R-25</t>
+        </is>
+      </c>
+      <c r="B44" s="6" t="inlineStr">
+        <is>
+          <t>網頁的品牌主題系統</t>
+        </is>
+      </c>
+      <c r="C44" s="13" t="inlineStr">
+        <is>
+          <t>2 內測準備</t>
+        </is>
+      </c>
+      <c r="D44" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E44" s="6" t="inlineStr">
+        <is>
+          <t>① 每個品牌一個資料夾：主題 token（顏色、字體、圓角）、logo 和圖示、文案、功能開關；首頁、上手流程、角色頁可以有品牌版本，其餘頁面共用 ② 由部署的環境變數選品牌（每套部署一個品牌，見 R-34），伺服器端渲染的第一屏就是對的主題，不閃爍 ③ 共用元件裡沒有品牌名稱和寫死的品牌顏色 ④ 加一個品牌只需要加資料夾、設定和一套部署，不用改共用元件</t>
+        </is>
+      </c>
+      <c r="F44" s="11" t="n"/>
+      <c r="G44" s="11" t="n"/>
+      <c r="H44" s="11" t="n"/>
+      <c r="I44" s="12" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="10" t="inlineStr">
         <is>
           <t>✅ 最近完成與測試效果</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="4" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
         <is>
           <t>編號</t>
         </is>
       </c>
-      <c r="B46" s="4" t="inlineStr">
+      <c r="B47" s="4" t="inlineStr">
         <is>
           <t>任務</t>
         </is>
       </c>
-      <c r="C46" s="4" t="inlineStr">
+      <c r="C47" s="4" t="inlineStr">
         <is>
           <t>測試結果</t>
         </is>
       </c>
-      <c r="D46" s="4" t="inlineStr">
+      <c r="D47" s="4" t="inlineStr">
         <is>
           <t>完成日期</t>
         </is>
       </c>
-      <c r="E46" s="4" t="inlineStr">
+      <c r="E47" s="4" t="inlineStr">
         <is>
           <t>測試證據</t>
-        </is>
-      </c>
-      <c r="F46" s="11" t="n"/>
-      <c r="G46" s="11" t="n"/>
-      <c r="H46" s="11" t="n"/>
-      <c r="I46" s="12" t="n"/>
-    </row>
-    <row r="47" ht="214" customHeight="1">
-      <c r="A47" s="13" t="inlineStr">
-        <is>
-          <t>P2-20</t>
-        </is>
-      </c>
-      <c r="B47" s="6" t="inlineStr">
-        <is>
-          <t>P2-16 ④ 從後台上傳與發佈韌體（取代手貼 service key）</t>
-        </is>
-      </c>
-      <c r="C47" s="13" t="inlineStr">
-        <is>
-          <t>通過</t>
-        </is>
-      </c>
-      <c r="D47" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="E47" s="6" t="inlineStr">
-        <is>
-          <t>node --test lib/firmwareImage.test.mjs 8/8（合成映像：dev build、無標記、未知板、晶片不符、非映像、截斷/損壞、超 4MB 拒；超 2MB 只警告）。分支 dev server + 本機 Supabase 端到端 16/16（GoTrue 真實登入的 cookie）：超管上傳 9.9.0 release build → 201 草稿（is_current f、rollout 0%），DB SHA-256 = 檔案、storage 原樣；審計 insert 記該超管；設備仍只拿到 current 1.6.2；已有 1.0.2 → 409；localall → 422 dev build；4MB+16 → 422；9MB → 413；PNG → 422；舊 1.6.1 映像（無標記）→ 422 指向 release_firmware.py；內容管理員上傳/刪除 → 403；未登入 → 401；刪 current → 409；超管刪草稿 → 行和映像都刪、審計 delete 記該超管。release_firmware.py list 照常。測試帳號與數據已清除</t>
         </is>
       </c>
       <c r="F47" s="11" t="n"/>
@@ -1995,15 +1996,15 @@
       <c r="H47" s="11" t="n"/>
       <c r="I47" s="12" t="n"/>
     </row>
-    <row r="48" ht="158" customHeight="1">
+    <row r="48" ht="214" customHeight="1">
       <c r="A48" s="13" t="inlineStr">
         <is>
-          <t>P2-19</t>
+          <t>P2-20</t>
         </is>
       </c>
       <c r="B48" s="6" t="inlineStr">
         <is>
-          <t>P2-16 ③ 回滾過多時自動暫停推送</t>
+          <t>P2-16 ④ 從後台上傳與發佈韌體（取代手貼 service key）</t>
         </is>
       </c>
       <c r="C48" s="13" t="inlineStr">
@@ -2018,7 +2019,7 @@
       </c>
       <c r="E48" s="6" t="inlineStr">
         <is>
-          <t>migration 20261014200000 BEGIN/ROLLBACK 套用兩次無錯並已套用本機。模擬 20 台連跑兩次 12/12：1/20 回滾不暫停、其餘 18 台照常；2/20 → 'Auto-paused: 2 of 20 boards rolled back (10%)'，其餘 0 台拿到 ota；已運行的設備記為 running 且不再下發；審計 1 筆 actor 空；恢復後 17 台拿到、保持恢復，第 3 台回滾 → 'Auto-paused: 3 of 20 (15%)'；白名單 2 台中 1 台回滾 → 50% 立即暫停、另一台不再下發；anon 呼叫 ota_maybe_pause → 401/42501。測試數據已清除，spotpear-ai-toy 1.6.2 仍 100% 未暫停</t>
+          <t>node --test lib/firmwareImage.test.mjs 8/8（合成映像：dev build、無標記、未知板、晶片不符、非映像、截斷/損壞、超 4MB 拒；超 2MB 只警告）。分支 dev server + 本機 Supabase 端到端 16/16（GoTrue 真實登入的 cookie）：超管上傳 9.9.0 release build → 201 草稿（is_current f、rollout 0%），DB SHA-256 = 檔案、storage 原樣；審計 insert 記該超管；設備仍只拿到 current 1.6.2；已有 1.0.2 → 409；localall → 422 dev build；4MB+16 → 422；9MB → 413；PNG → 422；舊 1.6.1 映像（無標記）→ 422 指向 release_firmware.py；內容管理員上傳/刪除 → 403；未登入 → 401；刪 current → 409；超管刪草稿 → 行和映像都刪、審計 delete 記該超管。release_firmware.py list 照常。測試帳號與數據已清除</t>
         </is>
       </c>
       <c r="F48" s="11" t="n"/>
@@ -2026,15 +2027,15 @@
       <c r="H48" s="11" t="n"/>
       <c r="I48" s="12" t="n"/>
     </row>
-    <row r="49" ht="200" customHeight="1">
+    <row r="49" ht="158" customHeight="1">
       <c r="A49" s="13" t="inlineStr">
         <is>
-          <t>P2-18</t>
+          <t>P2-19</t>
         </is>
       </c>
       <c r="B49" s="6" t="inlineStr">
         <is>
-          <t>P2-16 ② 按 MAC 雜湊穩定分組決定哪台收到 ota</t>
+          <t>P2-16 ③ 回滾過多時自動暫停推送</t>
         </is>
       </c>
       <c r="C49" s="13" t="inlineStr">
@@ -2049,7 +2050,7 @@
       </c>
       <c r="E49" s="6" t="inlineStr">
         <is>
-          <t>node --test lib/otaRollout.test.mjs 6/6：10,000 隨機 MAC 在 10%/50% 誤差 &lt; 1 個百分點、同 MAC（含大小寫/空白）結果一致、升階段只增不減、白名單各階段都在、不同版本選不同的 10%。tsc --noEmit 通過。分支 dev server（3216）+ 本機 Supabase 模擬 20 台（板型 p218-sim，連跑兩次 9/9）：白名單階段只有 1 台、重複不變；10% 拿到的正是雜湊預測的那組（2–5 台含白名單），重複不變；50% 包含 10% 全部；暫停 → 0 台且下載映像 404，恢復 → 200；100% → 除已更新和已回滾的 2 台外 18 台；每台下發次數與記錄一致；運行中/已回滾正確標記；審計 6 筆對應 6 次變更。真 spotpear-ai-toy（預設 100%）回報 1.6.1 → 仍拿到 1.6.2。測試數據已清除</t>
+          <t>migration 20261014200000 BEGIN/ROLLBACK 套用兩次無錯並已套用本機。模擬 20 台連跑兩次 12/12：1/20 回滾不暫停、其餘 18 台照常；2/20 → 'Auto-paused: 2 of 20 boards rolled back (10%)'，其餘 0 台拿到 ota；已運行的設備記為 running 且不再下發；審計 1 筆 actor 空；恢復後 17 台拿到、保持恢復，第 3 台回滾 → 'Auto-paused: 3 of 20 (15%)'；白名單 2 台中 1 台回滾 → 50% 立即暫停、另一台不再下發；anon 呼叫 ota_maybe_pause → 401/42501。測試數據已清除，spotpear-ai-toy 1.6.2 仍 100% 未暫停</t>
         </is>
       </c>
       <c r="F49" s="11" t="n"/>
@@ -2057,15 +2058,15 @@
       <c r="H49" s="11" t="n"/>
       <c r="I49" s="12" t="n"/>
     </row>
-    <row r="50" ht="172" customHeight="1">
+    <row r="50" ht="200" customHeight="1">
       <c r="A50" s="13" t="inlineStr">
         <is>
-          <t>P2-17</t>
+          <t>P2-18</t>
         </is>
       </c>
       <c r="B50" s="6" t="inlineStr">
         <is>
-          <t>P2-16 ① 分批推送的數據表：推送階段、白名單、每台安裝結果</t>
+          <t>P2-16 ② 按 MAC 雜湊穩定分組決定哪台收到 ota</t>
         </is>
       </c>
       <c r="C50" s="13" t="inlineStr">
@@ -2080,7 +2081,7 @@
       </c>
       <c r="E50" s="6" t="inlineStr">
         <is>
-          <t>migration 20261014190000 BEGIN/ROLLBACK 套用兩次無錯並已套用本機；行為：預設 100%、promote 記 stage_changed_at，7 種壞值（25%、小寫/空字串/NULL MAC、暫停缺原因等）全被 check 擋；ota_note_offer 1→2→3，report 正確標 running/failed、別板型不影響，刪發佈連帶刪記錄；審計 5 筆含 'test-board 9.9.9' 標籤。REST 13/13：超管可讀、內容管理員 0 行、anon 42501，三種身份寫入/改階段/呼叫 ota_note_offer 皆 42501。release_firmware.py promote spotpear-ai-toy 1.6.2 成功，token 查詢仍選 1.6.2，審計記 2 筆（actor 空＝service role）</t>
+          <t>node --test lib/otaRollout.test.mjs 6/6：10,000 隨機 MAC 在 10%/50% 誤差 &lt; 1 個百分點、同 MAC（含大小寫/空白）結果一致、升階段只增不減、白名單各階段都在、不同版本選不同的 10%。tsc --noEmit 通過。分支 dev server（3216）+ 本機 Supabase 模擬 20 台（板型 p218-sim，連跑兩次 9/9）：白名單階段只有 1 台、重複不變；10% 拿到的正是雜湊預測的那組（2–5 台含白名單），重複不變；50% 包含 10% 全部；暫停 → 0 台且下載映像 404，恢復 → 200；100% → 除已更新和已回滾的 2 台外 18 台；每台下發次數與記錄一致；運行中/已回滾正確標記；審計 6 筆對應 6 次變更。真 spotpear-ai-toy（預設 100%）回報 1.6.1 → 仍拿到 1.6.2。測試數據已清除</t>
         </is>
       </c>
       <c r="F50" s="11" t="n"/>
@@ -2088,15 +2089,15 @@
       <c r="H50" s="11" t="n"/>
       <c r="I50" s="12" t="n"/>
     </row>
-    <row r="51" ht="116" customHeight="1">
+    <row r="51" ht="172" customHeight="1">
       <c r="A51" s="13" t="inlineStr">
         <is>
-          <t>R-41</t>
+          <t>P2-17</t>
         </is>
       </c>
       <c r="B51" s="6" t="inlineStr">
         <is>
-          <t>App 顯示玩具電量狀態（低電量提示）</t>
+          <t>P2-16 ① 分批推送的數據表：推送階段、白名單、每台安裝結果</t>
         </is>
       </c>
       <c r="C51" s="13" t="inlineStr">
@@ -2111,7 +2112,7 @@
       </c>
       <c r="E51" s="6" t="inlineStr">
         <is>
-          <t>① pytest 33 passed；真 PATCH 本地 Supabase ② 62:70 刷 p212+R-41 強制低電 build（SUPPLY_LOW_RATIO_OVERRIDE=1.05）→ 串口 [WSc] power low:true，本地 DB battery_low=t ③ 刷回正常 1.6.2 → low:false，DB=f ④ App 讀 DB：低電紅標+Please charge+更新時間、72% 充電中、未上報不顯示 ⑤ 他人帳號 0 行、authenticated UPDATE 被拒。62:70 已還原為原 p212 build</t>
+          <t>migration 20261014190000 BEGIN/ROLLBACK 套用兩次無錯並已套用本機；行為：預設 100%、promote 記 stage_changed_at，7 種壞值（25%、小寫/空字串/NULL MAC、暫停缺原因等）全被 check 擋；ota_note_offer 1→2→3，report 正確標 running/failed、別板型不影響，刪發佈連帶刪記錄；審計 5 筆含 'test-board 9.9.9' 標籤。REST 13/13：超管可讀、內容管理員 0 行、anon 42501，三種身份寫入/改階段/呼叫 ota_note_offer 皆 42501。release_firmware.py promote spotpear-ai-toy 1.6.2 成功，token 查詢仍選 1.6.2，審計記 2 筆（actor 空＝service role）</t>
         </is>
       </c>
       <c r="F51" s="11" t="n"/>
@@ -2119,15 +2120,15 @@
       <c r="H51" s="11" t="n"/>
       <c r="I51" s="12" t="n"/>
     </row>
-    <row r="52" ht="102" customHeight="1">
+    <row r="52" ht="116" customHeight="1">
       <c r="A52" s="13" t="inlineStr">
         <is>
-          <t>P0-12</t>
+          <t>R-41</t>
         </is>
       </c>
       <c r="B52" s="6" t="inlineStr">
         <is>
-          <t>收緊 Admin 權限與路由保護</t>
+          <t>App 顯示玩具電量狀態（低電量提示）</t>
         </is>
       </c>
       <c r="C52" s="13" t="inlineStr">
@@ -2137,12 +2138,12 @@
       </c>
       <c r="D52" s="13" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E52" s="6" t="inlineStr">
         <is>
-          <t>線上 2026-10-12（bac24e9）：runbook 10/08 檢查 未登入 /admin→/login、/api/admin→401、has_role() 只看角色、無管理員 policy 觸及 conversations/記憶表、超管≥1；未登入 /home、/admin→/login；用戶確認：家長帳號開 /admin 轉回 /home、管理員在 /admin 修改角色保存成功；角色細分權限沿用本機 61/61</t>
+          <t>① pytest 33 passed；真 PATCH 本地 Supabase ② 62:70 刷 p212+R-41 強制低電 build（SUPPLY_LOW_RATIO_OVERRIDE=1.05）→ 串口 [WSc] power low:true，本地 DB battery_low=t ③ 刷回正常 1.6.2 → low:false，DB=f ④ App 讀 DB：低電紅標+Please charge+更新時間、72% 充電中、未上報不顯示 ⑤ 他人帳號 0 行、authenticated UPDATE 被拒。62:70 已還原為原 p212 build</t>
         </is>
       </c>
       <c r="F52" s="11" t="n"/>
@@ -2150,15 +2151,15 @@
       <c r="H52" s="11" t="n"/>
       <c r="I52" s="12" t="n"/>
     </row>
-    <row r="53" ht="88" customHeight="1">
+    <row r="53" ht="102" customHeight="1">
       <c r="A53" s="13" t="inlineStr">
         <is>
-          <t>P0-15</t>
+          <t>P0-12</t>
         </is>
       </c>
       <c r="B53" s="6" t="inlineStr">
         <is>
-          <t>角色表權限：只有內容管理員能發佈，關閉家長自建角色</t>
+          <t>收緊 Admin 權限與路由保護</t>
         </is>
       </c>
       <c r="C53" s="13" t="inlineStr">
@@ -2173,7 +2174,7 @@
       </c>
       <c r="E53" s="6" t="inlineStr">
         <is>
-          <t>線上 2026-10-12：② anon 只見 6 個已發佈 hk_ 內建，查隱藏/醫生/家長自建 → []，anon POST → 401；① authenticated 寫入權限由 20261007140000 REVOKE（runbook 10/08 已套用）；用戶確認：④ 家長登入後 /home/create 轉回 /home ③ 管理員在 /admin 修改角色保存成功</t>
+          <t>線上 2026-10-12（bac24e9）：runbook 10/08 檢查 未登入 /admin→/login、/api/admin→401、has_role() 只看角色、無管理員 policy 觸及 conversations/記憶表、超管≥1；未登入 /home、/admin→/login；用戶確認：家長帳號開 /admin 轉回 /home、管理員在 /admin 修改角色保存成功；角色細分權限沿用本機 61/61</t>
         </is>
       </c>
       <c r="F53" s="11" t="n"/>
@@ -2184,12 +2185,12 @@
     <row r="54" ht="88" customHeight="1">
       <c r="A54" s="13" t="inlineStr">
         <is>
-          <t>P0-16</t>
+          <t>P0-15</t>
         </is>
       </c>
       <c r="B54" s="6" t="inlineStr">
         <is>
-          <t>移除「醫生」身份與寫死的通關碼</t>
+          <t>角色表權限：只有內容管理員能發佈，關閉家長自建角色</t>
         </is>
       </c>
       <c r="C54" s="13" t="inlineStr">
@@ -2204,7 +2205,7 @@
       </c>
       <c r="E54" s="6" t="inlineStr">
         <is>
-          <t>線上 2026-10-12：生產 commit bac24e9 git grep checkDoctorAction/kiwi-subtle-emu/=== "doctor"/isDoctor → 0；線上 13 個 JS（/、/login、/onboard）grep 通關碼/"doctor"/Santa/patient → 0；anon 讀角色只見 6 個 hk_ 角色、is_doctor 全 false；用戶今日線上登入及 playground 正常</t>
+          <t>線上 2026-10-12：② anon 只見 6 個已發佈 hk_ 內建，查隱藏/醫生/家長自建 → []，anon POST → 401；① authenticated 寫入權限由 20261007140000 REVOKE（runbook 10/08 已套用）；用戶確認：④ 家長登入後 /home/create 轉回 /home ③ 管理員在 /admin 修改角色保存成功</t>
         </is>
       </c>
       <c r="F54" s="11" t="n"/>
@@ -2212,50 +2213,58 @@
       <c r="H54" s="11" t="n"/>
       <c r="I54" s="12" t="n"/>
     </row>
-    <row r="56">
-      <c r="A56" s="10" t="inlineStr">
+    <row r="55" ht="88" customHeight="1">
+      <c r="A55" s="13" t="inlineStr">
+        <is>
+          <t>P0-16</t>
+        </is>
+      </c>
+      <c r="B55" s="6" t="inlineStr">
+        <is>
+          <t>移除「醫生」身份與寫死的通關碼</t>
+        </is>
+      </c>
+      <c r="C55" s="13" t="inlineStr">
+        <is>
+          <t>通過</t>
+        </is>
+      </c>
+      <c r="D55" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="E55" s="6" t="inlineStr">
+        <is>
+          <t>線上 2026-10-12：生產 commit bac24e9 git grep checkDoctorAction/kiwi-subtle-emu/=== "doctor"/isDoctor → 0；線上 13 個 JS（/、/login、/onboard）grep 通關碼/"doctor"/Santa/patient → 0；anon 讀角色只見 6 個 hk_ 角色、is_doctor 全 false；用戶今日線上登入及 playground 正常</t>
+        </is>
+      </c>
+      <c r="F55" s="11" t="n"/>
+      <c r="G55" s="11" t="n"/>
+      <c r="H55" s="11" t="n"/>
+      <c r="I55" s="12" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="10" t="inlineStr">
         <is>
           <t>⏳ 等待依賴 / ⛔ 阻塞</t>
         </is>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="4" t="inlineStr">
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
         <is>
           <t>編號</t>
         </is>
       </c>
-      <c r="B57" s="4" t="inlineStr">
+      <c r="B58" s="4" t="inlineStr">
         <is>
           <t>任務</t>
         </is>
       </c>
-      <c r="C57" s="4" t="inlineStr">
+      <c r="C58" s="4" t="inlineStr">
         <is>
           <t>在等什麼</t>
-        </is>
-      </c>
-      <c r="D57" s="11" t="n"/>
-      <c r="E57" s="11" t="n"/>
-      <c r="F57" s="11" t="n"/>
-      <c r="G57" s="11" t="n"/>
-      <c r="H57" s="11" t="n"/>
-      <c r="I57" s="12" t="n"/>
-    </row>
-    <row r="58" ht="88" customHeight="1">
-      <c r="A58" s="13" t="inlineStr">
-        <is>
-          <t>R-17</t>
-        </is>
-      </c>
-      <c r="B58" s="6" t="inlineStr">
-        <is>
-          <t>Spotpear 電池耗盡時插電能否正常開機（供電路徑）</t>
-        </is>
-      </c>
-      <c r="C58" s="6" t="inlineStr">
-        <is>
-          <t>阻塞：[2026-10-08] 2026-10-08 開發板 63:64 插著 USB 時兩次無法解釋的完全斷電重開：09:13:26（崩潰循環中）、10:44:33（閒置、用戶確認沒碰）。都是 USB 先斷線再以 ESP_RST_POWERON 開機，非 brownout；斷電前 6 秒 GPIO0 讀數 99.9% 參考值，屬突然切斷而非緩降（SupplyMonitor 取樣太疏抓不到瞬間）。韌體無法造成 POWERON，指向充電芯片/電池保護/供電路徑，應一併問 Spotpear；放電實測時留意插 USB 閒置時是否也會斷電</t>
         </is>
       </c>
       <c r="D58" s="11" t="n"/>
@@ -2265,20 +2274,20 @@
       <c r="H58" s="11" t="n"/>
       <c r="I58" s="12" t="n"/>
     </row>
-    <row r="59" ht="60" customHeight="1">
+    <row r="59" ht="88" customHeight="1">
       <c r="A59" s="13" t="inlineStr">
         <is>
-          <t>P1-01</t>
+          <t>R-17</t>
         </is>
       </c>
       <c r="B59" s="6" t="inlineStr">
         <is>
-          <t>加入內容審核層（輸入與輸出）</t>
+          <t>Spotpear 電池耗盡時插電能否正常開機（供電路徑）</t>
         </is>
       </c>
       <c r="C59" s="6" t="inlineStr">
         <is>
-          <t>阻塞：[2026-10-14] 2026-10-14 用戶決定：先不定審核服務商，本項暫停。候選：Azure Content Safety（建議，香港區、可在每句回覆說出口前檢查）、OpenRouter 安全模型、OpenAI Moderation、只用本機字詞表。未寫任何程式。</t>
+          <t>阻塞：[2026-10-08] 2026-10-08 開發板 63:64 插著 USB 時兩次無法解釋的完全斷電重開：09:13:26（崩潰循環中）、10:44:33（閒置、用戶確認沒碰）。都是 USB 先斷線再以 ESP_RST_POWERON 開機，非 brownout；斷電前 6 秒 GPIO0 讀數 99.9% 參考值，屬突然切斷而非緩降（SupplyMonitor 取樣太疏抓不到瞬間）。韌體無法造成 POWERON，指向充電芯片/電池保護/供電路徑，應一併問 Spotpear；放電實測時留意插 USB 閒置時是否也會斷電</t>
         </is>
       </c>
       <c r="D59" s="11" t="n"/>
@@ -2288,20 +2297,20 @@
       <c r="H59" s="11" t="n"/>
       <c r="I59" s="12" t="n"/>
     </row>
-    <row r="60" ht="32" customHeight="1">
+    <row r="60" ht="60" customHeight="1">
       <c r="A60" s="13" t="inlineStr">
         <is>
-          <t>P1-09</t>
+          <t>P1-01</t>
         </is>
       </c>
       <c r="B60" s="6" t="inlineStr">
         <is>
-          <t>家長鎖：孩子模式進設定要輸入 PIN</t>
+          <t>加入內容審核層（輸入與輸出）</t>
         </is>
       </c>
       <c r="C60" s="6" t="inlineStr">
         <is>
-          <t>阻塞：[2026-10-13] 2026-10-13 用戶決定：AI Buddy（品牌 C）延到 1/15 之後，本項不卡 1/15 出廠；AI Buddy 啟動時再開。</t>
+          <t>阻塞：[2026-10-14] 2026-10-14 用戶決定：先不定審核服務商，本項暫停。候選：Azure Content Safety（建議，香港區、可在每句回覆說出口前檢查）、OpenRouter 安全模型、OpenAI Moderation、只用本機字詞表。未寫任何程式。</t>
         </is>
       </c>
       <c r="D60" s="11" t="n"/>
@@ -2314,12 +2323,12 @@
     <row r="61" ht="32" customHeight="1">
       <c r="A61" s="13" t="inlineStr">
         <is>
-          <t>R-12</t>
+          <t>P1-09</t>
         </is>
       </c>
       <c r="B61" s="6" t="inlineStr">
         <is>
-          <t>家長控制：每日使用上限和休息時段</t>
+          <t>家長鎖：孩子模式進設定要輸入 PIN</t>
         </is>
       </c>
       <c r="C61" s="6" t="inlineStr">
@@ -2337,12 +2346,12 @@
     <row r="62" ht="32" customHeight="1">
       <c r="A62" s="13" t="inlineStr">
         <is>
-          <t>R-29</t>
+          <t>R-12</t>
         </is>
       </c>
       <c r="B62" s="6" t="inlineStr">
         <is>
-          <t>AI Buddy App（品牌 C）頁面</t>
+          <t>家長控制：每日使用上限和休息時段</t>
         </is>
       </c>
       <c r="C62" s="6" t="inlineStr">
@@ -2357,20 +2366,20 @@
       <c r="H62" s="11" t="n"/>
       <c r="I62" s="12" t="n"/>
     </row>
-    <row r="63" ht="18" customHeight="1">
+    <row r="63" ht="32" customHeight="1">
       <c r="A63" s="13" t="inlineStr">
         <is>
-          <t>R-05</t>
+          <t>R-29</t>
         </is>
       </c>
       <c r="B63" s="6" t="inlineStr">
         <is>
-          <t>內測版外殼（3D 打印 20 台）</t>
+          <t>AI Buddy App（品牌 C）頁面</t>
         </is>
       </c>
       <c r="C63" s="6" t="inlineStr">
         <is>
-          <t>等 R-01</t>
+          <t>阻塞：[2026-10-13] 2026-10-13 用戶決定：AI Buddy（品牌 C）延到 1/15 之後，本項不卡 1/15 出廠；AI Buddy 啟動時再開。</t>
         </is>
       </c>
       <c r="D63" s="11" t="n"/>
@@ -2383,17 +2392,17 @@
     <row r="64" ht="18" customHeight="1">
       <c r="A64" s="13" t="inlineStr">
         <is>
-          <t>R-06</t>
+          <t>R-05</t>
         </is>
       </c>
       <c r="B64" s="6" t="inlineStr">
         <is>
-          <t>家長自助上手流程</t>
+          <t>內測版外殼（3D 打印 20 台）</t>
         </is>
       </c>
       <c r="C64" s="6" t="inlineStr">
         <is>
-          <t>等 P0-11</t>
+          <t>等 R-01</t>
         </is>
       </c>
       <c r="D64" s="11" t="n"/>
@@ -2403,20 +2412,20 @@
       <c r="H64" s="11" t="n"/>
       <c r="I64" s="12" t="n"/>
     </row>
-    <row r="65" ht="32" customHeight="1">
+    <row r="65" ht="18" customHeight="1">
       <c r="A65" s="13" t="inlineStr">
         <is>
-          <t>R-13</t>
+          <t>R-06</t>
         </is>
       </c>
       <c r="B65" s="6" t="inlineStr">
         <is>
-          <t>CP1 內測就緒檢查（10/30）</t>
+          <t>家長自助上手流程</t>
         </is>
       </c>
       <c r="C65" s="6" t="inlineStr">
         <is>
-          <t>等 P0-07、P0-11、P1-01、P1-02、P2-09、R-01、R-02、R-04、R-05、R-06、P1-11</t>
+          <t>等 P0-11</t>
         </is>
       </c>
       <c r="D65" s="11" t="n"/>
@@ -2429,17 +2438,17 @@
     <row r="66" ht="32" customHeight="1">
       <c r="A66" s="13" t="inlineStr">
         <is>
-          <t>R-18</t>
+          <t>R-13</t>
         </is>
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
-          <t>長按 BOOT 重新配網（開 AIBuddy-XXXX 熱點）</t>
+          <t>CP1 內測就緒檢查（10/30）</t>
         </is>
       </c>
       <c r="C66" s="6" t="inlineStr">
         <is>
-          <t>等 R-01</t>
+          <t>等 P0-07、P0-11、P1-01、P1-02、P2-09、R-01、R-02、R-04、R-05、R-06、P1-11</t>
         </is>
       </c>
       <c r="D66" s="11" t="n"/>
@@ -2452,12 +2461,12 @@
     <row r="67" ht="32" customHeight="1">
       <c r="A67" s="13" t="inlineStr">
         <is>
-          <t>R-19</t>
+          <t>R-18</t>
         </is>
       </c>
       <c r="B67" s="6" t="inlineStr">
         <is>
-          <t>外接按鈕：量產板加 I2C 擴展晶片（TCA9555）</t>
+          <t>長按 BOOT 重新配網（開 AIBuddy-XXXX 熱點）</t>
         </is>
       </c>
       <c r="C67" s="6" t="inlineStr">
@@ -2472,20 +2481,20 @@
       <c r="H67" s="11" t="n"/>
       <c r="I67" s="12" t="n"/>
     </row>
-    <row r="68" ht="18" customHeight="1">
+    <row r="68" ht="32" customHeight="1">
       <c r="A68" s="13" t="inlineStr">
         <is>
-          <t>R-20</t>
+          <t>R-19</t>
         </is>
       </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t>孩子資料與角色改成每台設備一份</t>
+          <t>外接按鈕：量產板加 I2C 擴展晶片（TCA9555）</t>
         </is>
       </c>
       <c r="C68" s="6" t="inlineStr">
         <is>
-          <t>等 P1-12</t>
+          <t>等 R-01</t>
         </is>
       </c>
       <c r="D68" s="11" t="n"/>
@@ -2495,20 +2504,20 @@
       <c r="H68" s="11" t="n"/>
       <c r="I68" s="12" t="n"/>
     </row>
-    <row r="69" ht="32" customHeight="1">
+    <row r="69" ht="18" customHeight="1">
       <c r="A69" s="13" t="inlineStr">
         <is>
-          <t>R-27</t>
+          <t>R-20</t>
         </is>
       </c>
       <c r="B69" s="6" t="inlineStr">
         <is>
-          <t>App 內登入：驗證碼、原生社交登入、刪除帳號</t>
+          <t>孩子資料與角色改成每台設備一份</t>
         </is>
       </c>
       <c r="C69" s="6" t="inlineStr">
         <is>
-          <t>等 R-26</t>
+          <t>等 P1-12</t>
         </is>
       </c>
       <c r="D69" s="11" t="n"/>
@@ -2518,20 +2527,20 @@
       <c r="H69" s="11" t="n"/>
       <c r="I69" s="12" t="n"/>
     </row>
-    <row r="70" ht="18" customHeight="1">
+    <row r="70" ht="32" customHeight="1">
       <c r="A70" s="13" t="inlineStr">
         <is>
-          <t>P0-14</t>
+          <t>R-27</t>
         </is>
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>韌體簽章、Secure Boot 與 Flash 加密</t>
+          <t>App 內登入：驗證碼、原生社交登入、刪除帳號</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr">
         <is>
-          <t>等 R-01</t>
+          <t>等 R-26</t>
         </is>
       </c>
       <c r="D70" s="11" t="n"/>
@@ -2544,17 +2553,17 @@
     <row r="71" ht="18" customHeight="1">
       <c r="A71" s="13" t="inlineStr">
         <is>
-          <t>P1-06</t>
+          <t>P0-14</t>
         </is>
       </c>
       <c r="B71" s="6" t="inlineStr">
         <is>
-          <t>處理 GPL-3.0 依賴（arduino-audio-tools）</t>
+          <t>韌體簽章、Secure Boot 與 Flash 加密</t>
         </is>
       </c>
       <c r="C71" s="6" t="inlineStr">
         <is>
-          <t>等 Q3</t>
+          <t>等 R-01</t>
         </is>
       </c>
       <c r="D71" s="11" t="n"/>
@@ -2567,12 +2576,12 @@
     <row r="72" ht="18" customHeight="1">
       <c r="A72" s="13" t="inlineStr">
         <is>
-          <t>P1-07</t>
+          <t>P1-06</t>
         </is>
       </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>LGPL 合規與第三方授權聲明</t>
+          <t>處理 GPL-3.0 依賴（arduino-audio-tools）</t>
         </is>
       </c>
       <c r="C72" s="6" t="inlineStr">
@@ -2590,17 +2599,17 @@
     <row r="73" ht="18" customHeight="1">
       <c r="A73" s="13" t="inlineStr">
         <is>
-          <t>P1-08</t>
+          <t>P1-07</t>
         </is>
       </c>
       <c r="B73" s="6" t="inlineStr">
         <is>
-          <t>硬件認證</t>
+          <t>LGPL 合規與第三方授權聲明</t>
         </is>
       </c>
       <c r="C73" s="6" t="inlineStr">
         <is>
-          <t>等 R-01、R-05</t>
+          <t>等 Q3</t>
         </is>
       </c>
       <c r="D73" s="11" t="n"/>
@@ -2613,17 +2622,17 @@
     <row r="74" ht="18" customHeight="1">
       <c r="A74" s="13" t="inlineStr">
         <is>
-          <t>P1-14</t>
+          <t>P1-08</t>
         </is>
       </c>
       <c r="B74" s="6" t="inlineStr">
         <is>
-          <t>Admin 內容安全頁：審核事件只按類別統計</t>
+          <t>硬件認證</t>
         </is>
       </c>
       <c r="C74" s="6" t="inlineStr">
         <is>
-          <t>等 P1-01、P2-13</t>
+          <t>等 R-01、R-05</t>
         </is>
       </c>
       <c r="D74" s="11" t="n"/>
@@ -2633,20 +2642,20 @@
       <c r="H74" s="11" t="n"/>
       <c r="I74" s="12" t="n"/>
     </row>
-    <row r="75" ht="32" customHeight="1">
+    <row r="75" ht="18" customHeight="1">
       <c r="A75" s="13" t="inlineStr">
         <is>
-          <t>P2-15</t>
+          <t>P1-14</t>
         </is>
       </c>
       <c r="B75" s="6" t="inlineStr">
         <is>
-          <t>Admin 總覽頁：在線、用量、成本與待處理事項</t>
+          <t>Admin 內容安全頁：審核事件只按類別統計</t>
         </is>
       </c>
       <c r="C75" s="6" t="inlineStr">
         <is>
-          <t>等 P2-14、P2-09</t>
+          <t>等 P1-01、P2-13</t>
         </is>
       </c>
       <c r="D75" s="11" t="n"/>
@@ -2656,20 +2665,20 @@
       <c r="H75" s="11" t="n"/>
       <c r="I75" s="12" t="n"/>
     </row>
-    <row r="76" ht="46" customHeight="1">
+    <row r="76" ht="32" customHeight="1">
       <c r="A76" s="13" t="inlineStr">
         <is>
-          <t>P2-22</t>
+          <t>P2-15</t>
         </is>
       </c>
       <c r="B76" s="6" t="inlineStr">
         <is>
-          <t>改服務器網址也不失聯：語音網址由後端下發、後端網址可遷移、已確認韌體長期連不上時自救</t>
+          <t>Admin 總覽頁：在線、用量、成本與待處理事項</t>
         </is>
       </c>
       <c r="C76" s="6" t="inlineStr">
         <is>
-          <t>等 R-35</t>
+          <t>等 P2-14、P2-09</t>
         </is>
       </c>
       <c r="D76" s="11" t="n"/>
@@ -3213,9 +3222,9 @@
     </row>
   </sheetData>
   <mergeCells count="87">
+    <mergeCell ref="E55:I55"/>
     <mergeCell ref="C82:I82"/>
     <mergeCell ref="E52:I52"/>
-    <mergeCell ref="A56:I56"/>
     <mergeCell ref="E39:I39"/>
     <mergeCell ref="C67:I67"/>
     <mergeCell ref="E48:I48"/>
@@ -3236,11 +3245,12 @@
     <mergeCell ref="C60:I60"/>
     <mergeCell ref="C71:I71"/>
     <mergeCell ref="E50:I50"/>
+    <mergeCell ref="A46:I46"/>
     <mergeCell ref="E42:I42"/>
     <mergeCell ref="C91:I91"/>
     <mergeCell ref="A105:I105"/>
-    <mergeCell ref="C57:I57"/>
     <mergeCell ref="C66:I66"/>
+    <mergeCell ref="E44:I44"/>
     <mergeCell ref="E20:I20"/>
     <mergeCell ref="E28:I28"/>
     <mergeCell ref="C77:I77"/>
@@ -3249,7 +3259,6 @@
     <mergeCell ref="C58:I58"/>
     <mergeCell ref="E30:I30"/>
     <mergeCell ref="E22:I22"/>
-    <mergeCell ref="E46:I46"/>
     <mergeCell ref="A102:I102"/>
     <mergeCell ref="C85:I85"/>
     <mergeCell ref="C65:I65"/>
@@ -3261,7 +3270,6 @@
     <mergeCell ref="C59:I59"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="E41:I41"/>
-    <mergeCell ref="A45:I45"/>
     <mergeCell ref="A94:I94"/>
     <mergeCell ref="E47:I47"/>
     <mergeCell ref="C61:I61"/>
@@ -3271,6 +3279,7 @@
     <mergeCell ref="E33:I33"/>
     <mergeCell ref="A3:I3"/>
     <mergeCell ref="A104:I104"/>
+    <mergeCell ref="A57:I57"/>
     <mergeCell ref="E35:I35"/>
     <mergeCell ref="A106:I106"/>
     <mergeCell ref="C74:I74"/>
@@ -10246,12 +10255,12 @@
       </c>
       <c r="F95" s="13" t="inlineStr">
         <is>
-          <t>未開始</t>
+          <t>進行中</t>
         </is>
       </c>
       <c r="G95" s="13" t="inlineStr">
         <is>
-          <t>未測試</t>
+          <t>部分通過</t>
         </is>
       </c>
       <c r="I95" s="6" t="inlineStr">
@@ -10279,10 +10288,21 @@
           <t>R-35</t>
         </is>
       </c>
+      <c r="N95" s="6" t="inlineStr">
+        <is>
+          <t>後端部分（分支 p2-22-server-urls）：node --test lib/deviceServerUrls.test.mjs 5/5、tsc 0 錯誤。worktree dev server 3222 + 本機 Supabase，兩塊假板（02:22:…:01/02）：已認領 200 帶 voice_url + backend_url；未認領 202 只帶 backend_url；DEVICE_VOICE_URL=ws://fastapi:7860/… → 不發、日誌記錯誤；兩個變數都不設 → 兩個欄位都不帶；生產值 → wss://elatoai.hkqft.com/fastapi/ws/esp32、https://elatoai.hkqft.com。測試數據已清除</t>
+        </is>
+      </c>
+      <c r="O95" s="13" t="inlineStr">
+        <is>
+          <t>c0f0e29</t>
+        </is>
+      </c>
       <c r="P95" s="6" t="inlineStr">
         <is>
           <t>[2026-10-14] 新增
-[2026-10-14] 2026-10-14 用戶要求：日後改 FastAPI 網址，板子仍要能 OTA 並連上。① 後端改動可隨時部署；②–⑦ 的韌體部分必須在 11/27 交 Spotpear 的出廠映像之前完成，出廠後才加的話，已出貨的板子靠 OTA 也能拿到，但前提是當時的網址還連得上。</t>
+[2026-10-14] 2026-10-14 用戶要求：日後改 FastAPI 網址，板子仍要能 OTA 並連上。① 後端改動可隨時部署；②–⑦ 的韌體部分必須在 11/27 交 Spotpear 的出廠映像之前完成，出廠後才加的話，已出貨的板子靠 OTA 也能拿到，但前提是當時的網址還連得上。
+[2026-10-15] 未完成：韌體部分（①② 使用 voice_url 並在 NVS 記上次成功的值、③ 候選 backend_url、④⑤ 連續 10 次開機連不上就切槽、⑦ 允許的網域後綴）未開始，要用 62:70 實機測；runbook（③ 舊網址保留多久、⑥ 證書鏈檢查）未寫。部署：.env.production 加 DEVICE_VOICE_URL、DEVICE_BACKEND_URL；舊韌體會忽略這兩個欄位，可以先上後端。分支未合併 dev、未推送</t>
         </is>
       </c>
     </row>
@@ -10868,7 +10888,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I301"/>
+  <dimension ref="A1:I303"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -21297,8 +21317,86 @@
         </is>
       </c>
     </row>
+    <row r="302" ht="46" customHeight="1">
+      <c r="A302" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-15 09:15</t>
+        </is>
+      </c>
+      <c r="B302" s="13" t="inlineStr">
+        <is>
+          <t>P2-22</t>
+        </is>
+      </c>
+      <c r="C302" s="6" t="inlineStr">
+        <is>
+          <t>改服務器網址也不失聯：語音網址由後端下發、後端網址可遷移、已確認韌體長期連不上時自救</t>
+        </is>
+      </c>
+      <c r="D302" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E302" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F302" s="13" t="n"/>
+      <c r="G302" s="6" t="n"/>
+      <c r="H302" s="13" t="n"/>
+      <c r="I302" s="6" t="n"/>
+    </row>
+    <row r="303" ht="144" customHeight="1">
+      <c r="A303" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-15 09:15</t>
+        </is>
+      </c>
+      <c r="B303" s="13" t="inlineStr">
+        <is>
+          <t>P2-22</t>
+        </is>
+      </c>
+      <c r="C303" s="6" t="inlineStr">
+        <is>
+          <t>改服務器網址也不失聯：語音網址由後端下發、後端網址可遷移、已確認韌體長期連不上時自救</t>
+        </is>
+      </c>
+      <c r="D303" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="E303" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F303" s="13" t="inlineStr">
+        <is>
+          <t>部分通過</t>
+        </is>
+      </c>
+      <c r="G303" s="6" t="inlineStr">
+        <is>
+          <t>後端部分（分支 p2-22-server-urls）：node --test lib/deviceServerUrls.test.mjs 5/5、tsc 0 錯誤。worktree dev server 3222 + 本機 Supabase，兩塊假板（02:22:…:01/02）：已認領 200 帶 voice_url + backend_url；未認領 202 只帶 backend_url；DEVICE_VOICE_URL=ws://fastapi:7860/… → 不發、日誌記錯誤；兩個變數都不設 → 兩個欄位都不帶；生產值 → wss://elatoai.hkqft.com/fastapi/ws/esp32、https://elatoai.hkqft.com。測試數據已清除</t>
+        </is>
+      </c>
+      <c r="H303" s="13" t="inlineStr">
+        <is>
+          <t>c0f0e29</t>
+        </is>
+      </c>
+      <c r="I303" s="6" t="inlineStr">
+        <is>
+          <t>未完成：韌體部分（①② 使用 voice_url 並在 NVS 記上次成功的值、③ 候選 backend_url、④⑤ 連續 10 次開機連不上就切槽、⑦ 允許的網域後綴）未開始，要用 62:70 實機測；runbook（③ 舊網址保留多久、⑥ 證書鏈檢查）未寫。部署：.env.production 加 DEVICE_VOICE_URL、DEVICE_BACKEND_URL；舊韌體會忽略這兩個欄位，可以先上後端。分支未合併 dev、未推送</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I301"/>
+  <autoFilter ref="A1:I303"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Track the 62:70 hardware run: P2-14, P2-16, P2-21 pass; R-36 partly.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/production-readiness.xlsx
+++ b/docs/production-readiness.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'任務清單'!$A$1:$P$95</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'待確認問題'!$A$1:$G$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$303</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$307</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -641,7 +641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I106"/>
+  <dimension ref="A1:I103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -665,14 +665,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>最後更新：2026-10-15 09:15　·　本頁由 tracker.py 自動生成，請勿手動編輯</t>
+          <t>最後更新：2026-10-15 09:48　·　本頁由 tracker.py 自動生成，請勿手動編輯</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>總進度：22/90 已完成（24%）　·　目前階段：1 止血定案（10/5–10/16）</t>
+          <t>總進度：25/90 已完成（28%）　·　目前階段：1 止血定案（10/5–10/16）</t>
         </is>
       </c>
     </row>
@@ -824,11 +824,11 @@
       </c>
       <c r="E8" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A8,'任務清單'!$F:$F,E$5)</f>
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="F8" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A8,'任務清單'!$F:$F,F$5)</f>
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="G8" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A8,'任務清單'!$F:$F,G$5)</f>
@@ -840,7 +840,7 @@
       </c>
       <c r="I8" s="8">
         <f>IFERROR(F8/(C8-H8),0)</f>
-        <v>0.3181818181818182</v>
+        <v>0.45454545454545453</v>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1">
@@ -900,11 +900,11 @@
       </c>
       <c r="E10" s="5">
         <f>SUM(E6:E9)</f>
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="F10" s="5">
         <f>SUM(F6:F9)</f>
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="G10" s="5">
         <f>SUM(G6:G9)</f>
@@ -916,7 +916,7 @@
       </c>
       <c r="I10" s="9">
         <f>IFERROR(F10/(C10-H10),0)</f>
-        <v>0.24444444444444444</v>
+        <v>0.2777777777777778</v>
       </c>
     </row>
     <row r="12">
@@ -1027,11 +1027,11 @@
       </c>
       <c r="E14" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A14,'任務清單'!$F:$F,E$12)</f>
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="F14" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A14,'任務清單'!$F:$F,F$12)</f>
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="G14" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A14,'任務清單'!$F:$F,G$12)</f>
@@ -1043,7 +1043,7 @@
       </c>
       <c r="I14" s="8">
         <f>IFERROR(F14/(C14-H14),0)</f>
-        <v>0.21212121212121213</v>
+        <v>0.30303030303030304</v>
       </c>
     </row>
     <row r="15" ht="46" customHeight="1">
@@ -1143,11 +1143,11 @@
       </c>
       <c r="E17" s="5">
         <f>SUM(E13:E16)</f>
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="F17" s="5">
         <f>SUM(F13:F16)</f>
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="G17" s="5">
         <f>SUM(G13:G16)</f>
@@ -1159,7 +1159,7 @@
       </c>
       <c r="I17" s="9">
         <f>IFERROR(F17/(C17-H17),0)</f>
-        <v>0.24444444444444444</v>
+        <v>0.2777777777777778</v>
       </c>
     </row>
     <row r="19">
@@ -1518,15 +1518,15 @@
       <c r="H30" s="11" t="n"/>
       <c r="I30" s="12" t="n"/>
     </row>
-    <row r="31" ht="298" customHeight="1">
+    <row r="31" ht="200" customHeight="1">
       <c r="A31" s="13" t="inlineStr">
         <is>
-          <t>P2-14</t>
+          <t>R-21</t>
         </is>
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>Admin 設備頁：每台玩具的狀態、韌體與基本操作</t>
+          <t>藍牙配網與綁定（取代熱點配網）</t>
         </is>
       </c>
       <c r="C31" s="13" t="inlineStr">
@@ -1541,8 +1541,7 @@
       </c>
       <c r="E31" s="6" t="inlineStr">
         <is>
-          <t>上次測試：部分通過 — 本機（未 commit）：migration 20261014140000 套用兩次無錯。探測腳本用 GoTrue 真實登入：超管 admin_list_devices 200（不含 user_code）；④ 內容管理員 → 42501、anon → 42501；超管直接讀 device_secrets → 42501；空原因 → 22023；重置密鑰 → device_secrets 行刪除；解綁 → user_id/claimed_at 清空；兩者各寫 1 筆含原因與前後值的審計，超管改審計 → 403。網頁（獨立副本+獨立語音伺服器 7871）：模擬 62:70 連上 → 15 秒內不刷新顯示 Online、-52 dBm；斷線後下一次輪詢變 Offline；按 f214 搜尋、強制解綁、重置密鑰、審計頁都看到兩筆；375px 無橫向捲動。pytest 71 passed。未做：① ② ③ 需真板 62:70，且要用新代碼重啟 7860 語音伺服器
-列出全部設備，可按 MAC、設備名、家長 email 搜尋，按狀態和韌體篩選；顯示在線／離線（取自語音伺服器）、上次上線、韌體版本、OTA 失敗版本、綁定帳號與時間、出廠鎖定的 IP；單台詳情可做「重置設備密鑰」「強制解綁」，兩者都要填原因並寫入審計記錄（P1-10）；不顯示任何對話、記憶或孩子資料（Q7）；只有超級管理員能讀。</t>
+          <t>① 設備在「未配網、Wi-Fi 連不上、未綁定、長按 BOOT」時以 AIBuddy-XXXX 名稱廣播藍牙，廣播資料帶品牌，品牌 App 只列出自己品牌的設備。② 設備經藍牙回傳它掃描到的 2.4GHz Wi-Fi 清單，App 讓用戶選擇並填密碼。③ App 經藍牙把 SSID、密碼和綁定票（P0-11）一起交給設備；藍牙通道加密（ESP 標準配網協定 security 1/2 或同等）。④ 設備連上 Wi-Fi 後自己完成認領，App 顯示綁定成功或失敗原因（密碼錯、設備已有主人、票過期）。⑤ 配網期間不啟動音訊；完成後釋放藍牙記憶體再開語音（必要時重開機），對話中最低 heap 不比現在差。⑥ 解綁在 App 內完成（P1-12），解綁後設備進入藍牙待綁定狀態。⑦ SoftAP 熱點配網保留給開發和運維（隱藏觸發方式或編譯開關），量產用戶流程不出現。</t>
         </is>
       </c>
       <c r="F31" s="11" t="n"/>
@@ -1550,15 +1549,15 @@
       <c r="H31" s="11" t="n"/>
       <c r="I31" s="12" t="n"/>
     </row>
-    <row r="32" ht="214" customHeight="1">
+    <row r="32" ht="256" customHeight="1">
       <c r="A32" s="13" t="inlineStr">
         <is>
-          <t>P2-16</t>
+          <t>R-36</t>
         </is>
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>OTA 分批推送與後台發佈頁</t>
+          <t>未認領的設備停在配對狀態，不再每秒重連 websocket</t>
         </is>
       </c>
       <c r="C32" s="13" t="inlineStr">
@@ -1573,8 +1572,8 @@
       </c>
       <c r="E32" s="6" t="inlineStr">
         <is>
-          <t>上次測試：部分通過 — 子任務 P2-17～P2-20 通過、P2-21 部分通過（等 P2-14）。① 10% 階段只有雜湊預測的那組拿到、重複不變（P2-18、P2-21）② 2 台回滾 → 自動暫停、其餘不再拿到（P2-19、P2-21）③ 100% 全部拿到 ⑤ 審計表有每次階段變更（P2-21 9 筆）。未做：④ 開發板 62:70 實機走一次白名單階段（用戶目前手上沒有板子），同時驗證新韌體開機印出 BUILD_INFO
-後台可上傳韌體（伺服器算 SHA-256、寫 firmware_releases）、填說明、設為 current；推送分階段：白名單 MAC → 10% → 50% → 100%，按 MAC 雜湊穩定分組；回滾率超過 5% 即自動暫停（2026-10-14 拿走「同一台重啟 3 次」，見 P2-19）；顯示每個版本已更新、回滾台數與回滾設備清單；顯示 app 分區用量（P2-12）；每個發佈操作寫入審計記錄。</t>
+          <t>上次測試：部分通過 — 真機 62:70（2026-10-15，r-36 rebase 到 dev 1bd85ac，-localall 1.7.2，本機 3230/7870）：① 09:45:10 後台解綁 → 語音伺服器只在 09:45:11 拒絕 1 次，串口『device token refused, pausing』，之後只見 generate_auth_token 202 輪詢（約 70 秒 4 次）② 09:46:36 重新認領 → 09:46:53 自動連上（17 秒）並播出開場白，沒按鍵、沒重開 ④ 對照：改動前 1.7.0 解綁後每秒被拒 1 次（約 57 次/分鐘）。未做：③ 已綁定時斷網 30 秒再恢復；洋紅慢閃燈號未目視；⑤ 隨 OTA 推出
+① 拿到 202 或 websocket 被 4401 拒絕後，設備停掉 websocket 自動重連，進入待綁定狀態（燈號可分辨）。② 待綁定時只按退避（5 秒起、上限 PROVISION_BACKOFF_MAX）呼叫 generate_auth_token，不開 websocket。③ 被認領後下一次輪詢拿到 200，在 10 秒內（加退避）自動開 websocket 並能對話，不用重開機。④ 已綁定設備網絡斷線重連的行為不變。⑤ 隨 OTA 推出。</t>
         </is>
       </c>
       <c r="F32" s="11" t="n"/>
@@ -1582,20 +1581,20 @@
       <c r="H32" s="11" t="n"/>
       <c r="I32" s="12" t="n"/>
     </row>
-    <row r="33" ht="382" customHeight="1">
+    <row r="33" ht="228" customHeight="1">
       <c r="A33" s="13" t="inlineStr">
         <is>
-          <t>P2-21</t>
+          <t>P2-12</t>
         </is>
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>P2-16 ⑤ 後台 OTA 頁換成真實數據與操作</t>
+          <t>量產燒錄前加大 app 分區</t>
         </is>
       </c>
       <c r="C33" s="13" t="inlineStr">
         <is>
-          <t>2 內測準備</t>
+          <t>3 封閉內測</t>
         </is>
       </c>
       <c r="D33" s="13" t="inlineStr">
@@ -1605,8 +1604,8 @@
       </c>
       <c r="E33" s="6" t="inlineStr">
         <is>
-          <t>上次測試：部分通過 — 本機（分支 dev server 3216 + 本機 Supabase，GoTrue 真實登入的超管 cookie），用 xmini-c3 板型 + 20 台模擬設備以免碰到真開發板：頁面上傳 9.9.0 → 草稿；白名單加 1 台（UI 選單）→ 存檔；設為 current → 頁面預測 1 台、模擬 1 台；推進 10% → 預測 4、實得 4（重複不變）；50% → 預測 9、實得 9 且包含 10% 全部；100% → 20/20。2 台回滾 → 頁面顯示 'Paused … by the server: Auto-paused: 2 of 20 boards rolled back (10%)' 與回滾清單 2 台；點回滾設備 → 設備頁已帶 MAC 搜尋；恢復 → 其餘 18 台再拿到、回滾的 2 台不再下發；手動暫停未填原因不能確認、填後顯示 'by an admin'。審計頁 9 筆（上傳、白名單、current、10/50/100%、系統暫停、恢復、手動暫停），系統暫停顯示 System。375px scrollWidth=375。內容管理員側欄只有 Characters/IPs、#ota 退回 Characters、頁面無 OTA 數據，直接呼叫 admin_change_firmware_rollout → 403/42501。測試中發現並修正：舊版本（含 63:64 仍在跑的 1.6.1）被當成可刪除的草稿（6c2dc9d）。測試數據已清除
-按板型列出版本：狀態（草稿／推送中＋階段／暫停＋原因／現行／舊版）、已更新／目標台數、回滾台數、大小、發佈時間、說明；單一版本可編輯白名單、推進下一階段、暫停／恢復、撤下；回滾設備清單可點進設備頁；顯示 app 分區用量（P2-12）；每個操作要確認並寫審計記錄；只有超級管理員可見；375px 無橫向捲動。</t>
+          <t>上次測試：部分通過 — 62:70（spotpear-ai-toy-p212 原型，現已併入 spotpear-ai-toy）：① 本機 OTA 1.6.1→1.6.2 寫入新 app1，120s 後 confirmed ② 3 秒 abort 的 1.6.3 → PANIC → 回到 1.6.2，ota_failed_version=1.6.3 ③ 崩潰寫入 coredump 14.8KB ④ 資源分區 9 個聲音 504KB/2MB，開機 CRC 63ms，OTA 後照常；損壞/清空 → 退回內建聲音無崩潰 ⑤ pio 全部 18 個 env 編譯通過，映像都在各自 app 槽內（Spotpear 4 個 1.59–1.60MB / 4MB；其他板仍 2MB 槽）；R-21 藍牙探針版 2,326,128 bytes &lt; 4MB ⑥ release_firmware.py 映像 &gt; app 槽即拒發。未做：雲端 OTA 一次（等上 UAT）、出廠腳本寫入資源包（R-10）
+新分區表（例如 app0/app1 各 4MB，保留 nvs/otadata 位置）在出廠前定案並寫入出廠腳本；OTA 與回滾在新分區表上照常</t>
         </is>
       </c>
       <c r="F33" s="11" t="n"/>
@@ -1614,20 +1613,20 @@
       <c r="H33" s="11" t="n"/>
       <c r="I33" s="12" t="n"/>
     </row>
-    <row r="34" ht="200" customHeight="1">
+    <row r="34" ht="409" customHeight="1">
       <c r="A34" s="13" t="inlineStr">
         <is>
-          <t>R-21</t>
+          <t>P2-22</t>
         </is>
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>藍牙配網與綁定（取代熱點配網）</t>
+          <t>改服務器網址也不失聯：語音網址由後端下發、後端網址可遷移、已確認韌體長期連不上時自救</t>
         </is>
       </c>
       <c r="C34" s="13" t="inlineStr">
         <is>
-          <t>2 內測準備</t>
+          <t>3 封閉內測</t>
         </is>
       </c>
       <c r="D34" s="13" t="inlineStr">
@@ -1637,7 +1636,8 @@
       </c>
       <c r="E34" s="6" t="inlineStr">
         <is>
-          <t>① 設備在「未配網、Wi-Fi 連不上、未綁定、長按 BOOT」時以 AIBuddy-XXXX 名稱廣播藍牙，廣播資料帶品牌，品牌 App 只列出自己品牌的設備。② 設備經藍牙回傳它掃描到的 2.4GHz Wi-Fi 清單，App 讓用戶選擇並填密碼。③ App 經藍牙把 SSID、密碼和綁定票（P0-11）一起交給設備；藍牙通道加密（ESP 標準配網協定 security 1/2 或同等）。④ 設備連上 Wi-Fi 後自己完成認領，App 顯示綁定成功或失敗原因（密碼錯、設備已有主人、票過期）。⑤ 配網期間不啟動音訊；完成後釋放藍牙記憶體再開語音（必要時重開機），對話中最低 heap 不比現在差。⑥ 解綁在 App 內完成（P1-12），解綁後設備進入藍牙待綁定狀態。⑦ SoftAP 熱點配網保留給開發和運維（隱藏觸發方式或編譯開關），量產用戶流程不出現。</t>
+          <t>上次測試：部分通過 — 後端部分（分支 p2-22-server-urls）：node --test lib/deviceServerUrls.test.mjs 5/5、tsc 0 錯誤。worktree dev server 3222 + 本機 Supabase，兩塊假板（02:22:…:01/02）：已認領 200 帶 voice_url + backend_url；未認領 202 只帶 backend_url；DEVICE_VOICE_URL=ws://fastapi:7860/… → 不發、日誌記錯誤；兩個變數都不設 → 兩個欄位都不帶；生產值 → wss://elatoai.hkqft.com/fastapi/ws/esp32、https://elatoai.hkqft.com。測試數據已清除
+① /api/generate_auth_token 的回應帶 voice_url（wss 主機＋端口＋路徑，來自後端環境變數）；韌體用它連 /ws，並把最後一次成功的值存進 NVS；改 FastAPI 網址只改伺服器設定，不需新韌體 ② 回應沒有 voice_url（舊後端）或新網址連不上時，退回 NVS 上次成功的值，再退回出廠／編譯時的預設值 ③ 後端網址可遷移：回應可帶 backend_url；韌體先存為候選，下次開機用新網址取 token 成功才正式替換，失敗就繼續用舊網址；舊網址在遷移期內保持可用（runbook 寫明保留多久） ④ 已確認的韌體若連續 N 次開機（預設 10 次、跨度至少 24 小時，計數存 NVS）Wi-Fi 已拿到 IP 卻取不到 token：先依次試 NVS、出廠的後端網址；仍失敗且另一個槽可用，就切到另一個槽一次，並在下次連上時把本版本報為失敗 ⑤ 純斷網（拿不到 IP、路由器沒外網）不計入 ④ ⑥ 新網址的證書必須鏈到 CF_CA_bundle 裡的根（GTS Root R4、ISRG Root X1）；換主機或離開 Cloudflare 前先查證書鏈，runbook 寫明 ⑦ 只接受 https 的 backend_url 和 wss 的 voice_url，主機須在韌體內允許的網域後綴之下，防止後端被冒充時把板子引去別處</t>
         </is>
       </c>
       <c r="F34" s="11" t="n"/>
@@ -1645,20 +1645,20 @@
       <c r="H34" s="11" t="n"/>
       <c r="I34" s="12" t="n"/>
     </row>
-    <row r="35" ht="116" customHeight="1">
+    <row r="35" ht="242" customHeight="1">
       <c r="A35" s="13" t="inlineStr">
         <is>
-          <t>R-36</t>
+          <t>R-37</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>未認領的設備停在配對狀態，不再每秒重連 websocket</t>
+          <t>網頁設定玩具的 Wi-Fi：查看、新增、刪除</t>
         </is>
       </c>
       <c r="C35" s="13" t="inlineStr">
         <is>
-          <t>2 內測準備</t>
+          <t>3 封閉內測</t>
         </is>
       </c>
       <c r="D35" s="13" t="inlineStr">
@@ -1668,7 +1668,8 @@
       </c>
       <c r="E35" s="6" t="inlineStr">
         <is>
-          <t>① 拿到 202 或 websocket 被 4401 拒絕後，設備停掉 websocket 自動重連，進入待綁定狀態（燈號可分辨）。② 待綁定時只按退避（5 秒起、上限 PROVISION_BACKOFF_MAX）呼叫 generate_auth_token，不開 websocket。③ 被認領後下一次輪詢拿到 200，在 10 秒內（加退避）自動開 websocket 並能對話，不用重開機。④ 已綁定設備網絡斷線重連的行為不變。⑤ 隨 OTA 推出。</t>
+          <t>上次測試：部分通過 — 模擬玩具經本機語音服務器＋網頁：status/scan/add/delete 正常；刪除目前 Wi-Fi → current 被拒；斷線 5 秒內頁面顯示睡著、按鈕停用；測試密碼在語音服務器日誌、網頁服務器日誌、資料庫均搜不到；用別人裝置 ID 重放 server action → forbidden；pytest 17 項通過（全套 230）；韌體 spotpear-ai-toy-localall 編譯通過（RAM 17.5%、Flash 75.9%）。未測：真機 ①② 及 OTA 推出
+① 設定頁顯示玩具在線／離線、目前 Wi-Fi 和訊號、已記住的 Wi-Fi 清單（只有名稱，不顯示密碼）② 在線時可新增 Wi-Fi（輸入或從玩具掃描到的清單選）、刪除 Wi-Fi；不能刪除正在使用的那個 ③ 經 /ws/esp32 轉送：伺服器先確認是設備主人；密碼不寫入資料庫、不寫入日誌 ④ 新增不切換網絡，目前 Wi-Fi 消失時才按訊號選；清單標示「連過／未連過」⑤ 上限 8 個 ⑥ 韌體改動經 OTA 推出</t>
         </is>
       </c>
       <c r="F35" s="11" t="n"/>
@@ -1676,31 +1677,30 @@
       <c r="H35" s="11" t="n"/>
       <c r="I35" s="12" t="n"/>
     </row>
-    <row r="36" ht="228" customHeight="1">
+    <row r="36" ht="102" customHeight="1">
       <c r="A36" s="13" t="inlineStr">
         <is>
-          <t>P2-12</t>
+          <t>R-16</t>
         </is>
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>量產燒錄前加大 app 分區</t>
+          <t>Spotpear 量產版加電池電壓檢測（GPIO0 分壓）</t>
         </is>
       </c>
       <c r="C36" s="13" t="inlineStr">
         <is>
-          <t>3 封閉內測</t>
+          <t>1 止血定案</t>
         </is>
       </c>
       <c r="D36" s="13" t="inlineStr">
         <is>
-          <t>進行中</t>
+          <t>未開始</t>
         </is>
       </c>
       <c r="E36" s="6" t="inlineStr">
         <is>
-          <t>上次測試：部分通過 — 62:70（spotpear-ai-toy-p212 原型，現已併入 spotpear-ai-toy）：① 本機 OTA 1.6.1→1.6.2 寫入新 app1，120s 後 confirmed ② 3 秒 abort 的 1.6.3 → PANIC → 回到 1.6.2，ota_failed_version=1.6.3 ③ 崩潰寫入 coredump 14.8KB ④ 資源分區 9 個聲音 504KB/2MB，開機 CRC 63ms，OTA 後照常；損壞/清空 → 退回內建聲音無崩潰 ⑤ pio 全部 18 個 env 編譯通過，映像都在各自 app 槽內（Spotpear 4 個 1.59–1.60MB / 4MB；其他板仍 2MB 槽）；R-21 藍牙探針版 2,326,128 bytes &lt; 4MB ⑥ release_firmware.py 映像 &gt; app 槽即拒發。未做：雲端 OTA 一次（等上 UAT）、出廠腳本寫入資源包（R-10）
-新分區表（例如 app0/app1 各 4MB，保留 nvs/otadata 位置）在出廠前定案並寫入出廠腳本；OTA 與回滾在新分區表上照常</t>
+          <t>Spotpear 書面確認量產版：GPIO1（屏幕 DC；本版不接屏幕，可空出來）接電芯正極（保護 IC 之後）100k/100k 分壓、100nF 濾波，屏幕不接該腳；GPIO0 保留給現有的 VDD 低電提醒；最好另把充電芯片 CHRG 接到 GPIO12 或 13。樣板到手後，固件讀到的電芯電壓與萬用表相差 ≤50mV，App（R-41）顯示百分比與充電中。</t>
         </is>
       </c>
       <c r="F36" s="11" t="n"/>
@@ -1708,31 +1708,30 @@
       <c r="H36" s="11" t="n"/>
       <c r="I36" s="12" t="n"/>
     </row>
-    <row r="37" ht="409" customHeight="1">
+    <row r="37" ht="46" customHeight="1">
       <c r="A37" s="13" t="inlineStr">
         <is>
-          <t>P2-22</t>
+          <t>P1-11</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>改服務器網址也不失聯：語音網址由後端下發、後端網址可遷移、已確認韌體長期連不上時自救</t>
+          <t>伺服器與資料庫直接存取的管控</t>
         </is>
       </c>
       <c r="C37" s="13" t="inlineStr">
         <is>
-          <t>3 封閉內測</t>
+          <t>2 內測準備</t>
         </is>
       </c>
       <c r="D37" s="13" t="inlineStr">
         <is>
-          <t>進行中</t>
+          <t>未開始</t>
         </is>
       </c>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>上次測試：部分通過 — 後端部分（分支 p2-22-server-urls）：node --test lib/deviceServerUrls.test.mjs 5/5、tsc 0 錯誤。worktree dev server 3222 + 本機 Supabase，兩塊假板（02:22:…:01/02）：已認領 200 帶 voice_url + backend_url；未認領 202 只帶 backend_url；DEVICE_VOICE_URL=ws://fastapi:7860/… → 不發、日誌記錯誤；兩個變數都不設 → 兩個欄位都不帶；生產值 → wss://elatoai.hkqft.com/fastapi/ws/esp32、https://elatoai.hkqft.com。測試數據已清除
-① /api/generate_auth_token 的回應帶 voice_url（wss 主機＋端口＋路徑，來自後端環境變數）；韌體用它連 /ws，並把最後一次成功的值存進 NVS；改 FastAPI 網址只改伺服器設定，不需新韌體 ② 回應沒有 voice_url（舊後端）或新網址連不上時，退回 NVS 上次成功的值，再退回出廠／編譯時的預設值 ③ 後端網址可遷移：回應可帶 backend_url；韌體先存為候選，下次開機用新網址取 token 成功才正式替換，失敗就繼續用舊網址；舊網址在遷移期內保持可用（runbook 寫明保留多久） ④ 已確認的韌體若連續 N 次開機（預設 10 次、跨度至少 24 小時，計數存 NVS）Wi-Fi 已拿到 IP 卻取不到 token：先依次試 NVS、出廠的後端網址；仍失敗且另一個槽可用，就切到另一個槽一次，並在下次連上時把本版本報為失敗 ⑤ 純斷網（拿不到 IP、路由器沒外網）不計入 ④ ⑥ 新網址的證書必須鏈到 CF_CA_bundle 裡的根（GTS Root R4、ISRG Root X1）；換主機或離開 Cloudflare 前先查證書鏈，runbook 寫明 ⑦ 只接受 https 的 backend_url 和 wss 的 voice_url，主機須在韌體內允許的網域後綴之下，防止後端被冒充時把板子引去別處</t>
+          <t>列出誰有 SSH 與資料庫直連權限（越少越好）；service_role key 只存在伺服器的 env；私隱政策寫明這類存取的範圍；每次直接查看生產資料都留記錄。</t>
         </is>
       </c>
       <c r="F37" s="11" t="n"/>
@@ -1740,31 +1739,30 @@
       <c r="H37" s="11" t="n"/>
       <c r="I37" s="12" t="n"/>
     </row>
-    <row r="38" ht="242" customHeight="1">
+    <row r="38" ht="46" customHeight="1">
       <c r="A38" s="13" t="inlineStr">
         <is>
-          <t>R-37</t>
+          <t>P2-02</t>
         </is>
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>網頁設定玩具的 Wi-Fi：查看、新增、刪除</t>
+          <t>CI 跑測試與靜態檢查</t>
         </is>
       </c>
       <c r="C38" s="13" t="inlineStr">
         <is>
-          <t>3 封閉內測</t>
+          <t>2 內測準備</t>
         </is>
       </c>
       <c r="D38" s="13" t="inlineStr">
         <is>
-          <t>進行中</t>
+          <t>未開始</t>
         </is>
       </c>
       <c r="E38" s="6" t="inlineStr">
         <is>
-          <t>上次測試：部分通過 — 模擬玩具經本機語音服務器＋網頁：status/scan/add/delete 正常；刪除目前 Wi-Fi → current 被拒；斷線 5 秒內頁面顯示睡著、按鈕停用；測試密碼在語音服務器日誌、網頁服務器日誌、資料庫均搜不到；用別人裝置 ID 重放 server action → forbidden；pytest 17 項通過（全套 230）；韌體 spotpear-ai-toy-localall 編譯通過（RAM 17.5%、Flash 75.9%）。未測：真機 ①② 及 OTA 推出
-① 設定頁顯示玩具在線／離線、目前 Wi-Fi 和訊號、已記住的 Wi-Fi 清單（只有名稱，不顯示密碼）② 在線時可新增 Wi-Fi（輸入或從玩具掃描到的清單選）、刪除 Wi-Fi；不能刪除正在使用的那個 ③ 經 /ws/esp32 轉送：伺服器先確認是設備主人；密碼不寫入資料庫、不寫入日誌 ④ 新增不切換網絡，目前 Wi-Fi 消失時才按訊號選；清單標示「連過／未連過」⑤ 上限 8 個 ⑥ 韌體改動經 OTA 推出</t>
+          <t>推送與 PR 時跑 pytest、ruff、pyright、next lint、tsc --noEmit、pio run；任何一項失敗就不發佈 image。</t>
         </is>
       </c>
       <c r="F38" s="11" t="n"/>
@@ -1772,20 +1770,20 @@
       <c r="H38" s="11" t="n"/>
       <c r="I38" s="12" t="n"/>
     </row>
-    <row r="39" ht="102" customHeight="1">
+    <row r="39" ht="32" customHeight="1">
       <c r="A39" s="13" t="inlineStr">
         <is>
-          <t>R-16</t>
+          <t>P2-04</t>
         </is>
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>Spotpear 量產版加電池電壓檢測（GPIO0 分壓）</t>
+          <t>容器改用非 root 用戶</t>
         </is>
       </c>
       <c r="C39" s="13" t="inlineStr">
         <is>
-          <t>1 止血定案</t>
+          <t>2 內測準備</t>
         </is>
       </c>
       <c r="D39" s="13" t="inlineStr">
@@ -1795,7 +1793,7 @@
       </c>
       <c r="E39" s="6" t="inlineStr">
         <is>
-          <t>Spotpear 書面確認量產版：GPIO1（屏幕 DC；本版不接屏幕，可空出來）接電芯正極（保護 IC 之後）100k/100k 分壓、100nF 濾波，屏幕不接該腳；GPIO0 保留給現有的 VDD 低電提醒；最好另把充電芯片 CHRG 接到 GPIO12 或 13。樣板到手後，固件讀到的電芯電壓與萬用表相差 ≤50mV，App（R-41）顯示百分比與充電中。</t>
+          <t>兩個 Dockerfile 都設定非 root 的 USER。</t>
         </is>
       </c>
       <c r="F39" s="11" t="n"/>
@@ -1806,12 +1804,12 @@
     <row r="40" ht="46" customHeight="1">
       <c r="A40" s="13" t="inlineStr">
         <is>
-          <t>P1-11</t>
+          <t>R-04</t>
         </is>
       </c>
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>伺服器與資料庫直接存取的管控</t>
+          <t>粵語質量評測</t>
         </is>
       </c>
       <c r="C40" s="13" t="inlineStr">
@@ -1826,7 +1824,7 @@
       </c>
       <c r="E40" s="6" t="inlineStr">
         <is>
-          <t>列出誰有 SSH 與資料庫直連權限（越少越好）；service_role key 只存在伺服器的 env；私隱政策寫明這類存取的範圍；每次直接查看生產資料都留記錄。</t>
+          <t>有一套粵語評測集（兒童錄音＋文字提示）；選定的 STT 與 LLM 達到門檻：兒童語音字錯率 ≤15%、口語粵語回覆 ≥90%、中英夾雜句能正確理解。</t>
         </is>
       </c>
       <c r="F40" s="11" t="n"/>
@@ -1834,15 +1832,15 @@
       <c r="H40" s="11" t="n"/>
       <c r="I40" s="12" t="n"/>
     </row>
-    <row r="41" ht="46" customHeight="1">
+    <row r="41" ht="116" customHeight="1">
       <c r="A41" s="13" t="inlineStr">
         <is>
-          <t>P2-02</t>
+          <t>R-25</t>
         </is>
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>CI 跑測試與靜態檢查</t>
+          <t>網頁的品牌主題系統</t>
         </is>
       </c>
       <c r="C41" s="13" t="inlineStr">
@@ -1857,7 +1855,7 @@
       </c>
       <c r="E41" s="6" t="inlineStr">
         <is>
-          <t>推送與 PR 時跑 pytest、ruff、pyright、next lint、tsc --noEmit、pio run；任何一項失敗就不發佈 image。</t>
+          <t>① 每個品牌一個資料夾：主題 token（顏色、字體、圓角）、logo 和圖示、文案、功能開關；首頁、上手流程、角色頁可以有品牌版本，其餘頁面共用 ② 由部署的環境變數選品牌（每套部署一個品牌，見 R-34），伺服器端渲染的第一屏就是對的主題，不閃爍 ③ 共用元件裡沒有品牌名稱和寫死的品牌顏色 ④ 加一個品牌只需要加資料夾、設定和一套部署，不用改共用元件</t>
         </is>
       </c>
       <c r="F41" s="11" t="n"/>
@@ -1865,92 +1863,37 @@
       <c r="H41" s="11" t="n"/>
       <c r="I41" s="12" t="n"/>
     </row>
-    <row r="42" ht="32" customHeight="1">
-      <c r="A42" s="13" t="inlineStr">
-        <is>
-          <t>P2-04</t>
-        </is>
-      </c>
-      <c r="B42" s="6" t="inlineStr">
-        <is>
-          <t>容器改用非 root 用戶</t>
-        </is>
-      </c>
-      <c r="C42" s="13" t="inlineStr">
-        <is>
-          <t>2 內測準備</t>
-        </is>
-      </c>
-      <c r="D42" s="13" t="inlineStr">
-        <is>
-          <t>未開始</t>
-        </is>
-      </c>
-      <c r="E42" s="6" t="inlineStr">
-        <is>
-          <t>兩個 Dockerfile 都設定非 root 的 USER。</t>
-        </is>
-      </c>
-      <c r="F42" s="11" t="n"/>
-      <c r="G42" s="11" t="n"/>
-      <c r="H42" s="11" t="n"/>
-      <c r="I42" s="12" t="n"/>
-    </row>
-    <row r="43" ht="46" customHeight="1">
-      <c r="A43" s="13" t="inlineStr">
-        <is>
-          <t>R-04</t>
-        </is>
-      </c>
-      <c r="B43" s="6" t="inlineStr">
-        <is>
-          <t>粵語質量評測</t>
-        </is>
-      </c>
-      <c r="C43" s="13" t="inlineStr">
-        <is>
-          <t>2 內測準備</t>
-        </is>
-      </c>
-      <c r="D43" s="13" t="inlineStr">
-        <is>
-          <t>未開始</t>
-        </is>
-      </c>
-      <c r="E43" s="6" t="inlineStr">
-        <is>
-          <t>有一套粵語評測集（兒童錄音＋文字提示）；選定的 STT 與 LLM 達到門檻：兒童語音字錯率 ≤15%、口語粵語回覆 ≥90%、中英夾雜句能正確理解。</t>
-        </is>
-      </c>
-      <c r="F43" s="11" t="n"/>
-      <c r="G43" s="11" t="n"/>
-      <c r="H43" s="11" t="n"/>
-      <c r="I43" s="12" t="n"/>
-    </row>
-    <row r="44" ht="116" customHeight="1">
-      <c r="A44" s="13" t="inlineStr">
-        <is>
-          <t>R-25</t>
-        </is>
-      </c>
-      <c r="B44" s="6" t="inlineStr">
-        <is>
-          <t>網頁的品牌主題系統</t>
-        </is>
-      </c>
-      <c r="C44" s="13" t="inlineStr">
-        <is>
-          <t>2 內測準備</t>
-        </is>
-      </c>
-      <c r="D44" s="13" t="inlineStr">
-        <is>
-          <t>未開始</t>
-        </is>
-      </c>
-      <c r="E44" s="6" t="inlineStr">
-        <is>
-          <t>① 每個品牌一個資料夾：主題 token（顏色、字體、圓角）、logo 和圖示、文案、功能開關；首頁、上手流程、角色頁可以有品牌版本，其餘頁面共用 ② 由部署的環境變數選品牌（每套部署一個品牌，見 R-34），伺服器端渲染的第一屏就是對的主題，不閃爍 ③ 共用元件裡沒有品牌名稱和寫死的品牌顏色 ④ 加一個品牌只需要加資料夾、設定和一套部署，不用改共用元件</t>
+    <row r="43">
+      <c r="A43" s="10" t="inlineStr">
+        <is>
+          <t>✅ 最近完成與測試效果</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>編號</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>任務</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>測試結果</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>完成日期</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="inlineStr">
+        <is>
+          <t>測試證據</t>
         </is>
       </c>
       <c r="F44" s="11" t="n"/>
@@ -1958,37 +1901,92 @@
       <c r="H44" s="11" t="n"/>
       <c r="I44" s="12" t="n"/>
     </row>
-    <row r="46">
-      <c r="A46" s="10" t="inlineStr">
-        <is>
-          <t>✅ 最近完成與測試效果</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="4" t="inlineStr">
-        <is>
-          <t>編號</t>
-        </is>
-      </c>
-      <c r="B47" s="4" t="inlineStr">
-        <is>
-          <t>任務</t>
-        </is>
-      </c>
-      <c r="C47" s="4" t="inlineStr">
-        <is>
-          <t>測試結果</t>
-        </is>
-      </c>
-      <c r="D47" s="4" t="inlineStr">
-        <is>
-          <t>完成日期</t>
-        </is>
-      </c>
-      <c r="E47" s="4" t="inlineStr">
-        <is>
-          <t>測試證據</t>
+    <row r="45" ht="88" customHeight="1">
+      <c r="A45" s="13" t="inlineStr">
+        <is>
+          <t>P2-21</t>
+        </is>
+      </c>
+      <c r="B45" s="6" t="inlineStr">
+        <is>
+          <t>P2-16 ⑤ 後台 OTA 頁換成真實數據與操作</t>
+        </is>
+      </c>
+      <c r="C45" s="13" t="inlineStr">
+        <is>
+          <t>通過</t>
+        </is>
+      </c>
+      <c r="D45" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="E45" s="6" t="inlineStr">
+        <is>
+          <t>10-14 模擬 20 台全部通過（見上次）；2026-10-15 真機補做：OTA 頁對 1.7.1 白名單加 62:70（UI MAC 欄）→ 存檔確認框 → 『Narrow to Whitelist』確認 → Make current（用戶點）→ 62:70 安裝並確認，頁面顯示 Rolling out · Whitelist、運行 1、回滾 0；每步一筆審計。依賴 P2-14 已完成</t>
+        </is>
+      </c>
+      <c r="F45" s="11" t="n"/>
+      <c r="G45" s="11" t="n"/>
+      <c r="H45" s="11" t="n"/>
+      <c r="I45" s="12" t="n"/>
+    </row>
+    <row r="46" ht="158" customHeight="1">
+      <c r="A46" s="13" t="inlineStr">
+        <is>
+          <t>P2-16</t>
+        </is>
+      </c>
+      <c r="B46" s="6" t="inlineStr">
+        <is>
+          <t>OTA 分批推送與後台發佈頁</t>
+        </is>
+      </c>
+      <c r="C46" s="13" t="inlineStr">
+        <is>
+          <t>通過</t>
+        </is>
+      </c>
+      <c r="D46" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="E46" s="6" t="inlineStr">
+        <is>
+          <t>④ 真機 62:70（2026-10-15）：USB 刷 1.7.0（開機印 aibuddy-build;kind=dev;…;version=1.7.0）→ release_firmware.py publish --dev 1.7.1 → 後台白名單加 62:70、改白名單階段、設為 current → 按 BOOT 喚醒：取 token 200、下載 12.8s、重開進 app1，09:39:36 連上語音伺服器；09:42 重開 → 『Firmware 1.7.1 on app1』無 probation、Up to date；頁面『Rolling out · Whitelist』運行 1 台、回滾 0；審計 5 筆（發佈、白名單、階段、1.6.2 取消 current、1.7.1 設 current）。①②③⑤ 見 P2-17～P2-21 模擬 20 台</t>
+        </is>
+      </c>
+      <c r="F46" s="11" t="n"/>
+      <c r="G46" s="11" t="n"/>
+      <c r="H46" s="11" t="n"/>
+      <c r="I46" s="12" t="n"/>
+    </row>
+    <row r="47" ht="144" customHeight="1">
+      <c r="A47" s="13" t="inlineStr">
+        <is>
+          <t>P2-14</t>
+        </is>
+      </c>
+      <c r="B47" s="6" t="inlineStr">
+        <is>
+          <t>Admin 設備頁：每台玩具的狀態、韌體與基本操作</t>
+        </is>
+      </c>
+      <c r="C47" s="13" t="inlineStr">
+        <is>
+          <t>通過</t>
+        </is>
+      </c>
+      <c r="D47" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="E47" s="6" t="inlineStr">
+        <is>
+          <t>真機 62:70（2026-10-15，分支 hw-test-1015 = dev+P2-16，-localall 1.7.0，本機網頁 3230 + 語音 7870）：① 開機 → 設備頁 Online、-67 dBm、1.7.0；板子停在 bootloader 約 38 秒後語音伺服器判離線（uvicorn ping 超時），頁面 0 台在線 ② 重置設備密鑰 → device_secrets 行刪除，板子重開印『Device secret issued and stored』並連上，行恢復 ③ 強制解綁 → 板子拿 202（配對碼 UKDM7N），語音伺服器拒絕連線；兩項審計各 1 筆含操作者與原因 ④ 內容管理員/anon → 42501（10-14 探測腳本）</t>
         </is>
       </c>
       <c r="F47" s="11" t="n"/>
@@ -2151,120 +2149,96 @@
       <c r="H52" s="11" t="n"/>
       <c r="I52" s="12" t="n"/>
     </row>
-    <row r="53" ht="102" customHeight="1">
-      <c r="A53" s="13" t="inlineStr">
-        <is>
-          <t>P0-12</t>
-        </is>
-      </c>
-      <c r="B53" s="6" t="inlineStr">
-        <is>
-          <t>收緊 Admin 權限與路由保護</t>
-        </is>
-      </c>
-      <c r="C53" s="13" t="inlineStr">
-        <is>
-          <t>通過</t>
-        </is>
-      </c>
-      <c r="D53" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-12</t>
-        </is>
-      </c>
-      <c r="E53" s="6" t="inlineStr">
-        <is>
-          <t>線上 2026-10-12（bac24e9）：runbook 10/08 檢查 未登入 /admin→/login、/api/admin→401、has_role() 只看角色、無管理員 policy 觸及 conversations/記憶表、超管≥1；未登入 /home、/admin→/login；用戶確認：家長帳號開 /admin 轉回 /home、管理員在 /admin 修改角色保存成功；角色細分權限沿用本機 61/61</t>
-        </is>
-      </c>
-      <c r="F53" s="11" t="n"/>
-      <c r="G53" s="11" t="n"/>
-      <c r="H53" s="11" t="n"/>
-      <c r="I53" s="12" t="n"/>
-    </row>
-    <row r="54" ht="88" customHeight="1">
-      <c r="A54" s="13" t="inlineStr">
-        <is>
-          <t>P0-15</t>
-        </is>
-      </c>
-      <c r="B54" s="6" t="inlineStr">
-        <is>
-          <t>角色表權限：只有內容管理員能發佈，關閉家長自建角色</t>
-        </is>
-      </c>
-      <c r="C54" s="13" t="inlineStr">
-        <is>
-          <t>通過</t>
-        </is>
-      </c>
-      <c r="D54" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-12</t>
-        </is>
-      </c>
-      <c r="E54" s="6" t="inlineStr">
-        <is>
-          <t>線上 2026-10-12：② anon 只見 6 個已發佈 hk_ 內建，查隱藏/醫生/家長自建 → []，anon POST → 401；① authenticated 寫入權限由 20261007140000 REVOKE（runbook 10/08 已套用）；用戶確認：④ 家長登入後 /home/create 轉回 /home ③ 管理員在 /admin 修改角色保存成功</t>
-        </is>
-      </c>
-      <c r="F54" s="11" t="n"/>
-      <c r="G54" s="11" t="n"/>
-      <c r="H54" s="11" t="n"/>
-      <c r="I54" s="12" t="n"/>
-    </row>
-    <row r="55" ht="88" customHeight="1">
-      <c r="A55" s="13" t="inlineStr">
-        <is>
-          <t>P0-16</t>
-        </is>
-      </c>
-      <c r="B55" s="6" t="inlineStr">
-        <is>
-          <t>移除「醫生」身份與寫死的通關碼</t>
-        </is>
-      </c>
-      <c r="C55" s="13" t="inlineStr">
-        <is>
-          <t>通過</t>
-        </is>
-      </c>
-      <c r="D55" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-12</t>
-        </is>
-      </c>
-      <c r="E55" s="6" t="inlineStr">
-        <is>
-          <t>線上 2026-10-12：生產 commit bac24e9 git grep checkDoctorAction/kiwi-subtle-emu/=== "doctor"/isDoctor → 0；線上 13 個 JS（/、/login、/onboard）grep 通關碼/"doctor"/Santa/patient → 0；anon 讀角色只見 6 個 hk_ 角色、is_doctor 全 false；用戶今日線上登入及 playground 正常</t>
-        </is>
-      </c>
+    <row r="54">
+      <c r="A54" s="10" t="inlineStr">
+        <is>
+          <t>⏳ 等待依賴 / ⛔ 阻塞</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>編號</t>
+        </is>
+      </c>
+      <c r="B55" s="4" t="inlineStr">
+        <is>
+          <t>任務</t>
+        </is>
+      </c>
+      <c r="C55" s="4" t="inlineStr">
+        <is>
+          <t>在等什麼</t>
+        </is>
+      </c>
+      <c r="D55" s="11" t="n"/>
+      <c r="E55" s="11" t="n"/>
       <c r="F55" s="11" t="n"/>
       <c r="G55" s="11" t="n"/>
       <c r="H55" s="11" t="n"/>
       <c r="I55" s="12" t="n"/>
     </row>
-    <row r="57">
-      <c r="A57" s="10" t="inlineStr">
-        <is>
-          <t>⏳ 等待依賴 / ⛔ 阻塞</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="4" t="inlineStr">
-        <is>
-          <t>編號</t>
-        </is>
-      </c>
-      <c r="B58" s="4" t="inlineStr">
-        <is>
-          <t>任務</t>
-        </is>
-      </c>
-      <c r="C58" s="4" t="inlineStr">
-        <is>
-          <t>在等什麼</t>
+    <row r="56" ht="88" customHeight="1">
+      <c r="A56" s="13" t="inlineStr">
+        <is>
+          <t>R-17</t>
+        </is>
+      </c>
+      <c r="B56" s="6" t="inlineStr">
+        <is>
+          <t>Spotpear 電池耗盡時插電能否正常開機（供電路徑）</t>
+        </is>
+      </c>
+      <c r="C56" s="6" t="inlineStr">
+        <is>
+          <t>阻塞：[2026-10-08] 2026-10-08 開發板 63:64 插著 USB 時兩次無法解釋的完全斷電重開：09:13:26（崩潰循環中）、10:44:33（閒置、用戶確認沒碰）。都是 USB 先斷線再以 ESP_RST_POWERON 開機，非 brownout；斷電前 6 秒 GPIO0 讀數 99.9% 參考值，屬突然切斷而非緩降（SupplyMonitor 取樣太疏抓不到瞬間）。韌體無法造成 POWERON，指向充電芯片/電池保護/供電路徑，應一併問 Spotpear；放電實測時留意插 USB 閒置時是否也會斷電</t>
+        </is>
+      </c>
+      <c r="D56" s="11" t="n"/>
+      <c r="E56" s="11" t="n"/>
+      <c r="F56" s="11" t="n"/>
+      <c r="G56" s="11" t="n"/>
+      <c r="H56" s="11" t="n"/>
+      <c r="I56" s="12" t="n"/>
+    </row>
+    <row r="57" ht="60" customHeight="1">
+      <c r="A57" s="13" t="inlineStr">
+        <is>
+          <t>P1-01</t>
+        </is>
+      </c>
+      <c r="B57" s="6" t="inlineStr">
+        <is>
+          <t>加入內容審核層（輸入與輸出）</t>
+        </is>
+      </c>
+      <c r="C57" s="6" t="inlineStr">
+        <is>
+          <t>阻塞：[2026-10-14] 2026-10-14 用戶決定：先不定審核服務商，本項暫停。候選：Azure Content Safety（建議，香港區、可在每句回覆說出口前檢查）、OpenRouter 安全模型、OpenAI Moderation、只用本機字詞表。未寫任何程式。</t>
+        </is>
+      </c>
+      <c r="D57" s="11" t="n"/>
+      <c r="E57" s="11" t="n"/>
+      <c r="F57" s="11" t="n"/>
+      <c r="G57" s="11" t="n"/>
+      <c r="H57" s="11" t="n"/>
+      <c r="I57" s="12" t="n"/>
+    </row>
+    <row r="58" ht="32" customHeight="1">
+      <c r="A58" s="13" t="inlineStr">
+        <is>
+          <t>P1-09</t>
+        </is>
+      </c>
+      <c r="B58" s="6" t="inlineStr">
+        <is>
+          <t>家長鎖：孩子模式進設定要輸入 PIN</t>
+        </is>
+      </c>
+      <c r="C58" s="6" t="inlineStr">
+        <is>
+          <t>阻塞：[2026-10-13] 2026-10-13 用戶決定：AI Buddy（品牌 C）延到 1/15 之後，本項不卡 1/15 出廠；AI Buddy 啟動時再開。</t>
         </is>
       </c>
       <c r="D58" s="11" t="n"/>
@@ -2274,20 +2248,20 @@
       <c r="H58" s="11" t="n"/>
       <c r="I58" s="12" t="n"/>
     </row>
-    <row r="59" ht="88" customHeight="1">
+    <row r="59" ht="32" customHeight="1">
       <c r="A59" s="13" t="inlineStr">
         <is>
-          <t>R-17</t>
+          <t>R-12</t>
         </is>
       </c>
       <c r="B59" s="6" t="inlineStr">
         <is>
-          <t>Spotpear 電池耗盡時插電能否正常開機（供電路徑）</t>
+          <t>家長控制：每日使用上限和休息時段</t>
         </is>
       </c>
       <c r="C59" s="6" t="inlineStr">
         <is>
-          <t>阻塞：[2026-10-08] 2026-10-08 開發板 63:64 插著 USB 時兩次無法解釋的完全斷電重開：09:13:26（崩潰循環中）、10:44:33（閒置、用戶確認沒碰）。都是 USB 先斷線再以 ESP_RST_POWERON 開機，非 brownout；斷電前 6 秒 GPIO0 讀數 99.9% 參考值，屬突然切斷而非緩降（SupplyMonitor 取樣太疏抓不到瞬間）。韌體無法造成 POWERON，指向充電芯片/電池保護/供電路徑，應一併問 Spotpear；放電實測時留意插 USB 閒置時是否也會斷電</t>
+          <t>阻塞：[2026-10-13] 2026-10-13 用戶決定：AI Buddy（品牌 C）延到 1/15 之後，本項不卡 1/15 出廠；AI Buddy 啟動時再開。</t>
         </is>
       </c>
       <c r="D59" s="11" t="n"/>
@@ -2297,20 +2271,20 @@
       <c r="H59" s="11" t="n"/>
       <c r="I59" s="12" t="n"/>
     </row>
-    <row r="60" ht="60" customHeight="1">
+    <row r="60" ht="32" customHeight="1">
       <c r="A60" s="13" t="inlineStr">
         <is>
-          <t>P1-01</t>
+          <t>R-29</t>
         </is>
       </c>
       <c r="B60" s="6" t="inlineStr">
         <is>
-          <t>加入內容審核層（輸入與輸出）</t>
+          <t>AI Buddy App（品牌 C）頁面</t>
         </is>
       </c>
       <c r="C60" s="6" t="inlineStr">
         <is>
-          <t>阻塞：[2026-10-14] 2026-10-14 用戶決定：先不定審核服務商，本項暫停。候選：Azure Content Safety（建議，香港區、可在每句回覆說出口前檢查）、OpenRouter 安全模型、OpenAI Moderation、只用本機字詞表。未寫任何程式。</t>
+          <t>阻塞：[2026-10-13] 2026-10-13 用戶決定：AI Buddy（品牌 C）延到 1/15 之後，本項不卡 1/15 出廠；AI Buddy 啟動時再開。</t>
         </is>
       </c>
       <c r="D60" s="11" t="n"/>
@@ -2320,20 +2294,20 @@
       <c r="H60" s="11" t="n"/>
       <c r="I60" s="12" t="n"/>
     </row>
-    <row r="61" ht="32" customHeight="1">
+    <row r="61" ht="18" customHeight="1">
       <c r="A61" s="13" t="inlineStr">
         <is>
-          <t>P1-09</t>
+          <t>R-05</t>
         </is>
       </c>
       <c r="B61" s="6" t="inlineStr">
         <is>
-          <t>家長鎖：孩子模式進設定要輸入 PIN</t>
+          <t>內測版外殼（3D 打印 20 台）</t>
         </is>
       </c>
       <c r="C61" s="6" t="inlineStr">
         <is>
-          <t>阻塞：[2026-10-13] 2026-10-13 用戶決定：AI Buddy（品牌 C）延到 1/15 之後，本項不卡 1/15 出廠；AI Buddy 啟動時再開。</t>
+          <t>等 R-01</t>
         </is>
       </c>
       <c r="D61" s="11" t="n"/>
@@ -2343,20 +2317,20 @@
       <c r="H61" s="11" t="n"/>
       <c r="I61" s="12" t="n"/>
     </row>
-    <row r="62" ht="32" customHeight="1">
+    <row r="62" ht="18" customHeight="1">
       <c r="A62" s="13" t="inlineStr">
         <is>
-          <t>R-12</t>
+          <t>R-06</t>
         </is>
       </c>
       <c r="B62" s="6" t="inlineStr">
         <is>
-          <t>家長控制：每日使用上限和休息時段</t>
+          <t>家長自助上手流程</t>
         </is>
       </c>
       <c r="C62" s="6" t="inlineStr">
         <is>
-          <t>阻塞：[2026-10-13] 2026-10-13 用戶決定：AI Buddy（品牌 C）延到 1/15 之後，本項不卡 1/15 出廠；AI Buddy 啟動時再開。</t>
+          <t>等 P0-11</t>
         </is>
       </c>
       <c r="D62" s="11" t="n"/>
@@ -2369,17 +2343,17 @@
     <row r="63" ht="32" customHeight="1">
       <c r="A63" s="13" t="inlineStr">
         <is>
-          <t>R-29</t>
+          <t>R-13</t>
         </is>
       </c>
       <c r="B63" s="6" t="inlineStr">
         <is>
-          <t>AI Buddy App（品牌 C）頁面</t>
+          <t>CP1 內測就緒檢查（10/30）</t>
         </is>
       </c>
       <c r="C63" s="6" t="inlineStr">
         <is>
-          <t>阻塞：[2026-10-13] 2026-10-13 用戶決定：AI Buddy（品牌 C）延到 1/15 之後，本項不卡 1/15 出廠；AI Buddy 啟動時再開。</t>
+          <t>等 P0-07、P0-11、P1-01、P1-02、P2-09、R-01、R-02、R-04、R-05、R-06、P1-11</t>
         </is>
       </c>
       <c r="D63" s="11" t="n"/>
@@ -2389,15 +2363,15 @@
       <c r="H63" s="11" t="n"/>
       <c r="I63" s="12" t="n"/>
     </row>
-    <row r="64" ht="18" customHeight="1">
+    <row r="64" ht="32" customHeight="1">
       <c r="A64" s="13" t="inlineStr">
         <is>
-          <t>R-05</t>
+          <t>R-18</t>
         </is>
       </c>
       <c r="B64" s="6" t="inlineStr">
         <is>
-          <t>內測版外殼（3D 打印 20 台）</t>
+          <t>長按 BOOT 重新配網（開 AIBuddy-XXXX 熱點）</t>
         </is>
       </c>
       <c r="C64" s="6" t="inlineStr">
@@ -2412,20 +2386,20 @@
       <c r="H64" s="11" t="n"/>
       <c r="I64" s="12" t="n"/>
     </row>
-    <row r="65" ht="18" customHeight="1">
+    <row r="65" ht="32" customHeight="1">
       <c r="A65" s="13" t="inlineStr">
         <is>
-          <t>R-06</t>
+          <t>R-19</t>
         </is>
       </c>
       <c r="B65" s="6" t="inlineStr">
         <is>
-          <t>家長自助上手流程</t>
+          <t>外接按鈕：量產板加 I2C 擴展晶片（TCA9555）</t>
         </is>
       </c>
       <c r="C65" s="6" t="inlineStr">
         <is>
-          <t>等 P0-11</t>
+          <t>等 R-01</t>
         </is>
       </c>
       <c r="D65" s="11" t="n"/>
@@ -2435,20 +2409,20 @@
       <c r="H65" s="11" t="n"/>
       <c r="I65" s="12" t="n"/>
     </row>
-    <row r="66" ht="32" customHeight="1">
+    <row r="66" ht="18" customHeight="1">
       <c r="A66" s="13" t="inlineStr">
         <is>
-          <t>R-13</t>
+          <t>R-20</t>
         </is>
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
-          <t>CP1 內測就緒檢查（10/30）</t>
+          <t>孩子資料與角色改成每台設備一份</t>
         </is>
       </c>
       <c r="C66" s="6" t="inlineStr">
         <is>
-          <t>等 P0-07、P0-11、P1-01、P1-02、P2-09、R-01、R-02、R-04、R-05、R-06、P1-11</t>
+          <t>等 P1-12</t>
         </is>
       </c>
       <c r="D66" s="11" t="n"/>
@@ -2461,17 +2435,17 @@
     <row r="67" ht="32" customHeight="1">
       <c r="A67" s="13" t="inlineStr">
         <is>
-          <t>R-18</t>
+          <t>R-27</t>
         </is>
       </c>
       <c r="B67" s="6" t="inlineStr">
         <is>
-          <t>長按 BOOT 重新配網（開 AIBuddy-XXXX 熱點）</t>
+          <t>App 內登入：驗證碼、原生社交登入、刪除帳號</t>
         </is>
       </c>
       <c r="C67" s="6" t="inlineStr">
         <is>
-          <t>等 R-01</t>
+          <t>等 R-26</t>
         </is>
       </c>
       <c r="D67" s="11" t="n"/>
@@ -2481,15 +2455,15 @@
       <c r="H67" s="11" t="n"/>
       <c r="I67" s="12" t="n"/>
     </row>
-    <row r="68" ht="32" customHeight="1">
+    <row r="68" ht="18" customHeight="1">
       <c r="A68" s="13" t="inlineStr">
         <is>
-          <t>R-19</t>
+          <t>P0-14</t>
         </is>
       </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t>外接按鈕：量產板加 I2C 擴展晶片（TCA9555）</t>
+          <t>韌體簽章、Secure Boot 與 Flash 加密</t>
         </is>
       </c>
       <c r="C68" s="6" t="inlineStr">
@@ -2507,17 +2481,17 @@
     <row r="69" ht="18" customHeight="1">
       <c r="A69" s="13" t="inlineStr">
         <is>
-          <t>R-20</t>
+          <t>P1-06</t>
         </is>
       </c>
       <c r="B69" s="6" t="inlineStr">
         <is>
-          <t>孩子資料與角色改成每台設備一份</t>
+          <t>處理 GPL-3.0 依賴（arduino-audio-tools）</t>
         </is>
       </c>
       <c r="C69" s="6" t="inlineStr">
         <is>
-          <t>等 P1-12</t>
+          <t>等 Q3</t>
         </is>
       </c>
       <c r="D69" s="11" t="n"/>
@@ -2527,20 +2501,20 @@
       <c r="H69" s="11" t="n"/>
       <c r="I69" s="12" t="n"/>
     </row>
-    <row r="70" ht="32" customHeight="1">
+    <row r="70" ht="18" customHeight="1">
       <c r="A70" s="13" t="inlineStr">
         <is>
-          <t>R-27</t>
+          <t>P1-07</t>
         </is>
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>App 內登入：驗證碼、原生社交登入、刪除帳號</t>
+          <t>LGPL 合規與第三方授權聲明</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr">
         <is>
-          <t>等 R-26</t>
+          <t>等 Q3</t>
         </is>
       </c>
       <c r="D70" s="11" t="n"/>
@@ -2553,17 +2527,17 @@
     <row r="71" ht="18" customHeight="1">
       <c r="A71" s="13" t="inlineStr">
         <is>
-          <t>P0-14</t>
+          <t>P1-08</t>
         </is>
       </c>
       <c r="B71" s="6" t="inlineStr">
         <is>
-          <t>韌體簽章、Secure Boot 與 Flash 加密</t>
+          <t>硬件認證</t>
         </is>
       </c>
       <c r="C71" s="6" t="inlineStr">
         <is>
-          <t>等 R-01</t>
+          <t>等 R-01、R-05</t>
         </is>
       </c>
       <c r="D71" s="11" t="n"/>
@@ -2576,17 +2550,17 @@
     <row r="72" ht="18" customHeight="1">
       <c r="A72" s="13" t="inlineStr">
         <is>
-          <t>P1-06</t>
+          <t>P1-14</t>
         </is>
       </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>處理 GPL-3.0 依賴（arduino-audio-tools）</t>
+          <t>Admin 內容安全頁：審核事件只按類別統計</t>
         </is>
       </c>
       <c r="C72" s="6" t="inlineStr">
         <is>
-          <t>等 Q3</t>
+          <t>等 P1-01、P2-13</t>
         </is>
       </c>
       <c r="D72" s="11" t="n"/>
@@ -2596,20 +2570,20 @@
       <c r="H72" s="11" t="n"/>
       <c r="I72" s="12" t="n"/>
     </row>
-    <row r="73" ht="18" customHeight="1">
+    <row r="73" ht="32" customHeight="1">
       <c r="A73" s="13" t="inlineStr">
         <is>
-          <t>P1-07</t>
+          <t>P2-15</t>
         </is>
       </c>
       <c r="B73" s="6" t="inlineStr">
         <is>
-          <t>LGPL 合規與第三方授權聲明</t>
+          <t>Admin 總覽頁：在線、用量、成本與待處理事項</t>
         </is>
       </c>
       <c r="C73" s="6" t="inlineStr">
         <is>
-          <t>等 Q3</t>
+          <t>等 P2-09</t>
         </is>
       </c>
       <c r="D73" s="11" t="n"/>
@@ -2622,17 +2596,17 @@
     <row r="74" ht="18" customHeight="1">
       <c r="A74" s="13" t="inlineStr">
         <is>
-          <t>P1-08</t>
+          <t>R-07</t>
         </is>
       </c>
       <c r="B74" s="6" t="inlineStr">
         <is>
-          <t>硬件認證</t>
+          <t>20 個家庭封閉內測</t>
         </is>
       </c>
       <c r="C74" s="6" t="inlineStr">
         <is>
-          <t>等 R-01、R-05</t>
+          <t>等 R-13</t>
         </is>
       </c>
       <c r="D74" s="11" t="n"/>
@@ -2645,17 +2619,17 @@
     <row r="75" ht="18" customHeight="1">
       <c r="A75" s="13" t="inlineStr">
         <is>
-          <t>P1-14</t>
+          <t>R-08</t>
         </is>
       </c>
       <c r="B75" s="6" t="inlineStr">
         <is>
-          <t>Admin 內容安全頁：審核事件只按類別統計</t>
+          <t>第 8 週關卡決策</t>
         </is>
       </c>
       <c r="C75" s="6" t="inlineStr">
         <is>
-          <t>等 P1-01、P2-13</t>
+          <t>等 R-07、P2-09、P1-08</t>
         </is>
       </c>
       <c r="D75" s="11" t="n"/>
@@ -2665,20 +2639,20 @@
       <c r="H75" s="11" t="n"/>
       <c r="I75" s="12" t="n"/>
     </row>
-    <row r="76" ht="32" customHeight="1">
+    <row r="76" ht="18" customHeight="1">
       <c r="A76" s="13" t="inlineStr">
         <is>
-          <t>P2-15</t>
+          <t>R-14</t>
         </is>
       </c>
       <c r="B76" s="6" t="inlineStr">
         <is>
-          <t>Admin 總覽頁：在線、用量、成本與待處理事項</t>
+          <t>離線兒歌與故事</t>
         </is>
       </c>
       <c r="C76" s="6" t="inlineStr">
         <is>
-          <t>等 P2-14、P2-09</t>
+          <t>等 R-01</t>
         </is>
       </c>
       <c r="D76" s="11" t="n"/>
@@ -2691,17 +2665,17 @@
     <row r="77" ht="18" customHeight="1">
       <c r="A77" s="13" t="inlineStr">
         <is>
-          <t>R-07</t>
+          <t>R-24</t>
         </is>
       </c>
       <c r="B77" s="6" t="inlineStr">
         <is>
-          <t>20 個家庭封閉內測</t>
+          <t>設備只能用自己品牌的角色</t>
         </is>
       </c>
       <c r="C77" s="6" t="inlineStr">
         <is>
-          <t>等 R-13</t>
+          <t>等 R-34</t>
         </is>
       </c>
       <c r="D77" s="11" t="n"/>
@@ -2714,17 +2688,17 @@
     <row r="78" ht="18" customHeight="1">
       <c r="A78" s="13" t="inlineStr">
         <is>
-          <t>R-08</t>
+          <t>R-28</t>
         </is>
       </c>
       <c r="B78" s="6" t="inlineStr">
         <is>
-          <t>第 8 週關卡決策</t>
+          <t>三個 App 的殼：品牌版本與測試版</t>
         </is>
       </c>
       <c r="C78" s="6" t="inlineStr">
         <is>
-          <t>等 R-07、P2-09、P1-08</t>
+          <t>等 R-25、R-26</t>
         </is>
       </c>
       <c r="D78" s="11" t="n"/>
@@ -2737,17 +2711,17 @@
     <row r="79" ht="18" customHeight="1">
       <c r="A79" s="13" t="inlineStr">
         <is>
-          <t>R-14</t>
+          <t>R-30</t>
         </is>
       </c>
       <c r="B79" s="6" t="inlineStr">
         <is>
-          <t>離線兒歌與故事</t>
+          <t>快活 App（品牌 A）頁面</t>
         </is>
       </c>
       <c r="C79" s="6" t="inlineStr">
         <is>
-          <t>等 R-01</t>
+          <t>等 R-25、R-34、Q12</t>
         </is>
       </c>
       <c r="D79" s="11" t="n"/>
@@ -2760,17 +2734,17 @@
     <row r="80" ht="18" customHeight="1">
       <c r="A80" s="13" t="inlineStr">
         <is>
-          <t>R-24</t>
+          <t>R-31</t>
         </is>
       </c>
       <c r="B80" s="6" t="inlineStr">
         <is>
-          <t>設備只能用自己品牌的角色</t>
+          <t>政協青年聯會版 App（品牌 B）頁面</t>
         </is>
       </c>
       <c r="C80" s="6" t="inlineStr">
         <is>
-          <t>等 R-34</t>
+          <t>等 R-25、R-34、Q13</t>
         </is>
       </c>
       <c r="D80" s="11" t="n"/>
@@ -2783,17 +2757,17 @@
     <row r="81" ht="18" customHeight="1">
       <c r="A81" s="13" t="inlineStr">
         <is>
-          <t>R-28</t>
+          <t>R-35</t>
         </is>
       </c>
       <c r="B81" s="6" t="inlineStr">
         <is>
-          <t>三個 App 的殼：品牌版本與測試版</t>
+          <t>韌體按品牌連線：伺服器網址在出廠時寫入</t>
         </is>
       </c>
       <c r="C81" s="6" t="inlineStr">
         <is>
-          <t>等 R-25、R-26</t>
+          <t>等 R-34</t>
         </is>
       </c>
       <c r="D81" s="11" t="n"/>
@@ -2803,20 +2777,20 @@
       <c r="H81" s="11" t="n"/>
       <c r="I81" s="12" t="n"/>
     </row>
-    <row r="82" ht="18" customHeight="1">
+    <row r="82" ht="32" customHeight="1">
       <c r="A82" s="13" t="inlineStr">
         <is>
-          <t>R-30</t>
+          <t>R-38</t>
         </is>
       </c>
       <c r="B82" s="6" t="inlineStr">
         <is>
-          <t>快活 App（品牌 A）頁面</t>
+          <t>公仔出廠鎖死所屬 IP，綁定時顯示該 IP 頭像</t>
         </is>
       </c>
       <c r="C82" s="6" t="inlineStr">
         <is>
-          <t>等 R-25、R-34、Q12</t>
+          <t>等 P0-11</t>
         </is>
       </c>
       <c r="D82" s="11" t="n"/>
@@ -2826,20 +2800,20 @@
       <c r="H82" s="11" t="n"/>
       <c r="I82" s="12" t="n"/>
     </row>
-    <row r="83" ht="18" customHeight="1">
+    <row r="83" ht="32" customHeight="1">
       <c r="A83" s="13" t="inlineStr">
         <is>
-          <t>R-31</t>
+          <t>R-39</t>
         </is>
       </c>
       <c r="B83" s="6" t="inlineStr">
         <is>
-          <t>政協青年聯會版 App（品牌 B）頁面</t>
+          <t>Admin 出廠登記頁：匯入 MAC 清單、指定公仔、查看自檢結果</t>
         </is>
       </c>
       <c r="C83" s="6" t="inlineStr">
         <is>
-          <t>等 R-25、R-34、Q13</t>
+          <t>等 R-38、P1-10</t>
         </is>
       </c>
       <c r="D83" s="11" t="n"/>
@@ -2852,17 +2826,17 @@
     <row r="84" ht="18" customHeight="1">
       <c r="A84" s="13" t="inlineStr">
         <is>
-          <t>R-35</t>
+          <t>R-09</t>
         </is>
       </c>
       <c r="B84" s="6" t="inlineStr">
         <is>
-          <t>韌體按品牌連線：伺服器網址在出廠時寫入</t>
+          <t>量產外殼（真空複模）</t>
         </is>
       </c>
       <c r="C84" s="6" t="inlineStr">
         <is>
-          <t>等 R-34</t>
+          <t>等 R-08、R-05、Q11</t>
         </is>
       </c>
       <c r="D84" s="11" t="n"/>
@@ -2872,20 +2846,20 @@
       <c r="H84" s="11" t="n"/>
       <c r="I84" s="12" t="n"/>
     </row>
-    <row r="85" ht="32" customHeight="1">
+    <row r="85" ht="18" customHeight="1">
       <c r="A85" s="13" t="inlineStr">
         <is>
-          <t>R-38</t>
+          <t>R-10</t>
         </is>
       </c>
       <c r="B85" s="6" t="inlineStr">
         <is>
-          <t>公仔出廠鎖死所屬 IP，綁定時顯示該 IP 頭像</t>
+          <t>出廠流程</t>
         </is>
       </c>
       <c r="C85" s="6" t="inlineStr">
         <is>
-          <t>等 P0-11</t>
+          <t>等 P0-14、R-01、P2-12、R-34、R-35、R-38、R-39</t>
         </is>
       </c>
       <c r="D85" s="11" t="n"/>
@@ -2895,20 +2869,20 @@
       <c r="H85" s="11" t="n"/>
       <c r="I85" s="12" t="n"/>
     </row>
-    <row r="86" ht="32" customHeight="1">
+    <row r="86" ht="18" customHeight="1">
       <c r="A86" s="13" t="inlineStr">
         <is>
-          <t>R-39</t>
+          <t>R-11</t>
         </is>
       </c>
       <c r="B86" s="6" t="inlineStr">
         <is>
-          <t>Admin 出廠登記頁：匯入 MAC 清單、指定公仔、查看自檢結果</t>
+          <t>售後：客服、保修與換機</t>
         </is>
       </c>
       <c r="C86" s="6" t="inlineStr">
         <is>
-          <t>等 R-38、P1-10</t>
+          <t>等 R-40</t>
         </is>
       </c>
       <c r="D86" s="11" t="n"/>
@@ -2921,17 +2895,17 @@
     <row r="87" ht="18" customHeight="1">
       <c r="A87" s="13" t="inlineStr">
         <is>
-          <t>R-09</t>
+          <t>R-15</t>
         </is>
       </c>
       <c r="B87" s="6" t="inlineStr">
         <is>
-          <t>量產外殼（真空複模）</t>
+          <t>農曆新年前交付（生產 1/15、送達 1/29）</t>
         </is>
       </c>
       <c r="C87" s="6" t="inlineStr">
         <is>
-          <t>等 R-08、R-05、Q11</t>
+          <t>等 R-09、R-10</t>
         </is>
       </c>
       <c r="D87" s="11" t="n"/>
@@ -2944,17 +2918,17 @@
     <row r="88" ht="18" customHeight="1">
       <c r="A88" s="13" t="inlineStr">
         <is>
-          <t>R-10</t>
+          <t>R-33</t>
         </is>
       </c>
       <c r="B88" s="6" t="inlineStr">
         <is>
-          <t>出廠流程</t>
+          <t>三個 App 送審並通過</t>
         </is>
       </c>
       <c r="C88" s="6" t="inlineStr">
         <is>
-          <t>等 P0-14、R-01、P2-12、R-34、R-35、R-38、R-39</t>
+          <t>等 R-27、R-21、R-28、R-29、R-30、R-31、R-32</t>
         </is>
       </c>
       <c r="D88" s="11" t="n"/>
@@ -2964,20 +2938,20 @@
       <c r="H88" s="11" t="n"/>
       <c r="I88" s="12" t="n"/>
     </row>
-    <row r="89" ht="18" customHeight="1">
+    <row r="89" ht="32" customHeight="1">
       <c r="A89" s="13" t="inlineStr">
         <is>
-          <t>R-11</t>
+          <t>R-40</t>
         </is>
       </c>
       <c r="B89" s="6" t="inlineStr">
         <is>
-          <t>售後：客服、保修與換機</t>
+          <t>Admin 客服查詢頁：查帳號、名下設備與最近事件</t>
         </is>
       </c>
       <c r="C89" s="6" t="inlineStr">
         <is>
-          <t>等 P2-14、R-40</t>
+          <t>等 P1-10、P1-12</t>
         </is>
       </c>
       <c r="D89" s="11" t="n"/>
@@ -2987,66 +2961,27 @@
       <c r="H89" s="11" t="n"/>
       <c r="I89" s="12" t="n"/>
     </row>
-    <row r="90" ht="18" customHeight="1">
-      <c r="A90" s="13" t="inlineStr">
-        <is>
-          <t>R-15</t>
-        </is>
-      </c>
-      <c r="B90" s="6" t="inlineStr">
-        <is>
-          <t>農曆新年前交付（生產 1/15、送達 1/29）</t>
-        </is>
-      </c>
-      <c r="C90" s="6" t="inlineStr">
-        <is>
-          <t>等 R-09、R-10</t>
-        </is>
-      </c>
-      <c r="D90" s="11" t="n"/>
-      <c r="E90" s="11" t="n"/>
-      <c r="F90" s="11" t="n"/>
-      <c r="G90" s="11" t="n"/>
-      <c r="H90" s="11" t="n"/>
-      <c r="I90" s="12" t="n"/>
-    </row>
-    <row r="91" ht="18" customHeight="1">
-      <c r="A91" s="13" t="inlineStr">
-        <is>
-          <t>R-33</t>
-        </is>
-      </c>
-      <c r="B91" s="6" t="inlineStr">
-        <is>
-          <t>三個 App 送審並通過</t>
-        </is>
-      </c>
-      <c r="C91" s="6" t="inlineStr">
-        <is>
-          <t>等 R-27、R-21、R-28、R-29、R-30、R-31、R-32</t>
-        </is>
-      </c>
-      <c r="D91" s="11" t="n"/>
-      <c r="E91" s="11" t="n"/>
-      <c r="F91" s="11" t="n"/>
-      <c r="G91" s="11" t="n"/>
-      <c r="H91" s="11" t="n"/>
-      <c r="I91" s="12" t="n"/>
-    </row>
-    <row r="92" ht="32" customHeight="1">
-      <c r="A92" s="13" t="inlineStr">
-        <is>
-          <t>R-40</t>
-        </is>
-      </c>
-      <c r="B92" s="6" t="inlineStr">
-        <is>
-          <t>Admin 客服查詢頁：查帳號、名下設備與最近事件</t>
-        </is>
-      </c>
-      <c r="C92" s="6" t="inlineStr">
-        <is>
-          <t>等 P2-14、P1-10、P1-12</t>
+    <row r="91">
+      <c r="A91" s="10" t="inlineStr">
+        <is>
+          <t>❓ 待確認問題</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="4" t="inlineStr">
+        <is>
+          <t>編號</t>
+        </is>
+      </c>
+      <c r="B92" s="4" t="inlineStr">
+        <is>
+          <t>問題</t>
+        </is>
+      </c>
+      <c r="C92" s="4" t="inlineStr">
+        <is>
+          <t>影響的任務 / 為什麼重要</t>
         </is>
       </c>
       <c r="D92" s="11" t="n"/>
@@ -3056,27 +2991,66 @@
       <c r="H92" s="11" t="n"/>
       <c r="I92" s="12" t="n"/>
     </row>
-    <row r="94">
-      <c r="A94" s="10" t="inlineStr">
-        <is>
-          <t>❓ 待確認問題</t>
-        </is>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" s="4" t="inlineStr">
-        <is>
-          <t>編號</t>
-        </is>
-      </c>
-      <c r="B95" s="4" t="inlineStr">
-        <is>
-          <t>問題</t>
-        </is>
-      </c>
-      <c r="C95" s="4" t="inlineStr">
-        <is>
-          <t>影響的任務 / 為什麼重要</t>
+    <row r="93" ht="18" customHeight="1">
+      <c r="A93" s="13" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="B93" s="6" t="inlineStr">
+        <is>
+          <t>韌體打算閉源商業銷售嗎？</t>
+        </is>
+      </c>
+      <c r="C93" s="6" t="inlineStr">
+        <is>
+          <t>P1-06, P1-07：決定 GPL／LGPL 依賴要開源還是替換。</t>
+        </is>
+      </c>
+      <c r="D93" s="11" t="n"/>
+      <c r="E93" s="11" t="n"/>
+      <c r="F93" s="11" t="n"/>
+      <c r="G93" s="11" t="n"/>
+      <c r="H93" s="11" t="n"/>
+      <c r="I93" s="12" t="n"/>
+    </row>
+    <row r="94" ht="32" customHeight="1">
+      <c r="A94" s="13" t="inlineStr">
+        <is>
+          <t>Q11</t>
+        </is>
+      </c>
+      <c r="B94" s="6" t="inlineStr">
+        <is>
+          <t>馬會快活的賽馬日版和新春版各多少隻（共 2,500）？</t>
+        </is>
+      </c>
+      <c r="C94" s="6" t="inlineStr">
+        <is>
+          <t>R-09, R-15：兩款的服裝和配件要分開訂料；11/20 前不知道，PP 樣和大貨單（11/27）會被拖慢。由馬會決定。</t>
+        </is>
+      </c>
+      <c r="D94" s="11" t="n"/>
+      <c r="E94" s="11" t="n"/>
+      <c r="F94" s="11" t="n"/>
+      <c r="G94" s="11" t="n"/>
+      <c r="H94" s="11" t="n"/>
+      <c r="I94" s="12" t="n"/>
+    </row>
+    <row r="95" ht="60" customHeight="1">
+      <c r="A95" s="13" t="inlineStr">
+        <is>
+          <t>Q12</t>
+        </is>
+      </c>
+      <c r="B95" s="6" t="inlineStr">
+        <is>
+          <t>快活 App 的「會員綁定」是指甚麼：用我們自己的帳號（email 驗證碼），還是接馬會的會員帳號登入（SSO）？</t>
+        </is>
+      </c>
+      <c r="C95" s="6" t="inlineStr">
+        <is>
+          <t>P0-11, 快活 App（未入追蹤表）：接馬會 SSO 的話，登入、帳號刪除和資料歸屬都要按馬會的介面重做，工作量和排期要另估，而且 W5（11/9–11/13）就要做快活 App 的綁定；用我們的帳號則和其他品牌共用同一套流程。由馬會決定，要盡早問。</t>
         </is>
       </c>
       <c r="D95" s="11" t="n"/>
@@ -3086,20 +3060,20 @@
       <c r="H95" s="11" t="n"/>
       <c r="I95" s="12" t="n"/>
     </row>
-    <row r="96" ht="18" customHeight="1">
+    <row r="96" ht="46" customHeight="1">
       <c r="A96" s="13" t="inlineStr">
         <is>
-          <t>Q3</t>
+          <t>Q13</t>
         </is>
       </c>
       <c r="B96" s="6" t="inlineStr">
         <is>
-          <t>韌體打算閉源商業銷售嗎？</t>
+          <t>政協青年聯會版的角色、語言和內容由誰提供？什麼時候交？</t>
         </is>
       </c>
       <c r="C96" s="6" t="inlineStr">
         <is>
-          <t>P1-06, P1-07：決定 GPL／LGPL 依賴要開源還是替換。</t>
+          <t>品牌 B 的 App 頁面：品牌 B 的用戶是成人會員，但角色、說話語言、內容規則都還沒有。最遲 11/13 要拿到，才趕得及內部測試和 App 頁面（W6）。</t>
         </is>
       </c>
       <c r="D96" s="11" t="n"/>
@@ -3109,120 +3083,51 @@
       <c r="H96" s="11" t="n"/>
       <c r="I96" s="12" t="n"/>
     </row>
-    <row r="97" ht="32" customHeight="1">
-      <c r="A97" s="13" t="inlineStr">
-        <is>
-          <t>Q11</t>
-        </is>
-      </c>
-      <c r="B97" s="6" t="inlineStr">
-        <is>
-          <t>馬會快活的賽馬日版和新春版各多少隻（共 2,500）？</t>
-        </is>
-      </c>
-      <c r="C97" s="6" t="inlineStr">
-        <is>
-          <t>R-09, R-15：兩款的服裝和配件要分開訂料；11/20 前不知道，PP 樣和大貨單（11/27）會被拖慢。由馬會決定。</t>
-        </is>
-      </c>
-      <c r="D97" s="11" t="n"/>
-      <c r="E97" s="11" t="n"/>
-      <c r="F97" s="11" t="n"/>
-      <c r="G97" s="11" t="n"/>
-      <c r="H97" s="11" t="n"/>
-      <c r="I97" s="12" t="n"/>
-    </row>
-    <row r="98" ht="60" customHeight="1">
-      <c r="A98" s="13" t="inlineStr">
-        <is>
-          <t>Q12</t>
-        </is>
-      </c>
-      <c r="B98" s="6" t="inlineStr">
-        <is>
-          <t>快活 App 的「會員綁定」是指甚麼：用我們自己的帳號（email 驗證碼），還是接馬會的會員帳號登入（SSO）？</t>
-        </is>
-      </c>
-      <c r="C98" s="6" t="inlineStr">
-        <is>
-          <t>P0-11, 快活 App（未入追蹤表）：接馬會 SSO 的話，登入、帳號刪除和資料歸屬都要按馬會的介面重做，工作量和排期要另估，而且 W5（11/9–11/13）就要做快活 App 的綁定；用我們的帳號則和其他品牌共用同一套流程。由馬會決定，要盡早問。</t>
-        </is>
-      </c>
-      <c r="D98" s="11" t="n"/>
-      <c r="E98" s="11" t="n"/>
-      <c r="F98" s="11" t="n"/>
-      <c r="G98" s="11" t="n"/>
-      <c r="H98" s="11" t="n"/>
-      <c r="I98" s="12" t="n"/>
-    </row>
-    <row r="99" ht="46" customHeight="1">
-      <c r="A99" s="13" t="inlineStr">
-        <is>
-          <t>Q13</t>
-        </is>
-      </c>
-      <c r="B99" s="6" t="inlineStr">
-        <is>
-          <t>政協青年聯會版的角色、語言和內容由誰提供？什麼時候交？</t>
-        </is>
-      </c>
-      <c r="C99" s="6" t="inlineStr">
-        <is>
-          <t>品牌 B 的 App 頁面：品牌 B 的用戶是成人會員，但角色、說話語言、內容規則都還沒有。最遲 11/13 要拿到，才趕得及內部測試和 App 頁面（W6）。</t>
-        </is>
-      </c>
-      <c r="D99" s="11" t="n"/>
-      <c r="E99" s="11" t="n"/>
-      <c r="F99" s="11" t="n"/>
-      <c r="G99" s="11" t="n"/>
-      <c r="H99" s="11" t="n"/>
-      <c r="I99" s="12" t="n"/>
-    </row>
-    <row r="101">
-      <c r="A101" s="10" t="inlineStr">
+    <row r="98">
+      <c r="A98" s="10" t="inlineStr">
         <is>
           <t>說明</t>
         </is>
       </c>
     </row>
-    <row r="102" ht="32" customHeight="1">
+    <row r="99" ht="32" customHeight="1">
+      <c r="A99" s="14" t="inlineStr">
+        <is>
+          <t>・狀態：未開始 → 進行中 → 已完成。只有測試真的跑過而且通過才算已完成；阻塞要在備註寫原因；不再需要的任務標不適用，不要刪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" ht="18" customHeight="1">
+      <c r="A100" s="14" t="inlineStr">
+        <is>
+          <t>・測試結果：未測試 / 通過 / 失敗 / 部分通過。測試證據寫跑了什麼、看到什麼，完整歷史在「更新記錄」。</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" ht="18" customHeight="1">
+      <c r="A101" s="14" t="inlineStr">
+        <is>
+          <t>・「接下來」按階段排序，同一階段內再按優先級；依賴還沒滿足的任務不會出現在「接下來」。</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="18" customHeight="1">
       <c r="A102" s="14" t="inlineStr">
         <is>
-          <t>・狀態：未開始 → 進行中 → 已完成。只有測試真的跑過而且通過才算已完成；阻塞要在備註寫原因；不再需要的任務標不適用，不要刪。</t>
-        </is>
-      </c>
-    </row>
-    <row r="103" ht="18" customHeight="1">
+          <t>・可以手動改：「任務清單」的狀態、測試結果、測試證據、Commit、備註，以及「待確認問題」的回答。其餘欄位和本頁由腳本維護。</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" ht="32" customHeight="1">
       <c r="A103" s="14" t="inlineStr">
         <is>
-          <t>・測試結果：未測試 / 通過 / 失敗 / 部分通過。測試證據寫跑了什麼、看到什麼，完整歷史在「更新記錄」。</t>
-        </is>
-      </c>
-    </row>
-    <row r="104" ht="18" customHeight="1">
-      <c r="A104" s="14" t="inlineStr">
-        <is>
-          <t>・「接下來」按階段排序，同一階段內再按優先級；依賴還沒滿足的任務不會出現在「接下來」。</t>
-        </is>
-      </c>
-    </row>
-    <row r="105" ht="18" customHeight="1">
-      <c r="A105" s="14" t="inlineStr">
-        <is>
-          <t>・可以手動改：「任務清單」的狀態、測試結果、測試證據、Commit、備註，以及「待確認問題」的回答。其餘欄位和本頁由腳本維護。</t>
-        </is>
-      </c>
-    </row>
-    <row r="106" ht="32" customHeight="1">
-      <c r="A106" s="14" t="inlineStr">
-        <is>
           <t>・建議用法：在 Claude Code 對 Claude 說「P0-02 做完了」或輸入 /prod-readiness。Claude 會先跑測試再更新，並寫進「更新記錄」。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="87">
-    <mergeCell ref="E55:I55"/>
+  <mergeCells count="84">
+    <mergeCell ref="A99:I99"/>
     <mergeCell ref="C82:I82"/>
     <mergeCell ref="E52:I52"/>
     <mergeCell ref="E39:I39"/>
@@ -3236,7 +3141,6 @@
     <mergeCell ref="C92:I92"/>
     <mergeCell ref="E31:I31"/>
     <mergeCell ref="E40:I40"/>
-    <mergeCell ref="C97:I97"/>
     <mergeCell ref="A19:I19"/>
     <mergeCell ref="E26:I26"/>
     <mergeCell ref="A103:I103"/>
@@ -3245,10 +3149,7 @@
     <mergeCell ref="C60:I60"/>
     <mergeCell ref="C71:I71"/>
     <mergeCell ref="E50:I50"/>
-    <mergeCell ref="A46:I46"/>
-    <mergeCell ref="E42:I42"/>
-    <mergeCell ref="C91:I91"/>
-    <mergeCell ref="A105:I105"/>
+    <mergeCell ref="C57:I57"/>
     <mergeCell ref="C66:I66"/>
     <mergeCell ref="E44:I44"/>
     <mergeCell ref="E20:I20"/>
@@ -3256,35 +3157,34 @@
     <mergeCell ref="C77:I77"/>
     <mergeCell ref="C86:I86"/>
     <mergeCell ref="C68:I68"/>
+    <mergeCell ref="A91:I91"/>
+    <mergeCell ref="A100:I100"/>
     <mergeCell ref="C58:I58"/>
     <mergeCell ref="E30:I30"/>
-    <mergeCell ref="E22:I22"/>
+    <mergeCell ref="E46:I46"/>
     <mergeCell ref="A102:I102"/>
     <mergeCell ref="C85:I85"/>
+    <mergeCell ref="C94:I94"/>
     <mergeCell ref="C65:I65"/>
     <mergeCell ref="C75:I75"/>
     <mergeCell ref="C84:I84"/>
     <mergeCell ref="C80:I80"/>
-    <mergeCell ref="E54:I54"/>
     <mergeCell ref="E32:I32"/>
     <mergeCell ref="C59:I59"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="E41:I41"/>
-    <mergeCell ref="A94:I94"/>
     <mergeCell ref="E47:I47"/>
     <mergeCell ref="C61:I61"/>
-    <mergeCell ref="E43:I43"/>
     <mergeCell ref="C70:I70"/>
     <mergeCell ref="E24:I24"/>
     <mergeCell ref="E33:I33"/>
     <mergeCell ref="A3:I3"/>
-    <mergeCell ref="A104:I104"/>
-    <mergeCell ref="A57:I57"/>
     <mergeCell ref="E35:I35"/>
-    <mergeCell ref="A106:I106"/>
+    <mergeCell ref="A43:I43"/>
     <mergeCell ref="C74:I74"/>
     <mergeCell ref="C88:I88"/>
-    <mergeCell ref="C99:I99"/>
+    <mergeCell ref="E45:I45"/>
+    <mergeCell ref="C55:I55"/>
     <mergeCell ref="E37:I37"/>
     <mergeCell ref="E21:I21"/>
     <mergeCell ref="E23:I23"/>
@@ -3296,7 +3196,6 @@
     <mergeCell ref="C78:I78"/>
     <mergeCell ref="C87:I87"/>
     <mergeCell ref="C62:I62"/>
-    <mergeCell ref="C98:I98"/>
     <mergeCell ref="C89:I89"/>
     <mergeCell ref="E34:I34"/>
     <mergeCell ref="C64:I64"/>
@@ -3306,9 +3205,12 @@
     <mergeCell ref="E27:I27"/>
     <mergeCell ref="E36:I36"/>
     <mergeCell ref="C63:I63"/>
-    <mergeCell ref="C90:I90"/>
-    <mergeCell ref="E53:I53"/>
+    <mergeCell ref="C93:I93"/>
+    <mergeCell ref="A98:I98"/>
+    <mergeCell ref="C56:I56"/>
+    <mergeCell ref="E22:I22"/>
     <mergeCell ref="C76:I76"/>
+    <mergeCell ref="A54:I54"/>
   </mergeCells>
   <conditionalFormatting sqref="I6:I10">
     <cfRule type="dataBar" priority="1">
@@ -8963,7 +8865,7 @@
         </is>
       </c>
     </row>
-    <row r="78" ht="228" customHeight="1">
+    <row r="78" ht="298" customHeight="1">
       <c r="A78" s="13" t="inlineStr">
         <is>
           <t>R-36</t>
@@ -8996,7 +8898,7 @@
       </c>
       <c r="G78" s="13" t="inlineStr">
         <is>
-          <t>未測試</t>
+          <t>部分通過</t>
         </is>
       </c>
       <c r="I78" s="6" t="inlineStr">
@@ -9024,15 +8926,21 @@
           <t>P1-12</t>
         </is>
       </c>
+      <c r="N78" s="6" t="inlineStr">
+        <is>
+          <t>真機 62:70（2026-10-15，r-36 rebase 到 dev 1bd85ac，-localall 1.7.2，本機 3230/7870）：① 09:45:10 後台解綁 → 語音伺服器只在 09:45:11 拒絕 1 次，串口『device token refused, pausing』，之後只見 generate_auth_token 202 輪詢（約 70 秒 4 次）② 09:46:36 重新認領 → 09:46:53 自動連上（17 秒）並播出開場白，沒按鍵、沒重開 ④ 對照：改動前 1.7.0 解綁後每秒被拒 1 次（約 57 次/分鐘）。未做：③ 已綁定時斷網 30 秒再恢復；洋紅慢閃燈號未目視；⑤ 隨 OTA 推出</t>
+        </is>
+      </c>
       <c r="O78" s="13" t="inlineStr">
         <is>
-          <t>e964851</t>
+          <t>1bd85ac</t>
         </is>
       </c>
       <c r="P78" s="6" t="inlineStr">
         <is>
           <t>[2026-10-12] 新增：2026-10-12 從 P1-12 真機測試拆出。
-[2026-10-12] 2026-10-12 韌體已改（分支 r-36-unclaimed-idle，以 mygithub/main 為基礎）：token 在 auth 前被拒就暫停 websocket（networkTask 不再呼叫 webSocket.loop），只有 startSessionIfReady 拿到新 token 才恢復；202 時清掉舊 token、標記未認領，閒置時 LED 慢閃洋紅（有螢幕的板顯示 NOT PAIRED）。spotpear-ai-toy 和 -localall 都編譯通過（Flash 75.6%）。真機測試未做：62:70 未接上，Mac 當時不在公司網絡。</t>
+[2026-10-12] 2026-10-12 韌體已改（分支 r-36-unclaimed-idle，以 mygithub/main 為基礎）：token 在 auth 前被拒就暫停 websocket（networkTask 不再呼叫 webSocket.loop），只有 startSessionIfReady 拿到新 token 才恢復；202 時清掉舊 token、標記未認領，閒置時 LED 慢閃洋紅（有螢幕的板顯示 NOT PAIRED）。spotpear-ai-toy 和 -localall 都編譯通過（Flash 75.6%）。真機測試未做：62:70 未接上，Mac 當時不在公司網絡。
+[2026-10-15] rebase 衝突在 networkTask：R-36 的暫停條件和 R-41 的 reportPower() 都保留（reportPower 自己檢查連線）。分支未推送。</t>
         </is>
       </c>
     </row>
@@ -9306,7 +9214,7 @@
         </is>
       </c>
     </row>
-    <row r="83" ht="214" customHeight="1">
+    <row r="83" ht="172" customHeight="1">
       <c r="A83" s="13" t="inlineStr">
         <is>
           <t>P2-14</t>
@@ -9334,12 +9242,17 @@
       </c>
       <c r="F83" s="13" t="inlineStr">
         <is>
-          <t>進行中</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="G83" s="13" t="inlineStr">
         <is>
-          <t>部分通過</t>
+          <t>通過</t>
+        </is>
+      </c>
+      <c r="H83" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="I83" s="6" t="inlineStr">
@@ -9371,13 +9284,19 @@
       </c>
       <c r="N83" s="6" t="inlineStr">
         <is>
-          <t>本機（未 commit）：migration 20261014140000 套用兩次無錯。探測腳本用 GoTrue 真實登入：超管 admin_list_devices 200（不含 user_code）；④ 內容管理員 → 42501、anon → 42501；超管直接讀 device_secrets → 42501；空原因 → 22023；重置密鑰 → device_secrets 行刪除；解綁 → user_id/claimed_at 清空；兩者各寫 1 筆含原因與前後值的審計，超管改審計 → 403。網頁（獨立副本+獨立語音伺服器 7871）：模擬 62:70 連上 → 15 秒內不刷新顯示 Online、-52 dBm；斷線後下一次輪詢變 Offline；按 f214 搜尋、強制解綁、重置密鑰、審計頁都看到兩筆；375px 無橫向捲動。pytest 71 passed。未做：① ② ③ 需真板 62:70，且要用新代碼重啟 7860 語音伺服器</t>
+          <t>真機 62:70（2026-10-15，分支 hw-test-1015 = dev+P2-16，-localall 1.7.0，本機網頁 3230 + 語音 7870）：① 開機 → 設備頁 Online、-67 dBm、1.7.0；板子停在 bootloader 約 38 秒後語音伺服器判離線（uvicorn ping 超時），頁面 0 台在線 ② 重置設備密鑰 → device_secrets 行刪除，板子重開印『Device secret issued and stored』並連上，行恢復 ③ 強制解綁 → 板子拿 202（配對碼 UKDM7N），語音伺服器拒絕連線；兩項審計各 1 筆含操作者與原因 ④ 內容管理員/anon → 42501（10-14 探測腳本）</t>
+        </is>
+      </c>
+      <c r="O83" s="13" t="inlineStr">
+        <is>
+          <t>1d31bb0</t>
         </is>
       </c>
       <c r="P83" s="6" t="inlineStr">
         <is>
           <t>[2026-10-14] 新增
-[2026-10-14] devices.ip_key 未有（R-38），IP 欄暫顯示「未鎖定」。部署要三件一起：migration、語音伺服器（/internal/devices_presence）、網頁。在線只代表有語音連線，睡眠和關機都算離線。</t>
+[2026-10-14] devices.ip_key 未有（R-38），IP 欄暫顯示「未鎖定」。部署要三件一起：migration、語音伺服器（/internal/devices_presence）、網頁。在線只代表有語音連線，睡眠和關機都算離線。
+[2026-10-15] 頁面在分頁不可見時不輪詢（設計如此），可見時立即刷新。測完已用 SQL 把 62:70 綁回 multi-device-test@example.test。</t>
         </is>
       </c>
     </row>
@@ -9448,7 +9367,7 @@
         </is>
       </c>
     </row>
-    <row r="85" ht="326" customHeight="1">
+    <row r="85" ht="409" customHeight="1">
       <c r="A85" s="13" t="inlineStr">
         <is>
           <t>P2-16</t>
@@ -9476,12 +9395,17 @@
       </c>
       <c r="F85" s="13" t="inlineStr">
         <is>
-          <t>進行中</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="G85" s="13" t="inlineStr">
         <is>
-          <t>部分通過</t>
+          <t>通過</t>
+        </is>
+      </c>
+      <c r="H85" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="I85" s="6" t="inlineStr">
@@ -9513,7 +9437,12 @@
       </c>
       <c r="N85" s="6" t="inlineStr">
         <is>
-          <t>子任務 P2-17～P2-20 通過、P2-21 部分通過（等 P2-14）。① 10% 階段只有雜湊預測的那組拿到、重複不變（P2-18、P2-21）② 2 台回滾 → 自動暫停、其餘不再拿到（P2-19、P2-21）③ 100% 全部拿到 ⑤ 審計表有每次階段變更（P2-21 9 筆）。未做：④ 開發板 62:70 實機走一次白名單階段（用戶目前手上沒有板子），同時驗證新韌體開機印出 BUILD_INFO</t>
+          <t>④ 真機 62:70（2026-10-15）：USB 刷 1.7.0（開機印 aibuddy-build;kind=dev;…;version=1.7.0）→ release_firmware.py publish --dev 1.7.1 → 後台白名單加 62:70、改白名單階段、設為 current → 按 BOOT 喚醒：取 token 200、下載 12.8s、重開進 app1，09:39:36 連上語音伺服器；09:42 重開 → 『Firmware 1.7.1 on app1』無 probation、Up to date；頁面『Rolling out · Whitelist』運行 1 台、回滾 0；審計 5 筆（發佈、白名單、階段、1.6.2 取消 current、1.7.1 設 current）。①②③⑤ 見 P2-17～P2-21 模擬 20 台</t>
+        </is>
+      </c>
+      <c r="O85" s="13" t="inlineStr">
+        <is>
+          <t>e0d7ac6</t>
         </is>
       </c>
       <c r="P85" s="6" t="inlineStr">
@@ -9522,7 +9451,8 @@
 [2026-10-14] 2026-10-14 開分支 p2-16-ota-rollout（worktree ../aibuddy-p216，從 dev cac98aa）；拆成 P2-17～P2-21 五項子任務，本項的測試方法即整體驗收（含 62:70 實機白名單）。
 [2026-10-14] 2026-10-14 用戶決定提前到第 2 階段，現在開始做
 [2026-10-14] 2026-10-14 用戶決定拿走「同一台重啟 3 次即暫停」，原因見 P2-19
-[2026-10-14] 部署清單：① migrations 20261014190000、200000、210000、220000（依序，在 10-14 release 的 7 個之後）② 網頁 image ③ nginx 網頁 location 加 client_max_body_size 16m，curl 上傳 2MB 不得 413 ④ 韌體 BUILD_INFO 隨下一版韌體出，之前的版本仍用 release_firmware.py 發佈。分支 p2-16-ota-rollout 6 個 commit，未合併 dev、未推送</t>
+[2026-10-14] 部署清單：① migrations 20261014190000、200000、210000、220000（依序，在 10-14 release 的 7 個之後）② 網頁 image ③ nginx 網頁 location 加 client_max_body_size 16m，curl 上傳 2MB 不得 413 ④ 韌體 BUILD_INFO 隨下一版韌體出，之前的版本仍用 release_firmware.py 發佈。分支 p2-16-ota-rollout 6 個 commit，未合併 dev、未推送
+[2026-10-15] 附帶：一開始本機 current 是 1.6.2（以舊 IP/端口編譯），1.7.0 開機就被推 1.6.2，裝上後連不上，試用期內重開即回到 1.7.0（非崩潰，判定會再試），回滾路徑實機正常。之後用 SQL 暫停 1.6.2。用腳本發佈的新版本要重新載入 OTA 頁才出現。</t>
         </is>
       </c>
     </row>
@@ -10148,7 +10078,7 @@
         </is>
       </c>
     </row>
-    <row r="94" ht="312" customHeight="1">
+    <row r="94" ht="116" customHeight="1">
       <c r="A94" s="13" t="inlineStr">
         <is>
           <t>P2-21</t>
@@ -10176,12 +10106,17 @@
       </c>
       <c r="F94" s="13" t="inlineStr">
         <is>
-          <t>進行中</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="G94" s="13" t="inlineStr">
         <is>
-          <t>部分通過</t>
+          <t>通過</t>
+        </is>
+      </c>
+      <c r="H94" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="I94" s="6" t="inlineStr">
@@ -10211,7 +10146,7 @@
       </c>
       <c r="N94" s="6" t="inlineStr">
         <is>
-          <t>本機（分支 dev server 3216 + 本機 Supabase，GoTrue 真實登入的超管 cookie），用 xmini-c3 板型 + 20 台模擬設備以免碰到真開發板：頁面上傳 9.9.0 → 草稿；白名單加 1 台（UI 選單）→ 存檔；設為 current → 頁面預測 1 台、模擬 1 台；推進 10% → 預測 4、實得 4（重複不變）；50% → 預測 9、實得 9 且包含 10% 全部；100% → 20/20。2 台回滾 → 頁面顯示 'Paused … by the server: Auto-paused: 2 of 20 boards rolled back (10%)' 與回滾清單 2 台；點回滾設備 → 設備頁已帶 MAC 搜尋；恢復 → 其餘 18 台再拿到、回滾的 2 台不再下發；手動暫停未填原因不能確認、填後顯示 'by an admin'。審計頁 9 筆（上傳、白名單、current、10/50/100%、系統暫停、恢復、手動暫停），系統暫停顯示 System。375px scrollWidth=375。內容管理員側欄只有 Characters/IPs、#ota 退回 Characters、頁面無 OTA 數據，直接呼叫 admin_change_firmware_rollout → 403/42501。測試中發現並修正：舊版本（含 63:64 仍在跑的 1.6.1）被當成可刪除的草稿（6c2dc9d）。測試數據已清除</t>
+          <t>10-14 模擬 20 台全部通過（見上次）；2026-10-15 真機補做：OTA 頁對 1.7.1 白名單加 62:70（UI MAC 欄）→ 存檔確認框 → 『Narrow to Whitelist』確認 → Make current（用戶點）→ 62:70 安裝並確認，頁面顯示 Rolling out · Whitelist、運行 1、回滾 0；每步一筆審計。依賴 P2-14 已完成</t>
         </is>
       </c>
       <c r="O94" s="13" t="inlineStr">
@@ -10888,7 +10823,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I303"/>
+  <dimension ref="A1:I307"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -21395,8 +21330,192 @@
         </is>
       </c>
     </row>
+    <row r="304" ht="144" customHeight="1">
+      <c r="A304" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-15 09:43</t>
+        </is>
+      </c>
+      <c r="B304" s="13" t="inlineStr">
+        <is>
+          <t>P2-14</t>
+        </is>
+      </c>
+      <c r="C304" s="6" t="inlineStr">
+        <is>
+          <t>Admin 設備頁：每台玩具的狀態、韌體與基本操作</t>
+        </is>
+      </c>
+      <c r="D304" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="E304" s="13" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="F304" s="13" t="inlineStr">
+        <is>
+          <t>通過</t>
+        </is>
+      </c>
+      <c r="G304" s="6" t="inlineStr">
+        <is>
+          <t>真機 62:70（2026-10-15，分支 hw-test-1015 = dev+P2-16，-localall 1.7.0，本機網頁 3230 + 語音 7870）：① 開機 → 設備頁 Online、-67 dBm、1.7.0；板子停在 bootloader 約 38 秒後語音伺服器判離線（uvicorn ping 超時），頁面 0 台在線 ② 重置設備密鑰 → device_secrets 行刪除，板子重開印『Device secret issued and stored』並連上，行恢復 ③ 強制解綁 → 板子拿 202（配對碼 UKDM7N），語音伺服器拒絕連線；兩項審計各 1 筆含操作者與原因 ④ 內容管理員/anon → 42501（10-14 探測腳本）</t>
+        </is>
+      </c>
+      <c r="H304" s="13" t="inlineStr">
+        <is>
+          <t>1d31bb0</t>
+        </is>
+      </c>
+      <c r="I304" s="6" t="inlineStr">
+        <is>
+          <t>頁面在分頁不可見時不輪詢（設計如此），可見時立即刷新。測完已用 SQL 把 62:70 綁回 multi-device-test@example.test。</t>
+        </is>
+      </c>
+    </row>
+    <row r="305" ht="144" customHeight="1">
+      <c r="A305" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-15 09:43</t>
+        </is>
+      </c>
+      <c r="B305" s="13" t="inlineStr">
+        <is>
+          <t>P2-16</t>
+        </is>
+      </c>
+      <c r="C305" s="6" t="inlineStr">
+        <is>
+          <t>OTA 分批推送與後台發佈頁</t>
+        </is>
+      </c>
+      <c r="D305" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="E305" s="13" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="F305" s="13" t="inlineStr">
+        <is>
+          <t>通過</t>
+        </is>
+      </c>
+      <c r="G305" s="6" t="inlineStr">
+        <is>
+          <t>④ 真機 62:70（2026-10-15）：USB 刷 1.7.0（開機印 aibuddy-build;kind=dev;…;version=1.7.0）→ release_firmware.py publish --dev 1.7.1 → 後台白名單加 62:70、改白名單階段、設為 current → 按 BOOT 喚醒：取 token 200、下載 12.8s、重開進 app1，09:39:36 連上語音伺服器；09:42 重開 → 『Firmware 1.7.1 on app1』無 probation、Up to date；頁面『Rolling out · Whitelist』運行 1 台、回滾 0；審計 5 筆（發佈、白名單、階段、1.6.2 取消 current、1.7.1 設 current）。①②③⑤ 見 P2-17～P2-21 模擬 20 台</t>
+        </is>
+      </c>
+      <c r="H305" s="13" t="inlineStr">
+        <is>
+          <t>e0d7ac6</t>
+        </is>
+      </c>
+      <c r="I305" s="6" t="inlineStr">
+        <is>
+          <t>附帶：一開始本機 current 是 1.6.2（以舊 IP/端口編譯），1.7.0 開機就被推 1.6.2，裝上後連不上，試用期內重開即回到 1.7.0（非崩潰，判定會再試），回滾路徑實機正常。之後用 SQL 暫停 1.6.2。用腳本發佈的新版本要重新載入 OTA 頁才出現。</t>
+        </is>
+      </c>
+    </row>
+    <row r="306" ht="88" customHeight="1">
+      <c r="A306" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-15 09:43</t>
+        </is>
+      </c>
+      <c r="B306" s="13" t="inlineStr">
+        <is>
+          <t>P2-21</t>
+        </is>
+      </c>
+      <c r="C306" s="6" t="inlineStr">
+        <is>
+          <t>P2-16 ⑤ 後台 OTA 頁換成真實數據與操作</t>
+        </is>
+      </c>
+      <c r="D306" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="E306" s="13" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="F306" s="13" t="inlineStr">
+        <is>
+          <t>通過</t>
+        </is>
+      </c>
+      <c r="G306" s="6" t="inlineStr">
+        <is>
+          <t>10-14 模擬 20 台全部通過（見上次）；2026-10-15 真機補做：OTA 頁對 1.7.1 白名單加 62:70（UI MAC 欄）→ 存檔確認框 → 『Narrow to Whitelist』確認 → Make current（用戶點）→ 62:70 安裝並確認，頁面顯示 Rolling out · Whitelist、運行 1、回滾 0；每步一筆審計。依賴 P2-14 已完成</t>
+        </is>
+      </c>
+      <c r="H306" s="13" t="inlineStr">
+        <is>
+          <t>e0d7ac6</t>
+        </is>
+      </c>
+      <c r="I306" s="6" t="n"/>
+    </row>
+    <row r="307" ht="144" customHeight="1">
+      <c r="A307" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-15 09:48</t>
+        </is>
+      </c>
+      <c r="B307" s="13" t="inlineStr">
+        <is>
+          <t>R-36</t>
+        </is>
+      </c>
+      <c r="C307" s="6" t="inlineStr">
+        <is>
+          <t>未認領的設備停在配對狀態，不再每秒重連 websocket</t>
+        </is>
+      </c>
+      <c r="D307" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="E307" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F307" s="13" t="inlineStr">
+        <is>
+          <t>部分通過</t>
+        </is>
+      </c>
+      <c r="G307" s="6" t="inlineStr">
+        <is>
+          <t>真機 62:70（2026-10-15，r-36 rebase 到 dev 1bd85ac，-localall 1.7.2，本機 3230/7870）：① 09:45:10 後台解綁 → 語音伺服器只在 09:45:11 拒絕 1 次，串口『device token refused, pausing』，之後只見 generate_auth_token 202 輪詢（約 70 秒 4 次）② 09:46:36 重新認領 → 09:46:53 自動連上（17 秒）並播出開場白，沒按鍵、沒重開 ④ 對照：改動前 1.7.0 解綁後每秒被拒 1 次（約 57 次/分鐘）。未做：③ 已綁定時斷網 30 秒再恢復；洋紅慢閃燈號未目視；⑤ 隨 OTA 推出</t>
+        </is>
+      </c>
+      <c r="H307" s="13" t="inlineStr">
+        <is>
+          <t>1bd85ac</t>
+        </is>
+      </c>
+      <c r="I307" s="6" t="inlineStr">
+        <is>
+          <t>rebase 衝突在 networkTask：R-36 的暫停條件和 R-41 的 reportPower() 都保留（reportPower 自己檢查連線）。分支未推送。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I303"/>
+  <autoFilter ref="A1:I307"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Track P2-23: seamless OTA, downloaded before idle sleep and applied on wake.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/production-readiness.xlsx
+++ b/docs/production-readiness.xlsx
@@ -13,9 +13,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="更新記錄" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'任務清單'!$A$1:$P$95</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'任務清單'!$A$1:$P$96</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'待確認問題'!$A$1:$G$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$307</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$309</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -665,14 +665,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>最後更新：2026-10-15 09:48　·　本頁由 tracker.py 自動生成，請勿手動編輯</t>
+          <t>最後更新：2026-10-15 09:50　·　本頁由 tracker.py 自動生成，請勿手動編輯</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>總進度：25/90 已完成（28%）　·　目前階段：1 止血定案（10/5–10/16）</t>
+          <t>總進度：25/91 已完成（27%）　·　目前階段：1 止血定案（10/5–10/16）</t>
         </is>
       </c>
     </row>
@@ -816,11 +816,11 @@
       </c>
       <c r="C8" s="7">
         <f>COUNTIF('任務清單'!$B:$B,$A8)</f>
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D8" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A8,'任務清單'!$F:$F,D$5)</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E8" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A8,'任務清單'!$F:$F,E$5)</f>
@@ -840,7 +840,7 @@
       </c>
       <c r="I8" s="8">
         <f>IFERROR(F8/(C8-H8),0)</f>
-        <v>0.45454545454545453</v>
+        <v>0.43478260869565216</v>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1">
@@ -892,11 +892,11 @@
       <c r="B10" s="6" t="n"/>
       <c r="C10" s="5">
         <f>SUM(C6:C9)</f>
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D10" s="5">
         <f>SUM(D6:D9)</f>
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E10" s="5">
         <f>SUM(E6:E9)</f>
@@ -916,7 +916,7 @@
       </c>
       <c r="I10" s="9">
         <f>IFERROR(F10/(C10-H10),0)</f>
-        <v>0.2777777777777778</v>
+        <v>0.27472527472527475</v>
       </c>
     </row>
     <row r="12">
@@ -1059,11 +1059,11 @@
       </c>
       <c r="C15" s="7">
         <f>COUNTIF('任務清單'!$C:$C,$A15)</f>
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D15" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A15,'任務清單'!$F:$F,D$12)</f>
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E15" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A15,'任務清單'!$F:$F,E$12)</f>
@@ -1135,11 +1135,11 @@
       <c r="B17" s="6" t="n"/>
       <c r="C17" s="5">
         <f>SUM(C13:C16)</f>
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D17" s="5">
         <f>SUM(D13:D16)</f>
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E17" s="5">
         <f>SUM(E13:E16)</f>
@@ -1159,7 +1159,7 @@
       </c>
       <c r="I17" s="9">
         <f>IFERROR(F17/(C17-H17),0)</f>
-        <v>0.2777777777777778</v>
+        <v>0.27472527472527475</v>
       </c>
     </row>
     <row r="19">
@@ -3240,7 +3240,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P95"/>
+  <dimension ref="A1:P96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -10241,8 +10241,76 @@
         </is>
       </c>
     </row>
+    <row r="96" ht="200" customHeight="1">
+      <c r="A96" s="13" t="inlineStr">
+        <is>
+          <t>P2-23</t>
+        </is>
+      </c>
+      <c r="B96" s="13" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C96" s="13" t="inlineStr">
+        <is>
+          <t>3 封閉內測</t>
+        </is>
+      </c>
+      <c r="D96" s="6" t="inlineStr">
+        <is>
+          <t>OTA/韌體</t>
+        </is>
+      </c>
+      <c r="E96" s="6" t="inlineStr">
+        <is>
+          <t>無感 OTA：閒置入睡前在背景下載，下次喚醒時生效</t>
+        </is>
+      </c>
+      <c r="F96" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="G96" s="13" t="inlineStr">
+        <is>
+          <t>未測試</t>
+        </is>
+      </c>
+      <c r="I96" s="6" t="inlineStr">
+        <is>
+          <t>現在 OTA 在開機時進行：開機取 token 時後端說要更新，板子就下載、重開，之後才開語音。2026-10-15 在 62:70 實測（本機 HTTP、1.52 MB），從開機到新版本能對話約 15 秒，其中下載 12.8 秒；雲端經 HTTPS／Cloudflare 未量，應更長。孩子按開機後要等這麼久玩具才說話，會覺得壞了。</t>
+        </is>
+      </c>
+      <c r="J96" s="6" t="inlineStr">
+        <is>
+          <t>firmware-arduino/src/OTA.cpp（otaCheckAndUpdate、installImage）、src/Audio.cpp（enterSleep、閒置睡眠 IDLE_SLEEP_SECONDS）、src/SupplyMonitor.cpp（低電判斷）；伺服器不用改（offer 仍隨 /api/generate_auth_token 回來）</t>
+        </is>
+      </c>
+      <c r="K96" s="6" t="inlineStr">
+        <is>
+          <t>① 開機只記下 offer，不下載、不重開；照常開 websocket 對話 ② 閒置準備入睡時（websocket 已關，C3 只有一條 TLS），如有未裝的 offer 就下載到另一個槽並校驗 SHA-256，成功後才入睡；下次喚醒的重開即進新版本，試用期與回滾照舊 ③ 下載中按 BOOT（孩子要說話）→ Update.abort，立即回到對話，下次入睡再試；不算失敗次數 ④ 電量低（supplyLow／電池低）不下載 ⑤ 已下載但未生效時再開機，不重複下載（slot 已設為下次啟動） ⑥ 有 offer 超過 N 天（預設 3 天）都沒機會在入睡時裝，就退回開機時安裝 ⑦ 下載期間 LED 和平時入睡一致，不播提示音 ⑧ 可選：映像 gzip 壓縮下載（10-15 實測 1,592,176 → 999,108 bytes），固件邊下邊解壓</t>
+        </is>
+      </c>
+      <c r="L96" s="6" t="inlineStr">
+        <is>
+          <t>62:70（-localall）：① 發佈新版本後開機 → 串口記下 offer，3 秒內連上語音並播開場白，無下載 ② 閒置至入睡 → 串口顯示下載與 SHA-256 通過後才 Sleeping；按 BOOT 喚醒 → 新版本 on 新槽、probation，120 秒後 confirmed，從按鍵到開場白的時間和沒有更新時相差 ≤ 2 秒 ③ 入睡下載中按 BOOT → 1 秒內回到對話，新槽不生效，下次入睡重下成功 ④ 強制低電 build → 入睡時跳過下載 ⑤ 已下載未生效時拔電重開 → 進新版本、不重下 ⑥ 把 N 調成 0 → 開機即安裝（舊行為）⑦ 量一次雲端 HTTPS 下載時間（等雲端可測時）</t>
+        </is>
+      </c>
+      <c r="M96" s="13" t="inlineStr">
+        <is>
+          <t>P2-16</t>
+        </is>
+      </c>
+      <c r="P96" s="6" t="inlineStr">
+        <is>
+          <t>[2026-10-15] 新增
+[2026-10-15] 2026-10-15 用戶要求。最好趕上 11/27 交 Spotpear 的出廠映像；趕不上也能經 OTA 推出，只是那一次更新仍要開機時等。依賴 P2-16（分批推送，已完成）。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P95"/>
+  <autoFilter ref="A1:P96"/>
   <conditionalFormatting sqref="F2:F1000">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"已完成"</formula>
@@ -10823,7 +10891,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I307"/>
+  <dimension ref="A1:I309"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -21514,8 +21582,70 @@
         </is>
       </c>
     </row>
+    <row r="308" ht="32" customHeight="1">
+      <c r="A308" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-15 09:50</t>
+        </is>
+      </c>
+      <c r="B308" s="13" t="inlineStr">
+        <is>
+          <t>P2-23</t>
+        </is>
+      </c>
+      <c r="C308" s="6" t="inlineStr">
+        <is>
+          <t>無感 OTA：閒置入睡前在背景下載，下次喚醒時生效</t>
+        </is>
+      </c>
+      <c r="E308" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="I308" s="6" t="inlineStr">
+        <is>
+          <t>新增任務</t>
+        </is>
+      </c>
+    </row>
+    <row r="309" ht="74" customHeight="1">
+      <c r="A309" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-15 09:50</t>
+        </is>
+      </c>
+      <c r="B309" s="13" t="inlineStr">
+        <is>
+          <t>P2-23</t>
+        </is>
+      </c>
+      <c r="C309" s="6" t="inlineStr">
+        <is>
+          <t>無感 OTA：閒置入睡前在背景下載，下次喚醒時生效</t>
+        </is>
+      </c>
+      <c r="D309" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E309" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="F309" s="13" t="n"/>
+      <c r="G309" s="6" t="n"/>
+      <c r="H309" s="13" t="n"/>
+      <c r="I309" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-15 用戶要求。最好趕上 11/27 交 Spotpear 的出廠映像；趕不上也能經 OTA 推出，只是那一次更新仍要開機時等。依賴 P2-16（分批推送，已完成）。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I307"/>
+  <autoFilter ref="A1:I309"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Track R-37 ⑦ (switch Wi-Fi) on 62:70: both fallbacks pass, success path to do.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/production-readiness.xlsx
+++ b/docs/production-readiness.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'任務清單'!$A$1:$P$96</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'待確認問題'!$A$1:$G$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$309</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$312</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -665,7 +665,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>最後更新：2026-10-15 09:50　·　本頁由 tracker.py 自動生成，請勿手動編輯</t>
+          <t>最後更新：2026-10-15 10:26　·　本頁由 tracker.py 自動生成，請勿手動編輯</t>
         </is>
       </c>
     </row>
@@ -1549,7 +1549,7 @@
       <c r="H31" s="11" t="n"/>
       <c r="I31" s="12" t="n"/>
     </row>
-    <row r="32" ht="256" customHeight="1">
+    <row r="32" ht="172" customHeight="1">
       <c r="A32" s="13" t="inlineStr">
         <is>
           <t>R-36</t>
@@ -1572,7 +1572,7 @@
       </c>
       <c r="E32" s="6" t="inlineStr">
         <is>
-          <t>上次測試：部分通過 — 真機 62:70（2026-10-15，r-36 rebase 到 dev 1bd85ac，-localall 1.7.2，本機 3230/7870）：① 09:45:10 後台解綁 → 語音伺服器只在 09:45:11 拒絕 1 次，串口『device token refused, pausing』，之後只見 generate_auth_token 202 輪詢（約 70 秒 4 次）② 09:46:36 重新認領 → 09:46:53 自動連上（17 秒）並播出開場白，沒按鍵、沒重開 ④ 對照：改動前 1.7.0 解綁後每秒被拒 1 次（約 57 次/分鐘）。未做：③ 已綁定時斷網 30 秒再恢復；洋紅慢閃燈號未目視；⑤ 隨 OTA 推出
+          <t>上次測試：部分通過 — 補充 2026-10-15（1.7.5，含 R-36）：已綁定時兩次 Wi-Fi 切換各斷網 9–11 秒，都自動重連並重新 auth，沒有停在暫停狀態；30 秒斷網仍未做
 ① 拿到 202 或 websocket 被 4401 拒絕後，設備停掉 websocket 自動重連，進入待綁定狀態（燈號可分辨）。② 待綁定時只按退避（5 秒起、上限 PROVISION_BACKOFF_MAX）呼叫 generate_auth_token，不開 websocket。③ 被認領後下一次輪詢拿到 200，在 10 秒內（加退避）自動開 websocket 並能對話，不用重開機。④ 已綁定設備網絡斷線重連的行為不變。⑤ 隨 OTA 推出。</t>
         </is>
       </c>
@@ -1645,7 +1645,7 @@
       <c r="H34" s="11" t="n"/>
       <c r="I34" s="12" t="n"/>
     </row>
-    <row r="35" ht="242" customHeight="1">
+    <row r="35" ht="409" customHeight="1">
       <c r="A35" s="13" t="inlineStr">
         <is>
           <t>R-37</t>
@@ -1668,8 +1668,8 @@
       </c>
       <c r="E35" s="6" t="inlineStr">
         <is>
-          <t>上次測試：部分通過 — 模擬玩具經本機語音服務器＋網頁：status/scan/add/delete 正常；刪除目前 Wi-Fi → current 被拒；斷線 5 秒內頁面顯示睡著、按鈕停用；測試密碼在語音服務器日誌、網頁服務器日誌、資料庫均搜不到；用別人裝置 ID 重放 server action → forbidden；pytest 17 項通過（全套 230）；韌體 spotpear-ai-toy-localall 編譯通過（RAM 17.5%、Flash 75.9%）。未測：真機 ①② 及 OTA 推出
-① 設定頁顯示玩具在線／離線、目前 Wi-Fi 和訊號、已記住的 Wi-Fi 清單（只有名稱，不顯示密碼）② 在線時可新增 Wi-Fi（輸入或從玩具掃描到的清單選）、刪除 Wi-Fi；不能刪除正在使用的那個 ③ 經 /ws/esp32 轉送：伺服器先確認是設備主人；密碼不寫入資料庫、不寫入日誌 ④ 新增不切換網絡，目前 Wi-Fi 消失時才按訊號選；清單標示「連過／未連過」⑤ 上限 8 個 ⑥ 韌體改動經 OTA 推出</t>
+          <t>上次測試：部分通過 — 2026-10-15 真機 62:70（hw-test-1015 = dev + P2-16 + R-36 + r-37-wifi-switch，1.7.5，本機 3230/7870）：① 熱點關掉 → 醒來重開後改連 HKQF - Guest 並上線（運行中途消失未單獨測）⑦ Use 按鈕、確認框（寫明 20 秒退回原網絡）、切換中提示都正常；熱點關著按 Use → 11 秒內頁面『couldn't find … nearby. It's back on HKQF - Guest』；熱點開著（到不了 Mac）→ 9 秒內『joined … but couldn't reach the internet … back on HKQF - Guest』，串口 failed (no_internet) → Back on；切換到目前網絡 → current、未存 SSID → unknown，板子不動。pytest 272 passed（新增 6 項），tsc 0 錯誤。未做：⑦ 成功切換（要第二個到得了 Mac 的網絡）、別人設備呼叫 switch → 403（同一個擁有者檢查，未對 switch 重測）、② 密碼打錯
+① 設定頁顯示玩具在線／離線、目前 Wi-Fi 和訊號、已記住的 Wi-Fi 清單（只有名稱，不顯示密碼）② 在線時可新增 Wi-Fi（輸入或從玩具掃描到的清單選）、刪除 Wi-Fi；不能刪除正在使用的那個 ③ 經 /ws/esp32 轉送：伺服器先確認是設備主人；密碼不寫入資料庫、不寫入日誌 ④ 新增不自動切換網絡；目前 Wi-Fi 消失時按訊號選，或由家長按「改用這個」（⑦）；清單標示「連過／未連過」⑤ 上限 8 個 ⑥ 韌體改動經 OTA 推出 ⑦ 已記住、未在使用的 Wi-Fi 可按「改用這個」：玩具斷開目前網絡改連它，最多 20 秒，要連上我們的伺服器才算成功；失敗就自動連回原網絡，頁面顯示「連不上 X，已回到 Y」；切換中頁面顯示切換中，玩具重新連上後刷新；成功後標示連過</t>
         </is>
       </c>
       <c r="F35" s="11" t="n"/>
@@ -8928,7 +8928,7 @@
       </c>
       <c r="N78" s="6" t="inlineStr">
         <is>
-          <t>真機 62:70（2026-10-15，r-36 rebase 到 dev 1bd85ac，-localall 1.7.2，本機 3230/7870）：① 09:45:10 後台解綁 → 語音伺服器只在 09:45:11 拒絕 1 次，串口『device token refused, pausing』，之後只見 generate_auth_token 202 輪詢（約 70 秒 4 次）② 09:46:36 重新認領 → 09:46:53 自動連上（17 秒）並播出開場白，沒按鍵、沒重開 ④ 對照：改動前 1.7.0 解綁後每秒被拒 1 次（約 57 次/分鐘）。未做：③ 已綁定時斷網 30 秒再恢復；洋紅慢閃燈號未目視；⑤ 隨 OTA 推出</t>
+          <t>補充 2026-10-15（1.7.5，含 R-36）：已綁定時兩次 Wi-Fi 切換各斷網 9–11 秒，都自動重連並重新 auth，沒有停在暫停狀態；30 秒斷網仍未做</t>
         </is>
       </c>
       <c r="O78" s="13" t="inlineStr">
@@ -8944,7 +8944,7 @@
         </is>
       </c>
     </row>
-    <row r="79" ht="270" customHeight="1">
+    <row r="79" ht="409" customHeight="1">
       <c r="A79" s="13" t="inlineStr">
         <is>
           <t>R-37</t>
@@ -8992,24 +8992,31 @@
       </c>
       <c r="K79" s="6" t="inlineStr">
         <is>
-          <t>① 設定頁顯示玩具在線／離線、目前 Wi-Fi 和訊號、已記住的 Wi-Fi 清單（只有名稱，不顯示密碼）② 在線時可新增 Wi-Fi（輸入或從玩具掃描到的清單選）、刪除 Wi-Fi；不能刪除正在使用的那個 ③ 經 /ws/esp32 轉送：伺服器先確認是設備主人；密碼不寫入資料庫、不寫入日誌 ④ 新增不切換網絡，目前 Wi-Fi 消失時才按訊號選；清單標示「連過／未連過」⑤ 上限 8 個 ⑥ 韌體改動經 OTA 推出</t>
+          <t>① 設定頁顯示玩具在線／離線、目前 Wi-Fi 和訊號、已記住的 Wi-Fi 清單（只有名稱，不顯示密碼）② 在線時可新增 Wi-Fi（輸入或從玩具掃描到的清單選）、刪除 Wi-Fi；不能刪除正在使用的那個 ③ 經 /ws/esp32 轉送：伺服器先確認是設備主人；密碼不寫入資料庫、不寫入日誌 ④ 新增不自動切換網絡；目前 Wi-Fi 消失時按訊號選，或由家長按「改用這個」（⑦）；清單標示「連過／未連過」⑤ 上限 8 個 ⑥ 韌體改動經 OTA 推出 ⑦ 已記住、未在使用的 Wi-Fi 可按「改用這個」：玩具斷開目前網絡改連它，最多 20 秒，要連上我們的伺服器才算成功；失敗就自動連回原網絡，頁面顯示「連不上 X，已回到 Y」；切換中頁面顯示切換中，玩具重新連上後刷新；成功後標示連過</t>
         </is>
       </c>
       <c r="L79" s="6" t="inlineStr">
         <is>
-          <t>① 網頁新增 Wi-Fi B，關掉 A → 玩具自動改連 B ② B 密碼打錯 → 玩具留在 A，B 標示未連過 ③ 嘗試刪除目前 Wi-Fi → 被拒 ④ 另一帳號呼叫同一接口 → 403 ⑤ 搜尋資料庫和伺服器日誌，找不到測試密碼 ⑥ 玩具離線時頁面顯示離線，新增按鈕停用</t>
+          <t>① 網頁新增 Wi-Fi B，關掉 A → 玩具自動改連 B ② B 密碼打錯 → 玩具留在 A，B 標示未連過 ③ 嘗試刪除目前 Wi-Fi → 被拒 ④ 另一帳號呼叫同一接口 → 403 ⑤ 搜尋資料庫和伺服器日誌，找不到測試密碼 ⑥ 玩具離線時頁面顯示離線，新增按鈕停用 ⑦ 62:70：對已存的手機熱點按「改用這個」→ 玩具改連熱點並在 30 秒內重新在線、頁面顯示熱點為目前 Wi-Fi；熱點關掉時按「改用這個」→ 20 秒後回到原網絡、頁面顯示失敗原因；對目前 Wi-Fi、未存的 SSID、別人的設備 → 被拒</t>
         </is>
       </c>
       <c r="M79" s="13" t="n"/>
       <c r="N79" s="6" t="inlineStr">
         <is>
-          <t>模擬玩具經本機語音服務器＋網頁：status/scan/add/delete 正常；刪除目前 Wi-Fi → current 被拒；斷線 5 秒內頁面顯示睡著、按鈕停用；測試密碼在語音服務器日誌、網頁服務器日誌、資料庫均搜不到；用別人裝置 ID 重放 server action → forbidden；pytest 17 項通過（全套 230）；韌體 spotpear-ai-toy-localall 編譯通過（RAM 17.5%、Flash 75.9%）。未測：真機 ①② 及 OTA 推出</t>
+          <t>2026-10-15 真機 62:70（hw-test-1015 = dev + P2-16 + R-36 + r-37-wifi-switch，1.7.5，本機 3230/7870）：① 熱點關掉 → 醒來重開後改連 HKQF - Guest 並上線（運行中途消失未單獨測）⑦ Use 按鈕、確認框（寫明 20 秒退回原網絡）、切換中提示都正常；熱點關著按 Use → 11 秒內頁面『couldn't find … nearby. It's back on HKQF - Guest』；熱點開著（到不了 Mac）→ 9 秒內『joined … but couldn't reach the internet … back on HKQF - Guest』，串口 failed (no_internet) → Back on；切換到目前網絡 → current、未存 SSID → unknown，板子不動。pytest 272 passed（新增 6 項），tsc 0 錯誤。未做：⑦ 成功切換（要第二個到得了 Mac 的網絡）、別人設備呼叫 switch → 403（同一個擁有者檢查，未對 switch 重測）、② 密碼打錯</t>
+        </is>
+      </c>
+      <c r="O79" s="13" t="inlineStr">
+        <is>
+          <t>3c180cd</t>
         </is>
       </c>
       <c r="P79" s="6" t="inlineStr">
         <is>
           <t>[2026-10-13] 新增：時間表（project-schedule.xlsx「Jacky 開發與測試」）排在 W4 11/2–11/6，和快活網頁核心一起；內部測試的家庭要加家裡的 Wi-Fi。
-[2026-10-13] 2026-10-13 應 Jacky 要求從 W4 提前開始。韌體：上限 8 個、NVS apOk%d 記錄連過、經 /ws/esp32 收 status/add/delete/scan、不刪不改目前 Wi-Fi、Wi-Fi 指令不印串口、修 delWifi 計數 bug。伺服器：device_wifi.py＋/internal/device_wifi（含 peek），密碼只轉送不留存。網頁：我 &gt; 裝置 &gt; Network &gt; Wi-Fi（Figma C4），deviceWifiAction 檢查擁有者。剩真機測試 ①②（需 62:70 刷 -localall＋兩個真實網絡）與 OTA。</t>
+[2026-10-13] 2026-10-13 應 Jacky 要求從 W4 提前開始。韌體：上限 8 個、NVS apOk%d 記錄連過、經 /ws/esp32 收 status/add/delete/scan、不刪不改目前 Wi-Fi、Wi-Fi 指令不印串口、修 delWifi 計數 bug。伺服器：device_wifi.py＋/internal/device_wifi（含 peek），密碼只轉送不留存。網頁：我 &gt; 裝置 &gt; Network &gt; Wi-Fi（Figma C4），deviceWifiAction 檢查擁有者。剩真機測試 ①②（需 62:70 刷 -localall＋兩個真實網絡）與 OTA。
+[2026-10-15] 2026-10-15 用戶決定：加「改用這個 Wi-Fi」（⑦），④ 改為新增不自動切換、可由家長手動切換。起因：62:70 實測加了 iPhone 熱點也無法讓玩具改用。另：離線一律顯示「睡著了」會誤導（63:64 已 6 天未上線仍叫人按按鈕），待改為按上次上線時間分開提示。
+[2026-10-15] 測試中修了原有 bug（a4 之後第二個 commit）：驅動在沒連上的網絡斷開時不發事件，WiFi.status() 留著上次的『找不到』，新嘗試一開始就被當失敗；1.7.4 切換失敗後連不回 Guest 並掉進 SoftAP，tryConnect() 也同樣。joinFor() 改為 6 秒後才相信失敗，tryConnect() 共用。雲端韌體同樣有這 bug。另：開機時 tryConnect() 挑最強的網絡但不檢查能否到伺服器，62:70 開機連上到不了 Mac 的熱點後一直卡著（見 P2-22 ④ 或另開任務）。分支 r-37-wifi-switch 未推送。</t>
         </is>
       </c>
     </row>
@@ -10891,7 +10898,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I309"/>
+  <dimension ref="A1:I312"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -21644,8 +21651,129 @@
         </is>
       </c>
     </row>
+    <row r="310" ht="116" customHeight="1">
+      <c r="A310" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-15 10:04</t>
+        </is>
+      </c>
+      <c r="B310" s="13" t="inlineStr">
+        <is>
+          <t>R-37</t>
+        </is>
+      </c>
+      <c r="C310" s="6" t="inlineStr">
+        <is>
+          <t>網頁設定玩具的 Wi-Fi：查看、新增、刪除</t>
+        </is>
+      </c>
+      <c r="D310" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="E310" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F310" s="13" t="n"/>
+      <c r="G310" s="6" t="n"/>
+      <c r="H310" s="13" t="n"/>
+      <c r="I310" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-15 用戶決定：加「改用這個 Wi-Fi」（⑦），④ 改為新增不自動切換、可由家長手動切換。起因：62:70 實測加了 iPhone 熱點也無法讓玩具改用。另：離線一律顯示「睡著了」會誤導（63:64 已 6 天未上線仍叫人按按鈕），待改為按上次上線時間分開提示。；修改了驗收標準、測試方法</t>
+        </is>
+      </c>
+    </row>
+    <row r="311" ht="200" customHeight="1">
+      <c r="A311" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-15 10:26</t>
+        </is>
+      </c>
+      <c r="B311" s="13" t="inlineStr">
+        <is>
+          <t>R-37</t>
+        </is>
+      </c>
+      <c r="C311" s="6" t="inlineStr">
+        <is>
+          <t>網頁設定玩具的 Wi-Fi：查看、新增、刪除</t>
+        </is>
+      </c>
+      <c r="D311" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="E311" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F311" s="13" t="inlineStr">
+        <is>
+          <t>部分通過</t>
+        </is>
+      </c>
+      <c r="G311" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-15 真機 62:70（hw-test-1015 = dev + P2-16 + R-36 + r-37-wifi-switch，1.7.5，本機 3230/7870）：① 熱點關掉 → 醒來重開後改連 HKQF - Guest 並上線（運行中途消失未單獨測）⑦ Use 按鈕、確認框（寫明 20 秒退回原網絡）、切換中提示都正常；熱點關著按 Use → 11 秒內頁面『couldn't find … nearby. It's back on HKQF - Guest』；熱點開著（到不了 Mac）→ 9 秒內『joined … but couldn't reach the internet … back on HKQF - Guest』，串口 failed (no_internet) → Back on；切換到目前網絡 → current、未存 SSID → unknown，板子不動。pytest 272 passed（新增 6 項），tsc 0 錯誤。未做：⑦ 成功切換（要第二個到得了 Mac 的網絡）、別人設備呼叫 switch → 403（同一個擁有者檢查，未對 switch 重測）、② 密碼打錯</t>
+        </is>
+      </c>
+      <c r="H311" s="13" t="inlineStr">
+        <is>
+          <t>3c180cd</t>
+        </is>
+      </c>
+      <c r="I311" s="6" t="inlineStr">
+        <is>
+          <t>測試中修了原有 bug（a4 之後第二個 commit）：驅動在沒連上的網絡斷開時不發事件，WiFi.status() 留著上次的『找不到』，新嘗試一開始就被當失敗；1.7.4 切換失敗後連不回 Guest 並掉進 SoftAP，tryConnect() 也同樣。joinFor() 改為 6 秒後才相信失敗，tryConnect() 共用。雲端韌體同樣有這 bug。另：開機時 tryConnect() 挑最強的網絡但不檢查能否到伺服器，62:70 開機連上到不了 Mac 的熱點後一直卡著（見 P2-22 ④ 或另開任務）。分支 r-37-wifi-switch 未推送。</t>
+        </is>
+      </c>
+    </row>
+    <row r="312" ht="46" customHeight="1">
+      <c r="A312" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-15 10:26</t>
+        </is>
+      </c>
+      <c r="B312" s="13" t="inlineStr">
+        <is>
+          <t>R-36</t>
+        </is>
+      </c>
+      <c r="C312" s="6" t="inlineStr">
+        <is>
+          <t>未認領的設備停在配對狀態，不再每秒重連 websocket</t>
+        </is>
+      </c>
+      <c r="D312" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="E312" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F312" s="13" t="inlineStr">
+        <is>
+          <t>部分通過</t>
+        </is>
+      </c>
+      <c r="G312" s="6" t="inlineStr">
+        <is>
+          <t>補充 2026-10-15（1.7.5，含 R-36）：已綁定時兩次 Wi-Fi 切換各斷網 9–11 秒，都自動重連並重新 auth，沒有停在暫停狀態；30 秒斷網仍未做</t>
+        </is>
+      </c>
+      <c r="H312" s="13" t="n"/>
+      <c r="I312" s="6" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I309"/>
+  <autoFilter ref="A1:I312"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Point R-37 at the Wi-Fi join fix.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/production-readiness.xlsx
+++ b/docs/production-readiness.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'任務清單'!$A$1:$P$96</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'待確認問題'!$A$1:$G$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$312</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$313</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -9008,7 +9008,7 @@
       </c>
       <c r="O79" s="13" t="inlineStr">
         <is>
-          <t>3c180cd</t>
+          <t>22d7674</t>
         </is>
       </c>
       <c r="P79" s="6" t="inlineStr">
@@ -9016,7 +9016,8 @@
           <t>[2026-10-13] 新增：時間表（project-schedule.xlsx「Jacky 開發與測試」）排在 W4 11/2–11/6，和快活網頁核心一起；內部測試的家庭要加家裡的 Wi-Fi。
 [2026-10-13] 2026-10-13 應 Jacky 要求從 W4 提前開始。韌體：上限 8 個、NVS apOk%d 記錄連過、經 /ws/esp32 收 status/add/delete/scan、不刪不改目前 Wi-Fi、Wi-Fi 指令不印串口、修 delWifi 計數 bug。伺服器：device_wifi.py＋/internal/device_wifi（含 peek），密碼只轉送不留存。網頁：我 &gt; 裝置 &gt; Network &gt; Wi-Fi（Figma C4），deviceWifiAction 檢查擁有者。剩真機測試 ①②（需 62:70 刷 -localall＋兩個真實網絡）與 OTA。
 [2026-10-15] 2026-10-15 用戶決定：加「改用這個 Wi-Fi」（⑦），④ 改為新增不自動切換、可由家長手動切換。起因：62:70 實測加了 iPhone 熱點也無法讓玩具改用。另：離線一律顯示「睡著了」會誤導（63:64 已 6 天未上線仍叫人按按鈕），待改為按上次上線時間分開提示。
-[2026-10-15] 測試中修了原有 bug（a4 之後第二個 commit）：驅動在沒連上的網絡斷開時不發事件，WiFi.status() 留著上次的『找不到』，新嘗試一開始就被當失敗；1.7.4 切換失敗後連不回 Guest 並掉進 SoftAP，tryConnect() 也同樣。joinFor() 改為 6 秒後才相信失敗，tryConnect() 共用。雲端韌體同樣有這 bug。另：開機時 tryConnect() 挑最強的網絡但不檢查能否到伺服器，62:70 開機連上到不了 Mac 的熱點後一直卡著（見 P2-22 ④ 或另開任務）。分支 r-37-wifi-switch 未推送。</t>
+[2026-10-15] 測試中修了原有 bug（a4 之後第二個 commit）：驅動在沒連上的網絡斷開時不發事件，WiFi.status() 留著上次的『找不到』，新嘗試一開始就被當失敗；1.7.4 切換失敗後連不回 Guest 並掉進 SoftAP，tryConnect() 也同樣。joinFor() 改為 6 秒後才相信失敗，tryConnect() 共用。雲端韌體同樣有這 bug。另：開機時 tryConnect() 挑最強的網絡但不檢查能否到伺服器，62:70 開機連上到不了 Mac 的熱點後一直卡著（見 P2-22 ④ 或另開任務）。分支 r-37-wifi-switch 未推送。
+[2026-10-15] 更正上一條備註：stale『找不到』的修正是 22d7674（切換功能本身是 3c180cd）。</t>
         </is>
       </c>
     </row>
@@ -10898,7 +10899,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I312"/>
+  <dimension ref="A1:I313"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -21772,8 +21773,47 @@
       <c r="H312" s="13" t="n"/>
       <c r="I312" s="6" t="n"/>
     </row>
+    <row r="313" ht="46" customHeight="1">
+      <c r="A313" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-15 10:26</t>
+        </is>
+      </c>
+      <c r="B313" s="13" t="inlineStr">
+        <is>
+          <t>R-37</t>
+        </is>
+      </c>
+      <c r="C313" s="6" t="inlineStr">
+        <is>
+          <t>網頁設定玩具的 Wi-Fi：查看、新增、刪除</t>
+        </is>
+      </c>
+      <c r="D313" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="E313" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F313" s="13" t="n"/>
+      <c r="G313" s="6" t="n"/>
+      <c r="H313" s="13" t="inlineStr">
+        <is>
+          <t>22d7674</t>
+        </is>
+      </c>
+      <c r="I313" s="6" t="inlineStr">
+        <is>
+          <t>更正上一條備註：stale『找不到』的修正是 22d7674（切換功能本身是 3c180cd）。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I312"/>
+  <autoFilter ref="A1:I313"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Track P2-24 (ADPCM mic uplink) and P2-25 (C3 reconnect self-recovery).
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/production-readiness.xlsx
+++ b/docs/production-readiness.xlsx
@@ -13,9 +13,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="更新記錄" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'任務清單'!$A$1:$P$96</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'任務清單'!$A$1:$P$98</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'待確認問題'!$A$1:$G$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$313</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$315</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -641,7 +641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I103"/>
+  <dimension ref="A1:I104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -665,14 +665,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>最後更新：2026-10-15 10:26　·　本頁由 tracker.py 自動生成，請勿手動編輯</t>
+          <t>最後更新：2026-10-15 10:29　·　本頁由 tracker.py 自動生成，請勿手動編輯</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>總進度：25/91 已完成（27%）　·　目前階段：1 止血定案（10/5–10/16）</t>
+          <t>總進度：25/93 已完成（27%）　·　目前階段：1 止血定案（10/5–10/16）</t>
         </is>
       </c>
     </row>
@@ -816,11 +816,11 @@
       </c>
       <c r="C8" s="7">
         <f>COUNTIF('任務清單'!$B:$B,$A8)</f>
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D8" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A8,'任務清單'!$F:$F,D$5)</f>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E8" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A8,'任務清單'!$F:$F,E$5)</f>
@@ -840,7 +840,7 @@
       </c>
       <c r="I8" s="8">
         <f>IFERROR(F8/(C8-H8),0)</f>
-        <v>0.43478260869565216</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1">
@@ -892,11 +892,11 @@
       <c r="B10" s="6" t="n"/>
       <c r="C10" s="5">
         <f>SUM(C6:C9)</f>
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="D10" s="5">
         <f>SUM(D6:D9)</f>
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="E10" s="5">
         <f>SUM(E6:E9)</f>
@@ -916,7 +916,7 @@
       </c>
       <c r="I10" s="9">
         <f>IFERROR(F10/(C10-H10),0)</f>
-        <v>0.27472527472527475</v>
+        <v>0.26881720430107525</v>
       </c>
     </row>
     <row r="12">
@@ -1019,11 +1019,11 @@
       </c>
       <c r="C14" s="7">
         <f>COUNTIF('任務清單'!$C:$C,$A14)</f>
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D14" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A14,'任務清單'!$F:$F,D$12)</f>
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E14" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A14,'任務清單'!$F:$F,E$12)</f>
@@ -1043,7 +1043,7 @@
       </c>
       <c r="I14" s="8">
         <f>IFERROR(F14/(C14-H14),0)</f>
-        <v>0.30303030303030304</v>
+        <v>0.2857142857142857</v>
       </c>
     </row>
     <row r="15" ht="46" customHeight="1">
@@ -1135,11 +1135,11 @@
       <c r="B17" s="6" t="n"/>
       <c r="C17" s="5">
         <f>SUM(C13:C16)</f>
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="D17" s="5">
         <f>SUM(D13:D16)</f>
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="E17" s="5">
         <f>SUM(E13:E16)</f>
@@ -1159,7 +1159,7 @@
       </c>
       <c r="I17" s="9">
         <f>IFERROR(F17/(C17-H17),0)</f>
-        <v>0.27472527472527475</v>
+        <v>0.26881720430107525</v>
       </c>
     </row>
     <row r="19">
@@ -1801,15 +1801,15 @@
       <c r="H39" s="11" t="n"/>
       <c r="I39" s="12" t="n"/>
     </row>
-    <row r="40" ht="46" customHeight="1">
+    <row r="40" ht="102" customHeight="1">
       <c r="A40" s="13" t="inlineStr">
         <is>
-          <t>R-04</t>
+          <t>P2-24</t>
         </is>
       </c>
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>粵語質量評測</t>
+          <t>麥克風上行改用 IMA ADPCM（減少 4 倍頻寬）</t>
         </is>
       </c>
       <c r="C40" s="13" t="inlineStr">
@@ -1824,7 +1824,7 @@
       </c>
       <c r="E40" s="6" t="inlineStr">
         <is>
-          <t>有一套粵語評測集（兒童錄音＋文字提示）；選定的 STT 與 LLM 達到門檻：兒童語音字錯率 ≤15%、口語粵語回覆 ≥90%、中英夾雜句能正確理解。</t>
+          <t>① 新韌體上行用 IMA ADPCM（64 kbps），每幀帶解碼狀態（預測值＋步長索引），掉幀或重連後下一幀即可正確解碼 ② 連線時以 header 聲明編碼；伺服器據此解碼成 16kHz PCM 再交給 STT；沒有聲明的舊韌體照舊當 PCM ③ 韌體編碼與伺服器解碼位元一致（同一算法）④ 編碼 CPU &lt; 2%、不增加延遲 ⑤ 語音辨識品質與 PCM 相當</t>
         </is>
       </c>
       <c r="F40" s="11" t="n"/>
@@ -1832,15 +1832,15 @@
       <c r="H40" s="11" t="n"/>
       <c r="I40" s="12" t="n"/>
     </row>
-    <row r="41" ht="116" customHeight="1">
+    <row r="41" ht="46" customHeight="1">
       <c r="A41" s="13" t="inlineStr">
         <is>
-          <t>R-25</t>
+          <t>R-04</t>
         </is>
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>網頁的品牌主題系統</t>
+          <t>粵語質量評測</t>
         </is>
       </c>
       <c r="C41" s="13" t="inlineStr">
@@ -1855,7 +1855,7 @@
       </c>
       <c r="E41" s="6" t="inlineStr">
         <is>
-          <t>① 每個品牌一個資料夾：主題 token（顏色、字體、圓角）、logo 和圖示、文案、功能開關；首頁、上手流程、角色頁可以有品牌版本，其餘頁面共用 ② 由部署的環境變數選品牌（每套部署一個品牌，見 R-34），伺服器端渲染的第一屏就是對的主題，不閃爍 ③ 共用元件裡沒有品牌名稱和寫死的品牌顏色 ④ 加一個品牌只需要加資料夾、設定和一套部署，不用改共用元件</t>
+          <t>有一套粵語評測集（兒童錄音＋文字提示）；選定的 STT 與 LLM 達到門檻：兒童語音字錯率 ≤15%、口語粵語回覆 ≥90%、中英夾雜句能正確理解。</t>
         </is>
       </c>
       <c r="F41" s="11" t="n"/>
@@ -2294,20 +2294,20 @@
       <c r="H60" s="11" t="n"/>
       <c r="I60" s="12" t="n"/>
     </row>
-    <row r="61" ht="18" customHeight="1">
+    <row r="61" ht="32" customHeight="1">
       <c r="A61" s="13" t="inlineStr">
         <is>
-          <t>R-05</t>
+          <t>P2-25</t>
         </is>
       </c>
       <c r="B61" s="6" t="inlineStr">
         <is>
-          <t>內測版外殼（3D 打印 20 台）</t>
+          <t>C3 斷線後自救：TLS 握手超時縮短、連續失敗重設 Wi-Fi 或重開、修重試漏記憶體</t>
         </is>
       </c>
       <c r="C61" s="6" t="inlineStr">
         <is>
-          <t>等 R-01</t>
+          <t>等 P2-24</t>
         </is>
       </c>
       <c r="D61" s="11" t="n"/>
@@ -2320,17 +2320,17 @@
     <row r="62" ht="18" customHeight="1">
       <c r="A62" s="13" t="inlineStr">
         <is>
-          <t>R-06</t>
+          <t>R-05</t>
         </is>
       </c>
       <c r="B62" s="6" t="inlineStr">
         <is>
-          <t>家長自助上手流程</t>
+          <t>內測版外殼（3D 打印 20 台）</t>
         </is>
       </c>
       <c r="C62" s="6" t="inlineStr">
         <is>
-          <t>等 P0-11</t>
+          <t>等 R-01</t>
         </is>
       </c>
       <c r="D62" s="11" t="n"/>
@@ -2340,20 +2340,20 @@
       <c r="H62" s="11" t="n"/>
       <c r="I62" s="12" t="n"/>
     </row>
-    <row r="63" ht="32" customHeight="1">
+    <row r="63" ht="18" customHeight="1">
       <c r="A63" s="13" t="inlineStr">
         <is>
-          <t>R-13</t>
+          <t>R-06</t>
         </is>
       </c>
       <c r="B63" s="6" t="inlineStr">
         <is>
-          <t>CP1 內測就緒檢查（10/30）</t>
+          <t>家長自助上手流程</t>
         </is>
       </c>
       <c r="C63" s="6" t="inlineStr">
         <is>
-          <t>等 P0-07、P0-11、P1-01、P1-02、P2-09、R-01、R-02、R-04、R-05、R-06、P1-11</t>
+          <t>等 P0-11</t>
         </is>
       </c>
       <c r="D63" s="11" t="n"/>
@@ -2366,17 +2366,17 @@
     <row r="64" ht="32" customHeight="1">
       <c r="A64" s="13" t="inlineStr">
         <is>
-          <t>R-18</t>
+          <t>R-13</t>
         </is>
       </c>
       <c r="B64" s="6" t="inlineStr">
         <is>
-          <t>長按 BOOT 重新配網（開 AIBuddy-XXXX 熱點）</t>
+          <t>CP1 內測就緒檢查（10/30）</t>
         </is>
       </c>
       <c r="C64" s="6" t="inlineStr">
         <is>
-          <t>等 R-01</t>
+          <t>等 P0-07、P0-11、P1-01、P1-02、P2-09、R-01、R-02、R-04、R-05、R-06、P1-11</t>
         </is>
       </c>
       <c r="D64" s="11" t="n"/>
@@ -2389,12 +2389,12 @@
     <row r="65" ht="32" customHeight="1">
       <c r="A65" s="13" t="inlineStr">
         <is>
-          <t>R-19</t>
+          <t>R-18</t>
         </is>
       </c>
       <c r="B65" s="6" t="inlineStr">
         <is>
-          <t>外接按鈕：量產板加 I2C 擴展晶片（TCA9555）</t>
+          <t>長按 BOOT 重新配網（開 AIBuddy-XXXX 熱點）</t>
         </is>
       </c>
       <c r="C65" s="6" t="inlineStr">
@@ -2409,20 +2409,20 @@
       <c r="H65" s="11" t="n"/>
       <c r="I65" s="12" t="n"/>
     </row>
-    <row r="66" ht="18" customHeight="1">
+    <row r="66" ht="32" customHeight="1">
       <c r="A66" s="13" t="inlineStr">
         <is>
-          <t>R-20</t>
+          <t>R-19</t>
         </is>
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
-          <t>孩子資料與角色改成每台設備一份</t>
+          <t>外接按鈕：量產板加 I2C 擴展晶片（TCA9555）</t>
         </is>
       </c>
       <c r="C66" s="6" t="inlineStr">
         <is>
-          <t>等 P1-12</t>
+          <t>等 R-01</t>
         </is>
       </c>
       <c r="D66" s="11" t="n"/>
@@ -2432,20 +2432,20 @@
       <c r="H66" s="11" t="n"/>
       <c r="I66" s="12" t="n"/>
     </row>
-    <row r="67" ht="32" customHeight="1">
+    <row r="67" ht="18" customHeight="1">
       <c r="A67" s="13" t="inlineStr">
         <is>
-          <t>R-27</t>
+          <t>R-20</t>
         </is>
       </c>
       <c r="B67" s="6" t="inlineStr">
         <is>
-          <t>App 內登入：驗證碼、原生社交登入、刪除帳號</t>
+          <t>孩子資料與角色改成每台設備一份</t>
         </is>
       </c>
       <c r="C67" s="6" t="inlineStr">
         <is>
-          <t>等 R-26</t>
+          <t>等 P1-12</t>
         </is>
       </c>
       <c r="D67" s="11" t="n"/>
@@ -2455,20 +2455,20 @@
       <c r="H67" s="11" t="n"/>
       <c r="I67" s="12" t="n"/>
     </row>
-    <row r="68" ht="18" customHeight="1">
+    <row r="68" ht="32" customHeight="1">
       <c r="A68" s="13" t="inlineStr">
         <is>
-          <t>P0-14</t>
+          <t>R-27</t>
         </is>
       </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t>韌體簽章、Secure Boot 與 Flash 加密</t>
+          <t>App 內登入：驗證碼、原生社交登入、刪除帳號</t>
         </is>
       </c>
       <c r="C68" s="6" t="inlineStr">
         <is>
-          <t>等 R-01</t>
+          <t>等 R-26</t>
         </is>
       </c>
       <c r="D68" s="11" t="n"/>
@@ -2481,17 +2481,17 @@
     <row r="69" ht="18" customHeight="1">
       <c r="A69" s="13" t="inlineStr">
         <is>
-          <t>P1-06</t>
+          <t>P0-14</t>
         </is>
       </c>
       <c r="B69" s="6" t="inlineStr">
         <is>
-          <t>處理 GPL-3.0 依賴（arduino-audio-tools）</t>
+          <t>韌體簽章、Secure Boot 與 Flash 加密</t>
         </is>
       </c>
       <c r="C69" s="6" t="inlineStr">
         <is>
-          <t>等 Q3</t>
+          <t>等 R-01</t>
         </is>
       </c>
       <c r="D69" s="11" t="n"/>
@@ -2504,12 +2504,12 @@
     <row r="70" ht="18" customHeight="1">
       <c r="A70" s="13" t="inlineStr">
         <is>
-          <t>P1-07</t>
+          <t>P1-06</t>
         </is>
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>LGPL 合規與第三方授權聲明</t>
+          <t>處理 GPL-3.0 依賴（arduino-audio-tools）</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr">
@@ -2527,17 +2527,17 @@
     <row r="71" ht="18" customHeight="1">
       <c r="A71" s="13" t="inlineStr">
         <is>
-          <t>P1-08</t>
+          <t>P1-07</t>
         </is>
       </c>
       <c r="B71" s="6" t="inlineStr">
         <is>
-          <t>硬件認證</t>
+          <t>LGPL 合規與第三方授權聲明</t>
         </is>
       </c>
       <c r="C71" s="6" t="inlineStr">
         <is>
-          <t>等 R-01、R-05</t>
+          <t>等 Q3</t>
         </is>
       </c>
       <c r="D71" s="11" t="n"/>
@@ -2550,17 +2550,17 @@
     <row r="72" ht="18" customHeight="1">
       <c r="A72" s="13" t="inlineStr">
         <is>
-          <t>P1-14</t>
+          <t>P1-08</t>
         </is>
       </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>Admin 內容安全頁：審核事件只按類別統計</t>
+          <t>硬件認證</t>
         </is>
       </c>
       <c r="C72" s="6" t="inlineStr">
         <is>
-          <t>等 P1-01、P2-13</t>
+          <t>等 R-01、R-05</t>
         </is>
       </c>
       <c r="D72" s="11" t="n"/>
@@ -2570,20 +2570,20 @@
       <c r="H72" s="11" t="n"/>
       <c r="I72" s="12" t="n"/>
     </row>
-    <row r="73" ht="32" customHeight="1">
+    <row r="73" ht="18" customHeight="1">
       <c r="A73" s="13" t="inlineStr">
         <is>
-          <t>P2-15</t>
+          <t>P1-14</t>
         </is>
       </c>
       <c r="B73" s="6" t="inlineStr">
         <is>
-          <t>Admin 總覽頁：在線、用量、成本與待處理事項</t>
+          <t>Admin 內容安全頁：審核事件只按類別統計</t>
         </is>
       </c>
       <c r="C73" s="6" t="inlineStr">
         <is>
-          <t>等 P2-09</t>
+          <t>等 P1-01、P2-13</t>
         </is>
       </c>
       <c r="D73" s="11" t="n"/>
@@ -2593,20 +2593,20 @@
       <c r="H73" s="11" t="n"/>
       <c r="I73" s="12" t="n"/>
     </row>
-    <row r="74" ht="18" customHeight="1">
+    <row r="74" ht="32" customHeight="1">
       <c r="A74" s="13" t="inlineStr">
         <is>
-          <t>R-07</t>
+          <t>P2-15</t>
         </is>
       </c>
       <c r="B74" s="6" t="inlineStr">
         <is>
-          <t>20 個家庭封閉內測</t>
+          <t>Admin 總覽頁：在線、用量、成本與待處理事項</t>
         </is>
       </c>
       <c r="C74" s="6" t="inlineStr">
         <is>
-          <t>等 R-13</t>
+          <t>等 P2-09</t>
         </is>
       </c>
       <c r="D74" s="11" t="n"/>
@@ -2619,17 +2619,17 @@
     <row r="75" ht="18" customHeight="1">
       <c r="A75" s="13" t="inlineStr">
         <is>
-          <t>R-08</t>
+          <t>R-07</t>
         </is>
       </c>
       <c r="B75" s="6" t="inlineStr">
         <is>
-          <t>第 8 週關卡決策</t>
+          <t>20 個家庭封閉內測</t>
         </is>
       </c>
       <c r="C75" s="6" t="inlineStr">
         <is>
-          <t>等 R-07、P2-09、P1-08</t>
+          <t>等 R-13</t>
         </is>
       </c>
       <c r="D75" s="11" t="n"/>
@@ -2642,17 +2642,17 @@
     <row r="76" ht="18" customHeight="1">
       <c r="A76" s="13" t="inlineStr">
         <is>
-          <t>R-14</t>
+          <t>R-08</t>
         </is>
       </c>
       <c r="B76" s="6" t="inlineStr">
         <is>
-          <t>離線兒歌與故事</t>
+          <t>第 8 週關卡決策</t>
         </is>
       </c>
       <c r="C76" s="6" t="inlineStr">
         <is>
-          <t>等 R-01</t>
+          <t>等 R-07、P2-09、P1-08</t>
         </is>
       </c>
       <c r="D76" s="11" t="n"/>
@@ -2665,17 +2665,17 @@
     <row r="77" ht="18" customHeight="1">
       <c r="A77" s="13" t="inlineStr">
         <is>
-          <t>R-24</t>
+          <t>R-14</t>
         </is>
       </c>
       <c r="B77" s="6" t="inlineStr">
         <is>
-          <t>設備只能用自己品牌的角色</t>
+          <t>離線兒歌與故事</t>
         </is>
       </c>
       <c r="C77" s="6" t="inlineStr">
         <is>
-          <t>等 R-34</t>
+          <t>等 R-01</t>
         </is>
       </c>
       <c r="D77" s="11" t="n"/>
@@ -2688,17 +2688,17 @@
     <row r="78" ht="18" customHeight="1">
       <c r="A78" s="13" t="inlineStr">
         <is>
-          <t>R-28</t>
+          <t>R-24</t>
         </is>
       </c>
       <c r="B78" s="6" t="inlineStr">
         <is>
-          <t>三個 App 的殼：品牌版本與測試版</t>
+          <t>設備只能用自己品牌的角色</t>
         </is>
       </c>
       <c r="C78" s="6" t="inlineStr">
         <is>
-          <t>等 R-25、R-26</t>
+          <t>等 R-34</t>
         </is>
       </c>
       <c r="D78" s="11" t="n"/>
@@ -2711,17 +2711,17 @@
     <row r="79" ht="18" customHeight="1">
       <c r="A79" s="13" t="inlineStr">
         <is>
-          <t>R-30</t>
+          <t>R-28</t>
         </is>
       </c>
       <c r="B79" s="6" t="inlineStr">
         <is>
-          <t>快活 App（品牌 A）頁面</t>
+          <t>三個 App 的殼：品牌版本與測試版</t>
         </is>
       </c>
       <c r="C79" s="6" t="inlineStr">
         <is>
-          <t>等 R-25、R-34、Q12</t>
+          <t>等 R-25、R-26</t>
         </is>
       </c>
       <c r="D79" s="11" t="n"/>
@@ -2734,17 +2734,17 @@
     <row r="80" ht="18" customHeight="1">
       <c r="A80" s="13" t="inlineStr">
         <is>
-          <t>R-31</t>
+          <t>R-30</t>
         </is>
       </c>
       <c r="B80" s="6" t="inlineStr">
         <is>
-          <t>政協青年聯會版 App（品牌 B）頁面</t>
+          <t>快活 App（品牌 A）頁面</t>
         </is>
       </c>
       <c r="C80" s="6" t="inlineStr">
         <is>
-          <t>等 R-25、R-34、Q13</t>
+          <t>等 R-25、R-34、Q12</t>
         </is>
       </c>
       <c r="D80" s="11" t="n"/>
@@ -2757,17 +2757,17 @@
     <row r="81" ht="18" customHeight="1">
       <c r="A81" s="13" t="inlineStr">
         <is>
-          <t>R-35</t>
+          <t>R-31</t>
         </is>
       </c>
       <c r="B81" s="6" t="inlineStr">
         <is>
-          <t>韌體按品牌連線：伺服器網址在出廠時寫入</t>
+          <t>政協青年聯會版 App（品牌 B）頁面</t>
         </is>
       </c>
       <c r="C81" s="6" t="inlineStr">
         <is>
-          <t>等 R-34</t>
+          <t>等 R-25、R-34、Q13</t>
         </is>
       </c>
       <c r="D81" s="11" t="n"/>
@@ -2777,20 +2777,20 @@
       <c r="H81" s="11" t="n"/>
       <c r="I81" s="12" t="n"/>
     </row>
-    <row r="82" ht="32" customHeight="1">
+    <row r="82" ht="18" customHeight="1">
       <c r="A82" s="13" t="inlineStr">
         <is>
-          <t>R-38</t>
+          <t>R-35</t>
         </is>
       </c>
       <c r="B82" s="6" t="inlineStr">
         <is>
-          <t>公仔出廠鎖死所屬 IP，綁定時顯示該 IP 頭像</t>
+          <t>韌體按品牌連線：伺服器網址在出廠時寫入</t>
         </is>
       </c>
       <c r="C82" s="6" t="inlineStr">
         <is>
-          <t>等 P0-11</t>
+          <t>等 R-34</t>
         </is>
       </c>
       <c r="D82" s="11" t="n"/>
@@ -2803,17 +2803,17 @@
     <row r="83" ht="32" customHeight="1">
       <c r="A83" s="13" t="inlineStr">
         <is>
-          <t>R-39</t>
+          <t>R-38</t>
         </is>
       </c>
       <c r="B83" s="6" t="inlineStr">
         <is>
-          <t>Admin 出廠登記頁：匯入 MAC 清單、指定公仔、查看自檢結果</t>
+          <t>公仔出廠鎖死所屬 IP，綁定時顯示該 IP 頭像</t>
         </is>
       </c>
       <c r="C83" s="6" t="inlineStr">
         <is>
-          <t>等 R-38、P1-10</t>
+          <t>等 P0-11</t>
         </is>
       </c>
       <c r="D83" s="11" t="n"/>
@@ -2823,20 +2823,20 @@
       <c r="H83" s="11" t="n"/>
       <c r="I83" s="12" t="n"/>
     </row>
-    <row r="84" ht="18" customHeight="1">
+    <row r="84" ht="32" customHeight="1">
       <c r="A84" s="13" t="inlineStr">
         <is>
-          <t>R-09</t>
+          <t>R-39</t>
         </is>
       </c>
       <c r="B84" s="6" t="inlineStr">
         <is>
-          <t>量產外殼（真空複模）</t>
+          <t>Admin 出廠登記頁：匯入 MAC 清單、指定公仔、查看自檢結果</t>
         </is>
       </c>
       <c r="C84" s="6" t="inlineStr">
         <is>
-          <t>等 R-08、R-05、Q11</t>
+          <t>等 R-38、P1-10</t>
         </is>
       </c>
       <c r="D84" s="11" t="n"/>
@@ -2849,17 +2849,17 @@
     <row r="85" ht="18" customHeight="1">
       <c r="A85" s="13" t="inlineStr">
         <is>
-          <t>R-10</t>
+          <t>R-09</t>
         </is>
       </c>
       <c r="B85" s="6" t="inlineStr">
         <is>
-          <t>出廠流程</t>
+          <t>量產外殼（真空複模）</t>
         </is>
       </c>
       <c r="C85" s="6" t="inlineStr">
         <is>
-          <t>等 P0-14、R-01、P2-12、R-34、R-35、R-38、R-39</t>
+          <t>等 R-08、R-05、Q11</t>
         </is>
       </c>
       <c r="D85" s="11" t="n"/>
@@ -2872,17 +2872,17 @@
     <row r="86" ht="18" customHeight="1">
       <c r="A86" s="13" t="inlineStr">
         <is>
-          <t>R-11</t>
+          <t>R-10</t>
         </is>
       </c>
       <c r="B86" s="6" t="inlineStr">
         <is>
-          <t>售後：客服、保修與換機</t>
+          <t>出廠流程</t>
         </is>
       </c>
       <c r="C86" s="6" t="inlineStr">
         <is>
-          <t>等 R-40</t>
+          <t>等 P0-14、R-01、P2-12、R-34、R-35、R-38、R-39</t>
         </is>
       </c>
       <c r="D86" s="11" t="n"/>
@@ -2895,17 +2895,17 @@
     <row r="87" ht="18" customHeight="1">
       <c r="A87" s="13" t="inlineStr">
         <is>
-          <t>R-15</t>
+          <t>R-11</t>
         </is>
       </c>
       <c r="B87" s="6" t="inlineStr">
         <is>
-          <t>農曆新年前交付（生產 1/15、送達 1/29）</t>
+          <t>售後：客服、保修與換機</t>
         </is>
       </c>
       <c r="C87" s="6" t="inlineStr">
         <is>
-          <t>等 R-09、R-10</t>
+          <t>等 R-40</t>
         </is>
       </c>
       <c r="D87" s="11" t="n"/>
@@ -2918,17 +2918,17 @@
     <row r="88" ht="18" customHeight="1">
       <c r="A88" s="13" t="inlineStr">
         <is>
-          <t>R-33</t>
+          <t>R-15</t>
         </is>
       </c>
       <c r="B88" s="6" t="inlineStr">
         <is>
-          <t>三個 App 送審並通過</t>
+          <t>農曆新年前交付（生產 1/15、送達 1/29）</t>
         </is>
       </c>
       <c r="C88" s="6" t="inlineStr">
         <is>
-          <t>等 R-27、R-21、R-28、R-29、R-30、R-31、R-32</t>
+          <t>等 R-09、R-10</t>
         </is>
       </c>
       <c r="D88" s="11" t="n"/>
@@ -2938,20 +2938,20 @@
       <c r="H88" s="11" t="n"/>
       <c r="I88" s="12" t="n"/>
     </row>
-    <row r="89" ht="32" customHeight="1">
+    <row r="89" ht="18" customHeight="1">
       <c r="A89" s="13" t="inlineStr">
         <is>
-          <t>R-40</t>
+          <t>R-33</t>
         </is>
       </c>
       <c r="B89" s="6" t="inlineStr">
         <is>
-          <t>Admin 客服查詢頁：查帳號、名下設備與最近事件</t>
+          <t>三個 App 送審並通過</t>
         </is>
       </c>
       <c r="C89" s="6" t="inlineStr">
         <is>
-          <t>等 P1-10、P1-12</t>
+          <t>等 R-27、R-21、R-28、R-29、R-30、R-31、R-32</t>
         </is>
       </c>
       <c r="D89" s="11" t="n"/>
@@ -2961,50 +2961,50 @@
       <c r="H89" s="11" t="n"/>
       <c r="I89" s="12" t="n"/>
     </row>
-    <row r="91">
-      <c r="A91" s="10" t="inlineStr">
+    <row r="90" ht="32" customHeight="1">
+      <c r="A90" s="13" t="inlineStr">
+        <is>
+          <t>R-40</t>
+        </is>
+      </c>
+      <c r="B90" s="6" t="inlineStr">
+        <is>
+          <t>Admin 客服查詢頁：查帳號、名下設備與最近事件</t>
+        </is>
+      </c>
+      <c r="C90" s="6" t="inlineStr">
+        <is>
+          <t>等 P1-10、P1-12</t>
+        </is>
+      </c>
+      <c r="D90" s="11" t="n"/>
+      <c r="E90" s="11" t="n"/>
+      <c r="F90" s="11" t="n"/>
+      <c r="G90" s="11" t="n"/>
+      <c r="H90" s="11" t="n"/>
+      <c r="I90" s="12" t="n"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="10" t="inlineStr">
         <is>
           <t>❓ 待確認問題</t>
         </is>
       </c>
     </row>
-    <row r="92">
-      <c r="A92" s="4" t="inlineStr">
+    <row r="93">
+      <c r="A93" s="4" t="inlineStr">
         <is>
           <t>編號</t>
         </is>
       </c>
-      <c r="B92" s="4" t="inlineStr">
+      <c r="B93" s="4" t="inlineStr">
         <is>
           <t>問題</t>
         </is>
       </c>
-      <c r="C92" s="4" t="inlineStr">
+      <c r="C93" s="4" t="inlineStr">
         <is>
           <t>影響的任務 / 為什麼重要</t>
-        </is>
-      </c>
-      <c r="D92" s="11" t="n"/>
-      <c r="E92" s="11" t="n"/>
-      <c r="F92" s="11" t="n"/>
-      <c r="G92" s="11" t="n"/>
-      <c r="H92" s="11" t="n"/>
-      <c r="I92" s="12" t="n"/>
-    </row>
-    <row r="93" ht="18" customHeight="1">
-      <c r="A93" s="13" t="inlineStr">
-        <is>
-          <t>Q3</t>
-        </is>
-      </c>
-      <c r="B93" s="6" t="inlineStr">
-        <is>
-          <t>韌體打算閉源商業銷售嗎？</t>
-        </is>
-      </c>
-      <c r="C93" s="6" t="inlineStr">
-        <is>
-          <t>P1-06, P1-07：決定 GPL／LGPL 依賴要開源還是替換。</t>
         </is>
       </c>
       <c r="D93" s="11" t="n"/>
@@ -3014,20 +3014,20 @@
       <c r="H93" s="11" t="n"/>
       <c r="I93" s="12" t="n"/>
     </row>
-    <row r="94" ht="32" customHeight="1">
+    <row r="94" ht="18" customHeight="1">
       <c r="A94" s="13" t="inlineStr">
         <is>
-          <t>Q11</t>
+          <t>Q3</t>
         </is>
       </c>
       <c r="B94" s="6" t="inlineStr">
         <is>
-          <t>馬會快活的賽馬日版和新春版各多少隻（共 2,500）？</t>
+          <t>韌體打算閉源商業銷售嗎？</t>
         </is>
       </c>
       <c r="C94" s="6" t="inlineStr">
         <is>
-          <t>R-09, R-15：兩款的服裝和配件要分開訂料；11/20 前不知道，PP 樣和大貨單（11/27）會被拖慢。由馬會決定。</t>
+          <t>P1-06, P1-07：決定 GPL／LGPL 依賴要開源還是替換。</t>
         </is>
       </c>
       <c r="D94" s="11" t="n"/>
@@ -3037,20 +3037,20 @@
       <c r="H94" s="11" t="n"/>
       <c r="I94" s="12" t="n"/>
     </row>
-    <row r="95" ht="60" customHeight="1">
+    <row r="95" ht="32" customHeight="1">
       <c r="A95" s="13" t="inlineStr">
         <is>
-          <t>Q12</t>
+          <t>Q11</t>
         </is>
       </c>
       <c r="B95" s="6" t="inlineStr">
         <is>
-          <t>快活 App 的「會員綁定」是指甚麼：用我們自己的帳號（email 驗證碼），還是接馬會的會員帳號登入（SSO）？</t>
+          <t>馬會快活的賽馬日版和新春版各多少隻（共 2,500）？</t>
         </is>
       </c>
       <c r="C95" s="6" t="inlineStr">
         <is>
-          <t>P0-11, 快活 App（未入追蹤表）：接馬會 SSO 的話，登入、帳號刪除和資料歸屬都要按馬會的介面重做，工作量和排期要另估，而且 W5（11/9–11/13）就要做快活 App 的綁定；用我們的帳號則和其他品牌共用同一套流程。由馬會決定，要盡早問。</t>
+          <t>R-09, R-15：兩款的服裝和配件要分開訂料；11/20 前不知道，PP 樣和大貨單（11/27）會被拖慢。由馬會決定。</t>
         </is>
       </c>
       <c r="D95" s="11" t="n"/>
@@ -3060,20 +3060,20 @@
       <c r="H95" s="11" t="n"/>
       <c r="I95" s="12" t="n"/>
     </row>
-    <row r="96" ht="46" customHeight="1">
+    <row r="96" ht="60" customHeight="1">
       <c r="A96" s="13" t="inlineStr">
         <is>
-          <t>Q13</t>
+          <t>Q12</t>
         </is>
       </c>
       <c r="B96" s="6" t="inlineStr">
         <is>
-          <t>政協青年聯會版的角色、語言和內容由誰提供？什麼時候交？</t>
+          <t>快活 App 的「會員綁定」是指甚麼：用我們自己的帳號（email 驗證碼），還是接馬會的會員帳號登入（SSO）？</t>
         </is>
       </c>
       <c r="C96" s="6" t="inlineStr">
         <is>
-          <t>品牌 B 的 App 頁面：品牌 B 的用戶是成人會員，但角色、說話語言、內容規則都還沒有。最遲 11/13 要拿到，才趕得及內部測試和 App 頁面（W6）。</t>
+          <t>P0-11, 快活 App（未入追蹤表）：接馬會 SSO 的話，登入、帳號刪除和資料歸屬都要按馬會的介面重做，工作量和排期要另估，而且 W5（11/9–11/13）就要做快活 App 的綁定；用我們的帳號則和其他品牌共用同一套流程。由馬會決定，要盡早問。</t>
         </is>
       </c>
       <c r="D96" s="11" t="n"/>
@@ -3083,50 +3083,73 @@
       <c r="H96" s="11" t="n"/>
       <c r="I96" s="12" t="n"/>
     </row>
-    <row r="98">
-      <c r="A98" s="10" t="inlineStr">
+    <row r="97" ht="46" customHeight="1">
+      <c r="A97" s="13" t="inlineStr">
+        <is>
+          <t>Q13</t>
+        </is>
+      </c>
+      <c r="B97" s="6" t="inlineStr">
+        <is>
+          <t>政協青年聯會版的角色、語言和內容由誰提供？什麼時候交？</t>
+        </is>
+      </c>
+      <c r="C97" s="6" t="inlineStr">
+        <is>
+          <t>品牌 B 的 App 頁面：品牌 B 的用戶是成人會員，但角色、說話語言、內容規則都還沒有。最遲 11/13 要拿到，才趕得及內部測試和 App 頁面（W6）。</t>
+        </is>
+      </c>
+      <c r="D97" s="11" t="n"/>
+      <c r="E97" s="11" t="n"/>
+      <c r="F97" s="11" t="n"/>
+      <c r="G97" s="11" t="n"/>
+      <c r="H97" s="11" t="n"/>
+      <c r="I97" s="12" t="n"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="10" t="inlineStr">
         <is>
           <t>說明</t>
         </is>
       </c>
     </row>
-    <row r="99" ht="32" customHeight="1">
-      <c r="A99" s="14" t="inlineStr">
+    <row r="100" ht="32" customHeight="1">
+      <c r="A100" s="14" t="inlineStr">
         <is>
           <t>・狀態：未開始 → 進行中 → 已完成。只有測試真的跑過而且通過才算已完成；阻塞要在備註寫原因；不再需要的任務標不適用，不要刪。</t>
-        </is>
-      </c>
-    </row>
-    <row r="100" ht="18" customHeight="1">
-      <c r="A100" s="14" t="inlineStr">
-        <is>
-          <t>・測試結果：未測試 / 通過 / 失敗 / 部分通過。測試證據寫跑了什麼、看到什麼，完整歷史在「更新記錄」。</t>
         </is>
       </c>
     </row>
     <row r="101" ht="18" customHeight="1">
       <c r="A101" s="14" t="inlineStr">
         <is>
-          <t>・「接下來」按階段排序，同一階段內再按優先級；依賴還沒滿足的任務不會出現在「接下來」。</t>
+          <t>・測試結果：未測試 / 通過 / 失敗 / 部分通過。測試證據寫跑了什麼、看到什麼，完整歷史在「更新記錄」。</t>
         </is>
       </c>
     </row>
     <row r="102" ht="18" customHeight="1">
       <c r="A102" s="14" t="inlineStr">
         <is>
+          <t>・「接下來」按階段排序，同一階段內再按優先級；依賴還沒滿足的任務不會出現在「接下來」。</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" ht="18" customHeight="1">
+      <c r="A103" s="14" t="inlineStr">
+        <is>
           <t>・可以手動改：「任務清單」的狀態、測試結果、測試證據、Commit、備註，以及「待確認問題」的回答。其餘欄位和本頁由腳本維護。</t>
         </is>
       </c>
     </row>
-    <row r="103" ht="32" customHeight="1">
-      <c r="A103" s="14" t="inlineStr">
+    <row r="104" ht="32" customHeight="1">
+      <c r="A104" s="14" t="inlineStr">
         <is>
           <t>・建議用法：在 Claude Code 對 Claude 說「P0-02 做完了」或輸入 /prod-readiness。Claude 會先跑測試再更新，並寫進「更新記錄」。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="84">
+  <mergeCells count="85">
     <mergeCell ref="A99:I99"/>
     <mergeCell ref="C82:I82"/>
     <mergeCell ref="E52:I52"/>
@@ -3138,9 +3161,9 @@
     <mergeCell ref="E29:I29"/>
     <mergeCell ref="E38:I38"/>
     <mergeCell ref="C83:I83"/>
-    <mergeCell ref="C92:I92"/>
     <mergeCell ref="E31:I31"/>
     <mergeCell ref="E40:I40"/>
+    <mergeCell ref="C97:I97"/>
     <mergeCell ref="A19:I19"/>
     <mergeCell ref="E26:I26"/>
     <mergeCell ref="A103:I103"/>
@@ -3157,7 +3180,6 @@
     <mergeCell ref="C77:I77"/>
     <mergeCell ref="C86:I86"/>
     <mergeCell ref="C68:I68"/>
-    <mergeCell ref="A91:I91"/>
     <mergeCell ref="A100:I100"/>
     <mergeCell ref="C58:I58"/>
     <mergeCell ref="E30:I30"/>
@@ -3166,6 +3188,7 @@
     <mergeCell ref="C85:I85"/>
     <mergeCell ref="C94:I94"/>
     <mergeCell ref="C65:I65"/>
+    <mergeCell ref="A92:I92"/>
     <mergeCell ref="C75:I75"/>
     <mergeCell ref="C84:I84"/>
     <mergeCell ref="C80:I80"/>
@@ -3179,6 +3202,7 @@
     <mergeCell ref="E24:I24"/>
     <mergeCell ref="E33:I33"/>
     <mergeCell ref="A3:I3"/>
+    <mergeCell ref="A104:I104"/>
     <mergeCell ref="E35:I35"/>
     <mergeCell ref="A43:I43"/>
     <mergeCell ref="C74:I74"/>
@@ -3206,8 +3230,8 @@
     <mergeCell ref="E36:I36"/>
     <mergeCell ref="C63:I63"/>
     <mergeCell ref="C93:I93"/>
-    <mergeCell ref="A98:I98"/>
     <mergeCell ref="C56:I56"/>
+    <mergeCell ref="C90:I90"/>
     <mergeCell ref="E22:I22"/>
     <mergeCell ref="C76:I76"/>
     <mergeCell ref="A54:I54"/>
@@ -3240,7 +3264,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P96"/>
+  <dimension ref="A1:P98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -10317,8 +10341,138 @@
         </is>
       </c>
     </row>
+    <row r="97" ht="144" customHeight="1">
+      <c r="A97" s="13" t="inlineStr">
+        <is>
+          <t>P2-24</t>
+        </is>
+      </c>
+      <c r="B97" s="13" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C97" s="13" t="inlineStr">
+        <is>
+          <t>2 內測準備</t>
+        </is>
+      </c>
+      <c r="D97" s="6" t="inlineStr">
+        <is>
+          <t>韌體-音訊</t>
+        </is>
+      </c>
+      <c r="E97" s="6" t="inlineStr">
+        <is>
+          <t>麥克風上行改用 IMA ADPCM（減少 4 倍頻寬）</t>
+        </is>
+      </c>
+      <c r="F97" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="G97" s="13" t="inlineStr">
+        <is>
+          <t>未測試</t>
+        </is>
+      </c>
+      <c r="I97" s="6" t="inlineStr">
+        <is>
+          <t>上行仍是從上游 ElatoAI 沿用的未壓縮 16kHz PCM（256 kbps）。2026-10-13 在 51:16:c0 實測：iPhone 熱點上發送最長卡 330ms、說話時 heap 13–20KB、最低 788B、約 5 輪斷 3 次；同板在 HKQF - Guest 20 輪 0 斷、最低 40.9KB。內部測試的家庭有人會用手機熱點。</t>
+        </is>
+      </c>
+      <c r="J97" s="6" t="inlineStr">
+        <is>
+          <t>firmware-arduino/src/Audio.cpp（麥克風上行發送、websocketExtraHeaders）；server/fastapi/esp32_transport.py（RawPCMFrameSerializer 的輸入）、server.py（/ws/esp32 接受連線）；Python 3.11 內建 audioop，3.13+ 用 audioop-lts</t>
+        </is>
+      </c>
+      <c r="K97" s="6" t="inlineStr">
+        <is>
+          <t>① 新韌體上行用 IMA ADPCM（64 kbps），每幀帶解碼狀態（預測值＋步長索引），掉幀或重連後下一幀即可正確解碼 ② 連線時以 header 聲明編碼；伺服器據此解碼成 16kHz PCM 再交給 STT；沒有聲明的舊韌體照舊當 PCM ③ 韌體編碼與伺服器解碼位元一致（同一算法）④ 編碼 CPU &lt; 2%、不增加延遲 ⑤ 語音辨識品質與 PCM 相當</t>
+        </is>
+      </c>
+      <c r="L97" s="6" t="inlineStr">
+        <is>
+          <t>① C 編碼器與 Python audioop 交叉驗證：同一段 PCM，韌體算法編碼 → audioop 解碼 = audioop 自己編碼再解碼的結果 ② pytest：帶 header 的連線解碼正確、無 header 照舊 PCM、壞幀不崩潰 ③ 62:70（Guest）：粵語對話 10 輪，STT 文字與 PCM 版本相當；上行位元組數約為原來 1/4 ④ 雲端可測時：雲端板在 iPhone 熱點重跑 10/13 的量度（發送最長卡頓、說話時 heap、斷線次數），對照 PCM 版本 ⑤ 舊韌體（1.0.1）連新伺服器照常對話</t>
+        </is>
+      </c>
+      <c r="M97" s="13" t="n"/>
+      <c r="P97" s="6" t="inlineStr">
+        <is>
+          <t>[2026-10-15] 新增</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" ht="102" customHeight="1">
+      <c r="A98" s="13" t="inlineStr">
+        <is>
+          <t>P2-25</t>
+        </is>
+      </c>
+      <c r="B98" s="13" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C98" s="13" t="inlineStr">
+        <is>
+          <t>2 內測準備</t>
+        </is>
+      </c>
+      <c r="D98" s="6" t="inlineStr">
+        <is>
+          <t>韌體-網絡</t>
+        </is>
+      </c>
+      <c r="E98" s="6" t="inlineStr">
+        <is>
+          <t>C3 斷線後自救：TLS 握手超時縮短、連續失敗重設 Wi-Fi 或重開、修重試漏記憶體</t>
+        </is>
+      </c>
+      <c r="F98" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="G98" s="13" t="inlineStr">
+        <is>
+          <t>未測試</t>
+        </is>
+      </c>
+      <c r="I98" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-13 在 51:16:c0（熱點）斷線後每次重連卡約 121 秒（TLS 握手超時），持續 26 分鐘不恢復；debug 版本顯示每次失敗的重連漏約 170B heap；韌體不會重設 Wi-Fi 或重開，孩子只見玩具不回應。</t>
+        </is>
+      </c>
+      <c r="J98" s="6" t="inlineStr">
+        <is>
+          <t>firmware-arduino/src/Audio.cpp（websocketSetup、networkTask 重連）、src/WifiManager.cpp；debug 分支 debug-1.0.1-iwdt 的 heap 記錄工具</t>
+        </is>
+      </c>
+      <c r="K98" s="6" t="inlineStr">
+        <is>
+          <t>① websocket / HTTPS 的 TLS 握手超時約 15 秒（可調）② 連續 N 次（預設 5）連不上伺服器就重設 Wi-Fi 重連；再連續失敗就 ESP.restart()（試用期內的重開照 OTA 規則處理）③ 失敗的重連不再漏 heap：連續 50 次失敗前後 free heap 差 &lt; 1KB ④ 已綁定設備的正常斷網重連行為不變（R-36 ④）</t>
+        </is>
+      </c>
+      <c r="L98" s="6" t="inlineStr">
+        <is>
+          <t>① 62:70：停掉語音伺服器 → 串口每次握手失敗 ≤ 15 秒，第 N 次後重設 Wi-Fi、再後重開，恢復伺服器後自動連上 ② 記錄 50 次失敗重連前後的 free heap ③ 雲端可測時在 iPhone 熱點重跑 10/13 情境，斷線後 1 分鐘內恢復對話</t>
+        </is>
+      </c>
+      <c r="M98" s="13" t="inlineStr">
+        <is>
+          <t>P2-24</t>
+        </is>
+      </c>
+      <c r="P98" s="6" t="inlineStr">
+        <is>
+          <t>[2026-10-15] 新增</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P96"/>
+  <autoFilter ref="A1:P98"/>
   <conditionalFormatting sqref="F2:F1000">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"已完成"</formula>
@@ -10899,7 +11053,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I313"/>
+  <dimension ref="A1:I315"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -21812,8 +21966,62 @@
         </is>
       </c>
     </row>
+    <row r="314" ht="32" customHeight="1">
+      <c r="A314" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-15 10:29</t>
+        </is>
+      </c>
+      <c r="B314" s="13" t="inlineStr">
+        <is>
+          <t>P2-24</t>
+        </is>
+      </c>
+      <c r="C314" s="6" t="inlineStr">
+        <is>
+          <t>麥克風上行改用 IMA ADPCM（減少 4 倍頻寬）</t>
+        </is>
+      </c>
+      <c r="E314" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="I314" s="6" t="inlineStr">
+        <is>
+          <t>新增任務</t>
+        </is>
+      </c>
+    </row>
+    <row r="315" ht="46" customHeight="1">
+      <c r="A315" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-15 10:29</t>
+        </is>
+      </c>
+      <c r="B315" s="13" t="inlineStr">
+        <is>
+          <t>P2-25</t>
+        </is>
+      </c>
+      <c r="C315" s="6" t="inlineStr">
+        <is>
+          <t>C3 斷線後自救：TLS 握手超時縮短、連續失敗重設 Wi-Fi 或重開、修重試漏記憶體</t>
+        </is>
+      </c>
+      <c r="E315" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="I315" s="6" t="inlineStr">
+        <is>
+          <t>新增任務</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I313"/>
+  <autoFilter ref="A1:I315"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
P2-25 does not wait for P2-24; start P2-24.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/production-readiness.xlsx
+++ b/docs/production-readiness.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'任務清單'!$A$1:$P$98</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'待確認問題'!$A$1:$G$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$315</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$317</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -641,7 +641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I104"/>
+  <dimension ref="A1:I105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -820,11 +820,11 @@
       </c>
       <c r="D8" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A8,'任務清單'!$F:$F,D$5)</f>
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E8" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A8,'任務清單'!$F:$F,E$5)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F8" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A8,'任務清單'!$F:$F,F$5)</f>
@@ -896,11 +896,11 @@
       </c>
       <c r="D10" s="5">
         <f>SUM(D6:D9)</f>
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E10" s="5">
         <f>SUM(E6:E9)</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F10" s="5">
         <f>SUM(F6:F9)</f>
@@ -1023,11 +1023,11 @@
       </c>
       <c r="D14" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A14,'任務清單'!$F:$F,D$12)</f>
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E14" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A14,'任務清單'!$F:$F,E$12)</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F14" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A14,'任務清單'!$F:$F,F$12)</f>
@@ -1139,11 +1139,11 @@
       </c>
       <c r="D17" s="5">
         <f>SUM(D13:D16)</f>
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E17" s="5">
         <f>SUM(E13:E16)</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F17" s="5">
         <f>SUM(F13:F16)</f>
@@ -1518,15 +1518,15 @@
       <c r="H30" s="11" t="n"/>
       <c r="I30" s="12" t="n"/>
     </row>
-    <row r="31" ht="200" customHeight="1">
+    <row r="31" ht="102" customHeight="1">
       <c r="A31" s="13" t="inlineStr">
         <is>
-          <t>R-21</t>
+          <t>P2-24</t>
         </is>
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>藍牙配網與綁定（取代熱點配網）</t>
+          <t>麥克風上行改用 IMA ADPCM（減少 4 倍頻寬）</t>
         </is>
       </c>
       <c r="C31" s="13" t="inlineStr">
@@ -1541,7 +1541,7 @@
       </c>
       <c r="E31" s="6" t="inlineStr">
         <is>
-          <t>① 設備在「未配網、Wi-Fi 連不上、未綁定、長按 BOOT」時以 AIBuddy-XXXX 名稱廣播藍牙，廣播資料帶品牌，品牌 App 只列出自己品牌的設備。② 設備經藍牙回傳它掃描到的 2.4GHz Wi-Fi 清單，App 讓用戶選擇並填密碼。③ App 經藍牙把 SSID、密碼和綁定票（P0-11）一起交給設備；藍牙通道加密（ESP 標準配網協定 security 1/2 或同等）。④ 設備連上 Wi-Fi 後自己完成認領，App 顯示綁定成功或失敗原因（密碼錯、設備已有主人、票過期）。⑤ 配網期間不啟動音訊；完成後釋放藍牙記憶體再開語音（必要時重開機），對話中最低 heap 不比現在差。⑥ 解綁在 App 內完成（P1-12），解綁後設備進入藍牙待綁定狀態。⑦ SoftAP 熱點配網保留給開發和運維（隱藏觸發方式或編譯開關），量產用戶流程不出現。</t>
+          <t>① 新韌體上行用 IMA ADPCM（64 kbps），每幀帶解碼狀態（預測值＋步長索引），掉幀或重連後下一幀即可正確解碼 ② 連線時以 header 聲明編碼；伺服器據此解碼成 16kHz PCM 再交給 STT；沒有聲明的舊韌體照舊當 PCM ③ 韌體編碼與伺服器解碼位元一致（同一算法）④ 編碼 CPU &lt; 2%、不增加延遲 ⑤ 語音辨識品質與 PCM 相當</t>
         </is>
       </c>
       <c r="F31" s="11" t="n"/>
@@ -1549,15 +1549,15 @@
       <c r="H31" s="11" t="n"/>
       <c r="I31" s="12" t="n"/>
     </row>
-    <row r="32" ht="172" customHeight="1">
+    <row r="32" ht="200" customHeight="1">
       <c r="A32" s="13" t="inlineStr">
         <is>
-          <t>R-36</t>
+          <t>R-21</t>
         </is>
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>未認領的設備停在配對狀態，不再每秒重連 websocket</t>
+          <t>藍牙配網與綁定（取代熱點配網）</t>
         </is>
       </c>
       <c r="C32" s="13" t="inlineStr">
@@ -1572,8 +1572,7 @@
       </c>
       <c r="E32" s="6" t="inlineStr">
         <is>
-          <t>上次測試：部分通過 — 補充 2026-10-15（1.7.5，含 R-36）：已綁定時兩次 Wi-Fi 切換各斷網 9–11 秒，都自動重連並重新 auth，沒有停在暫停狀態；30 秒斷網仍未做
-① 拿到 202 或 websocket 被 4401 拒絕後，設備停掉 websocket 自動重連，進入待綁定狀態（燈號可分辨）。② 待綁定時只按退避（5 秒起、上限 PROVISION_BACKOFF_MAX）呼叫 generate_auth_token，不開 websocket。③ 被認領後下一次輪詢拿到 200，在 10 秒內（加退避）自動開 websocket 並能對話，不用重開機。④ 已綁定設備網絡斷線重連的行為不變。⑤ 隨 OTA 推出。</t>
+          <t>① 設備在「未配網、Wi-Fi 連不上、未綁定、長按 BOOT」時以 AIBuddy-XXXX 名稱廣播藍牙，廣播資料帶品牌，品牌 App 只列出自己品牌的設備。② 設備經藍牙回傳它掃描到的 2.4GHz Wi-Fi 清單，App 讓用戶選擇並填密碼。③ App 經藍牙把 SSID、密碼和綁定票（P0-11）一起交給設備；藍牙通道加密（ESP 標準配網協定 security 1/2 或同等）。④ 設備連上 Wi-Fi 後自己完成認領，App 顯示綁定成功或失敗原因（密碼錯、設備已有主人、票過期）。⑤ 配網期間不啟動音訊；完成後釋放藍牙記憶體再開語音（必要時重開機），對話中最低 heap 不比現在差。⑥ 解綁在 App 內完成（P1-12），解綁後設備進入藍牙待綁定狀態。⑦ SoftAP 熱點配網保留給開發和運維（隱藏觸發方式或編譯開關），量產用戶流程不出現。</t>
         </is>
       </c>
       <c r="F32" s="11" t="n"/>
@@ -1581,20 +1580,20 @@
       <c r="H32" s="11" t="n"/>
       <c r="I32" s="12" t="n"/>
     </row>
-    <row r="33" ht="228" customHeight="1">
+    <row r="33" ht="172" customHeight="1">
       <c r="A33" s="13" t="inlineStr">
         <is>
-          <t>P2-12</t>
+          <t>R-36</t>
         </is>
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>量產燒錄前加大 app 分區</t>
+          <t>未認領的設備停在配對狀態，不再每秒重連 websocket</t>
         </is>
       </c>
       <c r="C33" s="13" t="inlineStr">
         <is>
-          <t>3 封閉內測</t>
+          <t>2 內測準備</t>
         </is>
       </c>
       <c r="D33" s="13" t="inlineStr">
@@ -1604,8 +1603,8 @@
       </c>
       <c r="E33" s="6" t="inlineStr">
         <is>
-          <t>上次測試：部分通過 — 62:70（spotpear-ai-toy-p212 原型，現已併入 spotpear-ai-toy）：① 本機 OTA 1.6.1→1.6.2 寫入新 app1，120s 後 confirmed ② 3 秒 abort 的 1.6.3 → PANIC → 回到 1.6.2，ota_failed_version=1.6.3 ③ 崩潰寫入 coredump 14.8KB ④ 資源分區 9 個聲音 504KB/2MB，開機 CRC 63ms，OTA 後照常；損壞/清空 → 退回內建聲音無崩潰 ⑤ pio 全部 18 個 env 編譯通過，映像都在各自 app 槽內（Spotpear 4 個 1.59–1.60MB / 4MB；其他板仍 2MB 槽）；R-21 藍牙探針版 2,326,128 bytes &lt; 4MB ⑥ release_firmware.py 映像 &gt; app 槽即拒發。未做：雲端 OTA 一次（等上 UAT）、出廠腳本寫入資源包（R-10）
-新分區表（例如 app0/app1 各 4MB，保留 nvs/otadata 位置）在出廠前定案並寫入出廠腳本；OTA 與回滾在新分區表上照常</t>
+          <t>上次測試：部分通過 — 補充 2026-10-15（1.7.5，含 R-36）：已綁定時兩次 Wi-Fi 切換各斷網 9–11 秒，都自動重連並重新 auth，沒有停在暫停狀態；30 秒斷網仍未做
+① 拿到 202 或 websocket 被 4401 拒絕後，設備停掉 websocket 自動重連，進入待綁定狀態（燈號可分辨）。② 待綁定時只按退避（5 秒起、上限 PROVISION_BACKOFF_MAX）呼叫 generate_auth_token，不開 websocket。③ 被認領後下一次輪詢拿到 200，在 10 秒內（加退避）自動開 websocket 並能對話，不用重開機。④ 已綁定設備網絡斷線重連的行為不變。⑤ 隨 OTA 推出。</t>
         </is>
       </c>
       <c r="F33" s="11" t="n"/>
@@ -1613,15 +1612,15 @@
       <c r="H33" s="11" t="n"/>
       <c r="I33" s="12" t="n"/>
     </row>
-    <row r="34" ht="409" customHeight="1">
+    <row r="34" ht="228" customHeight="1">
       <c r="A34" s="13" t="inlineStr">
         <is>
-          <t>P2-22</t>
+          <t>P2-12</t>
         </is>
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>改服務器網址也不失聯：語音網址由後端下發、後端網址可遷移、已確認韌體長期連不上時自救</t>
+          <t>量產燒錄前加大 app 分區</t>
         </is>
       </c>
       <c r="C34" s="13" t="inlineStr">
@@ -1636,8 +1635,8 @@
       </c>
       <c r="E34" s="6" t="inlineStr">
         <is>
-          <t>上次測試：部分通過 — 後端部分（分支 p2-22-server-urls）：node --test lib/deviceServerUrls.test.mjs 5/5、tsc 0 錯誤。worktree dev server 3222 + 本機 Supabase，兩塊假板（02:22:…:01/02）：已認領 200 帶 voice_url + backend_url；未認領 202 只帶 backend_url；DEVICE_VOICE_URL=ws://fastapi:7860/… → 不發、日誌記錯誤；兩個變數都不設 → 兩個欄位都不帶；生產值 → wss://elatoai.hkqft.com/fastapi/ws/esp32、https://elatoai.hkqft.com。測試數據已清除
-① /api/generate_auth_token 的回應帶 voice_url（wss 主機＋端口＋路徑，來自後端環境變數）；韌體用它連 /ws，並把最後一次成功的值存進 NVS；改 FastAPI 網址只改伺服器設定，不需新韌體 ② 回應沒有 voice_url（舊後端）或新網址連不上時，退回 NVS 上次成功的值，再退回出廠／編譯時的預設值 ③ 後端網址可遷移：回應可帶 backend_url；韌體先存為候選，下次開機用新網址取 token 成功才正式替換，失敗就繼續用舊網址；舊網址在遷移期內保持可用（runbook 寫明保留多久） ④ 已確認的韌體若連續 N 次開機（預設 10 次、跨度至少 24 小時，計數存 NVS）Wi-Fi 已拿到 IP 卻取不到 token：先依次試 NVS、出廠的後端網址；仍失敗且另一個槽可用，就切到另一個槽一次，並在下次連上時把本版本報為失敗 ⑤ 純斷網（拿不到 IP、路由器沒外網）不計入 ④ ⑥ 新網址的證書必須鏈到 CF_CA_bundle 裡的根（GTS Root R4、ISRG Root X1）；換主機或離開 Cloudflare 前先查證書鏈，runbook 寫明 ⑦ 只接受 https 的 backend_url 和 wss 的 voice_url，主機須在韌體內允許的網域後綴之下，防止後端被冒充時把板子引去別處</t>
+          <t>上次測試：部分通過 — 62:70（spotpear-ai-toy-p212 原型，現已併入 spotpear-ai-toy）：① 本機 OTA 1.6.1→1.6.2 寫入新 app1，120s 後 confirmed ② 3 秒 abort 的 1.6.3 → PANIC → 回到 1.6.2，ota_failed_version=1.6.3 ③ 崩潰寫入 coredump 14.8KB ④ 資源分區 9 個聲音 504KB/2MB，開機 CRC 63ms，OTA 後照常；損壞/清空 → 退回內建聲音無崩潰 ⑤ pio 全部 18 個 env 編譯通過，映像都在各自 app 槽內（Spotpear 4 個 1.59–1.60MB / 4MB；其他板仍 2MB 槽）；R-21 藍牙探針版 2,326,128 bytes &lt; 4MB ⑥ release_firmware.py 映像 &gt; app 槽即拒發。未做：雲端 OTA 一次（等上 UAT）、出廠腳本寫入資源包（R-10）
+新分區表（例如 app0/app1 各 4MB，保留 nvs/otadata 位置）在出廠前定案並寫入出廠腳本；OTA 與回滾在新分區表上照常</t>
         </is>
       </c>
       <c r="F34" s="11" t="n"/>
@@ -1648,12 +1647,12 @@
     <row r="35" ht="409" customHeight="1">
       <c r="A35" s="13" t="inlineStr">
         <is>
-          <t>R-37</t>
+          <t>P2-22</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>網頁設定玩具的 Wi-Fi：查看、新增、刪除</t>
+          <t>改服務器網址也不失聯：語音網址由後端下發、後端網址可遷移、已確認韌體長期連不上時自救</t>
         </is>
       </c>
       <c r="C35" s="13" t="inlineStr">
@@ -1668,8 +1667,8 @@
       </c>
       <c r="E35" s="6" t="inlineStr">
         <is>
-          <t>上次測試：部分通過 — 2026-10-15 真機 62:70（hw-test-1015 = dev + P2-16 + R-36 + r-37-wifi-switch，1.7.5，本機 3230/7870）：① 熱點關掉 → 醒來重開後改連 HKQF - Guest 並上線（運行中途消失未單獨測）⑦ Use 按鈕、確認框（寫明 20 秒退回原網絡）、切換中提示都正常；熱點關著按 Use → 11 秒內頁面『couldn't find … nearby. It's back on HKQF - Guest』；熱點開著（到不了 Mac）→ 9 秒內『joined … but couldn't reach the internet … back on HKQF - Guest』，串口 failed (no_internet) → Back on；切換到目前網絡 → current、未存 SSID → unknown，板子不動。pytest 272 passed（新增 6 項），tsc 0 錯誤。未做：⑦ 成功切換（要第二個到得了 Mac 的網絡）、別人設備呼叫 switch → 403（同一個擁有者檢查，未對 switch 重測）、② 密碼打錯
-① 設定頁顯示玩具在線／離線、目前 Wi-Fi 和訊號、已記住的 Wi-Fi 清單（只有名稱，不顯示密碼）② 在線時可新增 Wi-Fi（輸入或從玩具掃描到的清單選）、刪除 Wi-Fi；不能刪除正在使用的那個 ③ 經 /ws/esp32 轉送：伺服器先確認是設備主人；密碼不寫入資料庫、不寫入日誌 ④ 新增不自動切換網絡；目前 Wi-Fi 消失時按訊號選，或由家長按「改用這個」（⑦）；清單標示「連過／未連過」⑤ 上限 8 個 ⑥ 韌體改動經 OTA 推出 ⑦ 已記住、未在使用的 Wi-Fi 可按「改用這個」：玩具斷開目前網絡改連它，最多 20 秒，要連上我們的伺服器才算成功；失敗就自動連回原網絡，頁面顯示「連不上 X，已回到 Y」；切換中頁面顯示切換中，玩具重新連上後刷新；成功後標示連過</t>
+          <t>上次測試：部分通過 — 後端部分（分支 p2-22-server-urls）：node --test lib/deviceServerUrls.test.mjs 5/5、tsc 0 錯誤。worktree dev server 3222 + 本機 Supabase，兩塊假板（02:22:…:01/02）：已認領 200 帶 voice_url + backend_url；未認領 202 只帶 backend_url；DEVICE_VOICE_URL=ws://fastapi:7860/… → 不發、日誌記錯誤；兩個變數都不設 → 兩個欄位都不帶；生產值 → wss://elatoai.hkqft.com/fastapi/ws/esp32、https://elatoai.hkqft.com。測試數據已清除
+① /api/generate_auth_token 的回應帶 voice_url（wss 主機＋端口＋路徑，來自後端環境變數）；韌體用它連 /ws，並把最後一次成功的值存進 NVS；改 FastAPI 網址只改伺服器設定，不需新韌體 ② 回應沒有 voice_url（舊後端）或新網址連不上時，退回 NVS 上次成功的值，再退回出廠／編譯時的預設值 ③ 後端網址可遷移：回應可帶 backend_url；韌體先存為候選，下次開機用新網址取 token 成功才正式替換，失敗就繼續用舊網址；舊網址在遷移期內保持可用（runbook 寫明保留多久） ④ 已確認的韌體若連續 N 次開機（預設 10 次、跨度至少 24 小時，計數存 NVS）Wi-Fi 已拿到 IP 卻取不到 token：先依次試 NVS、出廠的後端網址；仍失敗且另一個槽可用，就切到另一個槽一次，並在下次連上時把本版本報為失敗 ⑤ 純斷網（拿不到 IP、路由器沒外網）不計入 ④ ⑥ 新網址的證書必須鏈到 CF_CA_bundle 裡的根（GTS Root R4、ISRG Root X1）；換主機或離開 Cloudflare 前先查證書鏈，runbook 寫明 ⑦ 只接受 https 的 backend_url 和 wss 的 voice_url，主機須在韌體內允許的網域後綴之下，防止後端被冒充時把板子引去別處</t>
         </is>
       </c>
       <c r="F35" s="11" t="n"/>
@@ -1677,30 +1676,31 @@
       <c r="H35" s="11" t="n"/>
       <c r="I35" s="12" t="n"/>
     </row>
-    <row r="36" ht="102" customHeight="1">
+    <row r="36" ht="409" customHeight="1">
       <c r="A36" s="13" t="inlineStr">
         <is>
-          <t>R-16</t>
+          <t>R-37</t>
         </is>
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>Spotpear 量產版加電池電壓檢測（GPIO0 分壓）</t>
+          <t>網頁設定玩具的 Wi-Fi：查看、新增、刪除</t>
         </is>
       </c>
       <c r="C36" s="13" t="inlineStr">
         <is>
-          <t>1 止血定案</t>
+          <t>3 封閉內測</t>
         </is>
       </c>
       <c r="D36" s="13" t="inlineStr">
         <is>
-          <t>未開始</t>
+          <t>進行中</t>
         </is>
       </c>
       <c r="E36" s="6" t="inlineStr">
         <is>
-          <t>Spotpear 書面確認量產版：GPIO1（屏幕 DC；本版不接屏幕，可空出來）接電芯正極（保護 IC 之後）100k/100k 分壓、100nF 濾波，屏幕不接該腳；GPIO0 保留給現有的 VDD 低電提醒；最好另把充電芯片 CHRG 接到 GPIO12 或 13。樣板到手後，固件讀到的電芯電壓與萬用表相差 ≤50mV，App（R-41）顯示百分比與充電中。</t>
+          <t>上次測試：部分通過 — 2026-10-15 真機 62:70（hw-test-1015 = dev + P2-16 + R-36 + r-37-wifi-switch，1.7.5，本機 3230/7870）：① 熱點關掉 → 醒來重開後改連 HKQF - Guest 並上線（運行中途消失未單獨測）⑦ Use 按鈕、確認框（寫明 20 秒退回原網絡）、切換中提示都正常；熱點關著按 Use → 11 秒內頁面『couldn't find … nearby. It's back on HKQF - Guest』；熱點開著（到不了 Mac）→ 9 秒內『joined … but couldn't reach the internet … back on HKQF - Guest』，串口 failed (no_internet) → Back on；切換到目前網絡 → current、未存 SSID → unknown，板子不動。pytest 272 passed（新增 6 項），tsc 0 錯誤。未做：⑦ 成功切換（要第二個到得了 Mac 的網絡）、別人設備呼叫 switch → 403（同一個擁有者檢查，未對 switch 重測）、② 密碼打錯
+① 設定頁顯示玩具在線／離線、目前 Wi-Fi 和訊號、已記住的 Wi-Fi 清單（只有名稱，不顯示密碼）② 在線時可新增 Wi-Fi（輸入或從玩具掃描到的清單選）、刪除 Wi-Fi；不能刪除正在使用的那個 ③ 經 /ws/esp32 轉送：伺服器先確認是設備主人；密碼不寫入資料庫、不寫入日誌 ④ 新增不自動切換網絡；目前 Wi-Fi 消失時按訊號選，或由家長按「改用這個」（⑦）；清單標示「連過／未連過」⑤ 上限 8 個 ⑥ 韌體改動經 OTA 推出 ⑦ 已記住、未在使用的 Wi-Fi 可按「改用這個」：玩具斷開目前網絡改連它，最多 20 秒，要連上我們的伺服器才算成功；失敗就自動連回原網絡，頁面顯示「連不上 X，已回到 Y」；切換中頁面顯示切換中，玩具重新連上後刷新；成功後標示連過</t>
         </is>
       </c>
       <c r="F36" s="11" t="n"/>
@@ -1708,20 +1708,20 @@
       <c r="H36" s="11" t="n"/>
       <c r="I36" s="12" t="n"/>
     </row>
-    <row r="37" ht="46" customHeight="1">
+    <row r="37" ht="102" customHeight="1">
       <c r="A37" s="13" t="inlineStr">
         <is>
-          <t>P1-11</t>
+          <t>R-16</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>伺服器與資料庫直接存取的管控</t>
+          <t>Spotpear 量產版加電池電壓檢測（GPIO0 分壓）</t>
         </is>
       </c>
       <c r="C37" s="13" t="inlineStr">
         <is>
-          <t>2 內測準備</t>
+          <t>1 止血定案</t>
         </is>
       </c>
       <c r="D37" s="13" t="inlineStr">
@@ -1731,7 +1731,7 @@
       </c>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>列出誰有 SSH 與資料庫直連權限（越少越好）；service_role key 只存在伺服器的 env；私隱政策寫明這類存取的範圍；每次直接查看生產資料都留記錄。</t>
+          <t>Spotpear 書面確認量產版：GPIO1（屏幕 DC；本版不接屏幕，可空出來）接電芯正極（保護 IC 之後）100k/100k 分壓、100nF 濾波，屏幕不接該腳；GPIO0 保留給現有的 VDD 低電提醒；最好另把充電芯片 CHRG 接到 GPIO12 或 13。樣板到手後，固件讀到的電芯電壓與萬用表相差 ≤50mV，App（R-41）顯示百分比與充電中。</t>
         </is>
       </c>
       <c r="F37" s="11" t="n"/>
@@ -1742,12 +1742,12 @@
     <row r="38" ht="46" customHeight="1">
       <c r="A38" s="13" t="inlineStr">
         <is>
-          <t>P2-02</t>
+          <t>P1-11</t>
         </is>
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>CI 跑測試與靜態檢查</t>
+          <t>伺服器與資料庫直接存取的管控</t>
         </is>
       </c>
       <c r="C38" s="13" t="inlineStr">
@@ -1762,7 +1762,7 @@
       </c>
       <c r="E38" s="6" t="inlineStr">
         <is>
-          <t>推送與 PR 時跑 pytest、ruff、pyright、next lint、tsc --noEmit、pio run；任何一項失敗就不發佈 image。</t>
+          <t>列出誰有 SSH 與資料庫直連權限（越少越好）；service_role key 只存在伺服器的 env；私隱政策寫明這類存取的範圍；每次直接查看生產資料都留記錄。</t>
         </is>
       </c>
       <c r="F38" s="11" t="n"/>
@@ -1770,15 +1770,15 @@
       <c r="H38" s="11" t="n"/>
       <c r="I38" s="12" t="n"/>
     </row>
-    <row r="39" ht="32" customHeight="1">
+    <row r="39" ht="46" customHeight="1">
       <c r="A39" s="13" t="inlineStr">
         <is>
-          <t>P2-04</t>
+          <t>P2-02</t>
         </is>
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>容器改用非 root 用戶</t>
+          <t>CI 跑測試與靜態檢查</t>
         </is>
       </c>
       <c r="C39" s="13" t="inlineStr">
@@ -1793,7 +1793,7 @@
       </c>
       <c r="E39" s="6" t="inlineStr">
         <is>
-          <t>兩個 Dockerfile 都設定非 root 的 USER。</t>
+          <t>推送與 PR 時跑 pytest、ruff、pyright、next lint、tsc --noEmit、pio run；任何一項失敗就不發佈 image。</t>
         </is>
       </c>
       <c r="F39" s="11" t="n"/>
@@ -1801,15 +1801,15 @@
       <c r="H39" s="11" t="n"/>
       <c r="I39" s="12" t="n"/>
     </row>
-    <row r="40" ht="102" customHeight="1">
+    <row r="40" ht="32" customHeight="1">
       <c r="A40" s="13" t="inlineStr">
         <is>
-          <t>P2-24</t>
+          <t>P2-04</t>
         </is>
       </c>
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>麥克風上行改用 IMA ADPCM（減少 4 倍頻寬）</t>
+          <t>容器改用非 root 用戶</t>
         </is>
       </c>
       <c r="C40" s="13" t="inlineStr">
@@ -1824,7 +1824,7 @@
       </c>
       <c r="E40" s="6" t="inlineStr">
         <is>
-          <t>① 新韌體上行用 IMA ADPCM（64 kbps），每幀帶解碼狀態（預測值＋步長索引），掉幀或重連後下一幀即可正確解碼 ② 連線時以 header 聲明編碼；伺服器據此解碼成 16kHz PCM 再交給 STT；沒有聲明的舊韌體照舊當 PCM ③ 韌體編碼與伺服器解碼位元一致（同一算法）④ 編碼 CPU &lt; 2%、不增加延遲 ⑤ 語音辨識品質與 PCM 相當</t>
+          <t>兩個 Dockerfile 都設定非 root 的 USER。</t>
         </is>
       </c>
       <c r="F40" s="11" t="n"/>
@@ -1863,68 +1863,68 @@
       <c r="H41" s="11" t="n"/>
       <c r="I41" s="12" t="n"/>
     </row>
-    <row r="43">
-      <c r="A43" s="10" t="inlineStr">
+    <row r="42" ht="116" customHeight="1">
+      <c r="A42" s="13" t="inlineStr">
+        <is>
+          <t>R-25</t>
+        </is>
+      </c>
+      <c r="B42" s="6" t="inlineStr">
+        <is>
+          <t>網頁的品牌主題系統</t>
+        </is>
+      </c>
+      <c r="C42" s="13" t="inlineStr">
+        <is>
+          <t>2 內測準備</t>
+        </is>
+      </c>
+      <c r="D42" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E42" s="6" t="inlineStr">
+        <is>
+          <t>① 每個品牌一個資料夾：主題 token（顏色、字體、圓角）、logo 和圖示、文案、功能開關；首頁、上手流程、角色頁可以有品牌版本，其餘頁面共用 ② 由部署的環境變數選品牌（每套部署一個品牌，見 R-34），伺服器端渲染的第一屏就是對的主題，不閃爍 ③ 共用元件裡沒有品牌名稱和寫死的品牌顏色 ④ 加一個品牌只需要加資料夾、設定和一套部署，不用改共用元件</t>
+        </is>
+      </c>
+      <c r="F42" s="11" t="n"/>
+      <c r="G42" s="11" t="n"/>
+      <c r="H42" s="11" t="n"/>
+      <c r="I42" s="12" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="10" t="inlineStr">
         <is>
           <t>✅ 最近完成與測試效果</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="4" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
         <is>
           <t>編號</t>
         </is>
       </c>
-      <c r="B44" s="4" t="inlineStr">
+      <c r="B45" s="4" t="inlineStr">
         <is>
           <t>任務</t>
         </is>
       </c>
-      <c r="C44" s="4" t="inlineStr">
+      <c r="C45" s="4" t="inlineStr">
         <is>
           <t>測試結果</t>
         </is>
       </c>
-      <c r="D44" s="4" t="inlineStr">
+      <c r="D45" s="4" t="inlineStr">
         <is>
           <t>完成日期</t>
         </is>
       </c>
-      <c r="E44" s="4" t="inlineStr">
+      <c r="E45" s="4" t="inlineStr">
         <is>
           <t>測試證據</t>
-        </is>
-      </c>
-      <c r="F44" s="11" t="n"/>
-      <c r="G44" s="11" t="n"/>
-      <c r="H44" s="11" t="n"/>
-      <c r="I44" s="12" t="n"/>
-    </row>
-    <row r="45" ht="88" customHeight="1">
-      <c r="A45" s="13" t="inlineStr">
-        <is>
-          <t>P2-21</t>
-        </is>
-      </c>
-      <c r="B45" s="6" t="inlineStr">
-        <is>
-          <t>P2-16 ⑤ 後台 OTA 頁換成真實數據與操作</t>
-        </is>
-      </c>
-      <c r="C45" s="13" t="inlineStr">
-        <is>
-          <t>通過</t>
-        </is>
-      </c>
-      <c r="D45" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
-      <c r="E45" s="6" t="inlineStr">
-        <is>
-          <t>10-14 模擬 20 台全部通過（見上次）；2026-10-15 真機補做：OTA 頁對 1.7.1 白名單加 62:70（UI MAC 欄）→ 存檔確認框 → 『Narrow to Whitelist』確認 → Make current（用戶點）→ 62:70 安裝並確認，頁面顯示 Rolling out · Whitelist、運行 1、回滾 0；每步一筆審計。依賴 P2-14 已完成</t>
         </is>
       </c>
       <c r="F45" s="11" t="n"/>
@@ -1932,15 +1932,15 @@
       <c r="H45" s="11" t="n"/>
       <c r="I45" s="12" t="n"/>
     </row>
-    <row r="46" ht="158" customHeight="1">
+    <row r="46" ht="88" customHeight="1">
       <c r="A46" s="13" t="inlineStr">
         <is>
-          <t>P2-16</t>
+          <t>P2-21</t>
         </is>
       </c>
       <c r="B46" s="6" t="inlineStr">
         <is>
-          <t>OTA 分批推送與後台發佈頁</t>
+          <t>P2-16 ⑤ 後台 OTA 頁換成真實數據與操作</t>
         </is>
       </c>
       <c r="C46" s="13" t="inlineStr">
@@ -1955,7 +1955,7 @@
       </c>
       <c r="E46" s="6" t="inlineStr">
         <is>
-          <t>④ 真機 62:70（2026-10-15）：USB 刷 1.7.0（開機印 aibuddy-build;kind=dev;…;version=1.7.0）→ release_firmware.py publish --dev 1.7.1 → 後台白名單加 62:70、改白名單階段、設為 current → 按 BOOT 喚醒：取 token 200、下載 12.8s、重開進 app1，09:39:36 連上語音伺服器；09:42 重開 → 『Firmware 1.7.1 on app1』無 probation、Up to date；頁面『Rolling out · Whitelist』運行 1 台、回滾 0；審計 5 筆（發佈、白名單、階段、1.6.2 取消 current、1.7.1 設 current）。①②③⑤ 見 P2-17～P2-21 模擬 20 台</t>
+          <t>10-14 模擬 20 台全部通過（見上次）；2026-10-15 真機補做：OTA 頁對 1.7.1 白名單加 62:70（UI MAC 欄）→ 存檔確認框 → 『Narrow to Whitelist』確認 → Make current（用戶點）→ 62:70 安裝並確認，頁面顯示 Rolling out · Whitelist、運行 1、回滾 0；每步一筆審計。依賴 P2-14 已完成</t>
         </is>
       </c>
       <c r="F46" s="11" t="n"/>
@@ -1963,15 +1963,15 @@
       <c r="H46" s="11" t="n"/>
       <c r="I46" s="12" t="n"/>
     </row>
-    <row r="47" ht="144" customHeight="1">
+    <row r="47" ht="158" customHeight="1">
       <c r="A47" s="13" t="inlineStr">
         <is>
-          <t>P2-14</t>
+          <t>P2-16</t>
         </is>
       </c>
       <c r="B47" s="6" t="inlineStr">
         <is>
-          <t>Admin 設備頁：每台玩具的狀態、韌體與基本操作</t>
+          <t>OTA 分批推送與後台發佈頁</t>
         </is>
       </c>
       <c r="C47" s="13" t="inlineStr">
@@ -1986,7 +1986,7 @@
       </c>
       <c r="E47" s="6" t="inlineStr">
         <is>
-          <t>真機 62:70（2026-10-15，分支 hw-test-1015 = dev+P2-16，-localall 1.7.0，本機網頁 3230 + 語音 7870）：① 開機 → 設備頁 Online、-67 dBm、1.7.0；板子停在 bootloader 約 38 秒後語音伺服器判離線（uvicorn ping 超時），頁面 0 台在線 ② 重置設備密鑰 → device_secrets 行刪除，板子重開印『Device secret issued and stored』並連上，行恢復 ③ 強制解綁 → 板子拿 202（配對碼 UKDM7N），語音伺服器拒絕連線；兩項審計各 1 筆含操作者與原因 ④ 內容管理員/anon → 42501（10-14 探測腳本）</t>
+          <t>④ 真機 62:70（2026-10-15）：USB 刷 1.7.0（開機印 aibuddy-build;kind=dev;…;version=1.7.0）→ release_firmware.py publish --dev 1.7.1 → 後台白名單加 62:70、改白名單階段、設為 current → 按 BOOT 喚醒：取 token 200、下載 12.8s、重開進 app1，09:39:36 連上語音伺服器；09:42 重開 → 『Firmware 1.7.1 on app1』無 probation、Up to date；頁面『Rolling out · Whitelist』運行 1 台、回滾 0；審計 5 筆（發佈、白名單、階段、1.6.2 取消 current、1.7.1 設 current）。①②③⑤ 見 P2-17～P2-21 模擬 20 台</t>
         </is>
       </c>
       <c r="F47" s="11" t="n"/>
@@ -1994,15 +1994,15 @@
       <c r="H47" s="11" t="n"/>
       <c r="I47" s="12" t="n"/>
     </row>
-    <row r="48" ht="214" customHeight="1">
+    <row r="48" ht="144" customHeight="1">
       <c r="A48" s="13" t="inlineStr">
         <is>
-          <t>P2-20</t>
+          <t>P2-14</t>
         </is>
       </c>
       <c r="B48" s="6" t="inlineStr">
         <is>
-          <t>P2-16 ④ 從後台上傳與發佈韌體（取代手貼 service key）</t>
+          <t>Admin 設備頁：每台玩具的狀態、韌體與基本操作</t>
         </is>
       </c>
       <c r="C48" s="13" t="inlineStr">
@@ -2012,12 +2012,12 @@
       </c>
       <c r="D48" s="13" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E48" s="6" t="inlineStr">
         <is>
-          <t>node --test lib/firmwareImage.test.mjs 8/8（合成映像：dev build、無標記、未知板、晶片不符、非映像、截斷/損壞、超 4MB 拒；超 2MB 只警告）。分支 dev server + 本機 Supabase 端到端 16/16（GoTrue 真實登入的 cookie）：超管上傳 9.9.0 release build → 201 草稿（is_current f、rollout 0%），DB SHA-256 = 檔案、storage 原樣；審計 insert 記該超管；設備仍只拿到 current 1.6.2；已有 1.0.2 → 409；localall → 422 dev build；4MB+16 → 422；9MB → 413；PNG → 422；舊 1.6.1 映像（無標記）→ 422 指向 release_firmware.py；內容管理員上傳/刪除 → 403；未登入 → 401；刪 current → 409；超管刪草稿 → 行和映像都刪、審計 delete 記該超管。release_firmware.py list 照常。測試帳號與數據已清除</t>
+          <t>真機 62:70（2026-10-15，分支 hw-test-1015 = dev+P2-16，-localall 1.7.0，本機網頁 3230 + 語音 7870）：① 開機 → 設備頁 Online、-67 dBm、1.7.0；板子停在 bootloader 約 38 秒後語音伺服器判離線（uvicorn ping 超時），頁面 0 台在線 ② 重置設備密鑰 → device_secrets 行刪除，板子重開印『Device secret issued and stored』並連上，行恢復 ③ 強制解綁 → 板子拿 202（配對碼 UKDM7N），語音伺服器拒絕連線；兩項審計各 1 筆含操作者與原因 ④ 內容管理員/anon → 42501（10-14 探測腳本）</t>
         </is>
       </c>
       <c r="F48" s="11" t="n"/>
@@ -2025,15 +2025,15 @@
       <c r="H48" s="11" t="n"/>
       <c r="I48" s="12" t="n"/>
     </row>
-    <row r="49" ht="158" customHeight="1">
+    <row r="49" ht="214" customHeight="1">
       <c r="A49" s="13" t="inlineStr">
         <is>
-          <t>P2-19</t>
+          <t>P2-20</t>
         </is>
       </c>
       <c r="B49" s="6" t="inlineStr">
         <is>
-          <t>P2-16 ③ 回滾過多時自動暫停推送</t>
+          <t>P2-16 ④ 從後台上傳與發佈韌體（取代手貼 service key）</t>
         </is>
       </c>
       <c r="C49" s="13" t="inlineStr">
@@ -2048,7 +2048,7 @@
       </c>
       <c r="E49" s="6" t="inlineStr">
         <is>
-          <t>migration 20261014200000 BEGIN/ROLLBACK 套用兩次無錯並已套用本機。模擬 20 台連跑兩次 12/12：1/20 回滾不暫停、其餘 18 台照常；2/20 → 'Auto-paused: 2 of 20 boards rolled back (10%)'，其餘 0 台拿到 ota；已運行的設備記為 running 且不再下發；審計 1 筆 actor 空；恢復後 17 台拿到、保持恢復，第 3 台回滾 → 'Auto-paused: 3 of 20 (15%)'；白名單 2 台中 1 台回滾 → 50% 立即暫停、另一台不再下發；anon 呼叫 ota_maybe_pause → 401/42501。測試數據已清除，spotpear-ai-toy 1.6.2 仍 100% 未暫停</t>
+          <t>node --test lib/firmwareImage.test.mjs 8/8（合成映像：dev build、無標記、未知板、晶片不符、非映像、截斷/損壞、超 4MB 拒；超 2MB 只警告）。分支 dev server + 本機 Supabase 端到端 16/16（GoTrue 真實登入的 cookie）：超管上傳 9.9.0 release build → 201 草稿（is_current f、rollout 0%），DB SHA-256 = 檔案、storage 原樣；審計 insert 記該超管；設備仍只拿到 current 1.6.2；已有 1.0.2 → 409；localall → 422 dev build；4MB+16 → 422；9MB → 413；PNG → 422；舊 1.6.1 映像（無標記）→ 422 指向 release_firmware.py；內容管理員上傳/刪除 → 403；未登入 → 401；刪 current → 409；超管刪草稿 → 行和映像都刪、審計 delete 記該超管。release_firmware.py list 照常。測試帳號與數據已清除</t>
         </is>
       </c>
       <c r="F49" s="11" t="n"/>
@@ -2056,15 +2056,15 @@
       <c r="H49" s="11" t="n"/>
       <c r="I49" s="12" t="n"/>
     </row>
-    <row r="50" ht="200" customHeight="1">
+    <row r="50" ht="158" customHeight="1">
       <c r="A50" s="13" t="inlineStr">
         <is>
-          <t>P2-18</t>
+          <t>P2-19</t>
         </is>
       </c>
       <c r="B50" s="6" t="inlineStr">
         <is>
-          <t>P2-16 ② 按 MAC 雜湊穩定分組決定哪台收到 ota</t>
+          <t>P2-16 ③ 回滾過多時自動暫停推送</t>
         </is>
       </c>
       <c r="C50" s="13" t="inlineStr">
@@ -2079,7 +2079,7 @@
       </c>
       <c r="E50" s="6" t="inlineStr">
         <is>
-          <t>node --test lib/otaRollout.test.mjs 6/6：10,000 隨機 MAC 在 10%/50% 誤差 &lt; 1 個百分點、同 MAC（含大小寫/空白）結果一致、升階段只增不減、白名單各階段都在、不同版本選不同的 10%。tsc --noEmit 通過。分支 dev server（3216）+ 本機 Supabase 模擬 20 台（板型 p218-sim，連跑兩次 9/9）：白名單階段只有 1 台、重複不變；10% 拿到的正是雜湊預測的那組（2–5 台含白名單），重複不變；50% 包含 10% 全部；暫停 → 0 台且下載映像 404，恢復 → 200；100% → 除已更新和已回滾的 2 台外 18 台；每台下發次數與記錄一致；運行中/已回滾正確標記；審計 6 筆對應 6 次變更。真 spotpear-ai-toy（預設 100%）回報 1.6.1 → 仍拿到 1.6.2。測試數據已清除</t>
+          <t>migration 20261014200000 BEGIN/ROLLBACK 套用兩次無錯並已套用本機。模擬 20 台連跑兩次 12/12：1/20 回滾不暫停、其餘 18 台照常；2/20 → 'Auto-paused: 2 of 20 boards rolled back (10%)'，其餘 0 台拿到 ota；已運行的設備記為 running 且不再下發；審計 1 筆 actor 空；恢復後 17 台拿到、保持恢復，第 3 台回滾 → 'Auto-paused: 3 of 20 (15%)'；白名單 2 台中 1 台回滾 → 50% 立即暫停、另一台不再下發；anon 呼叫 ota_maybe_pause → 401/42501。測試數據已清除，spotpear-ai-toy 1.6.2 仍 100% 未暫停</t>
         </is>
       </c>
       <c r="F50" s="11" t="n"/>
@@ -2087,15 +2087,15 @@
       <c r="H50" s="11" t="n"/>
       <c r="I50" s="12" t="n"/>
     </row>
-    <row r="51" ht="172" customHeight="1">
+    <row r="51" ht="200" customHeight="1">
       <c r="A51" s="13" t="inlineStr">
         <is>
-          <t>P2-17</t>
+          <t>P2-18</t>
         </is>
       </c>
       <c r="B51" s="6" t="inlineStr">
         <is>
-          <t>P2-16 ① 分批推送的數據表：推送階段、白名單、每台安裝結果</t>
+          <t>P2-16 ② 按 MAC 雜湊穩定分組決定哪台收到 ota</t>
         </is>
       </c>
       <c r="C51" s="13" t="inlineStr">
@@ -2110,7 +2110,7 @@
       </c>
       <c r="E51" s="6" t="inlineStr">
         <is>
-          <t>migration 20261014190000 BEGIN/ROLLBACK 套用兩次無錯並已套用本機；行為：預設 100%、promote 記 stage_changed_at，7 種壞值（25%、小寫/空字串/NULL MAC、暫停缺原因等）全被 check 擋；ota_note_offer 1→2→3，report 正確標 running/failed、別板型不影響，刪發佈連帶刪記錄；審計 5 筆含 'test-board 9.9.9' 標籤。REST 13/13：超管可讀、內容管理員 0 行、anon 42501，三種身份寫入/改階段/呼叫 ota_note_offer 皆 42501。release_firmware.py promote spotpear-ai-toy 1.6.2 成功，token 查詢仍選 1.6.2，審計記 2 筆（actor 空＝service role）</t>
+          <t>node --test lib/otaRollout.test.mjs 6/6：10,000 隨機 MAC 在 10%/50% 誤差 &lt; 1 個百分點、同 MAC（含大小寫/空白）結果一致、升階段只增不減、白名單各階段都在、不同版本選不同的 10%。tsc --noEmit 通過。分支 dev server（3216）+ 本機 Supabase 模擬 20 台（板型 p218-sim，連跑兩次 9/9）：白名單階段只有 1 台、重複不變；10% 拿到的正是雜湊預測的那組（2–5 台含白名單），重複不變；50% 包含 10% 全部；暫停 → 0 台且下載映像 404，恢復 → 200；100% → 除已更新和已回滾的 2 台外 18 台；每台下發次數與記錄一致；運行中/已回滾正確標記；審計 6 筆對應 6 次變更。真 spotpear-ai-toy（預設 100%）回報 1.6.1 → 仍拿到 1.6.2。測試數據已清除</t>
         </is>
       </c>
       <c r="F51" s="11" t="n"/>
@@ -2118,15 +2118,15 @@
       <c r="H51" s="11" t="n"/>
       <c r="I51" s="12" t="n"/>
     </row>
-    <row r="52" ht="116" customHeight="1">
+    <row r="52" ht="172" customHeight="1">
       <c r="A52" s="13" t="inlineStr">
         <is>
-          <t>R-41</t>
+          <t>P2-17</t>
         </is>
       </c>
       <c r="B52" s="6" t="inlineStr">
         <is>
-          <t>App 顯示玩具電量狀態（低電量提示）</t>
+          <t>P2-16 ① 分批推送的數據表：推送階段、白名單、每台安裝結果</t>
         </is>
       </c>
       <c r="C52" s="13" t="inlineStr">
@@ -2141,7 +2141,7 @@
       </c>
       <c r="E52" s="6" t="inlineStr">
         <is>
-          <t>① pytest 33 passed；真 PATCH 本地 Supabase ② 62:70 刷 p212+R-41 強制低電 build（SUPPLY_LOW_RATIO_OVERRIDE=1.05）→ 串口 [WSc] power low:true，本地 DB battery_low=t ③ 刷回正常 1.6.2 → low:false，DB=f ④ App 讀 DB：低電紅標+Please charge+更新時間、72% 充電中、未上報不顯示 ⑤ 他人帳號 0 行、authenticated UPDATE 被拒。62:70 已還原為原 p212 build</t>
+          <t>migration 20261014190000 BEGIN/ROLLBACK 套用兩次無錯並已套用本機；行為：預設 100%、promote 記 stage_changed_at，7 種壞值（25%、小寫/空字串/NULL MAC、暫停缺原因等）全被 check 擋；ota_note_offer 1→2→3，report 正確標 running/failed、別板型不影響，刪發佈連帶刪記錄；審計 5 筆含 'test-board 9.9.9' 標籤。REST 13/13：超管可讀、內容管理員 0 行、anon 42501，三種身份寫入/改階段/呼叫 ota_note_offer 皆 42501。release_firmware.py promote spotpear-ai-toy 1.6.2 成功，token 查詢仍選 1.6.2，審計記 2 筆（actor 空＝service role）</t>
         </is>
       </c>
       <c r="F52" s="11" t="n"/>
@@ -2149,50 +2149,58 @@
       <c r="H52" s="11" t="n"/>
       <c r="I52" s="12" t="n"/>
     </row>
-    <row r="54">
-      <c r="A54" s="10" t="inlineStr">
+    <row r="53" ht="116" customHeight="1">
+      <c r="A53" s="13" t="inlineStr">
+        <is>
+          <t>R-41</t>
+        </is>
+      </c>
+      <c r="B53" s="6" t="inlineStr">
+        <is>
+          <t>App 顯示玩具電量狀態（低電量提示）</t>
+        </is>
+      </c>
+      <c r="C53" s="13" t="inlineStr">
+        <is>
+          <t>通過</t>
+        </is>
+      </c>
+      <c r="D53" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="E53" s="6" t="inlineStr">
+        <is>
+          <t>① pytest 33 passed；真 PATCH 本地 Supabase ② 62:70 刷 p212+R-41 強制低電 build（SUPPLY_LOW_RATIO_OVERRIDE=1.05）→ 串口 [WSc] power low:true，本地 DB battery_low=t ③ 刷回正常 1.6.2 → low:false，DB=f ④ App 讀 DB：低電紅標+Please charge+更新時間、72% 充電中、未上報不顯示 ⑤ 他人帳號 0 行、authenticated UPDATE 被拒。62:70 已還原為原 p212 build</t>
+        </is>
+      </c>
+      <c r="F53" s="11" t="n"/>
+      <c r="G53" s="11" t="n"/>
+      <c r="H53" s="11" t="n"/>
+      <c r="I53" s="12" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="10" t="inlineStr">
         <is>
           <t>⏳ 等待依賴 / ⛔ 阻塞</t>
         </is>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="4" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
         <is>
           <t>編號</t>
         </is>
       </c>
-      <c r="B55" s="4" t="inlineStr">
+      <c r="B56" s="4" t="inlineStr">
         <is>
           <t>任務</t>
         </is>
       </c>
-      <c r="C55" s="4" t="inlineStr">
+      <c r="C56" s="4" t="inlineStr">
         <is>
           <t>在等什麼</t>
-        </is>
-      </c>
-      <c r="D55" s="11" t="n"/>
-      <c r="E55" s="11" t="n"/>
-      <c r="F55" s="11" t="n"/>
-      <c r="G55" s="11" t="n"/>
-      <c r="H55" s="11" t="n"/>
-      <c r="I55" s="12" t="n"/>
-    </row>
-    <row r="56" ht="88" customHeight="1">
-      <c r="A56" s="13" t="inlineStr">
-        <is>
-          <t>R-17</t>
-        </is>
-      </c>
-      <c r="B56" s="6" t="inlineStr">
-        <is>
-          <t>Spotpear 電池耗盡時插電能否正常開機（供電路徑）</t>
-        </is>
-      </c>
-      <c r="C56" s="6" t="inlineStr">
-        <is>
-          <t>阻塞：[2026-10-08] 2026-10-08 開發板 63:64 插著 USB 時兩次無法解釋的完全斷電重開：09:13:26（崩潰循環中）、10:44:33（閒置、用戶確認沒碰）。都是 USB 先斷線再以 ESP_RST_POWERON 開機，非 brownout；斷電前 6 秒 GPIO0 讀數 99.9% 參考值，屬突然切斷而非緩降（SupplyMonitor 取樣太疏抓不到瞬間）。韌體無法造成 POWERON，指向充電芯片/電池保護/供電路徑，應一併問 Spotpear；放電實測時留意插 USB 閒置時是否也會斷電</t>
         </is>
       </c>
       <c r="D56" s="11" t="n"/>
@@ -2202,20 +2210,20 @@
       <c r="H56" s="11" t="n"/>
       <c r="I56" s="12" t="n"/>
     </row>
-    <row r="57" ht="60" customHeight="1">
+    <row r="57" ht="88" customHeight="1">
       <c r="A57" s="13" t="inlineStr">
         <is>
-          <t>P1-01</t>
+          <t>R-17</t>
         </is>
       </c>
       <c r="B57" s="6" t="inlineStr">
         <is>
-          <t>加入內容審核層（輸入與輸出）</t>
+          <t>Spotpear 電池耗盡時插電能否正常開機（供電路徑）</t>
         </is>
       </c>
       <c r="C57" s="6" t="inlineStr">
         <is>
-          <t>阻塞：[2026-10-14] 2026-10-14 用戶決定：先不定審核服務商，本項暫停。候選：Azure Content Safety（建議，香港區、可在每句回覆說出口前檢查）、OpenRouter 安全模型、OpenAI Moderation、只用本機字詞表。未寫任何程式。</t>
+          <t>阻塞：[2026-10-08] 2026-10-08 開發板 63:64 插著 USB 時兩次無法解釋的完全斷電重開：09:13:26（崩潰循環中）、10:44:33（閒置、用戶確認沒碰）。都是 USB 先斷線再以 ESP_RST_POWERON 開機，非 brownout；斷電前 6 秒 GPIO0 讀數 99.9% 參考值，屬突然切斷而非緩降（SupplyMonitor 取樣太疏抓不到瞬間）。韌體無法造成 POWERON，指向充電芯片/電池保護/供電路徑，應一併問 Spotpear；放電實測時留意插 USB 閒置時是否也會斷電</t>
         </is>
       </c>
       <c r="D57" s="11" t="n"/>
@@ -2225,20 +2233,20 @@
       <c r="H57" s="11" t="n"/>
       <c r="I57" s="12" t="n"/>
     </row>
-    <row r="58" ht="32" customHeight="1">
+    <row r="58" ht="60" customHeight="1">
       <c r="A58" s="13" t="inlineStr">
         <is>
-          <t>P1-09</t>
+          <t>P1-01</t>
         </is>
       </c>
       <c r="B58" s="6" t="inlineStr">
         <is>
-          <t>家長鎖：孩子模式進設定要輸入 PIN</t>
+          <t>加入內容審核層（輸入與輸出）</t>
         </is>
       </c>
       <c r="C58" s="6" t="inlineStr">
         <is>
-          <t>阻塞：[2026-10-13] 2026-10-13 用戶決定：AI Buddy（品牌 C）延到 1/15 之後，本項不卡 1/15 出廠；AI Buddy 啟動時再開。</t>
+          <t>阻塞：[2026-10-14] 2026-10-14 用戶決定：先不定審核服務商，本項暫停。候選：Azure Content Safety（建議，香港區、可在每句回覆說出口前檢查）、OpenRouter 安全模型、OpenAI Moderation、只用本機字詞表。未寫任何程式。</t>
         </is>
       </c>
       <c r="D58" s="11" t="n"/>
@@ -2251,12 +2259,12 @@
     <row r="59" ht="32" customHeight="1">
       <c r="A59" s="13" t="inlineStr">
         <is>
-          <t>R-12</t>
+          <t>P1-09</t>
         </is>
       </c>
       <c r="B59" s="6" t="inlineStr">
         <is>
-          <t>家長控制：每日使用上限和休息時段</t>
+          <t>家長鎖：孩子模式進設定要輸入 PIN</t>
         </is>
       </c>
       <c r="C59" s="6" t="inlineStr">
@@ -2274,12 +2282,12 @@
     <row r="60" ht="32" customHeight="1">
       <c r="A60" s="13" t="inlineStr">
         <is>
-          <t>R-29</t>
+          <t>R-12</t>
         </is>
       </c>
       <c r="B60" s="6" t="inlineStr">
         <is>
-          <t>AI Buddy App（品牌 C）頁面</t>
+          <t>家長控制：每日使用上限和休息時段</t>
         </is>
       </c>
       <c r="C60" s="6" t="inlineStr">
@@ -2297,17 +2305,17 @@
     <row r="61" ht="32" customHeight="1">
       <c r="A61" s="13" t="inlineStr">
         <is>
-          <t>P2-25</t>
+          <t>R-29</t>
         </is>
       </c>
       <c r="B61" s="6" t="inlineStr">
         <is>
-          <t>C3 斷線後自救：TLS 握手超時縮短、連續失敗重設 Wi-Fi 或重開、修重試漏記憶體</t>
+          <t>AI Buddy App（品牌 C）頁面</t>
         </is>
       </c>
       <c r="C61" s="6" t="inlineStr">
         <is>
-          <t>等 P2-24</t>
+          <t>阻塞：[2026-10-13] 2026-10-13 用戶決定：AI Buddy（品牌 C）延到 1/15 之後，本項不卡 1/15 出廠；AI Buddy 啟動時再開。</t>
         </is>
       </c>
       <c r="D61" s="11" t="n"/>
@@ -2317,20 +2325,20 @@
       <c r="H61" s="11" t="n"/>
       <c r="I61" s="12" t="n"/>
     </row>
-    <row r="62" ht="18" customHeight="1">
+    <row r="62" ht="32" customHeight="1">
       <c r="A62" s="13" t="inlineStr">
         <is>
-          <t>R-05</t>
+          <t>P2-25</t>
         </is>
       </c>
       <c r="B62" s="6" t="inlineStr">
         <is>
-          <t>內測版外殼（3D 打印 20 台）</t>
+          <t>C3 斷線後自救：TLS 握手超時縮短、連續失敗重設 Wi-Fi 或重開、修重試漏記憶體</t>
         </is>
       </c>
       <c r="C62" s="6" t="inlineStr">
         <is>
-          <t>等 R-01</t>
+          <t>等 P2-24</t>
         </is>
       </c>
       <c r="D62" s="11" t="n"/>
@@ -2343,17 +2351,17 @@
     <row r="63" ht="18" customHeight="1">
       <c r="A63" s="13" t="inlineStr">
         <is>
-          <t>R-06</t>
+          <t>R-05</t>
         </is>
       </c>
       <c r="B63" s="6" t="inlineStr">
         <is>
-          <t>家長自助上手流程</t>
+          <t>內測版外殼（3D 打印 20 台）</t>
         </is>
       </c>
       <c r="C63" s="6" t="inlineStr">
         <is>
-          <t>等 P0-11</t>
+          <t>等 R-01</t>
         </is>
       </c>
       <c r="D63" s="11" t="n"/>
@@ -2363,20 +2371,20 @@
       <c r="H63" s="11" t="n"/>
       <c r="I63" s="12" t="n"/>
     </row>
-    <row r="64" ht="32" customHeight="1">
+    <row r="64" ht="18" customHeight="1">
       <c r="A64" s="13" t="inlineStr">
         <is>
-          <t>R-13</t>
+          <t>R-06</t>
         </is>
       </c>
       <c r="B64" s="6" t="inlineStr">
         <is>
-          <t>CP1 內測就緒檢查（10/30）</t>
+          <t>家長自助上手流程</t>
         </is>
       </c>
       <c r="C64" s="6" t="inlineStr">
         <is>
-          <t>等 P0-07、P0-11、P1-01、P1-02、P2-09、R-01、R-02、R-04、R-05、R-06、P1-11</t>
+          <t>等 P0-11</t>
         </is>
       </c>
       <c r="D64" s="11" t="n"/>
@@ -2389,17 +2397,17 @@
     <row r="65" ht="32" customHeight="1">
       <c r="A65" s="13" t="inlineStr">
         <is>
-          <t>R-18</t>
+          <t>R-13</t>
         </is>
       </c>
       <c r="B65" s="6" t="inlineStr">
         <is>
-          <t>長按 BOOT 重新配網（開 AIBuddy-XXXX 熱點）</t>
+          <t>CP1 內測就緒檢查（10/30）</t>
         </is>
       </c>
       <c r="C65" s="6" t="inlineStr">
         <is>
-          <t>等 R-01</t>
+          <t>等 P0-07、P0-11、P1-01、P1-02、P2-09、R-01、R-02、R-04、R-05、R-06、P1-11</t>
         </is>
       </c>
       <c r="D65" s="11" t="n"/>
@@ -2412,12 +2420,12 @@
     <row r="66" ht="32" customHeight="1">
       <c r="A66" s="13" t="inlineStr">
         <is>
-          <t>R-19</t>
+          <t>R-18</t>
         </is>
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
-          <t>外接按鈕：量產板加 I2C 擴展晶片（TCA9555）</t>
+          <t>長按 BOOT 重新配網（開 AIBuddy-XXXX 熱點）</t>
         </is>
       </c>
       <c r="C66" s="6" t="inlineStr">
@@ -2432,20 +2440,20 @@
       <c r="H66" s="11" t="n"/>
       <c r="I66" s="12" t="n"/>
     </row>
-    <row r="67" ht="18" customHeight="1">
+    <row r="67" ht="32" customHeight="1">
       <c r="A67" s="13" t="inlineStr">
         <is>
-          <t>R-20</t>
+          <t>R-19</t>
         </is>
       </c>
       <c r="B67" s="6" t="inlineStr">
         <is>
-          <t>孩子資料與角色改成每台設備一份</t>
+          <t>外接按鈕：量產板加 I2C 擴展晶片（TCA9555）</t>
         </is>
       </c>
       <c r="C67" s="6" t="inlineStr">
         <is>
-          <t>等 P1-12</t>
+          <t>等 R-01</t>
         </is>
       </c>
       <c r="D67" s="11" t="n"/>
@@ -2455,20 +2463,20 @@
       <c r="H67" s="11" t="n"/>
       <c r="I67" s="12" t="n"/>
     </row>
-    <row r="68" ht="32" customHeight="1">
+    <row r="68" ht="18" customHeight="1">
       <c r="A68" s="13" t="inlineStr">
         <is>
-          <t>R-27</t>
+          <t>R-20</t>
         </is>
       </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t>App 內登入：驗證碼、原生社交登入、刪除帳號</t>
+          <t>孩子資料與角色改成每台設備一份</t>
         </is>
       </c>
       <c r="C68" s="6" t="inlineStr">
         <is>
-          <t>等 R-26</t>
+          <t>等 P1-12</t>
         </is>
       </c>
       <c r="D68" s="11" t="n"/>
@@ -2478,20 +2486,20 @@
       <c r="H68" s="11" t="n"/>
       <c r="I68" s="12" t="n"/>
     </row>
-    <row r="69" ht="18" customHeight="1">
+    <row r="69" ht="32" customHeight="1">
       <c r="A69" s="13" t="inlineStr">
         <is>
-          <t>P0-14</t>
+          <t>R-27</t>
         </is>
       </c>
       <c r="B69" s="6" t="inlineStr">
         <is>
-          <t>韌體簽章、Secure Boot 與 Flash 加密</t>
+          <t>App 內登入：驗證碼、原生社交登入、刪除帳號</t>
         </is>
       </c>
       <c r="C69" s="6" t="inlineStr">
         <is>
-          <t>等 R-01</t>
+          <t>等 R-26</t>
         </is>
       </c>
       <c r="D69" s="11" t="n"/>
@@ -2504,17 +2512,17 @@
     <row r="70" ht="18" customHeight="1">
       <c r="A70" s="13" t="inlineStr">
         <is>
-          <t>P1-06</t>
+          <t>P0-14</t>
         </is>
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>處理 GPL-3.0 依賴（arduino-audio-tools）</t>
+          <t>韌體簽章、Secure Boot 與 Flash 加密</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr">
         <is>
-          <t>等 Q3</t>
+          <t>等 R-01</t>
         </is>
       </c>
       <c r="D70" s="11" t="n"/>
@@ -2527,12 +2535,12 @@
     <row r="71" ht="18" customHeight="1">
       <c r="A71" s="13" t="inlineStr">
         <is>
-          <t>P1-07</t>
+          <t>P1-06</t>
         </is>
       </c>
       <c r="B71" s="6" t="inlineStr">
         <is>
-          <t>LGPL 合規與第三方授權聲明</t>
+          <t>處理 GPL-3.0 依賴（arduino-audio-tools）</t>
         </is>
       </c>
       <c r="C71" s="6" t="inlineStr">
@@ -2550,17 +2558,17 @@
     <row r="72" ht="18" customHeight="1">
       <c r="A72" s="13" t="inlineStr">
         <is>
-          <t>P1-08</t>
+          <t>P1-07</t>
         </is>
       </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>硬件認證</t>
+          <t>LGPL 合規與第三方授權聲明</t>
         </is>
       </c>
       <c r="C72" s="6" t="inlineStr">
         <is>
-          <t>等 R-01、R-05</t>
+          <t>等 Q3</t>
         </is>
       </c>
       <c r="D72" s="11" t="n"/>
@@ -2573,17 +2581,17 @@
     <row r="73" ht="18" customHeight="1">
       <c r="A73" s="13" t="inlineStr">
         <is>
-          <t>P1-14</t>
+          <t>P1-08</t>
         </is>
       </c>
       <c r="B73" s="6" t="inlineStr">
         <is>
-          <t>Admin 內容安全頁：審核事件只按類別統計</t>
+          <t>硬件認證</t>
         </is>
       </c>
       <c r="C73" s="6" t="inlineStr">
         <is>
-          <t>等 P1-01、P2-13</t>
+          <t>等 R-01、R-05</t>
         </is>
       </c>
       <c r="D73" s="11" t="n"/>
@@ -2593,20 +2601,20 @@
       <c r="H73" s="11" t="n"/>
       <c r="I73" s="12" t="n"/>
     </row>
-    <row r="74" ht="32" customHeight="1">
+    <row r="74" ht="18" customHeight="1">
       <c r="A74" s="13" t="inlineStr">
         <is>
-          <t>P2-15</t>
+          <t>P1-14</t>
         </is>
       </c>
       <c r="B74" s="6" t="inlineStr">
         <is>
-          <t>Admin 總覽頁：在線、用量、成本與待處理事項</t>
+          <t>Admin 內容安全頁：審核事件只按類別統計</t>
         </is>
       </c>
       <c r="C74" s="6" t="inlineStr">
         <is>
-          <t>等 P2-09</t>
+          <t>等 P1-01、P2-13</t>
         </is>
       </c>
       <c r="D74" s="11" t="n"/>
@@ -2616,20 +2624,20 @@
       <c r="H74" s="11" t="n"/>
       <c r="I74" s="12" t="n"/>
     </row>
-    <row r="75" ht="18" customHeight="1">
+    <row r="75" ht="32" customHeight="1">
       <c r="A75" s="13" t="inlineStr">
         <is>
-          <t>R-07</t>
+          <t>P2-15</t>
         </is>
       </c>
       <c r="B75" s="6" t="inlineStr">
         <is>
-          <t>20 個家庭封閉內測</t>
+          <t>Admin 總覽頁：在線、用量、成本與待處理事項</t>
         </is>
       </c>
       <c r="C75" s="6" t="inlineStr">
         <is>
-          <t>等 R-13</t>
+          <t>等 P2-09</t>
         </is>
       </c>
       <c r="D75" s="11" t="n"/>
@@ -2642,17 +2650,17 @@
     <row r="76" ht="18" customHeight="1">
       <c r="A76" s="13" t="inlineStr">
         <is>
-          <t>R-08</t>
+          <t>R-07</t>
         </is>
       </c>
       <c r="B76" s="6" t="inlineStr">
         <is>
-          <t>第 8 週關卡決策</t>
+          <t>20 個家庭封閉內測</t>
         </is>
       </c>
       <c r="C76" s="6" t="inlineStr">
         <is>
-          <t>等 R-07、P2-09、P1-08</t>
+          <t>等 R-13</t>
         </is>
       </c>
       <c r="D76" s="11" t="n"/>
@@ -2665,17 +2673,17 @@
     <row r="77" ht="18" customHeight="1">
       <c r="A77" s="13" t="inlineStr">
         <is>
-          <t>R-14</t>
+          <t>R-08</t>
         </is>
       </c>
       <c r="B77" s="6" t="inlineStr">
         <is>
-          <t>離線兒歌與故事</t>
+          <t>第 8 週關卡決策</t>
         </is>
       </c>
       <c r="C77" s="6" t="inlineStr">
         <is>
-          <t>等 R-01</t>
+          <t>等 R-07、P2-09、P1-08</t>
         </is>
       </c>
       <c r="D77" s="11" t="n"/>
@@ -2688,17 +2696,17 @@
     <row r="78" ht="18" customHeight="1">
       <c r="A78" s="13" t="inlineStr">
         <is>
-          <t>R-24</t>
+          <t>R-14</t>
         </is>
       </c>
       <c r="B78" s="6" t="inlineStr">
         <is>
-          <t>設備只能用自己品牌的角色</t>
+          <t>離線兒歌與故事</t>
         </is>
       </c>
       <c r="C78" s="6" t="inlineStr">
         <is>
-          <t>等 R-34</t>
+          <t>等 R-01</t>
         </is>
       </c>
       <c r="D78" s="11" t="n"/>
@@ -2711,17 +2719,17 @@
     <row r="79" ht="18" customHeight="1">
       <c r="A79" s="13" t="inlineStr">
         <is>
-          <t>R-28</t>
+          <t>R-24</t>
         </is>
       </c>
       <c r="B79" s="6" t="inlineStr">
         <is>
-          <t>三個 App 的殼：品牌版本與測試版</t>
+          <t>設備只能用自己品牌的角色</t>
         </is>
       </c>
       <c r="C79" s="6" t="inlineStr">
         <is>
-          <t>等 R-25、R-26</t>
+          <t>等 R-34</t>
         </is>
       </c>
       <c r="D79" s="11" t="n"/>
@@ -2734,17 +2742,17 @@
     <row r="80" ht="18" customHeight="1">
       <c r="A80" s="13" t="inlineStr">
         <is>
-          <t>R-30</t>
+          <t>R-28</t>
         </is>
       </c>
       <c r="B80" s="6" t="inlineStr">
         <is>
-          <t>快活 App（品牌 A）頁面</t>
+          <t>三個 App 的殼：品牌版本與測試版</t>
         </is>
       </c>
       <c r="C80" s="6" t="inlineStr">
         <is>
-          <t>等 R-25、R-34、Q12</t>
+          <t>等 R-25、R-26</t>
         </is>
       </c>
       <c r="D80" s="11" t="n"/>
@@ -2757,17 +2765,17 @@
     <row r="81" ht="18" customHeight="1">
       <c r="A81" s="13" t="inlineStr">
         <is>
-          <t>R-31</t>
+          <t>R-30</t>
         </is>
       </c>
       <c r="B81" s="6" t="inlineStr">
         <is>
-          <t>政協青年聯會版 App（品牌 B）頁面</t>
+          <t>快活 App（品牌 A）頁面</t>
         </is>
       </c>
       <c r="C81" s="6" t="inlineStr">
         <is>
-          <t>等 R-25、R-34、Q13</t>
+          <t>等 R-25、R-34、Q12</t>
         </is>
       </c>
       <c r="D81" s="11" t="n"/>
@@ -2780,17 +2788,17 @@
     <row r="82" ht="18" customHeight="1">
       <c r="A82" s="13" t="inlineStr">
         <is>
-          <t>R-35</t>
+          <t>R-31</t>
         </is>
       </c>
       <c r="B82" s="6" t="inlineStr">
         <is>
-          <t>韌體按品牌連線：伺服器網址在出廠時寫入</t>
+          <t>政協青年聯會版 App（品牌 B）頁面</t>
         </is>
       </c>
       <c r="C82" s="6" t="inlineStr">
         <is>
-          <t>等 R-34</t>
+          <t>等 R-25、R-34、Q13</t>
         </is>
       </c>
       <c r="D82" s="11" t="n"/>
@@ -2800,20 +2808,20 @@
       <c r="H82" s="11" t="n"/>
       <c r="I82" s="12" t="n"/>
     </row>
-    <row r="83" ht="32" customHeight="1">
+    <row r="83" ht="18" customHeight="1">
       <c r="A83" s="13" t="inlineStr">
         <is>
-          <t>R-38</t>
+          <t>R-35</t>
         </is>
       </c>
       <c r="B83" s="6" t="inlineStr">
         <is>
-          <t>公仔出廠鎖死所屬 IP，綁定時顯示該 IP 頭像</t>
+          <t>韌體按品牌連線：伺服器網址在出廠時寫入</t>
         </is>
       </c>
       <c r="C83" s="6" t="inlineStr">
         <is>
-          <t>等 P0-11</t>
+          <t>等 R-34</t>
         </is>
       </c>
       <c r="D83" s="11" t="n"/>
@@ -2826,17 +2834,17 @@
     <row r="84" ht="32" customHeight="1">
       <c r="A84" s="13" t="inlineStr">
         <is>
-          <t>R-39</t>
+          <t>R-38</t>
         </is>
       </c>
       <c r="B84" s="6" t="inlineStr">
         <is>
-          <t>Admin 出廠登記頁：匯入 MAC 清單、指定公仔、查看自檢結果</t>
+          <t>公仔出廠鎖死所屬 IP，綁定時顯示該 IP 頭像</t>
         </is>
       </c>
       <c r="C84" s="6" t="inlineStr">
         <is>
-          <t>等 R-38、P1-10</t>
+          <t>等 P0-11</t>
         </is>
       </c>
       <c r="D84" s="11" t="n"/>
@@ -2846,20 +2854,20 @@
       <c r="H84" s="11" t="n"/>
       <c r="I84" s="12" t="n"/>
     </row>
-    <row r="85" ht="18" customHeight="1">
+    <row r="85" ht="32" customHeight="1">
       <c r="A85" s="13" t="inlineStr">
         <is>
-          <t>R-09</t>
+          <t>R-39</t>
         </is>
       </c>
       <c r="B85" s="6" t="inlineStr">
         <is>
-          <t>量產外殼（真空複模）</t>
+          <t>Admin 出廠登記頁：匯入 MAC 清單、指定公仔、查看自檢結果</t>
         </is>
       </c>
       <c r="C85" s="6" t="inlineStr">
         <is>
-          <t>等 R-08、R-05、Q11</t>
+          <t>等 R-38、P1-10</t>
         </is>
       </c>
       <c r="D85" s="11" t="n"/>
@@ -2872,17 +2880,17 @@
     <row r="86" ht="18" customHeight="1">
       <c r="A86" s="13" t="inlineStr">
         <is>
-          <t>R-10</t>
+          <t>R-09</t>
         </is>
       </c>
       <c r="B86" s="6" t="inlineStr">
         <is>
-          <t>出廠流程</t>
+          <t>量產外殼（真空複模）</t>
         </is>
       </c>
       <c r="C86" s="6" t="inlineStr">
         <is>
-          <t>等 P0-14、R-01、P2-12、R-34、R-35、R-38、R-39</t>
+          <t>等 R-08、R-05、Q11</t>
         </is>
       </c>
       <c r="D86" s="11" t="n"/>
@@ -2895,17 +2903,17 @@
     <row r="87" ht="18" customHeight="1">
       <c r="A87" s="13" t="inlineStr">
         <is>
-          <t>R-11</t>
+          <t>R-10</t>
         </is>
       </c>
       <c r="B87" s="6" t="inlineStr">
         <is>
-          <t>售後：客服、保修與換機</t>
+          <t>出廠流程</t>
         </is>
       </c>
       <c r="C87" s="6" t="inlineStr">
         <is>
-          <t>等 R-40</t>
+          <t>等 P0-14、R-01、P2-12、R-34、R-35、R-38、R-39</t>
         </is>
       </c>
       <c r="D87" s="11" t="n"/>
@@ -2918,17 +2926,17 @@
     <row r="88" ht="18" customHeight="1">
       <c r="A88" s="13" t="inlineStr">
         <is>
-          <t>R-15</t>
+          <t>R-11</t>
         </is>
       </c>
       <c r="B88" s="6" t="inlineStr">
         <is>
-          <t>農曆新年前交付（生產 1/15、送達 1/29）</t>
+          <t>售後：客服、保修與換機</t>
         </is>
       </c>
       <c r="C88" s="6" t="inlineStr">
         <is>
-          <t>等 R-09、R-10</t>
+          <t>等 R-40</t>
         </is>
       </c>
       <c r="D88" s="11" t="n"/>
@@ -2941,17 +2949,17 @@
     <row r="89" ht="18" customHeight="1">
       <c r="A89" s="13" t="inlineStr">
         <is>
-          <t>R-33</t>
+          <t>R-15</t>
         </is>
       </c>
       <c r="B89" s="6" t="inlineStr">
         <is>
-          <t>三個 App 送審並通過</t>
+          <t>農曆新年前交付（生產 1/15、送達 1/29）</t>
         </is>
       </c>
       <c r="C89" s="6" t="inlineStr">
         <is>
-          <t>等 R-27、R-21、R-28、R-29、R-30、R-31、R-32</t>
+          <t>等 R-09、R-10</t>
         </is>
       </c>
       <c r="D89" s="11" t="n"/>
@@ -2961,20 +2969,20 @@
       <c r="H89" s="11" t="n"/>
       <c r="I89" s="12" t="n"/>
     </row>
-    <row r="90" ht="32" customHeight="1">
+    <row r="90" ht="18" customHeight="1">
       <c r="A90" s="13" t="inlineStr">
         <is>
-          <t>R-40</t>
+          <t>R-33</t>
         </is>
       </c>
       <c r="B90" s="6" t="inlineStr">
         <is>
-          <t>Admin 客服查詢頁：查帳號、名下設備與最近事件</t>
+          <t>三個 App 送審並通過</t>
         </is>
       </c>
       <c r="C90" s="6" t="inlineStr">
         <is>
-          <t>等 P1-10、P1-12</t>
+          <t>等 R-27、R-21、R-28、R-29、R-30、R-31、R-32</t>
         </is>
       </c>
       <c r="D90" s="11" t="n"/>
@@ -2984,50 +2992,50 @@
       <c r="H90" s="11" t="n"/>
       <c r="I90" s="12" t="n"/>
     </row>
-    <row r="92">
-      <c r="A92" s="10" t="inlineStr">
+    <row r="91" ht="32" customHeight="1">
+      <c r="A91" s="13" t="inlineStr">
+        <is>
+          <t>R-40</t>
+        </is>
+      </c>
+      <c r="B91" s="6" t="inlineStr">
+        <is>
+          <t>Admin 客服查詢頁：查帳號、名下設備與最近事件</t>
+        </is>
+      </c>
+      <c r="C91" s="6" t="inlineStr">
+        <is>
+          <t>等 P1-10、P1-12</t>
+        </is>
+      </c>
+      <c r="D91" s="11" t="n"/>
+      <c r="E91" s="11" t="n"/>
+      <c r="F91" s="11" t="n"/>
+      <c r="G91" s="11" t="n"/>
+      <c r="H91" s="11" t="n"/>
+      <c r="I91" s="12" t="n"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="10" t="inlineStr">
         <is>
           <t>❓ 待確認問題</t>
         </is>
       </c>
     </row>
-    <row r="93">
-      <c r="A93" s="4" t="inlineStr">
+    <row r="94">
+      <c r="A94" s="4" t="inlineStr">
         <is>
           <t>編號</t>
         </is>
       </c>
-      <c r="B93" s="4" t="inlineStr">
+      <c r="B94" s="4" t="inlineStr">
         <is>
           <t>問題</t>
         </is>
       </c>
-      <c r="C93" s="4" t="inlineStr">
+      <c r="C94" s="4" t="inlineStr">
         <is>
           <t>影響的任務 / 為什麼重要</t>
-        </is>
-      </c>
-      <c r="D93" s="11" t="n"/>
-      <c r="E93" s="11" t="n"/>
-      <c r="F93" s="11" t="n"/>
-      <c r="G93" s="11" t="n"/>
-      <c r="H93" s="11" t="n"/>
-      <c r="I93" s="12" t="n"/>
-    </row>
-    <row r="94" ht="18" customHeight="1">
-      <c r="A94" s="13" t="inlineStr">
-        <is>
-          <t>Q3</t>
-        </is>
-      </c>
-      <c r="B94" s="6" t="inlineStr">
-        <is>
-          <t>韌體打算閉源商業銷售嗎？</t>
-        </is>
-      </c>
-      <c r="C94" s="6" t="inlineStr">
-        <is>
-          <t>P1-06, P1-07：決定 GPL／LGPL 依賴要開源還是替換。</t>
         </is>
       </c>
       <c r="D94" s="11" t="n"/>
@@ -3037,20 +3045,20 @@
       <c r="H94" s="11" t="n"/>
       <c r="I94" s="12" t="n"/>
     </row>
-    <row r="95" ht="32" customHeight="1">
+    <row r="95" ht="18" customHeight="1">
       <c r="A95" s="13" t="inlineStr">
         <is>
-          <t>Q11</t>
+          <t>Q3</t>
         </is>
       </c>
       <c r="B95" s="6" t="inlineStr">
         <is>
-          <t>馬會快活的賽馬日版和新春版各多少隻（共 2,500）？</t>
+          <t>韌體打算閉源商業銷售嗎？</t>
         </is>
       </c>
       <c r="C95" s="6" t="inlineStr">
         <is>
-          <t>R-09, R-15：兩款的服裝和配件要分開訂料；11/20 前不知道，PP 樣和大貨單（11/27）會被拖慢。由馬會決定。</t>
+          <t>P1-06, P1-07：決定 GPL／LGPL 依賴要開源還是替換。</t>
         </is>
       </c>
       <c r="D95" s="11" t="n"/>
@@ -3060,20 +3068,20 @@
       <c r="H95" s="11" t="n"/>
       <c r="I95" s="12" t="n"/>
     </row>
-    <row r="96" ht="60" customHeight="1">
+    <row r="96" ht="32" customHeight="1">
       <c r="A96" s="13" t="inlineStr">
         <is>
-          <t>Q12</t>
+          <t>Q11</t>
         </is>
       </c>
       <c r="B96" s="6" t="inlineStr">
         <is>
-          <t>快活 App 的「會員綁定」是指甚麼：用我們自己的帳號（email 驗證碼），還是接馬會的會員帳號登入（SSO）？</t>
+          <t>馬會快活的賽馬日版和新春版各多少隻（共 2,500）？</t>
         </is>
       </c>
       <c r="C96" s="6" t="inlineStr">
         <is>
-          <t>P0-11, 快活 App（未入追蹤表）：接馬會 SSO 的話，登入、帳號刪除和資料歸屬都要按馬會的介面重做，工作量和排期要另估，而且 W5（11/9–11/13）就要做快活 App 的綁定；用我們的帳號則和其他品牌共用同一套流程。由馬會決定，要盡早問。</t>
+          <t>R-09, R-15：兩款的服裝和配件要分開訂料；11/20 前不知道，PP 樣和大貨單（11/27）會被拖慢。由馬會決定。</t>
         </is>
       </c>
       <c r="D96" s="11" t="n"/>
@@ -3083,20 +3091,20 @@
       <c r="H96" s="11" t="n"/>
       <c r="I96" s="12" t="n"/>
     </row>
-    <row r="97" ht="46" customHeight="1">
+    <row r="97" ht="60" customHeight="1">
       <c r="A97" s="13" t="inlineStr">
         <is>
-          <t>Q13</t>
+          <t>Q12</t>
         </is>
       </c>
       <c r="B97" s="6" t="inlineStr">
         <is>
-          <t>政協青年聯會版的角色、語言和內容由誰提供？什麼時候交？</t>
+          <t>快活 App 的「會員綁定」是指甚麼：用我們自己的帳號（email 驗證碼），還是接馬會的會員帳號登入（SSO）？</t>
         </is>
       </c>
       <c r="C97" s="6" t="inlineStr">
         <is>
-          <t>品牌 B 的 App 頁面：品牌 B 的用戶是成人會員，但角色、說話語言、內容規則都還沒有。最遲 11/13 要拿到，才趕得及內部測試和 App 頁面（W6）。</t>
+          <t>P0-11, 快活 App（未入追蹤表）：接馬會 SSO 的話，登入、帳號刪除和資料歸屬都要按馬會的介面重做，工作量和排期要另估，而且 W5（11/9–11/13）就要做快活 App 的綁定；用我們的帳號則和其他品牌共用同一套流程。由馬會決定，要盡早問。</t>
         </is>
       </c>
       <c r="D97" s="11" t="n"/>
@@ -3106,51 +3114,73 @@
       <c r="H97" s="11" t="n"/>
       <c r="I97" s="12" t="n"/>
     </row>
-    <row r="99">
-      <c r="A99" s="10" t="inlineStr">
+    <row r="98" ht="46" customHeight="1">
+      <c r="A98" s="13" t="inlineStr">
+        <is>
+          <t>Q13</t>
+        </is>
+      </c>
+      <c r="B98" s="6" t="inlineStr">
+        <is>
+          <t>政協青年聯會版的角色、語言和內容由誰提供？什麼時候交？</t>
+        </is>
+      </c>
+      <c r="C98" s="6" t="inlineStr">
+        <is>
+          <t>品牌 B 的 App 頁面：品牌 B 的用戶是成人會員，但角色、說話語言、內容規則都還沒有。最遲 11/13 要拿到，才趕得及內部測試和 App 頁面（W6）。</t>
+        </is>
+      </c>
+      <c r="D98" s="11" t="n"/>
+      <c r="E98" s="11" t="n"/>
+      <c r="F98" s="11" t="n"/>
+      <c r="G98" s="11" t="n"/>
+      <c r="H98" s="11" t="n"/>
+      <c r="I98" s="12" t="n"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="10" t="inlineStr">
         <is>
           <t>說明</t>
         </is>
       </c>
     </row>
-    <row r="100" ht="32" customHeight="1">
-      <c r="A100" s="14" t="inlineStr">
+    <row r="101" ht="32" customHeight="1">
+      <c r="A101" s="14" t="inlineStr">
         <is>
           <t>・狀態：未開始 → 進行中 → 已完成。只有測試真的跑過而且通過才算已完成；阻塞要在備註寫原因；不再需要的任務標不適用，不要刪。</t>
-        </is>
-      </c>
-    </row>
-    <row r="101" ht="18" customHeight="1">
-      <c r="A101" s="14" t="inlineStr">
-        <is>
-          <t>・測試結果：未測試 / 通過 / 失敗 / 部分通過。測試證據寫跑了什麼、看到什麼，完整歷史在「更新記錄」。</t>
         </is>
       </c>
     </row>
     <row r="102" ht="18" customHeight="1">
       <c r="A102" s="14" t="inlineStr">
         <is>
-          <t>・「接下來」按階段排序，同一階段內再按優先級；依賴還沒滿足的任務不會出現在「接下來」。</t>
+          <t>・測試結果：未測試 / 通過 / 失敗 / 部分通過。測試證據寫跑了什麼、看到什麼，完整歷史在「更新記錄」。</t>
         </is>
       </c>
     </row>
     <row r="103" ht="18" customHeight="1">
       <c r="A103" s="14" t="inlineStr">
         <is>
+          <t>・「接下來」按階段排序，同一階段內再按優先級；依賴還沒滿足的任務不會出現在「接下來」。</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" ht="18" customHeight="1">
+      <c r="A104" s="14" t="inlineStr">
+        <is>
           <t>・可以手動改：「任務清單」的狀態、測試結果、測試證據、Commit、備註，以及「待確認問題」的回答。其餘欄位和本頁由腳本維護。</t>
         </is>
       </c>
     </row>
-    <row r="104" ht="32" customHeight="1">
-      <c r="A104" s="14" t="inlineStr">
+    <row r="105" ht="32" customHeight="1">
+      <c r="A105" s="14" t="inlineStr">
         <is>
           <t>・建議用法：在 Claude Code 對 Claude 說「P0-02 做完了」或輸入 /prod-readiness。Claude 會先跑測試再更新，並寫進「更新記錄」。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="85">
-    <mergeCell ref="A99:I99"/>
+  <mergeCells count="86">
     <mergeCell ref="C82:I82"/>
     <mergeCell ref="E52:I52"/>
     <mergeCell ref="E39:I39"/>
@@ -3172,9 +3202,11 @@
     <mergeCell ref="C60:I60"/>
     <mergeCell ref="C71:I71"/>
     <mergeCell ref="E50:I50"/>
+    <mergeCell ref="E42:I42"/>
+    <mergeCell ref="C91:I91"/>
+    <mergeCell ref="A105:I105"/>
     <mergeCell ref="C57:I57"/>
     <mergeCell ref="C66:I66"/>
-    <mergeCell ref="E44:I44"/>
     <mergeCell ref="E20:I20"/>
     <mergeCell ref="E28:I28"/>
     <mergeCell ref="C77:I77"/>
@@ -3183,12 +3215,13 @@
     <mergeCell ref="A100:I100"/>
     <mergeCell ref="C58:I58"/>
     <mergeCell ref="E30:I30"/>
+    <mergeCell ref="E22:I22"/>
+    <mergeCell ref="A93:I93"/>
     <mergeCell ref="E46:I46"/>
     <mergeCell ref="A102:I102"/>
     <mergeCell ref="C85:I85"/>
     <mergeCell ref="C94:I94"/>
     <mergeCell ref="C65:I65"/>
-    <mergeCell ref="A92:I92"/>
     <mergeCell ref="C75:I75"/>
     <mergeCell ref="C84:I84"/>
     <mergeCell ref="C80:I80"/>
@@ -3202,13 +3235,12 @@
     <mergeCell ref="E24:I24"/>
     <mergeCell ref="E33:I33"/>
     <mergeCell ref="A3:I3"/>
+    <mergeCell ref="A55:I55"/>
     <mergeCell ref="A104:I104"/>
     <mergeCell ref="E35:I35"/>
-    <mergeCell ref="A43:I43"/>
     <mergeCell ref="C74:I74"/>
     <mergeCell ref="C88:I88"/>
     <mergeCell ref="E45:I45"/>
-    <mergeCell ref="C55:I55"/>
     <mergeCell ref="E37:I37"/>
     <mergeCell ref="E21:I21"/>
     <mergeCell ref="E23:I23"/>
@@ -3220,21 +3252,21 @@
     <mergeCell ref="C78:I78"/>
     <mergeCell ref="C87:I87"/>
     <mergeCell ref="C62:I62"/>
+    <mergeCell ref="C98:I98"/>
     <mergeCell ref="C89:I89"/>
     <mergeCell ref="E34:I34"/>
     <mergeCell ref="C64:I64"/>
     <mergeCell ref="C79:I79"/>
     <mergeCell ref="C73:I73"/>
+    <mergeCell ref="A44:I44"/>
     <mergeCell ref="E49:I49"/>
     <mergeCell ref="E27:I27"/>
     <mergeCell ref="E36:I36"/>
     <mergeCell ref="C63:I63"/>
-    <mergeCell ref="C93:I93"/>
     <mergeCell ref="C56:I56"/>
     <mergeCell ref="C90:I90"/>
-    <mergeCell ref="E22:I22"/>
+    <mergeCell ref="E53:I53"/>
     <mergeCell ref="C76:I76"/>
-    <mergeCell ref="A54:I54"/>
   </mergeCells>
   <conditionalFormatting sqref="I6:I10">
     <cfRule type="dataBar" priority="1">
@@ -10369,7 +10401,7 @@
       </c>
       <c r="F97" s="13" t="inlineStr">
         <is>
-          <t>未開始</t>
+          <t>進行中</t>
         </is>
       </c>
       <c r="G97" s="13" t="inlineStr">
@@ -11053,7 +11085,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I315"/>
+  <dimension ref="A1:I317"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -22020,8 +22052,74 @@
         </is>
       </c>
     </row>
+    <row r="316" ht="46" customHeight="1">
+      <c r="A316" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-15 10:29</t>
+        </is>
+      </c>
+      <c r="B316" s="13" t="inlineStr">
+        <is>
+          <t>P2-25</t>
+        </is>
+      </c>
+      <c r="C316" s="6" t="inlineStr">
+        <is>
+          <t>C3 斷線後自救：TLS 握手超時縮短、連續失敗重設 Wi-Fi 或重開、修重試漏記憶體</t>
+        </is>
+      </c>
+      <c r="D316" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E316" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="F316" s="13" t="n"/>
+      <c r="G316" s="6" t="n"/>
+      <c r="H316" s="13" t="n"/>
+      <c r="I316" s="6" t="inlineStr">
+        <is>
+          <t>修改了依賴→</t>
+        </is>
+      </c>
+    </row>
+    <row r="317" ht="32" customHeight="1">
+      <c r="A317" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-15 10:29</t>
+        </is>
+      </c>
+      <c r="B317" s="13" t="inlineStr">
+        <is>
+          <t>P2-24</t>
+        </is>
+      </c>
+      <c r="C317" s="6" t="inlineStr">
+        <is>
+          <t>麥克風上行改用 IMA ADPCM（減少 4 倍頻寬）</t>
+        </is>
+      </c>
+      <c r="D317" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E317" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F317" s="13" t="n"/>
+      <c r="G317" s="6" t="n"/>
+      <c r="H317" s="13" t="n"/>
+      <c r="I317" s="6" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I315"/>
+  <autoFilter ref="A1:I317"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Note on P2-22 the boot-time pick of a saved Wi-Fi that cannot reach the server.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/production-readiness.xlsx
+++ b/docs/production-readiness.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'任務清單'!$A$1:$P$98</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'待確認問題'!$A$1:$G$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$317</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$319</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -9073,7 +9073,8 @@
 [2026-10-13] 2026-10-13 應 Jacky 要求從 W4 提前開始。韌體：上限 8 個、NVS apOk%d 記錄連過、經 /ws/esp32 收 status/add/delete/scan、不刪不改目前 Wi-Fi、Wi-Fi 指令不印串口、修 delWifi 計數 bug。伺服器：device_wifi.py＋/internal/device_wifi（含 peek），密碼只轉送不留存。網頁：我 &gt; 裝置 &gt; Network &gt; Wi-Fi（Figma C4），deviceWifiAction 檢查擁有者。剩真機測試 ①②（需 62:70 刷 -localall＋兩個真實網絡）與 OTA。
 [2026-10-15] 2026-10-15 用戶決定：加「改用這個 Wi-Fi」（⑦），④ 改為新增不自動切換、可由家長手動切換。起因：62:70 實測加了 iPhone 熱點也無法讓玩具改用。另：離線一律顯示「睡著了」會誤導（63:64 已 6 天未上線仍叫人按按鈕），待改為按上次上線時間分開提示。
 [2026-10-15] 測試中修了原有 bug（a4 之後第二個 commit）：驅動在沒連上的網絡斷開時不發事件，WiFi.status() 留著上次的『找不到』，新嘗試一開始就被當失敗；1.7.4 切換失敗後連不回 Guest 並掉進 SoftAP，tryConnect() 也同樣。joinFor() 改為 6 秒後才相信失敗，tryConnect() 共用。雲端韌體同樣有這 bug。另：開機時 tryConnect() 挑最強的網絡但不檢查能否到伺服器，62:70 開機連上到不了 Mac 的熱點後一直卡著（見 P2-22 ④ 或另開任務）。分支 r-37-wifi-switch 未推送。
-[2026-10-15] 更正上一條備註：stale『找不到』的修正是 22d7674（切換功能本身是 3c180cd）。</t>
+[2026-10-15] 更正上一條備註：stale『找不到』的修正是 22d7674（切換功能本身是 3c180cd）。
+[2026-10-15] 2026-10-15：⑦ 的成功切換在本機測不到（熱點到不了 Mac 上的伺服器），留到部署上 UAT 或雲端後用 iPhone 熱點測一次。</t>
         </is>
       </c>
     </row>
@@ -10226,7 +10227,7 @@
         </is>
       </c>
     </row>
-    <row r="95" ht="298" customHeight="1">
+    <row r="95" ht="409" customHeight="1">
       <c r="A95" s="13" t="inlineStr">
         <is>
           <t>P2-22</t>
@@ -10301,7 +10302,8 @@
         <is>
           <t>[2026-10-14] 新增
 [2026-10-14] 2026-10-14 用戶要求：日後改 FastAPI 網址，板子仍要能 OTA 並連上。① 後端改動可隨時部署；②–⑦ 的韌體部分必須在 11/27 交 Spotpear 的出廠映像之前完成，出廠後才加的話，已出貨的板子靠 OTA 也能拿到，但前提是當時的網址還連得上。
-[2026-10-15] 未完成：韌體部分（①② 使用 voice_url 並在 NVS 記上次成功的值、③ 候選 backend_url、④⑤ 連續 10 次開機連不上就切槽、⑦ 允許的網域後綴）未開始，要用 62:70 實機測；runbook（③ 舊網址保留多久、⑥ 證書鏈檢查）未寫。部署：.env.production 加 DEVICE_VOICE_URL、DEVICE_BACKEND_URL；舊韌體會忽略這兩個欄位，可以先上後端。分支未合併 dev、未推送</t>
+[2026-10-15] 未完成：韌體部分（①② 使用 voice_url 並在 NVS 記上次成功的值、③ 候選 backend_url、④⑤ 連續 10 次開機連不上就切槽、⑦ 允許的網域後綴）未開始，要用 62:70 實機測；runbook（③ 舊網址保留多久、⑥ 證書鏈檢查）未寫。部署：.env.production 加 DEVICE_VOICE_URL、DEVICE_BACKEND_URL；舊韌體會忽略這兩個欄位，可以先上後端。分支未合併 dev、未推送
+[2026-10-15] 2026-10-15（用戶決定只記備註、不另開任務）：開機時 tryConnect() 挑訊號最強的已存網絡，但不檢查能否到伺服器。若該網絡本身上不了網（熱點關了流動數據、要網頁登入的酒店 Wi-Fi、寬頻斷了），玩具每次開機都會卡在那裡，即使另一個已存網絡可用。做 ④ 時一併考慮：連上後取不到 token 就改試下一個已存網絡。62:70 連著到不了本機伺服器的 iPhone 熱點時出現過，但那是本機測試環境造成的，雲端不會。</t>
         </is>
       </c>
     </row>
@@ -11085,7 +11087,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I317"/>
+  <dimension ref="A1:I319"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -22118,8 +22120,78 @@
       <c r="H317" s="13" t="n"/>
       <c r="I317" s="6" t="n"/>
     </row>
+    <row r="318" ht="158" customHeight="1">
+      <c r="A318" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-15 10:29</t>
+        </is>
+      </c>
+      <c r="B318" s="13" t="inlineStr">
+        <is>
+          <t>P2-22</t>
+        </is>
+      </c>
+      <c r="C318" s="6" t="inlineStr">
+        <is>
+          <t>改服務器網址也不失聯：語音網址由後端下發、後端網址可遷移、已確認韌體長期連不上時自救</t>
+        </is>
+      </c>
+      <c r="D318" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="E318" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F318" s="13" t="n"/>
+      <c r="G318" s="6" t="n"/>
+      <c r="H318" s="13" t="n"/>
+      <c r="I318" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-15（用戶決定只記備註、不另開任務）：開機時 tryConnect() 挑訊號最強的已存網絡，但不檢查能否到伺服器。若該網絡本身上不了網（熱點關了流動數據、要網頁登入的酒店 Wi-Fi、寬頻斷了），玩具每次開機都會卡在那裡，即使另一個已存網絡可用。做 ④ 時一併考慮：連上後取不到 token 就改試下一個已存網絡。62:70 連著到不了本機伺服器的 iPhone 熱點時出現過，但那是本機測試環境造成的，雲端不會。</t>
+        </is>
+      </c>
+    </row>
+    <row r="319" ht="60" customHeight="1">
+      <c r="A319" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-15 10:29</t>
+        </is>
+      </c>
+      <c r="B319" s="13" t="inlineStr">
+        <is>
+          <t>R-37</t>
+        </is>
+      </c>
+      <c r="C319" s="6" t="inlineStr">
+        <is>
+          <t>網頁設定玩具的 Wi-Fi：查看、新增、刪除</t>
+        </is>
+      </c>
+      <c r="D319" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="E319" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F319" s="13" t="n"/>
+      <c r="G319" s="6" t="n"/>
+      <c r="H319" s="13" t="n"/>
+      <c r="I319" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-15：⑦ 的成功切換在本機測不到（熱點到不了 Mac 上的伺服器），留到部署上 UAT 或雲端後用 iPhone 熱點測一次。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I317"/>
+  <autoFilter ref="A1:I319"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Track P2-24 and R-37 hardware results on 62:70.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/production-readiness.xlsx
+++ b/docs/production-readiness.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'任務清單'!$A$1:$P$98</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'待確認問題'!$A$1:$G$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$319</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$320</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -665,7 +665,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>最後更新：2026-10-15 10:29　·　本頁由 tracker.py 自動生成，請勿手動編輯</t>
+          <t>最後更新：2026-10-15 10:42　·　本頁由 tracker.py 自動生成，請勿手動編輯</t>
         </is>
       </c>
     </row>
@@ -1518,7 +1518,7 @@
       <c r="H30" s="11" t="n"/>
       <c r="I30" s="12" t="n"/>
     </row>
-    <row r="31" ht="102" customHeight="1">
+    <row r="31" ht="270" customHeight="1">
       <c r="A31" s="13" t="inlineStr">
         <is>
           <t>P2-24</t>
@@ -1541,7 +1541,8 @@
       </c>
       <c r="E31" s="6" t="inlineStr">
         <is>
-          <t>① 新韌體上行用 IMA ADPCM（64 kbps），每幀帶解碼狀態（預測值＋步長索引），掉幀或重連後下一幀即可正確解碼 ② 連線時以 header 聲明編碼；伺服器據此解碼成 16kHz PCM 再交給 STT；沒有聲明的舊韌體照舊當 PCM ③ 韌體編碼與伺服器解碼位元一致（同一算法）④ 編碼 CPU &lt; 2%、不增加延遲 ⑤ 語音辨識品質與 PCM 相當</t>
+          <t>上次測試：部分通過 — ① pytest test_mic_adpcm 10 項：Mac 上編譯 firmware MicAdpcm.cpp，與 audioop 逐 byte 一致（改壞一個表值即失敗）；分塊解碼 = 連續流解碼；掉一塊只損失該塊；人聲段 SNR &gt; 20dB；全套 275 passed ② 伺服器按 X-Mic-Codec 解碼，無 header 照舊 PCM（10:37 1.7.5 → mic=pcm，10:40 1.7.6 → mic=adpcm）③ 62:70 Guest（2026-10-15）：ADPCM 3 輪 Azure zh-HK 辨識通順完整（如『但係點解依家望到外邊係陰天嘅？』），STT 431–526ms，對照同場 PCM 560ms；上行 27,650B/3,370ms 與 16,625B/2,026ms = 8.2 B/ms（PCM 32），發送最長 3ms、最低 heap 55KB
+① 新韌體上行用 IMA ADPCM（64 kbps），每幀帶解碼狀態（預測值＋步長索引），掉幀或重連後下一幀即可正確解碼 ② 連線時以 header 聲明編碼；伺服器據此解碼成 16kHz PCM 再交給 STT；沒有聲明的舊韌體照舊當 PCM ③ 韌體編碼與伺服器解碼位元一致（同一算法）④ 編碼 CPU &lt; 2%、不增加延遲 ⑤ 語音辨識品質與 PCM 相當</t>
         </is>
       </c>
       <c r="F31" s="11" t="n"/>
@@ -10375,7 +10376,7 @@
         </is>
       </c>
     </row>
-    <row r="97" ht="144" customHeight="1">
+    <row r="97" ht="186" customHeight="1">
       <c r="A97" s="13" t="inlineStr">
         <is>
           <t>P2-24</t>
@@ -10408,7 +10409,7 @@
       </c>
       <c r="G97" s="13" t="inlineStr">
         <is>
-          <t>未測試</t>
+          <t>部分通過</t>
         </is>
       </c>
       <c r="I97" s="6" t="inlineStr">
@@ -10432,9 +10433,20 @@
         </is>
       </c>
       <c r="M97" s="13" t="n"/>
+      <c r="N97" s="6" t="inlineStr">
+        <is>
+          <t>① pytest test_mic_adpcm 10 項：Mac 上編譯 firmware MicAdpcm.cpp，與 audioop 逐 byte 一致（改壞一個表值即失敗）；分塊解碼 = 連續流解碼；掉一塊只損失該塊；人聲段 SNR &gt; 20dB；全套 275 passed ② 伺服器按 X-Mic-Codec 解碼，無 header 照舊 PCM（10:37 1.7.5 → mic=pcm，10:40 1.7.6 → mic=adpcm）③ 62:70 Guest（2026-10-15）：ADPCM 3 輪 Azure zh-HK 辨識通順完整（如『但係點解依家望到外邊係陰天嘅？』），STT 431–526ms，對照同場 PCM 560ms；上行 27,650B/3,370ms 與 16,625B/2,026ms = 8.2 B/ms（PCM 32），發送最長 3ms、最低 heap 55KB</t>
+        </is>
+      </c>
+      <c r="O97" s="13" t="inlineStr">
+        <is>
+          <t>1ed9d3b</t>
+        </is>
+      </c>
       <c r="P97" s="6" t="inlineStr">
         <is>
-          <t>[2026-10-15] 新增</t>
+          <t>[2026-10-15] 新增
+[2026-10-15] 未做：④ 雲端板在 iPhone 熱點重跑 10/13 量度（等雲端可測）；⑤ 舊韌體 1.0.1 連新伺服器（邏輯上無 header 即 PCM，pytest 已覆蓋，未實機）；用戶確認辨識文字與原話一致。分支 p2-24-adpcm-uplink 未合併、未推送。</t>
         </is>
       </c>
     </row>
@@ -11087,7 +11099,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I319"/>
+  <dimension ref="A1:I320"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -22190,8 +22202,55 @@
         </is>
       </c>
     </row>
+    <row r="320" ht="158" customHeight="1">
+      <c r="A320" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-15 10:42</t>
+        </is>
+      </c>
+      <c r="B320" s="13" t="inlineStr">
+        <is>
+          <t>P2-24</t>
+        </is>
+      </c>
+      <c r="C320" s="6" t="inlineStr">
+        <is>
+          <t>麥克風上行改用 IMA ADPCM（減少 4 倍頻寬）</t>
+        </is>
+      </c>
+      <c r="D320" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="E320" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F320" s="13" t="inlineStr">
+        <is>
+          <t>部分通過</t>
+        </is>
+      </c>
+      <c r="G320" s="6" t="inlineStr">
+        <is>
+          <t>① pytest test_mic_adpcm 10 項：Mac 上編譯 firmware MicAdpcm.cpp，與 audioop 逐 byte 一致（改壞一個表值即失敗）；分塊解碼 = 連續流解碼；掉一塊只損失該塊；人聲段 SNR &gt; 20dB；全套 275 passed ② 伺服器按 X-Mic-Codec 解碼，無 header 照舊 PCM（10:37 1.7.5 → mic=pcm，10:40 1.7.6 → mic=adpcm）③ 62:70 Guest（2026-10-15）：ADPCM 3 輪 Azure zh-HK 辨識通順完整（如『但係點解依家望到外邊係陰天嘅？』），STT 431–526ms，對照同場 PCM 560ms；上行 27,650B/3,370ms 與 16,625B/2,026ms = 8.2 B/ms（PCM 32），發送最長 3ms、最低 heap 55KB</t>
+        </is>
+      </c>
+      <c r="H320" s="13" t="inlineStr">
+        <is>
+          <t>1ed9d3b</t>
+        </is>
+      </c>
+      <c r="I320" s="6" t="inlineStr">
+        <is>
+          <t>未做：④ 雲端板在 iPhone 熱點重跑 10/13 量度（等雲端可測）；⑤ 舊韌體 1.0.1 連新伺服器（邏輯上無 header 即 PCM，pytest 已覆蓋，未實機）；用戶確認辨識文字與原話一致。分支 p2-24-adpcm-uplink 未合併、未推送。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I319"/>
+  <autoFilter ref="A1:I320"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Track R-37 hardware results on 62:70.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/production-readiness.xlsx
+++ b/docs/production-readiness.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'任務清單'!$A$1:$P$98</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'待確認問題'!$A$1:$G$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$320</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$321</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1677,7 +1677,7 @@
       <c r="H35" s="11" t="n"/>
       <c r="I35" s="12" t="n"/>
     </row>
-    <row r="36" ht="409" customHeight="1">
+    <row r="36" ht="340" customHeight="1">
       <c r="A36" s="13" t="inlineStr">
         <is>
           <t>R-37</t>
@@ -1700,7 +1700,7 @@
       </c>
       <c r="E36" s="6" t="inlineStr">
         <is>
-          <t>上次測試：部分通過 — 2026-10-15 真機 62:70（hw-test-1015 = dev + P2-16 + R-36 + r-37-wifi-switch，1.7.5，本機 3230/7870）：① 熱點關掉 → 醒來重開後改連 HKQF - Guest 並上線（運行中途消失未單獨測）⑦ Use 按鈕、確認框（寫明 20 秒退回原網絡）、切換中提示都正常；熱點關著按 Use → 11 秒內頁面『couldn't find … nearby. It's back on HKQF - Guest』；熱點開著（到不了 Mac）→ 9 秒內『joined … but couldn't reach the internet … back on HKQF - Guest』，串口 failed (no_internet) → Back on；切換到目前網絡 → current、未存 SSID → unknown，板子不動。pytest 272 passed（新增 6 項），tsc 0 錯誤。未做：⑦ 成功切換（要第二個到得了 Mac 的網絡）、別人設備呼叫 switch → 403（同一個擁有者檢查，未對 switch 重測）、② 密碼打錯
+          <t>上次測試：部分通過 — 62:70（1.7.4/1.7.5，2026-10-15）：① 熱點關掉後醒來改連 HKQF - Guest 並上線（發生在醒來重開時）⑦ Use 按鈕、確認框、『Moving to…』；熱點關著時按 Use → 11 秒內頁面顯示『couldn't find lee’s iPhone nearby. It's back on HKQF - Guest』，串口 not_found → Back on Guest → 重連。過程中發現並修正：驅動殘留上一次的『找不到』令連回原網絡立即失敗並掉進 SoftAP（joinFor 6 秒內不信失敗，tryConnect 同用）。pytest 272 passed
 ① 設定頁顯示玩具在線／離線、目前 Wi-Fi 和訊號、已記住的 Wi-Fi 清單（只有名稱，不顯示密碼）② 在線時可新增 Wi-Fi（輸入或從玩具掃描到的清單選）、刪除 Wi-Fi；不能刪除正在使用的那個 ③ 經 /ws/esp32 轉送：伺服器先確認是設備主人；密碼不寫入資料庫、不寫入日誌 ④ 新增不自動切換網絡；目前 Wi-Fi 消失時按訊號選，或由家長按「改用這個」（⑦）；清單標示「連過／未連過」⑤ 上限 8 個 ⑥ 韌體改動經 OTA 推出 ⑦ 已記住、未在使用的 Wi-Fi 可按「改用這個」：玩具斷開目前網絡改連它，最多 20 秒，要連上我們的伺服器才算成功；失敗就自動連回原網絡，頁面顯示「連不上 X，已回到 Y」；切換中頁面顯示切換中，玩具重新連上後刷新；成功後標示連過</t>
         </is>
       </c>
@@ -9060,12 +9060,12 @@
       <c r="M79" s="13" t="n"/>
       <c r="N79" s="6" t="inlineStr">
         <is>
-          <t>2026-10-15 真機 62:70（hw-test-1015 = dev + P2-16 + R-36 + r-37-wifi-switch，1.7.5，本機 3230/7870）：① 熱點關掉 → 醒來重開後改連 HKQF - Guest 並上線（運行中途消失未單獨測）⑦ Use 按鈕、確認框（寫明 20 秒退回原網絡）、切換中提示都正常；熱點關著按 Use → 11 秒內頁面『couldn't find … nearby. It's back on HKQF - Guest』；熱點開著（到不了 Mac）→ 9 秒內『joined … but couldn't reach the internet … back on HKQF - Guest』，串口 failed (no_internet) → Back on；切換到目前網絡 → current、未存 SSID → unknown，板子不動。pytest 272 passed（新增 6 項），tsc 0 錯誤。未做：⑦ 成功切換（要第二個到得了 Mac 的網絡）、別人設備呼叫 switch → 403（同一個擁有者檢查，未對 switch 重測）、② 密碼打錯</t>
+          <t>62:70（1.7.4/1.7.5，2026-10-15）：① 熱點關掉後醒來改連 HKQF - Guest 並上線（發生在醒來重開時）⑦ Use 按鈕、確認框、『Moving to…』；熱點關著時按 Use → 11 秒內頁面顯示『couldn't find lee’s iPhone nearby. It's back on HKQF - Guest』，串口 not_found → Back on Guest → 重連。過程中發現並修正：驅動殘留上一次的『找不到』令連回原網絡立即失敗並掉進 SoftAP（joinFor 6 秒內不信失敗，tryConnect 同用）。pytest 272 passed</t>
         </is>
       </c>
       <c r="O79" s="13" t="inlineStr">
         <is>
-          <t>22d7674</t>
+          <t>3c180cd</t>
         </is>
       </c>
       <c r="P79" s="6" t="inlineStr">
@@ -9075,7 +9075,8 @@
 [2026-10-15] 2026-10-15 用戶決定：加「改用這個 Wi-Fi」（⑦），④ 改為新增不自動切換、可由家長手動切換。起因：62:70 實測加了 iPhone 熱點也無法讓玩具改用。另：離線一律顯示「睡著了」會誤導（63:64 已 6 天未上線仍叫人按按鈕），待改為按上次上線時間分開提示。
 [2026-10-15] 測試中修了原有 bug（a4 之後第二個 commit）：驅動在沒連上的網絡斷開時不發事件，WiFi.status() 留著上次的『找不到』，新嘗試一開始就被當失敗；1.7.4 切換失敗後連不回 Guest 並掉進 SoftAP，tryConnect() 也同樣。joinFor() 改為 6 秒後才相信失敗，tryConnect() 共用。雲端韌體同樣有這 bug。另：開機時 tryConnect() 挑最強的網絡但不檢查能否到伺服器，62:70 開機連上到不了 Mac 的熱點後一直卡著（見 P2-22 ④ 或另開任務）。分支 r-37-wifi-switch 未推送。
 [2026-10-15] 更正上一條備註：stale『找不到』的修正是 22d7674（切換功能本身是 3c180cd）。
-[2026-10-15] 2026-10-15：⑦ 的成功切換在本機測不到（熱點到不了 Mac 上的伺服器），留到部署上 UAT 或雲端後用 iPhone 熱點測一次。</t>
+[2026-10-15] 2026-10-15：⑦ 的成功切換在本機測不到（熱點到不了 Mac 上的伺服器），留到部署上 UAT 或雲端後用 iPhone 熱點測一次。
+[2026-10-15] 未做：⑦ 熱點開著但到不了伺服器（no_internet）→ 退回；⑦ 成功切換（需第二個能到 Mac 的網絡）；② 密碼打錯。發現：開機挑最強訊號、不檢查能否到伺服器，62:70 開機時連上 iPhone 熱點就一直取不到 token（本機伺服器到不了），建議併入 P2-22 ④ 或另開。分支 r-37-wifi-switch（3c180cd + 修正）未合併、未推送。</t>
         </is>
       </c>
     </row>
@@ -11099,7 +11100,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I320"/>
+  <dimension ref="A1:I321"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -22249,8 +22250,55 @@
         </is>
       </c>
     </row>
+    <row r="321" ht="130" customHeight="1">
+      <c r="A321" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-15 10:42</t>
+        </is>
+      </c>
+      <c r="B321" s="13" t="inlineStr">
+        <is>
+          <t>R-37</t>
+        </is>
+      </c>
+      <c r="C321" s="6" t="inlineStr">
+        <is>
+          <t>網頁設定玩具的 Wi-Fi：查看、新增、刪除</t>
+        </is>
+      </c>
+      <c r="D321" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="E321" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F321" s="13" t="inlineStr">
+        <is>
+          <t>部分通過</t>
+        </is>
+      </c>
+      <c r="G321" s="6" t="inlineStr">
+        <is>
+          <t>62:70（1.7.4/1.7.5，2026-10-15）：① 熱點關掉後醒來改連 HKQF - Guest 並上線（發生在醒來重開時）⑦ Use 按鈕、確認框、『Moving to…』；熱點關著時按 Use → 11 秒內頁面顯示『couldn't find lee’s iPhone nearby. It's back on HKQF - Guest』，串口 not_found → Back on Guest → 重連。過程中發現並修正：驅動殘留上一次的『找不到』令連回原網絡立即失敗並掉進 SoftAP（joinFor 6 秒內不信失敗，tryConnect 同用）。pytest 272 passed</t>
+        </is>
+      </c>
+      <c r="H321" s="13" t="inlineStr">
+        <is>
+          <t>3c180cd</t>
+        </is>
+      </c>
+      <c r="I321" s="6" t="inlineStr">
+        <is>
+          <t>未做：⑦ 熱點開著但到不了伺服器（no_internet）→ 退回；⑦ 成功切換（需第二個能到 Mac 的網絡）；② 密碼打錯。發現：開機挑最強訊號、不檢查能否到伺服器，62:70 開機時連上 iPhone 熱點就一直取不到 token（本機伺服器到不了），建議併入 P2-22 ④ 或另開。分支 r-37-wifi-switch（3c180cd + 修正）未合併、未推送。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I320"/>
+  <autoFilter ref="A1:I321"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Track P2-25 hardware results on 62:70.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/production-readiness.xlsx
+++ b/docs/production-readiness.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'任務清單'!$A$1:$P$98</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'待確認問題'!$A$1:$G$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$321</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$322</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -665,7 +665,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>最後更新：2026-10-15 10:42　·　本頁由 tracker.py 自動生成，請勿手動編輯</t>
+          <t>最後更新：2026-10-15 11:31　·　本頁由 tracker.py 自動生成，請勿手動編輯</t>
         </is>
       </c>
     </row>
@@ -820,11 +820,11 @@
       </c>
       <c r="D8" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A8,'任務清單'!$F:$F,D$5)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E8" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A8,'任務清單'!$F:$F,E$5)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F8" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A8,'任務清單'!$F:$F,F$5)</f>
@@ -896,11 +896,11 @@
       </c>
       <c r="D10" s="5">
         <f>SUM(D6:D9)</f>
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E10" s="5">
         <f>SUM(E6:E9)</f>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F10" s="5">
         <f>SUM(F6:F9)</f>
@@ -1023,11 +1023,11 @@
       </c>
       <c r="D14" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A14,'任務清單'!$F:$F,D$12)</f>
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E14" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A14,'任務清單'!$F:$F,E$12)</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F14" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A14,'任務清單'!$F:$F,F$12)</f>
@@ -1139,11 +1139,11 @@
       </c>
       <c r="D17" s="5">
         <f>SUM(D13:D16)</f>
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E17" s="5">
         <f>SUM(E13:E16)</f>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F17" s="5">
         <f>SUM(F13:F16)</f>
@@ -1550,15 +1550,15 @@
       <c r="H31" s="11" t="n"/>
       <c r="I31" s="12" t="n"/>
     </row>
-    <row r="32" ht="200" customHeight="1">
+    <row r="32" ht="270" customHeight="1">
       <c r="A32" s="13" t="inlineStr">
         <is>
-          <t>R-21</t>
+          <t>P2-25</t>
         </is>
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>藍牙配網與綁定（取代熱點配網）</t>
+          <t>C3 斷線後自救：TLS 握手超時縮短、連續失敗重設 Wi-Fi 或重開、修重試漏記憶體</t>
         </is>
       </c>
       <c r="C32" s="13" t="inlineStr">
@@ -1573,7 +1573,8 @@
       </c>
       <c r="E32" s="6" t="inlineStr">
         <is>
-          <t>① 設備在「未配網、Wi-Fi 連不上、未綁定、長按 BOOT」時以 AIBuddy-XXXX 名稱廣播藍牙，廣播資料帶品牌，品牌 App 只列出自己品牌的設備。② 設備經藍牙回傳它掃描到的 2.4GHz Wi-Fi 清單，App 讓用戶選擇並填密碼。③ App 經藍牙把 SSID、密碼和綁定票（P0-11）一起交給設備；藍牙通道加密（ESP 標準配網協定 security 1/2 或同等）。④ 設備連上 Wi-Fi 後自己完成認領，App 顯示綁定成功或失敗原因（密碼錯、設備已有主人、票過期）。⑤ 配網期間不啟動音訊；完成後釋放藍牙記憶體再開語音（必要時重開機），對話中最低 heap 不比現在差。⑥ 解綁在 App 內完成（P1-12），解綁後設備進入藍牙待綁定狀態。⑦ SoftAP 熱點配網保留給開發和運維（隱藏觸發方式或編譯開關），量產用戶流程不出現。</t>
+          <t>上次測試：部分通過 — 62:70（2026-10-15，分支 p2-25-reconnect-recovery，1.7.7/1.7.8，wss 連 Mac 上只接受不回應的端口）：① 握手每 16 秒失敗一次（15s 超時 + 1s 重連；以前 121s），objdump 確認 WiFiClientSecure 兩處呼叫都經 __wrap ② 63s、129s 重設 Wi-Fi，193s 靜默重開（Chime: boot skipped），重開後只重設 Wi-Fi（63/127/191/240s），不再重開 ③ 3s 超時版 65 次失敗握手：heap 64,424 → 64,300（波動 64,068–64,504），無漏 ④ 健康連線 2 分鐘無誤判；語音伺服器停 40 秒，恢復後 1 秒內重連。測試中發現並修正兩個問題：token 200 曾清除失聯記錄（每 3 分鐘重開）；只看事件不看狀態曾在健康連線 60 秒後重設 Wi-Fi
+① websocket / HTTPS 的 TLS 握手超時約 15 秒 ② Wi-Fi 在線但沒有開著的連線、也不是在等認領：累計 60 秒重設 Wi-Fi，3 分鐘靜默重開一次（同一次失聯只一次），之後每 60 秒重設 Wi-Fi ③ 失敗的重連不漏 heap：連續 50 次失敗前後差 &lt; 1KB ④ 已綁定設備的正常斷網重連行為不變</t>
         </is>
       </c>
       <c r="F32" s="11" t="n"/>
@@ -1581,15 +1582,15 @@
       <c r="H32" s="11" t="n"/>
       <c r="I32" s="12" t="n"/>
     </row>
-    <row r="33" ht="172" customHeight="1">
+    <row r="33" ht="200" customHeight="1">
       <c r="A33" s="13" t="inlineStr">
         <is>
-          <t>R-36</t>
+          <t>R-21</t>
         </is>
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>未認領的設備停在配對狀態，不再每秒重連 websocket</t>
+          <t>藍牙配網與綁定（取代熱點配網）</t>
         </is>
       </c>
       <c r="C33" s="13" t="inlineStr">
@@ -1604,8 +1605,7 @@
       </c>
       <c r="E33" s="6" t="inlineStr">
         <is>
-          <t>上次測試：部分通過 — 補充 2026-10-15（1.7.5，含 R-36）：已綁定時兩次 Wi-Fi 切換各斷網 9–11 秒，都自動重連並重新 auth，沒有停在暫停狀態；30 秒斷網仍未做
-① 拿到 202 或 websocket 被 4401 拒絕後，設備停掉 websocket 自動重連，進入待綁定狀態（燈號可分辨）。② 待綁定時只按退避（5 秒起、上限 PROVISION_BACKOFF_MAX）呼叫 generate_auth_token，不開 websocket。③ 被認領後下一次輪詢拿到 200，在 10 秒內（加退避）自動開 websocket 並能對話，不用重開機。④ 已綁定設備網絡斷線重連的行為不變。⑤ 隨 OTA 推出。</t>
+          <t>① 設備在「未配網、Wi-Fi 連不上、未綁定、長按 BOOT」時以 AIBuddy-XXXX 名稱廣播藍牙，廣播資料帶品牌，品牌 App 只列出自己品牌的設備。② 設備經藍牙回傳它掃描到的 2.4GHz Wi-Fi 清單，App 讓用戶選擇並填密碼。③ App 經藍牙把 SSID、密碼和綁定票（P0-11）一起交給設備；藍牙通道加密（ESP 標準配網協定 security 1/2 或同等）。④ 設備連上 Wi-Fi 後自己完成認領，App 顯示綁定成功或失敗原因（密碼錯、設備已有主人、票過期）。⑤ 配網期間不啟動音訊；完成後釋放藍牙記憶體再開語音（必要時重開機），對話中最低 heap 不比現在差。⑥ 解綁在 App 內完成（P1-12），解綁後設備進入藍牙待綁定狀態。⑦ SoftAP 熱點配網保留給開發和運維（隱藏觸發方式或編譯開關），量產用戶流程不出現。</t>
         </is>
       </c>
       <c r="F33" s="11" t="n"/>
@@ -1613,20 +1613,20 @@
       <c r="H33" s="11" t="n"/>
       <c r="I33" s="12" t="n"/>
     </row>
-    <row r="34" ht="228" customHeight="1">
+    <row r="34" ht="172" customHeight="1">
       <c r="A34" s="13" t="inlineStr">
         <is>
-          <t>P2-12</t>
+          <t>R-36</t>
         </is>
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>量產燒錄前加大 app 分區</t>
+          <t>未認領的設備停在配對狀態，不再每秒重連 websocket</t>
         </is>
       </c>
       <c r="C34" s="13" t="inlineStr">
         <is>
-          <t>3 封閉內測</t>
+          <t>2 內測準備</t>
         </is>
       </c>
       <c r="D34" s="13" t="inlineStr">
@@ -1636,8 +1636,8 @@
       </c>
       <c r="E34" s="6" t="inlineStr">
         <is>
-          <t>上次測試：部分通過 — 62:70（spotpear-ai-toy-p212 原型，現已併入 spotpear-ai-toy）：① 本機 OTA 1.6.1→1.6.2 寫入新 app1，120s 後 confirmed ② 3 秒 abort 的 1.6.3 → PANIC → 回到 1.6.2，ota_failed_version=1.6.3 ③ 崩潰寫入 coredump 14.8KB ④ 資源分區 9 個聲音 504KB/2MB，開機 CRC 63ms，OTA 後照常；損壞/清空 → 退回內建聲音無崩潰 ⑤ pio 全部 18 個 env 編譯通過，映像都在各自 app 槽內（Spotpear 4 個 1.59–1.60MB / 4MB；其他板仍 2MB 槽）；R-21 藍牙探針版 2,326,128 bytes &lt; 4MB ⑥ release_firmware.py 映像 &gt; app 槽即拒發。未做：雲端 OTA 一次（等上 UAT）、出廠腳本寫入資源包（R-10）
-新分區表（例如 app0/app1 各 4MB，保留 nvs/otadata 位置）在出廠前定案並寫入出廠腳本；OTA 與回滾在新分區表上照常</t>
+          <t>上次測試：部分通過 — 補充 2026-10-15（1.7.5，含 R-36）：已綁定時兩次 Wi-Fi 切換各斷網 9–11 秒，都自動重連並重新 auth，沒有停在暫停狀態；30 秒斷網仍未做
+① 拿到 202 或 websocket 被 4401 拒絕後，設備停掉 websocket 自動重連，進入待綁定狀態（燈號可分辨）。② 待綁定時只按退避（5 秒起、上限 PROVISION_BACKOFF_MAX）呼叫 generate_auth_token，不開 websocket。③ 被認領後下一次輪詢拿到 200，在 10 秒內（加退避）自動開 websocket 並能對話，不用重開機。④ 已綁定設備網絡斷線重連的行為不變。⑤ 隨 OTA 推出。</t>
         </is>
       </c>
       <c r="F34" s="11" t="n"/>
@@ -1645,15 +1645,15 @@
       <c r="H34" s="11" t="n"/>
       <c r="I34" s="12" t="n"/>
     </row>
-    <row r="35" ht="409" customHeight="1">
+    <row r="35" ht="228" customHeight="1">
       <c r="A35" s="13" t="inlineStr">
         <is>
-          <t>P2-22</t>
+          <t>P2-12</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>改服務器網址也不失聯：語音網址由後端下發、後端網址可遷移、已確認韌體長期連不上時自救</t>
+          <t>量產燒錄前加大 app 分區</t>
         </is>
       </c>
       <c r="C35" s="13" t="inlineStr">
@@ -1668,8 +1668,8 @@
       </c>
       <c r="E35" s="6" t="inlineStr">
         <is>
-          <t>上次測試：部分通過 — 後端部分（分支 p2-22-server-urls）：node --test lib/deviceServerUrls.test.mjs 5/5、tsc 0 錯誤。worktree dev server 3222 + 本機 Supabase，兩塊假板（02:22:…:01/02）：已認領 200 帶 voice_url + backend_url；未認領 202 只帶 backend_url；DEVICE_VOICE_URL=ws://fastapi:7860/… → 不發、日誌記錯誤；兩個變數都不設 → 兩個欄位都不帶；生產值 → wss://elatoai.hkqft.com/fastapi/ws/esp32、https://elatoai.hkqft.com。測試數據已清除
-① /api/generate_auth_token 的回應帶 voice_url（wss 主機＋端口＋路徑，來自後端環境變數）；韌體用它連 /ws，並把最後一次成功的值存進 NVS；改 FastAPI 網址只改伺服器設定，不需新韌體 ② 回應沒有 voice_url（舊後端）或新網址連不上時，退回 NVS 上次成功的值，再退回出廠／編譯時的預設值 ③ 後端網址可遷移：回應可帶 backend_url；韌體先存為候選，下次開機用新網址取 token 成功才正式替換，失敗就繼續用舊網址；舊網址在遷移期內保持可用（runbook 寫明保留多久） ④ 已確認的韌體若連續 N 次開機（預設 10 次、跨度至少 24 小時，計數存 NVS）Wi-Fi 已拿到 IP 卻取不到 token：先依次試 NVS、出廠的後端網址；仍失敗且另一個槽可用，就切到另一個槽一次，並在下次連上時把本版本報為失敗 ⑤ 純斷網（拿不到 IP、路由器沒外網）不計入 ④ ⑥ 新網址的證書必須鏈到 CF_CA_bundle 裡的根（GTS Root R4、ISRG Root X1）；換主機或離開 Cloudflare 前先查證書鏈，runbook 寫明 ⑦ 只接受 https 的 backend_url 和 wss 的 voice_url，主機須在韌體內允許的網域後綴之下，防止後端被冒充時把板子引去別處</t>
+          <t>上次測試：部分通過 — 62:70（spotpear-ai-toy-p212 原型，現已併入 spotpear-ai-toy）：① 本機 OTA 1.6.1→1.6.2 寫入新 app1，120s 後 confirmed ② 3 秒 abort 的 1.6.3 → PANIC → 回到 1.6.2，ota_failed_version=1.6.3 ③ 崩潰寫入 coredump 14.8KB ④ 資源分區 9 個聲音 504KB/2MB，開機 CRC 63ms，OTA 後照常；損壞/清空 → 退回內建聲音無崩潰 ⑤ pio 全部 18 個 env 編譯通過，映像都在各自 app 槽內（Spotpear 4 個 1.59–1.60MB / 4MB；其他板仍 2MB 槽）；R-21 藍牙探針版 2,326,128 bytes &lt; 4MB ⑥ release_firmware.py 映像 &gt; app 槽即拒發。未做：雲端 OTA 一次（等上 UAT）、出廠腳本寫入資源包（R-10）
+新分區表（例如 app0/app1 各 4MB，保留 nvs/otadata 位置）在出廠前定案並寫入出廠腳本；OTA 與回滾在新分區表上照常</t>
         </is>
       </c>
       <c r="F35" s="11" t="n"/>
@@ -1677,15 +1677,15 @@
       <c r="H35" s="11" t="n"/>
       <c r="I35" s="12" t="n"/>
     </row>
-    <row r="36" ht="340" customHeight="1">
+    <row r="36" ht="409" customHeight="1">
       <c r="A36" s="13" t="inlineStr">
         <is>
-          <t>R-37</t>
+          <t>P2-22</t>
         </is>
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>網頁設定玩具的 Wi-Fi：查看、新增、刪除</t>
+          <t>改服務器網址也不失聯：語音網址由後端下發、後端網址可遷移、已確認韌體長期連不上時自救</t>
         </is>
       </c>
       <c r="C36" s="13" t="inlineStr">
@@ -1700,8 +1700,8 @@
       </c>
       <c r="E36" s="6" t="inlineStr">
         <is>
-          <t>上次測試：部分通過 — 62:70（1.7.4/1.7.5，2026-10-15）：① 熱點關掉後醒來改連 HKQF - Guest 並上線（發生在醒來重開時）⑦ Use 按鈕、確認框、『Moving to…』；熱點關著時按 Use → 11 秒內頁面顯示『couldn't find lee’s iPhone nearby. It's back on HKQF - Guest』，串口 not_found → Back on Guest → 重連。過程中發現並修正：驅動殘留上一次的『找不到』令連回原網絡立即失敗並掉進 SoftAP（joinFor 6 秒內不信失敗，tryConnect 同用）。pytest 272 passed
-① 設定頁顯示玩具在線／離線、目前 Wi-Fi 和訊號、已記住的 Wi-Fi 清單（只有名稱，不顯示密碼）② 在線時可新增 Wi-Fi（輸入或從玩具掃描到的清單選）、刪除 Wi-Fi；不能刪除正在使用的那個 ③ 經 /ws/esp32 轉送：伺服器先確認是設備主人；密碼不寫入資料庫、不寫入日誌 ④ 新增不自動切換網絡；目前 Wi-Fi 消失時按訊號選，或由家長按「改用這個」（⑦）；清單標示「連過／未連過」⑤ 上限 8 個 ⑥ 韌體改動經 OTA 推出 ⑦ 已記住、未在使用的 Wi-Fi 可按「改用這個」：玩具斷開目前網絡改連它，最多 20 秒，要連上我們的伺服器才算成功；失敗就自動連回原網絡，頁面顯示「連不上 X，已回到 Y」；切換中頁面顯示切換中，玩具重新連上後刷新；成功後標示連過</t>
+          <t>上次測試：部分通過 — 後端部分（分支 p2-22-server-urls）：node --test lib/deviceServerUrls.test.mjs 5/5、tsc 0 錯誤。worktree dev server 3222 + 本機 Supabase，兩塊假板（02:22:…:01/02）：已認領 200 帶 voice_url + backend_url；未認領 202 只帶 backend_url；DEVICE_VOICE_URL=ws://fastapi:7860/… → 不發、日誌記錯誤；兩個變數都不設 → 兩個欄位都不帶；生產值 → wss://elatoai.hkqft.com/fastapi/ws/esp32、https://elatoai.hkqft.com。測試數據已清除
+① /api/generate_auth_token 的回應帶 voice_url（wss 主機＋端口＋路徑，來自後端環境變數）；韌體用它連 /ws，並把最後一次成功的值存進 NVS；改 FastAPI 網址只改伺服器設定，不需新韌體 ② 回應沒有 voice_url（舊後端）或新網址連不上時，退回 NVS 上次成功的值，再退回出廠／編譯時的預設值 ③ 後端網址可遷移：回應可帶 backend_url；韌體先存為候選，下次開機用新網址取 token 成功才正式替換，失敗就繼續用舊網址；舊網址在遷移期內保持可用（runbook 寫明保留多久） ④ 已確認的韌體若連續 N 次開機（預設 10 次、跨度至少 24 小時，計數存 NVS）Wi-Fi 已拿到 IP 卻取不到 token：先依次試 NVS、出廠的後端網址；仍失敗且另一個槽可用，就切到另一個槽一次，並在下次連上時把本版本報為失敗 ⑤ 純斷網（拿不到 IP、路由器沒外網）不計入 ④ ⑥ 新網址的證書必須鏈到 CF_CA_bundle 裡的根（GTS Root R4、ISRG Root X1）；換主機或離開 Cloudflare 前先查證書鏈，runbook 寫明 ⑦ 只接受 https 的 backend_url 和 wss 的 voice_url，主機須在韌體內允許的網域後綴之下，防止後端被冒充時把板子引去別處</t>
         </is>
       </c>
       <c r="F36" s="11" t="n"/>
@@ -1709,30 +1709,31 @@
       <c r="H36" s="11" t="n"/>
       <c r="I36" s="12" t="n"/>
     </row>
-    <row r="37" ht="102" customHeight="1">
+    <row r="37" ht="340" customHeight="1">
       <c r="A37" s="13" t="inlineStr">
         <is>
-          <t>R-16</t>
+          <t>R-37</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>Spotpear 量產版加電池電壓檢測（GPIO0 分壓）</t>
+          <t>網頁設定玩具的 Wi-Fi：查看、新增、刪除</t>
         </is>
       </c>
       <c r="C37" s="13" t="inlineStr">
         <is>
-          <t>1 止血定案</t>
+          <t>3 封閉內測</t>
         </is>
       </c>
       <c r="D37" s="13" t="inlineStr">
         <is>
-          <t>未開始</t>
+          <t>進行中</t>
         </is>
       </c>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>Spotpear 書面確認量產版：GPIO1（屏幕 DC；本版不接屏幕，可空出來）接電芯正極（保護 IC 之後）100k/100k 分壓、100nF 濾波，屏幕不接該腳；GPIO0 保留給現有的 VDD 低電提醒；最好另把充電芯片 CHRG 接到 GPIO12 或 13。樣板到手後，固件讀到的電芯電壓與萬用表相差 ≤50mV，App（R-41）顯示百分比與充電中。</t>
+          <t>上次測試：部分通過 — 62:70（1.7.4/1.7.5，2026-10-15）：① 熱點關掉後醒來改連 HKQF - Guest 並上線（發生在醒來重開時）⑦ Use 按鈕、確認框、『Moving to…』；熱點關著時按 Use → 11 秒內頁面顯示『couldn't find lee’s iPhone nearby. It's back on HKQF - Guest』，串口 not_found → Back on Guest → 重連。過程中發現並修正：驅動殘留上一次的『找不到』令連回原網絡立即失敗並掉進 SoftAP（joinFor 6 秒內不信失敗，tryConnect 同用）。pytest 272 passed
+① 設定頁顯示玩具在線／離線、目前 Wi-Fi 和訊號、已記住的 Wi-Fi 清單（只有名稱，不顯示密碼）② 在線時可新增 Wi-Fi（輸入或從玩具掃描到的清單選）、刪除 Wi-Fi；不能刪除正在使用的那個 ③ 經 /ws/esp32 轉送：伺服器先確認是設備主人；密碼不寫入資料庫、不寫入日誌 ④ 新增不自動切換網絡；目前 Wi-Fi 消失時按訊號選，或由家長按「改用這個」（⑦）；清單標示「連過／未連過」⑤ 上限 8 個 ⑥ 韌體改動經 OTA 推出 ⑦ 已記住、未在使用的 Wi-Fi 可按「改用這個」：玩具斷開目前網絡改連它，最多 20 秒，要連上我們的伺服器才算成功；失敗就自動連回原網絡，頁面顯示「連不上 X，已回到 Y」；切換中頁面顯示切換中，玩具重新連上後刷新；成功後標示連過</t>
         </is>
       </c>
       <c r="F37" s="11" t="n"/>
@@ -1740,20 +1741,20 @@
       <c r="H37" s="11" t="n"/>
       <c r="I37" s="12" t="n"/>
     </row>
-    <row r="38" ht="46" customHeight="1">
+    <row r="38" ht="102" customHeight="1">
       <c r="A38" s="13" t="inlineStr">
         <is>
-          <t>P1-11</t>
+          <t>R-16</t>
         </is>
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>伺服器與資料庫直接存取的管控</t>
+          <t>Spotpear 量產版加電池電壓檢測（GPIO0 分壓）</t>
         </is>
       </c>
       <c r="C38" s="13" t="inlineStr">
         <is>
-          <t>2 內測準備</t>
+          <t>1 止血定案</t>
         </is>
       </c>
       <c r="D38" s="13" t="inlineStr">
@@ -1763,7 +1764,7 @@
       </c>
       <c r="E38" s="6" t="inlineStr">
         <is>
-          <t>列出誰有 SSH 與資料庫直連權限（越少越好）；service_role key 只存在伺服器的 env；私隱政策寫明這類存取的範圍；每次直接查看生產資料都留記錄。</t>
+          <t>Spotpear 書面確認量產版：GPIO1（屏幕 DC；本版不接屏幕，可空出來）接電芯正極（保護 IC 之後）100k/100k 分壓、100nF 濾波，屏幕不接該腳；GPIO0 保留給現有的 VDD 低電提醒；最好另把充電芯片 CHRG 接到 GPIO12 或 13。樣板到手後，固件讀到的電芯電壓與萬用表相差 ≤50mV，App（R-41）顯示百分比與充電中。</t>
         </is>
       </c>
       <c r="F38" s="11" t="n"/>
@@ -1774,12 +1775,12 @@
     <row r="39" ht="46" customHeight="1">
       <c r="A39" s="13" t="inlineStr">
         <is>
-          <t>P2-02</t>
+          <t>P1-11</t>
         </is>
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>CI 跑測試與靜態檢查</t>
+          <t>伺服器與資料庫直接存取的管控</t>
         </is>
       </c>
       <c r="C39" s="13" t="inlineStr">
@@ -1794,7 +1795,7 @@
       </c>
       <c r="E39" s="6" t="inlineStr">
         <is>
-          <t>推送與 PR 時跑 pytest、ruff、pyright、next lint、tsc --noEmit、pio run；任何一項失敗就不發佈 image。</t>
+          <t>列出誰有 SSH 與資料庫直連權限（越少越好）；service_role key 只存在伺服器的 env；私隱政策寫明這類存取的範圍；每次直接查看生產資料都留記錄。</t>
         </is>
       </c>
       <c r="F39" s="11" t="n"/>
@@ -1802,15 +1803,15 @@
       <c r="H39" s="11" t="n"/>
       <c r="I39" s="12" t="n"/>
     </row>
-    <row r="40" ht="32" customHeight="1">
+    <row r="40" ht="46" customHeight="1">
       <c r="A40" s="13" t="inlineStr">
         <is>
-          <t>P2-04</t>
+          <t>P2-02</t>
         </is>
       </c>
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>容器改用非 root 用戶</t>
+          <t>CI 跑測試與靜態檢查</t>
         </is>
       </c>
       <c r="C40" s="13" t="inlineStr">
@@ -1825,7 +1826,7 @@
       </c>
       <c r="E40" s="6" t="inlineStr">
         <is>
-          <t>兩個 Dockerfile 都設定非 root 的 USER。</t>
+          <t>推送與 PR 時跑 pytest、ruff、pyright、next lint、tsc --noEmit、pio run；任何一項失敗就不發佈 image。</t>
         </is>
       </c>
       <c r="F40" s="11" t="n"/>
@@ -1833,15 +1834,15 @@
       <c r="H40" s="11" t="n"/>
       <c r="I40" s="12" t="n"/>
     </row>
-    <row r="41" ht="46" customHeight="1">
+    <row r="41" ht="32" customHeight="1">
       <c r="A41" s="13" t="inlineStr">
         <is>
-          <t>R-04</t>
+          <t>P2-04</t>
         </is>
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>粵語質量評測</t>
+          <t>容器改用非 root 用戶</t>
         </is>
       </c>
       <c r="C41" s="13" t="inlineStr">
@@ -1856,7 +1857,7 @@
       </c>
       <c r="E41" s="6" t="inlineStr">
         <is>
-          <t>有一套粵語評測集（兒童錄音＋文字提示）；選定的 STT 與 LLM 達到門檻：兒童語音字錯率 ≤15%、口語粵語回覆 ≥90%、中英夾雜句能正確理解。</t>
+          <t>兩個 Dockerfile 都設定非 root 的 USER。</t>
         </is>
       </c>
       <c r="F41" s="11" t="n"/>
@@ -1864,15 +1865,15 @@
       <c r="H41" s="11" t="n"/>
       <c r="I41" s="12" t="n"/>
     </row>
-    <row r="42" ht="116" customHeight="1">
+    <row r="42" ht="46" customHeight="1">
       <c r="A42" s="13" t="inlineStr">
         <is>
-          <t>R-25</t>
+          <t>R-04</t>
         </is>
       </c>
       <c r="B42" s="6" t="inlineStr">
         <is>
-          <t>網頁的品牌主題系統</t>
+          <t>粵語質量評測</t>
         </is>
       </c>
       <c r="C42" s="13" t="inlineStr">
@@ -1887,7 +1888,7 @@
       </c>
       <c r="E42" s="6" t="inlineStr">
         <is>
-          <t>① 每個品牌一個資料夾：主題 token（顏色、字體、圓角）、logo 和圖示、文案、功能開關；首頁、上手流程、角色頁可以有品牌版本，其餘頁面共用 ② 由部署的環境變數選品牌（每套部署一個品牌，見 R-34），伺服器端渲染的第一屏就是對的主題，不閃爍 ③ 共用元件裡沒有品牌名稱和寫死的品牌顏色 ④ 加一個品牌只需要加資料夾、設定和一套部署，不用改共用元件</t>
+          <t>有一套粵語評測集（兒童錄音＋文字提示）；選定的 STT 與 LLM 達到門檻：兒童語音字錯率 ≤15%、口語粵語回覆 ≥90%、中英夾雜句能正確理解。</t>
         </is>
       </c>
       <c r="F42" s="11" t="n"/>
@@ -1895,68 +1896,68 @@
       <c r="H42" s="11" t="n"/>
       <c r="I42" s="12" t="n"/>
     </row>
-    <row r="44">
-      <c r="A44" s="10" t="inlineStr">
+    <row r="43" ht="116" customHeight="1">
+      <c r="A43" s="13" t="inlineStr">
+        <is>
+          <t>R-25</t>
+        </is>
+      </c>
+      <c r="B43" s="6" t="inlineStr">
+        <is>
+          <t>網頁的品牌主題系統</t>
+        </is>
+      </c>
+      <c r="C43" s="13" t="inlineStr">
+        <is>
+          <t>2 內測準備</t>
+        </is>
+      </c>
+      <c r="D43" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E43" s="6" t="inlineStr">
+        <is>
+          <t>① 每個品牌一個資料夾：主題 token（顏色、字體、圓角）、logo 和圖示、文案、功能開關；首頁、上手流程、角色頁可以有品牌版本，其餘頁面共用 ② 由部署的環境變數選品牌（每套部署一個品牌，見 R-34），伺服器端渲染的第一屏就是對的主題，不閃爍 ③ 共用元件裡沒有品牌名稱和寫死的品牌顏色 ④ 加一個品牌只需要加資料夾、設定和一套部署，不用改共用元件</t>
+        </is>
+      </c>
+      <c r="F43" s="11" t="n"/>
+      <c r="G43" s="11" t="n"/>
+      <c r="H43" s="11" t="n"/>
+      <c r="I43" s="12" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="10" t="inlineStr">
         <is>
           <t>✅ 最近完成與測試效果</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="4" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
         <is>
           <t>編號</t>
         </is>
       </c>
-      <c r="B45" s="4" t="inlineStr">
+      <c r="B46" s="4" t="inlineStr">
         <is>
           <t>任務</t>
         </is>
       </c>
-      <c r="C45" s="4" t="inlineStr">
+      <c r="C46" s="4" t="inlineStr">
         <is>
           <t>測試結果</t>
         </is>
       </c>
-      <c r="D45" s="4" t="inlineStr">
+      <c r="D46" s="4" t="inlineStr">
         <is>
           <t>完成日期</t>
         </is>
       </c>
-      <c r="E45" s="4" t="inlineStr">
+      <c r="E46" s="4" t="inlineStr">
         <is>
           <t>測試證據</t>
-        </is>
-      </c>
-      <c r="F45" s="11" t="n"/>
-      <c r="G45" s="11" t="n"/>
-      <c r="H45" s="11" t="n"/>
-      <c r="I45" s="12" t="n"/>
-    </row>
-    <row r="46" ht="88" customHeight="1">
-      <c r="A46" s="13" t="inlineStr">
-        <is>
-          <t>P2-21</t>
-        </is>
-      </c>
-      <c r="B46" s="6" t="inlineStr">
-        <is>
-          <t>P2-16 ⑤ 後台 OTA 頁換成真實數據與操作</t>
-        </is>
-      </c>
-      <c r="C46" s="13" t="inlineStr">
-        <is>
-          <t>通過</t>
-        </is>
-      </c>
-      <c r="D46" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
-      <c r="E46" s="6" t="inlineStr">
-        <is>
-          <t>10-14 模擬 20 台全部通過（見上次）；2026-10-15 真機補做：OTA 頁對 1.7.1 白名單加 62:70（UI MAC 欄）→ 存檔確認框 → 『Narrow to Whitelist』確認 → Make current（用戶點）→ 62:70 安裝並確認，頁面顯示 Rolling out · Whitelist、運行 1、回滾 0；每步一筆審計。依賴 P2-14 已完成</t>
         </is>
       </c>
       <c r="F46" s="11" t="n"/>
@@ -1964,15 +1965,15 @@
       <c r="H46" s="11" t="n"/>
       <c r="I46" s="12" t="n"/>
     </row>
-    <row r="47" ht="158" customHeight="1">
+    <row r="47" ht="88" customHeight="1">
       <c r="A47" s="13" t="inlineStr">
         <is>
-          <t>P2-16</t>
+          <t>P2-21</t>
         </is>
       </c>
       <c r="B47" s="6" t="inlineStr">
         <is>
-          <t>OTA 分批推送與後台發佈頁</t>
+          <t>P2-16 ⑤ 後台 OTA 頁換成真實數據與操作</t>
         </is>
       </c>
       <c r="C47" s="13" t="inlineStr">
@@ -1987,7 +1988,7 @@
       </c>
       <c r="E47" s="6" t="inlineStr">
         <is>
-          <t>④ 真機 62:70（2026-10-15）：USB 刷 1.7.0（開機印 aibuddy-build;kind=dev;…;version=1.7.0）→ release_firmware.py publish --dev 1.7.1 → 後台白名單加 62:70、改白名單階段、設為 current → 按 BOOT 喚醒：取 token 200、下載 12.8s、重開進 app1，09:39:36 連上語音伺服器；09:42 重開 → 『Firmware 1.7.1 on app1』無 probation、Up to date；頁面『Rolling out · Whitelist』運行 1 台、回滾 0；審計 5 筆（發佈、白名單、階段、1.6.2 取消 current、1.7.1 設 current）。①②③⑤ 見 P2-17～P2-21 模擬 20 台</t>
+          <t>10-14 模擬 20 台全部通過（見上次）；2026-10-15 真機補做：OTA 頁對 1.7.1 白名單加 62:70（UI MAC 欄）→ 存檔確認框 → 『Narrow to Whitelist』確認 → Make current（用戶點）→ 62:70 安裝並確認，頁面顯示 Rolling out · Whitelist、運行 1、回滾 0；每步一筆審計。依賴 P2-14 已完成</t>
         </is>
       </c>
       <c r="F47" s="11" t="n"/>
@@ -1995,15 +1996,15 @@
       <c r="H47" s="11" t="n"/>
       <c r="I47" s="12" t="n"/>
     </row>
-    <row r="48" ht="144" customHeight="1">
+    <row r="48" ht="158" customHeight="1">
       <c r="A48" s="13" t="inlineStr">
         <is>
-          <t>P2-14</t>
+          <t>P2-16</t>
         </is>
       </c>
       <c r="B48" s="6" t="inlineStr">
         <is>
-          <t>Admin 設備頁：每台玩具的狀態、韌體與基本操作</t>
+          <t>OTA 分批推送與後台發佈頁</t>
         </is>
       </c>
       <c r="C48" s="13" t="inlineStr">
@@ -2018,7 +2019,7 @@
       </c>
       <c r="E48" s="6" t="inlineStr">
         <is>
-          <t>真機 62:70（2026-10-15，分支 hw-test-1015 = dev+P2-16，-localall 1.7.0，本機網頁 3230 + 語音 7870）：① 開機 → 設備頁 Online、-67 dBm、1.7.0；板子停在 bootloader 約 38 秒後語音伺服器判離線（uvicorn ping 超時），頁面 0 台在線 ② 重置設備密鑰 → device_secrets 行刪除，板子重開印『Device secret issued and stored』並連上，行恢復 ③ 強制解綁 → 板子拿 202（配對碼 UKDM7N），語音伺服器拒絕連線；兩項審計各 1 筆含操作者與原因 ④ 內容管理員/anon → 42501（10-14 探測腳本）</t>
+          <t>④ 真機 62:70（2026-10-15）：USB 刷 1.7.0（開機印 aibuddy-build;kind=dev;…;version=1.7.0）→ release_firmware.py publish --dev 1.7.1 → 後台白名單加 62:70、改白名單階段、設為 current → 按 BOOT 喚醒：取 token 200、下載 12.8s、重開進 app1，09:39:36 連上語音伺服器；09:42 重開 → 『Firmware 1.7.1 on app1』無 probation、Up to date；頁面『Rolling out · Whitelist』運行 1 台、回滾 0；審計 5 筆（發佈、白名單、階段、1.6.2 取消 current、1.7.1 設 current）。①②③⑤ 見 P2-17～P2-21 模擬 20 台</t>
         </is>
       </c>
       <c r="F48" s="11" t="n"/>
@@ -2026,15 +2027,15 @@
       <c r="H48" s="11" t="n"/>
       <c r="I48" s="12" t="n"/>
     </row>
-    <row r="49" ht="214" customHeight="1">
+    <row r="49" ht="144" customHeight="1">
       <c r="A49" s="13" t="inlineStr">
         <is>
-          <t>P2-20</t>
+          <t>P2-14</t>
         </is>
       </c>
       <c r="B49" s="6" t="inlineStr">
         <is>
-          <t>P2-16 ④ 從後台上傳與發佈韌體（取代手貼 service key）</t>
+          <t>Admin 設備頁：每台玩具的狀態、韌體與基本操作</t>
         </is>
       </c>
       <c r="C49" s="13" t="inlineStr">
@@ -2044,12 +2045,12 @@
       </c>
       <c r="D49" s="13" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E49" s="6" t="inlineStr">
         <is>
-          <t>node --test lib/firmwareImage.test.mjs 8/8（合成映像：dev build、無標記、未知板、晶片不符、非映像、截斷/損壞、超 4MB 拒；超 2MB 只警告）。分支 dev server + 本機 Supabase 端到端 16/16（GoTrue 真實登入的 cookie）：超管上傳 9.9.0 release build → 201 草稿（is_current f、rollout 0%），DB SHA-256 = 檔案、storage 原樣；審計 insert 記該超管；設備仍只拿到 current 1.6.2；已有 1.0.2 → 409；localall → 422 dev build；4MB+16 → 422；9MB → 413；PNG → 422；舊 1.6.1 映像（無標記）→ 422 指向 release_firmware.py；內容管理員上傳/刪除 → 403；未登入 → 401；刪 current → 409；超管刪草稿 → 行和映像都刪、審計 delete 記該超管。release_firmware.py list 照常。測試帳號與數據已清除</t>
+          <t>真機 62:70（2026-10-15，分支 hw-test-1015 = dev+P2-16，-localall 1.7.0，本機網頁 3230 + 語音 7870）：① 開機 → 設備頁 Online、-67 dBm、1.7.0；板子停在 bootloader 約 38 秒後語音伺服器判離線（uvicorn ping 超時），頁面 0 台在線 ② 重置設備密鑰 → device_secrets 行刪除，板子重開印『Device secret issued and stored』並連上，行恢復 ③ 強制解綁 → 板子拿 202（配對碼 UKDM7N），語音伺服器拒絕連線；兩項審計各 1 筆含操作者與原因 ④ 內容管理員/anon → 42501（10-14 探測腳本）</t>
         </is>
       </c>
       <c r="F49" s="11" t="n"/>
@@ -2057,15 +2058,15 @@
       <c r="H49" s="11" t="n"/>
       <c r="I49" s="12" t="n"/>
     </row>
-    <row r="50" ht="158" customHeight="1">
+    <row r="50" ht="214" customHeight="1">
       <c r="A50" s="13" t="inlineStr">
         <is>
-          <t>P2-19</t>
+          <t>P2-20</t>
         </is>
       </c>
       <c r="B50" s="6" t="inlineStr">
         <is>
-          <t>P2-16 ③ 回滾過多時自動暫停推送</t>
+          <t>P2-16 ④ 從後台上傳與發佈韌體（取代手貼 service key）</t>
         </is>
       </c>
       <c r="C50" s="13" t="inlineStr">
@@ -2080,7 +2081,7 @@
       </c>
       <c r="E50" s="6" t="inlineStr">
         <is>
-          <t>migration 20261014200000 BEGIN/ROLLBACK 套用兩次無錯並已套用本機。模擬 20 台連跑兩次 12/12：1/20 回滾不暫停、其餘 18 台照常；2/20 → 'Auto-paused: 2 of 20 boards rolled back (10%)'，其餘 0 台拿到 ota；已運行的設備記為 running 且不再下發；審計 1 筆 actor 空；恢復後 17 台拿到、保持恢復，第 3 台回滾 → 'Auto-paused: 3 of 20 (15%)'；白名單 2 台中 1 台回滾 → 50% 立即暫停、另一台不再下發；anon 呼叫 ota_maybe_pause → 401/42501。測試數據已清除，spotpear-ai-toy 1.6.2 仍 100% 未暫停</t>
+          <t>node --test lib/firmwareImage.test.mjs 8/8（合成映像：dev build、無標記、未知板、晶片不符、非映像、截斷/損壞、超 4MB 拒；超 2MB 只警告）。分支 dev server + 本機 Supabase 端到端 16/16（GoTrue 真實登入的 cookie）：超管上傳 9.9.0 release build → 201 草稿（is_current f、rollout 0%），DB SHA-256 = 檔案、storage 原樣；審計 insert 記該超管；設備仍只拿到 current 1.6.2；已有 1.0.2 → 409；localall → 422 dev build；4MB+16 → 422；9MB → 413；PNG → 422；舊 1.6.1 映像（無標記）→ 422 指向 release_firmware.py；內容管理員上傳/刪除 → 403；未登入 → 401；刪 current → 409；超管刪草稿 → 行和映像都刪、審計 delete 記該超管。release_firmware.py list 照常。測試帳號與數據已清除</t>
         </is>
       </c>
       <c r="F50" s="11" t="n"/>
@@ -2088,15 +2089,15 @@
       <c r="H50" s="11" t="n"/>
       <c r="I50" s="12" t="n"/>
     </row>
-    <row r="51" ht="200" customHeight="1">
+    <row r="51" ht="158" customHeight="1">
       <c r="A51" s="13" t="inlineStr">
         <is>
-          <t>P2-18</t>
+          <t>P2-19</t>
         </is>
       </c>
       <c r="B51" s="6" t="inlineStr">
         <is>
-          <t>P2-16 ② 按 MAC 雜湊穩定分組決定哪台收到 ota</t>
+          <t>P2-16 ③ 回滾過多時自動暫停推送</t>
         </is>
       </c>
       <c r="C51" s="13" t="inlineStr">
@@ -2111,7 +2112,7 @@
       </c>
       <c r="E51" s="6" t="inlineStr">
         <is>
-          <t>node --test lib/otaRollout.test.mjs 6/6：10,000 隨機 MAC 在 10%/50% 誤差 &lt; 1 個百分點、同 MAC（含大小寫/空白）結果一致、升階段只增不減、白名單各階段都在、不同版本選不同的 10%。tsc --noEmit 通過。分支 dev server（3216）+ 本機 Supabase 模擬 20 台（板型 p218-sim，連跑兩次 9/9）：白名單階段只有 1 台、重複不變；10% 拿到的正是雜湊預測的那組（2–5 台含白名單），重複不變；50% 包含 10% 全部；暫停 → 0 台且下載映像 404，恢復 → 200；100% → 除已更新和已回滾的 2 台外 18 台；每台下發次數與記錄一致；運行中/已回滾正確標記；審計 6 筆對應 6 次變更。真 spotpear-ai-toy（預設 100%）回報 1.6.1 → 仍拿到 1.6.2。測試數據已清除</t>
+          <t>migration 20261014200000 BEGIN/ROLLBACK 套用兩次無錯並已套用本機。模擬 20 台連跑兩次 12/12：1/20 回滾不暫停、其餘 18 台照常；2/20 → 'Auto-paused: 2 of 20 boards rolled back (10%)'，其餘 0 台拿到 ota；已運行的設備記為 running 且不再下發；審計 1 筆 actor 空；恢復後 17 台拿到、保持恢復，第 3 台回滾 → 'Auto-paused: 3 of 20 (15%)'；白名單 2 台中 1 台回滾 → 50% 立即暫停、另一台不再下發；anon 呼叫 ota_maybe_pause → 401/42501。測試數據已清除，spotpear-ai-toy 1.6.2 仍 100% 未暫停</t>
         </is>
       </c>
       <c r="F51" s="11" t="n"/>
@@ -2119,15 +2120,15 @@
       <c r="H51" s="11" t="n"/>
       <c r="I51" s="12" t="n"/>
     </row>
-    <row r="52" ht="172" customHeight="1">
+    <row r="52" ht="200" customHeight="1">
       <c r="A52" s="13" t="inlineStr">
         <is>
-          <t>P2-17</t>
+          <t>P2-18</t>
         </is>
       </c>
       <c r="B52" s="6" t="inlineStr">
         <is>
-          <t>P2-16 ① 分批推送的數據表：推送階段、白名單、每台安裝結果</t>
+          <t>P2-16 ② 按 MAC 雜湊穩定分組決定哪台收到 ota</t>
         </is>
       </c>
       <c r="C52" s="13" t="inlineStr">
@@ -2142,7 +2143,7 @@
       </c>
       <c r="E52" s="6" t="inlineStr">
         <is>
-          <t>migration 20261014190000 BEGIN/ROLLBACK 套用兩次無錯並已套用本機；行為：預設 100%、promote 記 stage_changed_at，7 種壞值（25%、小寫/空字串/NULL MAC、暫停缺原因等）全被 check 擋；ota_note_offer 1→2→3，report 正確標 running/failed、別板型不影響，刪發佈連帶刪記錄；審計 5 筆含 'test-board 9.9.9' 標籤。REST 13/13：超管可讀、內容管理員 0 行、anon 42501，三種身份寫入/改階段/呼叫 ota_note_offer 皆 42501。release_firmware.py promote spotpear-ai-toy 1.6.2 成功，token 查詢仍選 1.6.2，審計記 2 筆（actor 空＝service role）</t>
+          <t>node --test lib/otaRollout.test.mjs 6/6：10,000 隨機 MAC 在 10%/50% 誤差 &lt; 1 個百分點、同 MAC（含大小寫/空白）結果一致、升階段只增不減、白名單各階段都在、不同版本選不同的 10%。tsc --noEmit 通過。分支 dev server（3216）+ 本機 Supabase 模擬 20 台（板型 p218-sim，連跑兩次 9/9）：白名單階段只有 1 台、重複不變；10% 拿到的正是雜湊預測的那組（2–5 台含白名單），重複不變；50% 包含 10% 全部；暫停 → 0 台且下載映像 404，恢復 → 200；100% → 除已更新和已回滾的 2 台外 18 台；每台下發次數與記錄一致；運行中/已回滾正確標記；審計 6 筆對應 6 次變更。真 spotpear-ai-toy（預設 100%）回報 1.6.1 → 仍拿到 1.6.2。測試數據已清除</t>
         </is>
       </c>
       <c r="F52" s="11" t="n"/>
@@ -2150,15 +2151,15 @@
       <c r="H52" s="11" t="n"/>
       <c r="I52" s="12" t="n"/>
     </row>
-    <row r="53" ht="116" customHeight="1">
+    <row r="53" ht="172" customHeight="1">
       <c r="A53" s="13" t="inlineStr">
         <is>
-          <t>R-41</t>
+          <t>P2-17</t>
         </is>
       </c>
       <c r="B53" s="6" t="inlineStr">
         <is>
-          <t>App 顯示玩具電量狀態（低電量提示）</t>
+          <t>P2-16 ① 分批推送的數據表：推送階段、白名單、每台安裝結果</t>
         </is>
       </c>
       <c r="C53" s="13" t="inlineStr">
@@ -2173,7 +2174,7 @@
       </c>
       <c r="E53" s="6" t="inlineStr">
         <is>
-          <t>① pytest 33 passed；真 PATCH 本地 Supabase ② 62:70 刷 p212+R-41 強制低電 build（SUPPLY_LOW_RATIO_OVERRIDE=1.05）→ 串口 [WSc] power low:true，本地 DB battery_low=t ③ 刷回正常 1.6.2 → low:false，DB=f ④ App 讀 DB：低電紅標+Please charge+更新時間、72% 充電中、未上報不顯示 ⑤ 他人帳號 0 行、authenticated UPDATE 被拒。62:70 已還原為原 p212 build</t>
+          <t>migration 20261014190000 BEGIN/ROLLBACK 套用兩次無錯並已套用本機；行為：預設 100%、promote 記 stage_changed_at，7 種壞值（25%、小寫/空字串/NULL MAC、暫停缺原因等）全被 check 擋；ota_note_offer 1→2→3，report 正確標 running/failed、別板型不影響，刪發佈連帶刪記錄；審計 5 筆含 'test-board 9.9.9' 標籤。REST 13/13：超管可讀、內容管理員 0 行、anon 42501，三種身份寫入/改階段/呼叫 ota_note_offer 皆 42501。release_firmware.py promote spotpear-ai-toy 1.6.2 成功，token 查詢仍選 1.6.2，審計記 2 筆（actor 空＝service role）</t>
         </is>
       </c>
       <c r="F53" s="11" t="n"/>
@@ -2181,50 +2182,58 @@
       <c r="H53" s="11" t="n"/>
       <c r="I53" s="12" t="n"/>
     </row>
-    <row r="55">
-      <c r="A55" s="10" t="inlineStr">
+    <row r="54" ht="116" customHeight="1">
+      <c r="A54" s="13" t="inlineStr">
+        <is>
+          <t>R-41</t>
+        </is>
+      </c>
+      <c r="B54" s="6" t="inlineStr">
+        <is>
+          <t>App 顯示玩具電量狀態（低電量提示）</t>
+        </is>
+      </c>
+      <c r="C54" s="13" t="inlineStr">
+        <is>
+          <t>通過</t>
+        </is>
+      </c>
+      <c r="D54" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="E54" s="6" t="inlineStr">
+        <is>
+          <t>① pytest 33 passed；真 PATCH 本地 Supabase ② 62:70 刷 p212+R-41 強制低電 build（SUPPLY_LOW_RATIO_OVERRIDE=1.05）→ 串口 [WSc] power low:true，本地 DB battery_low=t ③ 刷回正常 1.6.2 → low:false，DB=f ④ App 讀 DB：低電紅標+Please charge+更新時間、72% 充電中、未上報不顯示 ⑤ 他人帳號 0 行、authenticated UPDATE 被拒。62:70 已還原為原 p212 build</t>
+        </is>
+      </c>
+      <c r="F54" s="11" t="n"/>
+      <c r="G54" s="11" t="n"/>
+      <c r="H54" s="11" t="n"/>
+      <c r="I54" s="12" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="10" t="inlineStr">
         <is>
           <t>⏳ 等待依賴 / ⛔ 阻塞</t>
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="4" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
         <is>
           <t>編號</t>
         </is>
       </c>
-      <c r="B56" s="4" t="inlineStr">
+      <c r="B57" s="4" t="inlineStr">
         <is>
           <t>任務</t>
         </is>
       </c>
-      <c r="C56" s="4" t="inlineStr">
+      <c r="C57" s="4" t="inlineStr">
         <is>
           <t>在等什麼</t>
-        </is>
-      </c>
-      <c r="D56" s="11" t="n"/>
-      <c r="E56" s="11" t="n"/>
-      <c r="F56" s="11" t="n"/>
-      <c r="G56" s="11" t="n"/>
-      <c r="H56" s="11" t="n"/>
-      <c r="I56" s="12" t="n"/>
-    </row>
-    <row r="57" ht="88" customHeight="1">
-      <c r="A57" s="13" t="inlineStr">
-        <is>
-          <t>R-17</t>
-        </is>
-      </c>
-      <c r="B57" s="6" t="inlineStr">
-        <is>
-          <t>Spotpear 電池耗盡時插電能否正常開機（供電路徑）</t>
-        </is>
-      </c>
-      <c r="C57" s="6" t="inlineStr">
-        <is>
-          <t>阻塞：[2026-10-08] 2026-10-08 開發板 63:64 插著 USB 時兩次無法解釋的完全斷電重開：09:13:26（崩潰循環中）、10:44:33（閒置、用戶確認沒碰）。都是 USB 先斷線再以 ESP_RST_POWERON 開機，非 brownout；斷電前 6 秒 GPIO0 讀數 99.9% 參考值，屬突然切斷而非緩降（SupplyMonitor 取樣太疏抓不到瞬間）。韌體無法造成 POWERON，指向充電芯片/電池保護/供電路徑，應一併問 Spotpear；放電實測時留意插 USB 閒置時是否也會斷電</t>
         </is>
       </c>
       <c r="D57" s="11" t="n"/>
@@ -2234,20 +2243,20 @@
       <c r="H57" s="11" t="n"/>
       <c r="I57" s="12" t="n"/>
     </row>
-    <row r="58" ht="60" customHeight="1">
+    <row r="58" ht="88" customHeight="1">
       <c r="A58" s="13" t="inlineStr">
         <is>
-          <t>P1-01</t>
+          <t>R-17</t>
         </is>
       </c>
       <c r="B58" s="6" t="inlineStr">
         <is>
-          <t>加入內容審核層（輸入與輸出）</t>
+          <t>Spotpear 電池耗盡時插電能否正常開機（供電路徑）</t>
         </is>
       </c>
       <c r="C58" s="6" t="inlineStr">
         <is>
-          <t>阻塞：[2026-10-14] 2026-10-14 用戶決定：先不定審核服務商，本項暫停。候選：Azure Content Safety（建議，香港區、可在每句回覆說出口前檢查）、OpenRouter 安全模型、OpenAI Moderation、只用本機字詞表。未寫任何程式。</t>
+          <t>阻塞：[2026-10-08] 2026-10-08 開發板 63:64 插著 USB 時兩次無法解釋的完全斷電重開：09:13:26（崩潰循環中）、10:44:33（閒置、用戶確認沒碰）。都是 USB 先斷線再以 ESP_RST_POWERON 開機，非 brownout；斷電前 6 秒 GPIO0 讀數 99.9% 參考值，屬突然切斷而非緩降（SupplyMonitor 取樣太疏抓不到瞬間）。韌體無法造成 POWERON，指向充電芯片/電池保護/供電路徑，應一併問 Spotpear；放電實測時留意插 USB 閒置時是否也會斷電</t>
         </is>
       </c>
       <c r="D58" s="11" t="n"/>
@@ -2257,20 +2266,20 @@
       <c r="H58" s="11" t="n"/>
       <c r="I58" s="12" t="n"/>
     </row>
-    <row r="59" ht="32" customHeight="1">
+    <row r="59" ht="60" customHeight="1">
       <c r="A59" s="13" t="inlineStr">
         <is>
-          <t>P1-09</t>
+          <t>P1-01</t>
         </is>
       </c>
       <c r="B59" s="6" t="inlineStr">
         <is>
-          <t>家長鎖：孩子模式進設定要輸入 PIN</t>
+          <t>加入內容審核層（輸入與輸出）</t>
         </is>
       </c>
       <c r="C59" s="6" t="inlineStr">
         <is>
-          <t>阻塞：[2026-10-13] 2026-10-13 用戶決定：AI Buddy（品牌 C）延到 1/15 之後，本項不卡 1/15 出廠；AI Buddy 啟動時再開。</t>
+          <t>阻塞：[2026-10-14] 2026-10-14 用戶決定：先不定審核服務商，本項暫停。候選：Azure Content Safety（建議，香港區、可在每句回覆說出口前檢查）、OpenRouter 安全模型、OpenAI Moderation、只用本機字詞表。未寫任何程式。</t>
         </is>
       </c>
       <c r="D59" s="11" t="n"/>
@@ -2283,12 +2292,12 @@
     <row r="60" ht="32" customHeight="1">
       <c r="A60" s="13" t="inlineStr">
         <is>
-          <t>R-12</t>
+          <t>P1-09</t>
         </is>
       </c>
       <c r="B60" s="6" t="inlineStr">
         <is>
-          <t>家長控制：每日使用上限和休息時段</t>
+          <t>家長鎖：孩子模式進設定要輸入 PIN</t>
         </is>
       </c>
       <c r="C60" s="6" t="inlineStr">
@@ -2306,12 +2315,12 @@
     <row r="61" ht="32" customHeight="1">
       <c r="A61" s="13" t="inlineStr">
         <is>
-          <t>R-29</t>
+          <t>R-12</t>
         </is>
       </c>
       <c r="B61" s="6" t="inlineStr">
         <is>
-          <t>AI Buddy App（品牌 C）頁面</t>
+          <t>家長控制：每日使用上限和休息時段</t>
         </is>
       </c>
       <c r="C61" s="6" t="inlineStr">
@@ -2329,17 +2338,17 @@
     <row r="62" ht="32" customHeight="1">
       <c r="A62" s="13" t="inlineStr">
         <is>
-          <t>P2-25</t>
+          <t>R-29</t>
         </is>
       </c>
       <c r="B62" s="6" t="inlineStr">
         <is>
-          <t>C3 斷線後自救：TLS 握手超時縮短、連續失敗重設 Wi-Fi 或重開、修重試漏記憶體</t>
+          <t>AI Buddy App（品牌 C）頁面</t>
         </is>
       </c>
       <c r="C62" s="6" t="inlineStr">
         <is>
-          <t>等 P2-24</t>
+          <t>阻塞：[2026-10-13] 2026-10-13 用戶決定：AI Buddy（品牌 C）延到 1/15 之後，本項不卡 1/15 出廠；AI Buddy 啟動時再開。</t>
         </is>
       </c>
       <c r="D62" s="11" t="n"/>
@@ -3184,6 +3193,7 @@
   <mergeCells count="86">
     <mergeCell ref="C82:I82"/>
     <mergeCell ref="E52:I52"/>
+    <mergeCell ref="A56:I56"/>
     <mergeCell ref="E39:I39"/>
     <mergeCell ref="C67:I67"/>
     <mergeCell ref="E48:I48"/>
@@ -3226,22 +3236,23 @@
     <mergeCell ref="C75:I75"/>
     <mergeCell ref="C84:I84"/>
     <mergeCell ref="C80:I80"/>
+    <mergeCell ref="E54:I54"/>
     <mergeCell ref="E32:I32"/>
     <mergeCell ref="C59:I59"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="E41:I41"/>
+    <mergeCell ref="A45:I45"/>
     <mergeCell ref="E47:I47"/>
     <mergeCell ref="C61:I61"/>
+    <mergeCell ref="E43:I43"/>
     <mergeCell ref="C70:I70"/>
     <mergeCell ref="E24:I24"/>
     <mergeCell ref="E33:I33"/>
     <mergeCell ref="A3:I3"/>
-    <mergeCell ref="A55:I55"/>
     <mergeCell ref="A104:I104"/>
     <mergeCell ref="E35:I35"/>
     <mergeCell ref="C74:I74"/>
     <mergeCell ref="C88:I88"/>
-    <mergeCell ref="E45:I45"/>
     <mergeCell ref="E37:I37"/>
     <mergeCell ref="E21:I21"/>
     <mergeCell ref="E23:I23"/>
@@ -3259,12 +3270,10 @@
     <mergeCell ref="C64:I64"/>
     <mergeCell ref="C79:I79"/>
     <mergeCell ref="C73:I73"/>
-    <mergeCell ref="A44:I44"/>
     <mergeCell ref="E49:I49"/>
     <mergeCell ref="E27:I27"/>
     <mergeCell ref="E36:I36"/>
     <mergeCell ref="C63:I63"/>
-    <mergeCell ref="C56:I56"/>
     <mergeCell ref="C90:I90"/>
     <mergeCell ref="E53:I53"/>
     <mergeCell ref="C76:I76"/>
@@ -10451,7 +10460,7 @@
         </is>
       </c>
     </row>
-    <row r="98" ht="102" customHeight="1">
+    <row r="98" ht="200" customHeight="1">
       <c r="A98" s="13" t="inlineStr">
         <is>
           <t>P2-25</t>
@@ -10479,12 +10488,12 @@
       </c>
       <c r="F98" s="13" t="inlineStr">
         <is>
-          <t>未開始</t>
+          <t>進行中</t>
         </is>
       </c>
       <c r="G98" s="13" t="inlineStr">
         <is>
-          <t>未測試</t>
+          <t>部分通過</t>
         </is>
       </c>
       <c r="I98" s="6" t="inlineStr">
@@ -10499,7 +10508,7 @@
       </c>
       <c r="K98" s="6" t="inlineStr">
         <is>
-          <t>① websocket / HTTPS 的 TLS 握手超時約 15 秒（可調）② 連續 N 次（預設 5）連不上伺服器就重設 Wi-Fi 重連；再連續失敗就 ESP.restart()（試用期內的重開照 OTA 規則處理）③ 失敗的重連不再漏 heap：連續 50 次失敗前後 free heap 差 &lt; 1KB ④ 已綁定設備的正常斷網重連行為不變（R-36 ④）</t>
+          <t>① websocket / HTTPS 的 TLS 握手超時約 15 秒 ② Wi-Fi 在線但沒有開著的連線、也不是在等認領：累計 60 秒重設 Wi-Fi，3 分鐘靜默重開一次（同一次失聯只一次），之後每 60 秒重設 Wi-Fi ③ 失敗的重連不漏 heap：連續 50 次失敗前後差 &lt; 1KB ④ 已綁定設備的正常斷網重連行為不變</t>
         </is>
       </c>
       <c r="L98" s="6" t="inlineStr">
@@ -10512,9 +10521,20 @@
           <t>P2-24</t>
         </is>
       </c>
+      <c r="N98" s="6" t="inlineStr">
+        <is>
+          <t>62:70（2026-10-15，分支 p2-25-reconnect-recovery，1.7.7/1.7.8，wss 連 Mac 上只接受不回應的端口）：① 握手每 16 秒失敗一次（15s 超時 + 1s 重連；以前 121s），objdump 確認 WiFiClientSecure 兩處呼叫都經 __wrap ② 63s、129s 重設 Wi-Fi，193s 靜默重開（Chime: boot skipped），重開後只重設 Wi-Fi（63/127/191/240s），不再重開 ③ 3s 超時版 65 次失敗握手：heap 64,424 → 64,300（波動 64,068–64,504），無漏 ④ 健康連線 2 分鐘無誤判；語音伺服器停 40 秒，恢復後 1 秒內重連。測試中發現並修正兩個問題：token 200 曾清除失聯記錄（每 3 分鐘重開）；只看事件不看狀態曾在健康連線 60 秒後重設 Wi-Fi</t>
+        </is>
+      </c>
+      <c r="O98" s="13" t="inlineStr">
+        <is>
+          <t>dc5598a</t>
+        </is>
+      </c>
       <c r="P98" s="6" t="inlineStr">
         <is>
-          <t>[2026-10-15] 新增</t>
+          <t>[2026-10-15] 新增
+[2026-10-15] 改為按時間而非次數：websocket 函式庫連線失敗時不發事件。未做：③ 的 10/13 熱點漏記憶體情境未重現（本次測的是握手超時路徑）；雲端板在 iPhone 熱點實測斷線後 1 分鐘內恢復（等雲端可測）。分支未合併、未推送。</t>
         </is>
       </c>
     </row>
@@ -11100,7 +11120,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I321"/>
+  <dimension ref="A1:I322"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -22297,8 +22317,55 @@
         </is>
       </c>
     </row>
+    <row r="322" ht="172" customHeight="1">
+      <c r="A322" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-15 11:31</t>
+        </is>
+      </c>
+      <c r="B322" s="13" t="inlineStr">
+        <is>
+          <t>P2-25</t>
+        </is>
+      </c>
+      <c r="C322" s="6" t="inlineStr">
+        <is>
+          <t>C3 斷線後自救：TLS 握手超時縮短、連續失敗重設 Wi-Fi 或重開、修重試漏記憶體</t>
+        </is>
+      </c>
+      <c r="D322" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E322" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F322" s="13" t="inlineStr">
+        <is>
+          <t>部分通過</t>
+        </is>
+      </c>
+      <c r="G322" s="6" t="inlineStr">
+        <is>
+          <t>62:70（2026-10-15，分支 p2-25-reconnect-recovery，1.7.7/1.7.8，wss 連 Mac 上只接受不回應的端口）：① 握手每 16 秒失敗一次（15s 超時 + 1s 重連；以前 121s），objdump 確認 WiFiClientSecure 兩處呼叫都經 __wrap ② 63s、129s 重設 Wi-Fi，193s 靜默重開（Chime: boot skipped），重開後只重設 Wi-Fi（63/127/191/240s），不再重開 ③ 3s 超時版 65 次失敗握手：heap 64,424 → 64,300（波動 64,068–64,504），無漏 ④ 健康連線 2 分鐘無誤判；語音伺服器停 40 秒，恢復後 1 秒內重連。測試中發現並修正兩個問題：token 200 曾清除失聯記錄（每 3 分鐘重開）；只看事件不看狀態曾在健康連線 60 秒後重設 Wi-Fi</t>
+        </is>
+      </c>
+      <c r="H322" s="13" t="inlineStr">
+        <is>
+          <t>dc5598a</t>
+        </is>
+      </c>
+      <c r="I322" s="6" t="inlineStr">
+        <is>
+          <t>改為按時間而非次數：websocket 函式庫連線失敗時不發事件。未做：③ 的 10/13 熱點漏記憶體情境未重現（本次測的是握手超時路徑）；雲端板在 iPhone 熱點實測斷線後 1 分鐘內恢復（等雲端可測）。分支未合併、未推送。；修改了驗收標準</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I321"/>
+  <autoFilter ref="A1:I322"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Track P2-25: network feedback and setup fallback tested on 62:70.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/production-readiness.xlsx
+++ b/docs/production-readiness.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'任務清單'!$A$1:$P$98</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'待確認問題'!$A$1:$G$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$322</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$323</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -665,7 +665,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>最後更新：2026-10-15 11:31　·　本頁由 tracker.py 自動生成，請勿手動編輯</t>
+          <t>最後更新：2026-10-15 14:49　·　本頁由 tracker.py 自動生成，請勿手動編輯</t>
         </is>
       </c>
     </row>
@@ -1550,7 +1550,7 @@
       <c r="H31" s="11" t="n"/>
       <c r="I31" s="12" t="n"/>
     </row>
-    <row r="32" ht="270" customHeight="1">
+    <row r="32" ht="409" customHeight="1">
       <c r="A32" s="13" t="inlineStr">
         <is>
           <t>P2-25</t>
@@ -1573,8 +1573,8 @@
       </c>
       <c r="E32" s="6" t="inlineStr">
         <is>
-          <t>上次測試：部分通過 — 62:70（2026-10-15，分支 p2-25-reconnect-recovery，1.7.7/1.7.8，wss 連 Mac 上只接受不回應的端口）：① 握手每 16 秒失敗一次（15s 超時 + 1s 重連；以前 121s），objdump 確認 WiFiClientSecure 兩處呼叫都經 __wrap ② 63s、129s 重設 Wi-Fi，193s 靜默重開（Chime: boot skipped），重開後只重設 Wi-Fi（63/127/191/240s），不再重開 ③ 3s 超時版 65 次失敗握手：heap 64,424 → 64,300（波動 64,068–64,504），無漏 ④ 健康連線 2 分鐘無誤判；語音伺服器停 40 秒，恢復後 1 秒內重連。測試中發現並修正兩個問題：token 200 曾清除失聯記錄（每 3 分鐘重開）；只看事件不看狀態曾在健康連線 60 秒後重設 Wi-Fi
-① websocket / HTTPS 的 TLS 握手超時約 15 秒 ② Wi-Fi 在線但沒有開著的連線、也不是在等認領：累計 60 秒重設 Wi-Fi，3 分鐘靜默重開一次（同一次失聯只一次），之後每 60 秒重設 Wi-Fi ③ 失敗的重連不漏 heap：連續 50 次失敗前後差 &lt; 1KB ④ 已綁定設備的正常斷網重連行為不變</t>
+          <t>上次測試：部分通過 — 62:70（2026-10-15，hw-test-1015 1.8.1/1.8.2）：① 黑洞端口：開機音 → 8 秒 Chime: wifi_try（用戶：聽到「正在連接」、燈在閃，看似藍色）；63 秒『The internet answers and our server does not』→ 黃燈；192 秒靜默重開（boot skipped），修正後重開不再播 wifi_try ② 無互聯網版：63 秒 No internet through HKQF - Guest → 改試（熱點不在，回到 Guest）；128 秒 opening Wi-Fi setup → AP AIBuddy-6270 → Chime: wifi_no_ap、wifi_setup ③ 65 次失敗握手 heap 64,424 → 64,300 無漏 ④ 健康連線 2 分鐘無誤判；伺服器停 40 秒後 1 秒內重連；正常版開機即連上、不播 wifi_try。測試中修正四個問題：token 200 清除失聯記錄；只看事件不看狀態（健康連線被重設）；Audio.cpp 的 #include 只對降採樣板生效（S3 編譯失敗）；靜默重開後又播「正在連接」
+① websocket / HTTPS 的 TLS 握手超時約 15 秒 ② 失去連線超過 8 秒：燈青色慢閃，播一次「正在連接」（wifi_try；每次失聯一次，8 秒內連上不播）③ Wi-Fi 在線但到不了伺服器 60 秒：檢查互聯網（generate_204）。上不了網 → 先改試其他已存網絡一次，仍不行就打開配網（洋紅常亮，播「無法連接」＋「正在配網…」，最多每 10 分鐘一次）；上得了網 → 是我們伺服器掛了，不叫家長重設 Wi-Fi，燈黃色慢閃，自己重試，3 分鐘靜默重開一次（重開後不再播提示、不再重開）④ 失敗的重連不漏 heap：連續 50 次失敗前後差 &lt; 1KB ⑤ 已綁定設備的正常斷網重連行為不變，正常開機不多播提示 ⑥ 開機時附近沒有已存網絡而打開配網：播「正在配網…」（2026-10-15 用戶決定 ②③⑥）</t>
         </is>
       </c>
       <c r="F32" s="11" t="n"/>
@@ -10460,7 +10460,7 @@
         </is>
       </c>
     </row>
-    <row r="98" ht="200" customHeight="1">
+    <row r="98" ht="256" customHeight="1">
       <c r="A98" s="13" t="inlineStr">
         <is>
           <t>P2-25</t>
@@ -10508,12 +10508,12 @@
       </c>
       <c r="K98" s="6" t="inlineStr">
         <is>
-          <t>① websocket / HTTPS 的 TLS 握手超時約 15 秒 ② Wi-Fi 在線但沒有開著的連線、也不是在等認領：累計 60 秒重設 Wi-Fi，3 分鐘靜默重開一次（同一次失聯只一次），之後每 60 秒重設 Wi-Fi ③ 失敗的重連不漏 heap：連續 50 次失敗前後差 &lt; 1KB ④ 已綁定設備的正常斷網重連行為不變</t>
+          <t>① websocket / HTTPS 的 TLS 握手超時約 15 秒 ② 失去連線超過 8 秒：燈青色慢閃，播一次「正在連接」（wifi_try；每次失聯一次，8 秒內連上不播）③ Wi-Fi 在線但到不了伺服器 60 秒：檢查互聯網（generate_204）。上不了網 → 先改試其他已存網絡一次，仍不行就打開配網（洋紅常亮，播「無法連接」＋「正在配網…」，最多每 10 分鐘一次）；上得了網 → 是我們伺服器掛了，不叫家長重設 Wi-Fi，燈黃色慢閃，自己重試，3 分鐘靜默重開一次（重開後不再播提示、不再重開）④ 失敗的重連不漏 heap：連續 50 次失敗前後差 &lt; 1KB ⑤ 已綁定設備的正常斷網重連行為不變，正常開機不多播提示 ⑥ 開機時附近沒有已存網絡而打開配網：播「正在配網…」（2026-10-15 用戶決定 ②③⑥）</t>
         </is>
       </c>
       <c r="L98" s="6" t="inlineStr">
         <is>
-          <t>① 62:70：停掉語音伺服器 → 串口每次握手失敗 ≤ 15 秒，第 N 次後重設 Wi-Fi、再後重開，恢復伺服器後自動連上 ② 記錄 50 次失敗重連前後的 free heap ③ 雲端可測時在 iPhone 熱點重跑 10/13 情境，斷線後 1 分鐘內恢復對話</t>
+          <t>① 62:70 wss 連 Mac 上只接受不回應的端口（測試編譯開關 LOCAL_WS_TLS）：握手 ≤ 15 秒失敗；8 秒播 wifi_try、青色慢閃；60 秒判定「上得了網」→ 黃色慢閃；3 分鐘靜默重開，重開後不播提示、不再重開 ② 同上再加 INTERNET_PROBE_URL 指向不存在的地址：60 秒改試其他已存網絡，再 60 秒打開配網（洋紅），播 wifi_no_ap、wifi_setup ③ 3 秒超時版記錄 50 次失敗前後 heap ④ 停語音伺服器 40 秒再恢復 → 1 秒內重連、健康連線不誤判、正常開機不播 wifi_try ⑤ 用戶目視燈號、聽提示音 ⑥ 雲端可測時在 iPhone 熱點重跑 10/13 情境</t>
         </is>
       </c>
       <c r="M98" s="13" t="inlineStr">
@@ -10523,18 +10523,19 @@
       </c>
       <c r="N98" s="6" t="inlineStr">
         <is>
-          <t>62:70（2026-10-15，分支 p2-25-reconnect-recovery，1.7.7/1.7.8，wss 連 Mac 上只接受不回應的端口）：① 握手每 16 秒失敗一次（15s 超時 + 1s 重連；以前 121s），objdump 確認 WiFiClientSecure 兩處呼叫都經 __wrap ② 63s、129s 重設 Wi-Fi，193s 靜默重開（Chime: boot skipped），重開後只重設 Wi-Fi（63/127/191/240s），不再重開 ③ 3s 超時版 65 次失敗握手：heap 64,424 → 64,300（波動 64,068–64,504），無漏 ④ 健康連線 2 分鐘無誤判；語音伺服器停 40 秒，恢復後 1 秒內重連。測試中發現並修正兩個問題：token 200 曾清除失聯記錄（每 3 分鐘重開）；只看事件不看狀態曾在健康連線 60 秒後重設 Wi-Fi</t>
+          <t>62:70（2026-10-15，hw-test-1015 1.8.1/1.8.2）：① 黑洞端口：開機音 → 8 秒 Chime: wifi_try（用戶：聽到「正在連接」、燈在閃，看似藍色）；63 秒『The internet answers and our server does not』→ 黃燈；192 秒靜默重開（boot skipped），修正後重開不再播 wifi_try ② 無互聯網版：63 秒 No internet through HKQF - Guest → 改試（熱點不在，回到 Guest）；128 秒 opening Wi-Fi setup → AP AIBuddy-6270 → Chime: wifi_no_ap、wifi_setup ③ 65 次失敗握手 heap 64,424 → 64,300 無漏 ④ 健康連線 2 分鐘無誤判；伺服器停 40 秒後 1 秒內重連；正常版開機即連上、不播 wifi_try。測試中修正四個問題：token 200 清除失聯記錄；只看事件不看狀態（健康連線被重設）；Audio.cpp 的 #include 只對降採樣板生效（S3 編譯失敗）；靜默重開後又播「正在連接」</t>
         </is>
       </c>
       <c r="O98" s="13" t="inlineStr">
         <is>
-          <t>dc5598a</t>
+          <t>45961e4</t>
         </is>
       </c>
       <c r="P98" s="6" t="inlineStr">
         <is>
           <t>[2026-10-15] 新增
-[2026-10-15] 改為按時間而非次數：websocket 函式庫連線失敗時不發事件。未做：③ 的 10/13 熱點漏記憶體情境未重現（本次測的是握手超時路徑）；雲端板在 iPhone 熱點實測斷線後 1 分鐘內恢復（等雲端可測）。分支未合併、未推送。</t>
+[2026-10-15] 改為按時間而非次數：websocket 函式庫連線失敗時不發事件。未做：③ 的 10/13 熱點漏記憶體情境未重現（本次測的是握手超時路徑）；雲端板在 iPhone 熱點實測斷線後 1 分鐘內恢復（等雲端可測）。分支未合併、未推送。
+[2026-10-15] 未做：⑤ 用戶確認黃燈、洋紅燈和兩句配網提示；⑥ 雲端板在熱點實測；10/13 的熱點漏記憶體情境未重現。配網目前是『連接 AI Buddy 嘅熱點』，App 經藍牙配網等 R-21，屆時換提示錄音；『正在尋找網絡』錄音未有，暫用 wifi_try。分支 p2-25-reconnect-recovery 未合併、未推送。</t>
         </is>
       </c>
     </row>
@@ -11120,7 +11121,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I322"/>
+  <dimension ref="A1:I323"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -22364,8 +22365,55 @@
         </is>
       </c>
     </row>
+    <row r="323" ht="214" customHeight="1">
+      <c r="A323" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-15 14:49</t>
+        </is>
+      </c>
+      <c r="B323" s="13" t="inlineStr">
+        <is>
+          <t>P2-25</t>
+        </is>
+      </c>
+      <c r="C323" s="6" t="inlineStr">
+        <is>
+          <t>C3 斷線後自救：TLS 握手超時縮短、連續失敗重設 Wi-Fi 或重開、修重試漏記憶體</t>
+        </is>
+      </c>
+      <c r="D323" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="E323" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F323" s="13" t="inlineStr">
+        <is>
+          <t>部分通過</t>
+        </is>
+      </c>
+      <c r="G323" s="6" t="inlineStr">
+        <is>
+          <t>62:70（2026-10-15，hw-test-1015 1.8.1/1.8.2）：① 黑洞端口：開機音 → 8 秒 Chime: wifi_try（用戶：聽到「正在連接」、燈在閃，看似藍色）；63 秒『The internet answers and our server does not』→ 黃燈；192 秒靜默重開（boot skipped），修正後重開不再播 wifi_try ② 無互聯網版：63 秒 No internet through HKQF - Guest → 改試（熱點不在，回到 Guest）；128 秒 opening Wi-Fi setup → AP AIBuddy-6270 → Chime: wifi_no_ap、wifi_setup ③ 65 次失敗握手 heap 64,424 → 64,300 無漏 ④ 健康連線 2 分鐘無誤判；伺服器停 40 秒後 1 秒內重連；正常版開機即連上、不播 wifi_try。測試中修正四個問題：token 200 清除失聯記錄；只看事件不看狀態（健康連線被重設）；Audio.cpp 的 #include 只對降採樣板生效（S3 編譯失敗）；靜默重開後又播「正在連接」</t>
+        </is>
+      </c>
+      <c r="H323" s="13" t="inlineStr">
+        <is>
+          <t>45961e4</t>
+        </is>
+      </c>
+      <c r="I323" s="6" t="inlineStr">
+        <is>
+          <t>未做：⑤ 用戶確認黃燈、洋紅燈和兩句配網提示；⑥ 雲端板在熱點實測；10/13 的熱點漏記憶體情境未重現。配網目前是『連接 AI Buddy 嘅熱點』，App 經藍牙配網等 R-21，屆時換提示錄音；『正在尋找網絡』錄音未有，暫用 wifi_try。分支 p2-25-reconnect-recovery 未合併、未推送。；修改了驗收標準、測試方法</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I322"/>
+  <autoFilter ref="A1:I323"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Track P0-11 merged into dev; UAT needs DEVICE_CLAIM_LIST until the app can bind.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/production-readiness.xlsx
+++ b/docs/production-readiness.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'任務清單'!$A$1:$P$98</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'待確認問題'!$A$1:$G$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$323</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$324</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -665,7 +665,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>最後更新：2026-10-15 14:49　·　本頁由 tracker.py 自動生成，請勿手動編輯</t>
+          <t>最後更新：2026-10-15 21:46　·　本頁由 tracker.py 自動生成，請勿手動編輯</t>
         </is>
       </c>
     </row>
@@ -4281,7 +4281,8 @@
 [2026-10-12] 2026-10-12 用戶確認綁定設計：Spotpear 沒有螢幕、也不讀出配對碼（韌體只印在序列埠），所以改為配網時綁定；已有主人的設備要原主先解綁，否則找客服；第一版一台設備只屬一個帳號。現況漏洞仍在：設定頁列出全球未認領設備可直接認領（AppSettings.tsx、getUnclaimedDevices）；addUserToDevice 沒有檢查 user_id IS NULL，也不寫 claimed_at。
 [2026-10-12] 2026-10-12 再改：用戶決定用藍牙配網（R-21），不用熱點綁定碼。改為「App 取綁定票，經藍牙交給設備，設備自己認領」，本項只管伺服器端，不用等藍牙就能先做和測試。
 [2026-10-12] 伺服器端完成並在本機全部通過，未部署。注意：DEVICE_CLAIM_LIST 在生產預設關閉，部署後網頁不能再加新設備，要等 R-21 藍牙配網（或臨時在生產開 DEVICE_CLAIM_LIST）。分支以 mygithub/main（8db9d9c）為基礎；本機 main 落後且沒有 P1-12。
-[2026-10-12] 2026-10-12 用戶決定：P0-11 不單獨部署，等 R-21 藍牙配網做好後一起上線，避免生產網頁在中間這段時間不能加新設備。</t>
+[2026-10-12] 2026-10-12 用戶決定：P0-11 不單獨部署，等 R-21 藍牙配網做好後一起上線，避免生產網頁在中間這段時間不能加新設備。
+[2026-10-15] 2026-10-15 併入 dev（41be698，未推送）。dev 已刪舊設定頁，認領清單開關移到 Account/AddDevice.tsx：DEVICE_CLAIM_LIST 關閉時清單回 null、停止輪詢、提示用 App 加設備。合併後 pytest 293、tsc 0、node 19/19、pio 18 env 全過；本機 DB 以 BEGIN/ROLLBACK 重套 migration 無錯。部署注意：沒有藍牙 App（R-21）前 UAT 要設 DEVICE_CLAIM_LIST=True，否則無法加板。</t>
         </is>
       </c>
     </row>
@@ -11121,7 +11122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I323"/>
+  <dimension ref="A1:I324"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -22412,8 +22413,43 @@
         </is>
       </c>
     </row>
+    <row r="324" ht="158" customHeight="1">
+      <c r="A324" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-15 21:46</t>
+        </is>
+      </c>
+      <c r="B324" s="13" t="inlineStr">
+        <is>
+          <t>P0-11</t>
+        </is>
+      </c>
+      <c r="C324" s="6" t="inlineStr">
+        <is>
+          <t>設備認領要求持有證明</t>
+        </is>
+      </c>
+      <c r="D324" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="E324" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F324" s="13" t="n"/>
+      <c r="G324" s="6" t="n"/>
+      <c r="H324" s="13" t="n"/>
+      <c r="I324" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-15 併入 dev（41be698，未推送）。dev 已刪舊設定頁，認領清單開關移到 Account/AddDevice.tsx：DEVICE_CLAIM_LIST 關閉時清單回 null、停止輪詢、提示用 App 加設備。合併後 pytest 293、tsc 0、node 19/19、pio 18 env 全過；本機 DB 以 BEGIN/ROLLBACK 重套 migration 無錯。部署注意：沒有藍牙 App（R-21）前 UAT 要設 DEVICE_CLAIM_LIST=True，否則無法加板。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I323"/>
+  <autoFilter ref="A1:I324"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Prepare the handover: add HANDOVER.md, mark design and app-shell owners as unassigned.
Navy and Neo are off the project from 2026-10-22, so the roadmap, plan,
schedule, tracker and app-shell interface doc now name the design and
app-shell roles as 待定, and the admin preview data no longer names them.
docs/HANDOVER.md covers deployment, boards, branches and known traps.
launch.json gains the dev-server entries for the side worktrees.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/production-readiness.xlsx
+++ b/docs/production-readiness.xlsx
@@ -13,9 +13,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="更新記錄" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'任務清單'!$A$1:$P$98</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'任務清單'!$A$1:$P$101</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'待確認問題'!$A$1:$G$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$324</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'更新記錄'!$A$1:$I$338</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -641,7 +641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I105"/>
+  <dimension ref="A1:I109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -665,14 +665,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>最後更新：2026-10-15 21:46　·　本頁由 tracker.py 自動生成，請勿手動編輯</t>
+          <t>最後更新：2026-10-20 16:45　·　本頁由 tracker.py 自動生成，請勿手動編輯</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>總進度：25/93 已完成（27%）　·　目前階段：1 止血定案（10/5–10/16）</t>
+          <t>總進度：25/96 已完成（26%）　·　目前階段：1 止血定案（10/5–10/16）</t>
         </is>
       </c>
     </row>
@@ -856,7 +856,7 @@
       </c>
       <c r="C9" s="7">
         <f>COUNTIF('任務清單'!$B:$B,$A9)</f>
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="D9" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A9,'任務清單'!$F:$F,D$5)</f>
@@ -864,7 +864,7 @@
       </c>
       <c r="E9" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A9,'任務清單'!$F:$F,E$5)</f>
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="F9" s="7">
         <f>COUNTIFS('任務清單'!$B:$B,$A9,'任務清單'!$F:$F,F$5)</f>
@@ -880,7 +880,7 @@
       </c>
       <c r="I9" s="8">
         <f>IFERROR(F9/(C9-H9),0)</f>
-        <v>0.05128205128205128</v>
+        <v>0.047619047619047616</v>
       </c>
     </row>
     <row r="10">
@@ -892,7 +892,7 @@
       <c r="B10" s="6" t="n"/>
       <c r="C10" s="5">
         <f>SUM(C6:C9)</f>
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="D10" s="5">
         <f>SUM(D6:D9)</f>
@@ -900,7 +900,7 @@
       </c>
       <c r="E10" s="5">
         <f>SUM(E6:E9)</f>
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="F10" s="5">
         <f>SUM(F6:F9)</f>
@@ -916,7 +916,7 @@
       </c>
       <c r="I10" s="9">
         <f>IFERROR(F10/(C10-H10),0)</f>
-        <v>0.26881720430107525</v>
+        <v>0.2604166666666667</v>
       </c>
     </row>
     <row r="12">
@@ -1023,11 +1023,11 @@
       </c>
       <c r="D14" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A14,'任務清單'!$F:$F,D$12)</f>
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E14" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A14,'任務清單'!$F:$F,E$12)</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F14" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A14,'任務清單'!$F:$F,F$12)</f>
@@ -1059,15 +1059,15 @@
       </c>
       <c r="C15" s="7">
         <f>COUNTIF('任務清單'!$C:$C,$A15)</f>
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D15" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A15,'任務清單'!$F:$F,D$12)</f>
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E15" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A15,'任務清單'!$F:$F,E$12)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F15" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A15,'任務清單'!$F:$F,F$12)</f>
@@ -1099,7 +1099,7 @@
       </c>
       <c r="C16" s="7">
         <f>COUNTIF('任務清單'!$C:$C,$A16)</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D16" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A16,'任務清單'!$F:$F,D$12)</f>
@@ -1107,7 +1107,7 @@
       </c>
       <c r="E16" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A16,'任務清單'!$F:$F,E$12)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F16" s="7">
         <f>COUNTIFS('任務清單'!$C:$C,$A16,'任務清單'!$F:$F,F$12)</f>
@@ -1135,7 +1135,7 @@
       <c r="B17" s="6" t="n"/>
       <c r="C17" s="5">
         <f>SUM(C13:C16)</f>
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="D17" s="5">
         <f>SUM(D13:D16)</f>
@@ -1143,7 +1143,7 @@
       </c>
       <c r="E17" s="5">
         <f>SUM(E13:E16)</f>
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="F17" s="5">
         <f>SUM(F13:F16)</f>
@@ -1159,7 +1159,7 @@
       </c>
       <c r="I17" s="9">
         <f>IFERROR(F17/(C17-H17),0)</f>
-        <v>0.26881720430107525</v>
+        <v>0.2604166666666667</v>
       </c>
     </row>
     <row r="19">
@@ -1613,15 +1613,15 @@
       <c r="H33" s="11" t="n"/>
       <c r="I33" s="12" t="n"/>
     </row>
-    <row r="34" ht="172" customHeight="1">
+    <row r="34" ht="382" customHeight="1">
       <c r="A34" s="13" t="inlineStr">
         <is>
-          <t>R-36</t>
+          <t>R-25</t>
         </is>
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>未認領的設備停在配對狀態，不再每秒重連 websocket</t>
+          <t>網頁的品牌主題系統</t>
         </is>
       </c>
       <c r="C34" s="13" t="inlineStr">
@@ -1636,8 +1636,8 @@
       </c>
       <c r="E34" s="6" t="inlineStr">
         <is>
-          <t>上次測試：部分通過 — 補充 2026-10-15（1.7.5，含 R-36）：已綁定時兩次 Wi-Fi 切換各斷網 9–11 秒，都自動重連並重新 auth，沒有停在暫停狀態；30 秒斷網仍未做
-① 拿到 202 或 websocket 被 4401 拒絕後，設備停掉 websocket 自動重連，進入待綁定狀態（燈號可分辨）。② 待綁定時只按退避（5 秒起、上限 PROVISION_BACKOFF_MAX）呼叫 generate_auth_token，不開 websocket。③ 被認領後下一次輪詢拿到 200，在 10 秒內（加退避）自動開 websocket 並能對話，不用重開機。④ 已綁定設備網絡斷線重連的行為不變。⑤ 隨 OTA 推出。</t>
+          <t>上次測試：部分通過 — 分支 r-25-brand-themes（3e59883 + c6654ed，worktree aibuddy-brands）：同一個 next build 的 standalone server.js 以 BRAND=aibuddy/hkjc/genex 各啟動一次 → /login 標題『Login | AI Buddy／快活／GEN-EX』、SSR &lt;head&gt; 內 :root --brand-primary 各自不同（無閃爍）、標誌與標語對；cp -R genex zz-test 改 JSON、不改程式不重 build → 『Login | Test Brand』；BRAND=nope → 500 並記錄 brands/nope/brand.json does not exist；brand.json 填錯 → 500 並逐欄報錯。dev 實測 hkjc：設備預設名『快活』、中文加設備提示、無方案徽章、/home/account/child 404。grep 共用程式碼：無品牌名、無 AI Buddy 色值（剩韌體熱點前綴、JWT audience、seed 帳號等技術識別碼）。tsc 0 錯、next build 通過、node --test 22/22。未做：① 首頁、上手流程、角色頁的整頁品牌版本（只有文案、圖片、功能開關可按品牌）和圖片 logo，等設計負責人（待定）10/23 的設計；hkjc/genex 名稱、顏色、文案是佔位。
+① 每個品牌一個資料夾：主題 token（顏色、字體、圓角）、logo 和圖示、文案、功能開關；首頁、上手流程、角色頁可以有品牌版本，其餘頁面共用 ② 由部署的環境變數選品牌（每套部署一個品牌，見 R-34），伺服器端渲染的第一屏就是對的主題，不閃爍 ③ 共用元件裡沒有品牌名稱和寫死的品牌顏色 ④ 加一個品牌只需要加資料夾、設定和一套部署，不用改共用元件</t>
         </is>
       </c>
       <c r="F34" s="11" t="n"/>
@@ -1645,20 +1645,20 @@
       <c r="H34" s="11" t="n"/>
       <c r="I34" s="12" t="n"/>
     </row>
-    <row r="35" ht="228" customHeight="1">
+    <row r="35" ht="172" customHeight="1">
       <c r="A35" s="13" t="inlineStr">
         <is>
-          <t>P2-12</t>
+          <t>R-36</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>量產燒錄前加大 app 分區</t>
+          <t>未認領的設備停在配對狀態，不再每秒重連 websocket</t>
         </is>
       </c>
       <c r="C35" s="13" t="inlineStr">
         <is>
-          <t>3 封閉內測</t>
+          <t>2 內測準備</t>
         </is>
       </c>
       <c r="D35" s="13" t="inlineStr">
@@ -1668,8 +1668,8 @@
       </c>
       <c r="E35" s="6" t="inlineStr">
         <is>
-          <t>上次測試：部分通過 — 62:70（spotpear-ai-toy-p212 原型，現已併入 spotpear-ai-toy）：① 本機 OTA 1.6.1→1.6.2 寫入新 app1，120s 後 confirmed ② 3 秒 abort 的 1.6.3 → PANIC → 回到 1.6.2，ota_failed_version=1.6.3 ③ 崩潰寫入 coredump 14.8KB ④ 資源分區 9 個聲音 504KB/2MB，開機 CRC 63ms，OTA 後照常；損壞/清空 → 退回內建聲音無崩潰 ⑤ pio 全部 18 個 env 編譯通過，映像都在各自 app 槽內（Spotpear 4 個 1.59–1.60MB / 4MB；其他板仍 2MB 槽）；R-21 藍牙探針版 2,326,128 bytes &lt; 4MB ⑥ release_firmware.py 映像 &gt; app 槽即拒發。未做：雲端 OTA 一次（等上 UAT）、出廠腳本寫入資源包（R-10）
-新分區表（例如 app0/app1 各 4MB，保留 nvs/otadata 位置）在出廠前定案並寫入出廠腳本；OTA 與回滾在新分區表上照常</t>
+          <t>上次測試：部分通過 — 補充 2026-10-15（1.7.5，含 R-36）：已綁定時兩次 Wi-Fi 切換各斷網 9–11 秒，都自動重連並重新 auth，沒有停在暫停狀態；30 秒斷網仍未做
+① 拿到 202 或 websocket 被 4401 拒絕後，設備停掉 websocket 自動重連，進入待綁定狀態（燈號可分辨）。② 待綁定時只按退避（5 秒起、上限 PROVISION_BACKOFF_MAX）呼叫 generate_auth_token，不開 websocket。③ 被認領後下一次輪詢拿到 200，在 10 秒內（加退避）自動開 websocket 並能對話，不用重開機。④ 已綁定設備網絡斷線重連的行為不變。⑤ 隨 OTA 推出。</t>
         </is>
       </c>
       <c r="F35" s="11" t="n"/>
@@ -1677,15 +1677,15 @@
       <c r="H35" s="11" t="n"/>
       <c r="I35" s="12" t="n"/>
     </row>
-    <row r="36" ht="409" customHeight="1">
+    <row r="36" ht="228" customHeight="1">
       <c r="A36" s="13" t="inlineStr">
         <is>
-          <t>P2-22</t>
+          <t>P2-12</t>
         </is>
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>改服務器網址也不失聯：語音網址由後端下發、後端網址可遷移、已確認韌體長期連不上時自救</t>
+          <t>量產燒錄前加大 app 分區</t>
         </is>
       </c>
       <c r="C36" s="13" t="inlineStr">
@@ -1700,8 +1700,8 @@
       </c>
       <c r="E36" s="6" t="inlineStr">
         <is>
-          <t>上次測試：部分通過 — 後端部分（分支 p2-22-server-urls）：node --test lib/deviceServerUrls.test.mjs 5/5、tsc 0 錯誤。worktree dev server 3222 + 本機 Supabase，兩塊假板（02:22:…:01/02）：已認領 200 帶 voice_url + backend_url；未認領 202 只帶 backend_url；DEVICE_VOICE_URL=ws://fastapi:7860/… → 不發、日誌記錯誤；兩個變數都不設 → 兩個欄位都不帶；生產值 → wss://elatoai.hkqft.com/fastapi/ws/esp32、https://elatoai.hkqft.com。測試數據已清除
-① /api/generate_auth_token 的回應帶 voice_url（wss 主機＋端口＋路徑，來自後端環境變數）；韌體用它連 /ws，並把最後一次成功的值存進 NVS；改 FastAPI 網址只改伺服器設定，不需新韌體 ② 回應沒有 voice_url（舊後端）或新網址連不上時，退回 NVS 上次成功的值，再退回出廠／編譯時的預設值 ③ 後端網址可遷移：回應可帶 backend_url；韌體先存為候選，下次開機用新網址取 token 成功才正式替換，失敗就繼續用舊網址；舊網址在遷移期內保持可用（runbook 寫明保留多久） ④ 已確認的韌體若連續 N 次開機（預設 10 次、跨度至少 24 小時，計數存 NVS）Wi-Fi 已拿到 IP 卻取不到 token：先依次試 NVS、出廠的後端網址；仍失敗且另一個槽可用，就切到另一個槽一次，並在下次連上時把本版本報為失敗 ⑤ 純斷網（拿不到 IP、路由器沒外網）不計入 ④ ⑥ 新網址的證書必須鏈到 CF_CA_bundle 裡的根（GTS Root R4、ISRG Root X1）；換主機或離開 Cloudflare 前先查證書鏈，runbook 寫明 ⑦ 只接受 https 的 backend_url 和 wss 的 voice_url，主機須在韌體內允許的網域後綴之下，防止後端被冒充時把板子引去別處</t>
+          <t>上次測試：部分通過 — 62:70（spotpear-ai-toy-p212 原型，現已併入 spotpear-ai-toy）：① 本機 OTA 1.6.1→1.6.2 寫入新 app1，120s 後 confirmed ② 3 秒 abort 的 1.6.3 → PANIC → 回到 1.6.2，ota_failed_version=1.6.3 ③ 崩潰寫入 coredump 14.8KB ④ 資源分區 9 個聲音 504KB/2MB，開機 CRC 63ms，OTA 後照常；損壞/清空 → 退回內建聲音無崩潰 ⑤ pio 全部 18 個 env 編譯通過，映像都在各自 app 槽內（Spotpear 4 個 1.59–1.60MB / 4MB；其他板仍 2MB 槽）；R-21 藍牙探針版 2,326,128 bytes &lt; 4MB ⑥ release_firmware.py 映像 &gt; app 槽即拒發。未做：雲端 OTA 一次（等上 UAT）、出廠腳本寫入資源包（R-10）
+新分區表（例如 app0/app1 各 4MB，保留 nvs/otadata 位置）在出廠前定案並寫入出廠腳本；OTA 與回滾在新分區表上照常</t>
         </is>
       </c>
       <c r="F36" s="11" t="n"/>
@@ -1709,15 +1709,15 @@
       <c r="H36" s="11" t="n"/>
       <c r="I36" s="12" t="n"/>
     </row>
-    <row r="37" ht="340" customHeight="1">
+    <row r="37" ht="409" customHeight="1">
       <c r="A37" s="13" t="inlineStr">
         <is>
-          <t>R-37</t>
+          <t>P2-22</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>網頁設定玩具的 Wi-Fi：查看、新增、刪除</t>
+          <t>改服務器網址也不失聯：語音網址由後端下發、後端網址可遷移、已確認韌體長期連不上時自救</t>
         </is>
       </c>
       <c r="C37" s="13" t="inlineStr">
@@ -1732,8 +1732,8 @@
       </c>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>上次測試：部分通過 — 62:70（1.7.4/1.7.5，2026-10-15）：① 熱點關掉後醒來改連 HKQF - Guest 並上線（發生在醒來重開時）⑦ Use 按鈕、確認框、『Moving to…』；熱點關著時按 Use → 11 秒內頁面顯示『couldn't find lee’s iPhone nearby. It's back on HKQF - Guest』，串口 not_found → Back on Guest → 重連。過程中發現並修正：驅動殘留上一次的『找不到』令連回原網絡立即失敗並掉進 SoftAP（joinFor 6 秒內不信失敗，tryConnect 同用）。pytest 272 passed
-① 設定頁顯示玩具在線／離線、目前 Wi-Fi 和訊號、已記住的 Wi-Fi 清單（只有名稱，不顯示密碼）② 在線時可新增 Wi-Fi（輸入或從玩具掃描到的清單選）、刪除 Wi-Fi；不能刪除正在使用的那個 ③ 經 /ws/esp32 轉送：伺服器先確認是設備主人；密碼不寫入資料庫、不寫入日誌 ④ 新增不自動切換網絡；目前 Wi-Fi 消失時按訊號選，或由家長按「改用這個」（⑦）；清單標示「連過／未連過」⑤ 上限 8 個 ⑥ 韌體改動經 OTA 推出 ⑦ 已記住、未在使用的 Wi-Fi 可按「改用這個」：玩具斷開目前網絡改連它，最多 20 秒，要連上我們的伺服器才算成功；失敗就自動連回原網絡，頁面顯示「連不上 X，已回到 Y」；切換中頁面顯示切換中，玩具重新連上後刷新；成功後標示連過</t>
+          <t>上次測試：部分通過 — 後端部分（分支 p2-22-server-urls）：node --test lib/deviceServerUrls.test.mjs 5/5、tsc 0 錯誤。worktree dev server 3222 + 本機 Supabase，兩塊假板（02:22:…:01/02）：已認領 200 帶 voice_url + backend_url；未認領 202 只帶 backend_url；DEVICE_VOICE_URL=ws://fastapi:7860/… → 不發、日誌記錯誤；兩個變數都不設 → 兩個欄位都不帶；生產值 → wss://elatoai.hkqft.com/fastapi/ws/esp32、https://elatoai.hkqft.com。測試數據已清除
+① /api/generate_auth_token 的回應帶 voice_url（wss 主機＋端口＋路徑，來自後端環境變數）；韌體用它連 /ws，並把最後一次成功的值存進 NVS；改 FastAPI 網址只改伺服器設定，不需新韌體 ② 回應沒有 voice_url（舊後端）或新網址連不上時，退回 NVS 上次成功的值，再退回出廠／編譯時的預設值 ③ 後端網址可遷移：回應可帶 backend_url；韌體先存為候選，下次開機用新網址取 token 成功才正式替換，失敗就繼續用舊網址；舊網址在遷移期內保持可用（runbook 寫明保留多久） ④ 已確認的韌體若連續 N 次開機（預設 10 次、跨度至少 24 小時，計數存 NVS）Wi-Fi 已拿到 IP 卻取不到 token：先依次試 NVS、出廠的後端網址；仍失敗且另一個槽可用，就切到另一個槽一次，並在下次連上時把本版本報為失敗 ⑤ 純斷網（拿不到 IP、路由器沒外網）不計入 ④ ⑥ 新網址的證書必須鏈到 CF_CA_bundle 裡的根（GTS Root R4、ISRG Root X1）；換主機或離開 Cloudflare 前先查證書鏈，runbook 寫明 ⑦ 只接受 https 的 backend_url 和 wss 的 voice_url，主機須在韌體內允許的網域後綴之下，防止後端被冒充時把板子引去別處</t>
         </is>
       </c>
       <c r="F37" s="11" t="n"/>
@@ -1741,30 +1741,31 @@
       <c r="H37" s="11" t="n"/>
       <c r="I37" s="12" t="n"/>
     </row>
-    <row r="38" ht="102" customHeight="1">
+    <row r="38" ht="340" customHeight="1">
       <c r="A38" s="13" t="inlineStr">
         <is>
-          <t>R-16</t>
+          <t>R-37</t>
         </is>
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>Spotpear 量產版加電池電壓檢測（GPIO0 分壓）</t>
+          <t>網頁設定玩具的 Wi-Fi：查看、新增、刪除</t>
         </is>
       </c>
       <c r="C38" s="13" t="inlineStr">
         <is>
-          <t>1 止血定案</t>
+          <t>3 封閉內測</t>
         </is>
       </c>
       <c r="D38" s="13" t="inlineStr">
         <is>
-          <t>未開始</t>
+          <t>進行中</t>
         </is>
       </c>
       <c r="E38" s="6" t="inlineStr">
         <is>
-          <t>Spotpear 書面確認量產版：GPIO1（屏幕 DC；本版不接屏幕，可空出來）接電芯正極（保護 IC 之後）100k/100k 分壓、100nF 濾波，屏幕不接該腳；GPIO0 保留給現有的 VDD 低電提醒；最好另把充電芯片 CHRG 接到 GPIO12 或 13。樣板到手後，固件讀到的電芯電壓與萬用表相差 ≤50mV，App（R-41）顯示百分比與充電中。</t>
+          <t>上次測試：部分通過 — 62:70（1.7.4/1.7.5，2026-10-15）：① 熱點關掉後醒來改連 HKQF - Guest 並上線（發生在醒來重開時）⑦ Use 按鈕、確認框、『Moving to…』；熱點關著時按 Use → 11 秒內頁面顯示『couldn't find lee’s iPhone nearby. It's back on HKQF - Guest』，串口 not_found → Back on Guest → 重連。過程中發現並修正：驅動殘留上一次的『找不到』令連回原網絡立即失敗並掉進 SoftAP（joinFor 6 秒內不信失敗，tryConnect 同用）。pytest 272 passed
+① 設定頁顯示玩具在線／離線、目前 Wi-Fi 和訊號、已記住的 Wi-Fi 清單（只有名稱，不顯示密碼）② 在線時可新增 Wi-Fi（輸入或從玩具掃描到的清單選）、刪除 Wi-Fi；不能刪除正在使用的那個 ③ 經 /ws/esp32 轉送：伺服器先確認是設備主人；密碼不寫入資料庫、不寫入日誌 ④ 新增不自動切換網絡；目前 Wi-Fi 消失時按訊號選，或由家長按「改用這個」（⑦）；清單標示「連過／未連過」⑤ 上限 8 個 ⑥ 韌體改動經 OTA 推出 ⑦ 已記住、未在使用的 Wi-Fi 可按「改用這個」：玩具斷開目前網絡改連它，最多 20 秒，要連上我們的伺服器才算成功；失敗就自動連回原網絡，頁面顯示「連不上 X，已回到 Y」；切換中頁面顯示切換中，玩具重新連上後刷新；成功後標示連過</t>
         </is>
       </c>
       <c r="F38" s="11" t="n"/>
@@ -1772,30 +1773,31 @@
       <c r="H38" s="11" t="n"/>
       <c r="I38" s="12" t="n"/>
     </row>
-    <row r="39" ht="46" customHeight="1">
+    <row r="39" ht="326" customHeight="1">
       <c r="A39" s="13" t="inlineStr">
         <is>
-          <t>P1-11</t>
+          <t>R-42</t>
         </is>
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>伺服器與資料庫直接存取的管控</t>
+          <t>Tool call v1：調音量、結束對話</t>
         </is>
       </c>
       <c r="C39" s="13" t="inlineStr">
         <is>
-          <t>2 內測準備</t>
+          <t>3 封閉內測</t>
         </is>
       </c>
       <c r="D39" s="13" t="inlineStr">
         <is>
-          <t>未開始</t>
+          <t>進行中</t>
         </is>
       </c>
       <c r="E39" s="6" t="inlineStr">
         <is>
-          <t>列出誰有 SSH 與資料庫直連權限（越少越好）；service_role key 只存在伺服器的 env；私隱政策寫明這類存取的範圍；每次直接查看生產資料都留記錄。</t>
+          <t>上次測試：部分通過 — 分支 tool-call-rag（e80784b、f24b809、f90a657，worktree aibuddy-tools）：evals/voice_tools 真實模型、伺服器提示詞同工具定義，每案 ×3：調音量 gemma 60/60、DeepSeek 59/60；結束對話 gemma 30/30＋50/50、DeepSeek 30/30＋49/50（唯一失敗係 DeepSeek 空回覆）；誤觸發 0/144（電視、鄰居、媽媽話我大聲、故事入面講拜拜等）。首字延遲：gemma 無增加（p50 856 vs 871ms），DeepSeek +150ms。本機端到端（simulate_device，Sinji 粵語錄音，7895 worktree 伺服器）：『你大聲啲啦』→ volume+auth 喺 RESPONSE.CREATED 前、70→85、devices.volume=85；『拜拜，我要瞓覺喇』→ 道別後 1.5s SESSION.END；記憶記錄三輪都正確。DeepSeek 先講『等我查吓先』再查：RESPONSE.COMPLETE 延後到答案講完（一個週期 22–33s 音頻）。pytest 325 passed。未做：真機 62:70 每個工具真實語音 20 次、合併 dev、部署。
+① 兩個工具各用真實語音在玩具上觸發 20 次，成功率 ≥ 95% ② 不相關的話（其他嘢好大聲、故事入面講拜拜等）不會誤觸發 ③ 首字延遲增加不超過 300 毫秒 ④ 1.0.1 同新固件都即時變音量，網頁音量同步 ⑤ 道別講完先瞓覺，用戶再講嘢就取消 ⑥ 工具輪嘅記憶記錄正確</t>
         </is>
       </c>
       <c r="F39" s="11" t="n"/>
@@ -1803,30 +1805,31 @@
       <c r="H39" s="11" t="n"/>
       <c r="I39" s="12" t="n"/>
     </row>
-    <row r="40" ht="46" customHeight="1">
+    <row r="40" ht="200" customHeight="1">
       <c r="A40" s="13" t="inlineStr">
         <is>
-          <t>P2-02</t>
+          <t>R-43</t>
         </is>
       </c>
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>CI 跑測試與靜態檢查</t>
+          <t>快活知識庫 RAG v1（檢索與回答）</t>
         </is>
       </c>
       <c r="C40" s="13" t="inlineStr">
         <is>
-          <t>2 內測準備</t>
+          <t>4 量產出貨</t>
         </is>
       </c>
       <c r="D40" s="13" t="inlineStr">
         <is>
-          <t>未開始</t>
+          <t>進行中</t>
         </is>
       </c>
       <c r="E40" s="6" t="inlineStr">
         <is>
-          <t>推送與 PR 時跑 pytest、ruff、pyright、next lint、tsc --noEmit、pio run；任何一項失敗就不發佈 image。</t>
+          <t>上次測試：部分通過 — BM25 檢索搬入伺服器（knowledge.py），KNOWLEDGE_BASE_FILE 指定，工具描述、查唔到嘅回覆、額外規則（唔畀貼士）都喺資料檔。用 13 條示範資料：evals/voice_tools 命中題 gemma 答對事實 12/12、DeepSeek 11–12/12；查唔到 → 固定句或者講唔清楚，冇自己作；貼士三題兩個模型都婉拒。已知問題：部分命中（沙田馬場有冇餐廳）DeepSeek 3 次有 2 次用自己知識補充（『係有餐廳㗎』），gemma 冇。未做：馬會資料、設計負責人（待定）100 條測試問題、MIN_SCORE 重新量、入庫審批流程。
+① v1 只放第一批馬會資料；設計負責人（待定）寫嘅 100 條測試問題答對率 ≥ 80% ② 知識庫冇嘅內容講唔肯定並建議查詢，唔自己作 ③ 問貼士、賠率、賽果預測 100% 婉拒 ④ 更新知識庫唔使重新燒錄玩具</t>
         </is>
       </c>
       <c r="F40" s="11" t="n"/>
@@ -1834,20 +1837,20 @@
       <c r="H40" s="11" t="n"/>
       <c r="I40" s="12" t="n"/>
     </row>
-    <row r="41" ht="32" customHeight="1">
+    <row r="41" ht="102" customHeight="1">
       <c r="A41" s="13" t="inlineStr">
         <is>
-          <t>P2-04</t>
+          <t>R-16</t>
         </is>
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>容器改用非 root 用戶</t>
+          <t>Spotpear 量產版加電池電壓檢測（GPIO0 分壓）</t>
         </is>
       </c>
       <c r="C41" s="13" t="inlineStr">
         <is>
-          <t>2 內測準備</t>
+          <t>1 止血定案</t>
         </is>
       </c>
       <c r="D41" s="13" t="inlineStr">
@@ -1857,7 +1860,7 @@
       </c>
       <c r="E41" s="6" t="inlineStr">
         <is>
-          <t>兩個 Dockerfile 都設定非 root 的 USER。</t>
+          <t>Spotpear 書面確認量產版：GPIO1（屏幕 DC；本版不接屏幕，可空出來）接電芯正極（保護 IC 之後）100k/100k 分壓、100nF 濾波，屏幕不接該腳；GPIO0 保留給現有的 VDD 低電提醒；最好另把充電芯片 CHRG 接到 GPIO12 或 13。樣板到手後，固件讀到的電芯電壓與萬用表相差 ≤50mV，App（R-41）顯示百分比與充電中。</t>
         </is>
       </c>
       <c r="F41" s="11" t="n"/>
@@ -1868,12 +1871,12 @@
     <row r="42" ht="46" customHeight="1">
       <c r="A42" s="13" t="inlineStr">
         <is>
-          <t>R-04</t>
+          <t>P1-11</t>
         </is>
       </c>
       <c r="B42" s="6" t="inlineStr">
         <is>
-          <t>粵語質量評測</t>
+          <t>伺服器與資料庫直接存取的管控</t>
         </is>
       </c>
       <c r="C42" s="13" t="inlineStr">
@@ -1888,7 +1891,7 @@
       </c>
       <c r="E42" s="6" t="inlineStr">
         <is>
-          <t>有一套粵語評測集（兒童錄音＋文字提示）；選定的 STT 與 LLM 達到門檻：兒童語音字錯率 ≤15%、口語粵語回覆 ≥90%、中英夾雜句能正確理解。</t>
+          <t>列出誰有 SSH 與資料庫直連權限（越少越好）；service_role key 只存在伺服器的 env；私隱政策寫明這類存取的範圍；每次直接查看生產資料都留記錄。</t>
         </is>
       </c>
       <c r="F42" s="11" t="n"/>
@@ -1896,15 +1899,15 @@
       <c r="H42" s="11" t="n"/>
       <c r="I42" s="12" t="n"/>
     </row>
-    <row r="43" ht="116" customHeight="1">
+    <row r="43" ht="46" customHeight="1">
       <c r="A43" s="13" t="inlineStr">
         <is>
-          <t>R-25</t>
+          <t>P2-02</t>
         </is>
       </c>
       <c r="B43" s="6" t="inlineStr">
         <is>
-          <t>網頁的品牌主題系統</t>
+          <t>CI 跑測試與靜態檢查</t>
         </is>
       </c>
       <c r="C43" s="13" t="inlineStr">
@@ -1919,7 +1922,7 @@
       </c>
       <c r="E43" s="6" t="inlineStr">
         <is>
-          <t>① 每個品牌一個資料夾：主題 token（顏色、字體、圓角）、logo 和圖示、文案、功能開關；首頁、上手流程、角色頁可以有品牌版本，其餘頁面共用 ② 由部署的環境變數選品牌（每套部署一個品牌，見 R-34），伺服器端渲染的第一屏就是對的主題，不閃爍 ③ 共用元件裡沒有品牌名稱和寫死的品牌顏色 ④ 加一個品牌只需要加資料夾、設定和一套部署，不用改共用元件</t>
+          <t>推送與 PR 時跑 pytest、ruff、pyright、next lint、tsc --noEmit、pio run；任何一項失敗就不發佈 image。</t>
         </is>
       </c>
       <c r="F43" s="11" t="n"/>
@@ -1927,37 +1930,92 @@
       <c r="H43" s="11" t="n"/>
       <c r="I43" s="12" t="n"/>
     </row>
-    <row r="45">
-      <c r="A45" s="10" t="inlineStr">
-        <is>
-          <t>✅ 最近完成與測試效果</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="4" t="inlineStr">
-        <is>
-          <t>編號</t>
-        </is>
-      </c>
-      <c r="B46" s="4" t="inlineStr">
-        <is>
-          <t>任務</t>
-        </is>
-      </c>
-      <c r="C46" s="4" t="inlineStr">
-        <is>
-          <t>測試結果</t>
-        </is>
-      </c>
-      <c r="D46" s="4" t="inlineStr">
-        <is>
-          <t>完成日期</t>
-        </is>
-      </c>
-      <c r="E46" s="4" t="inlineStr">
-        <is>
-          <t>測試證據</t>
+    <row r="44" ht="32" customHeight="1">
+      <c r="A44" s="13" t="inlineStr">
+        <is>
+          <t>P2-04</t>
+        </is>
+      </c>
+      <c r="B44" s="6" t="inlineStr">
+        <is>
+          <t>容器改用非 root 用戶</t>
+        </is>
+      </c>
+      <c r="C44" s="13" t="inlineStr">
+        <is>
+          <t>2 內測準備</t>
+        </is>
+      </c>
+      <c r="D44" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E44" s="6" t="inlineStr">
+        <is>
+          <t>兩個 Dockerfile 都設定非 root 的 USER。</t>
+        </is>
+      </c>
+      <c r="F44" s="11" t="n"/>
+      <c r="G44" s="11" t="n"/>
+      <c r="H44" s="11" t="n"/>
+      <c r="I44" s="12" t="n"/>
+    </row>
+    <row r="45" ht="46" customHeight="1">
+      <c r="A45" s="13" t="inlineStr">
+        <is>
+          <t>R-04</t>
+        </is>
+      </c>
+      <c r="B45" s="6" t="inlineStr">
+        <is>
+          <t>粵語質量評測</t>
+        </is>
+      </c>
+      <c r="C45" s="13" t="inlineStr">
+        <is>
+          <t>2 內測準備</t>
+        </is>
+      </c>
+      <c r="D45" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E45" s="6" t="inlineStr">
+        <is>
+          <t>有一套粵語評測集（兒童錄音＋文字提示）；選定的 STT 與 LLM 達到門檻：兒童語音字錯率 ≤15%、口語粵語回覆 ≥90%、中英夾雜句能正確理解。</t>
+        </is>
+      </c>
+      <c r="F45" s="11" t="n"/>
+      <c r="G45" s="11" t="n"/>
+      <c r="H45" s="11" t="n"/>
+      <c r="I45" s="12" t="n"/>
+    </row>
+    <row r="46" ht="102" customHeight="1">
+      <c r="A46" s="13" t="inlineStr">
+        <is>
+          <t>R-26</t>
+        </is>
+      </c>
+      <c r="B46" s="6" t="inlineStr">
+        <is>
+          <t>原生殼與網頁的橋接清單</t>
+        </is>
+      </c>
+      <c r="C46" s="13" t="inlineStr">
+        <is>
+          <t>2 內測準備</t>
+        </is>
+      </c>
+      <c r="D46" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E46" s="6" t="inlineStr">
+        <is>
+          <t>① docs/app-bridge.md 列出每項能力的 JS 介面、參數、回傳和錯誤：藍牙配網與綁定（R-21：掃描、Wi-Fi 清單、送 SSID／密碼／綁定票）、原生 Google／Apple 登入回傳 id token、推送 token 登記、麥克風權限、App 內刪除帳號入口、深層連結、殼告訴網頁自己的品牌和版本 ② 做殼的同事確認 ③ 偵測不到殼時（普通瀏覽器），每項都有替代做法或明確提示</t>
         </is>
       </c>
       <c r="F46" s="11" t="n"/>
@@ -1965,92 +2023,37 @@
       <c r="H46" s="11" t="n"/>
       <c r="I46" s="12" t="n"/>
     </row>
-    <row r="47" ht="88" customHeight="1">
-      <c r="A47" s="13" t="inlineStr">
-        <is>
-          <t>P2-21</t>
-        </is>
-      </c>
-      <c r="B47" s="6" t="inlineStr">
-        <is>
-          <t>P2-16 ⑤ 後台 OTA 頁換成真實數據與操作</t>
-        </is>
-      </c>
-      <c r="C47" s="13" t="inlineStr">
-        <is>
-          <t>通過</t>
-        </is>
-      </c>
-      <c r="D47" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
-      <c r="E47" s="6" t="inlineStr">
-        <is>
-          <t>10-14 模擬 20 台全部通過（見上次）；2026-10-15 真機補做：OTA 頁對 1.7.1 白名單加 62:70（UI MAC 欄）→ 存檔確認框 → 『Narrow to Whitelist』確認 → Make current（用戶點）→ 62:70 安裝並確認，頁面顯示 Rolling out · Whitelist、運行 1、回滾 0；每步一筆審計。依賴 P2-14 已完成</t>
-        </is>
-      </c>
-      <c r="F47" s="11" t="n"/>
-      <c r="G47" s="11" t="n"/>
-      <c r="H47" s="11" t="n"/>
-      <c r="I47" s="12" t="n"/>
-    </row>
-    <row r="48" ht="158" customHeight="1">
-      <c r="A48" s="13" t="inlineStr">
-        <is>
-          <t>P2-16</t>
-        </is>
-      </c>
-      <c r="B48" s="6" t="inlineStr">
-        <is>
-          <t>OTA 分批推送與後台發佈頁</t>
-        </is>
-      </c>
-      <c r="C48" s="13" t="inlineStr">
-        <is>
-          <t>通過</t>
-        </is>
-      </c>
-      <c r="D48" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
-      <c r="E48" s="6" t="inlineStr">
-        <is>
-          <t>④ 真機 62:70（2026-10-15）：USB 刷 1.7.0（開機印 aibuddy-build;kind=dev;…;version=1.7.0）→ release_firmware.py publish --dev 1.7.1 → 後台白名單加 62:70、改白名單階段、設為 current → 按 BOOT 喚醒：取 token 200、下載 12.8s、重開進 app1，09:39:36 連上語音伺服器；09:42 重開 → 『Firmware 1.7.1 on app1』無 probation、Up to date；頁面『Rolling out · Whitelist』運行 1 台、回滾 0；審計 5 筆（發佈、白名單、階段、1.6.2 取消 current、1.7.1 設 current）。①②③⑤ 見 P2-17～P2-21 模擬 20 台</t>
-        </is>
-      </c>
-      <c r="F48" s="11" t="n"/>
-      <c r="G48" s="11" t="n"/>
-      <c r="H48" s="11" t="n"/>
-      <c r="I48" s="12" t="n"/>
-    </row>
-    <row r="49" ht="144" customHeight="1">
-      <c r="A49" s="13" t="inlineStr">
-        <is>
-          <t>P2-14</t>
-        </is>
-      </c>
-      <c r="B49" s="6" t="inlineStr">
-        <is>
-          <t>Admin 設備頁：每台玩具的狀態、韌體與基本操作</t>
-        </is>
-      </c>
-      <c r="C49" s="13" t="inlineStr">
-        <is>
-          <t>通過</t>
-        </is>
-      </c>
-      <c r="D49" s="13" t="inlineStr">
-        <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
-      <c r="E49" s="6" t="inlineStr">
-        <is>
-          <t>真機 62:70（2026-10-15，分支 hw-test-1015 = dev+P2-16，-localall 1.7.0，本機網頁 3230 + 語音 7870）：① 開機 → 設備頁 Online、-67 dBm、1.7.0；板子停在 bootloader 約 38 秒後語音伺服器判離線（uvicorn ping 超時），頁面 0 台在線 ② 重置設備密鑰 → device_secrets 行刪除，板子重開印『Device secret issued and stored』並連上，行恢復 ③ 強制解綁 → 板子拿 202（配對碼 UKDM7N），語音伺服器拒絕連線；兩項審計各 1 筆含操作者與原因 ④ 內容管理員/anon → 42501（10-14 探測腳本）</t>
+    <row r="48">
+      <c r="A48" s="10" t="inlineStr">
+        <is>
+          <t>✅ 最近完成與測試效果</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>編號</t>
+        </is>
+      </c>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>任務</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="inlineStr">
+        <is>
+          <t>測試結果</t>
+        </is>
+      </c>
+      <c r="D49" s="4" t="inlineStr">
+        <is>
+          <t>完成日期</t>
+        </is>
+      </c>
+      <c r="E49" s="4" t="inlineStr">
+        <is>
+          <t>測試證據</t>
         </is>
       </c>
       <c r="F49" s="11" t="n"/>
@@ -2089,15 +2092,15 @@
       <c r="H50" s="11" t="n"/>
       <c r="I50" s="12" t="n"/>
     </row>
-    <row r="51" ht="158" customHeight="1">
+    <row r="51" ht="88" customHeight="1">
       <c r="A51" s="13" t="inlineStr">
         <is>
-          <t>P2-19</t>
+          <t>P2-21</t>
         </is>
       </c>
       <c r="B51" s="6" t="inlineStr">
         <is>
-          <t>P2-16 ③ 回滾過多時自動暫停推送</t>
+          <t>P2-16 ⑤ 後台 OTA 頁換成真實數據與操作</t>
         </is>
       </c>
       <c r="C51" s="13" t="inlineStr">
@@ -2107,12 +2110,12 @@
       </c>
       <c r="D51" s="13" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E51" s="6" t="inlineStr">
         <is>
-          <t>migration 20261014200000 BEGIN/ROLLBACK 套用兩次無錯並已套用本機。模擬 20 台連跑兩次 12/12：1/20 回滾不暫停、其餘 18 台照常；2/20 → 'Auto-paused: 2 of 20 boards rolled back (10%)'，其餘 0 台拿到 ota；已運行的設備記為 running 且不再下發；審計 1 筆 actor 空；恢復後 17 台拿到、保持恢復，第 3 台回滾 → 'Auto-paused: 3 of 20 (15%)'；白名單 2 台中 1 台回滾 → 50% 立即暫停、另一台不再下發；anon 呼叫 ota_maybe_pause → 401/42501。測試數據已清除，spotpear-ai-toy 1.6.2 仍 100% 未暫停</t>
+          <t>10-14 模擬 20 台全部通過（見上次）；2026-10-15 真機補做：OTA 頁對 1.7.1 白名單加 62:70（UI MAC 欄）→ 存檔確認框 → 『Narrow to Whitelist』確認 → Make current（用戶點）→ 62:70 安裝並確認，頁面顯示 Rolling out · Whitelist、運行 1、回滾 0；每步一筆審計。依賴 P2-14 已完成</t>
         </is>
       </c>
       <c r="F51" s="11" t="n"/>
@@ -2120,15 +2123,15 @@
       <c r="H51" s="11" t="n"/>
       <c r="I51" s="12" t="n"/>
     </row>
-    <row r="52" ht="200" customHeight="1">
+    <row r="52" ht="158" customHeight="1">
       <c r="A52" s="13" t="inlineStr">
         <is>
-          <t>P2-18</t>
+          <t>P2-16</t>
         </is>
       </c>
       <c r="B52" s="6" t="inlineStr">
         <is>
-          <t>P2-16 ② 按 MAC 雜湊穩定分組決定哪台收到 ota</t>
+          <t>OTA 分批推送與後台發佈頁</t>
         </is>
       </c>
       <c r="C52" s="13" t="inlineStr">
@@ -2138,12 +2141,12 @@
       </c>
       <c r="D52" s="13" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E52" s="6" t="inlineStr">
         <is>
-          <t>node --test lib/otaRollout.test.mjs 6/6：10,000 隨機 MAC 在 10%/50% 誤差 &lt; 1 個百分點、同 MAC（含大小寫/空白）結果一致、升階段只增不減、白名單各階段都在、不同版本選不同的 10%。tsc --noEmit 通過。分支 dev server（3216）+ 本機 Supabase 模擬 20 台（板型 p218-sim，連跑兩次 9/9）：白名單階段只有 1 台、重複不變；10% 拿到的正是雜湊預測的那組（2–5 台含白名單），重複不變；50% 包含 10% 全部；暫停 → 0 台且下載映像 404，恢復 → 200；100% → 除已更新和已回滾的 2 台外 18 台；每台下發次數與記錄一致；運行中/已回滾正確標記；審計 6 筆對應 6 次變更。真 spotpear-ai-toy（預設 100%）回報 1.6.1 → 仍拿到 1.6.2。測試數據已清除</t>
+          <t>④ 真機 62:70（2026-10-15）：USB 刷 1.7.0（開機印 aibuddy-build;kind=dev;…;version=1.7.0）→ release_firmware.py publish --dev 1.7.1 → 後台白名單加 62:70、改白名單階段、設為 current → 按 BOOT 喚醒：取 token 200、下載 12.8s、重開進 app1，09:39:36 連上語音伺服器；09:42 重開 → 『Firmware 1.7.1 on app1』無 probation、Up to date；頁面『Rolling out · Whitelist』運行 1 台、回滾 0；審計 5 筆（發佈、白名單、階段、1.6.2 取消 current、1.7.1 設 current）。①②③⑤ 見 P2-17～P2-21 模擬 20 台</t>
         </is>
       </c>
       <c r="F52" s="11" t="n"/>
@@ -2151,15 +2154,15 @@
       <c r="H52" s="11" t="n"/>
       <c r="I52" s="12" t="n"/>
     </row>
-    <row r="53" ht="172" customHeight="1">
+    <row r="53" ht="144" customHeight="1">
       <c r="A53" s="13" t="inlineStr">
         <is>
-          <t>P2-17</t>
+          <t>P2-14</t>
         </is>
       </c>
       <c r="B53" s="6" t="inlineStr">
         <is>
-          <t>P2-16 ① 分批推送的數據表：推送階段、白名單、每台安裝結果</t>
+          <t>Admin 設備頁：每台玩具的狀態、韌體與基本操作</t>
         </is>
       </c>
       <c r="C53" s="13" t="inlineStr">
@@ -2169,12 +2172,12 @@
       </c>
       <c r="D53" s="13" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E53" s="6" t="inlineStr">
         <is>
-          <t>migration 20261014190000 BEGIN/ROLLBACK 套用兩次無錯並已套用本機；行為：預設 100%、promote 記 stage_changed_at，7 種壞值（25%、小寫/空字串/NULL MAC、暫停缺原因等）全被 check 擋；ota_note_offer 1→2→3，report 正確標 running/failed、別板型不影響，刪發佈連帶刪記錄；審計 5 筆含 'test-board 9.9.9' 標籤。REST 13/13：超管可讀、內容管理員 0 行、anon 42501，三種身份寫入/改階段/呼叫 ota_note_offer 皆 42501。release_firmware.py promote spotpear-ai-toy 1.6.2 成功，token 查詢仍選 1.6.2，審計記 2 筆（actor 空＝service role）</t>
+          <t>真機 62:70（2026-10-15，分支 hw-test-1015 = dev+P2-16，-localall 1.7.0，本機網頁 3230 + 語音 7870）：① 開機 → 設備頁 Online、-67 dBm、1.7.0；板子停在 bootloader 約 38 秒後語音伺服器判離線（uvicorn ping 超時），頁面 0 台在線 ② 重置設備密鑰 → device_secrets 行刪除，板子重開印『Device secret issued and stored』並連上，行恢復 ③ 強制解綁 → 板子拿 202（配對碼 UKDM7N），語音伺服器拒絕連線；兩項審計各 1 筆含操作者與原因 ④ 內容管理員/anon → 42501（10-14 探測腳本）</t>
         </is>
       </c>
       <c r="F53" s="11" t="n"/>
@@ -2182,15 +2185,15 @@
       <c r="H53" s="11" t="n"/>
       <c r="I53" s="12" t="n"/>
     </row>
-    <row r="54" ht="116" customHeight="1">
+    <row r="54" ht="158" customHeight="1">
       <c r="A54" s="13" t="inlineStr">
         <is>
-          <t>R-41</t>
+          <t>P2-19</t>
         </is>
       </c>
       <c r="B54" s="6" t="inlineStr">
         <is>
-          <t>App 顯示玩具電量狀態（低電量提示）</t>
+          <t>P2-16 ③ 回滾過多時自動暫停推送</t>
         </is>
       </c>
       <c r="C54" s="13" t="inlineStr">
@@ -2205,7 +2208,7 @@
       </c>
       <c r="E54" s="6" t="inlineStr">
         <is>
-          <t>① pytest 33 passed；真 PATCH 本地 Supabase ② 62:70 刷 p212+R-41 強制低電 build（SUPPLY_LOW_RATIO_OVERRIDE=1.05）→ 串口 [WSc] power low:true，本地 DB battery_low=t ③ 刷回正常 1.6.2 → low:false，DB=f ④ App 讀 DB：低電紅標+Please charge+更新時間、72% 充電中、未上報不顯示 ⑤ 他人帳號 0 行、authenticated UPDATE 被拒。62:70 已還原為原 p212 build</t>
+          <t>migration 20261014200000 BEGIN/ROLLBACK 套用兩次無錯並已套用本機。模擬 20 台連跑兩次 12/12：1/20 回滾不暫停、其餘 18 台照常；2/20 → 'Auto-paused: 2 of 20 boards rolled back (10%)'，其餘 0 台拿到 ota；已運行的設備記為 running 且不再下發；審計 1 筆 actor 空；恢復後 17 台拿到、保持恢復，第 3 台回滾 → 'Auto-paused: 3 of 20 (15%)'；白名單 2 台中 1 台回滾 → 50% 立即暫停、另一台不再下發；anon 呼叫 ota_maybe_pause → 401/42501。測試數據已清除，spotpear-ai-toy 1.6.2 仍 100% 未暫停</t>
         </is>
       </c>
       <c r="F54" s="11" t="n"/>
@@ -2213,96 +2216,120 @@
       <c r="H54" s="11" t="n"/>
       <c r="I54" s="12" t="n"/>
     </row>
-    <row r="56">
-      <c r="A56" s="10" t="inlineStr">
-        <is>
-          <t>⏳ 等待依賴 / ⛔ 阻塞</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="4" t="inlineStr">
-        <is>
-          <t>編號</t>
-        </is>
-      </c>
-      <c r="B57" s="4" t="inlineStr">
-        <is>
-          <t>任務</t>
-        </is>
-      </c>
-      <c r="C57" s="4" t="inlineStr">
-        <is>
-          <t>在等什麼</t>
-        </is>
-      </c>
-      <c r="D57" s="11" t="n"/>
-      <c r="E57" s="11" t="n"/>
+    <row r="55" ht="200" customHeight="1">
+      <c r="A55" s="13" t="inlineStr">
+        <is>
+          <t>P2-18</t>
+        </is>
+      </c>
+      <c r="B55" s="6" t="inlineStr">
+        <is>
+          <t>P2-16 ② 按 MAC 雜湊穩定分組決定哪台收到 ota</t>
+        </is>
+      </c>
+      <c r="C55" s="13" t="inlineStr">
+        <is>
+          <t>通過</t>
+        </is>
+      </c>
+      <c r="D55" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="E55" s="6" t="inlineStr">
+        <is>
+          <t>node --test lib/otaRollout.test.mjs 6/6：10,000 隨機 MAC 在 10%/50% 誤差 &lt; 1 個百分點、同 MAC（含大小寫/空白）結果一致、升階段只增不減、白名單各階段都在、不同版本選不同的 10%。tsc --noEmit 通過。分支 dev server（3216）+ 本機 Supabase 模擬 20 台（板型 p218-sim，連跑兩次 9/9）：白名單階段只有 1 台、重複不變；10% 拿到的正是雜湊預測的那組（2–5 台含白名單），重複不變；50% 包含 10% 全部；暫停 → 0 台且下載映像 404，恢復 → 200；100% → 除已更新和已回滾的 2 台外 18 台；每台下發次數與記錄一致；運行中/已回滾正確標記；審計 6 筆對應 6 次變更。真 spotpear-ai-toy（預設 100%）回報 1.6.1 → 仍拿到 1.6.2。測試數據已清除</t>
+        </is>
+      </c>
+      <c r="F55" s="11" t="n"/>
+      <c r="G55" s="11" t="n"/>
+      <c r="H55" s="11" t="n"/>
+      <c r="I55" s="12" t="n"/>
+    </row>
+    <row r="56" ht="172" customHeight="1">
+      <c r="A56" s="13" t="inlineStr">
+        <is>
+          <t>P2-17</t>
+        </is>
+      </c>
+      <c r="B56" s="6" t="inlineStr">
+        <is>
+          <t>P2-16 ① 分批推送的數據表：推送階段、白名單、每台安裝結果</t>
+        </is>
+      </c>
+      <c r="C56" s="13" t="inlineStr">
+        <is>
+          <t>通過</t>
+        </is>
+      </c>
+      <c r="D56" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="E56" s="6" t="inlineStr">
+        <is>
+          <t>migration 20261014190000 BEGIN/ROLLBACK 套用兩次無錯並已套用本機；行為：預設 100%、promote 記 stage_changed_at，7 種壞值（25%、小寫/空字串/NULL MAC、暫停缺原因等）全被 check 擋；ota_note_offer 1→2→3，report 正確標 running/failed、別板型不影響，刪發佈連帶刪記錄；審計 5 筆含 'test-board 9.9.9' 標籤。REST 13/13：超管可讀、內容管理員 0 行、anon 42501，三種身份寫入/改階段/呼叫 ota_note_offer 皆 42501。release_firmware.py promote spotpear-ai-toy 1.6.2 成功，token 查詢仍選 1.6.2，審計記 2 筆（actor 空＝service role）</t>
+        </is>
+      </c>
+      <c r="F56" s="11" t="n"/>
+      <c r="G56" s="11" t="n"/>
+      <c r="H56" s="11" t="n"/>
+      <c r="I56" s="12" t="n"/>
+    </row>
+    <row r="57" ht="116" customHeight="1">
+      <c r="A57" s="13" t="inlineStr">
+        <is>
+          <t>R-41</t>
+        </is>
+      </c>
+      <c r="B57" s="6" t="inlineStr">
+        <is>
+          <t>App 顯示玩具電量狀態（低電量提示）</t>
+        </is>
+      </c>
+      <c r="C57" s="13" t="inlineStr">
+        <is>
+          <t>通過</t>
+        </is>
+      </c>
+      <c r="D57" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="E57" s="6" t="inlineStr">
+        <is>
+          <t>① pytest 33 passed；真 PATCH 本地 Supabase ② 62:70 刷 p212+R-41 強制低電 build（SUPPLY_LOW_RATIO_OVERRIDE=1.05）→ 串口 [WSc] power low:true，本地 DB battery_low=t ③ 刷回正常 1.6.2 → low:false，DB=f ④ App 讀 DB：低電紅標+Please charge+更新時間、72% 充電中、未上報不顯示 ⑤ 他人帳號 0 行、authenticated UPDATE 被拒。62:70 已還原為原 p212 build</t>
+        </is>
+      </c>
       <c r="F57" s="11" t="n"/>
       <c r="G57" s="11" t="n"/>
       <c r="H57" s="11" t="n"/>
       <c r="I57" s="12" t="n"/>
     </row>
-    <row r="58" ht="88" customHeight="1">
-      <c r="A58" s="13" t="inlineStr">
-        <is>
-          <t>R-17</t>
-        </is>
-      </c>
-      <c r="B58" s="6" t="inlineStr">
-        <is>
-          <t>Spotpear 電池耗盡時插電能否正常開機（供電路徑）</t>
-        </is>
-      </c>
-      <c r="C58" s="6" t="inlineStr">
-        <is>
-          <t>阻塞：[2026-10-08] 2026-10-08 開發板 63:64 插著 USB 時兩次無法解釋的完全斷電重開：09:13:26（崩潰循環中）、10:44:33（閒置、用戶確認沒碰）。都是 USB 先斷線再以 ESP_RST_POWERON 開機，非 brownout；斷電前 6 秒 GPIO0 讀數 99.9% 參考值，屬突然切斷而非緩降（SupplyMonitor 取樣太疏抓不到瞬間）。韌體無法造成 POWERON，指向充電芯片/電池保護/供電路徑，應一併問 Spotpear；放電實測時留意插 USB 閒置時是否也會斷電</t>
-        </is>
-      </c>
-      <c r="D58" s="11" t="n"/>
-      <c r="E58" s="11" t="n"/>
-      <c r="F58" s="11" t="n"/>
-      <c r="G58" s="11" t="n"/>
-      <c r="H58" s="11" t="n"/>
-      <c r="I58" s="12" t="n"/>
-    </row>
-    <row r="59" ht="60" customHeight="1">
-      <c r="A59" s="13" t="inlineStr">
-        <is>
-          <t>P1-01</t>
-        </is>
-      </c>
-      <c r="B59" s="6" t="inlineStr">
-        <is>
-          <t>加入內容審核層（輸入與輸出）</t>
-        </is>
-      </c>
-      <c r="C59" s="6" t="inlineStr">
-        <is>
-          <t>阻塞：[2026-10-14] 2026-10-14 用戶決定：先不定審核服務商，本項暫停。候選：Azure Content Safety（建議，香港區、可在每句回覆說出口前檢查）、OpenRouter 安全模型、OpenAI Moderation、只用本機字詞表。未寫任何程式。</t>
-        </is>
-      </c>
-      <c r="D59" s="11" t="n"/>
-      <c r="E59" s="11" t="n"/>
-      <c r="F59" s="11" t="n"/>
-      <c r="G59" s="11" t="n"/>
-      <c r="H59" s="11" t="n"/>
-      <c r="I59" s="12" t="n"/>
-    </row>
-    <row r="60" ht="32" customHeight="1">
-      <c r="A60" s="13" t="inlineStr">
-        <is>
-          <t>P1-09</t>
-        </is>
-      </c>
-      <c r="B60" s="6" t="inlineStr">
-        <is>
-          <t>家長鎖：孩子模式進設定要輸入 PIN</t>
-        </is>
-      </c>
-      <c r="C60" s="6" t="inlineStr">
-        <is>
-          <t>阻塞：[2026-10-13] 2026-10-13 用戶決定：AI Buddy（品牌 C）延到 1/15 之後，本項不卡 1/15 出廠；AI Buddy 啟動時再開。</t>
+    <row r="59">
+      <c r="A59" s="10" t="inlineStr">
+        <is>
+          <t>⏳ 等待依賴 / ⛔ 阻塞</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="4" t="inlineStr">
+        <is>
+          <t>編號</t>
+        </is>
+      </c>
+      <c r="B60" s="4" t="inlineStr">
+        <is>
+          <t>任務</t>
+        </is>
+      </c>
+      <c r="C60" s="4" t="inlineStr">
+        <is>
+          <t>在等什麼</t>
         </is>
       </c>
       <c r="D60" s="11" t="n"/>
@@ -2312,20 +2339,20 @@
       <c r="H60" s="11" t="n"/>
       <c r="I60" s="12" t="n"/>
     </row>
-    <row r="61" ht="32" customHeight="1">
+    <row r="61" ht="88" customHeight="1">
       <c r="A61" s="13" t="inlineStr">
         <is>
-          <t>R-12</t>
+          <t>R-17</t>
         </is>
       </c>
       <c r="B61" s="6" t="inlineStr">
         <is>
-          <t>家長控制：每日使用上限和休息時段</t>
+          <t>Spotpear 電池耗盡時插電能否正常開機（供電路徑）</t>
         </is>
       </c>
       <c r="C61" s="6" t="inlineStr">
         <is>
-          <t>阻塞：[2026-10-13] 2026-10-13 用戶決定：AI Buddy（品牌 C）延到 1/15 之後，本項不卡 1/15 出廠；AI Buddy 啟動時再開。</t>
+          <t>阻塞：[2026-10-08] 2026-10-08 開發板 63:64 插著 USB 時兩次無法解釋的完全斷電重開：09:13:26（崩潰循環中）、10:44:33（閒置、用戶確認沒碰）。都是 USB 先斷線再以 ESP_RST_POWERON 開機，非 brownout；斷電前 6 秒 GPIO0 讀數 99.9% 參考值，屬突然切斷而非緩降（SupplyMonitor 取樣太疏抓不到瞬間）。韌體無法造成 POWERON，指向充電芯片/電池保護/供電路徑，應一併問 Spotpear；放電實測時留意插 USB 閒置時是否也會斷電</t>
         </is>
       </c>
       <c r="D61" s="11" t="n"/>
@@ -2335,20 +2362,20 @@
       <c r="H61" s="11" t="n"/>
       <c r="I61" s="12" t="n"/>
     </row>
-    <row r="62" ht="32" customHeight="1">
+    <row r="62" ht="60" customHeight="1">
       <c r="A62" s="13" t="inlineStr">
         <is>
-          <t>R-29</t>
+          <t>P1-01</t>
         </is>
       </c>
       <c r="B62" s="6" t="inlineStr">
         <is>
-          <t>AI Buddy App（品牌 C）頁面</t>
+          <t>加入內容審核層（輸入與輸出）</t>
         </is>
       </c>
       <c r="C62" s="6" t="inlineStr">
         <is>
-          <t>阻塞：[2026-10-13] 2026-10-13 用戶決定：AI Buddy（品牌 C）延到 1/15 之後，本項不卡 1/15 出廠；AI Buddy 啟動時再開。</t>
+          <t>阻塞：[2026-10-14] 2026-10-14 用戶決定：先不定審核服務商，本項暫停。候選：Azure Content Safety（建議，香港區、可在每句回覆說出口前檢查）、OpenRouter 安全模型、OpenAI Moderation、只用本機字詞表。未寫任何程式。</t>
         </is>
       </c>
       <c r="D62" s="11" t="n"/>
@@ -2358,20 +2385,20 @@
       <c r="H62" s="11" t="n"/>
       <c r="I62" s="12" t="n"/>
     </row>
-    <row r="63" ht="18" customHeight="1">
+    <row r="63" ht="32" customHeight="1">
       <c r="A63" s="13" t="inlineStr">
         <is>
-          <t>R-05</t>
+          <t>P1-09</t>
         </is>
       </c>
       <c r="B63" s="6" t="inlineStr">
         <is>
-          <t>內測版外殼（3D 打印 20 台）</t>
+          <t>家長鎖：孩子模式進設定要輸入 PIN</t>
         </is>
       </c>
       <c r="C63" s="6" t="inlineStr">
         <is>
-          <t>等 R-01</t>
+          <t>阻塞：[2026-10-13] 2026-10-13 用戶決定：AI Buddy（品牌 C）延到 1/15 之後，本項不卡 1/15 出廠；AI Buddy 啟動時再開。</t>
         </is>
       </c>
       <c r="D63" s="11" t="n"/>
@@ -2381,20 +2408,20 @@
       <c r="H63" s="11" t="n"/>
       <c r="I63" s="12" t="n"/>
     </row>
-    <row r="64" ht="18" customHeight="1">
+    <row r="64" ht="32" customHeight="1">
       <c r="A64" s="13" t="inlineStr">
         <is>
-          <t>R-06</t>
+          <t>R-12</t>
         </is>
       </c>
       <c r="B64" s="6" t="inlineStr">
         <is>
-          <t>家長自助上手流程</t>
+          <t>家長控制：每日使用上限和休息時段</t>
         </is>
       </c>
       <c r="C64" s="6" t="inlineStr">
         <is>
-          <t>等 P0-11</t>
+          <t>阻塞：[2026-10-13] 2026-10-13 用戶決定：AI Buddy（品牌 C）延到 1/15 之後，本項不卡 1/15 出廠；AI Buddy 啟動時再開。</t>
         </is>
       </c>
       <c r="D64" s="11" t="n"/>
@@ -2407,17 +2434,17 @@
     <row r="65" ht="32" customHeight="1">
       <c r="A65" s="13" t="inlineStr">
         <is>
-          <t>R-13</t>
+          <t>R-29</t>
         </is>
       </c>
       <c r="B65" s="6" t="inlineStr">
         <is>
-          <t>CP1 內測就緒檢查（10/30）</t>
+          <t>AI Buddy App（品牌 C）頁面</t>
         </is>
       </c>
       <c r="C65" s="6" t="inlineStr">
         <is>
-          <t>等 P0-07、P0-11、P1-01、P1-02、P2-09、R-01、R-02、R-04、R-05、R-06、P1-11</t>
+          <t>阻塞：[2026-10-13] 2026-10-13 用戶決定：AI Buddy（品牌 C）延到 1/15 之後，本項不卡 1/15 出廠；AI Buddy 啟動時再開。</t>
         </is>
       </c>
       <c r="D65" s="11" t="n"/>
@@ -2427,15 +2454,15 @@
       <c r="H65" s="11" t="n"/>
       <c r="I65" s="12" t="n"/>
     </row>
-    <row r="66" ht="32" customHeight="1">
+    <row r="66" ht="18" customHeight="1">
       <c r="A66" s="13" t="inlineStr">
         <is>
-          <t>R-18</t>
+          <t>R-05</t>
         </is>
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
-          <t>長按 BOOT 重新配網（開 AIBuddy-XXXX 熱點）</t>
+          <t>內測版外殼（3D 打印 20 台）</t>
         </is>
       </c>
       <c r="C66" s="6" t="inlineStr">
@@ -2450,20 +2477,20 @@
       <c r="H66" s="11" t="n"/>
       <c r="I66" s="12" t="n"/>
     </row>
-    <row r="67" ht="32" customHeight="1">
+    <row r="67" ht="18" customHeight="1">
       <c r="A67" s="13" t="inlineStr">
         <is>
-          <t>R-19</t>
+          <t>R-06</t>
         </is>
       </c>
       <c r="B67" s="6" t="inlineStr">
         <is>
-          <t>外接按鈕：量產板加 I2C 擴展晶片（TCA9555）</t>
+          <t>家長自助上手流程</t>
         </is>
       </c>
       <c r="C67" s="6" t="inlineStr">
         <is>
-          <t>等 R-01</t>
+          <t>等 P0-11</t>
         </is>
       </c>
       <c r="D67" s="11" t="n"/>
@@ -2473,20 +2500,20 @@
       <c r="H67" s="11" t="n"/>
       <c r="I67" s="12" t="n"/>
     </row>
-    <row r="68" ht="18" customHeight="1">
+    <row r="68" ht="32" customHeight="1">
       <c r="A68" s="13" t="inlineStr">
         <is>
-          <t>R-20</t>
+          <t>R-13</t>
         </is>
       </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t>孩子資料與角色改成每台設備一份</t>
+          <t>CP1 內測就緒檢查（10/30）</t>
         </is>
       </c>
       <c r="C68" s="6" t="inlineStr">
         <is>
-          <t>等 P1-12</t>
+          <t>等 P0-07、P0-11、P1-01、P1-02、P2-09、R-01、R-02、R-04、R-05、R-06、P1-11</t>
         </is>
       </c>
       <c r="D68" s="11" t="n"/>
@@ -2499,17 +2526,17 @@
     <row r="69" ht="32" customHeight="1">
       <c r="A69" s="13" t="inlineStr">
         <is>
-          <t>R-27</t>
+          <t>R-18</t>
         </is>
       </c>
       <c r="B69" s="6" t="inlineStr">
         <is>
-          <t>App 內登入：驗證碼、原生社交登入、刪除帳號</t>
+          <t>長按 BOOT 重新配網（開 AIBuddy-XXXX 熱點）</t>
         </is>
       </c>
       <c r="C69" s="6" t="inlineStr">
         <is>
-          <t>等 R-26</t>
+          <t>等 R-01</t>
         </is>
       </c>
       <c r="D69" s="11" t="n"/>
@@ -2519,15 +2546,15 @@
       <c r="H69" s="11" t="n"/>
       <c r="I69" s="12" t="n"/>
     </row>
-    <row r="70" ht="18" customHeight="1">
+    <row r="70" ht="32" customHeight="1">
       <c r="A70" s="13" t="inlineStr">
         <is>
-          <t>P0-14</t>
+          <t>R-19</t>
         </is>
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>韌體簽章、Secure Boot 與 Flash 加密</t>
+          <t>外接按鈕：量產板加 I2C 擴展晶片（TCA9555）</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr">
@@ -2545,17 +2572,17 @@
     <row r="71" ht="18" customHeight="1">
       <c r="A71" s="13" t="inlineStr">
         <is>
-          <t>P1-06</t>
+          <t>R-20</t>
         </is>
       </c>
       <c r="B71" s="6" t="inlineStr">
         <is>
-          <t>處理 GPL-3.0 依賴（arduino-audio-tools）</t>
+          <t>孩子資料與角色改成每台設備一份</t>
         </is>
       </c>
       <c r="C71" s="6" t="inlineStr">
         <is>
-          <t>等 Q3</t>
+          <t>等 P1-12</t>
         </is>
       </c>
       <c r="D71" s="11" t="n"/>
@@ -2565,20 +2592,20 @@
       <c r="H71" s="11" t="n"/>
       <c r="I71" s="12" t="n"/>
     </row>
-    <row r="72" ht="18" customHeight="1">
+    <row r="72" ht="32" customHeight="1">
       <c r="A72" s="13" t="inlineStr">
         <is>
-          <t>P1-07</t>
+          <t>R-27</t>
         </is>
       </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>LGPL 合規與第三方授權聲明</t>
+          <t>App 內登入：驗證碼、原生社交登入、刪除帳號</t>
         </is>
       </c>
       <c r="C72" s="6" t="inlineStr">
         <is>
-          <t>等 Q3</t>
+          <t>等 R-26</t>
         </is>
       </c>
       <c r="D72" s="11" t="n"/>
@@ -2591,17 +2618,17 @@
     <row r="73" ht="18" customHeight="1">
       <c r="A73" s="13" t="inlineStr">
         <is>
-          <t>P1-08</t>
+          <t>P0-14</t>
         </is>
       </c>
       <c r="B73" s="6" t="inlineStr">
         <is>
-          <t>硬件認證</t>
+          <t>韌體簽章、Secure Boot 與 Flash 加密</t>
         </is>
       </c>
       <c r="C73" s="6" t="inlineStr">
         <is>
-          <t>等 R-01、R-05</t>
+          <t>等 R-01</t>
         </is>
       </c>
       <c r="D73" s="11" t="n"/>
@@ -2614,17 +2641,17 @@
     <row r="74" ht="18" customHeight="1">
       <c r="A74" s="13" t="inlineStr">
         <is>
-          <t>P1-14</t>
+          <t>P1-06</t>
         </is>
       </c>
       <c r="B74" s="6" t="inlineStr">
         <is>
-          <t>Admin 內容安全頁：審核事件只按類別統計</t>
+          <t>處理 GPL-3.0 依賴（arduino-audio-tools）</t>
         </is>
       </c>
       <c r="C74" s="6" t="inlineStr">
         <is>
-          <t>等 P1-01、P2-13</t>
+          <t>等 Q3</t>
         </is>
       </c>
       <c r="D74" s="11" t="n"/>
@@ -2634,20 +2661,20 @@
       <c r="H74" s="11" t="n"/>
       <c r="I74" s="12" t="n"/>
     </row>
-    <row r="75" ht="32" customHeight="1">
+    <row r="75" ht="18" customHeight="1">
       <c r="A75" s="13" t="inlineStr">
         <is>
-          <t>P2-15</t>
+          <t>P1-07</t>
         </is>
       </c>
       <c r="B75" s="6" t="inlineStr">
         <is>
-          <t>Admin 總覽頁：在線、用量、成本與待處理事項</t>
+          <t>LGPL 合規與第三方授權聲明</t>
         </is>
       </c>
       <c r="C75" s="6" t="inlineStr">
         <is>
-          <t>等 P2-09</t>
+          <t>等 Q3</t>
         </is>
       </c>
       <c r="D75" s="11" t="n"/>
@@ -2660,17 +2687,17 @@
     <row r="76" ht="18" customHeight="1">
       <c r="A76" s="13" t="inlineStr">
         <is>
-          <t>R-07</t>
+          <t>P1-08</t>
         </is>
       </c>
       <c r="B76" s="6" t="inlineStr">
         <is>
-          <t>20 個家庭封閉內測</t>
+          <t>硬件認證</t>
         </is>
       </c>
       <c r="C76" s="6" t="inlineStr">
         <is>
-          <t>等 R-13</t>
+          <t>等 R-01、R-05</t>
         </is>
       </c>
       <c r="D76" s="11" t="n"/>
@@ -2683,17 +2710,17 @@
     <row r="77" ht="18" customHeight="1">
       <c r="A77" s="13" t="inlineStr">
         <is>
-          <t>R-08</t>
+          <t>P1-14</t>
         </is>
       </c>
       <c r="B77" s="6" t="inlineStr">
         <is>
-          <t>第 8 週關卡決策</t>
+          <t>Admin 內容安全頁：審核事件只按類別統計</t>
         </is>
       </c>
       <c r="C77" s="6" t="inlineStr">
         <is>
-          <t>等 R-07、P2-09、P1-08</t>
+          <t>等 P1-01、P2-13</t>
         </is>
       </c>
       <c r="D77" s="11" t="n"/>
@@ -2703,20 +2730,20 @@
       <c r="H77" s="11" t="n"/>
       <c r="I77" s="12" t="n"/>
     </row>
-    <row r="78" ht="18" customHeight="1">
+    <row r="78" ht="32" customHeight="1">
       <c r="A78" s="13" t="inlineStr">
         <is>
-          <t>R-14</t>
+          <t>P2-15</t>
         </is>
       </c>
       <c r="B78" s="6" t="inlineStr">
         <is>
-          <t>離線兒歌與故事</t>
+          <t>Admin 總覽頁：在線、用量、成本與待處理事項</t>
         </is>
       </c>
       <c r="C78" s="6" t="inlineStr">
         <is>
-          <t>等 R-01</t>
+          <t>等 P2-09</t>
         </is>
       </c>
       <c r="D78" s="11" t="n"/>
@@ -2729,17 +2756,17 @@
     <row r="79" ht="18" customHeight="1">
       <c r="A79" s="13" t="inlineStr">
         <is>
-          <t>R-24</t>
+          <t>R-07</t>
         </is>
       </c>
       <c r="B79" s="6" t="inlineStr">
         <is>
-          <t>設備只能用自己品牌的角色</t>
+          <t>20 個家庭封閉內測</t>
         </is>
       </c>
       <c r="C79" s="6" t="inlineStr">
         <is>
-          <t>等 R-34</t>
+          <t>等 R-13</t>
         </is>
       </c>
       <c r="D79" s="11" t="n"/>
@@ -2752,17 +2779,17 @@
     <row r="80" ht="18" customHeight="1">
       <c r="A80" s="13" t="inlineStr">
         <is>
-          <t>R-28</t>
+          <t>R-08</t>
         </is>
       </c>
       <c r="B80" s="6" t="inlineStr">
         <is>
-          <t>三個 App 的殼：品牌版本與測試版</t>
+          <t>第 8 週關卡決策</t>
         </is>
       </c>
       <c r="C80" s="6" t="inlineStr">
         <is>
-          <t>等 R-25、R-26</t>
+          <t>等 R-07、P2-09、P1-08</t>
         </is>
       </c>
       <c r="D80" s="11" t="n"/>
@@ -2775,17 +2802,17 @@
     <row r="81" ht="18" customHeight="1">
       <c r="A81" s="13" t="inlineStr">
         <is>
-          <t>R-30</t>
+          <t>R-14</t>
         </is>
       </c>
       <c r="B81" s="6" t="inlineStr">
         <is>
-          <t>快活 App（品牌 A）頁面</t>
+          <t>離線兒歌與故事</t>
         </is>
       </c>
       <c r="C81" s="6" t="inlineStr">
         <is>
-          <t>等 R-25、R-34、Q12</t>
+          <t>等 R-01</t>
         </is>
       </c>
       <c r="D81" s="11" t="n"/>
@@ -2798,17 +2825,17 @@
     <row r="82" ht="18" customHeight="1">
       <c r="A82" s="13" t="inlineStr">
         <is>
-          <t>R-31</t>
+          <t>R-24</t>
         </is>
       </c>
       <c r="B82" s="6" t="inlineStr">
         <is>
-          <t>政協青年聯會版 App（品牌 B）頁面</t>
+          <t>設備只能用自己品牌的角色</t>
         </is>
       </c>
       <c r="C82" s="6" t="inlineStr">
         <is>
-          <t>等 R-25、R-34、Q13</t>
+          <t>等 R-34</t>
         </is>
       </c>
       <c r="D82" s="11" t="n"/>
@@ -2821,17 +2848,17 @@
     <row r="83" ht="18" customHeight="1">
       <c r="A83" s="13" t="inlineStr">
         <is>
-          <t>R-35</t>
+          <t>R-28</t>
         </is>
       </c>
       <c r="B83" s="6" t="inlineStr">
         <is>
-          <t>韌體按品牌連線：伺服器網址在出廠時寫入</t>
+          <t>三個 App 的殼：品牌版本與測試版</t>
         </is>
       </c>
       <c r="C83" s="6" t="inlineStr">
         <is>
-          <t>等 R-34</t>
+          <t>等 R-25、R-26</t>
         </is>
       </c>
       <c r="D83" s="11" t="n"/>
@@ -2841,20 +2868,20 @@
       <c r="H83" s="11" t="n"/>
       <c r="I83" s="12" t="n"/>
     </row>
-    <row r="84" ht="32" customHeight="1">
+    <row r="84" ht="18" customHeight="1">
       <c r="A84" s="13" t="inlineStr">
         <is>
-          <t>R-38</t>
+          <t>R-30</t>
         </is>
       </c>
       <c r="B84" s="6" t="inlineStr">
         <is>
-          <t>公仔出廠鎖死所屬 IP，綁定時顯示該 IP 頭像</t>
+          <t>快活 App（品牌 A）頁面</t>
         </is>
       </c>
       <c r="C84" s="6" t="inlineStr">
         <is>
-          <t>等 P0-11</t>
+          <t>等 R-25、R-34、Q12</t>
         </is>
       </c>
       <c r="D84" s="11" t="n"/>
@@ -2864,20 +2891,20 @@
       <c r="H84" s="11" t="n"/>
       <c r="I84" s="12" t="n"/>
     </row>
-    <row r="85" ht="32" customHeight="1">
+    <row r="85" ht="18" customHeight="1">
       <c r="A85" s="13" t="inlineStr">
         <is>
-          <t>R-39</t>
+          <t>R-31</t>
         </is>
       </c>
       <c r="B85" s="6" t="inlineStr">
         <is>
-          <t>Admin 出廠登記頁：匯入 MAC 清單、指定公仔、查看自檢結果</t>
+          <t>政協青年聯會版 App（品牌 B）頁面</t>
         </is>
       </c>
       <c r="C85" s="6" t="inlineStr">
         <is>
-          <t>等 R-38、P1-10</t>
+          <t>等 R-25、R-34、Q13</t>
         </is>
       </c>
       <c r="D85" s="11" t="n"/>
@@ -2890,17 +2917,17 @@
     <row r="86" ht="18" customHeight="1">
       <c r="A86" s="13" t="inlineStr">
         <is>
-          <t>R-09</t>
+          <t>R-35</t>
         </is>
       </c>
       <c r="B86" s="6" t="inlineStr">
         <is>
-          <t>量產外殼（真空複模）</t>
+          <t>韌體按品牌連線：伺服器網址在出廠時寫入</t>
         </is>
       </c>
       <c r="C86" s="6" t="inlineStr">
         <is>
-          <t>等 R-08、R-05、Q11</t>
+          <t>等 R-34</t>
         </is>
       </c>
       <c r="D86" s="11" t="n"/>
@@ -2910,20 +2937,20 @@
       <c r="H86" s="11" t="n"/>
       <c r="I86" s="12" t="n"/>
     </row>
-    <row r="87" ht="18" customHeight="1">
+    <row r="87" ht="32" customHeight="1">
       <c r="A87" s="13" t="inlineStr">
         <is>
-          <t>R-10</t>
+          <t>R-38</t>
         </is>
       </c>
       <c r="B87" s="6" t="inlineStr">
         <is>
-          <t>出廠流程</t>
+          <t>公仔出廠鎖死所屬 IP，綁定時顯示該 IP 頭像</t>
         </is>
       </c>
       <c r="C87" s="6" t="inlineStr">
         <is>
-          <t>等 P0-14、R-01、P2-12、R-34、R-35、R-38、R-39</t>
+          <t>等 P0-11</t>
         </is>
       </c>
       <c r="D87" s="11" t="n"/>
@@ -2933,20 +2960,20 @@
       <c r="H87" s="11" t="n"/>
       <c r="I87" s="12" t="n"/>
     </row>
-    <row r="88" ht="18" customHeight="1">
+    <row r="88" ht="32" customHeight="1">
       <c r="A88" s="13" t="inlineStr">
         <is>
-          <t>R-11</t>
+          <t>R-39</t>
         </is>
       </c>
       <c r="B88" s="6" t="inlineStr">
         <is>
-          <t>售後：客服、保修與換機</t>
+          <t>Admin 出廠登記頁：匯入 MAC 清單、指定公仔、查看自檢結果</t>
         </is>
       </c>
       <c r="C88" s="6" t="inlineStr">
         <is>
-          <t>等 R-40</t>
+          <t>等 R-38、P1-10</t>
         </is>
       </c>
       <c r="D88" s="11" t="n"/>
@@ -2959,17 +2986,17 @@
     <row r="89" ht="18" customHeight="1">
       <c r="A89" s="13" t="inlineStr">
         <is>
-          <t>R-15</t>
+          <t>R-44</t>
         </is>
       </c>
       <c r="B89" s="6" t="inlineStr">
         <is>
-          <t>農曆新年前交付（生產 1/15、送達 1/29）</t>
+          <t>知識庫後台頁面與審批流程</t>
         </is>
       </c>
       <c r="C89" s="6" t="inlineStr">
         <is>
-          <t>等 R-09、R-10</t>
+          <t>等 P1-10</t>
         </is>
       </c>
       <c r="D89" s="11" t="n"/>
@@ -2982,17 +3009,17 @@
     <row r="90" ht="18" customHeight="1">
       <c r="A90" s="13" t="inlineStr">
         <is>
-          <t>R-33</t>
+          <t>R-09</t>
         </is>
       </c>
       <c r="B90" s="6" t="inlineStr">
         <is>
-          <t>三個 App 送審並通過</t>
+          <t>量產外殼（真空複模）</t>
         </is>
       </c>
       <c r="C90" s="6" t="inlineStr">
         <is>
-          <t>等 R-27、R-21、R-28、R-29、R-30、R-31、R-32</t>
+          <t>等 R-08、R-05、Q11</t>
         </is>
       </c>
       <c r="D90" s="11" t="n"/>
@@ -3002,20 +3029,20 @@
       <c r="H90" s="11" t="n"/>
       <c r="I90" s="12" t="n"/>
     </row>
-    <row r="91" ht="32" customHeight="1">
+    <row r="91" ht="18" customHeight="1">
       <c r="A91" s="13" t="inlineStr">
         <is>
-          <t>R-40</t>
+          <t>R-10</t>
         </is>
       </c>
       <c r="B91" s="6" t="inlineStr">
         <is>
-          <t>Admin 客服查詢頁：查帳號、名下設備與最近事件</t>
+          <t>出廠流程</t>
         </is>
       </c>
       <c r="C91" s="6" t="inlineStr">
         <is>
-          <t>等 P1-10、P1-12</t>
+          <t>等 P0-14、R-01、P2-12、R-34、R-35、R-38、R-39</t>
         </is>
       </c>
       <c r="D91" s="11" t="n"/>
@@ -3025,27 +3052,66 @@
       <c r="H91" s="11" t="n"/>
       <c r="I91" s="12" t="n"/>
     </row>
-    <row r="93">
-      <c r="A93" s="10" t="inlineStr">
-        <is>
-          <t>❓ 待確認問題</t>
-        </is>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" s="4" t="inlineStr">
-        <is>
-          <t>編號</t>
-        </is>
-      </c>
-      <c r="B94" s="4" t="inlineStr">
-        <is>
-          <t>問題</t>
-        </is>
-      </c>
-      <c r="C94" s="4" t="inlineStr">
-        <is>
-          <t>影響的任務 / 為什麼重要</t>
+    <row r="92" ht="18" customHeight="1">
+      <c r="A92" s="13" t="inlineStr">
+        <is>
+          <t>R-11</t>
+        </is>
+      </c>
+      <c r="B92" s="6" t="inlineStr">
+        <is>
+          <t>售後：客服、保修與換機</t>
+        </is>
+      </c>
+      <c r="C92" s="6" t="inlineStr">
+        <is>
+          <t>等 R-40</t>
+        </is>
+      </c>
+      <c r="D92" s="11" t="n"/>
+      <c r="E92" s="11" t="n"/>
+      <c r="F92" s="11" t="n"/>
+      <c r="G92" s="11" t="n"/>
+      <c r="H92" s="11" t="n"/>
+      <c r="I92" s="12" t="n"/>
+    </row>
+    <row r="93" ht="18" customHeight="1">
+      <c r="A93" s="13" t="inlineStr">
+        <is>
+          <t>R-15</t>
+        </is>
+      </c>
+      <c r="B93" s="6" t="inlineStr">
+        <is>
+          <t>農曆新年前交付（生產 1/15、送達 1/29）</t>
+        </is>
+      </c>
+      <c r="C93" s="6" t="inlineStr">
+        <is>
+          <t>等 R-09、R-10</t>
+        </is>
+      </c>
+      <c r="D93" s="11" t="n"/>
+      <c r="E93" s="11" t="n"/>
+      <c r="F93" s="11" t="n"/>
+      <c r="G93" s="11" t="n"/>
+      <c r="H93" s="11" t="n"/>
+      <c r="I93" s="12" t="n"/>
+    </row>
+    <row r="94" ht="18" customHeight="1">
+      <c r="A94" s="13" t="inlineStr">
+        <is>
+          <t>R-33</t>
+        </is>
+      </c>
+      <c r="B94" s="6" t="inlineStr">
+        <is>
+          <t>三個 App 送審並通過</t>
+        </is>
+      </c>
+      <c r="C94" s="6" t="inlineStr">
+        <is>
+          <t>等 R-27、R-21、R-28、R-29、R-30、R-31、R-32</t>
         </is>
       </c>
       <c r="D94" s="11" t="n"/>
@@ -3055,20 +3121,20 @@
       <c r="H94" s="11" t="n"/>
       <c r="I94" s="12" t="n"/>
     </row>
-    <row r="95" ht="18" customHeight="1">
+    <row r="95" ht="32" customHeight="1">
       <c r="A95" s="13" t="inlineStr">
         <is>
-          <t>Q3</t>
+          <t>R-40</t>
         </is>
       </c>
       <c r="B95" s="6" t="inlineStr">
         <is>
-          <t>韌體打算閉源商業銷售嗎？</t>
+          <t>Admin 客服查詢頁：查帳號、名下設備與最近事件</t>
         </is>
       </c>
       <c r="C95" s="6" t="inlineStr">
         <is>
-          <t>P1-06, P1-07：決定 GPL／LGPL 依賴要開源還是替換。</t>
+          <t>等 P1-10、P1-12</t>
         </is>
       </c>
       <c r="D95" s="11" t="n"/>
@@ -3078,66 +3144,27 @@
       <c r="H95" s="11" t="n"/>
       <c r="I95" s="12" t="n"/>
     </row>
-    <row r="96" ht="32" customHeight="1">
-      <c r="A96" s="13" t="inlineStr">
-        <is>
-          <t>Q11</t>
-        </is>
-      </c>
-      <c r="B96" s="6" t="inlineStr">
-        <is>
-          <t>馬會快活的賽馬日版和新春版各多少隻（共 2,500）？</t>
-        </is>
-      </c>
-      <c r="C96" s="6" t="inlineStr">
-        <is>
-          <t>R-09, R-15：兩款的服裝和配件要分開訂料；11/20 前不知道，PP 樣和大貨單（11/27）會被拖慢。由馬會決定。</t>
-        </is>
-      </c>
-      <c r="D96" s="11" t="n"/>
-      <c r="E96" s="11" t="n"/>
-      <c r="F96" s="11" t="n"/>
-      <c r="G96" s="11" t="n"/>
-      <c r="H96" s="11" t="n"/>
-      <c r="I96" s="12" t="n"/>
-    </row>
-    <row r="97" ht="60" customHeight="1">
-      <c r="A97" s="13" t="inlineStr">
-        <is>
-          <t>Q12</t>
-        </is>
-      </c>
-      <c r="B97" s="6" t="inlineStr">
-        <is>
-          <t>快活 App 的「會員綁定」是指甚麼：用我們自己的帳號（email 驗證碼），還是接馬會的會員帳號登入（SSO）？</t>
-        </is>
-      </c>
-      <c r="C97" s="6" t="inlineStr">
-        <is>
-          <t>P0-11, 快活 App（未入追蹤表）：接馬會 SSO 的話，登入、帳號刪除和資料歸屬都要按馬會的介面重做，工作量和排期要另估，而且 W5（11/9–11/13）就要做快活 App 的綁定；用我們的帳號則和其他品牌共用同一套流程。由馬會決定，要盡早問。</t>
-        </is>
-      </c>
-      <c r="D97" s="11" t="n"/>
-      <c r="E97" s="11" t="n"/>
-      <c r="F97" s="11" t="n"/>
-      <c r="G97" s="11" t="n"/>
-      <c r="H97" s="11" t="n"/>
-      <c r="I97" s="12" t="n"/>
-    </row>
-    <row r="98" ht="46" customHeight="1">
-      <c r="A98" s="13" t="inlineStr">
-        <is>
-          <t>Q13</t>
-        </is>
-      </c>
-      <c r="B98" s="6" t="inlineStr">
-        <is>
-          <t>政協青年聯會版的角色、語言和內容由誰提供？什麼時候交？</t>
-        </is>
-      </c>
-      <c r="C98" s="6" t="inlineStr">
-        <is>
-          <t>品牌 B 的 App 頁面：品牌 B 的用戶是成人會員，但角色、說話語言、內容規則都還沒有。最遲 11/13 要拿到，才趕得及內部測試和 App 頁面（W6）。</t>
+    <row r="97">
+      <c r="A97" s="10" t="inlineStr">
+        <is>
+          <t>❓ 待確認問題</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="4" t="inlineStr">
+        <is>
+          <t>編號</t>
+        </is>
+      </c>
+      <c r="B98" s="4" t="inlineStr">
+        <is>
+          <t>問題</t>
+        </is>
+      </c>
+      <c r="C98" s="4" t="inlineStr">
+        <is>
+          <t>影響的任務 / 為什麼重要</t>
         </is>
       </c>
       <c r="D98" s="11" t="n"/>
@@ -3147,67 +3174,160 @@
       <c r="H98" s="11" t="n"/>
       <c r="I98" s="12" t="n"/>
     </row>
-    <row r="100">
-      <c r="A100" s="10" t="inlineStr">
+    <row r="99" ht="18" customHeight="1">
+      <c r="A99" s="13" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="B99" s="6" t="inlineStr">
+        <is>
+          <t>韌體打算閉源商業銷售嗎？</t>
+        </is>
+      </c>
+      <c r="C99" s="6" t="inlineStr">
+        <is>
+          <t>P1-06, P1-07：決定 GPL／LGPL 依賴要開源還是替換。</t>
+        </is>
+      </c>
+      <c r="D99" s="11" t="n"/>
+      <c r="E99" s="11" t="n"/>
+      <c r="F99" s="11" t="n"/>
+      <c r="G99" s="11" t="n"/>
+      <c r="H99" s="11" t="n"/>
+      <c r="I99" s="12" t="n"/>
+    </row>
+    <row r="100" ht="32" customHeight="1">
+      <c r="A100" s="13" t="inlineStr">
+        <is>
+          <t>Q11</t>
+        </is>
+      </c>
+      <c r="B100" s="6" t="inlineStr">
+        <is>
+          <t>馬會快活的賽馬日版和新春版各多少隻（共 2,500）？</t>
+        </is>
+      </c>
+      <c r="C100" s="6" t="inlineStr">
+        <is>
+          <t>R-09, R-15：兩款的服裝和配件要分開訂料；11/20 前不知道，PP 樣和大貨單（11/27）會被拖慢。由馬會決定。</t>
+        </is>
+      </c>
+      <c r="D100" s="11" t="n"/>
+      <c r="E100" s="11" t="n"/>
+      <c r="F100" s="11" t="n"/>
+      <c r="G100" s="11" t="n"/>
+      <c r="H100" s="11" t="n"/>
+      <c r="I100" s="12" t="n"/>
+    </row>
+    <row r="101" ht="60" customHeight="1">
+      <c r="A101" s="13" t="inlineStr">
+        <is>
+          <t>Q12</t>
+        </is>
+      </c>
+      <c r="B101" s="6" t="inlineStr">
+        <is>
+          <t>快活 App 的「會員綁定」是指甚麼：用我們自己的帳號（email 驗證碼），還是接馬會的會員帳號登入（SSO）？</t>
+        </is>
+      </c>
+      <c r="C101" s="6" t="inlineStr">
+        <is>
+          <t>P0-11, 快活 App（未入追蹤表）：接馬會 SSO 的話，登入、帳號刪除和資料歸屬都要按馬會的介面重做，工作量和排期要另估，而且 W5（11/9–11/13）就要做快活 App 的綁定；用我們的帳號則和其他品牌共用同一套流程。由馬會決定，要盡早問。</t>
+        </is>
+      </c>
+      <c r="D101" s="11" t="n"/>
+      <c r="E101" s="11" t="n"/>
+      <c r="F101" s="11" t="n"/>
+      <c r="G101" s="11" t="n"/>
+      <c r="H101" s="11" t="n"/>
+      <c r="I101" s="12" t="n"/>
+    </row>
+    <row r="102" ht="46" customHeight="1">
+      <c r="A102" s="13" t="inlineStr">
+        <is>
+          <t>Q13</t>
+        </is>
+      </c>
+      <c r="B102" s="6" t="inlineStr">
+        <is>
+          <t>政協青年聯會版的角色、語言和內容由誰提供？什麼時候交？</t>
+        </is>
+      </c>
+      <c r="C102" s="6" t="inlineStr">
+        <is>
+          <t>品牌 B 的 App 頁面：品牌 B 的用戶是成人會員，但角色、說話語言、內容規則都還沒有。最遲 11/13 要拿到，才趕得及內部測試和 App 頁面（W6）。</t>
+        </is>
+      </c>
+      <c r="D102" s="11" t="n"/>
+      <c r="E102" s="11" t="n"/>
+      <c r="F102" s="11" t="n"/>
+      <c r="G102" s="11" t="n"/>
+      <c r="H102" s="11" t="n"/>
+      <c r="I102" s="12" t="n"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="10" t="inlineStr">
         <is>
           <t>說明</t>
-        </is>
-      </c>
-    </row>
-    <row r="101" ht="32" customHeight="1">
-      <c r="A101" s="14" t="inlineStr">
-        <is>
-          <t>・狀態：未開始 → 進行中 → 已完成。只有測試真的跑過而且通過才算已完成；阻塞要在備註寫原因；不再需要的任務標不適用，不要刪。</t>
-        </is>
-      </c>
-    </row>
-    <row r="102" ht="18" customHeight="1">
-      <c r="A102" s="14" t="inlineStr">
-        <is>
-          <t>・測試結果：未測試 / 通過 / 失敗 / 部分通過。測試證據寫跑了什麼、看到什麼，完整歷史在「更新記錄」。</t>
-        </is>
-      </c>
-    </row>
-    <row r="103" ht="18" customHeight="1">
-      <c r="A103" s="14" t="inlineStr">
-        <is>
-          <t>・「接下來」按階段排序，同一階段內再按優先級；依賴還沒滿足的任務不會出現在「接下來」。</t>
-        </is>
-      </c>
-    </row>
-    <row r="104" ht="18" customHeight="1">
-      <c r="A104" s="14" t="inlineStr">
-        <is>
-          <t>・可以手動改：「任務清單」的狀態、測試結果、測試證據、Commit、備註，以及「待確認問題」的回答。其餘欄位和本頁由腳本維護。</t>
         </is>
       </c>
     </row>
     <row r="105" ht="32" customHeight="1">
       <c r="A105" s="14" t="inlineStr">
         <is>
+          <t>・狀態：未開始 → 進行中 → 已完成。只有測試真的跑過而且通過才算已完成；阻塞要在備註寫原因；不再需要的任務標不適用，不要刪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="18" customHeight="1">
+      <c r="A106" s="14" t="inlineStr">
+        <is>
+          <t>・測試結果：未測試 / 通過 / 失敗 / 部分通過。測試證據寫跑了什麼、看到什麼，完整歷史在「更新記錄」。</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" ht="18" customHeight="1">
+      <c r="A107" s="14" t="inlineStr">
+        <is>
+          <t>・「接下來」按階段排序，同一階段內再按優先級；依賴還沒滿足的任務不會出現在「接下來」。</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" ht="18" customHeight="1">
+      <c r="A108" s="14" t="inlineStr">
+        <is>
+          <t>・可以手動改：「任務清單」的狀態、測試結果、測試證據、Commit、備註，以及「待確認問題」的回答。其餘欄位和本頁由腳本維護。</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" ht="32" customHeight="1">
+      <c r="A109" s="14" t="inlineStr">
+        <is>
           <t>・建議用法：在 Claude Code 對 Claude 說「P0-02 做完了」或輸入 /prod-readiness。Claude 會先跑測試再更新，並寫進「更新記錄」。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="86">
+  <mergeCells count="90">
+    <mergeCell ref="E55:I55"/>
+    <mergeCell ref="A108:I108"/>
     <mergeCell ref="C82:I82"/>
     <mergeCell ref="E52:I52"/>
-    <mergeCell ref="A56:I56"/>
     <mergeCell ref="E39:I39"/>
     <mergeCell ref="C67:I67"/>
-    <mergeCell ref="E48:I48"/>
-    <mergeCell ref="A101:I101"/>
     <mergeCell ref="A2:I2"/>
     <mergeCell ref="E29:I29"/>
     <mergeCell ref="E38:I38"/>
     <mergeCell ref="C83:I83"/>
+    <mergeCell ref="C92:I92"/>
+    <mergeCell ref="A109:I109"/>
     <mergeCell ref="E31:I31"/>
     <mergeCell ref="E40:I40"/>
-    <mergeCell ref="C97:I97"/>
     <mergeCell ref="A19:I19"/>
+    <mergeCell ref="A48:I48"/>
     <mergeCell ref="E26:I26"/>
-    <mergeCell ref="A103:I103"/>
+    <mergeCell ref="A59:I59"/>
     <mergeCell ref="E25:I25"/>
     <mergeCell ref="C95:I95"/>
     <mergeCell ref="C60:I60"/>
@@ -3216,33 +3336,30 @@
     <mergeCell ref="E42:I42"/>
     <mergeCell ref="C91:I91"/>
     <mergeCell ref="A105:I105"/>
-    <mergeCell ref="C57:I57"/>
     <mergeCell ref="C66:I66"/>
+    <mergeCell ref="E44:I44"/>
+    <mergeCell ref="C102:I102"/>
     <mergeCell ref="E20:I20"/>
     <mergeCell ref="E28:I28"/>
     <mergeCell ref="C77:I77"/>
     <mergeCell ref="C86:I86"/>
     <mergeCell ref="C68:I68"/>
-    <mergeCell ref="A100:I100"/>
-    <mergeCell ref="C58:I58"/>
     <mergeCell ref="E30:I30"/>
     <mergeCell ref="E22:I22"/>
-    <mergeCell ref="A93:I93"/>
     <mergeCell ref="E46:I46"/>
-    <mergeCell ref="A102:I102"/>
     <mergeCell ref="C85:I85"/>
+    <mergeCell ref="C100:I100"/>
     <mergeCell ref="C94:I94"/>
     <mergeCell ref="C65:I65"/>
     <mergeCell ref="C75:I75"/>
     <mergeCell ref="C84:I84"/>
+    <mergeCell ref="E57:I57"/>
     <mergeCell ref="C80:I80"/>
     <mergeCell ref="E54:I54"/>
     <mergeCell ref="E32:I32"/>
-    <mergeCell ref="C59:I59"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="E41:I41"/>
-    <mergeCell ref="A45:I45"/>
-    <mergeCell ref="E47:I47"/>
+    <mergeCell ref="E56:I56"/>
     <mergeCell ref="C61:I61"/>
     <mergeCell ref="E43:I43"/>
     <mergeCell ref="C70:I70"/>
@@ -3251,8 +3368,12 @@
     <mergeCell ref="A3:I3"/>
     <mergeCell ref="A104:I104"/>
     <mergeCell ref="E35:I35"/>
+    <mergeCell ref="C101:I101"/>
+    <mergeCell ref="A106:I106"/>
     <mergeCell ref="C74:I74"/>
     <mergeCell ref="C88:I88"/>
+    <mergeCell ref="E45:I45"/>
+    <mergeCell ref="C99:I99"/>
     <mergeCell ref="E37:I37"/>
     <mergeCell ref="E21:I21"/>
     <mergeCell ref="E23:I23"/>
@@ -3260,10 +3381,10 @@
     <mergeCell ref="C81:I81"/>
     <mergeCell ref="C69:I69"/>
     <mergeCell ref="E51:I51"/>
-    <mergeCell ref="C96:I96"/>
     <mergeCell ref="C78:I78"/>
     <mergeCell ref="C87:I87"/>
     <mergeCell ref="C62:I62"/>
+    <mergeCell ref="A97:I97"/>
     <mergeCell ref="C98:I98"/>
     <mergeCell ref="C89:I89"/>
     <mergeCell ref="E34:I34"/>
@@ -3274,6 +3395,8 @@
     <mergeCell ref="E27:I27"/>
     <mergeCell ref="E36:I36"/>
     <mergeCell ref="C63:I63"/>
+    <mergeCell ref="C93:I93"/>
+    <mergeCell ref="A107:I107"/>
     <mergeCell ref="C90:I90"/>
     <mergeCell ref="E53:I53"/>
     <mergeCell ref="C76:I76"/>
@@ -3306,7 +3429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P98"/>
+  <dimension ref="A1:P101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -8003,7 +8126,7 @@
         <is>
           <t>[2026-10-12] 新增：2026-10-12 用戶決定。綁定的持有證明由「在藍牙範圍內」提供，取代上一版的熱點綁定碼。橋接清單要改：原生配網由 NEHotspotConfiguration／WifiNetworkSpecifier 改為藍牙（例如 Capacitor BLE 插件或 Espressif 的 ESP Provisioning iOS/Android 庫）。iOS 要 NSBluetoothAlwaysUsageDescription。純瀏覽器只有桌面和 Android 的 Chrome 有 Web Bluetooth，iPhone Safari 沒有，所以網頁版不能配網。
 [2026-10-12] 2026-10-12（路線圖）：用戶第一次設定時設備還沒有 Wi-Fi，藍牙配網不能經 OTA 補上，所以必須包含在 11/27 交 Spotpear 量產燒錄的共用出廠韌體裡；藍牙佔用的分區大小要在 11/13 分區表凍結（P2-12）前確定。趕不上的話，量產機只能用 SoftAP 熱點配網，或在玩具廠工位經工廠 Wi-Fi 做一次 OTA。
-[2026-10-13] 2026-10-13 量度（分支 r-21-ble-provisioning，測試版 spotpear-ai-toy-bleprobe，Espressif wifi_provisioning BLE + security 1）：韌體 1,585,162 → 2,254,868 bytes（+670KB，超出 2MB app 分區，P2-12 必須改 4MB，partition_4m.csv 已編譯通過）；靜態 RAM 57,0→78,1KB（+21KB）。62:70 實機：開 WiFi STA 後 heap 153.8KB，藍牙廣播中 89.2KB（最大塊 69.6KB）。仍未量：藍牙開著時連 WiFi + HTTPS 的最低 heap（決定綁定結果經藍牙回傳還是由 App 查伺服器）。協定選 Espressif 標準，Neo 可用官方 ESP Provisioning iOS/Android 庫，綁定票走自訂 endpoint。
+[2026-10-13] 2026-10-13 量度（分支 r-21-ble-provisioning，測試版 spotpear-ai-toy-bleprobe，Espressif wifi_provisioning BLE + security 1）：韌體 1,585,162 → 2,254,868 bytes（+670KB，超出 2MB app 分區，P2-12 必須改 4MB，partition_4m.csv 已編譯通過）；靜態 RAM 57,0→78,1KB（+21KB）。62:70 實機：開 WiFi STA 後 heap 153.8KB，藍牙廣播中 89.2KB（最大塊 69.6KB）。仍未量：藍牙開著時連 WiFi + HTTPS 的最低 heap（決定綁定結果經藍牙回傳還是由 App 查伺服器）。協定選 Espressif 標準，App 殼負責人（待定）可用官方 ESP Provisioning iOS/Android 庫，綁定票走自訂 endpoint。
 [2026-10-13] 更正上一條：靜態 RAM 56,988 → 78,092 bytes（+21KB）。</t>
         </is>
       </c>
@@ -8208,7 +8331,7 @@
         </is>
       </c>
     </row>
-    <row r="67" ht="116" customHeight="1">
+    <row r="67" ht="284" customHeight="1">
       <c r="A67" s="13" t="inlineStr">
         <is>
           <t>R-25</t>
@@ -8236,12 +8359,12 @@
       </c>
       <c r="F67" s="13" t="inlineStr">
         <is>
-          <t>未開始</t>
+          <t>進行中</t>
         </is>
       </c>
       <c r="G67" s="13" t="inlineStr">
         <is>
-          <t>未測試</t>
+          <t>部分通過</t>
         </is>
       </c>
       <c r="I67" s="6" t="inlineStr">
@@ -8265,10 +8388,21 @@
         </is>
       </c>
       <c r="M67" s="13" t="n"/>
+      <c r="N67" s="6" t="inlineStr">
+        <is>
+          <t>分支 r-25-brand-themes（3e59883 + c6654ed，worktree aibuddy-brands）：同一個 next build 的 standalone server.js 以 BRAND=aibuddy/hkjc/genex 各啟動一次 → /login 標題『Login | AI Buddy／快活／GEN-EX』、SSR &lt;head&gt; 內 :root --brand-primary 各自不同（無閃爍）、標誌與標語對；cp -R genex zz-test 改 JSON、不改程式不重 build → 『Login | Test Brand』；BRAND=nope → 500 並記錄 brands/nope/brand.json does not exist；brand.json 填錯 → 500 並逐欄報錯。dev 實測 hkjc：設備預設名『快活』、中文加設備提示、無方案徽章、/home/account/child 404。grep 共用程式碼：無品牌名、無 AI Buddy 色值（剩韌體熱點前綴、JWT audience、seed 帳號等技術識別碼）。tsc 0 錯、next build 通過、node --test 22/22。未做：① 首頁、上手流程、角色頁的整頁品牌版本（只有文案、圖片、功能開關可按品牌）和圖片 logo，等設計負責人（待定）10/23 的設計；hkjc/genex 名稱、顏色、文案是佔位。</t>
+        </is>
+      </c>
+      <c r="O67" s="13" t="inlineStr">
+        <is>
+          <t>3e59883</t>
+        </is>
+      </c>
       <c r="P67" s="6" t="inlineStr">
         <is>
           <t>[2026-10-12] 新增
-[2026-10-12] 2026-10-12：品牌改由部署的環境變數決定，不再按網址判斷（三套分開部署，R-34）。</t>
+[2026-10-12] 2026-10-12：品牌改由部署的環境變數決定，不再按網址判斷（三套分開部署，R-34）。
+[2026-10-19] 品牌由執行時的 BRAND 環境變數決定（同一個 image 服務三個品牌）；另刪除 52 個沒有路由使用的 Elato 舊元件和約 30MB 無引用圖片。未合併 dev、未部署。</t>
         </is>
       </c>
     </row>
@@ -10071,7 +10205,7 @@
         </is>
       </c>
     </row>
-    <row r="93" ht="270" customHeight="1">
+    <row r="93" ht="368" customHeight="1">
       <c r="A93" s="13" t="inlineStr">
         <is>
           <t>P2-20</t>
@@ -10151,7 +10285,8 @@
         <is>
           <t>[2026-10-14] 新增
 [2026-10-14] 2026-10-14 用戶決定提前到第 2 階段，現在開始做
-[2026-10-14] 做法：韌體 OTA.cpp 加 BUILD_INFO 字串（kind=release/dev;board;version），伺服器從映像讀板型和版本，不用手填；DEV_MODE/LOCAL_WS_HOST/LOCAL_BACKEND_HOST/AUDIO_SELFTEST 為 dev。只有加了標記之後編譯的韌體能從後台上傳，之前的仍用 release_firmware.py。部署注意：① 網頁的 nginx location 很可能仍是預設 1MB 上限（/supabase-api/ 已改 16m），上傳 1.6MB 映像會 413，部署時要加 client_max_body_size 16m 並用 curl 驗證 ② 依賴 P1-10 的審計表（本機已有，線上隨 10-14 release 部署）</t>
+[2026-10-14] 做法：韌體 OTA.cpp 加 BUILD_INFO 字串（kind=release/dev;board;version），伺服器從映像讀板型和版本，不用手填；DEV_MODE/LOCAL_WS_HOST/LOCAL_BACKEND_HOST/AUDIO_SELFTEST 為 dev。只有加了標記之後編譯的韌體能從後台上傳，之前的仍用 release_firmware.py。部署注意：① 網頁的 nginx location 很可能仍是預設 1MB 上限（/supabase-api/ 已改 16m），上傳 1.6MB 映像會 413，部署時要加 client_max_body_size 16m 並用 curl 驗證 ② 依賴 P1-10 的審計表（本機已有，線上隨 10-14 release 部署）
+[2026-10-16] 部署：nginx 上傳上限已寫進上線腳本 step 3c（conf.d/00-upload-limit.conf，16m，nginx -t 後 reload，並以 2MB POST 驗證不是 413；step 5 再查一次），本機 nginx 容器測過 4 種情況。commit b1e9d20，未推送</t>
         </is>
       </c>
     </row>
@@ -10540,8 +10675,226 @@
         </is>
       </c>
     </row>
+    <row r="99" ht="256" customHeight="1">
+      <c r="A99" s="13" t="inlineStr">
+        <is>
+          <t>R-42</t>
+        </is>
+      </c>
+      <c r="B99" s="13" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="C99" s="13" t="inlineStr">
+        <is>
+          <t>3 封閉內測</t>
+        </is>
+      </c>
+      <c r="D99" s="6" t="inlineStr">
+        <is>
+          <t>語音</t>
+        </is>
+      </c>
+      <c r="E99" s="6" t="inlineStr">
+        <is>
+          <t>Tool call v1：調音量、結束對話</t>
+        </is>
+      </c>
+      <c r="F99" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="G99" s="13" t="inlineStr">
+        <is>
+          <t>部分通過</t>
+        </is>
+      </c>
+      <c r="I99" s="6" t="inlineStr">
+        <is>
+          <t>1/15 只做兩個工具（路線圖 10/13）。誤觸發會令玩具突然變細聲或者瞓覺；舊固件 1.0.1 唔認 volume 訊息、收到 RESPONSE.COMPLETE 後一秒內丟音頻。</t>
+        </is>
+      </c>
+      <c r="J99" s="6" t="inlineStr">
+        <is>
+          <t>server/fastapi/voice_tools.py、bot.py（SESSION.END、RESPONSE.COMPLETE 延後）、llm_output_guard.py、memory/processors.py、evals/voice_tools</t>
+        </is>
+      </c>
+      <c r="K99" s="6" t="inlineStr">
+        <is>
+          <t>① 兩個工具各用真實語音在玩具上觸發 20 次，成功率 ≥ 95% ② 不相關的話（其他嘢好大聲、故事入面講拜拜等）不會誤觸發 ③ 首字延遲增加不超過 300 毫秒 ④ 1.0.1 同新固件都即時變音量，網頁音量同步 ⑤ 道別講完先瞓覺，用戶再講嘢就取消 ⑥ 工具輪嘅記憶記錄正確</t>
+        </is>
+      </c>
+      <c r="L99" s="6" t="inlineStr">
+        <is>
+          <t>evals/voice_tools 用真實模型跑 cases.yaml（兩個模型 ×3）；simulate_device 本機端到端（--wait-session-end）；真機 62:70 每個工具真實語音 20 次，聽確認句音量、睇串口 SESSION.END</t>
+        </is>
+      </c>
+      <c r="M99" s="13" t="n"/>
+      <c r="N99" s="6" t="inlineStr">
+        <is>
+          <t>分支 tool-call-rag（e80784b、f24b809、f90a657，worktree aibuddy-tools）：evals/voice_tools 真實模型、伺服器提示詞同工具定義，每案 ×3：調音量 gemma 60/60、DeepSeek 59/60；結束對話 gemma 30/30＋50/50、DeepSeek 30/30＋49/50（唯一失敗係 DeepSeek 空回覆）；誤觸發 0/144（電視、鄰居、媽媽話我大聲、故事入面講拜拜等）。首字延遲：gemma 無增加（p50 856 vs 871ms），DeepSeek +150ms。本機端到端（simulate_device，Sinji 粵語錄音，7895 worktree 伺服器）：『你大聲啲啦』→ volume+auth 喺 RESPONSE.CREATED 前、70→85、devices.volume=85；『拜拜，我要瞓覺喇』→ 道別後 1.5s SESSION.END；記憶記錄三輪都正確。DeepSeek 先講『等我查吓先』再查：RESPONSE.COMPLETE 延後到答案講完（一個週期 22–33s 音頻）。pytest 325 passed。未做：真機 62:70 每個工具真實語音 20 次、合併 dev、部署。</t>
+        </is>
+      </c>
+      <c r="O99" s="13" t="inlineStr">
+        <is>
+          <t>f24b809</t>
+        </is>
+      </c>
+      <c r="P99" s="6" t="inlineStr">
+        <is>
+          <t>[2026-10-19] 新增</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" ht="158" customHeight="1">
+      <c r="A100" s="13" t="inlineStr">
+        <is>
+          <t>R-43</t>
+        </is>
+      </c>
+      <c r="B100" s="13" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="C100" s="13" t="inlineStr">
+        <is>
+          <t>4 量產出貨</t>
+        </is>
+      </c>
+      <c r="D100" s="6" t="inlineStr">
+        <is>
+          <t>語音</t>
+        </is>
+      </c>
+      <c r="E100" s="6" t="inlineStr">
+        <is>
+          <t>快活知識庫 RAG v1（檢索與回答）</t>
+        </is>
+      </c>
+      <c r="F100" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="G100" s="13" t="inlineStr">
+        <is>
+          <t>部分通過</t>
+        </is>
+      </c>
+      <c r="I100" s="6" t="inlineStr">
+        <is>
+          <t>快活只可以按馬會審核過嘅知識庫答（路線圖）。模型用自己知識補充或者畀貼士都係合規風險。</t>
+        </is>
+      </c>
+      <c r="J100" s="6" t="inlineStr">
+        <is>
+          <t>server/fastapi/knowledge.py、voice_tools.py search_knowledge、content/knowledge/（KNOWLEDGE_BASE_FILE）、evals/voice_tools</t>
+        </is>
+      </c>
+      <c r="K100" s="6" t="inlineStr">
+        <is>
+          <t>① v1 只放第一批馬會資料；設計負責人（待定）寫嘅 100 條測試問題答對率 ≥ 80% ② 知識庫冇嘅內容講唔肯定並建議查詢，唔自己作 ③ 問貼士、賠率、賽果預測 100% 婉拒 ④ 更新知識庫唔使重新燒錄玩具</t>
+        </is>
+      </c>
+      <c r="L100" s="6" t="inlineStr">
+        <is>
+          <t>用馬會資料重新量 MIN_SCORE；evals/voice_tools 加入 100 條測試問題同標準答案；檢查部分命中時唔補充知識庫以外嘅內容</t>
+        </is>
+      </c>
+      <c r="M100" s="13" t="inlineStr">
+        <is>
+          <t>R-42</t>
+        </is>
+      </c>
+      <c r="N100" s="6" t="inlineStr">
+        <is>
+          <t>BM25 檢索搬入伺服器（knowledge.py），KNOWLEDGE_BASE_FILE 指定，工具描述、查唔到嘅回覆、額外規則（唔畀貼士）都喺資料檔。用 13 條示範資料：evals/voice_tools 命中題 gemma 答對事實 12/12、DeepSeek 11–12/12；查唔到 → 固定句或者講唔清楚，冇自己作；貼士三題兩個模型都婉拒。已知問題：部分命中（沙田馬場有冇餐廳）DeepSeek 3 次有 2 次用自己知識補充（『係有餐廳㗎』），gemma 冇。未做：馬會資料、設計負責人（待定）100 條測試問題、MIN_SCORE 重新量、入庫審批流程。</t>
+        </is>
+      </c>
+      <c r="O100" s="13" t="inlineStr">
+        <is>
+          <t>e80784b</t>
+        </is>
+      </c>
+      <c r="P100" s="6" t="inlineStr">
+        <is>
+          <t>[2026-10-19] 新增
+[2026-10-20] 2026-10-20 用戶同意先用 Excel 收資料：docs/knowledge/快活知識庫_範本.xlsx + scripts/knowledge_excel.py（check／import，測試問題只測檢索）。示範資料 + 96 條口語測試：62/88（70%），換講法 6/28。後台頁面另立 R-44。</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" ht="116" customHeight="1">
+      <c r="A101" s="13" t="inlineStr">
+        <is>
+          <t>R-44</t>
+        </is>
+      </c>
+      <c r="B101" s="13" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="C101" s="13" t="inlineStr">
+        <is>
+          <t>3 封閉內測</t>
+        </is>
+      </c>
+      <c r="D101" s="6" t="inlineStr">
+        <is>
+          <t>後台</t>
+        </is>
+      </c>
+      <c r="E101" s="6" t="inlineStr">
+        <is>
+          <t>知識庫後台頁面與審批流程</t>
+        </is>
+      </c>
+      <c r="F101" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="G101" s="13" t="inlineStr">
+        <is>
+          <t>未測試</t>
+        </is>
+      </c>
+      <c r="I101" s="6" t="inlineStr">
+        <is>
+          <t>Excel 階段（scripts/knowledge_excel.py）只適合少量人手更新；要有版本、送審、批准、發佈同回滾記錄，馬會先肯簽，更新知識庫亦唔使重開伺服器或者燒錄玩具。</t>
+        </is>
+      </c>
+      <c r="J101" s="6" t="inlineStr">
+        <is>
+          <t>frontend-nextjs Admin（內容管理員角色、P1-10 審計）、快活嗰套 Supabase 新表（kb_versions、kb_entries、kb_aliases）、server/fastapi/knowledge.py 改為讀已發佈版本</t>
+        </is>
+      </c>
+      <c r="K101" s="6" t="inlineStr">
+        <is>
+          <t>① 內容管理員可以列出、搜尋、編輯條目，亦可以直接匯入 Excel 範本 ② 「試問一句」即時顯示命中邊條、分數、模型會收到咩 ③ 版本：草稿 → 送審 → 批准 → 發佈，每步記錄邊個、幾時；兩個版本可以比較差異，可以回滾 ④ 發佈後語音伺服器喺下一個對話開始用新版本，唔使重開 ⑤ 每個版本可以匯出 Excel／PDF 俾馬會簽批，批准人同日期記入後台 ⑥ 知識庫資料只存喺快活自己嗰套 Supabase</t>
+        </is>
+      </c>
+      <c r="L101" s="6" t="inlineStr">
+        <is>
+          <t>本機：匯入範本 → 送審 → 批准 → 發佈，網頁 playground 問一條新加嘅問題答得到；回滾後答返舊版本；非內容管理員讀寫 → 42501；審計記錄每一步</t>
+        </is>
+      </c>
+      <c r="M101" s="13" t="inlineStr">
+        <is>
+          <t>P1-10</t>
+        </is>
+      </c>
+      <c r="P101" s="6" t="inlineStr">
+        <is>
+          <t>[2026-10-20] 新增</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P98"/>
+  <autoFilter ref="A1:P101"/>
   <conditionalFormatting sqref="F2:F1000">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"已完成"</formula>
@@ -11122,7 +11475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I324"/>
+  <dimension ref="A1:I338"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -18639,7 +18992,7 @@
       <c r="H217" s="13" t="n"/>
       <c r="I217" s="6" t="inlineStr">
         <is>
-          <t>2026-10-13 量度（分支 r-21-ble-provisioning，測試版 spotpear-ai-toy-bleprobe，Espressif wifi_provisioning BLE + security 1）：韌體 1,585,162 → 2,254,868 bytes（+670KB，超出 2MB app 分區，P2-12 必須改 4MB，partition_4m.csv 已編譯通過）；靜態 RAM 57,0→78,1KB（+21KB）。62:70 實機：開 WiFi STA 後 heap 153.8KB，藍牙廣播中 89.2KB（最大塊 69.6KB）。仍未量：藍牙開著時連 WiFi + HTTPS 的最低 heap（決定綁定結果經藍牙回傳還是由 App 查伺服器）。協定選 Espressif 標準，Neo 可用官方 ESP Provisioning iOS/Android 庫，綁定票走自訂 endpoint。</t>
+          <t>2026-10-13 量度（分支 r-21-ble-provisioning，測試版 spotpear-ai-toy-bleprobe，Espressif wifi_provisioning BLE + security 1）：韌體 1,585,162 → 2,254,868 bytes（+670KB，超出 2MB app 分區，P2-12 必須改 4MB，partition_4m.csv 已編譯通過）；靜態 RAM 57,0→78,1KB（+21KB）。62:70 實機：開 WiFi STA 後 heap 153.8KB，藍牙廣播中 89.2KB（最大塊 69.6KB）。仍未量：藍牙開著時連 WiFi + HTTPS 的最低 heap（決定綁定結果經藍牙回傳還是由 App 查伺服器）。協定選 Espressif 標準，App 殼負責人（待定）可用官方 ESP Provisioning iOS/Android 庫，綁定票走自訂 endpoint。</t>
         </is>
       </c>
     </row>
@@ -22448,8 +22801,490 @@
         </is>
       </c>
     </row>
+    <row r="325" ht="88" customHeight="1">
+      <c r="A325" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-16 10:04</t>
+        </is>
+      </c>
+      <c r="B325" s="13" t="inlineStr">
+        <is>
+          <t>P2-20</t>
+        </is>
+      </c>
+      <c r="C325" s="6" t="inlineStr">
+        <is>
+          <t>P2-16 ④ 從後台上傳與發佈韌體（取代手貼 service key）</t>
+        </is>
+      </c>
+      <c r="D325" s="13" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="E325" s="13" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="F325" s="13" t="n"/>
+      <c r="G325" s="6" t="n"/>
+      <c r="H325" s="13" t="n"/>
+      <c r="I325" s="6" t="inlineStr">
+        <is>
+          <t>部署：nginx 上傳上限已寫進上線腳本 step 3c（conf.d/00-upload-limit.conf，16m，nginx -t 後 reload，並以 2MB POST 驗證不是 413；step 5 再查一次），本機 nginx 容器測過 4 種情況。commit b1e9d20，未推送</t>
+        </is>
+      </c>
+    </row>
+    <row r="326" ht="32" customHeight="1">
+      <c r="A326" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-19 11:57</t>
+        </is>
+      </c>
+      <c r="B326" s="13" t="inlineStr">
+        <is>
+          <t>R-25</t>
+        </is>
+      </c>
+      <c r="C326" s="6" t="inlineStr">
+        <is>
+          <t>網頁的品牌主題系統</t>
+        </is>
+      </c>
+      <c r="D326" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E326" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F326" s="13" t="n"/>
+      <c r="G326" s="6" t="n"/>
+      <c r="H326" s="13" t="n"/>
+      <c r="I326" s="6" t="n"/>
+    </row>
+    <row r="327" ht="256" customHeight="1">
+      <c r="A327" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-19 11:57</t>
+        </is>
+      </c>
+      <c r="B327" s="13" t="inlineStr">
+        <is>
+          <t>R-25</t>
+        </is>
+      </c>
+      <c r="C327" s="6" t="inlineStr">
+        <is>
+          <t>網頁的品牌主題系統</t>
+        </is>
+      </c>
+      <c r="D327" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="E327" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F327" s="13" t="inlineStr">
+        <is>
+          <t>部分通過</t>
+        </is>
+      </c>
+      <c r="G327" s="6" t="inlineStr">
+        <is>
+          <t>分支 r-25-brand-themes（3e59883 + c6654ed，worktree aibuddy-brands）：同一個 next build 的 standalone server.js 以 BRAND=aibuddy/hkjc/genex 各啟動一次 → /login 標題『Login | AI Buddy／快活／GEN-EX』、SSR &lt;head&gt; 內 :root --brand-primary 各自不同（無閃爍）、標誌與標語對；cp -R genex zz-test 改 JSON、不改程式不重 build → 『Login | Test Brand』；BRAND=nope → 500 並記錄 brands/nope/brand.json does not exist；brand.json 填錯 → 500 並逐欄報錯。dev 實測 hkjc：設備預設名『快活』、中文加設備提示、無方案徽章、/home/account/child 404。grep 共用程式碼：無品牌名、無 AI Buddy 色值（剩韌體熱點前綴、JWT audience、seed 帳號等技術識別碼）。tsc 0 錯、next build 通過、node --test 22/22。未做：① 首頁、上手流程、角色頁的整頁品牌版本（只有文案、圖片、功能開關可按品牌）和圖片 logo，等設計負責人（待定）10/23 的設計；hkjc/genex 名稱、顏色、文案是佔位。</t>
+        </is>
+      </c>
+      <c r="H327" s="13" t="inlineStr">
+        <is>
+          <t>3e59883</t>
+        </is>
+      </c>
+      <c r="I327" s="6" t="inlineStr">
+        <is>
+          <t>品牌由執行時的 BRAND 環境變數決定（同一個 image 服務三個品牌）；另刪除 52 個沒有路由使用的 Elato 舊元件和約 30MB 無引用圖片。未合併 dev、未部署。</t>
+        </is>
+      </c>
+    </row>
+    <row r="328" ht="32" customHeight="1">
+      <c r="A328" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-19 12:57</t>
+        </is>
+      </c>
+      <c r="B328" s="13" t="inlineStr">
+        <is>
+          <t>R-42</t>
+        </is>
+      </c>
+      <c r="C328" s="6" t="inlineStr">
+        <is>
+          <t>Tool call v1：調音量、結束對話</t>
+        </is>
+      </c>
+      <c r="E328" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="I328" s="6" t="inlineStr">
+        <is>
+          <t>新增任務</t>
+        </is>
+      </c>
+    </row>
+    <row r="329" ht="32" customHeight="1">
+      <c r="A329" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-19 12:57</t>
+        </is>
+      </c>
+      <c r="B329" s="13" t="inlineStr">
+        <is>
+          <t>R-43</t>
+        </is>
+      </c>
+      <c r="C329" s="6" t="inlineStr">
+        <is>
+          <t>快活知識庫 RAG v1（檢索與回答）</t>
+        </is>
+      </c>
+      <c r="E329" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="I329" s="6" t="inlineStr">
+        <is>
+          <t>新增任務</t>
+        </is>
+      </c>
+    </row>
+    <row r="330" ht="32" customHeight="1">
+      <c r="A330" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-19 12:58</t>
+        </is>
+      </c>
+      <c r="B330" s="13" t="inlineStr">
+        <is>
+          <t>R-42</t>
+        </is>
+      </c>
+      <c r="C330" s="6" t="inlineStr">
+        <is>
+          <t>Tool call v1：調音量、結束對話</t>
+        </is>
+      </c>
+      <c r="D330" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E330" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F330" s="13" t="n"/>
+      <c r="G330" s="6" t="n"/>
+      <c r="H330" s="13" t="n"/>
+      <c r="I330" s="6" t="n"/>
+    </row>
+    <row r="331" ht="228" customHeight="1">
+      <c r="A331" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-19 12:58</t>
+        </is>
+      </c>
+      <c r="B331" s="13" t="inlineStr">
+        <is>
+          <t>R-42</t>
+        </is>
+      </c>
+      <c r="C331" s="6" t="inlineStr">
+        <is>
+          <t>Tool call v1：調音量、結束對話</t>
+        </is>
+      </c>
+      <c r="D331" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="E331" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F331" s="13" t="inlineStr">
+        <is>
+          <t>部分通過</t>
+        </is>
+      </c>
+      <c r="G331" s="6" t="inlineStr">
+        <is>
+          <t>分支 tool-call-rag（e80784b、f24b809、f90a657，worktree aibuddy-tools）：evals/voice_tools 真實模型、伺服器提示詞同工具定義，每案 ×3：調音量 gemma 60/60、DeepSeek 59/60；結束對話 gemma 30/30＋50/50、DeepSeek 30/30＋49/50（唯一失敗係 DeepSeek 空回覆）；誤觸發 0/144（電視、鄰居、媽媽話我大聲、故事入面講拜拜等）。首字延遲：gemma 無增加（p50 856 vs 871ms），DeepSeek +150ms。本機端到端（simulate_device，Sinji 粵語錄音，7895 worktree 伺服器）：『你大聲啲啦』→ volume+auth 喺 RESPONSE.CREATED 前、70→85、devices.volume=85；『拜拜，我要瞓覺喇』→ 道別後 1.5s SESSION.END；記憶記錄三輪都正確。DeepSeek 先講『等我查吓先』再查：RESPONSE.COMPLETE 延後到答案講完（一個週期 22–33s 音頻）。pytest 325 passed。未做：真機 62:70 每個工具真實語音 20 次、合併 dev、部署。</t>
+        </is>
+      </c>
+      <c r="H331" s="13" t="inlineStr">
+        <is>
+          <t>f24b809</t>
+        </is>
+      </c>
+      <c r="I331" s="6" t="n"/>
+    </row>
+    <row r="332" ht="32" customHeight="1">
+      <c r="A332" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-19 12:58</t>
+        </is>
+      </c>
+      <c r="B332" s="13" t="inlineStr">
+        <is>
+          <t>R-43</t>
+        </is>
+      </c>
+      <c r="C332" s="6" t="inlineStr">
+        <is>
+          <t>快活知識庫 RAG v1（檢索與回答）</t>
+        </is>
+      </c>
+      <c r="D332" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E332" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F332" s="13" t="n"/>
+      <c r="G332" s="6" t="n"/>
+      <c r="H332" s="13" t="n"/>
+      <c r="I332" s="6" t="n"/>
+    </row>
+    <row r="333" ht="144" customHeight="1">
+      <c r="A333" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-19 12:58</t>
+        </is>
+      </c>
+      <c r="B333" s="13" t="inlineStr">
+        <is>
+          <t>R-43</t>
+        </is>
+      </c>
+      <c r="C333" s="6" t="inlineStr">
+        <is>
+          <t>快活知識庫 RAG v1（檢索與回答）</t>
+        </is>
+      </c>
+      <c r="D333" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="E333" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F333" s="13" t="inlineStr">
+        <is>
+          <t>部分通過</t>
+        </is>
+      </c>
+      <c r="G333" s="6" t="inlineStr">
+        <is>
+          <t>BM25 檢索搬入伺服器（knowledge.py），KNOWLEDGE_BASE_FILE 指定，工具描述、查唔到嘅回覆、額外規則（唔畀貼士）都喺資料檔。用 13 條示範資料：evals/voice_tools 命中題 gemma 答對事實 12/12、DeepSeek 11–12/12；查唔到 → 固定句或者講唔清楚，冇自己作；貼士三題兩個模型都婉拒。已知問題：部分命中（沙田馬場有冇餐廳）DeepSeek 3 次有 2 次用自己知識補充（『係有餐廳㗎』），gemma 冇。未做：馬會資料、設計負責人（待定）100 條測試問題、MIN_SCORE 重新量、入庫審批流程。</t>
+        </is>
+      </c>
+      <c r="H333" s="13" t="inlineStr">
+        <is>
+          <t>e80784b</t>
+        </is>
+      </c>
+      <c r="I333" s="6" t="n"/>
+    </row>
+    <row r="334" ht="32" customHeight="1">
+      <c r="A334" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-19 12:58</t>
+        </is>
+      </c>
+      <c r="B334" s="13" t="inlineStr">
+        <is>
+          <t>R-43</t>
+        </is>
+      </c>
+      <c r="C334" s="6" t="inlineStr">
+        <is>
+          <t>快活知識庫 RAG v1（檢索與回答）</t>
+        </is>
+      </c>
+      <c r="D334" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="E334" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F334" s="13" t="n"/>
+      <c r="G334" s="6" t="n"/>
+      <c r="H334" s="13" t="n"/>
+      <c r="I334" s="6" t="inlineStr">
+        <is>
+          <t>修改了依賴→R-42</t>
+        </is>
+      </c>
+    </row>
+    <row r="335" ht="32" customHeight="1">
+      <c r="A335" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-19 12:58</t>
+        </is>
+      </c>
+      <c r="B335" s="13" t="inlineStr">
+        <is>
+          <t>R-43</t>
+        </is>
+      </c>
+      <c r="C335" s="6" t="inlineStr">
+        <is>
+          <t>快活知識庫 RAG v1（檢索與回答）</t>
+        </is>
+      </c>
+      <c r="D335" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="E335" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F335" s="13" t="n"/>
+      <c r="G335" s="6" t="n"/>
+      <c r="H335" s="13" t="n"/>
+      <c r="I335" s="6" t="inlineStr">
+        <is>
+          <t>修改了依賴→</t>
+        </is>
+      </c>
+    </row>
+    <row r="336" ht="32" customHeight="1">
+      <c r="A336" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-20 16:45</t>
+        </is>
+      </c>
+      <c r="B336" s="13" t="inlineStr">
+        <is>
+          <t>R-44</t>
+        </is>
+      </c>
+      <c r="C336" s="6" t="inlineStr">
+        <is>
+          <t>知識庫後台頁面與審批流程</t>
+        </is>
+      </c>
+      <c r="E336" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="I336" s="6" t="inlineStr">
+        <is>
+          <t>新增任務</t>
+        </is>
+      </c>
+    </row>
+    <row r="337" ht="32" customHeight="1">
+      <c r="A337" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-20 16:45</t>
+        </is>
+      </c>
+      <c r="B337" s="13" t="inlineStr">
+        <is>
+          <t>R-44</t>
+        </is>
+      </c>
+      <c r="C337" s="6" t="inlineStr">
+        <is>
+          <t>知識庫後台頁面與審批流程</t>
+        </is>
+      </c>
+      <c r="D337" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="E337" s="13" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="F337" s="13" t="n"/>
+      <c r="G337" s="6" t="n"/>
+      <c r="H337" s="13" t="n"/>
+      <c r="I337" s="6" t="inlineStr">
+        <is>
+          <t>修改了依賴→P1-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="338" ht="102" customHeight="1">
+      <c r="A338" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-20 16:45</t>
+        </is>
+      </c>
+      <c r="B338" s="13" t="inlineStr">
+        <is>
+          <t>R-43</t>
+        </is>
+      </c>
+      <c r="C338" s="6" t="inlineStr">
+        <is>
+          <t>快活知識庫 RAG v1（檢索與回答）</t>
+        </is>
+      </c>
+      <c r="D338" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="E338" s="13" t="inlineStr">
+        <is>
+          <t>進行中</t>
+        </is>
+      </c>
+      <c r="F338" s="13" t="n"/>
+      <c r="G338" s="6" t="n"/>
+      <c r="H338" s="13" t="n"/>
+      <c r="I338" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-20 用戶同意先用 Excel 收資料：docs/knowledge/快活知識庫_範本.xlsx + scripts/knowledge_excel.py（check／import，測試問題只測檢索）。示範資料 + 96 條口語測試：62/88（70%），換講法 6/28。後台頁面另立 R-44。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I324"/>
+  <autoFilter ref="A1:I338"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>